<commit_message>
Atualização automática: pagamentos (08/07/2026 14:38)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/01_Bases_Originais/005_CELOG_2025/005_CELOG-PAMALS_2025 online.xlsx
+++ b/Contrato 005/Dashboard/01_Bases_Originais/005_CELOG_2025/005_CELOG-PAMALS_2025 online.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="201">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="200">
   <si>
     <t>Controle de pagamentos</t>
   </si>
@@ -403,7 +403,7 @@
     <t>Módulo III – Orçamento 19 GPS</t>
   </si>
   <si>
-    <t>Aprovado e aguardando itens.</t>
+    <t>2025NE001065</t>
   </si>
   <si>
     <t>Saldo</t>
@@ -636,9 +636,6 @@
   </si>
   <si>
     <t>219C</t>
-  </si>
-  <si>
-    <t>2025NE001065</t>
   </si>
   <si>
     <r>
@@ -3210,13 +3207,19 @@
         <v>122</v>
       </c>
       <c r="E39" s="56"/>
-      <c r="F39" s="56"/>
-      <c r="G39" s="60"/>
-      <c r="H39" s="56"/>
-      <c r="I39" s="61" t="s">
+      <c r="F39" s="56">
+        <v>1882.0</v>
+      </c>
+      <c r="G39" s="60">
+        <v>46199.0</v>
+      </c>
+      <c r="H39" s="56" t="s">
         <v>123</v>
       </c>
-      <c r="J39" s="60"/>
+      <c r="I39" s="61"/>
+      <c r="J39" s="60">
+        <v>46233.0</v>
+      </c>
       <c r="K39" s="36">
         <v>58868.35</v>
       </c>
@@ -8645,13 +8648,13 @@
     </row>
     <row r="13">
       <c r="A13" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="B13" s="12" t="s">
         <v>157</v>
       </c>
-      <c r="B13" s="12" t="s">
+      <c r="C13" s="12" t="s">
         <v>158</v>
-      </c>
-      <c r="C13" s="12" t="s">
-        <v>159</v>
       </c>
       <c r="D13" s="12" t="s">
         <v>127</v>
@@ -8694,10 +8697,10 @@
         <v>59</v>
       </c>
       <c r="B14" s="12" t="s">
+        <v>159</v>
+      </c>
+      <c r="C14" s="12" t="s">
         <v>160</v>
-      </c>
-      <c r="C14" s="12" t="s">
-        <v>161</v>
       </c>
       <c r="D14" s="12" t="s">
         <v>127</v>
@@ -8736,13 +8739,13 @@
     </row>
     <row r="15">
       <c r="A15" s="12" t="s">
+        <v>161</v>
+      </c>
+      <c r="B15" s="12" t="s">
         <v>162</v>
       </c>
-      <c r="B15" s="12" t="s">
+      <c r="C15" s="12" t="s">
         <v>163</v>
-      </c>
-      <c r="C15" s="12" t="s">
-        <v>164</v>
       </c>
       <c r="D15" s="12" t="s">
         <v>127</v>
@@ -8781,13 +8784,13 @@
     </row>
     <row r="16">
       <c r="A16" s="12" t="s">
+        <v>164</v>
+      </c>
+      <c r="B16" s="12" t="s">
         <v>165</v>
       </c>
-      <c r="B16" s="12" t="s">
+      <c r="C16" s="12" t="s">
         <v>166</v>
-      </c>
-      <c r="C16" s="12" t="s">
-        <v>167</v>
       </c>
       <c r="D16" s="12" t="s">
         <v>127</v>
@@ -8826,13 +8829,13 @@
     </row>
     <row r="17">
       <c r="A17" s="12" t="s">
+        <v>167</v>
+      </c>
+      <c r="B17" s="12" t="s">
         <v>168</v>
       </c>
-      <c r="B17" s="12" t="s">
+      <c r="C17" s="12" t="s">
         <v>169</v>
-      </c>
-      <c r="C17" s="12" t="s">
-        <v>170</v>
       </c>
       <c r="D17" s="12" t="s">
         <v>127</v>
@@ -8874,10 +8877,10 @@
         <v>110</v>
       </c>
       <c r="B18" s="12" t="s">
+        <v>170</v>
+      </c>
+      <c r="C18" s="12" t="s">
         <v>171</v>
-      </c>
-      <c r="C18" s="12" t="s">
-        <v>172</v>
       </c>
       <c r="D18" s="12" t="s">
         <v>127</v>
@@ -8916,13 +8919,13 @@
     </row>
     <row r="19">
       <c r="A19" s="12" t="s">
+        <v>172</v>
+      </c>
+      <c r="B19" s="12" t="s">
         <v>173</v>
       </c>
-      <c r="B19" s="12" t="s">
+      <c r="C19" s="12" t="s">
         <v>174</v>
-      </c>
-      <c r="C19" s="12" t="s">
-        <v>175</v>
       </c>
       <c r="D19" s="12" t="s">
         <v>127</v>
@@ -8961,13 +8964,13 @@
     </row>
     <row r="20">
       <c r="A20" s="12" t="s">
+        <v>175</v>
+      </c>
+      <c r="B20" s="12" t="s">
         <v>176</v>
       </c>
-      <c r="B20" s="12" t="s">
+      <c r="C20" s="12" t="s">
         <v>177</v>
-      </c>
-      <c r="C20" s="12" t="s">
-        <v>178</v>
       </c>
       <c r="D20" s="12" t="s">
         <v>127</v>
@@ -9006,13 +9009,13 @@
     </row>
     <row r="21">
       <c r="A21" s="12" t="s">
+        <v>178</v>
+      </c>
+      <c r="B21" s="12" t="s">
         <v>179</v>
       </c>
-      <c r="B21" s="12" t="s">
+      <c r="C21" s="12" t="s">
         <v>180</v>
-      </c>
-      <c r="C21" s="12" t="s">
-        <v>181</v>
       </c>
       <c r="D21" s="12" t="s">
         <v>127</v>
@@ -9054,10 +9057,10 @@
         <v>74</v>
       </c>
       <c r="B22" s="12" t="s">
+        <v>181</v>
+      </c>
+      <c r="C22" s="12" t="s">
         <v>182</v>
-      </c>
-      <c r="C22" s="12" t="s">
-        <v>183</v>
       </c>
       <c r="D22" s="12" t="s">
         <v>127</v>
@@ -9099,10 +9102,10 @@
         <v>114</v>
       </c>
       <c r="B23" s="12" t="s">
+        <v>183</v>
+      </c>
+      <c r="C23" s="12" t="s">
         <v>184</v>
-      </c>
-      <c r="C23" s="12" t="s">
-        <v>185</v>
       </c>
       <c r="D23" s="12" t="s">
         <v>127</v>
@@ -9120,7 +9123,7 @@
         <v>339039.0</v>
       </c>
       <c r="I23" s="12" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="J23" s="14">
         <v>1000001.64</v>
@@ -9141,13 +9144,13 @@
     </row>
     <row r="24">
       <c r="A24" s="12" t="s">
+        <v>186</v>
+      </c>
+      <c r="B24" s="12" t="s">
         <v>187</v>
       </c>
-      <c r="B24" s="12" t="s">
+      <c r="C24" s="12" t="s">
         <v>188</v>
-      </c>
-      <c r="C24" s="12" t="s">
-        <v>189</v>
       </c>
       <c r="D24" s="12" t="s">
         <v>127</v>
@@ -9189,10 +9192,10 @@
         <v>105</v>
       </c>
       <c r="B25" s="12" t="s">
+        <v>189</v>
+      </c>
+      <c r="C25" s="12" t="s">
         <v>190</v>
-      </c>
-      <c r="C25" s="12" t="s">
-        <v>191</v>
       </c>
       <c r="D25" s="12" t="s">
         <v>127</v>
@@ -9210,7 +9213,7 @@
         <v>339039.0</v>
       </c>
       <c r="I25" s="12" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="J25" s="14">
         <v>1157673.06</v>
@@ -9231,13 +9234,13 @@
     </row>
     <row r="26">
       <c r="A26" s="12" t="s">
+        <v>191</v>
+      </c>
+      <c r="B26" s="12" t="s">
         <v>192</v>
       </c>
-      <c r="B26" s="12" t="s">
+      <c r="C26" s="12" t="s">
         <v>193</v>
-      </c>
-      <c r="C26" s="12" t="s">
-        <v>194</v>
       </c>
       <c r="D26" s="12" t="s">
         <v>127</v>
@@ -9276,13 +9279,13 @@
     </row>
     <row r="27">
       <c r="A27" s="12" t="s">
+        <v>194</v>
+      </c>
+      <c r="B27" s="12" t="s">
         <v>195</v>
       </c>
-      <c r="B27" s="12" t="s">
+      <c r="C27" s="12" t="s">
         <v>196</v>
-      </c>
-      <c r="C27" s="12" t="s">
-        <v>197</v>
       </c>
       <c r="D27" s="12" t="s">
         <v>127</v>
@@ -9321,13 +9324,13 @@
     </row>
     <row r="28">
       <c r="A28" s="12" t="s">
+        <v>197</v>
+      </c>
+      <c r="B28" s="12" t="s">
         <v>198</v>
       </c>
-      <c r="B28" s="12" t="s">
+      <c r="C28" s="12" t="s">
         <v>199</v>
-      </c>
-      <c r="C28" s="12" t="s">
-        <v>200</v>
       </c>
       <c r="D28" s="12" t="s">
         <v>127</v>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (09/07/2026 10:29)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/01_Bases_Originais/005_CELOG_2025/005_CELOG-PAMALS_2025 online.xlsx
+++ b/Contrato 005/Dashboard/01_Bases_Originais/005_CELOG_2025/005_CELOG-PAMALS_2025 online.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="198">
   <si>
     <t>Controle de pagamentos</t>
   </si>
@@ -412,14 +412,7 @@
     <t>2025NE000005</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <color rgb="FF1155CC"/>
-        <u/>
-      </rPr>
-      <t>C25375</t>
-    </r>
+    <t>C25375</t>
   </si>
   <si>
     <t>Ordenador de Despesas</t>
@@ -431,93 +424,34 @@
     <t>2025NE000367</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <color rgb="FF1155CC"/>
-        <u/>
-      </rPr>
-      <t>C25512</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <color rgb="FF1155CC"/>
-        <u/>
-      </rPr>
-      <t>25E0385</t>
-    </r>
+    <t>C25512</t>
+  </si>
+  <si>
+    <t>25E0385</t>
   </si>
   <si>
     <t>2025NE000369</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <color rgb="FF1155CC"/>
-        <u/>
-      </rPr>
-      <t>C25516</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <color rgb="FF1155CC"/>
-        <u/>
-      </rPr>
-      <t>25E0387</t>
-    </r>
+    <t>C25516</t>
+  </si>
+  <si>
+    <t>25E0387</t>
   </si>
   <si>
     <t>2025NE000371</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <color rgb="FF1155CC"/>
-        <u/>
-      </rPr>
-      <t>C25516</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <color rgb="FF1155CC"/>
-        <u/>
-      </rPr>
-      <t>25E0389</t>
-    </r>
+    <t>25E0389</t>
   </si>
   <si>
     <t>2025NE000413</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <color rgb="FF1155CC"/>
-        <u/>
-      </rPr>
-      <t>C25501</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <color rgb="FF1155CC"/>
-        <u/>
-      </rPr>
-      <t>25E0403</t>
-    </r>
+    <t>C25501</t>
+  </si>
+  <si>
+    <t>25E0403</t>
   </si>
   <si>
     <t>20SP</t>
@@ -526,354 +460,106 @@
     <t>2025NE000414</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <color rgb="FF1155CC"/>
-        <u/>
-      </rPr>
-      <t>C25525</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <color rgb="FF1155CC"/>
-        <u/>
-      </rPr>
-      <t>25E0431</t>
-    </r>
+    <t>C25525</t>
+  </si>
+  <si>
+    <t>25E0431</t>
   </si>
   <si>
     <t>21EM</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <color rgb="FF1155CC"/>
-        <u/>
-      </rPr>
-      <t>C25545</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <color rgb="FF1155CC"/>
-        <u/>
-      </rPr>
-      <t>25E0524</t>
-    </r>
+    <t>C25545</t>
+  </si>
+  <si>
+    <t>25E0524</t>
   </si>
   <si>
     <t>20X7</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <color rgb="FF1155CC"/>
-        <u/>
-      </rPr>
-      <t>C25512</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <color rgb="FF1155CC"/>
-        <u/>
-      </rPr>
-      <t>25E0731</t>
-    </r>
+    <t>25E0731</t>
   </si>
   <si>
     <t>2025NE000774</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <color rgb="FF1155CC"/>
-        <u/>
-      </rPr>
-      <t>C25516</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <color rgb="FF1155CC"/>
-        <u/>
-      </rPr>
-      <t>25E0737</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <color rgb="FF1155CC"/>
-        <u/>
-      </rPr>
-      <t>C25630</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <color rgb="FF1155CC"/>
-        <u/>
-      </rPr>
-      <t>25E0787</t>
-    </r>
+    <t>25E0737</t>
+  </si>
+  <si>
+    <t>C25630</t>
+  </si>
+  <si>
+    <t>25E0787</t>
   </si>
   <si>
     <t>219C</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <color rgb="FF1155CC"/>
-        <u/>
-      </rPr>
-      <t>C25512</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <color rgb="FF1155CC"/>
-        <u/>
-      </rPr>
-      <t>25E0999</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <color rgb="FF1155CC"/>
-        <u/>
-      </rPr>
-      <t>C25590</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <color rgb="FF1155CC"/>
-        <u/>
-      </rPr>
-      <t>25E1128</t>
-    </r>
+    <t>25E0999</t>
+  </si>
+  <si>
+    <t>C25590</t>
+  </si>
+  <si>
+    <t>25E1128</t>
   </si>
   <si>
     <t>2025NE001598</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <color rgb="FF1155CC"/>
-        <u/>
-      </rPr>
-      <t>C25814</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <color rgb="FF1155CC"/>
-        <u/>
-      </rPr>
-      <t>25E1446</t>
-    </r>
+    <t>C25814</t>
+  </si>
+  <si>
+    <t>25E1446</t>
   </si>
   <si>
     <t>2025NE001627</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <color rgb="FF1155CC"/>
-        <u/>
-      </rPr>
-      <t>C25512</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <color rgb="FF1155CC"/>
-        <u/>
-      </rPr>
-      <t>25E1475</t>
-    </r>
+    <t>25E1475</t>
   </si>
   <si>
     <t>2025NE001629</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <color rgb="FF1155CC"/>
-        <u/>
-      </rPr>
-      <t>C25820</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <color rgb="FF1155CC"/>
-        <u/>
-      </rPr>
-      <t>25E1477</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <color rgb="FF1155CC"/>
-        <u/>
-      </rPr>
-      <t>C25590</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <color rgb="FF1155CC"/>
-        <u/>
-      </rPr>
-      <t>25E1535</t>
-    </r>
+    <t>C25820</t>
+  </si>
+  <si>
+    <t>25E1477</t>
+  </si>
+  <si>
+    <t>25E1535</t>
   </si>
   <si>
     <t>2025NE001688</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <color rgb="FF1155CC"/>
-        <u/>
-      </rPr>
-      <t>C25630</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <color rgb="FF1155CC"/>
-        <u/>
-      </rPr>
-      <t>25E1536</t>
-    </r>
+    <t>25E1536</t>
   </si>
   <si>
     <t>2025NE001689</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <color rgb="FF1155CC"/>
-        <u/>
-      </rPr>
-      <t>C25512</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <color rgb="FF1155CC"/>
-        <u/>
-      </rPr>
-      <t>25E1537</t>
-    </r>
+    <t>25E1537</t>
   </si>
   <si>
     <t>2025NE001690</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <color rgb="FF1155CC"/>
-        <u/>
-      </rPr>
-      <t>C25516</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <color rgb="FF1155CC"/>
-        <u/>
-      </rPr>
-      <t>25E1538</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <color rgb="FF1155CC"/>
-        <u/>
-      </rPr>
-      <t>C25865</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <color rgb="FF1155CC"/>
-        <u/>
-      </rPr>
-      <t>25E1666</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <color rgb="FF1155CC"/>
-        <u/>
-      </rPr>
-      <t>C25869</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <color rgb="FF1155CC"/>
-        <u/>
-      </rPr>
-      <t>25E1667</t>
-    </r>
+    <t>25E1538</t>
+  </si>
+  <si>
+    <t>C25865</t>
+  </si>
+  <si>
+    <t>25E1666</t>
+  </si>
+  <si>
+    <t>C25869</t>
+  </si>
+  <si>
+    <t>25E1667</t>
   </si>
   <si>
     <t>20YJ</t>
@@ -882,113 +568,64 @@
     <t>2025NE001830</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <color rgb="FF1155CC"/>
-        <u/>
-      </rPr>
-      <t>C25516</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <color rgb="FF1155CC"/>
-        <u/>
-      </rPr>
-      <t>25E1669</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <color rgb="FF1155CC"/>
-        <u/>
-      </rPr>
-      <t>C25863</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <color rgb="FF1155CC"/>
-        <u/>
-      </rPr>
-      <t>25E2021</t>
-    </r>
+    <t>25E1669</t>
+  </si>
+  <si>
+    <t>C25863</t>
+  </si>
+  <si>
+    <t>25E2021</t>
   </si>
   <si>
     <t>2025NE002237</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <color rgb="FF1155CC"/>
-        <u/>
-      </rPr>
-      <t>C25512</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <color rgb="FF1155CC"/>
-        <u/>
-      </rPr>
-      <t>25E2058</t>
-    </r>
+    <t>25E2058</t>
   </si>
   <si>
     <t>2026NE000330</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <color rgb="FF1155CC"/>
-        <u/>
-      </rPr>
-      <t>C26163</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <color rgb="FF1155CC"/>
-        <u/>
-      </rPr>
-      <t>26E0320</t>
-    </r>
+    <t>C26163</t>
+  </si>
+  <si>
+    <t>26E0320</t>
   </si>
   <si>
     <t>2026NE000388</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <color rgb="FF1155CC"/>
-        <u/>
-      </rPr>
-      <t>C26193</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <color rgb="FF1155CC"/>
-        <u/>
-      </rPr>
-      <t>26E0375</t>
-    </r>
+    <t>C26193</t>
+  </si>
+  <si>
+    <t>26E0375</t>
+  </si>
+  <si>
+    <t>2026NE000748</t>
+  </si>
+  <si>
+    <t>C26312</t>
+  </si>
+  <si>
+    <t>26E0709</t>
+  </si>
+  <si>
+    <t>2026NE000816</t>
+  </si>
+  <si>
+    <t>C26324</t>
+  </si>
+  <si>
+    <t>26E0776</t>
+  </si>
+  <si>
+    <t>2026NE000817</t>
+  </si>
+  <si>
+    <t>C26326</t>
+  </si>
+  <si>
+    <t>26E0777</t>
   </si>
 </sst>
 </file>
@@ -8182,7 +7819,7 @@
     </row>
     <row r="2">
       <c r="A2" s="66">
-        <v>46154.0</v>
+        <v>46212.0</v>
       </c>
       <c r="L2" s="67" t="s">
         <v>124</v>
@@ -8335,10 +7972,10 @@
         <v>135</v>
       </c>
       <c r="B6" s="12" t="s">
+        <v>133</v>
+      </c>
+      <c r="C6" s="12" t="s">
         <v>136</v>
-      </c>
-      <c r="C6" s="12" t="s">
-        <v>137</v>
       </c>
       <c r="D6" s="12" t="s">
         <v>127</v>
@@ -8377,13 +8014,13 @@
     </row>
     <row r="7">
       <c r="A7" s="12" t="s">
+        <v>137</v>
+      </c>
+      <c r="B7" s="12" t="s">
         <v>138</v>
       </c>
-      <c r="B7" s="12" t="s">
+      <c r="C7" s="12" t="s">
         <v>139</v>
-      </c>
-      <c r="C7" s="12" t="s">
-        <v>140</v>
       </c>
       <c r="D7" s="12" t="s">
         <v>127</v>
@@ -8401,7 +8038,7 @@
         <v>339039.0</v>
       </c>
       <c r="I7" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="J7" s="14">
         <v>949835.78</v>
@@ -8422,13 +8059,13 @@
     </row>
     <row r="8">
       <c r="A8" s="12" t="s">
+        <v>141</v>
+      </c>
+      <c r="B8" s="12" t="s">
         <v>142</v>
       </c>
-      <c r="B8" s="12" t="s">
+      <c r="C8" s="12" t="s">
         <v>143</v>
-      </c>
-      <c r="C8" s="12" t="s">
-        <v>144</v>
       </c>
       <c r="D8" s="12" t="s">
         <v>127</v>
@@ -8446,7 +8083,7 @@
         <v>339039.0</v>
       </c>
       <c r="I8" s="12" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="J8" s="14">
         <v>524584.95</v>
@@ -8471,10 +8108,10 @@
         <v>91</v>
       </c>
       <c r="B9" s="12" t="s">
+        <v>145</v>
+      </c>
+      <c r="C9" s="12" t="s">
         <v>146</v>
-      </c>
-      <c r="C9" s="12" t="s">
-        <v>147</v>
       </c>
       <c r="D9" s="12" t="s">
         <v>127</v>
@@ -8492,7 +8129,7 @@
         <v>339039.0</v>
       </c>
       <c r="I9" s="12" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="J9" s="14">
         <v>211614.23</v>
@@ -8516,10 +8153,10 @@
         <v>98</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>149</v>
+        <v>130</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="D10" s="12" t="s">
         <v>127</v>
@@ -8558,13 +8195,13 @@
     </row>
     <row r="11">
       <c r="A11" s="12" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>152</v>
+        <v>133</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="D11" s="12" t="s">
         <v>127</v>
@@ -8606,10 +8243,10 @@
         <v>50</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="C12" s="12" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="D12" s="12" t="s">
         <v>127</v>
@@ -8627,7 +8264,7 @@
         <v>339039.0</v>
       </c>
       <c r="I12" s="12" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="J12" s="14">
         <v>1600334.09</v>
@@ -8651,10 +8288,10 @@
         <v>123</v>
       </c>
       <c r="B13" s="12" t="s">
-        <v>157</v>
+        <v>130</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="D13" s="12" t="s">
         <v>127</v>
@@ -8678,10 +8315,10 @@
         <v>2364771.07</v>
       </c>
       <c r="K13" s="14">
-        <v>259050.36</v>
+        <v>1867169.54</v>
       </c>
       <c r="L13" s="14">
-        <v>2105720.71</v>
+        <v>497601.53</v>
       </c>
       <c r="M13" s="72"/>
       <c r="AB13" s="65"/>
@@ -8697,10 +8334,10 @@
         <v>59</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="D14" s="12" t="s">
         <v>127</v>
@@ -8718,7 +8355,7 @@
         <v>339039.0</v>
       </c>
       <c r="I14" s="12" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="J14" s="14">
         <v>968237.39</v>
@@ -8739,13 +8376,13 @@
     </row>
     <row r="15">
       <c r="A15" s="12" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="B15" s="12" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="D15" s="12" t="s">
         <v>127</v>
@@ -8763,7 +8400,7 @@
         <v>339039.0</v>
       </c>
       <c r="I15" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="J15" s="14">
         <v>1011677.95</v>
@@ -8784,13 +8421,13 @@
     </row>
     <row r="16">
       <c r="A16" s="12" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="B16" s="12" t="s">
-        <v>165</v>
+        <v>130</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="D16" s="12" t="s">
         <v>127</v>
@@ -8829,13 +8466,13 @@
     </row>
     <row r="17">
       <c r="A17" s="12" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
       <c r="B17" s="12" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="D17" s="12" t="s">
         <v>127</v>
@@ -8877,10 +8514,10 @@
         <v>110</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>170</v>
+        <v>155</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="D18" s="12" t="s">
         <v>127</v>
@@ -8898,7 +8535,7 @@
         <v>339039.0</v>
       </c>
       <c r="I18" s="12" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="J18" s="14">
         <v>63746.85</v>
@@ -8919,13 +8556,13 @@
     </row>
     <row r="19">
       <c r="A19" s="12" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>173</v>
+        <v>151</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>174</v>
+        <v>167</v>
       </c>
       <c r="D19" s="12" t="s">
         <v>127</v>
@@ -8943,7 +8580,7 @@
         <v>339039.0</v>
       </c>
       <c r="I19" s="12" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="J19" s="14">
         <v>947931.1</v>
@@ -8964,13 +8601,13 @@
     </row>
     <row r="20">
       <c r="A20" s="12" t="s">
-        <v>175</v>
+        <v>168</v>
       </c>
       <c r="B20" s="12" t="s">
-        <v>176</v>
+        <v>130</v>
       </c>
       <c r="C20" s="12" t="s">
-        <v>177</v>
+        <v>169</v>
       </c>
       <c r="D20" s="12" t="s">
         <v>127</v>
@@ -9009,13 +8646,13 @@
     </row>
     <row r="21">
       <c r="A21" s="12" t="s">
-        <v>178</v>
+        <v>170</v>
       </c>
       <c r="B21" s="12" t="s">
-        <v>179</v>
+        <v>133</v>
       </c>
       <c r="C21" s="12" t="s">
-        <v>180</v>
+        <v>171</v>
       </c>
       <c r="D21" s="12" t="s">
         <v>127</v>
@@ -9057,10 +8694,10 @@
         <v>74</v>
       </c>
       <c r="B22" s="12" t="s">
-        <v>181</v>
+        <v>172</v>
       </c>
       <c r="C22" s="12" t="s">
-        <v>182</v>
+        <v>173</v>
       </c>
       <c r="D22" s="12" t="s">
         <v>127</v>
@@ -9102,10 +8739,10 @@
         <v>114</v>
       </c>
       <c r="B23" s="12" t="s">
-        <v>183</v>
+        <v>174</v>
       </c>
       <c r="C23" s="12" t="s">
-        <v>184</v>
+        <v>175</v>
       </c>
       <c r="D23" s="12" t="s">
         <v>127</v>
@@ -9123,7 +8760,7 @@
         <v>339039.0</v>
       </c>
       <c r="I23" s="12" t="s">
-        <v>185</v>
+        <v>176</v>
       </c>
       <c r="J23" s="14">
         <v>1000001.64</v>
@@ -9144,13 +8781,13 @@
     </row>
     <row r="24">
       <c r="A24" s="12" t="s">
-        <v>186</v>
+        <v>177</v>
       </c>
       <c r="B24" s="12" t="s">
-        <v>187</v>
+        <v>133</v>
       </c>
       <c r="C24" s="12" t="s">
-        <v>188</v>
+        <v>178</v>
       </c>
       <c r="D24" s="12" t="s">
         <v>127</v>
@@ -9192,10 +8829,10 @@
         <v>105</v>
       </c>
       <c r="B25" s="12" t="s">
-        <v>189</v>
+        <v>179</v>
       </c>
       <c r="C25" s="12" t="s">
-        <v>190</v>
+        <v>180</v>
       </c>
       <c r="D25" s="12" t="s">
         <v>127</v>
@@ -9213,7 +8850,7 @@
         <v>339039.0</v>
       </c>
       <c r="I25" s="12" t="s">
-        <v>185</v>
+        <v>176</v>
       </c>
       <c r="J25" s="14">
         <v>1157673.06</v>
@@ -9234,13 +8871,13 @@
     </row>
     <row r="26">
       <c r="A26" s="12" t="s">
-        <v>191</v>
+        <v>181</v>
       </c>
       <c r="B26" s="12" t="s">
-        <v>192</v>
+        <v>130</v>
       </c>
       <c r="C26" s="12" t="s">
-        <v>193</v>
+        <v>182</v>
       </c>
       <c r="D26" s="12" t="s">
         <v>127</v>
@@ -9279,13 +8916,13 @@
     </row>
     <row r="27">
       <c r="A27" s="12" t="s">
-        <v>194</v>
+        <v>183</v>
       </c>
       <c r="B27" s="12" t="s">
-        <v>195</v>
+        <v>184</v>
       </c>
       <c r="C27" s="12" t="s">
-        <v>196</v>
+        <v>185</v>
       </c>
       <c r="D27" s="12" t="s">
         <v>127</v>
@@ -9324,13 +8961,13 @@
     </row>
     <row r="28">
       <c r="A28" s="12" t="s">
-        <v>197</v>
+        <v>186</v>
       </c>
       <c r="B28" s="12" t="s">
-        <v>198</v>
+        <v>187</v>
       </c>
       <c r="C28" s="12" t="s">
-        <v>199</v>
+        <v>188</v>
       </c>
       <c r="D28" s="12" t="s">
         <v>127</v>
@@ -9348,7 +8985,7 @@
         <v>339039.0</v>
       </c>
       <c r="I28" s="12" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="J28" s="14">
         <v>1912292.52</v>
@@ -9368,6 +9005,42 @@
       <c r="AH28" s="65"/>
     </row>
     <row r="29">
+      <c r="A29" s="67" t="s">
+        <v>189</v>
+      </c>
+      <c r="B29" s="67" t="s">
+        <v>190</v>
+      </c>
+      <c r="C29" s="67" t="s">
+        <v>191</v>
+      </c>
+      <c r="D29" s="67" t="s">
+        <v>127</v>
+      </c>
+      <c r="E29" s="66">
+        <v>46196.0</v>
+      </c>
+      <c r="F29" s="67" t="s">
+        <v>128</v>
+      </c>
+      <c r="G29" s="67">
+        <v>12.0</v>
+      </c>
+      <c r="H29" s="67">
+        <v>339039.0</v>
+      </c>
+      <c r="I29" s="67">
+        <v>2048.0</v>
+      </c>
+      <c r="J29" s="55">
+        <v>1496713.48</v>
+      </c>
+      <c r="K29" s="67">
+        <v>0.0</v>
+      </c>
+      <c r="L29" s="55">
+        <v>1496713.48</v>
+      </c>
       <c r="AB29" s="65"/>
       <c r="AC29" s="65"/>
       <c r="AD29" s="65"/>
@@ -9377,6 +9050,42 @@
       <c r="AH29" s="65"/>
     </row>
     <row r="30">
+      <c r="A30" s="67" t="s">
+        <v>192</v>
+      </c>
+      <c r="B30" s="67" t="s">
+        <v>193</v>
+      </c>
+      <c r="C30" s="67" t="s">
+        <v>194</v>
+      </c>
+      <c r="D30" s="67" t="s">
+        <v>127</v>
+      </c>
+      <c r="E30" s="66">
+        <v>46205.0</v>
+      </c>
+      <c r="F30" s="67" t="s">
+        <v>128</v>
+      </c>
+      <c r="G30" s="67">
+        <v>12.0</v>
+      </c>
+      <c r="H30" s="67">
+        <v>339039.0</v>
+      </c>
+      <c r="I30" s="67" t="s">
+        <v>140</v>
+      </c>
+      <c r="J30" s="55">
+        <v>624166.14</v>
+      </c>
+      <c r="K30" s="67">
+        <v>0.0</v>
+      </c>
+      <c r="L30" s="55">
+        <v>624166.14</v>
+      </c>
       <c r="AB30" s="65"/>
       <c r="AC30" s="65"/>
       <c r="AD30" s="65"/>
@@ -9386,6 +9095,42 @@
       <c r="AH30" s="65"/>
     </row>
     <row r="31">
+      <c r="A31" s="67" t="s">
+        <v>195</v>
+      </c>
+      <c r="B31" s="67" t="s">
+        <v>196</v>
+      </c>
+      <c r="C31" s="67" t="s">
+        <v>197</v>
+      </c>
+      <c r="D31" s="67" t="s">
+        <v>127</v>
+      </c>
+      <c r="E31" s="66">
+        <v>46205.0</v>
+      </c>
+      <c r="F31" s="67" t="s">
+        <v>128</v>
+      </c>
+      <c r="G31" s="67">
+        <v>12.0</v>
+      </c>
+      <c r="H31" s="67">
+        <v>339039.0</v>
+      </c>
+      <c r="I31" s="67" t="s">
+        <v>176</v>
+      </c>
+      <c r="J31" s="55">
+        <v>18462.36</v>
+      </c>
+      <c r="K31" s="67">
+        <v>0.0</v>
+      </c>
+      <c r="L31" s="55">
+        <v>18462.36</v>
+      </c>
       <c r="AB31" s="65"/>
       <c r="AC31" s="65"/>
       <c r="AD31" s="65"/>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (09/07/2026 15:31)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/01_Bases_Originais/005_CELOG_2025/005_CELOG-PAMALS_2025 online.xlsx
+++ b/Contrato 005/Dashboard/01_Bases_Originais/005_CELOG_2025/005_CELOG-PAMALS_2025 online.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="198">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="199">
   <si>
     <t>Controle de pagamentos</t>
   </si>
@@ -395,6 +395,9 @@
   </si>
   <si>
     <t>Aprovado e aguardando itens</t>
+  </si>
+  <si>
+    <t>Módulo II – Orçamento 03/26</t>
   </si>
   <si>
     <t>Módulo III – Orçamento 17 Manuais</t>
@@ -2755,7 +2758,7 @@
     <row r="37" ht="12.75" customHeight="1">
       <c r="A37" s="16"/>
       <c r="B37" s="16"/>
-      <c r="C37" s="47"/>
+      <c r="C37" s="32"/>
       <c r="D37" s="52" t="s">
         <v>119</v>
       </c>
@@ -2792,34 +2795,22 @@
     <row r="38" ht="12.75" customHeight="1">
       <c r="A38" s="16"/>
       <c r="B38" s="16"/>
-      <c r="C38" s="24">
-        <v>3.0</v>
-      </c>
+      <c r="C38" s="47"/>
       <c r="D38" s="52" t="s">
         <v>121</v>
       </c>
       <c r="E38" s="56"/>
-      <c r="F38" s="56">
-        <v>1465.0</v>
-      </c>
-      <c r="G38" s="60">
-        <v>46104.0</v>
-      </c>
-      <c r="H38" s="56" t="s">
-        <v>74</v>
-      </c>
-      <c r="I38" s="61"/>
-      <c r="J38" s="60">
-        <v>46106.0</v>
-      </c>
-      <c r="K38" s="36">
-        <v>27801.11</v>
-      </c>
+      <c r="F38" s="56"/>
+      <c r="G38" s="60"/>
+      <c r="H38" s="56"/>
+      <c r="I38" s="56"/>
+      <c r="J38" s="60"/>
+      <c r="K38" s="36"/>
       <c r="L38" s="26"/>
-      <c r="M38" s="62">
-        <v>27801.11</v>
-      </c>
-      <c r="N38" s="41"/>
+      <c r="M38" s="30"/>
+      <c r="N38" s="41">
+        <v>24962.38</v>
+      </c>
       <c r="O38" s="18"/>
       <c r="P38" s="20"/>
       <c r="Q38" s="20"/>
@@ -2837,42 +2828,81 @@
       <c r="AC38" s="20"/>
     </row>
     <row r="39" ht="12.75" customHeight="1">
-      <c r="A39" s="8"/>
-      <c r="B39" s="8"/>
-      <c r="C39" s="32"/>
+      <c r="A39" s="16"/>
+      <c r="B39" s="16"/>
+      <c r="C39" s="24">
+        <v>3.0</v>
+      </c>
       <c r="D39" s="52" t="s">
         <v>122</v>
       </c>
       <c r="E39" s="56"/>
       <c r="F39" s="56">
-        <v>1882.0</v>
+        <v>1465.0</v>
       </c>
       <c r="G39" s="60">
-        <v>46199.0</v>
+        <v>46104.0</v>
       </c>
       <c r="H39" s="56" t="s">
-        <v>123</v>
+        <v>74</v>
       </c>
       <c r="I39" s="61"/>
       <c r="J39" s="60">
-        <v>46233.0</v>
+        <v>46106.0</v>
       </c>
       <c r="K39" s="36">
-        <v>58868.35</v>
+        <v>27801.11</v>
       </c>
       <c r="L39" s="26"/>
       <c r="M39" s="62">
-        <v>58868.35</v>
+        <v>27801.11</v>
       </c>
       <c r="N39" s="41"/>
-      <c r="V39" s="2"/>
+      <c r="O39" s="18"/>
+      <c r="P39" s="20"/>
+      <c r="Q39" s="20"/>
+      <c r="R39" s="20"/>
+      <c r="S39" s="20"/>
+      <c r="T39" s="20"/>
+      <c r="U39" s="20"/>
+      <c r="V39" s="42"/>
+      <c r="W39" s="20"/>
+      <c r="X39" s="20"/>
+      <c r="Y39" s="20"/>
+      <c r="Z39" s="20"/>
+      <c r="AA39" s="20"/>
+      <c r="AB39" s="20"/>
+      <c r="AC39" s="20"/>
     </row>
     <row r="40" ht="12.75" customHeight="1">
       <c r="A40" s="8"/>
       <c r="B40" s="8"/>
       <c r="C40" s="32"/>
-      <c r="K40" s="63"/>
-      <c r="M40" s="63"/>
+      <c r="D40" s="52" t="s">
+        <v>123</v>
+      </c>
+      <c r="E40" s="56"/>
+      <c r="F40" s="56">
+        <v>1882.0</v>
+      </c>
+      <c r="G40" s="60">
+        <v>46199.0</v>
+      </c>
+      <c r="H40" s="56" t="s">
+        <v>124</v>
+      </c>
+      <c r="I40" s="61"/>
+      <c r="J40" s="60">
+        <v>46233.0</v>
+      </c>
+      <c r="K40" s="36">
+        <v>58868.35</v>
+      </c>
+      <c r="L40" s="26"/>
+      <c r="M40" s="62">
+        <v>58868.35</v>
+      </c>
+      <c r="N40" s="41"/>
       <c r="V40" s="2"/>
     </row>
     <row r="41" ht="12.75" customHeight="1">
@@ -2887,6 +2917,8 @@
       <c r="A42" s="8"/>
       <c r="B42" s="8"/>
       <c r="C42" s="32"/>
+      <c r="K42" s="63"/>
+      <c r="M42" s="63"/>
       <c r="V42" s="2"/>
     </row>
     <row r="43" ht="12.75" customHeight="1">
@@ -2910,38 +2942,40 @@
     <row r="46" ht="12.75" customHeight="1">
       <c r="A46" s="8"/>
       <c r="B46" s="8"/>
-      <c r="C46" s="47"/>
-      <c r="K46" s="63"/>
-      <c r="M46" s="63"/>
+      <c r="C46" s="32"/>
       <c r="V46" s="2"/>
     </row>
     <row r="47" ht="12.75" customHeight="1">
       <c r="A47" s="8"/>
       <c r="B47" s="8"/>
-      <c r="C47" s="8"/>
-      <c r="D47" s="8"/>
-      <c r="E47" s="8"/>
-      <c r="F47" s="8"/>
-      <c r="G47" s="8"/>
-      <c r="H47" s="8"/>
-      <c r="I47" s="8"/>
-      <c r="J47" s="8"/>
-      <c r="K47" s="8"/>
-      <c r="L47" s="8"/>
-      <c r="M47" s="8"/>
-      <c r="N47" s="8"/>
-      <c r="O47" s="8"/>
-      <c r="P47" s="64"/>
-      <c r="Q47" s="64"/>
-      <c r="R47" s="64"/>
-      <c r="S47" s="64"/>
-      <c r="T47" s="64"/>
-      <c r="U47" s="64"/>
+      <c r="C47" s="47"/>
+      <c r="K47" s="63"/>
+      <c r="M47" s="63"/>
       <c r="V47" s="2"/>
     </row>
     <row r="48" ht="12.75" customHeight="1">
       <c r="A48" s="8"/>
       <c r="B48" s="8"/>
+      <c r="C48" s="8"/>
+      <c r="D48" s="8"/>
+      <c r="E48" s="8"/>
+      <c r="F48" s="8"/>
+      <c r="G48" s="8"/>
+      <c r="H48" s="8"/>
+      <c r="I48" s="8"/>
+      <c r="J48" s="8"/>
+      <c r="K48" s="8"/>
+      <c r="L48" s="8"/>
+      <c r="M48" s="8"/>
+      <c r="N48" s="8"/>
+      <c r="O48" s="8"/>
+      <c r="P48" s="64"/>
+      <c r="Q48" s="64"/>
+      <c r="R48" s="64"/>
+      <c r="S48" s="64"/>
+      <c r="T48" s="64"/>
+      <c r="U48" s="64"/>
+      <c r="V48" s="2"/>
     </row>
     <row r="49" ht="12.75" customHeight="1">
       <c r="A49" s="8"/>
@@ -3154,7 +3188,6 @@
     <row r="101" ht="12.75" customHeight="1">
       <c r="A101" s="8"/>
       <c r="B101" s="8"/>
-      <c r="L101" s="15"/>
     </row>
     <row r="102" ht="12.75" customHeight="1">
       <c r="A102" s="8"/>
@@ -7771,12 +7804,17 @@
       <c r="B1024" s="8"/>
       <c r="L1024" s="15"/>
     </row>
+    <row r="1025" ht="12.75" customHeight="1">
+      <c r="A1025" s="8"/>
+      <c r="B1025" s="8"/>
+      <c r="L1025" s="15"/>
+    </row>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="B2:U2"/>
     <mergeCell ref="C9:C26"/>
-    <mergeCell ref="C28:C37"/>
-    <mergeCell ref="C38:C46"/>
+    <mergeCell ref="C28:C38"/>
+    <mergeCell ref="C39:C47"/>
   </mergeCells>
   <printOptions/>
   <pageMargins bottom="0.7875" footer="0.0" header="0.0" left="0.7875" right="0.7875" top="0.7875"/>
@@ -7822,7 +7860,7 @@
         <v>46212.0</v>
       </c>
       <c r="L2" s="67" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="AB2" s="65"/>
       <c r="AC2" s="65"/>
@@ -7834,22 +7872,22 @@
     </row>
     <row r="3">
       <c r="A3" s="12" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C3" s="68">
         <v>2.5E32</v>
       </c>
       <c r="D3" s="12" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E3" s="69">
         <v>45686.0</v>
       </c>
       <c r="F3" s="12" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G3" s="12">
         <v>12.0</v>
@@ -7879,22 +7917,22 @@
     </row>
     <row r="4">
       <c r="A4" s="12" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E4" s="69">
         <v>45762.0</v>
       </c>
       <c r="F4" s="12" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G4" s="12">
         <v>12.0</v>
@@ -7924,22 +7962,22 @@
     </row>
     <row r="5">
       <c r="A5" s="12" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E5" s="69">
         <v>45762.0</v>
       </c>
       <c r="F5" s="12" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G5" s="12">
         <v>12.0</v>
@@ -7969,22 +8007,22 @@
     </row>
     <row r="6">
       <c r="A6" s="12" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E6" s="69">
         <v>45762.0</v>
       </c>
       <c r="F6" s="12" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G6" s="12">
         <v>12.0</v>
@@ -8014,22 +8052,22 @@
     </row>
     <row r="7">
       <c r="A7" s="12" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E7" s="69">
         <v>45763.0</v>
       </c>
       <c r="F7" s="12" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G7" s="12">
         <v>12.0</v>
@@ -8038,7 +8076,7 @@
         <v>339039.0</v>
       </c>
       <c r="I7" s="12" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="J7" s="14">
         <v>949835.78</v>
@@ -8059,22 +8097,22 @@
     </row>
     <row r="8">
       <c r="A8" s="12" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E8" s="69">
         <v>45763.0</v>
       </c>
       <c r="F8" s="12" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G8" s="12">
         <v>12.0</v>
@@ -8083,7 +8121,7 @@
         <v>339039.0</v>
       </c>
       <c r="I8" s="12" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="J8" s="14">
         <v>524584.95</v>
@@ -8108,19 +8146,19 @@
         <v>91</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E9" s="69">
         <v>45792.0</v>
       </c>
       <c r="F9" s="12" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G9" s="12">
         <v>12.0</v>
@@ -8129,7 +8167,7 @@
         <v>339039.0</v>
       </c>
       <c r="I9" s="12" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="J9" s="14">
         <v>211614.23</v>
@@ -8153,19 +8191,19 @@
         <v>98</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E10" s="69">
         <v>45825.0</v>
       </c>
       <c r="F10" s="12" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G10" s="12">
         <v>12.0</v>
@@ -8195,22 +8233,22 @@
     </row>
     <row r="11">
       <c r="A11" s="12" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D11" s="12" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E11" s="69">
         <v>45825.0</v>
       </c>
       <c r="F11" s="12" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G11" s="12">
         <v>12.0</v>
@@ -8243,19 +8281,19 @@
         <v>50</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C12" s="12" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D12" s="12" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E12" s="69">
         <v>45832.0</v>
       </c>
       <c r="F12" s="12" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G12" s="12">
         <v>12.0</v>
@@ -8264,7 +8302,7 @@
         <v>339039.0</v>
       </c>
       <c r="I12" s="12" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J12" s="14">
         <v>1600334.09</v>
@@ -8285,22 +8323,22 @@
     </row>
     <row r="13">
       <c r="A13" s="12" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B13" s="12" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D13" s="12" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E13" s="69">
         <v>45863.0</v>
       </c>
       <c r="F13" s="12" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G13" s="12">
         <v>12.0</v>
@@ -8334,19 +8372,19 @@
         <v>59</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D14" s="12" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E14" s="69">
         <v>45887.0</v>
       </c>
       <c r="F14" s="12" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G14" s="12">
         <v>12.0</v>
@@ -8355,7 +8393,7 @@
         <v>339039.0</v>
       </c>
       <c r="I14" s="12" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="J14" s="14">
         <v>968237.39</v>
@@ -8376,22 +8414,22 @@
     </row>
     <row r="15">
       <c r="A15" s="12" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B15" s="12" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D15" s="12" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E15" s="69">
         <v>45924.0</v>
       </c>
       <c r="F15" s="12" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G15" s="12">
         <v>12.0</v>
@@ -8400,7 +8438,7 @@
         <v>339039.0</v>
       </c>
       <c r="I15" s="12" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="J15" s="14">
         <v>1011677.95</v>
@@ -8421,22 +8459,22 @@
     </row>
     <row r="16">
       <c r="A16" s="12" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B16" s="12" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D16" s="12" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E16" s="69">
         <v>45929.0</v>
       </c>
       <c r="F16" s="12" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G16" s="12">
         <v>12.0</v>
@@ -8466,22 +8504,22 @@
     </row>
     <row r="17">
       <c r="A17" s="12" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B17" s="12" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D17" s="12" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E17" s="69">
         <v>45930.0</v>
       </c>
       <c r="F17" s="12" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G17" s="12">
         <v>12.0</v>
@@ -8514,19 +8552,19 @@
         <v>110</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D18" s="12" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E18" s="69">
         <v>45938.0</v>
       </c>
       <c r="F18" s="12" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G18" s="12">
         <v>12.0</v>
@@ -8535,7 +8573,7 @@
         <v>339039.0</v>
       </c>
       <c r="I18" s="12" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="J18" s="14">
         <v>63746.85</v>
@@ -8556,22 +8594,22 @@
     </row>
     <row r="19">
       <c r="A19" s="12" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D19" s="12" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E19" s="69">
         <v>45938.0</v>
       </c>
       <c r="F19" s="12" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G19" s="12">
         <v>12.0</v>
@@ -8580,7 +8618,7 @@
         <v>339039.0</v>
       </c>
       <c r="I19" s="12" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J19" s="14">
         <v>947931.1</v>
@@ -8601,22 +8639,22 @@
     </row>
     <row r="20">
       <c r="A20" s="12" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B20" s="12" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C20" s="12" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D20" s="12" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E20" s="69">
         <v>45938.0</v>
       </c>
       <c r="F20" s="12" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G20" s="12">
         <v>12.0</v>
@@ -8646,22 +8684,22 @@
     </row>
     <row r="21">
       <c r="A21" s="12" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B21" s="12" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C21" s="12" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="D21" s="12" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E21" s="69">
         <v>45938.0</v>
       </c>
       <c r="F21" s="12" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G21" s="12">
         <v>12.0</v>
@@ -8694,19 +8732,19 @@
         <v>74</v>
       </c>
       <c r="B22" s="12" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C22" s="12" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D22" s="12" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E22" s="73">
         <v>45953.0</v>
       </c>
       <c r="F22" s="12" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G22" s="12">
         <v>12.0</v>
@@ -8739,19 +8777,19 @@
         <v>114</v>
       </c>
       <c r="B23" s="12" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="C23" s="12" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D23" s="12" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E23" s="73">
         <v>45953.0</v>
       </c>
       <c r="F23" s="12" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G23" s="12">
         <v>12.0</v>
@@ -8760,7 +8798,7 @@
         <v>339039.0</v>
       </c>
       <c r="I23" s="12" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="J23" s="14">
         <v>1000001.64</v>
@@ -8781,22 +8819,22 @@
     </row>
     <row r="24">
       <c r="A24" s="12" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B24" s="12" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C24" s="12" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="D24" s="12" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E24" s="73">
         <v>45953.0</v>
       </c>
       <c r="F24" s="12" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G24" s="12">
         <v>12.0</v>
@@ -8829,19 +8867,19 @@
         <v>105</v>
       </c>
       <c r="B25" s="12" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C25" s="12" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D25" s="12" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E25" s="73">
         <v>45975.0</v>
       </c>
       <c r="F25" s="12" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G25" s="12">
         <v>12.0</v>
@@ -8850,7 +8888,7 @@
         <v>339039.0</v>
       </c>
       <c r="I25" s="12" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="J25" s="14">
         <v>1157673.06</v>
@@ -8871,22 +8909,22 @@
     </row>
     <row r="26">
       <c r="A26" s="12" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B26" s="12" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C26" s="12" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D26" s="12" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E26" s="73">
         <v>45989.0</v>
       </c>
       <c r="F26" s="12" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G26" s="12">
         <v>12.0</v>
@@ -8916,22 +8954,22 @@
     </row>
     <row r="27">
       <c r="A27" s="12" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B27" s="12" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C27" s="12" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="D27" s="12" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E27" s="69">
         <v>46104.0</v>
       </c>
       <c r="F27" s="12" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G27" s="12">
         <v>12.0</v>
@@ -8961,22 +8999,22 @@
     </row>
     <row r="28">
       <c r="A28" s="12" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B28" s="12" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="C28" s="12" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D28" s="12" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E28" s="69">
         <v>46120.0</v>
       </c>
       <c r="F28" s="12" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G28" s="12">
         <v>12.0</v>
@@ -8985,7 +9023,7 @@
         <v>339039.0</v>
       </c>
       <c r="I28" s="12" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="J28" s="14">
         <v>1912292.52</v>
@@ -9006,22 +9044,22 @@
     </row>
     <row r="29">
       <c r="A29" s="67" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B29" s="67" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C29" s="67" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D29" s="67" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E29" s="66">
         <v>46196.0</v>
       </c>
       <c r="F29" s="67" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G29" s="67">
         <v>12.0</v>
@@ -9051,22 +9089,22 @@
     </row>
     <row r="30">
       <c r="A30" s="67" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B30" s="67" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C30" s="67" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="D30" s="67" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E30" s="66">
         <v>46205.0</v>
       </c>
       <c r="F30" s="67" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G30" s="67">
         <v>12.0</v>
@@ -9075,7 +9113,7 @@
         <v>339039.0</v>
       </c>
       <c r="I30" s="67" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="J30" s="55">
         <v>624166.14</v>
@@ -9096,22 +9134,22 @@
     </row>
     <row r="31">
       <c r="A31" s="67" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B31" s="67" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C31" s="67" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="D31" s="67" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E31" s="66">
         <v>46205.0</v>
       </c>
       <c r="F31" s="67" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G31" s="67">
         <v>12.0</v>
@@ -9120,7 +9158,7 @@
         <v>339039.0</v>
       </c>
       <c r="I31" s="67" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="J31" s="55">
         <v>18462.36</v>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (16/07/2026 20:15)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/01_Bases_Originais/005_CELOG_2025/005_CELOG-PAMALS_2025 online.xlsx
+++ b/Contrato 005/Dashboard/01_Bases_Originais/005_CELOG_2025/005_CELOG-PAMALS_2025 online.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="317" uniqueCount="201">
   <si>
     <t>Controle de pagamentos</t>
   </si>
@@ -629,6 +629,12 @@
   </si>
   <si>
     <t>26E0777</t>
+  </si>
+  <si>
+    <t>2026NE000842</t>
+  </si>
+  <si>
+    <t>26E0803</t>
   </si>
 </sst>
 </file>
@@ -9178,7 +9184,42 @@
       <c r="AH31" s="65"/>
     </row>
     <row r="32">
-      <c r="C32" s="55"/>
+      <c r="A32" s="67" t="s">
+        <v>199</v>
+      </c>
+      <c r="B32" s="67" t="s">
+        <v>197</v>
+      </c>
+      <c r="C32" s="55" t="s">
+        <v>200</v>
+      </c>
+      <c r="D32" s="67" t="s">
+        <v>128</v>
+      </c>
+      <c r="E32" s="66">
+        <v>46213.0</v>
+      </c>
+      <c r="F32" s="67" t="s">
+        <v>129</v>
+      </c>
+      <c r="G32" s="67">
+        <v>12.0</v>
+      </c>
+      <c r="H32" s="67">
+        <v>339039.0</v>
+      </c>
+      <c r="I32" s="67" t="s">
+        <v>177</v>
+      </c>
+      <c r="J32" s="55">
+        <v>1530656.62</v>
+      </c>
+      <c r="K32" s="67">
+        <v>0.0</v>
+      </c>
+      <c r="L32" s="55">
+        <v>1530656.62</v>
+      </c>
       <c r="AB32" s="65"/>
       <c r="AC32" s="65"/>
       <c r="AD32" s="65"/>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (23/07/2026 20:41)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/01_Bases_Originais/005_CELOG_2025/005_CELOG-PAMALS_2025 online.xlsx
+++ b/Contrato 005/Dashboard/01_Bases_Originais/005_CELOG_2025/005_CELOG-PAMALS_2025 online.xlsx
@@ -30,12 +30,12 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="204">
   <si>
+    <t>Saldo</t>
+  </si>
+  <si>
     <t>Controle de pagamentos</t>
   </si>
   <si>
-    <t>Saldo</t>
-  </si>
-  <si>
     <t>2025NE000005</t>
   </si>
   <si>
@@ -72,6 +72,15 @@
     <t>Prazo Final de Execução</t>
   </si>
   <si>
+    <t>2025NE000369</t>
+  </si>
+  <si>
+    <t>C25516</t>
+  </si>
+  <si>
+    <t>25E0387</t>
+  </si>
+  <si>
     <t>Prazo Final de Vigência</t>
   </si>
   <si>
@@ -90,21 +99,12 @@
     <t>Valor Total do Contrato</t>
   </si>
   <si>
-    <t>2025NE000369</t>
-  </si>
-  <si>
     <t>Valor a Empenhar</t>
   </si>
   <si>
-    <t>C25516</t>
-  </si>
-  <si>
     <t>Valor Empenhado</t>
   </si>
   <si>
-    <t>25E0387</t>
-  </si>
-  <si>
     <t>Valor Liquidado</t>
   </si>
   <si>
@@ -120,12 +120,12 @@
     <t>Abrir</t>
   </si>
   <si>
+    <t>2025NE000371</t>
+  </si>
+  <si>
     <t>Editar</t>
   </si>
   <si>
-    <t>2025NE000371</t>
-  </si>
-  <si>
     <t>25E0389</t>
   </si>
   <si>
@@ -138,6 +138,15 @@
     <t>PAMALS</t>
   </si>
   <si>
+    <t>2025NE000413</t>
+  </si>
+  <si>
+    <t>C25501</t>
+  </si>
+  <si>
+    <t>25E0403</t>
+  </si>
+  <si>
     <t>Vigente</t>
   </si>
   <si>
@@ -147,24 +156,15 @@
     <t>67101.001510/2024-12</t>
   </si>
   <si>
+    <t>20SP</t>
+  </si>
+  <si>
     <t>R$</t>
   </si>
   <si>
-    <t>2025NE000413</t>
-  </si>
-  <si>
-    <t>C25501</t>
-  </si>
-  <si>
-    <t>25E0403</t>
-  </si>
-  <si>
     <t>VEE ONE-MANUTENCAO E SERVICOS TECNICOS LTDA</t>
   </si>
   <si>
-    <t>20SP</t>
-  </si>
-  <si>
     <t>2025NE000414</t>
   </si>
   <si>
@@ -177,22 +177,46 @@
     <t>21EM</t>
   </si>
   <si>
+    <t>2025NE000559</t>
+  </si>
+  <si>
+    <t>C25545</t>
+  </si>
+  <si>
+    <t>25E0524</t>
+  </si>
+  <si>
+    <t>20X7</t>
+  </si>
+  <si>
+    <t>2025NE000770</t>
+  </si>
+  <si>
+    <t>25E0731</t>
+  </si>
+  <si>
     <t>Módulo</t>
   </si>
   <si>
+    <t>2025NE000774</t>
+  </si>
+  <si>
+    <t>25E0737</t>
+  </si>
+  <si>
     <t>Referência</t>
   </si>
   <si>
-    <t>2025NE000559</t>
-  </si>
-  <si>
     <t>Nº recibo</t>
   </si>
   <si>
-    <t>C25545</t>
-  </si>
-  <si>
-    <t>25E0524</t>
+    <t>2025NE000843</t>
+  </si>
+  <si>
+    <t>C25630</t>
+  </si>
+  <si>
+    <t>25E0787</t>
   </si>
   <si>
     <t>Nº</t>
@@ -201,12 +225,12 @@
     <t>Data</t>
   </si>
   <si>
+    <t>219C</t>
+  </si>
+  <si>
     <t>Empenho</t>
   </si>
   <si>
-    <t>20X7</t>
-  </si>
-  <si>
     <t>Observações</t>
   </si>
   <si>
@@ -219,10 +243,10 @@
     <t>Ordem de Pagamento</t>
   </si>
   <si>
-    <t>2025NE000770</t>
-  </si>
-  <si>
-    <t>25E0731</t>
+    <t>2025NE001065</t>
+  </si>
+  <si>
+    <t>25E0999</t>
   </si>
   <si>
     <t>Faturado</t>
@@ -231,10 +255,13 @@
     <t>Pendente</t>
   </si>
   <si>
-    <t>2025NE000774</t>
-  </si>
-  <si>
-    <t>25E0737</t>
+    <t>2025NE001200</t>
+  </si>
+  <si>
+    <t>C25590</t>
+  </si>
+  <si>
+    <t>25E1128</t>
   </si>
   <si>
     <t>FEV/25</t>
@@ -243,40 +270,61 @@
     <t>-</t>
   </si>
   <si>
-    <t>2025NE000843</t>
+    <t>2025NE001598</t>
+  </si>
+  <si>
+    <t>C25814</t>
+  </si>
+  <si>
+    <t>25E1446</t>
+  </si>
+  <si>
+    <t>2025NE001627</t>
+  </si>
+  <si>
+    <t>25E1475</t>
   </si>
   <si>
     <t xml:space="preserve">2025NE000369 </t>
   </si>
   <si>
-    <t>C25630</t>
-  </si>
-  <si>
-    <t>25E0787</t>
-  </si>
-  <si>
-    <t>219C</t>
+    <t>2025NE001629</t>
+  </si>
+  <si>
+    <t>C25820</t>
+  </si>
+  <si>
+    <t>25E1477</t>
   </si>
   <si>
     <t>2025NP001980</t>
   </si>
   <si>
-    <t>2025NE001065</t>
-  </si>
-  <si>
-    <t>25E0999</t>
+    <t>2025NE001687</t>
+  </si>
+  <si>
+    <t>25E1535</t>
+  </si>
+  <si>
+    <t>2025NE001688</t>
+  </si>
+  <si>
+    <t>25E1536</t>
+  </si>
+  <si>
+    <t>2025NE001689</t>
+  </si>
+  <si>
+    <t>25E1537</t>
   </si>
   <si>
     <t>MAR/25</t>
   </si>
   <si>
-    <t>2025NE001200</t>
-  </si>
-  <si>
-    <t>C25590</t>
-  </si>
-  <si>
-    <t>25E1128</t>
+    <t>2025NE001690</t>
+  </si>
+  <si>
+    <t>25E1538</t>
   </si>
   <si>
     <t>2025NE000367, 2025NE000369, 2025NE000371, 2025NE000413</t>
@@ -285,58 +333,100 @@
     <t>2025NP001979</t>
   </si>
   <si>
-    <t>2025NE001598</t>
-  </si>
-  <si>
-    <t>C25814</t>
-  </si>
-  <si>
-    <t>25E1446</t>
+    <t>2025NE001823</t>
+  </si>
+  <si>
+    <t>C25865</t>
+  </si>
+  <si>
+    <t>25E1666</t>
+  </si>
+  <si>
+    <t>2025NE001828</t>
+  </si>
+  <si>
+    <t>C25869</t>
+  </si>
+  <si>
+    <t>25E1667</t>
+  </si>
+  <si>
+    <t>20YJ</t>
   </si>
   <si>
     <t>ABR/25</t>
   </si>
   <si>
+    <t>2025NE001830</t>
+  </si>
+  <si>
     <t>2025NE000413, 2025NE000414, 2025NE000559</t>
   </si>
   <si>
-    <t>2025NE001627</t>
-  </si>
-  <si>
-    <t>25E1475</t>
+    <t>25E1669</t>
   </si>
   <si>
     <t>2025NP002341</t>
   </si>
   <si>
+    <t>2025NE002200</t>
+  </si>
+  <si>
+    <t>C25863</t>
+  </si>
+  <si>
+    <t>25E2021</t>
+  </si>
+  <si>
     <t>MAI/25</t>
   </si>
   <si>
-    <t>2025NE001629</t>
-  </si>
-  <si>
-    <t>C25820</t>
-  </si>
-  <si>
-    <t>25E1477</t>
+    <t>2025NE002237</t>
+  </si>
+  <si>
+    <t>25E2058</t>
+  </si>
+  <si>
+    <t>2026NE000330</t>
+  </si>
+  <si>
+    <t>C26163</t>
+  </si>
+  <si>
+    <t>26E0320</t>
+  </si>
+  <si>
+    <t>2026NE000388</t>
+  </si>
+  <si>
+    <t>C26193</t>
   </si>
   <si>
     <t>2025NP002884</t>
   </si>
   <si>
-    <t>2025NE001687</t>
-  </si>
-  <si>
-    <t>25E1535</t>
+    <t>26E0375</t>
+  </si>
+  <si>
+    <t>2026NE000748</t>
+  </si>
+  <si>
+    <t>C26312</t>
+  </si>
+  <si>
+    <t>26E0709</t>
   </si>
   <si>
     <t>JUN/25</t>
   </si>
   <si>
-    <t>2025NE001688</t>
-  </si>
-  <si>
-    <t>25E1536</t>
+    <t>2026NE000816</t>
+  </si>
+  <si>
+    <t>C26324</t>
+  </si>
+  <si>
+    <t>26E0776</t>
   </si>
   <si>
     <t>2025NE000005,
@@ -348,176 +438,86 @@
     <t>2025NP400522</t>
   </si>
   <si>
-    <t>2025NE001689</t>
-  </si>
-  <si>
-    <t>25E1537</t>
+    <t>2026NE000817</t>
+  </si>
+  <si>
+    <t>C26326</t>
+  </si>
+  <si>
+    <t>26E0777</t>
   </si>
   <si>
     <t>JUL/25</t>
   </si>
   <si>
+    <t>2026NE000842</t>
+  </si>
+  <si>
+    <t>26E0803</t>
+  </si>
+  <si>
     <t>2025NE000843, 2025NE001200</t>
   </si>
   <si>
     <t>2025NP003724</t>
   </si>
   <si>
-    <t>2025NE001690</t>
-  </si>
-  <si>
-    <t>25E1538</t>
-  </si>
-  <si>
     <t>AGO/25</t>
   </si>
   <si>
-    <t>2025NE001823</t>
-  </si>
-  <si>
-    <t>C25865</t>
-  </si>
-  <si>
-    <t>25E1666</t>
-  </si>
-  <si>
     <t>2025NP004558</t>
   </si>
   <si>
     <t>SET/25</t>
-  </si>
-  <si>
-    <t>2025NE001828</t>
-  </si>
-  <si>
-    <t>C25869</t>
-  </si>
-  <si>
-    <t>25E1667</t>
   </si>
   <si>
     <t>2025NE001688 
 2025NE001828</t>
   </si>
   <si>
-    <t>20YJ</t>
-  </si>
-  <si>
     <t>2025NP004897</t>
   </si>
   <si>
-    <t>2025NE001830</t>
-  </si>
-  <si>
-    <t>25E1669</t>
-  </si>
-  <si>
     <t>OUT/25</t>
   </si>
   <si>
     <t>2025NE001688, 2025NE001828, 2025NE002200</t>
   </si>
   <si>
-    <t>2025NE002200</t>
-  </si>
-  <si>
-    <t>C25863</t>
-  </si>
-  <si>
-    <t>25E2021</t>
-  </si>
-  <si>
     <t>2025NP004932</t>
   </si>
   <si>
-    <t>2025NE002237</t>
-  </si>
-  <si>
-    <t>25E2058</t>
-  </si>
-  <si>
     <t>NOV/25</t>
   </si>
   <si>
     <t>2025NE001687, 2025NE001689, 2025NE001690, 2025NE001823, 2025NE001830, 2025NE002237</t>
   </si>
   <si>
-    <t>2026NE000330</t>
-  </si>
-  <si>
-    <t>C26163</t>
-  </si>
-  <si>
-    <t>26E0320</t>
-  </si>
-  <si>
     <t>2026NP400440</t>
   </si>
   <si>
-    <t>2026NE000388</t>
-  </si>
-  <si>
     <t>DEZ/25</t>
   </si>
   <si>
-    <t>C26193</t>
-  </si>
-  <si>
-    <t>26E0375</t>
-  </si>
-  <si>
     <t>2025NE001065, 2025NE002200</t>
   </si>
   <si>
     <t>2026NP400412</t>
   </si>
   <si>
-    <t>2026NE000748</t>
-  </si>
-  <si>
-    <t>C26312</t>
-  </si>
-  <si>
-    <t>26E0709</t>
-  </si>
-  <si>
     <t>JAN/26</t>
   </si>
   <si>
-    <t>2026NE000816</t>
-  </si>
-  <si>
     <t>2026NP401035</t>
   </si>
   <si>
-    <t>C26324</t>
-  </si>
-  <si>
-    <t>26E0776</t>
-  </si>
-  <si>
     <t>FEV/26</t>
   </si>
   <si>
-    <t>2026NE000817</t>
-  </si>
-  <si>
-    <t>C26326</t>
-  </si>
-  <si>
-    <t>26E0777</t>
-  </si>
-  <si>
     <t>2025NE001627, 2025NE001629, 2025NE001823</t>
   </si>
   <si>
     <t>2026NP402272</t>
-  </si>
-  <si>
-    <t>2026NE000842</t>
-  </si>
-  <si>
-    <t>26E0803</t>
   </si>
   <si>
     <t>MAR/26</t>
@@ -656,8 +656,8 @@
     <numFmt numFmtId="166" formatCode="dd/MM/yyyy"/>
     <numFmt numFmtId="167" formatCode="R$ #,##0.00"/>
     <numFmt numFmtId="168" formatCode="[$R$-416]\ #,##0.00;[RED]\-[$R$-416]\ #,##0.00"/>
-    <numFmt numFmtId="169" formatCode="MM/DD/YY"/>
-    <numFmt numFmtId="170" formatCode="d/m/yyyy"/>
+    <numFmt numFmtId="169" formatCode="d/m/yyyy"/>
+    <numFmt numFmtId="170" formatCode="MM/DD/YY"/>
     <numFmt numFmtId="171" formatCode="_([$R$ -416]* #,##0.00_);_([$R$ -416]* \(#,##0.00\);_([$R$ -416]* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="12">
@@ -852,35 +852,35 @@
     </xf>
     <xf borderId="0" fillId="3" fontId="2" numFmtId="0" xfId="0" applyFill="1" applyFont="1"/>
     <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyFill="1" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0"/>
+    </xf>
     <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="5" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
+      <alignment horizontal="left" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="11" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="left" readingOrder="0"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="11" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="left" readingOrder="0"/>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="right" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="right" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="4" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="right" readingOrder="0"/>
@@ -907,6 +907,9 @@
     <xf borderId="0" fillId="2" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
+    <xf borderId="1" fillId="0" fontId="6" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
@@ -919,9 +922,6 @@
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="6" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf borderId="1" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
@@ -931,6 +931,7 @@
     <xf borderId="1" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="165" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="2" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
@@ -955,15 +956,17 @@
     <xf borderId="1" fillId="8" fontId="7" numFmtId="168" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="165" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="3" fillId="0" fontId="10" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="169" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="right" readingOrder="0"/>
+    </xf>
     <xf borderId="1" fillId="8" fontId="9" numFmtId="168" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="8" numFmtId="166" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="8" numFmtId="169" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="8" numFmtId="170" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="7" fontId="9" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
@@ -975,23 +978,20 @@
     <xf borderId="1" fillId="8" fontId="9" numFmtId="168" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="4" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0"/>
+    </xf>
     <xf borderId="1" fillId="0" fontId="7" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="170" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="right" readingOrder="0"/>
-    </xf>
     <xf borderId="1" fillId="9" fontId="9" numFmtId="168" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="4" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="4" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0"/>
     </xf>
     <xf borderId="1" fillId="9" fontId="9" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
@@ -1400,42 +1400,42 @@
       <c r="V1" s="3"/>
     </row>
     <row r="2" ht="59.25" customHeight="1">
-      <c r="A2" s="4"/>
-      <c r="B2" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="V2" s="8"/>
-      <c r="W2" s="9"/>
-      <c r="X2" s="9"/>
-      <c r="Y2" s="9"/>
-      <c r="Z2" s="9"/>
-      <c r="AA2" s="9"/>
-      <c r="AB2" s="9"/>
-      <c r="AC2" s="9"/>
-      <c r="AD2" s="9"/>
+      <c r="A2" s="5"/>
+      <c r="B2" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="V2" s="9"/>
+      <c r="W2" s="11"/>
+      <c r="X2" s="11"/>
+      <c r="Y2" s="11"/>
+      <c r="Z2" s="11"/>
+      <c r="AA2" s="11"/>
+      <c r="AB2" s="11"/>
+      <c r="AC2" s="11"/>
+      <c r="AD2" s="11"/>
     </row>
     <row r="3" ht="12.75" customHeight="1">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
-      <c r="C3" s="12"/>
-      <c r="D3" s="12"/>
-      <c r="E3" s="12"/>
-      <c r="F3" s="12"/>
-      <c r="G3" s="12"/>
-      <c r="H3" s="12"/>
-      <c r="I3" s="12"/>
-      <c r="J3" s="12"/>
-      <c r="K3" s="12"/>
-      <c r="L3" s="12"/>
-      <c r="M3" s="12"/>
-      <c r="N3" s="12"/>
-      <c r="O3" s="12"/>
-      <c r="P3" s="12"/>
-      <c r="Q3" s="12"/>
-      <c r="R3" s="12"/>
-      <c r="S3" s="12"/>
-      <c r="T3" s="12"/>
-      <c r="U3" s="12"/>
+      <c r="C3" s="13"/>
+      <c r="D3" s="13"/>
+      <c r="E3" s="13"/>
+      <c r="F3" s="13"/>
+      <c r="G3" s="13"/>
+      <c r="H3" s="13"/>
+      <c r="I3" s="13"/>
+      <c r="J3" s="13"/>
+      <c r="K3" s="13"/>
+      <c r="L3" s="13"/>
+      <c r="M3" s="13"/>
+      <c r="N3" s="13"/>
+      <c r="O3" s="13"/>
+      <c r="P3" s="13"/>
+      <c r="Q3" s="13"/>
+      <c r="R3" s="13"/>
+      <c r="S3" s="13"/>
+      <c r="T3" s="13"/>
+      <c r="U3" s="13"/>
       <c r="V3" s="3"/>
     </row>
     <row r="4" ht="12.75" customHeight="1">
@@ -1457,28 +1457,28 @@
         <v>13</v>
       </c>
       <c r="H4" s="18" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="I4" s="17" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="J4" s="17" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="K4" s="17" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="L4" s="17" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="M4" s="18" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="N4" s="18" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="O4" s="18" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="P4" s="18" t="s">
         <v>25</v>
@@ -1496,7 +1496,7 @@
         <v>29</v>
       </c>
       <c r="U4" s="17" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="V4" s="3"/>
     </row>
@@ -1504,16 +1504,16 @@
       <c r="A5" s="16"/>
       <c r="B5" s="16"/>
       <c r="C5" s="19"/>
-      <c r="D5" s="10" t="s">
+      <c r="D5" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="E5" s="10" t="s">
+      <c r="E5" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="F5" s="10" t="s">
+      <c r="F5" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="G5" s="10" t="s">
+      <c r="G5" s="8" t="s">
         <v>35</v>
       </c>
       <c r="H5" s="20">
@@ -1522,17 +1522,17 @@
       <c r="I5" s="20">
         <v>1564.0</v>
       </c>
-      <c r="J5" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="K5" s="10" t="s">
-        <v>37</v>
-      </c>
-      <c r="L5" s="10" t="s">
-        <v>38</v>
-      </c>
-      <c r="M5" s="10" t="s">
+      <c r="J5" s="8" t="s">
         <v>39</v>
+      </c>
+      <c r="K5" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="L5" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="M5" s="8" t="s">
+        <v>43</v>
       </c>
       <c r="N5" s="14">
         <v>9.165159737E7</v>
@@ -1549,8 +1549,8 @@
       <c r="R5" s="14">
         <v>1.085943044E7</v>
       </c>
-      <c r="S5" s="10" t="s">
-        <v>43</v>
+      <c r="S5" s="8" t="s">
+        <v>44</v>
       </c>
       <c r="V5" s="3"/>
     </row>
@@ -1563,829 +1563,829 @@
     <row r="7" ht="12.75" customHeight="1">
       <c r="A7" s="22"/>
       <c r="B7" s="22"/>
-      <c r="C7" s="23"/>
-      <c r="D7" s="24"/>
-      <c r="E7" s="24"/>
-      <c r="F7" s="24"/>
-      <c r="G7" s="24"/>
-      <c r="H7" s="24"/>
-      <c r="I7" s="24"/>
-      <c r="J7" s="24"/>
-      <c r="K7" s="24"/>
-      <c r="L7" s="25"/>
-      <c r="M7" s="24"/>
-      <c r="N7" s="24"/>
-      <c r="O7" s="24"/>
-      <c r="P7" s="26"/>
+      <c r="C7" s="24"/>
+      <c r="D7" s="25"/>
+      <c r="E7" s="25"/>
+      <c r="F7" s="25"/>
+      <c r="G7" s="25"/>
+      <c r="H7" s="25"/>
+      <c r="I7" s="25"/>
+      <c r="J7" s="25"/>
+      <c r="K7" s="25"/>
+      <c r="L7" s="26"/>
+      <c r="M7" s="25"/>
+      <c r="N7" s="25"/>
+      <c r="O7" s="25"/>
+      <c r="P7" s="27"/>
       <c r="V7" s="3"/>
     </row>
     <row r="8" ht="12.75" customHeight="1">
       <c r="A8" s="22"/>
       <c r="B8" s="22"/>
       <c r="C8" s="28" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="D8" s="28" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="E8" s="29" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="F8" s="28" t="s">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="G8" s="28" t="s">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="H8" s="28" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="I8" s="29" t="s">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="J8" s="28" t="s">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="K8" s="28" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="L8" s="30" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="M8" s="29" t="s">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="N8" s="28" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="O8" s="28"/>
-      <c r="P8" s="26"/>
+      <c r="P8" s="27"/>
       <c r="V8" s="3"/>
     </row>
     <row r="9" ht="19.5" customHeight="1">
       <c r="A9" s="22"/>
       <c r="B9" s="22"/>
-      <c r="C9" s="31">
+      <c r="C9" s="32">
         <v>1.0</v>
       </c>
-      <c r="D9" s="32" t="s">
-        <v>69</v>
-      </c>
-      <c r="E9" s="33" t="s">
-        <v>70</v>
-      </c>
-      <c r="F9" s="34">
+      <c r="D9" s="33" t="s">
+        <v>78</v>
+      </c>
+      <c r="E9" s="34" t="s">
+        <v>79</v>
+      </c>
+      <c r="F9" s="35">
         <v>594.0</v>
       </c>
-      <c r="G9" s="35">
+      <c r="G9" s="36">
         <v>45740.0</v>
       </c>
-      <c r="H9" s="34" t="s">
-        <v>72</v>
-      </c>
-      <c r="I9" s="35"/>
-      <c r="J9" s="35">
+      <c r="H9" s="35" t="s">
+        <v>85</v>
+      </c>
+      <c r="I9" s="36"/>
+      <c r="J9" s="36">
         <v>45778.0</v>
       </c>
-      <c r="K9" s="36">
+      <c r="K9" s="37">
         <v>748504.24</v>
       </c>
-      <c r="L9" s="34" t="s">
-        <v>76</v>
-      </c>
-      <c r="M9" s="37">
+      <c r="L9" s="35" t="s">
+        <v>89</v>
+      </c>
+      <c r="M9" s="38">
         <f t="shared" ref="M9:M10" si="1">K9</f>
         <v>748504.24</v>
       </c>
-      <c r="N9" s="38"/>
-      <c r="O9" s="24"/>
-      <c r="P9" s="26"/>
+      <c r="N9" s="39"/>
+      <c r="O9" s="25"/>
+      <c r="P9" s="27"/>
       <c r="V9" s="3"/>
     </row>
     <row r="10" ht="51.0" customHeight="1">
       <c r="A10" s="22"/>
       <c r="B10" s="22"/>
       <c r="C10" s="40"/>
-      <c r="D10" s="32" t="s">
+      <c r="D10" s="33" t="s">
+        <v>96</v>
+      </c>
+      <c r="E10" s="34" t="s">
         <v>79</v>
       </c>
-      <c r="E10" s="33" t="s">
-        <v>70</v>
-      </c>
-      <c r="F10" s="34">
+      <c r="F10" s="35">
         <v>620.0</v>
       </c>
-      <c r="G10" s="35">
+      <c r="G10" s="36">
         <v>45775.0</v>
       </c>
-      <c r="H10" s="34" t="s">
-        <v>83</v>
-      </c>
-      <c r="I10" s="35"/>
-      <c r="J10" s="35">
+      <c r="H10" s="35" t="s">
+        <v>99</v>
+      </c>
+      <c r="I10" s="36"/>
+      <c r="J10" s="36">
         <v>45806.0</v>
       </c>
-      <c r="K10" s="36">
+      <c r="K10" s="37">
         <v>1110378.24</v>
       </c>
-      <c r="L10" s="34" t="s">
-        <v>84</v>
-      </c>
-      <c r="M10" s="37">
+      <c r="L10" s="35" t="s">
+        <v>100</v>
+      </c>
+      <c r="M10" s="38">
         <f t="shared" si="1"/>
         <v>1110378.24</v>
       </c>
-      <c r="N10" s="41"/>
-      <c r="O10" s="24"/>
-      <c r="P10" s="26"/>
+      <c r="N10" s="42"/>
+      <c r="O10" s="25"/>
+      <c r="P10" s="27"/>
       <c r="V10" s="3"/>
     </row>
     <row r="11" ht="12.75" customHeight="1">
       <c r="A11" s="22"/>
       <c r="B11" s="22"/>
       <c r="C11" s="40"/>
-      <c r="D11" s="32" t="s">
-        <v>88</v>
-      </c>
-      <c r="E11" s="33" t="s">
-        <v>70</v>
-      </c>
-      <c r="F11" s="34">
+      <c r="D11" s="33" t="s">
+        <v>108</v>
+      </c>
+      <c r="E11" s="34" t="s">
+        <v>79</v>
+      </c>
+      <c r="F11" s="35">
         <v>634.0</v>
       </c>
-      <c r="G11" s="35">
+      <c r="G11" s="36">
         <v>45799.0</v>
       </c>
-      <c r="H11" s="34" t="s">
-        <v>89</v>
-      </c>
-      <c r="I11" s="35"/>
-      <c r="J11" s="35">
+      <c r="H11" s="35" t="s">
+        <v>110</v>
+      </c>
+      <c r="I11" s="36"/>
+      <c r="J11" s="36">
         <v>45844.0</v>
       </c>
-      <c r="K11" s="36">
+      <c r="K11" s="37">
         <v>974557.12</v>
       </c>
-      <c r="L11" s="33" t="s">
-        <v>92</v>
-      </c>
-      <c r="M11" s="37">
+      <c r="L11" s="34" t="s">
+        <v>112</v>
+      </c>
+      <c r="M11" s="38">
         <v>974557.12</v>
       </c>
-      <c r="N11" s="41"/>
-      <c r="O11" s="24"/>
-      <c r="P11" s="26"/>
+      <c r="N11" s="42"/>
+      <c r="O11" s="25"/>
+      <c r="P11" s="27"/>
       <c r="V11" s="3"/>
     </row>
     <row r="12" ht="27.75" customHeight="1">
       <c r="A12" s="22"/>
       <c r="B12" s="22"/>
       <c r="C12" s="40"/>
-      <c r="D12" s="32" t="s">
-        <v>93</v>
-      </c>
-      <c r="E12" s="33" t="s">
-        <v>70</v>
-      </c>
-      <c r="F12" s="33">
+      <c r="D12" s="33" t="s">
+        <v>116</v>
+      </c>
+      <c r="E12" s="34" t="s">
+        <v>79</v>
+      </c>
+      <c r="F12" s="34">
         <v>660.0</v>
       </c>
-      <c r="G12" s="42">
+      <c r="G12" s="43">
         <v>45856.0</v>
       </c>
-      <c r="H12" s="43" t="s">
-        <v>71</v>
-      </c>
-      <c r="I12" s="35"/>
-      <c r="J12" s="35">
+      <c r="H12" s="44" t="s">
+        <v>60</v>
+      </c>
+      <c r="I12" s="36"/>
+      <c r="J12" s="36">
         <v>45891.0</v>
       </c>
-      <c r="K12" s="44">
+      <c r="K12" s="45">
         <v>1402001.34</v>
       </c>
-      <c r="L12" s="45" t="s">
-        <v>97</v>
-      </c>
-      <c r="M12" s="37">
+      <c r="L12" s="46" t="s">
+        <v>124</v>
+      </c>
+      <c r="M12" s="38">
         <v>1402001.34</v>
       </c>
-      <c r="N12" s="46"/>
-      <c r="O12" s="24"/>
-      <c r="P12" s="26"/>
+      <c r="N12" s="47"/>
+      <c r="O12" s="25"/>
+      <c r="P12" s="27"/>
       <c r="V12" s="3"/>
     </row>
     <row r="13">
       <c r="A13" s="22"/>
       <c r="B13" s="22"/>
       <c r="C13" s="40"/>
-      <c r="D13" s="47" t="s">
-        <v>100</v>
-      </c>
-      <c r="E13" s="33" t="s">
-        <v>70</v>
-      </c>
-      <c r="F13" s="34">
+      <c r="D13" s="49" t="s">
+        <v>129</v>
+      </c>
+      <c r="E13" s="34" t="s">
+        <v>79</v>
+      </c>
+      <c r="F13" s="35">
         <v>661.0</v>
       </c>
-      <c r="G13" s="35">
+      <c r="G13" s="36">
         <v>45856.0</v>
       </c>
-      <c r="H13" s="34" t="s">
-        <v>103</v>
-      </c>
-      <c r="I13" s="42"/>
-      <c r="J13" s="42">
+      <c r="H13" s="35" t="s">
+        <v>133</v>
+      </c>
+      <c r="I13" s="43"/>
+      <c r="J13" s="43">
         <v>45891.0</v>
       </c>
-      <c r="K13" s="44">
+      <c r="K13" s="45">
         <v>1223702.3</v>
       </c>
-      <c r="L13" s="33" t="s">
-        <v>104</v>
-      </c>
-      <c r="M13" s="37">
+      <c r="L13" s="34" t="s">
+        <v>134</v>
+      </c>
+      <c r="M13" s="38">
         <v>1223702.3</v>
       </c>
-      <c r="N13" s="46"/>
-      <c r="O13" s="24"/>
-      <c r="P13" s="48"/>
+      <c r="N13" s="47"/>
+      <c r="O13" s="25"/>
+      <c r="P13" s="50"/>
       <c r="V13" s="3"/>
     </row>
     <row r="14">
       <c r="A14" s="22"/>
       <c r="B14" s="22"/>
       <c r="C14" s="40"/>
-      <c r="D14" s="47" t="s">
-        <v>107</v>
-      </c>
-      <c r="E14" s="33" t="s">
-        <v>70</v>
-      </c>
-      <c r="F14" s="33">
+      <c r="D14" s="49" t="s">
+        <v>138</v>
+      </c>
+      <c r="E14" s="34" t="s">
+        <v>79</v>
+      </c>
+      <c r="F14" s="34">
         <v>688.0</v>
       </c>
-      <c r="G14" s="35">
+      <c r="G14" s="36">
         <v>45901.0</v>
       </c>
-      <c r="H14" s="33" t="s">
-        <v>108</v>
-      </c>
-      <c r="I14" s="42"/>
-      <c r="J14" s="42">
+      <c r="H14" s="34" t="s">
+        <v>141</v>
+      </c>
+      <c r="I14" s="43"/>
+      <c r="J14" s="43">
         <v>45938.0</v>
       </c>
-      <c r="K14" s="44">
+      <c r="K14" s="45">
         <v>1011677.95</v>
       </c>
-      <c r="L14" s="33" t="s">
-        <v>109</v>
-      </c>
-      <c r="M14" s="37">
+      <c r="L14" s="34" t="s">
+        <v>142</v>
+      </c>
+      <c r="M14" s="38">
         <v>1011677.95</v>
       </c>
-      <c r="N14" s="41"/>
-      <c r="O14" s="24"/>
-      <c r="P14" s="26"/>
+      <c r="N14" s="42"/>
+      <c r="O14" s="25"/>
+      <c r="P14" s="27"/>
       <c r="V14" s="3"/>
     </row>
     <row r="15">
       <c r="A15" s="22"/>
       <c r="B15" s="22"/>
       <c r="C15" s="40"/>
-      <c r="D15" s="47" t="s">
-        <v>112</v>
-      </c>
-      <c r="E15" s="33" t="s">
-        <v>70</v>
-      </c>
-      <c r="F15" s="33">
+      <c r="D15" s="49" t="s">
+        <v>143</v>
+      </c>
+      <c r="E15" s="34" t="s">
+        <v>79</v>
+      </c>
+      <c r="F15" s="34">
         <v>696.0</v>
       </c>
-      <c r="G15" s="35">
+      <c r="G15" s="36">
         <v>45923.0</v>
       </c>
-      <c r="H15" s="33" t="s">
-        <v>80</v>
-      </c>
-      <c r="I15" s="42"/>
-      <c r="J15" s="42">
+      <c r="H15" s="34" t="s">
+        <v>75</v>
+      </c>
+      <c r="I15" s="43"/>
+      <c r="J15" s="43">
         <v>45938.0</v>
       </c>
-      <c r="K15" s="44">
+      <c r="K15" s="45">
         <v>896744.06</v>
       </c>
-      <c r="L15" s="33" t="s">
-        <v>116</v>
-      </c>
-      <c r="M15" s="37">
+      <c r="L15" s="34" t="s">
+        <v>144</v>
+      </c>
+      <c r="M15" s="38">
         <v>896744.06</v>
       </c>
-      <c r="N15" s="46"/>
-      <c r="O15" s="24"/>
+      <c r="N15" s="47"/>
+      <c r="O15" s="25"/>
       <c r="V15" s="3"/>
     </row>
     <row r="16">
       <c r="A16" s="22"/>
       <c r="B16" s="22"/>
       <c r="C16" s="40"/>
-      <c r="D16" s="47" t="s">
-        <v>117</v>
-      </c>
-      <c r="E16" s="33" t="s">
-        <v>70</v>
-      </c>
-      <c r="F16" s="33">
+      <c r="D16" s="49" t="s">
+        <v>145</v>
+      </c>
+      <c r="E16" s="34" t="s">
+        <v>79</v>
+      </c>
+      <c r="F16" s="34">
         <v>704.0</v>
       </c>
-      <c r="G16" s="35">
+      <c r="G16" s="36">
         <v>45957.0</v>
       </c>
-      <c r="H16" s="33" t="s">
-        <v>121</v>
-      </c>
-      <c r="I16" s="42"/>
-      <c r="J16" s="42">
+      <c r="H16" s="34" t="s">
+        <v>146</v>
+      </c>
+      <c r="I16" s="43"/>
+      <c r="J16" s="43">
         <v>46003.0</v>
       </c>
-      <c r="K16" s="44">
+      <c r="K16" s="45">
         <v>919329.06</v>
       </c>
-      <c r="L16" s="33" t="s">
-        <v>123</v>
-      </c>
-      <c r="M16" s="37">
+      <c r="L16" s="34" t="s">
+        <v>147</v>
+      </c>
+      <c r="M16" s="38">
         <v>919329.06</v>
       </c>
-      <c r="N16" s="41"/>
-      <c r="O16" s="24"/>
+      <c r="N16" s="42"/>
+      <c r="O16" s="25"/>
       <c r="V16" s="3"/>
     </row>
     <row r="17">
       <c r="A17" s="22"/>
       <c r="B17" s="22"/>
       <c r="C17" s="40"/>
-      <c r="D17" s="47" t="s">
-        <v>126</v>
-      </c>
-      <c r="E17" s="33"/>
-      <c r="F17" s="33">
+      <c r="D17" s="49" t="s">
+        <v>148</v>
+      </c>
+      <c r="E17" s="34"/>
+      <c r="F17" s="34">
         <v>705.0</v>
       </c>
-      <c r="G17" s="42">
+      <c r="G17" s="43">
         <v>45972.0</v>
       </c>
-      <c r="H17" s="33" t="s">
-        <v>127</v>
-      </c>
-      <c r="I17" s="33"/>
-      <c r="J17" s="42">
+      <c r="H17" s="34" t="s">
+        <v>149</v>
+      </c>
+      <c r="I17" s="34"/>
+      <c r="J17" s="43">
         <v>46016.0</v>
       </c>
-      <c r="K17" s="44">
+      <c r="K17" s="45">
         <v>1157009.26</v>
       </c>
-      <c r="L17" s="33" t="s">
-        <v>131</v>
-      </c>
-      <c r="M17" s="37">
+      <c r="L17" s="34" t="s">
+        <v>150</v>
+      </c>
+      <c r="M17" s="38">
         <v>1157009.26</v>
       </c>
-      <c r="N17" s="50"/>
-      <c r="O17" s="24"/>
+      <c r="N17" s="51"/>
+      <c r="O17" s="25"/>
       <c r="V17" s="3"/>
     </row>
     <row r="18">
       <c r="A18" s="22"/>
       <c r="B18" s="22"/>
       <c r="C18" s="40"/>
-      <c r="D18" s="47" t="s">
-        <v>134</v>
-      </c>
-      <c r="E18" s="33" t="s">
-        <v>70</v>
-      </c>
-      <c r="F18" s="33">
+      <c r="D18" s="49" t="s">
+        <v>151</v>
+      </c>
+      <c r="E18" s="34" t="s">
+        <v>79</v>
+      </c>
+      <c r="F18" s="34">
         <v>728.0</v>
       </c>
-      <c r="G18" s="42">
+      <c r="G18" s="43">
         <v>46008.0</v>
       </c>
-      <c r="H18" s="33" t="s">
-        <v>135</v>
-      </c>
-      <c r="I18" s="33"/>
-      <c r="J18" s="42">
+      <c r="H18" s="34" t="s">
+        <v>152</v>
+      </c>
+      <c r="I18" s="34"/>
+      <c r="J18" s="43">
         <v>46040.0</v>
       </c>
-      <c r="K18" s="44">
+      <c r="K18" s="45">
         <v>1214597.952</v>
       </c>
-      <c r="L18" s="33" t="s">
-        <v>139</v>
-      </c>
-      <c r="M18" s="37">
+      <c r="L18" s="34" t="s">
+        <v>153</v>
+      </c>
+      <c r="M18" s="38">
         <v>1214597.952</v>
       </c>
-      <c r="N18" s="50"/>
-      <c r="O18" s="24"/>
-      <c r="R18" s="26"/>
-      <c r="S18" s="26"/>
-      <c r="T18" s="26"/>
-      <c r="U18" s="26"/>
-      <c r="V18" s="51"/>
+      <c r="N18" s="51"/>
+      <c r="O18" s="25"/>
+      <c r="R18" s="27"/>
+      <c r="S18" s="27"/>
+      <c r="T18" s="27"/>
+      <c r="U18" s="27"/>
+      <c r="V18" s="52"/>
     </row>
     <row r="19">
       <c r="A19" s="22"/>
       <c r="B19" s="22"/>
       <c r="C19" s="40"/>
-      <c r="D19" s="47" t="s">
-        <v>141</v>
-      </c>
-      <c r="E19" s="33" t="s">
-        <v>70</v>
-      </c>
-      <c r="F19" s="33">
+      <c r="D19" s="49" t="s">
+        <v>154</v>
+      </c>
+      <c r="E19" s="34" t="s">
+        <v>79</v>
+      </c>
+      <c r="F19" s="34">
         <v>278.0</v>
       </c>
-      <c r="G19" s="42">
+      <c r="G19" s="43">
         <v>46042.0</v>
       </c>
-      <c r="H19" s="33" t="s">
-        <v>144</v>
-      </c>
-      <c r="I19" s="42"/>
-      <c r="J19" s="42">
+      <c r="H19" s="34" t="s">
+        <v>155</v>
+      </c>
+      <c r="I19" s="43"/>
+      <c r="J19" s="43">
         <v>46074.0</v>
       </c>
-      <c r="K19" s="44">
+      <c r="K19" s="45">
         <v>967082.09</v>
       </c>
-      <c r="L19" s="33" t="s">
-        <v>145</v>
-      </c>
-      <c r="M19" s="37">
+      <c r="L19" s="34" t="s">
+        <v>156</v>
+      </c>
+      <c r="M19" s="38">
         <v>967082.09</v>
       </c>
-      <c r="N19" s="50"/>
-      <c r="O19" s="24"/>
-      <c r="R19" s="26"/>
-      <c r="S19" s="26"/>
-      <c r="T19" s="26"/>
-      <c r="U19" s="26"/>
-      <c r="V19" s="51"/>
+      <c r="N19" s="51"/>
+      <c r="O19" s="25"/>
+      <c r="R19" s="27"/>
+      <c r="S19" s="27"/>
+      <c r="T19" s="27"/>
+      <c r="U19" s="27"/>
+      <c r="V19" s="52"/>
     </row>
     <row r="20">
       <c r="A20" s="22"/>
       <c r="B20" s="22"/>
       <c r="C20" s="40"/>
-      <c r="D20" s="47" t="s">
-        <v>149</v>
-      </c>
-      <c r="E20" s="33"/>
-      <c r="F20" s="33">
+      <c r="D20" s="49" t="s">
+        <v>157</v>
+      </c>
+      <c r="E20" s="34"/>
+      <c r="F20" s="34">
         <v>10.0</v>
       </c>
-      <c r="G20" s="42">
+      <c r="G20" s="43">
         <v>46078.0</v>
       </c>
-      <c r="H20" s="33" t="s">
-        <v>113</v>
-      </c>
-      <c r="I20" s="42"/>
-      <c r="J20" s="42">
+      <c r="H20" s="34" t="s">
+        <v>101</v>
+      </c>
+      <c r="I20" s="43"/>
+      <c r="J20" s="43">
         <v>46106.0</v>
       </c>
-      <c r="K20" s="44">
+      <c r="K20" s="45">
         <v>719561.08</v>
       </c>
-      <c r="L20" s="33" t="s">
-        <v>151</v>
-      </c>
-      <c r="M20" s="37">
+      <c r="L20" s="34" t="s">
+        <v>158</v>
+      </c>
+      <c r="M20" s="38">
         <v>719561.08</v>
       </c>
-      <c r="N20" s="50"/>
-      <c r="O20" s="24"/>
-      <c r="R20" s="26"/>
-      <c r="S20" s="26"/>
-      <c r="T20" s="26"/>
-      <c r="U20" s="26"/>
-      <c r="V20" s="51"/>
+      <c r="N20" s="51"/>
+      <c r="O20" s="25"/>
+      <c r="R20" s="27"/>
+      <c r="S20" s="27"/>
+      <c r="T20" s="27"/>
+      <c r="U20" s="27"/>
+      <c r="V20" s="52"/>
     </row>
     <row r="21">
       <c r="A21" s="22"/>
       <c r="B21" s="22"/>
       <c r="C21" s="40"/>
-      <c r="D21" s="47" t="s">
-        <v>154</v>
-      </c>
-      <c r="E21" s="33"/>
-      <c r="F21" s="33">
+      <c r="D21" s="49" t="s">
+        <v>159</v>
+      </c>
+      <c r="E21" s="34"/>
+      <c r="F21" s="34">
         <v>15.0</v>
       </c>
-      <c r="G21" s="42">
+      <c r="G21" s="43">
         <v>46094.0</v>
       </c>
-      <c r="H21" s="33" t="s">
-        <v>158</v>
-      </c>
-      <c r="I21" s="42"/>
-      <c r="J21" s="42">
+      <c r="H21" s="34" t="s">
+        <v>160</v>
+      </c>
+      <c r="I21" s="43"/>
+      <c r="J21" s="43">
         <v>46128.0</v>
       </c>
-      <c r="K21" s="44">
+      <c r="K21" s="45">
         <v>885881.08</v>
       </c>
-      <c r="L21" s="33" t="s">
-        <v>159</v>
-      </c>
-      <c r="M21" s="37">
+      <c r="L21" s="34" t="s">
+        <v>161</v>
+      </c>
+      <c r="M21" s="38">
         <v>885881.08</v>
       </c>
-      <c r="N21" s="50"/>
-      <c r="O21" s="24"/>
-      <c r="R21" s="26"/>
-      <c r="S21" s="26"/>
-      <c r="T21" s="26"/>
-      <c r="U21" s="26"/>
-      <c r="V21" s="51"/>
+      <c r="N21" s="51"/>
+      <c r="O21" s="25"/>
+      <c r="R21" s="27"/>
+      <c r="S21" s="27"/>
+      <c r="T21" s="27"/>
+      <c r="U21" s="27"/>
+      <c r="V21" s="52"/>
     </row>
     <row r="22">
       <c r="A22" s="22"/>
       <c r="B22" s="22"/>
       <c r="C22" s="40"/>
-      <c r="D22" s="47" t="s">
+      <c r="D22" s="49" t="s">
         <v>162</v>
       </c>
-      <c r="E22" s="33"/>
-      <c r="F22" s="33">
+      <c r="E22" s="34"/>
+      <c r="F22" s="34">
         <v>28.0</v>
       </c>
-      <c r="G22" s="42">
+      <c r="G22" s="43">
         <v>46128.0</v>
       </c>
-      <c r="H22" s="33" t="s">
+      <c r="H22" s="34" t="s">
         <v>163</v>
       </c>
-      <c r="I22" s="42"/>
-      <c r="J22" s="42">
+      <c r="I22" s="43"/>
+      <c r="J22" s="43">
         <v>46164.0</v>
       </c>
-      <c r="K22" s="44" t="s">
+      <c r="K22" s="45" t="s">
         <v>164</v>
       </c>
-      <c r="L22" s="33" t="s">
+      <c r="L22" s="34" t="s">
         <v>165</v>
       </c>
-      <c r="M22" s="37" t="s">
+      <c r="M22" s="38" t="s">
         <v>164</v>
       </c>
-      <c r="N22" s="50"/>
-      <c r="O22" s="24"/>
-      <c r="R22" s="26"/>
-      <c r="S22" s="26"/>
-      <c r="T22" s="26"/>
-      <c r="U22" s="26"/>
-      <c r="V22" s="51"/>
+      <c r="N22" s="51"/>
+      <c r="O22" s="25"/>
+      <c r="R22" s="27"/>
+      <c r="S22" s="27"/>
+      <c r="T22" s="27"/>
+      <c r="U22" s="27"/>
+      <c r="V22" s="52"/>
     </row>
     <row r="23">
       <c r="A23" s="22"/>
       <c r="B23" s="22"/>
       <c r="C23" s="40"/>
-      <c r="D23" s="47" t="s">
+      <c r="D23" s="49" t="s">
         <v>166</v>
       </c>
-      <c r="E23" s="33"/>
-      <c r="F23" s="33">
+      <c r="E23" s="34"/>
+      <c r="F23" s="34">
         <v>33.0</v>
       </c>
-      <c r="G23" s="42">
+      <c r="G23" s="43">
         <v>46156.0</v>
       </c>
-      <c r="H23" s="33" t="s">
+      <c r="H23" s="34" t="s">
         <v>167</v>
       </c>
-      <c r="I23" s="42"/>
-      <c r="J23" s="42">
+      <c r="I23" s="43"/>
+      <c r="J23" s="43">
         <v>46191.0</v>
       </c>
-      <c r="K23" s="44">
+      <c r="K23" s="45">
         <v>1108954.4358333333</v>
       </c>
-      <c r="L23" s="33" t="s">
-        <v>159</v>
-      </c>
-      <c r="M23" s="37">
+      <c r="L23" s="34" t="s">
+        <v>161</v>
+      </c>
+      <c r="M23" s="38">
         <v>1108954.4358333333</v>
       </c>
       <c r="N23" s="53"/>
-      <c r="O23" s="24"/>
-      <c r="R23" s="26"/>
-      <c r="S23" s="26"/>
-      <c r="T23" s="26"/>
-      <c r="U23" s="26"/>
-      <c r="V23" s="51"/>
+      <c r="O23" s="25"/>
+      <c r="R23" s="27"/>
+      <c r="S23" s="27"/>
+      <c r="T23" s="27"/>
+      <c r="U23" s="27"/>
+      <c r="V23" s="52"/>
     </row>
     <row r="24">
       <c r="A24" s="22"/>
       <c r="B24" s="22"/>
       <c r="C24" s="40"/>
-      <c r="D24" s="47" t="s">
+      <c r="D24" s="49" t="s">
         <v>168</v>
       </c>
-      <c r="E24" s="33"/>
-      <c r="F24" s="33">
+      <c r="E24" s="34"/>
+      <c r="F24" s="34">
         <v>29.0</v>
       </c>
-      <c r="G24" s="42">
+      <c r="G24" s="43">
         <v>46149.0</v>
       </c>
-      <c r="H24" s="33" t="s">
+      <c r="H24" s="34" t="s">
         <v>167</v>
       </c>
-      <c r="I24" s="42"/>
-      <c r="J24" s="42">
+      <c r="I24" s="43"/>
+      <c r="J24" s="43">
         <v>46185.0</v>
       </c>
-      <c r="K24" s="44">
+      <c r="K24" s="45">
         <v>218206.1</v>
       </c>
-      <c r="L24" s="33" t="s">
+      <c r="L24" s="34" t="s">
         <v>169</v>
       </c>
-      <c r="M24" s="37">
+      <c r="M24" s="38">
         <v>218206.1</v>
       </c>
       <c r="N24" s="54"/>
-      <c r="O24" s="24"/>
-      <c r="R24" s="26"/>
-      <c r="S24" s="26"/>
-      <c r="T24" s="26"/>
-      <c r="U24" s="26"/>
-      <c r="V24" s="51"/>
+      <c r="O24" s="25"/>
+      <c r="R24" s="27"/>
+      <c r="S24" s="27"/>
+      <c r="T24" s="27"/>
+      <c r="U24" s="27"/>
+      <c r="V24" s="52"/>
     </row>
     <row r="25">
       <c r="A25" s="22"/>
       <c r="B25" s="22"/>
       <c r="C25" s="40"/>
-      <c r="D25" s="47" t="s">
+      <c r="D25" s="49" t="s">
         <v>170</v>
       </c>
-      <c r="E25" s="33"/>
+      <c r="E25" s="34"/>
       <c r="F25" s="55">
         <v>40.0</v>
       </c>
-      <c r="G25" s="42">
+      <c r="G25" s="43">
         <v>46156.0</v>
       </c>
       <c r="H25" s="55" t="s">
         <v>167</v>
       </c>
-      <c r="I25" s="42"/>
+      <c r="I25" s="43"/>
       <c r="J25" s="56">
         <v>46191.0</v>
       </c>
-      <c r="K25" s="44">
+      <c r="K25" s="45">
         <v>1549250.84</v>
       </c>
-      <c r="L25" s="33" t="s">
+      <c r="L25" s="34" t="s">
         <v>171</v>
       </c>
-      <c r="M25" s="37">
+      <c r="M25" s="38">
         <v>1549250.84</v>
       </c>
       <c r="N25" s="53"/>
-      <c r="O25" s="24"/>
-      <c r="R25" s="26"/>
-      <c r="S25" s="26"/>
-      <c r="T25" s="26"/>
-      <c r="U25" s="26"/>
-      <c r="V25" s="51"/>
+      <c r="O25" s="25"/>
+      <c r="R25" s="27"/>
+      <c r="S25" s="27"/>
+      <c r="T25" s="27"/>
+      <c r="U25" s="27"/>
+      <c r="V25" s="52"/>
     </row>
     <row r="26">
       <c r="A26" s="22"/>
       <c r="B26" s="22"/>
       <c r="C26" s="57"/>
-      <c r="D26" s="47" t="s">
+      <c r="D26" s="49" t="s">
         <v>172</v>
       </c>
-      <c r="E26" s="33"/>
+      <c r="E26" s="34"/>
       <c r="F26" s="55"/>
-      <c r="G26" s="42"/>
+      <c r="G26" s="43"/>
       <c r="H26" s="55"/>
-      <c r="I26" s="42"/>
+      <c r="I26" s="43"/>
       <c r="J26" s="56"/>
-      <c r="K26" s="44"/>
-      <c r="L26" s="33" t="s">
-        <v>65</v>
-      </c>
-      <c r="M26" s="37" t="s">
+      <c r="K26" s="45"/>
+      <c r="L26" s="34" t="s">
+        <v>73</v>
+      </c>
+      <c r="M26" s="38" t="s">
         <v>173</v>
       </c>
       <c r="N26" s="53"/>
-      <c r="O26" s="24"/>
-      <c r="R26" s="26"/>
-      <c r="S26" s="26"/>
-      <c r="T26" s="26"/>
-      <c r="U26" s="26"/>
-      <c r="V26" s="51"/>
+      <c r="O26" s="25"/>
+      <c r="R26" s="27"/>
+      <c r="S26" s="27"/>
+      <c r="T26" s="27"/>
+      <c r="U26" s="27"/>
+      <c r="V26" s="52"/>
     </row>
     <row r="27" ht="30.75" customHeight="1">
       <c r="A27" s="22"/>
       <c r="B27" s="22"/>
       <c r="C27" s="28" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="D27" s="28" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="E27" s="29" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="F27" s="28" t="s">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="G27" s="28"/>
       <c r="H27" s="28" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="I27" s="28"/>
       <c r="J27" s="28"/>
       <c r="K27" s="58" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="L27" s="30" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="M27" s="59" t="s">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="N27" s="28" t="s">
-        <v>66</v>
-      </c>
-      <c r="O27" s="24"/>
-      <c r="P27" s="26"/>
-      <c r="R27" s="26"/>
-      <c r="S27" s="26"/>
-      <c r="T27" s="26"/>
-      <c r="U27" s="26"/>
-      <c r="V27" s="51"/>
-      <c r="W27" s="26"/>
-      <c r="X27" s="26"/>
-      <c r="Y27" s="26"/>
-      <c r="Z27" s="26"/>
-      <c r="AA27" s="26"/>
-      <c r="AB27" s="26"/>
-      <c r="AC27" s="26"/>
+        <v>74</v>
+      </c>
+      <c r="O27" s="25"/>
+      <c r="P27" s="27"/>
+      <c r="R27" s="27"/>
+      <c r="S27" s="27"/>
+      <c r="T27" s="27"/>
+      <c r="U27" s="27"/>
+      <c r="V27" s="52"/>
+      <c r="W27" s="27"/>
+      <c r="X27" s="27"/>
+      <c r="Y27" s="27"/>
+      <c r="Z27" s="27"/>
+      <c r="AA27" s="27"/>
+      <c r="AB27" s="27"/>
+      <c r="AC27" s="27"/>
     </row>
     <row r="28" ht="12.75" customHeight="1">
       <c r="A28" s="22"/>
       <c r="B28" s="22"/>
-      <c r="C28" s="31">
+      <c r="C28" s="32">
         <v>2.0</v>
       </c>
       <c r="D28" s="60" t="s">
         <v>174</v>
       </c>
-      <c r="E28" s="34"/>
-      <c r="F28" s="34">
+      <c r="E28" s="35"/>
+      <c r="F28" s="35">
         <v>402.0</v>
       </c>
-      <c r="G28" s="35">
+      <c r="G28" s="36">
         <v>45791.0</v>
       </c>
-      <c r="H28" s="34" t="s">
-        <v>51</v>
-      </c>
-      <c r="I28" s="35"/>
-      <c r="J28" s="35">
+      <c r="H28" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="I28" s="36"/>
+      <c r="J28" s="36">
         <v>45834.0</v>
       </c>
-      <c r="K28" s="36">
+      <c r="K28" s="37">
         <v>188246.17</v>
       </c>
-      <c r="L28" s="33" t="s">
+      <c r="L28" s="34" t="s">
         <v>175</v>
       </c>
       <c r="M28" s="61">
         <v>188246.17</v>
       </c>
-      <c r="N28" s="50"/>
-      <c r="O28" s="24"/>
-      <c r="P28" s="26"/>
-      <c r="Q28" s="26"/>
-      <c r="R28" s="26"/>
-      <c r="S28" s="26"/>
-      <c r="T28" s="26"/>
-      <c r="U28" s="26"/>
-      <c r="V28" s="51"/>
-      <c r="W28" s="26"/>
-      <c r="X28" s="26"/>
-      <c r="Y28" s="26"/>
-      <c r="Z28" s="26"/>
-      <c r="AA28" s="26"/>
-      <c r="AB28" s="26"/>
-      <c r="AC28" s="26"/>
+      <c r="N28" s="51"/>
+      <c r="O28" s="25"/>
+      <c r="P28" s="27"/>
+      <c r="Q28" s="27"/>
+      <c r="R28" s="27"/>
+      <c r="S28" s="27"/>
+      <c r="T28" s="27"/>
+      <c r="U28" s="27"/>
+      <c r="V28" s="52"/>
+      <c r="W28" s="27"/>
+      <c r="X28" s="27"/>
+      <c r="Y28" s="27"/>
+      <c r="Z28" s="27"/>
+      <c r="AA28" s="27"/>
+      <c r="AB28" s="27"/>
+      <c r="AC28" s="27"/>
     </row>
     <row r="29">
       <c r="A29" s="22"/>
@@ -2397,44 +2397,44 @@
       <c r="E29" s="55">
         <v>46.0</v>
       </c>
-      <c r="F29" s="34">
+      <c r="F29" s="35">
         <v>447.0</v>
       </c>
-      <c r="G29" s="35">
+      <c r="G29" s="36">
         <v>45814.0</v>
       </c>
-      <c r="H29" s="33" t="s">
+      <c r="H29" s="34" t="s">
         <v>177</v>
       </c>
-      <c r="I29" s="42"/>
-      <c r="J29" s="42">
+      <c r="I29" s="43"/>
+      <c r="J29" s="43">
         <v>45955.0</v>
       </c>
-      <c r="K29" s="36">
+      <c r="K29" s="37">
         <v>112720.77</v>
       </c>
-      <c r="L29" s="33" t="s">
+      <c r="L29" s="34" t="s">
         <v>178</v>
       </c>
-      <c r="M29" s="37">
+      <c r="M29" s="38">
         <v>112720.77</v>
       </c>
-      <c r="N29" s="50"/>
-      <c r="O29" s="24"/>
-      <c r="P29" s="26"/>
-      <c r="Q29" s="26"/>
-      <c r="R29" s="26"/>
-      <c r="S29" s="26"/>
-      <c r="T29" s="26"/>
-      <c r="U29" s="26"/>
-      <c r="V29" s="51"/>
-      <c r="W29" s="26"/>
-      <c r="X29" s="26"/>
-      <c r="Y29" s="26"/>
-      <c r="Z29" s="26"/>
-      <c r="AA29" s="26"/>
-      <c r="AB29" s="26"/>
-      <c r="AC29" s="26"/>
+      <c r="N29" s="51"/>
+      <c r="O29" s="25"/>
+      <c r="P29" s="27"/>
+      <c r="Q29" s="27"/>
+      <c r="R29" s="27"/>
+      <c r="S29" s="27"/>
+      <c r="T29" s="27"/>
+      <c r="U29" s="27"/>
+      <c r="V29" s="52"/>
+      <c r="W29" s="27"/>
+      <c r="X29" s="27"/>
+      <c r="Y29" s="27"/>
+      <c r="Z29" s="27"/>
+      <c r="AA29" s="27"/>
+      <c r="AB29" s="27"/>
+      <c r="AC29" s="27"/>
     </row>
     <row r="30" ht="12.75" customHeight="1">
       <c r="A30" s="22"/>
@@ -2446,44 +2446,44 @@
       <c r="E30" s="63" t="s">
         <v>180</v>
       </c>
-      <c r="F30" s="34">
+      <c r="F30" s="35">
         <v>529.0</v>
       </c>
       <c r="G30" s="64">
         <v>45853.0</v>
       </c>
-      <c r="H30" s="33" t="s">
-        <v>63</v>
-      </c>
-      <c r="I30" s="42"/>
-      <c r="J30" s="42">
+      <c r="H30" s="34" t="s">
+        <v>53</v>
+      </c>
+      <c r="I30" s="43"/>
+      <c r="J30" s="43">
         <v>45939.0</v>
       </c>
-      <c r="K30" s="44">
+      <c r="K30" s="45">
         <v>378307.61</v>
       </c>
-      <c r="L30" s="33" t="s">
+      <c r="L30" s="34" t="s">
         <v>181</v>
       </c>
-      <c r="M30" s="37">
+      <c r="M30" s="38">
         <v>378307.61</v>
       </c>
-      <c r="N30" s="50"/>
-      <c r="O30" s="24"/>
-      <c r="P30" s="52"/>
-      <c r="Q30" s="26"/>
-      <c r="R30" s="26"/>
-      <c r="S30" s="26"/>
-      <c r="T30" s="26"/>
-      <c r="U30" s="26"/>
-      <c r="V30" s="51"/>
-      <c r="W30" s="26"/>
-      <c r="X30" s="26"/>
-      <c r="Y30" s="26"/>
-      <c r="Z30" s="26"/>
-      <c r="AA30" s="26"/>
-      <c r="AB30" s="26"/>
-      <c r="AC30" s="26"/>
+      <c r="N30" s="51"/>
+      <c r="O30" s="25"/>
+      <c r="P30" s="48"/>
+      <c r="Q30" s="27"/>
+      <c r="R30" s="27"/>
+      <c r="S30" s="27"/>
+      <c r="T30" s="27"/>
+      <c r="U30" s="27"/>
+      <c r="V30" s="52"/>
+      <c r="W30" s="27"/>
+      <c r="X30" s="27"/>
+      <c r="Y30" s="27"/>
+      <c r="Z30" s="27"/>
+      <c r="AA30" s="27"/>
+      <c r="AB30" s="27"/>
+      <c r="AC30" s="27"/>
     </row>
     <row r="31" ht="60.0" customHeight="1">
       <c r="A31" s="22"/>
@@ -2495,44 +2495,44 @@
       <c r="E31" s="63" t="s">
         <v>180</v>
       </c>
-      <c r="F31" s="33">
+      <c r="F31" s="34">
         <v>691.0</v>
       </c>
       <c r="G31" s="64">
         <v>45910.0</v>
       </c>
-      <c r="H31" s="33" t="s">
-        <v>63</v>
-      </c>
-      <c r="I31" s="42"/>
-      <c r="J31" s="42">
+      <c r="H31" s="34" t="s">
+        <v>53</v>
+      </c>
+      <c r="I31" s="43"/>
+      <c r="J31" s="43">
         <v>45941.0</v>
       </c>
-      <c r="K31" s="36">
+      <c r="K31" s="37">
         <v>3315.0471000000252</v>
       </c>
-      <c r="L31" s="33" t="s">
+      <c r="L31" s="34" t="s">
         <v>183</v>
       </c>
-      <c r="M31" s="37">
+      <c r="M31" s="38">
         <v>3315.04710000003</v>
       </c>
-      <c r="N31" s="50"/>
-      <c r="O31" s="24"/>
-      <c r="P31" s="52"/>
-      <c r="Q31" s="26"/>
-      <c r="R31" s="26"/>
-      <c r="S31" s="26"/>
-      <c r="T31" s="26"/>
-      <c r="U31" s="26"/>
-      <c r="V31" s="51"/>
-      <c r="W31" s="26"/>
-      <c r="X31" s="26"/>
-      <c r="Y31" s="26"/>
-      <c r="Z31" s="26"/>
-      <c r="AA31" s="26"/>
-      <c r="AB31" s="26"/>
-      <c r="AC31" s="26"/>
+      <c r="N31" s="51"/>
+      <c r="O31" s="25"/>
+      <c r="P31" s="48"/>
+      <c r="Q31" s="27"/>
+      <c r="R31" s="27"/>
+      <c r="S31" s="27"/>
+      <c r="T31" s="27"/>
+      <c r="U31" s="27"/>
+      <c r="V31" s="52"/>
+      <c r="W31" s="27"/>
+      <c r="X31" s="27"/>
+      <c r="Y31" s="27"/>
+      <c r="Z31" s="27"/>
+      <c r="AA31" s="27"/>
+      <c r="AB31" s="27"/>
+      <c r="AC31" s="27"/>
     </row>
     <row r="32" ht="12.75" customHeight="1">
       <c r="A32" s="22"/>
@@ -2544,44 +2544,44 @@
       <c r="E32" s="65">
         <v>135.0</v>
       </c>
-      <c r="F32" s="33">
+      <c r="F32" s="34">
         <v>677.0</v>
       </c>
       <c r="G32" s="64">
         <v>45904.0</v>
       </c>
-      <c r="H32" s="33" t="s">
-        <v>71</v>
+      <c r="H32" s="34" t="s">
+        <v>60</v>
       </c>
       <c r="I32" s="66"/>
       <c r="J32" s="66">
         <v>45935.0</v>
       </c>
-      <c r="K32" s="44">
+      <c r="K32" s="45">
         <v>198332.75</v>
       </c>
-      <c r="L32" s="33" t="s">
+      <c r="L32" s="34" t="s">
         <v>185</v>
       </c>
-      <c r="M32" s="37">
+      <c r="M32" s="38">
         <v>198332.75</v>
       </c>
-      <c r="N32" s="50"/>
-      <c r="O32" s="24"/>
-      <c r="P32" s="52"/>
-      <c r="Q32" s="26"/>
-      <c r="R32" s="26"/>
-      <c r="S32" s="26"/>
-      <c r="T32" s="26"/>
-      <c r="U32" s="26"/>
-      <c r="V32" s="51"/>
-      <c r="W32" s="26"/>
-      <c r="X32" s="26"/>
-      <c r="Y32" s="26"/>
-      <c r="Z32" s="26"/>
-      <c r="AA32" s="26"/>
-      <c r="AB32" s="26"/>
-      <c r="AC32" s="26"/>
+      <c r="N32" s="51"/>
+      <c r="O32" s="25"/>
+      <c r="P32" s="48"/>
+      <c r="Q32" s="27"/>
+      <c r="R32" s="27"/>
+      <c r="S32" s="27"/>
+      <c r="T32" s="27"/>
+      <c r="U32" s="27"/>
+      <c r="V32" s="52"/>
+      <c r="W32" s="27"/>
+      <c r="X32" s="27"/>
+      <c r="Y32" s="27"/>
+      <c r="Z32" s="27"/>
+      <c r="AA32" s="27"/>
+      <c r="AB32" s="27"/>
+      <c r="AC32" s="27"/>
     </row>
     <row r="33" ht="12.75" customHeight="1">
       <c r="A33" s="22"/>
@@ -2593,20 +2593,20 @@
       <c r="E33" s="65">
         <v>40.0</v>
       </c>
-      <c r="F33" s="33">
+      <c r="F33" s="34">
         <v>278.0</v>
       </c>
       <c r="G33" s="64">
         <v>46008.0</v>
       </c>
-      <c r="H33" s="33" t="s">
-        <v>128</v>
+      <c r="H33" s="34" t="s">
+        <v>113</v>
       </c>
       <c r="I33" s="66"/>
       <c r="J33" s="66">
         <v>46066.0</v>
       </c>
-      <c r="K33" s="44">
+      <c r="K33" s="45">
         <v>1528.62</v>
       </c>
       <c r="L33" s="67" t="s">
@@ -2615,22 +2615,22 @@
       <c r="M33" s="68" t="s">
         <v>188</v>
       </c>
-      <c r="N33" s="50"/>
-      <c r="O33" s="24"/>
-      <c r="P33" s="52"/>
-      <c r="Q33" s="26"/>
-      <c r="R33" s="26"/>
-      <c r="S33" s="26"/>
-      <c r="T33" s="26"/>
-      <c r="U33" s="26"/>
-      <c r="V33" s="51"/>
-      <c r="W33" s="26"/>
-      <c r="X33" s="26"/>
-      <c r="Y33" s="26"/>
-      <c r="Z33" s="26"/>
-      <c r="AA33" s="26"/>
-      <c r="AB33" s="26"/>
-      <c r="AC33" s="26"/>
+      <c r="N33" s="51"/>
+      <c r="O33" s="25"/>
+      <c r="P33" s="48"/>
+      <c r="Q33" s="27"/>
+      <c r="R33" s="27"/>
+      <c r="S33" s="27"/>
+      <c r="T33" s="27"/>
+      <c r="U33" s="27"/>
+      <c r="V33" s="52"/>
+      <c r="W33" s="27"/>
+      <c r="X33" s="27"/>
+      <c r="Y33" s="27"/>
+      <c r="Z33" s="27"/>
+      <c r="AA33" s="27"/>
+      <c r="AB33" s="27"/>
+      <c r="AC33" s="27"/>
     </row>
     <row r="34" ht="12.75" customHeight="1">
       <c r="A34" s="22"/>
@@ -2642,44 +2642,44 @@
       <c r="E34" s="65" t="s">
         <v>190</v>
       </c>
-      <c r="F34" s="33">
+      <c r="F34" s="34">
         <v>748.0</v>
       </c>
       <c r="G34" s="64">
         <v>45930.0</v>
       </c>
-      <c r="H34" s="33" t="s">
-        <v>98</v>
+      <c r="H34" s="34" t="s">
+        <v>90</v>
       </c>
       <c r="I34" s="66"/>
       <c r="J34" s="66">
         <v>45935.0</v>
       </c>
-      <c r="K34" s="44">
+      <c r="K34" s="45">
         <v>38718.58</v>
       </c>
-      <c r="L34" s="33" t="s">
+      <c r="L34" s="34" t="s">
         <v>191</v>
       </c>
       <c r="M34" s="61" t="s">
         <v>192</v>
       </c>
-      <c r="N34" s="50"/>
-      <c r="O34" s="24"/>
-      <c r="P34" s="52"/>
-      <c r="Q34" s="26"/>
-      <c r="R34" s="26"/>
-      <c r="S34" s="26"/>
-      <c r="T34" s="26"/>
-      <c r="U34" s="26"/>
-      <c r="V34" s="51"/>
-      <c r="W34" s="26"/>
-      <c r="X34" s="26"/>
-      <c r="Y34" s="26"/>
-      <c r="Z34" s="26"/>
-      <c r="AA34" s="26"/>
-      <c r="AB34" s="26"/>
-      <c r="AC34" s="26"/>
+      <c r="N34" s="51"/>
+      <c r="O34" s="25"/>
+      <c r="P34" s="48"/>
+      <c r="Q34" s="27"/>
+      <c r="R34" s="27"/>
+      <c r="S34" s="27"/>
+      <c r="T34" s="27"/>
+      <c r="U34" s="27"/>
+      <c r="V34" s="52"/>
+      <c r="W34" s="27"/>
+      <c r="X34" s="27"/>
+      <c r="Y34" s="27"/>
+      <c r="Z34" s="27"/>
+      <c r="AA34" s="27"/>
+      <c r="AB34" s="27"/>
+      <c r="AC34" s="27"/>
     </row>
     <row r="35" ht="12.75" customHeight="1">
       <c r="A35" s="22"/>
@@ -2691,44 +2691,44 @@
       <c r="E35" s="65">
         <v>154.0</v>
       </c>
-      <c r="F35" s="33">
+      <c r="F35" s="34">
         <v>822.0</v>
       </c>
       <c r="G35" s="64">
         <v>45968.0</v>
       </c>
-      <c r="H35" s="33" t="s">
-        <v>118</v>
+      <c r="H35" s="34" t="s">
+        <v>104</v>
       </c>
       <c r="I35" s="66"/>
       <c r="J35" s="66">
         <v>45935.0</v>
       </c>
-      <c r="K35" s="44">
+      <c r="K35" s="45">
         <v>133124.11</v>
       </c>
-      <c r="L35" s="33" t="s">
+      <c r="L35" s="34" t="s">
         <v>194</v>
       </c>
       <c r="M35" s="61" t="s">
         <v>195</v>
       </c>
-      <c r="N35" s="50"/>
-      <c r="O35" s="24"/>
-      <c r="P35" s="52"/>
-      <c r="Q35" s="26"/>
-      <c r="R35" s="26"/>
-      <c r="S35" s="26"/>
-      <c r="T35" s="26"/>
-      <c r="U35" s="26"/>
-      <c r="V35" s="51"/>
-      <c r="W35" s="26"/>
-      <c r="X35" s="26"/>
-      <c r="Y35" s="26"/>
-      <c r="Z35" s="26"/>
-      <c r="AA35" s="26"/>
-      <c r="AB35" s="26"/>
-      <c r="AC35" s="26"/>
+      <c r="N35" s="51"/>
+      <c r="O35" s="25"/>
+      <c r="P35" s="48"/>
+      <c r="Q35" s="27"/>
+      <c r="R35" s="27"/>
+      <c r="S35" s="27"/>
+      <c r="T35" s="27"/>
+      <c r="U35" s="27"/>
+      <c r="V35" s="52"/>
+      <c r="W35" s="27"/>
+      <c r="X35" s="27"/>
+      <c r="Y35" s="27"/>
+      <c r="Z35" s="27"/>
+      <c r="AA35" s="27"/>
+      <c r="AB35" s="27"/>
+      <c r="AC35" s="27"/>
     </row>
     <row r="36" ht="12.75" customHeight="1">
       <c r="A36" s="22"/>
@@ -2747,37 +2747,37 @@
         <v>46043.0</v>
       </c>
       <c r="H36" s="65" t="s">
-        <v>113</v>
+        <v>101</v>
       </c>
       <c r="I36" s="70"/>
       <c r="J36" s="69">
         <v>46075.0</v>
       </c>
-      <c r="K36" s="44">
+      <c r="K36" s="45">
         <v>11372.9</v>
       </c>
-      <c r="L36" s="33" t="s">
+      <c r="L36" s="34" t="s">
         <v>197</v>
       </c>
-      <c r="M36" s="37">
+      <c r="M36" s="38">
         <v>11372.9</v>
       </c>
-      <c r="N36" s="50"/>
-      <c r="O36" s="24"/>
-      <c r="P36" s="26"/>
-      <c r="Q36" s="26"/>
-      <c r="R36" s="26"/>
-      <c r="S36" s="26"/>
-      <c r="T36" s="26"/>
-      <c r="U36" s="26"/>
-      <c r="V36" s="51"/>
-      <c r="W36" s="26"/>
-      <c r="X36" s="26"/>
-      <c r="Y36" s="26"/>
-      <c r="Z36" s="26"/>
-      <c r="AA36" s="26"/>
-      <c r="AB36" s="26"/>
-      <c r="AC36" s="26"/>
+      <c r="N36" s="51"/>
+      <c r="O36" s="25"/>
+      <c r="P36" s="27"/>
+      <c r="Q36" s="27"/>
+      <c r="R36" s="27"/>
+      <c r="S36" s="27"/>
+      <c r="T36" s="27"/>
+      <c r="U36" s="27"/>
+      <c r="V36" s="52"/>
+      <c r="W36" s="27"/>
+      <c r="X36" s="27"/>
+      <c r="Y36" s="27"/>
+      <c r="Z36" s="27"/>
+      <c r="AA36" s="27"/>
+      <c r="AB36" s="27"/>
+      <c r="AC36" s="27"/>
     </row>
     <row r="37" ht="12.75" customHeight="1">
       <c r="A37" s="22"/>
@@ -2794,27 +2794,27 @@
         <v>199</v>
       </c>
       <c r="J37" s="69"/>
-      <c r="K37" s="44"/>
-      <c r="L37" s="33"/>
-      <c r="M37" s="37"/>
-      <c r="N37" s="50">
+      <c r="K37" s="45"/>
+      <c r="L37" s="34"/>
+      <c r="M37" s="38"/>
+      <c r="N37" s="51">
         <v>15854.78</v>
       </c>
-      <c r="O37" s="24"/>
-      <c r="P37" s="26"/>
-      <c r="Q37" s="26"/>
-      <c r="R37" s="26"/>
-      <c r="S37" s="26"/>
-      <c r="T37" s="26"/>
-      <c r="U37" s="26"/>
-      <c r="V37" s="51"/>
-      <c r="W37" s="26"/>
-      <c r="X37" s="26"/>
-      <c r="Y37" s="26"/>
-      <c r="Z37" s="26"/>
-      <c r="AA37" s="26"/>
-      <c r="AB37" s="26"/>
-      <c r="AC37" s="26"/>
+      <c r="O37" s="25"/>
+      <c r="P37" s="27"/>
+      <c r="Q37" s="27"/>
+      <c r="R37" s="27"/>
+      <c r="S37" s="27"/>
+      <c r="T37" s="27"/>
+      <c r="U37" s="27"/>
+      <c r="V37" s="52"/>
+      <c r="W37" s="27"/>
+      <c r="X37" s="27"/>
+      <c r="Y37" s="27"/>
+      <c r="Z37" s="27"/>
+      <c r="AA37" s="27"/>
+      <c r="AB37" s="27"/>
+      <c r="AC37" s="27"/>
     </row>
     <row r="38" ht="12.75" customHeight="1">
       <c r="A38" s="22"/>
@@ -2831,32 +2831,32 @@
         <v>199</v>
       </c>
       <c r="J38" s="69"/>
-      <c r="K38" s="44"/>
-      <c r="L38" s="33"/>
-      <c r="M38" s="37"/>
-      <c r="N38" s="50">
+      <c r="K38" s="45"/>
+      <c r="L38" s="34"/>
+      <c r="M38" s="38"/>
+      <c r="N38" s="51">
         <v>24962.38</v>
       </c>
-      <c r="O38" s="24"/>
-      <c r="P38" s="26"/>
-      <c r="Q38" s="26"/>
-      <c r="R38" s="26"/>
-      <c r="S38" s="26"/>
-      <c r="T38" s="26"/>
-      <c r="U38" s="26"/>
-      <c r="V38" s="51"/>
-      <c r="W38" s="26"/>
-      <c r="X38" s="26"/>
-      <c r="Y38" s="26"/>
-      <c r="Z38" s="26"/>
-      <c r="AA38" s="26"/>
-      <c r="AB38" s="26"/>
-      <c r="AC38" s="26"/>
+      <c r="O38" s="25"/>
+      <c r="P38" s="27"/>
+      <c r="Q38" s="27"/>
+      <c r="R38" s="27"/>
+      <c r="S38" s="27"/>
+      <c r="T38" s="27"/>
+      <c r="U38" s="27"/>
+      <c r="V38" s="52"/>
+      <c r="W38" s="27"/>
+      <c r="X38" s="27"/>
+      <c r="Y38" s="27"/>
+      <c r="Z38" s="27"/>
+      <c r="AA38" s="27"/>
+      <c r="AB38" s="27"/>
+      <c r="AC38" s="27"/>
     </row>
     <row r="39" ht="12.75" customHeight="1">
       <c r="A39" s="22"/>
       <c r="B39" s="22"/>
-      <c r="C39" s="31">
+      <c r="C39" s="32">
         <v>3.0</v>
       </c>
       <c r="D39" s="62" t="s">
@@ -2870,13 +2870,13 @@
         <v>46104.0</v>
       </c>
       <c r="H39" s="65" t="s">
-        <v>113</v>
+        <v>101</v>
       </c>
       <c r="I39" s="70"/>
       <c r="J39" s="69">
         <v>46106.0</v>
       </c>
-      <c r="K39" s="44">
+      <c r="K39" s="45">
         <v>27801.11</v>
       </c>
       <c r="L39" s="71" t="s">
@@ -2885,22 +2885,22 @@
       <c r="M39" s="72">
         <v>27801.11</v>
       </c>
-      <c r="N39" s="50"/>
-      <c r="O39" s="24"/>
-      <c r="P39" s="26"/>
-      <c r="Q39" s="26"/>
-      <c r="R39" s="26"/>
-      <c r="S39" s="26"/>
-      <c r="T39" s="26"/>
-      <c r="U39" s="26"/>
-      <c r="V39" s="51"/>
-      <c r="W39" s="26"/>
-      <c r="X39" s="26"/>
-      <c r="Y39" s="26"/>
-      <c r="Z39" s="26"/>
-      <c r="AA39" s="26"/>
-      <c r="AB39" s="26"/>
-      <c r="AC39" s="26"/>
+      <c r="N39" s="51"/>
+      <c r="O39" s="25"/>
+      <c r="P39" s="27"/>
+      <c r="Q39" s="27"/>
+      <c r="R39" s="27"/>
+      <c r="S39" s="27"/>
+      <c r="T39" s="27"/>
+      <c r="U39" s="27"/>
+      <c r="V39" s="52"/>
+      <c r="W39" s="27"/>
+      <c r="X39" s="27"/>
+      <c r="Y39" s="27"/>
+      <c r="Z39" s="27"/>
+      <c r="AA39" s="27"/>
+      <c r="AB39" s="27"/>
+      <c r="AC39" s="27"/>
     </row>
     <row r="40" ht="12.75" customHeight="1">
       <c r="A40" s="16"/>
@@ -2917,22 +2917,22 @@
         <v>46199.0</v>
       </c>
       <c r="H40" s="65" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="I40" s="70"/>
       <c r="J40" s="69">
         <v>46233.0</v>
       </c>
-      <c r="K40" s="44">
+      <c r="K40" s="45">
         <v>58868.35</v>
       </c>
-      <c r="L40" s="33" t="s">
-        <v>65</v>
+      <c r="L40" s="34" t="s">
+        <v>73</v>
       </c>
       <c r="M40" s="72">
         <v>58868.35</v>
       </c>
-      <c r="N40" s="50"/>
+      <c r="N40" s="51"/>
       <c r="V40" s="3"/>
     </row>
     <row r="41" ht="12.75" customHeight="1">
@@ -7886,11 +7886,11 @@
       <c r="AH1" s="2"/>
     </row>
     <row r="2">
-      <c r="A2" s="5">
+      <c r="A2" s="4">
         <v>46212.0</v>
       </c>
-      <c r="L2" s="7" t="s">
-        <v>1</v>
+      <c r="L2" s="6" t="s">
+        <v>0</v>
       </c>
       <c r="AB2" s="2"/>
       <c r="AC2" s="2"/>
@@ -7901,31 +7901,31 @@
       <c r="AH2" s="2"/>
     </row>
     <row r="3">
-      <c r="A3" s="10" t="s">
+      <c r="A3" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="B3" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="11">
+      <c r="C3" s="10">
         <v>2.5E32</v>
       </c>
-      <c r="D3" s="10" t="s">
+      <c r="D3" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="13">
+      <c r="E3" s="12">
         <v>45686.0</v>
       </c>
-      <c r="F3" s="10" t="s">
+      <c r="F3" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G3" s="10">
+      <c r="G3" s="8">
         <v>12.0</v>
       </c>
-      <c r="H3" s="10">
+      <c r="H3" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I3" s="10">
+      <c r="I3" s="8">
         <v>2048.0</v>
       </c>
       <c r="J3" s="14">
@@ -7946,31 +7946,31 @@
       <c r="AH3" s="2"/>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="s">
+      <c r="A4" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="B4" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="C4" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="D4" s="10" t="s">
+      <c r="D4" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="13">
+      <c r="E4" s="12">
         <v>45762.0</v>
       </c>
-      <c r="F4" s="10" t="s">
+      <c r="F4" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G4" s="10">
+      <c r="G4" s="8">
         <v>12.0</v>
       </c>
-      <c r="H4" s="10">
+      <c r="H4" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I4" s="10">
+      <c r="I4" s="8">
         <v>2048.0</v>
       </c>
       <c r="J4" s="14">
@@ -7991,31 +7991,31 @@
       <c r="AH4" s="2"/>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="B5" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="C5" s="10" t="s">
-        <v>24</v>
-      </c>
-      <c r="D5" s="10" t="s">
+      <c r="A5" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E5" s="13">
+      <c r="E5" s="12">
         <v>45762.0</v>
       </c>
-      <c r="F5" s="10" t="s">
+      <c r="F5" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G5" s="10">
+      <c r="G5" s="8">
         <v>12.0</v>
       </c>
-      <c r="H5" s="10">
+      <c r="H5" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I5" s="10">
+      <c r="I5" s="8">
         <v>2048.0</v>
       </c>
       <c r="J5" s="14">
@@ -8036,31 +8036,31 @@
       <c r="AH5" s="2"/>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="B6" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="C6" s="10" t="s">
+      <c r="A6" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="D6" s="10" t="s">
+      <c r="D6" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E6" s="13">
+      <c r="E6" s="12">
         <v>45762.0</v>
       </c>
-      <c r="F6" s="10" t="s">
+      <c r="F6" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G6" s="10">
+      <c r="G6" s="8">
         <v>12.0</v>
       </c>
-      <c r="H6" s="10">
+      <c r="H6" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I6" s="10">
+      <c r="I6" s="8">
         <v>2048.0</v>
       </c>
       <c r="J6" s="14">
@@ -8081,32 +8081,32 @@
       <c r="AH6" s="2"/>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="s">
-        <v>40</v>
-      </c>
-      <c r="B7" s="10" t="s">
-        <v>41</v>
-      </c>
-      <c r="C7" s="10" t="s">
+      <c r="A7" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="E7" s="12">
+        <v>45763.0</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="G7" s="8">
+        <v>12.0</v>
+      </c>
+      <c r="H7" s="8">
+        <v>339039.0</v>
+      </c>
+      <c r="I7" s="8" t="s">
         <v>42</v>
-      </c>
-      <c r="D7" s="10" t="s">
-        <v>4</v>
-      </c>
-      <c r="E7" s="13">
-        <v>45763.0</v>
-      </c>
-      <c r="F7" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="G7" s="10">
-        <v>12.0</v>
-      </c>
-      <c r="H7" s="10">
-        <v>339039.0</v>
-      </c>
-      <c r="I7" s="10" t="s">
-        <v>44</v>
       </c>
       <c r="J7" s="14">
         <v>949835.78</v>
@@ -8126,31 +8126,31 @@
       <c r="AH7" s="2"/>
     </row>
     <row r="8">
-      <c r="A8" s="10" t="s">
+      <c r="A8" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="B8" s="10" t="s">
+      <c r="B8" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="C8" s="10" t="s">
+      <c r="C8" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="D8" s="10" t="s">
+      <c r="D8" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E8" s="13">
+      <c r="E8" s="12">
         <v>45763.0</v>
       </c>
-      <c r="F8" s="10" t="s">
+      <c r="F8" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G8" s="10">
+      <c r="G8" s="8">
         <v>12.0</v>
       </c>
-      <c r="H8" s="10">
+      <c r="H8" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I8" s="10" t="s">
+      <c r="I8" s="8" t="s">
         <v>48</v>
       </c>
       <c r="J8" s="14">
@@ -8162,7 +8162,7 @@
       <c r="L8" s="15">
         <v>0.0</v>
       </c>
-      <c r="O8" s="27"/>
+      <c r="O8" s="23"/>
       <c r="AB8" s="2"/>
       <c r="AC8" s="2"/>
       <c r="AD8" s="2"/>
@@ -8172,32 +8172,32 @@
       <c r="AH8" s="2"/>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="s">
+      <c r="A9" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="C9" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="B9" s="10" t="s">
-        <v>53</v>
-      </c>
-      <c r="C9" s="10" t="s">
-        <v>54</v>
-      </c>
-      <c r="D9" s="10" t="s">
+      <c r="D9" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E9" s="13">
+      <c r="E9" s="12">
         <v>45792.0</v>
       </c>
-      <c r="F9" s="10" t="s">
+      <c r="F9" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G9" s="10">
+      <c r="G9" s="8">
         <v>12.0</v>
       </c>
-      <c r="H9" s="10">
+      <c r="H9" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I9" s="10" t="s">
-        <v>58</v>
+      <c r="I9" s="8" t="s">
+        <v>52</v>
       </c>
       <c r="J9" s="14">
         <v>211614.23</v>
@@ -8217,31 +8217,31 @@
       <c r="AH9" s="2"/>
     </row>
     <row r="10">
-      <c r="A10" s="10" t="s">
-        <v>63</v>
-      </c>
-      <c r="B10" s="10" t="s">
+      <c r="A10" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="B10" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="C10" s="10" t="s">
-        <v>64</v>
-      </c>
-      <c r="D10" s="10" t="s">
+      <c r="C10" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="D10" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E10" s="13">
+      <c r="E10" s="12">
         <v>45825.0</v>
       </c>
-      <c r="F10" s="10" t="s">
+      <c r="F10" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G10" s="10">
+      <c r="G10" s="8">
         <v>12.0</v>
       </c>
-      <c r="H10" s="10">
+      <c r="H10" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I10" s="10">
+      <c r="I10" s="8">
         <v>2048.0</v>
       </c>
       <c r="J10" s="14">
@@ -8262,31 +8262,31 @@
       <c r="AH10" s="2"/>
     </row>
     <row r="11">
-      <c r="A11" s="10" t="s">
-        <v>67</v>
-      </c>
-      <c r="B11" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="C11" s="10" t="s">
-        <v>68</v>
-      </c>
-      <c r="D11" s="10" t="s">
+      <c r="A11" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="D11" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E11" s="13">
+      <c r="E11" s="12">
         <v>45825.0</v>
       </c>
-      <c r="F11" s="10" t="s">
+      <c r="F11" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G11" s="10">
+      <c r="G11" s="8">
         <v>12.0</v>
       </c>
-      <c r="H11" s="10">
+      <c r="H11" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I11" s="10">
+      <c r="I11" s="8">
         <v>2048.0</v>
       </c>
       <c r="J11" s="14">
@@ -8307,32 +8307,32 @@
       <c r="AH11" s="2"/>
     </row>
     <row r="12">
-      <c r="A12" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="B12" s="10" t="s">
-        <v>73</v>
-      </c>
-      <c r="C12" s="10" t="s">
-        <v>74</v>
-      </c>
-      <c r="D12" s="10" t="s">
+      <c r="A12" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="D12" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E12" s="13">
+      <c r="E12" s="12">
         <v>45832.0</v>
       </c>
-      <c r="F12" s="10" t="s">
+      <c r="F12" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G12" s="10">
+      <c r="G12" s="8">
         <v>12.0</v>
       </c>
-      <c r="H12" s="10">
+      <c r="H12" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I12" s="10" t="s">
-        <v>75</v>
+      <c r="I12" s="8" t="s">
+        <v>65</v>
       </c>
       <c r="J12" s="14">
         <v>1600334.09</v>
@@ -8352,31 +8352,31 @@
       <c r="AH12" s="2"/>
     </row>
     <row r="13">
-      <c r="A13" s="10" t="s">
-        <v>77</v>
-      </c>
-      <c r="B13" s="10" t="s">
+      <c r="A13" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="B13" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="C13" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="D13" s="10" t="s">
+      <c r="C13" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="D13" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E13" s="13">
+      <c r="E13" s="12">
         <v>45863.0</v>
       </c>
-      <c r="F13" s="10" t="s">
+      <c r="F13" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G13" s="10">
+      <c r="G13" s="8">
         <v>12.0</v>
       </c>
-      <c r="H13" s="10">
+      <c r="H13" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I13" s="10">
+      <c r="I13" s="8">
         <v>2048.0</v>
       </c>
       <c r="J13" s="14">
@@ -8388,7 +8388,7 @@
       <c r="L13" s="14">
         <v>497601.53</v>
       </c>
-      <c r="M13" s="39"/>
+      <c r="M13" s="31"/>
       <c r="AB13" s="2"/>
       <c r="AC13" s="2"/>
       <c r="AD13" s="2"/>
@@ -8398,32 +8398,32 @@
       <c r="AH13" s="2"/>
     </row>
     <row r="14">
-      <c r="A14" s="10" t="s">
-        <v>80</v>
-      </c>
-      <c r="B14" s="10" t="s">
-        <v>81</v>
-      </c>
-      <c r="C14" s="10" t="s">
-        <v>82</v>
-      </c>
-      <c r="D14" s="10" t="s">
+      <c r="A14" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="D14" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E14" s="13">
+      <c r="E14" s="12">
         <v>45887.0</v>
       </c>
-      <c r="F14" s="10" t="s">
+      <c r="F14" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G14" s="10">
+      <c r="G14" s="8">
         <v>12.0</v>
       </c>
-      <c r="H14" s="10">
+      <c r="H14" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I14" s="10" t="s">
-        <v>58</v>
+      <c r="I14" s="8" t="s">
+        <v>52</v>
       </c>
       <c r="J14" s="14">
         <v>968237.39</v>
@@ -8443,32 +8443,32 @@
       <c r="AH14" s="2"/>
     </row>
     <row r="15">
-      <c r="A15" s="10" t="s">
-        <v>85</v>
-      </c>
-      <c r="B15" s="10" t="s">
-        <v>86</v>
-      </c>
-      <c r="C15" s="10" t="s">
-        <v>87</v>
-      </c>
-      <c r="D15" s="10" t="s">
+      <c r="A15" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="B15" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="C15" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="D15" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E15" s="13">
+      <c r="E15" s="12">
         <v>45924.0</v>
       </c>
-      <c r="F15" s="10" t="s">
+      <c r="F15" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G15" s="10">
+      <c r="G15" s="8">
         <v>12.0</v>
       </c>
-      <c r="H15" s="10">
+      <c r="H15" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I15" s="10" t="s">
-        <v>44</v>
+      <c r="I15" s="8" t="s">
+        <v>42</v>
       </c>
       <c r="J15" s="14">
         <v>1011677.95</v>
@@ -8488,31 +8488,31 @@
       <c r="AH15" s="2"/>
     </row>
     <row r="16">
-      <c r="A16" s="10" t="s">
-        <v>90</v>
-      </c>
-      <c r="B16" s="10" t="s">
+      <c r="A16" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="B16" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="C16" s="10" t="s">
-        <v>91</v>
-      </c>
-      <c r="D16" s="10" t="s">
+      <c r="C16" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="D16" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E16" s="13">
+      <c r="E16" s="12">
         <v>45929.0</v>
       </c>
-      <c r="F16" s="10" t="s">
+      <c r="F16" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G16" s="10">
+      <c r="G16" s="8">
         <v>12.0</v>
       </c>
-      <c r="H16" s="10">
+      <c r="H16" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I16" s="10">
+      <c r="I16" s="8">
         <v>2048.0</v>
       </c>
       <c r="J16" s="14">
@@ -8533,31 +8533,31 @@
       <c r="AH16" s="2"/>
     </row>
     <row r="17">
-      <c r="A17" s="10" t="s">
-        <v>94</v>
-      </c>
-      <c r="B17" s="10" t="s">
-        <v>95</v>
-      </c>
-      <c r="C17" s="10" t="s">
-        <v>96</v>
-      </c>
-      <c r="D17" s="10" t="s">
+      <c r="A17" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="B17" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="C17" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="D17" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E17" s="13">
+      <c r="E17" s="12">
         <v>45930.0</v>
       </c>
-      <c r="F17" s="10" t="s">
+      <c r="F17" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G17" s="10">
+      <c r="G17" s="8">
         <v>12.0</v>
       </c>
-      <c r="H17" s="10">
+      <c r="H17" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I17" s="10">
+      <c r="I17" s="8">
         <v>2048.0</v>
       </c>
       <c r="J17" s="14">
@@ -8578,32 +8578,32 @@
       <c r="AH17" s="2"/>
     </row>
     <row r="18">
-      <c r="A18" s="10" t="s">
-        <v>98</v>
-      </c>
-      <c r="B18" s="10" t="s">
-        <v>81</v>
-      </c>
-      <c r="C18" s="10" t="s">
-        <v>99</v>
-      </c>
-      <c r="D18" s="10" t="s">
+      <c r="A18" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="B18" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="C18" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="D18" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E18" s="13">
+      <c r="E18" s="12">
         <v>45938.0</v>
       </c>
-      <c r="F18" s="10" t="s">
+      <c r="F18" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G18" s="10">
+      <c r="G18" s="8">
         <v>12.0</v>
       </c>
-      <c r="H18" s="10">
+      <c r="H18" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I18" s="10" t="s">
-        <v>58</v>
+      <c r="I18" s="8" t="s">
+        <v>52</v>
       </c>
       <c r="J18" s="14">
         <v>63746.85</v>
@@ -8623,32 +8623,32 @@
       <c r="AH18" s="2"/>
     </row>
     <row r="19">
-      <c r="A19" s="10" t="s">
-        <v>101</v>
-      </c>
-      <c r="B19" s="10" t="s">
-        <v>73</v>
-      </c>
-      <c r="C19" s="10" t="s">
-        <v>102</v>
-      </c>
-      <c r="D19" s="10" t="s">
+      <c r="A19" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="B19" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="C19" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="D19" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E19" s="13">
+      <c r="E19" s="12">
         <v>45938.0</v>
       </c>
-      <c r="F19" s="10" t="s">
+      <c r="F19" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G19" s="10">
+      <c r="G19" s="8">
         <v>12.0</v>
       </c>
-      <c r="H19" s="10">
+      <c r="H19" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I19" s="10" t="s">
-        <v>75</v>
+      <c r="I19" s="8" t="s">
+        <v>65</v>
       </c>
       <c r="J19" s="14">
         <v>947931.1</v>
@@ -8668,31 +8668,31 @@
       <c r="AH19" s="2"/>
     </row>
     <row r="20">
-      <c r="A20" s="10" t="s">
-        <v>105</v>
-      </c>
-      <c r="B20" s="10" t="s">
+      <c r="A20" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="B20" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="C20" s="10" t="s">
-        <v>106</v>
-      </c>
-      <c r="D20" s="10" t="s">
+      <c r="C20" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="D20" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E20" s="13">
+      <c r="E20" s="12">
         <v>45938.0</v>
       </c>
-      <c r="F20" s="10" t="s">
+      <c r="F20" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G20" s="10">
+      <c r="G20" s="8">
         <v>12.0</v>
       </c>
-      <c r="H20" s="10">
+      <c r="H20" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I20" s="10">
+      <c r="I20" s="8">
         <v>2048.0</v>
       </c>
       <c r="J20" s="14">
@@ -8713,31 +8713,31 @@
       <c r="AH20" s="2"/>
     </row>
     <row r="21">
-      <c r="A21" s="10" t="s">
-        <v>110</v>
-      </c>
-      <c r="B21" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="C21" s="10" t="s">
-        <v>111</v>
-      </c>
-      <c r="D21" s="10" t="s">
+      <c r="A21" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="B21" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C21" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="D21" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E21" s="13">
+      <c r="E21" s="12">
         <v>45938.0</v>
       </c>
-      <c r="F21" s="10" t="s">
+      <c r="F21" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G21" s="10">
+      <c r="G21" s="8">
         <v>12.0</v>
       </c>
-      <c r="H21" s="10">
+      <c r="H21" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I21" s="10">
+      <c r="I21" s="8">
         <v>2048.0</v>
       </c>
       <c r="J21" s="14">
@@ -8758,31 +8758,31 @@
       <c r="AH21" s="2"/>
     </row>
     <row r="22">
-      <c r="A22" s="10" t="s">
-        <v>113</v>
-      </c>
-      <c r="B22" s="10" t="s">
-        <v>114</v>
-      </c>
-      <c r="C22" s="10" t="s">
-        <v>115</v>
-      </c>
-      <c r="D22" s="10" t="s">
+      <c r="A22" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="B22" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="C22" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="D22" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E22" s="49">
+      <c r="E22" s="41">
         <v>45953.0</v>
       </c>
-      <c r="F22" s="10" t="s">
+      <c r="F22" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G22" s="10">
+      <c r="G22" s="8">
         <v>12.0</v>
       </c>
-      <c r="H22" s="10">
+      <c r="H22" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I22" s="10">
+      <c r="I22" s="8">
         <v>2000.0</v>
       </c>
       <c r="J22" s="14">
@@ -8803,32 +8803,32 @@
       <c r="AH22" s="2"/>
     </row>
     <row r="23">
-      <c r="A23" s="10" t="s">
-        <v>118</v>
-      </c>
-      <c r="B23" s="10" t="s">
-        <v>119</v>
-      </c>
-      <c r="C23" s="10" t="s">
-        <v>120</v>
-      </c>
-      <c r="D23" s="10" t="s">
+      <c r="A23" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="B23" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="C23" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="D23" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E23" s="49">
+      <c r="E23" s="41">
         <v>45953.0</v>
       </c>
-      <c r="F23" s="10" t="s">
+      <c r="F23" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G23" s="10">
+      <c r="G23" s="8">
         <v>12.0</v>
       </c>
-      <c r="H23" s="10">
+      <c r="H23" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I23" s="10" t="s">
-        <v>122</v>
+      <c r="I23" s="8" t="s">
+        <v>107</v>
       </c>
       <c r="J23" s="14">
         <v>1000001.64</v>
@@ -8848,31 +8848,31 @@
       <c r="AH23" s="2"/>
     </row>
     <row r="24">
-      <c r="A24" s="10" t="s">
-        <v>124</v>
-      </c>
-      <c r="B24" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="C24" s="10" t="s">
-        <v>125</v>
-      </c>
-      <c r="D24" s="10" t="s">
+      <c r="A24" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="B24" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C24" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="D24" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E24" s="49">
+      <c r="E24" s="41">
         <v>45953.0</v>
       </c>
-      <c r="F24" s="10" t="s">
+      <c r="F24" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G24" s="10">
+      <c r="G24" s="8">
         <v>12.0</v>
       </c>
-      <c r="H24" s="10">
+      <c r="H24" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I24" s="10">
+      <c r="I24" s="8">
         <v>2048.0</v>
       </c>
       <c r="J24" s="14">
@@ -8893,32 +8893,32 @@
       <c r="AH24" s="2"/>
     </row>
     <row r="25">
-      <c r="A25" s="10" t="s">
-        <v>128</v>
-      </c>
-      <c r="B25" s="10" t="s">
-        <v>129</v>
-      </c>
-      <c r="C25" s="10" t="s">
-        <v>130</v>
-      </c>
-      <c r="D25" s="10" t="s">
+      <c r="A25" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="B25" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="C25" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="D25" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E25" s="49">
+      <c r="E25" s="41">
         <v>45975.0</v>
       </c>
-      <c r="F25" s="10" t="s">
+      <c r="F25" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G25" s="10">
+      <c r="G25" s="8">
         <v>12.0</v>
       </c>
-      <c r="H25" s="10">
+      <c r="H25" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I25" s="10" t="s">
-        <v>122</v>
+      <c r="I25" s="8" t="s">
+        <v>107</v>
       </c>
       <c r="J25" s="14">
         <v>1157673.06</v>
@@ -8938,31 +8938,31 @@
       <c r="AH25" s="2"/>
     </row>
     <row r="26">
-      <c r="A26" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="B26" s="10" t="s">
+      <c r="A26" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="B26" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="C26" s="10" t="s">
-        <v>133</v>
-      </c>
-      <c r="D26" s="10" t="s">
+      <c r="C26" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="D26" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E26" s="49">
+      <c r="E26" s="41">
         <v>45989.0</v>
       </c>
-      <c r="F26" s="10" t="s">
+      <c r="F26" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G26" s="10">
+      <c r="G26" s="8">
         <v>12.0</v>
       </c>
-      <c r="H26" s="10">
+      <c r="H26" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I26" s="10">
+      <c r="I26" s="8">
         <v>2048.0</v>
       </c>
       <c r="J26" s="14">
@@ -8983,31 +8983,31 @@
       <c r="AH26" s="2"/>
     </row>
     <row r="27">
-      <c r="A27" s="10" t="s">
-        <v>136</v>
-      </c>
-      <c r="B27" s="10" t="s">
-        <v>137</v>
-      </c>
-      <c r="C27" s="10" t="s">
-        <v>138</v>
-      </c>
-      <c r="D27" s="10" t="s">
+      <c r="A27" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="B27" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="C27" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="D27" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E27" s="13">
+      <c r="E27" s="12">
         <v>46104.0</v>
       </c>
-      <c r="F27" s="10" t="s">
+      <c r="F27" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G27" s="10">
+      <c r="G27" s="8">
         <v>12.0</v>
       </c>
-      <c r="H27" s="10">
+      <c r="H27" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I27" s="10">
+      <c r="I27" s="8">
         <v>2048.0</v>
       </c>
       <c r="J27" s="14">
@@ -9028,31 +9028,31 @@
       <c r="AH27" s="2"/>
     </row>
     <row r="28">
-      <c r="A28" s="10" t="s">
-        <v>140</v>
-      </c>
-      <c r="B28" s="10" t="s">
-        <v>142</v>
-      </c>
-      <c r="C28" s="10" t="s">
-        <v>143</v>
-      </c>
-      <c r="D28" s="10" t="s">
+      <c r="A28" s="8" t="s">
+        <v>122</v>
+      </c>
+      <c r="B28" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="C28" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="D28" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E28" s="13">
+      <c r="E28" s="12">
         <v>46120.0</v>
       </c>
-      <c r="F28" s="10" t="s">
+      <c r="F28" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G28" s="10">
+      <c r="G28" s="8">
         <v>12.0</v>
       </c>
-      <c r="H28" s="10">
+      <c r="H28" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I28" s="10" t="s">
+      <c r="I28" s="8" t="s">
         <v>48</v>
       </c>
       <c r="J28" s="14">
@@ -9073,40 +9073,40 @@
       <c r="AH28" s="2"/>
     </row>
     <row r="29">
-      <c r="A29" s="7" t="s">
-        <v>146</v>
-      </c>
-      <c r="B29" s="7" t="s">
-        <v>147</v>
-      </c>
-      <c r="C29" s="7" t="s">
-        <v>148</v>
-      </c>
-      <c r="D29" s="7" t="s">
+      <c r="A29" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="D29" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="E29" s="5">
+      <c r="E29" s="4">
         <v>46196.0</v>
       </c>
-      <c r="F29" s="7" t="s">
+      <c r="F29" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G29" s="7">
+      <c r="G29" s="6">
         <v>12.0</v>
       </c>
-      <c r="H29" s="7">
+      <c r="H29" s="6">
         <v>339039.0</v>
       </c>
-      <c r="I29" s="7">
+      <c r="I29" s="6">
         <v>2048.0</v>
       </c>
-      <c r="J29" s="52">
+      <c r="J29" s="48">
         <v>1496713.48</v>
       </c>
-      <c r="K29" s="7">
+      <c r="K29" s="6">
         <v>0.0</v>
       </c>
-      <c r="L29" s="52">
+      <c r="L29" s="48">
         <v>1496713.48</v>
       </c>
       <c r="AB29" s="2"/>
@@ -9118,40 +9118,40 @@
       <c r="AH29" s="2"/>
     </row>
     <row r="30">
-      <c r="A30" s="7" t="s">
-        <v>150</v>
-      </c>
-      <c r="B30" s="7" t="s">
-        <v>152</v>
-      </c>
-      <c r="C30" s="7" t="s">
-        <v>153</v>
-      </c>
-      <c r="D30" s="7" t="s">
+      <c r="A30" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="B30" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="C30" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="D30" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="E30" s="5">
+      <c r="E30" s="4">
         <v>46205.0</v>
       </c>
-      <c r="F30" s="7" t="s">
+      <c r="F30" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G30" s="7">
+      <c r="G30" s="6">
         <v>12.0</v>
       </c>
-      <c r="H30" s="7">
+      <c r="H30" s="6">
         <v>339039.0</v>
       </c>
-      <c r="I30" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="J30" s="52">
+      <c r="I30" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="J30" s="48">
         <v>624166.14</v>
       </c>
-      <c r="K30" s="7">
+      <c r="K30" s="6">
         <v>0.0</v>
       </c>
-      <c r="L30" s="52">
+      <c r="L30" s="48">
         <v>624166.14</v>
       </c>
       <c r="AB30" s="2"/>
@@ -9163,40 +9163,40 @@
       <c r="AH30" s="2"/>
     </row>
     <row r="31">
-      <c r="A31" s="7" t="s">
-        <v>155</v>
-      </c>
-      <c r="B31" s="7" t="s">
-        <v>156</v>
-      </c>
-      <c r="C31" s="7" t="s">
-        <v>157</v>
-      </c>
-      <c r="D31" s="7" t="s">
+      <c r="A31" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="B31" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="C31" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="D31" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="E31" s="5">
+      <c r="E31" s="4">
         <v>46205.0</v>
       </c>
-      <c r="F31" s="7" t="s">
+      <c r="F31" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G31" s="7">
+      <c r="G31" s="6">
         <v>12.0</v>
       </c>
-      <c r="H31" s="7">
+      <c r="H31" s="6">
         <v>339039.0</v>
       </c>
-      <c r="I31" s="7" t="s">
-        <v>122</v>
-      </c>
-      <c r="J31" s="52">
+      <c r="I31" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="J31" s="48">
         <v>18462.36</v>
       </c>
-      <c r="K31" s="7">
+      <c r="K31" s="6">
         <v>0.0</v>
       </c>
-      <c r="L31" s="52">
+      <c r="L31" s="48">
         <v>18462.36</v>
       </c>
       <c r="AB31" s="2"/>
@@ -9208,40 +9208,40 @@
       <c r="AH31" s="2"/>
     </row>
     <row r="32">
-      <c r="A32" s="7" t="s">
-        <v>160</v>
-      </c>
-      <c r="B32" s="7" t="s">
-        <v>156</v>
-      </c>
-      <c r="C32" s="52" t="s">
-        <v>161</v>
-      </c>
-      <c r="D32" s="7" t="s">
+      <c r="A32" s="6" t="s">
+        <v>139</v>
+      </c>
+      <c r="B32" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="C32" s="48" t="s">
+        <v>140</v>
+      </c>
+      <c r="D32" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="E32" s="5">
+      <c r="E32" s="4">
         <v>46213.0</v>
       </c>
-      <c r="F32" s="7" t="s">
+      <c r="F32" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G32" s="7">
+      <c r="G32" s="6">
         <v>12.0</v>
       </c>
-      <c r="H32" s="7">
+      <c r="H32" s="6">
         <v>339039.0</v>
       </c>
-      <c r="I32" s="7" t="s">
-        <v>122</v>
-      </c>
-      <c r="J32" s="52">
+      <c r="I32" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="J32" s="48">
         <v>1530656.62</v>
       </c>
-      <c r="K32" s="7">
+      <c r="K32" s="6">
         <v>0.0</v>
       </c>
-      <c r="L32" s="52">
+      <c r="L32" s="48">
         <v>1530656.62</v>
       </c>
       <c r="AB32" s="2"/>
@@ -9253,7 +9253,7 @@
       <c r="AH32" s="2"/>
     </row>
     <row r="33">
-      <c r="C33" s="52"/>
+      <c r="C33" s="48"/>
       <c r="AB33" s="2"/>
       <c r="AC33" s="2"/>
       <c r="AD33" s="2"/>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (03/08/2026 19:38)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/01_Bases_Originais/005_CELOG_2025/005_CELOG-PAMALS_2025 online.xlsx
+++ b/Contrato 005/Dashboard/01_Bases_Originais/005_CELOG_2025/005_CELOG-PAMALS_2025 online.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="207">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="331" uniqueCount="209">
   <si>
     <t>Saldo</t>
   </si>
@@ -69,42 +69,42 @@
     <t>UG Fiscalizadora</t>
   </si>
   <si>
+    <t>Prazo Final de Execução</t>
+  </si>
+  <si>
+    <t>Prazo Final de Vigência</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Ação</t>
+  </si>
+  <si>
+    <t>PAG</t>
+  </si>
+  <si>
+    <t>Moeda</t>
+  </si>
+  <si>
     <t>2025NE000369</t>
   </si>
   <si>
-    <t>Prazo Final de Execução</t>
+    <t>Valor Total do Contrato</t>
+  </si>
+  <si>
+    <t>Valor a Empenhar</t>
   </si>
   <si>
     <t>C25516</t>
   </si>
   <si>
-    <t>Prazo Final de Vigência</t>
+    <t>Valor Empenhado</t>
   </si>
   <si>
     <t>25E0387</t>
   </si>
   <si>
-    <t>Status</t>
-  </si>
-  <si>
-    <t>Ação</t>
-  </si>
-  <si>
-    <t>PAG</t>
-  </si>
-  <si>
-    <t>Moeda</t>
-  </si>
-  <si>
-    <t>Valor Total do Contrato</t>
-  </si>
-  <si>
-    <t>Valor a Empenhar</t>
-  </si>
-  <si>
-    <t>Valor Empenhado</t>
-  </si>
-  <si>
     <t>Valor Liquidado</t>
   </si>
   <si>
@@ -123,30 +123,30 @@
     <t>Editar</t>
   </si>
   <si>
+    <t>005/CELOG-PAMALS/2025</t>
+  </si>
+  <si>
+    <t>CELOG</t>
+  </si>
+  <si>
+    <t>PAMALS</t>
+  </si>
+  <si>
     <t>2025NE000371</t>
   </si>
   <si>
-    <t>005/CELOG-PAMALS/2025</t>
+    <t>Vigente</t>
+  </si>
+  <si>
+    <t>2048 20YJ 21EM 219C 20SP 20X7 2000</t>
+  </si>
+  <si>
+    <t>67101.001510/2024-12</t>
   </si>
   <si>
     <t>25E0389</t>
   </si>
   <si>
-    <t>CELOG</t>
-  </si>
-  <si>
-    <t>PAMALS</t>
-  </si>
-  <si>
-    <t>Vigente</t>
-  </si>
-  <si>
-    <t>2048 20YJ 21EM 219C 20SP 20X7 2000</t>
-  </si>
-  <si>
-    <t>67101.001510/2024-12</t>
-  </si>
-  <si>
     <t>R$</t>
   </si>
   <si>
@@ -174,69 +174,78 @@
     <t>25E0431</t>
   </si>
   <si>
+    <t>Módulo</t>
+  </si>
+  <si>
     <t>21EM</t>
   </si>
   <si>
-    <t>Módulo</t>
-  </si>
-  <si>
     <t>Referência</t>
   </si>
   <si>
+    <t>Nº recibo</t>
+  </si>
+  <si>
+    <t>Nº</t>
+  </si>
+  <si>
+    <t>Data</t>
+  </si>
+  <si>
+    <t>Empenho</t>
+  </si>
+  <si>
     <t>2025NE000559</t>
   </si>
   <si>
     <t>C25545</t>
   </si>
   <si>
+    <t>Observações</t>
+  </si>
+  <si>
     <t>25E0524</t>
   </si>
   <si>
-    <t>Nº recibo</t>
+    <t>Vencimento</t>
+  </si>
+  <si>
+    <t>Valor das Nfs</t>
+  </si>
+  <si>
+    <t>Ordem de Pagamento</t>
   </si>
   <si>
     <t>20X7</t>
   </si>
   <si>
-    <t>Nº</t>
+    <t>Faturado</t>
+  </si>
+  <si>
+    <t>Pendente</t>
   </si>
   <si>
     <t>2025NE000770</t>
   </si>
   <si>
-    <t>Data</t>
-  </si>
-  <si>
     <t>25E0731</t>
   </si>
   <si>
-    <t>Empenho</t>
-  </si>
-  <si>
-    <t>Observações</t>
-  </si>
-  <si>
-    <t>Vencimento</t>
-  </si>
-  <si>
-    <t>Valor das Nfs</t>
-  </si>
-  <si>
-    <t>Ordem de Pagamento</t>
-  </si>
-  <si>
-    <t>Faturado</t>
+    <t>FEV/25</t>
   </si>
   <si>
     <t>2025NE000774</t>
   </si>
   <si>
-    <t>Pendente</t>
+    <t>-</t>
   </si>
   <si>
     <t>25E0737</t>
   </si>
   <si>
+    <t xml:space="preserve">2025NE000369 </t>
+  </si>
+  <si>
     <t>2025NE000843</t>
   </si>
   <si>
@@ -246,13 +255,10 @@
     <t>25E0787</t>
   </si>
   <si>
-    <t>FEV/25</t>
-  </si>
-  <si>
     <t>219C</t>
   </si>
   <si>
-    <t>-</t>
+    <t>2025NP001980</t>
   </si>
   <si>
     <t>2025NE001065</t>
@@ -261,12 +267,6 @@
     <t>25E0999</t>
   </si>
   <si>
-    <t xml:space="preserve">2025NE000369 </t>
-  </si>
-  <si>
-    <t>2025NP001980</t>
-  </si>
-  <si>
     <t>2025NE001200</t>
   </si>
   <si>
@@ -276,6 +276,9 @@
     <t>25E1128</t>
   </si>
   <si>
+    <t>MAR/25</t>
+  </si>
+  <si>
     <t>2025NE001598</t>
   </si>
   <si>
@@ -285,15 +288,18 @@
     <t>25E1446</t>
   </si>
   <si>
+    <t>2025NE000367, 2025NE000369, 2025NE000371, 2025NE000413</t>
+  </si>
+  <si>
     <t>2025NE001627</t>
   </si>
   <si>
-    <t>MAR/25</t>
-  </si>
-  <si>
     <t>25E1475</t>
   </si>
   <si>
+    <t>2025NP001979</t>
+  </si>
+  <si>
     <t>2025NE001629</t>
   </si>
   <si>
@@ -303,151 +309,46 @@
     <t>25E1477</t>
   </si>
   <si>
+    <t>ABR/25</t>
+  </si>
+  <si>
+    <t>2025NE000413, 2025NE000414, 2025NE000559</t>
+  </si>
+  <si>
     <t>2025NE001687</t>
   </si>
   <si>
     <t>25E1535</t>
   </si>
   <si>
+    <t>2025NP002341</t>
+  </si>
+  <si>
+    <t>MAI/25</t>
+  </si>
+  <si>
     <t>2025NE001688</t>
   </si>
   <si>
     <t>25E1536</t>
   </si>
   <si>
+    <t>2025NP002884</t>
+  </si>
+  <si>
     <t>2025NE001689</t>
   </si>
   <si>
     <t>25E1537</t>
   </si>
   <si>
+    <t>JUN/25</t>
+  </si>
+  <si>
     <t>2025NE001690</t>
   </si>
   <si>
     <t>25E1538</t>
-  </si>
-  <si>
-    <t>2025NE001823</t>
-  </si>
-  <si>
-    <t>C25865</t>
-  </si>
-  <si>
-    <t>25E1666</t>
-  </si>
-  <si>
-    <t>2025NE001828</t>
-  </si>
-  <si>
-    <t>C25869</t>
-  </si>
-  <si>
-    <t>25E1667</t>
-  </si>
-  <si>
-    <t>20YJ</t>
-  </si>
-  <si>
-    <t>2025NE001830</t>
-  </si>
-  <si>
-    <t>25E1669</t>
-  </si>
-  <si>
-    <t>2025NE002200</t>
-  </si>
-  <si>
-    <t>C25863</t>
-  </si>
-  <si>
-    <t>25E2021</t>
-  </si>
-  <si>
-    <t>2025NE000367, 2025NE000369, 2025NE000371, 2025NE000413</t>
-  </si>
-  <si>
-    <t>2025NE002237</t>
-  </si>
-  <si>
-    <t>25E2058</t>
-  </si>
-  <si>
-    <t>2025NP001979</t>
-  </si>
-  <si>
-    <t>2026NE000330</t>
-  </si>
-  <si>
-    <t>C26163</t>
-  </si>
-  <si>
-    <t>26E0320</t>
-  </si>
-  <si>
-    <t>2026NE000388</t>
-  </si>
-  <si>
-    <t>C26193</t>
-  </si>
-  <si>
-    <t>26E0375</t>
-  </si>
-  <si>
-    <t>2026NE000748</t>
-  </si>
-  <si>
-    <t>C26312</t>
-  </si>
-  <si>
-    <t>26E0709</t>
-  </si>
-  <si>
-    <t>2026NE000816</t>
-  </si>
-  <si>
-    <t>C26324</t>
-  </si>
-  <si>
-    <t>26E0776</t>
-  </si>
-  <si>
-    <t>2026NE000817</t>
-  </si>
-  <si>
-    <t>C26326</t>
-  </si>
-  <si>
-    <t>26E0777</t>
-  </si>
-  <si>
-    <t>2026NE000842</t>
-  </si>
-  <si>
-    <t>26E0803</t>
-  </si>
-  <si>
-    <t>2026NE000944</t>
-  </si>
-  <si>
-    <t>26E0906</t>
-  </si>
-  <si>
-    <t>ABR/25</t>
-  </si>
-  <si>
-    <t>2025NE000413, 2025NE000414, 2025NE000559</t>
-  </si>
-  <si>
-    <t>2025NP002341</t>
-  </si>
-  <si>
-    <t>MAI/25</t>
-  </si>
-  <si>
-    <t>2025NP002884</t>
-  </si>
-  <si>
-    <t>JUN/25</t>
   </si>
   <si>
     <t>2025NE000005,
@@ -459,22 +360,64 @@
     <t>2025NP400522</t>
   </si>
   <si>
+    <t>2025NE001823</t>
+  </si>
+  <si>
+    <t>C25865</t>
+  </si>
+  <si>
+    <t>25E1666</t>
+  </si>
+  <si>
     <t>JUL/25</t>
   </si>
   <si>
+    <t>2025NE001828</t>
+  </si>
+  <si>
     <t>2025NE000843, 2025NE001200</t>
   </si>
   <si>
+    <t>C25869</t>
+  </si>
+  <si>
+    <t>25E1667</t>
+  </si>
+  <si>
+    <t>20YJ</t>
+  </si>
+  <si>
     <t>2025NP003724</t>
   </si>
   <si>
+    <t>2025NE001830</t>
+  </si>
+  <si>
+    <t>25E1669</t>
+  </si>
+  <si>
     <t>AGO/25</t>
   </si>
   <si>
     <t>2025NP004558</t>
   </si>
   <si>
+    <t>2025NE002200</t>
+  </si>
+  <si>
+    <t>C25863</t>
+  </si>
+  <si>
+    <t>25E2021</t>
+  </si>
+  <si>
     <t>SET/25</t>
+  </si>
+  <si>
+    <t>2025NE002237</t>
+  </si>
+  <si>
+    <t>25E2058</t>
   </si>
   <si>
     <t>2025NE001688 
@@ -484,15 +427,42 @@
     <t>2025NP004897</t>
   </si>
   <si>
+    <t>2026NE000330</t>
+  </si>
+  <si>
+    <t>C26163</t>
+  </si>
+  <si>
+    <t>26E0320</t>
+  </si>
+  <si>
     <t>OUT/25</t>
   </si>
   <si>
     <t>2025NE001688, 2025NE001828, 2025NE002200</t>
   </si>
   <si>
+    <t>2026NE000388</t>
+  </si>
+  <si>
+    <t>C26193</t>
+  </si>
+  <si>
+    <t>26E0375</t>
+  </si>
+  <si>
     <t>2025NP004932</t>
   </si>
   <si>
+    <t>2026NE000748</t>
+  </si>
+  <si>
+    <t>C26312</t>
+  </si>
+  <si>
+    <t>26E0709</t>
+  </si>
+  <si>
     <t>NOV/25</t>
   </si>
   <si>
@@ -502,21 +472,51 @@
     <t>2026NP400440</t>
   </si>
   <si>
+    <t>2026NE000816</t>
+  </si>
+  <si>
+    <t>C26324</t>
+  </si>
+  <si>
+    <t>26E0776</t>
+  </si>
+  <si>
     <t>DEZ/25</t>
   </si>
   <si>
+    <t>2026NE000817</t>
+  </si>
+  <si>
+    <t>C26326</t>
+  </si>
+  <si>
+    <t>26E0777</t>
+  </si>
+  <si>
     <t>2025NE001065, 2025NE002200</t>
   </si>
   <si>
     <t>2026NP400412</t>
   </si>
   <si>
+    <t>2026NE000842</t>
+  </si>
+  <si>
+    <t>26E0803</t>
+  </si>
+  <si>
     <t>JAN/26</t>
   </si>
   <si>
+    <t>2026NE000944</t>
+  </si>
+  <si>
     <t>2026NP401035</t>
   </si>
   <si>
+    <t>26E0906</t>
+  </si>
+  <si>
     <t>FEV/26</t>
   </si>
   <si>
@@ -559,7 +559,13 @@
     <t>JUNHO/26</t>
   </si>
   <si>
+    <t>2025NE001065, 2026NE000330</t>
+  </si>
+  <si>
     <t>R$ 1.340.865,98</t>
+  </si>
+  <si>
+    <t>2026NP402899</t>
   </si>
   <si>
     <t>Módulo II – Parcial Orçamento 10 (FAB 2728)</t>
@@ -665,8 +671,8 @@
     <numFmt numFmtId="166" formatCode="dd/MM/yyyy"/>
     <numFmt numFmtId="167" formatCode="R$ #,##0.00"/>
     <numFmt numFmtId="168" formatCode="[$R$-416]\ #,##0.00;[RED]\-[$R$-416]\ #,##0.00"/>
-    <numFmt numFmtId="169" formatCode="d/m/yyyy"/>
-    <numFmt numFmtId="170" formatCode="MM/DD/YY"/>
+    <numFmt numFmtId="169" formatCode="MM/DD/YY"/>
+    <numFmt numFmtId="170" formatCode="d/m/yyyy"/>
     <numFmt numFmtId="171" formatCode="_([$R$ -416]* #,##0.00_);_([$R$ -416]* \(#,##0.00\);_([$R$ -416]* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="12">
@@ -852,7 +858,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="78">
+  <cellXfs count="77">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -879,11 +885,11 @@
     <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="11" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="11" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
@@ -958,10 +964,10 @@
     <xf borderId="1" fillId="0" fontId="8" numFmtId="166" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="165" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="1" fillId="7" fontId="9" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="165" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="1" fillId="5" fontId="9" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
@@ -969,16 +975,13 @@
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="3" fillId="0" fontId="10" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="169" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
     <xf borderId="1" fillId="8" fontId="9" numFmtId="168" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="8" numFmtId="166" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="8" numFmtId="170" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="8" numFmtId="169" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="7" fontId="9" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
@@ -996,6 +999,9 @@
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="170" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
     <xf borderId="1" fillId="9" fontId="9" numFmtId="168" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
@@ -1007,12 +1013,6 @@
     </xf>
     <xf borderId="1" fillId="9" fontId="9" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="9" numFmtId="166" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="4" fillId="0" fontId="10" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="1" fillId="0" fontId="6" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
@@ -1026,6 +1026,9 @@
     </xf>
     <xf borderId="1" fillId="5" fontId="9" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="6" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
@@ -1417,14 +1420,14 @@
         <v>1</v>
       </c>
       <c r="V2" s="9"/>
-      <c r="W2" s="10"/>
-      <c r="X2" s="10"/>
-      <c r="Y2" s="10"/>
-      <c r="Z2" s="10"/>
-      <c r="AA2" s="10"/>
-      <c r="AB2" s="10"/>
-      <c r="AC2" s="10"/>
-      <c r="AD2" s="10"/>
+      <c r="W2" s="11"/>
+      <c r="X2" s="11"/>
+      <c r="Y2" s="11"/>
+      <c r="Z2" s="11"/>
+      <c r="AA2" s="11"/>
+      <c r="AB2" s="11"/>
+      <c r="AC2" s="11"/>
+      <c r="AD2" s="11"/>
     </row>
     <row r="3" ht="12.75" customHeight="1">
       <c r="A3" s="1"/>
@@ -1466,31 +1469,31 @@
         <v>12</v>
       </c>
       <c r="G4" s="17" t="s">
+        <v>13</v>
+      </c>
+      <c r="H4" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="H4" s="17" t="s">
+      <c r="I4" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="J4" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="I4" s="16" t="s">
+      <c r="K4" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="L4" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="J4" s="16" t="s">
-        <v>19</v>
-      </c>
-      <c r="K4" s="16" t="s">
+      <c r="M4" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="L4" s="16" t="s">
+      <c r="N4" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="M4" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="N4" s="17" t="s">
+      <c r="O4" s="17" t="s">
         <v>23</v>
-      </c>
-      <c r="O4" s="17" t="s">
-        <v>24</v>
       </c>
       <c r="P4" s="17" t="s">
         <v>25</v>
@@ -1517,16 +1520,16 @@
       <c r="B5" s="15"/>
       <c r="C5" s="18"/>
       <c r="D5" s="19" t="s">
+        <v>31</v>
+      </c>
+      <c r="E5" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="E5" s="19" t="s">
-        <v>34</v>
-      </c>
       <c r="F5" s="19" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="G5" s="19" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="H5" s="20">
         <v>1564.0</v>
@@ -1535,13 +1538,13 @@
         <v>1564.0</v>
       </c>
       <c r="J5" s="19" t="s">
+        <v>35</v>
+      </c>
+      <c r="K5" s="19" t="s">
         <v>36</v>
       </c>
-      <c r="K5" s="19" t="s">
+      <c r="L5" s="19" t="s">
         <v>37</v>
-      </c>
-      <c r="L5" s="19" t="s">
-        <v>38</v>
       </c>
       <c r="M5" s="19" t="s">
         <v>39</v>
@@ -1595,40 +1598,40 @@
       <c r="A8" s="23"/>
       <c r="B8" s="23"/>
       <c r="C8" s="28" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D8" s="28" t="s">
         <v>50</v>
       </c>
       <c r="E8" s="30" t="s">
+        <v>51</v>
+      </c>
+      <c r="F8" s="28" t="s">
+        <v>52</v>
+      </c>
+      <c r="G8" s="28" t="s">
+        <v>53</v>
+      </c>
+      <c r="H8" s="28" t="s">
         <v>54</v>
       </c>
-      <c r="F8" s="28" t="s">
-        <v>56</v>
-      </c>
-      <c r="G8" s="28" t="s">
-        <v>58</v>
-      </c>
-      <c r="H8" s="28" t="s">
+      <c r="I8" s="30" t="s">
+        <v>57</v>
+      </c>
+      <c r="J8" s="28" t="s">
+        <v>59</v>
+      </c>
+      <c r="K8" s="28" t="s">
         <v>60</v>
       </c>
-      <c r="I8" s="30" t="s">
+      <c r="L8" s="31" t="s">
         <v>61</v>
       </c>
-      <c r="J8" s="28" t="s">
-        <v>62</v>
-      </c>
-      <c r="K8" s="28" t="s">
+      <c r="M8" s="30" t="s">
         <v>63</v>
       </c>
-      <c r="L8" s="31" t="s">
+      <c r="N8" s="28" t="s">
         <v>64</v>
-      </c>
-      <c r="M8" s="30" t="s">
-        <v>65</v>
-      </c>
-      <c r="N8" s="28" t="s">
-        <v>67</v>
       </c>
       <c r="O8" s="28"/>
       <c r="P8" s="27"/>
@@ -1641,10 +1644,10 @@
         <v>1.0</v>
       </c>
       <c r="D9" s="33" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="E9" s="34" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="F9" s="35">
         <v>594.0</v>
@@ -1653,17 +1656,17 @@
         <v>45740.0</v>
       </c>
       <c r="H9" s="35" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="I9" s="36"/>
       <c r="J9" s="36">
         <v>45778.0</v>
       </c>
-      <c r="K9" s="38">
+      <c r="K9" s="37">
         <v>748504.24</v>
       </c>
       <c r="L9" s="35" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="M9" s="39">
         <f t="shared" ref="M9:M10" si="1">K9</f>
@@ -1679,10 +1682,10 @@
       <c r="B10" s="23"/>
       <c r="C10" s="41"/>
       <c r="D10" s="33" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="E10" s="34" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="F10" s="35">
         <v>620.0</v>
@@ -1691,23 +1694,23 @@
         <v>45775.0</v>
       </c>
       <c r="H10" s="35" t="s">
-        <v>111</v>
+        <v>86</v>
       </c>
       <c r="I10" s="36"/>
       <c r="J10" s="36">
         <v>45806.0</v>
       </c>
-      <c r="K10" s="38">
+      <c r="K10" s="37">
         <v>1110378.24</v>
       </c>
       <c r="L10" s="35" t="s">
-        <v>114</v>
+        <v>89</v>
       </c>
       <c r="M10" s="39">
         <f t="shared" si="1"/>
         <v>1110378.24</v>
       </c>
-      <c r="N10" s="43"/>
+      <c r="N10" s="42"/>
       <c r="O10" s="25"/>
       <c r="P10" s="27"/>
       <c r="V10" s="4"/>
@@ -1717,10 +1720,10 @@
       <c r="B11" s="23"/>
       <c r="C11" s="41"/>
       <c r="D11" s="33" t="s">
-        <v>134</v>
+        <v>93</v>
       </c>
       <c r="E11" s="34" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="F11" s="35">
         <v>634.0</v>
@@ -1729,22 +1732,22 @@
         <v>45799.0</v>
       </c>
       <c r="H11" s="35" t="s">
-        <v>135</v>
+        <v>94</v>
       </c>
       <c r="I11" s="36"/>
       <c r="J11" s="36">
         <v>45844.0</v>
       </c>
-      <c r="K11" s="38">
+      <c r="K11" s="37">
         <v>974557.12</v>
       </c>
       <c r="L11" s="34" t="s">
-        <v>136</v>
+        <v>97</v>
       </c>
       <c r="M11" s="39">
         <v>974557.12</v>
       </c>
-      <c r="N11" s="43"/>
+      <c r="N11" s="42"/>
       <c r="O11" s="25"/>
       <c r="P11" s="27"/>
       <c r="V11" s="4"/>
@@ -1754,34 +1757,34 @@
       <c r="B12" s="23"/>
       <c r="C12" s="41"/>
       <c r="D12" s="33" t="s">
-        <v>137</v>
+        <v>98</v>
       </c>
       <c r="E12" s="34" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="F12" s="34">
         <v>660.0</v>
       </c>
-      <c r="G12" s="44">
+      <c r="G12" s="43">
         <v>45856.0</v>
       </c>
-      <c r="H12" s="45" t="s">
-        <v>69</v>
+      <c r="H12" s="44" t="s">
+        <v>72</v>
       </c>
       <c r="I12" s="36"/>
       <c r="J12" s="36">
         <v>45891.0</v>
       </c>
-      <c r="K12" s="46">
+      <c r="K12" s="45">
         <v>1402001.34</v>
       </c>
-      <c r="L12" s="47" t="s">
-        <v>138</v>
+      <c r="L12" s="46" t="s">
+        <v>101</v>
       </c>
       <c r="M12" s="39">
         <v>1402001.34</v>
       </c>
-      <c r="N12" s="48"/>
+      <c r="N12" s="47"/>
       <c r="O12" s="25"/>
       <c r="P12" s="27"/>
       <c r="V12" s="4"/>
@@ -1790,11 +1793,11 @@
       <c r="A13" s="23"/>
       <c r="B13" s="23"/>
       <c r="C13" s="41"/>
-      <c r="D13" s="49" t="s">
-        <v>139</v>
+      <c r="D13" s="48" t="s">
+        <v>104</v>
       </c>
       <c r="E13" s="34" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="F13" s="35">
         <v>661.0</v>
@@ -1803,35 +1806,35 @@
         <v>45856.0</v>
       </c>
       <c r="H13" s="35" t="s">
-        <v>140</v>
-      </c>
-      <c r="I13" s="44"/>
-      <c r="J13" s="44">
+        <v>107</v>
+      </c>
+      <c r="I13" s="43"/>
+      <c r="J13" s="43">
         <v>45891.0</v>
       </c>
-      <c r="K13" s="46">
+      <c r="K13" s="45">
         <v>1223702.3</v>
       </c>
       <c r="L13" s="34" t="s">
-        <v>141</v>
+        <v>108</v>
       </c>
       <c r="M13" s="39">
         <v>1223702.3</v>
       </c>
-      <c r="N13" s="48"/>
+      <c r="N13" s="47"/>
       <c r="O13" s="25"/>
-      <c r="P13" s="50"/>
+      <c r="P13" s="49"/>
       <c r="V13" s="4"/>
     </row>
     <row r="14">
       <c r="A14" s="23"/>
       <c r="B14" s="23"/>
       <c r="C14" s="41"/>
-      <c r="D14" s="49" t="s">
-        <v>142</v>
+      <c r="D14" s="48" t="s">
+        <v>112</v>
       </c>
       <c r="E14" s="34" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="F14" s="34">
         <v>688.0</v>
@@ -1840,22 +1843,22 @@
         <v>45901.0</v>
       </c>
       <c r="H14" s="34" t="s">
-        <v>143</v>
-      </c>
-      <c r="I14" s="44"/>
-      <c r="J14" s="44">
+        <v>114</v>
+      </c>
+      <c r="I14" s="43"/>
+      <c r="J14" s="43">
         <v>45938.0</v>
       </c>
-      <c r="K14" s="46">
+      <c r="K14" s="45">
         <v>1011677.95</v>
       </c>
       <c r="L14" s="34" t="s">
-        <v>144</v>
+        <v>118</v>
       </c>
       <c r="M14" s="39">
         <v>1011677.95</v>
       </c>
-      <c r="N14" s="43"/>
+      <c r="N14" s="42"/>
       <c r="O14" s="25"/>
       <c r="P14" s="27"/>
       <c r="V14" s="4"/>
@@ -1864,11 +1867,11 @@
       <c r="A15" s="23"/>
       <c r="B15" s="23"/>
       <c r="C15" s="41"/>
-      <c r="D15" s="49" t="s">
-        <v>145</v>
+      <c r="D15" s="48" t="s">
+        <v>121</v>
       </c>
       <c r="E15" s="34" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="F15" s="34">
         <v>696.0</v>
@@ -1879,20 +1882,20 @@
       <c r="H15" s="34" t="s">
         <v>79</v>
       </c>
-      <c r="I15" s="44"/>
-      <c r="J15" s="44">
+      <c r="I15" s="43"/>
+      <c r="J15" s="43">
         <v>45938.0</v>
       </c>
-      <c r="K15" s="46">
+      <c r="K15" s="45">
         <v>896744.06</v>
       </c>
       <c r="L15" s="34" t="s">
-        <v>146</v>
+        <v>122</v>
       </c>
       <c r="M15" s="39">
         <v>896744.06</v>
       </c>
-      <c r="N15" s="48"/>
+      <c r="N15" s="47"/>
       <c r="O15" s="25"/>
       <c r="V15" s="4"/>
     </row>
@@ -1900,11 +1903,11 @@
       <c r="A16" s="23"/>
       <c r="B16" s="23"/>
       <c r="C16" s="41"/>
-      <c r="D16" s="49" t="s">
-        <v>147</v>
+      <c r="D16" s="48" t="s">
+        <v>126</v>
       </c>
       <c r="E16" s="34" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="F16" s="34">
         <v>704.0</v>
@@ -1913,22 +1916,22 @@
         <v>45957.0</v>
       </c>
       <c r="H16" s="34" t="s">
-        <v>148</v>
-      </c>
-      <c r="I16" s="44"/>
-      <c r="J16" s="44">
+        <v>129</v>
+      </c>
+      <c r="I16" s="43"/>
+      <c r="J16" s="43">
         <v>46003.0</v>
       </c>
-      <c r="K16" s="46">
+      <c r="K16" s="45">
         <v>919329.06</v>
       </c>
       <c r="L16" s="34" t="s">
-        <v>149</v>
+        <v>130</v>
       </c>
       <c r="M16" s="39">
         <v>919329.06</v>
       </c>
-      <c r="N16" s="43"/>
+      <c r="N16" s="42"/>
       <c r="O16" s="25"/>
       <c r="V16" s="4"/>
     </row>
@@ -1936,28 +1939,28 @@
       <c r="A17" s="23"/>
       <c r="B17" s="23"/>
       <c r="C17" s="41"/>
-      <c r="D17" s="49" t="s">
-        <v>150</v>
+      <c r="D17" s="48" t="s">
+        <v>134</v>
       </c>
       <c r="E17" s="34"/>
       <c r="F17" s="34">
         <v>705.0</v>
       </c>
-      <c r="G17" s="44">
+      <c r="G17" s="43">
         <v>45972.0</v>
       </c>
       <c r="H17" s="34" t="s">
-        <v>151</v>
+        <v>135</v>
       </c>
       <c r="I17" s="34"/>
-      <c r="J17" s="44">
+      <c r="J17" s="43">
         <v>46016.0</v>
       </c>
-      <c r="K17" s="46">
+      <c r="K17" s="45">
         <v>1157009.26</v>
       </c>
       <c r="L17" s="34" t="s">
-        <v>152</v>
+        <v>139</v>
       </c>
       <c r="M17" s="39">
         <v>1157009.26</v>
@@ -1970,30 +1973,30 @@
       <c r="A18" s="23"/>
       <c r="B18" s="23"/>
       <c r="C18" s="41"/>
-      <c r="D18" s="49" t="s">
-        <v>153</v>
+      <c r="D18" s="48" t="s">
+        <v>143</v>
       </c>
       <c r="E18" s="34" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="F18" s="34">
         <v>728.0</v>
       </c>
-      <c r="G18" s="44">
+      <c r="G18" s="43">
         <v>46008.0</v>
       </c>
       <c r="H18" s="34" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="I18" s="34"/>
-      <c r="J18" s="44">
+      <c r="J18" s="43">
         <v>46040.0</v>
       </c>
-      <c r="K18" s="46">
+      <c r="K18" s="45">
         <v>1214597.952</v>
       </c>
       <c r="L18" s="34" t="s">
-        <v>155</v>
+        <v>145</v>
       </c>
       <c r="M18" s="39">
         <v>1214597.952</v>
@@ -2010,30 +2013,30 @@
       <c r="A19" s="23"/>
       <c r="B19" s="23"/>
       <c r="C19" s="41"/>
-      <c r="D19" s="49" t="s">
-        <v>156</v>
+      <c r="D19" s="48" t="s">
+        <v>149</v>
       </c>
       <c r="E19" s="34" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="F19" s="34">
         <v>278.0</v>
       </c>
-      <c r="G19" s="44">
+      <c r="G19" s="43">
         <v>46042.0</v>
       </c>
       <c r="H19" s="34" t="s">
-        <v>157</v>
-      </c>
-      <c r="I19" s="44"/>
-      <c r="J19" s="44">
+        <v>153</v>
+      </c>
+      <c r="I19" s="43"/>
+      <c r="J19" s="43">
         <v>46074.0</v>
       </c>
-      <c r="K19" s="46">
+      <c r="K19" s="45">
         <v>967082.09</v>
       </c>
       <c r="L19" s="34" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="M19" s="39">
         <v>967082.09</v>
@@ -2050,28 +2053,28 @@
       <c r="A20" s="23"/>
       <c r="B20" s="23"/>
       <c r="C20" s="41"/>
-      <c r="D20" s="49" t="s">
-        <v>159</v>
+      <c r="D20" s="48" t="s">
+        <v>157</v>
       </c>
       <c r="E20" s="34"/>
       <c r="F20" s="34">
         <v>10.0</v>
       </c>
-      <c r="G20" s="44">
+      <c r="G20" s="43">
         <v>46078.0</v>
       </c>
       <c r="H20" s="34" t="s">
-        <v>99</v>
-      </c>
-      <c r="I20" s="44"/>
-      <c r="J20" s="44">
+        <v>109</v>
+      </c>
+      <c r="I20" s="43"/>
+      <c r="J20" s="43">
         <v>46106.0</v>
       </c>
-      <c r="K20" s="46">
+      <c r="K20" s="45">
         <v>719561.08</v>
       </c>
       <c r="L20" s="34" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="M20" s="39">
         <v>719561.08</v>
@@ -2088,24 +2091,24 @@
       <c r="A21" s="23"/>
       <c r="B21" s="23"/>
       <c r="C21" s="41"/>
-      <c r="D21" s="49" t="s">
+      <c r="D21" s="48" t="s">
         <v>161</v>
       </c>
       <c r="E21" s="34"/>
       <c r="F21" s="34">
         <v>15.0</v>
       </c>
-      <c r="G21" s="44">
+      <c r="G21" s="43">
         <v>46094.0</v>
       </c>
       <c r="H21" s="34" t="s">
         <v>162</v>
       </c>
-      <c r="I21" s="44"/>
-      <c r="J21" s="44">
+      <c r="I21" s="43"/>
+      <c r="J21" s="43">
         <v>46128.0</v>
       </c>
-      <c r="K21" s="46">
+      <c r="K21" s="45">
         <v>885881.08</v>
       </c>
       <c r="L21" s="34" t="s">
@@ -2126,24 +2129,24 @@
       <c r="A22" s="23"/>
       <c r="B22" s="23"/>
       <c r="C22" s="41"/>
-      <c r="D22" s="49" t="s">
+      <c r="D22" s="48" t="s">
         <v>164</v>
       </c>
       <c r="E22" s="34"/>
       <c r="F22" s="34">
         <v>28.0</v>
       </c>
-      <c r="G22" s="44">
+      <c r="G22" s="43">
         <v>46128.0</v>
       </c>
       <c r="H22" s="34" t="s">
         <v>165</v>
       </c>
-      <c r="I22" s="44"/>
-      <c r="J22" s="44">
+      <c r="I22" s="43"/>
+      <c r="J22" s="43">
         <v>46164.0</v>
       </c>
-      <c r="K22" s="46" t="s">
+      <c r="K22" s="45" t="s">
         <v>166</v>
       </c>
       <c r="L22" s="34" t="s">
@@ -2164,24 +2167,24 @@
       <c r="A23" s="23"/>
       <c r="B23" s="23"/>
       <c r="C23" s="41"/>
-      <c r="D23" s="49" t="s">
+      <c r="D23" s="48" t="s">
         <v>168</v>
       </c>
       <c r="E23" s="34"/>
       <c r="F23" s="34">
         <v>33.0</v>
       </c>
-      <c r="G23" s="44">
+      <c r="G23" s="43">
         <v>46156.0</v>
       </c>
       <c r="H23" s="34" t="s">
         <v>169</v>
       </c>
-      <c r="I23" s="44"/>
-      <c r="J23" s="44">
+      <c r="I23" s="43"/>
+      <c r="J23" s="43">
         <v>46191.0</v>
       </c>
-      <c r="K23" s="46">
+      <c r="K23" s="45">
         <v>1108954.4358333333</v>
       </c>
       <c r="L23" s="34" t="s">
@@ -2202,24 +2205,24 @@
       <c r="A24" s="23"/>
       <c r="B24" s="23"/>
       <c r="C24" s="41"/>
-      <c r="D24" s="49" t="s">
+      <c r="D24" s="48" t="s">
         <v>170</v>
       </c>
       <c r="E24" s="34"/>
       <c r="F24" s="34">
         <v>29.0</v>
       </c>
-      <c r="G24" s="44">
+      <c r="G24" s="43">
         <v>46149.0</v>
       </c>
       <c r="H24" s="34" t="s">
         <v>169</v>
       </c>
-      <c r="I24" s="44"/>
-      <c r="J24" s="44">
+      <c r="I24" s="43"/>
+      <c r="J24" s="43">
         <v>46185.0</v>
       </c>
-      <c r="K24" s="46">
+      <c r="K24" s="45">
         <v>218206.1</v>
       </c>
       <c r="L24" s="34" t="s">
@@ -2240,24 +2243,24 @@
       <c r="A25" s="23"/>
       <c r="B25" s="23"/>
       <c r="C25" s="41"/>
-      <c r="D25" s="49" t="s">
+      <c r="D25" s="48" t="s">
         <v>172</v>
       </c>
       <c r="E25" s="34"/>
-      <c r="F25" s="55">
+      <c r="F25" s="34">
         <v>40.0</v>
       </c>
-      <c r="G25" s="44">
+      <c r="G25" s="43">
         <v>46156.0</v>
       </c>
-      <c r="H25" s="55" t="s">
+      <c r="H25" s="34" t="s">
         <v>169</v>
       </c>
-      <c r="I25" s="44"/>
-      <c r="J25" s="56">
+      <c r="I25" s="43"/>
+      <c r="J25" s="43">
         <v>46191.0</v>
       </c>
-      <c r="K25" s="46">
+      <c r="K25" s="45">
         <v>1549250.84</v>
       </c>
       <c r="L25" s="34" t="s">
@@ -2266,7 +2269,7 @@
       <c r="M25" s="39">
         <v>1549250.84</v>
       </c>
-      <c r="N25" s="53"/>
+      <c r="N25" s="54"/>
       <c r="O25" s="25"/>
       <c r="R25" s="27"/>
       <c r="S25" s="27"/>
@@ -2277,24 +2280,34 @@
     <row r="26">
       <c r="A26" s="23"/>
       <c r="B26" s="23"/>
-      <c r="C26" s="57"/>
-      <c r="D26" s="49" t="s">
+      <c r="C26" s="55"/>
+      <c r="D26" s="48" t="s">
         <v>174</v>
       </c>
       <c r="E26" s="34"/>
-      <c r="F26" s="55"/>
-      <c r="G26" s="44"/>
-      <c r="H26" s="55"/>
-      <c r="I26" s="44"/>
-      <c r="J26" s="56"/>
-      <c r="K26" s="46"/>
+      <c r="F26" s="34">
+        <v>48.0</v>
+      </c>
+      <c r="G26" s="43">
+        <v>46230.0</v>
+      </c>
+      <c r="H26" s="34" t="s">
+        <v>175</v>
+      </c>
+      <c r="I26" s="43"/>
+      <c r="J26" s="43">
+        <v>46262.0</v>
+      </c>
+      <c r="K26" s="45" t="s">
+        <v>176</v>
+      </c>
       <c r="L26" s="34" t="s">
-        <v>65</v>
+        <v>177</v>
       </c>
       <c r="M26" s="39" t="s">
-        <v>175</v>
-      </c>
-      <c r="N26" s="53"/>
+        <v>176</v>
+      </c>
+      <c r="N26" s="54"/>
       <c r="O26" s="25"/>
       <c r="R26" s="27"/>
       <c r="S26" s="27"/>
@@ -2306,34 +2319,34 @@
       <c r="A27" s="23"/>
       <c r="B27" s="23"/>
       <c r="C27" s="28" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D27" s="28" t="s">
         <v>50</v>
       </c>
       <c r="E27" s="30" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="F27" s="28" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="G27" s="28"/>
       <c r="H27" s="28" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="I27" s="28"/>
       <c r="J27" s="28"/>
-      <c r="K27" s="58" t="s">
+      <c r="K27" s="56" t="s">
+        <v>60</v>
+      </c>
+      <c r="L27" s="31" t="s">
+        <v>61</v>
+      </c>
+      <c r="M27" s="57" t="s">
         <v>63</v>
       </c>
-      <c r="L27" s="31" t="s">
+      <c r="N27" s="28" t="s">
         <v>64</v>
-      </c>
-      <c r="M27" s="59" t="s">
-        <v>65</v>
-      </c>
-      <c r="N27" s="28" t="s">
-        <v>67</v>
       </c>
       <c r="O27" s="25"/>
       <c r="P27" s="27"/>
@@ -2356,8 +2369,8 @@
       <c r="C28" s="32">
         <v>2.0</v>
       </c>
-      <c r="D28" s="60" t="s">
-        <v>176</v>
+      <c r="D28" s="58" t="s">
+        <v>178</v>
       </c>
       <c r="E28" s="35"/>
       <c r="F28" s="35">
@@ -2367,19 +2380,19 @@
         <v>45791.0</v>
       </c>
       <c r="H28" s="35" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="I28" s="36"/>
       <c r="J28" s="36">
         <v>45834.0</v>
       </c>
-      <c r="K28" s="38">
+      <c r="K28" s="37">
         <v>188246.17</v>
       </c>
       <c r="L28" s="34" t="s">
-        <v>177</v>
-      </c>
-      <c r="M28" s="61">
+        <v>179</v>
+      </c>
+      <c r="M28" s="59">
         <v>188246.17</v>
       </c>
       <c r="N28" s="51"/>
@@ -2403,10 +2416,10 @@
       <c r="A29" s="23"/>
       <c r="B29" s="23"/>
       <c r="C29" s="41"/>
-      <c r="D29" s="60" t="s">
-        <v>178</v>
-      </c>
-      <c r="E29" s="55">
+      <c r="D29" s="58" t="s">
+        <v>180</v>
+      </c>
+      <c r="E29" s="60">
         <v>46.0</v>
       </c>
       <c r="F29" s="35">
@@ -2416,17 +2429,17 @@
         <v>45814.0</v>
       </c>
       <c r="H29" s="34" t="s">
-        <v>179</v>
-      </c>
-      <c r="I29" s="44"/>
-      <c r="J29" s="44">
+        <v>181</v>
+      </c>
+      <c r="I29" s="43"/>
+      <c r="J29" s="43">
         <v>45955.0</v>
       </c>
-      <c r="K29" s="38">
+      <c r="K29" s="37">
         <v>112720.77</v>
       </c>
       <c r="L29" s="34" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="M29" s="39">
         <v>112720.77</v>
@@ -2452,37 +2465,37 @@
       <c r="A30" s="23"/>
       <c r="B30" s="23"/>
       <c r="C30" s="41"/>
-      <c r="D30" s="62" t="s">
-        <v>181</v>
-      </c>
-      <c r="E30" s="63" t="s">
-        <v>182</v>
+      <c r="D30" s="61" t="s">
+        <v>183</v>
+      </c>
+      <c r="E30" s="62" t="s">
+        <v>184</v>
       </c>
       <c r="F30" s="35">
         <v>529.0</v>
       </c>
-      <c r="G30" s="64">
+      <c r="G30" s="63">
         <v>45853.0</v>
       </c>
       <c r="H30" s="34" t="s">
-        <v>57</v>
-      </c>
-      <c r="I30" s="44"/>
-      <c r="J30" s="44">
+        <v>65</v>
+      </c>
+      <c r="I30" s="43"/>
+      <c r="J30" s="43">
         <v>45939.0</v>
       </c>
-      <c r="K30" s="46">
+      <c r="K30" s="45">
         <v>378307.61</v>
       </c>
       <c r="L30" s="34" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="M30" s="39">
         <v>378307.61</v>
       </c>
       <c r="N30" s="51"/>
       <c r="O30" s="25"/>
-      <c r="P30" s="65"/>
+      <c r="P30" s="64"/>
       <c r="Q30" s="27"/>
       <c r="R30" s="27"/>
       <c r="S30" s="27"/>
@@ -2501,37 +2514,37 @@
       <c r="A31" s="23"/>
       <c r="B31" s="23"/>
       <c r="C31" s="41"/>
-      <c r="D31" s="62" t="s">
+      <c r="D31" s="61" t="s">
+        <v>186</v>
+      </c>
+      <c r="E31" s="62" t="s">
         <v>184</v>
-      </c>
-      <c r="E31" s="63" t="s">
-        <v>182</v>
       </c>
       <c r="F31" s="34">
         <v>691.0</v>
       </c>
-      <c r="G31" s="64">
+      <c r="G31" s="63">
         <v>45910.0</v>
       </c>
       <c r="H31" s="34" t="s">
-        <v>57</v>
-      </c>
-      <c r="I31" s="44"/>
-      <c r="J31" s="44">
+        <v>65</v>
+      </c>
+      <c r="I31" s="43"/>
+      <c r="J31" s="43">
         <v>45941.0</v>
       </c>
-      <c r="K31" s="38">
+      <c r="K31" s="37">
         <v>3315.0471000000252</v>
       </c>
       <c r="L31" s="34" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="M31" s="39">
         <v>3315.04710000003</v>
       </c>
       <c r="N31" s="51"/>
       <c r="O31" s="25"/>
-      <c r="P31" s="65"/>
+      <c r="P31" s="64"/>
       <c r="Q31" s="27"/>
       <c r="R31" s="27"/>
       <c r="S31" s="27"/>
@@ -2550,37 +2563,37 @@
       <c r="A32" s="23"/>
       <c r="B32" s="23"/>
       <c r="C32" s="41"/>
-      <c r="D32" s="62" t="s">
-        <v>186</v>
-      </c>
-      <c r="E32" s="66">
+      <c r="D32" s="61" t="s">
+        <v>188</v>
+      </c>
+      <c r="E32" s="65">
         <v>135.0</v>
       </c>
       <c r="F32" s="34">
         <v>677.0</v>
       </c>
-      <c r="G32" s="64">
+      <c r="G32" s="63">
         <v>45904.0</v>
       </c>
       <c r="H32" s="34" t="s">
-        <v>69</v>
-      </c>
-      <c r="I32" s="67"/>
-      <c r="J32" s="67">
+        <v>72</v>
+      </c>
+      <c r="I32" s="66"/>
+      <c r="J32" s="66">
         <v>45935.0</v>
       </c>
-      <c r="K32" s="46">
+      <c r="K32" s="45">
         <v>198332.75</v>
       </c>
       <c r="L32" s="34" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="M32" s="39">
         <v>198332.75</v>
       </c>
       <c r="N32" s="51"/>
       <c r="O32" s="25"/>
-      <c r="P32" s="65"/>
+      <c r="P32" s="64"/>
       <c r="Q32" s="27"/>
       <c r="R32" s="27"/>
       <c r="S32" s="27"/>
@@ -2599,37 +2612,37 @@
       <c r="A33" s="23"/>
       <c r="B33" s="23"/>
       <c r="C33" s="41"/>
-      <c r="D33" s="62" t="s">
-        <v>188</v>
-      </c>
-      <c r="E33" s="66">
+      <c r="D33" s="61" t="s">
+        <v>190</v>
+      </c>
+      <c r="E33" s="65">
         <v>40.0</v>
       </c>
       <c r="F33" s="34">
         <v>278.0</v>
       </c>
-      <c r="G33" s="64">
+      <c r="G33" s="63">
         <v>46008.0</v>
       </c>
       <c r="H33" s="34" t="s">
-        <v>108</v>
-      </c>
-      <c r="I33" s="67"/>
-      <c r="J33" s="67">
+        <v>123</v>
+      </c>
+      <c r="I33" s="66"/>
+      <c r="J33" s="66">
         <v>46066.0</v>
       </c>
-      <c r="K33" s="46">
+      <c r="K33" s="45">
         <v>1528.62</v>
       </c>
-      <c r="L33" s="68" t="s">
-        <v>189</v>
-      </c>
-      <c r="M33" s="69" t="s">
-        <v>190</v>
+      <c r="L33" s="67" t="s">
+        <v>191</v>
+      </c>
+      <c r="M33" s="68" t="s">
+        <v>192</v>
       </c>
       <c r="N33" s="51"/>
       <c r="O33" s="25"/>
-      <c r="P33" s="65"/>
+      <c r="P33" s="64"/>
       <c r="Q33" s="27"/>
       <c r="R33" s="27"/>
       <c r="S33" s="27"/>
@@ -2648,37 +2661,37 @@
       <c r="A34" s="23"/>
       <c r="B34" s="23"/>
       <c r="C34" s="41"/>
-      <c r="D34" s="62" t="s">
-        <v>191</v>
-      </c>
-      <c r="E34" s="66" t="s">
-        <v>192</v>
+      <c r="D34" s="61" t="s">
+        <v>193</v>
+      </c>
+      <c r="E34" s="65" t="s">
+        <v>194</v>
       </c>
       <c r="F34" s="34">
         <v>748.0</v>
       </c>
-      <c r="G34" s="64">
+      <c r="G34" s="63">
         <v>45930.0</v>
       </c>
       <c r="H34" s="34" t="s">
-        <v>91</v>
-      </c>
-      <c r="I34" s="67"/>
-      <c r="J34" s="67">
+        <v>95</v>
+      </c>
+      <c r="I34" s="66"/>
+      <c r="J34" s="66">
         <v>45935.0</v>
       </c>
-      <c r="K34" s="46">
+      <c r="K34" s="45">
         <v>38718.58</v>
       </c>
       <c r="L34" s="34" t="s">
-        <v>193</v>
-      </c>
-      <c r="M34" s="61" t="s">
-        <v>194</v>
+        <v>195</v>
+      </c>
+      <c r="M34" s="59" t="s">
+        <v>196</v>
       </c>
       <c r="N34" s="51"/>
       <c r="O34" s="25"/>
-      <c r="P34" s="65"/>
+      <c r="P34" s="64"/>
       <c r="Q34" s="27"/>
       <c r="R34" s="27"/>
       <c r="S34" s="27"/>
@@ -2697,37 +2710,37 @@
       <c r="A35" s="23"/>
       <c r="B35" s="23"/>
       <c r="C35" s="41"/>
-      <c r="D35" s="62" t="s">
-        <v>195</v>
-      </c>
-      <c r="E35" s="66">
+      <c r="D35" s="61" t="s">
+        <v>197</v>
+      </c>
+      <c r="E35" s="65">
         <v>154.0</v>
       </c>
       <c r="F35" s="34">
         <v>822.0</v>
       </c>
-      <c r="G35" s="64">
+      <c r="G35" s="63">
         <v>45968.0</v>
       </c>
       <c r="H35" s="34" t="s">
-        <v>102</v>
-      </c>
-      <c r="I35" s="67"/>
-      <c r="J35" s="67">
+        <v>113</v>
+      </c>
+      <c r="I35" s="66"/>
+      <c r="J35" s="66">
         <v>45935.0</v>
       </c>
-      <c r="K35" s="46">
+      <c r="K35" s="45">
         <v>133124.11</v>
       </c>
       <c r="L35" s="34" t="s">
-        <v>196</v>
-      </c>
-      <c r="M35" s="61" t="s">
-        <v>197</v>
+        <v>198</v>
+      </c>
+      <c r="M35" s="59" t="s">
+        <v>199</v>
       </c>
       <c r="N35" s="51"/>
       <c r="O35" s="25"/>
-      <c r="P35" s="65"/>
+      <c r="P35" s="64"/>
       <c r="Q35" s="27"/>
       <c r="R35" s="27"/>
       <c r="S35" s="27"/>
@@ -2746,30 +2759,30 @@
       <c r="A36" s="23"/>
       <c r="B36" s="23"/>
       <c r="C36" s="41"/>
-      <c r="D36" s="62" t="s">
-        <v>198</v>
-      </c>
-      <c r="E36" s="66">
+      <c r="D36" s="61" t="s">
+        <v>200</v>
+      </c>
+      <c r="E36" s="65">
         <v>252.0</v>
       </c>
-      <c r="F36" s="66">
+      <c r="F36" s="65">
         <v>360.0</v>
       </c>
-      <c r="G36" s="70">
+      <c r="G36" s="69">
         <v>46043.0</v>
       </c>
-      <c r="H36" s="66" t="s">
-        <v>99</v>
-      </c>
-      <c r="I36" s="71"/>
-      <c r="J36" s="70">
+      <c r="H36" s="65" t="s">
+        <v>109</v>
+      </c>
+      <c r="I36" s="70"/>
+      <c r="J36" s="69">
         <v>46075.0</v>
       </c>
-      <c r="K36" s="46">
+      <c r="K36" s="45">
         <v>11372.9</v>
       </c>
       <c r="L36" s="34" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="M36" s="39">
         <v>11372.9</v>
@@ -2795,18 +2808,18 @@
       <c r="A37" s="23"/>
       <c r="B37" s="23"/>
       <c r="C37" s="41"/>
-      <c r="D37" s="62" t="s">
-        <v>200</v>
-      </c>
-      <c r="E37" s="66"/>
-      <c r="F37" s="66"/>
-      <c r="G37" s="70"/>
-      <c r="H37" s="66"/>
-      <c r="I37" s="66" t="s">
-        <v>201</v>
-      </c>
-      <c r="J37" s="70"/>
-      <c r="K37" s="46"/>
+      <c r="D37" s="61" t="s">
+        <v>202</v>
+      </c>
+      <c r="E37" s="65"/>
+      <c r="F37" s="65"/>
+      <c r="G37" s="69"/>
+      <c r="H37" s="65"/>
+      <c r="I37" s="65" t="s">
+        <v>203</v>
+      </c>
+      <c r="J37" s="69"/>
+      <c r="K37" s="45"/>
       <c r="L37" s="34"/>
       <c r="M37" s="39"/>
       <c r="N37" s="51">
@@ -2831,23 +2844,23 @@
     <row r="38" ht="12.75" customHeight="1">
       <c r="A38" s="23"/>
       <c r="B38" s="23"/>
-      <c r="C38" s="57"/>
-      <c r="D38" s="62" t="s">
-        <v>202</v>
-      </c>
-      <c r="E38" s="66"/>
-      <c r="F38" s="66"/>
-      <c r="G38" s="70"/>
-      <c r="H38" s="66"/>
-      <c r="I38" s="66" t="s">
-        <v>201</v>
-      </c>
-      <c r="J38" s="70"/>
-      <c r="K38" s="46"/>
+      <c r="C38" s="55"/>
+      <c r="D38" s="61" t="s">
+        <v>204</v>
+      </c>
+      <c r="E38" s="65"/>
+      <c r="F38" s="65"/>
+      <c r="G38" s="69"/>
+      <c r="H38" s="65"/>
+      <c r="I38" s="65" t="s">
+        <v>203</v>
+      </c>
+      <c r="J38" s="69"/>
+      <c r="K38" s="45"/>
       <c r="L38" s="34"/>
       <c r="M38" s="39"/>
       <c r="N38" s="51" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="O38" s="25"/>
       <c r="P38" s="27"/>
@@ -2871,30 +2884,30 @@
       <c r="C39" s="32">
         <v>3.0</v>
       </c>
-      <c r="D39" s="62" t="s">
-        <v>204</v>
-      </c>
-      <c r="E39" s="66"/>
-      <c r="F39" s="66">
+      <c r="D39" s="61" t="s">
+        <v>206</v>
+      </c>
+      <c r="E39" s="65"/>
+      <c r="F39" s="65">
         <v>1465.0</v>
       </c>
-      <c r="G39" s="70">
+      <c r="G39" s="69">
         <v>46104.0</v>
       </c>
-      <c r="H39" s="66" t="s">
-        <v>99</v>
-      </c>
-      <c r="I39" s="71"/>
-      <c r="J39" s="70">
+      <c r="H39" s="65" t="s">
+        <v>109</v>
+      </c>
+      <c r="I39" s="70"/>
+      <c r="J39" s="69">
         <v>46106.0</v>
       </c>
-      <c r="K39" s="46">
+      <c r="K39" s="45">
         <v>27801.11</v>
       </c>
-      <c r="L39" s="72" t="s">
-        <v>205</v>
-      </c>
-      <c r="M39" s="73">
+      <c r="L39" s="71" t="s">
+        <v>207</v>
+      </c>
+      <c r="M39" s="72">
         <v>27801.11</v>
       </c>
       <c r="N39" s="51"/>
@@ -2918,30 +2931,30 @@
       <c r="A40" s="15"/>
       <c r="B40" s="15"/>
       <c r="C40" s="41"/>
-      <c r="D40" s="62" t="s">
-        <v>206</v>
-      </c>
-      <c r="E40" s="66"/>
-      <c r="F40" s="66">
+      <c r="D40" s="61" t="s">
+        <v>208</v>
+      </c>
+      <c r="E40" s="65"/>
+      <c r="F40" s="65">
         <v>1882.0</v>
       </c>
-      <c r="G40" s="70">
+      <c r="G40" s="69">
         <v>46199.0</v>
       </c>
-      <c r="H40" s="66" t="s">
-        <v>75</v>
-      </c>
-      <c r="I40" s="71"/>
-      <c r="J40" s="70">
+      <c r="H40" s="65" t="s">
+        <v>77</v>
+      </c>
+      <c r="I40" s="70"/>
+      <c r="J40" s="69">
         <v>46233.0</v>
       </c>
-      <c r="K40" s="46">
+      <c r="K40" s="45">
         <v>58868.35</v>
       </c>
       <c r="L40" s="34" t="s">
-        <v>65</v>
-      </c>
-      <c r="M40" s="73">
+        <v>63</v>
+      </c>
+      <c r="M40" s="72">
         <v>58868.35</v>
       </c>
       <c r="N40" s="51"/>
@@ -2951,16 +2964,16 @@
       <c r="A41" s="15"/>
       <c r="B41" s="15"/>
       <c r="C41" s="41"/>
-      <c r="K41" s="74"/>
-      <c r="M41" s="74"/>
+      <c r="K41" s="73"/>
+      <c r="M41" s="73"/>
       <c r="V41" s="4"/>
     </row>
     <row r="42" ht="12.75" customHeight="1">
       <c r="A42" s="15"/>
       <c r="B42" s="15"/>
       <c r="C42" s="41"/>
-      <c r="K42" s="74"/>
-      <c r="M42" s="74"/>
+      <c r="K42" s="73"/>
+      <c r="M42" s="73"/>
       <c r="V42" s="4"/>
     </row>
     <row r="43" ht="12.75" customHeight="1">
@@ -2990,9 +3003,9 @@
     <row r="47" ht="12.75" customHeight="1">
       <c r="A47" s="15"/>
       <c r="B47" s="15"/>
-      <c r="C47" s="57"/>
-      <c r="K47" s="74"/>
-      <c r="M47" s="74"/>
+      <c r="C47" s="55"/>
+      <c r="K47" s="73"/>
+      <c r="M47" s="73"/>
       <c r="V47" s="4"/>
     </row>
     <row r="48" ht="12.75" customHeight="1">
@@ -3011,12 +3024,12 @@
       <c r="M48" s="15"/>
       <c r="N48" s="15"/>
       <c r="O48" s="15"/>
-      <c r="P48" s="75"/>
-      <c r="Q48" s="75"/>
-      <c r="R48" s="75"/>
-      <c r="S48" s="75"/>
-      <c r="T48" s="75"/>
-      <c r="U48" s="75"/>
+      <c r="P48" s="74"/>
+      <c r="Q48" s="74"/>
+      <c r="R48" s="74"/>
+      <c r="S48" s="74"/>
+      <c r="T48" s="74"/>
+      <c r="U48" s="74"/>
       <c r="V48" s="4"/>
     </row>
     <row r="49" ht="12.75" customHeight="1">
@@ -7919,7 +7932,7 @@
       <c r="B3" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="11">
+      <c r="C3" s="10">
         <v>2.5E32</v>
       </c>
       <c r="D3" s="8" t="s">
@@ -8004,13 +8017,13 @@
     </row>
     <row r="5">
       <c r="A5" s="8" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="D5" s="8" t="s">
         <v>4</v>
@@ -8049,13 +8062,13 @@
     </row>
     <row r="6">
       <c r="A6" s="8" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="D6" s="8" t="s">
         <v>4</v>
@@ -8163,7 +8176,7 @@
         <v>339039.0</v>
       </c>
       <c r="I8" s="8" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="J8" s="14">
         <v>524584.95</v>
@@ -8185,13 +8198,13 @@
     </row>
     <row r="9">
       <c r="A9" s="8" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="D9" s="8" t="s">
         <v>4</v>
@@ -8209,7 +8222,7 @@
         <v>339039.0</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="J9" s="14">
         <v>211614.23</v>
@@ -8230,13 +8243,13 @@
     </row>
     <row r="10">
       <c r="A10" s="8" t="s">
-        <v>57</v>
+        <v>65</v>
       </c>
       <c r="B10" s="8" t="s">
         <v>7</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="D10" s="8" t="s">
         <v>4</v>
@@ -8275,13 +8288,13 @@
     </row>
     <row r="11">
       <c r="A11" s="8" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D11" s="8" t="s">
         <v>4</v>
@@ -8320,13 +8333,13 @@
     </row>
     <row r="12">
       <c r="A12" s="8" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="D12" s="8" t="s">
         <v>4</v>
@@ -8344,7 +8357,7 @@
         <v>339039.0</v>
       </c>
       <c r="I12" s="8" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="J12" s="14">
         <v>1600334.09</v>
@@ -8365,13 +8378,13 @@
     </row>
     <row r="13">
       <c r="A13" s="8" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B13" s="8" t="s">
         <v>7</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D13" s="8" t="s">
         <v>4</v>
@@ -8400,7 +8413,7 @@
       <c r="L13" s="14">
         <v>0.0</v>
       </c>
-      <c r="M13" s="37"/>
+      <c r="M13" s="38"/>
       <c r="AB13" s="2"/>
       <c r="AC13" s="2"/>
       <c r="AD13" s="2"/>
@@ -8435,7 +8448,7 @@
         <v>339039.0</v>
       </c>
       <c r="I14" s="8" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="J14" s="14">
         <v>968237.39</v>
@@ -8456,13 +8469,13 @@
     </row>
     <row r="15">
       <c r="A15" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D15" s="8" t="s">
         <v>4</v>
@@ -8501,13 +8514,13 @@
     </row>
     <row r="16">
       <c r="A16" s="8" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B16" s="8" t="s">
         <v>7</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D16" s="8" t="s">
         <v>4</v>
@@ -8546,13 +8559,13 @@
     </row>
     <row r="17">
       <c r="A17" s="8" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D17" s="8" t="s">
         <v>4</v>
@@ -8591,13 +8604,13 @@
     </row>
     <row r="18">
       <c r="A18" s="8" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="B18" s="8" t="s">
         <v>80</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D18" s="8" t="s">
         <v>4</v>
@@ -8615,7 +8628,7 @@
         <v>339039.0</v>
       </c>
       <c r="I18" s="8" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="J18" s="14">
         <v>63746.85</v>
@@ -8636,13 +8649,13 @@
     </row>
     <row r="19">
       <c r="A19" s="8" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="D19" s="8" t="s">
         <v>4</v>
@@ -8660,7 +8673,7 @@
         <v>339039.0</v>
       </c>
       <c r="I19" s="8" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="J19" s="14">
         <v>947931.1</v>
@@ -8681,13 +8694,13 @@
     </row>
     <row r="20">
       <c r="A20" s="8" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="B20" s="8" t="s">
         <v>7</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="D20" s="8" t="s">
         <v>4</v>
@@ -8726,13 +8739,13 @@
     </row>
     <row r="21">
       <c r="A21" s="8" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="D21" s="8" t="s">
         <v>4</v>
@@ -8771,18 +8784,18 @@
     </row>
     <row r="22">
       <c r="A22" s="8" t="s">
-        <v>99</v>
+        <v>109</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="D22" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E22" s="42">
+      <c r="E22" s="50">
         <v>45953.0</v>
       </c>
       <c r="F22" s="8" t="s">
@@ -8816,18 +8829,18 @@
     </row>
     <row r="23">
       <c r="A23" s="8" t="s">
-        <v>102</v>
+        <v>113</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>103</v>
+        <v>115</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>104</v>
+        <v>116</v>
       </c>
       <c r="D23" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E23" s="42">
+      <c r="E23" s="50">
         <v>45953.0</v>
       </c>
       <c r="F23" s="8" t="s">
@@ -8840,7 +8853,7 @@
         <v>339039.0</v>
       </c>
       <c r="I23" s="8" t="s">
-        <v>105</v>
+        <v>117</v>
       </c>
       <c r="J23" s="14">
         <v>1000001.64</v>
@@ -8861,18 +8874,18 @@
     </row>
     <row r="24">
       <c r="A24" s="8" t="s">
-        <v>106</v>
+        <v>119</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>107</v>
+        <v>120</v>
       </c>
       <c r="D24" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E24" s="42">
+      <c r="E24" s="50">
         <v>45953.0</v>
       </c>
       <c r="F24" s="8" t="s">
@@ -8906,18 +8919,18 @@
     </row>
     <row r="25">
       <c r="A25" s="8" t="s">
-        <v>108</v>
+        <v>123</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>109</v>
+        <v>124</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>110</v>
+        <v>125</v>
       </c>
       <c r="D25" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E25" s="42">
+      <c r="E25" s="50">
         <v>45975.0</v>
       </c>
       <c r="F25" s="8" t="s">
@@ -8930,7 +8943,7 @@
         <v>339039.0</v>
       </c>
       <c r="I25" s="8" t="s">
-        <v>105</v>
+        <v>117</v>
       </c>
       <c r="J25" s="14">
         <v>1157673.06</v>
@@ -8951,18 +8964,18 @@
     </row>
     <row r="26">
       <c r="A26" s="8" t="s">
-        <v>112</v>
+        <v>127</v>
       </c>
       <c r="B26" s="8" t="s">
         <v>7</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>113</v>
+        <v>128</v>
       </c>
       <c r="D26" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E26" s="42">
+      <c r="E26" s="50">
         <v>45989.0</v>
       </c>
       <c r="F26" s="8" t="s">
@@ -8996,13 +9009,13 @@
     </row>
     <row r="27">
       <c r="A27" s="8" t="s">
-        <v>115</v>
+        <v>131</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>116</v>
+        <v>132</v>
       </c>
       <c r="C27" s="8" t="s">
-        <v>117</v>
+        <v>133</v>
       </c>
       <c r="D27" s="8" t="s">
         <v>4</v>
@@ -9041,13 +9054,13 @@
     </row>
     <row r="28">
       <c r="A28" s="8" t="s">
-        <v>118</v>
+        <v>136</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>119</v>
+        <v>137</v>
       </c>
       <c r="C28" s="8" t="s">
-        <v>120</v>
+        <v>138</v>
       </c>
       <c r="D28" s="8" t="s">
         <v>4</v>
@@ -9065,7 +9078,7 @@
         <v>339039.0</v>
       </c>
       <c r="I28" s="8" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="J28" s="14">
         <v>1912292.52</v>
@@ -9086,13 +9099,13 @@
     </row>
     <row r="29">
       <c r="A29" s="8" t="s">
-        <v>121</v>
+        <v>140</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>122</v>
+        <v>141</v>
       </c>
       <c r="C29" s="8" t="s">
-        <v>123</v>
+        <v>142</v>
       </c>
       <c r="D29" s="8" t="s">
         <v>4</v>
@@ -9131,13 +9144,13 @@
     </row>
     <row r="30">
       <c r="A30" s="8" t="s">
-        <v>124</v>
+        <v>146</v>
       </c>
       <c r="B30" s="8" t="s">
-        <v>125</v>
+        <v>147</v>
       </c>
       <c r="C30" s="8" t="s">
-        <v>126</v>
+        <v>148</v>
       </c>
       <c r="D30" s="8" t="s">
         <v>4</v>
@@ -9176,13 +9189,13 @@
     </row>
     <row r="31">
       <c r="A31" s="8" t="s">
-        <v>127</v>
+        <v>150</v>
       </c>
       <c r="B31" s="8" t="s">
-        <v>128</v>
+        <v>151</v>
       </c>
       <c r="C31" s="8" t="s">
-        <v>129</v>
+        <v>152</v>
       </c>
       <c r="D31" s="8" t="s">
         <v>4</v>
@@ -9200,7 +9213,7 @@
         <v>339039.0</v>
       </c>
       <c r="I31" s="8" t="s">
-        <v>105</v>
+        <v>117</v>
       </c>
       <c r="J31" s="14">
         <v>18462.36</v>
@@ -9221,13 +9234,13 @@
     </row>
     <row r="32">
       <c r="A32" s="8" t="s">
-        <v>130</v>
+        <v>155</v>
       </c>
       <c r="B32" s="8" t="s">
-        <v>128</v>
+        <v>151</v>
       </c>
       <c r="C32" s="14" t="s">
-        <v>131</v>
+        <v>156</v>
       </c>
       <c r="D32" s="8" t="s">
         <v>4</v>
@@ -9245,7 +9258,7 @@
         <v>339039.0</v>
       </c>
       <c r="I32" s="8" t="s">
-        <v>105</v>
+        <v>117</v>
       </c>
       <c r="J32" s="14">
         <v>1530656.62</v>
@@ -9266,13 +9279,13 @@
     </row>
     <row r="33">
       <c r="A33" s="8" t="s">
-        <v>132</v>
+        <v>158</v>
       </c>
       <c r="B33" s="8" t="s">
-        <v>122</v>
+        <v>141</v>
       </c>
       <c r="C33" s="14" t="s">
-        <v>133</v>
+        <v>160</v>
       </c>
       <c r="D33" s="8" t="s">
         <v>4</v>
@@ -17610,18 +17623,18 @@
       <c r="I955" s="2"/>
       <c r="J955" s="2"/>
       <c r="K955" s="2"/>
-      <c r="L955" s="76"/>
+      <c r="L955" s="75"/>
       <c r="M955" s="2"/>
       <c r="N955" s="2"/>
       <c r="O955" s="2"/>
       <c r="P955" s="2"/>
       <c r="Q955" s="2"/>
-      <c r="R955" s="77"/>
-      <c r="S955" s="77"/>
-      <c r="T955" s="77"/>
-      <c r="U955" s="77"/>
-      <c r="V955" s="77"/>
-      <c r="W955" s="76"/>
+      <c r="R955" s="76"/>
+      <c r="S955" s="76"/>
+      <c r="T955" s="76"/>
+      <c r="U955" s="76"/>
+      <c r="V955" s="76"/>
+      <c r="W955" s="75"/>
       <c r="X955" s="2"/>
       <c r="Y955" s="2"/>
       <c r="Z955" s="2"/>
@@ -17646,18 +17659,18 @@
       <c r="I956" s="2"/>
       <c r="J956" s="2"/>
       <c r="K956" s="2"/>
-      <c r="L956" s="76"/>
+      <c r="L956" s="75"/>
       <c r="M956" s="2"/>
       <c r="N956" s="2"/>
       <c r="O956" s="2"/>
       <c r="P956" s="2"/>
       <c r="Q956" s="2"/>
-      <c r="R956" s="77"/>
-      <c r="S956" s="77"/>
-      <c r="T956" s="77"/>
-      <c r="U956" s="77"/>
-      <c r="V956" s="77"/>
-      <c r="W956" s="76"/>
+      <c r="R956" s="76"/>
+      <c r="S956" s="76"/>
+      <c r="T956" s="76"/>
+      <c r="U956" s="76"/>
+      <c r="V956" s="76"/>
+      <c r="W956" s="75"/>
       <c r="X956" s="2"/>
       <c r="Y956" s="2"/>
       <c r="Z956" s="2"/>
@@ -17682,18 +17695,18 @@
       <c r="I957" s="2"/>
       <c r="J957" s="2"/>
       <c r="K957" s="2"/>
-      <c r="L957" s="76"/>
+      <c r="L957" s="75"/>
       <c r="M957" s="2"/>
       <c r="N957" s="2"/>
       <c r="O957" s="2"/>
       <c r="P957" s="2"/>
       <c r="Q957" s="2"/>
-      <c r="R957" s="77"/>
-      <c r="S957" s="77"/>
-      <c r="T957" s="77"/>
-      <c r="U957" s="77"/>
-      <c r="V957" s="77"/>
-      <c r="W957" s="76"/>
+      <c r="R957" s="76"/>
+      <c r="S957" s="76"/>
+      <c r="T957" s="76"/>
+      <c r="U957" s="76"/>
+      <c r="V957" s="76"/>
+      <c r="W957" s="75"/>
       <c r="X957" s="2"/>
       <c r="Y957" s="2"/>
       <c r="Z957" s="2"/>
@@ -17718,18 +17731,18 @@
       <c r="I958" s="2"/>
       <c r="J958" s="2"/>
       <c r="K958" s="2"/>
-      <c r="L958" s="76"/>
+      <c r="L958" s="75"/>
       <c r="M958" s="2"/>
       <c r="N958" s="2"/>
       <c r="O958" s="2"/>
       <c r="P958" s="2"/>
       <c r="Q958" s="2"/>
-      <c r="R958" s="77"/>
-      <c r="S958" s="77"/>
-      <c r="T958" s="77"/>
-      <c r="U958" s="77"/>
-      <c r="V958" s="77"/>
-      <c r="W958" s="76"/>
+      <c r="R958" s="76"/>
+      <c r="S958" s="76"/>
+      <c r="T958" s="76"/>
+      <c r="U958" s="76"/>
+      <c r="V958" s="76"/>
+      <c r="W958" s="75"/>
       <c r="X958" s="2"/>
       <c r="Y958" s="2"/>
       <c r="Z958" s="2"/>
@@ -17754,18 +17767,18 @@
       <c r="I959" s="2"/>
       <c r="J959" s="2"/>
       <c r="K959" s="2"/>
-      <c r="L959" s="76"/>
+      <c r="L959" s="75"/>
       <c r="M959" s="2"/>
       <c r="N959" s="2"/>
       <c r="O959" s="2"/>
       <c r="P959" s="2"/>
       <c r="Q959" s="2"/>
-      <c r="R959" s="77"/>
-      <c r="S959" s="77"/>
-      <c r="T959" s="77"/>
-      <c r="U959" s="77"/>
-      <c r="V959" s="77"/>
-      <c r="W959" s="76"/>
+      <c r="R959" s="76"/>
+      <c r="S959" s="76"/>
+      <c r="T959" s="76"/>
+      <c r="U959" s="76"/>
+      <c r="V959" s="76"/>
+      <c r="W959" s="75"/>
       <c r="X959" s="2"/>
       <c r="Y959" s="2"/>
       <c r="Z959" s="2"/>
@@ -17790,18 +17803,18 @@
       <c r="I960" s="2"/>
       <c r="J960" s="2"/>
       <c r="K960" s="2"/>
-      <c r="L960" s="76"/>
+      <c r="L960" s="75"/>
       <c r="M960" s="2"/>
       <c r="N960" s="2"/>
       <c r="O960" s="2"/>
       <c r="P960" s="2"/>
       <c r="Q960" s="2"/>
-      <c r="R960" s="77"/>
-      <c r="S960" s="77"/>
-      <c r="T960" s="77"/>
-      <c r="U960" s="77"/>
-      <c r="V960" s="77"/>
-      <c r="W960" s="76"/>
+      <c r="R960" s="76"/>
+      <c r="S960" s="76"/>
+      <c r="T960" s="76"/>
+      <c r="U960" s="76"/>
+      <c r="V960" s="76"/>
+      <c r="W960" s="75"/>
       <c r="X960" s="2"/>
       <c r="Y960" s="2"/>
       <c r="Z960" s="2"/>
@@ -17826,18 +17839,18 @@
       <c r="I961" s="2"/>
       <c r="J961" s="2"/>
       <c r="K961" s="2"/>
-      <c r="L961" s="76"/>
+      <c r="L961" s="75"/>
       <c r="M961" s="2"/>
       <c r="N961" s="2"/>
       <c r="O961" s="2"/>
       <c r="P961" s="2"/>
       <c r="Q961" s="2"/>
-      <c r="R961" s="77"/>
-      <c r="S961" s="77"/>
-      <c r="T961" s="77"/>
-      <c r="U961" s="77"/>
-      <c r="V961" s="77"/>
-      <c r="W961" s="76"/>
+      <c r="R961" s="76"/>
+      <c r="S961" s="76"/>
+      <c r="T961" s="76"/>
+      <c r="U961" s="76"/>
+      <c r="V961" s="76"/>
+      <c r="W961" s="75"/>
       <c r="X961" s="2"/>
       <c r="Y961" s="2"/>
       <c r="Z961" s="2"/>
@@ -17862,18 +17875,18 @@
       <c r="I962" s="2"/>
       <c r="J962" s="2"/>
       <c r="K962" s="2"/>
-      <c r="L962" s="76"/>
+      <c r="L962" s="75"/>
       <c r="M962" s="2"/>
       <c r="N962" s="2"/>
       <c r="O962" s="2"/>
       <c r="P962" s="2"/>
       <c r="Q962" s="2"/>
-      <c r="R962" s="77"/>
-      <c r="S962" s="77"/>
-      <c r="T962" s="77"/>
-      <c r="U962" s="77"/>
-      <c r="V962" s="77"/>
-      <c r="W962" s="76"/>
+      <c r="R962" s="76"/>
+      <c r="S962" s="76"/>
+      <c r="T962" s="76"/>
+      <c r="U962" s="76"/>
+      <c r="V962" s="76"/>
+      <c r="W962" s="75"/>
       <c r="X962" s="2"/>
       <c r="Y962" s="2"/>
       <c r="Z962" s="2"/>
@@ -17898,18 +17911,18 @@
       <c r="I963" s="2"/>
       <c r="J963" s="2"/>
       <c r="K963" s="2"/>
-      <c r="L963" s="76"/>
+      <c r="L963" s="75"/>
       <c r="M963" s="2"/>
       <c r="N963" s="2"/>
       <c r="O963" s="2"/>
       <c r="P963" s="2"/>
       <c r="Q963" s="2"/>
-      <c r="R963" s="77"/>
-      <c r="S963" s="77"/>
-      <c r="T963" s="77"/>
-      <c r="U963" s="77"/>
-      <c r="V963" s="77"/>
-      <c r="W963" s="76"/>
+      <c r="R963" s="76"/>
+      <c r="S963" s="76"/>
+      <c r="T963" s="76"/>
+      <c r="U963" s="76"/>
+      <c r="V963" s="76"/>
+      <c r="W963" s="75"/>
       <c r="X963" s="2"/>
       <c r="Y963" s="2"/>
       <c r="Z963" s="2"/>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (04/08/2026 05:11)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/01_Bases_Originais/005_CELOG_2025/005_CELOG-PAMALS_2025 online.xlsx
+++ b/Contrato 005/Dashboard/01_Bases_Originais/005_CELOG_2025/005_CELOG-PAMALS_2025 online.xlsx
@@ -30,12 +30,12 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="331" uniqueCount="209">
   <si>
+    <t>Controle de pagamentos</t>
+  </si>
+  <si>
     <t>Saldo</t>
   </si>
   <si>
-    <t>Controle de pagamentos</t>
-  </si>
-  <si>
     <t>2025NE000005</t>
   </si>
   <si>
@@ -81,13 +81,19 @@
     <t>Ação</t>
   </si>
   <si>
+    <t>2025NE000369</t>
+  </si>
+  <si>
     <t>PAG</t>
   </si>
   <si>
+    <t>C25516</t>
+  </si>
+  <si>
     <t>Moeda</t>
   </si>
   <si>
-    <t>2025NE000369</t>
+    <t>25E0387</t>
   </si>
   <si>
     <t>Valor Total do Contrato</t>
@@ -96,15 +102,9 @@
     <t>Valor a Empenhar</t>
   </si>
   <si>
-    <t>C25516</t>
-  </si>
-  <si>
     <t>Valor Empenhado</t>
   </si>
   <si>
-    <t>25E0387</t>
-  </si>
-  <si>
     <t>Valor Liquidado</t>
   </si>
   <si>
@@ -123,18 +123,21 @@
     <t>Editar</t>
   </si>
   <si>
+    <t>2025NE000371</t>
+  </si>
+  <si>
     <t>005/CELOG-PAMALS/2025</t>
   </si>
   <si>
+    <t>25E0389</t>
+  </si>
+  <si>
     <t>CELOG</t>
   </si>
   <si>
     <t>PAMALS</t>
   </si>
   <si>
-    <t>2025NE000371</t>
-  </si>
-  <si>
     <t>Vigente</t>
   </si>
   <si>
@@ -144,27 +147,24 @@
     <t>67101.001510/2024-12</t>
   </si>
   <si>
-    <t>25E0389</t>
-  </si>
-  <si>
     <t>R$</t>
   </si>
   <si>
+    <t>2025NE000413</t>
+  </si>
+  <si>
+    <t>C25501</t>
+  </si>
+  <si>
+    <t>25E0403</t>
+  </si>
+  <si>
+    <t>20SP</t>
+  </si>
+  <si>
     <t>VEE ONE-MANUTENCAO E SERVICOS TECNICOS LTDA</t>
   </si>
   <si>
-    <t>2025NE000413</t>
-  </si>
-  <si>
-    <t>C25501</t>
-  </si>
-  <si>
-    <t>25E0403</t>
-  </si>
-  <si>
-    <t>20SP</t>
-  </si>
-  <si>
     <t>2025NE000414</t>
   </si>
   <si>
@@ -174,10 +174,19 @@
     <t>25E0431</t>
   </si>
   <si>
+    <t>21EM</t>
+  </si>
+  <si>
     <t>Módulo</t>
   </si>
   <si>
-    <t>21EM</t>
+    <t>2025NE000559</t>
+  </si>
+  <si>
+    <t>C25545</t>
+  </si>
+  <si>
+    <t>25E0524</t>
   </si>
   <si>
     <t>Referência</t>
@@ -186,6 +195,9 @@
     <t>Nº recibo</t>
   </si>
   <si>
+    <t>20X7</t>
+  </si>
+  <si>
     <t>Nº</t>
   </si>
   <si>
@@ -195,16 +207,13 @@
     <t>Empenho</t>
   </si>
   <si>
-    <t>2025NE000559</t>
-  </si>
-  <si>
-    <t>C25545</t>
+    <t>2025NE000770</t>
   </si>
   <si>
     <t>Observações</t>
   </si>
   <si>
-    <t>25E0524</t>
+    <t>25E0731</t>
   </si>
   <si>
     <t>Vencimento</t>
@@ -216,57 +225,48 @@
     <t>Ordem de Pagamento</t>
   </si>
   <si>
-    <t>20X7</t>
-  </si>
-  <si>
     <t>Faturado</t>
   </si>
   <si>
     <t>Pendente</t>
   </si>
   <si>
-    <t>2025NE000770</t>
-  </si>
-  <si>
-    <t>25E0731</t>
+    <t>2025NE000774</t>
+  </si>
+  <si>
+    <t>25E0737</t>
   </si>
   <si>
     <t>FEV/25</t>
   </si>
   <si>
-    <t>2025NE000774</t>
+    <t>2025NE000843</t>
+  </si>
+  <si>
+    <t>C25630</t>
+  </si>
+  <si>
+    <t>25E0787</t>
   </si>
   <si>
     <t>-</t>
   </si>
   <si>
-    <t>25E0737</t>
+    <t>219C</t>
   </si>
   <si>
     <t xml:space="preserve">2025NE000369 </t>
   </si>
   <si>
-    <t>2025NE000843</t>
-  </si>
-  <si>
-    <t>C25630</t>
-  </si>
-  <si>
-    <t>25E0787</t>
-  </si>
-  <si>
-    <t>219C</t>
+    <t>2025NE001065</t>
+  </si>
+  <si>
+    <t>25E0999</t>
   </si>
   <si>
     <t>2025NP001980</t>
   </si>
   <si>
-    <t>2025NE001065</t>
-  </si>
-  <si>
-    <t>25E0999</t>
-  </si>
-  <si>
     <t>2025NE001200</t>
   </si>
   <si>
@@ -276,37 +276,43 @@
     <t>25E1128</t>
   </si>
   <si>
+    <t>2025NE001598</t>
+  </si>
+  <si>
+    <t>C25814</t>
+  </si>
+  <si>
+    <t>25E1446</t>
+  </si>
+  <si>
+    <t>2025NE001627</t>
+  </si>
+  <si>
+    <t>25E1475</t>
+  </si>
+  <si>
     <t>MAR/25</t>
   </si>
   <si>
-    <t>2025NE001598</t>
-  </si>
-  <si>
-    <t>C25814</t>
-  </si>
-  <si>
-    <t>25E1446</t>
-  </si>
-  <si>
     <t>2025NE000367, 2025NE000369, 2025NE000371, 2025NE000413</t>
   </si>
   <si>
-    <t>2025NE001627</t>
-  </si>
-  <si>
-    <t>25E1475</t>
+    <t>2025NE001629</t>
+  </si>
+  <si>
+    <t>C25820</t>
+  </si>
+  <si>
+    <t>25E1477</t>
   </si>
   <si>
     <t>2025NP001979</t>
   </si>
   <si>
-    <t>2025NE001629</t>
-  </si>
-  <si>
-    <t>C25820</t>
-  </si>
-  <si>
-    <t>25E1477</t>
+    <t>2025NE001687</t>
+  </si>
+  <si>
+    <t>25E1535</t>
   </si>
   <si>
     <t>ABR/25</t>
@@ -315,40 +321,46 @@
     <t>2025NE000413, 2025NE000414, 2025NE000559</t>
   </si>
   <si>
-    <t>2025NE001687</t>
-  </si>
-  <si>
-    <t>25E1535</t>
+    <t>2025NE001688</t>
+  </si>
+  <si>
+    <t>25E1536</t>
   </si>
   <si>
     <t>2025NP002341</t>
   </si>
   <si>
+    <t>2025NE001689</t>
+  </si>
+  <si>
+    <t>25E1537</t>
+  </si>
+  <si>
     <t>MAI/25</t>
   </si>
   <si>
-    <t>2025NE001688</t>
-  </si>
-  <si>
-    <t>25E1536</t>
+    <t>2025NE001690</t>
+  </si>
+  <si>
+    <t>25E1538</t>
   </si>
   <si>
     <t>2025NP002884</t>
   </si>
   <si>
-    <t>2025NE001689</t>
-  </si>
-  <si>
-    <t>25E1537</t>
+    <t>2025NE001823</t>
+  </si>
+  <si>
+    <t>C25865</t>
+  </si>
+  <si>
+    <t>25E1666</t>
   </si>
   <si>
     <t>JUN/25</t>
   </si>
   <si>
-    <t>2025NE001690</t>
-  </si>
-  <si>
-    <t>25E1538</t>
+    <t>2025NE001828</t>
   </si>
   <si>
     <t>2025NE000005,
@@ -357,164 +369,152 @@
 2025NE000774</t>
   </si>
   <si>
+    <t>C25869</t>
+  </si>
+  <si>
+    <t>25E1667</t>
+  </si>
+  <si>
+    <t>20YJ</t>
+  </si>
+  <si>
     <t>2025NP400522</t>
   </si>
   <si>
-    <t>2025NE001823</t>
-  </si>
-  <si>
-    <t>C25865</t>
-  </si>
-  <si>
-    <t>25E1666</t>
+    <t>2025NE001830</t>
+  </si>
+  <si>
+    <t>25E1669</t>
   </si>
   <si>
     <t>JUL/25</t>
   </si>
   <si>
-    <t>2025NE001828</t>
-  </si>
-  <si>
     <t>2025NE000843, 2025NE001200</t>
   </si>
   <si>
-    <t>C25869</t>
-  </si>
-  <si>
-    <t>25E1667</t>
-  </si>
-  <si>
-    <t>20YJ</t>
+    <t>2025NE002200</t>
+  </si>
+  <si>
+    <t>C25863</t>
   </si>
   <si>
     <t>2025NP003724</t>
   </si>
   <si>
-    <t>2025NE001830</t>
-  </si>
-  <si>
-    <t>25E1669</t>
+    <t>25E2021</t>
   </si>
   <si>
     <t>AGO/25</t>
   </si>
   <si>
+    <t>2025NE002237</t>
+  </si>
+  <si>
+    <t>25E2058</t>
+  </si>
+  <si>
     <t>2025NP004558</t>
   </si>
   <si>
-    <t>2025NE002200</t>
-  </si>
-  <si>
-    <t>C25863</t>
-  </si>
-  <si>
-    <t>25E2021</t>
+    <t>2026NE000330</t>
+  </si>
+  <si>
+    <t>C26163</t>
+  </si>
+  <si>
+    <t>26E0320</t>
   </si>
   <si>
     <t>SET/25</t>
-  </si>
-  <si>
-    <t>2025NE002237</t>
-  </si>
-  <si>
-    <t>25E2058</t>
   </si>
   <si>
     <t>2025NE001688 
 2025NE001828</t>
   </si>
   <si>
+    <t>2026NE000388</t>
+  </si>
+  <si>
+    <t>C26193</t>
+  </si>
+  <si>
     <t>2025NP004897</t>
   </si>
   <si>
-    <t>2026NE000330</t>
-  </si>
-  <si>
-    <t>C26163</t>
-  </si>
-  <si>
-    <t>26E0320</t>
+    <t>26E0375</t>
   </si>
   <si>
     <t>OUT/25</t>
   </si>
   <si>
+    <t>2026NE000748</t>
+  </si>
+  <si>
+    <t>C26312</t>
+  </si>
+  <si>
+    <t>26E0709</t>
+  </si>
+  <si>
     <t>2025NE001688, 2025NE001828, 2025NE002200</t>
   </si>
   <si>
-    <t>2026NE000388</t>
-  </si>
-  <si>
-    <t>C26193</t>
-  </si>
-  <si>
-    <t>26E0375</t>
-  </si>
-  <si>
     <t>2025NP004932</t>
   </si>
   <si>
-    <t>2026NE000748</t>
-  </si>
-  <si>
-    <t>C26312</t>
-  </si>
-  <si>
-    <t>26E0709</t>
+    <t>2026NE000816</t>
+  </si>
+  <si>
+    <t>C26324</t>
+  </si>
+  <si>
+    <t>26E0776</t>
   </si>
   <si>
     <t>NOV/25</t>
   </si>
   <si>
+    <t>2026NE000817</t>
+  </si>
+  <si>
     <t>2025NE001687, 2025NE001689, 2025NE001690, 2025NE001823, 2025NE001830, 2025NE002237</t>
   </si>
   <si>
+    <t>C26326</t>
+  </si>
+  <si>
+    <t>26E0777</t>
+  </si>
+  <si>
     <t>2026NP400440</t>
   </si>
   <si>
-    <t>2026NE000816</t>
-  </si>
-  <si>
-    <t>C26324</t>
-  </si>
-  <si>
-    <t>26E0776</t>
+    <t>2026NE000842</t>
+  </si>
+  <si>
+    <t>26E0803</t>
   </si>
   <si>
     <t>DEZ/25</t>
   </si>
   <si>
-    <t>2026NE000817</t>
-  </si>
-  <si>
-    <t>C26326</t>
-  </si>
-  <si>
-    <t>26E0777</t>
+    <t>2026NE000944</t>
   </si>
   <si>
     <t>2025NE001065, 2025NE002200</t>
   </si>
   <si>
+    <t>26E0906</t>
+  </si>
+  <si>
     <t>2026NP400412</t>
   </si>
   <si>
-    <t>2026NE000842</t>
-  </si>
-  <si>
-    <t>26E0803</t>
-  </si>
-  <si>
     <t>JAN/26</t>
   </si>
   <si>
-    <t>2026NE000944</t>
-  </si>
-  <si>
     <t>2026NP401035</t>
-  </si>
-  <si>
-    <t>26E0906</t>
   </si>
   <si>
     <t>FEV/26</t>
@@ -715,13 +715,13 @@
       <b/>
       <sz val="10.0"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Century Gothic"/>
     </font>
     <font>
       <b/>
       <sz val="10.0"/>
       <color theme="1"/>
-      <name val="Century Gothic"/>
+      <name val="Arial"/>
     </font>
     <font>
       <sz val="10.0"/>
@@ -866,35 +866,35 @@
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="3" fontId="2" numFmtId="0" xfId="0" applyFill="1" applyFont="1"/>
+    <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyFill="1" applyFont="1"/>
+    <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyFill="1" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
     <xf borderId="0" fillId="5" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
+      <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="11" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="center"/>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="4" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
@@ -931,28 +931,28 @@
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
+    <xf borderId="1" fillId="0" fontId="6" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="7" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="2" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="6" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="7" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -971,7 +971,7 @@
     <xf borderId="1" fillId="5" fontId="9" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="8" fontId="6" numFmtId="168" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="8" fontId="7" numFmtId="168" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="3" fillId="0" fontId="10" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
@@ -993,14 +993,14 @@
     <xf borderId="1" fillId="8" fontId="9" numFmtId="168" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="6" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="170" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="7" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="170" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="1" fillId="9" fontId="9" numFmtId="168" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
@@ -1015,13 +1015,13 @@
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="4" fillId="0" fontId="10" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="1" fillId="0" fontId="6" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="7" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="6" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="7" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="6" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="7" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="5" fontId="9" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
@@ -1030,7 +1030,7 @@
     <xf borderId="1" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="6" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="7" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="5" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -1412,46 +1412,46 @@
       <c r="S1" s="1"/>
       <c r="T1" s="1"/>
       <c r="U1" s="1"/>
-      <c r="V1" s="4"/>
+      <c r="V1" s="3"/>
     </row>
     <row r="2" ht="59.25" customHeight="1">
-      <c r="A2" s="6"/>
-      <c r="B2" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="V2" s="9"/>
-      <c r="W2" s="11"/>
-      <c r="X2" s="11"/>
-      <c r="Y2" s="11"/>
-      <c r="Z2" s="11"/>
-      <c r="AA2" s="11"/>
-      <c r="AB2" s="11"/>
-      <c r="AC2" s="11"/>
-      <c r="AD2" s="11"/>
+      <c r="A2" s="4"/>
+      <c r="B2" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="V2" s="8"/>
+      <c r="W2" s="9"/>
+      <c r="X2" s="9"/>
+      <c r="Y2" s="9"/>
+      <c r="Z2" s="9"/>
+      <c r="AA2" s="9"/>
+      <c r="AB2" s="9"/>
+      <c r="AC2" s="9"/>
+      <c r="AD2" s="9"/>
     </row>
     <row r="3" ht="12.75" customHeight="1">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
-      <c r="E3" s="13"/>
-      <c r="F3" s="13"/>
-      <c r="G3" s="13"/>
-      <c r="H3" s="13"/>
-      <c r="I3" s="13"/>
-      <c r="J3" s="13"/>
-      <c r="K3" s="13"/>
-      <c r="L3" s="13"/>
-      <c r="M3" s="13"/>
-      <c r="N3" s="13"/>
-      <c r="O3" s="13"/>
-      <c r="P3" s="13"/>
-      <c r="Q3" s="13"/>
-      <c r="R3" s="13"/>
-      <c r="S3" s="13"/>
-      <c r="T3" s="13"/>
-      <c r="U3" s="13"/>
-      <c r="V3" s="4"/>
+      <c r="C3" s="12"/>
+      <c r="D3" s="12"/>
+      <c r="E3" s="12"/>
+      <c r="F3" s="12"/>
+      <c r="G3" s="12"/>
+      <c r="H3" s="12"/>
+      <c r="I3" s="12"/>
+      <c r="J3" s="12"/>
+      <c r="K3" s="12"/>
+      <c r="L3" s="12"/>
+      <c r="M3" s="12"/>
+      <c r="N3" s="12"/>
+      <c r="O3" s="12"/>
+      <c r="P3" s="12"/>
+      <c r="Q3" s="12"/>
+      <c r="R3" s="12"/>
+      <c r="S3" s="12"/>
+      <c r="T3" s="12"/>
+      <c r="U3" s="12"/>
+      <c r="V3" s="3"/>
     </row>
     <row r="4" ht="12.75" customHeight="1">
       <c r="A4" s="15"/>
@@ -1481,19 +1481,19 @@
         <v>16</v>
       </c>
       <c r="K4" s="16" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="L4" s="16" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="M4" s="17" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="N4" s="17" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="O4" s="17" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="P4" s="17" t="s">
         <v>25</v>
@@ -1513,23 +1513,23 @@
       <c r="U4" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="V4" s="4"/>
+      <c r="V4" s="3"/>
     </row>
     <row r="5" ht="12.75" customHeight="1">
       <c r="A5" s="15"/>
       <c r="B5" s="15"/>
       <c r="C5" s="18"/>
       <c r="D5" s="19" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E5" s="19" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F5" s="19" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="G5" s="19" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="H5" s="20">
         <v>1564.0</v>
@@ -1538,13 +1538,13 @@
         <v>1564.0</v>
       </c>
       <c r="J5" s="19" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="K5" s="19" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="L5" s="19" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="M5" s="19" t="s">
         <v>39</v>
@@ -1565,15 +1565,15 @@
         <v>1.085943044E7</v>
       </c>
       <c r="S5" s="19" t="s">
-        <v>40</v>
-      </c>
-      <c r="V5" s="4"/>
+        <v>44</v>
+      </c>
+      <c r="V5" s="3"/>
     </row>
     <row r="6" ht="12.75" customHeight="1">
       <c r="A6" s="15"/>
       <c r="B6" s="15"/>
       <c r="L6" s="22"/>
-      <c r="V6" s="4"/>
+      <c r="V6" s="3"/>
     </row>
     <row r="7" ht="12.75" customHeight="1">
       <c r="A7" s="23"/>
@@ -1587,55 +1587,55 @@
       <c r="I7" s="25"/>
       <c r="J7" s="25"/>
       <c r="K7" s="25"/>
-      <c r="L7" s="26"/>
+      <c r="L7" s="27"/>
       <c r="M7" s="25"/>
       <c r="N7" s="25"/>
       <c r="O7" s="25"/>
-      <c r="P7" s="27"/>
-      <c r="V7" s="4"/>
+      <c r="P7" s="28"/>
+      <c r="V7" s="3"/>
     </row>
     <row r="8" ht="12.75" customHeight="1">
       <c r="A8" s="23"/>
       <c r="B8" s="23"/>
-      <c r="C8" s="28" t="s">
-        <v>48</v>
-      </c>
-      <c r="D8" s="28" t="s">
-        <v>50</v>
+      <c r="C8" s="29" t="s">
+        <v>49</v>
+      </c>
+      <c r="D8" s="29" t="s">
+        <v>53</v>
       </c>
       <c r="E8" s="30" t="s">
-        <v>51</v>
-      </c>
-      <c r="F8" s="28" t="s">
-        <v>52</v>
-      </c>
-      <c r="G8" s="28" t="s">
-        <v>53</v>
-      </c>
-      <c r="H8" s="28" t="s">
         <v>54</v>
       </c>
+      <c r="F8" s="29" t="s">
+        <v>56</v>
+      </c>
+      <c r="G8" s="29" t="s">
+        <v>57</v>
+      </c>
+      <c r="H8" s="29" t="s">
+        <v>58</v>
+      </c>
       <c r="I8" s="30" t="s">
-        <v>57</v>
-      </c>
-      <c r="J8" s="28" t="s">
-        <v>59</v>
-      </c>
-      <c r="K8" s="28" t="s">
         <v>60</v>
       </c>
+      <c r="J8" s="29" t="s">
+        <v>62</v>
+      </c>
+      <c r="K8" s="29" t="s">
+        <v>63</v>
+      </c>
       <c r="L8" s="31" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="M8" s="30" t="s">
-        <v>63</v>
-      </c>
-      <c r="N8" s="28" t="s">
-        <v>64</v>
-      </c>
-      <c r="O8" s="28"/>
-      <c r="P8" s="27"/>
-      <c r="V8" s="4"/>
+        <v>65</v>
+      </c>
+      <c r="N8" s="29" t="s">
+        <v>66</v>
+      </c>
+      <c r="O8" s="29"/>
+      <c r="P8" s="28"/>
+      <c r="V8" s="3"/>
     </row>
     <row r="9" ht="19.5" customHeight="1">
       <c r="A9" s="23"/>
@@ -1644,10 +1644,10 @@
         <v>1.0</v>
       </c>
       <c r="D9" s="33" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E9" s="34" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="F9" s="35">
         <v>594.0</v>
@@ -1656,7 +1656,7 @@
         <v>45740.0</v>
       </c>
       <c r="H9" s="35" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="I9" s="36"/>
       <c r="J9" s="36">
@@ -1666,7 +1666,7 @@
         <v>748504.24</v>
       </c>
       <c r="L9" s="35" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="M9" s="39">
         <f t="shared" ref="M9:M10" si="1">K9</f>
@@ -1674,18 +1674,18 @@
       </c>
       <c r="N9" s="40"/>
       <c r="O9" s="25"/>
-      <c r="P9" s="27"/>
-      <c r="V9" s="4"/>
+      <c r="P9" s="28"/>
+      <c r="V9" s="3"/>
     </row>
     <row r="10" ht="51.0" customHeight="1">
       <c r="A10" s="23"/>
       <c r="B10" s="23"/>
       <c r="C10" s="41"/>
       <c r="D10" s="33" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="E10" s="34" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="F10" s="35">
         <v>620.0</v>
@@ -1694,7 +1694,7 @@
         <v>45775.0</v>
       </c>
       <c r="H10" s="35" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="I10" s="36"/>
       <c r="J10" s="36">
@@ -1704,7 +1704,7 @@
         <v>1110378.24</v>
       </c>
       <c r="L10" s="35" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="M10" s="39">
         <f t="shared" si="1"/>
@@ -1712,18 +1712,18 @@
       </c>
       <c r="N10" s="42"/>
       <c r="O10" s="25"/>
-      <c r="P10" s="27"/>
-      <c r="V10" s="4"/>
+      <c r="P10" s="28"/>
+      <c r="V10" s="3"/>
     </row>
     <row r="11" ht="12.75" customHeight="1">
       <c r="A11" s="23"/>
       <c r="B11" s="23"/>
       <c r="C11" s="41"/>
       <c r="D11" s="33" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="E11" s="34" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="F11" s="35">
         <v>634.0</v>
@@ -1732,7 +1732,7 @@
         <v>45799.0</v>
       </c>
       <c r="H11" s="35" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="I11" s="36"/>
       <c r="J11" s="36">
@@ -1742,25 +1742,25 @@
         <v>974557.12</v>
       </c>
       <c r="L11" s="34" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="M11" s="39">
         <v>974557.12</v>
       </c>
       <c r="N11" s="42"/>
       <c r="O11" s="25"/>
-      <c r="P11" s="27"/>
-      <c r="V11" s="4"/>
+      <c r="P11" s="28"/>
+      <c r="V11" s="3"/>
     </row>
     <row r="12" ht="27.75" customHeight="1">
       <c r="A12" s="23"/>
       <c r="B12" s="23"/>
       <c r="C12" s="41"/>
       <c r="D12" s="33" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="E12" s="34" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="F12" s="34">
         <v>660.0</v>
@@ -1769,7 +1769,7 @@
         <v>45856.0</v>
       </c>
       <c r="H12" s="44" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="I12" s="36"/>
       <c r="J12" s="36">
@@ -1779,25 +1779,25 @@
         <v>1402001.34</v>
       </c>
       <c r="L12" s="46" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="M12" s="39">
         <v>1402001.34</v>
       </c>
       <c r="N12" s="47"/>
       <c r="O12" s="25"/>
-      <c r="P12" s="27"/>
-      <c r="V12" s="4"/>
+      <c r="P12" s="28"/>
+      <c r="V12" s="3"/>
     </row>
     <row r="13">
       <c r="A13" s="23"/>
       <c r="B13" s="23"/>
       <c r="C13" s="41"/>
-      <c r="D13" s="48" t="s">
-        <v>104</v>
+      <c r="D13" s="49" t="s">
+        <v>109</v>
       </c>
       <c r="E13" s="34" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="F13" s="35">
         <v>661.0</v>
@@ -1806,7 +1806,7 @@
         <v>45856.0</v>
       </c>
       <c r="H13" s="35" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="I13" s="43"/>
       <c r="J13" s="43">
@@ -1816,25 +1816,25 @@
         <v>1223702.3</v>
       </c>
       <c r="L13" s="34" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="M13" s="39">
         <v>1223702.3</v>
       </c>
       <c r="N13" s="47"/>
       <c r="O13" s="25"/>
-      <c r="P13" s="49"/>
-      <c r="V13" s="4"/>
+      <c r="P13" s="50"/>
+      <c r="V13" s="3"/>
     </row>
     <row r="14">
       <c r="A14" s="23"/>
       <c r="B14" s="23"/>
       <c r="C14" s="41"/>
-      <c r="D14" s="48" t="s">
-        <v>112</v>
+      <c r="D14" s="49" t="s">
+        <v>118</v>
       </c>
       <c r="E14" s="34" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="F14" s="34">
         <v>688.0</v>
@@ -1843,7 +1843,7 @@
         <v>45901.0</v>
       </c>
       <c r="H14" s="34" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="I14" s="43"/>
       <c r="J14" s="43">
@@ -1853,25 +1853,25 @@
         <v>1011677.95</v>
       </c>
       <c r="L14" s="34" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="M14" s="39">
         <v>1011677.95</v>
       </c>
       <c r="N14" s="42"/>
       <c r="O14" s="25"/>
-      <c r="P14" s="27"/>
-      <c r="V14" s="4"/>
+      <c r="P14" s="28"/>
+      <c r="V14" s="3"/>
     </row>
     <row r="15">
       <c r="A15" s="23"/>
       <c r="B15" s="23"/>
       <c r="C15" s="41"/>
-      <c r="D15" s="48" t="s">
-        <v>121</v>
+      <c r="D15" s="49" t="s">
+        <v>124</v>
       </c>
       <c r="E15" s="34" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="F15" s="34">
         <v>696.0</v>
@@ -1890,24 +1890,24 @@
         <v>896744.06</v>
       </c>
       <c r="L15" s="34" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="M15" s="39">
         <v>896744.06</v>
       </c>
       <c r="N15" s="47"/>
       <c r="O15" s="25"/>
-      <c r="V15" s="4"/>
+      <c r="V15" s="3"/>
     </row>
     <row r="16">
       <c r="A16" s="23"/>
       <c r="B16" s="23"/>
       <c r="C16" s="41"/>
-      <c r="D16" s="48" t="s">
-        <v>126</v>
+      <c r="D16" s="49" t="s">
+        <v>131</v>
       </c>
       <c r="E16" s="34" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="F16" s="34">
         <v>704.0</v>
@@ -1916,7 +1916,7 @@
         <v>45957.0</v>
       </c>
       <c r="H16" s="34" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="I16" s="43"/>
       <c r="J16" s="43">
@@ -1926,21 +1926,21 @@
         <v>919329.06</v>
       </c>
       <c r="L16" s="34" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="M16" s="39">
         <v>919329.06</v>
       </c>
       <c r="N16" s="42"/>
       <c r="O16" s="25"/>
-      <c r="V16" s="4"/>
+      <c r="V16" s="3"/>
     </row>
     <row r="17">
       <c r="A17" s="23"/>
       <c r="B17" s="23"/>
       <c r="C17" s="41"/>
-      <c r="D17" s="48" t="s">
-        <v>134</v>
+      <c r="D17" s="49" t="s">
+        <v>137</v>
       </c>
       <c r="E17" s="34"/>
       <c r="F17" s="34">
@@ -1950,7 +1950,7 @@
         <v>45972.0</v>
       </c>
       <c r="H17" s="34" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="I17" s="34"/>
       <c r="J17" s="43">
@@ -1960,24 +1960,24 @@
         <v>1157009.26</v>
       </c>
       <c r="L17" s="34" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="M17" s="39">
         <v>1157009.26</v>
       </c>
       <c r="N17" s="51"/>
       <c r="O17" s="25"/>
-      <c r="V17" s="4"/>
+      <c r="V17" s="3"/>
     </row>
     <row r="18">
       <c r="A18" s="23"/>
       <c r="B18" s="23"/>
       <c r="C18" s="41"/>
-      <c r="D18" s="48" t="s">
-        <v>143</v>
+      <c r="D18" s="49" t="s">
+        <v>146</v>
       </c>
       <c r="E18" s="34" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="F18" s="34">
         <v>728.0</v>
@@ -1986,7 +1986,7 @@
         <v>46008.0</v>
       </c>
       <c r="H18" s="34" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="I18" s="34"/>
       <c r="J18" s="43">
@@ -1996,28 +1996,28 @@
         <v>1214597.952</v>
       </c>
       <c r="L18" s="34" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="M18" s="39">
         <v>1214597.952</v>
       </c>
       <c r="N18" s="51"/>
       <c r="O18" s="25"/>
-      <c r="R18" s="27"/>
-      <c r="S18" s="27"/>
-      <c r="T18" s="27"/>
-      <c r="U18" s="27"/>
+      <c r="R18" s="28"/>
+      <c r="S18" s="28"/>
+      <c r="T18" s="28"/>
+      <c r="U18" s="28"/>
       <c r="V18" s="52"/>
     </row>
     <row r="19">
       <c r="A19" s="23"/>
       <c r="B19" s="23"/>
       <c r="C19" s="41"/>
-      <c r="D19" s="48" t="s">
-        <v>149</v>
+      <c r="D19" s="49" t="s">
+        <v>154</v>
       </c>
       <c r="E19" s="34" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="F19" s="34">
         <v>278.0</v>
@@ -2026,7 +2026,7 @@
         <v>46042.0</v>
       </c>
       <c r="H19" s="34" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="I19" s="43"/>
       <c r="J19" s="43">
@@ -2036,25 +2036,25 @@
         <v>967082.09</v>
       </c>
       <c r="L19" s="34" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="M19" s="39">
         <v>967082.09</v>
       </c>
       <c r="N19" s="51"/>
       <c r="O19" s="25"/>
-      <c r="R19" s="27"/>
-      <c r="S19" s="27"/>
-      <c r="T19" s="27"/>
-      <c r="U19" s="27"/>
+      <c r="R19" s="28"/>
+      <c r="S19" s="28"/>
+      <c r="T19" s="28"/>
+      <c r="U19" s="28"/>
       <c r="V19" s="52"/>
     </row>
     <row r="20">
       <c r="A20" s="23"/>
       <c r="B20" s="23"/>
       <c r="C20" s="41"/>
-      <c r="D20" s="48" t="s">
-        <v>157</v>
+      <c r="D20" s="49" t="s">
+        <v>159</v>
       </c>
       <c r="E20" s="34"/>
       <c r="F20" s="34">
@@ -2064,7 +2064,7 @@
         <v>46078.0</v>
       </c>
       <c r="H20" s="34" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="I20" s="43"/>
       <c r="J20" s="43">
@@ -2074,24 +2074,24 @@
         <v>719561.08</v>
       </c>
       <c r="L20" s="34" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="M20" s="39">
         <v>719561.08</v>
       </c>
       <c r="N20" s="51"/>
       <c r="O20" s="25"/>
-      <c r="R20" s="27"/>
-      <c r="S20" s="27"/>
-      <c r="T20" s="27"/>
-      <c r="U20" s="27"/>
+      <c r="R20" s="28"/>
+      <c r="S20" s="28"/>
+      <c r="T20" s="28"/>
+      <c r="U20" s="28"/>
       <c r="V20" s="52"/>
     </row>
     <row r="21">
       <c r="A21" s="23"/>
       <c r="B21" s="23"/>
       <c r="C21" s="41"/>
-      <c r="D21" s="48" t="s">
+      <c r="D21" s="49" t="s">
         <v>161</v>
       </c>
       <c r="E21" s="34"/>
@@ -2119,17 +2119,17 @@
       </c>
       <c r="N21" s="51"/>
       <c r="O21" s="25"/>
-      <c r="R21" s="27"/>
-      <c r="S21" s="27"/>
-      <c r="T21" s="27"/>
-      <c r="U21" s="27"/>
+      <c r="R21" s="28"/>
+      <c r="S21" s="28"/>
+      <c r="T21" s="28"/>
+      <c r="U21" s="28"/>
       <c r="V21" s="52"/>
     </row>
     <row r="22">
       <c r="A22" s="23"/>
       <c r="B22" s="23"/>
       <c r="C22" s="41"/>
-      <c r="D22" s="48" t="s">
+      <c r="D22" s="49" t="s">
         <v>164</v>
       </c>
       <c r="E22" s="34"/>
@@ -2157,17 +2157,17 @@
       </c>
       <c r="N22" s="51"/>
       <c r="O22" s="25"/>
-      <c r="R22" s="27"/>
-      <c r="S22" s="27"/>
-      <c r="T22" s="27"/>
-      <c r="U22" s="27"/>
+      <c r="R22" s="28"/>
+      <c r="S22" s="28"/>
+      <c r="T22" s="28"/>
+      <c r="U22" s="28"/>
       <c r="V22" s="52"/>
     </row>
     <row r="23">
       <c r="A23" s="23"/>
       <c r="B23" s="23"/>
       <c r="C23" s="41"/>
-      <c r="D23" s="48" t="s">
+      <c r="D23" s="49" t="s">
         <v>168</v>
       </c>
       <c r="E23" s="34"/>
@@ -2195,17 +2195,17 @@
       </c>
       <c r="N23" s="53"/>
       <c r="O23" s="25"/>
-      <c r="R23" s="27"/>
-      <c r="S23" s="27"/>
-      <c r="T23" s="27"/>
-      <c r="U23" s="27"/>
+      <c r="R23" s="28"/>
+      <c r="S23" s="28"/>
+      <c r="T23" s="28"/>
+      <c r="U23" s="28"/>
       <c r="V23" s="52"/>
     </row>
     <row r="24">
       <c r="A24" s="23"/>
       <c r="B24" s="23"/>
       <c r="C24" s="41"/>
-      <c r="D24" s="48" t="s">
+      <c r="D24" s="49" t="s">
         <v>170</v>
       </c>
       <c r="E24" s="34"/>
@@ -2233,17 +2233,17 @@
       </c>
       <c r="N24" s="54"/>
       <c r="O24" s="25"/>
-      <c r="R24" s="27"/>
-      <c r="S24" s="27"/>
-      <c r="T24" s="27"/>
-      <c r="U24" s="27"/>
+      <c r="R24" s="28"/>
+      <c r="S24" s="28"/>
+      <c r="T24" s="28"/>
+      <c r="U24" s="28"/>
       <c r="V24" s="52"/>
     </row>
     <row r="25">
       <c r="A25" s="23"/>
       <c r="B25" s="23"/>
       <c r="C25" s="41"/>
-      <c r="D25" s="48" t="s">
+      <c r="D25" s="49" t="s">
         <v>172</v>
       </c>
       <c r="E25" s="34"/>
@@ -2271,17 +2271,17 @@
       </c>
       <c r="N25" s="54"/>
       <c r="O25" s="25"/>
-      <c r="R25" s="27"/>
-      <c r="S25" s="27"/>
-      <c r="T25" s="27"/>
-      <c r="U25" s="27"/>
+      <c r="R25" s="28"/>
+      <c r="S25" s="28"/>
+      <c r="T25" s="28"/>
+      <c r="U25" s="28"/>
       <c r="V25" s="52"/>
     </row>
     <row r="26">
       <c r="A26" s="23"/>
       <c r="B26" s="23"/>
       <c r="C26" s="55"/>
-      <c r="D26" s="48" t="s">
+      <c r="D26" s="49" t="s">
         <v>174</v>
       </c>
       <c r="E26" s="34"/>
@@ -2309,59 +2309,59 @@
       </c>
       <c r="N26" s="54"/>
       <c r="O26" s="25"/>
-      <c r="R26" s="27"/>
-      <c r="S26" s="27"/>
-      <c r="T26" s="27"/>
-      <c r="U26" s="27"/>
+      <c r="R26" s="28"/>
+      <c r="S26" s="28"/>
+      <c r="T26" s="28"/>
+      <c r="U26" s="28"/>
       <c r="V26" s="52"/>
     </row>
     <row r="27" ht="30.75" customHeight="1">
       <c r="A27" s="23"/>
       <c r="B27" s="23"/>
-      <c r="C27" s="28" t="s">
-        <v>48</v>
-      </c>
-      <c r="D27" s="28" t="s">
-        <v>50</v>
+      <c r="C27" s="29" t="s">
+        <v>49</v>
+      </c>
+      <c r="D27" s="29" t="s">
+        <v>53</v>
       </c>
       <c r="E27" s="30" t="s">
-        <v>51</v>
-      </c>
-      <c r="F27" s="28" t="s">
-        <v>52</v>
-      </c>
-      <c r="G27" s="28"/>
-      <c r="H27" s="28" t="s">
         <v>54</v>
       </c>
-      <c r="I27" s="28"/>
-      <c r="J27" s="28"/>
+      <c r="F27" s="29" t="s">
+        <v>56</v>
+      </c>
+      <c r="G27" s="29"/>
+      <c r="H27" s="29" t="s">
+        <v>58</v>
+      </c>
+      <c r="I27" s="29"/>
+      <c r="J27" s="29"/>
       <c r="K27" s="56" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="L27" s="31" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="M27" s="57" t="s">
-        <v>63</v>
-      </c>
-      <c r="N27" s="28" t="s">
-        <v>64</v>
+        <v>65</v>
+      </c>
+      <c r="N27" s="29" t="s">
+        <v>66</v>
       </c>
       <c r="O27" s="25"/>
-      <c r="P27" s="27"/>
-      <c r="R27" s="27"/>
-      <c r="S27" s="27"/>
-      <c r="T27" s="27"/>
-      <c r="U27" s="27"/>
+      <c r="P27" s="28"/>
+      <c r="R27" s="28"/>
+      <c r="S27" s="28"/>
+      <c r="T27" s="28"/>
+      <c r="U27" s="28"/>
       <c r="V27" s="52"/>
-      <c r="W27" s="27"/>
-      <c r="X27" s="27"/>
-      <c r="Y27" s="27"/>
-      <c r="Z27" s="27"/>
-      <c r="AA27" s="27"/>
-      <c r="AB27" s="27"/>
-      <c r="AC27" s="27"/>
+      <c r="W27" s="28"/>
+      <c r="X27" s="28"/>
+      <c r="Y27" s="28"/>
+      <c r="Z27" s="28"/>
+      <c r="AA27" s="28"/>
+      <c r="AB27" s="28"/>
+      <c r="AC27" s="28"/>
     </row>
     <row r="28" ht="12.75" customHeight="1">
       <c r="A28" s="23"/>
@@ -2380,7 +2380,7 @@
         <v>45791.0</v>
       </c>
       <c r="H28" s="35" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="I28" s="36"/>
       <c r="J28" s="36">
@@ -2397,20 +2397,20 @@
       </c>
       <c r="N28" s="51"/>
       <c r="O28" s="25"/>
-      <c r="P28" s="27"/>
-      <c r="Q28" s="27"/>
-      <c r="R28" s="27"/>
-      <c r="S28" s="27"/>
-      <c r="T28" s="27"/>
-      <c r="U28" s="27"/>
+      <c r="P28" s="28"/>
+      <c r="Q28" s="28"/>
+      <c r="R28" s="28"/>
+      <c r="S28" s="28"/>
+      <c r="T28" s="28"/>
+      <c r="U28" s="28"/>
       <c r="V28" s="52"/>
-      <c r="W28" s="27"/>
-      <c r="X28" s="27"/>
-      <c r="Y28" s="27"/>
-      <c r="Z28" s="27"/>
-      <c r="AA28" s="27"/>
-      <c r="AB28" s="27"/>
-      <c r="AC28" s="27"/>
+      <c r="W28" s="28"/>
+      <c r="X28" s="28"/>
+      <c r="Y28" s="28"/>
+      <c r="Z28" s="28"/>
+      <c r="AA28" s="28"/>
+      <c r="AB28" s="28"/>
+      <c r="AC28" s="28"/>
     </row>
     <row r="29">
       <c r="A29" s="23"/>
@@ -2446,20 +2446,20 @@
       </c>
       <c r="N29" s="51"/>
       <c r="O29" s="25"/>
-      <c r="P29" s="27"/>
-      <c r="Q29" s="27"/>
-      <c r="R29" s="27"/>
-      <c r="S29" s="27"/>
-      <c r="T29" s="27"/>
-      <c r="U29" s="27"/>
+      <c r="P29" s="28"/>
+      <c r="Q29" s="28"/>
+      <c r="R29" s="28"/>
+      <c r="S29" s="28"/>
+      <c r="T29" s="28"/>
+      <c r="U29" s="28"/>
       <c r="V29" s="52"/>
-      <c r="W29" s="27"/>
-      <c r="X29" s="27"/>
-      <c r="Y29" s="27"/>
-      <c r="Z29" s="27"/>
-      <c r="AA29" s="27"/>
-      <c r="AB29" s="27"/>
-      <c r="AC29" s="27"/>
+      <c r="W29" s="28"/>
+      <c r="X29" s="28"/>
+      <c r="Y29" s="28"/>
+      <c r="Z29" s="28"/>
+      <c r="AA29" s="28"/>
+      <c r="AB29" s="28"/>
+      <c r="AC29" s="28"/>
     </row>
     <row r="30" ht="12.75" customHeight="1">
       <c r="A30" s="23"/>
@@ -2478,7 +2478,7 @@
         <v>45853.0</v>
       </c>
       <c r="H30" s="34" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="I30" s="43"/>
       <c r="J30" s="43">
@@ -2496,19 +2496,19 @@
       <c r="N30" s="51"/>
       <c r="O30" s="25"/>
       <c r="P30" s="64"/>
-      <c r="Q30" s="27"/>
-      <c r="R30" s="27"/>
-      <c r="S30" s="27"/>
-      <c r="T30" s="27"/>
-      <c r="U30" s="27"/>
+      <c r="Q30" s="28"/>
+      <c r="R30" s="28"/>
+      <c r="S30" s="28"/>
+      <c r="T30" s="28"/>
+      <c r="U30" s="28"/>
       <c r="V30" s="52"/>
-      <c r="W30" s="27"/>
-      <c r="X30" s="27"/>
-      <c r="Y30" s="27"/>
-      <c r="Z30" s="27"/>
-      <c r="AA30" s="27"/>
-      <c r="AB30" s="27"/>
-      <c r="AC30" s="27"/>
+      <c r="W30" s="28"/>
+      <c r="X30" s="28"/>
+      <c r="Y30" s="28"/>
+      <c r="Z30" s="28"/>
+      <c r="AA30" s="28"/>
+      <c r="AB30" s="28"/>
+      <c r="AC30" s="28"/>
     </row>
     <row r="31" ht="60.0" customHeight="1">
       <c r="A31" s="23"/>
@@ -2527,7 +2527,7 @@
         <v>45910.0</v>
       </c>
       <c r="H31" s="34" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="I31" s="43"/>
       <c r="J31" s="43">
@@ -2545,19 +2545,19 @@
       <c r="N31" s="51"/>
       <c r="O31" s="25"/>
       <c r="P31" s="64"/>
-      <c r="Q31" s="27"/>
-      <c r="R31" s="27"/>
-      <c r="S31" s="27"/>
-      <c r="T31" s="27"/>
-      <c r="U31" s="27"/>
+      <c r="Q31" s="28"/>
+      <c r="R31" s="28"/>
+      <c r="S31" s="28"/>
+      <c r="T31" s="28"/>
+      <c r="U31" s="28"/>
       <c r="V31" s="52"/>
-      <c r="W31" s="27"/>
-      <c r="X31" s="27"/>
-      <c r="Y31" s="27"/>
-      <c r="Z31" s="27"/>
-      <c r="AA31" s="27"/>
-      <c r="AB31" s="27"/>
-      <c r="AC31" s="27"/>
+      <c r="W31" s="28"/>
+      <c r="X31" s="28"/>
+      <c r="Y31" s="28"/>
+      <c r="Z31" s="28"/>
+      <c r="AA31" s="28"/>
+      <c r="AB31" s="28"/>
+      <c r="AC31" s="28"/>
     </row>
     <row r="32" ht="12.75" customHeight="1">
       <c r="A32" s="23"/>
@@ -2576,7 +2576,7 @@
         <v>45904.0</v>
       </c>
       <c r="H32" s="34" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="I32" s="66"/>
       <c r="J32" s="66">
@@ -2594,19 +2594,19 @@
       <c r="N32" s="51"/>
       <c r="O32" s="25"/>
       <c r="P32" s="64"/>
-      <c r="Q32" s="27"/>
-      <c r="R32" s="27"/>
-      <c r="S32" s="27"/>
-      <c r="T32" s="27"/>
-      <c r="U32" s="27"/>
+      <c r="Q32" s="28"/>
+      <c r="R32" s="28"/>
+      <c r="S32" s="28"/>
+      <c r="T32" s="28"/>
+      <c r="U32" s="28"/>
       <c r="V32" s="52"/>
-      <c r="W32" s="27"/>
-      <c r="X32" s="27"/>
-      <c r="Y32" s="27"/>
-      <c r="Z32" s="27"/>
-      <c r="AA32" s="27"/>
-      <c r="AB32" s="27"/>
-      <c r="AC32" s="27"/>
+      <c r="W32" s="28"/>
+      <c r="X32" s="28"/>
+      <c r="Y32" s="28"/>
+      <c r="Z32" s="28"/>
+      <c r="AA32" s="28"/>
+      <c r="AB32" s="28"/>
+      <c r="AC32" s="28"/>
     </row>
     <row r="33" ht="12.75" customHeight="1">
       <c r="A33" s="23"/>
@@ -2625,7 +2625,7 @@
         <v>46008.0</v>
       </c>
       <c r="H33" s="34" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="I33" s="66"/>
       <c r="J33" s="66">
@@ -2643,19 +2643,19 @@
       <c r="N33" s="51"/>
       <c r="O33" s="25"/>
       <c r="P33" s="64"/>
-      <c r="Q33" s="27"/>
-      <c r="R33" s="27"/>
-      <c r="S33" s="27"/>
-      <c r="T33" s="27"/>
-      <c r="U33" s="27"/>
+      <c r="Q33" s="28"/>
+      <c r="R33" s="28"/>
+      <c r="S33" s="28"/>
+      <c r="T33" s="28"/>
+      <c r="U33" s="28"/>
       <c r="V33" s="52"/>
-      <c r="W33" s="27"/>
-      <c r="X33" s="27"/>
-      <c r="Y33" s="27"/>
-      <c r="Z33" s="27"/>
-      <c r="AA33" s="27"/>
-      <c r="AB33" s="27"/>
-      <c r="AC33" s="27"/>
+      <c r="W33" s="28"/>
+      <c r="X33" s="28"/>
+      <c r="Y33" s="28"/>
+      <c r="Z33" s="28"/>
+      <c r="AA33" s="28"/>
+      <c r="AB33" s="28"/>
+      <c r="AC33" s="28"/>
     </row>
     <row r="34" ht="12.75" customHeight="1">
       <c r="A34" s="23"/>
@@ -2674,7 +2674,7 @@
         <v>45930.0</v>
       </c>
       <c r="H34" s="34" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="I34" s="66"/>
       <c r="J34" s="66">
@@ -2692,19 +2692,19 @@
       <c r="N34" s="51"/>
       <c r="O34" s="25"/>
       <c r="P34" s="64"/>
-      <c r="Q34" s="27"/>
-      <c r="R34" s="27"/>
-      <c r="S34" s="27"/>
-      <c r="T34" s="27"/>
-      <c r="U34" s="27"/>
+      <c r="Q34" s="28"/>
+      <c r="R34" s="28"/>
+      <c r="S34" s="28"/>
+      <c r="T34" s="28"/>
+      <c r="U34" s="28"/>
       <c r="V34" s="52"/>
-      <c r="W34" s="27"/>
-      <c r="X34" s="27"/>
-      <c r="Y34" s="27"/>
-      <c r="Z34" s="27"/>
-      <c r="AA34" s="27"/>
-      <c r="AB34" s="27"/>
-      <c r="AC34" s="27"/>
+      <c r="W34" s="28"/>
+      <c r="X34" s="28"/>
+      <c r="Y34" s="28"/>
+      <c r="Z34" s="28"/>
+      <c r="AA34" s="28"/>
+      <c r="AB34" s="28"/>
+      <c r="AC34" s="28"/>
     </row>
     <row r="35" ht="12.75" customHeight="1">
       <c r="A35" s="23"/>
@@ -2723,7 +2723,7 @@
         <v>45968.0</v>
       </c>
       <c r="H35" s="34" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="I35" s="66"/>
       <c r="J35" s="66">
@@ -2741,19 +2741,19 @@
       <c r="N35" s="51"/>
       <c r="O35" s="25"/>
       <c r="P35" s="64"/>
-      <c r="Q35" s="27"/>
-      <c r="R35" s="27"/>
-      <c r="S35" s="27"/>
-      <c r="T35" s="27"/>
-      <c r="U35" s="27"/>
+      <c r="Q35" s="28"/>
+      <c r="R35" s="28"/>
+      <c r="S35" s="28"/>
+      <c r="T35" s="28"/>
+      <c r="U35" s="28"/>
       <c r="V35" s="52"/>
-      <c r="W35" s="27"/>
-      <c r="X35" s="27"/>
-      <c r="Y35" s="27"/>
-      <c r="Z35" s="27"/>
-      <c r="AA35" s="27"/>
-      <c r="AB35" s="27"/>
-      <c r="AC35" s="27"/>
+      <c r="W35" s="28"/>
+      <c r="X35" s="28"/>
+      <c r="Y35" s="28"/>
+      <c r="Z35" s="28"/>
+      <c r="AA35" s="28"/>
+      <c r="AB35" s="28"/>
+      <c r="AC35" s="28"/>
     </row>
     <row r="36" ht="12.75" customHeight="1">
       <c r="A36" s="23"/>
@@ -2772,7 +2772,7 @@
         <v>46043.0</v>
       </c>
       <c r="H36" s="65" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="I36" s="70"/>
       <c r="J36" s="69">
@@ -2789,20 +2789,20 @@
       </c>
       <c r="N36" s="51"/>
       <c r="O36" s="25"/>
-      <c r="P36" s="27"/>
-      <c r="Q36" s="27"/>
-      <c r="R36" s="27"/>
-      <c r="S36" s="27"/>
-      <c r="T36" s="27"/>
-      <c r="U36" s="27"/>
+      <c r="P36" s="28"/>
+      <c r="Q36" s="28"/>
+      <c r="R36" s="28"/>
+      <c r="S36" s="28"/>
+      <c r="T36" s="28"/>
+      <c r="U36" s="28"/>
       <c r="V36" s="52"/>
-      <c r="W36" s="27"/>
-      <c r="X36" s="27"/>
-      <c r="Y36" s="27"/>
-      <c r="Z36" s="27"/>
-      <c r="AA36" s="27"/>
-      <c r="AB36" s="27"/>
-      <c r="AC36" s="27"/>
+      <c r="W36" s="28"/>
+      <c r="X36" s="28"/>
+      <c r="Y36" s="28"/>
+      <c r="Z36" s="28"/>
+      <c r="AA36" s="28"/>
+      <c r="AB36" s="28"/>
+      <c r="AC36" s="28"/>
     </row>
     <row r="37" ht="12.75" customHeight="1">
       <c r="A37" s="23"/>
@@ -2826,20 +2826,20 @@
         <v>15854.78</v>
       </c>
       <c r="O37" s="25"/>
-      <c r="P37" s="27"/>
-      <c r="Q37" s="27"/>
-      <c r="R37" s="27"/>
-      <c r="S37" s="27"/>
-      <c r="T37" s="27"/>
-      <c r="U37" s="27"/>
+      <c r="P37" s="28"/>
+      <c r="Q37" s="28"/>
+      <c r="R37" s="28"/>
+      <c r="S37" s="28"/>
+      <c r="T37" s="28"/>
+      <c r="U37" s="28"/>
       <c r="V37" s="52"/>
-      <c r="W37" s="27"/>
-      <c r="X37" s="27"/>
-      <c r="Y37" s="27"/>
-      <c r="Z37" s="27"/>
-      <c r="AA37" s="27"/>
-      <c r="AB37" s="27"/>
-      <c r="AC37" s="27"/>
+      <c r="W37" s="28"/>
+      <c r="X37" s="28"/>
+      <c r="Y37" s="28"/>
+      <c r="Z37" s="28"/>
+      <c r="AA37" s="28"/>
+      <c r="AB37" s="28"/>
+      <c r="AC37" s="28"/>
     </row>
     <row r="38" ht="12.75" customHeight="1">
       <c r="A38" s="23"/>
@@ -2863,20 +2863,20 @@
         <v>205</v>
       </c>
       <c r="O38" s="25"/>
-      <c r="P38" s="27"/>
-      <c r="Q38" s="27"/>
-      <c r="R38" s="27"/>
-      <c r="S38" s="27"/>
-      <c r="T38" s="27"/>
-      <c r="U38" s="27"/>
+      <c r="P38" s="28"/>
+      <c r="Q38" s="28"/>
+      <c r="R38" s="28"/>
+      <c r="S38" s="28"/>
+      <c r="T38" s="28"/>
+      <c r="U38" s="28"/>
       <c r="V38" s="52"/>
-      <c r="W38" s="27"/>
-      <c r="X38" s="27"/>
-      <c r="Y38" s="27"/>
-      <c r="Z38" s="27"/>
-      <c r="AA38" s="27"/>
-      <c r="AB38" s="27"/>
-      <c r="AC38" s="27"/>
+      <c r="W38" s="28"/>
+      <c r="X38" s="28"/>
+      <c r="Y38" s="28"/>
+      <c r="Z38" s="28"/>
+      <c r="AA38" s="28"/>
+      <c r="AB38" s="28"/>
+      <c r="AC38" s="28"/>
     </row>
     <row r="39" ht="12.75" customHeight="1">
       <c r="A39" s="23"/>
@@ -2895,7 +2895,7 @@
         <v>46104.0</v>
       </c>
       <c r="H39" s="65" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="I39" s="70"/>
       <c r="J39" s="69">
@@ -2912,20 +2912,20 @@
       </c>
       <c r="N39" s="51"/>
       <c r="O39" s="25"/>
-      <c r="P39" s="27"/>
-      <c r="Q39" s="27"/>
-      <c r="R39" s="27"/>
-      <c r="S39" s="27"/>
-      <c r="T39" s="27"/>
-      <c r="U39" s="27"/>
+      <c r="P39" s="28"/>
+      <c r="Q39" s="28"/>
+      <c r="R39" s="28"/>
+      <c r="S39" s="28"/>
+      <c r="T39" s="28"/>
+      <c r="U39" s="28"/>
       <c r="V39" s="52"/>
-      <c r="W39" s="27"/>
-      <c r="X39" s="27"/>
-      <c r="Y39" s="27"/>
-      <c r="Z39" s="27"/>
-      <c r="AA39" s="27"/>
-      <c r="AB39" s="27"/>
-      <c r="AC39" s="27"/>
+      <c r="W39" s="28"/>
+      <c r="X39" s="28"/>
+      <c r="Y39" s="28"/>
+      <c r="Z39" s="28"/>
+      <c r="AA39" s="28"/>
+      <c r="AB39" s="28"/>
+      <c r="AC39" s="28"/>
     </row>
     <row r="40" ht="12.75" customHeight="1">
       <c r="A40" s="15"/>
@@ -2942,7 +2942,7 @@
         <v>46199.0</v>
       </c>
       <c r="H40" s="65" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="I40" s="70"/>
       <c r="J40" s="69">
@@ -2952,13 +2952,13 @@
         <v>58868.35</v>
       </c>
       <c r="L40" s="34" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="M40" s="72">
         <v>58868.35</v>
       </c>
       <c r="N40" s="51"/>
-      <c r="V40" s="4"/>
+      <c r="V40" s="3"/>
     </row>
     <row r="41" ht="12.75" customHeight="1">
       <c r="A41" s="15"/>
@@ -2966,7 +2966,7 @@
       <c r="C41" s="41"/>
       <c r="K41" s="73"/>
       <c r="M41" s="73"/>
-      <c r="V41" s="4"/>
+      <c r="V41" s="3"/>
     </row>
     <row r="42" ht="12.75" customHeight="1">
       <c r="A42" s="15"/>
@@ -2974,31 +2974,31 @@
       <c r="C42" s="41"/>
       <c r="K42" s="73"/>
       <c r="M42" s="73"/>
-      <c r="V42" s="4"/>
+      <c r="V42" s="3"/>
     </row>
     <row r="43" ht="12.75" customHeight="1">
       <c r="A43" s="15"/>
       <c r="B43" s="15"/>
       <c r="C43" s="41"/>
-      <c r="V43" s="4"/>
+      <c r="V43" s="3"/>
     </row>
     <row r="44" ht="12.75" customHeight="1">
       <c r="A44" s="15"/>
       <c r="B44" s="15"/>
       <c r="C44" s="41"/>
-      <c r="V44" s="4"/>
+      <c r="V44" s="3"/>
     </row>
     <row r="45" ht="12.75" customHeight="1">
       <c r="A45" s="15"/>
       <c r="B45" s="15"/>
       <c r="C45" s="41"/>
-      <c r="V45" s="4"/>
+      <c r="V45" s="3"/>
     </row>
     <row r="46" ht="12.75" customHeight="1">
       <c r="A46" s="15"/>
       <c r="B46" s="15"/>
       <c r="C46" s="41"/>
-      <c r="V46" s="4"/>
+      <c r="V46" s="3"/>
     </row>
     <row r="47" ht="12.75" customHeight="1">
       <c r="A47" s="15"/>
@@ -3006,7 +3006,7 @@
       <c r="C47" s="55"/>
       <c r="K47" s="73"/>
       <c r="M47" s="73"/>
-      <c r="V47" s="4"/>
+      <c r="V47" s="3"/>
     </row>
     <row r="48" ht="12.75" customHeight="1">
       <c r="A48" s="15"/>
@@ -3030,7 +3030,7 @@
       <c r="S48" s="74"/>
       <c r="T48" s="74"/>
       <c r="U48" s="74"/>
-      <c r="V48" s="4"/>
+      <c r="V48" s="3"/>
     </row>
     <row r="49" ht="12.75" customHeight="1">
       <c r="A49" s="15"/>
@@ -7911,11 +7911,11 @@
       <c r="AH1" s="2"/>
     </row>
     <row r="2">
-      <c r="A2" s="3">
+      <c r="A2" s="5">
         <v>46212.0</v>
       </c>
-      <c r="L2" s="5" t="s">
-        <v>0</v>
+      <c r="L2" s="7" t="s">
+        <v>1</v>
       </c>
       <c r="AB2" s="2"/>
       <c r="AC2" s="2"/>
@@ -7926,31 +7926,31 @@
       <c r="AH2" s="2"/>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="10">
+      <c r="C3" s="11">
         <v>2.5E32</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="D3" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="12">
+      <c r="E3" s="13">
         <v>45686.0</v>
       </c>
-      <c r="F3" s="8" t="s">
+      <c r="F3" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G3" s="8">
+      <c r="G3" s="10">
         <v>12.0</v>
       </c>
-      <c r="H3" s="8">
+      <c r="H3" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I3" s="8">
+      <c r="I3" s="10">
         <v>2048.0</v>
       </c>
       <c r="J3" s="14">
@@ -7959,7 +7959,7 @@
       <c r="K3" s="14">
         <v>1000.0</v>
       </c>
-      <c r="L3" s="8">
+      <c r="L3" s="10">
         <v>0.0</v>
       </c>
       <c r="AB3" s="2"/>
@@ -7971,31 +7971,31 @@
       <c r="AH3" s="2"/>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="C4" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="D4" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="12">
+      <c r="E4" s="13">
         <v>45762.0</v>
       </c>
-      <c r="F4" s="8" t="s">
+      <c r="F4" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G4" s="8">
+      <c r="G4" s="10">
         <v>12.0</v>
       </c>
-      <c r="H4" s="8">
+      <c r="H4" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I4" s="8">
+      <c r="I4" s="10">
         <v>2048.0</v>
       </c>
       <c r="J4" s="14">
@@ -8004,7 +8004,7 @@
       <c r="K4" s="14">
         <v>52250.04</v>
       </c>
-      <c r="L4" s="8">
+      <c r="L4" s="10">
         <v>0.0</v>
       </c>
       <c r="AB4" s="2"/>
@@ -8016,31 +8016,31 @@
       <c r="AH4" s="2"/>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="B5" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="C5" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="D5" s="8" t="s">
+      <c r="C5" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="D5" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E5" s="12">
+      <c r="E5" s="13">
         <v>45762.0</v>
       </c>
-      <c r="F5" s="8" t="s">
+      <c r="F5" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G5" s="8">
+      <c r="G5" s="10">
         <v>12.0</v>
       </c>
-      <c r="H5" s="8">
+      <c r="H5" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I5" s="8">
+      <c r="I5" s="10">
         <v>2048.0</v>
       </c>
       <c r="J5" s="14">
@@ -8049,7 +8049,7 @@
       <c r="K5" s="14">
         <v>881914.18</v>
       </c>
-      <c r="L5" s="8">
+      <c r="L5" s="10">
         <v>0.0</v>
       </c>
       <c r="AB5" s="2"/>
@@ -8061,31 +8061,31 @@
       <c r="AH5" s="2"/>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="B6" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="C6" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="D6" s="8" t="s">
+      <c r="A6" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="D6" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E6" s="12">
+      <c r="E6" s="13">
         <v>45762.0</v>
       </c>
-      <c r="F6" s="8" t="s">
+      <c r="F6" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G6" s="8">
+      <c r="G6" s="10">
         <v>12.0</v>
       </c>
-      <c r="H6" s="8">
+      <c r="H6" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I6" s="8">
+      <c r="I6" s="10">
         <v>2048.0</v>
       </c>
       <c r="J6" s="14">
@@ -8094,7 +8094,7 @@
       <c r="K6" s="14">
         <v>750000.0</v>
       </c>
-      <c r="L6" s="8">
+      <c r="L6" s="10">
         <v>0.0</v>
       </c>
       <c r="AB6" s="2"/>
@@ -8106,32 +8106,32 @@
       <c r="AH6" s="2"/>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="s">
+      <c r="A7" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="B7" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="C7" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="D7" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="E7" s="13">
+        <v>45763.0</v>
+      </c>
+      <c r="F7" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="G7" s="10">
+        <v>12.0</v>
+      </c>
+      <c r="H7" s="10">
+        <v>339039.0</v>
+      </c>
+      <c r="I7" s="10" t="s">
         <v>43</v>
-      </c>
-      <c r="D7" s="8" t="s">
-        <v>4</v>
-      </c>
-      <c r="E7" s="12">
-        <v>45763.0</v>
-      </c>
-      <c r="F7" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="G7" s="8">
-        <v>12.0</v>
-      </c>
-      <c r="H7" s="8">
-        <v>339039.0</v>
-      </c>
-      <c r="I7" s="8" t="s">
-        <v>44</v>
       </c>
       <c r="J7" s="14">
         <v>949835.78</v>
@@ -8139,7 +8139,7 @@
       <c r="K7" s="14">
         <v>949835.78</v>
       </c>
-      <c r="L7" s="8">
+      <c r="L7" s="10">
         <v>0.0</v>
       </c>
       <c r="AB7" s="2"/>
@@ -8151,32 +8151,32 @@
       <c r="AH7" s="2"/>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="s">
+      <c r="A8" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="B8" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="C8" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="D8" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E8" s="12">
+      <c r="E8" s="13">
         <v>45763.0</v>
       </c>
-      <c r="F8" s="8" t="s">
+      <c r="F8" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G8" s="8">
+      <c r="G8" s="10">
         <v>12.0</v>
       </c>
-      <c r="H8" s="8">
+      <c r="H8" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I8" s="8" t="s">
-        <v>49</v>
+      <c r="I8" s="10" t="s">
+        <v>48</v>
       </c>
       <c r="J8" s="14">
         <v>524584.95</v>
@@ -8184,10 +8184,10 @@
       <c r="K8" s="14">
         <v>524584.95</v>
       </c>
-      <c r="L8" s="8">
+      <c r="L8" s="10">
         <v>0.0</v>
       </c>
-      <c r="O8" s="29"/>
+      <c r="O8" s="26"/>
       <c r="AB8" s="2"/>
       <c r="AC8" s="2"/>
       <c r="AD8" s="2"/>
@@ -8197,32 +8197,32 @@
       <c r="AH8" s="2"/>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="s">
+      <c r="A9" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="C9" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="D9" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="E9" s="13">
+        <v>45792.0</v>
+      </c>
+      <c r="F9" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="G9" s="10">
+        <v>12.0</v>
+      </c>
+      <c r="H9" s="10">
+        <v>339039.0</v>
+      </c>
+      <c r="I9" s="10" t="s">
         <v>55</v>
-      </c>
-      <c r="B9" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="C9" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="D9" s="8" t="s">
-        <v>4</v>
-      </c>
-      <c r="E9" s="12">
-        <v>45792.0</v>
-      </c>
-      <c r="F9" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="G9" s="8">
-        <v>12.0</v>
-      </c>
-      <c r="H9" s="8">
-        <v>339039.0</v>
-      </c>
-      <c r="I9" s="8" t="s">
-        <v>62</v>
       </c>
       <c r="J9" s="14">
         <v>211614.23</v>
@@ -8230,7 +8230,7 @@
       <c r="K9" s="14">
         <v>211614.23</v>
       </c>
-      <c r="L9" s="8">
+      <c r="L9" s="10">
         <v>0.0</v>
       </c>
       <c r="AB9" s="2"/>
@@ -8242,31 +8242,31 @@
       <c r="AH9" s="2"/>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="s">
-        <v>65</v>
-      </c>
-      <c r="B10" s="8" t="s">
+      <c r="A10" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="B10" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="C10" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="D10" s="8" t="s">
+      <c r="C10" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="D10" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E10" s="12">
+      <c r="E10" s="13">
         <v>45825.0</v>
       </c>
-      <c r="F10" s="8" t="s">
+      <c r="F10" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G10" s="8">
+      <c r="G10" s="10">
         <v>12.0</v>
       </c>
-      <c r="H10" s="8">
+      <c r="H10" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I10" s="8">
+      <c r="I10" s="10">
         <v>2048.0</v>
       </c>
       <c r="J10" s="14">
@@ -8287,31 +8287,31 @@
       <c r="AH10" s="2"/>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="s">
+      <c r="A11" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="C11" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="B11" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="C11" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="D11" s="8" t="s">
+      <c r="D11" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E11" s="12">
+      <c r="E11" s="13">
         <v>45825.0</v>
       </c>
-      <c r="F11" s="8" t="s">
+      <c r="F11" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G11" s="8">
+      <c r="G11" s="10">
         <v>12.0</v>
       </c>
-      <c r="H11" s="8">
+      <c r="H11" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I11" s="8">
+      <c r="I11" s="10">
         <v>2048.0</v>
       </c>
       <c r="J11" s="14">
@@ -8320,7 +8320,7 @@
       <c r="K11" s="14">
         <v>618154.38</v>
       </c>
-      <c r="L11" s="8">
+      <c r="L11" s="10">
         <v>0.01</v>
       </c>
       <c r="AB11" s="2"/>
@@ -8332,32 +8332,32 @@
       <c r="AH11" s="2"/>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="s">
+      <c r="A12" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="B12" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="C12" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="B12" s="8" t="s">
-        <v>73</v>
-      </c>
-      <c r="C12" s="8" t="s">
+      <c r="D12" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="E12" s="13">
+        <v>45832.0</v>
+      </c>
+      <c r="F12" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="G12" s="10">
+        <v>12.0</v>
+      </c>
+      <c r="H12" s="10">
+        <v>339039.0</v>
+      </c>
+      <c r="I12" s="10" t="s">
         <v>74</v>
-      </c>
-      <c r="D12" s="8" t="s">
-        <v>4</v>
-      </c>
-      <c r="E12" s="12">
-        <v>45832.0</v>
-      </c>
-      <c r="F12" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="G12" s="8">
-        <v>12.0</v>
-      </c>
-      <c r="H12" s="8">
-        <v>339039.0</v>
-      </c>
-      <c r="I12" s="8" t="s">
-        <v>75</v>
       </c>
       <c r="J12" s="14">
         <v>1600334.09</v>
@@ -8365,7 +8365,7 @@
       <c r="K12" s="14">
         <v>1600334.09</v>
       </c>
-      <c r="L12" s="8">
+      <c r="L12" s="10">
         <v>0.0</v>
       </c>
       <c r="AB12" s="2"/>
@@ -8377,31 +8377,31 @@
       <c r="AH12" s="2"/>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="s">
+      <c r="A13" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="B13" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C13" s="10" t="s">
         <v>77</v>
       </c>
-      <c r="B13" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="C13" s="8" t="s">
-        <v>78</v>
-      </c>
-      <c r="D13" s="8" t="s">
+      <c r="D13" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E13" s="12">
+      <c r="E13" s="13">
         <v>45863.0</v>
       </c>
-      <c r="F13" s="8" t="s">
+      <c r="F13" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G13" s="8">
+      <c r="G13" s="10">
         <v>12.0</v>
       </c>
-      <c r="H13" s="8">
+      <c r="H13" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I13" s="8">
+      <c r="I13" s="10">
         <v>2048.0</v>
       </c>
       <c r="J13" s="14">
@@ -8423,32 +8423,32 @@
       <c r="AH13" s="2"/>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="s">
+      <c r="A14" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="B14" s="8" t="s">
+      <c r="B14" s="10" t="s">
         <v>80</v>
       </c>
-      <c r="C14" s="8" t="s">
+      <c r="C14" s="10" t="s">
         <v>81</v>
       </c>
-      <c r="D14" s="8" t="s">
+      <c r="D14" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E14" s="12">
+      <c r="E14" s="13">
         <v>45887.0</v>
       </c>
-      <c r="F14" s="8" t="s">
+      <c r="F14" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G14" s="8">
+      <c r="G14" s="10">
         <v>12.0</v>
       </c>
-      <c r="H14" s="8">
+      <c r="H14" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I14" s="8" t="s">
-        <v>62</v>
+      <c r="I14" s="10" t="s">
+        <v>55</v>
       </c>
       <c r="J14" s="14">
         <v>968237.39</v>
@@ -8456,7 +8456,7 @@
       <c r="K14" s="14">
         <v>968237.39</v>
       </c>
-      <c r="L14" s="8">
+      <c r="L14" s="10">
         <v>0.0</v>
       </c>
       <c r="AB14" s="2"/>
@@ -8468,32 +8468,32 @@
       <c r="AH14" s="2"/>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="s">
+      <c r="A15" s="10" t="s">
+        <v>82</v>
+      </c>
+      <c r="B15" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="B15" s="8" t="s">
+      <c r="C15" s="10" t="s">
         <v>84</v>
       </c>
-      <c r="C15" s="8" t="s">
-        <v>85</v>
-      </c>
-      <c r="D15" s="8" t="s">
+      <c r="D15" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E15" s="12">
+      <c r="E15" s="13">
         <v>45924.0</v>
       </c>
-      <c r="F15" s="8" t="s">
+      <c r="F15" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G15" s="8">
+      <c r="G15" s="10">
         <v>12.0</v>
       </c>
-      <c r="H15" s="8">
+      <c r="H15" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I15" s="8" t="s">
-        <v>44</v>
+      <c r="I15" s="10" t="s">
+        <v>43</v>
       </c>
       <c r="J15" s="14">
         <v>1011677.95</v>
@@ -8501,7 +8501,7 @@
       <c r="K15" s="14">
         <v>1011677.95</v>
       </c>
-      <c r="L15" s="8">
+      <c r="L15" s="10">
         <v>0.0</v>
       </c>
       <c r="AB15" s="2"/>
@@ -8513,31 +8513,31 @@
       <c r="AH15" s="2"/>
     </row>
     <row r="16">
-      <c r="A16" s="8" t="s">
-        <v>87</v>
-      </c>
-      <c r="B16" s="8" t="s">
+      <c r="A16" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="B16" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="C16" s="8" t="s">
-        <v>88</v>
-      </c>
-      <c r="D16" s="8" t="s">
+      <c r="C16" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="D16" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E16" s="12">
+      <c r="E16" s="13">
         <v>45929.0</v>
       </c>
-      <c r="F16" s="8" t="s">
+      <c r="F16" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G16" s="8">
+      <c r="G16" s="10">
         <v>12.0</v>
       </c>
-      <c r="H16" s="8">
+      <c r="H16" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I16" s="8">
+      <c r="I16" s="10">
         <v>2048.0</v>
       </c>
       <c r="J16" s="14">
@@ -8558,37 +8558,37 @@
       <c r="AH16" s="2"/>
     </row>
     <row r="17">
-      <c r="A17" s="8" t="s">
+      <c r="A17" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="B17" s="10" t="s">
         <v>90</v>
       </c>
-      <c r="B17" s="8" t="s">
+      <c r="C17" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="C17" s="8" t="s">
-        <v>92</v>
-      </c>
-      <c r="D17" s="8" t="s">
+      <c r="D17" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E17" s="12">
+      <c r="E17" s="13">
         <v>45930.0</v>
       </c>
-      <c r="F17" s="8" t="s">
+      <c r="F17" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G17" s="8">
+      <c r="G17" s="10">
         <v>12.0</v>
       </c>
-      <c r="H17" s="8">
+      <c r="H17" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I17" s="8">
+      <c r="I17" s="10">
         <v>2048.0</v>
       </c>
       <c r="J17" s="14">
         <v>34065.36</v>
       </c>
-      <c r="K17" s="8">
+      <c r="K17" s="10">
         <v>0.0</v>
       </c>
       <c r="L17" s="14">
@@ -8603,32 +8603,32 @@
       <c r="AH17" s="2"/>
     </row>
     <row r="18">
-      <c r="A18" s="8" t="s">
-        <v>95</v>
-      </c>
-      <c r="B18" s="8" t="s">
+      <c r="A18" s="10" t="s">
+        <v>93</v>
+      </c>
+      <c r="B18" s="10" t="s">
         <v>80</v>
       </c>
-      <c r="C18" s="8" t="s">
-        <v>96</v>
-      </c>
-      <c r="D18" s="8" t="s">
+      <c r="C18" s="10" t="s">
+        <v>94</v>
+      </c>
+      <c r="D18" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E18" s="12">
+      <c r="E18" s="13">
         <v>45938.0</v>
       </c>
-      <c r="F18" s="8" t="s">
+      <c r="F18" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G18" s="8">
+      <c r="G18" s="10">
         <v>12.0</v>
       </c>
-      <c r="H18" s="8">
+      <c r="H18" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I18" s="8" t="s">
-        <v>62</v>
+      <c r="I18" s="10" t="s">
+        <v>55</v>
       </c>
       <c r="J18" s="14">
         <v>63746.85</v>
@@ -8636,7 +8636,7 @@
       <c r="K18" s="14">
         <v>63746.85</v>
       </c>
-      <c r="L18" s="8">
+      <c r="L18" s="10">
         <v>0.0</v>
       </c>
       <c r="AB18" s="2"/>
@@ -8648,32 +8648,32 @@
       <c r="AH18" s="2"/>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="s">
-        <v>99</v>
-      </c>
-      <c r="B19" s="8" t="s">
-        <v>73</v>
-      </c>
-      <c r="C19" s="8" t="s">
-        <v>100</v>
-      </c>
-      <c r="D19" s="8" t="s">
+      <c r="A19" s="10" t="s">
+        <v>97</v>
+      </c>
+      <c r="B19" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="C19" s="10" t="s">
+        <v>98</v>
+      </c>
+      <c r="D19" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E19" s="12">
+      <c r="E19" s="13">
         <v>45938.0</v>
       </c>
-      <c r="F19" s="8" t="s">
+      <c r="F19" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G19" s="8">
+      <c r="G19" s="10">
         <v>12.0</v>
       </c>
-      <c r="H19" s="8">
+      <c r="H19" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I19" s="8" t="s">
-        <v>75</v>
+      <c r="I19" s="10" t="s">
+        <v>74</v>
       </c>
       <c r="J19" s="14">
         <v>947931.1</v>
@@ -8681,7 +8681,7 @@
       <c r="K19" s="14">
         <v>947931.1</v>
       </c>
-      <c r="L19" s="8">
+      <c r="L19" s="10">
         <v>0.0</v>
       </c>
       <c r="AB19" s="2"/>
@@ -8693,31 +8693,31 @@
       <c r="AH19" s="2"/>
     </row>
     <row r="20">
-      <c r="A20" s="8" t="s">
-        <v>102</v>
-      </c>
-      <c r="B20" s="8" t="s">
+      <c r="A20" s="10" t="s">
+        <v>100</v>
+      </c>
+      <c r="B20" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="C20" s="8" t="s">
-        <v>103</v>
-      </c>
-      <c r="D20" s="8" t="s">
+      <c r="C20" s="10" t="s">
+        <v>101</v>
+      </c>
+      <c r="D20" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E20" s="12">
+      <c r="E20" s="13">
         <v>45938.0</v>
       </c>
-      <c r="F20" s="8" t="s">
+      <c r="F20" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G20" s="8">
+      <c r="G20" s="10">
         <v>12.0</v>
       </c>
-      <c r="H20" s="8">
+      <c r="H20" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I20" s="8">
+      <c r="I20" s="10">
         <v>2048.0</v>
       </c>
       <c r="J20" s="14">
@@ -8726,7 +8726,7 @@
       <c r="K20" s="14">
         <v>259790.57</v>
       </c>
-      <c r="L20" s="8">
+      <c r="L20" s="10">
         <v>0.0</v>
       </c>
       <c r="AB20" s="2"/>
@@ -8738,31 +8738,31 @@
       <c r="AH20" s="2"/>
     </row>
     <row r="21">
-      <c r="A21" s="8" t="s">
-        <v>105</v>
-      </c>
-      <c r="B21" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="C21" s="8" t="s">
-        <v>106</v>
-      </c>
-      <c r="D21" s="8" t="s">
+      <c r="A21" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="B21" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="C21" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="D21" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E21" s="12">
+      <c r="E21" s="13">
         <v>45938.0</v>
       </c>
-      <c r="F21" s="8" t="s">
+      <c r="F21" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G21" s="8">
+      <c r="G21" s="10">
         <v>12.0</v>
       </c>
-      <c r="H21" s="8">
+      <c r="H21" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I21" s="8">
+      <c r="I21" s="10">
         <v>2048.0</v>
       </c>
       <c r="J21" s="14">
@@ -8771,7 +8771,7 @@
       <c r="K21" s="14">
         <v>170479.3</v>
       </c>
-      <c r="L21" s="8">
+      <c r="L21" s="10">
         <v>0.0</v>
       </c>
       <c r="AB21" s="2"/>
@@ -8783,31 +8783,31 @@
       <c r="AH21" s="2"/>
     </row>
     <row r="22">
-      <c r="A22" s="8" t="s">
-        <v>109</v>
-      </c>
-      <c r="B22" s="8" t="s">
-        <v>110</v>
-      </c>
-      <c r="C22" s="8" t="s">
-        <v>111</v>
-      </c>
-      <c r="D22" s="8" t="s">
+      <c r="A22" s="10" t="s">
+        <v>106</v>
+      </c>
+      <c r="B22" s="10" t="s">
+        <v>107</v>
+      </c>
+      <c r="C22" s="10" t="s">
+        <v>108</v>
+      </c>
+      <c r="D22" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E22" s="50">
+      <c r="E22" s="48">
         <v>45953.0</v>
       </c>
-      <c r="F22" s="8" t="s">
+      <c r="F22" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G22" s="8">
+      <c r="G22" s="10">
         <v>12.0</v>
       </c>
-      <c r="H22" s="8">
+      <c r="H22" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I22" s="8">
+      <c r="I22" s="10">
         <v>2000.0</v>
       </c>
       <c r="J22" s="14">
@@ -8828,32 +8828,32 @@
       <c r="AH22" s="2"/>
     </row>
     <row r="23">
-      <c r="A23" s="8" t="s">
+      <c r="A23" s="10" t="s">
+        <v>110</v>
+      </c>
+      <c r="B23" s="10" t="s">
+        <v>112</v>
+      </c>
+      <c r="C23" s="10" t="s">
         <v>113</v>
       </c>
-      <c r="B23" s="8" t="s">
-        <v>115</v>
-      </c>
-      <c r="C23" s="8" t="s">
-        <v>116</v>
-      </c>
-      <c r="D23" s="8" t="s">
+      <c r="D23" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E23" s="50">
+      <c r="E23" s="48">
         <v>45953.0</v>
       </c>
-      <c r="F23" s="8" t="s">
+      <c r="F23" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G23" s="8">
+      <c r="G23" s="10">
         <v>12.0</v>
       </c>
-      <c r="H23" s="8">
+      <c r="H23" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I23" s="8" t="s">
-        <v>117</v>
+      <c r="I23" s="10" t="s">
+        <v>114</v>
       </c>
       <c r="J23" s="14">
         <v>1000001.64</v>
@@ -8861,7 +8861,7 @@
       <c r="K23" s="14">
         <v>1000001.64</v>
       </c>
-      <c r="L23" s="8">
+      <c r="L23" s="10">
         <v>0.0</v>
       </c>
       <c r="AB23" s="2"/>
@@ -8873,31 +8873,31 @@
       <c r="AH23" s="2"/>
     </row>
     <row r="24">
-      <c r="A24" s="8" t="s">
-        <v>119</v>
-      </c>
-      <c r="B24" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="C24" s="8" t="s">
-        <v>120</v>
-      </c>
-      <c r="D24" s="8" t="s">
+      <c r="A24" s="10" t="s">
+        <v>116</v>
+      </c>
+      <c r="B24" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="C24" s="10" t="s">
+        <v>117</v>
+      </c>
+      <c r="D24" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E24" s="50">
+      <c r="E24" s="48">
         <v>45953.0</v>
       </c>
-      <c r="F24" s="8" t="s">
+      <c r="F24" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G24" s="8">
+      <c r="G24" s="10">
         <v>12.0</v>
       </c>
-      <c r="H24" s="8">
+      <c r="H24" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I24" s="8">
+      <c r="I24" s="10">
         <v>2048.0</v>
       </c>
       <c r="J24" s="14">
@@ -8906,7 +8906,7 @@
       <c r="K24" s="14">
         <v>68405.66</v>
       </c>
-      <c r="L24" s="8">
+      <c r="L24" s="10">
         <v>0.0</v>
       </c>
       <c r="AB24" s="2"/>
@@ -8918,32 +8918,32 @@
       <c r="AH24" s="2"/>
     </row>
     <row r="25">
-      <c r="A25" s="8" t="s">
+      <c r="A25" s="10" t="s">
+        <v>120</v>
+      </c>
+      <c r="B25" s="10" t="s">
+        <v>121</v>
+      </c>
+      <c r="C25" s="10" t="s">
         <v>123</v>
       </c>
-      <c r="B25" s="8" t="s">
-        <v>124</v>
-      </c>
-      <c r="C25" s="8" t="s">
-        <v>125</v>
-      </c>
-      <c r="D25" s="8" t="s">
+      <c r="D25" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E25" s="50">
+      <c r="E25" s="48">
         <v>45975.0</v>
       </c>
-      <c r="F25" s="8" t="s">
+      <c r="F25" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G25" s="8">
+      <c r="G25" s="10">
         <v>12.0</v>
       </c>
-      <c r="H25" s="8">
+      <c r="H25" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I25" s="8" t="s">
-        <v>117</v>
+      <c r="I25" s="10" t="s">
+        <v>114</v>
       </c>
       <c r="J25" s="14">
         <v>1157673.06</v>
@@ -8951,7 +8951,7 @@
       <c r="K25" s="14">
         <v>1157673.06</v>
       </c>
-      <c r="L25" s="8">
+      <c r="L25" s="10">
         <v>0.0</v>
       </c>
       <c r="AB25" s="2"/>
@@ -8963,31 +8963,31 @@
       <c r="AH25" s="2"/>
     </row>
     <row r="26">
-      <c r="A26" s="8" t="s">
-        <v>127</v>
-      </c>
-      <c r="B26" s="8" t="s">
+      <c r="A26" s="10" t="s">
+        <v>125</v>
+      </c>
+      <c r="B26" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="C26" s="8" t="s">
-        <v>128</v>
-      </c>
-      <c r="D26" s="8" t="s">
+      <c r="C26" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="D26" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E26" s="50">
+      <c r="E26" s="48">
         <v>45989.0</v>
       </c>
-      <c r="F26" s="8" t="s">
+      <c r="F26" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G26" s="8">
+      <c r="G26" s="10">
         <v>12.0</v>
       </c>
-      <c r="H26" s="8">
+      <c r="H26" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I26" s="8">
+      <c r="I26" s="10">
         <v>2048.0</v>
       </c>
       <c r="J26" s="14">
@@ -8996,7 +8996,7 @@
       <c r="K26" s="14">
         <v>34065.36</v>
       </c>
-      <c r="L26" s="8">
+      <c r="L26" s="10">
         <v>0.0</v>
       </c>
       <c r="AB26" s="2"/>
@@ -9008,31 +9008,31 @@
       <c r="AH26" s="2"/>
     </row>
     <row r="27">
-      <c r="A27" s="8" t="s">
-        <v>131</v>
-      </c>
-      <c r="B27" s="8" t="s">
-        <v>132</v>
-      </c>
-      <c r="C27" s="8" t="s">
-        <v>133</v>
-      </c>
-      <c r="D27" s="8" t="s">
+      <c r="A27" s="10" t="s">
+        <v>128</v>
+      </c>
+      <c r="B27" s="10" t="s">
+        <v>129</v>
+      </c>
+      <c r="C27" s="10" t="s">
+        <v>130</v>
+      </c>
+      <c r="D27" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E27" s="12">
+      <c r="E27" s="13">
         <v>46104.0</v>
       </c>
-      <c r="F27" s="8" t="s">
+      <c r="F27" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G27" s="8">
+      <c r="G27" s="10">
         <v>12.0</v>
       </c>
-      <c r="H27" s="8">
+      <c r="H27" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I27" s="8">
+      <c r="I27" s="10">
         <v>2048.0</v>
       </c>
       <c r="J27" s="14">
@@ -9053,37 +9053,37 @@
       <c r="AH27" s="2"/>
     </row>
     <row r="28">
-      <c r="A28" s="8" t="s">
+      <c r="A28" s="10" t="s">
+        <v>133</v>
+      </c>
+      <c r="B28" s="10" t="s">
+        <v>134</v>
+      </c>
+      <c r="C28" s="10" t="s">
         <v>136</v>
       </c>
-      <c r="B28" s="8" t="s">
-        <v>137</v>
-      </c>
-      <c r="C28" s="8" t="s">
-        <v>138</v>
-      </c>
-      <c r="D28" s="8" t="s">
+      <c r="D28" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E28" s="12">
+      <c r="E28" s="13">
         <v>46120.0</v>
       </c>
-      <c r="F28" s="8" t="s">
+      <c r="F28" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G28" s="8">
+      <c r="G28" s="10">
         <v>12.0</v>
       </c>
-      <c r="H28" s="8">
+      <c r="H28" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I28" s="8" t="s">
-        <v>49</v>
+      <c r="I28" s="10" t="s">
+        <v>48</v>
       </c>
       <c r="J28" s="14">
         <v>1912292.52</v>
       </c>
-      <c r="K28" s="8">
+      <c r="K28" s="10">
         <v>0.0</v>
       </c>
       <c r="L28" s="14">
@@ -9098,37 +9098,37 @@
       <c r="AH28" s="2"/>
     </row>
     <row r="29">
-      <c r="A29" s="8" t="s">
+      <c r="A29" s="10" t="s">
+        <v>138</v>
+      </c>
+      <c r="B29" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="C29" s="10" t="s">
         <v>140</v>
       </c>
-      <c r="B29" s="8" t="s">
-        <v>141</v>
-      </c>
-      <c r="C29" s="8" t="s">
-        <v>142</v>
-      </c>
-      <c r="D29" s="8" t="s">
+      <c r="D29" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E29" s="12">
+      <c r="E29" s="13">
         <v>46196.0</v>
       </c>
-      <c r="F29" s="8" t="s">
+      <c r="F29" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G29" s="8">
+      <c r="G29" s="10">
         <v>12.0</v>
       </c>
-      <c r="H29" s="8">
+      <c r="H29" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I29" s="8">
+      <c r="I29" s="10">
         <v>2048.0</v>
       </c>
       <c r="J29" s="14">
         <v>1496713.48</v>
       </c>
-      <c r="K29" s="8">
+      <c r="K29" s="10">
         <v>0.0</v>
       </c>
       <c r="L29" s="14">
@@ -9143,37 +9143,37 @@
       <c r="AH29" s="2"/>
     </row>
     <row r="30">
-      <c r="A30" s="8" t="s">
-        <v>146</v>
-      </c>
-      <c r="B30" s="8" t="s">
-        <v>147</v>
-      </c>
-      <c r="C30" s="8" t="s">
-        <v>148</v>
-      </c>
-      <c r="D30" s="8" t="s">
+      <c r="A30" s="10" t="s">
+        <v>143</v>
+      </c>
+      <c r="B30" s="10" t="s">
+        <v>144</v>
+      </c>
+      <c r="C30" s="10" t="s">
+        <v>145</v>
+      </c>
+      <c r="D30" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E30" s="12">
+      <c r="E30" s="13">
         <v>46205.0</v>
       </c>
-      <c r="F30" s="8" t="s">
+      <c r="F30" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G30" s="8">
+      <c r="G30" s="10">
         <v>12.0</v>
       </c>
-      <c r="H30" s="8">
+      <c r="H30" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I30" s="8" t="s">
-        <v>44</v>
+      <c r="I30" s="10" t="s">
+        <v>43</v>
       </c>
       <c r="J30" s="14">
         <v>624166.14</v>
       </c>
-      <c r="K30" s="8">
+      <c r="K30" s="10">
         <v>0.0</v>
       </c>
       <c r="L30" s="14">
@@ -9188,37 +9188,37 @@
       <c r="AH30" s="2"/>
     </row>
     <row r="31">
-      <c r="A31" s="8" t="s">
+      <c r="A31" s="10" t="s">
+        <v>147</v>
+      </c>
+      <c r="B31" s="10" t="s">
+        <v>149</v>
+      </c>
+      <c r="C31" s="10" t="s">
         <v>150</v>
       </c>
-      <c r="B31" s="8" t="s">
-        <v>151</v>
-      </c>
-      <c r="C31" s="8" t="s">
-        <v>152</v>
-      </c>
-      <c r="D31" s="8" t="s">
+      <c r="D31" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E31" s="12">
+      <c r="E31" s="13">
         <v>46205.0</v>
       </c>
-      <c r="F31" s="8" t="s">
+      <c r="F31" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G31" s="8">
+      <c r="G31" s="10">
         <v>12.0</v>
       </c>
-      <c r="H31" s="8">
+      <c r="H31" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I31" s="8" t="s">
-        <v>117</v>
+      <c r="I31" s="10" t="s">
+        <v>114</v>
       </c>
       <c r="J31" s="14">
         <v>18462.36</v>
       </c>
-      <c r="K31" s="8">
+      <c r="K31" s="10">
         <v>0.0</v>
       </c>
       <c r="L31" s="14">
@@ -9233,37 +9233,37 @@
       <c r="AH31" s="2"/>
     </row>
     <row r="32">
-      <c r="A32" s="8" t="s">
-        <v>155</v>
-      </c>
-      <c r="B32" s="8" t="s">
-        <v>151</v>
+      <c r="A32" s="10" t="s">
+        <v>152</v>
+      </c>
+      <c r="B32" s="10" t="s">
+        <v>149</v>
       </c>
       <c r="C32" s="14" t="s">
-        <v>156</v>
-      </c>
-      <c r="D32" s="8" t="s">
+        <v>153</v>
+      </c>
+      <c r="D32" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E32" s="12">
+      <c r="E32" s="13">
         <v>46213.0</v>
       </c>
-      <c r="F32" s="8" t="s">
+      <c r="F32" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G32" s="8">
+      <c r="G32" s="10">
         <v>12.0</v>
       </c>
-      <c r="H32" s="8">
+      <c r="H32" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I32" s="8" t="s">
-        <v>117</v>
+      <c r="I32" s="10" t="s">
+        <v>114</v>
       </c>
       <c r="J32" s="14">
         <v>1530656.62</v>
       </c>
-      <c r="K32" s="8">
+      <c r="K32" s="10">
         <v>0.0</v>
       </c>
       <c r="L32" s="14">
@@ -9278,37 +9278,37 @@
       <c r="AH32" s="2"/>
     </row>
     <row r="33">
-      <c r="A33" s="8" t="s">
-        <v>158</v>
-      </c>
-      <c r="B33" s="8" t="s">
-        <v>141</v>
+      <c r="A33" s="10" t="s">
+        <v>155</v>
+      </c>
+      <c r="B33" s="10" t="s">
+        <v>139</v>
       </c>
       <c r="C33" s="14" t="s">
-        <v>160</v>
-      </c>
-      <c r="D33" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="D33" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E33" s="12">
+      <c r="E33" s="13">
         <v>46227.0</v>
       </c>
-      <c r="F33" s="8" t="s">
+      <c r="F33" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G33" s="8">
+      <c r="G33" s="10">
         <v>12.0</v>
       </c>
-      <c r="H33" s="8">
+      <c r="H33" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I33" s="8">
+      <c r="I33" s="10">
         <v>2048.0</v>
       </c>
       <c r="J33" s="14">
         <v>173846.38</v>
       </c>
-      <c r="K33" s="8">
+      <c r="K33" s="10">
         <v>0.0</v>
       </c>
       <c r="L33" s="14">

</xml_diff>

<commit_message>
Atualização automática: pagamentos (04/08/2026 14:16)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/01_Bases_Originais/005_CELOG_2025/005_CELOG-PAMALS_2025 online.xlsx
+++ b/Contrato 005/Dashboard/01_Bases_Originais/005_CELOG_2025/005_CELOG-PAMALS_2025 online.xlsx
@@ -81,33 +81,33 @@
     <t>Ação</t>
   </si>
   <si>
+    <t>PAG</t>
+  </si>
+  <si>
+    <t>Moeda</t>
+  </si>
+  <si>
+    <t>Valor Total do Contrato</t>
+  </si>
+  <si>
+    <t>Valor a Empenhar</t>
+  </si>
+  <si>
     <t>2025NE000369</t>
   </si>
   <si>
-    <t>PAG</t>
+    <t>Valor Empenhado</t>
   </si>
   <si>
     <t>C25516</t>
   </si>
   <si>
-    <t>Moeda</t>
+    <t>Valor Liquidado</t>
   </si>
   <si>
     <t>25E0387</t>
   </si>
   <si>
-    <t>Valor Total do Contrato</t>
-  </si>
-  <si>
-    <t>Valor a Empenhar</t>
-  </si>
-  <si>
-    <t>Valor Empenhado</t>
-  </si>
-  <si>
-    <t>Valor Liquidado</t>
-  </si>
-  <si>
     <t>Saldo (Valor a Faturar)</t>
   </si>
   <si>
@@ -123,21 +123,21 @@
     <t>Editar</t>
   </si>
   <si>
+    <t>005/CELOG-PAMALS/2025</t>
+  </si>
+  <si>
+    <t>CELOG</t>
+  </si>
+  <si>
+    <t>PAMALS</t>
+  </si>
+  <si>
     <t>2025NE000371</t>
   </si>
   <si>
-    <t>005/CELOG-PAMALS/2025</t>
-  </si>
-  <si>
     <t>25E0389</t>
   </si>
   <si>
-    <t>CELOG</t>
-  </si>
-  <si>
-    <t>PAMALS</t>
-  </si>
-  <si>
     <t>Vigente</t>
   </si>
   <si>
@@ -150,6 +150,9 @@
     <t>R$</t>
   </si>
   <si>
+    <t>VEE ONE-MANUTENCAO E SERVICOS TECNICOS LTDA</t>
+  </si>
+  <si>
     <t>2025NE000413</t>
   </si>
   <si>
@@ -162,9 +165,6 @@
     <t>20SP</t>
   </si>
   <si>
-    <t>VEE ONE-MANUTENCAO E SERVICOS TECNICOS LTDA</t>
-  </si>
-  <si>
     <t>2025NE000414</t>
   </si>
   <si>
@@ -180,55 +180,61 @@
     <t>Módulo</t>
   </si>
   <si>
+    <t>Referência</t>
+  </si>
+  <si>
+    <t>Nº recibo</t>
+  </si>
+  <si>
+    <t>Nº</t>
+  </si>
+  <si>
+    <t>Data</t>
+  </si>
+  <si>
     <t>2025NE000559</t>
   </si>
   <si>
     <t>C25545</t>
   </si>
   <si>
+    <t>Empenho</t>
+  </si>
+  <si>
     <t>25E0524</t>
   </si>
   <si>
-    <t>Referência</t>
-  </si>
-  <si>
-    <t>Nº recibo</t>
+    <t>Observações</t>
+  </si>
+  <si>
+    <t>Vencimento</t>
+  </si>
+  <si>
+    <t>Valor das Nfs</t>
   </si>
   <si>
     <t>20X7</t>
   </si>
   <si>
-    <t>Nº</t>
-  </si>
-  <si>
-    <t>Data</t>
-  </si>
-  <si>
-    <t>Empenho</t>
+    <t>Ordem de Pagamento</t>
+  </si>
+  <si>
+    <t>Faturado</t>
+  </si>
+  <si>
+    <t>Pendente</t>
   </si>
   <si>
     <t>2025NE000770</t>
   </si>
   <si>
-    <t>Observações</t>
-  </si>
-  <si>
     <t>25E0731</t>
   </si>
   <si>
-    <t>Vencimento</t>
-  </si>
-  <si>
-    <t>Valor das Nfs</t>
-  </si>
-  <si>
-    <t>Ordem de Pagamento</t>
-  </si>
-  <si>
-    <t>Faturado</t>
-  </si>
-  <si>
-    <t>Pendente</t>
+    <t>FEV/25</t>
+  </si>
+  <si>
+    <t>-</t>
   </si>
   <si>
     <t>2025NE000774</t>
@@ -237,7 +243,10 @@
     <t>25E0737</t>
   </si>
   <si>
-    <t>FEV/25</t>
+    <t xml:space="preserve">2025NE000369 </t>
+  </si>
+  <si>
+    <t>2025NP001980</t>
   </si>
   <si>
     <t>2025NE000843</t>
@@ -249,22 +258,22 @@
     <t>25E0787</t>
   </si>
   <si>
-    <t>-</t>
-  </si>
-  <si>
     <t>219C</t>
   </si>
   <si>
-    <t xml:space="preserve">2025NE000369 </t>
-  </si>
-  <si>
     <t>2025NE001065</t>
   </si>
   <si>
     <t>25E0999</t>
   </si>
   <si>
-    <t>2025NP001980</t>
+    <t>MAR/25</t>
+  </si>
+  <si>
+    <t>2025NE000367, 2025NE000369, 2025NE000371, 2025NE000413</t>
+  </si>
+  <si>
+    <t>2025NP001979</t>
   </si>
   <si>
     <t>2025NE001200</t>
@@ -279,22 +288,28 @@
     <t>2025NE001598</t>
   </si>
   <si>
+    <t>ABR/25</t>
+  </si>
+  <si>
     <t>C25814</t>
   </si>
   <si>
     <t>25E1446</t>
   </si>
   <si>
+    <t>2025NE000413, 2025NE000414, 2025NE000559</t>
+  </si>
+  <si>
+    <t>2025NP002341</t>
+  </si>
+  <si>
     <t>2025NE001627</t>
   </si>
   <si>
     <t>25E1475</t>
   </si>
   <si>
-    <t>MAR/25</t>
-  </si>
-  <si>
-    <t>2025NE000367, 2025NE000369, 2025NE000371, 2025NE000413</t>
+    <t>MAI/25</t>
   </si>
   <si>
     <t>2025NE001629</t>
@@ -306,61 +321,16 @@
     <t>25E1477</t>
   </si>
   <si>
-    <t>2025NP001979</t>
+    <t>2025NP002884</t>
   </si>
   <si>
     <t>2025NE001687</t>
   </si>
   <si>
+    <t>JUN/25</t>
+  </si>
+  <si>
     <t>25E1535</t>
-  </si>
-  <si>
-    <t>ABR/25</t>
-  </si>
-  <si>
-    <t>2025NE000413, 2025NE000414, 2025NE000559</t>
-  </si>
-  <si>
-    <t>2025NE001688</t>
-  </si>
-  <si>
-    <t>25E1536</t>
-  </si>
-  <si>
-    <t>2025NP002341</t>
-  </si>
-  <si>
-    <t>2025NE001689</t>
-  </si>
-  <si>
-    <t>25E1537</t>
-  </si>
-  <si>
-    <t>MAI/25</t>
-  </si>
-  <si>
-    <t>2025NE001690</t>
-  </si>
-  <si>
-    <t>25E1538</t>
-  </si>
-  <si>
-    <t>2025NP002884</t>
-  </si>
-  <si>
-    <t>2025NE001823</t>
-  </si>
-  <si>
-    <t>C25865</t>
-  </si>
-  <si>
-    <t>25E1666</t>
-  </si>
-  <si>
-    <t>JUN/25</t>
-  </si>
-  <si>
-    <t>2025NE001828</t>
   </si>
   <si>
     <t>2025NE000005,
@@ -369,22 +339,13 @@
 2025NE000774</t>
   </si>
   <si>
-    <t>C25869</t>
-  </si>
-  <si>
-    <t>25E1667</t>
-  </si>
-  <si>
-    <t>20YJ</t>
-  </si>
-  <si>
     <t>2025NP400522</t>
   </si>
   <si>
-    <t>2025NE001830</t>
-  </si>
-  <si>
-    <t>25E1669</t>
+    <t>2025NE001688</t>
+  </si>
+  <si>
+    <t>25E1536</t>
   </si>
   <si>
     <t>JUL/25</t>
@@ -393,59 +354,125 @@
     <t>2025NE000843, 2025NE001200</t>
   </si>
   <si>
-    <t>2025NE002200</t>
-  </si>
-  <si>
-    <t>C25863</t>
+    <t>2025NE001689</t>
   </si>
   <si>
     <t>2025NP003724</t>
   </si>
   <si>
-    <t>25E2021</t>
+    <t>25E1537</t>
   </si>
   <si>
     <t>AGO/25</t>
   </si>
   <si>
-    <t>2025NE002237</t>
-  </si>
-  <si>
-    <t>25E2058</t>
+    <t>2025NE001690</t>
+  </si>
+  <si>
+    <t>25E1538</t>
   </si>
   <si>
     <t>2025NP004558</t>
   </si>
   <si>
-    <t>2026NE000330</t>
-  </si>
-  <si>
-    <t>C26163</t>
-  </si>
-  <si>
-    <t>26E0320</t>
-  </si>
-  <si>
     <t>SET/25</t>
+  </si>
+  <si>
+    <t>2025NE001823</t>
+  </si>
+  <si>
+    <t>C25865</t>
+  </si>
+  <si>
+    <t>25E1666</t>
   </si>
   <si>
     <t>2025NE001688 
 2025NE001828</t>
   </si>
   <si>
+    <t>2025NP004897</t>
+  </si>
+  <si>
+    <t>2025NE001828</t>
+  </si>
+  <si>
+    <t>C25869</t>
+  </si>
+  <si>
+    <t>25E1667</t>
+  </si>
+  <si>
+    <t>OUT/25</t>
+  </si>
+  <si>
+    <t>20YJ</t>
+  </si>
+  <si>
+    <t>2025NE001688, 2025NE001828, 2025NE002200</t>
+  </si>
+  <si>
+    <t>2025NE001830</t>
+  </si>
+  <si>
+    <t>2025NP004932</t>
+  </si>
+  <si>
+    <t>25E1669</t>
+  </si>
+  <si>
+    <t>2025NE002200</t>
+  </si>
+  <si>
+    <t>C25863</t>
+  </si>
+  <si>
+    <t>25E2021</t>
+  </si>
+  <si>
+    <t>NOV/25</t>
+  </si>
+  <si>
+    <t>2025NE001687, 2025NE001689, 2025NE001690, 2025NE001823, 2025NE001830, 2025NE002237</t>
+  </si>
+  <si>
+    <t>2025NE002237</t>
+  </si>
+  <si>
+    <t>25E2058</t>
+  </si>
+  <si>
+    <t>2026NP400440</t>
+  </si>
+  <si>
+    <t>2026NE000330</t>
+  </si>
+  <si>
+    <t>C26163</t>
+  </si>
+  <si>
+    <t>26E0320</t>
+  </si>
+  <si>
+    <t>DEZ/25</t>
+  </si>
+  <si>
+    <t>2025NE001065, 2025NE002200</t>
+  </si>
+  <si>
+    <t>2026NP400412</t>
+  </si>
+  <si>
     <t>2026NE000388</t>
   </si>
   <si>
     <t>C26193</t>
   </si>
   <si>
-    <t>2025NP004897</t>
-  </si>
-  <si>
     <t>26E0375</t>
   </si>
   <si>
-    <t>OUT/25</t>
+    <t>JAN/26</t>
   </si>
   <si>
     <t>2026NE000748</t>
@@ -457,10 +484,7 @@
     <t>26E0709</t>
   </si>
   <si>
-    <t>2025NE001688, 2025NE001828, 2025NE002200</t>
-  </si>
-  <si>
-    <t>2025NP004932</t>
+    <t>2026NP401035</t>
   </si>
   <si>
     <t>2026NE000816</t>
@@ -472,22 +496,25 @@
     <t>26E0776</t>
   </si>
   <si>
-    <t>NOV/25</t>
+    <t>FEV/26</t>
+  </si>
+  <si>
+    <t>2025NE001627, 2025NE001629, 2025NE001823</t>
   </si>
   <si>
     <t>2026NE000817</t>
   </si>
   <si>
-    <t>2025NE001687, 2025NE001689, 2025NE001690, 2025NE001823, 2025NE001830, 2025NE002237</t>
-  </si>
-  <si>
     <t>C26326</t>
   </si>
   <si>
     <t>26E0777</t>
   </si>
   <si>
-    <t>2026NP400440</t>
+    <t>2026NP402272</t>
+  </si>
+  <si>
+    <t>MAR/26</t>
   </si>
   <si>
     <t>2026NE000842</t>
@@ -496,46 +523,19 @@
     <t>26E0803</t>
   </si>
   <si>
-    <t>DEZ/25</t>
+    <t>2025NE000770, 2025NE001627</t>
+  </si>
+  <si>
+    <t>R$ 1.350.542,52</t>
+  </si>
+  <si>
+    <t>2026NP401762</t>
   </si>
   <si>
     <t>2026NE000944</t>
   </si>
   <si>
-    <t>2025NE001065, 2025NE002200</t>
-  </si>
-  <si>
     <t>26E0906</t>
-  </si>
-  <si>
-    <t>2026NP400412</t>
-  </si>
-  <si>
-    <t>JAN/26</t>
-  </si>
-  <si>
-    <t>2026NP401035</t>
-  </si>
-  <si>
-    <t>FEV/26</t>
-  </si>
-  <si>
-    <t>2025NE001627, 2025NE001629, 2025NE001823</t>
-  </si>
-  <si>
-    <t>2026NP402272</t>
-  </si>
-  <si>
-    <t>MAR/26</t>
-  </si>
-  <si>
-    <t>2025NE000770, 2025NE001627</t>
-  </si>
-  <si>
-    <t>R$ 1.350.542,52</t>
-  </si>
-  <si>
-    <t>2026NP401762</t>
   </si>
   <si>
     <t>ABR/26</t>
@@ -715,13 +715,13 @@
       <b/>
       <sz val="10.0"/>
       <color theme="1"/>
-      <name val="Century Gothic"/>
+      <name val="Arial"/>
     </font>
     <font>
       <b/>
       <sz val="10.0"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Century Gothic"/>
     </font>
     <font>
       <sz val="10.0"/>
@@ -931,28 +931,28 @@
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="6" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="0" fontId="7" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="2" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="7" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="6" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -967,14 +967,14 @@
     <xf borderId="1" fillId="7" fontId="9" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="165" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="1" fillId="5" fontId="9" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="8" fontId="7" numFmtId="168" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="8" fontId="6" numFmtId="168" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="3" fillId="0" fontId="10" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="165" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="1" fillId="8" fontId="9" numFmtId="168" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
@@ -993,14 +993,14 @@
     <xf borderId="1" fillId="8" fontId="9" numFmtId="168" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="170" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="7" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="6" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="170" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="1" fillId="9" fontId="9" numFmtId="168" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
@@ -1015,13 +1015,13 @@
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="4" fillId="0" fontId="10" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="1" fillId="0" fontId="7" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="6" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="7" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="6" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="7" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="6" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="5" fontId="9" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
@@ -1030,7 +1030,7 @@
     <xf borderId="1" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="7" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="6" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="5" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -1481,22 +1481,22 @@
         <v>16</v>
       </c>
       <c r="K4" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="L4" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="L4" s="16" t="s">
+      <c r="M4" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="N4" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="M4" s="17" t="s">
+      <c r="O4" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="N4" s="17" t="s">
-        <v>23</v>
-      </c>
-      <c r="O4" s="17" t="s">
+      <c r="P4" s="17" t="s">
         <v>24</v>
-      </c>
-      <c r="P4" s="17" t="s">
-        <v>25</v>
       </c>
       <c r="Q4" s="17" t="s">
         <v>26</v>
@@ -1520,16 +1520,16 @@
       <c r="B5" s="15"/>
       <c r="C5" s="18"/>
       <c r="D5" s="19" t="s">
+        <v>31</v>
+      </c>
+      <c r="E5" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="E5" s="19" t="s">
-        <v>34</v>
-      </c>
       <c r="F5" s="19" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="G5" s="19" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="H5" s="20">
         <v>1564.0</v>
@@ -1565,7 +1565,7 @@
         <v>1.085943044E7</v>
       </c>
       <c r="S5" s="19" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="V5" s="3"/>
     </row>
@@ -1587,54 +1587,54 @@
       <c r="I7" s="25"/>
       <c r="J7" s="25"/>
       <c r="K7" s="25"/>
-      <c r="L7" s="27"/>
+      <c r="L7" s="26"/>
       <c r="M7" s="25"/>
       <c r="N7" s="25"/>
       <c r="O7" s="25"/>
-      <c r="P7" s="28"/>
+      <c r="P7" s="27"/>
       <c r="V7" s="3"/>
     </row>
     <row r="8" ht="12.75" customHeight="1">
       <c r="A8" s="23"/>
       <c r="B8" s="23"/>
-      <c r="C8" s="29" t="s">
+      <c r="C8" s="28" t="s">
         <v>49</v>
       </c>
-      <c r="D8" s="29" t="s">
+      <c r="D8" s="28" t="s">
+        <v>50</v>
+      </c>
+      <c r="E8" s="30" t="s">
+        <v>51</v>
+      </c>
+      <c r="F8" s="28" t="s">
+        <v>52</v>
+      </c>
+      <c r="G8" s="28" t="s">
         <v>53</v>
       </c>
-      <c r="E8" s="30" t="s">
-        <v>54</v>
-      </c>
-      <c r="F8" s="29" t="s">
+      <c r="H8" s="28" t="s">
         <v>56</v>
       </c>
-      <c r="G8" s="29" t="s">
-        <v>57</v>
-      </c>
-      <c r="H8" s="29" t="s">
+      <c r="I8" s="30" t="s">
         <v>58</v>
       </c>
-      <c r="I8" s="30" t="s">
+      <c r="J8" s="28" t="s">
+        <v>59</v>
+      </c>
+      <c r="K8" s="28" t="s">
         <v>60</v>
       </c>
-      <c r="J8" s="29" t="s">
+      <c r="L8" s="31" t="s">
         <v>62</v>
       </c>
-      <c r="K8" s="29" t="s">
+      <c r="M8" s="30" t="s">
         <v>63</v>
       </c>
-      <c r="L8" s="31" t="s">
+      <c r="N8" s="28" t="s">
         <v>64</v>
       </c>
-      <c r="M8" s="30" t="s">
-        <v>65</v>
-      </c>
-      <c r="N8" s="29" t="s">
-        <v>66</v>
-      </c>
-      <c r="O8" s="29"/>
-      <c r="P8" s="28"/>
+      <c r="O8" s="28"/>
+      <c r="P8" s="27"/>
       <c r="V8" s="3"/>
     </row>
     <row r="9" ht="19.5" customHeight="1">
@@ -1644,10 +1644,10 @@
         <v>1.0</v>
       </c>
       <c r="D9" s="33" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="E9" s="34" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="F9" s="35">
         <v>594.0</v>
@@ -1656,7 +1656,7 @@
         <v>45740.0</v>
       </c>
       <c r="H9" s="35" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="I9" s="36"/>
       <c r="J9" s="36">
@@ -1666,26 +1666,26 @@
         <v>748504.24</v>
       </c>
       <c r="L9" s="35" t="s">
-        <v>78</v>
-      </c>
-      <c r="M9" s="39">
+        <v>72</v>
+      </c>
+      <c r="M9" s="38">
         <f t="shared" ref="M9:M10" si="1">K9</f>
         <v>748504.24</v>
       </c>
-      <c r="N9" s="40"/>
+      <c r="N9" s="39"/>
       <c r="O9" s="25"/>
-      <c r="P9" s="28"/>
+      <c r="P9" s="27"/>
       <c r="V9" s="3"/>
     </row>
     <row r="10" ht="51.0" customHeight="1">
       <c r="A10" s="23"/>
       <c r="B10" s="23"/>
-      <c r="C10" s="41"/>
+      <c r="C10" s="40"/>
       <c r="D10" s="33" t="s">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="E10" s="34" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="F10" s="35">
         <v>620.0</v>
@@ -1694,7 +1694,7 @@
         <v>45775.0</v>
       </c>
       <c r="H10" s="35" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="I10" s="36"/>
       <c r="J10" s="36">
@@ -1704,26 +1704,26 @@
         <v>1110378.24</v>
       </c>
       <c r="L10" s="35" t="s">
-        <v>92</v>
-      </c>
-      <c r="M10" s="39">
+        <v>81</v>
+      </c>
+      <c r="M10" s="38">
         <f t="shared" si="1"/>
         <v>1110378.24</v>
       </c>
       <c r="N10" s="42"/>
       <c r="O10" s="25"/>
-      <c r="P10" s="28"/>
+      <c r="P10" s="27"/>
       <c r="V10" s="3"/>
     </row>
     <row r="11" ht="12.75" customHeight="1">
       <c r="A11" s="23"/>
       <c r="B11" s="23"/>
-      <c r="C11" s="41"/>
+      <c r="C11" s="40"/>
       <c r="D11" s="33" t="s">
-        <v>95</v>
+        <v>86</v>
       </c>
       <c r="E11" s="34" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="F11" s="35">
         <v>634.0</v>
@@ -1732,7 +1732,7 @@
         <v>45799.0</v>
       </c>
       <c r="H11" s="35" t="s">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="I11" s="36"/>
       <c r="J11" s="36">
@@ -1742,25 +1742,25 @@
         <v>974557.12</v>
       </c>
       <c r="L11" s="34" t="s">
-        <v>99</v>
-      </c>
-      <c r="M11" s="39">
+        <v>90</v>
+      </c>
+      <c r="M11" s="38">
         <v>974557.12</v>
       </c>
       <c r="N11" s="42"/>
       <c r="O11" s="25"/>
-      <c r="P11" s="28"/>
+      <c r="P11" s="27"/>
       <c r="V11" s="3"/>
     </row>
     <row r="12" ht="27.75" customHeight="1">
       <c r="A12" s="23"/>
       <c r="B12" s="23"/>
-      <c r="C12" s="41"/>
+      <c r="C12" s="40"/>
       <c r="D12" s="33" t="s">
-        <v>102</v>
+        <v>93</v>
       </c>
       <c r="E12" s="34" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="F12" s="34">
         <v>660.0</v>
@@ -1769,7 +1769,7 @@
         <v>45856.0</v>
       </c>
       <c r="H12" s="44" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="I12" s="36"/>
       <c r="J12" s="36">
@@ -1779,25 +1779,25 @@
         <v>1402001.34</v>
       </c>
       <c r="L12" s="46" t="s">
-        <v>105</v>
-      </c>
-      <c r="M12" s="39">
+        <v>97</v>
+      </c>
+      <c r="M12" s="38">
         <v>1402001.34</v>
       </c>
       <c r="N12" s="47"/>
       <c r="O12" s="25"/>
-      <c r="P12" s="28"/>
+      <c r="P12" s="27"/>
       <c r="V12" s="3"/>
     </row>
     <row r="13">
       <c r="A13" s="23"/>
       <c r="B13" s="23"/>
-      <c r="C13" s="41"/>
-      <c r="D13" s="49" t="s">
-        <v>109</v>
+      <c r="C13" s="40"/>
+      <c r="D13" s="48" t="s">
+        <v>99</v>
       </c>
       <c r="E13" s="34" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="F13" s="35">
         <v>661.0</v>
@@ -1806,7 +1806,7 @@
         <v>45856.0</v>
       </c>
       <c r="H13" s="35" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="I13" s="43"/>
       <c r="J13" s="43">
@@ -1816,25 +1816,25 @@
         <v>1223702.3</v>
       </c>
       <c r="L13" s="34" t="s">
-        <v>115</v>
-      </c>
-      <c r="M13" s="39">
+        <v>102</v>
+      </c>
+      <c r="M13" s="38">
         <v>1223702.3</v>
       </c>
       <c r="N13" s="47"/>
       <c r="O13" s="25"/>
-      <c r="P13" s="50"/>
+      <c r="P13" s="49"/>
       <c r="V13" s="3"/>
     </row>
     <row r="14">
       <c r="A14" s="23"/>
       <c r="B14" s="23"/>
-      <c r="C14" s="41"/>
-      <c r="D14" s="49" t="s">
-        <v>118</v>
+      <c r="C14" s="40"/>
+      <c r="D14" s="48" t="s">
+        <v>105</v>
       </c>
       <c r="E14" s="34" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="F14" s="34">
         <v>688.0</v>
@@ -1843,7 +1843,7 @@
         <v>45901.0</v>
       </c>
       <c r="H14" s="34" t="s">
-        <v>119</v>
+        <v>106</v>
       </c>
       <c r="I14" s="43"/>
       <c r="J14" s="43">
@@ -1853,25 +1853,25 @@
         <v>1011677.95</v>
       </c>
       <c r="L14" s="34" t="s">
-        <v>122</v>
-      </c>
-      <c r="M14" s="39">
+        <v>108</v>
+      </c>
+      <c r="M14" s="38">
         <v>1011677.95</v>
       </c>
       <c r="N14" s="42"/>
       <c r="O14" s="25"/>
-      <c r="P14" s="28"/>
+      <c r="P14" s="27"/>
       <c r="V14" s="3"/>
     </row>
     <row r="15">
       <c r="A15" s="23"/>
       <c r="B15" s="23"/>
-      <c r="C15" s="41"/>
-      <c r="D15" s="49" t="s">
-        <v>124</v>
+      <c r="C15" s="40"/>
+      <c r="D15" s="48" t="s">
+        <v>110</v>
       </c>
       <c r="E15" s="34" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="F15" s="34">
         <v>696.0</v>
@@ -1880,7 +1880,7 @@
         <v>45923.0</v>
       </c>
       <c r="H15" s="34" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="I15" s="43"/>
       <c r="J15" s="43">
@@ -1890,9 +1890,9 @@
         <v>896744.06</v>
       </c>
       <c r="L15" s="34" t="s">
-        <v>127</v>
-      </c>
-      <c r="M15" s="39">
+        <v>113</v>
+      </c>
+      <c r="M15" s="38">
         <v>896744.06</v>
       </c>
       <c r="N15" s="47"/>
@@ -1902,12 +1902,12 @@
     <row r="16">
       <c r="A16" s="23"/>
       <c r="B16" s="23"/>
-      <c r="C16" s="41"/>
-      <c r="D16" s="49" t="s">
-        <v>131</v>
+      <c r="C16" s="40"/>
+      <c r="D16" s="48" t="s">
+        <v>114</v>
       </c>
       <c r="E16" s="34" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="F16" s="34">
         <v>704.0</v>
@@ -1916,7 +1916,7 @@
         <v>45957.0</v>
       </c>
       <c r="H16" s="34" t="s">
-        <v>132</v>
+        <v>118</v>
       </c>
       <c r="I16" s="43"/>
       <c r="J16" s="43">
@@ -1926,9 +1926,9 @@
         <v>919329.06</v>
       </c>
       <c r="L16" s="34" t="s">
-        <v>135</v>
-      </c>
-      <c r="M16" s="39">
+        <v>119</v>
+      </c>
+      <c r="M16" s="38">
         <v>919329.06</v>
       </c>
       <c r="N16" s="42"/>
@@ -1938,9 +1938,9 @@
     <row r="17">
       <c r="A17" s="23"/>
       <c r="B17" s="23"/>
-      <c r="C17" s="41"/>
-      <c r="D17" s="49" t="s">
-        <v>137</v>
+      <c r="C17" s="40"/>
+      <c r="D17" s="48" t="s">
+        <v>123</v>
       </c>
       <c r="E17" s="34"/>
       <c r="F17" s="34">
@@ -1950,7 +1950,7 @@
         <v>45972.0</v>
       </c>
       <c r="H17" s="34" t="s">
-        <v>141</v>
+        <v>125</v>
       </c>
       <c r="I17" s="34"/>
       <c r="J17" s="43">
@@ -1960,9 +1960,9 @@
         <v>1157009.26</v>
       </c>
       <c r="L17" s="34" t="s">
-        <v>142</v>
-      </c>
-      <c r="M17" s="39">
+        <v>127</v>
+      </c>
+      <c r="M17" s="38">
         <v>1157009.26</v>
       </c>
       <c r="N17" s="51"/>
@@ -1972,12 +1972,12 @@
     <row r="18">
       <c r="A18" s="23"/>
       <c r="B18" s="23"/>
-      <c r="C18" s="41"/>
-      <c r="D18" s="49" t="s">
-        <v>146</v>
+      <c r="C18" s="40"/>
+      <c r="D18" s="48" t="s">
+        <v>132</v>
       </c>
       <c r="E18" s="34" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="F18" s="34">
         <v>728.0</v>
@@ -1986,7 +1986,7 @@
         <v>46008.0</v>
       </c>
       <c r="H18" s="34" t="s">
-        <v>148</v>
+        <v>133</v>
       </c>
       <c r="I18" s="34"/>
       <c r="J18" s="43">
@@ -1996,28 +1996,28 @@
         <v>1214597.952</v>
       </c>
       <c r="L18" s="34" t="s">
-        <v>151</v>
-      </c>
-      <c r="M18" s="39">
+        <v>136</v>
+      </c>
+      <c r="M18" s="38">
         <v>1214597.952</v>
       </c>
       <c r="N18" s="51"/>
       <c r="O18" s="25"/>
-      <c r="R18" s="28"/>
-      <c r="S18" s="28"/>
-      <c r="T18" s="28"/>
-      <c r="U18" s="28"/>
+      <c r="R18" s="27"/>
+      <c r="S18" s="27"/>
+      <c r="T18" s="27"/>
+      <c r="U18" s="27"/>
       <c r="V18" s="52"/>
     </row>
     <row r="19">
       <c r="A19" s="23"/>
       <c r="B19" s="23"/>
-      <c r="C19" s="41"/>
-      <c r="D19" s="49" t="s">
-        <v>154</v>
+      <c r="C19" s="40"/>
+      <c r="D19" s="48" t="s">
+        <v>140</v>
       </c>
       <c r="E19" s="34" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="F19" s="34">
         <v>278.0</v>
@@ -2026,7 +2026,7 @@
         <v>46042.0</v>
       </c>
       <c r="H19" s="34" t="s">
-        <v>156</v>
+        <v>141</v>
       </c>
       <c r="I19" s="43"/>
       <c r="J19" s="43">
@@ -2036,25 +2036,25 @@
         <v>967082.09</v>
       </c>
       <c r="L19" s="34" t="s">
-        <v>158</v>
-      </c>
-      <c r="M19" s="39">
+        <v>142</v>
+      </c>
+      <c r="M19" s="38">
         <v>967082.09</v>
       </c>
       <c r="N19" s="51"/>
       <c r="O19" s="25"/>
-      <c r="R19" s="28"/>
-      <c r="S19" s="28"/>
-      <c r="T19" s="28"/>
-      <c r="U19" s="28"/>
+      <c r="R19" s="27"/>
+      <c r="S19" s="27"/>
+      <c r="T19" s="27"/>
+      <c r="U19" s="27"/>
       <c r="V19" s="52"/>
     </row>
     <row r="20">
       <c r="A20" s="23"/>
       <c r="B20" s="23"/>
-      <c r="C20" s="41"/>
-      <c r="D20" s="49" t="s">
-        <v>159</v>
+      <c r="C20" s="40"/>
+      <c r="D20" s="48" t="s">
+        <v>146</v>
       </c>
       <c r="E20" s="34"/>
       <c r="F20" s="34">
@@ -2064,7 +2064,7 @@
         <v>46078.0</v>
       </c>
       <c r="H20" s="34" t="s">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="I20" s="43"/>
       <c r="J20" s="43">
@@ -2074,25 +2074,25 @@
         <v>719561.08</v>
       </c>
       <c r="L20" s="34" t="s">
-        <v>160</v>
-      </c>
-      <c r="M20" s="39">
+        <v>150</v>
+      </c>
+      <c r="M20" s="38">
         <v>719561.08</v>
       </c>
       <c r="N20" s="51"/>
       <c r="O20" s="25"/>
-      <c r="R20" s="28"/>
-      <c r="S20" s="28"/>
-      <c r="T20" s="28"/>
-      <c r="U20" s="28"/>
+      <c r="R20" s="27"/>
+      <c r="S20" s="27"/>
+      <c r="T20" s="27"/>
+      <c r="U20" s="27"/>
       <c r="V20" s="52"/>
     </row>
     <row r="21">
       <c r="A21" s="23"/>
       <c r="B21" s="23"/>
-      <c r="C21" s="41"/>
-      <c r="D21" s="49" t="s">
-        <v>161</v>
+      <c r="C21" s="40"/>
+      <c r="D21" s="48" t="s">
+        <v>154</v>
       </c>
       <c r="E21" s="34"/>
       <c r="F21" s="34">
@@ -2102,7 +2102,7 @@
         <v>46094.0</v>
       </c>
       <c r="H21" s="34" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="I21" s="43"/>
       <c r="J21" s="43">
@@ -2112,25 +2112,25 @@
         <v>885881.08</v>
       </c>
       <c r="L21" s="34" t="s">
-        <v>163</v>
-      </c>
-      <c r="M21" s="39">
+        <v>159</v>
+      </c>
+      <c r="M21" s="38">
         <v>885881.08</v>
       </c>
       <c r="N21" s="51"/>
       <c r="O21" s="25"/>
-      <c r="R21" s="28"/>
-      <c r="S21" s="28"/>
-      <c r="T21" s="28"/>
-      <c r="U21" s="28"/>
+      <c r="R21" s="27"/>
+      <c r="S21" s="27"/>
+      <c r="T21" s="27"/>
+      <c r="U21" s="27"/>
       <c r="V21" s="52"/>
     </row>
     <row r="22">
       <c r="A22" s="23"/>
       <c r="B22" s="23"/>
-      <c r="C22" s="41"/>
-      <c r="D22" s="49" t="s">
-        <v>164</v>
+      <c r="C22" s="40"/>
+      <c r="D22" s="48" t="s">
+        <v>160</v>
       </c>
       <c r="E22" s="34"/>
       <c r="F22" s="34">
@@ -2140,34 +2140,34 @@
         <v>46128.0</v>
       </c>
       <c r="H22" s="34" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="I22" s="43"/>
       <c r="J22" s="43">
         <v>46164.0</v>
       </c>
       <c r="K22" s="45" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="L22" s="34" t="s">
-        <v>167</v>
-      </c>
-      <c r="M22" s="39" t="s">
-        <v>166</v>
+        <v>165</v>
+      </c>
+      <c r="M22" s="38" t="s">
+        <v>164</v>
       </c>
       <c r="N22" s="51"/>
       <c r="O22" s="25"/>
-      <c r="R22" s="28"/>
-      <c r="S22" s="28"/>
-      <c r="T22" s="28"/>
-      <c r="U22" s="28"/>
+      <c r="R22" s="27"/>
+      <c r="S22" s="27"/>
+      <c r="T22" s="27"/>
+      <c r="U22" s="27"/>
       <c r="V22" s="52"/>
     </row>
     <row r="23">
       <c r="A23" s="23"/>
       <c r="B23" s="23"/>
-      <c r="C23" s="41"/>
-      <c r="D23" s="49" t="s">
+      <c r="C23" s="40"/>
+      <c r="D23" s="48" t="s">
         <v>168</v>
       </c>
       <c r="E23" s="34"/>
@@ -2188,24 +2188,24 @@
         <v>1108954.4358333333</v>
       </c>
       <c r="L23" s="34" t="s">
-        <v>163</v>
-      </c>
-      <c r="M23" s="39">
+        <v>159</v>
+      </c>
+      <c r="M23" s="38">
         <v>1108954.4358333333</v>
       </c>
       <c r="N23" s="53"/>
       <c r="O23" s="25"/>
-      <c r="R23" s="28"/>
-      <c r="S23" s="28"/>
-      <c r="T23" s="28"/>
-      <c r="U23" s="28"/>
+      <c r="R23" s="27"/>
+      <c r="S23" s="27"/>
+      <c r="T23" s="27"/>
+      <c r="U23" s="27"/>
       <c r="V23" s="52"/>
     </row>
     <row r="24">
       <c r="A24" s="23"/>
       <c r="B24" s="23"/>
-      <c r="C24" s="41"/>
-      <c r="D24" s="49" t="s">
+      <c r="C24" s="40"/>
+      <c r="D24" s="48" t="s">
         <v>170</v>
       </c>
       <c r="E24" s="34"/>
@@ -2228,22 +2228,22 @@
       <c r="L24" s="34" t="s">
         <v>171</v>
       </c>
-      <c r="M24" s="39">
+      <c r="M24" s="38">
         <v>218206.1</v>
       </c>
       <c r="N24" s="54"/>
       <c r="O24" s="25"/>
-      <c r="R24" s="28"/>
-      <c r="S24" s="28"/>
-      <c r="T24" s="28"/>
-      <c r="U24" s="28"/>
+      <c r="R24" s="27"/>
+      <c r="S24" s="27"/>
+      <c r="T24" s="27"/>
+      <c r="U24" s="27"/>
       <c r="V24" s="52"/>
     </row>
     <row r="25">
       <c r="A25" s="23"/>
       <c r="B25" s="23"/>
-      <c r="C25" s="41"/>
-      <c r="D25" s="49" t="s">
+      <c r="C25" s="40"/>
+      <c r="D25" s="48" t="s">
         <v>172</v>
       </c>
       <c r="E25" s="34"/>
@@ -2266,22 +2266,22 @@
       <c r="L25" s="34" t="s">
         <v>173</v>
       </c>
-      <c r="M25" s="39">
+      <c r="M25" s="38">
         <v>1549250.84</v>
       </c>
       <c r="N25" s="54"/>
       <c r="O25" s="25"/>
-      <c r="R25" s="28"/>
-      <c r="S25" s="28"/>
-      <c r="T25" s="28"/>
-      <c r="U25" s="28"/>
+      <c r="R25" s="27"/>
+      <c r="S25" s="27"/>
+      <c r="T25" s="27"/>
+      <c r="U25" s="27"/>
       <c r="V25" s="52"/>
     </row>
     <row r="26">
       <c r="A26" s="23"/>
       <c r="B26" s="23"/>
       <c r="C26" s="55"/>
-      <c r="D26" s="49" t="s">
+      <c r="D26" s="48" t="s">
         <v>174</v>
       </c>
       <c r="E26" s="34"/>
@@ -2304,64 +2304,64 @@
       <c r="L26" s="34" t="s">
         <v>177</v>
       </c>
-      <c r="M26" s="39" t="s">
+      <c r="M26" s="38" t="s">
         <v>176</v>
       </c>
       <c r="N26" s="54"/>
       <c r="O26" s="25"/>
-      <c r="R26" s="28"/>
-      <c r="S26" s="28"/>
-      <c r="T26" s="28"/>
-      <c r="U26" s="28"/>
+      <c r="R26" s="27"/>
+      <c r="S26" s="27"/>
+      <c r="T26" s="27"/>
+      <c r="U26" s="27"/>
       <c r="V26" s="52"/>
     </row>
     <row r="27" ht="30.75" customHeight="1">
       <c r="A27" s="23"/>
       <c r="B27" s="23"/>
-      <c r="C27" s="29" t="s">
+      <c r="C27" s="28" t="s">
         <v>49</v>
       </c>
-      <c r="D27" s="29" t="s">
-        <v>53</v>
+      <c r="D27" s="28" t="s">
+        <v>50</v>
       </c>
       <c r="E27" s="30" t="s">
-        <v>54</v>
-      </c>
-      <c r="F27" s="29" t="s">
+        <v>51</v>
+      </c>
+      <c r="F27" s="28" t="s">
+        <v>52</v>
+      </c>
+      <c r="G27" s="28"/>
+      <c r="H27" s="28" t="s">
         <v>56</v>
       </c>
-      <c r="G27" s="29"/>
-      <c r="H27" s="29" t="s">
-        <v>58</v>
-      </c>
-      <c r="I27" s="29"/>
-      <c r="J27" s="29"/>
+      <c r="I27" s="28"/>
+      <c r="J27" s="28"/>
       <c r="K27" s="56" t="s">
+        <v>60</v>
+      </c>
+      <c r="L27" s="31" t="s">
+        <v>62</v>
+      </c>
+      <c r="M27" s="57" t="s">
         <v>63</v>
       </c>
-      <c r="L27" s="31" t="s">
+      <c r="N27" s="28" t="s">
         <v>64</v>
       </c>
-      <c r="M27" s="57" t="s">
-        <v>65</v>
-      </c>
-      <c r="N27" s="29" t="s">
-        <v>66</v>
-      </c>
       <c r="O27" s="25"/>
-      <c r="P27" s="28"/>
-      <c r="R27" s="28"/>
-      <c r="S27" s="28"/>
-      <c r="T27" s="28"/>
-      <c r="U27" s="28"/>
+      <c r="P27" s="27"/>
+      <c r="R27" s="27"/>
+      <c r="S27" s="27"/>
+      <c r="T27" s="27"/>
+      <c r="U27" s="27"/>
       <c r="V27" s="52"/>
-      <c r="W27" s="28"/>
-      <c r="X27" s="28"/>
-      <c r="Y27" s="28"/>
-      <c r="Z27" s="28"/>
-      <c r="AA27" s="28"/>
-      <c r="AB27" s="28"/>
-      <c r="AC27" s="28"/>
+      <c r="W27" s="27"/>
+      <c r="X27" s="27"/>
+      <c r="Y27" s="27"/>
+      <c r="Z27" s="27"/>
+      <c r="AA27" s="27"/>
+      <c r="AB27" s="27"/>
+      <c r="AC27" s="27"/>
     </row>
     <row r="28" ht="12.75" customHeight="1">
       <c r="A28" s="23"/>
@@ -2380,7 +2380,7 @@
         <v>45791.0</v>
       </c>
       <c r="H28" s="35" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="I28" s="36"/>
       <c r="J28" s="36">
@@ -2397,25 +2397,25 @@
       </c>
       <c r="N28" s="51"/>
       <c r="O28" s="25"/>
-      <c r="P28" s="28"/>
-      <c r="Q28" s="28"/>
-      <c r="R28" s="28"/>
-      <c r="S28" s="28"/>
-      <c r="T28" s="28"/>
-      <c r="U28" s="28"/>
+      <c r="P28" s="27"/>
+      <c r="Q28" s="27"/>
+      <c r="R28" s="27"/>
+      <c r="S28" s="27"/>
+      <c r="T28" s="27"/>
+      <c r="U28" s="27"/>
       <c r="V28" s="52"/>
-      <c r="W28" s="28"/>
-      <c r="X28" s="28"/>
-      <c r="Y28" s="28"/>
-      <c r="Z28" s="28"/>
-      <c r="AA28" s="28"/>
-      <c r="AB28" s="28"/>
-      <c r="AC28" s="28"/>
+      <c r="W28" s="27"/>
+      <c r="X28" s="27"/>
+      <c r="Y28" s="27"/>
+      <c r="Z28" s="27"/>
+      <c r="AA28" s="27"/>
+      <c r="AB28" s="27"/>
+      <c r="AC28" s="27"/>
     </row>
     <row r="29">
       <c r="A29" s="23"/>
       <c r="B29" s="23"/>
-      <c r="C29" s="41"/>
+      <c r="C29" s="40"/>
       <c r="D29" s="58" t="s">
         <v>180</v>
       </c>
@@ -2441,30 +2441,30 @@
       <c r="L29" s="34" t="s">
         <v>182</v>
       </c>
-      <c r="M29" s="39">
+      <c r="M29" s="38">
         <v>112720.77</v>
       </c>
       <c r="N29" s="51"/>
       <c r="O29" s="25"/>
-      <c r="P29" s="28"/>
-      <c r="Q29" s="28"/>
-      <c r="R29" s="28"/>
-      <c r="S29" s="28"/>
-      <c r="T29" s="28"/>
-      <c r="U29" s="28"/>
+      <c r="P29" s="27"/>
+      <c r="Q29" s="27"/>
+      <c r="R29" s="27"/>
+      <c r="S29" s="27"/>
+      <c r="T29" s="27"/>
+      <c r="U29" s="27"/>
       <c r="V29" s="52"/>
-      <c r="W29" s="28"/>
-      <c r="X29" s="28"/>
-      <c r="Y29" s="28"/>
-      <c r="Z29" s="28"/>
-      <c r="AA29" s="28"/>
-      <c r="AB29" s="28"/>
-      <c r="AC29" s="28"/>
+      <c r="W29" s="27"/>
+      <c r="X29" s="27"/>
+      <c r="Y29" s="27"/>
+      <c r="Z29" s="27"/>
+      <c r="AA29" s="27"/>
+      <c r="AB29" s="27"/>
+      <c r="AC29" s="27"/>
     </row>
     <row r="30" ht="12.75" customHeight="1">
       <c r="A30" s="23"/>
       <c r="B30" s="23"/>
-      <c r="C30" s="41"/>
+      <c r="C30" s="40"/>
       <c r="D30" s="61" t="s">
         <v>183</v>
       </c>
@@ -2478,7 +2478,7 @@
         <v>45853.0</v>
       </c>
       <c r="H30" s="34" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="I30" s="43"/>
       <c r="J30" s="43">
@@ -2490,30 +2490,30 @@
       <c r="L30" s="34" t="s">
         <v>185</v>
       </c>
-      <c r="M30" s="39">
+      <c r="M30" s="38">
         <v>378307.61</v>
       </c>
       <c r="N30" s="51"/>
       <c r="O30" s="25"/>
       <c r="P30" s="64"/>
-      <c r="Q30" s="28"/>
-      <c r="R30" s="28"/>
-      <c r="S30" s="28"/>
-      <c r="T30" s="28"/>
-      <c r="U30" s="28"/>
+      <c r="Q30" s="27"/>
+      <c r="R30" s="27"/>
+      <c r="S30" s="27"/>
+      <c r="T30" s="27"/>
+      <c r="U30" s="27"/>
       <c r="V30" s="52"/>
-      <c r="W30" s="28"/>
-      <c r="X30" s="28"/>
-      <c r="Y30" s="28"/>
-      <c r="Z30" s="28"/>
-      <c r="AA30" s="28"/>
-      <c r="AB30" s="28"/>
-      <c r="AC30" s="28"/>
+      <c r="W30" s="27"/>
+      <c r="X30" s="27"/>
+      <c r="Y30" s="27"/>
+      <c r="Z30" s="27"/>
+      <c r="AA30" s="27"/>
+      <c r="AB30" s="27"/>
+      <c r="AC30" s="27"/>
     </row>
     <row r="31" ht="60.0" customHeight="1">
       <c r="A31" s="23"/>
       <c r="B31" s="23"/>
-      <c r="C31" s="41"/>
+      <c r="C31" s="40"/>
       <c r="D31" s="61" t="s">
         <v>186</v>
       </c>
@@ -2527,7 +2527,7 @@
         <v>45910.0</v>
       </c>
       <c r="H31" s="34" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="I31" s="43"/>
       <c r="J31" s="43">
@@ -2539,30 +2539,30 @@
       <c r="L31" s="34" t="s">
         <v>187</v>
       </c>
-      <c r="M31" s="39">
+      <c r="M31" s="38">
         <v>3315.04710000003</v>
       </c>
       <c r="N31" s="51"/>
       <c r="O31" s="25"/>
       <c r="P31" s="64"/>
-      <c r="Q31" s="28"/>
-      <c r="R31" s="28"/>
-      <c r="S31" s="28"/>
-      <c r="T31" s="28"/>
-      <c r="U31" s="28"/>
+      <c r="Q31" s="27"/>
+      <c r="R31" s="27"/>
+      <c r="S31" s="27"/>
+      <c r="T31" s="27"/>
+      <c r="U31" s="27"/>
       <c r="V31" s="52"/>
-      <c r="W31" s="28"/>
-      <c r="X31" s="28"/>
-      <c r="Y31" s="28"/>
-      <c r="Z31" s="28"/>
-      <c r="AA31" s="28"/>
-      <c r="AB31" s="28"/>
-      <c r="AC31" s="28"/>
+      <c r="W31" s="27"/>
+      <c r="X31" s="27"/>
+      <c r="Y31" s="27"/>
+      <c r="Z31" s="27"/>
+      <c r="AA31" s="27"/>
+      <c r="AB31" s="27"/>
+      <c r="AC31" s="27"/>
     </row>
     <row r="32" ht="12.75" customHeight="1">
       <c r="A32" s="23"/>
       <c r="B32" s="23"/>
-      <c r="C32" s="41"/>
+      <c r="C32" s="40"/>
       <c r="D32" s="61" t="s">
         <v>188</v>
       </c>
@@ -2576,7 +2576,7 @@
         <v>45904.0</v>
       </c>
       <c r="H32" s="34" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="I32" s="66"/>
       <c r="J32" s="66">
@@ -2588,30 +2588,30 @@
       <c r="L32" s="34" t="s">
         <v>189</v>
       </c>
-      <c r="M32" s="39">
+      <c r="M32" s="38">
         <v>198332.75</v>
       </c>
       <c r="N32" s="51"/>
       <c r="O32" s="25"/>
       <c r="P32" s="64"/>
-      <c r="Q32" s="28"/>
-      <c r="R32" s="28"/>
-      <c r="S32" s="28"/>
-      <c r="T32" s="28"/>
-      <c r="U32" s="28"/>
+      <c r="Q32" s="27"/>
+      <c r="R32" s="27"/>
+      <c r="S32" s="27"/>
+      <c r="T32" s="27"/>
+      <c r="U32" s="27"/>
       <c r="V32" s="52"/>
-      <c r="W32" s="28"/>
-      <c r="X32" s="28"/>
-      <c r="Y32" s="28"/>
-      <c r="Z32" s="28"/>
-      <c r="AA32" s="28"/>
-      <c r="AB32" s="28"/>
-      <c r="AC32" s="28"/>
+      <c r="W32" s="27"/>
+      <c r="X32" s="27"/>
+      <c r="Y32" s="27"/>
+      <c r="Z32" s="27"/>
+      <c r="AA32" s="27"/>
+      <c r="AB32" s="27"/>
+      <c r="AC32" s="27"/>
     </row>
     <row r="33" ht="12.75" customHeight="1">
       <c r="A33" s="23"/>
       <c r="B33" s="23"/>
-      <c r="C33" s="41"/>
+      <c r="C33" s="40"/>
       <c r="D33" s="61" t="s">
         <v>190</v>
       </c>
@@ -2625,7 +2625,7 @@
         <v>46008.0</v>
       </c>
       <c r="H33" s="34" t="s">
-        <v>120</v>
+        <v>129</v>
       </c>
       <c r="I33" s="66"/>
       <c r="J33" s="66">
@@ -2643,24 +2643,24 @@
       <c r="N33" s="51"/>
       <c r="O33" s="25"/>
       <c r="P33" s="64"/>
-      <c r="Q33" s="28"/>
-      <c r="R33" s="28"/>
-      <c r="S33" s="28"/>
-      <c r="T33" s="28"/>
-      <c r="U33" s="28"/>
+      <c r="Q33" s="27"/>
+      <c r="R33" s="27"/>
+      <c r="S33" s="27"/>
+      <c r="T33" s="27"/>
+      <c r="U33" s="27"/>
       <c r="V33" s="52"/>
-      <c r="W33" s="28"/>
-      <c r="X33" s="28"/>
-      <c r="Y33" s="28"/>
-      <c r="Z33" s="28"/>
-      <c r="AA33" s="28"/>
-      <c r="AB33" s="28"/>
-      <c r="AC33" s="28"/>
+      <c r="W33" s="27"/>
+      <c r="X33" s="27"/>
+      <c r="Y33" s="27"/>
+      <c r="Z33" s="27"/>
+      <c r="AA33" s="27"/>
+      <c r="AB33" s="27"/>
+      <c r="AC33" s="27"/>
     </row>
     <row r="34" ht="12.75" customHeight="1">
       <c r="A34" s="23"/>
       <c r="B34" s="23"/>
-      <c r="C34" s="41"/>
+      <c r="C34" s="40"/>
       <c r="D34" s="61" t="s">
         <v>193</v>
       </c>
@@ -2674,7 +2674,7 @@
         <v>45930.0</v>
       </c>
       <c r="H34" s="34" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="I34" s="66"/>
       <c r="J34" s="66">
@@ -2692,24 +2692,24 @@
       <c r="N34" s="51"/>
       <c r="O34" s="25"/>
       <c r="P34" s="64"/>
-      <c r="Q34" s="28"/>
-      <c r="R34" s="28"/>
-      <c r="S34" s="28"/>
-      <c r="T34" s="28"/>
-      <c r="U34" s="28"/>
+      <c r="Q34" s="27"/>
+      <c r="R34" s="27"/>
+      <c r="S34" s="27"/>
+      <c r="T34" s="27"/>
+      <c r="U34" s="27"/>
       <c r="V34" s="52"/>
-      <c r="W34" s="28"/>
-      <c r="X34" s="28"/>
-      <c r="Y34" s="28"/>
-      <c r="Z34" s="28"/>
-      <c r="AA34" s="28"/>
-      <c r="AB34" s="28"/>
-      <c r="AC34" s="28"/>
+      <c r="W34" s="27"/>
+      <c r="X34" s="27"/>
+      <c r="Y34" s="27"/>
+      <c r="Z34" s="27"/>
+      <c r="AA34" s="27"/>
+      <c r="AB34" s="27"/>
+      <c r="AC34" s="27"/>
     </row>
     <row r="35" ht="12.75" customHeight="1">
       <c r="A35" s="23"/>
       <c r="B35" s="23"/>
-      <c r="C35" s="41"/>
+      <c r="C35" s="40"/>
       <c r="D35" s="61" t="s">
         <v>197</v>
       </c>
@@ -2723,7 +2723,7 @@
         <v>45968.0</v>
       </c>
       <c r="H35" s="34" t="s">
-        <v>110</v>
+        <v>120</v>
       </c>
       <c r="I35" s="66"/>
       <c r="J35" s="66">
@@ -2741,24 +2741,24 @@
       <c r="N35" s="51"/>
       <c r="O35" s="25"/>
       <c r="P35" s="64"/>
-      <c r="Q35" s="28"/>
-      <c r="R35" s="28"/>
-      <c r="S35" s="28"/>
-      <c r="T35" s="28"/>
-      <c r="U35" s="28"/>
+      <c r="Q35" s="27"/>
+      <c r="R35" s="27"/>
+      <c r="S35" s="27"/>
+      <c r="T35" s="27"/>
+      <c r="U35" s="27"/>
       <c r="V35" s="52"/>
-      <c r="W35" s="28"/>
-      <c r="X35" s="28"/>
-      <c r="Y35" s="28"/>
-      <c r="Z35" s="28"/>
-      <c r="AA35" s="28"/>
-      <c r="AB35" s="28"/>
-      <c r="AC35" s="28"/>
+      <c r="W35" s="27"/>
+      <c r="X35" s="27"/>
+      <c r="Y35" s="27"/>
+      <c r="Z35" s="27"/>
+      <c r="AA35" s="27"/>
+      <c r="AB35" s="27"/>
+      <c r="AC35" s="27"/>
     </row>
     <row r="36" ht="12.75" customHeight="1">
       <c r="A36" s="23"/>
       <c r="B36" s="23"/>
-      <c r="C36" s="41"/>
+      <c r="C36" s="40"/>
       <c r="D36" s="61" t="s">
         <v>200</v>
       </c>
@@ -2772,7 +2772,7 @@
         <v>46043.0</v>
       </c>
       <c r="H36" s="65" t="s">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="I36" s="70"/>
       <c r="J36" s="69">
@@ -2784,30 +2784,30 @@
       <c r="L36" s="34" t="s">
         <v>201</v>
       </c>
-      <c r="M36" s="39">
+      <c r="M36" s="38">
         <v>11372.9</v>
       </c>
       <c r="N36" s="51"/>
       <c r="O36" s="25"/>
-      <c r="P36" s="28"/>
-      <c r="Q36" s="28"/>
-      <c r="R36" s="28"/>
-      <c r="S36" s="28"/>
-      <c r="T36" s="28"/>
-      <c r="U36" s="28"/>
+      <c r="P36" s="27"/>
+      <c r="Q36" s="27"/>
+      <c r="R36" s="27"/>
+      <c r="S36" s="27"/>
+      <c r="T36" s="27"/>
+      <c r="U36" s="27"/>
       <c r="V36" s="52"/>
-      <c r="W36" s="28"/>
-      <c r="X36" s="28"/>
-      <c r="Y36" s="28"/>
-      <c r="Z36" s="28"/>
-      <c r="AA36" s="28"/>
-      <c r="AB36" s="28"/>
-      <c r="AC36" s="28"/>
+      <c r="W36" s="27"/>
+      <c r="X36" s="27"/>
+      <c r="Y36" s="27"/>
+      <c r="Z36" s="27"/>
+      <c r="AA36" s="27"/>
+      <c r="AB36" s="27"/>
+      <c r="AC36" s="27"/>
     </row>
     <row r="37" ht="12.75" customHeight="1">
       <c r="A37" s="23"/>
       <c r="B37" s="23"/>
-      <c r="C37" s="41"/>
+      <c r="C37" s="40"/>
       <c r="D37" s="61" t="s">
         <v>202</v>
       </c>
@@ -2821,25 +2821,25 @@
       <c r="J37" s="69"/>
       <c r="K37" s="45"/>
       <c r="L37" s="34"/>
-      <c r="M37" s="39"/>
+      <c r="M37" s="38"/>
       <c r="N37" s="51">
         <v>15854.78</v>
       </c>
       <c r="O37" s="25"/>
-      <c r="P37" s="28"/>
-      <c r="Q37" s="28"/>
-      <c r="R37" s="28"/>
-      <c r="S37" s="28"/>
-      <c r="T37" s="28"/>
-      <c r="U37" s="28"/>
+      <c r="P37" s="27"/>
+      <c r="Q37" s="27"/>
+      <c r="R37" s="27"/>
+      <c r="S37" s="27"/>
+      <c r="T37" s="27"/>
+      <c r="U37" s="27"/>
       <c r="V37" s="52"/>
-      <c r="W37" s="28"/>
-      <c r="X37" s="28"/>
-      <c r="Y37" s="28"/>
-      <c r="Z37" s="28"/>
-      <c r="AA37" s="28"/>
-      <c r="AB37" s="28"/>
-      <c r="AC37" s="28"/>
+      <c r="W37" s="27"/>
+      <c r="X37" s="27"/>
+      <c r="Y37" s="27"/>
+      <c r="Z37" s="27"/>
+      <c r="AA37" s="27"/>
+      <c r="AB37" s="27"/>
+      <c r="AC37" s="27"/>
     </row>
     <row r="38" ht="12.75" customHeight="1">
       <c r="A38" s="23"/>
@@ -2858,25 +2858,25 @@
       <c r="J38" s="69"/>
       <c r="K38" s="45"/>
       <c r="L38" s="34"/>
-      <c r="M38" s="39"/>
+      <c r="M38" s="38"/>
       <c r="N38" s="51" t="s">
         <v>205</v>
       </c>
       <c r="O38" s="25"/>
-      <c r="P38" s="28"/>
-      <c r="Q38" s="28"/>
-      <c r="R38" s="28"/>
-      <c r="S38" s="28"/>
-      <c r="T38" s="28"/>
-      <c r="U38" s="28"/>
+      <c r="P38" s="27"/>
+      <c r="Q38" s="27"/>
+      <c r="R38" s="27"/>
+      <c r="S38" s="27"/>
+      <c r="T38" s="27"/>
+      <c r="U38" s="27"/>
       <c r="V38" s="52"/>
-      <c r="W38" s="28"/>
-      <c r="X38" s="28"/>
-      <c r="Y38" s="28"/>
-      <c r="Z38" s="28"/>
-      <c r="AA38" s="28"/>
-      <c r="AB38" s="28"/>
-      <c r="AC38" s="28"/>
+      <c r="W38" s="27"/>
+      <c r="X38" s="27"/>
+      <c r="Y38" s="27"/>
+      <c r="Z38" s="27"/>
+      <c r="AA38" s="27"/>
+      <c r="AB38" s="27"/>
+      <c r="AC38" s="27"/>
     </row>
     <row r="39" ht="12.75" customHeight="1">
       <c r="A39" s="23"/>
@@ -2895,7 +2895,7 @@
         <v>46104.0</v>
       </c>
       <c r="H39" s="65" t="s">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="I39" s="70"/>
       <c r="J39" s="69">
@@ -2912,25 +2912,25 @@
       </c>
       <c r="N39" s="51"/>
       <c r="O39" s="25"/>
-      <c r="P39" s="28"/>
-      <c r="Q39" s="28"/>
-      <c r="R39" s="28"/>
-      <c r="S39" s="28"/>
-      <c r="T39" s="28"/>
-      <c r="U39" s="28"/>
+      <c r="P39" s="27"/>
+      <c r="Q39" s="27"/>
+      <c r="R39" s="27"/>
+      <c r="S39" s="27"/>
+      <c r="T39" s="27"/>
+      <c r="U39" s="27"/>
       <c r="V39" s="52"/>
-      <c r="W39" s="28"/>
-      <c r="X39" s="28"/>
-      <c r="Y39" s="28"/>
-      <c r="Z39" s="28"/>
-      <c r="AA39" s="28"/>
-      <c r="AB39" s="28"/>
-      <c r="AC39" s="28"/>
+      <c r="W39" s="27"/>
+      <c r="X39" s="27"/>
+      <c r="Y39" s="27"/>
+      <c r="Z39" s="27"/>
+      <c r="AA39" s="27"/>
+      <c r="AB39" s="27"/>
+      <c r="AC39" s="27"/>
     </row>
     <row r="40" ht="12.75" customHeight="1">
       <c r="A40" s="15"/>
       <c r="B40" s="15"/>
-      <c r="C40" s="41"/>
+      <c r="C40" s="40"/>
       <c r="D40" s="61" t="s">
         <v>208</v>
       </c>
@@ -2942,7 +2942,7 @@
         <v>46199.0</v>
       </c>
       <c r="H40" s="65" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="I40" s="70"/>
       <c r="J40" s="69">
@@ -2952,7 +2952,7 @@
         <v>58868.35</v>
       </c>
       <c r="L40" s="34" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="M40" s="72">
         <v>58868.35</v>
@@ -2963,7 +2963,7 @@
     <row r="41" ht="12.75" customHeight="1">
       <c r="A41" s="15"/>
       <c r="B41" s="15"/>
-      <c r="C41" s="41"/>
+      <c r="C41" s="40"/>
       <c r="K41" s="73"/>
       <c r="M41" s="73"/>
       <c r="V41" s="3"/>
@@ -2971,7 +2971,7 @@
     <row r="42" ht="12.75" customHeight="1">
       <c r="A42" s="15"/>
       <c r="B42" s="15"/>
-      <c r="C42" s="41"/>
+      <c r="C42" s="40"/>
       <c r="K42" s="73"/>
       <c r="M42" s="73"/>
       <c r="V42" s="3"/>
@@ -2979,25 +2979,25 @@
     <row r="43" ht="12.75" customHeight="1">
       <c r="A43" s="15"/>
       <c r="B43" s="15"/>
-      <c r="C43" s="41"/>
+      <c r="C43" s="40"/>
       <c r="V43" s="3"/>
     </row>
     <row r="44" ht="12.75" customHeight="1">
       <c r="A44" s="15"/>
       <c r="B44" s="15"/>
-      <c r="C44" s="41"/>
+      <c r="C44" s="40"/>
       <c r="V44" s="3"/>
     </row>
     <row r="45" ht="12.75" customHeight="1">
       <c r="A45" s="15"/>
       <c r="B45" s="15"/>
-      <c r="C45" s="41"/>
+      <c r="C45" s="40"/>
       <c r="V45" s="3"/>
     </row>
     <row r="46" ht="12.75" customHeight="1">
       <c r="A46" s="15"/>
       <c r="B46" s="15"/>
-      <c r="C46" s="41"/>
+      <c r="C46" s="40"/>
       <c r="V46" s="3"/>
     </row>
     <row r="47" ht="12.75" customHeight="1">
@@ -8017,13 +8017,13 @@
     </row>
     <row r="5">
       <c r="A5" s="10" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D5" s="10" t="s">
         <v>4</v>
@@ -8062,13 +8062,13 @@
     </row>
     <row r="6">
       <c r="A6" s="10" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D6" s="10" t="s">
         <v>4</v>
@@ -8107,13 +8107,13 @@
     </row>
     <row r="7">
       <c r="A7" s="10" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D7" s="10" t="s">
         <v>4</v>
@@ -8131,7 +8131,7 @@
         <v>339039.0</v>
       </c>
       <c r="I7" s="10" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="J7" s="14">
         <v>949835.78</v>
@@ -8187,7 +8187,7 @@
       <c r="L8" s="10">
         <v>0.0</v>
       </c>
-      <c r="O8" s="26"/>
+      <c r="O8" s="29"/>
       <c r="AB8" s="2"/>
       <c r="AC8" s="2"/>
       <c r="AD8" s="2"/>
@@ -8198,13 +8198,13 @@
     </row>
     <row r="9">
       <c r="A9" s="10" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="D9" s="10" t="s">
         <v>4</v>
@@ -8222,7 +8222,7 @@
         <v>339039.0</v>
       </c>
       <c r="I9" s="10" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="J9" s="14">
         <v>211614.23</v>
@@ -8243,13 +8243,13 @@
     </row>
     <row r="10">
       <c r="A10" s="10" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="B10" s="10" t="s">
         <v>7</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="D10" s="10" t="s">
         <v>4</v>
@@ -8288,13 +8288,13 @@
     </row>
     <row r="11">
       <c r="A11" s="10" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D11" s="10" t="s">
         <v>4</v>
@@ -8333,13 +8333,13 @@
     </row>
     <row r="12">
       <c r="A12" s="10" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="D12" s="10" t="s">
         <v>4</v>
@@ -8357,7 +8357,7 @@
         <v>339039.0</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="J12" s="14">
         <v>1600334.09</v>
@@ -8378,13 +8378,13 @@
     </row>
     <row r="13">
       <c r="A13" s="10" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B13" s="10" t="s">
         <v>7</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D13" s="10" t="s">
         <v>4</v>
@@ -8413,7 +8413,7 @@
       <c r="L13" s="14">
         <v>0.0</v>
       </c>
-      <c r="M13" s="38"/>
+      <c r="M13" s="41"/>
       <c r="AB13" s="2"/>
       <c r="AC13" s="2"/>
       <c r="AD13" s="2"/>
@@ -8424,13 +8424,13 @@
     </row>
     <row r="14">
       <c r="A14" s="10" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="D14" s="10" t="s">
         <v>4</v>
@@ -8448,7 +8448,7 @@
         <v>339039.0</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="J14" s="14">
         <v>968237.39</v>
@@ -8469,13 +8469,13 @@
     </row>
     <row r="15">
       <c r="A15" s="10" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="D15" s="10" t="s">
         <v>4</v>
@@ -8493,7 +8493,7 @@
         <v>339039.0</v>
       </c>
       <c r="I15" s="10" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="J15" s="14">
         <v>1011677.95</v>
@@ -8514,13 +8514,13 @@
     </row>
     <row r="16">
       <c r="A16" s="10" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="B16" s="10" t="s">
         <v>7</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="D16" s="10" t="s">
         <v>4</v>
@@ -8559,13 +8559,13 @@
     </row>
     <row r="17">
       <c r="A17" s="10" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="D17" s="10" t="s">
         <v>4</v>
@@ -8604,13 +8604,13 @@
     </row>
     <row r="18">
       <c r="A18" s="10" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="D18" s="10" t="s">
         <v>4</v>
@@ -8628,7 +8628,7 @@
         <v>339039.0</v>
       </c>
       <c r="I18" s="10" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="J18" s="14">
         <v>63746.85</v>
@@ -8649,13 +8649,13 @@
     </row>
     <row r="19">
       <c r="A19" s="10" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="D19" s="10" t="s">
         <v>4</v>
@@ -8673,7 +8673,7 @@
         <v>339039.0</v>
       </c>
       <c r="I19" s="10" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="J19" s="14">
         <v>947931.1</v>
@@ -8694,13 +8694,13 @@
     </row>
     <row r="20">
       <c r="A20" s="10" t="s">
-        <v>100</v>
+        <v>107</v>
       </c>
       <c r="B20" s="10" t="s">
         <v>7</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>101</v>
+        <v>109</v>
       </c>
       <c r="D20" s="10" t="s">
         <v>4</v>
@@ -8739,13 +8739,13 @@
     </row>
     <row r="21">
       <c r="A21" s="10" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="D21" s="10" t="s">
         <v>4</v>
@@ -8784,18 +8784,18 @@
     </row>
     <row r="22">
       <c r="A22" s="10" t="s">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="B22" s="10" t="s">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="C22" s="10" t="s">
-        <v>108</v>
+        <v>117</v>
       </c>
       <c r="D22" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E22" s="48">
+      <c r="E22" s="50">
         <v>45953.0</v>
       </c>
       <c r="F22" s="10" t="s">
@@ -8829,18 +8829,18 @@
     </row>
     <row r="23">
       <c r="A23" s="10" t="s">
-        <v>110</v>
+        <v>120</v>
       </c>
       <c r="B23" s="10" t="s">
-        <v>112</v>
+        <v>121</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>113</v>
+        <v>122</v>
       </c>
       <c r="D23" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E23" s="48">
+      <c r="E23" s="50">
         <v>45953.0</v>
       </c>
       <c r="F23" s="10" t="s">
@@ -8853,7 +8853,7 @@
         <v>339039.0</v>
       </c>
       <c r="I23" s="10" t="s">
-        <v>114</v>
+        <v>124</v>
       </c>
       <c r="J23" s="14">
         <v>1000001.64</v>
@@ -8874,18 +8874,18 @@
     </row>
     <row r="24">
       <c r="A24" s="10" t="s">
-        <v>116</v>
+        <v>126</v>
       </c>
       <c r="B24" s="10" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="C24" s="10" t="s">
-        <v>117</v>
+        <v>128</v>
       </c>
       <c r="D24" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E24" s="48">
+      <c r="E24" s="50">
         <v>45953.0</v>
       </c>
       <c r="F24" s="10" t="s">
@@ -8919,18 +8919,18 @@
     </row>
     <row r="25">
       <c r="A25" s="10" t="s">
-        <v>120</v>
+        <v>129</v>
       </c>
       <c r="B25" s="10" t="s">
-        <v>121</v>
+        <v>130</v>
       </c>
       <c r="C25" s="10" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="D25" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E25" s="48">
+      <c r="E25" s="50">
         <v>45975.0</v>
       </c>
       <c r="F25" s="10" t="s">
@@ -8943,7 +8943,7 @@
         <v>339039.0</v>
       </c>
       <c r="I25" s="10" t="s">
-        <v>114</v>
+        <v>124</v>
       </c>
       <c r="J25" s="14">
         <v>1157673.06</v>
@@ -8964,18 +8964,18 @@
     </row>
     <row r="26">
       <c r="A26" s="10" t="s">
-        <v>125</v>
+        <v>134</v>
       </c>
       <c r="B26" s="10" t="s">
         <v>7</v>
       </c>
       <c r="C26" s="10" t="s">
-        <v>126</v>
+        <v>135</v>
       </c>
       <c r="D26" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E26" s="48">
+      <c r="E26" s="50">
         <v>45989.0</v>
       </c>
       <c r="F26" s="10" t="s">
@@ -9009,13 +9009,13 @@
     </row>
     <row r="27">
       <c r="A27" s="10" t="s">
-        <v>128</v>
+        <v>137</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>129</v>
+        <v>138</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>130</v>
+        <v>139</v>
       </c>
       <c r="D27" s="10" t="s">
         <v>4</v>
@@ -9054,13 +9054,13 @@
     </row>
     <row r="28">
       <c r="A28" s="10" t="s">
-        <v>133</v>
+        <v>143</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>134</v>
+        <v>144</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>136</v>
+        <v>145</v>
       </c>
       <c r="D28" s="10" t="s">
         <v>4</v>
@@ -9099,13 +9099,13 @@
     </row>
     <row r="29">
       <c r="A29" s="10" t="s">
-        <v>138</v>
+        <v>147</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>139</v>
+        <v>148</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>140</v>
+        <v>149</v>
       </c>
       <c r="D29" s="10" t="s">
         <v>4</v>
@@ -9144,13 +9144,13 @@
     </row>
     <row r="30">
       <c r="A30" s="10" t="s">
-        <v>143</v>
+        <v>151</v>
       </c>
       <c r="B30" s="10" t="s">
-        <v>144</v>
+        <v>152</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="D30" s="10" t="s">
         <v>4</v>
@@ -9168,7 +9168,7 @@
         <v>339039.0</v>
       </c>
       <c r="I30" s="10" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="J30" s="14">
         <v>624166.14</v>
@@ -9189,13 +9189,13 @@
     </row>
     <row r="31">
       <c r="A31" s="10" t="s">
-        <v>147</v>
+        <v>156</v>
       </c>
       <c r="B31" s="10" t="s">
-        <v>149</v>
+        <v>157</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
       <c r="D31" s="10" t="s">
         <v>4</v>
@@ -9213,7 +9213,7 @@
         <v>339039.0</v>
       </c>
       <c r="I31" s="10" t="s">
-        <v>114</v>
+        <v>124</v>
       </c>
       <c r="J31" s="14">
         <v>18462.36</v>
@@ -9234,13 +9234,13 @@
     </row>
     <row r="32">
       <c r="A32" s="10" t="s">
-        <v>152</v>
+        <v>161</v>
       </c>
       <c r="B32" s="10" t="s">
-        <v>149</v>
+        <v>157</v>
       </c>
       <c r="C32" s="14" t="s">
-        <v>153</v>
+        <v>162</v>
       </c>
       <c r="D32" s="10" t="s">
         <v>4</v>
@@ -9258,7 +9258,7 @@
         <v>339039.0</v>
       </c>
       <c r="I32" s="10" t="s">
-        <v>114</v>
+        <v>124</v>
       </c>
       <c r="J32" s="14">
         <v>1530656.62</v>
@@ -9279,13 +9279,13 @@
     </row>
     <row r="33">
       <c r="A33" s="10" t="s">
-        <v>155</v>
+        <v>166</v>
       </c>
       <c r="B33" s="10" t="s">
-        <v>139</v>
+        <v>148</v>
       </c>
       <c r="C33" s="14" t="s">
-        <v>157</v>
+        <v>167</v>
       </c>
       <c r="D33" s="10" t="s">
         <v>4</v>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (05/08/2026 12:22)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/01_Bases_Originais/005_CELOG_2025/005_CELOG-PAMALS_2025 online.xlsx
+++ b/Contrato 005/Dashboard/01_Bases_Originais/005_CELOG_2025/005_CELOG-PAMALS_2025 online.xlsx
@@ -30,12 +30,12 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="331" uniqueCount="209">
   <si>
+    <t>Saldo</t>
+  </si>
+  <si>
     <t>Controle de pagamentos</t>
   </si>
   <si>
-    <t>Saldo</t>
-  </si>
-  <si>
     <t>2025NE000005</t>
   </si>
   <si>
@@ -57,6 +57,15 @@
     <t>25E0385</t>
   </si>
   <si>
+    <t>2025NE000369</t>
+  </si>
+  <si>
+    <t>C25516</t>
+  </si>
+  <si>
+    <t>25E0387</t>
+  </si>
+  <si>
     <t>Número Contrato</t>
   </si>
   <si>
@@ -84,12 +93,18 @@
     <t>PAG</t>
   </si>
   <si>
+    <t>2025NE000371</t>
+  </si>
+  <si>
     <t>Moeda</t>
   </si>
   <si>
     <t>Valor Total do Contrato</t>
   </si>
   <si>
+    <t>25E0389</t>
+  </si>
+  <si>
     <t>Valor a Empenhar</t>
   </si>
   <si>
@@ -114,12 +129,21 @@
     <t>Editar</t>
   </si>
   <si>
+    <t>2025NE000413</t>
+  </si>
+  <si>
     <t>005/CELOG-PAMALS/2025</t>
   </si>
   <si>
+    <t>C25501</t>
+  </si>
+  <si>
     <t>CELOG</t>
   </si>
   <si>
+    <t>25E0403</t>
+  </si>
+  <si>
     <t>PAMALS</t>
   </si>
   <si>
@@ -129,6 +153,9 @@
     <t>2048 20YJ 21EM 219C 20SP 20X7 2000</t>
   </si>
   <si>
+    <t>20SP</t>
+  </si>
+  <si>
     <t>67101.001510/2024-12</t>
   </si>
   <si>
@@ -138,19 +165,25 @@
     <t>VEE ONE-MANUTENCAO E SERVICOS TECNICOS LTDA</t>
   </si>
   <si>
-    <t>2025NE000369</t>
-  </si>
-  <si>
-    <t>C25516</t>
-  </si>
-  <si>
-    <t>25E0387</t>
-  </si>
-  <si>
-    <t>2025NE000371</t>
-  </si>
-  <si>
-    <t>25E0389</t>
+    <t>2025NE000414</t>
+  </si>
+  <si>
+    <t>C25525</t>
+  </si>
+  <si>
+    <t>25E0431</t>
+  </si>
+  <si>
+    <t>21EM</t>
+  </si>
+  <si>
+    <t>2025NE000559</t>
+  </si>
+  <si>
+    <t>C25545</t>
+  </si>
+  <si>
+    <t>25E0524</t>
   </si>
   <si>
     <t>Módulo</t>
@@ -159,33 +192,30 @@
     <t>Referência</t>
   </si>
   <si>
+    <t>20X7</t>
+  </si>
+  <si>
     <t>Nº recibo</t>
   </si>
   <si>
-    <t>2025NE000413</t>
-  </si>
-  <si>
-    <t>C25501</t>
-  </si>
-  <si>
     <t>Nº</t>
   </si>
   <si>
-    <t>25E0403</t>
-  </si>
-  <si>
     <t>Data</t>
   </si>
   <si>
     <t>Empenho</t>
   </si>
   <si>
-    <t>20SP</t>
+    <t>2025NE000770</t>
   </si>
   <si>
     <t>Observações</t>
   </si>
   <si>
+    <t>25E0731</t>
+  </si>
+  <si>
     <t>Vencimento</t>
   </si>
   <si>
@@ -195,37 +225,34 @@
     <t>Ordem de Pagamento</t>
   </si>
   <si>
-    <t>2025NE000414</t>
-  </si>
-  <si>
     <t>Faturado</t>
   </si>
   <si>
-    <t>C25525</t>
-  </si>
-  <si>
-    <t>25E0431</t>
-  </si>
-  <si>
     <t>Pendente</t>
   </si>
   <si>
-    <t>21EM</t>
+    <t>2025NE000774</t>
+  </si>
+  <si>
+    <t>25E0737</t>
   </si>
   <si>
     <t>FEV/25</t>
   </si>
   <si>
-    <t>2025NE000559</t>
-  </si>
-  <si>
     <t>-</t>
   </si>
   <si>
-    <t>C25545</t>
-  </si>
-  <si>
-    <t>25E0524</t>
+    <t>2025NE000843</t>
+  </si>
+  <si>
+    <t>C25630</t>
+  </si>
+  <si>
+    <t>25E0787</t>
+  </si>
+  <si>
+    <t>219C</t>
   </si>
   <si>
     <t xml:space="preserve">2025NE000369 </t>
@@ -234,103 +261,103 @@
     <t>2025NP001980</t>
   </si>
   <si>
-    <t>20X7</t>
-  </si>
-  <si>
-    <t>2025NE000770</t>
-  </si>
-  <si>
-    <t>25E0731</t>
-  </si>
-  <si>
-    <t>2025NE000774</t>
-  </si>
-  <si>
-    <t>25E0737</t>
-  </si>
-  <si>
-    <t>2025NE000843</t>
-  </si>
-  <si>
-    <t>C25630</t>
-  </si>
-  <si>
-    <t>25E0787</t>
+    <t>2025NE001065</t>
+  </si>
+  <si>
+    <t>25E0999</t>
+  </si>
+  <si>
+    <t>2025NE001200</t>
+  </si>
+  <si>
+    <t>C25590</t>
+  </si>
+  <si>
+    <t>25E1128</t>
+  </si>
+  <si>
+    <t>2025NE001598</t>
+  </si>
+  <si>
+    <t>C25814</t>
+  </si>
+  <si>
+    <t>25E1446</t>
   </si>
   <si>
     <t>MAR/25</t>
   </si>
   <si>
-    <t>219C</t>
+    <t>2025NE001627</t>
   </si>
   <si>
     <t>2025NE000367, 2025NE000369, 2025NE000371, 2025NE000413</t>
   </si>
   <si>
-    <t>2025NE001065</t>
-  </si>
-  <si>
-    <t>25E0999</t>
+    <t>25E1475</t>
   </si>
   <si>
     <t>2025NP001979</t>
   </si>
   <si>
+    <t>2025NE001629</t>
+  </si>
+  <si>
+    <t>C25820</t>
+  </si>
+  <si>
+    <t>25E1477</t>
+  </si>
+  <si>
     <t>ABR/25</t>
   </si>
   <si>
-    <t>2025NE001200</t>
-  </si>
-  <si>
-    <t>C25590</t>
-  </si>
-  <si>
-    <t>25E1128</t>
+    <t>2025NE001687</t>
   </si>
   <si>
     <t>2025NE000413, 2025NE000414, 2025NE000559</t>
   </si>
   <si>
-    <t>2025NE001598</t>
-  </si>
-  <si>
-    <t>C25814</t>
-  </si>
-  <si>
-    <t>25E1446</t>
+    <t>25E1535</t>
   </si>
   <si>
     <t>2025NP002341</t>
   </si>
   <si>
-    <t>2025NE001627</t>
+    <t>2025NE001688</t>
+  </si>
+  <si>
+    <t>25E1536</t>
   </si>
   <si>
     <t>MAI/25</t>
   </si>
   <si>
-    <t>25E1475</t>
-  </si>
-  <si>
-    <t>2025NE001629</t>
+    <t>2025NE001689</t>
+  </si>
+  <si>
+    <t>25E1537</t>
   </si>
   <si>
     <t>2025NP002884</t>
   </si>
   <si>
-    <t>C25820</t>
-  </si>
-  <si>
-    <t>25E1477</t>
+    <t>2025NE001690</t>
+  </si>
+  <si>
+    <t>25E1538</t>
   </si>
   <si>
     <t>JUN/25</t>
   </si>
   <si>
-    <t>2025NE001687</t>
-  </si>
-  <si>
-    <t>25E1535</t>
+    <t>2025NE001823</t>
+  </si>
+  <si>
+    <t>C25865</t>
+  </si>
+  <si>
+    <t>25E1666</t>
   </si>
   <si>
     <t>2025NE000005,
@@ -342,49 +369,73 @@
     <t>2025NP400522</t>
   </si>
   <si>
-    <t>2025NE001688</t>
-  </si>
-  <si>
-    <t>25E1536</t>
+    <t>2025NE001828</t>
+  </si>
+  <si>
+    <t>C25869</t>
+  </si>
+  <si>
+    <t>25E1667</t>
+  </si>
+  <si>
+    <t>20YJ</t>
   </si>
   <si>
     <t>JUL/25</t>
   </si>
   <si>
+    <t>2025NE001830</t>
+  </si>
+  <si>
+    <t>25E1669</t>
+  </si>
+  <si>
     <t>2025NE000843, 2025NE001200</t>
   </si>
   <si>
-    <t>2025NE001689</t>
+    <t>2025NE002200</t>
+  </si>
+  <si>
+    <t>C25863</t>
+  </si>
+  <si>
+    <t>25E2021</t>
   </si>
   <si>
     <t>2025NP003724</t>
   </si>
   <si>
-    <t>25E1537</t>
+    <t>2025NE002237</t>
+  </si>
+  <si>
+    <t>25E2058</t>
   </si>
   <si>
     <t>AGO/25</t>
   </si>
   <si>
-    <t>2025NE001690</t>
-  </si>
-  <si>
-    <t>25E1538</t>
+    <t>2026NE000330</t>
+  </si>
+  <si>
+    <t>C26163</t>
+  </si>
+  <si>
+    <t>26E0320</t>
   </si>
   <si>
     <t>2025NP004558</t>
   </si>
   <si>
-    <t>2025NE001823</t>
-  </si>
-  <si>
-    <t>C25865</t>
-  </si>
-  <si>
-    <t>25E1666</t>
-  </si>
-  <si>
     <t>SET/25</t>
+  </si>
+  <si>
+    <t>2026NE000388</t>
+  </si>
+  <si>
+    <t>C26193</t>
+  </si>
+  <si>
+    <t>26E0375</t>
   </si>
   <si>
     <t>2025NE001688 
@@ -394,43 +445,43 @@
     <t>2025NP004897</t>
   </si>
   <si>
-    <t>2025NE001828</t>
-  </si>
-  <si>
-    <t>C25869</t>
-  </si>
-  <si>
-    <t>25E1667</t>
+    <t>2026NE000748</t>
+  </si>
+  <si>
+    <t>C26312</t>
   </si>
   <si>
     <t>OUT/25</t>
   </si>
   <si>
-    <t>20YJ</t>
+    <t>26E0709</t>
   </si>
   <si>
     <t>2025NE001688, 2025NE001828, 2025NE002200</t>
   </si>
   <si>
-    <t>2025NE001830</t>
-  </si>
-  <si>
-    <t>25E1669</t>
-  </si>
-  <si>
     <t>2025NP004932</t>
   </si>
   <si>
+    <t>2026NE000816</t>
+  </si>
+  <si>
+    <t>C26324</t>
+  </si>
+  <si>
+    <t>26E0776</t>
+  </si>
+  <si>
     <t>NOV/25</t>
   </si>
   <si>
-    <t>2025NE002200</t>
-  </si>
-  <si>
-    <t>C25863</t>
-  </si>
-  <si>
-    <t>25E2021</t>
+    <t>2026NE000817</t>
+  </si>
+  <si>
+    <t>C26326</t>
+  </si>
+  <si>
+    <t>26E0777</t>
   </si>
   <si>
     <t>2025NE001687, 2025NE001689, 2025NE001690, 2025NE001823, 2025NE001830, 2025NE002237</t>
@@ -439,78 +490,48 @@
     <t>2026NP400440</t>
   </si>
   <si>
+    <t>2026NE000842</t>
+  </si>
+  <si>
+    <t>26E0803</t>
+  </si>
+  <si>
     <t>DEZ/25</t>
   </si>
   <si>
+    <t>2026NE000944</t>
+  </si>
+  <si>
     <t>2025NE001065, 2025NE002200</t>
   </si>
   <si>
+    <t>26E0906</t>
+  </si>
+  <si>
     <t>2026NP400412</t>
   </si>
   <si>
     <t>JAN/26</t>
   </si>
   <si>
-    <t>2025NE002237</t>
-  </si>
-  <si>
-    <t>25E2058</t>
-  </si>
-  <si>
     <t>2026NP401035</t>
   </si>
   <si>
-    <t>2026NE000330</t>
-  </si>
-  <si>
-    <t>C26163</t>
-  </si>
-  <si>
-    <t>26E0320</t>
-  </si>
-  <si>
-    <t>2026NE000388</t>
-  </si>
-  <si>
     <t>FEV/26</t>
   </si>
   <si>
-    <t>C26193</t>
-  </si>
-  <si>
-    <t>26E0375</t>
-  </si>
-  <si>
     <t>2025NE001627, 2025NE001629, 2025NE001823</t>
   </si>
   <si>
     <t>2026NP402272</t>
   </si>
   <si>
-    <t>2026NE000748</t>
-  </si>
-  <si>
-    <t>C26312</t>
-  </si>
-  <si>
-    <t>26E0709</t>
-  </si>
-  <si>
     <t>MAR/26</t>
   </si>
   <si>
     <t>2025NE000770, 2025NE001627</t>
   </si>
   <si>
-    <t>2026NE000816</t>
-  </si>
-  <si>
-    <t>C26324</t>
-  </si>
-  <si>
-    <t>26E0776</t>
-  </si>
-  <si>
     <t>R$ 1.350.542,52</t>
   </si>
   <si>
@@ -520,28 +541,7 @@
     <t>ABR/26</t>
   </si>
   <si>
-    <t>2026NE000817</t>
-  </si>
-  <si>
-    <t>C26326</t>
-  </si>
-  <si>
-    <t>26E0777</t>
-  </si>
-  <si>
     <t>2025NE000770, 2025NE001065, 2025NE001627</t>
-  </si>
-  <si>
-    <t>2026NE000842</t>
-  </si>
-  <si>
-    <t>26E0803</t>
-  </si>
-  <si>
-    <t>2026NE000944</t>
-  </si>
-  <si>
-    <t>26E0906</t>
   </si>
   <si>
     <t>REAJUSTE</t>
@@ -715,13 +715,13 @@
       <b/>
       <sz val="10.0"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Century Gothic"/>
     </font>
     <font>
       <b/>
       <sz val="10.0"/>
       <color theme="1"/>
-      <name val="Century Gothic"/>
+      <name val="Arial"/>
     </font>
     <font>
       <sz val="10.0"/>
@@ -866,15 +866,15 @@
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="3" fontId="2" numFmtId="0" xfId="0" applyFill="1" applyFont="1"/>
-    <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyFill="1" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyFill="1" applyFont="1"/>
     <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
@@ -888,11 +888,11 @@
     <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="center"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="4" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
@@ -931,28 +931,28 @@
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
+    <xf borderId="1" fillId="0" fontId="6" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="7" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment vertical="center"/>
     </xf>
     <xf borderId="2" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="6" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="7" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -967,17 +967,17 @@
     <xf borderId="1" fillId="7" fontId="9" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="165" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="1" fillId="5" fontId="9" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="8" fontId="6" numFmtId="168" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="8" fontId="7" numFmtId="168" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="3" fillId="0" fontId="10" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="1" fillId="8" fontId="9" numFmtId="168" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="165" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="1" fillId="0" fontId="8" numFmtId="166" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
@@ -993,14 +993,14 @@
     <xf borderId="1" fillId="8" fontId="9" numFmtId="168" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="6" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="7" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="170" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="170" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="1" fillId="9" fontId="9" numFmtId="168" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
@@ -1015,13 +1015,13 @@
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="4" fillId="0" fontId="10" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="1" fillId="0" fontId="6" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="7" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="6" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="7" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="6" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="7" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="5" fontId="9" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
@@ -1030,7 +1030,7 @@
     <xf borderId="1" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="6" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="7" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="5" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -1412,22 +1412,22 @@
       <c r="S1" s="1"/>
       <c r="T1" s="1"/>
       <c r="U1" s="1"/>
-      <c r="V1" s="3"/>
+      <c r="V1" s="5"/>
     </row>
     <row r="2" ht="59.25" customHeight="1">
-      <c r="A2" s="5"/>
+      <c r="A2" s="6"/>
       <c r="B2" s="8" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V2" s="10"/>
-      <c r="W2" s="12"/>
-      <c r="X2" s="12"/>
-      <c r="Y2" s="12"/>
-      <c r="Z2" s="12"/>
-      <c r="AA2" s="12"/>
-      <c r="AB2" s="12"/>
-      <c r="AC2" s="12"/>
-      <c r="AD2" s="12"/>
+      <c r="W2" s="11"/>
+      <c r="X2" s="11"/>
+      <c r="Y2" s="11"/>
+      <c r="Z2" s="11"/>
+      <c r="AA2" s="11"/>
+      <c r="AB2" s="11"/>
+      <c r="AC2" s="11"/>
+      <c r="AD2" s="11"/>
     </row>
     <row r="3" ht="12.75" customHeight="1">
       <c r="A3" s="1"/>
@@ -1451,85 +1451,85 @@
       <c r="S3" s="14"/>
       <c r="T3" s="14"/>
       <c r="U3" s="14"/>
-      <c r="V3" s="3"/>
+      <c r="V3" s="5"/>
     </row>
     <row r="4" ht="12.75" customHeight="1">
       <c r="A4" s="15"/>
       <c r="B4" s="15"/>
       <c r="C4" s="16" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D4" s="16" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="E4" s="16" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="F4" s="16" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="G4" s="17" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="H4" s="17" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="I4" s="16" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="J4" s="16" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="K4" s="16" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="L4" s="16" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="M4" s="17" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="N4" s="17" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="O4" s="17" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="P4" s="17" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="Q4" s="17" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="R4" s="16" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="S4" s="16" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="T4" s="16" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="U4" s="16" t="s">
-        <v>27</v>
-      </c>
-      <c r="V4" s="3"/>
+        <v>32</v>
+      </c>
+      <c r="V4" s="5"/>
     </row>
     <row r="5" ht="12.75" customHeight="1">
       <c r="A5" s="15"/>
       <c r="B5" s="15"/>
       <c r="C5" s="18"/>
       <c r="D5" s="19" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="E5" s="19" t="s">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="F5" s="19" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="G5" s="19" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="H5" s="20">
         <v>1564.0</v>
@@ -1538,16 +1538,16 @@
         <v>1564.0</v>
       </c>
       <c r="J5" s="19" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="K5" s="19" t="s">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="L5" s="19" t="s">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="M5" s="19" t="s">
-        <v>34</v>
+        <v>43</v>
       </c>
       <c r="N5" s="21">
         <v>9.165159737E7</v>
@@ -1565,15 +1565,15 @@
         <v>1.085943044E7</v>
       </c>
       <c r="S5" s="19" t="s">
-        <v>35</v>
-      </c>
-      <c r="V5" s="3"/>
+        <v>44</v>
+      </c>
+      <c r="V5" s="5"/>
     </row>
     <row r="6" ht="12.75" customHeight="1">
       <c r="A6" s="15"/>
       <c r="B6" s="15"/>
       <c r="L6" s="22"/>
-      <c r="V6" s="3"/>
+      <c r="V6" s="5"/>
     </row>
     <row r="7" ht="12.75" customHeight="1">
       <c r="A7" s="23"/>
@@ -1587,55 +1587,55 @@
       <c r="I7" s="25"/>
       <c r="J7" s="25"/>
       <c r="K7" s="25"/>
-      <c r="L7" s="26"/>
+      <c r="L7" s="27"/>
       <c r="M7" s="25"/>
       <c r="N7" s="25"/>
       <c r="O7" s="25"/>
-      <c r="P7" s="27"/>
-      <c r="V7" s="3"/>
+      <c r="P7" s="28"/>
+      <c r="V7" s="5"/>
     </row>
     <row r="8" ht="12.75" customHeight="1">
       <c r="A8" s="23"/>
       <c r="B8" s="23"/>
-      <c r="C8" s="28" t="s">
-        <v>41</v>
-      </c>
-      <c r="D8" s="28" t="s">
-        <v>42</v>
-      </c>
-      <c r="E8" s="29" t="s">
-        <v>43</v>
-      </c>
-      <c r="F8" s="28" t="s">
-        <v>46</v>
-      </c>
-      <c r="G8" s="28" t="s">
-        <v>48</v>
-      </c>
-      <c r="H8" s="28" t="s">
-        <v>49</v>
-      </c>
-      <c r="I8" s="29" t="s">
-        <v>51</v>
-      </c>
-      <c r="J8" s="28" t="s">
+      <c r="C8" s="29" t="s">
         <v>52</v>
       </c>
-      <c r="K8" s="28" t="s">
+      <c r="D8" s="29" t="s">
         <v>53</v>
       </c>
-      <c r="L8" s="30" t="s">
-        <v>54</v>
-      </c>
-      <c r="M8" s="29" t="s">
+      <c r="E8" s="30" t="s">
+        <v>55</v>
+      </c>
+      <c r="F8" s="29" t="s">
         <v>56</v>
       </c>
-      <c r="N8" s="28" t="s">
-        <v>59</v>
-      </c>
-      <c r="O8" s="28"/>
-      <c r="P8" s="27"/>
-      <c r="V8" s="3"/>
+      <c r="G8" s="29" t="s">
+        <v>57</v>
+      </c>
+      <c r="H8" s="29" t="s">
+        <v>58</v>
+      </c>
+      <c r="I8" s="30" t="s">
+        <v>60</v>
+      </c>
+      <c r="J8" s="29" t="s">
+        <v>62</v>
+      </c>
+      <c r="K8" s="29" t="s">
+        <v>63</v>
+      </c>
+      <c r="L8" s="31" t="s">
+        <v>64</v>
+      </c>
+      <c r="M8" s="30" t="s">
+        <v>65</v>
+      </c>
+      <c r="N8" s="29" t="s">
+        <v>66</v>
+      </c>
+      <c r="O8" s="29"/>
+      <c r="P8" s="28"/>
+      <c r="V8" s="5"/>
     </row>
     <row r="9" ht="19.5" customHeight="1">
       <c r="A9" s="23"/>
@@ -1644,10 +1644,10 @@
         <v>1.0</v>
       </c>
       <c r="D9" s="33" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="E9" s="34" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="F9" s="35">
         <v>594.0</v>
@@ -1656,7 +1656,7 @@
         <v>45740.0</v>
       </c>
       <c r="H9" s="35" t="s">
-        <v>66</v>
+        <v>75</v>
       </c>
       <c r="I9" s="36"/>
       <c r="J9" s="36">
@@ -1666,26 +1666,26 @@
         <v>748504.24</v>
       </c>
       <c r="L9" s="35" t="s">
-        <v>67</v>
-      </c>
-      <c r="M9" s="38">
+        <v>76</v>
+      </c>
+      <c r="M9" s="39">
         <f t="shared" ref="M9:M10" si="1">K9</f>
         <v>748504.24</v>
       </c>
-      <c r="N9" s="39"/>
+      <c r="N9" s="40"/>
       <c r="O9" s="25"/>
-      <c r="P9" s="27"/>
-      <c r="V9" s="3"/>
+      <c r="P9" s="28"/>
+      <c r="V9" s="5"/>
     </row>
     <row r="10" ht="51.0" customHeight="1">
       <c r="A10" s="23"/>
       <c r="B10" s="23"/>
-      <c r="C10" s="40"/>
+      <c r="C10" s="41"/>
       <c r="D10" s="33" t="s">
-        <v>76</v>
+        <v>85</v>
       </c>
       <c r="E10" s="34" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="F10" s="35">
         <v>620.0</v>
@@ -1694,7 +1694,7 @@
         <v>45775.0</v>
       </c>
       <c r="H10" s="35" t="s">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="I10" s="36"/>
       <c r="J10" s="36">
@@ -1704,26 +1704,26 @@
         <v>1110378.24</v>
       </c>
       <c r="L10" s="35" t="s">
-        <v>81</v>
-      </c>
-      <c r="M10" s="38">
+        <v>89</v>
+      </c>
+      <c r="M10" s="39">
         <f t="shared" si="1"/>
         <v>1110378.24</v>
       </c>
-      <c r="N10" s="41"/>
+      <c r="N10" s="42"/>
       <c r="O10" s="25"/>
-      <c r="P10" s="27"/>
-      <c r="V10" s="3"/>
+      <c r="P10" s="28"/>
+      <c r="V10" s="5"/>
     </row>
     <row r="11" ht="12.75" customHeight="1">
       <c r="A11" s="23"/>
       <c r="B11" s="23"/>
-      <c r="C11" s="40"/>
+      <c r="C11" s="41"/>
       <c r="D11" s="33" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="E11" s="34" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="F11" s="35">
         <v>634.0</v>
@@ -1732,7 +1732,7 @@
         <v>45799.0</v>
       </c>
       <c r="H11" s="35" t="s">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="I11" s="36"/>
       <c r="J11" s="36">
@@ -1742,25 +1742,25 @@
         <v>974557.12</v>
       </c>
       <c r="L11" s="34" t="s">
-        <v>90</v>
-      </c>
-      <c r="M11" s="38">
+        <v>97</v>
+      </c>
+      <c r="M11" s="39">
         <v>974557.12</v>
       </c>
-      <c r="N11" s="41"/>
+      <c r="N11" s="42"/>
       <c r="O11" s="25"/>
-      <c r="P11" s="27"/>
-      <c r="V11" s="3"/>
+      <c r="P11" s="28"/>
+      <c r="V11" s="5"/>
     </row>
     <row r="12" ht="27.75" customHeight="1">
       <c r="A12" s="23"/>
       <c r="B12" s="23"/>
-      <c r="C12" s="40"/>
+      <c r="C12" s="41"/>
       <c r="D12" s="33" t="s">
-        <v>92</v>
+        <v>100</v>
       </c>
       <c r="E12" s="34" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="F12" s="34">
         <v>660.0</v>
@@ -1769,7 +1769,7 @@
         <v>45856.0</v>
       </c>
       <c r="H12" s="44" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="I12" s="36"/>
       <c r="J12" s="36">
@@ -1779,25 +1779,25 @@
         <v>1402001.34</v>
       </c>
       <c r="L12" s="46" t="s">
-        <v>95</v>
-      </c>
-      <c r="M12" s="38">
+        <v>103</v>
+      </c>
+      <c r="M12" s="39">
         <v>1402001.34</v>
       </c>
       <c r="N12" s="47"/>
       <c r="O12" s="25"/>
-      <c r="P12" s="27"/>
-      <c r="V12" s="3"/>
+      <c r="P12" s="28"/>
+      <c r="V12" s="5"/>
     </row>
     <row r="13">
       <c r="A13" s="23"/>
       <c r="B13" s="23"/>
-      <c r="C13" s="40"/>
+      <c r="C13" s="41"/>
       <c r="D13" s="48" t="s">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="E13" s="34" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="F13" s="35">
         <v>661.0</v>
@@ -1806,7 +1806,7 @@
         <v>45856.0</v>
       </c>
       <c r="H13" s="35" t="s">
-        <v>101</v>
+        <v>110</v>
       </c>
       <c r="I13" s="43"/>
       <c r="J13" s="43">
@@ -1816,25 +1816,25 @@
         <v>1223702.3</v>
       </c>
       <c r="L13" s="34" t="s">
-        <v>102</v>
-      </c>
-      <c r="M13" s="38">
+        <v>111</v>
+      </c>
+      <c r="M13" s="39">
         <v>1223702.3</v>
       </c>
       <c r="N13" s="47"/>
       <c r="O13" s="25"/>
-      <c r="P13" s="49"/>
-      <c r="V13" s="3"/>
+      <c r="P13" s="50"/>
+      <c r="V13" s="5"/>
     </row>
     <row r="14">
       <c r="A14" s="23"/>
       <c r="B14" s="23"/>
-      <c r="C14" s="40"/>
+      <c r="C14" s="41"/>
       <c r="D14" s="48" t="s">
-        <v>105</v>
+        <v>116</v>
       </c>
       <c r="E14" s="34" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="F14" s="34">
         <v>688.0</v>
@@ -1843,7 +1843,7 @@
         <v>45901.0</v>
       </c>
       <c r="H14" s="34" t="s">
-        <v>106</v>
+        <v>119</v>
       </c>
       <c r="I14" s="43"/>
       <c r="J14" s="43">
@@ -1853,25 +1853,25 @@
         <v>1011677.95</v>
       </c>
       <c r="L14" s="34" t="s">
-        <v>108</v>
-      </c>
-      <c r="M14" s="38">
+        <v>123</v>
+      </c>
+      <c r="M14" s="39">
         <v>1011677.95</v>
       </c>
-      <c r="N14" s="41"/>
+      <c r="N14" s="42"/>
       <c r="O14" s="25"/>
-      <c r="P14" s="27"/>
-      <c r="V14" s="3"/>
+      <c r="P14" s="28"/>
+      <c r="V14" s="5"/>
     </row>
     <row r="15">
       <c r="A15" s="23"/>
       <c r="B15" s="23"/>
-      <c r="C15" s="40"/>
+      <c r="C15" s="41"/>
       <c r="D15" s="48" t="s">
-        <v>110</v>
+        <v>126</v>
       </c>
       <c r="E15" s="34" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="F15" s="34">
         <v>696.0</v>
@@ -1880,7 +1880,7 @@
         <v>45923.0</v>
       </c>
       <c r="H15" s="34" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="I15" s="43"/>
       <c r="J15" s="43">
@@ -1890,24 +1890,24 @@
         <v>896744.06</v>
       </c>
       <c r="L15" s="34" t="s">
-        <v>113</v>
-      </c>
-      <c r="M15" s="38">
+        <v>130</v>
+      </c>
+      <c r="M15" s="39">
         <v>896744.06</v>
       </c>
       <c r="N15" s="47"/>
       <c r="O15" s="25"/>
-      <c r="V15" s="3"/>
+      <c r="V15" s="5"/>
     </row>
     <row r="16">
       <c r="A16" s="23"/>
       <c r="B16" s="23"/>
-      <c r="C16" s="40"/>
+      <c r="C16" s="41"/>
       <c r="D16" s="48" t="s">
-        <v>117</v>
+        <v>131</v>
       </c>
       <c r="E16" s="34" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="F16" s="34">
         <v>704.0</v>
@@ -1916,7 +1916,7 @@
         <v>45957.0</v>
       </c>
       <c r="H16" s="34" t="s">
-        <v>118</v>
+        <v>135</v>
       </c>
       <c r="I16" s="43"/>
       <c r="J16" s="43">
@@ -1926,21 +1926,21 @@
         <v>919329.06</v>
       </c>
       <c r="L16" s="34" t="s">
-        <v>119</v>
-      </c>
-      <c r="M16" s="38">
+        <v>136</v>
+      </c>
+      <c r="M16" s="39">
         <v>919329.06</v>
       </c>
-      <c r="N16" s="41"/>
+      <c r="N16" s="42"/>
       <c r="O16" s="25"/>
-      <c r="V16" s="3"/>
+      <c r="V16" s="5"/>
     </row>
     <row r="17">
       <c r="A17" s="23"/>
       <c r="B17" s="23"/>
-      <c r="C17" s="40"/>
+      <c r="C17" s="41"/>
       <c r="D17" s="48" t="s">
-        <v>123</v>
+        <v>139</v>
       </c>
       <c r="E17" s="34"/>
       <c r="F17" s="34">
@@ -1950,7 +1950,7 @@
         <v>45972.0</v>
       </c>
       <c r="H17" s="34" t="s">
-        <v>125</v>
+        <v>141</v>
       </c>
       <c r="I17" s="34"/>
       <c r="J17" s="43">
@@ -1960,24 +1960,24 @@
         <v>1157009.26</v>
       </c>
       <c r="L17" s="34" t="s">
-        <v>128</v>
-      </c>
-      <c r="M17" s="38">
+        <v>142</v>
+      </c>
+      <c r="M17" s="39">
         <v>1157009.26</v>
       </c>
       <c r="N17" s="51"/>
       <c r="O17" s="25"/>
-      <c r="V17" s="3"/>
+      <c r="V17" s="5"/>
     </row>
     <row r="18">
       <c r="A18" s="23"/>
       <c r="B18" s="23"/>
-      <c r="C18" s="40"/>
+      <c r="C18" s="41"/>
       <c r="D18" s="48" t="s">
-        <v>129</v>
+        <v>146</v>
       </c>
       <c r="E18" s="34" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="F18" s="34">
         <v>728.0</v>
@@ -1986,7 +1986,7 @@
         <v>46008.0</v>
       </c>
       <c r="H18" s="34" t="s">
-        <v>133</v>
+        <v>150</v>
       </c>
       <c r="I18" s="34"/>
       <c r="J18" s="43">
@@ -1996,28 +1996,28 @@
         <v>1214597.952</v>
       </c>
       <c r="L18" s="34" t="s">
-        <v>134</v>
-      </c>
-      <c r="M18" s="38">
+        <v>151</v>
+      </c>
+      <c r="M18" s="39">
         <v>1214597.952</v>
       </c>
       <c r="N18" s="51"/>
       <c r="O18" s="25"/>
-      <c r="R18" s="27"/>
-      <c r="S18" s="27"/>
-      <c r="T18" s="27"/>
-      <c r="U18" s="27"/>
+      <c r="R18" s="28"/>
+      <c r="S18" s="28"/>
+      <c r="T18" s="28"/>
+      <c r="U18" s="28"/>
       <c r="V18" s="52"/>
     </row>
     <row r="19">
       <c r="A19" s="23"/>
       <c r="B19" s="23"/>
-      <c r="C19" s="40"/>
+      <c r="C19" s="41"/>
       <c r="D19" s="48" t="s">
-        <v>135</v>
+        <v>154</v>
       </c>
       <c r="E19" s="34" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="F19" s="34">
         <v>278.0</v>
@@ -2026,7 +2026,7 @@
         <v>46042.0</v>
       </c>
       <c r="H19" s="34" t="s">
-        <v>136</v>
+        <v>156</v>
       </c>
       <c r="I19" s="43"/>
       <c r="J19" s="43">
@@ -2036,25 +2036,25 @@
         <v>967082.09</v>
       </c>
       <c r="L19" s="34" t="s">
-        <v>137</v>
-      </c>
-      <c r="M19" s="38">
+        <v>158</v>
+      </c>
+      <c r="M19" s="39">
         <v>967082.09</v>
       </c>
       <c r="N19" s="51"/>
       <c r="O19" s="25"/>
-      <c r="R19" s="27"/>
-      <c r="S19" s="27"/>
-      <c r="T19" s="27"/>
-      <c r="U19" s="27"/>
+      <c r="R19" s="28"/>
+      <c r="S19" s="28"/>
+      <c r="T19" s="28"/>
+      <c r="U19" s="28"/>
       <c r="V19" s="52"/>
     </row>
     <row r="20">
       <c r="A20" s="23"/>
       <c r="B20" s="23"/>
-      <c r="C20" s="40"/>
+      <c r="C20" s="41"/>
       <c r="D20" s="48" t="s">
-        <v>138</v>
+        <v>159</v>
       </c>
       <c r="E20" s="34"/>
       <c r="F20" s="34">
@@ -2064,7 +2064,7 @@
         <v>46078.0</v>
       </c>
       <c r="H20" s="34" t="s">
-        <v>114</v>
+        <v>107</v>
       </c>
       <c r="I20" s="43"/>
       <c r="J20" s="43">
@@ -2074,25 +2074,25 @@
         <v>719561.08</v>
       </c>
       <c r="L20" s="34" t="s">
-        <v>141</v>
-      </c>
-      <c r="M20" s="38">
+        <v>160</v>
+      </c>
+      <c r="M20" s="39">
         <v>719561.08</v>
       </c>
       <c r="N20" s="51"/>
       <c r="O20" s="25"/>
-      <c r="R20" s="27"/>
-      <c r="S20" s="27"/>
-      <c r="T20" s="27"/>
-      <c r="U20" s="27"/>
+      <c r="R20" s="28"/>
+      <c r="S20" s="28"/>
+      <c r="T20" s="28"/>
+      <c r="U20" s="28"/>
       <c r="V20" s="52"/>
     </row>
     <row r="21">
       <c r="A21" s="23"/>
       <c r="B21" s="23"/>
-      <c r="C21" s="40"/>
+      <c r="C21" s="41"/>
       <c r="D21" s="48" t="s">
-        <v>146</v>
+        <v>161</v>
       </c>
       <c r="E21" s="34"/>
       <c r="F21" s="34">
@@ -2102,7 +2102,7 @@
         <v>46094.0</v>
       </c>
       <c r="H21" s="34" t="s">
-        <v>149</v>
+        <v>162</v>
       </c>
       <c r="I21" s="43"/>
       <c r="J21" s="43">
@@ -2112,25 +2112,25 @@
         <v>885881.08</v>
       </c>
       <c r="L21" s="34" t="s">
-        <v>150</v>
-      </c>
-      <c r="M21" s="38">
+        <v>163</v>
+      </c>
+      <c r="M21" s="39">
         <v>885881.08</v>
       </c>
       <c r="N21" s="51"/>
       <c r="O21" s="25"/>
-      <c r="R21" s="27"/>
-      <c r="S21" s="27"/>
-      <c r="T21" s="27"/>
-      <c r="U21" s="27"/>
+      <c r="R21" s="28"/>
+      <c r="S21" s="28"/>
+      <c r="T21" s="28"/>
+      <c r="U21" s="28"/>
       <c r="V21" s="52"/>
     </row>
     <row r="22">
       <c r="A22" s="23"/>
       <c r="B22" s="23"/>
-      <c r="C22" s="40"/>
+      <c r="C22" s="41"/>
       <c r="D22" s="48" t="s">
-        <v>154</v>
+        <v>164</v>
       </c>
       <c r="E22" s="34"/>
       <c r="F22" s="34">
@@ -2140,35 +2140,35 @@
         <v>46128.0</v>
       </c>
       <c r="H22" s="34" t="s">
-        <v>155</v>
+        <v>165</v>
       </c>
       <c r="I22" s="43"/>
       <c r="J22" s="43">
         <v>46164.0</v>
       </c>
       <c r="K22" s="45" t="s">
-        <v>159</v>
+        <v>166</v>
       </c>
       <c r="L22" s="34" t="s">
-        <v>160</v>
-      </c>
-      <c r="M22" s="38" t="s">
-        <v>159</v>
+        <v>167</v>
+      </c>
+      <c r="M22" s="39" t="s">
+        <v>166</v>
       </c>
       <c r="N22" s="51"/>
       <c r="O22" s="25"/>
-      <c r="R22" s="27"/>
-      <c r="S22" s="27"/>
-      <c r="T22" s="27"/>
-      <c r="U22" s="27"/>
+      <c r="R22" s="28"/>
+      <c r="S22" s="28"/>
+      <c r="T22" s="28"/>
+      <c r="U22" s="28"/>
       <c r="V22" s="52"/>
     </row>
     <row r="23">
       <c r="A23" s="23"/>
       <c r="B23" s="23"/>
-      <c r="C23" s="40"/>
+      <c r="C23" s="41"/>
       <c r="D23" s="48" t="s">
-        <v>161</v>
+        <v>168</v>
       </c>
       <c r="E23" s="34"/>
       <c r="F23" s="34">
@@ -2178,7 +2178,7 @@
         <v>46156.0</v>
       </c>
       <c r="H23" s="34" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="I23" s="43"/>
       <c r="J23" s="43">
@@ -2188,23 +2188,23 @@
         <v>1108954.4358333333</v>
       </c>
       <c r="L23" s="34" t="s">
-        <v>150</v>
-      </c>
-      <c r="M23" s="38">
+        <v>163</v>
+      </c>
+      <c r="M23" s="39">
         <v>1108954.4358333333</v>
       </c>
       <c r="N23" s="53"/>
       <c r="O23" s="25"/>
-      <c r="R23" s="27"/>
-      <c r="S23" s="27"/>
-      <c r="T23" s="27"/>
-      <c r="U23" s="27"/>
+      <c r="R23" s="28"/>
+      <c r="S23" s="28"/>
+      <c r="T23" s="28"/>
+      <c r="U23" s="28"/>
       <c r="V23" s="52"/>
     </row>
     <row r="24">
       <c r="A24" s="23"/>
       <c r="B24" s="23"/>
-      <c r="C24" s="40"/>
+      <c r="C24" s="41"/>
       <c r="D24" s="48" t="s">
         <v>170</v>
       </c>
@@ -2216,7 +2216,7 @@
         <v>46149.0</v>
       </c>
       <c r="H24" s="34" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="I24" s="43"/>
       <c r="J24" s="43">
@@ -2228,21 +2228,21 @@
       <c r="L24" s="34" t="s">
         <v>171</v>
       </c>
-      <c r="M24" s="38">
+      <c r="M24" s="39">
         <v>218206.1</v>
       </c>
       <c r="N24" s="54"/>
       <c r="O24" s="25"/>
-      <c r="R24" s="27"/>
-      <c r="S24" s="27"/>
-      <c r="T24" s="27"/>
-      <c r="U24" s="27"/>
+      <c r="R24" s="28"/>
+      <c r="S24" s="28"/>
+      <c r="T24" s="28"/>
+      <c r="U24" s="28"/>
       <c r="V24" s="52"/>
     </row>
     <row r="25">
       <c r="A25" s="23"/>
       <c r="B25" s="23"/>
-      <c r="C25" s="40"/>
+      <c r="C25" s="41"/>
       <c r="D25" s="48" t="s">
         <v>172</v>
       </c>
@@ -2254,7 +2254,7 @@
         <v>46156.0</v>
       </c>
       <c r="H25" s="34" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="I25" s="43"/>
       <c r="J25" s="43">
@@ -2266,15 +2266,15 @@
       <c r="L25" s="34" t="s">
         <v>173</v>
       </c>
-      <c r="M25" s="38">
+      <c r="M25" s="39">
         <v>1549250.84</v>
       </c>
       <c r="N25" s="54"/>
       <c r="O25" s="25"/>
-      <c r="R25" s="27"/>
-      <c r="S25" s="27"/>
-      <c r="T25" s="27"/>
-      <c r="U25" s="27"/>
+      <c r="R25" s="28"/>
+      <c r="S25" s="28"/>
+      <c r="T25" s="28"/>
+      <c r="U25" s="28"/>
       <c r="V25" s="52"/>
     </row>
     <row r="26">
@@ -2304,64 +2304,64 @@
       <c r="L26" s="34" t="s">
         <v>177</v>
       </c>
-      <c r="M26" s="38" t="s">
+      <c r="M26" s="39" t="s">
         <v>176</v>
       </c>
       <c r="N26" s="54"/>
       <c r="O26" s="25"/>
-      <c r="R26" s="27"/>
-      <c r="S26" s="27"/>
-      <c r="T26" s="27"/>
-      <c r="U26" s="27"/>
+      <c r="R26" s="28"/>
+      <c r="S26" s="28"/>
+      <c r="T26" s="28"/>
+      <c r="U26" s="28"/>
       <c r="V26" s="52"/>
     </row>
     <row r="27" ht="30.75" customHeight="1">
       <c r="A27" s="23"/>
       <c r="B27" s="23"/>
-      <c r="C27" s="28" t="s">
-        <v>41</v>
-      </c>
-      <c r="D27" s="28" t="s">
-        <v>42</v>
-      </c>
-      <c r="E27" s="29" t="s">
-        <v>43</v>
-      </c>
-      <c r="F27" s="28" t="s">
-        <v>46</v>
-      </c>
-      <c r="G27" s="28"/>
-      <c r="H27" s="28" t="s">
-        <v>49</v>
-      </c>
-      <c r="I27" s="28"/>
-      <c r="J27" s="28"/>
+      <c r="C27" s="29" t="s">
+        <v>52</v>
+      </c>
+      <c r="D27" s="29" t="s">
+        <v>53</v>
+      </c>
+      <c r="E27" s="30" t="s">
+        <v>55</v>
+      </c>
+      <c r="F27" s="29" t="s">
+        <v>56</v>
+      </c>
+      <c r="G27" s="29"/>
+      <c r="H27" s="29" t="s">
+        <v>58</v>
+      </c>
+      <c r="I27" s="29"/>
+      <c r="J27" s="29"/>
       <c r="K27" s="56" t="s">
-        <v>53</v>
-      </c>
-      <c r="L27" s="30" t="s">
-        <v>54</v>
+        <v>63</v>
+      </c>
+      <c r="L27" s="31" t="s">
+        <v>64</v>
       </c>
       <c r="M27" s="57" t="s">
-        <v>56</v>
-      </c>
-      <c r="N27" s="28" t="s">
-        <v>59</v>
+        <v>65</v>
+      </c>
+      <c r="N27" s="29" t="s">
+        <v>66</v>
       </c>
       <c r="O27" s="25"/>
-      <c r="P27" s="27"/>
-      <c r="R27" s="27"/>
-      <c r="S27" s="27"/>
-      <c r="T27" s="27"/>
-      <c r="U27" s="27"/>
+      <c r="P27" s="28"/>
+      <c r="R27" s="28"/>
+      <c r="S27" s="28"/>
+      <c r="T27" s="28"/>
+      <c r="U27" s="28"/>
       <c r="V27" s="52"/>
-      <c r="W27" s="27"/>
-      <c r="X27" s="27"/>
-      <c r="Y27" s="27"/>
-      <c r="Z27" s="27"/>
-      <c r="AA27" s="27"/>
-      <c r="AB27" s="27"/>
-      <c r="AC27" s="27"/>
+      <c r="W27" s="28"/>
+      <c r="X27" s="28"/>
+      <c r="Y27" s="28"/>
+      <c r="Z27" s="28"/>
+      <c r="AA27" s="28"/>
+      <c r="AB27" s="28"/>
+      <c r="AC27" s="28"/>
     </row>
     <row r="28" ht="12.75" customHeight="1">
       <c r="A28" s="23"/>
@@ -2380,7 +2380,7 @@
         <v>45791.0</v>
       </c>
       <c r="H28" s="35" t="s">
-        <v>62</v>
+        <v>49</v>
       </c>
       <c r="I28" s="36"/>
       <c r="J28" s="36">
@@ -2397,25 +2397,25 @@
       </c>
       <c r="N28" s="51"/>
       <c r="O28" s="25"/>
-      <c r="P28" s="27"/>
-      <c r="Q28" s="27"/>
-      <c r="R28" s="27"/>
-      <c r="S28" s="27"/>
-      <c r="T28" s="27"/>
-      <c r="U28" s="27"/>
+      <c r="P28" s="28"/>
+      <c r="Q28" s="28"/>
+      <c r="R28" s="28"/>
+      <c r="S28" s="28"/>
+      <c r="T28" s="28"/>
+      <c r="U28" s="28"/>
       <c r="V28" s="52"/>
-      <c r="W28" s="27"/>
-      <c r="X28" s="27"/>
-      <c r="Y28" s="27"/>
-      <c r="Z28" s="27"/>
-      <c r="AA28" s="27"/>
-      <c r="AB28" s="27"/>
-      <c r="AC28" s="27"/>
+      <c r="W28" s="28"/>
+      <c r="X28" s="28"/>
+      <c r="Y28" s="28"/>
+      <c r="Z28" s="28"/>
+      <c r="AA28" s="28"/>
+      <c r="AB28" s="28"/>
+      <c r="AC28" s="28"/>
     </row>
     <row r="29">
       <c r="A29" s="23"/>
       <c r="B29" s="23"/>
-      <c r="C29" s="40"/>
+      <c r="C29" s="41"/>
       <c r="D29" s="58" t="s">
         <v>180</v>
       </c>
@@ -2441,30 +2441,30 @@
       <c r="L29" s="34" t="s">
         <v>182</v>
       </c>
-      <c r="M29" s="38">
+      <c r="M29" s="39">
         <v>112720.77</v>
       </c>
       <c r="N29" s="51"/>
       <c r="O29" s="25"/>
-      <c r="P29" s="27"/>
-      <c r="Q29" s="27"/>
-      <c r="R29" s="27"/>
-      <c r="S29" s="27"/>
-      <c r="T29" s="27"/>
-      <c r="U29" s="27"/>
+      <c r="P29" s="28"/>
+      <c r="Q29" s="28"/>
+      <c r="R29" s="28"/>
+      <c r="S29" s="28"/>
+      <c r="T29" s="28"/>
+      <c r="U29" s="28"/>
       <c r="V29" s="52"/>
-      <c r="W29" s="27"/>
-      <c r="X29" s="27"/>
-      <c r="Y29" s="27"/>
-      <c r="Z29" s="27"/>
-      <c r="AA29" s="27"/>
-      <c r="AB29" s="27"/>
-      <c r="AC29" s="27"/>
+      <c r="W29" s="28"/>
+      <c r="X29" s="28"/>
+      <c r="Y29" s="28"/>
+      <c r="Z29" s="28"/>
+      <c r="AA29" s="28"/>
+      <c r="AB29" s="28"/>
+      <c r="AC29" s="28"/>
     </row>
     <row r="30" ht="12.75" customHeight="1">
       <c r="A30" s="23"/>
       <c r="B30" s="23"/>
-      <c r="C30" s="40"/>
+      <c r="C30" s="41"/>
       <c r="D30" s="61" t="s">
         <v>183</v>
       </c>
@@ -2478,7 +2478,7 @@
         <v>45853.0</v>
       </c>
       <c r="H30" s="34" t="s">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="I30" s="43"/>
       <c r="J30" s="43">
@@ -2490,30 +2490,30 @@
       <c r="L30" s="34" t="s">
         <v>185</v>
       </c>
-      <c r="M30" s="38">
+      <c r="M30" s="39">
         <v>378307.61</v>
       </c>
       <c r="N30" s="51"/>
       <c r="O30" s="25"/>
       <c r="P30" s="64"/>
-      <c r="Q30" s="27"/>
-      <c r="R30" s="27"/>
-      <c r="S30" s="27"/>
-      <c r="T30" s="27"/>
-      <c r="U30" s="27"/>
+      <c r="Q30" s="28"/>
+      <c r="R30" s="28"/>
+      <c r="S30" s="28"/>
+      <c r="T30" s="28"/>
+      <c r="U30" s="28"/>
       <c r="V30" s="52"/>
-      <c r="W30" s="27"/>
-      <c r="X30" s="27"/>
-      <c r="Y30" s="27"/>
-      <c r="Z30" s="27"/>
-      <c r="AA30" s="27"/>
-      <c r="AB30" s="27"/>
-      <c r="AC30" s="27"/>
+      <c r="W30" s="28"/>
+      <c r="X30" s="28"/>
+      <c r="Y30" s="28"/>
+      <c r="Z30" s="28"/>
+      <c r="AA30" s="28"/>
+      <c r="AB30" s="28"/>
+      <c r="AC30" s="28"/>
     </row>
     <row r="31" ht="60.0" customHeight="1">
       <c r="A31" s="23"/>
       <c r="B31" s="23"/>
-      <c r="C31" s="40"/>
+      <c r="C31" s="41"/>
       <c r="D31" s="61" t="s">
         <v>186</v>
       </c>
@@ -2527,7 +2527,7 @@
         <v>45910.0</v>
       </c>
       <c r="H31" s="34" t="s">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="I31" s="43"/>
       <c r="J31" s="43">
@@ -2539,30 +2539,30 @@
       <c r="L31" s="34" t="s">
         <v>187</v>
       </c>
-      <c r="M31" s="38">
+      <c r="M31" s="39">
         <v>3315.04710000003</v>
       </c>
       <c r="N31" s="51"/>
       <c r="O31" s="25"/>
       <c r="P31" s="64"/>
-      <c r="Q31" s="27"/>
-      <c r="R31" s="27"/>
-      <c r="S31" s="27"/>
-      <c r="T31" s="27"/>
-      <c r="U31" s="27"/>
+      <c r="Q31" s="28"/>
+      <c r="R31" s="28"/>
+      <c r="S31" s="28"/>
+      <c r="T31" s="28"/>
+      <c r="U31" s="28"/>
       <c r="V31" s="52"/>
-      <c r="W31" s="27"/>
-      <c r="X31" s="27"/>
-      <c r="Y31" s="27"/>
-      <c r="Z31" s="27"/>
-      <c r="AA31" s="27"/>
-      <c r="AB31" s="27"/>
-      <c r="AC31" s="27"/>
+      <c r="W31" s="28"/>
+      <c r="X31" s="28"/>
+      <c r="Y31" s="28"/>
+      <c r="Z31" s="28"/>
+      <c r="AA31" s="28"/>
+      <c r="AB31" s="28"/>
+      <c r="AC31" s="28"/>
     </row>
     <row r="32" ht="12.75" customHeight="1">
       <c r="A32" s="23"/>
       <c r="B32" s="23"/>
-      <c r="C32" s="40"/>
+      <c r="C32" s="41"/>
       <c r="D32" s="61" t="s">
         <v>188</v>
       </c>
@@ -2576,7 +2576,7 @@
         <v>45904.0</v>
       </c>
       <c r="H32" s="34" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="I32" s="66"/>
       <c r="J32" s="66">
@@ -2588,30 +2588,30 @@
       <c r="L32" s="34" t="s">
         <v>189</v>
       </c>
-      <c r="M32" s="38">
+      <c r="M32" s="39">
         <v>198332.75</v>
       </c>
       <c r="N32" s="51"/>
       <c r="O32" s="25"/>
       <c r="P32" s="64"/>
-      <c r="Q32" s="27"/>
-      <c r="R32" s="27"/>
-      <c r="S32" s="27"/>
-      <c r="T32" s="27"/>
-      <c r="U32" s="27"/>
+      <c r="Q32" s="28"/>
+      <c r="R32" s="28"/>
+      <c r="S32" s="28"/>
+      <c r="T32" s="28"/>
+      <c r="U32" s="28"/>
       <c r="V32" s="52"/>
-      <c r="W32" s="27"/>
-      <c r="X32" s="27"/>
-      <c r="Y32" s="27"/>
-      <c r="Z32" s="27"/>
-      <c r="AA32" s="27"/>
-      <c r="AB32" s="27"/>
-      <c r="AC32" s="27"/>
+      <c r="W32" s="28"/>
+      <c r="X32" s="28"/>
+      <c r="Y32" s="28"/>
+      <c r="Z32" s="28"/>
+      <c r="AA32" s="28"/>
+      <c r="AB32" s="28"/>
+      <c r="AC32" s="28"/>
     </row>
     <row r="33" ht="12.75" customHeight="1">
       <c r="A33" s="23"/>
       <c r="B33" s="23"/>
-      <c r="C33" s="40"/>
+      <c r="C33" s="41"/>
       <c r="D33" s="61" t="s">
         <v>190</v>
       </c>
@@ -2625,7 +2625,7 @@
         <v>46008.0</v>
       </c>
       <c r="H33" s="34" t="s">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="I33" s="66"/>
       <c r="J33" s="66">
@@ -2643,24 +2643,24 @@
       <c r="N33" s="51"/>
       <c r="O33" s="25"/>
       <c r="P33" s="64"/>
-      <c r="Q33" s="27"/>
-      <c r="R33" s="27"/>
-      <c r="S33" s="27"/>
-      <c r="T33" s="27"/>
-      <c r="U33" s="27"/>
+      <c r="Q33" s="28"/>
+      <c r="R33" s="28"/>
+      <c r="S33" s="28"/>
+      <c r="T33" s="28"/>
+      <c r="U33" s="28"/>
       <c r="V33" s="52"/>
-      <c r="W33" s="27"/>
-      <c r="X33" s="27"/>
-      <c r="Y33" s="27"/>
-      <c r="Z33" s="27"/>
-      <c r="AA33" s="27"/>
-      <c r="AB33" s="27"/>
-      <c r="AC33" s="27"/>
+      <c r="W33" s="28"/>
+      <c r="X33" s="28"/>
+      <c r="Y33" s="28"/>
+      <c r="Z33" s="28"/>
+      <c r="AA33" s="28"/>
+      <c r="AB33" s="28"/>
+      <c r="AC33" s="28"/>
     </row>
     <row r="34" ht="12.75" customHeight="1">
       <c r="A34" s="23"/>
       <c r="B34" s="23"/>
-      <c r="C34" s="40"/>
+      <c r="C34" s="41"/>
       <c r="D34" s="61" t="s">
         <v>193</v>
       </c>
@@ -2674,7 +2674,7 @@
         <v>45930.0</v>
       </c>
       <c r="H34" s="34" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="I34" s="66"/>
       <c r="J34" s="66">
@@ -2692,24 +2692,24 @@
       <c r="N34" s="51"/>
       <c r="O34" s="25"/>
       <c r="P34" s="64"/>
-      <c r="Q34" s="27"/>
-      <c r="R34" s="27"/>
-      <c r="S34" s="27"/>
-      <c r="T34" s="27"/>
-      <c r="U34" s="27"/>
+      <c r="Q34" s="28"/>
+      <c r="R34" s="28"/>
+      <c r="S34" s="28"/>
+      <c r="T34" s="28"/>
+      <c r="U34" s="28"/>
       <c r="V34" s="52"/>
-      <c r="W34" s="27"/>
-      <c r="X34" s="27"/>
-      <c r="Y34" s="27"/>
-      <c r="Z34" s="27"/>
-      <c r="AA34" s="27"/>
-      <c r="AB34" s="27"/>
-      <c r="AC34" s="27"/>
+      <c r="W34" s="28"/>
+      <c r="X34" s="28"/>
+      <c r="Y34" s="28"/>
+      <c r="Z34" s="28"/>
+      <c r="AA34" s="28"/>
+      <c r="AB34" s="28"/>
+      <c r="AC34" s="28"/>
     </row>
     <row r="35" ht="12.75" customHeight="1">
       <c r="A35" s="23"/>
       <c r="B35" s="23"/>
-      <c r="C35" s="40"/>
+      <c r="C35" s="41"/>
       <c r="D35" s="61" t="s">
         <v>197</v>
       </c>
@@ -2723,7 +2723,7 @@
         <v>45968.0</v>
       </c>
       <c r="H35" s="34" t="s">
-        <v>120</v>
+        <v>112</v>
       </c>
       <c r="I35" s="66"/>
       <c r="J35" s="66">
@@ -2741,24 +2741,24 @@
       <c r="N35" s="51"/>
       <c r="O35" s="25"/>
       <c r="P35" s="64"/>
-      <c r="Q35" s="27"/>
-      <c r="R35" s="27"/>
-      <c r="S35" s="27"/>
-      <c r="T35" s="27"/>
-      <c r="U35" s="27"/>
+      <c r="Q35" s="28"/>
+      <c r="R35" s="28"/>
+      <c r="S35" s="28"/>
+      <c r="T35" s="28"/>
+      <c r="U35" s="28"/>
       <c r="V35" s="52"/>
-      <c r="W35" s="27"/>
-      <c r="X35" s="27"/>
-      <c r="Y35" s="27"/>
-      <c r="Z35" s="27"/>
-      <c r="AA35" s="27"/>
-      <c r="AB35" s="27"/>
-      <c r="AC35" s="27"/>
+      <c r="W35" s="28"/>
+      <c r="X35" s="28"/>
+      <c r="Y35" s="28"/>
+      <c r="Z35" s="28"/>
+      <c r="AA35" s="28"/>
+      <c r="AB35" s="28"/>
+      <c r="AC35" s="28"/>
     </row>
     <row r="36" ht="12.75" customHeight="1">
       <c r="A36" s="23"/>
       <c r="B36" s="23"/>
-      <c r="C36" s="40"/>
+      <c r="C36" s="41"/>
       <c r="D36" s="61" t="s">
         <v>200</v>
       </c>
@@ -2772,7 +2772,7 @@
         <v>46043.0</v>
       </c>
       <c r="H36" s="65" t="s">
-        <v>114</v>
+        <v>107</v>
       </c>
       <c r="I36" s="70"/>
       <c r="J36" s="69">
@@ -2784,30 +2784,30 @@
       <c r="L36" s="34" t="s">
         <v>201</v>
       </c>
-      <c r="M36" s="38">
+      <c r="M36" s="39">
         <v>11372.9</v>
       </c>
       <c r="N36" s="51"/>
       <c r="O36" s="25"/>
-      <c r="P36" s="27"/>
-      <c r="Q36" s="27"/>
-      <c r="R36" s="27"/>
-      <c r="S36" s="27"/>
-      <c r="T36" s="27"/>
-      <c r="U36" s="27"/>
+      <c r="P36" s="28"/>
+      <c r="Q36" s="28"/>
+      <c r="R36" s="28"/>
+      <c r="S36" s="28"/>
+      <c r="T36" s="28"/>
+      <c r="U36" s="28"/>
       <c r="V36" s="52"/>
-      <c r="W36" s="27"/>
-      <c r="X36" s="27"/>
-      <c r="Y36" s="27"/>
-      <c r="Z36" s="27"/>
-      <c r="AA36" s="27"/>
-      <c r="AB36" s="27"/>
-      <c r="AC36" s="27"/>
+      <c r="W36" s="28"/>
+      <c r="X36" s="28"/>
+      <c r="Y36" s="28"/>
+      <c r="Z36" s="28"/>
+      <c r="AA36" s="28"/>
+      <c r="AB36" s="28"/>
+      <c r="AC36" s="28"/>
     </row>
     <row r="37" ht="12.75" customHeight="1">
       <c r="A37" s="23"/>
       <c r="B37" s="23"/>
-      <c r="C37" s="40"/>
+      <c r="C37" s="41"/>
       <c r="D37" s="61" t="s">
         <v>202</v>
       </c>
@@ -2821,25 +2821,25 @@
       <c r="J37" s="69"/>
       <c r="K37" s="45"/>
       <c r="L37" s="34"/>
-      <c r="M37" s="38"/>
+      <c r="M37" s="39"/>
       <c r="N37" s="51">
         <v>15854.78</v>
       </c>
       <c r="O37" s="25"/>
-      <c r="P37" s="27"/>
-      <c r="Q37" s="27"/>
-      <c r="R37" s="27"/>
-      <c r="S37" s="27"/>
-      <c r="T37" s="27"/>
-      <c r="U37" s="27"/>
+      <c r="P37" s="28"/>
+      <c r="Q37" s="28"/>
+      <c r="R37" s="28"/>
+      <c r="S37" s="28"/>
+      <c r="T37" s="28"/>
+      <c r="U37" s="28"/>
       <c r="V37" s="52"/>
-      <c r="W37" s="27"/>
-      <c r="X37" s="27"/>
-      <c r="Y37" s="27"/>
-      <c r="Z37" s="27"/>
-      <c r="AA37" s="27"/>
-      <c r="AB37" s="27"/>
-      <c r="AC37" s="27"/>
+      <c r="W37" s="28"/>
+      <c r="X37" s="28"/>
+      <c r="Y37" s="28"/>
+      <c r="Z37" s="28"/>
+      <c r="AA37" s="28"/>
+      <c r="AB37" s="28"/>
+      <c r="AC37" s="28"/>
     </row>
     <row r="38" ht="12.75" customHeight="1">
       <c r="A38" s="23"/>
@@ -2858,25 +2858,25 @@
       <c r="J38" s="69"/>
       <c r="K38" s="45"/>
       <c r="L38" s="34"/>
-      <c r="M38" s="38"/>
+      <c r="M38" s="39"/>
       <c r="N38" s="51" t="s">
         <v>205</v>
       </c>
       <c r="O38" s="25"/>
-      <c r="P38" s="27"/>
-      <c r="Q38" s="27"/>
-      <c r="R38" s="27"/>
-      <c r="S38" s="27"/>
-      <c r="T38" s="27"/>
-      <c r="U38" s="27"/>
+      <c r="P38" s="28"/>
+      <c r="Q38" s="28"/>
+      <c r="R38" s="28"/>
+      <c r="S38" s="28"/>
+      <c r="T38" s="28"/>
+      <c r="U38" s="28"/>
       <c r="V38" s="52"/>
-      <c r="W38" s="27"/>
-      <c r="X38" s="27"/>
-      <c r="Y38" s="27"/>
-      <c r="Z38" s="27"/>
-      <c r="AA38" s="27"/>
-      <c r="AB38" s="27"/>
-      <c r="AC38" s="27"/>
+      <c r="W38" s="28"/>
+      <c r="X38" s="28"/>
+      <c r="Y38" s="28"/>
+      <c r="Z38" s="28"/>
+      <c r="AA38" s="28"/>
+      <c r="AB38" s="28"/>
+      <c r="AC38" s="28"/>
     </row>
     <row r="39" ht="12.75" customHeight="1">
       <c r="A39" s="23"/>
@@ -2895,7 +2895,7 @@
         <v>46104.0</v>
       </c>
       <c r="H39" s="65" t="s">
-        <v>114</v>
+        <v>107</v>
       </c>
       <c r="I39" s="70"/>
       <c r="J39" s="69">
@@ -2912,25 +2912,25 @@
       </c>
       <c r="N39" s="51"/>
       <c r="O39" s="25"/>
-      <c r="P39" s="27"/>
-      <c r="Q39" s="27"/>
-      <c r="R39" s="27"/>
-      <c r="S39" s="27"/>
-      <c r="T39" s="27"/>
-      <c r="U39" s="27"/>
+      <c r="P39" s="28"/>
+      <c r="Q39" s="28"/>
+      <c r="R39" s="28"/>
+      <c r="S39" s="28"/>
+      <c r="T39" s="28"/>
+      <c r="U39" s="28"/>
       <c r="V39" s="52"/>
-      <c r="W39" s="27"/>
-      <c r="X39" s="27"/>
-      <c r="Y39" s="27"/>
-      <c r="Z39" s="27"/>
-      <c r="AA39" s="27"/>
-      <c r="AB39" s="27"/>
-      <c r="AC39" s="27"/>
+      <c r="W39" s="28"/>
+      <c r="X39" s="28"/>
+      <c r="Y39" s="28"/>
+      <c r="Z39" s="28"/>
+      <c r="AA39" s="28"/>
+      <c r="AB39" s="28"/>
+      <c r="AC39" s="28"/>
     </row>
     <row r="40" ht="12.75" customHeight="1">
       <c r="A40" s="15"/>
       <c r="B40" s="15"/>
-      <c r="C40" s="40"/>
+      <c r="C40" s="41"/>
       <c r="D40" s="61" t="s">
         <v>208</v>
       </c>
@@ -2942,7 +2942,7 @@
         <v>46199.0</v>
       </c>
       <c r="H40" s="65" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="I40" s="70"/>
       <c r="J40" s="69">
@@ -2952,53 +2952,53 @@
         <v>58868.35</v>
       </c>
       <c r="L40" s="34" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="M40" s="72">
         <v>58868.35</v>
       </c>
       <c r="N40" s="51"/>
-      <c r="V40" s="3"/>
+      <c r="V40" s="5"/>
     </row>
     <row r="41" ht="12.75" customHeight="1">
       <c r="A41" s="15"/>
       <c r="B41" s="15"/>
-      <c r="C41" s="40"/>
+      <c r="C41" s="41"/>
       <c r="K41" s="73"/>
       <c r="M41" s="73"/>
-      <c r="V41" s="3"/>
+      <c r="V41" s="5"/>
     </row>
     <row r="42" ht="12.75" customHeight="1">
       <c r="A42" s="15"/>
       <c r="B42" s="15"/>
-      <c r="C42" s="40"/>
+      <c r="C42" s="41"/>
       <c r="K42" s="73"/>
       <c r="M42" s="73"/>
-      <c r="V42" s="3"/>
+      <c r="V42" s="5"/>
     </row>
     <row r="43" ht="12.75" customHeight="1">
       <c r="A43" s="15"/>
       <c r="B43" s="15"/>
-      <c r="C43" s="40"/>
-      <c r="V43" s="3"/>
+      <c r="C43" s="41"/>
+      <c r="V43" s="5"/>
     </row>
     <row r="44" ht="12.75" customHeight="1">
       <c r="A44" s="15"/>
       <c r="B44" s="15"/>
-      <c r="C44" s="40"/>
-      <c r="V44" s="3"/>
+      <c r="C44" s="41"/>
+      <c r="V44" s="5"/>
     </row>
     <row r="45" ht="12.75" customHeight="1">
       <c r="A45" s="15"/>
       <c r="B45" s="15"/>
-      <c r="C45" s="40"/>
-      <c r="V45" s="3"/>
+      <c r="C45" s="41"/>
+      <c r="V45" s="5"/>
     </row>
     <row r="46" ht="12.75" customHeight="1">
       <c r="A46" s="15"/>
       <c r="B46" s="15"/>
-      <c r="C46" s="40"/>
-      <c r="V46" s="3"/>
+      <c r="C46" s="41"/>
+      <c r="V46" s="5"/>
     </row>
     <row r="47" ht="12.75" customHeight="1">
       <c r="A47" s="15"/>
@@ -3006,7 +3006,7 @@
       <c r="C47" s="55"/>
       <c r="K47" s="73"/>
       <c r="M47" s="73"/>
-      <c r="V47" s="3"/>
+      <c r="V47" s="5"/>
     </row>
     <row r="48" ht="12.75" customHeight="1">
       <c r="A48" s="15"/>
@@ -3030,7 +3030,7 @@
       <c r="S48" s="74"/>
       <c r="T48" s="74"/>
       <c r="U48" s="74"/>
-      <c r="V48" s="3"/>
+      <c r="V48" s="5"/>
     </row>
     <row r="49" ht="12.75" customHeight="1">
       <c r="A49" s="15"/>
@@ -7911,11 +7911,11 @@
       <c r="AH1" s="2"/>
     </row>
     <row r="2">
-      <c r="A2" s="4">
+      <c r="A2" s="3">
         <v>46212.0</v>
       </c>
-      <c r="L2" s="6" t="s">
-        <v>1</v>
+      <c r="L2" s="4" t="s">
+        <v>0</v>
       </c>
       <c r="AB2" s="2"/>
       <c r="AC2" s="2"/>
@@ -7938,7 +7938,7 @@
       <c r="D3" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="11">
+      <c r="E3" s="12">
         <v>45686.0</v>
       </c>
       <c r="F3" s="7" t="s">
@@ -7983,7 +7983,7 @@
       <c r="D4" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="11">
+      <c r="E4" s="12">
         <v>45762.0</v>
       </c>
       <c r="F4" s="7" t="s">
@@ -8017,18 +8017,18 @@
     </row>
     <row r="5">
       <c r="A5" s="7" t="s">
-        <v>36</v>
+        <v>9</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>37</v>
+        <v>10</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>38</v>
+        <v>11</v>
       </c>
       <c r="D5" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="E5" s="11">
+      <c r="E5" s="12">
         <v>45762.0</v>
       </c>
       <c r="F5" s="7" t="s">
@@ -8062,18 +8062,18 @@
     </row>
     <row r="6">
       <c r="A6" s="7" t="s">
-        <v>39</v>
+        <v>21</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>37</v>
+        <v>10</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>40</v>
+        <v>24</v>
       </c>
       <c r="D6" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="E6" s="11">
+      <c r="E6" s="12">
         <v>45762.0</v>
       </c>
       <c r="F6" s="7" t="s">
@@ -8107,18 +8107,18 @@
     </row>
     <row r="7">
       <c r="A7" s="7" t="s">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="D7" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="E7" s="11">
+      <c r="E7" s="12">
         <v>45763.0</v>
       </c>
       <c r="F7" s="7" t="s">
@@ -8131,7 +8131,7 @@
         <v>339039.0</v>
       </c>
       <c r="I7" s="7" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="J7" s="13">
         <v>949835.78</v>
@@ -8152,18 +8152,18 @@
     </row>
     <row r="8">
       <c r="A8" s="7" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>57</v>
+        <v>46</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>58</v>
+        <v>47</v>
       </c>
       <c r="D8" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="E8" s="11">
+      <c r="E8" s="12">
         <v>45763.0</v>
       </c>
       <c r="F8" s="7" t="s">
@@ -8176,7 +8176,7 @@
         <v>339039.0</v>
       </c>
       <c r="I8" s="7" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="J8" s="13">
         <v>524584.95</v>
@@ -8187,7 +8187,7 @@
       <c r="L8" s="7">
         <v>0.0</v>
       </c>
-      <c r="O8" s="31"/>
+      <c r="O8" s="26"/>
       <c r="AB8" s="2"/>
       <c r="AC8" s="2"/>
       <c r="AD8" s="2"/>
@@ -8198,18 +8198,18 @@
     </row>
     <row r="9">
       <c r="A9" s="7" t="s">
-        <v>62</v>
+        <v>49</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>64</v>
+        <v>50</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>65</v>
+        <v>51</v>
       </c>
       <c r="D9" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="E9" s="11">
+      <c r="E9" s="12">
         <v>45792.0</v>
       </c>
       <c r="F9" s="7" t="s">
@@ -8222,7 +8222,7 @@
         <v>339039.0</v>
       </c>
       <c r="I9" s="7" t="s">
-        <v>68</v>
+        <v>54</v>
       </c>
       <c r="J9" s="13">
         <v>211614.23</v>
@@ -8243,18 +8243,18 @@
     </row>
     <row r="10">
       <c r="A10" s="7" t="s">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="B10" s="7" t="s">
         <v>7</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="D10" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="E10" s="11">
+      <c r="E10" s="12">
         <v>45825.0</v>
       </c>
       <c r="F10" s="7" t="s">
@@ -8288,18 +8288,18 @@
     </row>
     <row r="11">
       <c r="A11" s="7" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>37</v>
+        <v>10</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="D11" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="E11" s="11">
+      <c r="E11" s="12">
         <v>45825.0</v>
       </c>
       <c r="F11" s="7" t="s">
@@ -8333,18 +8333,18 @@
     </row>
     <row r="12">
       <c r="A12" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="C12" s="7" t="s">
         <v>73</v>
-      </c>
-      <c r="B12" s="7" t="s">
-        <v>74</v>
-      </c>
-      <c r="C12" s="7" t="s">
-        <v>75</v>
       </c>
       <c r="D12" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="E12" s="11">
+      <c r="E12" s="12">
         <v>45832.0</v>
       </c>
       <c r="F12" s="7" t="s">
@@ -8357,7 +8357,7 @@
         <v>339039.0</v>
       </c>
       <c r="I12" s="7" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="J12" s="13">
         <v>1600334.09</v>
@@ -8378,18 +8378,18 @@
     </row>
     <row r="13">
       <c r="A13" s="7" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B13" s="7" t="s">
         <v>7</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="D13" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="E13" s="11">
+      <c r="E13" s="12">
         <v>45863.0</v>
       </c>
       <c r="F13" s="7" t="s">
@@ -8413,7 +8413,7 @@
       <c r="L13" s="13">
         <v>0.0</v>
       </c>
-      <c r="M13" s="42"/>
+      <c r="M13" s="38"/>
       <c r="AB13" s="2"/>
       <c r="AC13" s="2"/>
       <c r="AD13" s="2"/>
@@ -8424,18 +8424,18 @@
     </row>
     <row r="14">
       <c r="A14" s="7" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="D14" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="E14" s="11">
+      <c r="E14" s="12">
         <v>45887.0</v>
       </c>
       <c r="F14" s="7" t="s">
@@ -8448,7 +8448,7 @@
         <v>339039.0</v>
       </c>
       <c r="I14" s="7" t="s">
-        <v>68</v>
+        <v>54</v>
       </c>
       <c r="J14" s="13">
         <v>968237.39</v>
@@ -8469,18 +8469,18 @@
     </row>
     <row r="15">
       <c r="A15" s="7" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="D15" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="E15" s="11">
+      <c r="E15" s="12">
         <v>45924.0</v>
       </c>
       <c r="F15" s="7" t="s">
@@ -8493,7 +8493,7 @@
         <v>339039.0</v>
       </c>
       <c r="I15" s="7" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="J15" s="13">
         <v>1011677.95</v>
@@ -8514,18 +8514,18 @@
     </row>
     <row r="16">
       <c r="A16" s="7" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="B16" s="7" t="s">
         <v>7</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="D16" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="E16" s="11">
+      <c r="E16" s="12">
         <v>45929.0</v>
       </c>
       <c r="F16" s="7" t="s">
@@ -8559,18 +8559,18 @@
     </row>
     <row r="17">
       <c r="A17" s="7" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="D17" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="E17" s="11">
+      <c r="E17" s="12">
         <v>45930.0</v>
       </c>
       <c r="F17" s="7" t="s">
@@ -8604,18 +8604,18 @@
     </row>
     <row r="18">
       <c r="A18" s="7" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="D18" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="E18" s="11">
+      <c r="E18" s="12">
         <v>45938.0</v>
       </c>
       <c r="F18" s="7" t="s">
@@ -8628,7 +8628,7 @@
         <v>339039.0</v>
       </c>
       <c r="I18" s="7" t="s">
-        <v>68</v>
+        <v>54</v>
       </c>
       <c r="J18" s="13">
         <v>63746.85</v>
@@ -8649,18 +8649,18 @@
     </row>
     <row r="19">
       <c r="A19" s="7" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="D19" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="E19" s="11">
+      <c r="E19" s="12">
         <v>45938.0</v>
       </c>
       <c r="F19" s="7" t="s">
@@ -8673,7 +8673,7 @@
         <v>339039.0</v>
       </c>
       <c r="I19" s="7" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="J19" s="13">
         <v>947931.1</v>
@@ -8694,18 +8694,18 @@
     </row>
     <row r="20">
       <c r="A20" s="7" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="B20" s="7" t="s">
         <v>7</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>109</v>
+        <v>102</v>
       </c>
       <c r="D20" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="E20" s="11">
+      <c r="E20" s="12">
         <v>45938.0</v>
       </c>
       <c r="F20" s="7" t="s">
@@ -8739,18 +8739,18 @@
     </row>
     <row r="21">
       <c r="A21" s="7" t="s">
-        <v>111</v>
+        <v>104</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>37</v>
+        <v>10</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>112</v>
+        <v>105</v>
       </c>
       <c r="D21" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="E21" s="11">
+      <c r="E21" s="12">
         <v>45938.0</v>
       </c>
       <c r="F21" s="7" t="s">
@@ -8784,18 +8784,18 @@
     </row>
     <row r="22">
       <c r="A22" s="7" t="s">
-        <v>114</v>
+        <v>107</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>116</v>
+        <v>109</v>
       </c>
       <c r="D22" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="E22" s="50">
+      <c r="E22" s="49">
         <v>45953.0</v>
       </c>
       <c r="F22" s="7" t="s">
@@ -8829,18 +8829,18 @@
     </row>
     <row r="23">
       <c r="A23" s="7" t="s">
-        <v>120</v>
+        <v>112</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
       <c r="D23" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="E23" s="50">
+      <c r="E23" s="49">
         <v>45953.0</v>
       </c>
       <c r="F23" s="7" t="s">
@@ -8853,7 +8853,7 @@
         <v>339039.0</v>
       </c>
       <c r="I23" s="7" t="s">
-        <v>124</v>
+        <v>115</v>
       </c>
       <c r="J23" s="13">
         <v>1000001.64</v>
@@ -8874,18 +8874,18 @@
     </row>
     <row r="24">
       <c r="A24" s="7" t="s">
-        <v>126</v>
+        <v>117</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>37</v>
+        <v>10</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>127</v>
+        <v>118</v>
       </c>
       <c r="D24" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="E24" s="50">
+      <c r="E24" s="49">
         <v>45953.0</v>
       </c>
       <c r="F24" s="7" t="s">
@@ -8919,18 +8919,18 @@
     </row>
     <row r="25">
       <c r="A25" s="7" t="s">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>131</v>
+        <v>121</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>132</v>
+        <v>122</v>
       </c>
       <c r="D25" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="E25" s="50">
+      <c r="E25" s="49">
         <v>45975.0</v>
       </c>
       <c r="F25" s="7" t="s">
@@ -8943,7 +8943,7 @@
         <v>339039.0</v>
       </c>
       <c r="I25" s="7" t="s">
-        <v>124</v>
+        <v>115</v>
       </c>
       <c r="J25" s="13">
         <v>1157673.06</v>
@@ -8964,18 +8964,18 @@
     </row>
     <row r="26">
       <c r="A26" s="7" t="s">
-        <v>139</v>
+        <v>124</v>
       </c>
       <c r="B26" s="7" t="s">
         <v>7</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>140</v>
+        <v>125</v>
       </c>
       <c r="D26" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="E26" s="50">
+      <c r="E26" s="49">
         <v>45989.0</v>
       </c>
       <c r="F26" s="7" t="s">
@@ -9009,18 +9009,18 @@
     </row>
     <row r="27">
       <c r="A27" s="7" t="s">
-        <v>142</v>
+        <v>127</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>143</v>
+        <v>128</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>144</v>
+        <v>129</v>
       </c>
       <c r="D27" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="E27" s="11">
+      <c r="E27" s="12">
         <v>46104.0</v>
       </c>
       <c r="F27" s="7" t="s">
@@ -9054,18 +9054,18 @@
     </row>
     <row r="28">
       <c r="A28" s="7" t="s">
-        <v>145</v>
+        <v>132</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>147</v>
+        <v>133</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>148</v>
+        <v>134</v>
       </c>
       <c r="D28" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="E28" s="11">
+      <c r="E28" s="12">
         <v>46120.0</v>
       </c>
       <c r="F28" s="7" t="s">
@@ -9078,7 +9078,7 @@
         <v>339039.0</v>
       </c>
       <c r="I28" s="7" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="J28" s="13">
         <v>1912292.52</v>
@@ -9099,18 +9099,18 @@
     </row>
     <row r="29">
       <c r="A29" s="7" t="s">
-        <v>151</v>
+        <v>137</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>152</v>
+        <v>138</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>153</v>
+        <v>140</v>
       </c>
       <c r="D29" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="E29" s="11">
+      <c r="E29" s="12">
         <v>46196.0</v>
       </c>
       <c r="F29" s="7" t="s">
@@ -9144,18 +9144,18 @@
     </row>
     <row r="30">
       <c r="A30" s="7" t="s">
-        <v>156</v>
+        <v>143</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>157</v>
+        <v>144</v>
       </c>
       <c r="C30" s="7" t="s">
-        <v>158</v>
+        <v>145</v>
       </c>
       <c r="D30" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="E30" s="11">
+      <c r="E30" s="12">
         <v>46205.0</v>
       </c>
       <c r="F30" s="7" t="s">
@@ -9168,7 +9168,7 @@
         <v>339039.0</v>
       </c>
       <c r="I30" s="7" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="J30" s="13">
         <v>624166.14</v>
@@ -9189,18 +9189,18 @@
     </row>
     <row r="31">
       <c r="A31" s="7" t="s">
-        <v>162</v>
+        <v>147</v>
       </c>
       <c r="B31" s="7" t="s">
-        <v>163</v>
+        <v>148</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>164</v>
+        <v>149</v>
       </c>
       <c r="D31" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="E31" s="11">
+      <c r="E31" s="12">
         <v>46205.0</v>
       </c>
       <c r="F31" s="7" t="s">
@@ -9213,7 +9213,7 @@
         <v>339039.0</v>
       </c>
       <c r="I31" s="7" t="s">
-        <v>124</v>
+        <v>115</v>
       </c>
       <c r="J31" s="13">
         <v>18462.36</v>
@@ -9234,18 +9234,18 @@
     </row>
     <row r="32">
       <c r="A32" s="7" t="s">
-        <v>166</v>
+        <v>152</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>163</v>
+        <v>148</v>
       </c>
       <c r="C32" s="13" t="s">
-        <v>167</v>
+        <v>153</v>
       </c>
       <c r="D32" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="E32" s="11">
+      <c r="E32" s="12">
         <v>46213.0</v>
       </c>
       <c r="F32" s="7" t="s">
@@ -9258,7 +9258,7 @@
         <v>339039.0</v>
       </c>
       <c r="I32" s="7" t="s">
-        <v>124</v>
+        <v>115</v>
       </c>
       <c r="J32" s="13">
         <v>1530656.62</v>
@@ -9279,18 +9279,18 @@
     </row>
     <row r="33">
       <c r="A33" s="7" t="s">
-        <v>168</v>
+        <v>155</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>152</v>
+        <v>138</v>
       </c>
       <c r="C33" s="13" t="s">
-        <v>169</v>
+        <v>157</v>
       </c>
       <c r="D33" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="E33" s="11">
+      <c r="E33" s="12">
         <v>46227.0</v>
       </c>
       <c r="F33" s="7" t="s">

</xml_diff>

<commit_message>
Atualização automática: pagamentos (05/08/2026 15:41)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/01_Bases_Originais/005_CELOG_2025/005_CELOG-PAMALS_2025 online.xlsx
+++ b/Contrato 005/Dashboard/01_Bases_Originais/005_CELOG_2025/005_CELOG-PAMALS_2025 online.xlsx
@@ -57,30 +57,30 @@
     <t>25E0385</t>
   </si>
   <si>
+    <t>Número Contrato</t>
+  </si>
+  <si>
+    <t>UG Executora</t>
+  </si>
+  <si>
+    <t>UG Responsável</t>
+  </si>
+  <si>
     <t>2025NE000369</t>
   </si>
   <si>
+    <t>UG Fiscalizadora</t>
+  </si>
+  <si>
     <t>C25516</t>
   </si>
   <si>
+    <t>Prazo Final de Execução</t>
+  </si>
+  <si>
     <t>25E0387</t>
   </si>
   <si>
-    <t>Número Contrato</t>
-  </si>
-  <si>
-    <t>UG Executora</t>
-  </si>
-  <si>
-    <t>UG Responsável</t>
-  </si>
-  <si>
-    <t>UG Fiscalizadora</t>
-  </si>
-  <si>
-    <t>Prazo Final de Execução</t>
-  </si>
-  <si>
     <t>Prazo Final de Vigência</t>
   </si>
   <si>
@@ -93,75 +93,75 @@
     <t>PAG</t>
   </si>
   <si>
+    <t>Moeda</t>
+  </si>
+  <si>
+    <t>Valor Total do Contrato</t>
+  </si>
+  <si>
+    <t>Valor a Empenhar</t>
+  </si>
+  <si>
+    <t>Valor Empenhado</t>
+  </si>
+  <si>
+    <t>Valor Liquidado</t>
+  </si>
+  <si>
+    <t>Saldo (Valor a Faturar)</t>
+  </si>
+  <si>
+    <t>Fornecedor</t>
+  </si>
+  <si>
     <t>2025NE000371</t>
   </si>
   <si>
-    <t>Moeda</t>
-  </si>
-  <si>
-    <t>Valor Total do Contrato</t>
+    <t>Tipo Despesa /Receita</t>
+  </si>
+  <si>
+    <t>Abrir</t>
   </si>
   <si>
     <t>25E0389</t>
   </si>
   <si>
-    <t>Valor a Empenhar</t>
-  </si>
-  <si>
-    <t>Valor Empenhado</t>
-  </si>
-  <si>
-    <t>Valor Liquidado</t>
-  </si>
-  <si>
-    <t>Saldo (Valor a Faturar)</t>
-  </si>
-  <si>
-    <t>Fornecedor</t>
-  </si>
-  <si>
-    <t>Tipo Despesa /Receita</t>
-  </si>
-  <si>
-    <t>Abrir</t>
-  </si>
-  <si>
     <t>Editar</t>
   </si>
   <si>
+    <t>005/CELOG-PAMALS/2025</t>
+  </si>
+  <si>
+    <t>CELOG</t>
+  </si>
+  <si>
+    <t>PAMALS</t>
+  </si>
+  <si>
+    <t>Vigente</t>
+  </si>
+  <si>
+    <t>2048 20YJ 21EM 219C 20SP 20X7 2000</t>
+  </si>
+  <si>
+    <t>67101.001510/2024-12</t>
+  </si>
+  <si>
     <t>2025NE000413</t>
   </si>
   <si>
-    <t>005/CELOG-PAMALS/2025</t>
+    <t>R$</t>
   </si>
   <si>
     <t>C25501</t>
   </si>
   <si>
-    <t>CELOG</t>
-  </si>
-  <si>
     <t>25E0403</t>
   </si>
   <si>
-    <t>PAMALS</t>
-  </si>
-  <si>
-    <t>Vigente</t>
-  </si>
-  <si>
-    <t>2048 20YJ 21EM 219C 20SP 20X7 2000</t>
-  </si>
-  <si>
     <t>20SP</t>
   </si>
   <si>
-    <t>67101.001510/2024-12</t>
-  </si>
-  <si>
-    <t>R$</t>
-  </si>
-  <si>
     <t>VEE ONE-MANUTENCAO E SERVICOS TECNICOS LTDA</t>
   </si>
   <si>
@@ -186,13 +186,19 @@
     <t>25E0524</t>
   </si>
   <si>
+    <t>20X7</t>
+  </si>
+  <si>
     <t>Módulo</t>
   </si>
   <si>
     <t>Referência</t>
   </si>
   <si>
-    <t>20X7</t>
+    <t>2025NE000770</t>
+  </si>
+  <si>
+    <t>25E0731</t>
   </si>
   <si>
     <t>Nº recibo</t>
@@ -207,13 +213,13 @@
     <t>Empenho</t>
   </si>
   <si>
-    <t>2025NE000770</t>
+    <t>2025NE000774</t>
   </si>
   <si>
     <t>Observações</t>
   </si>
   <si>
-    <t>25E0731</t>
+    <t>25E0737</t>
   </si>
   <si>
     <t>Vencimento</t>
@@ -228,136 +234,190 @@
     <t>Faturado</t>
   </si>
   <si>
+    <t>2025NE000843</t>
+  </si>
+  <si>
+    <t>C25630</t>
+  </si>
+  <si>
     <t>Pendente</t>
   </si>
   <si>
-    <t>2025NE000774</t>
-  </si>
-  <si>
-    <t>25E0737</t>
+    <t>25E0787</t>
+  </si>
+  <si>
+    <t>219C</t>
+  </si>
+  <si>
+    <t>2025NE001065</t>
+  </si>
+  <si>
+    <t>25E0999</t>
   </si>
   <si>
     <t>FEV/25</t>
   </si>
   <si>
+    <t>2025NE001200</t>
+  </si>
+  <si>
     <t>-</t>
   </si>
   <si>
-    <t>2025NE000843</t>
-  </si>
-  <si>
-    <t>C25630</t>
-  </si>
-  <si>
-    <t>25E0787</t>
-  </si>
-  <si>
-    <t>219C</t>
+    <t>C25590</t>
+  </si>
+  <si>
+    <t>25E1128</t>
   </si>
   <si>
     <t xml:space="preserve">2025NE000369 </t>
   </si>
   <si>
+    <t>2025NE001598</t>
+  </si>
+  <si>
+    <t>C25814</t>
+  </si>
+  <si>
+    <t>25E1446</t>
+  </si>
+  <si>
     <t>2025NP001980</t>
   </si>
   <si>
-    <t>2025NE001065</t>
-  </si>
-  <si>
-    <t>25E0999</t>
-  </si>
-  <si>
-    <t>2025NE001200</t>
-  </si>
-  <si>
-    <t>C25590</t>
-  </si>
-  <si>
-    <t>25E1128</t>
-  </si>
-  <si>
-    <t>2025NE001598</t>
-  </si>
-  <si>
-    <t>C25814</t>
-  </si>
-  <si>
-    <t>25E1446</t>
+    <t>2025NE001627</t>
+  </si>
+  <si>
+    <t>25E1475</t>
+  </si>
+  <si>
+    <t>2025NE001629</t>
+  </si>
+  <si>
+    <t>C25820</t>
+  </si>
+  <si>
+    <t>25E1477</t>
+  </si>
+  <si>
+    <t>2025NE001687</t>
+  </si>
+  <si>
+    <t>25E1535</t>
+  </si>
+  <si>
+    <t>2025NE001688</t>
+  </si>
+  <si>
+    <t>25E1536</t>
   </si>
   <si>
     <t>MAR/25</t>
   </si>
   <si>
-    <t>2025NE001627</t>
+    <t>2025NE001689</t>
+  </si>
+  <si>
+    <t>25E1537</t>
   </si>
   <si>
     <t>2025NE000367, 2025NE000369, 2025NE000371, 2025NE000413</t>
   </si>
   <si>
-    <t>25E1475</t>
+    <t>2025NE001690</t>
   </si>
   <si>
     <t>2025NP001979</t>
   </si>
   <si>
-    <t>2025NE001629</t>
-  </si>
-  <si>
-    <t>C25820</t>
-  </si>
-  <si>
-    <t>25E1477</t>
+    <t>25E1538</t>
+  </si>
+  <si>
+    <t>2025NE001823</t>
+  </si>
+  <si>
+    <t>C25865</t>
+  </si>
+  <si>
+    <t>25E1666</t>
   </si>
   <si>
     <t>ABR/25</t>
   </si>
   <si>
-    <t>2025NE001687</t>
+    <t>2025NE001828</t>
+  </si>
+  <si>
+    <t>C25869</t>
+  </si>
+  <si>
+    <t>25E1667</t>
+  </si>
+  <si>
+    <t>20YJ</t>
   </si>
   <si>
     <t>2025NE000413, 2025NE000414, 2025NE000559</t>
   </si>
   <si>
-    <t>25E1535</t>
+    <t>2025NE001830</t>
+  </si>
+  <si>
+    <t>25E1669</t>
   </si>
   <si>
     <t>2025NP002341</t>
   </si>
   <si>
-    <t>2025NE001688</t>
-  </si>
-  <si>
-    <t>25E1536</t>
+    <t>2025NE002200</t>
+  </si>
+  <si>
+    <t>C25863</t>
+  </si>
+  <si>
+    <t>25E2021</t>
   </si>
   <si>
     <t>MAI/25</t>
   </si>
   <si>
-    <t>2025NE001689</t>
-  </si>
-  <si>
-    <t>25E1537</t>
+    <t>2025NE002237</t>
+  </si>
+  <si>
+    <t>25E2058</t>
+  </si>
+  <si>
+    <t>2026NE000330</t>
+  </si>
+  <si>
+    <t>C26163</t>
+  </si>
+  <si>
+    <t>26E0320</t>
   </si>
   <si>
     <t>2025NP002884</t>
   </si>
   <si>
-    <t>2025NE001690</t>
-  </si>
-  <si>
-    <t>25E1538</t>
+    <t>2026NE000388</t>
+  </si>
+  <si>
+    <t>C26193</t>
+  </si>
+  <si>
+    <t>26E0375</t>
+  </si>
+  <si>
+    <t>2026NE000748</t>
+  </si>
+  <si>
+    <t>C26312</t>
+  </si>
+  <si>
+    <t>26E0709</t>
   </si>
   <si>
     <t>JUN/25</t>
-  </si>
-  <si>
-    <t>2025NE001823</t>
-  </si>
-  <si>
-    <t>C25865</t>
-  </si>
-  <si>
-    <t>25E1666</t>
   </si>
   <si>
     <t>2025NE000005,
@@ -366,76 +426,55 @@
 2025NE000774</t>
   </si>
   <si>
+    <t>2026NE000816</t>
+  </si>
+  <si>
+    <t>C26324</t>
+  </si>
+  <si>
+    <t>26E0776</t>
+  </si>
+  <si>
     <t>2025NP400522</t>
   </si>
   <si>
-    <t>2025NE001828</t>
-  </si>
-  <si>
-    <t>C25869</t>
-  </si>
-  <si>
-    <t>25E1667</t>
-  </si>
-  <si>
-    <t>20YJ</t>
+    <t>2026NE000817</t>
+  </si>
+  <si>
+    <t>C26326</t>
+  </si>
+  <si>
+    <t>26E0777</t>
   </si>
   <si>
     <t>JUL/25</t>
   </si>
   <si>
-    <t>2025NE001830</t>
-  </si>
-  <si>
-    <t>25E1669</t>
-  </si>
-  <si>
     <t>2025NE000843, 2025NE001200</t>
   </si>
   <si>
-    <t>2025NE002200</t>
-  </si>
-  <si>
-    <t>C25863</t>
-  </si>
-  <si>
-    <t>25E2021</t>
-  </si>
-  <si>
     <t>2025NP003724</t>
   </si>
   <si>
-    <t>2025NE002237</t>
-  </si>
-  <si>
-    <t>25E2058</t>
+    <t>2026NE000842</t>
+  </si>
+  <si>
+    <t>26E0803</t>
   </si>
   <si>
     <t>AGO/25</t>
   </si>
   <si>
-    <t>2026NE000330</t>
-  </si>
-  <si>
-    <t>C26163</t>
-  </si>
-  <si>
-    <t>26E0320</t>
+    <t>2026NE000944</t>
+  </si>
+  <si>
+    <t>26E0906</t>
   </si>
   <si>
     <t>2025NP004558</t>
   </si>
   <si>
     <t>SET/25</t>
-  </si>
-  <si>
-    <t>2026NE000388</t>
-  </si>
-  <si>
-    <t>C26193</t>
-  </si>
-  <si>
-    <t>26E0375</t>
   </si>
   <si>
     <t>2025NE001688 
@@ -445,67 +484,28 @@
     <t>2025NP004897</t>
   </si>
   <si>
-    <t>2026NE000748</t>
-  </si>
-  <si>
-    <t>C26312</t>
-  </si>
-  <si>
     <t>OUT/25</t>
   </si>
   <si>
-    <t>26E0709</t>
-  </si>
-  <si>
     <t>2025NE001688, 2025NE001828, 2025NE002200</t>
   </si>
   <si>
     <t>2025NP004932</t>
   </si>
   <si>
-    <t>2026NE000816</t>
-  </si>
-  <si>
-    <t>C26324</t>
-  </si>
-  <si>
-    <t>26E0776</t>
-  </si>
-  <si>
     <t>NOV/25</t>
   </si>
   <si>
-    <t>2026NE000817</t>
-  </si>
-  <si>
-    <t>C26326</t>
-  </si>
-  <si>
-    <t>26E0777</t>
-  </si>
-  <si>
     <t>2025NE001687, 2025NE001689, 2025NE001690, 2025NE001823, 2025NE001830, 2025NE002237</t>
   </si>
   <si>
     <t>2026NP400440</t>
   </si>
   <si>
-    <t>2026NE000842</t>
-  </si>
-  <si>
-    <t>26E0803</t>
-  </si>
-  <si>
     <t>DEZ/25</t>
   </si>
   <si>
-    <t>2026NE000944</t>
-  </si>
-  <si>
     <t>2025NE001065, 2025NE002200</t>
-  </si>
-  <si>
-    <t>26E0906</t>
   </si>
   <si>
     <t>2026NP400412</t>
@@ -671,8 +671,8 @@
     <numFmt numFmtId="166" formatCode="dd/MM/yyyy"/>
     <numFmt numFmtId="167" formatCode="R$ #,##0.00"/>
     <numFmt numFmtId="168" formatCode="[$R$-416]\ #,##0.00;[RED]\-[$R$-416]\ #,##0.00"/>
-    <numFmt numFmtId="169" formatCode="MM/DD/YY"/>
-    <numFmt numFmtId="170" formatCode="d/m/yyyy"/>
+    <numFmt numFmtId="169" formatCode="d/m/yyyy"/>
+    <numFmt numFmtId="170" formatCode="MM/DD/YY"/>
     <numFmt numFmtId="171" formatCode="_([$R$ -416]* #,##0.00_);_([$R$ -416]* \(#,##0.00\);_([$R$ -416]* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="12">
@@ -866,24 +866,18 @@
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="3" fontId="2" numFmtId="0" xfId="0" applyFill="1" applyFont="1"/>
+    <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyFill="1" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyFill="1" applyFont="1"/>
-    <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
     <xf borderId="0" fillId="5" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="11" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="center"/>
@@ -891,13 +885,19 @@
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="11" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="4" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="4" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
@@ -952,6 +952,7 @@
     <xf borderId="2" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="165" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="1" fillId="0" fontId="7" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
@@ -967,7 +968,6 @@
     <xf borderId="1" fillId="7" fontId="9" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="165" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="1" fillId="5" fontId="9" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
@@ -978,10 +978,13 @@
     <xf borderId="1" fillId="8" fontId="9" numFmtId="168" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="169" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
     <xf borderId="1" fillId="0" fontId="8" numFmtId="166" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="8" numFmtId="169" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="8" numFmtId="170" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="7" fontId="9" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
@@ -995,9 +998,6 @@
     </xf>
     <xf borderId="1" fillId="0" fontId="7" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="170" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
@@ -1412,64 +1412,64 @@
       <c r="S1" s="1"/>
       <c r="T1" s="1"/>
       <c r="U1" s="1"/>
-      <c r="V1" s="5"/>
+      <c r="V1" s="3"/>
     </row>
     <row r="2" ht="59.25" customHeight="1">
-      <c r="A2" s="6"/>
-      <c r="B2" s="8" t="s">
+      <c r="A2" s="5"/>
+      <c r="B2" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="V2" s="10"/>
-      <c r="W2" s="11"/>
-      <c r="X2" s="11"/>
-      <c r="Y2" s="11"/>
-      <c r="Z2" s="11"/>
-      <c r="AA2" s="11"/>
-      <c r="AB2" s="11"/>
-      <c r="AC2" s="11"/>
-      <c r="AD2" s="11"/>
+      <c r="V2" s="8"/>
+      <c r="W2" s="9"/>
+      <c r="X2" s="9"/>
+      <c r="Y2" s="9"/>
+      <c r="Z2" s="9"/>
+      <c r="AA2" s="9"/>
+      <c r="AB2" s="9"/>
+      <c r="AC2" s="9"/>
+      <c r="AD2" s="9"/>
     </row>
     <row r="3" ht="12.75" customHeight="1">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
-      <c r="C3" s="14"/>
-      <c r="D3" s="14"/>
-      <c r="E3" s="14"/>
-      <c r="F3" s="14"/>
-      <c r="G3" s="14"/>
-      <c r="H3" s="14"/>
-      <c r="I3" s="14"/>
-      <c r="J3" s="14"/>
-      <c r="K3" s="14"/>
-      <c r="L3" s="14"/>
-      <c r="M3" s="14"/>
-      <c r="N3" s="14"/>
-      <c r="O3" s="14"/>
-      <c r="P3" s="14"/>
-      <c r="Q3" s="14"/>
-      <c r="R3" s="14"/>
-      <c r="S3" s="14"/>
-      <c r="T3" s="14"/>
-      <c r="U3" s="14"/>
-      <c r="V3" s="5"/>
+      <c r="C3" s="13"/>
+      <c r="D3" s="13"/>
+      <c r="E3" s="13"/>
+      <c r="F3" s="13"/>
+      <c r="G3" s="13"/>
+      <c r="H3" s="13"/>
+      <c r="I3" s="13"/>
+      <c r="J3" s="13"/>
+      <c r="K3" s="13"/>
+      <c r="L3" s="13"/>
+      <c r="M3" s="13"/>
+      <c r="N3" s="13"/>
+      <c r="O3" s="13"/>
+      <c r="P3" s="13"/>
+      <c r="Q3" s="13"/>
+      <c r="R3" s="13"/>
+      <c r="S3" s="13"/>
+      <c r="T3" s="13"/>
+      <c r="U3" s="13"/>
+      <c r="V3" s="3"/>
     </row>
     <row r="4" ht="12.75" customHeight="1">
       <c r="A4" s="15"/>
       <c r="B4" s="15"/>
       <c r="C4" s="16" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D4" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" s="16" t="s">
+        <v>11</v>
+      </c>
+      <c r="F4" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="E4" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="F4" s="16" t="s">
+      <c r="G4" s="17" t="s">
         <v>15</v>
-      </c>
-      <c r="G4" s="17" t="s">
-        <v>16</v>
       </c>
       <c r="H4" s="17" t="s">
         <v>17</v>
@@ -1484,52 +1484,52 @@
         <v>20</v>
       </c>
       <c r="L4" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="M4" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="M4" s="17" t="s">
+      <c r="N4" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="N4" s="17" t="s">
+      <c r="O4" s="17" t="s">
+        <v>24</v>
+      </c>
+      <c r="P4" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="O4" s="17" t="s">
+      <c r="Q4" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="P4" s="17" t="s">
+      <c r="R4" s="16" t="s">
         <v>27</v>
       </c>
-      <c r="Q4" s="17" t="s">
-        <v>28</v>
-      </c>
-      <c r="R4" s="16" t="s">
+      <c r="S4" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="S4" s="16" t="s">
+      <c r="T4" s="16" t="s">
         <v>30</v>
-      </c>
-      <c r="T4" s="16" t="s">
-        <v>31</v>
       </c>
       <c r="U4" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="V4" s="5"/>
+      <c r="V4" s="3"/>
     </row>
     <row r="5" ht="12.75" customHeight="1">
       <c r="A5" s="15"/>
       <c r="B5" s="15"/>
       <c r="C5" s="18"/>
       <c r="D5" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="E5" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="E5" s="19" t="s">
-        <v>36</v>
-      </c>
       <c r="F5" s="19" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="G5" s="19" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="H5" s="20">
         <v>1564.0</v>
@@ -1538,16 +1538,16 @@
         <v>1564.0</v>
       </c>
       <c r="J5" s="19" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="K5" s="19" t="s">
+        <v>37</v>
+      </c>
+      <c r="L5" s="19" t="s">
+        <v>38</v>
+      </c>
+      <c r="M5" s="19" t="s">
         <v>40</v>
-      </c>
-      <c r="L5" s="19" t="s">
-        <v>42</v>
-      </c>
-      <c r="M5" s="19" t="s">
-        <v>43</v>
       </c>
       <c r="N5" s="21">
         <v>9.165159737E7</v>
@@ -1567,13 +1567,13 @@
       <c r="S5" s="19" t="s">
         <v>44</v>
       </c>
-      <c r="V5" s="5"/>
+      <c r="V5" s="3"/>
     </row>
     <row r="6" ht="12.75" customHeight="1">
       <c r="A6" s="15"/>
       <c r="B6" s="15"/>
       <c r="L6" s="22"/>
-      <c r="V6" s="5"/>
+      <c r="V6" s="3"/>
     </row>
     <row r="7" ht="12.75" customHeight="1">
       <c r="A7" s="23"/>
@@ -1592,50 +1592,50 @@
       <c r="N7" s="25"/>
       <c r="O7" s="25"/>
       <c r="P7" s="28"/>
-      <c r="V7" s="5"/>
+      <c r="V7" s="3"/>
     </row>
     <row r="8" ht="12.75" customHeight="1">
       <c r="A8" s="23"/>
       <c r="B8" s="23"/>
       <c r="C8" s="29" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D8" s="29" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E8" s="30" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="F8" s="29" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="G8" s="29" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="H8" s="29" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="I8" s="30" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="J8" s="29" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="K8" s="29" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="L8" s="31" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="M8" s="30" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="N8" s="29" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="O8" s="29"/>
       <c r="P8" s="28"/>
-      <c r="V8" s="5"/>
+      <c r="V8" s="3"/>
     </row>
     <row r="9" ht="19.5" customHeight="1">
       <c r="A9" s="23"/>
@@ -1643,30 +1643,30 @@
       <c r="C9" s="32">
         <v>1.0</v>
       </c>
-      <c r="D9" s="33" t="s">
-        <v>69</v>
-      </c>
-      <c r="E9" s="34" t="s">
-        <v>70</v>
-      </c>
-      <c r="F9" s="35">
+      <c r="D9" s="34" t="s">
+        <v>75</v>
+      </c>
+      <c r="E9" s="35" t="s">
+        <v>77</v>
+      </c>
+      <c r="F9" s="36">
         <v>594.0</v>
       </c>
-      <c r="G9" s="36">
+      <c r="G9" s="37">
         <v>45740.0</v>
       </c>
-      <c r="H9" s="35" t="s">
-        <v>75</v>
-      </c>
-      <c r="I9" s="36"/>
-      <c r="J9" s="36">
+      <c r="H9" s="36" t="s">
+        <v>80</v>
+      </c>
+      <c r="I9" s="37"/>
+      <c r="J9" s="37">
         <v>45778.0</v>
       </c>
-      <c r="K9" s="37">
+      <c r="K9" s="38">
         <v>748504.24</v>
       </c>
-      <c r="L9" s="35" t="s">
-        <v>76</v>
+      <c r="L9" s="36" t="s">
+        <v>84</v>
       </c>
       <c r="M9" s="39">
         <f t="shared" ref="M9:M10" si="1">K9</f>
@@ -1675,36 +1675,36 @@
       <c r="N9" s="40"/>
       <c r="O9" s="25"/>
       <c r="P9" s="28"/>
-      <c r="V9" s="5"/>
+      <c r="V9" s="3"/>
     </row>
     <row r="10" ht="51.0" customHeight="1">
       <c r="A10" s="23"/>
       <c r="B10" s="23"/>
       <c r="C10" s="41"/>
-      <c r="D10" s="33" t="s">
-        <v>85</v>
-      </c>
-      <c r="E10" s="34" t="s">
-        <v>70</v>
-      </c>
-      <c r="F10" s="35">
+      <c r="D10" s="34" t="s">
+        <v>94</v>
+      </c>
+      <c r="E10" s="35" t="s">
+        <v>77</v>
+      </c>
+      <c r="F10" s="36">
         <v>620.0</v>
       </c>
-      <c r="G10" s="36">
+      <c r="G10" s="37">
         <v>45775.0</v>
       </c>
-      <c r="H10" s="35" t="s">
-        <v>87</v>
-      </c>
-      <c r="I10" s="36"/>
-      <c r="J10" s="36">
+      <c r="H10" s="36" t="s">
+        <v>97</v>
+      </c>
+      <c r="I10" s="37"/>
+      <c r="J10" s="37">
         <v>45806.0</v>
       </c>
-      <c r="K10" s="37">
+      <c r="K10" s="38">
         <v>1110378.24</v>
       </c>
-      <c r="L10" s="35" t="s">
-        <v>89</v>
+      <c r="L10" s="36" t="s">
+        <v>99</v>
       </c>
       <c r="M10" s="39">
         <f t="shared" si="1"/>
@@ -1713,36 +1713,36 @@
       <c r="N10" s="42"/>
       <c r="O10" s="25"/>
       <c r="P10" s="28"/>
-      <c r="V10" s="5"/>
+      <c r="V10" s="3"/>
     </row>
     <row r="11" ht="12.75" customHeight="1">
       <c r="A11" s="23"/>
       <c r="B11" s="23"/>
       <c r="C11" s="41"/>
-      <c r="D11" s="33" t="s">
-        <v>93</v>
-      </c>
-      <c r="E11" s="34" t="s">
-        <v>70</v>
-      </c>
-      <c r="F11" s="35">
+      <c r="D11" s="34" t="s">
+        <v>104</v>
+      </c>
+      <c r="E11" s="35" t="s">
+        <v>77</v>
+      </c>
+      <c r="F11" s="36">
         <v>634.0</v>
       </c>
-      <c r="G11" s="36">
+      <c r="G11" s="37">
         <v>45799.0</v>
       </c>
-      <c r="H11" s="35" t="s">
-        <v>95</v>
-      </c>
-      <c r="I11" s="36"/>
-      <c r="J11" s="36">
+      <c r="H11" s="36" t="s">
+        <v>109</v>
+      </c>
+      <c r="I11" s="37"/>
+      <c r="J11" s="37">
         <v>45844.0</v>
       </c>
-      <c r="K11" s="37">
+      <c r="K11" s="38">
         <v>974557.12</v>
       </c>
-      <c r="L11" s="34" t="s">
-        <v>97</v>
+      <c r="L11" s="35" t="s">
+        <v>112</v>
       </c>
       <c r="M11" s="39">
         <v>974557.12</v>
@@ -1750,110 +1750,110 @@
       <c r="N11" s="42"/>
       <c r="O11" s="25"/>
       <c r="P11" s="28"/>
-      <c r="V11" s="5"/>
+      <c r="V11" s="3"/>
     </row>
     <row r="12" ht="27.75" customHeight="1">
       <c r="A12" s="23"/>
       <c r="B12" s="23"/>
       <c r="C12" s="41"/>
-      <c r="D12" s="33" t="s">
-        <v>100</v>
-      </c>
-      <c r="E12" s="34" t="s">
-        <v>70</v>
-      </c>
-      <c r="F12" s="34">
+      <c r="D12" s="34" t="s">
+        <v>116</v>
+      </c>
+      <c r="E12" s="35" t="s">
+        <v>77</v>
+      </c>
+      <c r="F12" s="35">
         <v>660.0</v>
       </c>
-      <c r="G12" s="43">
+      <c r="G12" s="44">
         <v>45856.0</v>
       </c>
-      <c r="H12" s="44" t="s">
-        <v>71</v>
-      </c>
-      <c r="I12" s="36"/>
-      <c r="J12" s="36">
+      <c r="H12" s="45" t="s">
+        <v>68</v>
+      </c>
+      <c r="I12" s="37"/>
+      <c r="J12" s="37">
         <v>45891.0</v>
       </c>
-      <c r="K12" s="45">
+      <c r="K12" s="46">
         <v>1402001.34</v>
       </c>
-      <c r="L12" s="46" t="s">
-        <v>103</v>
+      <c r="L12" s="47" t="s">
+        <v>122</v>
       </c>
       <c r="M12" s="39">
         <v>1402001.34</v>
       </c>
-      <c r="N12" s="47"/>
+      <c r="N12" s="48"/>
       <c r="O12" s="25"/>
       <c r="P12" s="28"/>
-      <c r="V12" s="5"/>
+      <c r="V12" s="3"/>
     </row>
     <row r="13">
       <c r="A13" s="23"/>
       <c r="B13" s="23"/>
       <c r="C13" s="41"/>
-      <c r="D13" s="48" t="s">
-        <v>106</v>
-      </c>
-      <c r="E13" s="34" t="s">
-        <v>70</v>
-      </c>
-      <c r="F13" s="35">
+      <c r="D13" s="49" t="s">
+        <v>129</v>
+      </c>
+      <c r="E13" s="35" t="s">
+        <v>77</v>
+      </c>
+      <c r="F13" s="36">
         <v>661.0</v>
       </c>
-      <c r="G13" s="36">
+      <c r="G13" s="37">
         <v>45856.0</v>
       </c>
-      <c r="H13" s="35" t="s">
-        <v>110</v>
-      </c>
-      <c r="I13" s="43"/>
-      <c r="J13" s="43">
+      <c r="H13" s="36" t="s">
+        <v>130</v>
+      </c>
+      <c r="I13" s="44"/>
+      <c r="J13" s="44">
         <v>45891.0</v>
       </c>
-      <c r="K13" s="45">
+      <c r="K13" s="46">
         <v>1223702.3</v>
       </c>
-      <c r="L13" s="34" t="s">
-        <v>111</v>
+      <c r="L13" s="35" t="s">
+        <v>134</v>
       </c>
       <c r="M13" s="39">
         <v>1223702.3</v>
       </c>
-      <c r="N13" s="47"/>
+      <c r="N13" s="48"/>
       <c r="O13" s="25"/>
       <c r="P13" s="50"/>
-      <c r="V13" s="5"/>
+      <c r="V13" s="3"/>
     </row>
     <row r="14">
       <c r="A14" s="23"/>
       <c r="B14" s="23"/>
       <c r="C14" s="41"/>
-      <c r="D14" s="48" t="s">
-        <v>116</v>
-      </c>
-      <c r="E14" s="34" t="s">
-        <v>70</v>
-      </c>
-      <c r="F14" s="34">
+      <c r="D14" s="49" t="s">
+        <v>138</v>
+      </c>
+      <c r="E14" s="35" t="s">
+        <v>77</v>
+      </c>
+      <c r="F14" s="35">
         <v>688.0</v>
       </c>
-      <c r="G14" s="36">
+      <c r="G14" s="37">
         <v>45901.0</v>
       </c>
-      <c r="H14" s="34" t="s">
-        <v>119</v>
-      </c>
-      <c r="I14" s="43"/>
-      <c r="J14" s="43">
+      <c r="H14" s="35" t="s">
+        <v>139</v>
+      </c>
+      <c r="I14" s="44"/>
+      <c r="J14" s="44">
         <v>45938.0</v>
       </c>
-      <c r="K14" s="45">
+      <c r="K14" s="46">
         <v>1011677.95</v>
       </c>
-      <c r="L14" s="34" t="s">
-        <v>123</v>
+      <c r="L14" s="35" t="s">
+        <v>140</v>
       </c>
       <c r="M14" s="39">
         <v>1011677.95</v>
@@ -1861,142 +1861,142 @@
       <c r="N14" s="42"/>
       <c r="O14" s="25"/>
       <c r="P14" s="28"/>
-      <c r="V14" s="5"/>
+      <c r="V14" s="3"/>
     </row>
     <row r="15">
       <c r="A15" s="23"/>
       <c r="B15" s="23"/>
       <c r="C15" s="41"/>
-      <c r="D15" s="48" t="s">
-        <v>126</v>
-      </c>
-      <c r="E15" s="34" t="s">
-        <v>70</v>
-      </c>
-      <c r="F15" s="34">
+      <c r="D15" s="49" t="s">
+        <v>143</v>
+      </c>
+      <c r="E15" s="35" t="s">
+        <v>77</v>
+      </c>
+      <c r="F15" s="35">
         <v>696.0</v>
       </c>
-      <c r="G15" s="36">
+      <c r="G15" s="37">
         <v>45923.0</v>
       </c>
-      <c r="H15" s="34" t="s">
-        <v>79</v>
-      </c>
-      <c r="I15" s="43"/>
-      <c r="J15" s="43">
+      <c r="H15" s="35" t="s">
+        <v>76</v>
+      </c>
+      <c r="I15" s="44"/>
+      <c r="J15" s="44">
         <v>45938.0</v>
       </c>
-      <c r="K15" s="45">
+      <c r="K15" s="46">
         <v>896744.06</v>
       </c>
-      <c r="L15" s="34" t="s">
-        <v>130</v>
+      <c r="L15" s="35" t="s">
+        <v>146</v>
       </c>
       <c r="M15" s="39">
         <v>896744.06</v>
       </c>
-      <c r="N15" s="47"/>
+      <c r="N15" s="48"/>
       <c r="O15" s="25"/>
-      <c r="V15" s="5"/>
+      <c r="V15" s="3"/>
     </row>
     <row r="16">
       <c r="A16" s="23"/>
       <c r="B16" s="23"/>
       <c r="C16" s="41"/>
-      <c r="D16" s="48" t="s">
-        <v>131</v>
-      </c>
-      <c r="E16" s="34" t="s">
-        <v>70</v>
-      </c>
-      <c r="F16" s="34">
+      <c r="D16" s="49" t="s">
+        <v>147</v>
+      </c>
+      <c r="E16" s="35" t="s">
+        <v>77</v>
+      </c>
+      <c r="F16" s="35">
         <v>704.0</v>
       </c>
-      <c r="G16" s="36">
+      <c r="G16" s="37">
         <v>45957.0</v>
       </c>
-      <c r="H16" s="34" t="s">
-        <v>135</v>
-      </c>
-      <c r="I16" s="43"/>
-      <c r="J16" s="43">
+      <c r="H16" s="35" t="s">
+        <v>148</v>
+      </c>
+      <c r="I16" s="44"/>
+      <c r="J16" s="44">
         <v>46003.0</v>
       </c>
-      <c r="K16" s="45">
+      <c r="K16" s="46">
         <v>919329.06</v>
       </c>
-      <c r="L16" s="34" t="s">
-        <v>136</v>
+      <c r="L16" s="35" t="s">
+        <v>149</v>
       </c>
       <c r="M16" s="39">
         <v>919329.06</v>
       </c>
       <c r="N16" s="42"/>
       <c r="O16" s="25"/>
-      <c r="V16" s="5"/>
+      <c r="V16" s="3"/>
     </row>
     <row r="17">
       <c r="A17" s="23"/>
       <c r="B17" s="23"/>
       <c r="C17" s="41"/>
-      <c r="D17" s="48" t="s">
-        <v>139</v>
-      </c>
-      <c r="E17" s="34"/>
-      <c r="F17" s="34">
+      <c r="D17" s="49" t="s">
+        <v>150</v>
+      </c>
+      <c r="E17" s="35"/>
+      <c r="F17" s="35">
         <v>705.0</v>
       </c>
-      <c r="G17" s="43">
+      <c r="G17" s="44">
         <v>45972.0</v>
       </c>
-      <c r="H17" s="34" t="s">
-        <v>141</v>
-      </c>
-      <c r="I17" s="34"/>
-      <c r="J17" s="43">
+      <c r="H17" s="35" t="s">
+        <v>151</v>
+      </c>
+      <c r="I17" s="35"/>
+      <c r="J17" s="44">
         <v>46016.0</v>
       </c>
-      <c r="K17" s="45">
+      <c r="K17" s="46">
         <v>1157009.26</v>
       </c>
-      <c r="L17" s="34" t="s">
-        <v>142</v>
+      <c r="L17" s="35" t="s">
+        <v>152</v>
       </c>
       <c r="M17" s="39">
         <v>1157009.26</v>
       </c>
       <c r="N17" s="51"/>
       <c r="O17" s="25"/>
-      <c r="V17" s="5"/>
+      <c r="V17" s="3"/>
     </row>
     <row r="18">
       <c r="A18" s="23"/>
       <c r="B18" s="23"/>
       <c r="C18" s="41"/>
-      <c r="D18" s="48" t="s">
-        <v>146</v>
-      </c>
-      <c r="E18" s="34" t="s">
-        <v>70</v>
-      </c>
-      <c r="F18" s="34">
+      <c r="D18" s="49" t="s">
+        <v>153</v>
+      </c>
+      <c r="E18" s="35" t="s">
+        <v>77</v>
+      </c>
+      <c r="F18" s="35">
         <v>728.0</v>
       </c>
-      <c r="G18" s="43">
+      <c r="G18" s="44">
         <v>46008.0</v>
       </c>
-      <c r="H18" s="34" t="s">
-        <v>150</v>
-      </c>
-      <c r="I18" s="34"/>
-      <c r="J18" s="43">
+      <c r="H18" s="35" t="s">
+        <v>154</v>
+      </c>
+      <c r="I18" s="35"/>
+      <c r="J18" s="44">
         <v>46040.0</v>
       </c>
-      <c r="K18" s="45">
+      <c r="K18" s="46">
         <v>1214597.952</v>
       </c>
-      <c r="L18" s="34" t="s">
-        <v>151</v>
+      <c r="L18" s="35" t="s">
+        <v>155</v>
       </c>
       <c r="M18" s="39">
         <v>1214597.952</v>
@@ -2013,29 +2013,29 @@
       <c r="A19" s="23"/>
       <c r="B19" s="23"/>
       <c r="C19" s="41"/>
-      <c r="D19" s="48" t="s">
-        <v>154</v>
-      </c>
-      <c r="E19" s="34" t="s">
-        <v>70</v>
-      </c>
-      <c r="F19" s="34">
+      <c r="D19" s="49" t="s">
+        <v>156</v>
+      </c>
+      <c r="E19" s="35" t="s">
+        <v>77</v>
+      </c>
+      <c r="F19" s="35">
         <v>278.0</v>
       </c>
-      <c r="G19" s="43">
+      <c r="G19" s="44">
         <v>46042.0</v>
       </c>
-      <c r="H19" s="34" t="s">
-        <v>156</v>
-      </c>
-      <c r="I19" s="43"/>
-      <c r="J19" s="43">
+      <c r="H19" s="35" t="s">
+        <v>157</v>
+      </c>
+      <c r="I19" s="44"/>
+      <c r="J19" s="44">
         <v>46074.0</v>
       </c>
-      <c r="K19" s="45">
+      <c r="K19" s="46">
         <v>967082.09</v>
       </c>
-      <c r="L19" s="34" t="s">
+      <c r="L19" s="35" t="s">
         <v>158</v>
       </c>
       <c r="M19" s="39">
@@ -2053,27 +2053,27 @@
       <c r="A20" s="23"/>
       <c r="B20" s="23"/>
       <c r="C20" s="41"/>
-      <c r="D20" s="48" t="s">
+      <c r="D20" s="49" t="s">
         <v>159</v>
       </c>
-      <c r="E20" s="34"/>
-      <c r="F20" s="34">
+      <c r="E20" s="35"/>
+      <c r="F20" s="35">
         <v>10.0</v>
       </c>
-      <c r="G20" s="43">
+      <c r="G20" s="44">
         <v>46078.0</v>
       </c>
-      <c r="H20" s="34" t="s">
-        <v>107</v>
-      </c>
-      <c r="I20" s="43"/>
-      <c r="J20" s="43">
+      <c r="H20" s="35" t="s">
+        <v>101</v>
+      </c>
+      <c r="I20" s="44"/>
+      <c r="J20" s="44">
         <v>46106.0</v>
       </c>
-      <c r="K20" s="45">
+      <c r="K20" s="46">
         <v>719561.08</v>
       </c>
-      <c r="L20" s="34" t="s">
+      <c r="L20" s="35" t="s">
         <v>160</v>
       </c>
       <c r="M20" s="39">
@@ -2091,27 +2091,27 @@
       <c r="A21" s="23"/>
       <c r="B21" s="23"/>
       <c r="C21" s="41"/>
-      <c r="D21" s="48" t="s">
+      <c r="D21" s="49" t="s">
         <v>161</v>
       </c>
-      <c r="E21" s="34"/>
-      <c r="F21" s="34">
+      <c r="E21" s="35"/>
+      <c r="F21" s="35">
         <v>15.0</v>
       </c>
-      <c r="G21" s="43">
+      <c r="G21" s="44">
         <v>46094.0</v>
       </c>
-      <c r="H21" s="34" t="s">
+      <c r="H21" s="35" t="s">
         <v>162</v>
       </c>
-      <c r="I21" s="43"/>
-      <c r="J21" s="43">
+      <c r="I21" s="44"/>
+      <c r="J21" s="44">
         <v>46128.0</v>
       </c>
-      <c r="K21" s="45">
+      <c r="K21" s="46">
         <v>885881.08</v>
       </c>
-      <c r="L21" s="34" t="s">
+      <c r="L21" s="35" t="s">
         <v>163</v>
       </c>
       <c r="M21" s="39">
@@ -2129,27 +2129,27 @@
       <c r="A22" s="23"/>
       <c r="B22" s="23"/>
       <c r="C22" s="41"/>
-      <c r="D22" s="48" t="s">
+      <c r="D22" s="49" t="s">
         <v>164</v>
       </c>
-      <c r="E22" s="34"/>
-      <c r="F22" s="34">
+      <c r="E22" s="35"/>
+      <c r="F22" s="35">
         <v>28.0</v>
       </c>
-      <c r="G22" s="43">
+      <c r="G22" s="44">
         <v>46128.0</v>
       </c>
-      <c r="H22" s="34" t="s">
+      <c r="H22" s="35" t="s">
         <v>165</v>
       </c>
-      <c r="I22" s="43"/>
-      <c r="J22" s="43">
+      <c r="I22" s="44"/>
+      <c r="J22" s="44">
         <v>46164.0</v>
       </c>
-      <c r="K22" s="45" t="s">
+      <c r="K22" s="46" t="s">
         <v>166</v>
       </c>
-      <c r="L22" s="34" t="s">
+      <c r="L22" s="35" t="s">
         <v>167</v>
       </c>
       <c r="M22" s="39" t="s">
@@ -2167,27 +2167,27 @@
       <c r="A23" s="23"/>
       <c r="B23" s="23"/>
       <c r="C23" s="41"/>
-      <c r="D23" s="48" t="s">
+      <c r="D23" s="49" t="s">
         <v>168</v>
       </c>
-      <c r="E23" s="34"/>
-      <c r="F23" s="34">
+      <c r="E23" s="35"/>
+      <c r="F23" s="35">
         <v>33.0</v>
       </c>
-      <c r="G23" s="43">
+      <c r="G23" s="44">
         <v>46156.0</v>
       </c>
-      <c r="H23" s="34" t="s">
+      <c r="H23" s="35" t="s">
         <v>169</v>
       </c>
-      <c r="I23" s="43"/>
-      <c r="J23" s="43">
+      <c r="I23" s="44"/>
+      <c r="J23" s="44">
         <v>46191.0</v>
       </c>
-      <c r="K23" s="45">
+      <c r="K23" s="46">
         <v>1108954.4358333333</v>
       </c>
-      <c r="L23" s="34" t="s">
+      <c r="L23" s="35" t="s">
         <v>163</v>
       </c>
       <c r="M23" s="39">
@@ -2205,27 +2205,27 @@
       <c r="A24" s="23"/>
       <c r="B24" s="23"/>
       <c r="C24" s="41"/>
-      <c r="D24" s="48" t="s">
+      <c r="D24" s="49" t="s">
         <v>170</v>
       </c>
-      <c r="E24" s="34"/>
-      <c r="F24" s="34">
+      <c r="E24" s="35"/>
+      <c r="F24" s="35">
         <v>29.0</v>
       </c>
-      <c r="G24" s="43">
+      <c r="G24" s="44">
         <v>46149.0</v>
       </c>
-      <c r="H24" s="34" t="s">
+      <c r="H24" s="35" t="s">
         <v>169</v>
       </c>
-      <c r="I24" s="43"/>
-      <c r="J24" s="43">
+      <c r="I24" s="44"/>
+      <c r="J24" s="44">
         <v>46185.0</v>
       </c>
-      <c r="K24" s="45">
+      <c r="K24" s="46">
         <v>218206.1</v>
       </c>
-      <c r="L24" s="34" t="s">
+      <c r="L24" s="35" t="s">
         <v>171</v>
       </c>
       <c r="M24" s="39">
@@ -2243,27 +2243,27 @@
       <c r="A25" s="23"/>
       <c r="B25" s="23"/>
       <c r="C25" s="41"/>
-      <c r="D25" s="48" t="s">
+      <c r="D25" s="49" t="s">
         <v>172</v>
       </c>
-      <c r="E25" s="34"/>
-      <c r="F25" s="34">
+      <c r="E25" s="35"/>
+      <c r="F25" s="35">
         <v>40.0</v>
       </c>
-      <c r="G25" s="43">
+      <c r="G25" s="44">
         <v>46156.0</v>
       </c>
-      <c r="H25" s="34" t="s">
+      <c r="H25" s="35" t="s">
         <v>169</v>
       </c>
-      <c r="I25" s="43"/>
-      <c r="J25" s="43">
+      <c r="I25" s="44"/>
+      <c r="J25" s="44">
         <v>46191.0</v>
       </c>
-      <c r="K25" s="45">
+      <c r="K25" s="46">
         <v>1549250.84</v>
       </c>
-      <c r="L25" s="34" t="s">
+      <c r="L25" s="35" t="s">
         <v>173</v>
       </c>
       <c r="M25" s="39">
@@ -2281,27 +2281,27 @@
       <c r="A26" s="23"/>
       <c r="B26" s="23"/>
       <c r="C26" s="55"/>
-      <c r="D26" s="48" t="s">
+      <c r="D26" s="49" t="s">
         <v>174</v>
       </c>
-      <c r="E26" s="34"/>
-      <c r="F26" s="34">
+      <c r="E26" s="35"/>
+      <c r="F26" s="35">
         <v>48.0</v>
       </c>
-      <c r="G26" s="43">
+      <c r="G26" s="44">
         <v>46230.0</v>
       </c>
-      <c r="H26" s="34" t="s">
+      <c r="H26" s="35" t="s">
         <v>175</v>
       </c>
-      <c r="I26" s="43"/>
-      <c r="J26" s="43">
+      <c r="I26" s="44"/>
+      <c r="J26" s="44">
         <v>46262.0</v>
       </c>
-      <c r="K26" s="45" t="s">
+      <c r="K26" s="46" t="s">
         <v>176</v>
       </c>
-      <c r="L26" s="34" t="s">
+      <c r="L26" s="35" t="s">
         <v>177</v>
       </c>
       <c r="M26" s="39" t="s">
@@ -2319,34 +2319,34 @@
       <c r="A27" s="23"/>
       <c r="B27" s="23"/>
       <c r="C27" s="29" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D27" s="29" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E27" s="30" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="F27" s="29" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="G27" s="29"/>
       <c r="H27" s="29" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="I27" s="29"/>
       <c r="J27" s="29"/>
       <c r="K27" s="56" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="L27" s="31" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="M27" s="57" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="N27" s="29" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="O27" s="25"/>
       <c r="P27" s="28"/>
@@ -2372,24 +2372,24 @@
       <c r="D28" s="58" t="s">
         <v>178</v>
       </c>
-      <c r="E28" s="35"/>
-      <c r="F28" s="35">
+      <c r="E28" s="36"/>
+      <c r="F28" s="36">
         <v>402.0</v>
       </c>
-      <c r="G28" s="36">
+      <c r="G28" s="37">
         <v>45791.0</v>
       </c>
-      <c r="H28" s="35" t="s">
+      <c r="H28" s="36" t="s">
         <v>49</v>
       </c>
-      <c r="I28" s="36"/>
-      <c r="J28" s="36">
+      <c r="I28" s="37"/>
+      <c r="J28" s="37">
         <v>45834.0</v>
       </c>
-      <c r="K28" s="37">
+      <c r="K28" s="38">
         <v>188246.17</v>
       </c>
-      <c r="L28" s="34" t="s">
+      <c r="L28" s="35" t="s">
         <v>179</v>
       </c>
       <c r="M28" s="59">
@@ -2422,23 +2422,23 @@
       <c r="E29" s="60">
         <v>46.0</v>
       </c>
-      <c r="F29" s="35">
+      <c r="F29" s="36">
         <v>447.0</v>
       </c>
-      <c r="G29" s="36">
+      <c r="G29" s="37">
         <v>45814.0</v>
       </c>
-      <c r="H29" s="34" t="s">
+      <c r="H29" s="35" t="s">
         <v>181</v>
       </c>
-      <c r="I29" s="43"/>
-      <c r="J29" s="43">
+      <c r="I29" s="44"/>
+      <c r="J29" s="44">
         <v>45955.0</v>
       </c>
-      <c r="K29" s="37">
+      <c r="K29" s="38">
         <v>112720.77</v>
       </c>
-      <c r="L29" s="34" t="s">
+      <c r="L29" s="35" t="s">
         <v>182</v>
       </c>
       <c r="M29" s="39">
@@ -2471,23 +2471,23 @@
       <c r="E30" s="62" t="s">
         <v>184</v>
       </c>
-      <c r="F30" s="35">
+      <c r="F30" s="36">
         <v>529.0</v>
       </c>
       <c r="G30" s="63">
         <v>45853.0</v>
       </c>
-      <c r="H30" s="34" t="s">
-        <v>59</v>
-      </c>
-      <c r="I30" s="43"/>
-      <c r="J30" s="43">
+      <c r="H30" s="35" t="s">
+        <v>55</v>
+      </c>
+      <c r="I30" s="44"/>
+      <c r="J30" s="44">
         <v>45939.0</v>
       </c>
-      <c r="K30" s="45">
+      <c r="K30" s="46">
         <v>378307.61</v>
       </c>
-      <c r="L30" s="34" t="s">
+      <c r="L30" s="35" t="s">
         <v>185</v>
       </c>
       <c r="M30" s="39">
@@ -2520,23 +2520,23 @@
       <c r="E31" s="62" t="s">
         <v>184</v>
       </c>
-      <c r="F31" s="34">
+      <c r="F31" s="35">
         <v>691.0</v>
       </c>
       <c r="G31" s="63">
         <v>45910.0</v>
       </c>
-      <c r="H31" s="34" t="s">
-        <v>59</v>
-      </c>
-      <c r="I31" s="43"/>
-      <c r="J31" s="43">
+      <c r="H31" s="35" t="s">
+        <v>55</v>
+      </c>
+      <c r="I31" s="44"/>
+      <c r="J31" s="44">
         <v>45941.0</v>
       </c>
-      <c r="K31" s="37">
+      <c r="K31" s="38">
         <v>3315.0471000000252</v>
       </c>
-      <c r="L31" s="34" t="s">
+      <c r="L31" s="35" t="s">
         <v>187</v>
       </c>
       <c r="M31" s="39">
@@ -2569,23 +2569,23 @@
       <c r="E32" s="65">
         <v>135.0</v>
       </c>
-      <c r="F32" s="34">
+      <c r="F32" s="35">
         <v>677.0</v>
       </c>
       <c r="G32" s="63">
         <v>45904.0</v>
       </c>
-      <c r="H32" s="34" t="s">
-        <v>71</v>
+      <c r="H32" s="35" t="s">
+        <v>68</v>
       </c>
       <c r="I32" s="66"/>
       <c r="J32" s="66">
         <v>45935.0</v>
       </c>
-      <c r="K32" s="45">
+      <c r="K32" s="46">
         <v>198332.75</v>
       </c>
-      <c r="L32" s="34" t="s">
+      <c r="L32" s="35" t="s">
         <v>189</v>
       </c>
       <c r="M32" s="39">
@@ -2618,20 +2618,20 @@
       <c r="E33" s="65">
         <v>40.0</v>
       </c>
-      <c r="F33" s="34">
+      <c r="F33" s="35">
         <v>278.0</v>
       </c>
       <c r="G33" s="63">
         <v>46008.0</v>
       </c>
-      <c r="H33" s="34" t="s">
-        <v>120</v>
+      <c r="H33" s="35" t="s">
+        <v>113</v>
       </c>
       <c r="I33" s="66"/>
       <c r="J33" s="66">
         <v>46066.0</v>
       </c>
-      <c r="K33" s="45">
+      <c r="K33" s="46">
         <v>1528.62</v>
       </c>
       <c r="L33" s="67" t="s">
@@ -2667,23 +2667,23 @@
       <c r="E34" s="65" t="s">
         <v>194</v>
       </c>
-      <c r="F34" s="34">
+      <c r="F34" s="35">
         <v>748.0</v>
       </c>
       <c r="G34" s="63">
         <v>45930.0</v>
       </c>
-      <c r="H34" s="34" t="s">
-        <v>94</v>
+      <c r="H34" s="35" t="s">
+        <v>90</v>
       </c>
       <c r="I34" s="66"/>
       <c r="J34" s="66">
         <v>45935.0</v>
       </c>
-      <c r="K34" s="45">
+      <c r="K34" s="46">
         <v>38718.58</v>
       </c>
-      <c r="L34" s="34" t="s">
+      <c r="L34" s="35" t="s">
         <v>195</v>
       </c>
       <c r="M34" s="59" t="s">
@@ -2716,23 +2716,23 @@
       <c r="E35" s="65">
         <v>154.0</v>
       </c>
-      <c r="F35" s="34">
+      <c r="F35" s="35">
         <v>822.0</v>
       </c>
       <c r="G35" s="63">
         <v>45968.0</v>
       </c>
-      <c r="H35" s="34" t="s">
-        <v>112</v>
+      <c r="H35" s="35" t="s">
+        <v>105</v>
       </c>
       <c r="I35" s="66"/>
       <c r="J35" s="66">
         <v>45935.0</v>
       </c>
-      <c r="K35" s="45">
+      <c r="K35" s="46">
         <v>133124.11</v>
       </c>
-      <c r="L35" s="34" t="s">
+      <c r="L35" s="35" t="s">
         <v>198</v>
       </c>
       <c r="M35" s="59" t="s">
@@ -2772,16 +2772,16 @@
         <v>46043.0</v>
       </c>
       <c r="H36" s="65" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="I36" s="70"/>
       <c r="J36" s="69">
         <v>46075.0</v>
       </c>
-      <c r="K36" s="45">
+      <c r="K36" s="46">
         <v>11372.9</v>
       </c>
-      <c r="L36" s="34" t="s">
+      <c r="L36" s="35" t="s">
         <v>201</v>
       </c>
       <c r="M36" s="39">
@@ -2819,8 +2819,8 @@
         <v>203</v>
       </c>
       <c r="J37" s="69"/>
-      <c r="K37" s="45"/>
-      <c r="L37" s="34"/>
+      <c r="K37" s="46"/>
+      <c r="L37" s="35"/>
       <c r="M37" s="39"/>
       <c r="N37" s="51">
         <v>15854.78</v>
@@ -2856,8 +2856,8 @@
         <v>203</v>
       </c>
       <c r="J38" s="69"/>
-      <c r="K38" s="45"/>
-      <c r="L38" s="34"/>
+      <c r="K38" s="46"/>
+      <c r="L38" s="35"/>
       <c r="M38" s="39"/>
       <c r="N38" s="51" t="s">
         <v>205</v>
@@ -2895,13 +2895,13 @@
         <v>46104.0</v>
       </c>
       <c r="H39" s="65" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="I39" s="70"/>
       <c r="J39" s="69">
         <v>46106.0</v>
       </c>
-      <c r="K39" s="45">
+      <c r="K39" s="46">
         <v>27801.11</v>
       </c>
       <c r="L39" s="71" t="s">
@@ -2942,23 +2942,23 @@
         <v>46199.0</v>
       </c>
       <c r="H40" s="65" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="I40" s="70"/>
       <c r="J40" s="69">
         <v>46233.0</v>
       </c>
-      <c r="K40" s="45">
+      <c r="K40" s="46">
         <v>58868.35</v>
       </c>
-      <c r="L40" s="34" t="s">
-        <v>65</v>
+      <c r="L40" s="35" t="s">
+        <v>67</v>
       </c>
       <c r="M40" s="72">
         <v>58868.35</v>
       </c>
       <c r="N40" s="51"/>
-      <c r="V40" s="5"/>
+      <c r="V40" s="3"/>
     </row>
     <row r="41" ht="12.75" customHeight="1">
       <c r="A41" s="15"/>
@@ -2966,7 +2966,7 @@
       <c r="C41" s="41"/>
       <c r="K41" s="73"/>
       <c r="M41" s="73"/>
-      <c r="V41" s="5"/>
+      <c r="V41" s="3"/>
     </row>
     <row r="42" ht="12.75" customHeight="1">
       <c r="A42" s="15"/>
@@ -2974,31 +2974,31 @@
       <c r="C42" s="41"/>
       <c r="K42" s="73"/>
       <c r="M42" s="73"/>
-      <c r="V42" s="5"/>
+      <c r="V42" s="3"/>
     </row>
     <row r="43" ht="12.75" customHeight="1">
       <c r="A43" s="15"/>
       <c r="B43" s="15"/>
       <c r="C43" s="41"/>
-      <c r="V43" s="5"/>
+      <c r="V43" s="3"/>
     </row>
     <row r="44" ht="12.75" customHeight="1">
       <c r="A44" s="15"/>
       <c r="B44" s="15"/>
       <c r="C44" s="41"/>
-      <c r="V44" s="5"/>
+      <c r="V44" s="3"/>
     </row>
     <row r="45" ht="12.75" customHeight="1">
       <c r="A45" s="15"/>
       <c r="B45" s="15"/>
       <c r="C45" s="41"/>
-      <c r="V45" s="5"/>
+      <c r="V45" s="3"/>
     </row>
     <row r="46" ht="12.75" customHeight="1">
       <c r="A46" s="15"/>
       <c r="B46" s="15"/>
       <c r="C46" s="41"/>
-      <c r="V46" s="5"/>
+      <c r="V46" s="3"/>
     </row>
     <row r="47" ht="12.75" customHeight="1">
       <c r="A47" s="15"/>
@@ -3006,7 +3006,7 @@
       <c r="C47" s="55"/>
       <c r="K47" s="73"/>
       <c r="M47" s="73"/>
-      <c r="V47" s="5"/>
+      <c r="V47" s="3"/>
     </row>
     <row r="48" ht="12.75" customHeight="1">
       <c r="A48" s="15"/>
@@ -3030,7 +3030,7 @@
       <c r="S48" s="74"/>
       <c r="T48" s="74"/>
       <c r="U48" s="74"/>
-      <c r="V48" s="5"/>
+      <c r="V48" s="3"/>
     </row>
     <row r="49" ht="12.75" customHeight="1">
       <c r="A49" s="15"/>
@@ -7911,10 +7911,10 @@
       <c r="AH1" s="2"/>
     </row>
     <row r="2">
-      <c r="A2" s="3">
+      <c r="A2" s="4">
         <v>46212.0</v>
       </c>
-      <c r="L2" s="4" t="s">
+      <c r="L2" s="6" t="s">
         <v>0</v>
       </c>
       <c r="AB2" s="2"/>
@@ -7926,40 +7926,40 @@
       <c r="AH2" s="2"/>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="9">
+      <c r="C3" s="11">
         <v>2.5E32</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="D3" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E3" s="12">
         <v>45686.0</v>
       </c>
-      <c r="F3" s="7" t="s">
+      <c r="F3" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G3" s="7">
+      <c r="G3" s="10">
         <v>12.0</v>
       </c>
-      <c r="H3" s="7">
+      <c r="H3" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I3" s="7">
+      <c r="I3" s="10">
         <v>2048.0</v>
       </c>
-      <c r="J3" s="13">
+      <c r="J3" s="14">
         <v>1000.0</v>
       </c>
-      <c r="K3" s="13">
+      <c r="K3" s="14">
         <v>1000.0</v>
       </c>
-      <c r="L3" s="7">
+      <c r="L3" s="10">
         <v>0.0</v>
       </c>
       <c r="AB3" s="2"/>
@@ -7971,40 +7971,40 @@
       <c r="AH3" s="2"/>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="D4" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E4" s="12">
         <v>45762.0</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="F4" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G4" s="7">
+      <c r="G4" s="10">
         <v>12.0</v>
       </c>
-      <c r="H4" s="7">
+      <c r="H4" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I4" s="7">
+      <c r="I4" s="10">
         <v>2048.0</v>
       </c>
-      <c r="J4" s="13">
+      <c r="J4" s="14">
         <v>52250.04</v>
       </c>
-      <c r="K4" s="13">
+      <c r="K4" s="14">
         <v>52250.04</v>
       </c>
-      <c r="L4" s="7">
+      <c r="L4" s="10">
         <v>0.0</v>
       </c>
       <c r="AB4" s="2"/>
@@ -8016,40 +8016,40 @@
       <c r="AH4" s="2"/>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="C5" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="D5" s="7" t="s">
+      <c r="A5" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E5" s="12">
         <v>45762.0</v>
       </c>
-      <c r="F5" s="7" t="s">
+      <c r="F5" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G5" s="7">
+      <c r="G5" s="10">
         <v>12.0</v>
       </c>
-      <c r="H5" s="7">
+      <c r="H5" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I5" s="7">
+      <c r="I5" s="10">
         <v>2048.0</v>
       </c>
-      <c r="J5" s="13">
+      <c r="J5" s="14">
         <v>881914.18</v>
       </c>
-      <c r="K5" s="13">
+      <c r="K5" s="14">
         <v>881914.18</v>
       </c>
-      <c r="L5" s="7">
+      <c r="L5" s="10">
         <v>0.0</v>
       </c>
       <c r="AB5" s="2"/>
@@ -8061,40 +8061,40 @@
       <c r="AH5" s="2"/>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="B6" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="C6" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="D6" s="7" t="s">
+      <c r="A6" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="D6" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E6" s="12">
         <v>45762.0</v>
       </c>
-      <c r="F6" s="7" t="s">
+      <c r="F6" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G6" s="7">
+      <c r="G6" s="10">
         <v>12.0</v>
       </c>
-      <c r="H6" s="7">
+      <c r="H6" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I6" s="7">
+      <c r="I6" s="10">
         <v>2048.0</v>
       </c>
-      <c r="J6" s="13">
+      <c r="J6" s="14">
         <v>750000.0</v>
       </c>
-      <c r="K6" s="13">
+      <c r="K6" s="14">
         <v>750000.0</v>
       </c>
-      <c r="L6" s="7">
+      <c r="L6" s="10">
         <v>0.0</v>
       </c>
       <c r="AB6" s="2"/>
@@ -8106,40 +8106,40 @@
       <c r="AH6" s="2"/>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="B7" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="C7" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="D7" s="7" t="s">
+      <c r="A7" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="D7" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E7" s="12">
         <v>45763.0</v>
       </c>
-      <c r="F7" s="7" t="s">
+      <c r="F7" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G7" s="7">
+      <c r="G7" s="10">
         <v>12.0</v>
       </c>
-      <c r="H7" s="7">
+      <c r="H7" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I7" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="J7" s="13">
+      <c r="I7" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="J7" s="14">
         <v>949835.78</v>
       </c>
-      <c r="K7" s="13">
+      <c r="K7" s="14">
         <v>949835.78</v>
       </c>
-      <c r="L7" s="7">
+      <c r="L7" s="10">
         <v>0.0</v>
       </c>
       <c r="AB7" s="2"/>
@@ -8151,40 +8151,40 @@
       <c r="AH7" s="2"/>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="s">
+      <c r="A8" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E8" s="12">
         <v>45763.0</v>
       </c>
-      <c r="F8" s="7" t="s">
+      <c r="F8" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G8" s="7">
+      <c r="G8" s="10">
         <v>12.0</v>
       </c>
-      <c r="H8" s="7">
+      <c r="H8" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I8" s="7" t="s">
+      <c r="I8" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="J8" s="13">
+      <c r="J8" s="14">
         <v>524584.95</v>
       </c>
-      <c r="K8" s="13">
+      <c r="K8" s="14">
         <v>524584.95</v>
       </c>
-      <c r="L8" s="7">
+      <c r="L8" s="10">
         <v>0.0</v>
       </c>
       <c r="O8" s="26"/>
@@ -8197,40 +8197,40 @@
       <c r="AH8" s="2"/>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="s">
+      <c r="A9" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="C9" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="D9" s="7" t="s">
+      <c r="D9" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E9" s="12">
         <v>45792.0</v>
       </c>
-      <c r="F9" s="7" t="s">
+      <c r="F9" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G9" s="7">
+      <c r="G9" s="10">
         <v>12.0</v>
       </c>
-      <c r="H9" s="7">
+      <c r="H9" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I9" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="J9" s="13">
+      <c r="I9" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="J9" s="14">
         <v>211614.23</v>
       </c>
-      <c r="K9" s="13">
+      <c r="K9" s="14">
         <v>211614.23</v>
       </c>
-      <c r="L9" s="7">
+      <c r="L9" s="10">
         <v>0.0</v>
       </c>
       <c r="AB9" s="2"/>
@@ -8242,40 +8242,40 @@
       <c r="AH9" s="2"/>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="s">
-        <v>59</v>
-      </c>
-      <c r="B10" s="7" t="s">
+      <c r="A10" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="B10" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="C10" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="D10" s="7" t="s">
+      <c r="C10" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="D10" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E10" s="12">
         <v>45825.0</v>
       </c>
-      <c r="F10" s="7" t="s">
+      <c r="F10" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G10" s="7">
+      <c r="G10" s="10">
         <v>12.0</v>
       </c>
-      <c r="H10" s="7">
+      <c r="H10" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I10" s="7">
+      <c r="I10" s="10">
         <v>2048.0</v>
       </c>
-      <c r="J10" s="13">
+      <c r="J10" s="14">
         <v>2391157.42</v>
       </c>
-      <c r="K10" s="13">
+      <c r="K10" s="14">
         <v>2391157.41</v>
       </c>
-      <c r="L10" s="13">
+      <c r="L10" s="14">
         <v>0.01</v>
       </c>
       <c r="AB10" s="2"/>
@@ -8287,40 +8287,40 @@
       <c r="AH10" s="2"/>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="B11" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="C11" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="D11" s="7" t="s">
+      <c r="A11" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C11" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="D11" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E11" s="12">
         <v>45825.0</v>
       </c>
-      <c r="F11" s="7" t="s">
+      <c r="F11" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G11" s="7">
+      <c r="G11" s="10">
         <v>12.0</v>
       </c>
-      <c r="H11" s="7">
+      <c r="H11" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I11" s="7">
+      <c r="I11" s="10">
         <v>2048.0</v>
       </c>
-      <c r="J11" s="13">
+      <c r="J11" s="14">
         <v>618154.39</v>
       </c>
-      <c r="K11" s="13">
+      <c r="K11" s="14">
         <v>618154.38</v>
       </c>
-      <c r="L11" s="7">
+      <c r="L11" s="10">
         <v>0.01</v>
       </c>
       <c r="AB11" s="2"/>
@@ -8332,40 +8332,40 @@
       <c r="AH11" s="2"/>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="s">
+      <c r="A12" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="B12" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="C12" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="B12" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="C12" s="7" t="s">
-        <v>73</v>
-      </c>
-      <c r="D12" s="7" t="s">
+      <c r="D12" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E12" s="12">
         <v>45832.0</v>
       </c>
-      <c r="F12" s="7" t="s">
+      <c r="F12" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G12" s="7">
+      <c r="G12" s="10">
         <v>12.0</v>
       </c>
-      <c r="H12" s="7">
+      <c r="H12" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I12" s="7" t="s">
-        <v>74</v>
-      </c>
-      <c r="J12" s="13">
+      <c r="I12" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="J12" s="14">
         <v>1600334.09</v>
       </c>
-      <c r="K12" s="13">
+      <c r="K12" s="14">
         <v>1600334.09</v>
       </c>
-      <c r="L12" s="7">
+      <c r="L12" s="10">
         <v>0.0</v>
       </c>
       <c r="AB12" s="2"/>
@@ -8377,43 +8377,43 @@
       <c r="AH12" s="2"/>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="s">
-        <v>77</v>
-      </c>
-      <c r="B13" s="7" t="s">
+      <c r="A13" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="B13" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="C13" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="D13" s="7" t="s">
+      <c r="C13" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="D13" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E13" s="12">
         <v>45863.0</v>
       </c>
-      <c r="F13" s="7" t="s">
+      <c r="F13" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G13" s="7">
+      <c r="G13" s="10">
         <v>12.0</v>
       </c>
-      <c r="H13" s="7">
+      <c r="H13" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I13" s="7">
+      <c r="I13" s="10">
         <v>2048.0</v>
       </c>
-      <c r="J13" s="13">
+      <c r="J13" s="14">
         <v>2364771.07</v>
       </c>
-      <c r="K13" s="13">
+      <c r="K13" s="14">
         <v>2364771.07</v>
       </c>
-      <c r="L13" s="13">
+      <c r="L13" s="14">
         <v>0.0</v>
       </c>
-      <c r="M13" s="38"/>
+      <c r="M13" s="33"/>
       <c r="AB13" s="2"/>
       <c r="AC13" s="2"/>
       <c r="AD13" s="2"/>
@@ -8423,40 +8423,40 @@
       <c r="AH13" s="2"/>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="s">
+      <c r="A14" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="B14" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="C14" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="B14" s="7" t="s">
-        <v>80</v>
-      </c>
-      <c r="C14" s="7" t="s">
-        <v>81</v>
-      </c>
-      <c r="D14" s="7" t="s">
+      <c r="D14" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E14" s="12">
         <v>45887.0</v>
       </c>
-      <c r="F14" s="7" t="s">
+      <c r="F14" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G14" s="7">
+      <c r="G14" s="10">
         <v>12.0</v>
       </c>
-      <c r="H14" s="7">
+      <c r="H14" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I14" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="J14" s="13">
+      <c r="I14" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="J14" s="14">
         <v>968237.39</v>
       </c>
-      <c r="K14" s="13">
+      <c r="K14" s="14">
         <v>968237.39</v>
       </c>
-      <c r="L14" s="7">
+      <c r="L14" s="10">
         <v>0.0</v>
       </c>
       <c r="AB14" s="2"/>
@@ -8468,40 +8468,40 @@
       <c r="AH14" s="2"/>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="s">
+      <c r="A15" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="B15" s="10" t="s">
         <v>82</v>
       </c>
-      <c r="B15" s="7" t="s">
+      <c r="C15" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="C15" s="7" t="s">
-        <v>84</v>
-      </c>
-      <c r="D15" s="7" t="s">
+      <c r="D15" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E15" s="12">
         <v>45924.0</v>
       </c>
-      <c r="F15" s="7" t="s">
+      <c r="F15" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G15" s="7">
+      <c r="G15" s="10">
         <v>12.0</v>
       </c>
-      <c r="H15" s="7">
+      <c r="H15" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I15" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="J15" s="13">
+      <c r="I15" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="J15" s="14">
         <v>1011677.95</v>
       </c>
-      <c r="K15" s="13">
+      <c r="K15" s="14">
         <v>1011677.95</v>
       </c>
-      <c r="L15" s="7">
+      <c r="L15" s="10">
         <v>0.0</v>
       </c>
       <c r="AB15" s="2"/>
@@ -8513,40 +8513,40 @@
       <c r="AH15" s="2"/>
     </row>
     <row r="16">
-      <c r="A16" s="7" t="s">
+      <c r="A16" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="B16" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C16" s="10" t="s">
         <v>86</v>
       </c>
-      <c r="B16" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="C16" s="7" t="s">
-        <v>88</v>
-      </c>
-      <c r="D16" s="7" t="s">
+      <c r="D16" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E16" s="12">
         <v>45929.0</v>
       </c>
-      <c r="F16" s="7" t="s">
+      <c r="F16" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G16" s="7">
+      <c r="G16" s="10">
         <v>12.0</v>
       </c>
-      <c r="H16" s="7">
+      <c r="H16" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I16" s="7">
+      <c r="I16" s="10">
         <v>2048.0</v>
       </c>
-      <c r="J16" s="13">
+      <c r="J16" s="14">
         <v>1580293.02</v>
       </c>
-      <c r="K16" s="13">
+      <c r="K16" s="14">
         <v>1580293.02</v>
       </c>
-      <c r="L16" s="13">
+      <c r="L16" s="14">
         <v>0.0</v>
       </c>
       <c r="AB16" s="2"/>
@@ -8558,40 +8558,40 @@
       <c r="AH16" s="2"/>
     </row>
     <row r="17">
-      <c r="A17" s="7" t="s">
-        <v>90</v>
-      </c>
-      <c r="B17" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="C17" s="7" t="s">
-        <v>92</v>
-      </c>
-      <c r="D17" s="7" t="s">
+      <c r="A17" s="10" t="s">
+        <v>87</v>
+      </c>
+      <c r="B17" s="10" t="s">
+        <v>88</v>
+      </c>
+      <c r="C17" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="D17" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E17" s="12">
         <v>45930.0</v>
       </c>
-      <c r="F17" s="7" t="s">
+      <c r="F17" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G17" s="7">
+      <c r="G17" s="10">
         <v>12.0</v>
       </c>
-      <c r="H17" s="7">
+      <c r="H17" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I17" s="7">
+      <c r="I17" s="10">
         <v>2048.0</v>
       </c>
-      <c r="J17" s="13">
+      <c r="J17" s="14">
         <v>34065.36</v>
       </c>
-      <c r="K17" s="7">
+      <c r="K17" s="10">
         <v>0.0</v>
       </c>
-      <c r="L17" s="13">
+      <c r="L17" s="14">
         <v>34065.36</v>
       </c>
       <c r="AB17" s="2"/>
@@ -8603,40 +8603,40 @@
       <c r="AH17" s="2"/>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="s">
-        <v>94</v>
-      </c>
-      <c r="B18" s="7" t="s">
-        <v>80</v>
-      </c>
-      <c r="C18" s="7" t="s">
-        <v>96</v>
-      </c>
-      <c r="D18" s="7" t="s">
+      <c r="A18" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="B18" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="C18" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="D18" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E18" s="12">
         <v>45938.0</v>
       </c>
-      <c r="F18" s="7" t="s">
+      <c r="F18" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G18" s="7">
+      <c r="G18" s="10">
         <v>12.0</v>
       </c>
-      <c r="H18" s="7">
+      <c r="H18" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I18" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="J18" s="13">
+      <c r="I18" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="J18" s="14">
         <v>63746.85</v>
       </c>
-      <c r="K18" s="13">
+      <c r="K18" s="14">
         <v>63746.85</v>
       </c>
-      <c r="L18" s="7">
+      <c r="L18" s="10">
         <v>0.0</v>
       </c>
       <c r="AB18" s="2"/>
@@ -8648,40 +8648,40 @@
       <c r="AH18" s="2"/>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="s">
-        <v>98</v>
-      </c>
-      <c r="B19" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="C19" s="7" t="s">
-        <v>99</v>
-      </c>
-      <c r="D19" s="7" t="s">
+      <c r="A19" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="B19" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="C19" s="10" t="s">
+        <v>93</v>
+      </c>
+      <c r="D19" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E19" s="12">
         <v>45938.0</v>
       </c>
-      <c r="F19" s="7" t="s">
+      <c r="F19" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G19" s="7">
+      <c r="G19" s="10">
         <v>12.0</v>
       </c>
-      <c r="H19" s="7">
+      <c r="H19" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I19" s="7" t="s">
-        <v>74</v>
-      </c>
-      <c r="J19" s="13">
+      <c r="I19" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="J19" s="14">
         <v>947931.1</v>
       </c>
-      <c r="K19" s="13">
+      <c r="K19" s="14">
         <v>947931.1</v>
       </c>
-      <c r="L19" s="7">
+      <c r="L19" s="10">
         <v>0.0</v>
       </c>
       <c r="AB19" s="2"/>
@@ -8693,40 +8693,40 @@
       <c r="AH19" s="2"/>
     </row>
     <row r="20">
-      <c r="A20" s="7" t="s">
-        <v>101</v>
-      </c>
-      <c r="B20" s="7" t="s">
+      <c r="A20" s="10" t="s">
+        <v>95</v>
+      </c>
+      <c r="B20" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="C20" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="D20" s="7" t="s">
+      <c r="C20" s="10" t="s">
+        <v>96</v>
+      </c>
+      <c r="D20" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E20" s="12">
         <v>45938.0</v>
       </c>
-      <c r="F20" s="7" t="s">
+      <c r="F20" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G20" s="7">
+      <c r="G20" s="10">
         <v>12.0</v>
       </c>
-      <c r="H20" s="7">
+      <c r="H20" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I20" s="7">
+      <c r="I20" s="10">
         <v>2048.0</v>
       </c>
-      <c r="J20" s="13">
+      <c r="J20" s="14">
         <v>259790.57</v>
       </c>
-      <c r="K20" s="13">
+      <c r="K20" s="14">
         <v>259790.57</v>
       </c>
-      <c r="L20" s="7">
+      <c r="L20" s="10">
         <v>0.0</v>
       </c>
       <c r="AB20" s="2"/>
@@ -8738,40 +8738,40 @@
       <c r="AH20" s="2"/>
     </row>
     <row r="21">
-      <c r="A21" s="7" t="s">
-        <v>104</v>
-      </c>
-      <c r="B21" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="C21" s="7" t="s">
-        <v>105</v>
-      </c>
-      <c r="D21" s="7" t="s">
+      <c r="A21" s="10" t="s">
+        <v>98</v>
+      </c>
+      <c r="B21" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C21" s="10" t="s">
+        <v>100</v>
+      </c>
+      <c r="D21" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E21" s="12">
         <v>45938.0</v>
       </c>
-      <c r="F21" s="7" t="s">
+      <c r="F21" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G21" s="7">
+      <c r="G21" s="10">
         <v>12.0</v>
       </c>
-      <c r="H21" s="7">
+      <c r="H21" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I21" s="7">
+      <c r="I21" s="10">
         <v>2048.0</v>
       </c>
-      <c r="J21" s="13">
+      <c r="J21" s="14">
         <v>170479.3</v>
       </c>
-      <c r="K21" s="13">
+      <c r="K21" s="14">
         <v>170479.3</v>
       </c>
-      <c r="L21" s="7">
+      <c r="L21" s="10">
         <v>0.0</v>
       </c>
       <c r="AB21" s="2"/>
@@ -8783,40 +8783,40 @@
       <c r="AH21" s="2"/>
     </row>
     <row r="22">
-      <c r="A22" s="7" t="s">
-        <v>107</v>
-      </c>
-      <c r="B22" s="7" t="s">
-        <v>108</v>
-      </c>
-      <c r="C22" s="7" t="s">
-        <v>109</v>
-      </c>
-      <c r="D22" s="7" t="s">
+      <c r="A22" s="10" t="s">
+        <v>101</v>
+      </c>
+      <c r="B22" s="10" t="s">
+        <v>102</v>
+      </c>
+      <c r="C22" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="D22" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E22" s="49">
+      <c r="E22" s="43">
         <v>45953.0</v>
       </c>
-      <c r="F22" s="7" t="s">
+      <c r="F22" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G22" s="7">
+      <c r="G22" s="10">
         <v>12.0</v>
       </c>
-      <c r="H22" s="7">
+      <c r="H22" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I22" s="7">
+      <c r="I22" s="10">
         <v>2000.0</v>
       </c>
-      <c r="J22" s="13">
+      <c r="J22" s="14">
         <v>1500000.0</v>
       </c>
-      <c r="K22" s="13">
+      <c r="K22" s="14">
         <v>1500000.0</v>
       </c>
-      <c r="L22" s="13">
+      <c r="L22" s="14">
         <v>0.0</v>
       </c>
       <c r="AB22" s="2"/>
@@ -8828,40 +8828,40 @@
       <c r="AH22" s="2"/>
     </row>
     <row r="23">
-      <c r="A23" s="7" t="s">
-        <v>112</v>
-      </c>
-      <c r="B23" s="7" t="s">
-        <v>113</v>
-      </c>
-      <c r="C23" s="7" t="s">
-        <v>114</v>
-      </c>
-      <c r="D23" s="7" t="s">
+      <c r="A23" s="10" t="s">
+        <v>105</v>
+      </c>
+      <c r="B23" s="10" t="s">
+        <v>106</v>
+      </c>
+      <c r="C23" s="10" t="s">
+        <v>107</v>
+      </c>
+      <c r="D23" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E23" s="49">
+      <c r="E23" s="43">
         <v>45953.0</v>
       </c>
-      <c r="F23" s="7" t="s">
+      <c r="F23" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G23" s="7">
+      <c r="G23" s="10">
         <v>12.0</v>
       </c>
-      <c r="H23" s="7">
+      <c r="H23" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I23" s="7" t="s">
-        <v>115</v>
-      </c>
-      <c r="J23" s="13">
+      <c r="I23" s="10" t="s">
+        <v>108</v>
+      </c>
+      <c r="J23" s="14">
         <v>1000001.64</v>
       </c>
-      <c r="K23" s="13">
+      <c r="K23" s="14">
         <v>1000001.64</v>
       </c>
-      <c r="L23" s="7">
+      <c r="L23" s="10">
         <v>0.0</v>
       </c>
       <c r="AB23" s="2"/>
@@ -8873,40 +8873,40 @@
       <c r="AH23" s="2"/>
     </row>
     <row r="24">
-      <c r="A24" s="7" t="s">
-        <v>117</v>
-      </c>
-      <c r="B24" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="C24" s="7" t="s">
-        <v>118</v>
-      </c>
-      <c r="D24" s="7" t="s">
+      <c r="A24" s="10" t="s">
+        <v>110</v>
+      </c>
+      <c r="B24" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C24" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="D24" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E24" s="49">
+      <c r="E24" s="43">
         <v>45953.0</v>
       </c>
-      <c r="F24" s="7" t="s">
+      <c r="F24" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G24" s="7">
+      <c r="G24" s="10">
         <v>12.0</v>
       </c>
-      <c r="H24" s="7">
+      <c r="H24" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I24" s="7">
+      <c r="I24" s="10">
         <v>2048.0</v>
       </c>
-      <c r="J24" s="13">
+      <c r="J24" s="14">
         <v>68405.66</v>
       </c>
-      <c r="K24" s="13">
+      <c r="K24" s="14">
         <v>68405.66</v>
       </c>
-      <c r="L24" s="7">
+      <c r="L24" s="10">
         <v>0.0</v>
       </c>
       <c r="AB24" s="2"/>
@@ -8918,40 +8918,40 @@
       <c r="AH24" s="2"/>
     </row>
     <row r="25">
-      <c r="A25" s="7" t="s">
-        <v>120</v>
-      </c>
-      <c r="B25" s="7" t="s">
-        <v>121</v>
-      </c>
-      <c r="C25" s="7" t="s">
-        <v>122</v>
-      </c>
-      <c r="D25" s="7" t="s">
+      <c r="A25" s="10" t="s">
+        <v>113</v>
+      </c>
+      <c r="B25" s="10" t="s">
+        <v>114</v>
+      </c>
+      <c r="C25" s="10" t="s">
+        <v>115</v>
+      </c>
+      <c r="D25" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E25" s="49">
+      <c r="E25" s="43">
         <v>45975.0</v>
       </c>
-      <c r="F25" s="7" t="s">
+      <c r="F25" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G25" s="7">
+      <c r="G25" s="10">
         <v>12.0</v>
       </c>
-      <c r="H25" s="7">
+      <c r="H25" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I25" s="7" t="s">
-        <v>115</v>
-      </c>
-      <c r="J25" s="13">
+      <c r="I25" s="10" t="s">
+        <v>108</v>
+      </c>
+      <c r="J25" s="14">
         <v>1157673.06</v>
       </c>
-      <c r="K25" s="13">
+      <c r="K25" s="14">
         <v>1157673.06</v>
       </c>
-      <c r="L25" s="7">
+      <c r="L25" s="10">
         <v>0.0</v>
       </c>
       <c r="AB25" s="2"/>
@@ -8963,40 +8963,40 @@
       <c r="AH25" s="2"/>
     </row>
     <row r="26">
-      <c r="A26" s="7" t="s">
-        <v>124</v>
-      </c>
-      <c r="B26" s="7" t="s">
+      <c r="A26" s="10" t="s">
+        <v>117</v>
+      </c>
+      <c r="B26" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="C26" s="7" t="s">
-        <v>125</v>
-      </c>
-      <c r="D26" s="7" t="s">
+      <c r="C26" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="D26" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E26" s="49">
+      <c r="E26" s="43">
         <v>45989.0</v>
       </c>
-      <c r="F26" s="7" t="s">
+      <c r="F26" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G26" s="7">
+      <c r="G26" s="10">
         <v>12.0</v>
       </c>
-      <c r="H26" s="7">
+      <c r="H26" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I26" s="7">
+      <c r="I26" s="10">
         <v>2048.0</v>
       </c>
-      <c r="J26" s="13">
+      <c r="J26" s="14">
         <v>34065.36</v>
       </c>
-      <c r="K26" s="13">
+      <c r="K26" s="14">
         <v>34065.36</v>
       </c>
-      <c r="L26" s="7">
+      <c r="L26" s="10">
         <v>0.0</v>
       </c>
       <c r="AB26" s="2"/>
@@ -9008,40 +9008,40 @@
       <c r="AH26" s="2"/>
     </row>
     <row r="27">
-      <c r="A27" s="7" t="s">
-        <v>127</v>
-      </c>
-      <c r="B27" s="7" t="s">
-        <v>128</v>
-      </c>
-      <c r="C27" s="7" t="s">
-        <v>129</v>
-      </c>
-      <c r="D27" s="7" t="s">
+      <c r="A27" s="10" t="s">
+        <v>119</v>
+      </c>
+      <c r="B27" s="10" t="s">
+        <v>120</v>
+      </c>
+      <c r="C27" s="10" t="s">
+        <v>121</v>
+      </c>
+      <c r="D27" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E27" s="12">
         <v>46104.0</v>
       </c>
-      <c r="F27" s="7" t="s">
+      <c r="F27" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G27" s="7">
+      <c r="G27" s="10">
         <v>12.0</v>
       </c>
-      <c r="H27" s="7">
+      <c r="H27" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I27" s="7">
+      <c r="I27" s="10">
         <v>2048.0</v>
       </c>
-      <c r="J27" s="13">
+      <c r="J27" s="14">
         <v>1770880.5</v>
       </c>
-      <c r="K27" s="13">
+      <c r="K27" s="14">
         <v>843261.89</v>
       </c>
-      <c r="L27" s="13">
+      <c r="L27" s="14">
         <v>927618.61</v>
       </c>
       <c r="AB27" s="2"/>
@@ -9053,40 +9053,40 @@
       <c r="AH27" s="2"/>
     </row>
     <row r="28">
-      <c r="A28" s="7" t="s">
-        <v>132</v>
-      </c>
-      <c r="B28" s="7" t="s">
-        <v>133</v>
-      </c>
-      <c r="C28" s="7" t="s">
-        <v>134</v>
-      </c>
-      <c r="D28" s="7" t="s">
+      <c r="A28" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="B28" s="10" t="s">
+        <v>124</v>
+      </c>
+      <c r="C28" s="10" t="s">
+        <v>125</v>
+      </c>
+      <c r="D28" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E28" s="12">
         <v>46120.0</v>
       </c>
-      <c r="F28" s="7" t="s">
+      <c r="F28" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G28" s="7">
+      <c r="G28" s="10">
         <v>12.0</v>
       </c>
-      <c r="H28" s="7">
+      <c r="H28" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I28" s="7" t="s">
+      <c r="I28" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="J28" s="13">
+      <c r="J28" s="14">
         <v>1912292.52</v>
       </c>
-      <c r="K28" s="7">
+      <c r="K28" s="10">
         <v>0.0</v>
       </c>
-      <c r="L28" s="13">
+      <c r="L28" s="14">
         <v>1912292.52</v>
       </c>
       <c r="AB28" s="2"/>
@@ -9098,40 +9098,40 @@
       <c r="AH28" s="2"/>
     </row>
     <row r="29">
-      <c r="A29" s="7" t="s">
-        <v>137</v>
-      </c>
-      <c r="B29" s="7" t="s">
-        <v>138</v>
-      </c>
-      <c r="C29" s="7" t="s">
-        <v>140</v>
-      </c>
-      <c r="D29" s="7" t="s">
+      <c r="A29" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="B29" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="C29" s="10" t="s">
+        <v>128</v>
+      </c>
+      <c r="D29" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E29" s="12">
         <v>46196.0</v>
       </c>
-      <c r="F29" s="7" t="s">
+      <c r="F29" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G29" s="7">
+      <c r="G29" s="10">
         <v>12.0</v>
       </c>
-      <c r="H29" s="7">
+      <c r="H29" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I29" s="7">
+      <c r="I29" s="10">
         <v>2048.0</v>
       </c>
-      <c r="J29" s="13">
+      <c r="J29" s="14">
         <v>1496713.48</v>
       </c>
-      <c r="K29" s="7">
+      <c r="K29" s="10">
         <v>0.0</v>
       </c>
-      <c r="L29" s="13">
+      <c r="L29" s="14">
         <v>1496713.48</v>
       </c>
       <c r="AB29" s="2"/>
@@ -9143,40 +9143,40 @@
       <c r="AH29" s="2"/>
     </row>
     <row r="30">
-      <c r="A30" s="7" t="s">
-        <v>143</v>
-      </c>
-      <c r="B30" s="7" t="s">
-        <v>144</v>
-      </c>
-      <c r="C30" s="7" t="s">
-        <v>145</v>
-      </c>
-      <c r="D30" s="7" t="s">
+      <c r="A30" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="B30" s="10" t="s">
+        <v>132</v>
+      </c>
+      <c r="C30" s="10" t="s">
+        <v>133</v>
+      </c>
+      <c r="D30" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E30" s="12">
         <v>46205.0</v>
       </c>
-      <c r="F30" s="7" t="s">
+      <c r="F30" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G30" s="7">
+      <c r="G30" s="10">
         <v>12.0</v>
       </c>
-      <c r="H30" s="7">
+      <c r="H30" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I30" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="J30" s="13">
+      <c r="I30" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="J30" s="14">
         <v>624166.14</v>
       </c>
-      <c r="K30" s="7">
+      <c r="K30" s="10">
         <v>0.0</v>
       </c>
-      <c r="L30" s="13">
+      <c r="L30" s="14">
         <v>624166.14</v>
       </c>
       <c r="AB30" s="2"/>
@@ -9188,40 +9188,40 @@
       <c r="AH30" s="2"/>
     </row>
     <row r="31">
-      <c r="A31" s="7" t="s">
-        <v>147</v>
-      </c>
-      <c r="B31" s="7" t="s">
-        <v>148</v>
-      </c>
-      <c r="C31" s="7" t="s">
-        <v>149</v>
-      </c>
-      <c r="D31" s="7" t="s">
+      <c r="A31" s="10" t="s">
+        <v>135</v>
+      </c>
+      <c r="B31" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="C31" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="D31" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E31" s="12">
         <v>46205.0</v>
       </c>
-      <c r="F31" s="7" t="s">
+      <c r="F31" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G31" s="7">
+      <c r="G31" s="10">
         <v>12.0</v>
       </c>
-      <c r="H31" s="7">
+      <c r="H31" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I31" s="7" t="s">
-        <v>115</v>
-      </c>
-      <c r="J31" s="13">
+      <c r="I31" s="10" t="s">
+        <v>108</v>
+      </c>
+      <c r="J31" s="14">
         <v>18462.36</v>
       </c>
-      <c r="K31" s="7">
+      <c r="K31" s="10">
         <v>0.0</v>
       </c>
-      <c r="L31" s="13">
+      <c r="L31" s="14">
         <v>18462.36</v>
       </c>
       <c r="AB31" s="2"/>
@@ -9233,40 +9233,40 @@
       <c r="AH31" s="2"/>
     </row>
     <row r="32">
-      <c r="A32" s="7" t="s">
-        <v>152</v>
-      </c>
-      <c r="B32" s="7" t="s">
-        <v>148</v>
-      </c>
-      <c r="C32" s="13" t="s">
-        <v>153</v>
-      </c>
-      <c r="D32" s="7" t="s">
+      <c r="A32" s="10" t="s">
+        <v>141</v>
+      </c>
+      <c r="B32" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="C32" s="14" t="s">
+        <v>142</v>
+      </c>
+      <c r="D32" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E32" s="12">
         <v>46213.0</v>
       </c>
-      <c r="F32" s="7" t="s">
+      <c r="F32" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G32" s="7">
+      <c r="G32" s="10">
         <v>12.0</v>
       </c>
-      <c r="H32" s="7">
+      <c r="H32" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I32" s="7" t="s">
-        <v>115</v>
-      </c>
-      <c r="J32" s="13">
+      <c r="I32" s="10" t="s">
+        <v>108</v>
+      </c>
+      <c r="J32" s="14">
         <v>1530656.62</v>
       </c>
-      <c r="K32" s="7">
+      <c r="K32" s="10">
         <v>0.0</v>
       </c>
-      <c r="L32" s="13">
+      <c r="L32" s="14">
         <v>1530656.62</v>
       </c>
       <c r="AB32" s="2"/>
@@ -9278,40 +9278,40 @@
       <c r="AH32" s="2"/>
     </row>
     <row r="33">
-      <c r="A33" s="7" t="s">
-        <v>155</v>
-      </c>
-      <c r="B33" s="7" t="s">
-        <v>138</v>
-      </c>
-      <c r="C33" s="13" t="s">
-        <v>157</v>
-      </c>
-      <c r="D33" s="7" t="s">
+      <c r="A33" s="10" t="s">
+        <v>144</v>
+      </c>
+      <c r="B33" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="C33" s="14" t="s">
+        <v>145</v>
+      </c>
+      <c r="D33" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E33" s="12">
         <v>46227.0</v>
       </c>
-      <c r="F33" s="7" t="s">
+      <c r="F33" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G33" s="7">
+      <c r="G33" s="10">
         <v>12.0</v>
       </c>
-      <c r="H33" s="7">
+      <c r="H33" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I33" s="7">
+      <c r="I33" s="10">
         <v>2048.0</v>
       </c>
-      <c r="J33" s="13">
+      <c r="J33" s="14">
         <v>173846.38</v>
       </c>
-      <c r="K33" s="7">
+      <c r="K33" s="10">
         <v>0.0</v>
       </c>
-      <c r="L33" s="13">
+      <c r="L33" s="14">
         <v>173846.38</v>
       </c>
       <c r="AB33" s="2"/>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (05/08/2026 17:37)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/01_Bases_Originais/005_CELOG_2025/005_CELOG-PAMALS_2025 online.xlsx
+++ b/Contrato 005/Dashboard/01_Bases_Originais/005_CELOG_2025/005_CELOG-PAMALS_2025 online.xlsx
@@ -30,12 +30,12 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="331" uniqueCount="209">
   <si>
+    <t>Controle de pagamentos</t>
+  </si>
+  <si>
     <t>Saldo</t>
   </si>
   <si>
-    <t>Controle de pagamentos</t>
-  </si>
-  <si>
     <t>2025NE000005</t>
   </si>
   <si>
@@ -66,39 +66,39 @@
     <t>UG Responsável</t>
   </si>
   <si>
+    <t>UG Fiscalizadora</t>
+  </si>
+  <si>
+    <t>Prazo Final de Execução</t>
+  </si>
+  <si>
+    <t>Prazo Final de Vigência</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Ação</t>
+  </si>
+  <si>
+    <t>PAG</t>
+  </si>
+  <si>
     <t>2025NE000369</t>
   </si>
   <si>
-    <t>UG Fiscalizadora</t>
+    <t>Moeda</t>
   </si>
   <si>
     <t>C25516</t>
   </si>
   <si>
-    <t>Prazo Final de Execução</t>
+    <t>Valor Total do Contrato</t>
   </si>
   <si>
     <t>25E0387</t>
   </si>
   <si>
-    <t>Prazo Final de Vigência</t>
-  </si>
-  <si>
-    <t>Status</t>
-  </si>
-  <si>
-    <t>Ação</t>
-  </si>
-  <si>
-    <t>PAG</t>
-  </si>
-  <si>
-    <t>Moeda</t>
-  </si>
-  <si>
-    <t>Valor Total do Contrato</t>
-  </si>
-  <si>
     <t>Valor a Empenhar</t>
   </si>
   <si>
@@ -114,27 +114,27 @@
     <t>Fornecedor</t>
   </si>
   <si>
+    <t>Tipo Despesa /Receita</t>
+  </si>
+  <si>
+    <t>Abrir</t>
+  </si>
+  <si>
+    <t>Editar</t>
+  </si>
+  <si>
     <t>2025NE000371</t>
   </si>
   <si>
-    <t>Tipo Despesa /Receita</t>
-  </si>
-  <si>
-    <t>Abrir</t>
+    <t>005/CELOG-PAMALS/2025</t>
+  </si>
+  <si>
+    <t>CELOG</t>
   </si>
   <si>
     <t>25E0389</t>
   </si>
   <si>
-    <t>Editar</t>
-  </si>
-  <si>
-    <t>005/CELOG-PAMALS/2025</t>
-  </si>
-  <si>
-    <t>CELOG</t>
-  </si>
-  <si>
     <t>PAMALS</t>
   </si>
   <si>
@@ -147,24 +147,24 @@
     <t>67101.001510/2024-12</t>
   </si>
   <si>
+    <t>R$</t>
+  </si>
+  <si>
     <t>2025NE000413</t>
   </si>
   <si>
-    <t>R$</t>
-  </si>
-  <si>
     <t>C25501</t>
   </si>
   <si>
+    <t>VEE ONE-MANUTENCAO E SERVICOS TECNICOS LTDA</t>
+  </si>
+  <si>
     <t>25E0403</t>
   </si>
   <si>
     <t>20SP</t>
   </si>
   <si>
-    <t>VEE ONE-MANUTENCAO E SERVICOS TECNICOS LTDA</t>
-  </si>
-  <si>
     <t>2025NE000414</t>
   </si>
   <si>
@@ -177,6 +177,15 @@
     <t>21EM</t>
   </si>
   <si>
+    <t>Módulo</t>
+  </si>
+  <si>
+    <t>Referência</t>
+  </si>
+  <si>
+    <t>Nº recibo</t>
+  </si>
+  <si>
     <t>2025NE000559</t>
   </si>
   <si>
@@ -186,52 +195,55 @@
     <t>25E0524</t>
   </si>
   <si>
+    <t>Nº</t>
+  </si>
+  <si>
+    <t>Data</t>
+  </si>
+  <si>
+    <t>Empenho</t>
+  </si>
+  <si>
     <t>20X7</t>
   </si>
   <si>
-    <t>Módulo</t>
-  </si>
-  <si>
-    <t>Referência</t>
+    <t>Observações</t>
+  </si>
+  <si>
+    <t>Vencimento</t>
+  </si>
+  <si>
+    <t>Valor das Nfs</t>
+  </si>
+  <si>
+    <t>Ordem de Pagamento</t>
+  </si>
+  <si>
+    <t>Faturado</t>
   </si>
   <si>
     <t>2025NE000770</t>
   </si>
   <si>
+    <t>Pendente</t>
+  </si>
+  <si>
     <t>25E0731</t>
   </si>
   <si>
-    <t>Nº recibo</t>
-  </si>
-  <si>
-    <t>Nº</t>
-  </si>
-  <si>
-    <t>Data</t>
-  </si>
-  <si>
-    <t>Empenho</t>
-  </si>
-  <si>
     <t>2025NE000774</t>
   </si>
   <si>
-    <t>Observações</t>
-  </si>
-  <si>
     <t>25E0737</t>
   </si>
   <si>
-    <t>Vencimento</t>
-  </si>
-  <si>
-    <t>Valor das Nfs</t>
-  </si>
-  <si>
-    <t>Ordem de Pagamento</t>
-  </si>
-  <si>
-    <t>Faturado</t>
+    <t>FEV/25</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025NE000369 </t>
   </si>
   <si>
     <t>2025NE000843</t>
@@ -240,37 +252,31 @@
     <t>C25630</t>
   </si>
   <si>
-    <t>Pendente</t>
-  </si>
-  <si>
     <t>25E0787</t>
   </si>
   <si>
     <t>219C</t>
   </si>
   <si>
+    <t>2025NP001980</t>
+  </si>
+  <si>
     <t>2025NE001065</t>
   </si>
   <si>
     <t>25E0999</t>
   </si>
   <si>
-    <t>FEV/25</t>
-  </si>
-  <si>
     <t>2025NE001200</t>
   </si>
   <si>
-    <t>-</t>
-  </si>
-  <si>
     <t>C25590</t>
   </si>
   <si>
     <t>25E1128</t>
   </si>
   <si>
-    <t xml:space="preserve">2025NE000369 </t>
+    <t>MAR/25</t>
   </si>
   <si>
     <t>2025NE001598</t>
@@ -282,7 +288,10 @@
     <t>25E1446</t>
   </si>
   <si>
-    <t>2025NP001980</t>
+    <t>2025NE000367, 2025NE000369, 2025NE000371, 2025NE000413</t>
+  </si>
+  <si>
+    <t>2025NP001979</t>
   </si>
   <si>
     <t>2025NE001627</t>
@@ -300,121 +309,43 @@
     <t>25E1477</t>
   </si>
   <si>
+    <t>ABR/25</t>
+  </si>
+  <si>
+    <t>2025NE000413, 2025NE000414, 2025NE000559</t>
+  </si>
+  <si>
     <t>2025NE001687</t>
   </si>
   <si>
+    <t>2025NP002341</t>
+  </si>
+  <si>
     <t>25E1535</t>
   </si>
   <si>
+    <t>MAI/25</t>
+  </si>
+  <si>
     <t>2025NE001688</t>
   </si>
   <si>
     <t>25E1536</t>
   </si>
   <si>
-    <t>MAR/25</t>
-  </si>
-  <si>
     <t>2025NE001689</t>
   </si>
   <si>
+    <t>2025NP002884</t>
+  </si>
+  <si>
     <t>25E1537</t>
   </si>
   <si>
-    <t>2025NE000367, 2025NE000369, 2025NE000371, 2025NE000413</t>
-  </si>
-  <si>
     <t>2025NE001690</t>
   </si>
   <si>
-    <t>2025NP001979</t>
-  </si>
-  <si>
     <t>25E1538</t>
-  </si>
-  <si>
-    <t>2025NE001823</t>
-  </si>
-  <si>
-    <t>C25865</t>
-  </si>
-  <si>
-    <t>25E1666</t>
-  </si>
-  <si>
-    <t>ABR/25</t>
-  </si>
-  <si>
-    <t>2025NE001828</t>
-  </si>
-  <si>
-    <t>C25869</t>
-  </si>
-  <si>
-    <t>25E1667</t>
-  </si>
-  <si>
-    <t>20YJ</t>
-  </si>
-  <si>
-    <t>2025NE000413, 2025NE000414, 2025NE000559</t>
-  </si>
-  <si>
-    <t>2025NE001830</t>
-  </si>
-  <si>
-    <t>25E1669</t>
-  </si>
-  <si>
-    <t>2025NP002341</t>
-  </si>
-  <si>
-    <t>2025NE002200</t>
-  </si>
-  <si>
-    <t>C25863</t>
-  </si>
-  <si>
-    <t>25E2021</t>
-  </si>
-  <si>
-    <t>MAI/25</t>
-  </si>
-  <si>
-    <t>2025NE002237</t>
-  </si>
-  <si>
-    <t>25E2058</t>
-  </si>
-  <si>
-    <t>2026NE000330</t>
-  </si>
-  <si>
-    <t>C26163</t>
-  </si>
-  <si>
-    <t>26E0320</t>
-  </si>
-  <si>
-    <t>2025NP002884</t>
-  </si>
-  <si>
-    <t>2026NE000388</t>
-  </si>
-  <si>
-    <t>C26193</t>
-  </si>
-  <si>
-    <t>26E0375</t>
-  </si>
-  <si>
-    <t>2026NE000748</t>
-  </si>
-  <si>
-    <t>C26312</t>
-  </si>
-  <si>
-    <t>26E0709</t>
   </si>
   <si>
     <t>JUN/25</t>
@@ -426,52 +357,64 @@
 2025NE000774</t>
   </si>
   <si>
-    <t>2026NE000816</t>
-  </si>
-  <si>
-    <t>C26324</t>
-  </si>
-  <si>
-    <t>26E0776</t>
+    <t>2025NE001823</t>
+  </si>
+  <si>
+    <t>C25865</t>
   </si>
   <si>
     <t>2025NP400522</t>
   </si>
   <si>
-    <t>2026NE000817</t>
-  </si>
-  <si>
-    <t>C26326</t>
-  </si>
-  <si>
-    <t>26E0777</t>
+    <t>25E1666</t>
   </si>
   <si>
     <t>JUL/25</t>
   </si>
   <si>
+    <t>2025NE001828</t>
+  </si>
+  <si>
+    <t>C25869</t>
+  </si>
+  <si>
+    <t>25E1667</t>
+  </si>
+  <si>
     <t>2025NE000843, 2025NE001200</t>
   </si>
   <si>
+    <t>20YJ</t>
+  </si>
+  <si>
     <t>2025NP003724</t>
   </si>
   <si>
-    <t>2026NE000842</t>
-  </si>
-  <si>
-    <t>26E0803</t>
+    <t>2025NE001830</t>
+  </si>
+  <si>
+    <t>25E1669</t>
   </si>
   <si>
     <t>AGO/25</t>
   </si>
   <si>
-    <t>2026NE000944</t>
-  </si>
-  <si>
-    <t>26E0906</t>
+    <t>2025NE002200</t>
+  </si>
+  <si>
+    <t>C25863</t>
+  </si>
+  <si>
+    <t>25E2021</t>
   </si>
   <si>
     <t>2025NP004558</t>
+  </si>
+  <si>
+    <t>2025NE002237</t>
+  </si>
+  <si>
+    <t>25E2058</t>
   </si>
   <si>
     <t>SET/25</t>
@@ -481,25 +424,82 @@
 2025NE001828</t>
   </si>
   <si>
+    <t>2026NE000330</t>
+  </si>
+  <si>
+    <t>C26163</t>
+  </si>
+  <si>
+    <t>26E0320</t>
+  </si>
+  <si>
     <t>2025NP004897</t>
   </si>
   <si>
+    <t>2026NE000388</t>
+  </si>
+  <si>
+    <t>C26193</t>
+  </si>
+  <si>
+    <t>26E0375</t>
+  </si>
+  <si>
     <t>OUT/25</t>
   </si>
   <si>
+    <t>2026NE000748</t>
+  </si>
+  <si>
+    <t>C26312</t>
+  </si>
+  <si>
+    <t>26E0709</t>
+  </si>
+  <si>
     <t>2025NE001688, 2025NE001828, 2025NE002200</t>
   </si>
   <si>
     <t>2025NP004932</t>
   </si>
   <si>
+    <t>2026NE000816</t>
+  </si>
+  <si>
+    <t>C26324</t>
+  </si>
+  <si>
+    <t>26E0776</t>
+  </si>
+  <si>
+    <t>2026NE000817</t>
+  </si>
+  <si>
     <t>NOV/25</t>
   </si>
   <si>
+    <t>C26326</t>
+  </si>
+  <si>
+    <t>26E0777</t>
+  </si>
+  <si>
     <t>2025NE001687, 2025NE001689, 2025NE001690, 2025NE001823, 2025NE001830, 2025NE002237</t>
   </si>
   <si>
+    <t>2026NE000842</t>
+  </si>
+  <si>
     <t>2026NP400440</t>
+  </si>
+  <si>
+    <t>26E0803</t>
+  </si>
+  <si>
+    <t>2026NE000944</t>
+  </si>
+  <si>
+    <t>26E0906</t>
   </si>
   <si>
     <t>DEZ/25</t>
@@ -671,8 +671,8 @@
     <numFmt numFmtId="166" formatCode="dd/MM/yyyy"/>
     <numFmt numFmtId="167" formatCode="R$ #,##0.00"/>
     <numFmt numFmtId="168" formatCode="[$R$-416]\ #,##0.00;[RED]\-[$R$-416]\ #,##0.00"/>
-    <numFmt numFmtId="169" formatCode="d/m/yyyy"/>
-    <numFmt numFmtId="170" formatCode="MM/DD/YY"/>
+    <numFmt numFmtId="169" formatCode="MM/DD/YY"/>
+    <numFmt numFmtId="170" formatCode="d/m/yyyy"/>
     <numFmt numFmtId="171" formatCode="_([$R$ -416]* #,##0.00_);_([$R$ -416]* \(#,##0.00\);_([$R$ -416]* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="12">
@@ -867,11 +867,11 @@
     </xf>
     <xf borderId="0" fillId="3" fontId="2" numFmtId="0" xfId="0" applyFill="1" applyFont="1"/>
     <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyFill="1" applyFont="1"/>
+    <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
@@ -931,14 +931,14 @@
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="6" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="6" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment vertical="center"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
@@ -952,7 +952,6 @@
     <xf borderId="2" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="165" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="1" fillId="0" fontId="7" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
@@ -968,6 +967,7 @@
     <xf borderId="1" fillId="7" fontId="9" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="165" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="1" fillId="5" fontId="9" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
@@ -978,13 +978,10 @@
     <xf borderId="1" fillId="8" fontId="9" numFmtId="168" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="169" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
     <xf borderId="1" fillId="0" fontId="8" numFmtId="166" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="8" numFmtId="170" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="8" numFmtId="169" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="7" fontId="9" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
@@ -998,6 +995,9 @@
     </xf>
     <xf borderId="1" fillId="0" fontId="7" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="170" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
@@ -1415,9 +1415,9 @@
       <c r="V1" s="3"/>
     </row>
     <row r="2" ht="59.25" customHeight="1">
-      <c r="A2" s="5"/>
+      <c r="A2" s="4"/>
       <c r="B2" s="7" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V2" s="8"/>
       <c r="W2" s="9"/>
@@ -1466,28 +1466,28 @@
         <v>11</v>
       </c>
       <c r="F4" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="G4" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="G4" s="17" t="s">
+      <c r="H4" s="17" t="s">
+        <v>14</v>
+      </c>
+      <c r="I4" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="H4" s="17" t="s">
+      <c r="J4" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="K4" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="I4" s="16" t="s">
-        <v>18</v>
-      </c>
-      <c r="J4" s="16" t="s">
+      <c r="L4" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="K4" s="16" t="s">
-        <v>20</v>
-      </c>
-      <c r="L4" s="16" t="s">
+      <c r="M4" s="17" t="s">
         <v>21</v>
-      </c>
-      <c r="M4" s="17" t="s">
-        <v>22</v>
       </c>
       <c r="N4" s="17" t="s">
         <v>23</v>
@@ -1505,13 +1505,13 @@
         <v>27</v>
       </c>
       <c r="S4" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="T4" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="T4" s="16" t="s">
+      <c r="U4" s="16" t="s">
         <v>30</v>
-      </c>
-      <c r="U4" s="16" t="s">
-        <v>32</v>
       </c>
       <c r="V4" s="3"/>
     </row>
@@ -1520,10 +1520,10 @@
       <c r="B5" s="15"/>
       <c r="C5" s="18"/>
       <c r="D5" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="E5" s="19" t="s">
         <v>33</v>
-      </c>
-      <c r="E5" s="19" t="s">
-        <v>34</v>
       </c>
       <c r="F5" s="19" t="s">
         <v>35</v>
@@ -1547,7 +1547,7 @@
         <v>38</v>
       </c>
       <c r="M5" s="19" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="N5" s="21">
         <v>9.165159737E7</v>
@@ -1565,7 +1565,7 @@
         <v>1.085943044E7</v>
       </c>
       <c r="S5" s="19" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="V5" s="3"/>
     </row>
@@ -1587,54 +1587,54 @@
       <c r="I7" s="25"/>
       <c r="J7" s="25"/>
       <c r="K7" s="25"/>
-      <c r="L7" s="27"/>
+      <c r="L7" s="26"/>
       <c r="M7" s="25"/>
       <c r="N7" s="25"/>
       <c r="O7" s="25"/>
-      <c r="P7" s="28"/>
+      <c r="P7" s="27"/>
       <c r="V7" s="3"/>
     </row>
     <row r="8" ht="12.75" customHeight="1">
       <c r="A8" s="23"/>
       <c r="B8" s="23"/>
       <c r="C8" s="29" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="D8" s="29" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="E8" s="30" t="s">
+        <v>51</v>
+      </c>
+      <c r="F8" s="29" t="s">
+        <v>55</v>
+      </c>
+      <c r="G8" s="29" t="s">
+        <v>56</v>
+      </c>
+      <c r="H8" s="29" t="s">
         <v>57</v>
       </c>
-      <c r="F8" s="29" t="s">
-        <v>58</v>
-      </c>
-      <c r="G8" s="29" t="s">
+      <c r="I8" s="30" t="s">
         <v>59</v>
       </c>
-      <c r="H8" s="29" t="s">
+      <c r="J8" s="29" t="s">
         <v>60</v>
       </c>
-      <c r="I8" s="30" t="s">
+      <c r="K8" s="29" t="s">
+        <v>61</v>
+      </c>
+      <c r="L8" s="31" t="s">
         <v>62</v>
       </c>
-      <c r="J8" s="29" t="s">
-        <v>64</v>
-      </c>
-      <c r="K8" s="29" t="s">
+      <c r="M8" s="30" t="s">
+        <v>63</v>
+      </c>
+      <c r="N8" s="29" t="s">
         <v>65</v>
       </c>
-      <c r="L8" s="31" t="s">
-        <v>66</v>
-      </c>
-      <c r="M8" s="30" t="s">
-        <v>67</v>
-      </c>
-      <c r="N8" s="29" t="s">
-        <v>70</v>
-      </c>
       <c r="O8" s="29"/>
-      <c r="P8" s="28"/>
+      <c r="P8" s="27"/>
       <c r="V8" s="3"/>
     </row>
     <row r="9" ht="19.5" customHeight="1">
@@ -1643,30 +1643,30 @@
       <c r="C9" s="32">
         <v>1.0</v>
       </c>
-      <c r="D9" s="34" t="s">
-        <v>75</v>
-      </c>
-      <c r="E9" s="35" t="s">
-        <v>77</v>
-      </c>
-      <c r="F9" s="36">
+      <c r="D9" s="33" t="s">
+        <v>69</v>
+      </c>
+      <c r="E9" s="34" t="s">
+        <v>70</v>
+      </c>
+      <c r="F9" s="35">
         <v>594.0</v>
       </c>
-      <c r="G9" s="37">
+      <c r="G9" s="36">
         <v>45740.0</v>
       </c>
-      <c r="H9" s="36" t="s">
-        <v>80</v>
-      </c>
-      <c r="I9" s="37"/>
-      <c r="J9" s="37">
+      <c r="H9" s="35" t="s">
+        <v>71</v>
+      </c>
+      <c r="I9" s="36"/>
+      <c r="J9" s="36">
         <v>45778.0</v>
       </c>
-      <c r="K9" s="38">
+      <c r="K9" s="37">
         <v>748504.24</v>
       </c>
-      <c r="L9" s="36" t="s">
-        <v>84</v>
+      <c r="L9" s="35" t="s">
+        <v>76</v>
       </c>
       <c r="M9" s="39">
         <f t="shared" ref="M9:M10" si="1">K9</f>
@@ -1674,37 +1674,37 @@
       </c>
       <c r="N9" s="40"/>
       <c r="O9" s="25"/>
-      <c r="P9" s="28"/>
+      <c r="P9" s="27"/>
       <c r="V9" s="3"/>
     </row>
     <row r="10" ht="51.0" customHeight="1">
       <c r="A10" s="23"/>
       <c r="B10" s="23"/>
       <c r="C10" s="41"/>
-      <c r="D10" s="34" t="s">
-        <v>94</v>
-      </c>
-      <c r="E10" s="35" t="s">
-        <v>77</v>
-      </c>
-      <c r="F10" s="36">
+      <c r="D10" s="33" t="s">
+        <v>82</v>
+      </c>
+      <c r="E10" s="34" t="s">
+        <v>70</v>
+      </c>
+      <c r="F10" s="35">
         <v>620.0</v>
       </c>
-      <c r="G10" s="37">
+      <c r="G10" s="36">
         <v>45775.0</v>
       </c>
-      <c r="H10" s="36" t="s">
-        <v>97</v>
-      </c>
-      <c r="I10" s="37"/>
-      <c r="J10" s="37">
+      <c r="H10" s="35" t="s">
+        <v>86</v>
+      </c>
+      <c r="I10" s="36"/>
+      <c r="J10" s="36">
         <v>45806.0</v>
       </c>
-      <c r="K10" s="38">
+      <c r="K10" s="37">
         <v>1110378.24</v>
       </c>
-      <c r="L10" s="36" t="s">
-        <v>99</v>
+      <c r="L10" s="35" t="s">
+        <v>87</v>
       </c>
       <c r="M10" s="39">
         <f t="shared" si="1"/>
@@ -1712,116 +1712,116 @@
       </c>
       <c r="N10" s="42"/>
       <c r="O10" s="25"/>
-      <c r="P10" s="28"/>
+      <c r="P10" s="27"/>
       <c r="V10" s="3"/>
     </row>
     <row r="11" ht="12.75" customHeight="1">
       <c r="A11" s="23"/>
       <c r="B11" s="23"/>
       <c r="C11" s="41"/>
-      <c r="D11" s="34" t="s">
-        <v>104</v>
-      </c>
-      <c r="E11" s="35" t="s">
-        <v>77</v>
-      </c>
-      <c r="F11" s="36">
+      <c r="D11" s="33" t="s">
+        <v>93</v>
+      </c>
+      <c r="E11" s="34" t="s">
+        <v>70</v>
+      </c>
+      <c r="F11" s="35">
         <v>634.0</v>
       </c>
-      <c r="G11" s="37">
+      <c r="G11" s="36">
         <v>45799.0</v>
       </c>
-      <c r="H11" s="36" t="s">
-        <v>109</v>
-      </c>
-      <c r="I11" s="37"/>
-      <c r="J11" s="37">
+      <c r="H11" s="35" t="s">
+        <v>94</v>
+      </c>
+      <c r="I11" s="36"/>
+      <c r="J11" s="36">
         <v>45844.0</v>
       </c>
-      <c r="K11" s="38">
+      <c r="K11" s="37">
         <v>974557.12</v>
       </c>
-      <c r="L11" s="35" t="s">
-        <v>112</v>
+      <c r="L11" s="34" t="s">
+        <v>96</v>
       </c>
       <c r="M11" s="39">
         <v>974557.12</v>
       </c>
       <c r="N11" s="42"/>
       <c r="O11" s="25"/>
-      <c r="P11" s="28"/>
+      <c r="P11" s="27"/>
       <c r="V11" s="3"/>
     </row>
     <row r="12" ht="27.75" customHeight="1">
       <c r="A12" s="23"/>
       <c r="B12" s="23"/>
       <c r="C12" s="41"/>
-      <c r="D12" s="34" t="s">
-        <v>116</v>
-      </c>
-      <c r="E12" s="35" t="s">
-        <v>77</v>
-      </c>
-      <c r="F12" s="35">
+      <c r="D12" s="33" t="s">
+        <v>98</v>
+      </c>
+      <c r="E12" s="34" t="s">
+        <v>70</v>
+      </c>
+      <c r="F12" s="34">
         <v>660.0</v>
       </c>
-      <c r="G12" s="44">
+      <c r="G12" s="43">
         <v>45856.0</v>
       </c>
-      <c r="H12" s="45" t="s">
-        <v>68</v>
-      </c>
-      <c r="I12" s="37"/>
-      <c r="J12" s="37">
+      <c r="H12" s="44" t="s">
+        <v>72</v>
+      </c>
+      <c r="I12" s="36"/>
+      <c r="J12" s="36">
         <v>45891.0</v>
       </c>
-      <c r="K12" s="46">
+      <c r="K12" s="45">
         <v>1402001.34</v>
       </c>
-      <c r="L12" s="47" t="s">
-        <v>122</v>
+      <c r="L12" s="46" t="s">
+        <v>102</v>
       </c>
       <c r="M12" s="39">
         <v>1402001.34</v>
       </c>
-      <c r="N12" s="48"/>
+      <c r="N12" s="47"/>
       <c r="O12" s="25"/>
-      <c r="P12" s="28"/>
+      <c r="P12" s="27"/>
       <c r="V12" s="3"/>
     </row>
     <row r="13">
       <c r="A13" s="23"/>
       <c r="B13" s="23"/>
       <c r="C13" s="41"/>
-      <c r="D13" s="49" t="s">
-        <v>129</v>
-      </c>
-      <c r="E13" s="35" t="s">
-        <v>77</v>
-      </c>
-      <c r="F13" s="36">
+      <c r="D13" s="48" t="s">
+        <v>106</v>
+      </c>
+      <c r="E13" s="34" t="s">
+        <v>70</v>
+      </c>
+      <c r="F13" s="35">
         <v>661.0</v>
       </c>
-      <c r="G13" s="37">
+      <c r="G13" s="36">
         <v>45856.0</v>
       </c>
-      <c r="H13" s="36" t="s">
-        <v>130</v>
-      </c>
-      <c r="I13" s="44"/>
-      <c r="J13" s="44">
+      <c r="H13" s="35" t="s">
+        <v>107</v>
+      </c>
+      <c r="I13" s="43"/>
+      <c r="J13" s="43">
         <v>45891.0</v>
       </c>
-      <c r="K13" s="46">
+      <c r="K13" s="45">
         <v>1223702.3</v>
       </c>
-      <c r="L13" s="35" t="s">
-        <v>134</v>
+      <c r="L13" s="34" t="s">
+        <v>110</v>
       </c>
       <c r="M13" s="39">
         <v>1223702.3</v>
       </c>
-      <c r="N13" s="48"/>
+      <c r="N13" s="47"/>
       <c r="O13" s="25"/>
       <c r="P13" s="50"/>
       <c r="V13" s="3"/>
@@ -1830,72 +1830,72 @@
       <c r="A14" s="23"/>
       <c r="B14" s="23"/>
       <c r="C14" s="41"/>
-      <c r="D14" s="49" t="s">
-        <v>138</v>
-      </c>
-      <c r="E14" s="35" t="s">
-        <v>77</v>
-      </c>
-      <c r="F14" s="35">
+      <c r="D14" s="48" t="s">
+        <v>112</v>
+      </c>
+      <c r="E14" s="34" t="s">
+        <v>70</v>
+      </c>
+      <c r="F14" s="34">
         <v>688.0</v>
       </c>
-      <c r="G14" s="37">
+      <c r="G14" s="36">
         <v>45901.0</v>
       </c>
-      <c r="H14" s="35" t="s">
-        <v>139</v>
-      </c>
-      <c r="I14" s="44"/>
-      <c r="J14" s="44">
+      <c r="H14" s="34" t="s">
+        <v>116</v>
+      </c>
+      <c r="I14" s="43"/>
+      <c r="J14" s="43">
         <v>45938.0</v>
       </c>
-      <c r="K14" s="46">
+      <c r="K14" s="45">
         <v>1011677.95</v>
       </c>
-      <c r="L14" s="35" t="s">
-        <v>140</v>
+      <c r="L14" s="34" t="s">
+        <v>118</v>
       </c>
       <c r="M14" s="39">
         <v>1011677.95</v>
       </c>
       <c r="N14" s="42"/>
       <c r="O14" s="25"/>
-      <c r="P14" s="28"/>
+      <c r="P14" s="27"/>
       <c r="V14" s="3"/>
     </row>
     <row r="15">
       <c r="A15" s="23"/>
       <c r="B15" s="23"/>
       <c r="C15" s="41"/>
-      <c r="D15" s="49" t="s">
-        <v>143</v>
-      </c>
-      <c r="E15" s="35" t="s">
-        <v>77</v>
-      </c>
-      <c r="F15" s="35">
+      <c r="D15" s="48" t="s">
+        <v>121</v>
+      </c>
+      <c r="E15" s="34" t="s">
+        <v>70</v>
+      </c>
+      <c r="F15" s="34">
         <v>696.0</v>
       </c>
-      <c r="G15" s="37">
+      <c r="G15" s="36">
         <v>45923.0</v>
       </c>
-      <c r="H15" s="35" t="s">
-        <v>76</v>
-      </c>
-      <c r="I15" s="44"/>
-      <c r="J15" s="44">
+      <c r="H15" s="34" t="s">
+        <v>79</v>
+      </c>
+      <c r="I15" s="43"/>
+      <c r="J15" s="43">
         <v>45938.0</v>
       </c>
-      <c r="K15" s="46">
+      <c r="K15" s="45">
         <v>896744.06</v>
       </c>
-      <c r="L15" s="35" t="s">
-        <v>146</v>
+      <c r="L15" s="34" t="s">
+        <v>125</v>
       </c>
       <c r="M15" s="39">
         <v>896744.06</v>
       </c>
-      <c r="N15" s="48"/>
+      <c r="N15" s="47"/>
       <c r="O15" s="25"/>
       <c r="V15" s="3"/>
     </row>
@@ -1903,30 +1903,30 @@
       <c r="A16" s="23"/>
       <c r="B16" s="23"/>
       <c r="C16" s="41"/>
-      <c r="D16" s="49" t="s">
-        <v>147</v>
-      </c>
-      <c r="E16" s="35" t="s">
-        <v>77</v>
-      </c>
-      <c r="F16" s="35">
+      <c r="D16" s="48" t="s">
+        <v>128</v>
+      </c>
+      <c r="E16" s="34" t="s">
+        <v>70</v>
+      </c>
+      <c r="F16" s="34">
         <v>704.0</v>
       </c>
-      <c r="G16" s="37">
+      <c r="G16" s="36">
         <v>45957.0</v>
       </c>
-      <c r="H16" s="35" t="s">
-        <v>148</v>
-      </c>
-      <c r="I16" s="44"/>
-      <c r="J16" s="44">
+      <c r="H16" s="34" t="s">
+        <v>129</v>
+      </c>
+      <c r="I16" s="43"/>
+      <c r="J16" s="43">
         <v>46003.0</v>
       </c>
-      <c r="K16" s="46">
+      <c r="K16" s="45">
         <v>919329.06</v>
       </c>
-      <c r="L16" s="35" t="s">
-        <v>149</v>
+      <c r="L16" s="34" t="s">
+        <v>133</v>
       </c>
       <c r="M16" s="39">
         <v>919329.06</v>
@@ -1939,28 +1939,28 @@
       <c r="A17" s="23"/>
       <c r="B17" s="23"/>
       <c r="C17" s="41"/>
-      <c r="D17" s="49" t="s">
-        <v>150</v>
-      </c>
-      <c r="E17" s="35"/>
-      <c r="F17" s="35">
+      <c r="D17" s="48" t="s">
+        <v>137</v>
+      </c>
+      <c r="E17" s="34"/>
+      <c r="F17" s="34">
         <v>705.0</v>
       </c>
-      <c r="G17" s="44">
+      <c r="G17" s="43">
         <v>45972.0</v>
       </c>
-      <c r="H17" s="35" t="s">
-        <v>151</v>
-      </c>
-      <c r="I17" s="35"/>
-      <c r="J17" s="44">
+      <c r="H17" s="34" t="s">
+        <v>141</v>
+      </c>
+      <c r="I17" s="34"/>
+      <c r="J17" s="43">
         <v>46016.0</v>
       </c>
-      <c r="K17" s="46">
+      <c r="K17" s="45">
         <v>1157009.26</v>
       </c>
-      <c r="L17" s="35" t="s">
-        <v>152</v>
+      <c r="L17" s="34" t="s">
+        <v>142</v>
       </c>
       <c r="M17" s="39">
         <v>1157009.26</v>
@@ -1973,69 +1973,69 @@
       <c r="A18" s="23"/>
       <c r="B18" s="23"/>
       <c r="C18" s="41"/>
-      <c r="D18" s="49" t="s">
-        <v>153</v>
-      </c>
-      <c r="E18" s="35" t="s">
-        <v>77</v>
-      </c>
-      <c r="F18" s="35">
+      <c r="D18" s="48" t="s">
+        <v>147</v>
+      </c>
+      <c r="E18" s="34" t="s">
+        <v>70</v>
+      </c>
+      <c r="F18" s="34">
         <v>728.0</v>
       </c>
-      <c r="G18" s="44">
+      <c r="G18" s="43">
         <v>46008.0</v>
       </c>
-      <c r="H18" s="35" t="s">
-        <v>154</v>
-      </c>
-      <c r="I18" s="35"/>
-      <c r="J18" s="44">
+      <c r="H18" s="34" t="s">
+        <v>150</v>
+      </c>
+      <c r="I18" s="34"/>
+      <c r="J18" s="43">
         <v>46040.0</v>
       </c>
-      <c r="K18" s="46">
+      <c r="K18" s="45">
         <v>1214597.952</v>
       </c>
-      <c r="L18" s="35" t="s">
-        <v>155</v>
+      <c r="L18" s="34" t="s">
+        <v>152</v>
       </c>
       <c r="M18" s="39">
         <v>1214597.952</v>
       </c>
       <c r="N18" s="51"/>
       <c r="O18" s="25"/>
-      <c r="R18" s="28"/>
-      <c r="S18" s="28"/>
-      <c r="T18" s="28"/>
-      <c r="U18" s="28"/>
+      <c r="R18" s="27"/>
+      <c r="S18" s="27"/>
+      <c r="T18" s="27"/>
+      <c r="U18" s="27"/>
       <c r="V18" s="52"/>
     </row>
     <row r="19">
       <c r="A19" s="23"/>
       <c r="B19" s="23"/>
       <c r="C19" s="41"/>
-      <c r="D19" s="49" t="s">
+      <c r="D19" s="48" t="s">
         <v>156</v>
       </c>
-      <c r="E19" s="35" t="s">
-        <v>77</v>
-      </c>
-      <c r="F19" s="35">
+      <c r="E19" s="34" t="s">
+        <v>70</v>
+      </c>
+      <c r="F19" s="34">
         <v>278.0</v>
       </c>
-      <c r="G19" s="44">
+      <c r="G19" s="43">
         <v>46042.0</v>
       </c>
-      <c r="H19" s="35" t="s">
+      <c r="H19" s="34" t="s">
         <v>157</v>
       </c>
-      <c r="I19" s="44"/>
-      <c r="J19" s="44">
+      <c r="I19" s="43"/>
+      <c r="J19" s="43">
         <v>46074.0</v>
       </c>
-      <c r="K19" s="46">
+      <c r="K19" s="45">
         <v>967082.09</v>
       </c>
-      <c r="L19" s="35" t="s">
+      <c r="L19" s="34" t="s">
         <v>158</v>
       </c>
       <c r="M19" s="39">
@@ -2043,37 +2043,37 @@
       </c>
       <c r="N19" s="51"/>
       <c r="O19" s="25"/>
-      <c r="R19" s="28"/>
-      <c r="S19" s="28"/>
-      <c r="T19" s="28"/>
-      <c r="U19" s="28"/>
+      <c r="R19" s="27"/>
+      <c r="S19" s="27"/>
+      <c r="T19" s="27"/>
+      <c r="U19" s="27"/>
       <c r="V19" s="52"/>
     </row>
     <row r="20">
       <c r="A20" s="23"/>
       <c r="B20" s="23"/>
       <c r="C20" s="41"/>
-      <c r="D20" s="49" t="s">
+      <c r="D20" s="48" t="s">
         <v>159</v>
       </c>
-      <c r="E20" s="35"/>
-      <c r="F20" s="35">
+      <c r="E20" s="34"/>
+      <c r="F20" s="34">
         <v>10.0</v>
       </c>
-      <c r="G20" s="44">
+      <c r="G20" s="43">
         <v>46078.0</v>
       </c>
-      <c r="H20" s="35" t="s">
-        <v>101</v>
-      </c>
-      <c r="I20" s="44"/>
-      <c r="J20" s="44">
+      <c r="H20" s="34" t="s">
+        <v>108</v>
+      </c>
+      <c r="I20" s="43"/>
+      <c r="J20" s="43">
         <v>46106.0</v>
       </c>
-      <c r="K20" s="46">
+      <c r="K20" s="45">
         <v>719561.08</v>
       </c>
-      <c r="L20" s="35" t="s">
+      <c r="L20" s="34" t="s">
         <v>160</v>
       </c>
       <c r="M20" s="39">
@@ -2081,37 +2081,37 @@
       </c>
       <c r="N20" s="51"/>
       <c r="O20" s="25"/>
-      <c r="R20" s="28"/>
-      <c r="S20" s="28"/>
-      <c r="T20" s="28"/>
-      <c r="U20" s="28"/>
+      <c r="R20" s="27"/>
+      <c r="S20" s="27"/>
+      <c r="T20" s="27"/>
+      <c r="U20" s="27"/>
       <c r="V20" s="52"/>
     </row>
     <row r="21">
       <c r="A21" s="23"/>
       <c r="B21" s="23"/>
       <c r="C21" s="41"/>
-      <c r="D21" s="49" t="s">
+      <c r="D21" s="48" t="s">
         <v>161</v>
       </c>
-      <c r="E21" s="35"/>
-      <c r="F21" s="35">
+      <c r="E21" s="34"/>
+      <c r="F21" s="34">
         <v>15.0</v>
       </c>
-      <c r="G21" s="44">
+      <c r="G21" s="43">
         <v>46094.0</v>
       </c>
-      <c r="H21" s="35" t="s">
+      <c r="H21" s="34" t="s">
         <v>162</v>
       </c>
-      <c r="I21" s="44"/>
-      <c r="J21" s="44">
+      <c r="I21" s="43"/>
+      <c r="J21" s="43">
         <v>46128.0</v>
       </c>
-      <c r="K21" s="46">
+      <c r="K21" s="45">
         <v>885881.08</v>
       </c>
-      <c r="L21" s="35" t="s">
+      <c r="L21" s="34" t="s">
         <v>163</v>
       </c>
       <c r="M21" s="39">
@@ -2119,37 +2119,37 @@
       </c>
       <c r="N21" s="51"/>
       <c r="O21" s="25"/>
-      <c r="R21" s="28"/>
-      <c r="S21" s="28"/>
-      <c r="T21" s="28"/>
-      <c r="U21" s="28"/>
+      <c r="R21" s="27"/>
+      <c r="S21" s="27"/>
+      <c r="T21" s="27"/>
+      <c r="U21" s="27"/>
       <c r="V21" s="52"/>
     </row>
     <row r="22">
       <c r="A22" s="23"/>
       <c r="B22" s="23"/>
       <c r="C22" s="41"/>
-      <c r="D22" s="49" t="s">
+      <c r="D22" s="48" t="s">
         <v>164</v>
       </c>
-      <c r="E22" s="35"/>
-      <c r="F22" s="35">
+      <c r="E22" s="34"/>
+      <c r="F22" s="34">
         <v>28.0</v>
       </c>
-      <c r="G22" s="44">
+      <c r="G22" s="43">
         <v>46128.0</v>
       </c>
-      <c r="H22" s="35" t="s">
+      <c r="H22" s="34" t="s">
         <v>165</v>
       </c>
-      <c r="I22" s="44"/>
-      <c r="J22" s="44">
+      <c r="I22" s="43"/>
+      <c r="J22" s="43">
         <v>46164.0</v>
       </c>
-      <c r="K22" s="46" t="s">
+      <c r="K22" s="45" t="s">
         <v>166</v>
       </c>
-      <c r="L22" s="35" t="s">
+      <c r="L22" s="34" t="s">
         <v>167</v>
       </c>
       <c r="M22" s="39" t="s">
@@ -2157,37 +2157,37 @@
       </c>
       <c r="N22" s="51"/>
       <c r="O22" s="25"/>
-      <c r="R22" s="28"/>
-      <c r="S22" s="28"/>
-      <c r="T22" s="28"/>
-      <c r="U22" s="28"/>
+      <c r="R22" s="27"/>
+      <c r="S22" s="27"/>
+      <c r="T22" s="27"/>
+      <c r="U22" s="27"/>
       <c r="V22" s="52"/>
     </row>
     <row r="23">
       <c r="A23" s="23"/>
       <c r="B23" s="23"/>
       <c r="C23" s="41"/>
-      <c r="D23" s="49" t="s">
+      <c r="D23" s="48" t="s">
         <v>168</v>
       </c>
-      <c r="E23" s="35"/>
-      <c r="F23" s="35">
+      <c r="E23" s="34"/>
+      <c r="F23" s="34">
         <v>33.0</v>
       </c>
-      <c r="G23" s="44">
+      <c r="G23" s="43">
         <v>46156.0</v>
       </c>
-      <c r="H23" s="35" t="s">
+      <c r="H23" s="34" t="s">
         <v>169</v>
       </c>
-      <c r="I23" s="44"/>
-      <c r="J23" s="44">
+      <c r="I23" s="43"/>
+      <c r="J23" s="43">
         <v>46191.0</v>
       </c>
-      <c r="K23" s="46">
+      <c r="K23" s="45">
         <v>1108954.4358333333</v>
       </c>
-      <c r="L23" s="35" t="s">
+      <c r="L23" s="34" t="s">
         <v>163</v>
       </c>
       <c r="M23" s="39">
@@ -2195,37 +2195,37 @@
       </c>
       <c r="N23" s="53"/>
       <c r="O23" s="25"/>
-      <c r="R23" s="28"/>
-      <c r="S23" s="28"/>
-      <c r="T23" s="28"/>
-      <c r="U23" s="28"/>
+      <c r="R23" s="27"/>
+      <c r="S23" s="27"/>
+      <c r="T23" s="27"/>
+      <c r="U23" s="27"/>
       <c r="V23" s="52"/>
     </row>
     <row r="24">
       <c r="A24" s="23"/>
       <c r="B24" s="23"/>
       <c r="C24" s="41"/>
-      <c r="D24" s="49" t="s">
+      <c r="D24" s="48" t="s">
         <v>170</v>
       </c>
-      <c r="E24" s="35"/>
-      <c r="F24" s="35">
+      <c r="E24" s="34"/>
+      <c r="F24" s="34">
         <v>29.0</v>
       </c>
-      <c r="G24" s="44">
+      <c r="G24" s="43">
         <v>46149.0</v>
       </c>
-      <c r="H24" s="35" t="s">
+      <c r="H24" s="34" t="s">
         <v>169</v>
       </c>
-      <c r="I24" s="44"/>
-      <c r="J24" s="44">
+      <c r="I24" s="43"/>
+      <c r="J24" s="43">
         <v>46185.0</v>
       </c>
-      <c r="K24" s="46">
+      <c r="K24" s="45">
         <v>218206.1</v>
       </c>
-      <c r="L24" s="35" t="s">
+      <c r="L24" s="34" t="s">
         <v>171</v>
       </c>
       <c r="M24" s="39">
@@ -2233,37 +2233,37 @@
       </c>
       <c r="N24" s="54"/>
       <c r="O24" s="25"/>
-      <c r="R24" s="28"/>
-      <c r="S24" s="28"/>
-      <c r="T24" s="28"/>
-      <c r="U24" s="28"/>
+      <c r="R24" s="27"/>
+      <c r="S24" s="27"/>
+      <c r="T24" s="27"/>
+      <c r="U24" s="27"/>
       <c r="V24" s="52"/>
     </row>
     <row r="25">
       <c r="A25" s="23"/>
       <c r="B25" s="23"/>
       <c r="C25" s="41"/>
-      <c r="D25" s="49" t="s">
+      <c r="D25" s="48" t="s">
         <v>172</v>
       </c>
-      <c r="E25" s="35"/>
-      <c r="F25" s="35">
+      <c r="E25" s="34"/>
+      <c r="F25" s="34">
         <v>40.0</v>
       </c>
-      <c r="G25" s="44">
+      <c r="G25" s="43">
         <v>46156.0</v>
       </c>
-      <c r="H25" s="35" t="s">
+      <c r="H25" s="34" t="s">
         <v>169</v>
       </c>
-      <c r="I25" s="44"/>
-      <c r="J25" s="44">
+      <c r="I25" s="43"/>
+      <c r="J25" s="43">
         <v>46191.0</v>
       </c>
-      <c r="K25" s="46">
+      <c r="K25" s="45">
         <v>1549250.84</v>
       </c>
-      <c r="L25" s="35" t="s">
+      <c r="L25" s="34" t="s">
         <v>173</v>
       </c>
       <c r="M25" s="39">
@@ -2271,37 +2271,37 @@
       </c>
       <c r="N25" s="54"/>
       <c r="O25" s="25"/>
-      <c r="R25" s="28"/>
-      <c r="S25" s="28"/>
-      <c r="T25" s="28"/>
-      <c r="U25" s="28"/>
+      <c r="R25" s="27"/>
+      <c r="S25" s="27"/>
+      <c r="T25" s="27"/>
+      <c r="U25" s="27"/>
       <c r="V25" s="52"/>
     </row>
     <row r="26">
       <c r="A26" s="23"/>
       <c r="B26" s="23"/>
       <c r="C26" s="55"/>
-      <c r="D26" s="49" t="s">
+      <c r="D26" s="48" t="s">
         <v>174</v>
       </c>
-      <c r="E26" s="35"/>
-      <c r="F26" s="35">
+      <c r="E26" s="34"/>
+      <c r="F26" s="34">
         <v>48.0</v>
       </c>
-      <c r="G26" s="44">
+      <c r="G26" s="43">
         <v>46230.0</v>
       </c>
-      <c r="H26" s="35" t="s">
+      <c r="H26" s="34" t="s">
         <v>175</v>
       </c>
-      <c r="I26" s="44"/>
-      <c r="J26" s="44">
+      <c r="I26" s="43"/>
+      <c r="J26" s="43">
         <v>46262.0</v>
       </c>
-      <c r="K26" s="46" t="s">
+      <c r="K26" s="45" t="s">
         <v>176</v>
       </c>
-      <c r="L26" s="35" t="s">
+      <c r="L26" s="34" t="s">
         <v>177</v>
       </c>
       <c r="M26" s="39" t="s">
@@ -2309,59 +2309,59 @@
       </c>
       <c r="N26" s="54"/>
       <c r="O26" s="25"/>
-      <c r="R26" s="28"/>
-      <c r="S26" s="28"/>
-      <c r="T26" s="28"/>
-      <c r="U26" s="28"/>
+      <c r="R26" s="27"/>
+      <c r="S26" s="27"/>
+      <c r="T26" s="27"/>
+      <c r="U26" s="27"/>
       <c r="V26" s="52"/>
     </row>
     <row r="27" ht="30.75" customHeight="1">
       <c r="A27" s="23"/>
       <c r="B27" s="23"/>
       <c r="C27" s="29" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="D27" s="29" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="E27" s="30" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="F27" s="29" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="G27" s="29"/>
       <c r="H27" s="29" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="I27" s="29"/>
       <c r="J27" s="29"/>
       <c r="K27" s="56" t="s">
+        <v>61</v>
+      </c>
+      <c r="L27" s="31" t="s">
+        <v>62</v>
+      </c>
+      <c r="M27" s="57" t="s">
+        <v>63</v>
+      </c>
+      <c r="N27" s="29" t="s">
         <v>65</v>
       </c>
-      <c r="L27" s="31" t="s">
-        <v>66</v>
-      </c>
-      <c r="M27" s="57" t="s">
-        <v>67</v>
-      </c>
-      <c r="N27" s="29" t="s">
-        <v>70</v>
-      </c>
       <c r="O27" s="25"/>
-      <c r="P27" s="28"/>
-      <c r="R27" s="28"/>
-      <c r="S27" s="28"/>
-      <c r="T27" s="28"/>
-      <c r="U27" s="28"/>
+      <c r="P27" s="27"/>
+      <c r="R27" s="27"/>
+      <c r="S27" s="27"/>
+      <c r="T27" s="27"/>
+      <c r="U27" s="27"/>
       <c r="V27" s="52"/>
-      <c r="W27" s="28"/>
-      <c r="X27" s="28"/>
-      <c r="Y27" s="28"/>
-      <c r="Z27" s="28"/>
-      <c r="AA27" s="28"/>
-      <c r="AB27" s="28"/>
-      <c r="AC27" s="28"/>
+      <c r="W27" s="27"/>
+      <c r="X27" s="27"/>
+      <c r="Y27" s="27"/>
+      <c r="Z27" s="27"/>
+      <c r="AA27" s="27"/>
+      <c r="AB27" s="27"/>
+      <c r="AC27" s="27"/>
     </row>
     <row r="28" ht="12.75" customHeight="1">
       <c r="A28" s="23"/>
@@ -2372,24 +2372,24 @@
       <c r="D28" s="58" t="s">
         <v>178</v>
       </c>
-      <c r="E28" s="36"/>
-      <c r="F28" s="36">
+      <c r="E28" s="35"/>
+      <c r="F28" s="35">
         <v>402.0</v>
       </c>
-      <c r="G28" s="37">
+      <c r="G28" s="36">
         <v>45791.0</v>
       </c>
-      <c r="H28" s="36" t="s">
-        <v>49</v>
-      </c>
-      <c r="I28" s="37"/>
-      <c r="J28" s="37">
+      <c r="H28" s="35" t="s">
+        <v>52</v>
+      </c>
+      <c r="I28" s="36"/>
+      <c r="J28" s="36">
         <v>45834.0</v>
       </c>
-      <c r="K28" s="38">
+      <c r="K28" s="37">
         <v>188246.17</v>
       </c>
-      <c r="L28" s="35" t="s">
+      <c r="L28" s="34" t="s">
         <v>179</v>
       </c>
       <c r="M28" s="59">
@@ -2397,20 +2397,20 @@
       </c>
       <c r="N28" s="51"/>
       <c r="O28" s="25"/>
-      <c r="P28" s="28"/>
-      <c r="Q28" s="28"/>
-      <c r="R28" s="28"/>
-      <c r="S28" s="28"/>
-      <c r="T28" s="28"/>
-      <c r="U28" s="28"/>
+      <c r="P28" s="27"/>
+      <c r="Q28" s="27"/>
+      <c r="R28" s="27"/>
+      <c r="S28" s="27"/>
+      <c r="T28" s="27"/>
+      <c r="U28" s="27"/>
       <c r="V28" s="52"/>
-      <c r="W28" s="28"/>
-      <c r="X28" s="28"/>
-      <c r="Y28" s="28"/>
-      <c r="Z28" s="28"/>
-      <c r="AA28" s="28"/>
-      <c r="AB28" s="28"/>
-      <c r="AC28" s="28"/>
+      <c r="W28" s="27"/>
+      <c r="X28" s="27"/>
+      <c r="Y28" s="27"/>
+      <c r="Z28" s="27"/>
+      <c r="AA28" s="27"/>
+      <c r="AB28" s="27"/>
+      <c r="AC28" s="27"/>
     </row>
     <row r="29">
       <c r="A29" s="23"/>
@@ -2422,23 +2422,23 @@
       <c r="E29" s="60">
         <v>46.0</v>
       </c>
-      <c r="F29" s="36">
+      <c r="F29" s="35">
         <v>447.0</v>
       </c>
-      <c r="G29" s="37">
+      <c r="G29" s="36">
         <v>45814.0</v>
       </c>
-      <c r="H29" s="35" t="s">
+      <c r="H29" s="34" t="s">
         <v>181</v>
       </c>
-      <c r="I29" s="44"/>
-      <c r="J29" s="44">
+      <c r="I29" s="43"/>
+      <c r="J29" s="43">
         <v>45955.0</v>
       </c>
-      <c r="K29" s="38">
+      <c r="K29" s="37">
         <v>112720.77</v>
       </c>
-      <c r="L29" s="35" t="s">
+      <c r="L29" s="34" t="s">
         <v>182</v>
       </c>
       <c r="M29" s="39">
@@ -2446,20 +2446,20 @@
       </c>
       <c r="N29" s="51"/>
       <c r="O29" s="25"/>
-      <c r="P29" s="28"/>
-      <c r="Q29" s="28"/>
-      <c r="R29" s="28"/>
-      <c r="S29" s="28"/>
-      <c r="T29" s="28"/>
-      <c r="U29" s="28"/>
+      <c r="P29" s="27"/>
+      <c r="Q29" s="27"/>
+      <c r="R29" s="27"/>
+      <c r="S29" s="27"/>
+      <c r="T29" s="27"/>
+      <c r="U29" s="27"/>
       <c r="V29" s="52"/>
-      <c r="W29" s="28"/>
-      <c r="X29" s="28"/>
-      <c r="Y29" s="28"/>
-      <c r="Z29" s="28"/>
-      <c r="AA29" s="28"/>
-      <c r="AB29" s="28"/>
-      <c r="AC29" s="28"/>
+      <c r="W29" s="27"/>
+      <c r="X29" s="27"/>
+      <c r="Y29" s="27"/>
+      <c r="Z29" s="27"/>
+      <c r="AA29" s="27"/>
+      <c r="AB29" s="27"/>
+      <c r="AC29" s="27"/>
     </row>
     <row r="30" ht="12.75" customHeight="1">
       <c r="A30" s="23"/>
@@ -2471,23 +2471,23 @@
       <c r="E30" s="62" t="s">
         <v>184</v>
       </c>
-      <c r="F30" s="36">
+      <c r="F30" s="35">
         <v>529.0</v>
       </c>
       <c r="G30" s="63">
         <v>45853.0</v>
       </c>
-      <c r="H30" s="35" t="s">
-        <v>55</v>
-      </c>
-      <c r="I30" s="44"/>
-      <c r="J30" s="44">
+      <c r="H30" s="34" t="s">
+        <v>64</v>
+      </c>
+      <c r="I30" s="43"/>
+      <c r="J30" s="43">
         <v>45939.0</v>
       </c>
-      <c r="K30" s="46">
+      <c r="K30" s="45">
         <v>378307.61</v>
       </c>
-      <c r="L30" s="35" t="s">
+      <c r="L30" s="34" t="s">
         <v>185</v>
       </c>
       <c r="M30" s="39">
@@ -2496,19 +2496,19 @@
       <c r="N30" s="51"/>
       <c r="O30" s="25"/>
       <c r="P30" s="64"/>
-      <c r="Q30" s="28"/>
-      <c r="R30" s="28"/>
-      <c r="S30" s="28"/>
-      <c r="T30" s="28"/>
-      <c r="U30" s="28"/>
+      <c r="Q30" s="27"/>
+      <c r="R30" s="27"/>
+      <c r="S30" s="27"/>
+      <c r="T30" s="27"/>
+      <c r="U30" s="27"/>
       <c r="V30" s="52"/>
-      <c r="W30" s="28"/>
-      <c r="X30" s="28"/>
-      <c r="Y30" s="28"/>
-      <c r="Z30" s="28"/>
-      <c r="AA30" s="28"/>
-      <c r="AB30" s="28"/>
-      <c r="AC30" s="28"/>
+      <c r="W30" s="27"/>
+      <c r="X30" s="27"/>
+      <c r="Y30" s="27"/>
+      <c r="Z30" s="27"/>
+      <c r="AA30" s="27"/>
+      <c r="AB30" s="27"/>
+      <c r="AC30" s="27"/>
     </row>
     <row r="31" ht="60.0" customHeight="1">
       <c r="A31" s="23"/>
@@ -2520,23 +2520,23 @@
       <c r="E31" s="62" t="s">
         <v>184</v>
       </c>
-      <c r="F31" s="35">
+      <c r="F31" s="34">
         <v>691.0</v>
       </c>
       <c r="G31" s="63">
         <v>45910.0</v>
       </c>
-      <c r="H31" s="35" t="s">
-        <v>55</v>
-      </c>
-      <c r="I31" s="44"/>
-      <c r="J31" s="44">
+      <c r="H31" s="34" t="s">
+        <v>64</v>
+      </c>
+      <c r="I31" s="43"/>
+      <c r="J31" s="43">
         <v>45941.0</v>
       </c>
-      <c r="K31" s="38">
+      <c r="K31" s="37">
         <v>3315.0471000000252</v>
       </c>
-      <c r="L31" s="35" t="s">
+      <c r="L31" s="34" t="s">
         <v>187</v>
       </c>
       <c r="M31" s="39">
@@ -2545,19 +2545,19 @@
       <c r="N31" s="51"/>
       <c r="O31" s="25"/>
       <c r="P31" s="64"/>
-      <c r="Q31" s="28"/>
-      <c r="R31" s="28"/>
-      <c r="S31" s="28"/>
-      <c r="T31" s="28"/>
-      <c r="U31" s="28"/>
+      <c r="Q31" s="27"/>
+      <c r="R31" s="27"/>
+      <c r="S31" s="27"/>
+      <c r="T31" s="27"/>
+      <c r="U31" s="27"/>
       <c r="V31" s="52"/>
-      <c r="W31" s="28"/>
-      <c r="X31" s="28"/>
-      <c r="Y31" s="28"/>
-      <c r="Z31" s="28"/>
-      <c r="AA31" s="28"/>
-      <c r="AB31" s="28"/>
-      <c r="AC31" s="28"/>
+      <c r="W31" s="27"/>
+      <c r="X31" s="27"/>
+      <c r="Y31" s="27"/>
+      <c r="Z31" s="27"/>
+      <c r="AA31" s="27"/>
+      <c r="AB31" s="27"/>
+      <c r="AC31" s="27"/>
     </row>
     <row r="32" ht="12.75" customHeight="1">
       <c r="A32" s="23"/>
@@ -2569,23 +2569,23 @@
       <c r="E32" s="65">
         <v>135.0</v>
       </c>
-      <c r="F32" s="35">
+      <c r="F32" s="34">
         <v>677.0</v>
       </c>
       <c r="G32" s="63">
         <v>45904.0</v>
       </c>
-      <c r="H32" s="35" t="s">
-        <v>68</v>
+      <c r="H32" s="34" t="s">
+        <v>72</v>
       </c>
       <c r="I32" s="66"/>
       <c r="J32" s="66">
         <v>45935.0</v>
       </c>
-      <c r="K32" s="46">
+      <c r="K32" s="45">
         <v>198332.75</v>
       </c>
-      <c r="L32" s="35" t="s">
+      <c r="L32" s="34" t="s">
         <v>189</v>
       </c>
       <c r="M32" s="39">
@@ -2594,19 +2594,19 @@
       <c r="N32" s="51"/>
       <c r="O32" s="25"/>
       <c r="P32" s="64"/>
-      <c r="Q32" s="28"/>
-      <c r="R32" s="28"/>
-      <c r="S32" s="28"/>
-      <c r="T32" s="28"/>
-      <c r="U32" s="28"/>
+      <c r="Q32" s="27"/>
+      <c r="R32" s="27"/>
+      <c r="S32" s="27"/>
+      <c r="T32" s="27"/>
+      <c r="U32" s="27"/>
       <c r="V32" s="52"/>
-      <c r="W32" s="28"/>
-      <c r="X32" s="28"/>
-      <c r="Y32" s="28"/>
-      <c r="Z32" s="28"/>
-      <c r="AA32" s="28"/>
-      <c r="AB32" s="28"/>
-      <c r="AC32" s="28"/>
+      <c r="W32" s="27"/>
+      <c r="X32" s="27"/>
+      <c r="Y32" s="27"/>
+      <c r="Z32" s="27"/>
+      <c r="AA32" s="27"/>
+      <c r="AB32" s="27"/>
+      <c r="AC32" s="27"/>
     </row>
     <row r="33" ht="12.75" customHeight="1">
       <c r="A33" s="23"/>
@@ -2618,20 +2618,20 @@
       <c r="E33" s="65">
         <v>40.0</v>
       </c>
-      <c r="F33" s="35">
+      <c r="F33" s="34">
         <v>278.0</v>
       </c>
       <c r="G33" s="63">
         <v>46008.0</v>
       </c>
-      <c r="H33" s="35" t="s">
-        <v>113</v>
+      <c r="H33" s="34" t="s">
+        <v>122</v>
       </c>
       <c r="I33" s="66"/>
       <c r="J33" s="66">
         <v>46066.0</v>
       </c>
-      <c r="K33" s="46">
+      <c r="K33" s="45">
         <v>1528.62</v>
       </c>
       <c r="L33" s="67" t="s">
@@ -2643,19 +2643,19 @@
       <c r="N33" s="51"/>
       <c r="O33" s="25"/>
       <c r="P33" s="64"/>
-      <c r="Q33" s="28"/>
-      <c r="R33" s="28"/>
-      <c r="S33" s="28"/>
-      <c r="T33" s="28"/>
-      <c r="U33" s="28"/>
+      <c r="Q33" s="27"/>
+      <c r="R33" s="27"/>
+      <c r="S33" s="27"/>
+      <c r="T33" s="27"/>
+      <c r="U33" s="27"/>
       <c r="V33" s="52"/>
-      <c r="W33" s="28"/>
-      <c r="X33" s="28"/>
-      <c r="Y33" s="28"/>
-      <c r="Z33" s="28"/>
-      <c r="AA33" s="28"/>
-      <c r="AB33" s="28"/>
-      <c r="AC33" s="28"/>
+      <c r="W33" s="27"/>
+      <c r="X33" s="27"/>
+      <c r="Y33" s="27"/>
+      <c r="Z33" s="27"/>
+      <c r="AA33" s="27"/>
+      <c r="AB33" s="27"/>
+      <c r="AC33" s="27"/>
     </row>
     <row r="34" ht="12.75" customHeight="1">
       <c r="A34" s="23"/>
@@ -2667,23 +2667,23 @@
       <c r="E34" s="65" t="s">
         <v>194</v>
       </c>
-      <c r="F34" s="35">
+      <c r="F34" s="34">
         <v>748.0</v>
       </c>
       <c r="G34" s="63">
         <v>45930.0</v>
       </c>
-      <c r="H34" s="35" t="s">
-        <v>90</v>
+      <c r="H34" s="34" t="s">
+        <v>95</v>
       </c>
       <c r="I34" s="66"/>
       <c r="J34" s="66">
         <v>45935.0</v>
       </c>
-      <c r="K34" s="46">
+      <c r="K34" s="45">
         <v>38718.58</v>
       </c>
-      <c r="L34" s="35" t="s">
+      <c r="L34" s="34" t="s">
         <v>195</v>
       </c>
       <c r="M34" s="59" t="s">
@@ -2692,19 +2692,19 @@
       <c r="N34" s="51"/>
       <c r="O34" s="25"/>
       <c r="P34" s="64"/>
-      <c r="Q34" s="28"/>
-      <c r="R34" s="28"/>
-      <c r="S34" s="28"/>
-      <c r="T34" s="28"/>
-      <c r="U34" s="28"/>
+      <c r="Q34" s="27"/>
+      <c r="R34" s="27"/>
+      <c r="S34" s="27"/>
+      <c r="T34" s="27"/>
+      <c r="U34" s="27"/>
       <c r="V34" s="52"/>
-      <c r="W34" s="28"/>
-      <c r="X34" s="28"/>
-      <c r="Y34" s="28"/>
-      <c r="Z34" s="28"/>
-      <c r="AA34" s="28"/>
-      <c r="AB34" s="28"/>
-      <c r="AC34" s="28"/>
+      <c r="W34" s="27"/>
+      <c r="X34" s="27"/>
+      <c r="Y34" s="27"/>
+      <c r="Z34" s="27"/>
+      <c r="AA34" s="27"/>
+      <c r="AB34" s="27"/>
+      <c r="AC34" s="27"/>
     </row>
     <row r="35" ht="12.75" customHeight="1">
       <c r="A35" s="23"/>
@@ -2716,23 +2716,23 @@
       <c r="E35" s="65">
         <v>154.0</v>
       </c>
-      <c r="F35" s="35">
+      <c r="F35" s="34">
         <v>822.0</v>
       </c>
       <c r="G35" s="63">
         <v>45968.0</v>
       </c>
-      <c r="H35" s="35" t="s">
-        <v>105</v>
+      <c r="H35" s="34" t="s">
+        <v>113</v>
       </c>
       <c r="I35" s="66"/>
       <c r="J35" s="66">
         <v>45935.0</v>
       </c>
-      <c r="K35" s="46">
+      <c r="K35" s="45">
         <v>133124.11</v>
       </c>
-      <c r="L35" s="35" t="s">
+      <c r="L35" s="34" t="s">
         <v>198</v>
       </c>
       <c r="M35" s="59" t="s">
@@ -2741,19 +2741,19 @@
       <c r="N35" s="51"/>
       <c r="O35" s="25"/>
       <c r="P35" s="64"/>
-      <c r="Q35" s="28"/>
-      <c r="R35" s="28"/>
-      <c r="S35" s="28"/>
-      <c r="T35" s="28"/>
-      <c r="U35" s="28"/>
+      <c r="Q35" s="27"/>
+      <c r="R35" s="27"/>
+      <c r="S35" s="27"/>
+      <c r="T35" s="27"/>
+      <c r="U35" s="27"/>
       <c r="V35" s="52"/>
-      <c r="W35" s="28"/>
-      <c r="X35" s="28"/>
-      <c r="Y35" s="28"/>
-      <c r="Z35" s="28"/>
-      <c r="AA35" s="28"/>
-      <c r="AB35" s="28"/>
-      <c r="AC35" s="28"/>
+      <c r="W35" s="27"/>
+      <c r="X35" s="27"/>
+      <c r="Y35" s="27"/>
+      <c r="Z35" s="27"/>
+      <c r="AA35" s="27"/>
+      <c r="AB35" s="27"/>
+      <c r="AC35" s="27"/>
     </row>
     <row r="36" ht="12.75" customHeight="1">
       <c r="A36" s="23"/>
@@ -2772,16 +2772,16 @@
         <v>46043.0</v>
       </c>
       <c r="H36" s="65" t="s">
-        <v>101</v>
+        <v>108</v>
       </c>
       <c r="I36" s="70"/>
       <c r="J36" s="69">
         <v>46075.0</v>
       </c>
-      <c r="K36" s="46">
+      <c r="K36" s="45">
         <v>11372.9</v>
       </c>
-      <c r="L36" s="35" t="s">
+      <c r="L36" s="34" t="s">
         <v>201</v>
       </c>
       <c r="M36" s="39">
@@ -2789,20 +2789,20 @@
       </c>
       <c r="N36" s="51"/>
       <c r="O36" s="25"/>
-      <c r="P36" s="28"/>
-      <c r="Q36" s="28"/>
-      <c r="R36" s="28"/>
-      <c r="S36" s="28"/>
-      <c r="T36" s="28"/>
-      <c r="U36" s="28"/>
+      <c r="P36" s="27"/>
+      <c r="Q36" s="27"/>
+      <c r="R36" s="27"/>
+      <c r="S36" s="27"/>
+      <c r="T36" s="27"/>
+      <c r="U36" s="27"/>
       <c r="V36" s="52"/>
-      <c r="W36" s="28"/>
-      <c r="X36" s="28"/>
-      <c r="Y36" s="28"/>
-      <c r="Z36" s="28"/>
-      <c r="AA36" s="28"/>
-      <c r="AB36" s="28"/>
-      <c r="AC36" s="28"/>
+      <c r="W36" s="27"/>
+      <c r="X36" s="27"/>
+      <c r="Y36" s="27"/>
+      <c r="Z36" s="27"/>
+      <c r="AA36" s="27"/>
+      <c r="AB36" s="27"/>
+      <c r="AC36" s="27"/>
     </row>
     <row r="37" ht="12.75" customHeight="1">
       <c r="A37" s="23"/>
@@ -2819,27 +2819,27 @@
         <v>203</v>
       </c>
       <c r="J37" s="69"/>
-      <c r="K37" s="46"/>
-      <c r="L37" s="35"/>
+      <c r="K37" s="45"/>
+      <c r="L37" s="34"/>
       <c r="M37" s="39"/>
       <c r="N37" s="51">
         <v>15854.78</v>
       </c>
       <c r="O37" s="25"/>
-      <c r="P37" s="28"/>
-      <c r="Q37" s="28"/>
-      <c r="R37" s="28"/>
-      <c r="S37" s="28"/>
-      <c r="T37" s="28"/>
-      <c r="U37" s="28"/>
+      <c r="P37" s="27"/>
+      <c r="Q37" s="27"/>
+      <c r="R37" s="27"/>
+      <c r="S37" s="27"/>
+      <c r="T37" s="27"/>
+      <c r="U37" s="27"/>
       <c r="V37" s="52"/>
-      <c r="W37" s="28"/>
-      <c r="X37" s="28"/>
-      <c r="Y37" s="28"/>
-      <c r="Z37" s="28"/>
-      <c r="AA37" s="28"/>
-      <c r="AB37" s="28"/>
-      <c r="AC37" s="28"/>
+      <c r="W37" s="27"/>
+      <c r="X37" s="27"/>
+      <c r="Y37" s="27"/>
+      <c r="Z37" s="27"/>
+      <c r="AA37" s="27"/>
+      <c r="AB37" s="27"/>
+      <c r="AC37" s="27"/>
     </row>
     <row r="38" ht="12.75" customHeight="1">
       <c r="A38" s="23"/>
@@ -2856,27 +2856,27 @@
         <v>203</v>
       </c>
       <c r="J38" s="69"/>
-      <c r="K38" s="46"/>
-      <c r="L38" s="35"/>
+      <c r="K38" s="45"/>
+      <c r="L38" s="34"/>
       <c r="M38" s="39"/>
       <c r="N38" s="51" t="s">
         <v>205</v>
       </c>
       <c r="O38" s="25"/>
-      <c r="P38" s="28"/>
-      <c r="Q38" s="28"/>
-      <c r="R38" s="28"/>
-      <c r="S38" s="28"/>
-      <c r="T38" s="28"/>
-      <c r="U38" s="28"/>
+      <c r="P38" s="27"/>
+      <c r="Q38" s="27"/>
+      <c r="R38" s="27"/>
+      <c r="S38" s="27"/>
+      <c r="T38" s="27"/>
+      <c r="U38" s="27"/>
       <c r="V38" s="52"/>
-      <c r="W38" s="28"/>
-      <c r="X38" s="28"/>
-      <c r="Y38" s="28"/>
-      <c r="Z38" s="28"/>
-      <c r="AA38" s="28"/>
-      <c r="AB38" s="28"/>
-      <c r="AC38" s="28"/>
+      <c r="W38" s="27"/>
+      <c r="X38" s="27"/>
+      <c r="Y38" s="27"/>
+      <c r="Z38" s="27"/>
+      <c r="AA38" s="27"/>
+      <c r="AB38" s="27"/>
+      <c r="AC38" s="27"/>
     </row>
     <row r="39" ht="12.75" customHeight="1">
       <c r="A39" s="23"/>
@@ -2895,13 +2895,13 @@
         <v>46104.0</v>
       </c>
       <c r="H39" s="65" t="s">
-        <v>101</v>
+        <v>108</v>
       </c>
       <c r="I39" s="70"/>
       <c r="J39" s="69">
         <v>46106.0</v>
       </c>
-      <c r="K39" s="46">
+      <c r="K39" s="45">
         <v>27801.11</v>
       </c>
       <c r="L39" s="71" t="s">
@@ -2912,20 +2912,20 @@
       </c>
       <c r="N39" s="51"/>
       <c r="O39" s="25"/>
-      <c r="P39" s="28"/>
-      <c r="Q39" s="28"/>
-      <c r="R39" s="28"/>
-      <c r="S39" s="28"/>
-      <c r="T39" s="28"/>
-      <c r="U39" s="28"/>
+      <c r="P39" s="27"/>
+      <c r="Q39" s="27"/>
+      <c r="R39" s="27"/>
+      <c r="S39" s="27"/>
+      <c r="T39" s="27"/>
+      <c r="U39" s="27"/>
       <c r="V39" s="52"/>
-      <c r="W39" s="28"/>
-      <c r="X39" s="28"/>
-      <c r="Y39" s="28"/>
-      <c r="Z39" s="28"/>
-      <c r="AA39" s="28"/>
-      <c r="AB39" s="28"/>
-      <c r="AC39" s="28"/>
+      <c r="W39" s="27"/>
+      <c r="X39" s="27"/>
+      <c r="Y39" s="27"/>
+      <c r="Z39" s="27"/>
+      <c r="AA39" s="27"/>
+      <c r="AB39" s="27"/>
+      <c r="AC39" s="27"/>
     </row>
     <row r="40" ht="12.75" customHeight="1">
       <c r="A40" s="15"/>
@@ -2942,17 +2942,17 @@
         <v>46199.0</v>
       </c>
       <c r="H40" s="65" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="I40" s="70"/>
       <c r="J40" s="69">
         <v>46233.0</v>
       </c>
-      <c r="K40" s="46">
+      <c r="K40" s="45">
         <v>58868.35</v>
       </c>
-      <c r="L40" s="35" t="s">
-        <v>67</v>
+      <c r="L40" s="34" t="s">
+        <v>63</v>
       </c>
       <c r="M40" s="72">
         <v>58868.35</v>
@@ -7911,11 +7911,11 @@
       <c r="AH1" s="2"/>
     </row>
     <row r="2">
-      <c r="A2" s="4">
+      <c r="A2" s="5">
         <v>46212.0</v>
       </c>
       <c r="L2" s="6" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB2" s="2"/>
       <c r="AC2" s="2"/>
@@ -8017,13 +8017,13 @@
     </row>
     <row r="5">
       <c r="A5" s="10" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="D5" s="10" t="s">
         <v>4</v>
@@ -8062,13 +8062,13 @@
     </row>
     <row r="6">
       <c r="A6" s="10" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="D6" s="10" t="s">
         <v>4</v>
@@ -8107,13 +8107,13 @@
     </row>
     <row r="7">
       <c r="A7" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>41</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D7" s="10" t="s">
         <v>4</v>
@@ -8131,7 +8131,7 @@
         <v>339039.0</v>
       </c>
       <c r="I7" s="10" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="J7" s="14">
         <v>949835.78</v>
@@ -8187,7 +8187,7 @@
       <c r="L8" s="10">
         <v>0.0</v>
       </c>
-      <c r="O8" s="26"/>
+      <c r="O8" s="28"/>
       <c r="AB8" s="2"/>
       <c r="AC8" s="2"/>
       <c r="AD8" s="2"/>
@@ -8198,13 +8198,13 @@
     </row>
     <row r="9">
       <c r="A9" s="10" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="D9" s="10" t="s">
         <v>4</v>
@@ -8222,7 +8222,7 @@
         <v>339039.0</v>
       </c>
       <c r="I9" s="10" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="J9" s="14">
         <v>211614.23</v>
@@ -8243,13 +8243,13 @@
     </row>
     <row r="10">
       <c r="A10" s="10" t="s">
-        <v>55</v>
+        <v>64</v>
       </c>
       <c r="B10" s="10" t="s">
         <v>7</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>56</v>
+        <v>66</v>
       </c>
       <c r="D10" s="10" t="s">
         <v>4</v>
@@ -8288,13 +8288,13 @@
     </row>
     <row r="11">
       <c r="A11" s="10" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="D11" s="10" t="s">
         <v>4</v>
@@ -8333,13 +8333,13 @@
     </row>
     <row r="12">
       <c r="A12" s="10" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="D12" s="10" t="s">
         <v>4</v>
@@ -8357,7 +8357,7 @@
         <v>339039.0</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="J12" s="14">
         <v>1600334.09</v>
@@ -8378,13 +8378,13 @@
     </row>
     <row r="13">
       <c r="A13" s="10" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="B13" s="10" t="s">
         <v>7</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="D13" s="10" t="s">
         <v>4</v>
@@ -8413,7 +8413,7 @@
       <c r="L13" s="14">
         <v>0.0</v>
       </c>
-      <c r="M13" s="33"/>
+      <c r="M13" s="38"/>
       <c r="AB13" s="2"/>
       <c r="AC13" s="2"/>
       <c r="AD13" s="2"/>
@@ -8424,13 +8424,13 @@
     </row>
     <row r="14">
       <c r="A14" s="10" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="D14" s="10" t="s">
         <v>4</v>
@@ -8448,7 +8448,7 @@
         <v>339039.0</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="J14" s="14">
         <v>968237.39</v>
@@ -8469,13 +8469,13 @@
     </row>
     <row r="15">
       <c r="A15" s="10" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="D15" s="10" t="s">
         <v>4</v>
@@ -8493,7 +8493,7 @@
         <v>339039.0</v>
       </c>
       <c r="I15" s="10" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="J15" s="14">
         <v>1011677.95</v>
@@ -8514,13 +8514,13 @@
     </row>
     <row r="16">
       <c r="A16" s="10" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B16" s="10" t="s">
         <v>7</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="D16" s="10" t="s">
         <v>4</v>
@@ -8559,13 +8559,13 @@
     </row>
     <row r="17">
       <c r="A17" s="10" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="D17" s="10" t="s">
         <v>4</v>
@@ -8604,13 +8604,13 @@
     </row>
     <row r="18">
       <c r="A18" s="10" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="D18" s="10" t="s">
         <v>4</v>
@@ -8628,7 +8628,7 @@
         <v>339039.0</v>
       </c>
       <c r="I18" s="10" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="J18" s="14">
         <v>63746.85</v>
@@ -8649,13 +8649,13 @@
     </row>
     <row r="19">
       <c r="A19" s="10" t="s">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="D19" s="10" t="s">
         <v>4</v>
@@ -8673,7 +8673,7 @@
         <v>339039.0</v>
       </c>
       <c r="I19" s="10" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="J19" s="14">
         <v>947931.1</v>
@@ -8694,13 +8694,13 @@
     </row>
     <row r="20">
       <c r="A20" s="10" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="B20" s="10" t="s">
         <v>7</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="D20" s="10" t="s">
         <v>4</v>
@@ -8739,13 +8739,13 @@
     </row>
     <row r="21">
       <c r="A21" s="10" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="D21" s="10" t="s">
         <v>4</v>
@@ -8784,18 +8784,18 @@
     </row>
     <row r="22">
       <c r="A22" s="10" t="s">
-        <v>101</v>
+        <v>108</v>
       </c>
       <c r="B22" s="10" t="s">
-        <v>102</v>
+        <v>109</v>
       </c>
       <c r="C22" s="10" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="D22" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E22" s="43">
+      <c r="E22" s="49">
         <v>45953.0</v>
       </c>
       <c r="F22" s="10" t="s">
@@ -8829,18 +8829,18 @@
     </row>
     <row r="23">
       <c r="A23" s="10" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="B23" s="10" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>107</v>
+        <v>115</v>
       </c>
       <c r="D23" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E23" s="43">
+      <c r="E23" s="49">
         <v>45953.0</v>
       </c>
       <c r="F23" s="10" t="s">
@@ -8853,7 +8853,7 @@
         <v>339039.0</v>
       </c>
       <c r="I23" s="10" t="s">
-        <v>108</v>
+        <v>117</v>
       </c>
       <c r="J23" s="14">
         <v>1000001.64</v>
@@ -8874,18 +8874,18 @@
     </row>
     <row r="24">
       <c r="A24" s="10" t="s">
-        <v>110</v>
+        <v>119</v>
       </c>
       <c r="B24" s="10" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C24" s="10" t="s">
-        <v>111</v>
+        <v>120</v>
       </c>
       <c r="D24" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E24" s="43">
+      <c r="E24" s="49">
         <v>45953.0</v>
       </c>
       <c r="F24" s="10" t="s">
@@ -8919,18 +8919,18 @@
     </row>
     <row r="25">
       <c r="A25" s="10" t="s">
-        <v>113</v>
+        <v>122</v>
       </c>
       <c r="B25" s="10" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C25" s="10" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="D25" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E25" s="43">
+      <c r="E25" s="49">
         <v>45975.0</v>
       </c>
       <c r="F25" s="10" t="s">
@@ -8943,7 +8943,7 @@
         <v>339039.0</v>
       </c>
       <c r="I25" s="10" t="s">
-        <v>108</v>
+        <v>117</v>
       </c>
       <c r="J25" s="14">
         <v>1157673.06</v>
@@ -8964,18 +8964,18 @@
     </row>
     <row r="26">
       <c r="A26" s="10" t="s">
-        <v>117</v>
+        <v>126</v>
       </c>
       <c r="B26" s="10" t="s">
         <v>7</v>
       </c>
       <c r="C26" s="10" t="s">
-        <v>118</v>
+        <v>127</v>
       </c>
       <c r="D26" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E26" s="43">
+      <c r="E26" s="49">
         <v>45989.0</v>
       </c>
       <c r="F26" s="10" t="s">
@@ -9009,13 +9009,13 @@
     </row>
     <row r="27">
       <c r="A27" s="10" t="s">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>120</v>
+        <v>131</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>121</v>
+        <v>132</v>
       </c>
       <c r="D27" s="10" t="s">
         <v>4</v>
@@ -9054,13 +9054,13 @@
     </row>
     <row r="28">
       <c r="A28" s="10" t="s">
-        <v>123</v>
+        <v>134</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>124</v>
+        <v>135</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>125</v>
+        <v>136</v>
       </c>
       <c r="D28" s="10" t="s">
         <v>4</v>
@@ -9099,13 +9099,13 @@
     </row>
     <row r="29">
       <c r="A29" s="10" t="s">
-        <v>126</v>
+        <v>138</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>127</v>
+        <v>139</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>128</v>
+        <v>140</v>
       </c>
       <c r="D29" s="10" t="s">
         <v>4</v>
@@ -9144,13 +9144,13 @@
     </row>
     <row r="30">
       <c r="A30" s="10" t="s">
-        <v>131</v>
+        <v>143</v>
       </c>
       <c r="B30" s="10" t="s">
-        <v>132</v>
+        <v>144</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>133</v>
+        <v>145</v>
       </c>
       <c r="D30" s="10" t="s">
         <v>4</v>
@@ -9168,7 +9168,7 @@
         <v>339039.0</v>
       </c>
       <c r="I30" s="10" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="J30" s="14">
         <v>624166.14</v>
@@ -9189,13 +9189,13 @@
     </row>
     <row r="31">
       <c r="A31" s="10" t="s">
-        <v>135</v>
+        <v>146</v>
       </c>
       <c r="B31" s="10" t="s">
-        <v>136</v>
+        <v>148</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>137</v>
+        <v>149</v>
       </c>
       <c r="D31" s="10" t="s">
         <v>4</v>
@@ -9213,7 +9213,7 @@
         <v>339039.0</v>
       </c>
       <c r="I31" s="10" t="s">
-        <v>108</v>
+        <v>117</v>
       </c>
       <c r="J31" s="14">
         <v>18462.36</v>
@@ -9234,13 +9234,13 @@
     </row>
     <row r="32">
       <c r="A32" s="10" t="s">
-        <v>141</v>
+        <v>151</v>
       </c>
       <c r="B32" s="10" t="s">
-        <v>136</v>
+        <v>148</v>
       </c>
       <c r="C32" s="14" t="s">
-        <v>142</v>
+        <v>153</v>
       </c>
       <c r="D32" s="10" t="s">
         <v>4</v>
@@ -9258,7 +9258,7 @@
         <v>339039.0</v>
       </c>
       <c r="I32" s="10" t="s">
-        <v>108</v>
+        <v>117</v>
       </c>
       <c r="J32" s="14">
         <v>1530656.62</v>
@@ -9279,13 +9279,13 @@
     </row>
     <row r="33">
       <c r="A33" s="10" t="s">
-        <v>144</v>
+        <v>154</v>
       </c>
       <c r="B33" s="10" t="s">
-        <v>127</v>
+        <v>139</v>
       </c>
       <c r="C33" s="14" t="s">
-        <v>145</v>
+        <v>155</v>
       </c>
       <c r="D33" s="10" t="s">
         <v>4</v>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (12/08/2026 08:54)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/01_Bases_Originais/005_CELOG_2025/005_CELOG-PAMALS_2025 online.xlsx
+++ b/Contrato 005/Dashboard/01_Bases_Originais/005_CELOG_2025/005_CELOG-PAMALS_2025 online.xlsx
@@ -69,42 +69,42 @@
     <t>Status</t>
   </si>
   <si>
+    <t>Ação</t>
+  </si>
+  <si>
+    <t>PAG</t>
+  </si>
+  <si>
+    <t>Moeda</t>
+  </si>
+  <si>
+    <t>Valor Total do Contrato</t>
+  </si>
+  <si>
+    <t>Valor a Empenhar</t>
+  </si>
+  <si>
+    <t>Valor Empenhado</t>
+  </si>
+  <si>
     <t>2025NE000367</t>
   </si>
   <si>
-    <t>Ação</t>
+    <t>Valor Liquidado</t>
+  </si>
+  <si>
+    <t>Saldo (Valor a Faturar)</t>
   </si>
   <si>
     <t>C25512</t>
   </si>
   <si>
-    <t>PAG</t>
+    <t>Fornecedor</t>
   </si>
   <si>
     <t>25E0385</t>
   </si>
   <si>
-    <t>Moeda</t>
-  </si>
-  <si>
-    <t>Valor Total do Contrato</t>
-  </si>
-  <si>
-    <t>Valor a Empenhar</t>
-  </si>
-  <si>
-    <t>Valor Empenhado</t>
-  </si>
-  <si>
-    <t>Valor Liquidado</t>
-  </si>
-  <si>
-    <t>Saldo (Valor a Faturar)</t>
-  </si>
-  <si>
-    <t>Fornecedor</t>
-  </si>
-  <si>
     <t>Tipo Despesa /Receita</t>
   </si>
   <si>
@@ -114,58 +114,91 @@
     <t>Editar</t>
   </si>
   <si>
+    <t>005/CELOG-PAMALS/2025</t>
+  </si>
+  <si>
+    <t>CELOG</t>
+  </si>
+  <si>
+    <t>PAMALS</t>
+  </si>
+  <si>
+    <t>Vigente</t>
+  </si>
+  <si>
+    <t>2048 20YJ 21EM 219C 20SP 20X7 2000</t>
+  </si>
+  <si>
     <t>2025NE000369</t>
   </si>
   <si>
+    <t>67101.001510/2024-12</t>
+  </si>
+  <si>
+    <t>R$</t>
+  </si>
+  <si>
     <t>C25516</t>
   </si>
   <si>
     <t>25E0387</t>
   </si>
   <si>
-    <t>005/CELOG-PAMALS/2025</t>
-  </si>
-  <si>
-    <t>CELOG</t>
-  </si>
-  <si>
-    <t>PAMALS</t>
-  </si>
-  <si>
-    <t>Vigente</t>
-  </si>
-  <si>
-    <t>2048 20YJ 21EM 219C 20SP 20X7 2000</t>
+    <t>VEE ONE-MANUTENCAO E SERVICOS TECNICOS LTDA</t>
   </si>
   <si>
     <t>2025NE000371</t>
   </si>
   <si>
-    <t>67101.001510/2024-12</t>
-  </si>
-  <si>
-    <t>R$</t>
-  </si>
-  <si>
     <t>25E0389</t>
   </si>
   <si>
-    <t>VEE ONE-MANUTENCAO E SERVICOS TECNICOS LTDA</t>
+    <t>Módulo</t>
+  </si>
+  <si>
+    <t>Referência</t>
+  </si>
+  <si>
+    <t>Nº recibo</t>
   </si>
   <si>
     <t>2025NE000413</t>
   </si>
   <si>
+    <t>Nº</t>
+  </si>
+  <si>
     <t>C25501</t>
   </si>
   <si>
+    <t>Data</t>
+  </si>
+  <si>
     <t>25E0403</t>
   </si>
   <si>
+    <t>Empenho</t>
+  </si>
+  <si>
+    <t>Observações</t>
+  </si>
+  <si>
+    <t>Vencimento</t>
+  </si>
+  <si>
+    <t>Valor das Nfs</t>
+  </si>
+  <si>
+    <t>Ordem de Pagamento</t>
+  </si>
+  <si>
     <t>20SP</t>
   </si>
   <si>
-    <t>Módulo</t>
+    <t>Faturado</t>
+  </si>
+  <si>
+    <t>Pendente</t>
   </si>
   <si>
     <t>2025NE000414</t>
@@ -177,40 +210,16 @@
     <t>25E0431</t>
   </si>
   <si>
-    <t>Referência</t>
-  </si>
-  <si>
-    <t>Nº recibo</t>
+    <t>FEV/25</t>
   </si>
   <si>
     <t>21EM</t>
   </si>
   <si>
-    <t>Nº</t>
-  </si>
-  <si>
-    <t>Data</t>
-  </si>
-  <si>
-    <t>Empenho</t>
-  </si>
-  <si>
-    <t>Observações</t>
-  </si>
-  <si>
-    <t>Vencimento</t>
-  </si>
-  <si>
-    <t>Valor das Nfs</t>
-  </si>
-  <si>
-    <t>Ordem de Pagamento</t>
-  </si>
-  <si>
-    <t>Faturado</t>
-  </si>
-  <si>
-    <t>Pendente</t>
+    <t>-</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025NE000369 </t>
   </si>
   <si>
     <t>2025NE000559</t>
@@ -222,31 +231,31 @@
     <t>25E0524</t>
   </si>
   <si>
+    <t>2025NP001980</t>
+  </si>
+  <si>
     <t>20X7</t>
   </si>
   <si>
     <t>2025NE000770</t>
   </si>
   <si>
-    <t>FEV/25</t>
-  </si>
-  <si>
-    <t>-</t>
-  </si>
-  <si>
     <t>25E0731</t>
   </si>
   <si>
-    <t xml:space="preserve">2025NE000369 </t>
-  </si>
-  <si>
     <t>2025NE000774</t>
   </si>
   <si>
     <t>25E0737</t>
   </si>
   <si>
-    <t>2025NP001980</t>
+    <t>MAR/25</t>
+  </si>
+  <si>
+    <t>2025NE000367, 2025NE000369, 2025NE000371, 2025NE000413</t>
+  </si>
+  <si>
+    <t>2025NP001979</t>
   </si>
   <si>
     <t>2025NE000843</t>
@@ -261,12 +270,24 @@
     <t>219C</t>
   </si>
   <si>
+    <t>ABR/25</t>
+  </si>
+  <si>
     <t>2025NE001065</t>
   </si>
   <si>
+    <t>2025NE000413, 2025NE000414, 2025NE000559</t>
+  </si>
+  <si>
     <t>25E0999</t>
   </si>
   <si>
+    <t>2025NP002341</t>
+  </si>
+  <si>
+    <t>MAI/25</t>
+  </si>
+  <si>
     <t>2025NE001200</t>
   </si>
   <si>
@@ -276,6 +297,9 @@
     <t>25E1128</t>
   </si>
   <si>
+    <t>2025NP002884</t>
+  </si>
+  <si>
     <t>2025NE001598</t>
   </si>
   <si>
@@ -285,97 +309,10 @@
     <t>25E1446</t>
   </si>
   <si>
-    <t>MAR/25</t>
+    <t>JUN/25</t>
   </si>
   <si>
     <t>2025NE001627</t>
-  </si>
-  <si>
-    <t>25E1475</t>
-  </si>
-  <si>
-    <t>2025NE000367, 2025NE000369, 2025NE000371, 2025NE000413</t>
-  </si>
-  <si>
-    <t>2025NP001979</t>
-  </si>
-  <si>
-    <t>2025NE001629</t>
-  </si>
-  <si>
-    <t>C25820</t>
-  </si>
-  <si>
-    <t>25E1477</t>
-  </si>
-  <si>
-    <t>ABR/25</t>
-  </si>
-  <si>
-    <t>2025NE001687</t>
-  </si>
-  <si>
-    <t>25E1535</t>
-  </si>
-  <si>
-    <t>2025NE000413, 2025NE000414, 2025NE000559</t>
-  </si>
-  <si>
-    <t>2025NE001688</t>
-  </si>
-  <si>
-    <t>25E1536</t>
-  </si>
-  <si>
-    <t>2025NP002341</t>
-  </si>
-  <si>
-    <t>2025NE001689</t>
-  </si>
-  <si>
-    <t>25E1537</t>
-  </si>
-  <si>
-    <t>MAI/25</t>
-  </si>
-  <si>
-    <t>2025NE001690</t>
-  </si>
-  <si>
-    <t>25E1538</t>
-  </si>
-  <si>
-    <t>2025NE001823</t>
-  </si>
-  <si>
-    <t>C25865</t>
-  </si>
-  <si>
-    <t>25E1666</t>
-  </si>
-  <si>
-    <t>2025NP002884</t>
-  </si>
-  <si>
-    <t>2025NE001828</t>
-  </si>
-  <si>
-    <t>C25869</t>
-  </si>
-  <si>
-    <t>25E1667</t>
-  </si>
-  <si>
-    <t>20YJ</t>
-  </si>
-  <si>
-    <t>JUN/25</t>
-  </si>
-  <si>
-    <t>2025NE001830</t>
-  </si>
-  <si>
-    <t>25E1669</t>
   </si>
   <si>
     <t>2025NE000005,
@@ -384,61 +321,37 @@
 2025NE000774</t>
   </si>
   <si>
+    <t>25E1475</t>
+  </si>
+  <si>
     <t>2025NP400522</t>
   </si>
   <si>
-    <t>2025NE002200</t>
-  </si>
-  <si>
-    <t>C25863</t>
-  </si>
-  <si>
-    <t>25E2021</t>
-  </si>
-  <si>
     <t>JUL/25</t>
   </si>
   <si>
-    <t>2025NE002237</t>
-  </si>
-  <si>
-    <t>25E2058</t>
+    <t>2025NE001629</t>
+  </si>
+  <si>
+    <t>C25820</t>
+  </si>
+  <si>
+    <t>25E1477</t>
   </si>
   <si>
     <t>2025NE000843, 2025NE001200</t>
   </si>
   <si>
-    <t>2026NE000330</t>
-  </si>
-  <si>
-    <t>C26163</t>
-  </si>
-  <si>
-    <t>26E0320</t>
-  </si>
-  <si>
     <t>2025NP003724</t>
   </si>
   <si>
-    <t>2026NE000388</t>
-  </si>
-  <si>
     <t>AGO/25</t>
   </si>
   <si>
-    <t>C26193</t>
-  </si>
-  <si>
-    <t>26E0375</t>
-  </si>
-  <si>
-    <t>2026NE000748</t>
-  </si>
-  <si>
-    <t>C26312</t>
-  </si>
-  <si>
-    <t>26E0709</t>
+    <t>2025NE001687</t>
+  </si>
+  <si>
+    <t>25E1535</t>
   </si>
   <si>
     <t>2025NP004558</t>
@@ -447,52 +360,220 @@
     <t>SET/25</t>
   </si>
   <si>
-    <t>2026NE000816</t>
-  </si>
-  <si>
-    <t>C26324</t>
-  </si>
-  <si>
-    <t>26E0776</t>
+    <t>2025NE001688</t>
   </si>
   <si>
     <t>2025NE001688 
 2025NE001828</t>
   </si>
   <si>
+    <t>25E1536</t>
+  </si>
+  <si>
+    <t>2025NP004897</t>
+  </si>
+  <si>
+    <t>OUT/25</t>
+  </si>
+  <si>
+    <t>2025NE001688, 2025NE001828, 2025NE002200</t>
+  </si>
+  <si>
+    <t>2025NE001689</t>
+  </si>
+  <si>
+    <t>25E1537</t>
+  </si>
+  <si>
+    <t>2025NP004932</t>
+  </si>
+  <si>
+    <t>NOV/25</t>
+  </si>
+  <si>
+    <t>2025NE001690</t>
+  </si>
+  <si>
+    <t>25E1538</t>
+  </si>
+  <si>
+    <t>2025NE001687, 2025NE001689, 2025NE001690, 2025NE001823, 2025NE001830, 2025NE002237</t>
+  </si>
+  <si>
+    <t>2026NP400440</t>
+  </si>
+  <si>
+    <t>2025NE001823</t>
+  </si>
+  <si>
+    <t>C25865</t>
+  </si>
+  <si>
+    <t>25E1666</t>
+  </si>
+  <si>
+    <t>DEZ/25</t>
+  </si>
+  <si>
+    <t>2025NE001065, 2025NE002200</t>
+  </si>
+  <si>
+    <t>2026NP400412</t>
+  </si>
+  <si>
+    <t>2025NE001828</t>
+  </si>
+  <si>
+    <t>JAN/26</t>
+  </si>
+  <si>
+    <t>C25869</t>
+  </si>
+  <si>
+    <t>25E1667</t>
+  </si>
+  <si>
+    <t>2026NP401035</t>
+  </si>
+  <si>
+    <t>20YJ</t>
+  </si>
+  <si>
+    <t>2025NE001830</t>
+  </si>
+  <si>
+    <t>FEV/26</t>
+  </si>
+  <si>
+    <t>25E1669</t>
+  </si>
+  <si>
+    <t>2025NE001627, 2025NE001629, 2025NE001823</t>
+  </si>
+  <si>
+    <t>2026NP402272</t>
+  </si>
+  <si>
+    <t>2025NE002200</t>
+  </si>
+  <si>
+    <t>MAR/26</t>
+  </si>
+  <si>
+    <t>C25863</t>
+  </si>
+  <si>
+    <t>25E2021</t>
+  </si>
+  <si>
+    <t>2025NE000770, 2025NE001627</t>
+  </si>
+  <si>
+    <t>R$ 1.350.542,52</t>
+  </si>
+  <si>
+    <t>2026NP401762</t>
+  </si>
+  <si>
+    <t>2025NE002237</t>
+  </si>
+  <si>
+    <t>25E2058</t>
+  </si>
+  <si>
+    <t>ABR/26</t>
+  </si>
+  <si>
+    <t>2025NE000770, 2025NE001065, 2025NE001627</t>
+  </si>
+  <si>
+    <t>2026NE000330</t>
+  </si>
+  <si>
+    <t>C26163</t>
+  </si>
+  <si>
+    <t>26E0320</t>
+  </si>
+  <si>
+    <t>REAJUSTE</t>
+  </si>
+  <si>
+    <t>2026NE000388</t>
+  </si>
+  <si>
+    <t>C26193</t>
+  </si>
+  <si>
+    <t>2026NP402148</t>
+  </si>
+  <si>
+    <t>26E0375</t>
+  </si>
+  <si>
+    <t>MAIO/26</t>
+  </si>
+  <si>
+    <t>2026NE000748</t>
+  </si>
+  <si>
+    <t>C26312</t>
+  </si>
+  <si>
+    <t>26E0709</t>
+  </si>
+  <si>
+    <t>2026NP402373</t>
+  </si>
+  <si>
+    <t>2026NE000816</t>
+  </si>
+  <si>
+    <t>JUNHO/26</t>
+  </si>
+  <si>
+    <t>C26324</t>
+  </si>
+  <si>
+    <t>26E0776</t>
+  </si>
+  <si>
+    <t>2025NE001065, 2026NE000330</t>
+  </si>
+  <si>
+    <t>R$ 1.340.865,98</t>
+  </si>
+  <si>
+    <t>2026NP402899</t>
+  </si>
+  <si>
     <t>2026NE000817</t>
   </si>
   <si>
+    <t>JULHO/26</t>
+  </si>
+  <si>
     <t>C26326</t>
   </si>
   <si>
-    <t>2025NP004897</t>
-  </si>
-  <si>
     <t>26E0777</t>
   </si>
   <si>
-    <t>OUT/25</t>
-  </si>
-  <si>
     <t>2026NE000842</t>
   </si>
   <si>
     <t>26E0803</t>
   </si>
   <si>
-    <t>2025NE001688, 2025NE001828, 2025NE002200</t>
-  </si>
-  <si>
     <t>2026NE000944</t>
   </si>
   <si>
-    <t>2025NP004932</t>
-  </si>
-  <si>
     <t>26E0906</t>
   </si>
   <si>
+    <t>Módulo II – Parcial Orçamento 10 (FAB 2728)</t>
+  </si>
+  <si>
     <t>2026NE001015</t>
   </si>
   <si>
@@ -502,91 +583,10 @@
     <t>26E0959</t>
   </si>
   <si>
-    <t>NOV/25</t>
+    <t>2025NP002620</t>
   </si>
   <si>
     <t>20XV</t>
-  </si>
-  <si>
-    <t>2025NE001687, 2025NE001689, 2025NE001690, 2025NE001823, 2025NE001830, 2025NE002237</t>
-  </si>
-  <si>
-    <t>2026NP400440</t>
-  </si>
-  <si>
-    <t>DEZ/25</t>
-  </si>
-  <si>
-    <t>2025NE001065, 2025NE002200</t>
-  </si>
-  <si>
-    <t>2026NP400412</t>
-  </si>
-  <si>
-    <t>JAN/26</t>
-  </si>
-  <si>
-    <t>2026NP401035</t>
-  </si>
-  <si>
-    <t>FEV/26</t>
-  </si>
-  <si>
-    <t>2025NE001627, 2025NE001629, 2025NE001823</t>
-  </si>
-  <si>
-    <t>2026NP402272</t>
-  </si>
-  <si>
-    <t>MAR/26</t>
-  </si>
-  <si>
-    <t>2025NE000770, 2025NE001627</t>
-  </si>
-  <si>
-    <t>R$ 1.350.542,52</t>
-  </si>
-  <si>
-    <t>2026NP401762</t>
-  </si>
-  <si>
-    <t>ABR/26</t>
-  </si>
-  <si>
-    <t>2025NE000770, 2025NE001065, 2025NE001627</t>
-  </si>
-  <si>
-    <t>REAJUSTE</t>
-  </si>
-  <si>
-    <t>2026NP402148</t>
-  </si>
-  <si>
-    <t>MAIO/26</t>
-  </si>
-  <si>
-    <t>2026NP402373</t>
-  </si>
-  <si>
-    <t>JUNHO/26</t>
-  </si>
-  <si>
-    <t>2025NE001065, 2026NE000330</t>
-  </si>
-  <si>
-    <t>R$ 1.340.865,98</t>
-  </si>
-  <si>
-    <t>2026NP402899</t>
-  </si>
-  <si>
-    <t>JULHO/26</t>
-  </si>
-  <si>
-    <t>Módulo II – Parcial Orçamento 10 (FAB 2728)</t>
-  </si>
-  <si>
-    <t>2025NP002620</t>
   </si>
   <si>
     <t>Módulo II – Orçamento 06 (Hélice)</t>
@@ -740,15 +740,15 @@
       <name val="Arial"/>
     </font>
     <font>
+      <sz val="10.0"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+    </font>
+    <font>
       <b/>
       <sz val="10.0"/>
       <color theme="1"/>
       <name val="Century Gothic"/>
-    </font>
-    <font>
-      <sz val="10.0"/>
-      <color theme="1"/>
-      <name val="Times New Roman"/>
     </font>
     <font>
       <b/>
@@ -895,22 +895,22 @@
     <xf borderId="0" fillId="5" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
+    <xf borderId="0" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment vertical="center"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="11" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
@@ -965,31 +965,30 @@
     <xf borderId="1" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="7" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf borderId="1" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="2" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="2" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="6" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="8" numFmtId="166" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="8" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="7" numFmtId="166" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="7" fontId="9" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="165" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="1" fillId="5" fontId="9" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
@@ -1000,19 +999,17 @@
     <xf borderId="1" fillId="8" fontId="9" numFmtId="168" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="8" numFmtId="166" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="165" xfId="0" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="1" fillId="0" fontId="7" numFmtId="166" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="8" numFmtId="169" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="7" numFmtId="169" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="7" fontId="9" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="170" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="8" fontId="9" numFmtId="168" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
@@ -1029,6 +1026,9 @@
     </xf>
     <xf borderId="0" fillId="3" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="170" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="1" fillId="9" fontId="9" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
@@ -1058,7 +1058,7 @@
     <xf borderId="5" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="8" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="7" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="4" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
@@ -1067,10 +1067,10 @@
     <xf borderId="1" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="8" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="7" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="8" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="7" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="5" fontId="9" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
@@ -1447,38 +1447,38 @@
       <c r="B2" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="V2" s="6"/>
-      <c r="W2" s="7"/>
-      <c r="X2" s="7"/>
-      <c r="Y2" s="7"/>
-      <c r="Z2" s="7"/>
-      <c r="AA2" s="7"/>
-      <c r="AB2" s="7"/>
-      <c r="AC2" s="7"/>
-      <c r="AD2" s="7"/>
+      <c r="V2" s="7"/>
+      <c r="W2" s="9"/>
+      <c r="X2" s="9"/>
+      <c r="Y2" s="9"/>
+      <c r="Z2" s="9"/>
+      <c r="AA2" s="9"/>
+      <c r="AB2" s="9"/>
+      <c r="AC2" s="9"/>
+      <c r="AD2" s="9"/>
     </row>
     <row r="3" ht="12.75" customHeight="1">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
-      <c r="C3" s="9"/>
-      <c r="D3" s="9"/>
-      <c r="E3" s="9"/>
-      <c r="F3" s="9"/>
-      <c r="G3" s="9"/>
-      <c r="H3" s="9"/>
-      <c r="I3" s="9"/>
-      <c r="J3" s="9"/>
-      <c r="K3" s="9"/>
-      <c r="L3" s="9"/>
-      <c r="M3" s="9"/>
-      <c r="N3" s="9"/>
-      <c r="O3" s="9"/>
-      <c r="P3" s="9"/>
-      <c r="Q3" s="9"/>
-      <c r="R3" s="9"/>
-      <c r="S3" s="9"/>
-      <c r="T3" s="9"/>
-      <c r="U3" s="9"/>
+      <c r="C3" s="11"/>
+      <c r="D3" s="11"/>
+      <c r="E3" s="11"/>
+      <c r="F3" s="11"/>
+      <c r="G3" s="11"/>
+      <c r="H3" s="11"/>
+      <c r="I3" s="11"/>
+      <c r="J3" s="11"/>
+      <c r="K3" s="11"/>
+      <c r="L3" s="11"/>
+      <c r="M3" s="11"/>
+      <c r="N3" s="11"/>
+      <c r="O3" s="11"/>
+      <c r="P3" s="11"/>
+      <c r="Q3" s="11"/>
+      <c r="R3" s="11"/>
+      <c r="S3" s="11"/>
+      <c r="T3" s="11"/>
+      <c r="U3" s="11"/>
       <c r="V3" s="2"/>
     </row>
     <row r="4" ht="12.75" customHeight="1">
@@ -1506,31 +1506,31 @@
         <v>12</v>
       </c>
       <c r="J4" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="K4" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="K4" s="15" t="s">
+      <c r="L4" s="15" t="s">
+        <v>15</v>
+      </c>
+      <c r="M4" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="L4" s="15" t="s">
+      <c r="N4" s="17" t="s">
+        <v>17</v>
+      </c>
+      <c r="O4" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="M4" s="17" t="s">
-        <v>19</v>
-      </c>
-      <c r="N4" s="17" t="s">
+      <c r="P4" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="O4" s="17" t="s">
+      <c r="Q4" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="P4" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="Q4" s="17" t="s">
+      <c r="R4" s="15" t="s">
         <v>23</v>
-      </c>
-      <c r="R4" s="15" t="s">
-        <v>24</v>
       </c>
       <c r="S4" s="15" t="s">
         <v>25</v>
@@ -1548,16 +1548,16 @@
       <c r="B5" s="14"/>
       <c r="C5" s="18"/>
       <c r="D5" s="19" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="E5" s="19" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="F5" s="19" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="G5" s="19" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="H5" s="20">
         <v>1564.0</v>
@@ -1566,16 +1566,16 @@
         <v>1564.0</v>
       </c>
       <c r="J5" s="19" t="s">
+        <v>31</v>
+      </c>
+      <c r="K5" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="L5" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="K5" s="19" t="s">
+      <c r="M5" s="19" t="s">
         <v>35</v>
-      </c>
-      <c r="L5" s="19" t="s">
-        <v>37</v>
-      </c>
-      <c r="M5" s="19" t="s">
-        <v>38</v>
       </c>
       <c r="N5" s="21">
         <v>9.165159737E7</v>
@@ -1593,7 +1593,7 @@
         <v>1.085943044E7</v>
       </c>
       <c r="S5" s="19" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="V5" s="2"/>
     </row>
@@ -1626,40 +1626,40 @@
       <c r="A8" s="23"/>
       <c r="B8" s="23"/>
       <c r="C8" s="28" t="s">
+        <v>41</v>
+      </c>
+      <c r="D8" s="28" t="s">
+        <v>42</v>
+      </c>
+      <c r="E8" s="29" t="s">
+        <v>43</v>
+      </c>
+      <c r="F8" s="28" t="s">
         <v>45</v>
       </c>
-      <c r="D8" s="28" t="s">
+      <c r="G8" s="28" t="s">
+        <v>47</v>
+      </c>
+      <c r="H8" s="28" t="s">
         <v>49</v>
       </c>
-      <c r="E8" s="29" t="s">
+      <c r="I8" s="29" t="s">
         <v>50</v>
       </c>
-      <c r="F8" s="28" t="s">
+      <c r="J8" s="28" t="s">
+        <v>51</v>
+      </c>
+      <c r="K8" s="28" t="s">
         <v>52</v>
       </c>
-      <c r="G8" s="28" t="s">
+      <c r="L8" s="30" t="s">
         <v>53</v>
       </c>
-      <c r="H8" s="28" t="s">
-        <v>54</v>
-      </c>
-      <c r="I8" s="29" t="s">
+      <c r="M8" s="29" t="s">
         <v>55</v>
       </c>
-      <c r="J8" s="28" t="s">
+      <c r="N8" s="28" t="s">
         <v>56</v>
-      </c>
-      <c r="K8" s="28" t="s">
-        <v>57</v>
-      </c>
-      <c r="L8" s="31" t="s">
-        <v>58</v>
-      </c>
-      <c r="M8" s="29" t="s">
-        <v>59</v>
-      </c>
-      <c r="N8" s="28" t="s">
-        <v>60</v>
       </c>
       <c r="O8" s="28"/>
       <c r="P8" s="27"/>
@@ -1668,23 +1668,23 @@
     <row r="9" ht="19.5" customHeight="1">
       <c r="A9" s="23"/>
       <c r="B9" s="23"/>
-      <c r="C9" s="32">
+      <c r="C9" s="31">
         <v>1.0</v>
       </c>
-      <c r="D9" s="33" t="s">
-        <v>66</v>
-      </c>
-      <c r="E9" s="34" t="s">
-        <v>67</v>
-      </c>
-      <c r="F9" s="35">
+      <c r="D9" s="32" t="s">
+        <v>60</v>
+      </c>
+      <c r="E9" s="33" t="s">
+        <v>62</v>
+      </c>
+      <c r="F9" s="34">
         <v>594.0</v>
       </c>
       <c r="G9" s="36">
         <v>45740.0</v>
       </c>
-      <c r="H9" s="35" t="s">
-        <v>69</v>
+      <c r="H9" s="34" t="s">
+        <v>63</v>
       </c>
       <c r="I9" s="36"/>
       <c r="J9" s="36">
@@ -1693,14 +1693,14 @@
       <c r="K9" s="37">
         <v>748504.24</v>
       </c>
-      <c r="L9" s="35" t="s">
-        <v>72</v>
-      </c>
-      <c r="M9" s="39">
+      <c r="L9" s="34" t="s">
+        <v>67</v>
+      </c>
+      <c r="M9" s="38">
         <f t="shared" ref="M9:M10" si="1">K9</f>
         <v>748504.24</v>
       </c>
-      <c r="N9" s="40"/>
+      <c r="N9" s="39"/>
       <c r="O9" s="25"/>
       <c r="P9" s="27"/>
       <c r="V9" s="2"/>
@@ -1708,21 +1708,21 @@
     <row r="10" ht="51.0" customHeight="1">
       <c r="A10" s="23"/>
       <c r="B10" s="23"/>
-      <c r="C10" s="41"/>
-      <c r="D10" s="33" t="s">
-        <v>85</v>
-      </c>
-      <c r="E10" s="34" t="s">
-        <v>67</v>
-      </c>
-      <c r="F10" s="35">
+      <c r="C10" s="40"/>
+      <c r="D10" s="32" t="s">
+        <v>73</v>
+      </c>
+      <c r="E10" s="33" t="s">
+        <v>62</v>
+      </c>
+      <c r="F10" s="34">
         <v>620.0</v>
       </c>
       <c r="G10" s="36">
         <v>45775.0</v>
       </c>
-      <c r="H10" s="35" t="s">
-        <v>88</v>
+      <c r="H10" s="34" t="s">
+        <v>74</v>
       </c>
       <c r="I10" s="36"/>
       <c r="J10" s="36">
@@ -1731,14 +1731,14 @@
       <c r="K10" s="37">
         <v>1110378.24</v>
       </c>
-      <c r="L10" s="35" t="s">
-        <v>89</v>
-      </c>
-      <c r="M10" s="39">
+      <c r="L10" s="34" t="s">
+        <v>75</v>
+      </c>
+      <c r="M10" s="38">
         <f t="shared" si="1"/>
         <v>1110378.24</v>
       </c>
-      <c r="N10" s="42"/>
+      <c r="N10" s="41"/>
       <c r="O10" s="25"/>
       <c r="P10" s="27"/>
       <c r="V10" s="2"/>
@@ -1746,21 +1746,21 @@
     <row r="11" ht="12.75" customHeight="1">
       <c r="A11" s="23"/>
       <c r="B11" s="23"/>
-      <c r="C11" s="41"/>
-      <c r="D11" s="33" t="s">
-        <v>93</v>
-      </c>
-      <c r="E11" s="34" t="s">
-        <v>67</v>
-      </c>
-      <c r="F11" s="35">
+      <c r="C11" s="40"/>
+      <c r="D11" s="32" t="s">
+        <v>80</v>
+      </c>
+      <c r="E11" s="33" t="s">
+        <v>62</v>
+      </c>
+      <c r="F11" s="34">
         <v>634.0</v>
       </c>
       <c r="G11" s="36">
         <v>45799.0</v>
       </c>
-      <c r="H11" s="35" t="s">
-        <v>96</v>
+      <c r="H11" s="34" t="s">
+        <v>82</v>
       </c>
       <c r="I11" s="36"/>
       <c r="J11" s="36">
@@ -1769,13 +1769,13 @@
       <c r="K11" s="37">
         <v>974557.12</v>
       </c>
-      <c r="L11" s="34" t="s">
-        <v>99</v>
-      </c>
-      <c r="M11" s="39">
+      <c r="L11" s="33" t="s">
+        <v>84</v>
+      </c>
+      <c r="M11" s="38">
         <v>974557.12</v>
       </c>
-      <c r="N11" s="42"/>
+      <c r="N11" s="41"/>
       <c r="O11" s="25"/>
       <c r="P11" s="27"/>
       <c r="V11" s="2"/>
@@ -1783,21 +1783,21 @@
     <row r="12" ht="27.75" customHeight="1">
       <c r="A12" s="23"/>
       <c r="B12" s="23"/>
-      <c r="C12" s="41"/>
-      <c r="D12" s="33" t="s">
-        <v>102</v>
-      </c>
-      <c r="E12" s="34" t="s">
-        <v>67</v>
-      </c>
-      <c r="F12" s="34">
+      <c r="C12" s="40"/>
+      <c r="D12" s="32" t="s">
+        <v>85</v>
+      </c>
+      <c r="E12" s="33" t="s">
+        <v>62</v>
+      </c>
+      <c r="F12" s="33">
         <v>660.0</v>
       </c>
       <c r="G12" s="43">
         <v>45856.0</v>
       </c>
       <c r="H12" s="44" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I12" s="36"/>
       <c r="J12" s="36">
@@ -1806,13 +1806,13 @@
       <c r="K12" s="45">
         <v>1402001.34</v>
       </c>
-      <c r="L12" s="47" t="s">
-        <v>108</v>
-      </c>
-      <c r="M12" s="39">
+      <c r="L12" s="46" t="s">
+        <v>89</v>
+      </c>
+      <c r="M12" s="38">
         <v>1402001.34</v>
       </c>
-      <c r="N12" s="48"/>
+      <c r="N12" s="47"/>
       <c r="O12" s="25"/>
       <c r="P12" s="27"/>
       <c r="V12" s="2"/>
@@ -1820,21 +1820,21 @@
     <row r="13">
       <c r="A13" s="23"/>
       <c r="B13" s="23"/>
-      <c r="C13" s="41"/>
-      <c r="D13" s="49" t="s">
-        <v>113</v>
-      </c>
-      <c r="E13" s="34" t="s">
-        <v>67</v>
-      </c>
-      <c r="F13" s="35">
+      <c r="C13" s="40"/>
+      <c r="D13" s="48" t="s">
+        <v>93</v>
+      </c>
+      <c r="E13" s="33" t="s">
+        <v>62</v>
+      </c>
+      <c r="F13" s="34">
         <v>661.0</v>
       </c>
       <c r="G13" s="36">
         <v>45856.0</v>
       </c>
-      <c r="H13" s="35" t="s">
-        <v>116</v>
+      <c r="H13" s="34" t="s">
+        <v>95</v>
       </c>
       <c r="I13" s="43"/>
       <c r="J13" s="43">
@@ -1843,35 +1843,35 @@
       <c r="K13" s="45">
         <v>1223702.3</v>
       </c>
-      <c r="L13" s="34" t="s">
-        <v>117</v>
-      </c>
-      <c r="M13" s="39">
+      <c r="L13" s="33" t="s">
+        <v>97</v>
+      </c>
+      <c r="M13" s="38">
         <v>1223702.3</v>
       </c>
-      <c r="N13" s="48"/>
+      <c r="N13" s="47"/>
       <c r="O13" s="25"/>
-      <c r="P13" s="50"/>
+      <c r="P13" s="49"/>
       <c r="V13" s="2"/>
     </row>
     <row r="14">
       <c r="A14" s="23"/>
       <c r="B14" s="23"/>
-      <c r="C14" s="41"/>
-      <c r="D14" s="49" t="s">
-        <v>121</v>
-      </c>
-      <c r="E14" s="34" t="s">
-        <v>67</v>
-      </c>
-      <c r="F14" s="34">
+      <c r="C14" s="40"/>
+      <c r="D14" s="48" t="s">
+        <v>98</v>
+      </c>
+      <c r="E14" s="33" t="s">
+        <v>62</v>
+      </c>
+      <c r="F14" s="33">
         <v>688.0</v>
       </c>
       <c r="G14" s="36">
         <v>45901.0</v>
       </c>
-      <c r="H14" s="34" t="s">
-        <v>124</v>
+      <c r="H14" s="33" t="s">
+        <v>102</v>
       </c>
       <c r="I14" s="43"/>
       <c r="J14" s="43">
@@ -1880,13 +1880,13 @@
       <c r="K14" s="45">
         <v>1011677.95</v>
       </c>
-      <c r="L14" s="34" t="s">
-        <v>128</v>
-      </c>
-      <c r="M14" s="39">
+      <c r="L14" s="33" t="s">
+        <v>103</v>
+      </c>
+      <c r="M14" s="38">
         <v>1011677.95</v>
       </c>
-      <c r="N14" s="42"/>
+      <c r="N14" s="41"/>
       <c r="O14" s="25"/>
       <c r="P14" s="27"/>
       <c r="V14" s="2"/>
@@ -1894,21 +1894,21 @@
     <row r="15">
       <c r="A15" s="23"/>
       <c r="B15" s="23"/>
-      <c r="C15" s="41"/>
-      <c r="D15" s="49" t="s">
-        <v>130</v>
-      </c>
-      <c r="E15" s="34" t="s">
-        <v>67</v>
-      </c>
-      <c r="F15" s="34">
+      <c r="C15" s="40"/>
+      <c r="D15" s="48" t="s">
+        <v>104</v>
+      </c>
+      <c r="E15" s="33" t="s">
+        <v>62</v>
+      </c>
+      <c r="F15" s="33">
         <v>696.0</v>
       </c>
       <c r="G15" s="36">
         <v>45923.0</v>
       </c>
-      <c r="H15" s="34" t="s">
-        <v>79</v>
+      <c r="H15" s="33" t="s">
+        <v>86</v>
       </c>
       <c r="I15" s="43"/>
       <c r="J15" s="43">
@@ -1917,34 +1917,34 @@
       <c r="K15" s="45">
         <v>896744.06</v>
       </c>
-      <c r="L15" s="34" t="s">
-        <v>136</v>
-      </c>
-      <c r="M15" s="39">
+      <c r="L15" s="33" t="s">
+        <v>107</v>
+      </c>
+      <c r="M15" s="38">
         <v>896744.06</v>
       </c>
-      <c r="N15" s="48"/>
+      <c r="N15" s="47"/>
       <c r="O15" s="25"/>
       <c r="V15" s="2"/>
     </row>
     <row r="16">
       <c r="A16" s="23"/>
       <c r="B16" s="23"/>
-      <c r="C16" s="41"/>
-      <c r="D16" s="49" t="s">
-        <v>137</v>
-      </c>
-      <c r="E16" s="34" t="s">
-        <v>67</v>
-      </c>
-      <c r="F16" s="34">
+      <c r="C16" s="40"/>
+      <c r="D16" s="48" t="s">
+        <v>108</v>
+      </c>
+      <c r="E16" s="33" t="s">
+        <v>62</v>
+      </c>
+      <c r="F16" s="33">
         <v>704.0</v>
       </c>
       <c r="G16" s="36">
         <v>45957.0</v>
       </c>
-      <c r="H16" s="34" t="s">
-        <v>141</v>
+      <c r="H16" s="33" t="s">
+        <v>110</v>
       </c>
       <c r="I16" s="43"/>
       <c r="J16" s="43">
@@ -1953,108 +1953,108 @@
       <c r="K16" s="45">
         <v>919329.06</v>
       </c>
-      <c r="L16" s="34" t="s">
-        <v>144</v>
-      </c>
-      <c r="M16" s="39">
+      <c r="L16" s="33" t="s">
+        <v>112</v>
+      </c>
+      <c r="M16" s="38">
         <v>919329.06</v>
       </c>
-      <c r="N16" s="42"/>
+      <c r="N16" s="41"/>
       <c r="O16" s="25"/>
       <c r="V16" s="2"/>
     </row>
     <row r="17">
       <c r="A17" s="23"/>
       <c r="B17" s="23"/>
-      <c r="C17" s="41"/>
-      <c r="D17" s="49" t="s">
-        <v>146</v>
-      </c>
-      <c r="E17" s="34"/>
-      <c r="F17" s="34">
+      <c r="C17" s="40"/>
+      <c r="D17" s="48" t="s">
+        <v>113</v>
+      </c>
+      <c r="E17" s="33"/>
+      <c r="F17" s="33">
         <v>705.0</v>
       </c>
       <c r="G17" s="43">
         <v>45972.0</v>
       </c>
-      <c r="H17" s="34" t="s">
-        <v>149</v>
-      </c>
-      <c r="I17" s="34"/>
+      <c r="H17" s="33" t="s">
+        <v>114</v>
+      </c>
+      <c r="I17" s="33"/>
       <c r="J17" s="43">
         <v>46016.0</v>
       </c>
       <c r="K17" s="45">
         <v>1157009.26</v>
       </c>
-      <c r="L17" s="34" t="s">
-        <v>151</v>
-      </c>
-      <c r="M17" s="39">
+      <c r="L17" s="33" t="s">
+        <v>117</v>
+      </c>
+      <c r="M17" s="38">
         <v>1157009.26</v>
       </c>
-      <c r="N17" s="51"/>
+      <c r="N17" s="50"/>
       <c r="O17" s="25"/>
       <c r="V17" s="2"/>
     </row>
     <row r="18">
       <c r="A18" s="23"/>
       <c r="B18" s="23"/>
-      <c r="C18" s="41"/>
-      <c r="D18" s="49" t="s">
-        <v>156</v>
-      </c>
-      <c r="E18" s="34" t="s">
-        <v>67</v>
-      </c>
-      <c r="F18" s="34">
+      <c r="C18" s="40"/>
+      <c r="D18" s="48" t="s">
+        <v>118</v>
+      </c>
+      <c r="E18" s="33" t="s">
+        <v>62</v>
+      </c>
+      <c r="F18" s="33">
         <v>728.0</v>
       </c>
       <c r="G18" s="43">
         <v>46008.0</v>
       </c>
-      <c r="H18" s="34" t="s">
-        <v>158</v>
-      </c>
-      <c r="I18" s="34"/>
+      <c r="H18" s="33" t="s">
+        <v>121</v>
+      </c>
+      <c r="I18" s="33"/>
       <c r="J18" s="43">
         <v>46040.0</v>
       </c>
       <c r="K18" s="45">
         <v>1214597.952</v>
       </c>
-      <c r="L18" s="34" t="s">
-        <v>159</v>
-      </c>
-      <c r="M18" s="39">
+      <c r="L18" s="33" t="s">
+        <v>122</v>
+      </c>
+      <c r="M18" s="38">
         <v>1214597.952</v>
       </c>
-      <c r="N18" s="51"/>
+      <c r="N18" s="50"/>
       <c r="O18" s="25"/>
       <c r="R18" s="27"/>
       <c r="S18" s="27"/>
       <c r="T18" s="27"/>
       <c r="U18" s="27"/>
-      <c r="V18" s="52"/>
+      <c r="V18" s="51"/>
     </row>
     <row r="19">
       <c r="A19" s="23"/>
       <c r="B19" s="23"/>
-      <c r="C19" s="41"/>
-      <c r="D19" s="49" t="s">
-        <v>160</v>
-      </c>
-      <c r="E19" s="34" t="s">
-        <v>67</v>
-      </c>
-      <c r="F19" s="34">
+      <c r="C19" s="40"/>
+      <c r="D19" s="48" t="s">
+        <v>126</v>
+      </c>
+      <c r="E19" s="33" t="s">
+        <v>62</v>
+      </c>
+      <c r="F19" s="33">
         <v>278.0</v>
       </c>
       <c r="G19" s="43">
         <v>46042.0</v>
       </c>
-      <c r="H19" s="34" t="s">
-        <v>161</v>
+      <c r="H19" s="33" t="s">
+        <v>127</v>
       </c>
       <c r="I19" s="43"/>
       <c r="J19" s="43">
@@ -2063,36 +2063,36 @@
       <c r="K19" s="45">
         <v>967082.09</v>
       </c>
-      <c r="L19" s="34" t="s">
-        <v>162</v>
-      </c>
-      <c r="M19" s="39">
+      <c r="L19" s="33" t="s">
+        <v>128</v>
+      </c>
+      <c r="M19" s="38">
         <v>967082.09</v>
       </c>
-      <c r="N19" s="51"/>
+      <c r="N19" s="50"/>
       <c r="O19" s="25"/>
       <c r="R19" s="27"/>
       <c r="S19" s="27"/>
       <c r="T19" s="27"/>
       <c r="U19" s="27"/>
-      <c r="V19" s="52"/>
+      <c r="V19" s="51"/>
     </row>
     <row r="20">
       <c r="A20" s="23"/>
       <c r="B20" s="23"/>
-      <c r="C20" s="41"/>
-      <c r="D20" s="49" t="s">
-        <v>163</v>
-      </c>
-      <c r="E20" s="34"/>
-      <c r="F20" s="34">
+      <c r="C20" s="40"/>
+      <c r="D20" s="48" t="s">
+        <v>130</v>
+      </c>
+      <c r="E20" s="33"/>
+      <c r="F20" s="33">
         <v>10.0</v>
       </c>
       <c r="G20" s="43">
         <v>46078.0</v>
       </c>
-      <c r="H20" s="34" t="s">
-        <v>105</v>
+      <c r="H20" s="33" t="s">
+        <v>123</v>
       </c>
       <c r="I20" s="43"/>
       <c r="J20" s="43">
@@ -2101,36 +2101,36 @@
       <c r="K20" s="45">
         <v>719561.08</v>
       </c>
-      <c r="L20" s="34" t="s">
-        <v>164</v>
-      </c>
-      <c r="M20" s="39">
+      <c r="L20" s="33" t="s">
+        <v>133</v>
+      </c>
+      <c r="M20" s="38">
         <v>719561.08</v>
       </c>
-      <c r="N20" s="51"/>
+      <c r="N20" s="50"/>
       <c r="O20" s="25"/>
       <c r="R20" s="27"/>
       <c r="S20" s="27"/>
       <c r="T20" s="27"/>
       <c r="U20" s="27"/>
-      <c r="V20" s="52"/>
+      <c r="V20" s="51"/>
     </row>
     <row r="21">
       <c r="A21" s="23"/>
       <c r="B21" s="23"/>
-      <c r="C21" s="41"/>
-      <c r="D21" s="49" t="s">
-        <v>165</v>
-      </c>
-      <c r="E21" s="34"/>
-      <c r="F21" s="34">
+      <c r="C21" s="40"/>
+      <c r="D21" s="48" t="s">
+        <v>136</v>
+      </c>
+      <c r="E21" s="33"/>
+      <c r="F21" s="33">
         <v>15.0</v>
       </c>
       <c r="G21" s="43">
         <v>46094.0</v>
       </c>
-      <c r="H21" s="34" t="s">
-        <v>166</v>
+      <c r="H21" s="33" t="s">
+        <v>138</v>
       </c>
       <c r="I21" s="43"/>
       <c r="J21" s="43">
@@ -2139,74 +2139,74 @@
       <c r="K21" s="45">
         <v>885881.08</v>
       </c>
-      <c r="L21" s="34" t="s">
-        <v>167</v>
-      </c>
-      <c r="M21" s="39">
+      <c r="L21" s="33" t="s">
+        <v>139</v>
+      </c>
+      <c r="M21" s="38">
         <v>885881.08</v>
       </c>
-      <c r="N21" s="51"/>
+      <c r="N21" s="50"/>
       <c r="O21" s="25"/>
       <c r="R21" s="27"/>
       <c r="S21" s="27"/>
       <c r="T21" s="27"/>
       <c r="U21" s="27"/>
-      <c r="V21" s="52"/>
+      <c r="V21" s="51"/>
     </row>
     <row r="22">
       <c r="A22" s="23"/>
       <c r="B22" s="23"/>
-      <c r="C22" s="41"/>
-      <c r="D22" s="49" t="s">
-        <v>168</v>
-      </c>
-      <c r="E22" s="34"/>
-      <c r="F22" s="34">
+      <c r="C22" s="40"/>
+      <c r="D22" s="48" t="s">
+        <v>141</v>
+      </c>
+      <c r="E22" s="33"/>
+      <c r="F22" s="33">
         <v>28.0</v>
       </c>
       <c r="G22" s="43">
         <v>46128.0</v>
       </c>
-      <c r="H22" s="34" t="s">
-        <v>169</v>
+      <c r="H22" s="33" t="s">
+        <v>144</v>
       </c>
       <c r="I22" s="43"/>
       <c r="J22" s="43">
         <v>46164.0</v>
       </c>
       <c r="K22" s="45" t="s">
-        <v>170</v>
-      </c>
-      <c r="L22" s="34" t="s">
-        <v>171</v>
-      </c>
-      <c r="M22" s="39" t="s">
-        <v>170</v>
-      </c>
-      <c r="N22" s="51"/>
+        <v>145</v>
+      </c>
+      <c r="L22" s="33" t="s">
+        <v>146</v>
+      </c>
+      <c r="M22" s="38" t="s">
+        <v>145</v>
+      </c>
+      <c r="N22" s="50"/>
       <c r="O22" s="25"/>
       <c r="R22" s="27"/>
       <c r="S22" s="27"/>
       <c r="T22" s="27"/>
       <c r="U22" s="27"/>
-      <c r="V22" s="52"/>
+      <c r="V22" s="51"/>
     </row>
     <row r="23">
       <c r="A23" s="23"/>
       <c r="B23" s="23"/>
-      <c r="C23" s="41"/>
-      <c r="D23" s="49" t="s">
-        <v>172</v>
-      </c>
-      <c r="E23" s="34"/>
-      <c r="F23" s="34">
+      <c r="C23" s="40"/>
+      <c r="D23" s="48" t="s">
+        <v>149</v>
+      </c>
+      <c r="E23" s="33"/>
+      <c r="F23" s="33">
         <v>33.0</v>
       </c>
       <c r="G23" s="43">
         <v>46156.0</v>
       </c>
-      <c r="H23" s="34" t="s">
-        <v>173</v>
+      <c r="H23" s="33" t="s">
+        <v>150</v>
       </c>
       <c r="I23" s="43"/>
       <c r="J23" s="43">
@@ -2215,10 +2215,10 @@
       <c r="K23" s="45">
         <v>1108954.4358333333</v>
       </c>
-      <c r="L23" s="34" t="s">
-        <v>167</v>
-      </c>
-      <c r="M23" s="39">
+      <c r="L23" s="33" t="s">
+        <v>139</v>
+      </c>
+      <c r="M23" s="38">
         <v>1108954.4358333333</v>
       </c>
       <c r="N23" s="53"/>
@@ -2227,24 +2227,24 @@
       <c r="S23" s="27"/>
       <c r="T23" s="27"/>
       <c r="U23" s="27"/>
-      <c r="V23" s="52"/>
+      <c r="V23" s="51"/>
     </row>
     <row r="24">
       <c r="A24" s="23"/>
       <c r="B24" s="23"/>
-      <c r="C24" s="41"/>
-      <c r="D24" s="49" t="s">
-        <v>174</v>
-      </c>
-      <c r="E24" s="34"/>
-      <c r="F24" s="34">
+      <c r="C24" s="40"/>
+      <c r="D24" s="48" t="s">
+        <v>154</v>
+      </c>
+      <c r="E24" s="33"/>
+      <c r="F24" s="33">
         <v>29.0</v>
       </c>
       <c r="G24" s="43">
         <v>46149.0</v>
       </c>
-      <c r="H24" s="34" t="s">
-        <v>173</v>
+      <c r="H24" s="33" t="s">
+        <v>150</v>
       </c>
       <c r="I24" s="43"/>
       <c r="J24" s="43">
@@ -2253,10 +2253,10 @@
       <c r="K24" s="45">
         <v>218206.1</v>
       </c>
-      <c r="L24" s="34" t="s">
-        <v>175</v>
-      </c>
-      <c r="M24" s="39">
+      <c r="L24" s="33" t="s">
+        <v>157</v>
+      </c>
+      <c r="M24" s="38">
         <v>218206.1</v>
       </c>
       <c r="N24" s="54"/>
@@ -2265,24 +2265,24 @@
       <c r="S24" s="27"/>
       <c r="T24" s="27"/>
       <c r="U24" s="27"/>
-      <c r="V24" s="52"/>
+      <c r="V24" s="51"/>
     </row>
     <row r="25">
       <c r="A25" s="23"/>
       <c r="B25" s="23"/>
-      <c r="C25" s="41"/>
-      <c r="D25" s="49" t="s">
-        <v>176</v>
-      </c>
-      <c r="E25" s="34"/>
-      <c r="F25" s="34">
+      <c r="C25" s="40"/>
+      <c r="D25" s="48" t="s">
+        <v>159</v>
+      </c>
+      <c r="E25" s="33"/>
+      <c r="F25" s="33">
         <v>40.0</v>
       </c>
       <c r="G25" s="43">
         <v>46156.0</v>
       </c>
-      <c r="H25" s="34" t="s">
-        <v>173</v>
+      <c r="H25" s="33" t="s">
+        <v>150</v>
       </c>
       <c r="I25" s="43"/>
       <c r="J25" s="43">
@@ -2291,10 +2291,10 @@
       <c r="K25" s="45">
         <v>1549250.84</v>
       </c>
-      <c r="L25" s="34" t="s">
-        <v>177</v>
-      </c>
-      <c r="M25" s="39">
+      <c r="L25" s="33" t="s">
+        <v>163</v>
+      </c>
+      <c r="M25" s="38">
         <v>1549250.84</v>
       </c>
       <c r="N25" s="54"/>
@@ -2303,37 +2303,37 @@
       <c r="S25" s="27"/>
       <c r="T25" s="27"/>
       <c r="U25" s="27"/>
-      <c r="V25" s="52"/>
+      <c r="V25" s="51"/>
     </row>
     <row r="26">
       <c r="A26" s="23"/>
       <c r="B26" s="23"/>
       <c r="C26" s="55"/>
-      <c r="D26" s="49" t="s">
-        <v>178</v>
-      </c>
-      <c r="E26" s="34"/>
-      <c r="F26" s="34">
+      <c r="D26" s="48" t="s">
+        <v>165</v>
+      </c>
+      <c r="E26" s="33"/>
+      <c r="F26" s="33">
         <v>48.0</v>
       </c>
       <c r="G26" s="43">
         <v>46230.0</v>
       </c>
-      <c r="H26" s="34" t="s">
-        <v>179</v>
+      <c r="H26" s="33" t="s">
+        <v>168</v>
       </c>
       <c r="I26" s="43"/>
       <c r="J26" s="43">
         <v>46262.0</v>
       </c>
       <c r="K26" s="45" t="s">
-        <v>180</v>
-      </c>
-      <c r="L26" s="34" t="s">
-        <v>181</v>
-      </c>
-      <c r="M26" s="39" t="s">
-        <v>180</v>
+        <v>169</v>
+      </c>
+      <c r="L26" s="33" t="s">
+        <v>170</v>
+      </c>
+      <c r="M26" s="38" t="s">
+        <v>169</v>
       </c>
       <c r="N26" s="54"/>
       <c r="O26" s="25"/>
@@ -2341,64 +2341,64 @@
       <c r="S26" s="27"/>
       <c r="T26" s="27"/>
       <c r="U26" s="27"/>
-      <c r="V26" s="52"/>
+      <c r="V26" s="51"/>
     </row>
     <row r="27">
       <c r="A27" s="23"/>
       <c r="B27" s="23"/>
-      <c r="C27" s="35"/>
-      <c r="D27" s="49" t="s">
-        <v>182</v>
-      </c>
-      <c r="E27" s="34"/>
-      <c r="F27" s="34"/>
+      <c r="C27" s="34"/>
+      <c r="D27" s="48" t="s">
+        <v>172</v>
+      </c>
+      <c r="E27" s="33"/>
+      <c r="F27" s="33"/>
       <c r="G27" s="43"/>
-      <c r="H27" s="34"/>
+      <c r="H27" s="33"/>
       <c r="I27" s="43"/>
       <c r="J27" s="43"/>
       <c r="K27" s="45"/>
-      <c r="L27" s="34"/>
-      <c r="M27" s="39"/>
+      <c r="L27" s="33"/>
+      <c r="M27" s="38"/>
       <c r="N27" s="54"/>
       <c r="O27" s="25"/>
       <c r="R27" s="27"/>
       <c r="S27" s="27"/>
       <c r="T27" s="27"/>
       <c r="U27" s="27"/>
-      <c r="V27" s="52"/>
+      <c r="V27" s="51"/>
     </row>
     <row r="28" ht="30.75" customHeight="1">
       <c r="A28" s="23"/>
       <c r="B28" s="23"/>
       <c r="C28" s="28" t="s">
+        <v>41</v>
+      </c>
+      <c r="D28" s="28" t="s">
+        <v>42</v>
+      </c>
+      <c r="E28" s="29" t="s">
+        <v>43</v>
+      </c>
+      <c r="F28" s="28" t="s">
         <v>45</v>
-      </c>
-      <c r="D28" s="28" t="s">
-        <v>49</v>
-      </c>
-      <c r="E28" s="29" t="s">
-        <v>50</v>
-      </c>
-      <c r="F28" s="28" t="s">
-        <v>52</v>
       </c>
       <c r="G28" s="28"/>
       <c r="H28" s="28" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="I28" s="28"/>
       <c r="J28" s="28"/>
       <c r="K28" s="56" t="s">
-        <v>57</v>
-      </c>
-      <c r="L28" s="31" t="s">
-        <v>58</v>
+        <v>52</v>
+      </c>
+      <c r="L28" s="30" t="s">
+        <v>53</v>
       </c>
       <c r="M28" s="57" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="N28" s="28" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="O28" s="25"/>
       <c r="P28" s="27"/>
@@ -2406,7 +2406,7 @@
       <c r="S28" s="27"/>
       <c r="T28" s="27"/>
       <c r="U28" s="27"/>
-      <c r="V28" s="52"/>
+      <c r="V28" s="51"/>
       <c r="W28" s="27"/>
       <c r="X28" s="27"/>
       <c r="Y28" s="27"/>
@@ -2418,21 +2418,21 @@
     <row r="29" ht="12.75" customHeight="1">
       <c r="A29" s="23"/>
       <c r="B29" s="23"/>
-      <c r="C29" s="32">
+      <c r="C29" s="31">
         <v>2.0</v>
       </c>
       <c r="D29" s="58" t="s">
-        <v>183</v>
-      </c>
-      <c r="E29" s="35"/>
-      <c r="F29" s="35">
+        <v>179</v>
+      </c>
+      <c r="E29" s="34"/>
+      <c r="F29" s="34">
         <v>402.0</v>
       </c>
       <c r="G29" s="36">
         <v>45791.0</v>
       </c>
-      <c r="H29" s="35" t="s">
-        <v>61</v>
+      <c r="H29" s="34" t="s">
+        <v>64</v>
       </c>
       <c r="I29" s="36"/>
       <c r="J29" s="36">
@@ -2441,13 +2441,13 @@
       <c r="K29" s="37">
         <v>188246.17</v>
       </c>
-      <c r="L29" s="34" t="s">
-        <v>184</v>
+      <c r="L29" s="33" t="s">
+        <v>183</v>
       </c>
       <c r="M29" s="59">
         <v>188246.17</v>
       </c>
-      <c r="N29" s="51"/>
+      <c r="N29" s="50"/>
       <c r="O29" s="25"/>
       <c r="P29" s="27"/>
       <c r="Q29" s="27"/>
@@ -2455,7 +2455,7 @@
       <c r="S29" s="27"/>
       <c r="T29" s="27"/>
       <c r="U29" s="27"/>
-      <c r="V29" s="52"/>
+      <c r="V29" s="51"/>
       <c r="W29" s="27"/>
       <c r="X29" s="27"/>
       <c r="Y29" s="27"/>
@@ -2467,20 +2467,20 @@
     <row r="30">
       <c r="A30" s="23"/>
       <c r="B30" s="23"/>
-      <c r="C30" s="41"/>
+      <c r="C30" s="40"/>
       <c r="D30" s="58" t="s">
         <v>185</v>
       </c>
       <c r="E30" s="60">
         <v>46.0</v>
       </c>
-      <c r="F30" s="35">
+      <c r="F30" s="34">
         <v>447.0</v>
       </c>
       <c r="G30" s="36">
         <v>45814.0</v>
       </c>
-      <c r="H30" s="34" t="s">
+      <c r="H30" s="33" t="s">
         <v>186</v>
       </c>
       <c r="I30" s="43"/>
@@ -2490,13 +2490,13 @@
       <c r="K30" s="37">
         <v>112720.77</v>
       </c>
-      <c r="L30" s="34" t="s">
+      <c r="L30" s="33" t="s">
         <v>187</v>
       </c>
-      <c r="M30" s="39">
+      <c r="M30" s="38">
         <v>112720.77</v>
       </c>
-      <c r="N30" s="51"/>
+      <c r="N30" s="50"/>
       <c r="O30" s="25"/>
       <c r="P30" s="27"/>
       <c r="Q30" s="27"/>
@@ -2504,7 +2504,7 @@
       <c r="S30" s="27"/>
       <c r="T30" s="27"/>
       <c r="U30" s="27"/>
-      <c r="V30" s="52"/>
+      <c r="V30" s="51"/>
       <c r="W30" s="27"/>
       <c r="X30" s="27"/>
       <c r="Y30" s="27"/>
@@ -2516,21 +2516,21 @@
     <row r="31" ht="12.75" customHeight="1">
       <c r="A31" s="23"/>
       <c r="B31" s="23"/>
-      <c r="C31" s="41"/>
+      <c r="C31" s="40"/>
       <c r="D31" s="61" t="s">
         <v>188</v>
       </c>
       <c r="E31" s="62" t="s">
         <v>189</v>
       </c>
-      <c r="F31" s="35">
+      <c r="F31" s="34">
         <v>529.0</v>
       </c>
       <c r="G31" s="63">
         <v>45853.0</v>
       </c>
-      <c r="H31" s="34" t="s">
-        <v>65</v>
+      <c r="H31" s="33" t="s">
+        <v>69</v>
       </c>
       <c r="I31" s="43"/>
       <c r="J31" s="43">
@@ -2539,13 +2539,13 @@
       <c r="K31" s="45">
         <v>378307.61</v>
       </c>
-      <c r="L31" s="34" t="s">
+      <c r="L31" s="33" t="s">
         <v>190</v>
       </c>
-      <c r="M31" s="39">
+      <c r="M31" s="38">
         <v>378307.61</v>
       </c>
-      <c r="N31" s="51"/>
+      <c r="N31" s="50"/>
       <c r="O31" s="25"/>
       <c r="P31" s="64"/>
       <c r="Q31" s="27"/>
@@ -2553,7 +2553,7 @@
       <c r="S31" s="27"/>
       <c r="T31" s="27"/>
       <c r="U31" s="27"/>
-      <c r="V31" s="52"/>
+      <c r="V31" s="51"/>
       <c r="W31" s="27"/>
       <c r="X31" s="27"/>
       <c r="Y31" s="27"/>
@@ -2565,21 +2565,21 @@
     <row r="32" ht="60.0" customHeight="1">
       <c r="A32" s="23"/>
       <c r="B32" s="23"/>
-      <c r="C32" s="41"/>
+      <c r="C32" s="40"/>
       <c r="D32" s="61" t="s">
         <v>191</v>
       </c>
       <c r="E32" s="62" t="s">
         <v>189</v>
       </c>
-      <c r="F32" s="34">
+      <c r="F32" s="33">
         <v>691.0</v>
       </c>
       <c r="G32" s="63">
         <v>45910.0</v>
       </c>
-      <c r="H32" s="34" t="s">
-        <v>65</v>
+      <c r="H32" s="33" t="s">
+        <v>69</v>
       </c>
       <c r="I32" s="43"/>
       <c r="J32" s="43">
@@ -2588,13 +2588,13 @@
       <c r="K32" s="37">
         <v>3315.0471000000252</v>
       </c>
-      <c r="L32" s="34" t="s">
+      <c r="L32" s="33" t="s">
         <v>192</v>
       </c>
-      <c r="M32" s="39">
+      <c r="M32" s="38">
         <v>3315.04710000003</v>
       </c>
-      <c r="N32" s="51"/>
+      <c r="N32" s="50"/>
       <c r="O32" s="25"/>
       <c r="P32" s="64"/>
       <c r="Q32" s="27"/>
@@ -2602,7 +2602,7 @@
       <c r="S32" s="27"/>
       <c r="T32" s="27"/>
       <c r="U32" s="27"/>
-      <c r="V32" s="52"/>
+      <c r="V32" s="51"/>
       <c r="W32" s="27"/>
       <c r="X32" s="27"/>
       <c r="Y32" s="27"/>
@@ -2614,21 +2614,21 @@
     <row r="33" ht="12.75" customHeight="1">
       <c r="A33" s="23"/>
       <c r="B33" s="23"/>
-      <c r="C33" s="41"/>
+      <c r="C33" s="40"/>
       <c r="D33" s="61" t="s">
         <v>193</v>
       </c>
       <c r="E33" s="65">
         <v>135.0</v>
       </c>
-      <c r="F33" s="34">
+      <c r="F33" s="33">
         <v>677.0</v>
       </c>
       <c r="G33" s="63">
         <v>45904.0</v>
       </c>
-      <c r="H33" s="34" t="s">
-        <v>73</v>
+      <c r="H33" s="33" t="s">
+        <v>76</v>
       </c>
       <c r="I33" s="66"/>
       <c r="J33" s="66">
@@ -2637,13 +2637,13 @@
       <c r="K33" s="45">
         <v>198332.75</v>
       </c>
-      <c r="L33" s="34" t="s">
+      <c r="L33" s="33" t="s">
         <v>194</v>
       </c>
-      <c r="M33" s="39">
+      <c r="M33" s="38">
         <v>198332.75</v>
       </c>
-      <c r="N33" s="51"/>
+      <c r="N33" s="50"/>
       <c r="O33" s="25"/>
       <c r="P33" s="64"/>
       <c r="Q33" s="27"/>
@@ -2651,7 +2651,7 @@
       <c r="S33" s="27"/>
       <c r="T33" s="27"/>
       <c r="U33" s="27"/>
-      <c r="V33" s="52"/>
+      <c r="V33" s="51"/>
       <c r="W33" s="27"/>
       <c r="X33" s="27"/>
       <c r="Y33" s="27"/>
@@ -2663,21 +2663,21 @@
     <row r="34" ht="12.75" customHeight="1">
       <c r="A34" s="23"/>
       <c r="B34" s="23"/>
-      <c r="C34" s="41"/>
+      <c r="C34" s="40"/>
       <c r="D34" s="61" t="s">
         <v>195</v>
       </c>
       <c r="E34" s="65">
         <v>40.0</v>
       </c>
-      <c r="F34" s="34">
+      <c r="F34" s="33">
         <v>278.0</v>
       </c>
       <c r="G34" s="63">
         <v>46008.0</v>
       </c>
-      <c r="H34" s="34" t="s">
-        <v>118</v>
+      <c r="H34" s="33" t="s">
+        <v>140</v>
       </c>
       <c r="I34" s="66"/>
       <c r="J34" s="66">
@@ -2692,7 +2692,7 @@
       <c r="M34" s="68" t="s">
         <v>197</v>
       </c>
-      <c r="N34" s="51"/>
+      <c r="N34" s="50"/>
       <c r="O34" s="25"/>
       <c r="P34" s="64"/>
       <c r="Q34" s="27"/>
@@ -2700,7 +2700,7 @@
       <c r="S34" s="27"/>
       <c r="T34" s="27"/>
       <c r="U34" s="27"/>
-      <c r="V34" s="52"/>
+      <c r="V34" s="51"/>
       <c r="W34" s="27"/>
       <c r="X34" s="27"/>
       <c r="Y34" s="27"/>
@@ -2712,21 +2712,21 @@
     <row r="35" ht="12.75" customHeight="1">
       <c r="A35" s="23"/>
       <c r="B35" s="23"/>
-      <c r="C35" s="41"/>
+      <c r="C35" s="40"/>
       <c r="D35" s="61" t="s">
         <v>198</v>
       </c>
       <c r="E35" s="65" t="s">
         <v>199</v>
       </c>
-      <c r="F35" s="34">
+      <c r="F35" s="33">
         <v>748.0</v>
       </c>
       <c r="G35" s="63">
         <v>45930.0</v>
       </c>
-      <c r="H35" s="34" t="s">
-        <v>94</v>
+      <c r="H35" s="33" t="s">
+        <v>105</v>
       </c>
       <c r="I35" s="66"/>
       <c r="J35" s="66">
@@ -2735,13 +2735,13 @@
       <c r="K35" s="45">
         <v>38718.58</v>
       </c>
-      <c r="L35" s="34" t="s">
+      <c r="L35" s="33" t="s">
         <v>200</v>
       </c>
       <c r="M35" s="59" t="s">
         <v>201</v>
       </c>
-      <c r="N35" s="51"/>
+      <c r="N35" s="50"/>
       <c r="O35" s="25"/>
       <c r="P35" s="64"/>
       <c r="Q35" s="27"/>
@@ -2749,7 +2749,7 @@
       <c r="S35" s="27"/>
       <c r="T35" s="27"/>
       <c r="U35" s="27"/>
-      <c r="V35" s="52"/>
+      <c r="V35" s="51"/>
       <c r="W35" s="27"/>
       <c r="X35" s="27"/>
       <c r="Y35" s="27"/>
@@ -2761,21 +2761,21 @@
     <row r="36" ht="12.75" customHeight="1">
       <c r="A36" s="23"/>
       <c r="B36" s="23"/>
-      <c r="C36" s="41"/>
+      <c r="C36" s="40"/>
       <c r="D36" s="61" t="s">
         <v>202</v>
       </c>
       <c r="E36" s="65">
         <v>154.0</v>
       </c>
-      <c r="F36" s="34">
+      <c r="F36" s="33">
         <v>822.0</v>
       </c>
       <c r="G36" s="63">
         <v>45968.0</v>
       </c>
-      <c r="H36" s="34" t="s">
-        <v>109</v>
+      <c r="H36" s="33" t="s">
+        <v>129</v>
       </c>
       <c r="I36" s="66"/>
       <c r="J36" s="66">
@@ -2784,13 +2784,13 @@
       <c r="K36" s="45">
         <v>133124.11</v>
       </c>
-      <c r="L36" s="34" t="s">
+      <c r="L36" s="33" t="s">
         <v>203</v>
       </c>
       <c r="M36" s="59" t="s">
         <v>204</v>
       </c>
-      <c r="N36" s="51"/>
+      <c r="N36" s="50"/>
       <c r="O36" s="25"/>
       <c r="P36" s="64"/>
       <c r="Q36" s="27"/>
@@ -2798,7 +2798,7 @@
       <c r="S36" s="27"/>
       <c r="T36" s="27"/>
       <c r="U36" s="27"/>
-      <c r="V36" s="52"/>
+      <c r="V36" s="51"/>
       <c r="W36" s="27"/>
       <c r="X36" s="27"/>
       <c r="Y36" s="27"/>
@@ -2810,7 +2810,7 @@
     <row r="37" ht="12.75" customHeight="1">
       <c r="A37" s="23"/>
       <c r="B37" s="23"/>
-      <c r="C37" s="41"/>
+      <c r="C37" s="40"/>
       <c r="D37" s="61" t="s">
         <v>205</v>
       </c>
@@ -2824,7 +2824,7 @@
         <v>46043.0</v>
       </c>
       <c r="H37" s="65" t="s">
-        <v>105</v>
+        <v>123</v>
       </c>
       <c r="I37" s="70"/>
       <c r="J37" s="69">
@@ -2833,13 +2833,13 @@
       <c r="K37" s="45">
         <v>11372.9</v>
       </c>
-      <c r="L37" s="34" t="s">
+      <c r="L37" s="33" t="s">
         <v>206</v>
       </c>
-      <c r="M37" s="39">
+      <c r="M37" s="38">
         <v>11372.9</v>
       </c>
-      <c r="N37" s="51"/>
+      <c r="N37" s="50"/>
       <c r="O37" s="25"/>
       <c r="P37" s="27"/>
       <c r="Q37" s="27"/>
@@ -2847,7 +2847,7 @@
       <c r="S37" s="27"/>
       <c r="T37" s="27"/>
       <c r="U37" s="27"/>
-      <c r="V37" s="52"/>
+      <c r="V37" s="51"/>
       <c r="W37" s="27"/>
       <c r="X37" s="27"/>
       <c r="Y37" s="27"/>
@@ -2859,7 +2859,7 @@
     <row r="38" ht="12.75" customHeight="1">
       <c r="A38" s="23"/>
       <c r="B38" s="23"/>
-      <c r="C38" s="41"/>
+      <c r="C38" s="40"/>
       <c r="D38" s="61" t="s">
         <v>207</v>
       </c>
@@ -2872,9 +2872,9 @@
       </c>
       <c r="J38" s="69"/>
       <c r="K38" s="45"/>
-      <c r="L38" s="34"/>
-      <c r="M38" s="39"/>
-      <c r="N38" s="51">
+      <c r="L38" s="33"/>
+      <c r="M38" s="38"/>
+      <c r="N38" s="50">
         <v>15854.78</v>
       </c>
       <c r="O38" s="25"/>
@@ -2884,7 +2884,7 @@
       <c r="S38" s="27"/>
       <c r="T38" s="27"/>
       <c r="U38" s="27"/>
-      <c r="V38" s="52"/>
+      <c r="V38" s="51"/>
       <c r="W38" s="27"/>
       <c r="X38" s="27"/>
       <c r="Y38" s="27"/>
@@ -2909,8 +2909,8 @@
       </c>
       <c r="J39" s="69"/>
       <c r="K39" s="45"/>
-      <c r="L39" s="34"/>
-      <c r="M39" s="39"/>
+      <c r="L39" s="33"/>
+      <c r="M39" s="38"/>
       <c r="N39" s="71">
         <v>42229.72325</v>
       </c>
@@ -2921,7 +2921,7 @@
       <c r="S39" s="27"/>
       <c r="T39" s="27"/>
       <c r="U39" s="27"/>
-      <c r="V39" s="52"/>
+      <c r="V39" s="51"/>
       <c r="W39" s="27"/>
       <c r="X39" s="27"/>
       <c r="Y39" s="27"/>
@@ -2933,7 +2933,7 @@
     <row r="40" ht="12.75" customHeight="1">
       <c r="A40" s="23"/>
       <c r="B40" s="23"/>
-      <c r="C40" s="35"/>
+      <c r="C40" s="34"/>
       <c r="D40" s="61" t="s">
         <v>210</v>
       </c>
@@ -2946,8 +2946,8 @@
       </c>
       <c r="J40" s="69"/>
       <c r="K40" s="45"/>
-      <c r="L40" s="47"/>
-      <c r="M40" s="39"/>
+      <c r="L40" s="46"/>
+      <c r="M40" s="38"/>
       <c r="N40" s="72">
         <v>48857.395500000006</v>
       </c>
@@ -2958,7 +2958,7 @@
       <c r="S40" s="27"/>
       <c r="T40" s="27"/>
       <c r="U40" s="27"/>
-      <c r="V40" s="52"/>
+      <c r="V40" s="51"/>
       <c r="W40" s="27"/>
       <c r="X40" s="27"/>
       <c r="Y40" s="27"/>
@@ -2970,7 +2970,7 @@
     <row r="41" ht="12.75" customHeight="1">
       <c r="A41" s="23"/>
       <c r="B41" s="23"/>
-      <c r="C41" s="35"/>
+      <c r="C41" s="34"/>
       <c r="D41" s="61" t="s">
         <v>211</v>
       </c>
@@ -2983,8 +2983,8 @@
       </c>
       <c r="J41" s="69"/>
       <c r="K41" s="45"/>
-      <c r="L41" s="47"/>
-      <c r="M41" s="39"/>
+      <c r="L41" s="46"/>
+      <c r="M41" s="38"/>
       <c r="N41" s="72"/>
       <c r="O41" s="25"/>
       <c r="P41" s="27"/>
@@ -2993,7 +2993,7 @@
       <c r="S41" s="27"/>
       <c r="T41" s="27"/>
       <c r="U41" s="27"/>
-      <c r="V41" s="52"/>
+      <c r="V41" s="51"/>
       <c r="W41" s="27"/>
       <c r="X41" s="27"/>
       <c r="Y41" s="27"/>
@@ -3005,7 +3005,7 @@
     <row r="42" ht="12.75" customHeight="1">
       <c r="A42" s="23"/>
       <c r="B42" s="23"/>
-      <c r="C42" s="32">
+      <c r="C42" s="31">
         <v>3.0</v>
       </c>
       <c r="D42" s="61" t="s">
@@ -3019,7 +3019,7 @@
         <v>46104.0</v>
       </c>
       <c r="H42" s="65" t="s">
-        <v>105</v>
+        <v>123</v>
       </c>
       <c r="I42" s="70"/>
       <c r="J42" s="69">
@@ -3034,7 +3034,7 @@
       <c r="M42" s="74">
         <v>27801.11</v>
       </c>
-      <c r="N42" s="51"/>
+      <c r="N42" s="50"/>
       <c r="O42" s="25"/>
       <c r="P42" s="27"/>
       <c r="Q42" s="27"/>
@@ -3042,7 +3042,7 @@
       <c r="S42" s="27"/>
       <c r="T42" s="27"/>
       <c r="U42" s="27"/>
-      <c r="V42" s="52"/>
+      <c r="V42" s="51"/>
       <c r="W42" s="27"/>
       <c r="X42" s="27"/>
       <c r="Y42" s="27"/>
@@ -3054,7 +3054,7 @@
     <row r="43" ht="12.75" customHeight="1">
       <c r="A43" s="14"/>
       <c r="B43" s="14"/>
-      <c r="C43" s="41"/>
+      <c r="C43" s="40"/>
       <c r="D43" s="61" t="s">
         <v>215</v>
       </c>
@@ -3066,7 +3066,7 @@
         <v>46199.0</v>
       </c>
       <c r="H43" s="65" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="I43" s="70"/>
       <c r="J43" s="69">
@@ -3075,19 +3075,19 @@
       <c r="K43" s="45">
         <v>58868.35</v>
       </c>
-      <c r="L43" s="34" t="s">
-        <v>59</v>
+      <c r="L43" s="33" t="s">
+        <v>55</v>
       </c>
       <c r="M43" s="74">
         <v>58868.35</v>
       </c>
-      <c r="N43" s="51"/>
+      <c r="N43" s="50"/>
       <c r="V43" s="2"/>
     </row>
     <row r="44" ht="12.75" customHeight="1">
       <c r="A44" s="14"/>
       <c r="B44" s="14"/>
-      <c r="C44" s="41"/>
+      <c r="C44" s="40"/>
       <c r="K44" s="75"/>
       <c r="M44" s="75"/>
       <c r="V44" s="2"/>
@@ -3095,7 +3095,7 @@
     <row r="45" ht="12.75" customHeight="1">
       <c r="A45" s="14"/>
       <c r="B45" s="14"/>
-      <c r="C45" s="41"/>
+      <c r="C45" s="40"/>
       <c r="K45" s="75"/>
       <c r="M45" s="75"/>
       <c r="V45" s="2"/>
@@ -3103,25 +3103,25 @@
     <row r="46" ht="12.75" customHeight="1">
       <c r="A46" s="14"/>
       <c r="B46" s="14"/>
-      <c r="C46" s="41"/>
+      <c r="C46" s="40"/>
       <c r="V46" s="2"/>
     </row>
     <row r="47" ht="12.75" customHeight="1">
       <c r="A47" s="14"/>
       <c r="B47" s="14"/>
-      <c r="C47" s="41"/>
+      <c r="C47" s="40"/>
       <c r="V47" s="2"/>
     </row>
     <row r="48" ht="12.75" customHeight="1">
       <c r="A48" s="14"/>
       <c r="B48" s="14"/>
-      <c r="C48" s="41"/>
+      <c r="C48" s="40"/>
       <c r="V48" s="2"/>
     </row>
     <row r="49" ht="12.75" customHeight="1">
       <c r="A49" s="14"/>
       <c r="B49" s="14"/>
-      <c r="C49" s="41"/>
+      <c r="C49" s="40"/>
       <c r="V49" s="2"/>
     </row>
     <row r="50" ht="12.75" customHeight="1">
@@ -8035,10 +8035,10 @@
       <c r="AH1" s="4"/>
     </row>
     <row r="2">
-      <c r="A2" s="8">
+      <c r="A2" s="6">
         <v>46212.0</v>
       </c>
-      <c r="L2" s="10" t="s">
+      <c r="L2" s="8" t="s">
         <v>1</v>
       </c>
       <c r="AB2" s="4"/>
@@ -8050,31 +8050,31 @@
       <c r="AH2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="11" t="s">
+      <c r="A3" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="11" t="s">
+      <c r="B3" s="10" t="s">
         <v>3</v>
       </c>
       <c r="C3" s="12">
         <v>2.5E32</v>
       </c>
-      <c r="D3" s="11" t="s">
+      <c r="D3" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E3" s="13">
         <v>45686.0</v>
       </c>
-      <c r="F3" s="11" t="s">
+      <c r="F3" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G3" s="11">
+      <c r="G3" s="10">
         <v>12.0</v>
       </c>
-      <c r="H3" s="11">
+      <c r="H3" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I3" s="11">
+      <c r="I3" s="10">
         <v>2048.0</v>
       </c>
       <c r="J3" s="16">
@@ -8083,7 +8083,7 @@
       <c r="K3" s="16">
         <v>1000.0</v>
       </c>
-      <c r="L3" s="11">
+      <c r="L3" s="10">
         <v>0.0</v>
       </c>
       <c r="AB3" s="4"/>
@@ -8095,31 +8095,31 @@
       <c r="AH3" s="4"/>
     </row>
     <row r="4">
-      <c r="A4" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="B4" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="C4" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="D4" s="11" t="s">
+      <c r="A4" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="D4" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E4" s="13">
         <v>45762.0</v>
       </c>
-      <c r="F4" s="11" t="s">
+      <c r="F4" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G4" s="11">
+      <c r="G4" s="10">
         <v>12.0</v>
       </c>
-      <c r="H4" s="11">
+      <c r="H4" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I4" s="11">
+      <c r="I4" s="10">
         <v>2048.0</v>
       </c>
       <c r="J4" s="16">
@@ -8128,7 +8128,7 @@
       <c r="K4" s="16">
         <v>52250.04</v>
       </c>
-      <c r="L4" s="11">
+      <c r="L4" s="10">
         <v>0.0</v>
       </c>
       <c r="AB4" s="4"/>
@@ -8140,31 +8140,31 @@
       <c r="AH4" s="4"/>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="B5" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="C5" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="D5" s="11" t="s">
+      <c r="A5" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="D5" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E5" s="13">
         <v>45762.0</v>
       </c>
-      <c r="F5" s="11" t="s">
+      <c r="F5" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G5" s="11">
+      <c r="G5" s="10">
         <v>12.0</v>
       </c>
-      <c r="H5" s="11">
+      <c r="H5" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I5" s="11">
+      <c r="I5" s="10">
         <v>2048.0</v>
       </c>
       <c r="J5" s="16">
@@ -8173,7 +8173,7 @@
       <c r="K5" s="16">
         <v>881914.18</v>
       </c>
-      <c r="L5" s="11">
+      <c r="L5" s="10">
         <v>0.0</v>
       </c>
       <c r="AB5" s="4"/>
@@ -8185,31 +8185,31 @@
       <c r="AH5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="s">
+      <c r="A6" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="B6" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="B6" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="C6" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="D6" s="11" t="s">
+      <c r="C6" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="D6" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E6" s="13">
         <v>45762.0</v>
       </c>
-      <c r="F6" s="11" t="s">
+      <c r="F6" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G6" s="11">
+      <c r="G6" s="10">
         <v>12.0</v>
       </c>
-      <c r="H6" s="11">
+      <c r="H6" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I6" s="11">
+      <c r="I6" s="10">
         <v>2048.0</v>
       </c>
       <c r="J6" s="16">
@@ -8218,7 +8218,7 @@
       <c r="K6" s="16">
         <v>750000.0</v>
       </c>
-      <c r="L6" s="11">
+      <c r="L6" s="10">
         <v>0.0</v>
       </c>
       <c r="AB6" s="4"/>
@@ -8230,32 +8230,32 @@
       <c r="AH6" s="4"/>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="B7" s="11" t="s">
-        <v>42</v>
-      </c>
-      <c r="C7" s="11" t="s">
-        <v>43</v>
-      </c>
-      <c r="D7" s="11" t="s">
+      <c r="A7" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="D7" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E7" s="13">
         <v>45763.0</v>
       </c>
-      <c r="F7" s="11" t="s">
+      <c r="F7" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G7" s="11">
+      <c r="G7" s="10">
         <v>12.0</v>
       </c>
-      <c r="H7" s="11">
+      <c r="H7" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I7" s="11" t="s">
-        <v>44</v>
+      <c r="I7" s="10" t="s">
+        <v>54</v>
       </c>
       <c r="J7" s="16">
         <v>949835.78</v>
@@ -8263,7 +8263,7 @@
       <c r="K7" s="16">
         <v>949835.78</v>
       </c>
-      <c r="L7" s="11">
+      <c r="L7" s="10">
         <v>0.0</v>
       </c>
       <c r="AB7" s="4"/>
@@ -8275,32 +8275,32 @@
       <c r="AH7" s="4"/>
     </row>
     <row r="8">
-      <c r="A8" s="11" t="s">
-        <v>46</v>
-      </c>
-      <c r="B8" s="11" t="s">
-        <v>47</v>
-      </c>
-      <c r="C8" s="11" t="s">
-        <v>48</v>
-      </c>
-      <c r="D8" s="11" t="s">
+      <c r="A8" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="B8" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="C8" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="D8" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E8" s="13">
         <v>45763.0</v>
       </c>
-      <c r="F8" s="11" t="s">
+      <c r="F8" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G8" s="11">
+      <c r="G8" s="10">
         <v>12.0</v>
       </c>
-      <c r="H8" s="11">
+      <c r="H8" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I8" s="11" t="s">
-        <v>51</v>
+      <c r="I8" s="10" t="s">
+        <v>61</v>
       </c>
       <c r="J8" s="16">
         <v>524584.95</v>
@@ -8308,10 +8308,10 @@
       <c r="K8" s="16">
         <v>524584.95</v>
       </c>
-      <c r="L8" s="11">
+      <c r="L8" s="10">
         <v>0.0</v>
       </c>
-      <c r="O8" s="30"/>
+      <c r="O8" s="35"/>
       <c r="AB8" s="4"/>
       <c r="AC8" s="4"/>
       <c r="AD8" s="4"/>
@@ -8321,32 +8321,32 @@
       <c r="AH8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="11" t="s">
-        <v>61</v>
-      </c>
-      <c r="B9" s="11" t="s">
-        <v>62</v>
-      </c>
-      <c r="C9" s="11" t="s">
-        <v>63</v>
-      </c>
-      <c r="D9" s="11" t="s">
+      <c r="A9" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="C9" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="D9" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E9" s="13">
         <v>45792.0</v>
       </c>
-      <c r="F9" s="11" t="s">
+      <c r="F9" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G9" s="11">
+      <c r="G9" s="10">
         <v>12.0</v>
       </c>
-      <c r="H9" s="11">
+      <c r="H9" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I9" s="11" t="s">
-        <v>64</v>
+      <c r="I9" s="10" t="s">
+        <v>68</v>
       </c>
       <c r="J9" s="16">
         <v>211614.23</v>
@@ -8354,7 +8354,7 @@
       <c r="K9" s="16">
         <v>211614.23</v>
       </c>
-      <c r="L9" s="11">
+      <c r="L9" s="10">
         <v>0.0</v>
       </c>
       <c r="AB9" s="4"/>
@@ -8366,31 +8366,31 @@
       <c r="AH9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="11" t="s">
-        <v>65</v>
-      </c>
-      <c r="B10" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="C10" s="11" t="s">
-        <v>68</v>
-      </c>
-      <c r="D10" s="11" t="s">
+      <c r="A10" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="C10" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="D10" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E10" s="13">
         <v>45825.0</v>
       </c>
-      <c r="F10" s="11" t="s">
+      <c r="F10" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G10" s="11">
+      <c r="G10" s="10">
         <v>12.0</v>
       </c>
-      <c r="H10" s="11">
+      <c r="H10" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I10" s="11">
+      <c r="I10" s="10">
         <v>2048.0</v>
       </c>
       <c r="J10" s="16">
@@ -8411,31 +8411,31 @@
       <c r="AH10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="s">
-        <v>70</v>
-      </c>
-      <c r="B11" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="C11" s="11" t="s">
+      <c r="A11" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="D11" s="11" t="s">
+      <c r="B11" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="C11" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="D11" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E11" s="13">
         <v>45825.0</v>
       </c>
-      <c r="F11" s="11" t="s">
+      <c r="F11" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G11" s="11">
+      <c r="G11" s="10">
         <v>12.0</v>
       </c>
-      <c r="H11" s="11">
+      <c r="H11" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I11" s="11">
+      <c r="I11" s="10">
         <v>2048.0</v>
       </c>
       <c r="J11" s="16">
@@ -8444,7 +8444,7 @@
       <c r="K11" s="16">
         <v>618154.38</v>
       </c>
-      <c r="L11" s="11">
+      <c r="L11" s="10">
         <v>0.01</v>
       </c>
       <c r="AB11" s="4"/>
@@ -8456,32 +8456,32 @@
       <c r="AH11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="11" t="s">
-        <v>73</v>
-      </c>
-      <c r="B12" s="11" t="s">
-        <v>74</v>
-      </c>
-      <c r="C12" s="11" t="s">
-        <v>75</v>
-      </c>
-      <c r="D12" s="11" t="s">
+      <c r="A12" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="B12" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="C12" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="D12" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E12" s="13">
         <v>45832.0</v>
       </c>
-      <c r="F12" s="11" t="s">
+      <c r="F12" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G12" s="11">
+      <c r="G12" s="10">
         <v>12.0</v>
       </c>
-      <c r="H12" s="11">
+      <c r="H12" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I12" s="11" t="s">
-        <v>76</v>
+      <c r="I12" s="10" t="s">
+        <v>79</v>
       </c>
       <c r="J12" s="16">
         <v>1600334.09</v>
@@ -8489,7 +8489,7 @@
       <c r="K12" s="16">
         <v>1600334.09</v>
       </c>
-      <c r="L12" s="11">
+      <c r="L12" s="10">
         <v>0.0</v>
       </c>
       <c r="AB12" s="4"/>
@@ -8501,31 +8501,31 @@
       <c r="AH12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="11" t="s">
-        <v>77</v>
-      </c>
-      <c r="B13" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="C13" s="11" t="s">
-        <v>78</v>
-      </c>
-      <c r="D13" s="11" t="s">
+      <c r="A13" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="B13" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="C13" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="D13" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E13" s="13">
         <v>45863.0</v>
       </c>
-      <c r="F13" s="11" t="s">
+      <c r="F13" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G13" s="11">
+      <c r="G13" s="10">
         <v>12.0</v>
       </c>
-      <c r="H13" s="11">
+      <c r="H13" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I13" s="11">
+      <c r="I13" s="10">
         <v>2048.0</v>
       </c>
       <c r="J13" s="16">
@@ -8537,7 +8537,7 @@
       <c r="L13" s="16">
         <v>0.0</v>
       </c>
-      <c r="M13" s="38"/>
+      <c r="M13" s="42"/>
       <c r="AB13" s="4"/>
       <c r="AC13" s="4"/>
       <c r="AD13" s="4"/>
@@ -8547,32 +8547,32 @@
       <c r="AH13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="B14" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="C14" s="11" t="s">
-        <v>81</v>
-      </c>
-      <c r="D14" s="11" t="s">
+      <c r="A14" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="B14" s="10" t="s">
+        <v>87</v>
+      </c>
+      <c r="C14" s="10" t="s">
+        <v>88</v>
+      </c>
+      <c r="D14" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E14" s="13">
         <v>45887.0</v>
       </c>
-      <c r="F14" s="11" t="s">
+      <c r="F14" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G14" s="11">
+      <c r="G14" s="10">
         <v>12.0</v>
       </c>
-      <c r="H14" s="11">
+      <c r="H14" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I14" s="11" t="s">
-        <v>64</v>
+      <c r="I14" s="10" t="s">
+        <v>68</v>
       </c>
       <c r="J14" s="16">
         <v>968237.39</v>
@@ -8580,7 +8580,7 @@
       <c r="K14" s="16">
         <v>968237.39</v>
       </c>
-      <c r="L14" s="11">
+      <c r="L14" s="10">
         <v>0.0</v>
       </c>
       <c r="AB14" s="4"/>
@@ -8592,32 +8592,32 @@
       <c r="AH14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="11" t="s">
-        <v>82</v>
-      </c>
-      <c r="B15" s="11" t="s">
-        <v>83</v>
-      </c>
-      <c r="C15" s="11" t="s">
-        <v>84</v>
-      </c>
-      <c r="D15" s="11" t="s">
+      <c r="A15" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="B15" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="D15" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E15" s="13">
         <v>45924.0</v>
       </c>
-      <c r="F15" s="11" t="s">
+      <c r="F15" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G15" s="11">
+      <c r="G15" s="10">
         <v>12.0</v>
       </c>
-      <c r="H15" s="11">
+      <c r="H15" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I15" s="11" t="s">
-        <v>44</v>
+      <c r="I15" s="10" t="s">
+        <v>54</v>
       </c>
       <c r="J15" s="16">
         <v>1011677.95</v>
@@ -8625,7 +8625,7 @@
       <c r="K15" s="16">
         <v>1011677.95</v>
       </c>
-      <c r="L15" s="11">
+      <c r="L15" s="10">
         <v>0.0</v>
       </c>
       <c r="AB15" s="4"/>
@@ -8637,31 +8637,31 @@
       <c r="AH15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="11" t="s">
-        <v>86</v>
-      </c>
-      <c r="B16" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="C16" s="11" t="s">
-        <v>87</v>
-      </c>
-      <c r="D16" s="11" t="s">
+      <c r="A16" s="10" t="s">
+        <v>94</v>
+      </c>
+      <c r="B16" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="C16" s="10" t="s">
+        <v>96</v>
+      </c>
+      <c r="D16" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E16" s="13">
         <v>45929.0</v>
       </c>
-      <c r="F16" s="11" t="s">
+      <c r="F16" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G16" s="11">
+      <c r="G16" s="10">
         <v>12.0</v>
       </c>
-      <c r="H16" s="11">
+      <c r="H16" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I16" s="11">
+      <c r="I16" s="10">
         <v>2048.0</v>
       </c>
       <c r="J16" s="16">
@@ -8682,37 +8682,37 @@
       <c r="AH16" s="4"/>
     </row>
     <row r="17">
-      <c r="A17" s="11" t="s">
-        <v>90</v>
-      </c>
-      <c r="B17" s="11" t="s">
-        <v>91</v>
-      </c>
-      <c r="C17" s="11" t="s">
-        <v>92</v>
-      </c>
-      <c r="D17" s="11" t="s">
+      <c r="A17" s="10" t="s">
+        <v>99</v>
+      </c>
+      <c r="B17" s="10" t="s">
+        <v>100</v>
+      </c>
+      <c r="C17" s="10" t="s">
+        <v>101</v>
+      </c>
+      <c r="D17" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E17" s="13">
         <v>45930.0</v>
       </c>
-      <c r="F17" s="11" t="s">
+      <c r="F17" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G17" s="11">
+      <c r="G17" s="10">
         <v>12.0</v>
       </c>
-      <c r="H17" s="11">
+      <c r="H17" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I17" s="11">
+      <c r="I17" s="10">
         <v>2048.0</v>
       </c>
       <c r="J17" s="16">
         <v>34065.36</v>
       </c>
-      <c r="K17" s="11">
+      <c r="K17" s="10">
         <v>0.0</v>
       </c>
       <c r="L17" s="16">
@@ -8727,32 +8727,32 @@
       <c r="AH17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="11" t="s">
-        <v>94</v>
-      </c>
-      <c r="B18" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="C18" s="11" t="s">
-        <v>95</v>
-      </c>
-      <c r="D18" s="11" t="s">
+      <c r="A18" s="10" t="s">
+        <v>105</v>
+      </c>
+      <c r="B18" s="10" t="s">
+        <v>87</v>
+      </c>
+      <c r="C18" s="10" t="s">
+        <v>106</v>
+      </c>
+      <c r="D18" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E18" s="13">
         <v>45938.0</v>
       </c>
-      <c r="F18" s="11" t="s">
+      <c r="F18" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G18" s="11">
+      <c r="G18" s="10">
         <v>12.0</v>
       </c>
-      <c r="H18" s="11">
+      <c r="H18" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I18" s="11" t="s">
-        <v>64</v>
+      <c r="I18" s="10" t="s">
+        <v>68</v>
       </c>
       <c r="J18" s="16">
         <v>63746.85</v>
@@ -8760,7 +8760,7 @@
       <c r="K18" s="16">
         <v>63746.85</v>
       </c>
-      <c r="L18" s="11">
+      <c r="L18" s="10">
         <v>0.0</v>
       </c>
       <c r="AB18" s="4"/>
@@ -8772,32 +8772,32 @@
       <c r="AH18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="11" t="s">
-        <v>97</v>
-      </c>
-      <c r="B19" s="11" t="s">
-        <v>74</v>
-      </c>
-      <c r="C19" s="11" t="s">
-        <v>98</v>
-      </c>
-      <c r="D19" s="11" t="s">
+      <c r="A19" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="B19" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="C19" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="D19" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E19" s="13">
         <v>45938.0</v>
       </c>
-      <c r="F19" s="11" t="s">
+      <c r="F19" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G19" s="11">
+      <c r="G19" s="10">
         <v>12.0</v>
       </c>
-      <c r="H19" s="11">
+      <c r="H19" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I19" s="11" t="s">
-        <v>76</v>
+      <c r="I19" s="10" t="s">
+        <v>79</v>
       </c>
       <c r="J19" s="16">
         <v>947931.1</v>
@@ -8805,7 +8805,7 @@
       <c r="K19" s="16">
         <v>947931.1</v>
       </c>
-      <c r="L19" s="11">
+      <c r="L19" s="10">
         <v>0.0</v>
       </c>
       <c r="AB19" s="4"/>
@@ -8817,31 +8817,31 @@
       <c r="AH19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="11" t="s">
-        <v>100</v>
-      </c>
-      <c r="B20" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="C20" s="11" t="s">
-        <v>101</v>
-      </c>
-      <c r="D20" s="11" t="s">
+      <c r="A20" s="10" t="s">
+        <v>115</v>
+      </c>
+      <c r="B20" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="C20" s="10" t="s">
+        <v>116</v>
+      </c>
+      <c r="D20" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E20" s="13">
         <v>45938.0</v>
       </c>
-      <c r="F20" s="11" t="s">
+      <c r="F20" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G20" s="11">
+      <c r="G20" s="10">
         <v>12.0</v>
       </c>
-      <c r="H20" s="11">
+      <c r="H20" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I20" s="11">
+      <c r="I20" s="10">
         <v>2048.0</v>
       </c>
       <c r="J20" s="16">
@@ -8850,7 +8850,7 @@
       <c r="K20" s="16">
         <v>259790.57</v>
       </c>
-      <c r="L20" s="11">
+      <c r="L20" s="10">
         <v>0.0</v>
       </c>
       <c r="AB20" s="4"/>
@@ -8862,31 +8862,31 @@
       <c r="AH20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="11" t="s">
-        <v>103</v>
-      </c>
-      <c r="B21" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="C21" s="11" t="s">
-        <v>104</v>
-      </c>
-      <c r="D21" s="11" t="s">
+      <c r="A21" s="10" t="s">
+        <v>119</v>
+      </c>
+      <c r="B21" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="C21" s="10" t="s">
+        <v>120</v>
+      </c>
+      <c r="D21" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E21" s="13">
         <v>45938.0</v>
       </c>
-      <c r="F21" s="11" t="s">
+      <c r="F21" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G21" s="11">
+      <c r="G21" s="10">
         <v>12.0</v>
       </c>
-      <c r="H21" s="11">
+      <c r="H21" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I21" s="11">
+      <c r="I21" s="10">
         <v>2048.0</v>
       </c>
       <c r="J21" s="16">
@@ -8895,7 +8895,7 @@
       <c r="K21" s="16">
         <v>170479.3</v>
       </c>
-      <c r="L21" s="11">
+      <c r="L21" s="10">
         <v>0.0</v>
       </c>
       <c r="AB21" s="4"/>
@@ -8907,31 +8907,31 @@
       <c r="AH21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="11" t="s">
-        <v>105</v>
-      </c>
-      <c r="B22" s="11" t="s">
-        <v>106</v>
-      </c>
-      <c r="C22" s="11" t="s">
-        <v>107</v>
-      </c>
-      <c r="D22" s="11" t="s">
+      <c r="A22" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="B22" s="10" t="s">
+        <v>124</v>
+      </c>
+      <c r="C22" s="10" t="s">
+        <v>125</v>
+      </c>
+      <c r="D22" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E22" s="46">
+      <c r="E22" s="52">
         <v>45953.0</v>
       </c>
-      <c r="F22" s="11" t="s">
+      <c r="F22" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G22" s="11">
+      <c r="G22" s="10">
         <v>12.0</v>
       </c>
-      <c r="H22" s="11">
+      <c r="H22" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I22" s="11">
+      <c r="I22" s="10">
         <v>2000.0</v>
       </c>
       <c r="J22" s="16">
@@ -8952,32 +8952,32 @@
       <c r="AH22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="11" t="s">
-        <v>109</v>
-      </c>
-      <c r="B23" s="11" t="s">
-        <v>110</v>
-      </c>
-      <c r="C23" s="11" t="s">
-        <v>111</v>
-      </c>
-      <c r="D23" s="11" t="s">
+      <c r="A23" s="10" t="s">
+        <v>129</v>
+      </c>
+      <c r="B23" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C23" s="10" t="s">
+        <v>132</v>
+      </c>
+      <c r="D23" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E23" s="46">
+      <c r="E23" s="52">
         <v>45953.0</v>
       </c>
-      <c r="F23" s="11" t="s">
+      <c r="F23" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G23" s="11">
+      <c r="G23" s="10">
         <v>12.0</v>
       </c>
-      <c r="H23" s="11">
+      <c r="H23" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I23" s="11" t="s">
-        <v>112</v>
+      <c r="I23" s="10" t="s">
+        <v>134</v>
       </c>
       <c r="J23" s="16">
         <v>1000001.64</v>
@@ -8985,7 +8985,7 @@
       <c r="K23" s="16">
         <v>1000001.64</v>
       </c>
-      <c r="L23" s="11">
+      <c r="L23" s="10">
         <v>0.0</v>
       </c>
       <c r="AB23" s="4"/>
@@ -8997,31 +8997,31 @@
       <c r="AH23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="11" t="s">
-        <v>114</v>
-      </c>
-      <c r="B24" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="C24" s="11" t="s">
-        <v>115</v>
-      </c>
-      <c r="D24" s="11" t="s">
+      <c r="A24" s="10" t="s">
+        <v>135</v>
+      </c>
+      <c r="B24" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="C24" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="D24" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E24" s="46">
+      <c r="E24" s="52">
         <v>45953.0</v>
       </c>
-      <c r="F24" s="11" t="s">
+      <c r="F24" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G24" s="11">
+      <c r="G24" s="10">
         <v>12.0</v>
       </c>
-      <c r="H24" s="11">
+      <c r="H24" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I24" s="11">
+      <c r="I24" s="10">
         <v>2048.0</v>
       </c>
       <c r="J24" s="16">
@@ -9030,7 +9030,7 @@
       <c r="K24" s="16">
         <v>68405.66</v>
       </c>
-      <c r="L24" s="11">
+      <c r="L24" s="10">
         <v>0.0</v>
       </c>
       <c r="AB24" s="4"/>
@@ -9042,32 +9042,32 @@
       <c r="AH24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="11" t="s">
-        <v>118</v>
-      </c>
-      <c r="B25" s="11" t="s">
-        <v>119</v>
-      </c>
-      <c r="C25" s="11" t="s">
-        <v>120</v>
-      </c>
-      <c r="D25" s="11" t="s">
+      <c r="A25" s="10" t="s">
+        <v>140</v>
+      </c>
+      <c r="B25" s="10" t="s">
+        <v>142</v>
+      </c>
+      <c r="C25" s="10" t="s">
+        <v>143</v>
+      </c>
+      <c r="D25" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E25" s="46">
+      <c r="E25" s="52">
         <v>45975.0</v>
       </c>
-      <c r="F25" s="11" t="s">
+      <c r="F25" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G25" s="11">
+      <c r="G25" s="10">
         <v>12.0</v>
       </c>
-      <c r="H25" s="11">
+      <c r="H25" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I25" s="11" t="s">
-        <v>112</v>
+      <c r="I25" s="10" t="s">
+        <v>134</v>
       </c>
       <c r="J25" s="16">
         <v>1157673.06</v>
@@ -9075,7 +9075,7 @@
       <c r="K25" s="16">
         <v>1157673.06</v>
       </c>
-      <c r="L25" s="11">
+      <c r="L25" s="10">
         <v>0.0</v>
       </c>
       <c r="AB25" s="4"/>
@@ -9087,31 +9087,31 @@
       <c r="AH25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="11" t="s">
-        <v>122</v>
-      </c>
-      <c r="B26" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="C26" s="11" t="s">
-        <v>123</v>
-      </c>
-      <c r="D26" s="11" t="s">
+      <c r="A26" s="10" t="s">
+        <v>147</v>
+      </c>
+      <c r="B26" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="C26" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="D26" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E26" s="46">
+      <c r="E26" s="52">
         <v>45989.0</v>
       </c>
-      <c r="F26" s="11" t="s">
+      <c r="F26" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G26" s="11">
+      <c r="G26" s="10">
         <v>12.0</v>
       </c>
-      <c r="H26" s="11">
+      <c r="H26" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I26" s="11">
+      <c r="I26" s="10">
         <v>2048.0</v>
       </c>
       <c r="J26" s="16">
@@ -9120,7 +9120,7 @@
       <c r="K26" s="16">
         <v>34065.36</v>
       </c>
-      <c r="L26" s="11">
+      <c r="L26" s="10">
         <v>0.0</v>
       </c>
       <c r="AB26" s="4"/>
@@ -9132,31 +9132,31 @@
       <c r="AH26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="11" t="s">
-        <v>125</v>
-      </c>
-      <c r="B27" s="11" t="s">
-        <v>126</v>
-      </c>
-      <c r="C27" s="11" t="s">
-        <v>127</v>
-      </c>
-      <c r="D27" s="11" t="s">
+      <c r="A27" s="10" t="s">
+        <v>151</v>
+      </c>
+      <c r="B27" s="10" t="s">
+        <v>152</v>
+      </c>
+      <c r="C27" s="10" t="s">
+        <v>153</v>
+      </c>
+      <c r="D27" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E27" s="13">
         <v>46104.0</v>
       </c>
-      <c r="F27" s="11" t="s">
+      <c r="F27" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G27" s="11">
+      <c r="G27" s="10">
         <v>12.0</v>
       </c>
-      <c r="H27" s="11">
+      <c r="H27" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I27" s="11">
+      <c r="I27" s="10">
         <v>2048.0</v>
       </c>
       <c r="J27" s="16">
@@ -9177,37 +9177,37 @@
       <c r="AH27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="11" t="s">
-        <v>129</v>
-      </c>
-      <c r="B28" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="C28" s="11" t="s">
-        <v>132</v>
-      </c>
-      <c r="D28" s="11" t="s">
+      <c r="A28" s="10" t="s">
+        <v>155</v>
+      </c>
+      <c r="B28" s="10" t="s">
+        <v>156</v>
+      </c>
+      <c r="C28" s="10" t="s">
+        <v>158</v>
+      </c>
+      <c r="D28" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E28" s="13">
         <v>46120.0</v>
       </c>
-      <c r="F28" s="11" t="s">
+      <c r="F28" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G28" s="11">
+      <c r="G28" s="10">
         <v>12.0</v>
       </c>
-      <c r="H28" s="11">
+      <c r="H28" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I28" s="11" t="s">
-        <v>51</v>
+      <c r="I28" s="10" t="s">
+        <v>61</v>
       </c>
       <c r="J28" s="16">
         <v>1912292.52</v>
       </c>
-      <c r="K28" s="11">
+      <c r="K28" s="10">
         <v>0.0</v>
       </c>
       <c r="L28" s="16">
@@ -9222,37 +9222,37 @@
       <c r="AH28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="11" t="s">
-        <v>133</v>
-      </c>
-      <c r="B29" s="11" t="s">
-        <v>134</v>
-      </c>
-      <c r="C29" s="11" t="s">
-        <v>135</v>
-      </c>
-      <c r="D29" s="11" t="s">
+      <c r="A29" s="10" t="s">
+        <v>160</v>
+      </c>
+      <c r="B29" s="10" t="s">
+        <v>161</v>
+      </c>
+      <c r="C29" s="10" t="s">
+        <v>162</v>
+      </c>
+      <c r="D29" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E29" s="13">
         <v>46196.0</v>
       </c>
-      <c r="F29" s="11" t="s">
+      <c r="F29" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G29" s="11">
+      <c r="G29" s="10">
         <v>12.0</v>
       </c>
-      <c r="H29" s="11">
+      <c r="H29" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I29" s="11">
+      <c r="I29" s="10">
         <v>2048.0</v>
       </c>
       <c r="J29" s="16">
         <v>1496713.48</v>
       </c>
-      <c r="K29" s="11">
+      <c r="K29" s="10">
         <v>0.0</v>
       </c>
       <c r="L29" s="16">
@@ -9267,37 +9267,37 @@
       <c r="AH29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="11" t="s">
-        <v>138</v>
-      </c>
-      <c r="B30" s="11" t="s">
-        <v>139</v>
-      </c>
-      <c r="C30" s="11" t="s">
-        <v>140</v>
-      </c>
-      <c r="D30" s="11" t="s">
+      <c r="A30" s="10" t="s">
+        <v>164</v>
+      </c>
+      <c r="B30" s="10" t="s">
+        <v>166</v>
+      </c>
+      <c r="C30" s="10" t="s">
+        <v>167</v>
+      </c>
+      <c r="D30" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E30" s="13">
         <v>46205.0</v>
       </c>
-      <c r="F30" s="11" t="s">
+      <c r="F30" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G30" s="11">
+      <c r="G30" s="10">
         <v>12.0</v>
       </c>
-      <c r="H30" s="11">
+      <c r="H30" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I30" s="11" t="s">
-        <v>44</v>
+      <c r="I30" s="10" t="s">
+        <v>54</v>
       </c>
       <c r="J30" s="16">
         <v>624166.14</v>
       </c>
-      <c r="K30" s="11">
+      <c r="K30" s="10">
         <v>0.0</v>
       </c>
       <c r="L30" s="16">
@@ -9312,37 +9312,37 @@
       <c r="AH30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="11" t="s">
-        <v>142</v>
-      </c>
-      <c r="B31" s="11" t="s">
-        <v>143</v>
-      </c>
-      <c r="C31" s="11" t="s">
-        <v>145</v>
-      </c>
-      <c r="D31" s="11" t="s">
+      <c r="A31" s="10" t="s">
+        <v>171</v>
+      </c>
+      <c r="B31" s="10" t="s">
+        <v>173</v>
+      </c>
+      <c r="C31" s="10" t="s">
+        <v>174</v>
+      </c>
+      <c r="D31" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E31" s="13">
         <v>46205.0</v>
       </c>
-      <c r="F31" s="11" t="s">
+      <c r="F31" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G31" s="11">
+      <c r="G31" s="10">
         <v>12.0</v>
       </c>
-      <c r="H31" s="11">
+      <c r="H31" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I31" s="11" t="s">
-        <v>112</v>
+      <c r="I31" s="10" t="s">
+        <v>134</v>
       </c>
       <c r="J31" s="16">
         <v>18462.36</v>
       </c>
-      <c r="K31" s="11">
+      <c r="K31" s="10">
         <v>0.0</v>
       </c>
       <c r="L31" s="16">
@@ -9357,37 +9357,37 @@
       <c r="AH31" s="4"/>
     </row>
     <row r="32">
-      <c r="A32" s="11" t="s">
-        <v>147</v>
-      </c>
-      <c r="B32" s="11" t="s">
-        <v>143</v>
+      <c r="A32" s="10" t="s">
+        <v>175</v>
+      </c>
+      <c r="B32" s="10" t="s">
+        <v>173</v>
       </c>
       <c r="C32" s="16" t="s">
-        <v>148</v>
-      </c>
-      <c r="D32" s="11" t="s">
+        <v>176</v>
+      </c>
+      <c r="D32" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E32" s="13">
         <v>46213.0</v>
       </c>
-      <c r="F32" s="11" t="s">
+      <c r="F32" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G32" s="11">
+      <c r="G32" s="10">
         <v>12.0</v>
       </c>
-      <c r="H32" s="11">
+      <c r="H32" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I32" s="11" t="s">
-        <v>112</v>
+      <c r="I32" s="10" t="s">
+        <v>134</v>
       </c>
       <c r="J32" s="16">
         <v>1530656.62</v>
       </c>
-      <c r="K32" s="11">
+      <c r="K32" s="10">
         <v>0.0</v>
       </c>
       <c r="L32" s="16">
@@ -9402,37 +9402,37 @@
       <c r="AH32" s="4"/>
     </row>
     <row r="33">
-      <c r="A33" s="11" t="s">
-        <v>150</v>
-      </c>
-      <c r="B33" s="11" t="s">
-        <v>134</v>
+      <c r="A33" s="10" t="s">
+        <v>177</v>
+      </c>
+      <c r="B33" s="10" t="s">
+        <v>161</v>
       </c>
       <c r="C33" s="16" t="s">
-        <v>152</v>
-      </c>
-      <c r="D33" s="11" t="s">
+        <v>178</v>
+      </c>
+      <c r="D33" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E33" s="13">
         <v>46227.0</v>
       </c>
-      <c r="F33" s="11" t="s">
+      <c r="F33" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G33" s="11">
+      <c r="G33" s="10">
         <v>12.0</v>
       </c>
-      <c r="H33" s="11">
+      <c r="H33" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I33" s="11">
+      <c r="I33" s="10">
         <v>2048.0</v>
       </c>
       <c r="J33" s="16">
         <v>173846.38</v>
       </c>
-      <c r="K33" s="11">
+      <c r="K33" s="10">
         <v>0.0</v>
       </c>
       <c r="L33" s="16">
@@ -9447,37 +9447,37 @@
       <c r="AH33" s="4"/>
     </row>
     <row r="34">
-      <c r="A34" s="11" t="s">
-        <v>153</v>
-      </c>
-      <c r="B34" s="11" t="s">
-        <v>154</v>
-      </c>
-      <c r="C34" s="11" t="s">
-        <v>155</v>
-      </c>
-      <c r="D34" s="11" t="s">
+      <c r="A34" s="10" t="s">
+        <v>180</v>
+      </c>
+      <c r="B34" s="10" t="s">
+        <v>181</v>
+      </c>
+      <c r="C34" s="10" t="s">
+        <v>182</v>
+      </c>
+      <c r="D34" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E34" s="13">
         <v>46240.0</v>
       </c>
-      <c r="F34" s="11" t="s">
+      <c r="F34" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G34" s="11">
+      <c r="G34" s="10">
         <v>12.0</v>
       </c>
-      <c r="H34" s="11">
+      <c r="H34" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I34" s="11" t="s">
-        <v>157</v>
+      <c r="I34" s="10" t="s">
+        <v>184</v>
       </c>
       <c r="J34" s="16">
         <v>236343.68</v>
       </c>
-      <c r="K34" s="11">
+      <c r="K34" s="10">
         <v>0.0</v>
       </c>
       <c r="L34" s="16">

</xml_diff>

<commit_message>
Atualização automática: pagamentos (13/08/2026 13:04)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/01_Bases_Originais/005_CELOG_2025/005_CELOG-PAMALS_2025 online.xlsx
+++ b/Contrato 005/Dashboard/01_Bases_Originais/005_CELOG_2025/005_CELOG-PAMALS_2025 online.xlsx
@@ -30,12 +30,12 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="341" uniqueCount="216">
   <si>
+    <t>Saldo</t>
+  </si>
+  <si>
     <t>Controle de pagamentos</t>
   </si>
   <si>
-    <t>Saldo</t>
-  </si>
-  <si>
     <t>2025NE000005</t>
   </si>
   <si>
@@ -81,16 +81,22 @@
     <t>Ação</t>
   </si>
   <si>
+    <t>2025NE000369</t>
+  </si>
+  <si>
     <t>PAG</t>
   </si>
   <si>
+    <t>C25516</t>
+  </si>
+  <si>
     <t>Moeda</t>
   </si>
   <si>
     <t>Valor Total do Contrato</t>
   </si>
   <si>
-    <t>2025NE000369</t>
+    <t>25E0387</t>
   </si>
   <si>
     <t>Valor a Empenhar</t>
@@ -99,15 +105,9 @@
     <t>Valor Empenhado</t>
   </si>
   <si>
-    <t>C25516</t>
-  </si>
-  <si>
     <t>Valor Liquidado</t>
   </si>
   <si>
-    <t>25E0387</t>
-  </si>
-  <si>
     <t>Saldo (Valor a Faturar)</t>
   </si>
   <si>
@@ -135,12 +135,12 @@
     <t>2025NE000371</t>
   </si>
   <si>
+    <t>25E0389</t>
+  </si>
+  <si>
     <t>Vigente</t>
   </si>
   <si>
-    <t>25E0389</t>
-  </si>
-  <si>
     <t>2048 20YJ 21EM 219C 20SP 20X7 2000</t>
   </si>
   <si>
@@ -195,39 +195,39 @@
     <t>2025NE000559</t>
   </si>
   <si>
+    <t>Empenho</t>
+  </si>
+  <si>
     <t>C25545</t>
   </si>
   <si>
+    <t>Observações</t>
+  </si>
+  <si>
     <t>25E0524</t>
   </si>
   <si>
-    <t>Empenho</t>
-  </si>
-  <si>
-    <t>Observações</t>
-  </si>
-  <si>
     <t>Vencimento</t>
   </si>
   <si>
+    <t>Valor das Nfs</t>
+  </si>
+  <si>
+    <t>Ordem de Pagamento</t>
+  </si>
+  <si>
     <t>20X7</t>
   </si>
   <si>
-    <t>Valor das Nfs</t>
-  </si>
-  <si>
-    <t>Ordem de Pagamento</t>
-  </si>
-  <si>
     <t>Faturado</t>
   </si>
   <si>
+    <t>Pendente</t>
+  </si>
+  <si>
     <t>2025NE000770</t>
   </si>
   <si>
-    <t>Pendente</t>
-  </si>
-  <si>
     <t>25E0731</t>
   </si>
   <si>
@@ -243,6 +243,9 @@
     <t>-</t>
   </si>
   <si>
+    <t xml:space="preserve">2025NE000369 </t>
+  </si>
+  <si>
     <t>2025NE000843</t>
   </si>
   <si>
@@ -252,9 +255,6 @@
     <t>25E0787</t>
   </si>
   <si>
-    <t xml:space="preserve">2025NE000369 </t>
-  </si>
-  <si>
     <t>219C</t>
   </si>
   <si>
@@ -279,6 +279,9 @@
     <t>MAR/25</t>
   </si>
   <si>
+    <t>2025NE000367, 2025NE000369, 2025NE000371, 2025NE000413</t>
+  </si>
+  <si>
     <t>2025NE001598</t>
   </si>
   <si>
@@ -288,9 +291,6 @@
     <t>25E1446</t>
   </si>
   <si>
-    <t>2025NE000367, 2025NE000369, 2025NE000371, 2025NE000413</t>
-  </si>
-  <si>
     <t>2025NP001979</t>
   </si>
   <si>
@@ -300,6 +300,12 @@
     <t>25E1475</t>
   </si>
   <si>
+    <t>ABR/25</t>
+  </si>
+  <si>
+    <t>2025NE000413, 2025NE000414, 2025NE000559</t>
+  </si>
+  <si>
     <t>2025NE001629</t>
   </si>
   <si>
@@ -309,24 +315,18 @@
     <t>25E1477</t>
   </si>
   <si>
-    <t>ABR/25</t>
-  </si>
-  <si>
-    <t>2025NE000413, 2025NE000414, 2025NE000559</t>
+    <t>2025NP002341</t>
+  </si>
+  <si>
+    <t>MAI/25</t>
   </si>
   <si>
     <t>2025NE001687</t>
   </si>
   <si>
-    <t>2025NP002341</t>
-  </si>
-  <si>
     <t>25E1535</t>
   </si>
   <si>
-    <t>MAI/25</t>
-  </si>
-  <si>
     <t>2025NE001688</t>
   </si>
   <si>
@@ -336,13 +336,13 @@
     <t>2025NP002884</t>
   </si>
   <si>
+    <t>2025NE001689</t>
+  </si>
+  <si>
+    <t>25E1537</t>
+  </si>
+  <si>
     <t>JUN/25</t>
-  </si>
-  <si>
-    <t>2025NE001689</t>
-  </si>
-  <si>
-    <t>25E1537</t>
   </si>
   <si>
     <t>2025NE000005,
@@ -351,55 +351,64 @@
 2025NE000774</t>
   </si>
   <si>
+    <t>2025NE001690</t>
+  </si>
+  <si>
+    <t>25E1538</t>
+  </si>
+  <si>
     <t>2025NP400522</t>
   </si>
   <si>
-    <t>2025NE001690</t>
-  </si>
-  <si>
-    <t>25E1538</t>
+    <t>2025NE001823</t>
+  </si>
+  <si>
+    <t>C25865</t>
+  </si>
+  <si>
+    <t>25E1666</t>
   </si>
   <si>
     <t>JUL/25</t>
   </si>
   <si>
-    <t>2025NE001823</t>
-  </si>
-  <si>
-    <t>C25865</t>
-  </si>
-  <si>
-    <t>25E1666</t>
-  </si>
-  <si>
     <t>2025NE000843, 2025NE001200</t>
   </si>
   <si>
+    <t>2025NE001828</t>
+  </si>
+  <si>
+    <t>C25869</t>
+  </si>
+  <si>
+    <t>25E1667</t>
+  </si>
+  <si>
     <t>2025NP003724</t>
   </si>
   <si>
-    <t>2025NE001828</t>
-  </si>
-  <si>
-    <t>C25869</t>
-  </si>
-  <si>
-    <t>25E1667</t>
-  </si>
-  <si>
     <t>20YJ</t>
   </si>
   <si>
     <t>AGO/25</t>
   </si>
   <si>
+    <t>2025NE001830</t>
+  </si>
+  <si>
+    <t>25E1669</t>
+  </si>
+  <si>
     <t>2025NP004558</t>
   </si>
   <si>
-    <t>2025NE001830</t>
-  </si>
-  <si>
-    <t>25E1669</t>
+    <t>2025NE002200</t>
+  </si>
+  <si>
+    <t>C25863</t>
+  </si>
+  <si>
+    <t>25E2021</t>
   </si>
   <si>
     <t>SET/25</t>
@@ -409,13 +418,10 @@
 2025NE001828</t>
   </si>
   <si>
-    <t>2025NE002200</t>
-  </si>
-  <si>
-    <t>C25863</t>
-  </si>
-  <si>
-    <t>25E2021</t>
+    <t>2025NE002237</t>
+  </si>
+  <si>
+    <t>25E2058</t>
   </si>
   <si>
     <t>2025NP004897</t>
@@ -424,36 +430,30 @@
     <t>OUT/25</t>
   </si>
   <si>
-    <t>2025NE002237</t>
-  </si>
-  <si>
     <t>2025NE001688, 2025NE001828, 2025NE002200</t>
   </si>
   <si>
-    <t>25E2058</t>
+    <t>2026NE000330</t>
+  </si>
+  <si>
+    <t>C26163</t>
+  </si>
+  <si>
+    <t>26E0320</t>
   </si>
   <si>
     <t>2025NP004932</t>
   </si>
   <si>
-    <t>2026NE000330</t>
-  </si>
-  <si>
-    <t>C26163</t>
-  </si>
-  <si>
-    <t>26E0320</t>
-  </si>
-  <si>
     <t>NOV/25</t>
   </si>
   <si>
+    <t>2026NE000388</t>
+  </si>
+  <si>
     <t>2025NE001687, 2025NE001689, 2025NE001690, 2025NE001823, 2025NE001830, 2025NE002237</t>
   </si>
   <si>
-    <t>2026NE000388</t>
-  </si>
-  <si>
     <t>C26193</t>
   </si>
   <si>
@@ -481,6 +481,9 @@
     <t>2026NP400412</t>
   </si>
   <si>
+    <t>JAN/26</t>
+  </si>
+  <si>
     <t>2026NE000816</t>
   </si>
   <si>
@@ -490,7 +493,10 @@
     <t>26E0776</t>
   </si>
   <si>
-    <t>JAN/26</t>
+    <t>2026NP401035</t>
+  </si>
+  <si>
+    <t>FEV/26</t>
   </si>
   <si>
     <t>2026NE000817</t>
@@ -499,13 +505,13 @@
     <t>C26326</t>
   </si>
   <si>
-    <t>2026NP401035</t>
-  </si>
-  <si>
     <t>26E0777</t>
   </si>
   <si>
-    <t>FEV/26</t>
+    <t>2025NE001627, 2025NE001629, 2025NE001823</t>
+  </si>
+  <si>
+    <t>2026NP402272</t>
   </si>
   <si>
     <t>2026NE000842</t>
@@ -514,19 +520,28 @@
     <t>26E0803</t>
   </si>
   <si>
-    <t>2025NE001627, 2025NE001629, 2025NE001823</t>
+    <t>MAR/26</t>
+  </si>
+  <si>
+    <t>2025NE000770, 2025NE001627</t>
+  </si>
+  <si>
+    <t>R$ 1.350.542,52</t>
+  </si>
+  <si>
+    <t>2026NP401762</t>
   </si>
   <si>
     <t>2026NE000944</t>
   </si>
   <si>
-    <t>2026NP402272</t>
-  </si>
-  <si>
     <t>26E0906</t>
   </si>
   <si>
-    <t>MAR/26</t>
+    <t>ABR/26</t>
+  </si>
+  <si>
+    <t>2025NE000770, 2025NE001065, 2025NE001627</t>
   </si>
   <si>
     <t>2026NE001015</t>
@@ -539,21 +554,6 @@
   </si>
   <si>
     <t>20XV</t>
-  </si>
-  <si>
-    <t>2025NE000770, 2025NE001627</t>
-  </si>
-  <si>
-    <t>R$ 1.350.542,52</t>
-  </si>
-  <si>
-    <t>2026NP401762</t>
-  </si>
-  <si>
-    <t>ABR/26</t>
-  </si>
-  <si>
-    <t>2025NE000770, 2025NE001065, 2025NE001627</t>
   </si>
   <si>
     <t>REAJUSTE</t>
@@ -888,27 +888,27 @@
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="3" fontId="2" numFmtId="0" xfId="0" applyFill="1" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0"/>
+    </xf>
     <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyFill="1" applyFont="1"/>
     <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="5" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="11" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
@@ -1440,22 +1440,22 @@
       <c r="S1" s="1"/>
       <c r="T1" s="1"/>
       <c r="U1" s="1"/>
-      <c r="V1" s="3"/>
+      <c r="V1" s="4"/>
     </row>
     <row r="2" ht="59.25" customHeight="1">
-      <c r="A2" s="4"/>
-      <c r="B2" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="V2" s="8"/>
-      <c r="W2" s="9"/>
-      <c r="X2" s="9"/>
-      <c r="Y2" s="9"/>
-      <c r="Z2" s="9"/>
-      <c r="AA2" s="9"/>
-      <c r="AB2" s="9"/>
-      <c r="AC2" s="9"/>
-      <c r="AD2" s="9"/>
+      <c r="A2" s="5"/>
+      <c r="B2" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="V2" s="9"/>
+      <c r="W2" s="10"/>
+      <c r="X2" s="10"/>
+      <c r="Y2" s="10"/>
+      <c r="Z2" s="10"/>
+      <c r="AA2" s="10"/>
+      <c r="AB2" s="10"/>
+      <c r="AC2" s="10"/>
+      <c r="AD2" s="10"/>
     </row>
     <row r="3" ht="12.75" customHeight="1">
       <c r="A3" s="1"/>
@@ -1479,7 +1479,7 @@
       <c r="S3" s="13"/>
       <c r="T3" s="13"/>
       <c r="U3" s="13"/>
-      <c r="V3" s="3"/>
+      <c r="V3" s="4"/>
     </row>
     <row r="4" ht="12.75" customHeight="1">
       <c r="A4" s="15"/>
@@ -1509,22 +1509,22 @@
         <v>16</v>
       </c>
       <c r="K4" s="16" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="L4" s="16" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="M4" s="17" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="N4" s="17" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="O4" s="17" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="P4" s="17" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="Q4" s="17" t="s">
         <v>26</v>
@@ -1541,7 +1541,7 @@
       <c r="U4" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="V4" s="3"/>
+      <c r="V4" s="4"/>
     </row>
     <row r="5" ht="12.75" customHeight="1">
       <c r="A5" s="15"/>
@@ -1566,7 +1566,7 @@
         <v>1564.0</v>
       </c>
       <c r="J5" s="19" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="K5" s="19" t="s">
         <v>37</v>
@@ -1595,13 +1595,13 @@
       <c r="S5" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="V5" s="3"/>
+      <c r="V5" s="4"/>
     </row>
     <row r="6" ht="12.75" customHeight="1">
       <c r="A6" s="15"/>
       <c r="B6" s="15"/>
       <c r="L6" s="22"/>
-      <c r="V6" s="3"/>
+      <c r="V6" s="4"/>
     </row>
     <row r="7" ht="12.75" customHeight="1">
       <c r="A7" s="23"/>
@@ -1620,7 +1620,7 @@
       <c r="N7" s="25"/>
       <c r="O7" s="25"/>
       <c r="P7" s="27"/>
-      <c r="V7" s="3"/>
+      <c r="V7" s="4"/>
     </row>
     <row r="8" ht="12.75" customHeight="1">
       <c r="A8" s="23"/>
@@ -1641,29 +1641,29 @@
         <v>53</v>
       </c>
       <c r="H8" s="28" t="s">
+        <v>55</v>
+      </c>
+      <c r="I8" s="30" t="s">
         <v>57</v>
-      </c>
-      <c r="I8" s="30" t="s">
-        <v>58</v>
       </c>
       <c r="J8" s="28" t="s">
         <v>59</v>
       </c>
       <c r="K8" s="28" t="s">
+        <v>60</v>
+      </c>
+      <c r="L8" s="31" t="s">
         <v>61</v>
-      </c>
-      <c r="L8" s="31" t="s">
-        <v>62</v>
       </c>
       <c r="M8" s="30" t="s">
         <v>63</v>
       </c>
       <c r="N8" s="28" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="O8" s="28"/>
       <c r="P8" s="27"/>
-      <c r="V8" s="3"/>
+      <c r="V8" s="4"/>
     </row>
     <row r="9" ht="19.5" customHeight="1">
       <c r="A9" s="23"/>
@@ -1684,7 +1684,7 @@
         <v>45740.0</v>
       </c>
       <c r="H9" s="35" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="I9" s="36"/>
       <c r="J9" s="36">
@@ -1703,7 +1703,7 @@
       <c r="N9" s="40"/>
       <c r="O9" s="25"/>
       <c r="P9" s="27"/>
-      <c r="V9" s="3"/>
+      <c r="V9" s="4"/>
     </row>
     <row r="10" ht="51.0" customHeight="1">
       <c r="A10" s="23"/>
@@ -1722,7 +1722,7 @@
         <v>45775.0</v>
       </c>
       <c r="H10" s="35" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="I10" s="36"/>
       <c r="J10" s="36">
@@ -1741,14 +1741,14 @@
       <c r="N10" s="42"/>
       <c r="O10" s="25"/>
       <c r="P10" s="27"/>
-      <c r="V10" s="3"/>
+      <c r="V10" s="4"/>
     </row>
     <row r="11" ht="12.75" customHeight="1">
       <c r="A11" s="23"/>
       <c r="B11" s="23"/>
       <c r="C11" s="41"/>
       <c r="D11" s="33" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="E11" s="34" t="s">
         <v>70</v>
@@ -1760,7 +1760,7 @@
         <v>45799.0</v>
       </c>
       <c r="H11" s="35" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="I11" s="36"/>
       <c r="J11" s="36">
@@ -1770,7 +1770,7 @@
         <v>974557.12</v>
       </c>
       <c r="L11" s="34" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="M11" s="39">
         <v>974557.12</v>
@@ -1778,14 +1778,14 @@
       <c r="N11" s="42"/>
       <c r="O11" s="25"/>
       <c r="P11" s="27"/>
-      <c r="V11" s="3"/>
+      <c r="V11" s="4"/>
     </row>
     <row r="12" ht="27.75" customHeight="1">
       <c r="A12" s="23"/>
       <c r="B12" s="23"/>
       <c r="C12" s="41"/>
       <c r="D12" s="33" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="E12" s="34" t="s">
         <v>70</v>
@@ -1797,7 +1797,7 @@
         <v>45856.0</v>
       </c>
       <c r="H12" s="44" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="I12" s="36"/>
       <c r="J12" s="36">
@@ -1815,14 +1815,14 @@
       <c r="N12" s="47"/>
       <c r="O12" s="25"/>
       <c r="P12" s="27"/>
-      <c r="V12" s="3"/>
+      <c r="V12" s="4"/>
     </row>
     <row r="13">
       <c r="A13" s="23"/>
       <c r="B13" s="23"/>
       <c r="C13" s="41"/>
       <c r="D13" s="48" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="E13" s="34" t="s">
         <v>70</v>
@@ -1844,7 +1844,7 @@
         <v>1223702.3</v>
       </c>
       <c r="L13" s="34" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="M13" s="39">
         <v>1223702.3</v>
@@ -1852,14 +1852,14 @@
       <c r="N13" s="47"/>
       <c r="O13" s="25"/>
       <c r="P13" s="49"/>
-      <c r="V13" s="3"/>
+      <c r="V13" s="4"/>
     </row>
     <row r="14">
       <c r="A14" s="23"/>
       <c r="B14" s="23"/>
       <c r="C14" s="41"/>
       <c r="D14" s="48" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="E14" s="34" t="s">
         <v>70</v>
@@ -1881,7 +1881,7 @@
         <v>1011677.95</v>
       </c>
       <c r="L14" s="34" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="M14" s="39">
         <v>1011677.95</v>
@@ -1889,7 +1889,7 @@
       <c r="N14" s="42"/>
       <c r="O14" s="25"/>
       <c r="P14" s="27"/>
-      <c r="V14" s="3"/>
+      <c r="V14" s="4"/>
     </row>
     <row r="15">
       <c r="A15" s="23"/>
@@ -1918,21 +1918,21 @@
         <v>896744.06</v>
       </c>
       <c r="L15" s="34" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="M15" s="39">
         <v>896744.06</v>
       </c>
       <c r="N15" s="47"/>
       <c r="O15" s="25"/>
-      <c r="V15" s="3"/>
+      <c r="V15" s="4"/>
     </row>
     <row r="16">
       <c r="A16" s="23"/>
       <c r="B16" s="23"/>
       <c r="C16" s="41"/>
       <c r="D16" s="48" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="E16" s="34" t="s">
         <v>70</v>
@@ -1944,7 +1944,7 @@
         <v>45957.0</v>
       </c>
       <c r="H16" s="34" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="I16" s="43"/>
       <c r="J16" s="43">
@@ -1954,21 +1954,21 @@
         <v>919329.06</v>
       </c>
       <c r="L16" s="34" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="M16" s="39">
         <v>919329.06</v>
       </c>
       <c r="N16" s="42"/>
       <c r="O16" s="25"/>
-      <c r="V16" s="3"/>
+      <c r="V16" s="4"/>
     </row>
     <row r="17">
       <c r="A17" s="23"/>
       <c r="B17" s="23"/>
       <c r="C17" s="41"/>
       <c r="D17" s="48" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="E17" s="34"/>
       <c r="F17" s="34">
@@ -1978,7 +1978,7 @@
         <v>45972.0</v>
       </c>
       <c r="H17" s="34" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="I17" s="34"/>
       <c r="J17" s="43">
@@ -1988,14 +1988,14 @@
         <v>1157009.26</v>
       </c>
       <c r="L17" s="34" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="M17" s="39">
         <v>1157009.26</v>
       </c>
       <c r="N17" s="51"/>
       <c r="O17" s="25"/>
-      <c r="V17" s="3"/>
+      <c r="V17" s="4"/>
     </row>
     <row r="18">
       <c r="A18" s="23"/>
@@ -2014,7 +2014,7 @@
         <v>46008.0</v>
       </c>
       <c r="H18" s="34" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="I18" s="34"/>
       <c r="J18" s="43">
@@ -2082,7 +2082,7 @@
       <c r="B20" s="23"/>
       <c r="C20" s="41"/>
       <c r="D20" s="48" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="E20" s="34"/>
       <c r="F20" s="34">
@@ -2092,7 +2092,7 @@
         <v>46078.0</v>
       </c>
       <c r="H20" s="34" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="I20" s="43"/>
       <c r="J20" s="43">
@@ -2102,7 +2102,7 @@
         <v>719561.08</v>
       </c>
       <c r="L20" s="34" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="M20" s="39">
         <v>719561.08</v>
@@ -2120,7 +2120,7 @@
       <c r="B21" s="23"/>
       <c r="C21" s="41"/>
       <c r="D21" s="48" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="E21" s="34"/>
       <c r="F21" s="34">
@@ -2130,7 +2130,7 @@
         <v>46094.0</v>
       </c>
       <c r="H21" s="34" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="I21" s="43"/>
       <c r="J21" s="43">
@@ -2140,7 +2140,7 @@
         <v>885881.08</v>
       </c>
       <c r="L21" s="34" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="M21" s="39">
         <v>885881.08</v>
@@ -2158,7 +2158,7 @@
       <c r="B22" s="23"/>
       <c r="C22" s="41"/>
       <c r="D22" s="48" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="E22" s="34"/>
       <c r="F22" s="34">
@@ -2168,20 +2168,20 @@
         <v>46128.0</v>
       </c>
       <c r="H22" s="34" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
       <c r="I22" s="43"/>
       <c r="J22" s="43">
         <v>46164.0</v>
       </c>
       <c r="K22" s="45" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="L22" s="34" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="M22" s="39" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="N22" s="51"/>
       <c r="O22" s="25"/>
@@ -2196,7 +2196,7 @@
       <c r="B23" s="23"/>
       <c r="C23" s="41"/>
       <c r="D23" s="48" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="E23" s="34"/>
       <c r="F23" s="34">
@@ -2206,7 +2206,7 @@
         <v>46156.0</v>
       </c>
       <c r="H23" s="34" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="I23" s="43"/>
       <c r="J23" s="43">
@@ -2216,7 +2216,7 @@
         <v>1108954.4358333333</v>
       </c>
       <c r="L23" s="34" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="M23" s="39">
         <v>1108954.4358333333</v>
@@ -2244,7 +2244,7 @@
         <v>46149.0</v>
       </c>
       <c r="H24" s="34" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="I24" s="43"/>
       <c r="J24" s="43">
@@ -2282,7 +2282,7 @@
         <v>46156.0</v>
       </c>
       <c r="H25" s="34" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="I25" s="43"/>
       <c r="J25" s="43">
@@ -2384,21 +2384,21 @@
       </c>
       <c r="G28" s="28"/>
       <c r="H28" s="28" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="I28" s="28"/>
       <c r="J28" s="28"/>
       <c r="K28" s="56" t="s">
+        <v>60</v>
+      </c>
+      <c r="L28" s="31" t="s">
         <v>61</v>
-      </c>
-      <c r="L28" s="31" t="s">
-        <v>62</v>
       </c>
       <c r="M28" s="57" t="s">
         <v>63</v>
       </c>
       <c r="N28" s="28" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="O28" s="25"/>
       <c r="P28" s="27"/>
@@ -2530,7 +2530,7 @@
         <v>45853.0</v>
       </c>
       <c r="H31" s="34" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="I31" s="43"/>
       <c r="J31" s="43">
@@ -2579,7 +2579,7 @@
         <v>45910.0</v>
       </c>
       <c r="H32" s="34" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="I32" s="43"/>
       <c r="J32" s="43">
@@ -2628,7 +2628,7 @@
         <v>45904.0</v>
       </c>
       <c r="H33" s="34" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="I33" s="66"/>
       <c r="J33" s="66">
@@ -2677,7 +2677,7 @@
         <v>46008.0</v>
       </c>
       <c r="H34" s="34" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="I34" s="66"/>
       <c r="J34" s="66">
@@ -2726,7 +2726,7 @@
         <v>45930.0</v>
       </c>
       <c r="H35" s="34" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I35" s="66"/>
       <c r="J35" s="66">
@@ -2775,7 +2775,7 @@
         <v>45968.0</v>
       </c>
       <c r="H36" s="34" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="I36" s="66"/>
       <c r="J36" s="66">
@@ -2824,7 +2824,7 @@
         <v>46043.0</v>
       </c>
       <c r="H37" s="65" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="I37" s="70"/>
       <c r="J37" s="69">
@@ -3019,7 +3019,7 @@
         <v>46104.0</v>
       </c>
       <c r="H42" s="65" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="I42" s="70"/>
       <c r="J42" s="69">
@@ -3082,7 +3082,7 @@
         <v>58868.35</v>
       </c>
       <c r="N43" s="51"/>
-      <c r="V43" s="3"/>
+      <c r="V43" s="4"/>
     </row>
     <row r="44" ht="12.75" customHeight="1">
       <c r="A44" s="15"/>
@@ -3090,7 +3090,7 @@
       <c r="C44" s="41"/>
       <c r="K44" s="75"/>
       <c r="M44" s="75"/>
-      <c r="V44" s="3"/>
+      <c r="V44" s="4"/>
     </row>
     <row r="45" ht="12.75" customHeight="1">
       <c r="A45" s="15"/>
@@ -3098,31 +3098,31 @@
       <c r="C45" s="41"/>
       <c r="K45" s="75"/>
       <c r="M45" s="75"/>
-      <c r="V45" s="3"/>
+      <c r="V45" s="4"/>
     </row>
     <row r="46" ht="12.75" customHeight="1">
       <c r="A46" s="15"/>
       <c r="B46" s="15"/>
       <c r="C46" s="41"/>
-      <c r="V46" s="3"/>
+      <c r="V46" s="4"/>
     </row>
     <row r="47" ht="12.75" customHeight="1">
       <c r="A47" s="15"/>
       <c r="B47" s="15"/>
       <c r="C47" s="41"/>
-      <c r="V47" s="3"/>
+      <c r="V47" s="4"/>
     </row>
     <row r="48" ht="12.75" customHeight="1">
       <c r="A48" s="15"/>
       <c r="B48" s="15"/>
       <c r="C48" s="41"/>
-      <c r="V48" s="3"/>
+      <c r="V48" s="4"/>
     </row>
     <row r="49" ht="12.75" customHeight="1">
       <c r="A49" s="15"/>
       <c r="B49" s="15"/>
       <c r="C49" s="41"/>
-      <c r="V49" s="3"/>
+      <c r="V49" s="4"/>
     </row>
     <row r="50" ht="12.75" customHeight="1">
       <c r="A50" s="15"/>
@@ -3130,7 +3130,7 @@
       <c r="C50" s="55"/>
       <c r="K50" s="75"/>
       <c r="M50" s="75"/>
-      <c r="V50" s="3"/>
+      <c r="V50" s="4"/>
     </row>
     <row r="51" ht="12.75" customHeight="1">
       <c r="A51" s="15"/>
@@ -3154,7 +3154,7 @@
       <c r="S51" s="76"/>
       <c r="T51" s="76"/>
       <c r="U51" s="76"/>
-      <c r="V51" s="3"/>
+      <c r="V51" s="4"/>
     </row>
     <row r="52" ht="12.75" customHeight="1">
       <c r="A52" s="15"/>
@@ -8035,11 +8035,11 @@
       <c r="AH1" s="2"/>
     </row>
     <row r="2">
-      <c r="A2" s="5">
+      <c r="A2" s="3">
         <v>46212.0</v>
       </c>
-      <c r="L2" s="7" t="s">
-        <v>1</v>
+      <c r="L2" s="6" t="s">
+        <v>0</v>
       </c>
       <c r="AB2" s="2"/>
       <c r="AC2" s="2"/>
@@ -8050,31 +8050,31 @@
       <c r="AH2" s="2"/>
     </row>
     <row r="3">
-      <c r="A3" s="10" t="s">
+      <c r="A3" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="B3" s="8" t="s">
         <v>3</v>
       </c>
       <c r="C3" s="11">
         <v>2.5E32</v>
       </c>
-      <c r="D3" s="10" t="s">
+      <c r="D3" s="8" t="s">
         <v>4</v>
       </c>
       <c r="E3" s="12">
         <v>45686.0</v>
       </c>
-      <c r="F3" s="10" t="s">
+      <c r="F3" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G3" s="10">
+      <c r="G3" s="8">
         <v>12.0</v>
       </c>
-      <c r="H3" s="10">
+      <c r="H3" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I3" s="10">
+      <c r="I3" s="8">
         <v>2048.0</v>
       </c>
       <c r="J3" s="14">
@@ -8083,7 +8083,7 @@
       <c r="K3" s="14">
         <v>1000.0</v>
       </c>
-      <c r="L3" s="10">
+      <c r="L3" s="8">
         <v>0.0</v>
       </c>
       <c r="AB3" s="2"/>
@@ -8095,31 +8095,31 @@
       <c r="AH3" s="2"/>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="s">
+      <c r="A4" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="B4" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="C4" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="D4" s="10" t="s">
+      <c r="D4" s="8" t="s">
         <v>4</v>
       </c>
       <c r="E4" s="12">
         <v>45762.0</v>
       </c>
-      <c r="F4" s="10" t="s">
+      <c r="F4" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G4" s="10">
+      <c r="G4" s="8">
         <v>12.0</v>
       </c>
-      <c r="H4" s="10">
+      <c r="H4" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I4" s="10">
+      <c r="I4" s="8">
         <v>2048.0</v>
       </c>
       <c r="J4" s="14">
@@ -8128,7 +8128,7 @@
       <c r="K4" s="14">
         <v>52250.04</v>
       </c>
-      <c r="L4" s="10">
+      <c r="L4" s="8">
         <v>0.0</v>
       </c>
       <c r="AB4" s="2"/>
@@ -8140,31 +8140,31 @@
       <c r="AH4" s="2"/>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="B5" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="C5" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="D5" s="10" t="s">
+      <c r="A5" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D5" s="8" t="s">
         <v>4</v>
       </c>
       <c r="E5" s="12">
         <v>45762.0</v>
       </c>
-      <c r="F5" s="10" t="s">
+      <c r="F5" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G5" s="10">
+      <c r="G5" s="8">
         <v>12.0</v>
       </c>
-      <c r="H5" s="10">
+      <c r="H5" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I5" s="10">
+      <c r="I5" s="8">
         <v>2048.0</v>
       </c>
       <c r="J5" s="14">
@@ -8173,7 +8173,7 @@
       <c r="K5" s="14">
         <v>881914.18</v>
       </c>
-      <c r="L5" s="10">
+      <c r="L5" s="8">
         <v>0.0</v>
       </c>
       <c r="AB5" s="2"/>
@@ -8185,31 +8185,31 @@
       <c r="AH5" s="2"/>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="s">
+      <c r="A6" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="B6" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="C6" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="D6" s="10" t="s">
+      <c r="B6" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="D6" s="8" t="s">
         <v>4</v>
       </c>
       <c r="E6" s="12">
         <v>45762.0</v>
       </c>
-      <c r="F6" s="10" t="s">
+      <c r="F6" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G6" s="10">
+      <c r="G6" s="8">
         <v>12.0</v>
       </c>
-      <c r="H6" s="10">
+      <c r="H6" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I6" s="10">
+      <c r="I6" s="8">
         <v>2048.0</v>
       </c>
       <c r="J6" s="14">
@@ -8218,7 +8218,7 @@
       <c r="K6" s="14">
         <v>750000.0</v>
       </c>
-      <c r="L6" s="10">
+      <c r="L6" s="8">
         <v>0.0</v>
       </c>
       <c r="AB6" s="2"/>
@@ -8230,31 +8230,31 @@
       <c r="AH6" s="2"/>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="s">
+      <c r="A7" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="B7" s="10" t="s">
+      <c r="B7" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="C7" s="10" t="s">
+      <c r="C7" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="D7" s="10" t="s">
+      <c r="D7" s="8" t="s">
         <v>4</v>
       </c>
       <c r="E7" s="12">
         <v>45763.0</v>
       </c>
-      <c r="F7" s="10" t="s">
+      <c r="F7" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G7" s="10">
+      <c r="G7" s="8">
         <v>12.0</v>
       </c>
-      <c r="H7" s="10">
+      <c r="H7" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I7" s="10" t="s">
+      <c r="I7" s="8" t="s">
         <v>44</v>
       </c>
       <c r="J7" s="14">
@@ -8263,7 +8263,7 @@
       <c r="K7" s="14">
         <v>949835.78</v>
       </c>
-      <c r="L7" s="10">
+      <c r="L7" s="8">
         <v>0.0</v>
       </c>
       <c r="AB7" s="2"/>
@@ -8275,31 +8275,31 @@
       <c r="AH7" s="2"/>
     </row>
     <row r="8">
-      <c r="A8" s="10" t="s">
+      <c r="A8" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="B8" s="10" t="s">
+      <c r="B8" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="C8" s="10" t="s">
+      <c r="C8" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="D8" s="10" t="s">
+      <c r="D8" s="8" t="s">
         <v>4</v>
       </c>
       <c r="E8" s="12">
         <v>45763.0</v>
       </c>
-      <c r="F8" s="10" t="s">
+      <c r="F8" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G8" s="10">
+      <c r="G8" s="8">
         <v>12.0</v>
       </c>
-      <c r="H8" s="10">
+      <c r="H8" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I8" s="10" t="s">
+      <c r="I8" s="8" t="s">
         <v>49</v>
       </c>
       <c r="J8" s="14">
@@ -8308,7 +8308,7 @@
       <c r="K8" s="14">
         <v>524584.95</v>
       </c>
-      <c r="L8" s="10">
+      <c r="L8" s="8">
         <v>0.0</v>
       </c>
       <c r="O8" s="29"/>
@@ -8321,32 +8321,32 @@
       <c r="AH8" s="2"/>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="s">
+      <c r="A9" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="B9" s="10" t="s">
-        <v>55</v>
-      </c>
-      <c r="C9" s="10" t="s">
+      <c r="B9" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="D9" s="10" t="s">
+      <c r="C9" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D9" s="8" t="s">
         <v>4</v>
       </c>
       <c r="E9" s="12">
         <v>45792.0</v>
       </c>
-      <c r="F9" s="10" t="s">
+      <c r="F9" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G9" s="10">
+      <c r="G9" s="8">
         <v>12.0</v>
       </c>
-      <c r="H9" s="10">
+      <c r="H9" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I9" s="10" t="s">
-        <v>60</v>
+      <c r="I9" s="8" t="s">
+        <v>62</v>
       </c>
       <c r="J9" s="14">
         <v>211614.23</v>
@@ -8354,7 +8354,7 @@
       <c r="K9" s="14">
         <v>211614.23</v>
       </c>
-      <c r="L9" s="10">
+      <c r="L9" s="8">
         <v>0.0</v>
       </c>
       <c r="AB9" s="2"/>
@@ -8366,31 +8366,31 @@
       <c r="AH9" s="2"/>
     </row>
     <row r="10">
-      <c r="A10" s="10" t="s">
-        <v>64</v>
-      </c>
-      <c r="B10" s="10" t="s">
+      <c r="A10" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="B10" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="C10" s="10" t="s">
+      <c r="C10" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="D10" s="10" t="s">
+      <c r="D10" s="8" t="s">
         <v>4</v>
       </c>
       <c r="E10" s="12">
         <v>45825.0</v>
       </c>
-      <c r="F10" s="10" t="s">
+      <c r="F10" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G10" s="10">
+      <c r="G10" s="8">
         <v>12.0</v>
       </c>
-      <c r="H10" s="10">
+      <c r="H10" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I10" s="10">
+      <c r="I10" s="8">
         <v>2048.0</v>
       </c>
       <c r="J10" s="14">
@@ -8411,31 +8411,31 @@
       <c r="AH10" s="2"/>
     </row>
     <row r="11">
-      <c r="A11" s="10" t="s">
+      <c r="A11" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="B11" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="C11" s="10" t="s">
+      <c r="B11" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C11" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="D11" s="10" t="s">
+      <c r="D11" s="8" t="s">
         <v>4</v>
       </c>
       <c r="E11" s="12">
         <v>45825.0</v>
       </c>
-      <c r="F11" s="10" t="s">
+      <c r="F11" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G11" s="10">
+      <c r="G11" s="8">
         <v>12.0</v>
       </c>
-      <c r="H11" s="10">
+      <c r="H11" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I11" s="10">
+      <c r="I11" s="8">
         <v>2048.0</v>
       </c>
       <c r="J11" s="14">
@@ -8444,7 +8444,7 @@
       <c r="K11" s="14">
         <v>618154.38</v>
       </c>
-      <c r="L11" s="10">
+      <c r="L11" s="8">
         <v>0.01</v>
       </c>
       <c r="AB11" s="2"/>
@@ -8456,31 +8456,31 @@
       <c r="AH11" s="2"/>
     </row>
     <row r="12">
-      <c r="A12" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="B12" s="10" t="s">
+      <c r="A12" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="C12" s="10" t="s">
+      <c r="B12" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="D12" s="10" t="s">
+      <c r="C12" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="D12" s="8" t="s">
         <v>4</v>
       </c>
       <c r="E12" s="12">
         <v>45832.0</v>
       </c>
-      <c r="F12" s="10" t="s">
+      <c r="F12" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G12" s="10">
+      <c r="G12" s="8">
         <v>12.0</v>
       </c>
-      <c r="H12" s="10">
+      <c r="H12" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I12" s="10" t="s">
+      <c r="I12" s="8" t="s">
         <v>75</v>
       </c>
       <c r="J12" s="14">
@@ -8489,7 +8489,7 @@
       <c r="K12" s="14">
         <v>1600334.09</v>
       </c>
-      <c r="L12" s="10">
+      <c r="L12" s="8">
         <v>0.0</v>
       </c>
       <c r="AB12" s="2"/>
@@ -8501,31 +8501,31 @@
       <c r="AH12" s="2"/>
     </row>
     <row r="13">
-      <c r="A13" s="10" t="s">
+      <c r="A13" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="B13" s="10" t="s">
+      <c r="B13" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="C13" s="10" t="s">
+      <c r="C13" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="D13" s="10" t="s">
+      <c r="D13" s="8" t="s">
         <v>4</v>
       </c>
       <c r="E13" s="12">
         <v>45863.0</v>
       </c>
-      <c r="F13" s="10" t="s">
+      <c r="F13" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G13" s="10">
+      <c r="G13" s="8">
         <v>12.0</v>
       </c>
-      <c r="H13" s="10">
+      <c r="H13" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I13" s="10">
+      <c r="I13" s="8">
         <v>2048.0</v>
       </c>
       <c r="J13" s="14">
@@ -8547,32 +8547,32 @@
       <c r="AH13" s="2"/>
     </row>
     <row r="14">
-      <c r="A14" s="10" t="s">
+      <c r="A14" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="B14" s="10" t="s">
+      <c r="B14" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="C14" s="10" t="s">
+      <c r="C14" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="D14" s="10" t="s">
+      <c r="D14" s="8" t="s">
         <v>4</v>
       </c>
       <c r="E14" s="12">
         <v>45887.0</v>
       </c>
-      <c r="F14" s="10" t="s">
+      <c r="F14" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G14" s="10">
+      <c r="G14" s="8">
         <v>12.0</v>
       </c>
-      <c r="H14" s="10">
+      <c r="H14" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I14" s="10" t="s">
-        <v>60</v>
+      <c r="I14" s="8" t="s">
+        <v>62</v>
       </c>
       <c r="J14" s="14">
         <v>968237.39</v>
@@ -8580,7 +8580,7 @@
       <c r="K14" s="14">
         <v>968237.39</v>
       </c>
-      <c r="L14" s="10">
+      <c r="L14" s="8">
         <v>0.0</v>
       </c>
       <c r="AB14" s="2"/>
@@ -8592,31 +8592,31 @@
       <c r="AH14" s="2"/>
     </row>
     <row r="15">
-      <c r="A15" s="10" t="s">
-        <v>83</v>
-      </c>
-      <c r="B15" s="10" t="s">
+      <c r="A15" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="C15" s="10" t="s">
+      <c r="B15" s="8" t="s">
         <v>85</v>
       </c>
-      <c r="D15" s="10" t="s">
+      <c r="C15" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="D15" s="8" t="s">
         <v>4</v>
       </c>
       <c r="E15" s="12">
         <v>45924.0</v>
       </c>
-      <c r="F15" s="10" t="s">
+      <c r="F15" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G15" s="10">
+      <c r="G15" s="8">
         <v>12.0</v>
       </c>
-      <c r="H15" s="10">
+      <c r="H15" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I15" s="10" t="s">
+      <c r="I15" s="8" t="s">
         <v>44</v>
       </c>
       <c r="J15" s="14">
@@ -8625,7 +8625,7 @@
       <c r="K15" s="14">
         <v>1011677.95</v>
       </c>
-      <c r="L15" s="10">
+      <c r="L15" s="8">
         <v>0.0</v>
       </c>
       <c r="AB15" s="2"/>
@@ -8637,31 +8637,31 @@
       <c r="AH15" s="2"/>
     </row>
     <row r="16">
-      <c r="A16" s="10" t="s">
+      <c r="A16" s="8" t="s">
         <v>88</v>
       </c>
-      <c r="B16" s="10" t="s">
+      <c r="B16" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="C16" s="10" t="s">
+      <c r="C16" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="D16" s="10" t="s">
+      <c r="D16" s="8" t="s">
         <v>4</v>
       </c>
       <c r="E16" s="12">
         <v>45929.0</v>
       </c>
-      <c r="F16" s="10" t="s">
+      <c r="F16" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G16" s="10">
+      <c r="G16" s="8">
         <v>12.0</v>
       </c>
-      <c r="H16" s="10">
+      <c r="H16" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I16" s="10">
+      <c r="I16" s="8">
         <v>2048.0</v>
       </c>
       <c r="J16" s="14">
@@ -8682,37 +8682,37 @@
       <c r="AH16" s="2"/>
     </row>
     <row r="17">
-      <c r="A17" s="10" t="s">
-        <v>90</v>
-      </c>
-      <c r="B17" s="10" t="s">
-        <v>91</v>
-      </c>
-      <c r="C17" s="10" t="s">
+      <c r="A17" s="8" t="s">
         <v>92</v>
       </c>
-      <c r="D17" s="10" t="s">
+      <c r="B17" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="C17" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="D17" s="8" t="s">
         <v>4</v>
       </c>
       <c r="E17" s="12">
         <v>45930.0</v>
       </c>
-      <c r="F17" s="10" t="s">
+      <c r="F17" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G17" s="10">
+      <c r="G17" s="8">
         <v>12.0</v>
       </c>
-      <c r="H17" s="10">
+      <c r="H17" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I17" s="10">
+      <c r="I17" s="8">
         <v>2048.0</v>
       </c>
       <c r="J17" s="14">
         <v>34065.36</v>
       </c>
-      <c r="K17" s="10">
+      <c r="K17" s="8">
         <v>0.0</v>
       </c>
       <c r="L17" s="14">
@@ -8727,32 +8727,32 @@
       <c r="AH17" s="2"/>
     </row>
     <row r="18">
-      <c r="A18" s="10" t="s">
-        <v>95</v>
-      </c>
-      <c r="B18" s="10" t="s">
+      <c r="A18" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="B18" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="C18" s="10" t="s">
-        <v>97</v>
-      </c>
-      <c r="D18" s="10" t="s">
+      <c r="C18" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="D18" s="8" t="s">
         <v>4</v>
       </c>
       <c r="E18" s="12">
         <v>45938.0</v>
       </c>
-      <c r="F18" s="10" t="s">
+      <c r="F18" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G18" s="10">
+      <c r="G18" s="8">
         <v>12.0</v>
       </c>
-      <c r="H18" s="10">
+      <c r="H18" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I18" s="10" t="s">
-        <v>60</v>
+      <c r="I18" s="8" t="s">
+        <v>62</v>
       </c>
       <c r="J18" s="14">
         <v>63746.85</v>
@@ -8760,7 +8760,7 @@
       <c r="K18" s="14">
         <v>63746.85</v>
       </c>
-      <c r="L18" s="10">
+      <c r="L18" s="8">
         <v>0.0</v>
       </c>
       <c r="AB18" s="2"/>
@@ -8772,31 +8772,31 @@
       <c r="AH18" s="2"/>
     </row>
     <row r="19">
-      <c r="A19" s="10" t="s">
+      <c r="A19" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="B19" s="10" t="s">
-        <v>72</v>
-      </c>
-      <c r="C19" s="10" t="s">
+      <c r="B19" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="C19" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="D19" s="10" t="s">
+      <c r="D19" s="8" t="s">
         <v>4</v>
       </c>
       <c r="E19" s="12">
         <v>45938.0</v>
       </c>
-      <c r="F19" s="10" t="s">
+      <c r="F19" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G19" s="10">
+      <c r="G19" s="8">
         <v>12.0</v>
       </c>
-      <c r="H19" s="10">
+      <c r="H19" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I19" s="10" t="s">
+      <c r="I19" s="8" t="s">
         <v>75</v>
       </c>
       <c r="J19" s="14">
@@ -8805,7 +8805,7 @@
       <c r="K19" s="14">
         <v>947931.1</v>
       </c>
-      <c r="L19" s="10">
+      <c r="L19" s="8">
         <v>0.0</v>
       </c>
       <c r="AB19" s="2"/>
@@ -8817,31 +8817,31 @@
       <c r="AH19" s="2"/>
     </row>
     <row r="20">
-      <c r="A20" s="10" t="s">
+      <c r="A20" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="B20" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="C20" s="8" t="s">
         <v>103</v>
       </c>
-      <c r="B20" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="C20" s="10" t="s">
-        <v>104</v>
-      </c>
-      <c r="D20" s="10" t="s">
+      <c r="D20" s="8" t="s">
         <v>4</v>
       </c>
       <c r="E20" s="12">
         <v>45938.0</v>
       </c>
-      <c r="F20" s="10" t="s">
+      <c r="F20" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G20" s="10">
+      <c r="G20" s="8">
         <v>12.0</v>
       </c>
-      <c r="H20" s="10">
+      <c r="H20" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I20" s="10">
+      <c r="I20" s="8">
         <v>2048.0</v>
       </c>
       <c r="J20" s="14">
@@ -8850,7 +8850,7 @@
       <c r="K20" s="14">
         <v>259790.57</v>
       </c>
-      <c r="L20" s="10">
+      <c r="L20" s="8">
         <v>0.0</v>
       </c>
       <c r="AB20" s="2"/>
@@ -8862,31 +8862,31 @@
       <c r="AH20" s="2"/>
     </row>
     <row r="21">
-      <c r="A21" s="10" t="s">
+      <c r="A21" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="B21" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C21" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="B21" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="C21" s="10" t="s">
-        <v>108</v>
-      </c>
-      <c r="D21" s="10" t="s">
+      <c r="D21" s="8" t="s">
         <v>4</v>
       </c>
       <c r="E21" s="12">
         <v>45938.0</v>
       </c>
-      <c r="F21" s="10" t="s">
+      <c r="F21" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G21" s="10">
+      <c r="G21" s="8">
         <v>12.0</v>
       </c>
-      <c r="H21" s="10">
+      <c r="H21" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I21" s="10">
+      <c r="I21" s="8">
         <v>2048.0</v>
       </c>
       <c r="J21" s="14">
@@ -8895,7 +8895,7 @@
       <c r="K21" s="14">
         <v>170479.3</v>
       </c>
-      <c r="L21" s="10">
+      <c r="L21" s="8">
         <v>0.0</v>
       </c>
       <c r="AB21" s="2"/>
@@ -8907,31 +8907,31 @@
       <c r="AH21" s="2"/>
     </row>
     <row r="22">
-      <c r="A22" s="10" t="s">
+      <c r="A22" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="B22" s="8" t="s">
         <v>110</v>
       </c>
-      <c r="B22" s="10" t="s">
+      <c r="C22" s="8" t="s">
         <v>111</v>
       </c>
-      <c r="C22" s="10" t="s">
-        <v>112</v>
-      </c>
-      <c r="D22" s="10" t="s">
+      <c r="D22" s="8" t="s">
         <v>4</v>
       </c>
       <c r="E22" s="50">
         <v>45953.0</v>
       </c>
-      <c r="F22" s="10" t="s">
+      <c r="F22" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G22" s="10">
+      <c r="G22" s="8">
         <v>12.0</v>
       </c>
-      <c r="H22" s="10">
+      <c r="H22" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I22" s="10">
+      <c r="I22" s="8">
         <v>2000.0</v>
       </c>
       <c r="J22" s="14">
@@ -8952,31 +8952,31 @@
       <c r="AH22" s="2"/>
     </row>
     <row r="23">
-      <c r="A23" s="10" t="s">
+      <c r="A23" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="B23" s="8" t="s">
         <v>115</v>
       </c>
-      <c r="B23" s="10" t="s">
+      <c r="C23" s="8" t="s">
         <v>116</v>
       </c>
-      <c r="C23" s="10" t="s">
-        <v>117</v>
-      </c>
-      <c r="D23" s="10" t="s">
+      <c r="D23" s="8" t="s">
         <v>4</v>
       </c>
       <c r="E23" s="50">
         <v>45953.0</v>
       </c>
-      <c r="F23" s="10" t="s">
+      <c r="F23" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G23" s="10">
+      <c r="G23" s="8">
         <v>12.0</v>
       </c>
-      <c r="H23" s="10">
+      <c r="H23" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I23" s="10" t="s">
+      <c r="I23" s="8" t="s">
         <v>118</v>
       </c>
       <c r="J23" s="14">
@@ -8985,7 +8985,7 @@
       <c r="K23" s="14">
         <v>1000001.64</v>
       </c>
-      <c r="L23" s="10">
+      <c r="L23" s="8">
         <v>0.0</v>
       </c>
       <c r="AB23" s="2"/>
@@ -8997,31 +8997,31 @@
       <c r="AH23" s="2"/>
     </row>
     <row r="24">
-      <c r="A24" s="10" t="s">
+      <c r="A24" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="B24" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C24" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="B24" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="C24" s="10" t="s">
-        <v>122</v>
-      </c>
-      <c r="D24" s="10" t="s">
+      <c r="D24" s="8" t="s">
         <v>4</v>
       </c>
       <c r="E24" s="50">
         <v>45953.0</v>
       </c>
-      <c r="F24" s="10" t="s">
+      <c r="F24" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G24" s="10">
+      <c r="G24" s="8">
         <v>12.0</v>
       </c>
-      <c r="H24" s="10">
+      <c r="H24" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I24" s="10">
+      <c r="I24" s="8">
         <v>2048.0</v>
       </c>
       <c r="J24" s="14">
@@ -9030,7 +9030,7 @@
       <c r="K24" s="14">
         <v>68405.66</v>
       </c>
-      <c r="L24" s="10">
+      <c r="L24" s="8">
         <v>0.0</v>
       </c>
       <c r="AB24" s="2"/>
@@ -9042,31 +9042,31 @@
       <c r="AH24" s="2"/>
     </row>
     <row r="25">
-      <c r="A25" s="10" t="s">
+      <c r="A25" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="B25" s="8" t="s">
+        <v>124</v>
+      </c>
+      <c r="C25" s="8" t="s">
         <v>125</v>
       </c>
-      <c r="B25" s="10" t="s">
-        <v>126</v>
-      </c>
-      <c r="C25" s="10" t="s">
-        <v>127</v>
-      </c>
-      <c r="D25" s="10" t="s">
+      <c r="D25" s="8" t="s">
         <v>4</v>
       </c>
       <c r="E25" s="50">
         <v>45975.0</v>
       </c>
-      <c r="F25" s="10" t="s">
+      <c r="F25" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G25" s="10">
+      <c r="G25" s="8">
         <v>12.0</v>
       </c>
-      <c r="H25" s="10">
+      <c r="H25" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I25" s="10" t="s">
+      <c r="I25" s="8" t="s">
         <v>118</v>
       </c>
       <c r="J25" s="14">
@@ -9075,7 +9075,7 @@
       <c r="K25" s="14">
         <v>1157673.06</v>
       </c>
-      <c r="L25" s="10">
+      <c r="L25" s="8">
         <v>0.0</v>
       </c>
       <c r="AB25" s="2"/>
@@ -9087,31 +9087,31 @@
       <c r="AH25" s="2"/>
     </row>
     <row r="26">
-      <c r="A26" s="10" t="s">
-        <v>130</v>
-      </c>
-      <c r="B26" s="10" t="s">
+      <c r="A26" s="8" t="s">
+        <v>128</v>
+      </c>
+      <c r="B26" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="C26" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="D26" s="10" t="s">
+      <c r="C26" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="D26" s="8" t="s">
         <v>4</v>
       </c>
       <c r="E26" s="50">
         <v>45989.0</v>
       </c>
-      <c r="F26" s="10" t="s">
+      <c r="F26" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G26" s="10">
+      <c r="G26" s="8">
         <v>12.0</v>
       </c>
-      <c r="H26" s="10">
+      <c r="H26" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I26" s="10">
+      <c r="I26" s="8">
         <v>2048.0</v>
       </c>
       <c r="J26" s="14">
@@ -9120,7 +9120,7 @@
       <c r="K26" s="14">
         <v>34065.36</v>
       </c>
-      <c r="L26" s="10">
+      <c r="L26" s="8">
         <v>0.0</v>
       </c>
       <c r="AB26" s="2"/>
@@ -9132,31 +9132,31 @@
       <c r="AH26" s="2"/>
     </row>
     <row r="27">
-      <c r="A27" s="10" t="s">
+      <c r="A27" s="8" t="s">
+        <v>133</v>
+      </c>
+      <c r="B27" s="8" t="s">
         <v>134</v>
       </c>
-      <c r="B27" s="10" t="s">
+      <c r="C27" s="8" t="s">
         <v>135</v>
       </c>
-      <c r="C27" s="10" t="s">
-        <v>136</v>
-      </c>
-      <c r="D27" s="10" t="s">
+      <c r="D27" s="8" t="s">
         <v>4</v>
       </c>
       <c r="E27" s="12">
         <v>46104.0</v>
       </c>
-      <c r="F27" s="10" t="s">
+      <c r="F27" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G27" s="10">
+      <c r="G27" s="8">
         <v>12.0</v>
       </c>
-      <c r="H27" s="10">
+      <c r="H27" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I27" s="10">
+      <c r="I27" s="8">
         <v>2048.0</v>
       </c>
       <c r="J27" s="14">
@@ -9177,37 +9177,37 @@
       <c r="AH27" s="2"/>
     </row>
     <row r="28">
-      <c r="A28" s="10" t="s">
-        <v>139</v>
-      </c>
-      <c r="B28" s="10" t="s">
+      <c r="A28" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="B28" s="8" t="s">
         <v>140</v>
       </c>
-      <c r="C28" s="10" t="s">
+      <c r="C28" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="D28" s="10" t="s">
+      <c r="D28" s="8" t="s">
         <v>4</v>
       </c>
       <c r="E28" s="12">
         <v>46120.0</v>
       </c>
-      <c r="F28" s="10" t="s">
+      <c r="F28" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G28" s="10">
+      <c r="G28" s="8">
         <v>12.0</v>
       </c>
-      <c r="H28" s="10">
+      <c r="H28" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I28" s="10" t="s">
+      <c r="I28" s="8" t="s">
         <v>49</v>
       </c>
       <c r="J28" s="14">
         <v>1912292.52</v>
       </c>
-      <c r="K28" s="10">
+      <c r="K28" s="8">
         <v>0.0</v>
       </c>
       <c r="L28" s="14">
@@ -9222,37 +9222,37 @@
       <c r="AH28" s="2"/>
     </row>
     <row r="29">
-      <c r="A29" s="10" t="s">
+      <c r="A29" s="8" t="s">
         <v>144</v>
       </c>
-      <c r="B29" s="10" t="s">
+      <c r="B29" s="8" t="s">
         <v>145</v>
       </c>
-      <c r="C29" s="10" t="s">
+      <c r="C29" s="8" t="s">
         <v>146</v>
       </c>
-      <c r="D29" s="10" t="s">
+      <c r="D29" s="8" t="s">
         <v>4</v>
       </c>
       <c r="E29" s="12">
         <v>46196.0</v>
       </c>
-      <c r="F29" s="10" t="s">
+      <c r="F29" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G29" s="10">
+      <c r="G29" s="8">
         <v>12.0</v>
       </c>
-      <c r="H29" s="10">
+      <c r="H29" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I29" s="10">
+      <c r="I29" s="8">
         <v>2048.0</v>
       </c>
       <c r="J29" s="14">
         <v>1496713.48</v>
       </c>
-      <c r="K29" s="10">
+      <c r="K29" s="8">
         <v>0.0</v>
       </c>
       <c r="L29" s="14">
@@ -9267,37 +9267,37 @@
       <c r="AH29" s="2"/>
     </row>
     <row r="30">
-      <c r="A30" s="10" t="s">
-        <v>149</v>
-      </c>
-      <c r="B30" s="10" t="s">
+      <c r="A30" s="8" t="s">
         <v>150</v>
       </c>
-      <c r="C30" s="10" t="s">
+      <c r="B30" s="8" t="s">
         <v>151</v>
       </c>
-      <c r="D30" s="10" t="s">
+      <c r="C30" s="8" t="s">
+        <v>152</v>
+      </c>
+      <c r="D30" s="8" t="s">
         <v>4</v>
       </c>
       <c r="E30" s="12">
         <v>46205.0</v>
       </c>
-      <c r="F30" s="10" t="s">
+      <c r="F30" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G30" s="10">
+      <c r="G30" s="8">
         <v>12.0</v>
       </c>
-      <c r="H30" s="10">
+      <c r="H30" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I30" s="10" t="s">
+      <c r="I30" s="8" t="s">
         <v>44</v>
       </c>
       <c r="J30" s="14">
         <v>624166.14</v>
       </c>
-      <c r="K30" s="10">
+      <c r="K30" s="8">
         <v>0.0</v>
       </c>
       <c r="L30" s="14">
@@ -9312,37 +9312,37 @@
       <c r="AH30" s="2"/>
     </row>
     <row r="31">
-      <c r="A31" s="10" t="s">
-        <v>153</v>
-      </c>
-      <c r="B31" s="10" t="s">
-        <v>154</v>
-      </c>
-      <c r="C31" s="10" t="s">
+      <c r="A31" s="8" t="s">
+        <v>155</v>
+      </c>
+      <c r="B31" s="8" t="s">
         <v>156</v>
       </c>
-      <c r="D31" s="10" t="s">
+      <c r="C31" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="D31" s="8" t="s">
         <v>4</v>
       </c>
       <c r="E31" s="12">
         <v>46205.0</v>
       </c>
-      <c r="F31" s="10" t="s">
+      <c r="F31" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G31" s="10">
+      <c r="G31" s="8">
         <v>12.0</v>
       </c>
-      <c r="H31" s="10">
+      <c r="H31" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I31" s="10" t="s">
+      <c r="I31" s="8" t="s">
         <v>118</v>
       </c>
       <c r="J31" s="14">
         <v>18462.36</v>
       </c>
-      <c r="K31" s="10">
+      <c r="K31" s="8">
         <v>0.0</v>
       </c>
       <c r="L31" s="14">
@@ -9357,37 +9357,37 @@
       <c r="AH31" s="2"/>
     </row>
     <row r="32">
-      <c r="A32" s="10" t="s">
-        <v>158</v>
-      </c>
-      <c r="B32" s="10" t="s">
-        <v>154</v>
+      <c r="A32" s="8" t="s">
+        <v>160</v>
+      </c>
+      <c r="B32" s="8" t="s">
+        <v>156</v>
       </c>
       <c r="C32" s="14" t="s">
-        <v>159</v>
-      </c>
-      <c r="D32" s="10" t="s">
+        <v>161</v>
+      </c>
+      <c r="D32" s="8" t="s">
         <v>4</v>
       </c>
       <c r="E32" s="12">
         <v>46213.0</v>
       </c>
-      <c r="F32" s="10" t="s">
+      <c r="F32" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G32" s="10">
+      <c r="G32" s="8">
         <v>12.0</v>
       </c>
-      <c r="H32" s="10">
+      <c r="H32" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I32" s="10" t="s">
+      <c r="I32" s="8" t="s">
         <v>118</v>
       </c>
       <c r="J32" s="14">
         <v>1530656.62</v>
       </c>
-      <c r="K32" s="10">
+      <c r="K32" s="8">
         <v>0.0</v>
       </c>
       <c r="L32" s="14">
@@ -9402,37 +9402,37 @@
       <c r="AH32" s="2"/>
     </row>
     <row r="33">
-      <c r="A33" s="10" t="s">
-        <v>161</v>
-      </c>
-      <c r="B33" s="10" t="s">
+      <c r="A33" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="B33" s="8" t="s">
         <v>145</v>
       </c>
       <c r="C33" s="14" t="s">
-        <v>163</v>
-      </c>
-      <c r="D33" s="10" t="s">
+        <v>167</v>
+      </c>
+      <c r="D33" s="8" t="s">
         <v>4</v>
       </c>
       <c r="E33" s="12">
         <v>46227.0</v>
       </c>
-      <c r="F33" s="10" t="s">
+      <c r="F33" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G33" s="10">
+      <c r="G33" s="8">
         <v>12.0</v>
       </c>
-      <c r="H33" s="10">
+      <c r="H33" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I33" s="10">
+      <c r="I33" s="8">
         <v>2048.0</v>
       </c>
       <c r="J33" s="14">
         <v>173846.38</v>
       </c>
-      <c r="K33" s="10">
+      <c r="K33" s="8">
         <v>0.0</v>
       </c>
       <c r="L33" s="14">
@@ -9447,37 +9447,37 @@
       <c r="AH33" s="2"/>
     </row>
     <row r="34">
-      <c r="A34" s="10" t="s">
-        <v>165</v>
-      </c>
-      <c r="B34" s="10" t="s">
-        <v>166</v>
-      </c>
-      <c r="C34" s="10" t="s">
-        <v>167</v>
-      </c>
-      <c r="D34" s="10" t="s">
+      <c r="A34" s="8" t="s">
+        <v>170</v>
+      </c>
+      <c r="B34" s="8" t="s">
+        <v>171</v>
+      </c>
+      <c r="C34" s="8" t="s">
+        <v>172</v>
+      </c>
+      <c r="D34" s="8" t="s">
         <v>4</v>
       </c>
       <c r="E34" s="12">
         <v>46240.0</v>
       </c>
-      <c r="F34" s="10" t="s">
+      <c r="F34" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G34" s="10">
+      <c r="G34" s="8">
         <v>12.0</v>
       </c>
-      <c r="H34" s="10">
+      <c r="H34" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I34" s="10" t="s">
-        <v>168</v>
+      <c r="I34" s="8" t="s">
+        <v>173</v>
       </c>
       <c r="J34" s="14">
         <v>236343.68</v>
       </c>
-      <c r="K34" s="10">
+      <c r="K34" s="8">
         <v>0.0</v>
       </c>
       <c r="L34" s="14">

</xml_diff>

<commit_message>
Atualização automática: pagamentos (13/08/2026 18:56)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/01_Bases_Originais/005_CELOG_2025/005_CELOG-PAMALS_2025 online.xlsx
+++ b/Contrato 005/Dashboard/01_Bases_Originais/005_CELOG_2025/005_CELOG-PAMALS_2025 online.xlsx
@@ -30,12 +30,12 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="341" uniqueCount="216">
   <si>
+    <t>Controle de pagamentos</t>
+  </si>
+  <si>
     <t>Saldo</t>
   </si>
   <si>
-    <t>Controle de pagamentos</t>
-  </si>
-  <si>
     <t>2025NE000005</t>
   </si>
   <si>
@@ -108,27 +108,27 @@
     <t>Valor Liquidado</t>
   </si>
   <si>
+    <t>Saldo (Valor a Faturar)</t>
+  </si>
+  <si>
+    <t>Fornecedor</t>
+  </si>
+  <si>
+    <t>Tipo Despesa /Receita</t>
+  </si>
+  <si>
+    <t>Abrir</t>
+  </si>
+  <si>
+    <t>Editar</t>
+  </si>
+  <si>
     <t>2025NE000371</t>
   </si>
   <si>
-    <t>Saldo (Valor a Faturar)</t>
-  </si>
-  <si>
-    <t>Fornecedor</t>
-  </si>
-  <si>
     <t>25E0389</t>
   </si>
   <si>
-    <t>Tipo Despesa /Receita</t>
-  </si>
-  <si>
-    <t>Abrir</t>
-  </si>
-  <si>
-    <t>Editar</t>
-  </si>
-  <si>
     <t>005/CELOG-PAMALS/2025</t>
   </si>
   <si>
@@ -138,27 +138,27 @@
     <t>PAMALS</t>
   </si>
   <si>
+    <t>Vigente</t>
+  </si>
+  <si>
+    <t>2048 20YJ 21EM 219C 20SP 20X7 2000</t>
+  </si>
+  <si>
+    <t>67101.001510/2024-12</t>
+  </si>
+  <si>
+    <t>R$</t>
+  </si>
+  <si>
     <t>2025NE000413</t>
   </si>
   <si>
     <t>C25501</t>
   </si>
   <si>
-    <t>Vigente</t>
-  </si>
-  <si>
     <t>25E0403</t>
   </si>
   <si>
-    <t>2048 20YJ 21EM 219C 20SP 20X7 2000</t>
-  </si>
-  <si>
-    <t>67101.001510/2024-12</t>
-  </si>
-  <si>
-    <t>R$</t>
-  </si>
-  <si>
     <t>20SP</t>
   </si>
   <si>
@@ -180,13 +180,22 @@
     <t>2025NE000559</t>
   </si>
   <si>
+    <t>C25545</t>
+  </si>
+  <si>
+    <t>25E0524</t>
+  </si>
+  <si>
+    <t>20X7</t>
+  </si>
+  <si>
     <t>Módulo</t>
   </si>
   <si>
-    <t>C25545</t>
-  </si>
-  <si>
-    <t>25E0524</t>
+    <t>2025NE000770</t>
+  </si>
+  <si>
+    <t>25E0731</t>
   </si>
   <si>
     <t>Referência</t>
@@ -195,12 +204,15 @@
     <t>Nº recibo</t>
   </si>
   <si>
-    <t>20X7</t>
-  </si>
-  <si>
     <t>Nº</t>
   </si>
   <si>
+    <t>2025NE000774</t>
+  </si>
+  <si>
+    <t>25E0737</t>
+  </si>
+  <si>
     <t>Data</t>
   </si>
   <si>
@@ -213,16 +225,22 @@
     <t>Vencimento</t>
   </si>
   <si>
+    <t>2025NE000843</t>
+  </si>
+  <si>
     <t>Valor das Nfs</t>
   </si>
   <si>
+    <t>C25630</t>
+  </si>
+  <si>
+    <t>25E0787</t>
+  </si>
+  <si>
     <t>Ordem de Pagamento</t>
   </si>
   <si>
-    <t>2025NE000770</t>
-  </si>
-  <si>
-    <t>25E0731</t>
+    <t>219C</t>
   </si>
   <si>
     <t>Faturado</t>
@@ -231,118 +249,145 @@
     <t>Pendente</t>
   </si>
   <si>
-    <t>2025NE000774</t>
-  </si>
-  <si>
-    <t>25E0737</t>
+    <t>2025NE001065</t>
+  </si>
+  <si>
+    <t>25E0999</t>
+  </si>
+  <si>
+    <t>2025NE001200</t>
   </si>
   <si>
     <t>FEV/25</t>
   </si>
   <si>
+    <t>C25590</t>
+  </si>
+  <si>
+    <t>25E1128</t>
+  </si>
+  <si>
     <t>-</t>
   </si>
   <si>
-    <t>2025NE000843</t>
-  </si>
-  <si>
-    <t>C25630</t>
-  </si>
-  <si>
     <t xml:space="preserve">2025NE000369 </t>
   </si>
   <si>
-    <t>25E0787</t>
-  </si>
-  <si>
-    <t>219C</t>
+    <t>2025NE001598</t>
+  </si>
+  <si>
+    <t>C25814</t>
+  </si>
+  <si>
+    <t>25E1446</t>
   </si>
   <si>
     <t>2025NP001980</t>
   </si>
   <si>
-    <t>2025NE001065</t>
-  </si>
-  <si>
-    <t>25E0999</t>
-  </si>
-  <si>
-    <t>2025NE001200</t>
-  </si>
-  <si>
-    <t>C25590</t>
-  </si>
-  <si>
-    <t>25E1128</t>
+    <t>2025NE001627</t>
+  </si>
+  <si>
+    <t>25E1475</t>
+  </si>
+  <si>
+    <t>2025NE001629</t>
+  </si>
+  <si>
+    <t>C25820</t>
+  </si>
+  <si>
+    <t>25E1477</t>
+  </si>
+  <si>
+    <t>2025NE001687</t>
+  </si>
+  <si>
+    <t>25E1535</t>
   </si>
   <si>
     <t>MAR/25</t>
   </si>
   <si>
+    <t>2025NE001688</t>
+  </si>
+  <si>
+    <t>25E1536</t>
+  </si>
+  <si>
     <t>2025NE000367, 2025NE000369, 2025NE000371, 2025NE000413</t>
   </si>
   <si>
-    <t>2025NE001598</t>
-  </si>
-  <si>
-    <t>C25814</t>
-  </si>
-  <si>
-    <t>25E1446</t>
+    <t>2025NE001689</t>
+  </si>
+  <si>
+    <t>25E1537</t>
   </si>
   <si>
     <t>2025NP001979</t>
   </si>
   <si>
-    <t>2025NE001627</t>
+    <t>2025NE001690</t>
+  </si>
+  <si>
+    <t>25E1538</t>
   </si>
   <si>
     <t>ABR/25</t>
   </si>
   <si>
-    <t>25E1475</t>
+    <t>2025NE001823</t>
+  </si>
+  <si>
+    <t>C25865</t>
   </si>
   <si>
     <t>2025NE000413, 2025NE000414, 2025NE000559</t>
   </si>
   <si>
+    <t>25E1666</t>
+  </si>
+  <si>
     <t>2025NP002341</t>
   </si>
   <si>
-    <t>2025NE001629</t>
-  </si>
-  <si>
-    <t>C25820</t>
-  </si>
-  <si>
-    <t>25E1477</t>
+    <t>2025NE001828</t>
+  </si>
+  <si>
+    <t>C25869</t>
+  </si>
+  <si>
+    <t>25E1667</t>
   </si>
   <si>
     <t>MAI/25</t>
   </si>
   <si>
-    <t>2025NE001687</t>
-  </si>
-  <si>
-    <t>25E1535</t>
+    <t>20YJ</t>
+  </si>
+  <si>
+    <t>2025NE001830</t>
+  </si>
+  <si>
+    <t>25E1669</t>
   </si>
   <si>
     <t>2025NP002884</t>
   </si>
   <si>
-    <t>2025NE001688</t>
-  </si>
-  <si>
-    <t>25E1536</t>
+    <t>2025NE002200</t>
+  </si>
+  <si>
+    <t>C25863</t>
+  </si>
+  <si>
+    <t>25E2021</t>
   </si>
   <si>
     <t>JUN/25</t>
   </si>
   <si>
-    <t>2025NE001689</t>
-  </si>
-  <si>
-    <t>25E1537</t>
+    <t>2025NE002237</t>
   </si>
   <si>
     <t>2025NE000005,
@@ -351,13 +396,19 @@
 2025NE000774</t>
   </si>
   <si>
+    <t>25E2058</t>
+  </si>
+  <si>
     <t>2025NP400522</t>
   </si>
   <si>
-    <t>2025NE001690</t>
-  </si>
-  <si>
-    <t>25E1538</t>
+    <t>2026NE000330</t>
+  </si>
+  <si>
+    <t>C26163</t>
+  </si>
+  <si>
+    <t>26E0320</t>
   </si>
   <si>
     <t>JUL/25</t>
@@ -369,98 +420,98 @@
     <t>2025NP003724</t>
   </si>
   <si>
-    <t>2025NE001823</t>
-  </si>
-  <si>
-    <t>C25865</t>
-  </si>
-  <si>
-    <t>25E1666</t>
+    <t>2026NE000388</t>
+  </si>
+  <si>
+    <t>C26193</t>
+  </si>
+  <si>
+    <t>26E0375</t>
   </si>
   <si>
     <t>AGO/25</t>
   </si>
   <si>
+    <t>2026NE000748</t>
+  </si>
+  <si>
+    <t>C26312</t>
+  </si>
+  <si>
+    <t>26E0709</t>
+  </si>
+  <si>
     <t>2025NP004558</t>
   </si>
   <si>
-    <t>2025NE001828</t>
-  </si>
-  <si>
-    <t>C25869</t>
-  </si>
-  <si>
-    <t>25E1667</t>
-  </si>
-  <si>
-    <t>20YJ</t>
+    <t>2026NE000816</t>
   </si>
   <si>
     <t>SET/25</t>
+  </si>
+  <si>
+    <t>C26324</t>
+  </si>
+  <si>
+    <t>26E0776</t>
   </si>
   <si>
     <t>2025NE001688 
 2025NE001828</t>
   </si>
   <si>
-    <t>2025NE001830</t>
-  </si>
-  <si>
-    <t>25E1669</t>
-  </si>
-  <si>
     <t>2025NP004897</t>
   </si>
   <si>
+    <t>2026NE000817</t>
+  </si>
+  <si>
+    <t>C26326</t>
+  </si>
+  <si>
+    <t>26E0777</t>
+  </si>
+  <si>
     <t>OUT/25</t>
   </si>
   <si>
-    <t>2025NE002200</t>
-  </si>
-  <si>
-    <t>C25863</t>
-  </si>
-  <si>
-    <t>25E2021</t>
-  </si>
-  <si>
     <t>2025NE001688, 2025NE001828, 2025NE002200</t>
   </si>
   <si>
+    <t>2026NE000842</t>
+  </si>
+  <si>
+    <t>26E0803</t>
+  </si>
+  <si>
     <t>2025NP004932</t>
   </si>
   <si>
-    <t>2025NE002237</t>
+    <t>2026NE000944</t>
   </si>
   <si>
     <t>NOV/25</t>
   </si>
   <si>
-    <t>25E2058</t>
-  </si>
-  <si>
-    <t>2026NE000330</t>
+    <t>26E0906</t>
   </si>
   <si>
     <t>2025NE001687, 2025NE001689, 2025NE001690, 2025NE001823, 2025NE001830, 2025NE002237</t>
   </si>
   <si>
-    <t>C26163</t>
-  </si>
-  <si>
-    <t>26E0320</t>
-  </si>
-  <si>
     <t>2026NP400440</t>
   </si>
   <si>
-    <t>2026NE000388</t>
-  </si>
-  <si>
-    <t>C26193</t>
-  </si>
-  <si>
-    <t>26E0375</t>
+    <t>2026NE001015</t>
+  </si>
+  <si>
+    <t>C26363</t>
+  </si>
+  <si>
+    <t>26E0959</t>
+  </si>
+  <si>
+    <t>20XV</t>
   </si>
   <si>
     <t>DEZ/25</t>
@@ -469,76 +520,25 @@
     <t>2025NE001065, 2025NE002200</t>
   </si>
   <si>
-    <t>2026NE000748</t>
-  </si>
-  <si>
-    <t>C26312</t>
-  </si>
-  <si>
-    <t>26E0709</t>
-  </si>
-  <si>
     <t>2026NP400412</t>
   </si>
   <si>
-    <t>2026NE000816</t>
-  </si>
-  <si>
-    <t>C26324</t>
-  </si>
-  <si>
-    <t>26E0776</t>
-  </si>
-  <si>
     <t>JAN/26</t>
   </si>
   <si>
-    <t>2026NE000817</t>
-  </si>
-  <si>
-    <t>C26326</t>
-  </si>
-  <si>
-    <t>26E0777</t>
-  </si>
-  <si>
     <t>2026NP401035</t>
   </si>
   <si>
-    <t>2026NE000842</t>
-  </si>
-  <si>
     <t>FEV/26</t>
   </si>
   <si>
-    <t>26E0803</t>
-  </si>
-  <si>
     <t>2025NE001627, 2025NE001629, 2025NE001823</t>
   </si>
   <si>
-    <t>2026NE000944</t>
-  </si>
-  <si>
     <t>2026NP402272</t>
   </si>
   <si>
-    <t>26E0906</t>
-  </si>
-  <si>
-    <t>2026NE001015</t>
-  </si>
-  <si>
-    <t>C26363</t>
-  </si>
-  <si>
     <t>MAR/26</t>
-  </si>
-  <si>
-    <t>26E0959</t>
-  </si>
-  <si>
-    <t>20XV</t>
   </si>
   <si>
     <t>2025NE000770, 2025NE001627</t>
@@ -692,8 +692,8 @@
     <numFmt numFmtId="166" formatCode="dd/MM/yyyy"/>
     <numFmt numFmtId="167" formatCode="R$ #,##0.00"/>
     <numFmt numFmtId="168" formatCode="[$R$-416]\ #,##0.00;[RED]\-[$R$-416]\ #,##0.00"/>
-    <numFmt numFmtId="169" formatCode="MM/DD/YY"/>
-    <numFmt numFmtId="170" formatCode="d/m/yyyy"/>
+    <numFmt numFmtId="169" formatCode="d/m/yyyy"/>
+    <numFmt numFmtId="170" formatCode="MM/DD/YY"/>
     <numFmt numFmtId="171" formatCode="[$R$ -416]#,##0.00"/>
     <numFmt numFmtId="172" formatCode="_([$R$ -416]* #,##0.00_);_([$R$ -416]* \(#,##0.00\);_([$R$ -416]* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
@@ -889,20 +889,17 @@
     </xf>
     <xf borderId="0" fillId="3" fontId="2" numFmtId="0" xfId="0" applyFill="1" applyFont="1"/>
     <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyFill="1" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0"/>
-    </xf>
     <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="5" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
+      <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="center"/>
@@ -910,13 +907,16 @@
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="11" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="4" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
@@ -953,11 +953,11 @@
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
+    <xf borderId="1" fillId="0" fontId="6" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="6" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment vertical="center"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="0"/>
@@ -971,6 +971,7 @@
     <xf borderId="1" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="165" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="2" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
@@ -992,7 +993,6 @@
     <xf borderId="1" fillId="5" fontId="9" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="165" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="1" fillId="8" fontId="7" numFmtId="168" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
@@ -1000,10 +1000,13 @@
     <xf borderId="1" fillId="8" fontId="9" numFmtId="168" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="169" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
     <xf borderId="1" fillId="0" fontId="8" numFmtId="166" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="8" numFmtId="169" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="8" numFmtId="170" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="7" fontId="9" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
@@ -1020,9 +1023,6 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="170" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="1" fillId="9" fontId="9" numFmtId="168" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
@@ -1443,42 +1443,42 @@
       <c r="V1" s="3"/>
     </row>
     <row r="2" ht="59.25" customHeight="1">
-      <c r="A2" s="5"/>
-      <c r="B2" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="V2" s="9"/>
-      <c r="W2" s="10"/>
-      <c r="X2" s="10"/>
-      <c r="Y2" s="10"/>
-      <c r="Z2" s="10"/>
-      <c r="AA2" s="10"/>
-      <c r="AB2" s="10"/>
-      <c r="AC2" s="10"/>
-      <c r="AD2" s="10"/>
+      <c r="A2" s="4"/>
+      <c r="B2" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="V2" s="8"/>
+      <c r="W2" s="9"/>
+      <c r="X2" s="9"/>
+      <c r="Y2" s="9"/>
+      <c r="Z2" s="9"/>
+      <c r="AA2" s="9"/>
+      <c r="AB2" s="9"/>
+      <c r="AC2" s="9"/>
+      <c r="AD2" s="9"/>
     </row>
     <row r="3" ht="12.75" customHeight="1">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
-      <c r="E3" s="13"/>
-      <c r="F3" s="13"/>
-      <c r="G3" s="13"/>
-      <c r="H3" s="13"/>
-      <c r="I3" s="13"/>
-      <c r="J3" s="13"/>
-      <c r="K3" s="13"/>
-      <c r="L3" s="13"/>
-      <c r="M3" s="13"/>
-      <c r="N3" s="13"/>
-      <c r="O3" s="13"/>
-      <c r="P3" s="13"/>
-      <c r="Q3" s="13"/>
-      <c r="R3" s="13"/>
-      <c r="S3" s="13"/>
-      <c r="T3" s="13"/>
-      <c r="U3" s="13"/>
+      <c r="C3" s="11"/>
+      <c r="D3" s="11"/>
+      <c r="E3" s="11"/>
+      <c r="F3" s="11"/>
+      <c r="G3" s="11"/>
+      <c r="H3" s="11"/>
+      <c r="I3" s="11"/>
+      <c r="J3" s="11"/>
+      <c r="K3" s="11"/>
+      <c r="L3" s="11"/>
+      <c r="M3" s="11"/>
+      <c r="N3" s="11"/>
+      <c r="O3" s="11"/>
+      <c r="P3" s="11"/>
+      <c r="Q3" s="11"/>
+      <c r="R3" s="11"/>
+      <c r="S3" s="11"/>
+      <c r="T3" s="11"/>
+      <c r="U3" s="11"/>
       <c r="V3" s="3"/>
     </row>
     <row r="4" ht="12.75" customHeight="1">
@@ -1527,19 +1527,19 @@
         <v>25</v>
       </c>
       <c r="Q4" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="R4" s="16" t="s">
         <v>27</v>
       </c>
-      <c r="R4" s="16" t="s">
+      <c r="S4" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="S4" s="16" t="s">
+      <c r="T4" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="U4" s="16" t="s">
         <v>30</v>
-      </c>
-      <c r="T4" s="16" t="s">
-        <v>31</v>
-      </c>
-      <c r="U4" s="16" t="s">
-        <v>32</v>
       </c>
       <c r="V4" s="3"/>
     </row>
@@ -1566,16 +1566,16 @@
         <v>1564.0</v>
       </c>
       <c r="J5" s="19" t="s">
+        <v>36</v>
+      </c>
+      <c r="K5" s="19" t="s">
+        <v>37</v>
+      </c>
+      <c r="L5" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="K5" s="19" t="s">
-        <v>40</v>
-      </c>
-      <c r="L5" s="19" t="s">
-        <v>41</v>
-      </c>
       <c r="M5" s="19" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="N5" s="21">
         <v>9.165159737E7</v>
@@ -1615,7 +1615,7 @@
       <c r="I7" s="25"/>
       <c r="J7" s="25"/>
       <c r="K7" s="25"/>
-      <c r="L7" s="26"/>
+      <c r="L7" s="27"/>
       <c r="M7" s="25"/>
       <c r="N7" s="25"/>
       <c r="O7" s="25"/>
@@ -1626,40 +1626,40 @@
       <c r="A8" s="23"/>
       <c r="B8" s="23"/>
       <c r="C8" s="29" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="D8" s="29" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="E8" s="30" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="F8" s="29" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="G8" s="29" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="H8" s="29" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="I8" s="30" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="J8" s="29" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="K8" s="29" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="L8" s="31" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="M8" s="30" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="N8" s="29" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="O8" s="29"/>
       <c r="P8" s="28"/>
@@ -1668,35 +1668,35 @@
     <row r="9" ht="19.5" customHeight="1">
       <c r="A9" s="23"/>
       <c r="B9" s="23"/>
-      <c r="C9" s="32">
+      <c r="C9" s="33">
         <v>1.0</v>
       </c>
-      <c r="D9" s="33" t="s">
-        <v>69</v>
-      </c>
-      <c r="E9" s="34" t="s">
-        <v>70</v>
-      </c>
-      <c r="F9" s="35">
+      <c r="D9" s="34" t="s">
+        <v>76</v>
+      </c>
+      <c r="E9" s="35" t="s">
+        <v>79</v>
+      </c>
+      <c r="F9" s="36">
         <v>594.0</v>
       </c>
-      <c r="G9" s="36">
+      <c r="G9" s="37">
         <v>45740.0</v>
       </c>
-      <c r="H9" s="35" t="s">
-        <v>73</v>
-      </c>
-      <c r="I9" s="36"/>
-      <c r="J9" s="36">
+      <c r="H9" s="36" t="s">
+        <v>80</v>
+      </c>
+      <c r="I9" s="37"/>
+      <c r="J9" s="37">
         <v>45778.0</v>
       </c>
-      <c r="K9" s="37">
+      <c r="K9" s="38">
         <v>748504.24</v>
       </c>
-      <c r="L9" s="35" t="s">
-        <v>76</v>
-      </c>
-      <c r="M9" s="38">
+      <c r="L9" s="36" t="s">
+        <v>84</v>
+      </c>
+      <c r="M9" s="39">
         <f t="shared" ref="M9:M10" si="1">K9</f>
         <v>748504.24</v>
       </c>
@@ -1709,32 +1709,32 @@
       <c r="A10" s="23"/>
       <c r="B10" s="23"/>
       <c r="C10" s="41"/>
-      <c r="D10" s="33" t="s">
-        <v>82</v>
-      </c>
-      <c r="E10" s="34" t="s">
-        <v>70</v>
-      </c>
-      <c r="F10" s="35">
+      <c r="D10" s="34" t="s">
+        <v>92</v>
+      </c>
+      <c r="E10" s="35" t="s">
+        <v>79</v>
+      </c>
+      <c r="F10" s="36">
         <v>620.0</v>
       </c>
-      <c r="G10" s="36">
+      <c r="G10" s="37">
         <v>45775.0</v>
       </c>
-      <c r="H10" s="35" t="s">
-        <v>83</v>
-      </c>
-      <c r="I10" s="36"/>
-      <c r="J10" s="36">
+      <c r="H10" s="36" t="s">
+        <v>95</v>
+      </c>
+      <c r="I10" s="37"/>
+      <c r="J10" s="37">
         <v>45806.0</v>
       </c>
-      <c r="K10" s="37">
+      <c r="K10" s="38">
         <v>1110378.24</v>
       </c>
-      <c r="L10" s="35" t="s">
-        <v>87</v>
-      </c>
-      <c r="M10" s="38">
+      <c r="L10" s="36" t="s">
+        <v>98</v>
+      </c>
+      <c r="M10" s="39">
         <f t="shared" si="1"/>
         <v>1110378.24</v>
       </c>
@@ -1747,32 +1747,32 @@
       <c r="A11" s="23"/>
       <c r="B11" s="23"/>
       <c r="C11" s="41"/>
-      <c r="D11" s="33" t="s">
-        <v>89</v>
-      </c>
-      <c r="E11" s="34" t="s">
-        <v>70</v>
-      </c>
-      <c r="F11" s="35">
+      <c r="D11" s="34" t="s">
+        <v>101</v>
+      </c>
+      <c r="E11" s="35" t="s">
+        <v>79</v>
+      </c>
+      <c r="F11" s="36">
         <v>634.0</v>
       </c>
-      <c r="G11" s="36">
+      <c r="G11" s="37">
         <v>45799.0</v>
       </c>
-      <c r="H11" s="35" t="s">
-        <v>91</v>
-      </c>
-      <c r="I11" s="36"/>
-      <c r="J11" s="36">
+      <c r="H11" s="36" t="s">
+        <v>104</v>
+      </c>
+      <c r="I11" s="37"/>
+      <c r="J11" s="37">
         <v>45844.0</v>
       </c>
-      <c r="K11" s="37">
+      <c r="K11" s="38">
         <v>974557.12</v>
       </c>
-      <c r="L11" s="34" t="s">
-        <v>92</v>
-      </c>
-      <c r="M11" s="38">
+      <c r="L11" s="35" t="s">
+        <v>106</v>
+      </c>
+      <c r="M11" s="39">
         <v>974557.12</v>
       </c>
       <c r="N11" s="42"/>
@@ -1784,35 +1784,35 @@
       <c r="A12" s="23"/>
       <c r="B12" s="23"/>
       <c r="C12" s="41"/>
-      <c r="D12" s="33" t="s">
-        <v>96</v>
-      </c>
-      <c r="E12" s="34" t="s">
-        <v>70</v>
-      </c>
-      <c r="F12" s="34">
+      <c r="D12" s="34" t="s">
+        <v>110</v>
+      </c>
+      <c r="E12" s="35" t="s">
+        <v>79</v>
+      </c>
+      <c r="F12" s="35">
         <v>660.0</v>
       </c>
-      <c r="G12" s="43">
+      <c r="G12" s="44">
         <v>45856.0</v>
       </c>
-      <c r="H12" s="44" t="s">
-        <v>71</v>
-      </c>
-      <c r="I12" s="36"/>
-      <c r="J12" s="36">
+      <c r="H12" s="45" t="s">
+        <v>65</v>
+      </c>
+      <c r="I12" s="37"/>
+      <c r="J12" s="37">
         <v>45891.0</v>
       </c>
-      <c r="K12" s="45">
+      <c r="K12" s="46">
         <v>1402001.34</v>
       </c>
-      <c r="L12" s="46" t="s">
-        <v>99</v>
-      </c>
-      <c r="M12" s="38">
+      <c r="L12" s="47" t="s">
+        <v>114</v>
+      </c>
+      <c r="M12" s="39">
         <v>1402001.34</v>
       </c>
-      <c r="N12" s="47"/>
+      <c r="N12" s="48"/>
       <c r="O12" s="25"/>
       <c r="P12" s="28"/>
       <c r="V12" s="3"/>
@@ -1821,69 +1821,69 @@
       <c r="A13" s="23"/>
       <c r="B13" s="23"/>
       <c r="C13" s="41"/>
-      <c r="D13" s="48" t="s">
-        <v>102</v>
-      </c>
-      <c r="E13" s="34" t="s">
-        <v>70</v>
-      </c>
-      <c r="F13" s="35">
+      <c r="D13" s="49" t="s">
+        <v>118</v>
+      </c>
+      <c r="E13" s="35" t="s">
+        <v>79</v>
+      </c>
+      <c r="F13" s="36">
         <v>661.0</v>
       </c>
-      <c r="G13" s="36">
+      <c r="G13" s="37">
         <v>45856.0</v>
       </c>
-      <c r="H13" s="35" t="s">
-        <v>105</v>
-      </c>
-      <c r="I13" s="43"/>
-      <c r="J13" s="43">
+      <c r="H13" s="36" t="s">
+        <v>120</v>
+      </c>
+      <c r="I13" s="44"/>
+      <c r="J13" s="44">
         <v>45891.0</v>
       </c>
-      <c r="K13" s="45">
+      <c r="K13" s="46">
         <v>1223702.3</v>
       </c>
-      <c r="L13" s="34" t="s">
-        <v>106</v>
-      </c>
-      <c r="M13" s="38">
+      <c r="L13" s="35" t="s">
+        <v>122</v>
+      </c>
+      <c r="M13" s="39">
         <v>1223702.3</v>
       </c>
-      <c r="N13" s="47"/>
+      <c r="N13" s="48"/>
       <c r="O13" s="25"/>
-      <c r="P13" s="49"/>
+      <c r="P13" s="50"/>
       <c r="V13" s="3"/>
     </row>
     <row r="14">
       <c r="A14" s="23"/>
       <c r="B14" s="23"/>
       <c r="C14" s="41"/>
-      <c r="D14" s="48" t="s">
-        <v>109</v>
-      </c>
-      <c r="E14" s="34" t="s">
-        <v>70</v>
-      </c>
-      <c r="F14" s="34">
+      <c r="D14" s="49" t="s">
+        <v>126</v>
+      </c>
+      <c r="E14" s="35" t="s">
+        <v>79</v>
+      </c>
+      <c r="F14" s="35">
         <v>688.0</v>
       </c>
-      <c r="G14" s="36">
+      <c r="G14" s="37">
         <v>45901.0</v>
       </c>
-      <c r="H14" s="34" t="s">
-        <v>110</v>
-      </c>
-      <c r="I14" s="43"/>
-      <c r="J14" s="43">
+      <c r="H14" s="35" t="s">
+        <v>127</v>
+      </c>
+      <c r="I14" s="44"/>
+      <c r="J14" s="44">
         <v>45938.0</v>
       </c>
-      <c r="K14" s="45">
+      <c r="K14" s="46">
         <v>1011677.95</v>
       </c>
-      <c r="L14" s="34" t="s">
-        <v>111</v>
-      </c>
-      <c r="M14" s="38">
+      <c r="L14" s="35" t="s">
+        <v>128</v>
+      </c>
+      <c r="M14" s="39">
         <v>1011677.95</v>
       </c>
       <c r="N14" s="42"/>
@@ -1895,35 +1895,35 @@
       <c r="A15" s="23"/>
       <c r="B15" s="23"/>
       <c r="C15" s="41"/>
-      <c r="D15" s="48" t="s">
-        <v>115</v>
-      </c>
-      <c r="E15" s="34" t="s">
-        <v>70</v>
-      </c>
-      <c r="F15" s="34">
+      <c r="D15" s="49" t="s">
+        <v>132</v>
+      </c>
+      <c r="E15" s="35" t="s">
+        <v>79</v>
+      </c>
+      <c r="F15" s="35">
         <v>696.0</v>
       </c>
-      <c r="G15" s="36">
+      <c r="G15" s="37">
         <v>45923.0</v>
       </c>
-      <c r="H15" s="34" t="s">
-        <v>79</v>
-      </c>
-      <c r="I15" s="43"/>
-      <c r="J15" s="43">
+      <c r="H15" s="35" t="s">
+        <v>75</v>
+      </c>
+      <c r="I15" s="44"/>
+      <c r="J15" s="44">
         <v>45938.0</v>
       </c>
-      <c r="K15" s="45">
+      <c r="K15" s="46">
         <v>896744.06</v>
       </c>
-      <c r="L15" s="34" t="s">
-        <v>116</v>
-      </c>
-      <c r="M15" s="38">
+      <c r="L15" s="35" t="s">
+        <v>136</v>
+      </c>
+      <c r="M15" s="39">
         <v>896744.06</v>
       </c>
-      <c r="N15" s="47"/>
+      <c r="N15" s="48"/>
       <c r="O15" s="25"/>
       <c r="V15" s="3"/>
     </row>
@@ -1931,32 +1931,32 @@
       <c r="A16" s="23"/>
       <c r="B16" s="23"/>
       <c r="C16" s="41"/>
-      <c r="D16" s="48" t="s">
-        <v>121</v>
-      </c>
-      <c r="E16" s="34" t="s">
-        <v>70</v>
-      </c>
-      <c r="F16" s="34">
+      <c r="D16" s="49" t="s">
+        <v>138</v>
+      </c>
+      <c r="E16" s="35" t="s">
+        <v>79</v>
+      </c>
+      <c r="F16" s="35">
         <v>704.0</v>
       </c>
-      <c r="G16" s="36">
+      <c r="G16" s="37">
         <v>45957.0</v>
       </c>
-      <c r="H16" s="34" t="s">
-        <v>122</v>
-      </c>
-      <c r="I16" s="43"/>
-      <c r="J16" s="43">
+      <c r="H16" s="35" t="s">
+        <v>141</v>
+      </c>
+      <c r="I16" s="44"/>
+      <c r="J16" s="44">
         <v>46003.0</v>
       </c>
-      <c r="K16" s="45">
+      <c r="K16" s="46">
         <v>919329.06</v>
       </c>
-      <c r="L16" s="34" t="s">
-        <v>125</v>
-      </c>
-      <c r="M16" s="38">
+      <c r="L16" s="35" t="s">
+        <v>142</v>
+      </c>
+      <c r="M16" s="39">
         <v>919329.06</v>
       </c>
       <c r="N16" s="42"/>
@@ -1967,30 +1967,30 @@
       <c r="A17" s="23"/>
       <c r="B17" s="23"/>
       <c r="C17" s="41"/>
-      <c r="D17" s="48" t="s">
-        <v>126</v>
-      </c>
-      <c r="E17" s="34"/>
-      <c r="F17" s="34">
+      <c r="D17" s="49" t="s">
+        <v>146</v>
+      </c>
+      <c r="E17" s="35"/>
+      <c r="F17" s="35">
         <v>705.0</v>
       </c>
-      <c r="G17" s="43">
+      <c r="G17" s="44">
         <v>45972.0</v>
       </c>
-      <c r="H17" s="34" t="s">
-        <v>130</v>
-      </c>
-      <c r="I17" s="34"/>
-      <c r="J17" s="43">
+      <c r="H17" s="35" t="s">
+        <v>147</v>
+      </c>
+      <c r="I17" s="35"/>
+      <c r="J17" s="44">
         <v>46016.0</v>
       </c>
-      <c r="K17" s="45">
+      <c r="K17" s="46">
         <v>1157009.26</v>
       </c>
-      <c r="L17" s="34" t="s">
-        <v>131</v>
-      </c>
-      <c r="M17" s="38">
+      <c r="L17" s="35" t="s">
+        <v>150</v>
+      </c>
+      <c r="M17" s="39">
         <v>1157009.26</v>
       </c>
       <c r="N17" s="51"/>
@@ -2001,32 +2001,32 @@
       <c r="A18" s="23"/>
       <c r="B18" s="23"/>
       <c r="C18" s="41"/>
-      <c r="D18" s="48" t="s">
-        <v>133</v>
-      </c>
-      <c r="E18" s="34" t="s">
-        <v>70</v>
-      </c>
-      <c r="F18" s="34">
+      <c r="D18" s="49" t="s">
+        <v>152</v>
+      </c>
+      <c r="E18" s="35" t="s">
+        <v>79</v>
+      </c>
+      <c r="F18" s="35">
         <v>728.0</v>
       </c>
-      <c r="G18" s="43">
+      <c r="G18" s="44">
         <v>46008.0</v>
       </c>
-      <c r="H18" s="34" t="s">
-        <v>136</v>
-      </c>
-      <c r="I18" s="34"/>
-      <c r="J18" s="43">
+      <c r="H18" s="35" t="s">
+        <v>154</v>
+      </c>
+      <c r="I18" s="35"/>
+      <c r="J18" s="44">
         <v>46040.0</v>
       </c>
-      <c r="K18" s="45">
+      <c r="K18" s="46">
         <v>1214597.952</v>
       </c>
-      <c r="L18" s="34" t="s">
-        <v>139</v>
-      </c>
-      <c r="M18" s="38">
+      <c r="L18" s="35" t="s">
+        <v>155</v>
+      </c>
+      <c r="M18" s="39">
         <v>1214597.952</v>
       </c>
       <c r="N18" s="51"/>
@@ -2041,32 +2041,32 @@
       <c r="A19" s="23"/>
       <c r="B19" s="23"/>
       <c r="C19" s="41"/>
-      <c r="D19" s="48" t="s">
-        <v>143</v>
-      </c>
-      <c r="E19" s="34" t="s">
-        <v>70</v>
-      </c>
-      <c r="F19" s="34">
+      <c r="D19" s="49" t="s">
+        <v>160</v>
+      </c>
+      <c r="E19" s="35" t="s">
+        <v>79</v>
+      </c>
+      <c r="F19" s="35">
         <v>278.0</v>
       </c>
-      <c r="G19" s="43">
+      <c r="G19" s="44">
         <v>46042.0</v>
       </c>
-      <c r="H19" s="34" t="s">
-        <v>144</v>
-      </c>
-      <c r="I19" s="43"/>
-      <c r="J19" s="43">
+      <c r="H19" s="35" t="s">
+        <v>161</v>
+      </c>
+      <c r="I19" s="44"/>
+      <c r="J19" s="44">
         <v>46074.0</v>
       </c>
-      <c r="K19" s="45">
+      <c r="K19" s="46">
         <v>967082.09</v>
       </c>
-      <c r="L19" s="34" t="s">
-        <v>148</v>
-      </c>
-      <c r="M19" s="38">
+      <c r="L19" s="35" t="s">
+        <v>162</v>
+      </c>
+      <c r="M19" s="39">
         <v>967082.09</v>
       </c>
       <c r="N19" s="51"/>
@@ -2081,30 +2081,30 @@
       <c r="A20" s="23"/>
       <c r="B20" s="23"/>
       <c r="C20" s="41"/>
-      <c r="D20" s="48" t="s">
-        <v>152</v>
-      </c>
-      <c r="E20" s="34"/>
-      <c r="F20" s="34">
+      <c r="D20" s="49" t="s">
+        <v>163</v>
+      </c>
+      <c r="E20" s="35"/>
+      <c r="F20" s="35">
         <v>10.0</v>
       </c>
-      <c r="G20" s="43">
+      <c r="G20" s="44">
         <v>46078.0</v>
       </c>
-      <c r="H20" s="34" t="s">
-        <v>112</v>
-      </c>
-      <c r="I20" s="43"/>
-      <c r="J20" s="43">
+      <c r="H20" s="35" t="s">
+        <v>102</v>
+      </c>
+      <c r="I20" s="44"/>
+      <c r="J20" s="44">
         <v>46106.0</v>
       </c>
-      <c r="K20" s="45">
+      <c r="K20" s="46">
         <v>719561.08</v>
       </c>
-      <c r="L20" s="34" t="s">
-        <v>156</v>
-      </c>
-      <c r="M20" s="38">
+      <c r="L20" s="35" t="s">
+        <v>164</v>
+      </c>
+      <c r="M20" s="39">
         <v>719561.08</v>
       </c>
       <c r="N20" s="51"/>
@@ -2119,30 +2119,30 @@
       <c r="A21" s="23"/>
       <c r="B21" s="23"/>
       <c r="C21" s="41"/>
-      <c r="D21" s="48" t="s">
-        <v>158</v>
-      </c>
-      <c r="E21" s="34"/>
-      <c r="F21" s="34">
+      <c r="D21" s="49" t="s">
+        <v>165</v>
+      </c>
+      <c r="E21" s="35"/>
+      <c r="F21" s="35">
         <v>15.0</v>
       </c>
-      <c r="G21" s="43">
+      <c r="G21" s="44">
         <v>46094.0</v>
       </c>
-      <c r="H21" s="34" t="s">
-        <v>160</v>
-      </c>
-      <c r="I21" s="43"/>
-      <c r="J21" s="43">
+      <c r="H21" s="35" t="s">
+        <v>166</v>
+      </c>
+      <c r="I21" s="44"/>
+      <c r="J21" s="44">
         <v>46128.0</v>
       </c>
-      <c r="K21" s="45">
+      <c r="K21" s="46">
         <v>885881.08</v>
       </c>
-      <c r="L21" s="34" t="s">
-        <v>162</v>
-      </c>
-      <c r="M21" s="38">
+      <c r="L21" s="35" t="s">
+        <v>167</v>
+      </c>
+      <c r="M21" s="39">
         <v>885881.08</v>
       </c>
       <c r="N21" s="51"/>
@@ -2157,30 +2157,30 @@
       <c r="A22" s="23"/>
       <c r="B22" s="23"/>
       <c r="C22" s="41"/>
-      <c r="D22" s="48" t="s">
-        <v>166</v>
-      </c>
-      <c r="E22" s="34"/>
-      <c r="F22" s="34">
+      <c r="D22" s="49" t="s">
+        <v>168</v>
+      </c>
+      <c r="E22" s="35"/>
+      <c r="F22" s="35">
         <v>28.0</v>
       </c>
-      <c r="G22" s="43">
+      <c r="G22" s="44">
         <v>46128.0</v>
       </c>
-      <c r="H22" s="34" t="s">
+      <c r="H22" s="35" t="s">
         <v>169</v>
       </c>
-      <c r="I22" s="43"/>
-      <c r="J22" s="43">
+      <c r="I22" s="44"/>
+      <c r="J22" s="44">
         <v>46164.0</v>
       </c>
-      <c r="K22" s="45" t="s">
+      <c r="K22" s="46" t="s">
         <v>170</v>
       </c>
-      <c r="L22" s="34" t="s">
+      <c r="L22" s="35" t="s">
         <v>171</v>
       </c>
-      <c r="M22" s="38" t="s">
+      <c r="M22" s="39" t="s">
         <v>170</v>
       </c>
       <c r="N22" s="51"/>
@@ -2195,30 +2195,30 @@
       <c r="A23" s="23"/>
       <c r="B23" s="23"/>
       <c r="C23" s="41"/>
-      <c r="D23" s="48" t="s">
+      <c r="D23" s="49" t="s">
         <v>172</v>
       </c>
-      <c r="E23" s="34"/>
-      <c r="F23" s="34">
+      <c r="E23" s="35"/>
+      <c r="F23" s="35">
         <v>33.0</v>
       </c>
-      <c r="G23" s="43">
+      <c r="G23" s="44">
         <v>46156.0</v>
       </c>
-      <c r="H23" s="34" t="s">
+      <c r="H23" s="35" t="s">
         <v>173</v>
       </c>
-      <c r="I23" s="43"/>
-      <c r="J23" s="43">
+      <c r="I23" s="44"/>
+      <c r="J23" s="44">
         <v>46191.0</v>
       </c>
-      <c r="K23" s="45">
+      <c r="K23" s="46">
         <v>1108954.4358333333</v>
       </c>
-      <c r="L23" s="34" t="s">
-        <v>162</v>
-      </c>
-      <c r="M23" s="38">
+      <c r="L23" s="35" t="s">
+        <v>167</v>
+      </c>
+      <c r="M23" s="39">
         <v>1108954.4358333333</v>
       </c>
       <c r="N23" s="53"/>
@@ -2233,30 +2233,30 @@
       <c r="A24" s="23"/>
       <c r="B24" s="23"/>
       <c r="C24" s="41"/>
-      <c r="D24" s="48" t="s">
+      <c r="D24" s="49" t="s">
         <v>174</v>
       </c>
-      <c r="E24" s="34"/>
-      <c r="F24" s="34">
+      <c r="E24" s="35"/>
+      <c r="F24" s="35">
         <v>29.0</v>
       </c>
-      <c r="G24" s="43">
+      <c r="G24" s="44">
         <v>46149.0</v>
       </c>
-      <c r="H24" s="34" t="s">
+      <c r="H24" s="35" t="s">
         <v>173</v>
       </c>
-      <c r="I24" s="43"/>
-      <c r="J24" s="43">
+      <c r="I24" s="44"/>
+      <c r="J24" s="44">
         <v>46185.0</v>
       </c>
-      <c r="K24" s="45">
+      <c r="K24" s="46">
         <v>218206.1</v>
       </c>
-      <c r="L24" s="34" t="s">
+      <c r="L24" s="35" t="s">
         <v>175</v>
       </c>
-      <c r="M24" s="38">
+      <c r="M24" s="39">
         <v>218206.1</v>
       </c>
       <c r="N24" s="54"/>
@@ -2271,30 +2271,30 @@
       <c r="A25" s="23"/>
       <c r="B25" s="23"/>
       <c r="C25" s="41"/>
-      <c r="D25" s="48" t="s">
+      <c r="D25" s="49" t="s">
         <v>176</v>
       </c>
-      <c r="E25" s="34"/>
-      <c r="F25" s="34">
+      <c r="E25" s="35"/>
+      <c r="F25" s="35">
         <v>40.0</v>
       </c>
-      <c r="G25" s="43">
+      <c r="G25" s="44">
         <v>46156.0</v>
       </c>
-      <c r="H25" s="34" t="s">
+      <c r="H25" s="35" t="s">
         <v>173</v>
       </c>
-      <c r="I25" s="43"/>
-      <c r="J25" s="43">
+      <c r="I25" s="44"/>
+      <c r="J25" s="44">
         <v>46191.0</v>
       </c>
-      <c r="K25" s="45">
+      <c r="K25" s="46">
         <v>1549250.84</v>
       </c>
-      <c r="L25" s="34" t="s">
+      <c r="L25" s="35" t="s">
         <v>177</v>
       </c>
-      <c r="M25" s="38">
+      <c r="M25" s="39">
         <v>1549250.84</v>
       </c>
       <c r="N25" s="54"/>
@@ -2309,30 +2309,30 @@
       <c r="A26" s="23"/>
       <c r="B26" s="23"/>
       <c r="C26" s="55"/>
-      <c r="D26" s="48" t="s">
+      <c r="D26" s="49" t="s">
         <v>178</v>
       </c>
-      <c r="E26" s="34"/>
-      <c r="F26" s="34">
+      <c r="E26" s="35"/>
+      <c r="F26" s="35">
         <v>48.0</v>
       </c>
-      <c r="G26" s="43">
+      <c r="G26" s="44">
         <v>46230.0</v>
       </c>
-      <c r="H26" s="34" t="s">
+      <c r="H26" s="35" t="s">
         <v>179</v>
       </c>
-      <c r="I26" s="43"/>
-      <c r="J26" s="43">
+      <c r="I26" s="44"/>
+      <c r="J26" s="44">
         <v>46262.0</v>
       </c>
-      <c r="K26" s="45" t="s">
+      <c r="K26" s="46" t="s">
         <v>180</v>
       </c>
-      <c r="L26" s="34" t="s">
+      <c r="L26" s="35" t="s">
         <v>181</v>
       </c>
-      <c r="M26" s="38" t="s">
+      <c r="M26" s="39" t="s">
         <v>180</v>
       </c>
       <c r="N26" s="54"/>
@@ -2346,19 +2346,19 @@
     <row r="27">
       <c r="A27" s="23"/>
       <c r="B27" s="23"/>
-      <c r="C27" s="35"/>
-      <c r="D27" s="48" t="s">
+      <c r="C27" s="36"/>
+      <c r="D27" s="49" t="s">
         <v>182</v>
       </c>
-      <c r="E27" s="34"/>
-      <c r="F27" s="34"/>
-      <c r="G27" s="43"/>
-      <c r="H27" s="34"/>
-      <c r="I27" s="43"/>
-      <c r="J27" s="43"/>
-      <c r="K27" s="45"/>
-      <c r="L27" s="34"/>
-      <c r="M27" s="38"/>
+      <c r="E27" s="35"/>
+      <c r="F27" s="35"/>
+      <c r="G27" s="44"/>
+      <c r="H27" s="35"/>
+      <c r="I27" s="44"/>
+      <c r="J27" s="44"/>
+      <c r="K27" s="46"/>
+      <c r="L27" s="35"/>
+      <c r="M27" s="39"/>
       <c r="N27" s="54"/>
       <c r="O27" s="25"/>
       <c r="R27" s="28"/>
@@ -2371,34 +2371,34 @@
       <c r="A28" s="23"/>
       <c r="B28" s="23"/>
       <c r="C28" s="29" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="D28" s="29" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="E28" s="30" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="F28" s="29" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="G28" s="29"/>
       <c r="H28" s="29" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="I28" s="29"/>
       <c r="J28" s="29"/>
       <c r="K28" s="56" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="L28" s="31" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="M28" s="57" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="N28" s="29" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="O28" s="25"/>
       <c r="P28" s="28"/>
@@ -2418,30 +2418,30 @@
     <row r="29" ht="12.75" customHeight="1">
       <c r="A29" s="23"/>
       <c r="B29" s="23"/>
-      <c r="C29" s="32">
+      <c r="C29" s="33">
         <v>2.0</v>
       </c>
       <c r="D29" s="58" t="s">
         <v>183</v>
       </c>
-      <c r="E29" s="35"/>
-      <c r="F29" s="35">
+      <c r="E29" s="36"/>
+      <c r="F29" s="36">
         <v>402.0</v>
       </c>
-      <c r="G29" s="36">
+      <c r="G29" s="37">
         <v>45791.0</v>
       </c>
-      <c r="H29" s="35" t="s">
+      <c r="H29" s="36" t="s">
         <v>49</v>
       </c>
-      <c r="I29" s="36"/>
-      <c r="J29" s="36">
+      <c r="I29" s="37"/>
+      <c r="J29" s="37">
         <v>45834.0</v>
       </c>
-      <c r="K29" s="37">
+      <c r="K29" s="38">
         <v>188246.17</v>
       </c>
-      <c r="L29" s="34" t="s">
+      <c r="L29" s="35" t="s">
         <v>184</v>
       </c>
       <c r="M29" s="59">
@@ -2474,26 +2474,26 @@
       <c r="E30" s="60">
         <v>46.0</v>
       </c>
-      <c r="F30" s="35">
+      <c r="F30" s="36">
         <v>447.0</v>
       </c>
-      <c r="G30" s="36">
+      <c r="G30" s="37">
         <v>45814.0</v>
       </c>
-      <c r="H30" s="34" t="s">
+      <c r="H30" s="35" t="s">
         <v>186</v>
       </c>
-      <c r="I30" s="43"/>
-      <c r="J30" s="43">
+      <c r="I30" s="44"/>
+      <c r="J30" s="44">
         <v>45955.0</v>
       </c>
-      <c r="K30" s="37">
+      <c r="K30" s="38">
         <v>112720.77</v>
       </c>
-      <c r="L30" s="34" t="s">
+      <c r="L30" s="35" t="s">
         <v>187</v>
       </c>
-      <c r="M30" s="38">
+      <c r="M30" s="39">
         <v>112720.77</v>
       </c>
       <c r="N30" s="51"/>
@@ -2523,26 +2523,26 @@
       <c r="E31" s="62" t="s">
         <v>189</v>
       </c>
-      <c r="F31" s="35">
+      <c r="F31" s="36">
         <v>529.0</v>
       </c>
       <c r="G31" s="63">
         <v>45853.0</v>
       </c>
-      <c r="H31" s="34" t="s">
-        <v>63</v>
-      </c>
-      <c r="I31" s="43"/>
-      <c r="J31" s="43">
+      <c r="H31" s="35" t="s">
+        <v>54</v>
+      </c>
+      <c r="I31" s="44"/>
+      <c r="J31" s="44">
         <v>45939.0</v>
       </c>
-      <c r="K31" s="45">
+      <c r="K31" s="46">
         <v>378307.61</v>
       </c>
-      <c r="L31" s="34" t="s">
+      <c r="L31" s="35" t="s">
         <v>190</v>
       </c>
-      <c r="M31" s="38">
+      <c r="M31" s="39">
         <v>378307.61</v>
       </c>
       <c r="N31" s="51"/>
@@ -2572,26 +2572,26 @@
       <c r="E32" s="62" t="s">
         <v>189</v>
       </c>
-      <c r="F32" s="34">
+      <c r="F32" s="35">
         <v>691.0</v>
       </c>
       <c r="G32" s="63">
         <v>45910.0</v>
       </c>
-      <c r="H32" s="34" t="s">
-        <v>63</v>
-      </c>
-      <c r="I32" s="43"/>
-      <c r="J32" s="43">
+      <c r="H32" s="35" t="s">
+        <v>54</v>
+      </c>
+      <c r="I32" s="44"/>
+      <c r="J32" s="44">
         <v>45941.0</v>
       </c>
-      <c r="K32" s="37">
+      <c r="K32" s="38">
         <v>3315.0471000000252</v>
       </c>
-      <c r="L32" s="34" t="s">
+      <c r="L32" s="35" t="s">
         <v>192</v>
       </c>
-      <c r="M32" s="38">
+      <c r="M32" s="39">
         <v>3315.04710000003</v>
       </c>
       <c r="N32" s="51"/>
@@ -2621,26 +2621,26 @@
       <c r="E33" s="65">
         <v>135.0</v>
       </c>
-      <c r="F33" s="34">
+      <c r="F33" s="35">
         <v>677.0</v>
       </c>
       <c r="G33" s="63">
         <v>45904.0</v>
       </c>
-      <c r="H33" s="34" t="s">
-        <v>71</v>
+      <c r="H33" s="35" t="s">
+        <v>65</v>
       </c>
       <c r="I33" s="66"/>
       <c r="J33" s="66">
         <v>45935.0</v>
       </c>
-      <c r="K33" s="45">
+      <c r="K33" s="46">
         <v>198332.75</v>
       </c>
-      <c r="L33" s="34" t="s">
+      <c r="L33" s="35" t="s">
         <v>194</v>
       </c>
-      <c r="M33" s="38">
+      <c r="M33" s="39">
         <v>198332.75</v>
       </c>
       <c r="N33" s="51"/>
@@ -2670,20 +2670,20 @@
       <c r="E34" s="65">
         <v>40.0</v>
       </c>
-      <c r="F34" s="34">
+      <c r="F34" s="35">
         <v>278.0</v>
       </c>
       <c r="G34" s="63">
         <v>46008.0</v>
       </c>
-      <c r="H34" s="34" t="s">
-        <v>127</v>
+      <c r="H34" s="35" t="s">
+        <v>115</v>
       </c>
       <c r="I34" s="66"/>
       <c r="J34" s="66">
         <v>46066.0</v>
       </c>
-      <c r="K34" s="45">
+      <c r="K34" s="46">
         <v>1528.62</v>
       </c>
       <c r="L34" s="67" t="s">
@@ -2719,23 +2719,23 @@
       <c r="E35" s="65" t="s">
         <v>199</v>
       </c>
-      <c r="F35" s="34">
+      <c r="F35" s="35">
         <v>748.0</v>
       </c>
       <c r="G35" s="63">
         <v>45930.0</v>
       </c>
-      <c r="H35" s="34" t="s">
-        <v>97</v>
+      <c r="H35" s="35" t="s">
+        <v>90</v>
       </c>
       <c r="I35" s="66"/>
       <c r="J35" s="66">
         <v>45935.0</v>
       </c>
-      <c r="K35" s="45">
+      <c r="K35" s="46">
         <v>38718.58</v>
       </c>
-      <c r="L35" s="34" t="s">
+      <c r="L35" s="35" t="s">
         <v>200</v>
       </c>
       <c r="M35" s="59" t="s">
@@ -2768,23 +2768,23 @@
       <c r="E36" s="65">
         <v>154.0</v>
       </c>
-      <c r="F36" s="34">
+      <c r="F36" s="35">
         <v>822.0</v>
       </c>
       <c r="G36" s="63">
         <v>45968.0</v>
       </c>
-      <c r="H36" s="34" t="s">
-        <v>117</v>
+      <c r="H36" s="35" t="s">
+        <v>107</v>
       </c>
       <c r="I36" s="66"/>
       <c r="J36" s="66">
         <v>45935.0</v>
       </c>
-      <c r="K36" s="45">
+      <c r="K36" s="46">
         <v>133124.11</v>
       </c>
-      <c r="L36" s="34" t="s">
+      <c r="L36" s="35" t="s">
         <v>203</v>
       </c>
       <c r="M36" s="59" t="s">
@@ -2824,19 +2824,19 @@
         <v>46043.0</v>
       </c>
       <c r="H37" s="65" t="s">
-        <v>112</v>
+        <v>102</v>
       </c>
       <c r="I37" s="70"/>
       <c r="J37" s="69">
         <v>46075.0</v>
       </c>
-      <c r="K37" s="45">
+      <c r="K37" s="46">
         <v>11372.9</v>
       </c>
-      <c r="L37" s="34" t="s">
+      <c r="L37" s="35" t="s">
         <v>206</v>
       </c>
-      <c r="M37" s="38">
+      <c r="M37" s="39">
         <v>11372.9</v>
       </c>
       <c r="N37" s="51"/>
@@ -2871,9 +2871,9 @@
         <v>208</v>
       </c>
       <c r="J38" s="69"/>
-      <c r="K38" s="45"/>
-      <c r="L38" s="34"/>
-      <c r="M38" s="38"/>
+      <c r="K38" s="46"/>
+      <c r="L38" s="35"/>
+      <c r="M38" s="39"/>
       <c r="N38" s="51">
         <v>15854.78</v>
       </c>
@@ -2908,9 +2908,9 @@
         <v>208</v>
       </c>
       <c r="J39" s="69"/>
-      <c r="K39" s="45"/>
-      <c r="L39" s="34"/>
-      <c r="M39" s="38"/>
+      <c r="K39" s="46"/>
+      <c r="L39" s="35"/>
+      <c r="M39" s="39"/>
       <c r="N39" s="71">
         <v>42229.72325</v>
       </c>
@@ -2933,7 +2933,7 @@
     <row r="40" ht="12.75" customHeight="1">
       <c r="A40" s="23"/>
       <c r="B40" s="23"/>
-      <c r="C40" s="35"/>
+      <c r="C40" s="36"/>
       <c r="D40" s="61" t="s">
         <v>210</v>
       </c>
@@ -2945,9 +2945,9 @@
         <v>208</v>
       </c>
       <c r="J40" s="69"/>
-      <c r="K40" s="45"/>
-      <c r="L40" s="46"/>
-      <c r="M40" s="38"/>
+      <c r="K40" s="46"/>
+      <c r="L40" s="47"/>
+      <c r="M40" s="39"/>
       <c r="N40" s="72">
         <v>48857.395500000006</v>
       </c>
@@ -2970,7 +2970,7 @@
     <row r="41" ht="12.75" customHeight="1">
       <c r="A41" s="23"/>
       <c r="B41" s="23"/>
-      <c r="C41" s="35"/>
+      <c r="C41" s="36"/>
       <c r="D41" s="61" t="s">
         <v>211</v>
       </c>
@@ -2982,9 +2982,9 @@
         <v>212</v>
       </c>
       <c r="J41" s="69"/>
-      <c r="K41" s="45"/>
-      <c r="L41" s="46"/>
-      <c r="M41" s="38"/>
+      <c r="K41" s="46"/>
+      <c r="L41" s="47"/>
+      <c r="M41" s="39"/>
       <c r="N41" s="72"/>
       <c r="O41" s="25"/>
       <c r="P41" s="28"/>
@@ -3005,7 +3005,7 @@
     <row r="42" ht="12.75" customHeight="1">
       <c r="A42" s="23"/>
       <c r="B42" s="23"/>
-      <c r="C42" s="32">
+      <c r="C42" s="33">
         <v>3.0</v>
       </c>
       <c r="D42" s="61" t="s">
@@ -3019,13 +3019,13 @@
         <v>46104.0</v>
       </c>
       <c r="H42" s="65" t="s">
-        <v>112</v>
+        <v>102</v>
       </c>
       <c r="I42" s="70"/>
       <c r="J42" s="69">
         <v>46106.0</v>
       </c>
-      <c r="K42" s="45">
+      <c r="K42" s="46">
         <v>27801.11</v>
       </c>
       <c r="L42" s="73" t="s">
@@ -3066,17 +3066,17 @@
         <v>46199.0</v>
       </c>
       <c r="H43" s="65" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="I43" s="70"/>
       <c r="J43" s="69">
         <v>46233.0</v>
       </c>
-      <c r="K43" s="45">
+      <c r="K43" s="46">
         <v>58868.35</v>
       </c>
-      <c r="L43" s="34" t="s">
-        <v>65</v>
+      <c r="L43" s="35" t="s">
+        <v>71</v>
       </c>
       <c r="M43" s="74">
         <v>58868.35</v>
@@ -8035,11 +8035,11 @@
       <c r="AH1" s="2"/>
     </row>
     <row r="2">
-      <c r="A2" s="4">
+      <c r="A2" s="5">
         <v>46212.0</v>
       </c>
-      <c r="L2" s="6" t="s">
-        <v>0</v>
+      <c r="L2" s="7" t="s">
+        <v>1</v>
       </c>
       <c r="AB2" s="2"/>
       <c r="AC2" s="2"/>
@@ -8050,31 +8050,31 @@
       <c r="AH2" s="2"/>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="11">
+      <c r="C3" s="12">
         <v>2.5E32</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="D3" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="12">
+      <c r="E3" s="13">
         <v>45686.0</v>
       </c>
-      <c r="F3" s="8" t="s">
+      <c r="F3" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G3" s="8">
+      <c r="G3" s="10">
         <v>12.0</v>
       </c>
-      <c r="H3" s="8">
+      <c r="H3" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I3" s="8">
+      <c r="I3" s="10">
         <v>2048.0</v>
       </c>
       <c r="J3" s="14">
@@ -8083,7 +8083,7 @@
       <c r="K3" s="14">
         <v>1000.0</v>
       </c>
-      <c r="L3" s="8">
+      <c r="L3" s="10">
         <v>0.0</v>
       </c>
       <c r="AB3" s="2"/>
@@ -8095,31 +8095,31 @@
       <c r="AH3" s="2"/>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="C4" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="D4" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="12">
+      <c r="E4" s="13">
         <v>45762.0</v>
       </c>
-      <c r="F4" s="8" t="s">
+      <c r="F4" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G4" s="8">
+      <c r="G4" s="10">
         <v>12.0</v>
       </c>
-      <c r="H4" s="8">
+      <c r="H4" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I4" s="8">
+      <c r="I4" s="10">
         <v>2048.0</v>
       </c>
       <c r="J4" s="14">
@@ -8128,7 +8128,7 @@
       <c r="K4" s="14">
         <v>52250.04</v>
       </c>
-      <c r="L4" s="8">
+      <c r="L4" s="10">
         <v>0.0</v>
       </c>
       <c r="AB4" s="2"/>
@@ -8140,31 +8140,31 @@
       <c r="AH4" s="2"/>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="C5" s="8" t="s">
+      <c r="C5" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="D5" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E5" s="12">
+      <c r="E5" s="13">
         <v>45762.0</v>
       </c>
-      <c r="F5" s="8" t="s">
+      <c r="F5" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G5" s="8">
+      <c r="G5" s="10">
         <v>12.0</v>
       </c>
-      <c r="H5" s="8">
+      <c r="H5" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I5" s="8">
+      <c r="I5" s="10">
         <v>2048.0</v>
       </c>
       <c r="J5" s="14">
@@ -8173,7 +8173,7 @@
       <c r="K5" s="14">
         <v>881914.18</v>
       </c>
-      <c r="L5" s="8">
+      <c r="L5" s="10">
         <v>0.0</v>
       </c>
       <c r="AB5" s="2"/>
@@ -8185,31 +8185,31 @@
       <c r="AH5" s="2"/>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="B6" s="8" t="s">
+      <c r="A6" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="D6" s="8" t="s">
+      <c r="C6" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="D6" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E6" s="12">
+      <c r="E6" s="13">
         <v>45762.0</v>
       </c>
-      <c r="F6" s="8" t="s">
+      <c r="F6" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G6" s="8">
+      <c r="G6" s="10">
         <v>12.0</v>
       </c>
-      <c r="H6" s="8">
+      <c r="H6" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I6" s="8">
+      <c r="I6" s="10">
         <v>2048.0</v>
       </c>
       <c r="J6" s="14">
@@ -8218,7 +8218,7 @@
       <c r="K6" s="14">
         <v>750000.0</v>
       </c>
-      <c r="L6" s="8">
+      <c r="L6" s="10">
         <v>0.0</v>
       </c>
       <c r="AB6" s="2"/>
@@ -8230,31 +8230,31 @@
       <c r="AH6" s="2"/>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="B7" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="C7" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="D7" s="8" t="s">
+      <c r="A7" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="D7" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E7" s="12">
+      <c r="E7" s="13">
         <v>45763.0</v>
       </c>
-      <c r="F7" s="8" t="s">
+      <c r="F7" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G7" s="8">
+      <c r="G7" s="10">
         <v>12.0</v>
       </c>
-      <c r="H7" s="8">
+      <c r="H7" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I7" s="8" t="s">
+      <c r="I7" s="10" t="s">
         <v>43</v>
       </c>
       <c r="J7" s="14">
@@ -8263,7 +8263,7 @@
       <c r="K7" s="14">
         <v>949835.78</v>
       </c>
-      <c r="L7" s="8">
+      <c r="L7" s="10">
         <v>0.0</v>
       </c>
       <c r="AB7" s="2"/>
@@ -8275,31 +8275,31 @@
       <c r="AH7" s="2"/>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="s">
+      <c r="A8" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="B8" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="C8" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="D8" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E8" s="12">
+      <c r="E8" s="13">
         <v>45763.0</v>
       </c>
-      <c r="F8" s="8" t="s">
+      <c r="F8" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G8" s="8">
+      <c r="G8" s="10">
         <v>12.0</v>
       </c>
-      <c r="H8" s="8">
+      <c r="H8" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I8" s="8" t="s">
+      <c r="I8" s="10" t="s">
         <v>48</v>
       </c>
       <c r="J8" s="14">
@@ -8308,10 +8308,10 @@
       <c r="K8" s="14">
         <v>524584.95</v>
       </c>
-      <c r="L8" s="8">
+      <c r="L8" s="10">
         <v>0.0</v>
       </c>
-      <c r="O8" s="27"/>
+      <c r="O8" s="26"/>
       <c r="AB8" s="2"/>
       <c r="AC8" s="2"/>
       <c r="AD8" s="2"/>
@@ -8321,32 +8321,32 @@
       <c r="AH8" s="2"/>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="s">
+      <c r="A9" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="B9" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="C9" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="C9" s="8" t="s">
+      <c r="D9" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="E9" s="13">
+        <v>45792.0</v>
+      </c>
+      <c r="F9" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="G9" s="10">
+        <v>12.0</v>
+      </c>
+      <c r="H9" s="10">
+        <v>339039.0</v>
+      </c>
+      <c r="I9" s="10" t="s">
         <v>52</v>
-      </c>
-      <c r="D9" s="8" t="s">
-        <v>4</v>
-      </c>
-      <c r="E9" s="12">
-        <v>45792.0</v>
-      </c>
-      <c r="F9" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="G9" s="8">
-        <v>12.0</v>
-      </c>
-      <c r="H9" s="8">
-        <v>339039.0</v>
-      </c>
-      <c r="I9" s="8" t="s">
-        <v>55</v>
       </c>
       <c r="J9" s="14">
         <v>211614.23</v>
@@ -8354,7 +8354,7 @@
       <c r="K9" s="14">
         <v>211614.23</v>
       </c>
-      <c r="L9" s="8">
+      <c r="L9" s="10">
         <v>0.0</v>
       </c>
       <c r="AB9" s="2"/>
@@ -8366,31 +8366,31 @@
       <c r="AH9" s="2"/>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="s">
-        <v>63</v>
-      </c>
-      <c r="B10" s="8" t="s">
+      <c r="A10" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="B10" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="C10" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="D10" s="8" t="s">
+      <c r="C10" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="D10" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E10" s="12">
+      <c r="E10" s="13">
         <v>45825.0</v>
       </c>
-      <c r="F10" s="8" t="s">
+      <c r="F10" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G10" s="8">
+      <c r="G10" s="10">
         <v>12.0</v>
       </c>
-      <c r="H10" s="8">
+      <c r="H10" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I10" s="8">
+      <c r="I10" s="10">
         <v>2048.0</v>
       </c>
       <c r="J10" s="14">
@@ -8411,31 +8411,31 @@
       <c r="AH10" s="2"/>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="B11" s="8" t="s">
+      <c r="A11" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="B11" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="C11" s="8" t="s">
-        <v>68</v>
-      </c>
-      <c r="D11" s="8" t="s">
+      <c r="C11" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="D11" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E11" s="12">
+      <c r="E11" s="13">
         <v>45825.0</v>
       </c>
-      <c r="F11" s="8" t="s">
+      <c r="F11" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G11" s="8">
+      <c r="G11" s="10">
         <v>12.0</v>
       </c>
-      <c r="H11" s="8">
+      <c r="H11" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I11" s="8">
+      <c r="I11" s="10">
         <v>2048.0</v>
       </c>
       <c r="J11" s="14">
@@ -8444,7 +8444,7 @@
       <c r="K11" s="14">
         <v>618154.38</v>
       </c>
-      <c r="L11" s="8">
+      <c r="L11" s="10">
         <v>0.01</v>
       </c>
       <c r="AB11" s="2"/>
@@ -8456,32 +8456,32 @@
       <c r="AH11" s="2"/>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="B12" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="C12" s="8" t="s">
-        <v>74</v>
-      </c>
-      <c r="D12" s="8" t="s">
+      <c r="A12" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="B12" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="C12" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="D12" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E12" s="12">
+      <c r="E12" s="13">
         <v>45832.0</v>
       </c>
-      <c r="F12" s="8" t="s">
+      <c r="F12" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G12" s="8">
+      <c r="G12" s="10">
         <v>12.0</v>
       </c>
-      <c r="H12" s="8">
+      <c r="H12" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I12" s="8" t="s">
-        <v>75</v>
+      <c r="I12" s="10" t="s">
+        <v>70</v>
       </c>
       <c r="J12" s="14">
         <v>1600334.09</v>
@@ -8489,7 +8489,7 @@
       <c r="K12" s="14">
         <v>1600334.09</v>
       </c>
-      <c r="L12" s="8">
+      <c r="L12" s="10">
         <v>0.0</v>
       </c>
       <c r="AB12" s="2"/>
@@ -8501,31 +8501,31 @@
       <c r="AH12" s="2"/>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="s">
-        <v>77</v>
-      </c>
-      <c r="B13" s="8" t="s">
+      <c r="A13" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="B13" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="C13" s="8" t="s">
-        <v>78</v>
-      </c>
-      <c r="D13" s="8" t="s">
+      <c r="C13" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="D13" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E13" s="12">
+      <c r="E13" s="13">
         <v>45863.0</v>
       </c>
-      <c r="F13" s="8" t="s">
+      <c r="F13" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G13" s="8">
+      <c r="G13" s="10">
         <v>12.0</v>
       </c>
-      <c r="H13" s="8">
+      <c r="H13" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I13" s="8">
+      <c r="I13" s="10">
         <v>2048.0</v>
       </c>
       <c r="J13" s="14">
@@ -8537,7 +8537,7 @@
       <c r="L13" s="14">
         <v>0.0</v>
       </c>
-      <c r="M13" s="39"/>
+      <c r="M13" s="32"/>
       <c r="AB13" s="2"/>
       <c r="AC13" s="2"/>
       <c r="AD13" s="2"/>
@@ -8547,32 +8547,32 @@
       <c r="AH13" s="2"/>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="s">
-        <v>79</v>
-      </c>
-      <c r="B14" s="8" t="s">
-        <v>80</v>
-      </c>
-      <c r="C14" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="D14" s="8" t="s">
+      <c r="A14" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="B14" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="C14" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="D14" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E14" s="12">
+      <c r="E14" s="13">
         <v>45887.0</v>
       </c>
-      <c r="F14" s="8" t="s">
+      <c r="F14" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G14" s="8">
+      <c r="G14" s="10">
         <v>12.0</v>
       </c>
-      <c r="H14" s="8">
+      <c r="H14" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I14" s="8" t="s">
-        <v>55</v>
+      <c r="I14" s="10" t="s">
+        <v>52</v>
       </c>
       <c r="J14" s="14">
         <v>968237.39</v>
@@ -8580,7 +8580,7 @@
       <c r="K14" s="14">
         <v>968237.39</v>
       </c>
-      <c r="L14" s="8">
+      <c r="L14" s="10">
         <v>0.0</v>
       </c>
       <c r="AB14" s="2"/>
@@ -8592,31 +8592,31 @@
       <c r="AH14" s="2"/>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="B15" s="8" t="s">
-        <v>85</v>
-      </c>
-      <c r="C15" s="8" t="s">
-        <v>86</v>
-      </c>
-      <c r="D15" s="8" t="s">
+      <c r="A15" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="B15" s="10" t="s">
+        <v>82</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="D15" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E15" s="12">
+      <c r="E15" s="13">
         <v>45924.0</v>
       </c>
-      <c r="F15" s="8" t="s">
+      <c r="F15" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G15" s="8">
+      <c r="G15" s="10">
         <v>12.0</v>
       </c>
-      <c r="H15" s="8">
+      <c r="H15" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I15" s="8" t="s">
+      <c r="I15" s="10" t="s">
         <v>43</v>
       </c>
       <c r="J15" s="14">
@@ -8625,7 +8625,7 @@
       <c r="K15" s="14">
         <v>1011677.95</v>
       </c>
-      <c r="L15" s="8">
+      <c r="L15" s="10">
         <v>0.0</v>
       </c>
       <c r="AB15" s="2"/>
@@ -8637,31 +8637,31 @@
       <c r="AH15" s="2"/>
     </row>
     <row r="16">
-      <c r="A16" s="8" t="s">
-        <v>88</v>
-      </c>
-      <c r="B16" s="8" t="s">
+      <c r="A16" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="B16" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="C16" s="8" t="s">
-        <v>90</v>
-      </c>
-      <c r="D16" s="8" t="s">
+      <c r="C16" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="D16" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E16" s="12">
+      <c r="E16" s="13">
         <v>45929.0</v>
       </c>
-      <c r="F16" s="8" t="s">
+      <c r="F16" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G16" s="8">
+      <c r="G16" s="10">
         <v>12.0</v>
       </c>
-      <c r="H16" s="8">
+      <c r="H16" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I16" s="8">
+      <c r="I16" s="10">
         <v>2048.0</v>
       </c>
       <c r="J16" s="14">
@@ -8682,37 +8682,37 @@
       <c r="AH16" s="2"/>
     </row>
     <row r="17">
-      <c r="A17" s="8" t="s">
-        <v>93</v>
-      </c>
-      <c r="B17" s="8" t="s">
-        <v>94</v>
-      </c>
-      <c r="C17" s="8" t="s">
-        <v>95</v>
-      </c>
-      <c r="D17" s="8" t="s">
+      <c r="A17" s="10" t="s">
+        <v>87</v>
+      </c>
+      <c r="B17" s="10" t="s">
+        <v>88</v>
+      </c>
+      <c r="C17" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="D17" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E17" s="12">
+      <c r="E17" s="13">
         <v>45930.0</v>
       </c>
-      <c r="F17" s="8" t="s">
+      <c r="F17" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G17" s="8">
+      <c r="G17" s="10">
         <v>12.0</v>
       </c>
-      <c r="H17" s="8">
+      <c r="H17" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I17" s="8">
+      <c r="I17" s="10">
         <v>2048.0</v>
       </c>
       <c r="J17" s="14">
         <v>34065.36</v>
       </c>
-      <c r="K17" s="8">
+      <c r="K17" s="10">
         <v>0.0</v>
       </c>
       <c r="L17" s="14">
@@ -8727,32 +8727,32 @@
       <c r="AH17" s="2"/>
     </row>
     <row r="18">
-      <c r="A18" s="8" t="s">
-        <v>97</v>
-      </c>
-      <c r="B18" s="8" t="s">
-        <v>80</v>
-      </c>
-      <c r="C18" s="8" t="s">
-        <v>98</v>
-      </c>
-      <c r="D18" s="8" t="s">
+      <c r="A18" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="B18" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="C18" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="D18" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E18" s="12">
+      <c r="E18" s="13">
         <v>45938.0</v>
       </c>
-      <c r="F18" s="8" t="s">
+      <c r="F18" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G18" s="8">
+      <c r="G18" s="10">
         <v>12.0</v>
       </c>
-      <c r="H18" s="8">
+      <c r="H18" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I18" s="8" t="s">
-        <v>55</v>
+      <c r="I18" s="10" t="s">
+        <v>52</v>
       </c>
       <c r="J18" s="14">
         <v>63746.85</v>
@@ -8760,7 +8760,7 @@
       <c r="K18" s="14">
         <v>63746.85</v>
       </c>
-      <c r="L18" s="8">
+      <c r="L18" s="10">
         <v>0.0</v>
       </c>
       <c r="AB18" s="2"/>
@@ -8772,32 +8772,32 @@
       <c r="AH18" s="2"/>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="s">
-        <v>100</v>
-      </c>
-      <c r="B19" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="C19" s="8" t="s">
-        <v>101</v>
-      </c>
-      <c r="D19" s="8" t="s">
+      <c r="A19" s="10" t="s">
+        <v>93</v>
+      </c>
+      <c r="B19" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="C19" s="10" t="s">
+        <v>94</v>
+      </c>
+      <c r="D19" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E19" s="12">
+      <c r="E19" s="13">
         <v>45938.0</v>
       </c>
-      <c r="F19" s="8" t="s">
+      <c r="F19" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G19" s="8">
+      <c r="G19" s="10">
         <v>12.0</v>
       </c>
-      <c r="H19" s="8">
+      <c r="H19" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I19" s="8" t="s">
-        <v>75</v>
+      <c r="I19" s="10" t="s">
+        <v>70</v>
       </c>
       <c r="J19" s="14">
         <v>947931.1</v>
@@ -8805,7 +8805,7 @@
       <c r="K19" s="14">
         <v>947931.1</v>
       </c>
-      <c r="L19" s="8">
+      <c r="L19" s="10">
         <v>0.0</v>
       </c>
       <c r="AB19" s="2"/>
@@ -8817,31 +8817,31 @@
       <c r="AH19" s="2"/>
     </row>
     <row r="20">
-      <c r="A20" s="8" t="s">
-        <v>103</v>
-      </c>
-      <c r="B20" s="8" t="s">
+      <c r="A20" s="10" t="s">
+        <v>96</v>
+      </c>
+      <c r="B20" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="C20" s="8" t="s">
-        <v>104</v>
-      </c>
-      <c r="D20" s="8" t="s">
+      <c r="C20" s="10" t="s">
+        <v>97</v>
+      </c>
+      <c r="D20" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E20" s="12">
+      <c r="E20" s="13">
         <v>45938.0</v>
       </c>
-      <c r="F20" s="8" t="s">
+      <c r="F20" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G20" s="8">
+      <c r="G20" s="10">
         <v>12.0</v>
       </c>
-      <c r="H20" s="8">
+      <c r="H20" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I20" s="8">
+      <c r="I20" s="10">
         <v>2048.0</v>
       </c>
       <c r="J20" s="14">
@@ -8850,7 +8850,7 @@
       <c r="K20" s="14">
         <v>259790.57</v>
       </c>
-      <c r="L20" s="8">
+      <c r="L20" s="10">
         <v>0.0</v>
       </c>
       <c r="AB20" s="2"/>
@@ -8862,31 +8862,31 @@
       <c r="AH20" s="2"/>
     </row>
     <row r="21">
-      <c r="A21" s="8" t="s">
-        <v>107</v>
-      </c>
-      <c r="B21" s="8" t="s">
+      <c r="A21" s="10" t="s">
+        <v>99</v>
+      </c>
+      <c r="B21" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="C21" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="D21" s="8" t="s">
+      <c r="C21" s="10" t="s">
+        <v>100</v>
+      </c>
+      <c r="D21" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E21" s="12">
+      <c r="E21" s="13">
         <v>45938.0</v>
       </c>
-      <c r="F21" s="8" t="s">
+      <c r="F21" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G21" s="8">
+      <c r="G21" s="10">
         <v>12.0</v>
       </c>
-      <c r="H21" s="8">
+      <c r="H21" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I21" s="8">
+      <c r="I21" s="10">
         <v>2048.0</v>
       </c>
       <c r="J21" s="14">
@@ -8895,7 +8895,7 @@
       <c r="K21" s="14">
         <v>170479.3</v>
       </c>
-      <c r="L21" s="8">
+      <c r="L21" s="10">
         <v>0.0</v>
       </c>
       <c r="AB21" s="2"/>
@@ -8907,31 +8907,31 @@
       <c r="AH21" s="2"/>
     </row>
     <row r="22">
-      <c r="A22" s="8" t="s">
-        <v>112</v>
-      </c>
-      <c r="B22" s="8" t="s">
-        <v>113</v>
-      </c>
-      <c r="C22" s="8" t="s">
-        <v>114</v>
-      </c>
-      <c r="D22" s="8" t="s">
+      <c r="A22" s="10" t="s">
+        <v>102</v>
+      </c>
+      <c r="B22" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="C22" s="10" t="s">
+        <v>105</v>
+      </c>
+      <c r="D22" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E22" s="50">
+      <c r="E22" s="43">
         <v>45953.0</v>
       </c>
-      <c r="F22" s="8" t="s">
+      <c r="F22" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G22" s="8">
+      <c r="G22" s="10">
         <v>12.0</v>
       </c>
-      <c r="H22" s="8">
+      <c r="H22" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I22" s="8">
+      <c r="I22" s="10">
         <v>2000.0</v>
       </c>
       <c r="J22" s="14">
@@ -8952,32 +8952,32 @@
       <c r="AH22" s="2"/>
     </row>
     <row r="23">
-      <c r="A23" s="8" t="s">
-        <v>117</v>
-      </c>
-      <c r="B23" s="8" t="s">
-        <v>118</v>
-      </c>
-      <c r="C23" s="8" t="s">
-        <v>119</v>
-      </c>
-      <c r="D23" s="8" t="s">
+      <c r="A23" s="10" t="s">
+        <v>107</v>
+      </c>
+      <c r="B23" s="10" t="s">
+        <v>108</v>
+      </c>
+      <c r="C23" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="D23" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E23" s="50">
+      <c r="E23" s="43">
         <v>45953.0</v>
       </c>
-      <c r="F23" s="8" t="s">
+      <c r="F23" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G23" s="8">
+      <c r="G23" s="10">
         <v>12.0</v>
       </c>
-      <c r="H23" s="8">
+      <c r="H23" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I23" s="8" t="s">
-        <v>120</v>
+      <c r="I23" s="10" t="s">
+        <v>111</v>
       </c>
       <c r="J23" s="14">
         <v>1000001.64</v>
@@ -8985,7 +8985,7 @@
       <c r="K23" s="14">
         <v>1000001.64</v>
       </c>
-      <c r="L23" s="8">
+      <c r="L23" s="10">
         <v>0.0</v>
       </c>
       <c r="AB23" s="2"/>
@@ -8997,31 +8997,31 @@
       <c r="AH23" s="2"/>
     </row>
     <row r="24">
-      <c r="A24" s="8" t="s">
-        <v>123</v>
-      </c>
-      <c r="B24" s="8" t="s">
+      <c r="A24" s="10" t="s">
+        <v>112</v>
+      </c>
+      <c r="B24" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="C24" s="8" t="s">
-        <v>124</v>
-      </c>
-      <c r="D24" s="8" t="s">
+      <c r="C24" s="10" t="s">
+        <v>113</v>
+      </c>
+      <c r="D24" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E24" s="50">
+      <c r="E24" s="43">
         <v>45953.0</v>
       </c>
-      <c r="F24" s="8" t="s">
+      <c r="F24" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G24" s="8">
+      <c r="G24" s="10">
         <v>12.0</v>
       </c>
-      <c r="H24" s="8">
+      <c r="H24" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I24" s="8">
+      <c r="I24" s="10">
         <v>2048.0</v>
       </c>
       <c r="J24" s="14">
@@ -9030,7 +9030,7 @@
       <c r="K24" s="14">
         <v>68405.66</v>
       </c>
-      <c r="L24" s="8">
+      <c r="L24" s="10">
         <v>0.0</v>
       </c>
       <c r="AB24" s="2"/>
@@ -9042,32 +9042,32 @@
       <c r="AH24" s="2"/>
     </row>
     <row r="25">
-      <c r="A25" s="8" t="s">
-        <v>127</v>
-      </c>
-      <c r="B25" s="8" t="s">
-        <v>128</v>
-      </c>
-      <c r="C25" s="8" t="s">
-        <v>129</v>
-      </c>
-      <c r="D25" s="8" t="s">
+      <c r="A25" s="10" t="s">
+        <v>115</v>
+      </c>
+      <c r="B25" s="10" t="s">
+        <v>116</v>
+      </c>
+      <c r="C25" s="10" t="s">
+        <v>117</v>
+      </c>
+      <c r="D25" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E25" s="50">
+      <c r="E25" s="43">
         <v>45975.0</v>
       </c>
-      <c r="F25" s="8" t="s">
+      <c r="F25" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G25" s="8">
+      <c r="G25" s="10">
         <v>12.0</v>
       </c>
-      <c r="H25" s="8">
+      <c r="H25" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I25" s="8" t="s">
-        <v>120</v>
+      <c r="I25" s="10" t="s">
+        <v>111</v>
       </c>
       <c r="J25" s="14">
         <v>1157673.06</v>
@@ -9075,7 +9075,7 @@
       <c r="K25" s="14">
         <v>1157673.06</v>
       </c>
-      <c r="L25" s="8">
+      <c r="L25" s="10">
         <v>0.0</v>
       </c>
       <c r="AB25" s="2"/>
@@ -9087,31 +9087,31 @@
       <c r="AH25" s="2"/>
     </row>
     <row r="26">
-      <c r="A26" s="8" t="s">
-        <v>132</v>
-      </c>
-      <c r="B26" s="8" t="s">
+      <c r="A26" s="10" t="s">
+        <v>119</v>
+      </c>
+      <c r="B26" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="C26" s="8" t="s">
-        <v>134</v>
-      </c>
-      <c r="D26" s="8" t="s">
+      <c r="C26" s="10" t="s">
+        <v>121</v>
+      </c>
+      <c r="D26" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E26" s="50">
+      <c r="E26" s="43">
         <v>45989.0</v>
       </c>
-      <c r="F26" s="8" t="s">
+      <c r="F26" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G26" s="8">
+      <c r="G26" s="10">
         <v>12.0</v>
       </c>
-      <c r="H26" s="8">
+      <c r="H26" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I26" s="8">
+      <c r="I26" s="10">
         <v>2048.0</v>
       </c>
       <c r="J26" s="14">
@@ -9120,7 +9120,7 @@
       <c r="K26" s="14">
         <v>34065.36</v>
       </c>
-      <c r="L26" s="8">
+      <c r="L26" s="10">
         <v>0.0</v>
       </c>
       <c r="AB26" s="2"/>
@@ -9132,31 +9132,31 @@
       <c r="AH26" s="2"/>
     </row>
     <row r="27">
-      <c r="A27" s="8" t="s">
-        <v>135</v>
-      </c>
-      <c r="B27" s="8" t="s">
-        <v>137</v>
-      </c>
-      <c r="C27" s="8" t="s">
-        <v>138</v>
-      </c>
-      <c r="D27" s="8" t="s">
+      <c r="A27" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="B27" s="10" t="s">
+        <v>124</v>
+      </c>
+      <c r="C27" s="10" t="s">
+        <v>125</v>
+      </c>
+      <c r="D27" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E27" s="12">
+      <c r="E27" s="13">
         <v>46104.0</v>
       </c>
-      <c r="F27" s="8" t="s">
+      <c r="F27" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G27" s="8">
+      <c r="G27" s="10">
         <v>12.0</v>
       </c>
-      <c r="H27" s="8">
+      <c r="H27" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I27" s="8">
+      <c r="I27" s="10">
         <v>2048.0</v>
       </c>
       <c r="J27" s="14">
@@ -9177,37 +9177,37 @@
       <c r="AH27" s="2"/>
     </row>
     <row r="28">
-      <c r="A28" s="8" t="s">
-        <v>140</v>
-      </c>
-      <c r="B28" s="8" t="s">
-        <v>141</v>
-      </c>
-      <c r="C28" s="8" t="s">
-        <v>142</v>
-      </c>
-      <c r="D28" s="8" t="s">
+      <c r="A28" s="10" t="s">
+        <v>129</v>
+      </c>
+      <c r="B28" s="10" t="s">
+        <v>130</v>
+      </c>
+      <c r="C28" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="D28" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E28" s="12">
+      <c r="E28" s="13">
         <v>46120.0</v>
       </c>
-      <c r="F28" s="8" t="s">
+      <c r="F28" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G28" s="8">
+      <c r="G28" s="10">
         <v>12.0</v>
       </c>
-      <c r="H28" s="8">
+      <c r="H28" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I28" s="8" t="s">
+      <c r="I28" s="10" t="s">
         <v>48</v>
       </c>
       <c r="J28" s="14">
         <v>1912292.52</v>
       </c>
-      <c r="K28" s="8">
+      <c r="K28" s="10">
         <v>0.0</v>
       </c>
       <c r="L28" s="14">
@@ -9222,37 +9222,37 @@
       <c r="AH28" s="2"/>
     </row>
     <row r="29">
-      <c r="A29" s="8" t="s">
-        <v>145</v>
-      </c>
-      <c r="B29" s="8" t="s">
-        <v>146</v>
-      </c>
-      <c r="C29" s="8" t="s">
-        <v>147</v>
-      </c>
-      <c r="D29" s="8" t="s">
+      <c r="A29" s="10" t="s">
+        <v>133</v>
+      </c>
+      <c r="B29" s="10" t="s">
+        <v>134</v>
+      </c>
+      <c r="C29" s="10" t="s">
+        <v>135</v>
+      </c>
+      <c r="D29" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E29" s="12">
+      <c r="E29" s="13">
         <v>46196.0</v>
       </c>
-      <c r="F29" s="8" t="s">
+      <c r="F29" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G29" s="8">
+      <c r="G29" s="10">
         <v>12.0</v>
       </c>
-      <c r="H29" s="8">
+      <c r="H29" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I29" s="8">
+      <c r="I29" s="10">
         <v>2048.0</v>
       </c>
       <c r="J29" s="14">
         <v>1496713.48</v>
       </c>
-      <c r="K29" s="8">
+      <c r="K29" s="10">
         <v>0.0</v>
       </c>
       <c r="L29" s="14">
@@ -9267,37 +9267,37 @@
       <c r="AH29" s="2"/>
     </row>
     <row r="30">
-      <c r="A30" s="8" t="s">
-        <v>149</v>
-      </c>
-      <c r="B30" s="8" t="s">
-        <v>150</v>
-      </c>
-      <c r="C30" s="8" t="s">
-        <v>151</v>
-      </c>
-      <c r="D30" s="8" t="s">
+      <c r="A30" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="B30" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="C30" s="10" t="s">
+        <v>140</v>
+      </c>
+      <c r="D30" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E30" s="12">
+      <c r="E30" s="13">
         <v>46205.0</v>
       </c>
-      <c r="F30" s="8" t="s">
+      <c r="F30" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G30" s="8">
+      <c r="G30" s="10">
         <v>12.0</v>
       </c>
-      <c r="H30" s="8">
+      <c r="H30" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I30" s="8" t="s">
+      <c r="I30" s="10" t="s">
         <v>43</v>
       </c>
       <c r="J30" s="14">
         <v>624166.14</v>
       </c>
-      <c r="K30" s="8">
+      <c r="K30" s="10">
         <v>0.0</v>
       </c>
       <c r="L30" s="14">
@@ -9312,37 +9312,37 @@
       <c r="AH30" s="2"/>
     </row>
     <row r="31">
-      <c r="A31" s="8" t="s">
-        <v>153</v>
-      </c>
-      <c r="B31" s="8" t="s">
-        <v>154</v>
-      </c>
-      <c r="C31" s="8" t="s">
-        <v>155</v>
-      </c>
-      <c r="D31" s="8" t="s">
+      <c r="A31" s="10" t="s">
+        <v>143</v>
+      </c>
+      <c r="B31" s="10" t="s">
+        <v>144</v>
+      </c>
+      <c r="C31" s="10" t="s">
+        <v>145</v>
+      </c>
+      <c r="D31" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E31" s="12">
+      <c r="E31" s="13">
         <v>46205.0</v>
       </c>
-      <c r="F31" s="8" t="s">
+      <c r="F31" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G31" s="8">
+      <c r="G31" s="10">
         <v>12.0</v>
       </c>
-      <c r="H31" s="8">
+      <c r="H31" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I31" s="8" t="s">
-        <v>120</v>
+      <c r="I31" s="10" t="s">
+        <v>111</v>
       </c>
       <c r="J31" s="14">
         <v>18462.36</v>
       </c>
-      <c r="K31" s="8">
+      <c r="K31" s="10">
         <v>0.0</v>
       </c>
       <c r="L31" s="14">
@@ -9357,37 +9357,37 @@
       <c r="AH31" s="2"/>
     </row>
     <row r="32">
-      <c r="A32" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="B32" s="8" t="s">
-        <v>154</v>
+      <c r="A32" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="B32" s="10" t="s">
+        <v>144</v>
       </c>
       <c r="C32" s="14" t="s">
-        <v>159</v>
-      </c>
-      <c r="D32" s="8" t="s">
+        <v>149</v>
+      </c>
+      <c r="D32" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E32" s="12">
+      <c r="E32" s="13">
         <v>46213.0</v>
       </c>
-      <c r="F32" s="8" t="s">
+      <c r="F32" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G32" s="8">
+      <c r="G32" s="10">
         <v>12.0</v>
       </c>
-      <c r="H32" s="8">
+      <c r="H32" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I32" s="8" t="s">
-        <v>120</v>
+      <c r="I32" s="10" t="s">
+        <v>111</v>
       </c>
       <c r="J32" s="14">
         <v>1530656.62</v>
       </c>
-      <c r="K32" s="8">
+      <c r="K32" s="10">
         <v>0.0</v>
       </c>
       <c r="L32" s="14">
@@ -9402,37 +9402,37 @@
       <c r="AH32" s="2"/>
     </row>
     <row r="33">
-      <c r="A33" s="8" t="s">
-        <v>161</v>
-      </c>
-      <c r="B33" s="8" t="s">
-        <v>146</v>
+      <c r="A33" s="10" t="s">
+        <v>151</v>
+      </c>
+      <c r="B33" s="10" t="s">
+        <v>134</v>
       </c>
       <c r="C33" s="14" t="s">
-        <v>163</v>
-      </c>
-      <c r="D33" s="8" t="s">
+        <v>153</v>
+      </c>
+      <c r="D33" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E33" s="12">
+      <c r="E33" s="13">
         <v>46227.0</v>
       </c>
-      <c r="F33" s="8" t="s">
+      <c r="F33" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G33" s="8">
+      <c r="G33" s="10">
         <v>12.0</v>
       </c>
-      <c r="H33" s="8">
+      <c r="H33" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I33" s="8">
+      <c r="I33" s="10">
         <v>2048.0</v>
       </c>
       <c r="J33" s="14">
         <v>173846.38</v>
       </c>
-      <c r="K33" s="8">
+      <c r="K33" s="10">
         <v>0.0</v>
       </c>
       <c r="L33" s="14">
@@ -9447,37 +9447,37 @@
       <c r="AH33" s="2"/>
     </row>
     <row r="34">
-      <c r="A34" s="8" t="s">
-        <v>164</v>
-      </c>
-      <c r="B34" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="C34" s="8" t="s">
-        <v>167</v>
-      </c>
-      <c r="D34" s="8" t="s">
+      <c r="A34" s="10" t="s">
+        <v>156</v>
+      </c>
+      <c r="B34" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="C34" s="10" t="s">
+        <v>158</v>
+      </c>
+      <c r="D34" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E34" s="12">
+      <c r="E34" s="13">
         <v>46240.0</v>
       </c>
-      <c r="F34" s="8" t="s">
+      <c r="F34" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G34" s="8">
+      <c r="G34" s="10">
         <v>12.0</v>
       </c>
-      <c r="H34" s="8">
+      <c r="H34" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I34" s="8" t="s">
-        <v>168</v>
+      <c r="I34" s="10" t="s">
+        <v>159</v>
       </c>
       <c r="J34" s="14">
         <v>236343.68</v>
       </c>
-      <c r="K34" s="8">
+      <c r="K34" s="10">
         <v>0.0</v>
       </c>
       <c r="L34" s="14">

</xml_diff>

<commit_message>
Atualização automática: pagamentos (14/08/2026 12:59)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/01_Bases_Originais/005_CELOG_2025/005_CELOG-PAMALS_2025 online.xlsx
+++ b/Contrato 005/Dashboard/01_Bases_Originais/005_CELOG_2025/005_CELOG-PAMALS_2025 online.xlsx
@@ -63,120 +63,156 @@
     <t>UG Executora</t>
   </si>
   <si>
+    <t>UG Responsável</t>
+  </si>
+  <si>
+    <t>UG Fiscalizadora</t>
+  </si>
+  <si>
+    <t>Prazo Final de Execução</t>
+  </si>
+  <si>
+    <t>Prazo Final de Vigência</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Ação</t>
+  </si>
+  <si>
+    <t>PAG</t>
+  </si>
+  <si>
+    <t>Moeda</t>
+  </si>
+  <si>
+    <t>Valor Total do Contrato</t>
+  </si>
+  <si>
+    <t>Valor a Empenhar</t>
+  </si>
+  <si>
+    <t>Valor Empenhado</t>
+  </si>
+  <si>
+    <t>Valor Liquidado</t>
+  </si>
+  <si>
+    <t>Saldo (Valor a Faturar)</t>
+  </si>
+  <si>
     <t>2025NE000369</t>
   </si>
   <si>
-    <t>UG Responsável</t>
+    <t>Fornecedor</t>
+  </si>
+  <si>
+    <t>Tipo Despesa /Receita</t>
   </si>
   <si>
     <t>C25516</t>
   </si>
   <si>
-    <t>UG Fiscalizadora</t>
+    <t>Abrir</t>
+  </si>
+  <si>
+    <t>Editar</t>
   </si>
   <si>
     <t>25E0387</t>
   </si>
   <si>
-    <t>Prazo Final de Execução</t>
-  </si>
-  <si>
-    <t>Prazo Final de Vigência</t>
-  </si>
-  <si>
-    <t>Status</t>
-  </si>
-  <si>
-    <t>Ação</t>
-  </si>
-  <si>
-    <t>PAG</t>
-  </si>
-  <si>
-    <t>Moeda</t>
-  </si>
-  <si>
-    <t>Valor Total do Contrato</t>
-  </si>
-  <si>
-    <t>Valor a Empenhar</t>
-  </si>
-  <si>
-    <t>Valor Empenhado</t>
-  </si>
-  <si>
-    <t>Valor Liquidado</t>
-  </si>
-  <si>
-    <t>Saldo (Valor a Faturar)</t>
-  </si>
-  <si>
-    <t>Fornecedor</t>
+    <t>005/CELOG-PAMALS/2025</t>
+  </si>
+  <si>
+    <t>CELOG</t>
+  </si>
+  <si>
+    <t>PAMALS</t>
+  </si>
+  <si>
+    <t>Vigente</t>
+  </si>
+  <si>
+    <t>2048 20YJ 21EM 219C 20SP 20X7 2000</t>
+  </si>
+  <si>
+    <t>67101.001510/2024-12</t>
+  </si>
+  <si>
+    <t>R$</t>
   </si>
   <si>
     <t>2025NE000371</t>
   </si>
   <si>
-    <t>Tipo Despesa /Receita</t>
-  </si>
-  <si>
-    <t>Abrir</t>
-  </si>
-  <si>
     <t>25E0389</t>
   </si>
   <si>
-    <t>Editar</t>
-  </si>
-  <si>
-    <t>005/CELOG-PAMALS/2025</t>
-  </si>
-  <si>
-    <t>CELOG</t>
-  </si>
-  <si>
-    <t>PAMALS</t>
-  </si>
-  <si>
-    <t>Vigente</t>
+    <t>VEE ONE-MANUTENCAO E SERVICOS TECNICOS LTDA</t>
   </si>
   <si>
     <t>2025NE000413</t>
   </si>
   <si>
-    <t>2048 20YJ 21EM 219C 20SP 20X7 2000</t>
-  </si>
-  <si>
     <t>C25501</t>
   </si>
   <si>
     <t>25E0403</t>
   </si>
   <si>
-    <t>67101.001510/2024-12</t>
-  </si>
-  <si>
-    <t>R$</t>
+    <t>Módulo</t>
   </si>
   <si>
     <t>20SP</t>
   </si>
   <si>
-    <t>VEE ONE-MANUTENCAO E SERVICOS TECNICOS LTDA</t>
+    <t>Referência</t>
+  </si>
+  <si>
+    <t>Nº recibo</t>
+  </si>
+  <si>
+    <t>Nº</t>
   </si>
   <si>
     <t>2025NE000414</t>
   </si>
   <si>
+    <t>Data</t>
+  </si>
+  <si>
     <t>C25525</t>
   </si>
   <si>
     <t>25E0431</t>
   </si>
   <si>
+    <t>Empenho</t>
+  </si>
+  <si>
+    <t>Observações</t>
+  </si>
+  <si>
+    <t>Vencimento</t>
+  </si>
+  <si>
+    <t>Valor das Nfs</t>
+  </si>
+  <si>
     <t>21EM</t>
   </si>
   <si>
+    <t>Ordem de Pagamento</t>
+  </si>
+  <si>
+    <t>Faturado</t>
+  </si>
+  <si>
+    <t>Pendente</t>
+  </si>
+  <si>
     <t>2025NE000559</t>
   </si>
   <si>
@@ -186,57 +222,36 @@
     <t>25E0524</t>
   </si>
   <si>
-    <t>Módulo</t>
+    <t>FEV/25</t>
+  </si>
+  <si>
+    <t>-</t>
   </si>
   <si>
     <t>20X7</t>
   </si>
   <si>
-    <t>Referência</t>
-  </si>
-  <si>
-    <t>Nº recibo</t>
-  </si>
-  <si>
-    <t>Nº</t>
+    <t xml:space="preserve">2025NE000369 </t>
   </si>
   <si>
     <t>2025NE000770</t>
   </si>
   <si>
-    <t>Data</t>
-  </si>
-  <si>
     <t>25E0731</t>
   </si>
   <si>
-    <t>Empenho</t>
-  </si>
-  <si>
-    <t>Observações</t>
-  </si>
-  <si>
-    <t>Vencimento</t>
-  </si>
-  <si>
-    <t>Valor das Nfs</t>
-  </si>
-  <si>
-    <t>Ordem de Pagamento</t>
-  </si>
-  <si>
-    <t>Faturado</t>
+    <t>2025NP001980</t>
   </si>
   <si>
     <t>2025NE000774</t>
   </si>
   <si>
-    <t>Pendente</t>
-  </si>
-  <si>
     <t>25E0737</t>
   </si>
   <si>
+    <t>MAR/25</t>
+  </si>
+  <si>
     <t>2025NE000843</t>
   </si>
   <si>
@@ -246,118 +261,58 @@
     <t>25E0787</t>
   </si>
   <si>
+    <t>2025NE000367, 2025NE000369, 2025NE000371, 2025NE000413</t>
+  </si>
+  <si>
     <t>219C</t>
   </si>
   <si>
-    <t>FEV/25</t>
+    <t>2025NP001979</t>
   </si>
   <si>
     <t>2025NE001065</t>
   </si>
   <si>
-    <t>-</t>
-  </si>
-  <si>
     <t>25E0999</t>
   </si>
   <si>
-    <t xml:space="preserve">2025NE000369 </t>
+    <t>ABR/25</t>
+  </si>
+  <si>
+    <t>2025NE000413, 2025NE000414, 2025NE000559</t>
+  </si>
+  <si>
+    <t>2025NP002341</t>
   </si>
   <si>
     <t>2025NE001200</t>
   </si>
   <si>
+    <t>MAI/25</t>
+  </si>
+  <si>
     <t>C25590</t>
   </si>
   <si>
     <t>25E1128</t>
   </si>
   <si>
-    <t>2025NP001980</t>
-  </si>
-  <si>
     <t>2025NE001598</t>
   </si>
   <si>
+    <t>2025NP002884</t>
+  </si>
+  <si>
     <t>C25814</t>
   </si>
   <si>
     <t>25E1446</t>
   </si>
   <si>
+    <t>JUN/25</t>
+  </si>
+  <si>
     <t>2025NE001627</t>
-  </si>
-  <si>
-    <t>25E1475</t>
-  </si>
-  <si>
-    <t>2025NE001629</t>
-  </si>
-  <si>
-    <t>C25820</t>
-  </si>
-  <si>
-    <t>25E1477</t>
-  </si>
-  <si>
-    <t>MAR/25</t>
-  </si>
-  <si>
-    <t>2025NE000367, 2025NE000369, 2025NE000371, 2025NE000413</t>
-  </si>
-  <si>
-    <t>2025NE001687</t>
-  </si>
-  <si>
-    <t>25E1535</t>
-  </si>
-  <si>
-    <t>2025NP001979</t>
-  </si>
-  <si>
-    <t>2025NE001688</t>
-  </si>
-  <si>
-    <t>25E1536</t>
-  </si>
-  <si>
-    <t>ABR/25</t>
-  </si>
-  <si>
-    <t>2025NE000413, 2025NE000414, 2025NE000559</t>
-  </si>
-  <si>
-    <t>2025NE001689</t>
-  </si>
-  <si>
-    <t>25E1537</t>
-  </si>
-  <si>
-    <t>2025NP002341</t>
-  </si>
-  <si>
-    <t>2025NE001690</t>
-  </si>
-  <si>
-    <t>25E1538</t>
-  </si>
-  <si>
-    <t>MAI/25</t>
-  </si>
-  <si>
-    <t>2025NP002884</t>
-  </si>
-  <si>
-    <t>2025NE001823</t>
-  </si>
-  <si>
-    <t>C25865</t>
-  </si>
-  <si>
-    <t>25E1666</t>
-  </si>
-  <si>
-    <t>JUN/25</t>
   </si>
   <si>
     <t>2025NE000005,
@@ -366,28 +321,22 @@
 2025NE000774</t>
   </si>
   <si>
-    <t>2025NE001828</t>
-  </si>
-  <si>
-    <t>C25869</t>
-  </si>
-  <si>
-    <t>25E1667</t>
+    <t>25E1475</t>
   </si>
   <si>
     <t>2025NP400522</t>
   </si>
   <si>
-    <t>20YJ</t>
-  </si>
-  <si>
     <t>JUL/25</t>
   </si>
   <si>
-    <t>2025NE001830</t>
-  </si>
-  <si>
-    <t>25E1669</t>
+    <t>2025NE001629</t>
+  </si>
+  <si>
+    <t>C25820</t>
+  </si>
+  <si>
+    <t>25E1477</t>
   </si>
   <si>
     <t>2025NE000843, 2025NE001200</t>
@@ -396,56 +345,125 @@
     <t>2025NP003724</t>
   </si>
   <si>
-    <t>2025NE002200</t>
-  </si>
-  <si>
-    <t>C25863</t>
-  </si>
-  <si>
-    <t>25E2021</t>
+    <t>2025NE001687</t>
   </si>
   <si>
     <t>AGO/25</t>
   </si>
   <si>
-    <t>2025NE002237</t>
-  </si>
-  <si>
-    <t>25E2058</t>
+    <t>25E1535</t>
   </si>
   <si>
     <t>2025NP004558</t>
   </si>
   <si>
-    <t>2026NE000330</t>
-  </si>
-  <si>
-    <t>C26163</t>
-  </si>
-  <si>
-    <t>26E0320</t>
+    <t>2025NE001688</t>
+  </si>
+  <si>
+    <t>25E1536</t>
   </si>
   <si>
     <t>SET/25</t>
+  </si>
+  <si>
+    <t>2025NE001689</t>
+  </si>
+  <si>
+    <t>25E1537</t>
   </si>
   <si>
     <t>2025NE001688 
 2025NE001828</t>
   </si>
   <si>
+    <t>2025NE001690</t>
+  </si>
+  <si>
+    <t>25E1538</t>
+  </si>
+  <si>
+    <t>2025NP004897</t>
+  </si>
+  <si>
+    <t>2025NE001823</t>
+  </si>
+  <si>
+    <t>C25865</t>
+  </si>
+  <si>
+    <t>25E1666</t>
+  </si>
+  <si>
+    <t>OUT/25</t>
+  </si>
+  <si>
+    <t>2025NE001688, 2025NE001828, 2025NE002200</t>
+  </si>
+  <si>
+    <t>2025NE001828</t>
+  </si>
+  <si>
+    <t>C25869</t>
+  </si>
+  <si>
+    <t>25E1667</t>
+  </si>
+  <si>
+    <t>20YJ</t>
+  </si>
+  <si>
+    <t>2025NP004932</t>
+  </si>
+  <si>
+    <t>2025NE001830</t>
+  </si>
+  <si>
+    <t>25E1669</t>
+  </si>
+  <si>
+    <t>NOV/25</t>
+  </si>
+  <si>
+    <t>2025NE002200</t>
+  </si>
+  <si>
+    <t>C25863</t>
+  </si>
+  <si>
+    <t>25E2021</t>
+  </si>
+  <si>
+    <t>2025NE001687, 2025NE001689, 2025NE001690, 2025NE001823, 2025NE001830, 2025NE002237</t>
+  </si>
+  <si>
+    <t>2025NE002237</t>
+  </si>
+  <si>
+    <t>2026NP400440</t>
+  </si>
+  <si>
+    <t>25E2058</t>
+  </si>
+  <si>
+    <t>2026NE000330</t>
+  </si>
+  <si>
+    <t>C26163</t>
+  </si>
+  <si>
+    <t>26E0320</t>
+  </si>
+  <si>
     <t>2026NE000388</t>
   </si>
   <si>
     <t>C26193</t>
   </si>
   <si>
-    <t>2025NP004897</t>
-  </si>
-  <si>
     <t>26E0375</t>
   </si>
   <si>
-    <t>OUT/25</t>
+    <t>DEZ/25</t>
   </si>
   <si>
     <t>2026NE000748</t>
@@ -457,27 +475,21 @@
     <t>26E0709</t>
   </si>
   <si>
-    <t>2025NE001688, 2025NE001828, 2025NE002200</t>
-  </si>
-  <si>
-    <t>2025NP004932</t>
+    <t>2025NE001065, 2025NE002200</t>
   </si>
   <si>
     <t>2026NE000816</t>
   </si>
   <si>
+    <t>2026NP400412</t>
+  </si>
+  <si>
     <t>C26324</t>
   </si>
   <si>
     <t>26E0776</t>
   </si>
   <si>
-    <t>NOV/25</t>
-  </si>
-  <si>
-    <t>2025NE001687, 2025NE001689, 2025NE001690, 2025NE001823, 2025NE001830, 2025NE002237</t>
-  </si>
-  <si>
     <t>2026NE000817</t>
   </si>
   <si>
@@ -487,7 +499,7 @@
     <t>26E0777</t>
   </si>
   <si>
-    <t>2026NP400440</t>
+    <t>JAN/26</t>
   </si>
   <si>
     <t>2026NE000842</t>
@@ -496,22 +508,13 @@
     <t>26E0803</t>
   </si>
   <si>
-    <t>DEZ/25</t>
-  </si>
-  <si>
-    <t>2025NE001065, 2025NE002200</t>
-  </si>
-  <si>
     <t>2026NE000944</t>
   </si>
   <si>
-    <t>2026NP400412</t>
-  </si>
-  <si>
     <t>26E0906</t>
   </si>
   <si>
-    <t>JAN/26</t>
+    <t>2026NP401035</t>
   </si>
   <si>
     <t>2026NE001015</t>
@@ -524,9 +527,6 @@
   </si>
   <si>
     <t>20XV</t>
-  </si>
-  <si>
-    <t>2026NP401035</t>
   </si>
   <si>
     <t>FEV/26</t>
@@ -737,13 +737,13 @@
       <b/>
       <sz val="10.0"/>
       <color theme="1"/>
-      <name val="Century Gothic"/>
+      <name val="Arial"/>
     </font>
     <font>
       <b/>
       <sz val="10.0"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Century Gothic"/>
     </font>
     <font>
       <sz val="10.0"/>
@@ -898,10 +898,13 @@
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
     <xf borderId="0" fillId="5" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="11" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -909,9 +912,6 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="11" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
@@ -953,28 +953,28 @@
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="6" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="7" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment vertical="center"/>
     </xf>
     <xf borderId="2" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="7" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="6" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -986,20 +986,20 @@
     <xf borderId="1" fillId="0" fontId="8" numFmtId="166" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="165" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="1" fillId="7" fontId="9" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="5" fontId="9" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="8" fontId="7" numFmtId="168" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="8" fontId="6" numFmtId="168" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="3" fillId="0" fontId="10" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="1" fillId="8" fontId="9" numFmtId="168" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="165" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="1" fillId="0" fontId="8" numFmtId="166" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
@@ -1015,14 +1015,14 @@
     <xf borderId="1" fillId="8" fontId="9" numFmtId="168" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="170" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="7" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="6" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="170" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="1" fillId="9" fontId="9" numFmtId="168" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
@@ -1037,13 +1037,13 @@
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="4" fillId="0" fontId="10" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="1" fillId="0" fontId="7" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="6" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="7" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="6" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="7" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="6" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="5" fontId="9" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
@@ -1052,7 +1052,7 @@
     <xf borderId="1" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="7" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="6" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="5" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -1444,18 +1444,18 @@
     </row>
     <row r="2" ht="59.25" customHeight="1">
       <c r="A2" s="4"/>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="V2" s="9"/>
-      <c r="W2" s="10"/>
-      <c r="X2" s="10"/>
-      <c r="Y2" s="10"/>
-      <c r="Z2" s="10"/>
-      <c r="AA2" s="10"/>
-      <c r="AB2" s="10"/>
-      <c r="AC2" s="10"/>
-      <c r="AD2" s="10"/>
+      <c r="V2" s="10"/>
+      <c r="W2" s="11"/>
+      <c r="X2" s="11"/>
+      <c r="Y2" s="11"/>
+      <c r="Z2" s="11"/>
+      <c r="AA2" s="11"/>
+      <c r="AB2" s="11"/>
+      <c r="AC2" s="11"/>
+      <c r="AD2" s="11"/>
     </row>
     <row r="3" ht="12.75" customHeight="1">
       <c r="A3" s="1"/>
@@ -1491,55 +1491,55 @@
         <v>10</v>
       </c>
       <c r="E4" s="16" t="s">
+        <v>11</v>
+      </c>
+      <c r="F4" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="F4" s="16" t="s">
+      <c r="G4" s="17" t="s">
+        <v>13</v>
+      </c>
+      <c r="H4" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="G4" s="17" t="s">
+      <c r="I4" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="J4" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="H4" s="17" t="s">
+      <c r="K4" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="I4" s="16" t="s">
+      <c r="L4" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="J4" s="16" t="s">
+      <c r="M4" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="K4" s="16" t="s">
+      <c r="N4" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="L4" s="16" t="s">
+      <c r="O4" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="M4" s="17" t="s">
+      <c r="P4" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="N4" s="17" t="s">
+      <c r="Q4" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="O4" s="17" t="s">
-        <v>24</v>
-      </c>
-      <c r="P4" s="17" t="s">
+      <c r="R4" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="Q4" s="17" t="s">
+      <c r="S4" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="R4" s="16" t="s">
-        <v>27</v>
-      </c>
-      <c r="S4" s="16" t="s">
+      <c r="T4" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="U4" s="16" t="s">
         <v>29</v>
-      </c>
-      <c r="T4" s="16" t="s">
-        <v>30</v>
-      </c>
-      <c r="U4" s="16" t="s">
-        <v>32</v>
       </c>
       <c r="V4" s="3"/>
     </row>
@@ -1548,16 +1548,16 @@
       <c r="B5" s="15"/>
       <c r="C5" s="18"/>
       <c r="D5" s="19" t="s">
+        <v>31</v>
+      </c>
+      <c r="E5" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="F5" s="19" t="s">
         <v>33</v>
       </c>
-      <c r="E5" s="19" t="s">
-        <v>34</v>
-      </c>
-      <c r="F5" s="19" t="s">
-        <v>35</v>
-      </c>
       <c r="G5" s="19" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="H5" s="20">
         <v>1564.0</v>
@@ -1566,16 +1566,16 @@
         <v>1564.0</v>
       </c>
       <c r="J5" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="K5" s="19" t="s">
+        <v>35</v>
+      </c>
+      <c r="L5" s="19" t="s">
         <v>36</v>
       </c>
-      <c r="K5" s="19" t="s">
-        <v>38</v>
-      </c>
-      <c r="L5" s="19" t="s">
-        <v>41</v>
-      </c>
       <c r="M5" s="19" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="N5" s="21">
         <v>9.165159737E7</v>
@@ -1593,7 +1593,7 @@
         <v>1.085943044E7</v>
       </c>
       <c r="S5" s="19" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="V5" s="3"/>
     </row>
@@ -1615,54 +1615,54 @@
       <c r="I7" s="25"/>
       <c r="J7" s="25"/>
       <c r="K7" s="25"/>
-      <c r="L7" s="27"/>
+      <c r="L7" s="26"/>
       <c r="M7" s="25"/>
       <c r="N7" s="25"/>
       <c r="O7" s="25"/>
-      <c r="P7" s="28"/>
+      <c r="P7" s="27"/>
       <c r="V7" s="3"/>
     </row>
     <row r="8" ht="12.75" customHeight="1">
       <c r="A8" s="23"/>
       <c r="B8" s="23"/>
-      <c r="C8" s="29" t="s">
-        <v>52</v>
-      </c>
-      <c r="D8" s="29" t="s">
+      <c r="C8" s="28" t="s">
+        <v>44</v>
+      </c>
+      <c r="D8" s="28" t="s">
+        <v>46</v>
+      </c>
+      <c r="E8" s="29" t="s">
+        <v>47</v>
+      </c>
+      <c r="F8" s="28" t="s">
+        <v>48</v>
+      </c>
+      <c r="G8" s="28" t="s">
+        <v>50</v>
+      </c>
+      <c r="H8" s="28" t="s">
+        <v>53</v>
+      </c>
+      <c r="I8" s="29" t="s">
         <v>54</v>
       </c>
-      <c r="E8" s="30" t="s">
+      <c r="J8" s="28" t="s">
         <v>55</v>
       </c>
-      <c r="F8" s="29" t="s">
+      <c r="K8" s="28" t="s">
         <v>56</v>
       </c>
-      <c r="G8" s="29" t="s">
+      <c r="L8" s="30" t="s">
         <v>58</v>
       </c>
-      <c r="H8" s="29" t="s">
+      <c r="M8" s="29" t="s">
+        <v>59</v>
+      </c>
+      <c r="N8" s="28" t="s">
         <v>60</v>
       </c>
-      <c r="I8" s="30" t="s">
-        <v>61</v>
-      </c>
-      <c r="J8" s="29" t="s">
-        <v>62</v>
-      </c>
-      <c r="K8" s="29" t="s">
-        <v>63</v>
-      </c>
-      <c r="L8" s="31" t="s">
-        <v>64</v>
-      </c>
-      <c r="M8" s="30" t="s">
-        <v>65</v>
-      </c>
-      <c r="N8" s="29" t="s">
-        <v>67</v>
-      </c>
-      <c r="O8" s="29"/>
-      <c r="P8" s="28"/>
+      <c r="O8" s="28"/>
+      <c r="P8" s="27"/>
       <c r="V8" s="3"/>
     </row>
     <row r="9" ht="19.5" customHeight="1">
@@ -1672,10 +1672,10 @@
         <v>1.0</v>
       </c>
       <c r="D9" s="33" t="s">
-        <v>73</v>
+        <v>64</v>
       </c>
       <c r="E9" s="34" t="s">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="F9" s="35">
         <v>594.0</v>
@@ -1684,36 +1684,36 @@
         <v>45740.0</v>
       </c>
       <c r="H9" s="35" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="I9" s="36"/>
       <c r="J9" s="36">
         <v>45778.0</v>
       </c>
-      <c r="K9" s="38">
+      <c r="K9" s="37">
         <v>748504.24</v>
       </c>
       <c r="L9" s="35" t="s">
-        <v>81</v>
-      </c>
-      <c r="M9" s="39">
+        <v>70</v>
+      </c>
+      <c r="M9" s="38">
         <f t="shared" ref="M9:M10" si="1">K9</f>
         <v>748504.24</v>
       </c>
-      <c r="N9" s="40"/>
+      <c r="N9" s="39"/>
       <c r="O9" s="25"/>
-      <c r="P9" s="28"/>
+      <c r="P9" s="27"/>
       <c r="V9" s="3"/>
     </row>
     <row r="10" ht="51.0" customHeight="1">
       <c r="A10" s="23"/>
       <c r="B10" s="23"/>
-      <c r="C10" s="41"/>
+      <c r="C10" s="40"/>
       <c r="D10" s="33" t="s">
-        <v>90</v>
+        <v>73</v>
       </c>
       <c r="E10" s="34" t="s">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="F10" s="35">
         <v>620.0</v>
@@ -1722,36 +1722,36 @@
         <v>45775.0</v>
       </c>
       <c r="H10" s="35" t="s">
-        <v>91</v>
+        <v>77</v>
       </c>
       <c r="I10" s="36"/>
       <c r="J10" s="36">
         <v>45806.0</v>
       </c>
-      <c r="K10" s="38">
+      <c r="K10" s="37">
         <v>1110378.24</v>
       </c>
       <c r="L10" s="35" t="s">
-        <v>94</v>
-      </c>
-      <c r="M10" s="39">
+        <v>79</v>
+      </c>
+      <c r="M10" s="38">
         <f t="shared" si="1"/>
         <v>1110378.24</v>
       </c>
-      <c r="N10" s="42"/>
+      <c r="N10" s="41"/>
       <c r="O10" s="25"/>
-      <c r="P10" s="28"/>
+      <c r="P10" s="27"/>
       <c r="V10" s="3"/>
     </row>
     <row r="11" ht="12.75" customHeight="1">
       <c r="A11" s="23"/>
       <c r="B11" s="23"/>
-      <c r="C11" s="41"/>
+      <c r="C11" s="40"/>
       <c r="D11" s="33" t="s">
-        <v>97</v>
+        <v>82</v>
       </c>
       <c r="E11" s="34" t="s">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="F11" s="35">
         <v>634.0</v>
@@ -1760,35 +1760,35 @@
         <v>45799.0</v>
       </c>
       <c r="H11" s="35" t="s">
-        <v>98</v>
+        <v>83</v>
       </c>
       <c r="I11" s="36"/>
       <c r="J11" s="36">
         <v>45844.0</v>
       </c>
-      <c r="K11" s="38">
+      <c r="K11" s="37">
         <v>974557.12</v>
       </c>
       <c r="L11" s="34" t="s">
-        <v>101</v>
-      </c>
-      <c r="M11" s="39">
+        <v>84</v>
+      </c>
+      <c r="M11" s="38">
         <v>974557.12</v>
       </c>
-      <c r="N11" s="42"/>
+      <c r="N11" s="41"/>
       <c r="O11" s="25"/>
-      <c r="P11" s="28"/>
+      <c r="P11" s="27"/>
       <c r="V11" s="3"/>
     </row>
     <row r="12" ht="27.75" customHeight="1">
       <c r="A12" s="23"/>
       <c r="B12" s="23"/>
-      <c r="C12" s="41"/>
+      <c r="C12" s="40"/>
       <c r="D12" s="33" t="s">
-        <v>104</v>
+        <v>86</v>
       </c>
       <c r="E12" s="34" t="s">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="F12" s="34">
         <v>660.0</v>
@@ -1797,7 +1797,7 @@
         <v>45856.0</v>
       </c>
       <c r="H12" s="44" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="I12" s="36"/>
       <c r="J12" s="36">
@@ -1807,25 +1807,25 @@
         <v>1402001.34</v>
       </c>
       <c r="L12" s="46" t="s">
-        <v>105</v>
-      </c>
-      <c r="M12" s="39">
+        <v>90</v>
+      </c>
+      <c r="M12" s="38">
         <v>1402001.34</v>
       </c>
       <c r="N12" s="47"/>
       <c r="O12" s="25"/>
-      <c r="P12" s="28"/>
+      <c r="P12" s="27"/>
       <c r="V12" s="3"/>
     </row>
     <row r="13">
       <c r="A13" s="23"/>
       <c r="B13" s="23"/>
-      <c r="C13" s="41"/>
-      <c r="D13" s="49" t="s">
-        <v>109</v>
+      <c r="C13" s="40"/>
+      <c r="D13" s="48" t="s">
+        <v>93</v>
       </c>
       <c r="E13" s="34" t="s">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="F13" s="35">
         <v>661.0</v>
@@ -1834,7 +1834,7 @@
         <v>45856.0</v>
       </c>
       <c r="H13" s="35" t="s">
-        <v>110</v>
+        <v>95</v>
       </c>
       <c r="I13" s="43"/>
       <c r="J13" s="43">
@@ -1844,25 +1844,25 @@
         <v>1223702.3</v>
       </c>
       <c r="L13" s="34" t="s">
-        <v>114</v>
-      </c>
-      <c r="M13" s="39">
+        <v>97</v>
+      </c>
+      <c r="M13" s="38">
         <v>1223702.3</v>
       </c>
       <c r="N13" s="47"/>
       <c r="O13" s="25"/>
-      <c r="P13" s="50"/>
+      <c r="P13" s="49"/>
       <c r="V13" s="3"/>
     </row>
     <row r="14">
       <c r="A14" s="23"/>
       <c r="B14" s="23"/>
-      <c r="C14" s="41"/>
-      <c r="D14" s="49" t="s">
-        <v>116</v>
+      <c r="C14" s="40"/>
+      <c r="D14" s="48" t="s">
+        <v>98</v>
       </c>
       <c r="E14" s="34" t="s">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="F14" s="34">
         <v>688.0</v>
@@ -1871,7 +1871,7 @@
         <v>45901.0</v>
       </c>
       <c r="H14" s="34" t="s">
-        <v>119</v>
+        <v>102</v>
       </c>
       <c r="I14" s="43"/>
       <c r="J14" s="43">
@@ -1881,25 +1881,25 @@
         <v>1011677.95</v>
       </c>
       <c r="L14" s="34" t="s">
-        <v>120</v>
-      </c>
-      <c r="M14" s="39">
+        <v>103</v>
+      </c>
+      <c r="M14" s="38">
         <v>1011677.95</v>
       </c>
-      <c r="N14" s="42"/>
+      <c r="N14" s="41"/>
       <c r="O14" s="25"/>
-      <c r="P14" s="28"/>
+      <c r="P14" s="27"/>
       <c r="V14" s="3"/>
     </row>
     <row r="15">
       <c r="A15" s="23"/>
       <c r="B15" s="23"/>
-      <c r="C15" s="41"/>
-      <c r="D15" s="49" t="s">
-        <v>124</v>
+      <c r="C15" s="40"/>
+      <c r="D15" s="48" t="s">
+        <v>105</v>
       </c>
       <c r="E15" s="34" t="s">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="F15" s="34">
         <v>696.0</v>
@@ -1908,7 +1908,7 @@
         <v>45923.0</v>
       </c>
       <c r="H15" s="34" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="I15" s="43"/>
       <c r="J15" s="43">
@@ -1918,9 +1918,9 @@
         <v>896744.06</v>
       </c>
       <c r="L15" s="34" t="s">
-        <v>127</v>
-      </c>
-      <c r="M15" s="39">
+        <v>107</v>
+      </c>
+      <c r="M15" s="38">
         <v>896744.06</v>
       </c>
       <c r="N15" s="47"/>
@@ -1930,12 +1930,12 @@
     <row r="16">
       <c r="A16" s="23"/>
       <c r="B16" s="23"/>
-      <c r="C16" s="41"/>
-      <c r="D16" s="49" t="s">
-        <v>131</v>
+      <c r="C16" s="40"/>
+      <c r="D16" s="48" t="s">
+        <v>110</v>
       </c>
       <c r="E16" s="34" t="s">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="F16" s="34">
         <v>704.0</v>
@@ -1944,7 +1944,7 @@
         <v>45957.0</v>
       </c>
       <c r="H16" s="34" t="s">
-        <v>132</v>
+        <v>113</v>
       </c>
       <c r="I16" s="43"/>
       <c r="J16" s="43">
@@ -1954,21 +1954,21 @@
         <v>919329.06</v>
       </c>
       <c r="L16" s="34" t="s">
-        <v>135</v>
-      </c>
-      <c r="M16" s="39">
+        <v>116</v>
+      </c>
+      <c r="M16" s="38">
         <v>919329.06</v>
       </c>
-      <c r="N16" s="42"/>
+      <c r="N16" s="41"/>
       <c r="O16" s="25"/>
       <c r="V16" s="3"/>
     </row>
     <row r="17">
       <c r="A17" s="23"/>
       <c r="B17" s="23"/>
-      <c r="C17" s="41"/>
-      <c r="D17" s="49" t="s">
-        <v>137</v>
+      <c r="C17" s="40"/>
+      <c r="D17" s="48" t="s">
+        <v>120</v>
       </c>
       <c r="E17" s="34"/>
       <c r="F17" s="34">
@@ -1978,7 +1978,7 @@
         <v>45972.0</v>
       </c>
       <c r="H17" s="34" t="s">
-        <v>141</v>
+        <v>121</v>
       </c>
       <c r="I17" s="34"/>
       <c r="J17" s="43">
@@ -1988,9 +1988,9 @@
         <v>1157009.26</v>
       </c>
       <c r="L17" s="34" t="s">
-        <v>142</v>
-      </c>
-      <c r="M17" s="39">
+        <v>126</v>
+      </c>
+      <c r="M17" s="38">
         <v>1157009.26</v>
       </c>
       <c r="N17" s="51"/>
@@ -2000,12 +2000,12 @@
     <row r="18">
       <c r="A18" s="23"/>
       <c r="B18" s="23"/>
-      <c r="C18" s="41"/>
-      <c r="D18" s="49" t="s">
-        <v>146</v>
+      <c r="C18" s="40"/>
+      <c r="D18" s="48" t="s">
+        <v>129</v>
       </c>
       <c r="E18" s="34" t="s">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="F18" s="34">
         <v>728.0</v>
@@ -2014,7 +2014,7 @@
         <v>46008.0</v>
       </c>
       <c r="H18" s="34" t="s">
-        <v>147</v>
+        <v>133</v>
       </c>
       <c r="I18" s="34"/>
       <c r="J18" s="43">
@@ -2024,28 +2024,28 @@
         <v>1214597.952</v>
       </c>
       <c r="L18" s="34" t="s">
-        <v>151</v>
-      </c>
-      <c r="M18" s="39">
+        <v>135</v>
+      </c>
+      <c r="M18" s="38">
         <v>1214597.952</v>
       </c>
       <c r="N18" s="51"/>
       <c r="O18" s="25"/>
-      <c r="R18" s="28"/>
-      <c r="S18" s="28"/>
-      <c r="T18" s="28"/>
-      <c r="U18" s="28"/>
+      <c r="R18" s="27"/>
+      <c r="S18" s="27"/>
+      <c r="T18" s="27"/>
+      <c r="U18" s="27"/>
       <c r="V18" s="52"/>
     </row>
     <row r="19">
       <c r="A19" s="23"/>
       <c r="B19" s="23"/>
-      <c r="C19" s="41"/>
-      <c r="D19" s="49" t="s">
-        <v>154</v>
+      <c r="C19" s="40"/>
+      <c r="D19" s="48" t="s">
+        <v>143</v>
       </c>
       <c r="E19" s="34" t="s">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="F19" s="34">
         <v>278.0</v>
@@ -2054,7 +2054,7 @@
         <v>46042.0</v>
       </c>
       <c r="H19" s="34" t="s">
-        <v>155</v>
+        <v>147</v>
       </c>
       <c r="I19" s="43"/>
       <c r="J19" s="43">
@@ -2064,25 +2064,25 @@
         <v>967082.09</v>
       </c>
       <c r="L19" s="34" t="s">
-        <v>157</v>
-      </c>
-      <c r="M19" s="39">
+        <v>149</v>
+      </c>
+      <c r="M19" s="38">
         <v>967082.09</v>
       </c>
       <c r="N19" s="51"/>
       <c r="O19" s="25"/>
-      <c r="R19" s="28"/>
-      <c r="S19" s="28"/>
-      <c r="T19" s="28"/>
-      <c r="U19" s="28"/>
+      <c r="R19" s="27"/>
+      <c r="S19" s="27"/>
+      <c r="T19" s="27"/>
+      <c r="U19" s="27"/>
       <c r="V19" s="52"/>
     </row>
     <row r="20">
       <c r="A20" s="23"/>
       <c r="B20" s="23"/>
-      <c r="C20" s="41"/>
-      <c r="D20" s="49" t="s">
-        <v>159</v>
+      <c r="C20" s="40"/>
+      <c r="D20" s="48" t="s">
+        <v>155</v>
       </c>
       <c r="E20" s="34"/>
       <c r="F20" s="34">
@@ -2092,7 +2092,7 @@
         <v>46078.0</v>
       </c>
       <c r="H20" s="34" t="s">
-        <v>106</v>
+        <v>117</v>
       </c>
       <c r="I20" s="43"/>
       <c r="J20" s="43">
@@ -2102,24 +2102,24 @@
         <v>719561.08</v>
       </c>
       <c r="L20" s="34" t="s">
-        <v>164</v>
-      </c>
-      <c r="M20" s="39">
+        <v>160</v>
+      </c>
+      <c r="M20" s="38">
         <v>719561.08</v>
       </c>
       <c r="N20" s="51"/>
       <c r="O20" s="25"/>
-      <c r="R20" s="28"/>
-      <c r="S20" s="28"/>
-      <c r="T20" s="28"/>
-      <c r="U20" s="28"/>
+      <c r="R20" s="27"/>
+      <c r="S20" s="27"/>
+      <c r="T20" s="27"/>
+      <c r="U20" s="27"/>
       <c r="V20" s="52"/>
     </row>
     <row r="21">
       <c r="A21" s="23"/>
       <c r="B21" s="23"/>
-      <c r="C21" s="41"/>
-      <c r="D21" s="49" t="s">
+      <c r="C21" s="40"/>
+      <c r="D21" s="48" t="s">
         <v>165</v>
       </c>
       <c r="E21" s="34"/>
@@ -2142,22 +2142,22 @@
       <c r="L21" s="34" t="s">
         <v>167</v>
       </c>
-      <c r="M21" s="39">
+      <c r="M21" s="38">
         <v>885881.08</v>
       </c>
       <c r="N21" s="51"/>
       <c r="O21" s="25"/>
-      <c r="R21" s="28"/>
-      <c r="S21" s="28"/>
-      <c r="T21" s="28"/>
-      <c r="U21" s="28"/>
+      <c r="R21" s="27"/>
+      <c r="S21" s="27"/>
+      <c r="T21" s="27"/>
+      <c r="U21" s="27"/>
       <c r="V21" s="52"/>
     </row>
     <row r="22">
       <c r="A22" s="23"/>
       <c r="B22" s="23"/>
-      <c r="C22" s="41"/>
-      <c r="D22" s="49" t="s">
+      <c r="C22" s="40"/>
+      <c r="D22" s="48" t="s">
         <v>168</v>
       </c>
       <c r="E22" s="34"/>
@@ -2180,22 +2180,22 @@
       <c r="L22" s="34" t="s">
         <v>171</v>
       </c>
-      <c r="M22" s="39" t="s">
+      <c r="M22" s="38" t="s">
         <v>170</v>
       </c>
       <c r="N22" s="51"/>
       <c r="O22" s="25"/>
-      <c r="R22" s="28"/>
-      <c r="S22" s="28"/>
-      <c r="T22" s="28"/>
-      <c r="U22" s="28"/>
+      <c r="R22" s="27"/>
+      <c r="S22" s="27"/>
+      <c r="T22" s="27"/>
+      <c r="U22" s="27"/>
       <c r="V22" s="52"/>
     </row>
     <row r="23">
       <c r="A23" s="23"/>
       <c r="B23" s="23"/>
-      <c r="C23" s="41"/>
-      <c r="D23" s="49" t="s">
+      <c r="C23" s="40"/>
+      <c r="D23" s="48" t="s">
         <v>172</v>
       </c>
       <c r="E23" s="34"/>
@@ -2218,22 +2218,22 @@
       <c r="L23" s="34" t="s">
         <v>167</v>
       </c>
-      <c r="M23" s="39">
+      <c r="M23" s="38">
         <v>1108954.4358333333</v>
       </c>
       <c r="N23" s="53"/>
       <c r="O23" s="25"/>
-      <c r="R23" s="28"/>
-      <c r="S23" s="28"/>
-      <c r="T23" s="28"/>
-      <c r="U23" s="28"/>
+      <c r="R23" s="27"/>
+      <c r="S23" s="27"/>
+      <c r="T23" s="27"/>
+      <c r="U23" s="27"/>
       <c r="V23" s="52"/>
     </row>
     <row r="24">
       <c r="A24" s="23"/>
       <c r="B24" s="23"/>
-      <c r="C24" s="41"/>
-      <c r="D24" s="49" t="s">
+      <c r="C24" s="40"/>
+      <c r="D24" s="48" t="s">
         <v>174</v>
       </c>
       <c r="E24" s="34"/>
@@ -2256,22 +2256,22 @@
       <c r="L24" s="34" t="s">
         <v>175</v>
       </c>
-      <c r="M24" s="39">
+      <c r="M24" s="38">
         <v>218206.1</v>
       </c>
       <c r="N24" s="54"/>
       <c r="O24" s="25"/>
-      <c r="R24" s="28"/>
-      <c r="S24" s="28"/>
-      <c r="T24" s="28"/>
-      <c r="U24" s="28"/>
+      <c r="R24" s="27"/>
+      <c r="S24" s="27"/>
+      <c r="T24" s="27"/>
+      <c r="U24" s="27"/>
       <c r="V24" s="52"/>
     </row>
     <row r="25">
       <c r="A25" s="23"/>
       <c r="B25" s="23"/>
-      <c r="C25" s="41"/>
-      <c r="D25" s="49" t="s">
+      <c r="C25" s="40"/>
+      <c r="D25" s="48" t="s">
         <v>176</v>
       </c>
       <c r="E25" s="34"/>
@@ -2294,22 +2294,22 @@
       <c r="L25" s="34" t="s">
         <v>177</v>
       </c>
-      <c r="M25" s="39">
+      <c r="M25" s="38">
         <v>1549250.84</v>
       </c>
       <c r="N25" s="54"/>
       <c r="O25" s="25"/>
-      <c r="R25" s="28"/>
-      <c r="S25" s="28"/>
-      <c r="T25" s="28"/>
-      <c r="U25" s="28"/>
+      <c r="R25" s="27"/>
+      <c r="S25" s="27"/>
+      <c r="T25" s="27"/>
+      <c r="U25" s="27"/>
       <c r="V25" s="52"/>
     </row>
     <row r="26">
       <c r="A26" s="23"/>
       <c r="B26" s="23"/>
       <c r="C26" s="55"/>
-      <c r="D26" s="49" t="s">
+      <c r="D26" s="48" t="s">
         <v>178</v>
       </c>
       <c r="E26" s="34"/>
@@ -2332,22 +2332,22 @@
       <c r="L26" s="34" t="s">
         <v>181</v>
       </c>
-      <c r="M26" s="39" t="s">
+      <c r="M26" s="38" t="s">
         <v>180</v>
       </c>
       <c r="N26" s="54"/>
       <c r="O26" s="25"/>
-      <c r="R26" s="28"/>
-      <c r="S26" s="28"/>
-      <c r="T26" s="28"/>
-      <c r="U26" s="28"/>
+      <c r="R26" s="27"/>
+      <c r="S26" s="27"/>
+      <c r="T26" s="27"/>
+      <c r="U26" s="27"/>
       <c r="V26" s="52"/>
     </row>
     <row r="27">
       <c r="A27" s="23"/>
       <c r="B27" s="23"/>
       <c r="C27" s="35"/>
-      <c r="D27" s="49" t="s">
+      <c r="D27" s="48" t="s">
         <v>182</v>
       </c>
       <c r="E27" s="34"/>
@@ -2358,62 +2358,62 @@
       <c r="J27" s="43"/>
       <c r="K27" s="45"/>
       <c r="L27" s="34"/>
-      <c r="M27" s="39"/>
+      <c r="M27" s="38"/>
       <c r="N27" s="54"/>
       <c r="O27" s="25"/>
-      <c r="R27" s="28"/>
-      <c r="S27" s="28"/>
-      <c r="T27" s="28"/>
-      <c r="U27" s="28"/>
+      <c r="R27" s="27"/>
+      <c r="S27" s="27"/>
+      <c r="T27" s="27"/>
+      <c r="U27" s="27"/>
       <c r="V27" s="52"/>
     </row>
     <row r="28" ht="30.75" customHeight="1">
       <c r="A28" s="23"/>
       <c r="B28" s="23"/>
-      <c r="C28" s="29" t="s">
-        <v>52</v>
-      </c>
-      <c r="D28" s="29" t="s">
-        <v>54</v>
-      </c>
-      <c r="E28" s="30" t="s">
-        <v>55</v>
-      </c>
-      <c r="F28" s="29" t="s">
+      <c r="C28" s="28" t="s">
+        <v>44</v>
+      </c>
+      <c r="D28" s="28" t="s">
+        <v>46</v>
+      </c>
+      <c r="E28" s="29" t="s">
+        <v>47</v>
+      </c>
+      <c r="F28" s="28" t="s">
+        <v>48</v>
+      </c>
+      <c r="G28" s="28"/>
+      <c r="H28" s="28" t="s">
+        <v>53</v>
+      </c>
+      <c r="I28" s="28"/>
+      <c r="J28" s="28"/>
+      <c r="K28" s="56" t="s">
         <v>56</v>
       </c>
-      <c r="G28" s="29"/>
-      <c r="H28" s="29" t="s">
+      <c r="L28" s="30" t="s">
+        <v>58</v>
+      </c>
+      <c r="M28" s="57" t="s">
+        <v>59</v>
+      </c>
+      <c r="N28" s="28" t="s">
         <v>60</v>
       </c>
-      <c r="I28" s="29"/>
-      <c r="J28" s="29"/>
-      <c r="K28" s="56" t="s">
-        <v>63</v>
-      </c>
-      <c r="L28" s="31" t="s">
-        <v>64</v>
-      </c>
-      <c r="M28" s="57" t="s">
-        <v>65</v>
-      </c>
-      <c r="N28" s="29" t="s">
-        <v>67</v>
-      </c>
       <c r="O28" s="25"/>
-      <c r="P28" s="28"/>
-      <c r="R28" s="28"/>
-      <c r="S28" s="28"/>
-      <c r="T28" s="28"/>
-      <c r="U28" s="28"/>
+      <c r="P28" s="27"/>
+      <c r="R28" s="27"/>
+      <c r="S28" s="27"/>
+      <c r="T28" s="27"/>
+      <c r="U28" s="27"/>
       <c r="V28" s="52"/>
-      <c r="W28" s="28"/>
-      <c r="X28" s="28"/>
-      <c r="Y28" s="28"/>
-      <c r="Z28" s="28"/>
-      <c r="AA28" s="28"/>
-      <c r="AB28" s="28"/>
-      <c r="AC28" s="28"/>
+      <c r="W28" s="27"/>
+      <c r="X28" s="27"/>
+      <c r="Y28" s="27"/>
+      <c r="Z28" s="27"/>
+      <c r="AA28" s="27"/>
+      <c r="AB28" s="27"/>
+      <c r="AC28" s="27"/>
     </row>
     <row r="29" ht="12.75" customHeight="1">
       <c r="A29" s="23"/>
@@ -2432,13 +2432,13 @@
         <v>45791.0</v>
       </c>
       <c r="H29" s="35" t="s">
-        <v>49</v>
+        <v>61</v>
       </c>
       <c r="I29" s="36"/>
       <c r="J29" s="36">
         <v>45834.0</v>
       </c>
-      <c r="K29" s="38">
+      <c r="K29" s="37">
         <v>188246.17</v>
       </c>
       <c r="L29" s="34" t="s">
@@ -2449,25 +2449,25 @@
       </c>
       <c r="N29" s="51"/>
       <c r="O29" s="25"/>
-      <c r="P29" s="28"/>
-      <c r="Q29" s="28"/>
-      <c r="R29" s="28"/>
-      <c r="S29" s="28"/>
-      <c r="T29" s="28"/>
-      <c r="U29" s="28"/>
+      <c r="P29" s="27"/>
+      <c r="Q29" s="27"/>
+      <c r="R29" s="27"/>
+      <c r="S29" s="27"/>
+      <c r="T29" s="27"/>
+      <c r="U29" s="27"/>
       <c r="V29" s="52"/>
-      <c r="W29" s="28"/>
-      <c r="X29" s="28"/>
-      <c r="Y29" s="28"/>
-      <c r="Z29" s="28"/>
-      <c r="AA29" s="28"/>
-      <c r="AB29" s="28"/>
-      <c r="AC29" s="28"/>
+      <c r="W29" s="27"/>
+      <c r="X29" s="27"/>
+      <c r="Y29" s="27"/>
+      <c r="Z29" s="27"/>
+      <c r="AA29" s="27"/>
+      <c r="AB29" s="27"/>
+      <c r="AC29" s="27"/>
     </row>
     <row r="30">
       <c r="A30" s="23"/>
       <c r="B30" s="23"/>
-      <c r="C30" s="41"/>
+      <c r="C30" s="40"/>
       <c r="D30" s="58" t="s">
         <v>185</v>
       </c>
@@ -2487,36 +2487,36 @@
       <c r="J30" s="43">
         <v>45955.0</v>
       </c>
-      <c r="K30" s="38">
+      <c r="K30" s="37">
         <v>112720.77</v>
       </c>
       <c r="L30" s="34" t="s">
         <v>187</v>
       </c>
-      <c r="M30" s="39">
+      <c r="M30" s="38">
         <v>112720.77</v>
       </c>
       <c r="N30" s="51"/>
       <c r="O30" s="25"/>
-      <c r="P30" s="28"/>
-      <c r="Q30" s="28"/>
-      <c r="R30" s="28"/>
-      <c r="S30" s="28"/>
-      <c r="T30" s="28"/>
-      <c r="U30" s="28"/>
+      <c r="P30" s="27"/>
+      <c r="Q30" s="27"/>
+      <c r="R30" s="27"/>
+      <c r="S30" s="27"/>
+      <c r="T30" s="27"/>
+      <c r="U30" s="27"/>
       <c r="V30" s="52"/>
-      <c r="W30" s="28"/>
-      <c r="X30" s="28"/>
-      <c r="Y30" s="28"/>
-      <c r="Z30" s="28"/>
-      <c r="AA30" s="28"/>
-      <c r="AB30" s="28"/>
-      <c r="AC30" s="28"/>
+      <c r="W30" s="27"/>
+      <c r="X30" s="27"/>
+      <c r="Y30" s="27"/>
+      <c r="Z30" s="27"/>
+      <c r="AA30" s="27"/>
+      <c r="AB30" s="27"/>
+      <c r="AC30" s="27"/>
     </row>
     <row r="31" ht="12.75" customHeight="1">
       <c r="A31" s="23"/>
       <c r="B31" s="23"/>
-      <c r="C31" s="41"/>
+      <c r="C31" s="40"/>
       <c r="D31" s="61" t="s">
         <v>188</v>
       </c>
@@ -2530,7 +2530,7 @@
         <v>45853.0</v>
       </c>
       <c r="H31" s="34" t="s">
-        <v>57</v>
+        <v>68</v>
       </c>
       <c r="I31" s="43"/>
       <c r="J31" s="43">
@@ -2542,30 +2542,30 @@
       <c r="L31" s="34" t="s">
         <v>190</v>
       </c>
-      <c r="M31" s="39">
+      <c r="M31" s="38">
         <v>378307.61</v>
       </c>
       <c r="N31" s="51"/>
       <c r="O31" s="25"/>
       <c r="P31" s="64"/>
-      <c r="Q31" s="28"/>
-      <c r="R31" s="28"/>
-      <c r="S31" s="28"/>
-      <c r="T31" s="28"/>
-      <c r="U31" s="28"/>
+      <c r="Q31" s="27"/>
+      <c r="R31" s="27"/>
+      <c r="S31" s="27"/>
+      <c r="T31" s="27"/>
+      <c r="U31" s="27"/>
       <c r="V31" s="52"/>
-      <c r="W31" s="28"/>
-      <c r="X31" s="28"/>
-      <c r="Y31" s="28"/>
-      <c r="Z31" s="28"/>
-      <c r="AA31" s="28"/>
-      <c r="AB31" s="28"/>
-      <c r="AC31" s="28"/>
+      <c r="W31" s="27"/>
+      <c r="X31" s="27"/>
+      <c r="Y31" s="27"/>
+      <c r="Z31" s="27"/>
+      <c r="AA31" s="27"/>
+      <c r="AB31" s="27"/>
+      <c r="AC31" s="27"/>
     </row>
     <row r="32" ht="60.0" customHeight="1">
       <c r="A32" s="23"/>
       <c r="B32" s="23"/>
-      <c r="C32" s="41"/>
+      <c r="C32" s="40"/>
       <c r="D32" s="61" t="s">
         <v>191</v>
       </c>
@@ -2579,42 +2579,42 @@
         <v>45910.0</v>
       </c>
       <c r="H32" s="34" t="s">
-        <v>57</v>
+        <v>68</v>
       </c>
       <c r="I32" s="43"/>
       <c r="J32" s="43">
         <v>45941.0</v>
       </c>
-      <c r="K32" s="38">
+      <c r="K32" s="37">
         <v>3315.0471000000252</v>
       </c>
       <c r="L32" s="34" t="s">
         <v>192</v>
       </c>
-      <c r="M32" s="39">
+      <c r="M32" s="38">
         <v>3315.04710000003</v>
       </c>
       <c r="N32" s="51"/>
       <c r="O32" s="25"/>
       <c r="P32" s="64"/>
-      <c r="Q32" s="28"/>
-      <c r="R32" s="28"/>
-      <c r="S32" s="28"/>
-      <c r="T32" s="28"/>
-      <c r="U32" s="28"/>
+      <c r="Q32" s="27"/>
+      <c r="R32" s="27"/>
+      <c r="S32" s="27"/>
+      <c r="T32" s="27"/>
+      <c r="U32" s="27"/>
       <c r="V32" s="52"/>
-      <c r="W32" s="28"/>
-      <c r="X32" s="28"/>
-      <c r="Y32" s="28"/>
-      <c r="Z32" s="28"/>
-      <c r="AA32" s="28"/>
-      <c r="AB32" s="28"/>
-      <c r="AC32" s="28"/>
+      <c r="W32" s="27"/>
+      <c r="X32" s="27"/>
+      <c r="Y32" s="27"/>
+      <c r="Z32" s="27"/>
+      <c r="AA32" s="27"/>
+      <c r="AB32" s="27"/>
+      <c r="AC32" s="27"/>
     </row>
     <row r="33" ht="12.75" customHeight="1">
       <c r="A33" s="23"/>
       <c r="B33" s="23"/>
-      <c r="C33" s="41"/>
+      <c r="C33" s="40"/>
       <c r="D33" s="61" t="s">
         <v>193</v>
       </c>
@@ -2628,7 +2628,7 @@
         <v>45904.0</v>
       </c>
       <c r="H33" s="34" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="I33" s="66"/>
       <c r="J33" s="66">
@@ -2640,30 +2640,30 @@
       <c r="L33" s="34" t="s">
         <v>194</v>
       </c>
-      <c r="M33" s="39">
+      <c r="M33" s="38">
         <v>198332.75</v>
       </c>
       <c r="N33" s="51"/>
       <c r="O33" s="25"/>
       <c r="P33" s="64"/>
-      <c r="Q33" s="28"/>
-      <c r="R33" s="28"/>
-      <c r="S33" s="28"/>
-      <c r="T33" s="28"/>
-      <c r="U33" s="28"/>
+      <c r="Q33" s="27"/>
+      <c r="R33" s="27"/>
+      <c r="S33" s="27"/>
+      <c r="T33" s="27"/>
+      <c r="U33" s="27"/>
       <c r="V33" s="52"/>
-      <c r="W33" s="28"/>
-      <c r="X33" s="28"/>
-      <c r="Y33" s="28"/>
-      <c r="Z33" s="28"/>
-      <c r="AA33" s="28"/>
-      <c r="AB33" s="28"/>
-      <c r="AC33" s="28"/>
+      <c r="W33" s="27"/>
+      <c r="X33" s="27"/>
+      <c r="Y33" s="27"/>
+      <c r="Z33" s="27"/>
+      <c r="AA33" s="27"/>
+      <c r="AB33" s="27"/>
+      <c r="AC33" s="27"/>
     </row>
     <row r="34" ht="12.75" customHeight="1">
       <c r="A34" s="23"/>
       <c r="B34" s="23"/>
-      <c r="C34" s="41"/>
+      <c r="C34" s="40"/>
       <c r="D34" s="61" t="s">
         <v>195</v>
       </c>
@@ -2677,7 +2677,7 @@
         <v>46008.0</v>
       </c>
       <c r="H34" s="34" t="s">
-        <v>121</v>
+        <v>130</v>
       </c>
       <c r="I34" s="66"/>
       <c r="J34" s="66">
@@ -2695,24 +2695,24 @@
       <c r="N34" s="51"/>
       <c r="O34" s="25"/>
       <c r="P34" s="64"/>
-      <c r="Q34" s="28"/>
-      <c r="R34" s="28"/>
-      <c r="S34" s="28"/>
-      <c r="T34" s="28"/>
-      <c r="U34" s="28"/>
+      <c r="Q34" s="27"/>
+      <c r="R34" s="27"/>
+      <c r="S34" s="27"/>
+      <c r="T34" s="27"/>
+      <c r="U34" s="27"/>
       <c r="V34" s="52"/>
-      <c r="W34" s="28"/>
-      <c r="X34" s="28"/>
-      <c r="Y34" s="28"/>
-      <c r="Z34" s="28"/>
-      <c r="AA34" s="28"/>
-      <c r="AB34" s="28"/>
-      <c r="AC34" s="28"/>
+      <c r="W34" s="27"/>
+      <c r="X34" s="27"/>
+      <c r="Y34" s="27"/>
+      <c r="Z34" s="27"/>
+      <c r="AA34" s="27"/>
+      <c r="AB34" s="27"/>
+      <c r="AC34" s="27"/>
     </row>
     <row r="35" ht="12.75" customHeight="1">
       <c r="A35" s="23"/>
       <c r="B35" s="23"/>
-      <c r="C35" s="41"/>
+      <c r="C35" s="40"/>
       <c r="D35" s="61" t="s">
         <v>198</v>
       </c>
@@ -2726,7 +2726,7 @@
         <v>45930.0</v>
       </c>
       <c r="H35" s="34" t="s">
-        <v>92</v>
+        <v>104</v>
       </c>
       <c r="I35" s="66"/>
       <c r="J35" s="66">
@@ -2744,24 +2744,24 @@
       <c r="N35" s="51"/>
       <c r="O35" s="25"/>
       <c r="P35" s="64"/>
-      <c r="Q35" s="28"/>
-      <c r="R35" s="28"/>
-      <c r="S35" s="28"/>
-      <c r="T35" s="28"/>
-      <c r="U35" s="28"/>
+      <c r="Q35" s="27"/>
+      <c r="R35" s="27"/>
+      <c r="S35" s="27"/>
+      <c r="T35" s="27"/>
+      <c r="U35" s="27"/>
       <c r="V35" s="52"/>
-      <c r="W35" s="28"/>
-      <c r="X35" s="28"/>
-      <c r="Y35" s="28"/>
-      <c r="Z35" s="28"/>
-      <c r="AA35" s="28"/>
-      <c r="AB35" s="28"/>
-      <c r="AC35" s="28"/>
+      <c r="W35" s="27"/>
+      <c r="X35" s="27"/>
+      <c r="Y35" s="27"/>
+      <c r="Z35" s="27"/>
+      <c r="AA35" s="27"/>
+      <c r="AB35" s="27"/>
+      <c r="AC35" s="27"/>
     </row>
     <row r="36" ht="12.75" customHeight="1">
       <c r="A36" s="23"/>
       <c r="B36" s="23"/>
-      <c r="C36" s="41"/>
+      <c r="C36" s="40"/>
       <c r="D36" s="61" t="s">
         <v>202</v>
       </c>
@@ -2775,7 +2775,7 @@
         <v>45968.0</v>
       </c>
       <c r="H36" s="34" t="s">
-        <v>111</v>
+        <v>122</v>
       </c>
       <c r="I36" s="66"/>
       <c r="J36" s="66">
@@ -2793,24 +2793,24 @@
       <c r="N36" s="51"/>
       <c r="O36" s="25"/>
       <c r="P36" s="64"/>
-      <c r="Q36" s="28"/>
-      <c r="R36" s="28"/>
-      <c r="S36" s="28"/>
-      <c r="T36" s="28"/>
-      <c r="U36" s="28"/>
+      <c r="Q36" s="27"/>
+      <c r="R36" s="27"/>
+      <c r="S36" s="27"/>
+      <c r="T36" s="27"/>
+      <c r="U36" s="27"/>
       <c r="V36" s="52"/>
-      <c r="W36" s="28"/>
-      <c r="X36" s="28"/>
-      <c r="Y36" s="28"/>
-      <c r="Z36" s="28"/>
-      <c r="AA36" s="28"/>
-      <c r="AB36" s="28"/>
-      <c r="AC36" s="28"/>
+      <c r="W36" s="27"/>
+      <c r="X36" s="27"/>
+      <c r="Y36" s="27"/>
+      <c r="Z36" s="27"/>
+      <c r="AA36" s="27"/>
+      <c r="AB36" s="27"/>
+      <c r="AC36" s="27"/>
     </row>
     <row r="37" ht="12.75" customHeight="1">
       <c r="A37" s="23"/>
       <c r="B37" s="23"/>
-      <c r="C37" s="41"/>
+      <c r="C37" s="40"/>
       <c r="D37" s="61" t="s">
         <v>205</v>
       </c>
@@ -2824,7 +2824,7 @@
         <v>46043.0</v>
       </c>
       <c r="H37" s="65" t="s">
-        <v>106</v>
+        <v>117</v>
       </c>
       <c r="I37" s="70"/>
       <c r="J37" s="69">
@@ -2836,30 +2836,30 @@
       <c r="L37" s="34" t="s">
         <v>206</v>
       </c>
-      <c r="M37" s="39">
+      <c r="M37" s="38">
         <v>11372.9</v>
       </c>
       <c r="N37" s="51"/>
       <c r="O37" s="25"/>
-      <c r="P37" s="28"/>
-      <c r="Q37" s="28"/>
-      <c r="R37" s="28"/>
-      <c r="S37" s="28"/>
-      <c r="T37" s="28"/>
-      <c r="U37" s="28"/>
+      <c r="P37" s="27"/>
+      <c r="Q37" s="27"/>
+      <c r="R37" s="27"/>
+      <c r="S37" s="27"/>
+      <c r="T37" s="27"/>
+      <c r="U37" s="27"/>
       <c r="V37" s="52"/>
-      <c r="W37" s="28"/>
-      <c r="X37" s="28"/>
-      <c r="Y37" s="28"/>
-      <c r="Z37" s="28"/>
-      <c r="AA37" s="28"/>
-      <c r="AB37" s="28"/>
-      <c r="AC37" s="28"/>
+      <c r="W37" s="27"/>
+      <c r="X37" s="27"/>
+      <c r="Y37" s="27"/>
+      <c r="Z37" s="27"/>
+      <c r="AA37" s="27"/>
+      <c r="AB37" s="27"/>
+      <c r="AC37" s="27"/>
     </row>
     <row r="38" ht="12.75" customHeight="1">
       <c r="A38" s="23"/>
       <c r="B38" s="23"/>
-      <c r="C38" s="41"/>
+      <c r="C38" s="40"/>
       <c r="D38" s="61" t="s">
         <v>207</v>
       </c>
@@ -2873,25 +2873,25 @@
       <c r="J38" s="69"/>
       <c r="K38" s="45"/>
       <c r="L38" s="34"/>
-      <c r="M38" s="39"/>
+      <c r="M38" s="38"/>
       <c r="N38" s="51">
         <v>15854.78</v>
       </c>
       <c r="O38" s="25"/>
-      <c r="P38" s="28"/>
-      <c r="Q38" s="28"/>
-      <c r="R38" s="28"/>
-      <c r="S38" s="28"/>
-      <c r="T38" s="28"/>
-      <c r="U38" s="28"/>
+      <c r="P38" s="27"/>
+      <c r="Q38" s="27"/>
+      <c r="R38" s="27"/>
+      <c r="S38" s="27"/>
+      <c r="T38" s="27"/>
+      <c r="U38" s="27"/>
       <c r="V38" s="52"/>
-      <c r="W38" s="28"/>
-      <c r="X38" s="28"/>
-      <c r="Y38" s="28"/>
-      <c r="Z38" s="28"/>
-      <c r="AA38" s="28"/>
-      <c r="AB38" s="28"/>
-      <c r="AC38" s="28"/>
+      <c r="W38" s="27"/>
+      <c r="X38" s="27"/>
+      <c r="Y38" s="27"/>
+      <c r="Z38" s="27"/>
+      <c r="AA38" s="27"/>
+      <c r="AB38" s="27"/>
+      <c r="AC38" s="27"/>
     </row>
     <row r="39" ht="12.75" customHeight="1">
       <c r="A39" s="23"/>
@@ -2910,25 +2910,25 @@
       <c r="J39" s="69"/>
       <c r="K39" s="45"/>
       <c r="L39" s="34"/>
-      <c r="M39" s="39"/>
+      <c r="M39" s="38"/>
       <c r="N39" s="71">
         <v>42229.72325</v>
       </c>
       <c r="O39" s="25"/>
-      <c r="P39" s="28"/>
-      <c r="Q39" s="28"/>
-      <c r="R39" s="28"/>
-      <c r="S39" s="28"/>
-      <c r="T39" s="28"/>
-      <c r="U39" s="28"/>
+      <c r="P39" s="27"/>
+      <c r="Q39" s="27"/>
+      <c r="R39" s="27"/>
+      <c r="S39" s="27"/>
+      <c r="T39" s="27"/>
+      <c r="U39" s="27"/>
       <c r="V39" s="52"/>
-      <c r="W39" s="28"/>
-      <c r="X39" s="28"/>
-      <c r="Y39" s="28"/>
-      <c r="Z39" s="28"/>
-      <c r="AA39" s="28"/>
-      <c r="AB39" s="28"/>
-      <c r="AC39" s="28"/>
+      <c r="W39" s="27"/>
+      <c r="X39" s="27"/>
+      <c r="Y39" s="27"/>
+      <c r="Z39" s="27"/>
+      <c r="AA39" s="27"/>
+      <c r="AB39" s="27"/>
+      <c r="AC39" s="27"/>
     </row>
     <row r="40" ht="12.75" customHeight="1">
       <c r="A40" s="23"/>
@@ -2947,25 +2947,25 @@
       <c r="J40" s="69"/>
       <c r="K40" s="45"/>
       <c r="L40" s="46"/>
-      <c r="M40" s="39"/>
+      <c r="M40" s="38"/>
       <c r="N40" s="72">
         <v>48857.395500000006</v>
       </c>
       <c r="O40" s="25"/>
-      <c r="P40" s="28"/>
-      <c r="Q40" s="28"/>
-      <c r="R40" s="28"/>
-      <c r="S40" s="28"/>
-      <c r="T40" s="28"/>
-      <c r="U40" s="28"/>
+      <c r="P40" s="27"/>
+      <c r="Q40" s="27"/>
+      <c r="R40" s="27"/>
+      <c r="S40" s="27"/>
+      <c r="T40" s="27"/>
+      <c r="U40" s="27"/>
       <c r="V40" s="52"/>
-      <c r="W40" s="28"/>
-      <c r="X40" s="28"/>
-      <c r="Y40" s="28"/>
-      <c r="Z40" s="28"/>
-      <c r="AA40" s="28"/>
-      <c r="AB40" s="28"/>
-      <c r="AC40" s="28"/>
+      <c r="W40" s="27"/>
+      <c r="X40" s="27"/>
+      <c r="Y40" s="27"/>
+      <c r="Z40" s="27"/>
+      <c r="AA40" s="27"/>
+      <c r="AB40" s="27"/>
+      <c r="AC40" s="27"/>
     </row>
     <row r="41" ht="12.75" customHeight="1">
       <c r="A41" s="23"/>
@@ -2984,23 +2984,23 @@
       <c r="J41" s="69"/>
       <c r="K41" s="45"/>
       <c r="L41" s="46"/>
-      <c r="M41" s="39"/>
+      <c r="M41" s="38"/>
       <c r="N41" s="72"/>
       <c r="O41" s="25"/>
-      <c r="P41" s="28"/>
-      <c r="Q41" s="28"/>
-      <c r="R41" s="28"/>
-      <c r="S41" s="28"/>
-      <c r="T41" s="28"/>
-      <c r="U41" s="28"/>
+      <c r="P41" s="27"/>
+      <c r="Q41" s="27"/>
+      <c r="R41" s="27"/>
+      <c r="S41" s="27"/>
+      <c r="T41" s="27"/>
+      <c r="U41" s="27"/>
       <c r="V41" s="52"/>
-      <c r="W41" s="28"/>
-      <c r="X41" s="28"/>
-      <c r="Y41" s="28"/>
-      <c r="Z41" s="28"/>
-      <c r="AA41" s="28"/>
-      <c r="AB41" s="28"/>
-      <c r="AC41" s="28"/>
+      <c r="W41" s="27"/>
+      <c r="X41" s="27"/>
+      <c r="Y41" s="27"/>
+      <c r="Z41" s="27"/>
+      <c r="AA41" s="27"/>
+      <c r="AB41" s="27"/>
+      <c r="AC41" s="27"/>
     </row>
     <row r="42" ht="12.75" customHeight="1">
       <c r="A42" s="23"/>
@@ -3019,7 +3019,7 @@
         <v>46104.0</v>
       </c>
       <c r="H42" s="65" t="s">
-        <v>106</v>
+        <v>117</v>
       </c>
       <c r="I42" s="70"/>
       <c r="J42" s="69">
@@ -3036,25 +3036,25 @@
       </c>
       <c r="N42" s="51"/>
       <c r="O42" s="25"/>
-      <c r="P42" s="28"/>
-      <c r="Q42" s="28"/>
-      <c r="R42" s="28"/>
-      <c r="S42" s="28"/>
-      <c r="T42" s="28"/>
-      <c r="U42" s="28"/>
+      <c r="P42" s="27"/>
+      <c r="Q42" s="27"/>
+      <c r="R42" s="27"/>
+      <c r="S42" s="27"/>
+      <c r="T42" s="27"/>
+      <c r="U42" s="27"/>
       <c r="V42" s="52"/>
-      <c r="W42" s="28"/>
-      <c r="X42" s="28"/>
-      <c r="Y42" s="28"/>
-      <c r="Z42" s="28"/>
-      <c r="AA42" s="28"/>
-      <c r="AB42" s="28"/>
-      <c r="AC42" s="28"/>
+      <c r="W42" s="27"/>
+      <c r="X42" s="27"/>
+      <c r="Y42" s="27"/>
+      <c r="Z42" s="27"/>
+      <c r="AA42" s="27"/>
+      <c r="AB42" s="27"/>
+      <c r="AC42" s="27"/>
     </row>
     <row r="43" ht="12.75" customHeight="1">
       <c r="A43" s="15"/>
       <c r="B43" s="15"/>
-      <c r="C43" s="41"/>
+      <c r="C43" s="40"/>
       <c r="D43" s="61" t="s">
         <v>215</v>
       </c>
@@ -3066,7 +3066,7 @@
         <v>46199.0</v>
       </c>
       <c r="H43" s="65" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="I43" s="70"/>
       <c r="J43" s="69">
@@ -3076,7 +3076,7 @@
         <v>58868.35</v>
       </c>
       <c r="L43" s="34" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="M43" s="74">
         <v>58868.35</v>
@@ -3087,7 +3087,7 @@
     <row r="44" ht="12.75" customHeight="1">
       <c r="A44" s="15"/>
       <c r="B44" s="15"/>
-      <c r="C44" s="41"/>
+      <c r="C44" s="40"/>
       <c r="K44" s="75"/>
       <c r="M44" s="75"/>
       <c r="V44" s="3"/>
@@ -3095,7 +3095,7 @@
     <row r="45" ht="12.75" customHeight="1">
       <c r="A45" s="15"/>
       <c r="B45" s="15"/>
-      <c r="C45" s="41"/>
+      <c r="C45" s="40"/>
       <c r="K45" s="75"/>
       <c r="M45" s="75"/>
       <c r="V45" s="3"/>
@@ -3103,25 +3103,25 @@
     <row r="46" ht="12.75" customHeight="1">
       <c r="A46" s="15"/>
       <c r="B46" s="15"/>
-      <c r="C46" s="41"/>
+      <c r="C46" s="40"/>
       <c r="V46" s="3"/>
     </row>
     <row r="47" ht="12.75" customHeight="1">
       <c r="A47" s="15"/>
       <c r="B47" s="15"/>
-      <c r="C47" s="41"/>
+      <c r="C47" s="40"/>
       <c r="V47" s="3"/>
     </row>
     <row r="48" ht="12.75" customHeight="1">
       <c r="A48" s="15"/>
       <c r="B48" s="15"/>
-      <c r="C48" s="41"/>
+      <c r="C48" s="40"/>
       <c r="V48" s="3"/>
     </row>
     <row r="49" ht="12.75" customHeight="1">
       <c r="A49" s="15"/>
       <c r="B49" s="15"/>
-      <c r="C49" s="41"/>
+      <c r="C49" s="40"/>
       <c r="V49" s="3"/>
     </row>
     <row r="50" ht="12.75" customHeight="1">
@@ -8050,31 +8050,31 @@
       <c r="AH2" s="2"/>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="11">
+      <c r="C3" s="9">
         <v>2.5E32</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="D3" s="7" t="s">
         <v>4</v>
       </c>
       <c r="E3" s="12">
         <v>45686.0</v>
       </c>
-      <c r="F3" s="8" t="s">
+      <c r="F3" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G3" s="8">
+      <c r="G3" s="7">
         <v>12.0</v>
       </c>
-      <c r="H3" s="8">
+      <c r="H3" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I3" s="8">
+      <c r="I3" s="7">
         <v>2048.0</v>
       </c>
       <c r="J3" s="14">
@@ -8083,7 +8083,7 @@
       <c r="K3" s="14">
         <v>1000.0</v>
       </c>
-      <c r="L3" s="8">
+      <c r="L3" s="7">
         <v>0.0</v>
       </c>
       <c r="AB3" s="2"/>
@@ -8095,31 +8095,31 @@
       <c r="AH3" s="2"/>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="C4" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="D4" s="7" t="s">
         <v>4</v>
       </c>
       <c r="E4" s="12">
         <v>45762.0</v>
       </c>
-      <c r="F4" s="8" t="s">
+      <c r="F4" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G4" s="8">
+      <c r="G4" s="7">
         <v>12.0</v>
       </c>
-      <c r="H4" s="8">
+      <c r="H4" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I4" s="8">
+      <c r="I4" s="7">
         <v>2048.0</v>
       </c>
       <c r="J4" s="14">
@@ -8128,7 +8128,7 @@
       <c r="K4" s="14">
         <v>52250.04</v>
       </c>
-      <c r="L4" s="8">
+      <c r="L4" s="7">
         <v>0.0</v>
       </c>
       <c r="AB4" s="2"/>
@@ -8140,31 +8140,31 @@
       <c r="AH4" s="2"/>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="B5" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="D5" s="8" t="s">
+      <c r="A5" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="D5" s="7" t="s">
         <v>4</v>
       </c>
       <c r="E5" s="12">
         <v>45762.0</v>
       </c>
-      <c r="F5" s="8" t="s">
+      <c r="F5" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G5" s="8">
+      <c r="G5" s="7">
         <v>12.0</v>
       </c>
-      <c r="H5" s="8">
+      <c r="H5" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I5" s="8">
+      <c r="I5" s="7">
         <v>2048.0</v>
       </c>
       <c r="J5" s="14">
@@ -8173,7 +8173,7 @@
       <c r="K5" s="14">
         <v>881914.18</v>
       </c>
-      <c r="L5" s="8">
+      <c r="L5" s="7">
         <v>0.0</v>
       </c>
       <c r="AB5" s="2"/>
@@ -8185,31 +8185,31 @@
       <c r="AH5" s="2"/>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="B6" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="C6" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="D6" s="8" t="s">
+      <c r="A6" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="D6" s="7" t="s">
         <v>4</v>
       </c>
       <c r="E6" s="12">
         <v>45762.0</v>
       </c>
-      <c r="F6" s="8" t="s">
+      <c r="F6" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G6" s="8">
+      <c r="G6" s="7">
         <v>12.0</v>
       </c>
-      <c r="H6" s="8">
+      <c r="H6" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I6" s="8">
+      <c r="I6" s="7">
         <v>2048.0</v>
       </c>
       <c r="J6" s="14">
@@ -8218,7 +8218,7 @@
       <c r="K6" s="14">
         <v>750000.0</v>
       </c>
-      <c r="L6" s="8">
+      <c r="L6" s="7">
         <v>0.0</v>
       </c>
       <c r="AB6" s="2"/>
@@ -8230,32 +8230,32 @@
       <c r="AH6" s="2"/>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="B7" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="C7" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="D7" s="8" t="s">
+      <c r="A7" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="D7" s="7" t="s">
         <v>4</v>
       </c>
       <c r="E7" s="12">
         <v>45763.0</v>
       </c>
-      <c r="F7" s="8" t="s">
+      <c r="F7" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G7" s="8">
+      <c r="G7" s="7">
         <v>12.0</v>
       </c>
-      <c r="H7" s="8">
+      <c r="H7" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I7" s="8" t="s">
-        <v>43</v>
+      <c r="I7" s="7" t="s">
+        <v>45</v>
       </c>
       <c r="J7" s="14">
         <v>949835.78</v>
@@ -8263,7 +8263,7 @@
       <c r="K7" s="14">
         <v>949835.78</v>
       </c>
-      <c r="L7" s="8">
+      <c r="L7" s="7">
         <v>0.0</v>
       </c>
       <c r="AB7" s="2"/>
@@ -8275,32 +8275,32 @@
       <c r="AH7" s="2"/>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="B8" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="C8" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="D8" s="8" t="s">
+      <c r="A8" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="D8" s="7" t="s">
         <v>4</v>
       </c>
       <c r="E8" s="12">
         <v>45763.0</v>
       </c>
-      <c r="F8" s="8" t="s">
+      <c r="F8" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G8" s="8">
+      <c r="G8" s="7">
         <v>12.0</v>
       </c>
-      <c r="H8" s="8">
+      <c r="H8" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I8" s="8" t="s">
-        <v>48</v>
+      <c r="I8" s="7" t="s">
+        <v>57</v>
       </c>
       <c r="J8" s="14">
         <v>524584.95</v>
@@ -8308,10 +8308,10 @@
       <c r="K8" s="14">
         <v>524584.95</v>
       </c>
-      <c r="L8" s="8">
+      <c r="L8" s="7">
         <v>0.0</v>
       </c>
-      <c r="O8" s="26"/>
+      <c r="O8" s="31"/>
       <c r="AB8" s="2"/>
       <c r="AC8" s="2"/>
       <c r="AD8" s="2"/>
@@ -8321,32 +8321,32 @@
       <c r="AH8" s="2"/>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="B9" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="C9" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="D9" s="8" t="s">
+      <c r="A9" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="D9" s="7" t="s">
         <v>4</v>
       </c>
       <c r="E9" s="12">
         <v>45792.0</v>
       </c>
-      <c r="F9" s="8" t="s">
+      <c r="F9" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G9" s="8">
+      <c r="G9" s="7">
         <v>12.0</v>
       </c>
-      <c r="H9" s="8">
+      <c r="H9" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I9" s="8" t="s">
-        <v>53</v>
+      <c r="I9" s="7" t="s">
+        <v>66</v>
       </c>
       <c r="J9" s="14">
         <v>211614.23</v>
@@ -8354,7 +8354,7 @@
       <c r="K9" s="14">
         <v>211614.23</v>
       </c>
-      <c r="L9" s="8">
+      <c r="L9" s="7">
         <v>0.0</v>
       </c>
       <c r="AB9" s="2"/>
@@ -8366,31 +8366,31 @@
       <c r="AH9" s="2"/>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="B10" s="8" t="s">
+      <c r="A10" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="B10" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="C10" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="D10" s="8" t="s">
+      <c r="C10" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="D10" s="7" t="s">
         <v>4</v>
       </c>
       <c r="E10" s="12">
         <v>45825.0</v>
       </c>
-      <c r="F10" s="8" t="s">
+      <c r="F10" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G10" s="8">
+      <c r="G10" s="7">
         <v>12.0</v>
       </c>
-      <c r="H10" s="8">
+      <c r="H10" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I10" s="8">
+      <c r="I10" s="7">
         <v>2048.0</v>
       </c>
       <c r="J10" s="14">
@@ -8411,31 +8411,31 @@
       <c r="AH10" s="2"/>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="B11" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="C11" s="8" t="s">
-        <v>68</v>
-      </c>
-      <c r="D11" s="8" t="s">
+      <c r="A11" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="D11" s="7" t="s">
         <v>4</v>
       </c>
       <c r="E11" s="12">
         <v>45825.0</v>
       </c>
-      <c r="F11" s="8" t="s">
+      <c r="F11" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G11" s="8">
+      <c r="G11" s="7">
         <v>12.0</v>
       </c>
-      <c r="H11" s="8">
+      <c r="H11" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I11" s="8">
+      <c r="I11" s="7">
         <v>2048.0</v>
       </c>
       <c r="J11" s="14">
@@ -8444,7 +8444,7 @@
       <c r="K11" s="14">
         <v>618154.38</v>
       </c>
-      <c r="L11" s="8">
+      <c r="L11" s="7">
         <v>0.01</v>
       </c>
       <c r="AB11" s="2"/>
@@ -8456,32 +8456,32 @@
       <c r="AH11" s="2"/>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="B12" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="C12" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="D12" s="8" t="s">
+      <c r="A12" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="D12" s="7" t="s">
         <v>4</v>
       </c>
       <c r="E12" s="12">
         <v>45832.0</v>
       </c>
-      <c r="F12" s="8" t="s">
+      <c r="F12" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G12" s="8">
+      <c r="G12" s="7">
         <v>12.0</v>
       </c>
-      <c r="H12" s="8">
+      <c r="H12" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I12" s="8" t="s">
-        <v>72</v>
+      <c r="I12" s="7" t="s">
+        <v>78</v>
       </c>
       <c r="J12" s="14">
         <v>1600334.09</v>
@@ -8489,7 +8489,7 @@
       <c r="K12" s="14">
         <v>1600334.09</v>
       </c>
-      <c r="L12" s="8">
+      <c r="L12" s="7">
         <v>0.0</v>
       </c>
       <c r="AB12" s="2"/>
@@ -8501,31 +8501,31 @@
       <c r="AH12" s="2"/>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="s">
-        <v>74</v>
-      </c>
-      <c r="B13" s="8" t="s">
+      <c r="A13" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="B13" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="C13" s="8" t="s">
-        <v>76</v>
-      </c>
-      <c r="D13" s="8" t="s">
+      <c r="C13" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="D13" s="7" t="s">
         <v>4</v>
       </c>
       <c r="E13" s="12">
         <v>45863.0</v>
       </c>
-      <c r="F13" s="8" t="s">
+      <c r="F13" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G13" s="8">
+      <c r="G13" s="7">
         <v>12.0</v>
       </c>
-      <c r="H13" s="8">
+      <c r="H13" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I13" s="8">
+      <c r="I13" s="7">
         <v>2048.0</v>
       </c>
       <c r="J13" s="14">
@@ -8537,7 +8537,7 @@
       <c r="L13" s="14">
         <v>0.0</v>
       </c>
-      <c r="M13" s="37"/>
+      <c r="M13" s="42"/>
       <c r="AB13" s="2"/>
       <c r="AC13" s="2"/>
       <c r="AD13" s="2"/>
@@ -8547,32 +8547,32 @@
       <c r="AH13" s="2"/>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="s">
-        <v>78</v>
-      </c>
-      <c r="B14" s="8" t="s">
-        <v>79</v>
-      </c>
-      <c r="C14" s="8" t="s">
-        <v>80</v>
-      </c>
-      <c r="D14" s="8" t="s">
+      <c r="A14" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="D14" s="7" t="s">
         <v>4</v>
       </c>
       <c r="E14" s="12">
         <v>45887.0</v>
       </c>
-      <c r="F14" s="8" t="s">
+      <c r="F14" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G14" s="8">
+      <c r="G14" s="7">
         <v>12.0</v>
       </c>
-      <c r="H14" s="8">
+      <c r="H14" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I14" s="8" t="s">
-        <v>53</v>
+      <c r="I14" s="7" t="s">
+        <v>66</v>
       </c>
       <c r="J14" s="14">
         <v>968237.39</v>
@@ -8580,7 +8580,7 @@
       <c r="K14" s="14">
         <v>968237.39</v>
       </c>
-      <c r="L14" s="8">
+      <c r="L14" s="7">
         <v>0.0</v>
       </c>
       <c r="AB14" s="2"/>
@@ -8592,32 +8592,32 @@
       <c r="AH14" s="2"/>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="B15" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="C15" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="D15" s="8" t="s">
+      <c r="A15" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="D15" s="7" t="s">
         <v>4</v>
       </c>
       <c r="E15" s="12">
         <v>45924.0</v>
       </c>
-      <c r="F15" s="8" t="s">
+      <c r="F15" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G15" s="8">
+      <c r="G15" s="7">
         <v>12.0</v>
       </c>
-      <c r="H15" s="8">
+      <c r="H15" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I15" s="8" t="s">
-        <v>43</v>
+      <c r="I15" s="7" t="s">
+        <v>45</v>
       </c>
       <c r="J15" s="14">
         <v>1011677.95</v>
@@ -8625,7 +8625,7 @@
       <c r="K15" s="14">
         <v>1011677.95</v>
       </c>
-      <c r="L15" s="8">
+      <c r="L15" s="7">
         <v>0.0</v>
       </c>
       <c r="AB15" s="2"/>
@@ -8637,31 +8637,31 @@
       <c r="AH15" s="2"/>
     </row>
     <row r="16">
-      <c r="A16" s="8" t="s">
-        <v>85</v>
-      </c>
-      <c r="B16" s="8" t="s">
+      <c r="A16" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="B16" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="C16" s="8" t="s">
-        <v>86</v>
-      </c>
-      <c r="D16" s="8" t="s">
+      <c r="C16" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="D16" s="7" t="s">
         <v>4</v>
       </c>
       <c r="E16" s="12">
         <v>45929.0</v>
       </c>
-      <c r="F16" s="8" t="s">
+      <c r="F16" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G16" s="8">
+      <c r="G16" s="7">
         <v>12.0</v>
       </c>
-      <c r="H16" s="8">
+      <c r="H16" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I16" s="8">
+      <c r="I16" s="7">
         <v>2048.0</v>
       </c>
       <c r="J16" s="14">
@@ -8682,37 +8682,37 @@
       <c r="AH16" s="2"/>
     </row>
     <row r="17">
-      <c r="A17" s="8" t="s">
-        <v>87</v>
-      </c>
-      <c r="B17" s="8" t="s">
-        <v>88</v>
-      </c>
-      <c r="C17" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="D17" s="8" t="s">
+      <c r="A17" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="D17" s="7" t="s">
         <v>4</v>
       </c>
       <c r="E17" s="12">
         <v>45930.0</v>
       </c>
-      <c r="F17" s="8" t="s">
+      <c r="F17" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G17" s="8">
+      <c r="G17" s="7">
         <v>12.0</v>
       </c>
-      <c r="H17" s="8">
+      <c r="H17" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I17" s="8">
+      <c r="I17" s="7">
         <v>2048.0</v>
       </c>
       <c r="J17" s="14">
         <v>34065.36</v>
       </c>
-      <c r="K17" s="8">
+      <c r="K17" s="7">
         <v>0.0</v>
       </c>
       <c r="L17" s="14">
@@ -8727,32 +8727,32 @@
       <c r="AH17" s="2"/>
     </row>
     <row r="18">
-      <c r="A18" s="8" t="s">
-        <v>92</v>
-      </c>
-      <c r="B18" s="8" t="s">
-        <v>79</v>
-      </c>
-      <c r="C18" s="8" t="s">
-        <v>93</v>
-      </c>
-      <c r="D18" s="8" t="s">
+      <c r="A18" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="D18" s="7" t="s">
         <v>4</v>
       </c>
       <c r="E18" s="12">
         <v>45938.0</v>
       </c>
-      <c r="F18" s="8" t="s">
+      <c r="F18" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G18" s="8">
+      <c r="G18" s="7">
         <v>12.0</v>
       </c>
-      <c r="H18" s="8">
+      <c r="H18" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I18" s="8" t="s">
-        <v>53</v>
+      <c r="I18" s="7" t="s">
+        <v>66</v>
       </c>
       <c r="J18" s="14">
         <v>63746.85</v>
@@ -8760,7 +8760,7 @@
       <c r="K18" s="14">
         <v>63746.85</v>
       </c>
-      <c r="L18" s="8">
+      <c r="L18" s="7">
         <v>0.0</v>
       </c>
       <c r="AB18" s="2"/>
@@ -8772,32 +8772,32 @@
       <c r="AH18" s="2"/>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="s">
-        <v>95</v>
-      </c>
-      <c r="B19" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="C19" s="8" t="s">
-        <v>96</v>
-      </c>
-      <c r="D19" s="8" t="s">
+      <c r="A19" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="B19" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="C19" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="D19" s="7" t="s">
         <v>4</v>
       </c>
       <c r="E19" s="12">
         <v>45938.0</v>
       </c>
-      <c r="F19" s="8" t="s">
+      <c r="F19" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G19" s="8">
+      <c r="G19" s="7">
         <v>12.0</v>
       </c>
-      <c r="H19" s="8">
+      <c r="H19" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I19" s="8" t="s">
-        <v>72</v>
+      <c r="I19" s="7" t="s">
+        <v>78</v>
       </c>
       <c r="J19" s="14">
         <v>947931.1</v>
@@ -8805,7 +8805,7 @@
       <c r="K19" s="14">
         <v>947931.1</v>
       </c>
-      <c r="L19" s="8">
+      <c r="L19" s="7">
         <v>0.0</v>
       </c>
       <c r="AB19" s="2"/>
@@ -8817,31 +8817,31 @@
       <c r="AH19" s="2"/>
     </row>
     <row r="20">
-      <c r="A20" s="8" t="s">
-        <v>99</v>
-      </c>
-      <c r="B20" s="8" t="s">
+      <c r="A20" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="B20" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="C20" s="8" t="s">
-        <v>100</v>
-      </c>
-      <c r="D20" s="8" t="s">
+      <c r="C20" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="D20" s="7" t="s">
         <v>4</v>
       </c>
       <c r="E20" s="12">
         <v>45938.0</v>
       </c>
-      <c r="F20" s="8" t="s">
+      <c r="F20" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G20" s="8">
+      <c r="G20" s="7">
         <v>12.0</v>
       </c>
-      <c r="H20" s="8">
+      <c r="H20" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I20" s="8">
+      <c r="I20" s="7">
         <v>2048.0</v>
       </c>
       <c r="J20" s="14">
@@ -8850,7 +8850,7 @@
       <c r="K20" s="14">
         <v>259790.57</v>
       </c>
-      <c r="L20" s="8">
+      <c r="L20" s="7">
         <v>0.0</v>
       </c>
       <c r="AB20" s="2"/>
@@ -8862,31 +8862,31 @@
       <c r="AH20" s="2"/>
     </row>
     <row r="21">
-      <c r="A21" s="8" t="s">
-        <v>102</v>
-      </c>
-      <c r="B21" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="C21" s="8" t="s">
-        <v>103</v>
-      </c>
-      <c r="D21" s="8" t="s">
+      <c r="A21" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="B21" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="C21" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="D21" s="7" t="s">
         <v>4</v>
       </c>
       <c r="E21" s="12">
         <v>45938.0</v>
       </c>
-      <c r="F21" s="8" t="s">
+      <c r="F21" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G21" s="8">
+      <c r="G21" s="7">
         <v>12.0</v>
       </c>
-      <c r="H21" s="8">
+      <c r="H21" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I21" s="8">
+      <c r="I21" s="7">
         <v>2048.0</v>
       </c>
       <c r="J21" s="14">
@@ -8895,7 +8895,7 @@
       <c r="K21" s="14">
         <v>170479.3</v>
       </c>
-      <c r="L21" s="8">
+      <c r="L21" s="7">
         <v>0.0</v>
       </c>
       <c r="AB21" s="2"/>
@@ -8907,31 +8907,31 @@
       <c r="AH21" s="2"/>
     </row>
     <row r="22">
-      <c r="A22" s="8" t="s">
-        <v>106</v>
-      </c>
-      <c r="B22" s="8" t="s">
-        <v>107</v>
-      </c>
-      <c r="C22" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="D22" s="8" t="s">
+      <c r="A22" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="B22" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="C22" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="D22" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="E22" s="48">
+      <c r="E22" s="50">
         <v>45953.0</v>
       </c>
-      <c r="F22" s="8" t="s">
+      <c r="F22" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G22" s="8">
+      <c r="G22" s="7">
         <v>12.0</v>
       </c>
-      <c r="H22" s="8">
+      <c r="H22" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I22" s="8">
+      <c r="I22" s="7">
         <v>2000.0</v>
       </c>
       <c r="J22" s="14">
@@ -8952,32 +8952,32 @@
       <c r="AH22" s="2"/>
     </row>
     <row r="23">
-      <c r="A23" s="8" t="s">
-        <v>111</v>
-      </c>
-      <c r="B23" s="8" t="s">
-        <v>112</v>
-      </c>
-      <c r="C23" s="8" t="s">
-        <v>113</v>
-      </c>
-      <c r="D23" s="8" t="s">
+      <c r="A23" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="B23" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="C23" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="D23" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="E23" s="48">
+      <c r="E23" s="50">
         <v>45953.0</v>
       </c>
-      <c r="F23" s="8" t="s">
+      <c r="F23" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G23" s="8">
+      <c r="G23" s="7">
         <v>12.0</v>
       </c>
-      <c r="H23" s="8">
+      <c r="H23" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I23" s="8" t="s">
-        <v>115</v>
+      <c r="I23" s="7" t="s">
+        <v>125</v>
       </c>
       <c r="J23" s="14">
         <v>1000001.64</v>
@@ -8985,7 +8985,7 @@
       <c r="K23" s="14">
         <v>1000001.64</v>
       </c>
-      <c r="L23" s="8">
+      <c r="L23" s="7">
         <v>0.0</v>
       </c>
       <c r="AB23" s="2"/>
@@ -8997,31 +8997,31 @@
       <c r="AH23" s="2"/>
     </row>
     <row r="24">
-      <c r="A24" s="8" t="s">
-        <v>117</v>
-      </c>
-      <c r="B24" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="C24" s="8" t="s">
-        <v>118</v>
-      </c>
-      <c r="D24" s="8" t="s">
+      <c r="A24" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="B24" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="C24" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="D24" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="E24" s="48">
+      <c r="E24" s="50">
         <v>45953.0</v>
       </c>
-      <c r="F24" s="8" t="s">
+      <c r="F24" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G24" s="8">
+      <c r="G24" s="7">
         <v>12.0</v>
       </c>
-      <c r="H24" s="8">
+      <c r="H24" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I24" s="8">
+      <c r="I24" s="7">
         <v>2048.0</v>
       </c>
       <c r="J24" s="14">
@@ -9030,7 +9030,7 @@
       <c r="K24" s="14">
         <v>68405.66</v>
       </c>
-      <c r="L24" s="8">
+      <c r="L24" s="7">
         <v>0.0</v>
       </c>
       <c r="AB24" s="2"/>
@@ -9042,32 +9042,32 @@
       <c r="AH24" s="2"/>
     </row>
     <row r="25">
-      <c r="A25" s="8" t="s">
-        <v>121</v>
-      </c>
-      <c r="B25" s="8" t="s">
-        <v>122</v>
-      </c>
-      <c r="C25" s="8" t="s">
-        <v>123</v>
-      </c>
-      <c r="D25" s="8" t="s">
+      <c r="A25" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="B25" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="C25" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="D25" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="E25" s="48">
+      <c r="E25" s="50">
         <v>45975.0</v>
       </c>
-      <c r="F25" s="8" t="s">
+      <c r="F25" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G25" s="8">
+      <c r="G25" s="7">
         <v>12.0</v>
       </c>
-      <c r="H25" s="8">
+      <c r="H25" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I25" s="8" t="s">
-        <v>115</v>
+      <c r="I25" s="7" t="s">
+        <v>125</v>
       </c>
       <c r="J25" s="14">
         <v>1157673.06</v>
@@ -9075,7 +9075,7 @@
       <c r="K25" s="14">
         <v>1157673.06</v>
       </c>
-      <c r="L25" s="8">
+      <c r="L25" s="7">
         <v>0.0</v>
       </c>
       <c r="AB25" s="2"/>
@@ -9087,31 +9087,31 @@
       <c r="AH25" s="2"/>
     </row>
     <row r="26">
-      <c r="A26" s="8" t="s">
-        <v>125</v>
-      </c>
-      <c r="B26" s="8" t="s">
+      <c r="A26" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="B26" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="C26" s="8" t="s">
-        <v>126</v>
-      </c>
-      <c r="D26" s="8" t="s">
+      <c r="C26" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="D26" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="E26" s="48">
+      <c r="E26" s="50">
         <v>45989.0</v>
       </c>
-      <c r="F26" s="8" t="s">
+      <c r="F26" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G26" s="8">
+      <c r="G26" s="7">
         <v>12.0</v>
       </c>
-      <c r="H26" s="8">
+      <c r="H26" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I26" s="8">
+      <c r="I26" s="7">
         <v>2048.0</v>
       </c>
       <c r="J26" s="14">
@@ -9120,7 +9120,7 @@
       <c r="K26" s="14">
         <v>34065.36</v>
       </c>
-      <c r="L26" s="8">
+      <c r="L26" s="7">
         <v>0.0</v>
       </c>
       <c r="AB26" s="2"/>
@@ -9132,31 +9132,31 @@
       <c r="AH26" s="2"/>
     </row>
     <row r="27">
-      <c r="A27" s="8" t="s">
-        <v>128</v>
-      </c>
-      <c r="B27" s="8" t="s">
-        <v>129</v>
-      </c>
-      <c r="C27" s="8" t="s">
-        <v>130</v>
-      </c>
-      <c r="D27" s="8" t="s">
+      <c r="A27" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="B27" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="C27" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="D27" s="7" t="s">
         <v>4</v>
       </c>
       <c r="E27" s="12">
         <v>46104.0</v>
       </c>
-      <c r="F27" s="8" t="s">
+      <c r="F27" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G27" s="8">
+      <c r="G27" s="7">
         <v>12.0</v>
       </c>
-      <c r="H27" s="8">
+      <c r="H27" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I27" s="8">
+      <c r="I27" s="7">
         <v>2048.0</v>
       </c>
       <c r="J27" s="14">
@@ -9177,37 +9177,37 @@
       <c r="AH27" s="2"/>
     </row>
     <row r="28">
-      <c r="A28" s="8" t="s">
-        <v>133</v>
-      </c>
-      <c r="B28" s="8" t="s">
-        <v>134</v>
-      </c>
-      <c r="C28" s="8" t="s">
-        <v>136</v>
-      </c>
-      <c r="D28" s="8" t="s">
+      <c r="A28" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="B28" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="C28" s="7" t="s">
+        <v>142</v>
+      </c>
+      <c r="D28" s="7" t="s">
         <v>4</v>
       </c>
       <c r="E28" s="12">
         <v>46120.0</v>
       </c>
-      <c r="F28" s="8" t="s">
+      <c r="F28" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G28" s="8">
+      <c r="G28" s="7">
         <v>12.0</v>
       </c>
-      <c r="H28" s="8">
+      <c r="H28" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I28" s="8" t="s">
-        <v>48</v>
+      <c r="I28" s="7" t="s">
+        <v>57</v>
       </c>
       <c r="J28" s="14">
         <v>1912292.52</v>
       </c>
-      <c r="K28" s="8">
+      <c r="K28" s="7">
         <v>0.0</v>
       </c>
       <c r="L28" s="14">
@@ -9222,37 +9222,37 @@
       <c r="AH28" s="2"/>
     </row>
     <row r="29">
-      <c r="A29" s="8" t="s">
-        <v>138</v>
-      </c>
-      <c r="B29" s="8" t="s">
-        <v>139</v>
-      </c>
-      <c r="C29" s="8" t="s">
-        <v>140</v>
-      </c>
-      <c r="D29" s="8" t="s">
+      <c r="A29" s="7" t="s">
+        <v>144</v>
+      </c>
+      <c r="B29" s="7" t="s">
+        <v>145</v>
+      </c>
+      <c r="C29" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="D29" s="7" t="s">
         <v>4</v>
       </c>
       <c r="E29" s="12">
         <v>46196.0</v>
       </c>
-      <c r="F29" s="8" t="s">
+      <c r="F29" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G29" s="8">
+      <c r="G29" s="7">
         <v>12.0</v>
       </c>
-      <c r="H29" s="8">
+      <c r="H29" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I29" s="8">
+      <c r="I29" s="7">
         <v>2048.0</v>
       </c>
       <c r="J29" s="14">
         <v>1496713.48</v>
       </c>
-      <c r="K29" s="8">
+      <c r="K29" s="7">
         <v>0.0</v>
       </c>
       <c r="L29" s="14">
@@ -9267,37 +9267,37 @@
       <c r="AH29" s="2"/>
     </row>
     <row r="30">
-      <c r="A30" s="8" t="s">
-        <v>143</v>
-      </c>
-      <c r="B30" s="8" t="s">
-        <v>144</v>
-      </c>
-      <c r="C30" s="8" t="s">
-        <v>145</v>
-      </c>
-      <c r="D30" s="8" t="s">
+      <c r="A30" s="7" t="s">
+        <v>148</v>
+      </c>
+      <c r="B30" s="7" t="s">
+        <v>150</v>
+      </c>
+      <c r="C30" s="7" t="s">
+        <v>151</v>
+      </c>
+      <c r="D30" s="7" t="s">
         <v>4</v>
       </c>
       <c r="E30" s="12">
         <v>46205.0</v>
       </c>
-      <c r="F30" s="8" t="s">
+      <c r="F30" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G30" s="8">
+      <c r="G30" s="7">
         <v>12.0</v>
       </c>
-      <c r="H30" s="8">
+      <c r="H30" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I30" s="8" t="s">
-        <v>43</v>
+      <c r="I30" s="7" t="s">
+        <v>45</v>
       </c>
       <c r="J30" s="14">
         <v>624166.14</v>
       </c>
-      <c r="K30" s="8">
+      <c r="K30" s="7">
         <v>0.0</v>
       </c>
       <c r="L30" s="14">
@@ -9312,37 +9312,37 @@
       <c r="AH30" s="2"/>
     </row>
     <row r="31">
-      <c r="A31" s="8" t="s">
-        <v>148</v>
-      </c>
-      <c r="B31" s="8" t="s">
-        <v>149</v>
-      </c>
-      <c r="C31" s="8" t="s">
-        <v>150</v>
-      </c>
-      <c r="D31" s="8" t="s">
+      <c r="A31" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="B31" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="C31" s="7" t="s">
+        <v>154</v>
+      </c>
+      <c r="D31" s="7" t="s">
         <v>4</v>
       </c>
       <c r="E31" s="12">
         <v>46205.0</v>
       </c>
-      <c r="F31" s="8" t="s">
+      <c r="F31" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G31" s="8">
+      <c r="G31" s="7">
         <v>12.0</v>
       </c>
-      <c r="H31" s="8">
+      <c r="H31" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I31" s="8" t="s">
-        <v>115</v>
+      <c r="I31" s="7" t="s">
+        <v>125</v>
       </c>
       <c r="J31" s="14">
         <v>18462.36</v>
       </c>
-      <c r="K31" s="8">
+      <c r="K31" s="7">
         <v>0.0</v>
       </c>
       <c r="L31" s="14">
@@ -9357,37 +9357,37 @@
       <c r="AH31" s="2"/>
     </row>
     <row r="32">
-      <c r="A32" s="8" t="s">
-        <v>152</v>
-      </c>
-      <c r="B32" s="8" t="s">
-        <v>149</v>
+      <c r="A32" s="7" t="s">
+        <v>156</v>
+      </c>
+      <c r="B32" s="7" t="s">
+        <v>153</v>
       </c>
       <c r="C32" s="14" t="s">
-        <v>153</v>
-      </c>
-      <c r="D32" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="D32" s="7" t="s">
         <v>4</v>
       </c>
       <c r="E32" s="12">
         <v>46213.0</v>
       </c>
-      <c r="F32" s="8" t="s">
+      <c r="F32" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G32" s="8">
+      <c r="G32" s="7">
         <v>12.0</v>
       </c>
-      <c r="H32" s="8">
+      <c r="H32" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I32" s="8" t="s">
-        <v>115</v>
+      <c r="I32" s="7" t="s">
+        <v>125</v>
       </c>
       <c r="J32" s="14">
         <v>1530656.62</v>
       </c>
-      <c r="K32" s="8">
+      <c r="K32" s="7">
         <v>0.0</v>
       </c>
       <c r="L32" s="14">
@@ -9402,37 +9402,37 @@
       <c r="AH32" s="2"/>
     </row>
     <row r="33">
-      <c r="A33" s="8" t="s">
-        <v>156</v>
-      </c>
-      <c r="B33" s="8" t="s">
-        <v>139</v>
+      <c r="A33" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="B33" s="7" t="s">
+        <v>145</v>
       </c>
       <c r="C33" s="14" t="s">
-        <v>158</v>
-      </c>
-      <c r="D33" s="8" t="s">
+        <v>159</v>
+      </c>
+      <c r="D33" s="7" t="s">
         <v>4</v>
       </c>
       <c r="E33" s="12">
         <v>46227.0</v>
       </c>
-      <c r="F33" s="8" t="s">
+      <c r="F33" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G33" s="8">
+      <c r="G33" s="7">
         <v>12.0</v>
       </c>
-      <c r="H33" s="8">
+      <c r="H33" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I33" s="8">
+      <c r="I33" s="7">
         <v>2048.0</v>
       </c>
       <c r="J33" s="14">
         <v>173846.38</v>
       </c>
-      <c r="K33" s="8">
+      <c r="K33" s="7">
         <v>0.0</v>
       </c>
       <c r="L33" s="14">
@@ -9447,37 +9447,37 @@
       <c r="AH33" s="2"/>
     </row>
     <row r="34">
-      <c r="A34" s="8" t="s">
-        <v>160</v>
-      </c>
-      <c r="B34" s="8" t="s">
+      <c r="A34" s="7" t="s">
         <v>161</v>
       </c>
-      <c r="C34" s="8" t="s">
+      <c r="B34" s="7" t="s">
         <v>162</v>
       </c>
-      <c r="D34" s="8" t="s">
+      <c r="C34" s="7" t="s">
+        <v>163</v>
+      </c>
+      <c r="D34" s="7" t="s">
         <v>4</v>
       </c>
       <c r="E34" s="12">
         <v>46240.0</v>
       </c>
-      <c r="F34" s="8" t="s">
+      <c r="F34" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G34" s="8">
+      <c r="G34" s="7">
         <v>12.0</v>
       </c>
-      <c r="H34" s="8">
+      <c r="H34" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I34" s="8" t="s">
-        <v>163</v>
+      <c r="I34" s="7" t="s">
+        <v>164</v>
       </c>
       <c r="J34" s="14">
         <v>236343.68</v>
       </c>
-      <c r="K34" s="8">
+      <c r="K34" s="7">
         <v>0.0</v>
       </c>
       <c r="L34" s="14">

</xml_diff>

<commit_message>
Atualização automática: pagamentos (19/08/2026 14:34)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/01_Bases_Originais/005_CELOG_2025/005_CELOG-PAMALS_2025 online.xlsx
+++ b/Contrato 005/Dashboard/01_Bases_Originais/005_CELOG_2025/005_CELOG-PAMALS_2025 online.xlsx
@@ -117,24 +117,24 @@
     <t>005/CELOG-PAMALS/2025</t>
   </si>
   <si>
+    <t>2025NE000369</t>
+  </si>
+  <si>
+    <t>C25516</t>
+  </si>
+  <si>
     <t>CELOG</t>
   </si>
   <si>
     <t>PAMALS</t>
   </si>
   <si>
-    <t>2025NE000369</t>
-  </si>
-  <si>
-    <t>C25516</t>
+    <t>25E0387</t>
   </si>
   <si>
     <t>Vigente</t>
   </si>
   <si>
-    <t>25E0387</t>
-  </si>
-  <si>
     <t>2048 20YJ 21EM 219C 20SP 20X7 2000</t>
   </si>
   <si>
@@ -144,15 +144,15 @@
     <t>R$</t>
   </si>
   <si>
+    <t>2025NE000371</t>
+  </si>
+  <si>
+    <t>25E0389</t>
+  </si>
+  <si>
     <t>VEE ONE-MANUTENCAO E SERVICOS TECNICOS LTDA</t>
   </si>
   <si>
-    <t>2025NE000371</t>
-  </si>
-  <si>
-    <t>25E0389</t>
-  </si>
-  <si>
     <t>2025NE000413</t>
   </si>
   <si>
@@ -177,34 +177,73 @@
     <t>21EM</t>
   </si>
   <si>
+    <t>Módulo</t>
+  </si>
+  <si>
+    <t>Referência</t>
+  </si>
+  <si>
+    <t>Nº recibo</t>
+  </si>
+  <si>
+    <t>Nº</t>
+  </si>
+  <si>
     <t>2025NE000559</t>
   </si>
   <si>
+    <t>Data</t>
+  </si>
+  <si>
+    <t>Empenho</t>
+  </si>
+  <si>
     <t>C25545</t>
   </si>
   <si>
+    <t>Observações</t>
+  </si>
+  <si>
     <t>25E0524</t>
   </si>
   <si>
+    <t>Vencimento</t>
+  </si>
+  <si>
+    <t>Valor das Nfs</t>
+  </si>
+  <si>
+    <t>Ordem de Pagamento</t>
+  </si>
+  <si>
     <t>20X7</t>
   </si>
   <si>
+    <t>Faturado</t>
+  </si>
+  <si>
+    <t>Pendente</t>
+  </si>
+  <si>
     <t>2025NE000770</t>
   </si>
   <si>
     <t>25E0731</t>
   </si>
   <si>
+    <t>FEV/25</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
     <t>2025NE000774</t>
   </si>
   <si>
-    <t>Módulo</t>
-  </si>
-  <si>
     <t>25E0737</t>
   </si>
   <si>
-    <t>Referência</t>
+    <t xml:space="preserve">2025NE000369 </t>
   </si>
   <si>
     <t>2025NE000843</t>
@@ -213,48 +252,21 @@
     <t>C25630</t>
   </si>
   <si>
-    <t>Nº recibo</t>
-  </si>
-  <si>
     <t>25E0787</t>
   </si>
   <si>
+    <t>2025NP001980</t>
+  </si>
+  <si>
     <t>219C</t>
   </si>
   <si>
-    <t>Nº</t>
-  </si>
-  <si>
-    <t>Data</t>
-  </si>
-  <si>
-    <t>Empenho</t>
-  </si>
-  <si>
-    <t>Observações</t>
-  </si>
-  <si>
     <t>2025NE001065</t>
   </si>
   <si>
-    <t>Vencimento</t>
-  </si>
-  <si>
     <t>25E0999</t>
   </si>
   <si>
-    <t>Valor das Nfs</t>
-  </si>
-  <si>
-    <t>Ordem de Pagamento</t>
-  </si>
-  <si>
-    <t>Faturado</t>
-  </si>
-  <si>
-    <t>Pendente</t>
-  </si>
-  <si>
     <t>2025NE001200</t>
   </si>
   <si>
@@ -273,31 +285,37 @@
     <t>25E1446</t>
   </si>
   <si>
-    <t>FEV/25</t>
+    <t>MAR/25</t>
+  </si>
+  <si>
+    <t>2025NE000367, 2025NE000369, 2025NE000371, 2025NE000413</t>
+  </si>
+  <si>
+    <t>2025NP001979</t>
   </si>
   <si>
     <t>2025NE001627</t>
   </si>
   <si>
-    <t>-</t>
-  </si>
-  <si>
     <t>25E1475</t>
   </si>
   <si>
     <t>2025NE001629</t>
   </si>
   <si>
-    <t xml:space="preserve">2025NE000369 </t>
-  </si>
-  <si>
     <t>C25820</t>
   </si>
   <si>
     <t>25E1477</t>
   </si>
   <si>
-    <t>2025NP001980</t>
+    <t>ABR/25</t>
+  </si>
+  <si>
+    <t>2025NE000413, 2025NE000414, 2025NE000559</t>
+  </si>
+  <si>
+    <t>2025NP002341</t>
   </si>
   <si>
     <t>2025NE001687</t>
@@ -306,12 +324,18 @@
     <t>25E1535</t>
   </si>
   <si>
+    <t>MAI/25</t>
+  </si>
+  <si>
     <t>2025NE001688</t>
   </si>
   <si>
     <t>25E1536</t>
   </si>
   <si>
+    <t>2025NP002884</t>
+  </si>
+  <si>
     <t>2025NE001689</t>
   </si>
   <si>
@@ -324,91 +348,7 @@
     <t>25E1538</t>
   </si>
   <si>
-    <t>MAR/25</t>
-  </si>
-  <si>
-    <t>2025NE001823</t>
-  </si>
-  <si>
-    <t>C25865</t>
-  </si>
-  <si>
-    <t>25E1666</t>
-  </si>
-  <si>
-    <t>2025NE000367, 2025NE000369, 2025NE000371, 2025NE000413</t>
-  </si>
-  <si>
-    <t>2025NP001979</t>
-  </si>
-  <si>
-    <t>2025NE001828</t>
-  </si>
-  <si>
-    <t>C25869</t>
-  </si>
-  <si>
-    <t>25E1667</t>
-  </si>
-  <si>
-    <t>20YJ</t>
-  </si>
-  <si>
-    <t>ABR/25</t>
-  </si>
-  <si>
-    <t>2025NE001830</t>
-  </si>
-  <si>
-    <t>2025NE000413, 2025NE000414, 2025NE000559</t>
-  </si>
-  <si>
-    <t>25E1669</t>
-  </si>
-  <si>
-    <t>2025NP002341</t>
-  </si>
-  <si>
-    <t>2025NE002200</t>
-  </si>
-  <si>
-    <t>MAI/25</t>
-  </si>
-  <si>
-    <t>C25863</t>
-  </si>
-  <si>
-    <t>25E2021</t>
-  </si>
-  <si>
-    <t>2025NE002237</t>
-  </si>
-  <si>
-    <t>2025NP002884</t>
-  </si>
-  <si>
-    <t>25E2058</t>
-  </si>
-  <si>
-    <t>2026NE000330</t>
-  </si>
-  <si>
-    <t>C26163</t>
-  </si>
-  <si>
-    <t>26E0320</t>
-  </si>
-  <si>
     <t>JUN/25</t>
-  </si>
-  <si>
-    <t>2026NE000388</t>
-  </si>
-  <si>
-    <t>C26193</t>
-  </si>
-  <si>
-    <t>26E0375</t>
   </si>
   <si>
     <t>2025NE000005,
@@ -417,25 +357,16 @@
 2025NE000774</t>
   </si>
   <si>
-    <t>2026NE000748</t>
-  </si>
-  <si>
-    <t>C26312</t>
-  </si>
-  <si>
-    <t>26E0709</t>
+    <t>2025NE001823</t>
   </si>
   <si>
     <t>2025NP400522</t>
   </si>
   <si>
-    <t>2026NE000816</t>
-  </si>
-  <si>
-    <t>C26324</t>
-  </si>
-  <si>
-    <t>26E0776</t>
+    <t>C25865</t>
+  </si>
+  <si>
+    <t>25E1666</t>
   </si>
   <si>
     <t>JUL/25</t>
@@ -447,28 +378,40 @@
     <t>2025NP003724</t>
   </si>
   <si>
-    <t>2026NE000817</t>
-  </si>
-  <si>
-    <t>C26326</t>
-  </si>
-  <si>
-    <t>26E0777</t>
+    <t>2025NE001828</t>
+  </si>
+  <si>
+    <t>C25869</t>
+  </si>
+  <si>
+    <t>25E1667</t>
   </si>
   <si>
     <t>AGO/25</t>
   </si>
   <si>
+    <t>20YJ</t>
+  </si>
+  <si>
     <t>2025NP004558</t>
   </si>
   <si>
-    <t>2026NE000842</t>
+    <t>2025NE001830</t>
+  </si>
+  <si>
+    <t>25E1669</t>
   </si>
   <si>
     <t>SET/25</t>
   </si>
   <si>
-    <t>26E0803</t>
+    <t>2025NE002200</t>
+  </si>
+  <si>
+    <t>C25863</t>
+  </si>
+  <si>
+    <t>25E2021</t>
   </si>
   <si>
     <t>2025NE001688 
@@ -481,16 +424,127 @@
     <t>OUT/25</t>
   </si>
   <si>
+    <t>2025NE002237</t>
+  </si>
+  <si>
+    <t>2025NE001688, 2025NE001828, 2025NE002200</t>
+  </si>
+  <si>
+    <t>25E2058</t>
+  </si>
+  <si>
+    <t>2025NP004932</t>
+  </si>
+  <si>
+    <t>2026NE000330</t>
+  </si>
+  <si>
+    <t>C26163</t>
+  </si>
+  <si>
+    <t>26E0320</t>
+  </si>
+  <si>
+    <t>NOV/25</t>
+  </si>
+  <si>
+    <t>2025NE001687, 2025NE001689, 2025NE001690, 2025NE001823, 2025NE001830, 2025NE002237</t>
+  </si>
+  <si>
+    <t>2026NP400440</t>
+  </si>
+  <si>
+    <t>2026NE000388</t>
+  </si>
+  <si>
+    <t>C26193</t>
+  </si>
+  <si>
+    <t>26E0375</t>
+  </si>
+  <si>
+    <t>DEZ/25</t>
+  </si>
+  <si>
+    <t>2025NE001065, 2025NE002200</t>
+  </si>
+  <si>
+    <t>2026NP400412</t>
+  </si>
+  <si>
+    <t>2026NE000748</t>
+  </si>
+  <si>
+    <t>C26312</t>
+  </si>
+  <si>
+    <t>26E0709</t>
+  </si>
+  <si>
+    <t>JAN/26</t>
+  </si>
+  <si>
+    <t>2026NP401035</t>
+  </si>
+  <si>
+    <t>2026NE000816</t>
+  </si>
+  <si>
+    <t>C26324</t>
+  </si>
+  <si>
+    <t>26E0776</t>
+  </si>
+  <si>
+    <t>FEV/26</t>
+  </si>
+  <si>
+    <t>2025NE001627, 2025NE001629, 2025NE001823</t>
+  </si>
+  <si>
+    <t>2026NP402272</t>
+  </si>
+  <si>
+    <t>2026NE000817</t>
+  </si>
+  <si>
+    <t>C26326</t>
+  </si>
+  <si>
+    <t>26E0777</t>
+  </si>
+  <si>
+    <t>MAR/26</t>
+  </si>
+  <si>
+    <t>2025NE000770, 2025NE001627</t>
+  </si>
+  <si>
+    <t>R$ 1.350.542,52</t>
+  </si>
+  <si>
+    <t>2026NP401762</t>
+  </si>
+  <si>
+    <t>2026NE000842</t>
+  </si>
+  <si>
+    <t>26E0803</t>
+  </si>
+  <si>
+    <t>ABR/26</t>
+  </si>
+  <si>
+    <t>2025NE000770, 2025NE001065, 2025NE001627</t>
+  </si>
+  <si>
     <t>2026NE000944</t>
   </si>
   <si>
-    <t>2025NE001688, 2025NE001828, 2025NE002200</t>
-  </si>
-  <si>
     <t>26E0906</t>
   </si>
   <si>
-    <t>2025NP004932</t>
+    <t>REAJUSTE</t>
   </si>
   <si>
     <t>2026NE001015</t>
@@ -502,64 +556,10 @@
     <t>26E0959</t>
   </si>
   <si>
+    <t>2026NP402148</t>
+  </si>
+  <si>
     <t>20XV</t>
-  </si>
-  <si>
-    <t>NOV/25</t>
-  </si>
-  <si>
-    <t>2025NE001687, 2025NE001689, 2025NE001690, 2025NE001823, 2025NE001830, 2025NE002237</t>
-  </si>
-  <si>
-    <t>2026NP400440</t>
-  </si>
-  <si>
-    <t>DEZ/25</t>
-  </si>
-  <si>
-    <t>2025NE001065, 2025NE002200</t>
-  </si>
-  <si>
-    <t>2026NP400412</t>
-  </si>
-  <si>
-    <t>JAN/26</t>
-  </si>
-  <si>
-    <t>2026NP401035</t>
-  </si>
-  <si>
-    <t>FEV/26</t>
-  </si>
-  <si>
-    <t>2025NE001627, 2025NE001629, 2025NE001823</t>
-  </si>
-  <si>
-    <t>2026NP402272</t>
-  </si>
-  <si>
-    <t>MAR/26</t>
-  </si>
-  <si>
-    <t>2025NE000770, 2025NE001627</t>
-  </si>
-  <si>
-    <t>R$ 1.350.542,52</t>
-  </si>
-  <si>
-    <t>2026NP401762</t>
-  </si>
-  <si>
-    <t>ABR/26</t>
-  </si>
-  <si>
-    <t>2025NE000770, 2025NE001065, 2025NE001627</t>
-  </si>
-  <si>
-    <t>REAJUSTE</t>
-  </si>
-  <si>
-    <t>2026NP402148</t>
   </si>
   <si>
     <t>MAIO/26</t>
@@ -695,8 +695,8 @@
     <numFmt numFmtId="166" formatCode="dd/MM/yyyy"/>
     <numFmt numFmtId="167" formatCode="R$ #,##0.00"/>
     <numFmt numFmtId="168" formatCode="[$R$-416]\ #,##0.00;[RED]\-[$R$-416]\ #,##0.00"/>
-    <numFmt numFmtId="169" formatCode="d/m/yyyy"/>
-    <numFmt numFmtId="170" formatCode="MM/DD/YY"/>
+    <numFmt numFmtId="169" formatCode="MM/DD/YY"/>
+    <numFmt numFmtId="170" formatCode="d/m/yyyy"/>
     <numFmt numFmtId="171" formatCode="[$R$ -416]#,##0.00"/>
     <numFmt numFmtId="172" formatCode="_([$R$ -416]* #,##0.00_);_([$R$ -416]* \(#,##0.00\);_([$R$ -416]* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
@@ -740,13 +740,13 @@
       <b/>
       <sz val="10.0"/>
       <color theme="1"/>
-      <name val="Century Gothic"/>
+      <name val="Arial"/>
     </font>
     <font>
       <b/>
       <sz val="10.0"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Century Gothic"/>
     </font>
     <font>
       <sz val="10.0"/>
@@ -895,39 +895,39 @@
     <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
     <xf borderId="0" fillId="5" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
     <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="11" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="11" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="4" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="right" readingOrder="0"/>
@@ -959,26 +959,25 @@
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="6" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="0" fontId="7" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="165" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="2" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="7" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="6" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -993,23 +992,21 @@
     <xf borderId="1" fillId="7" fontId="9" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="165" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="1" fillId="5" fontId="9" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="8" fontId="7" numFmtId="168" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="8" fontId="6" numFmtId="168" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="3" fillId="0" fontId="10" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="169" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
     <xf borderId="1" fillId="8" fontId="9" numFmtId="168" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="8" numFmtId="166" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="8" numFmtId="170" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="8" numFmtId="169" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="7" fontId="9" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
@@ -1021,11 +1018,14 @@
     <xf borderId="1" fillId="8" fontId="9" numFmtId="168" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="7" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="6" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="170" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="1" fillId="9" fontId="9" numFmtId="168" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
@@ -1040,13 +1040,13 @@
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="4" fillId="0" fontId="10" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="1" fillId="0" fontId="7" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="6" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="7" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="6" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="7" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="6" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="5" fontId="9" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
@@ -1055,7 +1055,7 @@
     <xf borderId="1" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="7" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="6" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="5" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -1447,56 +1447,56 @@
     </row>
     <row r="2" ht="59.25" customHeight="1">
       <c r="A2" s="4"/>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="V2" s="8"/>
-      <c r="W2" s="10"/>
-      <c r="X2" s="10"/>
-      <c r="Y2" s="10"/>
-      <c r="Z2" s="10"/>
-      <c r="AA2" s="10"/>
-      <c r="AB2" s="10"/>
-      <c r="AC2" s="10"/>
-      <c r="AD2" s="10"/>
+      <c r="V2" s="6"/>
+      <c r="W2" s="8"/>
+      <c r="X2" s="8"/>
+      <c r="Y2" s="8"/>
+      <c r="Z2" s="8"/>
+      <c r="AA2" s="8"/>
+      <c r="AB2" s="8"/>
+      <c r="AC2" s="8"/>
+      <c r="AD2" s="8"/>
     </row>
     <row r="3" ht="12.75" customHeight="1">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
-      <c r="C3" s="12"/>
-      <c r="D3" s="12"/>
-      <c r="E3" s="12"/>
-      <c r="F3" s="12"/>
-      <c r="G3" s="12"/>
-      <c r="H3" s="12"/>
-      <c r="I3" s="12"/>
-      <c r="J3" s="12"/>
-      <c r="K3" s="12"/>
-      <c r="L3" s="12"/>
-      <c r="M3" s="12"/>
-      <c r="N3" s="12"/>
-      <c r="O3" s="12"/>
-      <c r="P3" s="12"/>
-      <c r="Q3" s="12"/>
-      <c r="R3" s="12"/>
-      <c r="S3" s="12"/>
-      <c r="T3" s="12"/>
-      <c r="U3" s="12"/>
+      <c r="C3" s="10"/>
+      <c r="D3" s="10"/>
+      <c r="E3" s="10"/>
+      <c r="F3" s="10"/>
+      <c r="G3" s="10"/>
+      <c r="H3" s="10"/>
+      <c r="I3" s="10"/>
+      <c r="J3" s="10"/>
+      <c r="K3" s="10"/>
+      <c r="L3" s="10"/>
+      <c r="M3" s="10"/>
+      <c r="N3" s="10"/>
+      <c r="O3" s="10"/>
+      <c r="P3" s="10"/>
+      <c r="Q3" s="10"/>
+      <c r="R3" s="10"/>
+      <c r="S3" s="10"/>
+      <c r="T3" s="10"/>
+      <c r="U3" s="10"/>
       <c r="V3" s="3"/>
     </row>
     <row r="4" ht="12.75" customHeight="1">
       <c r="A4" s="14"/>
       <c r="B4" s="14"/>
-      <c r="C4" s="16" t="s">
+      <c r="C4" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="D4" s="16" t="s">
+      <c r="D4" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="E4" s="16" t="s">
+      <c r="E4" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="F4" s="16" t="s">
+      <c r="F4" s="15" t="s">
         <v>9</v>
       </c>
       <c r="G4" s="17" t="s">
@@ -1505,16 +1505,16 @@
       <c r="H4" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="I4" s="16" t="s">
+      <c r="I4" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="J4" s="16" t="s">
+      <c r="J4" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="K4" s="16" t="s">
+      <c r="K4" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="L4" s="16" t="s">
+      <c r="L4" s="15" t="s">
         <v>15</v>
       </c>
       <c r="M4" s="17" t="s">
@@ -1532,16 +1532,16 @@
       <c r="Q4" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="R4" s="16" t="s">
+      <c r="R4" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="S4" s="16" t="s">
+      <c r="S4" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="T4" s="16" t="s">
+      <c r="T4" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="U4" s="16" t="s">
+      <c r="U4" s="15" t="s">
         <v>27</v>
       </c>
       <c r="V4" s="3"/>
@@ -1554,13 +1554,13 @@
         <v>28</v>
       </c>
       <c r="E5" s="19" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F5" s="19" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="G5" s="19" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="H5" s="20">
         <v>1564.0</v>
@@ -1569,7 +1569,7 @@
         <v>1564.0</v>
       </c>
       <c r="J5" s="19" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="K5" s="19" t="s">
         <v>35</v>
@@ -1596,7 +1596,7 @@
         <v>1.085943044E7</v>
       </c>
       <c r="S5" s="19" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="V5" s="3"/>
     </row>
@@ -1622,82 +1622,82 @@
       <c r="M7" s="25"/>
       <c r="N7" s="25"/>
       <c r="O7" s="25"/>
-      <c r="P7" s="28"/>
+      <c r="P7" s="27"/>
       <c r="V7" s="3"/>
     </row>
     <row r="8" ht="12.75" customHeight="1">
       <c r="A8" s="23"/>
       <c r="B8" s="23"/>
-      <c r="C8" s="29" t="s">
-        <v>56</v>
-      </c>
-      <c r="D8" s="29" t="s">
-        <v>58</v>
+      <c r="C8" s="28" t="s">
+        <v>49</v>
+      </c>
+      <c r="D8" s="28" t="s">
+        <v>50</v>
       </c>
       <c r="E8" s="30" t="s">
+        <v>51</v>
+      </c>
+      <c r="F8" s="28" t="s">
+        <v>52</v>
+      </c>
+      <c r="G8" s="28" t="s">
+        <v>54</v>
+      </c>
+      <c r="H8" s="28" t="s">
+        <v>55</v>
+      </c>
+      <c r="I8" s="30" t="s">
+        <v>57</v>
+      </c>
+      <c r="J8" s="28" t="s">
+        <v>59</v>
+      </c>
+      <c r="K8" s="28" t="s">
+        <v>60</v>
+      </c>
+      <c r="L8" s="31" t="s">
         <v>61</v>
       </c>
-      <c r="F8" s="29" t="s">
+      <c r="M8" s="30" t="s">
+        <v>63</v>
+      </c>
+      <c r="N8" s="28" t="s">
         <v>64</v>
       </c>
-      <c r="G8" s="29" t="s">
-        <v>65</v>
-      </c>
-      <c r="H8" s="29" t="s">
-        <v>66</v>
-      </c>
-      <c r="I8" s="30" t="s">
-        <v>67</v>
-      </c>
-      <c r="J8" s="29" t="s">
-        <v>69</v>
-      </c>
-      <c r="K8" s="29" t="s">
-        <v>71</v>
-      </c>
-      <c r="L8" s="31" t="s">
-        <v>72</v>
-      </c>
-      <c r="M8" s="30" t="s">
-        <v>73</v>
-      </c>
-      <c r="N8" s="29" t="s">
-        <v>74</v>
-      </c>
-      <c r="O8" s="29"/>
-      <c r="P8" s="28"/>
+      <c r="O8" s="28"/>
+      <c r="P8" s="27"/>
       <c r="V8" s="3"/>
     </row>
     <row r="9" ht="19.5" customHeight="1">
       <c r="A9" s="23"/>
       <c r="B9" s="23"/>
-      <c r="C9" s="33">
+      <c r="C9" s="32">
         <v>1.0</v>
       </c>
-      <c r="D9" s="34" t="s">
-        <v>81</v>
-      </c>
-      <c r="E9" s="35" t="s">
-        <v>83</v>
-      </c>
-      <c r="F9" s="36">
+      <c r="D9" s="33" t="s">
+        <v>67</v>
+      </c>
+      <c r="E9" s="34" t="s">
+        <v>68</v>
+      </c>
+      <c r="F9" s="35">
         <v>594.0</v>
       </c>
-      <c r="G9" s="37">
+      <c r="G9" s="36">
         <v>45740.0</v>
       </c>
-      <c r="H9" s="36" t="s">
-        <v>86</v>
-      </c>
-      <c r="I9" s="37"/>
-      <c r="J9" s="37">
+      <c r="H9" s="35" t="s">
+        <v>71</v>
+      </c>
+      <c r="I9" s="36"/>
+      <c r="J9" s="36">
         <v>45778.0</v>
       </c>
-      <c r="K9" s="38">
+      <c r="K9" s="37">
         <v>748504.24</v>
       </c>
-      <c r="L9" s="36" t="s">
-        <v>89</v>
+      <c r="L9" s="35" t="s">
+        <v>75</v>
       </c>
       <c r="M9" s="39">
         <f t="shared" ref="M9:M10" si="1">K9</f>
@@ -1705,228 +1705,228 @@
       </c>
       <c r="N9" s="40"/>
       <c r="O9" s="25"/>
-      <c r="P9" s="28"/>
+      <c r="P9" s="27"/>
       <c r="V9" s="3"/>
     </row>
     <row r="10" ht="51.0" customHeight="1">
       <c r="A10" s="23"/>
       <c r="B10" s="23"/>
       <c r="C10" s="41"/>
-      <c r="D10" s="34" t="s">
-        <v>98</v>
-      </c>
-      <c r="E10" s="35" t="s">
-        <v>83</v>
-      </c>
-      <c r="F10" s="36">
+      <c r="D10" s="33" t="s">
+        <v>85</v>
+      </c>
+      <c r="E10" s="34" t="s">
+        <v>68</v>
+      </c>
+      <c r="F10" s="35">
         <v>620.0</v>
       </c>
-      <c r="G10" s="37">
+      <c r="G10" s="36">
         <v>45775.0</v>
       </c>
-      <c r="H10" s="36" t="s">
-        <v>102</v>
-      </c>
-      <c r="I10" s="37"/>
-      <c r="J10" s="37">
+      <c r="H10" s="35" t="s">
+        <v>86</v>
+      </c>
+      <c r="I10" s="36"/>
+      <c r="J10" s="36">
         <v>45806.0</v>
       </c>
-      <c r="K10" s="38">
+      <c r="K10" s="37">
         <v>1110378.24</v>
       </c>
-      <c r="L10" s="36" t="s">
-        <v>103</v>
+      <c r="L10" s="35" t="s">
+        <v>87</v>
       </c>
       <c r="M10" s="39">
         <f t="shared" si="1"/>
         <v>1110378.24</v>
       </c>
-      <c r="N10" s="43"/>
+      <c r="N10" s="42"/>
       <c r="O10" s="25"/>
-      <c r="P10" s="28"/>
+      <c r="P10" s="27"/>
       <c r="V10" s="3"/>
     </row>
     <row r="11" ht="12.75" customHeight="1">
       <c r="A11" s="23"/>
       <c r="B11" s="23"/>
       <c r="C11" s="41"/>
-      <c r="D11" s="34" t="s">
-        <v>108</v>
-      </c>
-      <c r="E11" s="35" t="s">
-        <v>83</v>
-      </c>
-      <c r="F11" s="36">
+      <c r="D11" s="33" t="s">
+        <v>93</v>
+      </c>
+      <c r="E11" s="34" t="s">
+        <v>68</v>
+      </c>
+      <c r="F11" s="35">
         <v>634.0</v>
       </c>
-      <c r="G11" s="37">
+      <c r="G11" s="36">
         <v>45799.0</v>
       </c>
-      <c r="H11" s="36" t="s">
-        <v>110</v>
-      </c>
-      <c r="I11" s="37"/>
-      <c r="J11" s="37">
+      <c r="H11" s="35" t="s">
+        <v>94</v>
+      </c>
+      <c r="I11" s="36"/>
+      <c r="J11" s="36">
         <v>45844.0</v>
       </c>
-      <c r="K11" s="38">
+      <c r="K11" s="37">
         <v>974557.12</v>
       </c>
-      <c r="L11" s="35" t="s">
-        <v>112</v>
+      <c r="L11" s="34" t="s">
+        <v>95</v>
       </c>
       <c r="M11" s="39">
         <v>974557.12</v>
       </c>
-      <c r="N11" s="43"/>
+      <c r="N11" s="42"/>
       <c r="O11" s="25"/>
-      <c r="P11" s="28"/>
+      <c r="P11" s="27"/>
       <c r="V11" s="3"/>
     </row>
     <row r="12" ht="27.75" customHeight="1">
       <c r="A12" s="23"/>
       <c r="B12" s="23"/>
       <c r="C12" s="41"/>
-      <c r="D12" s="34" t="s">
-        <v>114</v>
-      </c>
-      <c r="E12" s="35" t="s">
-        <v>83</v>
-      </c>
-      <c r="F12" s="35">
+      <c r="D12" s="33" t="s">
+        <v>98</v>
+      </c>
+      <c r="E12" s="34" t="s">
+        <v>68</v>
+      </c>
+      <c r="F12" s="34">
         <v>660.0</v>
       </c>
-      <c r="G12" s="44">
+      <c r="G12" s="43">
         <v>45856.0</v>
       </c>
-      <c r="H12" s="45" t="s">
-        <v>59</v>
-      </c>
-      <c r="I12" s="37"/>
-      <c r="J12" s="37">
+      <c r="H12" s="44" t="s">
+        <v>72</v>
+      </c>
+      <c r="I12" s="36"/>
+      <c r="J12" s="36">
         <v>45891.0</v>
       </c>
-      <c r="K12" s="46">
+      <c r="K12" s="45">
         <v>1402001.34</v>
       </c>
-      <c r="L12" s="47" t="s">
-        <v>118</v>
+      <c r="L12" s="46" t="s">
+        <v>101</v>
       </c>
       <c r="M12" s="39">
         <v>1402001.34</v>
       </c>
-      <c r="N12" s="48"/>
+      <c r="N12" s="47"/>
       <c r="O12" s="25"/>
-      <c r="P12" s="28"/>
+      <c r="P12" s="27"/>
       <c r="V12" s="3"/>
     </row>
     <row r="13">
       <c r="A13" s="23"/>
       <c r="B13" s="23"/>
       <c r="C13" s="41"/>
-      <c r="D13" s="49" t="s">
-        <v>123</v>
-      </c>
-      <c r="E13" s="35" t="s">
-        <v>83</v>
-      </c>
-      <c r="F13" s="36">
+      <c r="D13" s="48" t="s">
+        <v>106</v>
+      </c>
+      <c r="E13" s="34" t="s">
+        <v>68</v>
+      </c>
+      <c r="F13" s="35">
         <v>661.0</v>
       </c>
-      <c r="G13" s="37">
+      <c r="G13" s="36">
         <v>45856.0</v>
       </c>
-      <c r="H13" s="36" t="s">
-        <v>127</v>
-      </c>
-      <c r="I13" s="44"/>
-      <c r="J13" s="44">
+      <c r="H13" s="35" t="s">
+        <v>107</v>
+      </c>
+      <c r="I13" s="43"/>
+      <c r="J13" s="43">
         <v>45891.0</v>
       </c>
-      <c r="K13" s="46">
+      <c r="K13" s="45">
         <v>1223702.3</v>
       </c>
-      <c r="L13" s="35" t="s">
-        <v>131</v>
+      <c r="L13" s="34" t="s">
+        <v>109</v>
       </c>
       <c r="M13" s="39">
         <v>1223702.3</v>
       </c>
-      <c r="N13" s="48"/>
+      <c r="N13" s="47"/>
       <c r="O13" s="25"/>
-      <c r="P13" s="50"/>
+      <c r="P13" s="49"/>
       <c r="V13" s="3"/>
     </row>
     <row r="14">
       <c r="A14" s="23"/>
       <c r="B14" s="23"/>
       <c r="C14" s="41"/>
-      <c r="D14" s="49" t="s">
-        <v>135</v>
-      </c>
-      <c r="E14" s="35" t="s">
-        <v>83</v>
-      </c>
-      <c r="F14" s="35">
+      <c r="D14" s="48" t="s">
+        <v>112</v>
+      </c>
+      <c r="E14" s="34" t="s">
+        <v>68</v>
+      </c>
+      <c r="F14" s="34">
         <v>688.0</v>
       </c>
-      <c r="G14" s="37">
+      <c r="G14" s="36">
         <v>45901.0</v>
       </c>
-      <c r="H14" s="35" t="s">
-        <v>136</v>
-      </c>
-      <c r="I14" s="44"/>
-      <c r="J14" s="44">
+      <c r="H14" s="34" t="s">
+        <v>113</v>
+      </c>
+      <c r="I14" s="43"/>
+      <c r="J14" s="43">
         <v>45938.0</v>
       </c>
-      <c r="K14" s="46">
+      <c r="K14" s="45">
         <v>1011677.95</v>
       </c>
-      <c r="L14" s="35" t="s">
-        <v>137</v>
+      <c r="L14" s="34" t="s">
+        <v>114</v>
       </c>
       <c r="M14" s="39">
         <v>1011677.95</v>
       </c>
-      <c r="N14" s="43"/>
+      <c r="N14" s="42"/>
       <c r="O14" s="25"/>
-      <c r="P14" s="28"/>
+      <c r="P14" s="27"/>
       <c r="V14" s="3"/>
     </row>
     <row r="15">
       <c r="A15" s="23"/>
       <c r="B15" s="23"/>
       <c r="C15" s="41"/>
-      <c r="D15" s="49" t="s">
-        <v>141</v>
-      </c>
-      <c r="E15" s="35" t="s">
-        <v>83</v>
-      </c>
-      <c r="F15" s="35">
+      <c r="D15" s="48" t="s">
+        <v>118</v>
+      </c>
+      <c r="E15" s="34" t="s">
+        <v>68</v>
+      </c>
+      <c r="F15" s="34">
         <v>696.0</v>
       </c>
-      <c r="G15" s="37">
+      <c r="G15" s="36">
         <v>45923.0</v>
       </c>
-      <c r="H15" s="35" t="s">
-        <v>75</v>
-      </c>
-      <c r="I15" s="44"/>
-      <c r="J15" s="44">
+      <c r="H15" s="34" t="s">
+        <v>79</v>
+      </c>
+      <c r="I15" s="43"/>
+      <c r="J15" s="43">
         <v>45938.0</v>
       </c>
-      <c r="K15" s="46">
+      <c r="K15" s="45">
         <v>896744.06</v>
       </c>
-      <c r="L15" s="35" t="s">
-        <v>142</v>
+      <c r="L15" s="34" t="s">
+        <v>120</v>
       </c>
       <c r="M15" s="39">
         <v>896744.06</v>
       </c>
-      <c r="N15" s="48"/>
+      <c r="N15" s="47"/>
       <c r="O15" s="25"/>
       <c r="V15" s="3"/>
     </row>
@@ -1934,35 +1934,35 @@
       <c r="A16" s="23"/>
       <c r="B16" s="23"/>
       <c r="C16" s="41"/>
-      <c r="D16" s="49" t="s">
-        <v>144</v>
-      </c>
-      <c r="E16" s="35" t="s">
-        <v>83</v>
-      </c>
-      <c r="F16" s="35">
+      <c r="D16" s="48" t="s">
+        <v>123</v>
+      </c>
+      <c r="E16" s="34" t="s">
+        <v>68</v>
+      </c>
+      <c r="F16" s="34">
         <v>704.0</v>
       </c>
-      <c r="G16" s="37">
+      <c r="G16" s="36">
         <v>45957.0</v>
       </c>
-      <c r="H16" s="35" t="s">
-        <v>146</v>
-      </c>
-      <c r="I16" s="44"/>
-      <c r="J16" s="44">
+      <c r="H16" s="34" t="s">
+        <v>127</v>
+      </c>
+      <c r="I16" s="43"/>
+      <c r="J16" s="43">
         <v>46003.0</v>
       </c>
-      <c r="K16" s="46">
+      <c r="K16" s="45">
         <v>919329.06</v>
       </c>
-      <c r="L16" s="35" t="s">
-        <v>147</v>
+      <c r="L16" s="34" t="s">
+        <v>128</v>
       </c>
       <c r="M16" s="39">
         <v>919329.06</v>
       </c>
-      <c r="N16" s="43"/>
+      <c r="N16" s="42"/>
       <c r="O16" s="25"/>
       <c r="V16" s="3"/>
     </row>
@@ -1970,28 +1970,28 @@
       <c r="A17" s="23"/>
       <c r="B17" s="23"/>
       <c r="C17" s="41"/>
-      <c r="D17" s="49" t="s">
-        <v>148</v>
-      </c>
-      <c r="E17" s="35"/>
-      <c r="F17" s="35">
+      <c r="D17" s="48" t="s">
+        <v>129</v>
+      </c>
+      <c r="E17" s="34"/>
+      <c r="F17" s="34">
         <v>705.0</v>
       </c>
-      <c r="G17" s="44">
+      <c r="G17" s="43">
         <v>45972.0</v>
       </c>
-      <c r="H17" s="35" t="s">
-        <v>150</v>
-      </c>
-      <c r="I17" s="35"/>
-      <c r="J17" s="44">
+      <c r="H17" s="34" t="s">
+        <v>131</v>
+      </c>
+      <c r="I17" s="34"/>
+      <c r="J17" s="43">
         <v>46016.0</v>
       </c>
-      <c r="K17" s="46">
+      <c r="K17" s="45">
         <v>1157009.26</v>
       </c>
-      <c r="L17" s="35" t="s">
-        <v>152</v>
+      <c r="L17" s="34" t="s">
+        <v>133</v>
       </c>
       <c r="M17" s="39">
         <v>1157009.26</v>
@@ -2004,297 +2004,297 @@
       <c r="A18" s="23"/>
       <c r="B18" s="23"/>
       <c r="C18" s="41"/>
-      <c r="D18" s="49" t="s">
-        <v>157</v>
-      </c>
-      <c r="E18" s="35" t="s">
-        <v>83</v>
-      </c>
-      <c r="F18" s="35">
+      <c r="D18" s="48" t="s">
+        <v>137</v>
+      </c>
+      <c r="E18" s="34" t="s">
+        <v>68</v>
+      </c>
+      <c r="F18" s="34">
         <v>728.0</v>
       </c>
-      <c r="G18" s="44">
+      <c r="G18" s="43">
         <v>46008.0</v>
       </c>
-      <c r="H18" s="35" t="s">
-        <v>158</v>
-      </c>
-      <c r="I18" s="35"/>
-      <c r="J18" s="44">
+      <c r="H18" s="34" t="s">
+        <v>138</v>
+      </c>
+      <c r="I18" s="34"/>
+      <c r="J18" s="43">
         <v>46040.0</v>
       </c>
-      <c r="K18" s="46">
+      <c r="K18" s="45">
         <v>1214597.952</v>
       </c>
-      <c r="L18" s="35" t="s">
-        <v>159</v>
+      <c r="L18" s="34" t="s">
+        <v>139</v>
       </c>
       <c r="M18" s="39">
         <v>1214597.952</v>
       </c>
       <c r="N18" s="51"/>
       <c r="O18" s="25"/>
-      <c r="R18" s="28"/>
-      <c r="S18" s="28"/>
-      <c r="T18" s="28"/>
-      <c r="U18" s="28"/>
+      <c r="R18" s="27"/>
+      <c r="S18" s="27"/>
+      <c r="T18" s="27"/>
+      <c r="U18" s="27"/>
       <c r="V18" s="52"/>
     </row>
     <row r="19">
       <c r="A19" s="23"/>
       <c r="B19" s="23"/>
       <c r="C19" s="41"/>
-      <c r="D19" s="49" t="s">
-        <v>160</v>
-      </c>
-      <c r="E19" s="35" t="s">
-        <v>83</v>
-      </c>
-      <c r="F19" s="35">
+      <c r="D19" s="48" t="s">
+        <v>143</v>
+      </c>
+      <c r="E19" s="34" t="s">
+        <v>68</v>
+      </c>
+      <c r="F19" s="34">
         <v>278.0</v>
       </c>
-      <c r="G19" s="44">
+      <c r="G19" s="43">
         <v>46042.0</v>
       </c>
-      <c r="H19" s="35" t="s">
-        <v>161</v>
-      </c>
-      <c r="I19" s="44"/>
-      <c r="J19" s="44">
+      <c r="H19" s="34" t="s">
+        <v>144</v>
+      </c>
+      <c r="I19" s="43"/>
+      <c r="J19" s="43">
         <v>46074.0</v>
       </c>
-      <c r="K19" s="46">
+      <c r="K19" s="45">
         <v>967082.09</v>
       </c>
-      <c r="L19" s="35" t="s">
-        <v>162</v>
+      <c r="L19" s="34" t="s">
+        <v>145</v>
       </c>
       <c r="M19" s="39">
         <v>967082.09</v>
       </c>
       <c r="N19" s="51"/>
       <c r="O19" s="25"/>
-      <c r="R19" s="28"/>
-      <c r="S19" s="28"/>
-      <c r="T19" s="28"/>
-      <c r="U19" s="28"/>
+      <c r="R19" s="27"/>
+      <c r="S19" s="27"/>
+      <c r="T19" s="27"/>
+      <c r="U19" s="27"/>
       <c r="V19" s="52"/>
     </row>
     <row r="20">
       <c r="A20" s="23"/>
       <c r="B20" s="23"/>
       <c r="C20" s="41"/>
-      <c r="D20" s="49" t="s">
-        <v>163</v>
-      </c>
-      <c r="E20" s="35"/>
-      <c r="F20" s="35">
+      <c r="D20" s="48" t="s">
+        <v>149</v>
+      </c>
+      <c r="E20" s="34"/>
+      <c r="F20" s="34">
         <v>10.0</v>
       </c>
-      <c r="G20" s="44">
+      <c r="G20" s="43">
         <v>46078.0</v>
       </c>
-      <c r="H20" s="35" t="s">
-        <v>99</v>
-      </c>
-      <c r="I20" s="44"/>
-      <c r="J20" s="44">
+      <c r="H20" s="34" t="s">
+        <v>108</v>
+      </c>
+      <c r="I20" s="43"/>
+      <c r="J20" s="43">
         <v>46106.0</v>
       </c>
-      <c r="K20" s="46">
+      <c r="K20" s="45">
         <v>719561.08</v>
       </c>
-      <c r="L20" s="35" t="s">
-        <v>164</v>
+      <c r="L20" s="34" t="s">
+        <v>150</v>
       </c>
       <c r="M20" s="39">
         <v>719561.08</v>
       </c>
       <c r="N20" s="51"/>
       <c r="O20" s="25"/>
-      <c r="R20" s="28"/>
-      <c r="S20" s="28"/>
-      <c r="T20" s="28"/>
-      <c r="U20" s="28"/>
+      <c r="R20" s="27"/>
+      <c r="S20" s="27"/>
+      <c r="T20" s="27"/>
+      <c r="U20" s="27"/>
       <c r="V20" s="52"/>
     </row>
     <row r="21">
       <c r="A21" s="23"/>
       <c r="B21" s="23"/>
       <c r="C21" s="41"/>
-      <c r="D21" s="49" t="s">
-        <v>165</v>
-      </c>
-      <c r="E21" s="35"/>
-      <c r="F21" s="35">
+      <c r="D21" s="48" t="s">
+        <v>154</v>
+      </c>
+      <c r="E21" s="34"/>
+      <c r="F21" s="34">
         <v>15.0</v>
       </c>
-      <c r="G21" s="44">
+      <c r="G21" s="43">
         <v>46094.0</v>
       </c>
-      <c r="H21" s="35" t="s">
-        <v>166</v>
-      </c>
-      <c r="I21" s="44"/>
-      <c r="J21" s="44">
+      <c r="H21" s="34" t="s">
+        <v>155</v>
+      </c>
+      <c r="I21" s="43"/>
+      <c r="J21" s="43">
         <v>46128.0</v>
       </c>
-      <c r="K21" s="46">
+      <c r="K21" s="45">
         <v>885881.08</v>
       </c>
-      <c r="L21" s="35" t="s">
-        <v>167</v>
+      <c r="L21" s="34" t="s">
+        <v>156</v>
       </c>
       <c r="M21" s="39">
         <v>885881.08</v>
       </c>
       <c r="N21" s="51"/>
       <c r="O21" s="25"/>
-      <c r="R21" s="28"/>
-      <c r="S21" s="28"/>
-      <c r="T21" s="28"/>
-      <c r="U21" s="28"/>
+      <c r="R21" s="27"/>
+      <c r="S21" s="27"/>
+      <c r="T21" s="27"/>
+      <c r="U21" s="27"/>
       <c r="V21" s="52"/>
     </row>
     <row r="22">
       <c r="A22" s="23"/>
       <c r="B22" s="23"/>
       <c r="C22" s="41"/>
-      <c r="D22" s="49" t="s">
-        <v>168</v>
-      </c>
-      <c r="E22" s="35"/>
-      <c r="F22" s="35">
+      <c r="D22" s="48" t="s">
+        <v>160</v>
+      </c>
+      <c r="E22" s="34"/>
+      <c r="F22" s="34">
         <v>28.0</v>
       </c>
-      <c r="G22" s="44">
+      <c r="G22" s="43">
         <v>46128.0</v>
       </c>
-      <c r="H22" s="35" t="s">
-        <v>169</v>
-      </c>
-      <c r="I22" s="44"/>
-      <c r="J22" s="44">
+      <c r="H22" s="34" t="s">
+        <v>161</v>
+      </c>
+      <c r="I22" s="43"/>
+      <c r="J22" s="43">
         <v>46164.0</v>
       </c>
-      <c r="K22" s="46" t="s">
-        <v>170</v>
-      </c>
-      <c r="L22" s="35" t="s">
-        <v>171</v>
+      <c r="K22" s="45" t="s">
+        <v>162</v>
+      </c>
+      <c r="L22" s="34" t="s">
+        <v>163</v>
       </c>
       <c r="M22" s="39" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="N22" s="51"/>
       <c r="O22" s="25"/>
-      <c r="R22" s="28"/>
-      <c r="S22" s="28"/>
-      <c r="T22" s="28"/>
-      <c r="U22" s="28"/>
+      <c r="R22" s="27"/>
+      <c r="S22" s="27"/>
+      <c r="T22" s="27"/>
+      <c r="U22" s="27"/>
       <c r="V22" s="52"/>
     </row>
     <row r="23">
       <c r="A23" s="23"/>
       <c r="B23" s="23"/>
       <c r="C23" s="41"/>
-      <c r="D23" s="49" t="s">
-        <v>172</v>
-      </c>
-      <c r="E23" s="35"/>
-      <c r="F23" s="35">
+      <c r="D23" s="48" t="s">
+        <v>166</v>
+      </c>
+      <c r="E23" s="34"/>
+      <c r="F23" s="34">
         <v>33.0</v>
       </c>
-      <c r="G23" s="44">
+      <c r="G23" s="43">
         <v>46156.0</v>
       </c>
-      <c r="H23" s="35" t="s">
-        <v>173</v>
-      </c>
-      <c r="I23" s="44"/>
-      <c r="J23" s="44">
+      <c r="H23" s="34" t="s">
+        <v>167</v>
+      </c>
+      <c r="I23" s="43"/>
+      <c r="J23" s="43">
         <v>46191.0</v>
       </c>
-      <c r="K23" s="46">
+      <c r="K23" s="45">
         <v>1108954.4358333333</v>
       </c>
-      <c r="L23" s="35" t="s">
-        <v>167</v>
+      <c r="L23" s="34" t="s">
+        <v>156</v>
       </c>
       <c r="M23" s="39">
         <v>1108954.4358333333</v>
       </c>
       <c r="N23" s="53"/>
       <c r="O23" s="25"/>
-      <c r="R23" s="28"/>
-      <c r="S23" s="28"/>
-      <c r="T23" s="28"/>
-      <c r="U23" s="28"/>
+      <c r="R23" s="27"/>
+      <c r="S23" s="27"/>
+      <c r="T23" s="27"/>
+      <c r="U23" s="27"/>
       <c r="V23" s="52"/>
     </row>
     <row r="24">
       <c r="A24" s="23"/>
       <c r="B24" s="23"/>
       <c r="C24" s="41"/>
-      <c r="D24" s="49" t="s">
+      <c r="D24" s="48" t="s">
+        <v>170</v>
+      </c>
+      <c r="E24" s="34"/>
+      <c r="F24" s="34">
+        <v>29.0</v>
+      </c>
+      <c r="G24" s="43">
+        <v>46149.0</v>
+      </c>
+      <c r="H24" s="34" t="s">
+        <v>167</v>
+      </c>
+      <c r="I24" s="43"/>
+      <c r="J24" s="43">
+        <v>46185.0</v>
+      </c>
+      <c r="K24" s="45">
+        <v>218206.1</v>
+      </c>
+      <c r="L24" s="34" t="s">
         <v>174</v>
-      </c>
-      <c r="E24" s="35"/>
-      <c r="F24" s="35">
-        <v>29.0</v>
-      </c>
-      <c r="G24" s="44">
-        <v>46149.0</v>
-      </c>
-      <c r="H24" s="35" t="s">
-        <v>173</v>
-      </c>
-      <c r="I24" s="44"/>
-      <c r="J24" s="44">
-        <v>46185.0</v>
-      </c>
-      <c r="K24" s="46">
-        <v>218206.1</v>
-      </c>
-      <c r="L24" s="35" t="s">
-        <v>175</v>
       </c>
       <c r="M24" s="39">
         <v>218206.1</v>
       </c>
       <c r="N24" s="54"/>
       <c r="O24" s="25"/>
-      <c r="R24" s="28"/>
-      <c r="S24" s="28"/>
-      <c r="T24" s="28"/>
-      <c r="U24" s="28"/>
+      <c r="R24" s="27"/>
+      <c r="S24" s="27"/>
+      <c r="T24" s="27"/>
+      <c r="U24" s="27"/>
       <c r="V24" s="52"/>
     </row>
     <row r="25">
       <c r="A25" s="23"/>
       <c r="B25" s="23"/>
       <c r="C25" s="41"/>
-      <c r="D25" s="49" t="s">
+      <c r="D25" s="48" t="s">
         <v>176</v>
       </c>
-      <c r="E25" s="35"/>
-      <c r="F25" s="35">
+      <c r="E25" s="34"/>
+      <c r="F25" s="34">
         <v>40.0</v>
       </c>
-      <c r="G25" s="44">
+      <c r="G25" s="43">
         <v>46156.0</v>
       </c>
-      <c r="H25" s="35" t="s">
-        <v>173</v>
-      </c>
-      <c r="I25" s="44"/>
-      <c r="J25" s="44">
+      <c r="H25" s="34" t="s">
+        <v>167</v>
+      </c>
+      <c r="I25" s="43"/>
+      <c r="J25" s="43">
         <v>46191.0</v>
       </c>
-      <c r="K25" s="46">
+      <c r="K25" s="45">
         <v>1549250.84</v>
       </c>
-      <c r="L25" s="35" t="s">
+      <c r="L25" s="34" t="s">
         <v>177</v>
       </c>
       <c r="M25" s="39">
@@ -2302,37 +2302,37 @@
       </c>
       <c r="N25" s="54"/>
       <c r="O25" s="25"/>
-      <c r="R25" s="28"/>
-      <c r="S25" s="28"/>
-      <c r="T25" s="28"/>
-      <c r="U25" s="28"/>
+      <c r="R25" s="27"/>
+      <c r="S25" s="27"/>
+      <c r="T25" s="27"/>
+      <c r="U25" s="27"/>
       <c r="V25" s="52"/>
     </row>
     <row r="26">
       <c r="A26" s="23"/>
       <c r="B26" s="23"/>
       <c r="C26" s="55"/>
-      <c r="D26" s="49" t="s">
+      <c r="D26" s="48" t="s">
         <v>178</v>
       </c>
-      <c r="E26" s="35"/>
-      <c r="F26" s="35">
+      <c r="E26" s="34"/>
+      <c r="F26" s="34">
         <v>48.0</v>
       </c>
-      <c r="G26" s="44">
+      <c r="G26" s="43">
         <v>46230.0</v>
       </c>
-      <c r="H26" s="35" t="s">
+      <c r="H26" s="34" t="s">
         <v>179</v>
       </c>
-      <c r="I26" s="44"/>
-      <c r="J26" s="44">
+      <c r="I26" s="43"/>
+      <c r="J26" s="43">
         <v>46262.0</v>
       </c>
-      <c r="K26" s="46" t="s">
+      <c r="K26" s="45" t="s">
         <v>180</v>
       </c>
-      <c r="L26" s="35" t="s">
+      <c r="L26" s="34" t="s">
         <v>181</v>
       </c>
       <c r="M26" s="39" t="s">
@@ -2340,113 +2340,113 @@
       </c>
       <c r="N26" s="54"/>
       <c r="O26" s="25"/>
-      <c r="R26" s="28"/>
-      <c r="S26" s="28"/>
-      <c r="T26" s="28"/>
-      <c r="U26" s="28"/>
+      <c r="R26" s="27"/>
+      <c r="S26" s="27"/>
+      <c r="T26" s="27"/>
+      <c r="U26" s="27"/>
       <c r="V26" s="52"/>
     </row>
     <row r="27">
       <c r="A27" s="23"/>
       <c r="B27" s="23"/>
-      <c r="C27" s="36"/>
-      <c r="D27" s="49" t="s">
+      <c r="C27" s="35"/>
+      <c r="D27" s="48" t="s">
         <v>182</v>
       </c>
-      <c r="E27" s="35"/>
-      <c r="F27" s="35"/>
-      <c r="G27" s="44"/>
-      <c r="H27" s="35"/>
-      <c r="I27" s="44"/>
-      <c r="J27" s="44"/>
-      <c r="K27" s="46"/>
-      <c r="L27" s="35"/>
+      <c r="E27" s="34"/>
+      <c r="F27" s="34"/>
+      <c r="G27" s="43"/>
+      <c r="H27" s="34"/>
+      <c r="I27" s="43"/>
+      <c r="J27" s="43"/>
+      <c r="K27" s="45"/>
+      <c r="L27" s="34"/>
       <c r="M27" s="39"/>
       <c r="N27" s="54" t="s">
         <v>183</v>
       </c>
       <c r="O27" s="25"/>
-      <c r="R27" s="28"/>
-      <c r="S27" s="28"/>
-      <c r="T27" s="28"/>
-      <c r="U27" s="28"/>
+      <c r="R27" s="27"/>
+      <c r="S27" s="27"/>
+      <c r="T27" s="27"/>
+      <c r="U27" s="27"/>
       <c r="V27" s="52"/>
     </row>
     <row r="28" ht="30.75" customHeight="1">
       <c r="A28" s="23"/>
       <c r="B28" s="23"/>
-      <c r="C28" s="29" t="s">
-        <v>56</v>
-      </c>
-      <c r="D28" s="29" t="s">
-        <v>58</v>
+      <c r="C28" s="28" t="s">
+        <v>49</v>
+      </c>
+      <c r="D28" s="28" t="s">
+        <v>50</v>
       </c>
       <c r="E28" s="30" t="s">
+        <v>51</v>
+      </c>
+      <c r="F28" s="28" t="s">
+        <v>52</v>
+      </c>
+      <c r="G28" s="28"/>
+      <c r="H28" s="28" t="s">
+        <v>55</v>
+      </c>
+      <c r="I28" s="28"/>
+      <c r="J28" s="28"/>
+      <c r="K28" s="56" t="s">
+        <v>60</v>
+      </c>
+      <c r="L28" s="31" t="s">
         <v>61</v>
       </c>
-      <c r="F28" s="29" t="s">
+      <c r="M28" s="57" t="s">
+        <v>63</v>
+      </c>
+      <c r="N28" s="28" t="s">
         <v>64</v>
       </c>
-      <c r="G28" s="29"/>
-      <c r="H28" s="29" t="s">
-        <v>66</v>
-      </c>
-      <c r="I28" s="29"/>
-      <c r="J28" s="29"/>
-      <c r="K28" s="56" t="s">
-        <v>71</v>
-      </c>
-      <c r="L28" s="31" t="s">
-        <v>72</v>
-      </c>
-      <c r="M28" s="57" t="s">
-        <v>73</v>
-      </c>
-      <c r="N28" s="29" t="s">
-        <v>74</v>
-      </c>
       <c r="O28" s="25"/>
-      <c r="P28" s="28"/>
-      <c r="R28" s="28"/>
-      <c r="S28" s="28"/>
-      <c r="T28" s="28"/>
-      <c r="U28" s="28"/>
+      <c r="P28" s="27"/>
+      <c r="R28" s="27"/>
+      <c r="S28" s="27"/>
+      <c r="T28" s="27"/>
+      <c r="U28" s="27"/>
       <c r="V28" s="52"/>
-      <c r="W28" s="28"/>
-      <c r="X28" s="28"/>
-      <c r="Y28" s="28"/>
-      <c r="Z28" s="28"/>
-      <c r="AA28" s="28"/>
-      <c r="AB28" s="28"/>
-      <c r="AC28" s="28"/>
+      <c r="W28" s="27"/>
+      <c r="X28" s="27"/>
+      <c r="Y28" s="27"/>
+      <c r="Z28" s="27"/>
+      <c r="AA28" s="27"/>
+      <c r="AB28" s="27"/>
+      <c r="AC28" s="27"/>
     </row>
     <row r="29" ht="12.75" customHeight="1">
       <c r="A29" s="23"/>
       <c r="B29" s="23"/>
-      <c r="C29" s="33">
+      <c r="C29" s="32">
         <v>2.0</v>
       </c>
       <c r="D29" s="58" t="s">
         <v>184</v>
       </c>
-      <c r="E29" s="36"/>
-      <c r="F29" s="36">
+      <c r="E29" s="35"/>
+      <c r="F29" s="35">
         <v>402.0</v>
       </c>
-      <c r="G29" s="37">
+      <c r="G29" s="36">
         <v>45791.0</v>
       </c>
-      <c r="H29" s="36" t="s">
-        <v>49</v>
-      </c>
-      <c r="I29" s="37"/>
-      <c r="J29" s="37">
+      <c r="H29" s="35" t="s">
+        <v>53</v>
+      </c>
+      <c r="I29" s="36"/>
+      <c r="J29" s="36">
         <v>45834.0</v>
       </c>
-      <c r="K29" s="38">
+      <c r="K29" s="37">
         <v>188246.17</v>
       </c>
-      <c r="L29" s="35" t="s">
+      <c r="L29" s="34" t="s">
         <v>185</v>
       </c>
       <c r="M29" s="59">
@@ -2454,20 +2454,20 @@
       </c>
       <c r="N29" s="51"/>
       <c r="O29" s="25"/>
-      <c r="P29" s="28"/>
-      <c r="Q29" s="28"/>
-      <c r="R29" s="28"/>
-      <c r="S29" s="28"/>
-      <c r="T29" s="28"/>
-      <c r="U29" s="28"/>
+      <c r="P29" s="27"/>
+      <c r="Q29" s="27"/>
+      <c r="R29" s="27"/>
+      <c r="S29" s="27"/>
+      <c r="T29" s="27"/>
+      <c r="U29" s="27"/>
       <c r="V29" s="52"/>
-      <c r="W29" s="28"/>
-      <c r="X29" s="28"/>
-      <c r="Y29" s="28"/>
-      <c r="Z29" s="28"/>
-      <c r="AA29" s="28"/>
-      <c r="AB29" s="28"/>
-      <c r="AC29" s="28"/>
+      <c r="W29" s="27"/>
+      <c r="X29" s="27"/>
+      <c r="Y29" s="27"/>
+      <c r="Z29" s="27"/>
+      <c r="AA29" s="27"/>
+      <c r="AB29" s="27"/>
+      <c r="AC29" s="27"/>
     </row>
     <row r="30">
       <c r="A30" s="23"/>
@@ -2479,23 +2479,23 @@
       <c r="E30" s="60">
         <v>46.0</v>
       </c>
-      <c r="F30" s="36">
+      <c r="F30" s="35">
         <v>447.0</v>
       </c>
-      <c r="G30" s="37">
+      <c r="G30" s="36">
         <v>45814.0</v>
       </c>
-      <c r="H30" s="35" t="s">
+      <c r="H30" s="34" t="s">
         <v>187</v>
       </c>
-      <c r="I30" s="44"/>
-      <c r="J30" s="44">
+      <c r="I30" s="43"/>
+      <c r="J30" s="43">
         <v>45955.0</v>
       </c>
-      <c r="K30" s="38">
+      <c r="K30" s="37">
         <v>112720.77</v>
       </c>
-      <c r="L30" s="35" t="s">
+      <c r="L30" s="34" t="s">
         <v>188</v>
       </c>
       <c r="M30" s="39">
@@ -2503,20 +2503,20 @@
       </c>
       <c r="N30" s="51"/>
       <c r="O30" s="25"/>
-      <c r="P30" s="28"/>
-      <c r="Q30" s="28"/>
-      <c r="R30" s="28"/>
-      <c r="S30" s="28"/>
-      <c r="T30" s="28"/>
-      <c r="U30" s="28"/>
+      <c r="P30" s="27"/>
+      <c r="Q30" s="27"/>
+      <c r="R30" s="27"/>
+      <c r="S30" s="27"/>
+      <c r="T30" s="27"/>
+      <c r="U30" s="27"/>
       <c r="V30" s="52"/>
-      <c r="W30" s="28"/>
-      <c r="X30" s="28"/>
-      <c r="Y30" s="28"/>
-      <c r="Z30" s="28"/>
-      <c r="AA30" s="28"/>
-      <c r="AB30" s="28"/>
-      <c r="AC30" s="28"/>
+      <c r="W30" s="27"/>
+      <c r="X30" s="27"/>
+      <c r="Y30" s="27"/>
+      <c r="Z30" s="27"/>
+      <c r="AA30" s="27"/>
+      <c r="AB30" s="27"/>
+      <c r="AC30" s="27"/>
     </row>
     <row r="31" ht="12.75" customHeight="1">
       <c r="A31" s="23"/>
@@ -2528,23 +2528,23 @@
       <c r="E31" s="62" t="s">
         <v>190</v>
       </c>
-      <c r="F31" s="36">
+      <c r="F31" s="35">
         <v>529.0</v>
       </c>
       <c r="G31" s="63">
         <v>45853.0</v>
       </c>
-      <c r="H31" s="35" t="s">
-        <v>53</v>
-      </c>
-      <c r="I31" s="44"/>
-      <c r="J31" s="44">
+      <c r="H31" s="34" t="s">
+        <v>65</v>
+      </c>
+      <c r="I31" s="43"/>
+      <c r="J31" s="43">
         <v>45939.0</v>
       </c>
-      <c r="K31" s="46">
+      <c r="K31" s="45">
         <v>378307.61</v>
       </c>
-      <c r="L31" s="35" t="s">
+      <c r="L31" s="34" t="s">
         <v>191</v>
       </c>
       <c r="M31" s="39">
@@ -2553,19 +2553,19 @@
       <c r="N31" s="51"/>
       <c r="O31" s="25"/>
       <c r="P31" s="64"/>
-      <c r="Q31" s="28"/>
-      <c r="R31" s="28"/>
-      <c r="S31" s="28"/>
-      <c r="T31" s="28"/>
-      <c r="U31" s="28"/>
+      <c r="Q31" s="27"/>
+      <c r="R31" s="27"/>
+      <c r="S31" s="27"/>
+      <c r="T31" s="27"/>
+      <c r="U31" s="27"/>
       <c r="V31" s="52"/>
-      <c r="W31" s="28"/>
-      <c r="X31" s="28"/>
-      <c r="Y31" s="28"/>
-      <c r="Z31" s="28"/>
-      <c r="AA31" s="28"/>
-      <c r="AB31" s="28"/>
-      <c r="AC31" s="28"/>
+      <c r="W31" s="27"/>
+      <c r="X31" s="27"/>
+      <c r="Y31" s="27"/>
+      <c r="Z31" s="27"/>
+      <c r="AA31" s="27"/>
+      <c r="AB31" s="27"/>
+      <c r="AC31" s="27"/>
     </row>
     <row r="32" ht="60.0" customHeight="1">
       <c r="A32" s="23"/>
@@ -2577,23 +2577,23 @@
       <c r="E32" s="62" t="s">
         <v>190</v>
       </c>
-      <c r="F32" s="35">
+      <c r="F32" s="34">
         <v>691.0</v>
       </c>
       <c r="G32" s="63">
         <v>45910.0</v>
       </c>
-      <c r="H32" s="35" t="s">
-        <v>53</v>
-      </c>
-      <c r="I32" s="44"/>
-      <c r="J32" s="44">
+      <c r="H32" s="34" t="s">
+        <v>65</v>
+      </c>
+      <c r="I32" s="43"/>
+      <c r="J32" s="43">
         <v>45941.0</v>
       </c>
-      <c r="K32" s="38">
+      <c r="K32" s="37">
         <v>3315.0471000000252</v>
       </c>
-      <c r="L32" s="35" t="s">
+      <c r="L32" s="34" t="s">
         <v>193</v>
       </c>
       <c r="M32" s="39">
@@ -2602,19 +2602,19 @@
       <c r="N32" s="51"/>
       <c r="O32" s="25"/>
       <c r="P32" s="64"/>
-      <c r="Q32" s="28"/>
-      <c r="R32" s="28"/>
-      <c r="S32" s="28"/>
-      <c r="T32" s="28"/>
-      <c r="U32" s="28"/>
+      <c r="Q32" s="27"/>
+      <c r="R32" s="27"/>
+      <c r="S32" s="27"/>
+      <c r="T32" s="27"/>
+      <c r="U32" s="27"/>
       <c r="V32" s="52"/>
-      <c r="W32" s="28"/>
-      <c r="X32" s="28"/>
-      <c r="Y32" s="28"/>
-      <c r="Z32" s="28"/>
-      <c r="AA32" s="28"/>
-      <c r="AB32" s="28"/>
-      <c r="AC32" s="28"/>
+      <c r="W32" s="27"/>
+      <c r="X32" s="27"/>
+      <c r="Y32" s="27"/>
+      <c r="Z32" s="27"/>
+      <c r="AA32" s="27"/>
+      <c r="AB32" s="27"/>
+      <c r="AC32" s="27"/>
     </row>
     <row r="33" ht="12.75" customHeight="1">
       <c r="A33" s="23"/>
@@ -2626,23 +2626,23 @@
       <c r="E33" s="65">
         <v>135.0</v>
       </c>
-      <c r="F33" s="35">
+      <c r="F33" s="34">
         <v>677.0</v>
       </c>
       <c r="G33" s="63">
         <v>45904.0</v>
       </c>
-      <c r="H33" s="35" t="s">
-        <v>59</v>
+      <c r="H33" s="34" t="s">
+        <v>72</v>
       </c>
       <c r="I33" s="66"/>
       <c r="J33" s="66">
         <v>45935.0</v>
       </c>
-      <c r="K33" s="46">
+      <c r="K33" s="45">
         <v>198332.75</v>
       </c>
-      <c r="L33" s="35" t="s">
+      <c r="L33" s="34" t="s">
         <v>195</v>
       </c>
       <c r="M33" s="39">
@@ -2651,19 +2651,19 @@
       <c r="N33" s="51"/>
       <c r="O33" s="25"/>
       <c r="P33" s="64"/>
-      <c r="Q33" s="28"/>
-      <c r="R33" s="28"/>
-      <c r="S33" s="28"/>
-      <c r="T33" s="28"/>
-      <c r="U33" s="28"/>
+      <c r="Q33" s="27"/>
+      <c r="R33" s="27"/>
+      <c r="S33" s="27"/>
+      <c r="T33" s="27"/>
+      <c r="U33" s="27"/>
       <c r="V33" s="52"/>
-      <c r="W33" s="28"/>
-      <c r="X33" s="28"/>
-      <c r="Y33" s="28"/>
-      <c r="Z33" s="28"/>
-      <c r="AA33" s="28"/>
-      <c r="AB33" s="28"/>
-      <c r="AC33" s="28"/>
+      <c r="W33" s="27"/>
+      <c r="X33" s="27"/>
+      <c r="Y33" s="27"/>
+      <c r="Z33" s="27"/>
+      <c r="AA33" s="27"/>
+      <c r="AB33" s="27"/>
+      <c r="AC33" s="27"/>
     </row>
     <row r="34" ht="12.75" customHeight="1">
       <c r="A34" s="23"/>
@@ -2675,20 +2675,20 @@
       <c r="E34" s="65">
         <v>40.0</v>
       </c>
-      <c r="F34" s="35">
+      <c r="F34" s="34">
         <v>278.0</v>
       </c>
       <c r="G34" s="63">
         <v>46008.0</v>
       </c>
-      <c r="H34" s="35" t="s">
-        <v>113</v>
+      <c r="H34" s="34" t="s">
+        <v>124</v>
       </c>
       <c r="I34" s="66"/>
       <c r="J34" s="66">
         <v>46066.0</v>
       </c>
-      <c r="K34" s="46">
+      <c r="K34" s="45">
         <v>1528.62</v>
       </c>
       <c r="L34" s="67" t="s">
@@ -2700,19 +2700,19 @@
       <c r="N34" s="51"/>
       <c r="O34" s="25"/>
       <c r="P34" s="64"/>
-      <c r="Q34" s="28"/>
-      <c r="R34" s="28"/>
-      <c r="S34" s="28"/>
-      <c r="T34" s="28"/>
-      <c r="U34" s="28"/>
+      <c r="Q34" s="27"/>
+      <c r="R34" s="27"/>
+      <c r="S34" s="27"/>
+      <c r="T34" s="27"/>
+      <c r="U34" s="27"/>
       <c r="V34" s="52"/>
-      <c r="W34" s="28"/>
-      <c r="X34" s="28"/>
-      <c r="Y34" s="28"/>
-      <c r="Z34" s="28"/>
-      <c r="AA34" s="28"/>
-      <c r="AB34" s="28"/>
-      <c r="AC34" s="28"/>
+      <c r="W34" s="27"/>
+      <c r="X34" s="27"/>
+      <c r="Y34" s="27"/>
+      <c r="Z34" s="27"/>
+      <c r="AA34" s="27"/>
+      <c r="AB34" s="27"/>
+      <c r="AC34" s="27"/>
     </row>
     <row r="35" ht="12.75" customHeight="1">
       <c r="A35" s="23"/>
@@ -2724,23 +2724,23 @@
       <c r="E35" s="65" t="s">
         <v>200</v>
       </c>
-      <c r="F35" s="35">
+      <c r="F35" s="34">
         <v>748.0</v>
       </c>
       <c r="G35" s="63">
         <v>45930.0</v>
       </c>
-      <c r="H35" s="35" t="s">
-        <v>90</v>
+      <c r="H35" s="34" t="s">
+        <v>96</v>
       </c>
       <c r="I35" s="66"/>
       <c r="J35" s="66">
         <v>45935.0</v>
       </c>
-      <c r="K35" s="46">
+      <c r="K35" s="45">
         <v>38718.58</v>
       </c>
-      <c r="L35" s="35" t="s">
+      <c r="L35" s="34" t="s">
         <v>201</v>
       </c>
       <c r="M35" s="59" t="s">
@@ -2749,19 +2749,19 @@
       <c r="N35" s="51"/>
       <c r="O35" s="25"/>
       <c r="P35" s="64"/>
-      <c r="Q35" s="28"/>
-      <c r="R35" s="28"/>
-      <c r="S35" s="28"/>
-      <c r="T35" s="28"/>
-      <c r="U35" s="28"/>
+      <c r="Q35" s="27"/>
+      <c r="R35" s="27"/>
+      <c r="S35" s="27"/>
+      <c r="T35" s="27"/>
+      <c r="U35" s="27"/>
       <c r="V35" s="52"/>
-      <c r="W35" s="28"/>
-      <c r="X35" s="28"/>
-      <c r="Y35" s="28"/>
-      <c r="Z35" s="28"/>
-      <c r="AA35" s="28"/>
-      <c r="AB35" s="28"/>
-      <c r="AC35" s="28"/>
+      <c r="W35" s="27"/>
+      <c r="X35" s="27"/>
+      <c r="Y35" s="27"/>
+      <c r="Z35" s="27"/>
+      <c r="AA35" s="27"/>
+      <c r="AB35" s="27"/>
+      <c r="AC35" s="27"/>
     </row>
     <row r="36" ht="12.75" customHeight="1">
       <c r="A36" s="23"/>
@@ -2773,23 +2773,23 @@
       <c r="E36" s="65">
         <v>154.0</v>
       </c>
-      <c r="F36" s="35">
+      <c r="F36" s="34">
         <v>822.0</v>
       </c>
       <c r="G36" s="63">
         <v>45968.0</v>
       </c>
-      <c r="H36" s="35" t="s">
-        <v>104</v>
+      <c r="H36" s="34" t="s">
+        <v>115</v>
       </c>
       <c r="I36" s="66"/>
       <c r="J36" s="66">
         <v>45935.0</v>
       </c>
-      <c r="K36" s="46">
+      <c r="K36" s="45">
         <v>133124.11</v>
       </c>
-      <c r="L36" s="35" t="s">
+      <c r="L36" s="34" t="s">
         <v>204</v>
       </c>
       <c r="M36" s="59" t="s">
@@ -2798,19 +2798,19 @@
       <c r="N36" s="51"/>
       <c r="O36" s="25"/>
       <c r="P36" s="64"/>
-      <c r="Q36" s="28"/>
-      <c r="R36" s="28"/>
-      <c r="S36" s="28"/>
-      <c r="T36" s="28"/>
-      <c r="U36" s="28"/>
+      <c r="Q36" s="27"/>
+      <c r="R36" s="27"/>
+      <c r="S36" s="27"/>
+      <c r="T36" s="27"/>
+      <c r="U36" s="27"/>
       <c r="V36" s="52"/>
-      <c r="W36" s="28"/>
-      <c r="X36" s="28"/>
-      <c r="Y36" s="28"/>
-      <c r="Z36" s="28"/>
-      <c r="AA36" s="28"/>
-      <c r="AB36" s="28"/>
-      <c r="AC36" s="28"/>
+      <c r="W36" s="27"/>
+      <c r="X36" s="27"/>
+      <c r="Y36" s="27"/>
+      <c r="Z36" s="27"/>
+      <c r="AA36" s="27"/>
+      <c r="AB36" s="27"/>
+      <c r="AC36" s="27"/>
     </row>
     <row r="37" ht="12.75" customHeight="1">
       <c r="A37" s="23"/>
@@ -2829,16 +2829,16 @@
         <v>46043.0</v>
       </c>
       <c r="H37" s="65" t="s">
-        <v>99</v>
+        <v>108</v>
       </c>
       <c r="I37" s="70"/>
       <c r="J37" s="69">
         <v>46075.0</v>
       </c>
-      <c r="K37" s="46">
+      <c r="K37" s="45">
         <v>11372.9</v>
       </c>
-      <c r="L37" s="35" t="s">
+      <c r="L37" s="34" t="s">
         <v>207</v>
       </c>
       <c r="M37" s="39">
@@ -2846,20 +2846,20 @@
       </c>
       <c r="N37" s="51"/>
       <c r="O37" s="25"/>
-      <c r="P37" s="28"/>
-      <c r="Q37" s="28"/>
-      <c r="R37" s="28"/>
-      <c r="S37" s="28"/>
-      <c r="T37" s="28"/>
-      <c r="U37" s="28"/>
+      <c r="P37" s="27"/>
+      <c r="Q37" s="27"/>
+      <c r="R37" s="27"/>
+      <c r="S37" s="27"/>
+      <c r="T37" s="27"/>
+      <c r="U37" s="27"/>
       <c r="V37" s="52"/>
-      <c r="W37" s="28"/>
-      <c r="X37" s="28"/>
-      <c r="Y37" s="28"/>
-      <c r="Z37" s="28"/>
-      <c r="AA37" s="28"/>
-      <c r="AB37" s="28"/>
-      <c r="AC37" s="28"/>
+      <c r="W37" s="27"/>
+      <c r="X37" s="27"/>
+      <c r="Y37" s="27"/>
+      <c r="Z37" s="27"/>
+      <c r="AA37" s="27"/>
+      <c r="AB37" s="27"/>
+      <c r="AC37" s="27"/>
     </row>
     <row r="38" ht="12.75" customHeight="1">
       <c r="A38" s="23"/>
@@ -2876,27 +2876,27 @@
         <v>209</v>
       </c>
       <c r="J38" s="69"/>
-      <c r="K38" s="46"/>
-      <c r="L38" s="35"/>
+      <c r="K38" s="45"/>
+      <c r="L38" s="34"/>
       <c r="M38" s="39"/>
       <c r="N38" s="51">
         <v>15854.78</v>
       </c>
       <c r="O38" s="25"/>
-      <c r="P38" s="28"/>
-      <c r="Q38" s="28"/>
-      <c r="R38" s="28"/>
-      <c r="S38" s="28"/>
-      <c r="T38" s="28"/>
-      <c r="U38" s="28"/>
+      <c r="P38" s="27"/>
+      <c r="Q38" s="27"/>
+      <c r="R38" s="27"/>
+      <c r="S38" s="27"/>
+      <c r="T38" s="27"/>
+      <c r="U38" s="27"/>
       <c r="V38" s="52"/>
-      <c r="W38" s="28"/>
-      <c r="X38" s="28"/>
-      <c r="Y38" s="28"/>
-      <c r="Z38" s="28"/>
-      <c r="AA38" s="28"/>
-      <c r="AB38" s="28"/>
-      <c r="AC38" s="28"/>
+      <c r="W38" s="27"/>
+      <c r="X38" s="27"/>
+      <c r="Y38" s="27"/>
+      <c r="Z38" s="27"/>
+      <c r="AA38" s="27"/>
+      <c r="AB38" s="27"/>
+      <c r="AC38" s="27"/>
     </row>
     <row r="39" ht="12.75" customHeight="1">
       <c r="A39" s="23"/>
@@ -2913,32 +2913,32 @@
         <v>209</v>
       </c>
       <c r="J39" s="69"/>
-      <c r="K39" s="46"/>
-      <c r="L39" s="35"/>
+      <c r="K39" s="45"/>
+      <c r="L39" s="34"/>
       <c r="M39" s="39"/>
       <c r="N39" s="71">
         <v>42229.72325</v>
       </c>
       <c r="O39" s="25"/>
-      <c r="P39" s="28"/>
-      <c r="Q39" s="28"/>
-      <c r="R39" s="28"/>
-      <c r="S39" s="28"/>
-      <c r="T39" s="28"/>
-      <c r="U39" s="28"/>
+      <c r="P39" s="27"/>
+      <c r="Q39" s="27"/>
+      <c r="R39" s="27"/>
+      <c r="S39" s="27"/>
+      <c r="T39" s="27"/>
+      <c r="U39" s="27"/>
       <c r="V39" s="52"/>
-      <c r="W39" s="28"/>
-      <c r="X39" s="28"/>
-      <c r="Y39" s="28"/>
-      <c r="Z39" s="28"/>
-      <c r="AA39" s="28"/>
-      <c r="AB39" s="28"/>
-      <c r="AC39" s="28"/>
+      <c r="W39" s="27"/>
+      <c r="X39" s="27"/>
+      <c r="Y39" s="27"/>
+      <c r="Z39" s="27"/>
+      <c r="AA39" s="27"/>
+      <c r="AB39" s="27"/>
+      <c r="AC39" s="27"/>
     </row>
     <row r="40" ht="12.75" customHeight="1">
       <c r="A40" s="23"/>
       <c r="B40" s="23"/>
-      <c r="C40" s="36"/>
+      <c r="C40" s="35"/>
       <c r="D40" s="61" t="s">
         <v>211</v>
       </c>
@@ -2950,32 +2950,32 @@
         <v>209</v>
       </c>
       <c r="J40" s="69"/>
-      <c r="K40" s="46"/>
-      <c r="L40" s="47"/>
+      <c r="K40" s="45"/>
+      <c r="L40" s="46"/>
       <c r="M40" s="39"/>
       <c r="N40" s="72">
         <v>48857.395500000006</v>
       </c>
       <c r="O40" s="25"/>
-      <c r="P40" s="28"/>
-      <c r="Q40" s="28"/>
-      <c r="R40" s="28"/>
-      <c r="S40" s="28"/>
-      <c r="T40" s="28"/>
-      <c r="U40" s="28"/>
+      <c r="P40" s="27"/>
+      <c r="Q40" s="27"/>
+      <c r="R40" s="27"/>
+      <c r="S40" s="27"/>
+      <c r="T40" s="27"/>
+      <c r="U40" s="27"/>
       <c r="V40" s="52"/>
-      <c r="W40" s="28"/>
-      <c r="X40" s="28"/>
-      <c r="Y40" s="28"/>
-      <c r="Z40" s="28"/>
-      <c r="AA40" s="28"/>
-      <c r="AB40" s="28"/>
-      <c r="AC40" s="28"/>
+      <c r="W40" s="27"/>
+      <c r="X40" s="27"/>
+      <c r="Y40" s="27"/>
+      <c r="Z40" s="27"/>
+      <c r="AA40" s="27"/>
+      <c r="AB40" s="27"/>
+      <c r="AC40" s="27"/>
     </row>
     <row r="41" ht="12.75" customHeight="1">
       <c r="A41" s="23"/>
       <c r="B41" s="23"/>
-      <c r="C41" s="36"/>
+      <c r="C41" s="35"/>
       <c r="D41" s="61" t="s">
         <v>212</v>
       </c>
@@ -2987,30 +2987,30 @@
         <v>213</v>
       </c>
       <c r="J41" s="69"/>
-      <c r="K41" s="46"/>
-      <c r="L41" s="47"/>
+      <c r="K41" s="45"/>
+      <c r="L41" s="46"/>
       <c r="M41" s="39"/>
       <c r="N41" s="72"/>
       <c r="O41" s="25"/>
-      <c r="P41" s="28"/>
-      <c r="Q41" s="28"/>
-      <c r="R41" s="28"/>
-      <c r="S41" s="28"/>
-      <c r="T41" s="28"/>
-      <c r="U41" s="28"/>
+      <c r="P41" s="27"/>
+      <c r="Q41" s="27"/>
+      <c r="R41" s="27"/>
+      <c r="S41" s="27"/>
+      <c r="T41" s="27"/>
+      <c r="U41" s="27"/>
       <c r="V41" s="52"/>
-      <c r="W41" s="28"/>
-      <c r="X41" s="28"/>
-      <c r="Y41" s="28"/>
-      <c r="Z41" s="28"/>
-      <c r="AA41" s="28"/>
-      <c r="AB41" s="28"/>
-      <c r="AC41" s="28"/>
+      <c r="W41" s="27"/>
+      <c r="X41" s="27"/>
+      <c r="Y41" s="27"/>
+      <c r="Z41" s="27"/>
+      <c r="AA41" s="27"/>
+      <c r="AB41" s="27"/>
+      <c r="AC41" s="27"/>
     </row>
     <row r="42" ht="12.75" customHeight="1">
       <c r="A42" s="23"/>
       <c r="B42" s="23"/>
-      <c r="C42" s="33">
+      <c r="C42" s="32">
         <v>3.0</v>
       </c>
       <c r="D42" s="61" t="s">
@@ -3024,13 +3024,13 @@
         <v>46104.0</v>
       </c>
       <c r="H42" s="65" t="s">
-        <v>99</v>
+        <v>108</v>
       </c>
       <c r="I42" s="70"/>
       <c r="J42" s="69">
         <v>46106.0</v>
       </c>
-      <c r="K42" s="46">
+      <c r="K42" s="45">
         <v>27801.11</v>
       </c>
       <c r="L42" s="73" t="s">
@@ -3041,20 +3041,20 @@
       </c>
       <c r="N42" s="51"/>
       <c r="O42" s="25"/>
-      <c r="P42" s="28"/>
-      <c r="Q42" s="28"/>
-      <c r="R42" s="28"/>
-      <c r="S42" s="28"/>
-      <c r="T42" s="28"/>
-      <c r="U42" s="28"/>
+      <c r="P42" s="27"/>
+      <c r="Q42" s="27"/>
+      <c r="R42" s="27"/>
+      <c r="S42" s="27"/>
+      <c r="T42" s="27"/>
+      <c r="U42" s="27"/>
       <c r="V42" s="52"/>
-      <c r="W42" s="28"/>
-      <c r="X42" s="28"/>
-      <c r="Y42" s="28"/>
-      <c r="Z42" s="28"/>
-      <c r="AA42" s="28"/>
-      <c r="AB42" s="28"/>
-      <c r="AC42" s="28"/>
+      <c r="W42" s="27"/>
+      <c r="X42" s="27"/>
+      <c r="Y42" s="27"/>
+      <c r="Z42" s="27"/>
+      <c r="AA42" s="27"/>
+      <c r="AB42" s="27"/>
+      <c r="AC42" s="27"/>
     </row>
     <row r="43" ht="12.75" customHeight="1">
       <c r="A43" s="14"/>
@@ -3071,17 +3071,17 @@
         <v>46199.0</v>
       </c>
       <c r="H43" s="65" t="s">
-        <v>68</v>
+        <v>77</v>
       </c>
       <c r="I43" s="70"/>
       <c r="J43" s="69">
         <v>46233.0</v>
       </c>
-      <c r="K43" s="46">
+      <c r="K43" s="45">
         <v>58868.35</v>
       </c>
-      <c r="L43" s="35" t="s">
-        <v>73</v>
+      <c r="L43" s="34" t="s">
+        <v>63</v>
       </c>
       <c r="M43" s="74">
         <v>58868.35</v>
@@ -8040,10 +8040,10 @@
       <c r="AH1" s="2"/>
     </row>
     <row r="2">
-      <c r="A2" s="5">
+      <c r="A2" s="7">
         <v>46212.0</v>
       </c>
-      <c r="L2" s="6" t="s">
+      <c r="L2" s="9" t="s">
         <v>1</v>
       </c>
       <c r="AB2" s="2"/>
@@ -8055,40 +8055,40 @@
       <c r="AH2" s="2"/>
     </row>
     <row r="3">
-      <c r="A3" s="9" t="s">
+      <c r="A3" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="9" t="s">
+      <c r="B3" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="11">
+      <c r="C3" s="12">
         <v>2.5E32</v>
       </c>
-      <c r="D3" s="9" t="s">
+      <c r="D3" s="11" t="s">
         <v>4</v>
       </c>
       <c r="E3" s="13">
         <v>45686.0</v>
       </c>
-      <c r="F3" s="9" t="s">
+      <c r="F3" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="G3" s="9">
+      <c r="G3" s="11">
         <v>12.0</v>
       </c>
-      <c r="H3" s="9">
+      <c r="H3" s="11">
         <v>339039.0</v>
       </c>
-      <c r="I3" s="9">
+      <c r="I3" s="11">
         <v>2048.0</v>
       </c>
-      <c r="J3" s="15">
+      <c r="J3" s="16">
         <v>1000.0</v>
       </c>
-      <c r="K3" s="15">
+      <c r="K3" s="16">
         <v>1000.0</v>
       </c>
-      <c r="L3" s="9">
+      <c r="L3" s="11">
         <v>0.0</v>
       </c>
       <c r="AB3" s="2"/>
@@ -8100,40 +8100,40 @@
       <c r="AH3" s="2"/>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="s">
+      <c r="A4" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="B4" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="9" t="s">
+      <c r="C4" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="D4" s="9" t="s">
+      <c r="D4" s="11" t="s">
         <v>4</v>
       </c>
       <c r="E4" s="13">
         <v>45762.0</v>
       </c>
-      <c r="F4" s="9" t="s">
+      <c r="F4" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="G4" s="9">
+      <c r="G4" s="11">
         <v>12.0</v>
       </c>
-      <c r="H4" s="9">
+      <c r="H4" s="11">
         <v>339039.0</v>
       </c>
-      <c r="I4" s="9">
+      <c r="I4" s="11">
         <v>2048.0</v>
       </c>
-      <c r="J4" s="15">
+      <c r="J4" s="16">
         <v>52250.04</v>
       </c>
-      <c r="K4" s="15">
+      <c r="K4" s="16">
         <v>52250.04</v>
       </c>
-      <c r="L4" s="9">
+      <c r="L4" s="11">
         <v>0.0</v>
       </c>
       <c r="AB4" s="2"/>
@@ -8145,40 +8145,40 @@
       <c r="AH4" s="2"/>
     </row>
     <row r="5">
-      <c r="A5" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="B5" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="C5" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="D5" s="9" t="s">
+      <c r="A5" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="B5" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="D5" s="11" t="s">
         <v>4</v>
       </c>
       <c r="E5" s="13">
         <v>45762.0</v>
       </c>
-      <c r="F5" s="9" t="s">
+      <c r="F5" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="G5" s="9">
+      <c r="G5" s="11">
         <v>12.0</v>
       </c>
-      <c r="H5" s="9">
+      <c r="H5" s="11">
         <v>339039.0</v>
       </c>
-      <c r="I5" s="9">
+      <c r="I5" s="11">
         <v>2048.0</v>
       </c>
-      <c r="J5" s="15">
+      <c r="J5" s="16">
         <v>881914.18</v>
       </c>
-      <c r="K5" s="15">
+      <c r="K5" s="16">
         <v>881914.18</v>
       </c>
-      <c r="L5" s="9">
+      <c r="L5" s="11">
         <v>0.0</v>
       </c>
       <c r="AB5" s="2"/>
@@ -8190,40 +8190,40 @@
       <c r="AH5" s="2"/>
     </row>
     <row r="6">
-      <c r="A6" s="9" t="s">
+      <c r="A6" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C6" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="B6" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="C6" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="D6" s="9" t="s">
+      <c r="D6" s="11" t="s">
         <v>4</v>
       </c>
       <c r="E6" s="13">
         <v>45762.0</v>
       </c>
-      <c r="F6" s="9" t="s">
+      <c r="F6" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="G6" s="9">
+      <c r="G6" s="11">
         <v>12.0</v>
       </c>
-      <c r="H6" s="9">
+      <c r="H6" s="11">
         <v>339039.0</v>
       </c>
-      <c r="I6" s="9">
+      <c r="I6" s="11">
         <v>2048.0</v>
       </c>
-      <c r="J6" s="15">
+      <c r="J6" s="16">
         <v>750000.0</v>
       </c>
-      <c r="K6" s="15">
+      <c r="K6" s="16">
         <v>750000.0</v>
       </c>
-      <c r="L6" s="9">
+      <c r="L6" s="11">
         <v>0.0</v>
       </c>
       <c r="AB6" s="2"/>
@@ -8235,40 +8235,40 @@
       <c r="AH6" s="2"/>
     </row>
     <row r="7">
-      <c r="A7" s="9" t="s">
+      <c r="A7" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="B7" s="9" t="s">
+      <c r="B7" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="C7" s="9" t="s">
+      <c r="C7" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="D7" s="9" t="s">
+      <c r="D7" s="11" t="s">
         <v>4</v>
       </c>
       <c r="E7" s="13">
         <v>45763.0</v>
       </c>
-      <c r="F7" s="9" t="s">
+      <c r="F7" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="G7" s="9">
+      <c r="G7" s="11">
         <v>12.0</v>
       </c>
-      <c r="H7" s="9">
+      <c r="H7" s="11">
         <v>339039.0</v>
       </c>
-      <c r="I7" s="9" t="s">
+      <c r="I7" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="J7" s="15">
+      <c r="J7" s="16">
         <v>949835.78</v>
       </c>
-      <c r="K7" s="15">
+      <c r="K7" s="16">
         <v>949835.78</v>
       </c>
-      <c r="L7" s="9">
+      <c r="L7" s="11">
         <v>0.0</v>
       </c>
       <c r="AB7" s="2"/>
@@ -8280,43 +8280,43 @@
       <c r="AH7" s="2"/>
     </row>
     <row r="8">
-      <c r="A8" s="9" t="s">
+      <c r="A8" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="B8" s="9" t="s">
+      <c r="B8" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="C8" s="9" t="s">
+      <c r="C8" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="D8" s="9" t="s">
+      <c r="D8" s="11" t="s">
         <v>4</v>
       </c>
       <c r="E8" s="13">
         <v>45763.0</v>
       </c>
-      <c r="F8" s="9" t="s">
+      <c r="F8" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="G8" s="9">
+      <c r="G8" s="11">
         <v>12.0</v>
       </c>
-      <c r="H8" s="9">
+      <c r="H8" s="11">
         <v>339039.0</v>
       </c>
-      <c r="I8" s="9" t="s">
+      <c r="I8" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="J8" s="15">
+      <c r="J8" s="16">
         <v>524584.95</v>
       </c>
-      <c r="K8" s="15">
+      <c r="K8" s="16">
         <v>524584.95</v>
       </c>
-      <c r="L8" s="9">
+      <c r="L8" s="11">
         <v>0.0</v>
       </c>
-      <c r="O8" s="27"/>
+      <c r="O8" s="29"/>
       <c r="AB8" s="2"/>
       <c r="AC8" s="2"/>
       <c r="AD8" s="2"/>
@@ -8326,40 +8326,40 @@
       <c r="AH8" s="2"/>
     </row>
     <row r="9">
-      <c r="A9" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="B9" s="9" t="s">
-        <v>50</v>
-      </c>
-      <c r="C9" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="D9" s="9" t="s">
+      <c r="A9" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="C9" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="D9" s="11" t="s">
         <v>4</v>
       </c>
       <c r="E9" s="13">
         <v>45792.0</v>
       </c>
-      <c r="F9" s="9" t="s">
+      <c r="F9" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="G9" s="9">
+      <c r="G9" s="11">
         <v>12.0</v>
       </c>
-      <c r="H9" s="9">
+      <c r="H9" s="11">
         <v>339039.0</v>
       </c>
-      <c r="I9" s="9" t="s">
-        <v>52</v>
-      </c>
-      <c r="J9" s="15">
+      <c r="I9" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="J9" s="16">
         <v>211614.23</v>
       </c>
-      <c r="K9" s="15">
+      <c r="K9" s="16">
         <v>211614.23</v>
       </c>
-      <c r="L9" s="9">
+      <c r="L9" s="11">
         <v>0.0</v>
       </c>
       <c r="AB9" s="2"/>
@@ -8371,40 +8371,40 @@
       <c r="AH9" s="2"/>
     </row>
     <row r="10">
-      <c r="A10" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="B10" s="9" t="s">
+      <c r="A10" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="B10" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="C10" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="D10" s="9" t="s">
+      <c r="C10" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="D10" s="11" t="s">
         <v>4</v>
       </c>
       <c r="E10" s="13">
         <v>45825.0</v>
       </c>
-      <c r="F10" s="9" t="s">
+      <c r="F10" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="G10" s="9">
+      <c r="G10" s="11">
         <v>12.0</v>
       </c>
-      <c r="H10" s="9">
+      <c r="H10" s="11">
         <v>339039.0</v>
       </c>
-      <c r="I10" s="9">
+      <c r="I10" s="11">
         <v>2048.0</v>
       </c>
-      <c r="J10" s="15">
+      <c r="J10" s="16">
         <v>2391157.42</v>
       </c>
-      <c r="K10" s="15">
+      <c r="K10" s="16">
         <v>2391157.41</v>
       </c>
-      <c r="L10" s="15">
+      <c r="L10" s="16">
         <v>0.01</v>
       </c>
       <c r="AB10" s="2"/>
@@ -8416,40 +8416,40 @@
       <c r="AH10" s="2"/>
     </row>
     <row r="11">
-      <c r="A11" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="B11" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="C11" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="D11" s="9" t="s">
+      <c r="A11" s="11" t="s">
+        <v>69</v>
+      </c>
+      <c r="B11" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C11" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="D11" s="11" t="s">
         <v>4</v>
       </c>
       <c r="E11" s="13">
         <v>45825.0</v>
       </c>
-      <c r="F11" s="9" t="s">
+      <c r="F11" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="G11" s="9">
+      <c r="G11" s="11">
         <v>12.0</v>
       </c>
-      <c r="H11" s="9">
+      <c r="H11" s="11">
         <v>339039.0</v>
       </c>
-      <c r="I11" s="9">
+      <c r="I11" s="11">
         <v>2048.0</v>
       </c>
-      <c r="J11" s="15">
+      <c r="J11" s="16">
         <v>618154.39</v>
       </c>
-      <c r="K11" s="15">
+      <c r="K11" s="16">
         <v>618154.38</v>
       </c>
-      <c r="L11" s="9">
+      <c r="L11" s="11">
         <v>0.01</v>
       </c>
       <c r="AB11" s="2"/>
@@ -8461,40 +8461,40 @@
       <c r="AH11" s="2"/>
     </row>
     <row r="12">
-      <c r="A12" s="9" t="s">
-        <v>59</v>
-      </c>
-      <c r="B12" s="9" t="s">
-        <v>60</v>
-      </c>
-      <c r="C12" s="9" t="s">
-        <v>62</v>
-      </c>
-      <c r="D12" s="9" t="s">
+      <c r="A12" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="B12" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="C12" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="D12" s="11" t="s">
         <v>4</v>
       </c>
       <c r="E12" s="13">
         <v>45832.0</v>
       </c>
-      <c r="F12" s="9" t="s">
+      <c r="F12" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="G12" s="9">
+      <c r="G12" s="11">
         <v>12.0</v>
       </c>
-      <c r="H12" s="9">
+      <c r="H12" s="11">
         <v>339039.0</v>
       </c>
-      <c r="I12" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="J12" s="15">
+      <c r="I12" s="11" t="s">
+        <v>76</v>
+      </c>
+      <c r="J12" s="16">
         <v>1600334.09</v>
       </c>
-      <c r="K12" s="15">
+      <c r="K12" s="16">
         <v>1600334.09</v>
       </c>
-      <c r="L12" s="9">
+      <c r="L12" s="11">
         <v>0.0</v>
       </c>
       <c r="AB12" s="2"/>
@@ -8506,43 +8506,43 @@
       <c r="AH12" s="2"/>
     </row>
     <row r="13">
-      <c r="A13" s="9" t="s">
-        <v>68</v>
-      </c>
-      <c r="B13" s="9" t="s">
+      <c r="A13" s="11" t="s">
+        <v>77</v>
+      </c>
+      <c r="B13" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="C13" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="D13" s="9" t="s">
+      <c r="C13" s="11" t="s">
+        <v>78</v>
+      </c>
+      <c r="D13" s="11" t="s">
         <v>4</v>
       </c>
       <c r="E13" s="13">
         <v>45863.0</v>
       </c>
-      <c r="F13" s="9" t="s">
+      <c r="F13" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="G13" s="9">
+      <c r="G13" s="11">
         <v>12.0</v>
       </c>
-      <c r="H13" s="9">
+      <c r="H13" s="11">
         <v>339039.0</v>
       </c>
-      <c r="I13" s="9">
+      <c r="I13" s="11">
         <v>2048.0</v>
       </c>
-      <c r="J13" s="15">
+      <c r="J13" s="16">
         <v>2364771.07</v>
       </c>
-      <c r="K13" s="15">
+      <c r="K13" s="16">
         <v>2364771.07</v>
       </c>
-      <c r="L13" s="15">
+      <c r="L13" s="16">
         <v>0.0</v>
       </c>
-      <c r="M13" s="32"/>
+      <c r="M13" s="38"/>
       <c r="AB13" s="2"/>
       <c r="AC13" s="2"/>
       <c r="AD13" s="2"/>
@@ -8552,40 +8552,40 @@
       <c r="AH13" s="2"/>
     </row>
     <row r="14">
-      <c r="A14" s="9" t="s">
-        <v>75</v>
-      </c>
-      <c r="B14" s="9" t="s">
-        <v>76</v>
-      </c>
-      <c r="C14" s="9" t="s">
-        <v>77</v>
-      </c>
-      <c r="D14" s="9" t="s">
+      <c r="A14" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="B14" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="C14" s="11" t="s">
+        <v>81</v>
+      </c>
+      <c r="D14" s="11" t="s">
         <v>4</v>
       </c>
       <c r="E14" s="13">
         <v>45887.0</v>
       </c>
-      <c r="F14" s="9" t="s">
+      <c r="F14" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="G14" s="9">
+      <c r="G14" s="11">
         <v>12.0</v>
       </c>
-      <c r="H14" s="9">
+      <c r="H14" s="11">
         <v>339039.0</v>
       </c>
-      <c r="I14" s="9" t="s">
-        <v>52</v>
-      </c>
-      <c r="J14" s="15">
+      <c r="I14" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="J14" s="16">
         <v>968237.39</v>
       </c>
-      <c r="K14" s="15">
+      <c r="K14" s="16">
         <v>968237.39</v>
       </c>
-      <c r="L14" s="9">
+      <c r="L14" s="11">
         <v>0.0</v>
       </c>
       <c r="AB14" s="2"/>
@@ -8597,40 +8597,40 @@
       <c r="AH14" s="2"/>
     </row>
     <row r="15">
-      <c r="A15" s="9" t="s">
-        <v>78</v>
-      </c>
-      <c r="B15" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="C15" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="D15" s="9" t="s">
+      <c r="A15" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="B15" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="C15" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="D15" s="11" t="s">
         <v>4</v>
       </c>
       <c r="E15" s="13">
         <v>45924.0</v>
       </c>
-      <c r="F15" s="9" t="s">
+      <c r="F15" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="G15" s="9">
+      <c r="G15" s="11">
         <v>12.0</v>
       </c>
-      <c r="H15" s="9">
+      <c r="H15" s="11">
         <v>339039.0</v>
       </c>
-      <c r="I15" s="9" t="s">
+      <c r="I15" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="J15" s="15">
+      <c r="J15" s="16">
         <v>1011677.95</v>
       </c>
-      <c r="K15" s="15">
+      <c r="K15" s="16">
         <v>1011677.95</v>
       </c>
-      <c r="L15" s="9">
+      <c r="L15" s="11">
         <v>0.0</v>
       </c>
       <c r="AB15" s="2"/>
@@ -8642,40 +8642,40 @@
       <c r="AH15" s="2"/>
     </row>
     <row r="16">
-      <c r="A16" s="9" t="s">
-        <v>82</v>
-      </c>
-      <c r="B16" s="9" t="s">
+      <c r="A16" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="B16" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="C16" s="9" t="s">
-        <v>84</v>
-      </c>
-      <c r="D16" s="9" t="s">
+      <c r="C16" s="11" t="s">
+        <v>89</v>
+      </c>
+      <c r="D16" s="11" t="s">
         <v>4</v>
       </c>
       <c r="E16" s="13">
         <v>45929.0</v>
       </c>
-      <c r="F16" s="9" t="s">
+      <c r="F16" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="G16" s="9">
+      <c r="G16" s="11">
         <v>12.0</v>
       </c>
-      <c r="H16" s="9">
+      <c r="H16" s="11">
         <v>339039.0</v>
       </c>
-      <c r="I16" s="9">
+      <c r="I16" s="11">
         <v>2048.0</v>
       </c>
-      <c r="J16" s="15">
+      <c r="J16" s="16">
         <v>1580293.02</v>
       </c>
-      <c r="K16" s="15">
+      <c r="K16" s="16">
         <v>1580293.02</v>
       </c>
-      <c r="L16" s="15">
+      <c r="L16" s="16">
         <v>0.0</v>
       </c>
       <c r="AB16" s="2"/>
@@ -8687,40 +8687,40 @@
       <c r="AH16" s="2"/>
     </row>
     <row r="17">
-      <c r="A17" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="B17" s="9" t="s">
-        <v>87</v>
-      </c>
-      <c r="C17" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="D17" s="9" t="s">
+      <c r="A17" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="B17" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="C17" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="D17" s="11" t="s">
         <v>4</v>
       </c>
       <c r="E17" s="13">
         <v>45930.0</v>
       </c>
-      <c r="F17" s="9" t="s">
+      <c r="F17" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="G17" s="9">
+      <c r="G17" s="11">
         <v>12.0</v>
       </c>
-      <c r="H17" s="9">
+      <c r="H17" s="11">
         <v>339039.0</v>
       </c>
-      <c r="I17" s="9">
+      <c r="I17" s="11">
         <v>2048.0</v>
       </c>
-      <c r="J17" s="15">
+      <c r="J17" s="16">
         <v>34065.36</v>
       </c>
-      <c r="K17" s="9">
+      <c r="K17" s="11">
         <v>0.0</v>
       </c>
-      <c r="L17" s="15">
+      <c r="L17" s="16">
         <v>34065.36</v>
       </c>
       <c r="AB17" s="2"/>
@@ -8732,40 +8732,40 @@
       <c r="AH17" s="2"/>
     </row>
     <row r="18">
-      <c r="A18" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="B18" s="9" t="s">
-        <v>76</v>
-      </c>
-      <c r="C18" s="9" t="s">
-        <v>91</v>
-      </c>
-      <c r="D18" s="9" t="s">
+      <c r="A18" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="B18" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="C18" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="D18" s="11" t="s">
         <v>4</v>
       </c>
       <c r="E18" s="13">
         <v>45938.0</v>
       </c>
-      <c r="F18" s="9" t="s">
+      <c r="F18" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="G18" s="9">
+      <c r="G18" s="11">
         <v>12.0</v>
       </c>
-      <c r="H18" s="9">
+      <c r="H18" s="11">
         <v>339039.0</v>
       </c>
-      <c r="I18" s="9" t="s">
-        <v>52</v>
-      </c>
-      <c r="J18" s="15">
+      <c r="I18" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="J18" s="16">
         <v>63746.85</v>
       </c>
-      <c r="K18" s="15">
+      <c r="K18" s="16">
         <v>63746.85</v>
       </c>
-      <c r="L18" s="9">
+      <c r="L18" s="11">
         <v>0.0</v>
       </c>
       <c r="AB18" s="2"/>
@@ -8777,40 +8777,40 @@
       <c r="AH18" s="2"/>
     </row>
     <row r="19">
-      <c r="A19" s="9" t="s">
-        <v>92</v>
-      </c>
-      <c r="B19" s="9" t="s">
-        <v>60</v>
-      </c>
-      <c r="C19" s="9" t="s">
-        <v>93</v>
-      </c>
-      <c r="D19" s="9" t="s">
+      <c r="A19" s="11" t="s">
+        <v>99</v>
+      </c>
+      <c r="B19" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="C19" s="11" t="s">
+        <v>100</v>
+      </c>
+      <c r="D19" s="11" t="s">
         <v>4</v>
       </c>
       <c r="E19" s="13">
         <v>45938.0</v>
       </c>
-      <c r="F19" s="9" t="s">
+      <c r="F19" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="G19" s="9">
+      <c r="G19" s="11">
         <v>12.0</v>
       </c>
-      <c r="H19" s="9">
+      <c r="H19" s="11">
         <v>339039.0</v>
       </c>
-      <c r="I19" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="J19" s="15">
+      <c r="I19" s="11" t="s">
+        <v>76</v>
+      </c>
+      <c r="J19" s="16">
         <v>947931.1</v>
       </c>
-      <c r="K19" s="15">
+      <c r="K19" s="16">
         <v>947931.1</v>
       </c>
-      <c r="L19" s="9">
+      <c r="L19" s="11">
         <v>0.0</v>
       </c>
       <c r="AB19" s="2"/>
@@ -8822,40 +8822,40 @@
       <c r="AH19" s="2"/>
     </row>
     <row r="20">
-      <c r="A20" s="9" t="s">
-        <v>94</v>
-      </c>
-      <c r="B20" s="9" t="s">
+      <c r="A20" s="11" t="s">
+        <v>102</v>
+      </c>
+      <c r="B20" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="C20" s="9" t="s">
-        <v>95</v>
-      </c>
-      <c r="D20" s="9" t="s">
+      <c r="C20" s="11" t="s">
+        <v>103</v>
+      </c>
+      <c r="D20" s="11" t="s">
         <v>4</v>
       </c>
       <c r="E20" s="13">
         <v>45938.0</v>
       </c>
-      <c r="F20" s="9" t="s">
+      <c r="F20" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="G20" s="9">
+      <c r="G20" s="11">
         <v>12.0</v>
       </c>
-      <c r="H20" s="9">
+      <c r="H20" s="11">
         <v>339039.0</v>
       </c>
-      <c r="I20" s="9">
+      <c r="I20" s="11">
         <v>2048.0</v>
       </c>
-      <c r="J20" s="15">
+      <c r="J20" s="16">
         <v>259790.57</v>
       </c>
-      <c r="K20" s="15">
+      <c r="K20" s="16">
         <v>259790.57</v>
       </c>
-      <c r="L20" s="9">
+      <c r="L20" s="11">
         <v>0.0</v>
       </c>
       <c r="AB20" s="2"/>
@@ -8867,40 +8867,40 @@
       <c r="AH20" s="2"/>
     </row>
     <row r="21">
-      <c r="A21" s="9" t="s">
-        <v>96</v>
-      </c>
-      <c r="B21" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="C21" s="9" t="s">
-        <v>97</v>
-      </c>
-      <c r="D21" s="9" t="s">
+      <c r="A21" s="11" t="s">
+        <v>104</v>
+      </c>
+      <c r="B21" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C21" s="11" t="s">
+        <v>105</v>
+      </c>
+      <c r="D21" s="11" t="s">
         <v>4</v>
       </c>
       <c r="E21" s="13">
         <v>45938.0</v>
       </c>
-      <c r="F21" s="9" t="s">
+      <c r="F21" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="G21" s="9">
+      <c r="G21" s="11">
         <v>12.0</v>
       </c>
-      <c r="H21" s="9">
+      <c r="H21" s="11">
         <v>339039.0</v>
       </c>
-      <c r="I21" s="9">
+      <c r="I21" s="11">
         <v>2048.0</v>
       </c>
-      <c r="J21" s="15">
+      <c r="J21" s="16">
         <v>170479.3</v>
       </c>
-      <c r="K21" s="15">
+      <c r="K21" s="16">
         <v>170479.3</v>
       </c>
-      <c r="L21" s="9">
+      <c r="L21" s="11">
         <v>0.0</v>
       </c>
       <c r="AB21" s="2"/>
@@ -8912,40 +8912,40 @@
       <c r="AH21" s="2"/>
     </row>
     <row r="22">
-      <c r="A22" s="9" t="s">
-        <v>99</v>
-      </c>
-      <c r="B22" s="9" t="s">
-        <v>100</v>
-      </c>
-      <c r="C22" s="9" t="s">
-        <v>101</v>
-      </c>
-      <c r="D22" s="9" t="s">
+      <c r="A22" s="11" t="s">
+        <v>108</v>
+      </c>
+      <c r="B22" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="C22" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="D22" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="E22" s="42">
+      <c r="E22" s="50">
         <v>45953.0</v>
       </c>
-      <c r="F22" s="9" t="s">
+      <c r="F22" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="G22" s="9">
+      <c r="G22" s="11">
         <v>12.0</v>
       </c>
-      <c r="H22" s="9">
+      <c r="H22" s="11">
         <v>339039.0</v>
       </c>
-      <c r="I22" s="9">
+      <c r="I22" s="11">
         <v>2000.0</v>
       </c>
-      <c r="J22" s="15">
+      <c r="J22" s="16">
         <v>1500000.0</v>
       </c>
-      <c r="K22" s="15">
+      <c r="K22" s="16">
         <v>1500000.0</v>
       </c>
-      <c r="L22" s="15">
+      <c r="L22" s="16">
         <v>0.0</v>
       </c>
       <c r="AB22" s="2"/>
@@ -8957,40 +8957,40 @@
       <c r="AH22" s="2"/>
     </row>
     <row r="23">
-      <c r="A23" s="9" t="s">
-        <v>104</v>
-      </c>
-      <c r="B23" s="9" t="s">
-        <v>105</v>
-      </c>
-      <c r="C23" s="9" t="s">
-        <v>106</v>
-      </c>
-      <c r="D23" s="9" t="s">
+      <c r="A23" s="11" t="s">
+        <v>115</v>
+      </c>
+      <c r="B23" s="11" t="s">
+        <v>116</v>
+      </c>
+      <c r="C23" s="11" t="s">
+        <v>117</v>
+      </c>
+      <c r="D23" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="E23" s="42">
+      <c r="E23" s="50">
         <v>45953.0</v>
       </c>
-      <c r="F23" s="9" t="s">
+      <c r="F23" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="G23" s="9">
+      <c r="G23" s="11">
         <v>12.0</v>
       </c>
-      <c r="H23" s="9">
+      <c r="H23" s="11">
         <v>339039.0</v>
       </c>
-      <c r="I23" s="9" t="s">
-        <v>107</v>
-      </c>
-      <c r="J23" s="15">
+      <c r="I23" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="J23" s="16">
         <v>1000001.64</v>
       </c>
-      <c r="K23" s="15">
+      <c r="K23" s="16">
         <v>1000001.64</v>
       </c>
-      <c r="L23" s="9">
+      <c r="L23" s="11">
         <v>0.0</v>
       </c>
       <c r="AB23" s="2"/>
@@ -9002,40 +9002,40 @@
       <c r="AH23" s="2"/>
     </row>
     <row r="24">
-      <c r="A24" s="9" t="s">
-        <v>109</v>
-      </c>
-      <c r="B24" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="C24" s="9" t="s">
-        <v>111</v>
-      </c>
-      <c r="D24" s="9" t="s">
+      <c r="A24" s="11" t="s">
+        <v>121</v>
+      </c>
+      <c r="B24" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C24" s="11" t="s">
+        <v>122</v>
+      </c>
+      <c r="D24" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="E24" s="42">
+      <c r="E24" s="50">
         <v>45953.0</v>
       </c>
-      <c r="F24" s="9" t="s">
+      <c r="F24" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="G24" s="9">
+      <c r="G24" s="11">
         <v>12.0</v>
       </c>
-      <c r="H24" s="9">
+      <c r="H24" s="11">
         <v>339039.0</v>
       </c>
-      <c r="I24" s="9">
+      <c r="I24" s="11">
         <v>2048.0</v>
       </c>
-      <c r="J24" s="15">
+      <c r="J24" s="16">
         <v>68405.66</v>
       </c>
-      <c r="K24" s="15">
+      <c r="K24" s="16">
         <v>68405.66</v>
       </c>
-      <c r="L24" s="9">
+      <c r="L24" s="11">
         <v>0.0</v>
       </c>
       <c r="AB24" s="2"/>
@@ -9047,40 +9047,40 @@
       <c r="AH24" s="2"/>
     </row>
     <row r="25">
-      <c r="A25" s="9" t="s">
-        <v>113</v>
-      </c>
-      <c r="B25" s="9" t="s">
-        <v>115</v>
-      </c>
-      <c r="C25" s="9" t="s">
-        <v>116</v>
-      </c>
-      <c r="D25" s="9" t="s">
+      <c r="A25" s="11" t="s">
+        <v>124</v>
+      </c>
+      <c r="B25" s="11" t="s">
+        <v>125</v>
+      </c>
+      <c r="C25" s="11" t="s">
+        <v>126</v>
+      </c>
+      <c r="D25" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="E25" s="42">
+      <c r="E25" s="50">
         <v>45975.0</v>
       </c>
-      <c r="F25" s="9" t="s">
+      <c r="F25" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="G25" s="9">
+      <c r="G25" s="11">
         <v>12.0</v>
       </c>
-      <c r="H25" s="9">
+      <c r="H25" s="11">
         <v>339039.0</v>
       </c>
-      <c r="I25" s="9" t="s">
-        <v>107</v>
-      </c>
-      <c r="J25" s="15">
+      <c r="I25" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="J25" s="16">
         <v>1157673.06</v>
       </c>
-      <c r="K25" s="15">
+      <c r="K25" s="16">
         <v>1157673.06</v>
       </c>
-      <c r="L25" s="9">
+      <c r="L25" s="11">
         <v>0.0</v>
       </c>
       <c r="AB25" s="2"/>
@@ -9092,40 +9092,40 @@
       <c r="AH25" s="2"/>
     </row>
     <row r="26">
-      <c r="A26" s="9" t="s">
-        <v>117</v>
-      </c>
-      <c r="B26" s="9" t="s">
+      <c r="A26" s="11" t="s">
+        <v>130</v>
+      </c>
+      <c r="B26" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="C26" s="9" t="s">
-        <v>119</v>
-      </c>
-      <c r="D26" s="9" t="s">
+      <c r="C26" s="11" t="s">
+        <v>132</v>
+      </c>
+      <c r="D26" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="E26" s="42">
+      <c r="E26" s="50">
         <v>45989.0</v>
       </c>
-      <c r="F26" s="9" t="s">
+      <c r="F26" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="G26" s="9">
+      <c r="G26" s="11">
         <v>12.0</v>
       </c>
-      <c r="H26" s="9">
+      <c r="H26" s="11">
         <v>339039.0</v>
       </c>
-      <c r="I26" s="9">
+      <c r="I26" s="11">
         <v>2048.0</v>
       </c>
-      <c r="J26" s="15">
+      <c r="J26" s="16">
         <v>34065.36</v>
       </c>
-      <c r="K26" s="15">
+      <c r="K26" s="16">
         <v>34065.36</v>
       </c>
-      <c r="L26" s="9">
+      <c r="L26" s="11">
         <v>0.0</v>
       </c>
       <c r="AB26" s="2"/>
@@ -9137,40 +9137,40 @@
       <c r="AH26" s="2"/>
     </row>
     <row r="27">
-      <c r="A27" s="9" t="s">
-        <v>120</v>
-      </c>
-      <c r="B27" s="9" t="s">
-        <v>121</v>
-      </c>
-      <c r="C27" s="9" t="s">
-        <v>122</v>
-      </c>
-      <c r="D27" s="9" t="s">
+      <c r="A27" s="11" t="s">
+        <v>134</v>
+      </c>
+      <c r="B27" s="11" t="s">
+        <v>135</v>
+      </c>
+      <c r="C27" s="11" t="s">
+        <v>136</v>
+      </c>
+      <c r="D27" s="11" t="s">
         <v>4</v>
       </c>
       <c r="E27" s="13">
         <v>46104.0</v>
       </c>
-      <c r="F27" s="9" t="s">
+      <c r="F27" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="G27" s="9">
+      <c r="G27" s="11">
         <v>12.0</v>
       </c>
-      <c r="H27" s="9">
+      <c r="H27" s="11">
         <v>339039.0</v>
       </c>
-      <c r="I27" s="9">
+      <c r="I27" s="11">
         <v>2048.0</v>
       </c>
-      <c r="J27" s="15">
+      <c r="J27" s="16">
         <v>1770880.5</v>
       </c>
-      <c r="K27" s="15">
+      <c r="K27" s="16">
         <v>843261.89</v>
       </c>
-      <c r="L27" s="15">
+      <c r="L27" s="16">
         <v>927618.61</v>
       </c>
       <c r="AB27" s="2"/>
@@ -9182,40 +9182,40 @@
       <c r="AH27" s="2"/>
     </row>
     <row r="28">
-      <c r="A28" s="9" t="s">
-        <v>124</v>
-      </c>
-      <c r="B28" s="9" t="s">
-        <v>125</v>
-      </c>
-      <c r="C28" s="9" t="s">
-        <v>126</v>
-      </c>
-      <c r="D28" s="9" t="s">
+      <c r="A28" s="11" t="s">
+        <v>140</v>
+      </c>
+      <c r="B28" s="11" t="s">
+        <v>141</v>
+      </c>
+      <c r="C28" s="11" t="s">
+        <v>142</v>
+      </c>
+      <c r="D28" s="11" t="s">
         <v>4</v>
       </c>
       <c r="E28" s="13">
         <v>46120.0</v>
       </c>
-      <c r="F28" s="9" t="s">
+      <c r="F28" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="G28" s="9">
+      <c r="G28" s="11">
         <v>12.0</v>
       </c>
-      <c r="H28" s="9">
+      <c r="H28" s="11">
         <v>339039.0</v>
       </c>
-      <c r="I28" s="9" t="s">
+      <c r="I28" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="J28" s="15">
+      <c r="J28" s="16">
         <v>1912292.52</v>
       </c>
-      <c r="K28" s="9">
+      <c r="K28" s="11">
         <v>0.0</v>
       </c>
-      <c r="L28" s="15">
+      <c r="L28" s="16">
         <v>1912292.52</v>
       </c>
       <c r="AB28" s="2"/>
@@ -9227,40 +9227,40 @@
       <c r="AH28" s="2"/>
     </row>
     <row r="29">
-      <c r="A29" s="9" t="s">
-        <v>128</v>
-      </c>
-      <c r="B29" s="9" t="s">
-        <v>129</v>
-      </c>
-      <c r="C29" s="9" t="s">
-        <v>130</v>
-      </c>
-      <c r="D29" s="9" t="s">
+      <c r="A29" s="11" t="s">
+        <v>146</v>
+      </c>
+      <c r="B29" s="11" t="s">
+        <v>147</v>
+      </c>
+      <c r="C29" s="11" t="s">
+        <v>148</v>
+      </c>
+      <c r="D29" s="11" t="s">
         <v>4</v>
       </c>
       <c r="E29" s="13">
         <v>46196.0</v>
       </c>
-      <c r="F29" s="9" t="s">
+      <c r="F29" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="G29" s="9">
+      <c r="G29" s="11">
         <v>12.0</v>
       </c>
-      <c r="H29" s="9">
+      <c r="H29" s="11">
         <v>339039.0</v>
       </c>
-      <c r="I29" s="9">
+      <c r="I29" s="11">
         <v>2048.0</v>
       </c>
-      <c r="J29" s="15">
+      <c r="J29" s="16">
         <v>1496713.48</v>
       </c>
-      <c r="K29" s="9">
+      <c r="K29" s="11">
         <v>0.0</v>
       </c>
-      <c r="L29" s="15">
+      <c r="L29" s="16">
         <v>1496713.48</v>
       </c>
       <c r="AB29" s="2"/>
@@ -9272,40 +9272,40 @@
       <c r="AH29" s="2"/>
     </row>
     <row r="30">
-      <c r="A30" s="9" t="s">
-        <v>132</v>
-      </c>
-      <c r="B30" s="9" t="s">
-        <v>133</v>
-      </c>
-      <c r="C30" s="9" t="s">
-        <v>134</v>
-      </c>
-      <c r="D30" s="9" t="s">
+      <c r="A30" s="11" t="s">
+        <v>151</v>
+      </c>
+      <c r="B30" s="11" t="s">
+        <v>152</v>
+      </c>
+      <c r="C30" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="D30" s="11" t="s">
         <v>4</v>
       </c>
       <c r="E30" s="13">
         <v>46205.0</v>
       </c>
-      <c r="F30" s="9" t="s">
+      <c r="F30" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="G30" s="9">
+      <c r="G30" s="11">
         <v>12.0</v>
       </c>
-      <c r="H30" s="9">
+      <c r="H30" s="11">
         <v>339039.0</v>
       </c>
-      <c r="I30" s="9" t="s">
+      <c r="I30" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="J30" s="15">
+      <c r="J30" s="16">
         <v>624166.14</v>
       </c>
-      <c r="K30" s="9">
+      <c r="K30" s="11">
         <v>0.0</v>
       </c>
-      <c r="L30" s="15">
+      <c r="L30" s="16">
         <v>624166.14</v>
       </c>
       <c r="AB30" s="2"/>
@@ -9317,40 +9317,40 @@
       <c r="AH30" s="2"/>
     </row>
     <row r="31">
-      <c r="A31" s="9" t="s">
-        <v>138</v>
-      </c>
-      <c r="B31" s="9" t="s">
-        <v>139</v>
-      </c>
-      <c r="C31" s="9" t="s">
-        <v>140</v>
-      </c>
-      <c r="D31" s="9" t="s">
+      <c r="A31" s="11" t="s">
+        <v>157</v>
+      </c>
+      <c r="B31" s="11" t="s">
+        <v>158</v>
+      </c>
+      <c r="C31" s="11" t="s">
+        <v>159</v>
+      </c>
+      <c r="D31" s="11" t="s">
         <v>4</v>
       </c>
       <c r="E31" s="13">
         <v>46205.0</v>
       </c>
-      <c r="F31" s="9" t="s">
+      <c r="F31" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="G31" s="9">
+      <c r="G31" s="11">
         <v>12.0</v>
       </c>
-      <c r="H31" s="9">
+      <c r="H31" s="11">
         <v>339039.0</v>
       </c>
-      <c r="I31" s="9" t="s">
-        <v>107</v>
-      </c>
-      <c r="J31" s="15">
+      <c r="I31" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="J31" s="16">
         <v>18462.36</v>
       </c>
-      <c r="K31" s="9">
+      <c r="K31" s="11">
         <v>0.0</v>
       </c>
-      <c r="L31" s="15">
+      <c r="L31" s="16">
         <v>18462.36</v>
       </c>
       <c r="AB31" s="2"/>
@@ -9362,40 +9362,40 @@
       <c r="AH31" s="2"/>
     </row>
     <row r="32">
-      <c r="A32" s="9" t="s">
-        <v>143</v>
-      </c>
-      <c r="B32" s="9" t="s">
-        <v>139</v>
-      </c>
-      <c r="C32" s="15" t="s">
-        <v>145</v>
-      </c>
-      <c r="D32" s="9" t="s">
+      <c r="A32" s="11" t="s">
+        <v>164</v>
+      </c>
+      <c r="B32" s="11" t="s">
+        <v>158</v>
+      </c>
+      <c r="C32" s="16" t="s">
+        <v>165</v>
+      </c>
+      <c r="D32" s="11" t="s">
         <v>4</v>
       </c>
       <c r="E32" s="13">
         <v>46213.0</v>
       </c>
-      <c r="F32" s="9" t="s">
+      <c r="F32" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="G32" s="9">
+      <c r="G32" s="11">
         <v>12.0</v>
       </c>
-      <c r="H32" s="9">
+      <c r="H32" s="11">
         <v>339039.0</v>
       </c>
-      <c r="I32" s="9" t="s">
-        <v>107</v>
-      </c>
-      <c r="J32" s="15">
+      <c r="I32" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="J32" s="16">
         <v>1530656.62</v>
       </c>
-      <c r="K32" s="9">
+      <c r="K32" s="11">
         <v>0.0</v>
       </c>
-      <c r="L32" s="15">
+      <c r="L32" s="16">
         <v>1530656.62</v>
       </c>
       <c r="AB32" s="2"/>
@@ -9407,40 +9407,40 @@
       <c r="AH32" s="2"/>
     </row>
     <row r="33">
-      <c r="A33" s="9" t="s">
-        <v>149</v>
-      </c>
-      <c r="B33" s="9" t="s">
-        <v>129</v>
-      </c>
-      <c r="C33" s="15" t="s">
-        <v>151</v>
-      </c>
-      <c r="D33" s="9" t="s">
+      <c r="A33" s="11" t="s">
+        <v>168</v>
+      </c>
+      <c r="B33" s="11" t="s">
+        <v>147</v>
+      </c>
+      <c r="C33" s="16" t="s">
+        <v>169</v>
+      </c>
+      <c r="D33" s="11" t="s">
         <v>4</v>
       </c>
       <c r="E33" s="13">
         <v>46227.0</v>
       </c>
-      <c r="F33" s="9" t="s">
+      <c r="F33" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="G33" s="9">
+      <c r="G33" s="11">
         <v>12.0</v>
       </c>
-      <c r="H33" s="9">
+      <c r="H33" s="11">
         <v>339039.0</v>
       </c>
-      <c r="I33" s="9">
+      <c r="I33" s="11">
         <v>2048.0</v>
       </c>
-      <c r="J33" s="15">
+      <c r="J33" s="16">
         <v>173846.38</v>
       </c>
-      <c r="K33" s="9">
+      <c r="K33" s="11">
         <v>0.0</v>
       </c>
-      <c r="L33" s="15">
+      <c r="L33" s="16">
         <v>173846.38</v>
       </c>
       <c r="AB33" s="2"/>
@@ -9452,40 +9452,40 @@
       <c r="AH33" s="2"/>
     </row>
     <row r="34">
-      <c r="A34" s="9" t="s">
-        <v>153</v>
-      </c>
-      <c r="B34" s="9" t="s">
-        <v>154</v>
-      </c>
-      <c r="C34" s="9" t="s">
-        <v>155</v>
-      </c>
-      <c r="D34" s="9" t="s">
+      <c r="A34" s="11" t="s">
+        <v>171</v>
+      </c>
+      <c r="B34" s="11" t="s">
+        <v>172</v>
+      </c>
+      <c r="C34" s="11" t="s">
+        <v>173</v>
+      </c>
+      <c r="D34" s="11" t="s">
         <v>4</v>
       </c>
       <c r="E34" s="13">
         <v>46240.0</v>
       </c>
-      <c r="F34" s="9" t="s">
+      <c r="F34" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="G34" s="9">
+      <c r="G34" s="11">
         <v>12.0</v>
       </c>
-      <c r="H34" s="9">
+      <c r="H34" s="11">
         <v>339039.0</v>
       </c>
-      <c r="I34" s="9" t="s">
-        <v>156</v>
-      </c>
-      <c r="J34" s="15">
+      <c r="I34" s="11" t="s">
+        <v>175</v>
+      </c>
+      <c r="J34" s="16">
         <v>236343.68</v>
       </c>
-      <c r="K34" s="9">
+      <c r="K34" s="11">
         <v>0.0</v>
       </c>
-      <c r="L34" s="15">
+      <c r="L34" s="16">
         <v>236343.68</v>
       </c>
       <c r="AB34" s="2"/>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (21/08/2026 08:33)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/01_Bases_Originais/005_CELOG_2025/005_CELOG-PAMALS_2025 online.xlsx
+++ b/Contrato 005/Dashboard/01_Bases_Originais/005_CELOG_2025/005_CELOG-PAMALS_2025 online.xlsx
@@ -48,36 +48,45 @@
     <t>S</t>
   </si>
   <si>
+    <t>2025NE000367</t>
+  </si>
+  <si>
+    <t>C25512</t>
+  </si>
+  <si>
+    <t>25E0385</t>
+  </si>
+  <si>
     <t>Número Contrato</t>
   </si>
   <si>
-    <t>2025NE000367</t>
-  </si>
-  <si>
     <t>UG Executora</t>
   </si>
   <si>
-    <t>C25512</t>
-  </si>
-  <si>
     <t>UG Responsável</t>
   </si>
   <si>
-    <t>25E0385</t>
-  </si>
-  <si>
     <t>UG Fiscalizadora</t>
   </si>
   <si>
     <t>Prazo Final de Execução</t>
   </si>
   <si>
+    <t>2025NE000369</t>
+  </si>
+  <si>
     <t>Prazo Final de Vigência</t>
   </si>
   <si>
+    <t>C25516</t>
+  </si>
+  <si>
     <t>Status</t>
   </si>
   <si>
+    <t>25E0387</t>
+  </si>
+  <si>
     <t>Ação</t>
   </si>
   <si>
@@ -114,18 +123,15 @@
     <t>Editar</t>
   </si>
   <si>
-    <t>2025NE000369</t>
+    <t>2025NE000371</t>
+  </si>
+  <si>
+    <t>25E0389</t>
   </si>
   <si>
     <t>005/CELOG-PAMALS/2025</t>
   </si>
   <si>
-    <t>C25516</t>
-  </si>
-  <si>
-    <t>25E0387</t>
-  </si>
-  <si>
     <t>CELOG</t>
   </si>
   <si>
@@ -144,51 +150,57 @@
     <t>R$</t>
   </si>
   <si>
-    <t>2025NE000371</t>
+    <t>2025NE000413</t>
+  </si>
+  <si>
+    <t>C25501</t>
+  </si>
+  <si>
+    <t>25E0403</t>
   </si>
   <si>
     <t>VEE ONE-MANUTENCAO E SERVICOS TECNICOS LTDA</t>
   </si>
   <si>
-    <t>25E0389</t>
-  </si>
-  <si>
-    <t>2025NE000413</t>
-  </si>
-  <si>
-    <t>C25501</t>
-  </si>
-  <si>
-    <t>25E0403</t>
-  </si>
-  <si>
     <t>20SP</t>
   </si>
   <si>
+    <t>2025NE000414</t>
+  </si>
+  <si>
+    <t>C25525</t>
+  </si>
+  <si>
+    <t>25E0431</t>
+  </si>
+  <si>
+    <t>21EM</t>
+  </si>
+  <si>
     <t>Módulo</t>
   </si>
   <si>
+    <t>2025NE000559</t>
+  </si>
+  <si>
     <t>Referência</t>
   </si>
   <si>
+    <t>C25545</t>
+  </si>
+  <si>
+    <t>25E0524</t>
+  </si>
+  <si>
     <t>Nº recibo</t>
   </si>
   <si>
-    <t>2025NE000414</t>
-  </si>
-  <si>
-    <t>C25525</t>
-  </si>
-  <si>
-    <t>25E0431</t>
-  </si>
-  <si>
-    <t>21EM</t>
-  </si>
-  <si>
     <t>Nº</t>
   </si>
   <si>
+    <t>20X7</t>
+  </si>
+  <si>
     <t>Data</t>
   </si>
   <si>
@@ -201,34 +213,28 @@
     <t>Vencimento</t>
   </si>
   <si>
+    <t>2025NE000770</t>
+  </si>
+  <si>
     <t>Valor das Nfs</t>
   </si>
   <si>
+    <t>25E0731</t>
+  </si>
+  <si>
     <t>Ordem de Pagamento</t>
   </si>
   <si>
     <t>Faturado</t>
   </si>
   <si>
-    <t>2025NE000559</t>
-  </si>
-  <si>
-    <t>C25545</t>
-  </si>
-  <si>
     <t>Pendente</t>
   </si>
   <si>
-    <t>25E0524</t>
-  </si>
-  <si>
-    <t>20X7</t>
-  </si>
-  <si>
-    <t>2025NE000770</t>
-  </si>
-  <si>
-    <t>25E0731</t>
+    <t>2025NE000774</t>
+  </si>
+  <si>
+    <t>25E0737</t>
   </si>
   <si>
     <t>FEV/25</t>
@@ -237,24 +243,18 @@
     <t>-</t>
   </si>
   <si>
-    <t>2025NE000774</t>
-  </si>
-  <si>
-    <t>25E0737</t>
+    <t>2025NE000843</t>
+  </si>
+  <si>
+    <t>C25630</t>
+  </si>
+  <si>
+    <t>25E0787</t>
   </si>
   <si>
     <t xml:space="preserve">2025NE000369 </t>
   </si>
   <si>
-    <t>2025NE000843</t>
-  </si>
-  <si>
-    <t>C25630</t>
-  </si>
-  <si>
-    <t>25E0787</t>
-  </si>
-  <si>
     <t>219C</t>
   </si>
   <si>
@@ -300,6 +300,12 @@
     <t>25E1475</t>
   </si>
   <si>
+    <t>ABR/25</t>
+  </si>
+  <si>
+    <t>2025NE000413, 2025NE000414, 2025NE000559</t>
+  </si>
+  <si>
     <t>2025NE001629</t>
   </si>
   <si>
@@ -309,10 +315,10 @@
     <t>25E1477</t>
   </si>
   <si>
-    <t>ABR/25</t>
-  </si>
-  <si>
-    <t>2025NE000413, 2025NE000414, 2025NE000559</t>
+    <t>2025NP002341</t>
+  </si>
+  <si>
+    <t>MAI/25</t>
   </si>
   <si>
     <t>2025NE001687</t>
@@ -321,52 +327,22 @@
     <t>25E1535</t>
   </si>
   <si>
-    <t>2025NP002341</t>
-  </si>
-  <si>
-    <t>MAI/25</t>
-  </si>
-  <si>
     <t>2025NE001688</t>
   </si>
   <si>
     <t>25E1536</t>
   </si>
   <si>
+    <t>2025NP002884</t>
+  </si>
+  <si>
     <t>2025NE001689</t>
   </si>
   <si>
     <t>25E1537</t>
   </si>
   <si>
-    <t>2025NE001690</t>
-  </si>
-  <si>
-    <t>2025NP002884</t>
-  </si>
-  <si>
-    <t>25E1538</t>
-  </si>
-  <si>
-    <t>2025NE001823</t>
-  </si>
-  <si>
-    <t>C25865</t>
-  </si>
-  <si>
-    <t>25E1666</t>
-  </si>
-  <si>
     <t>JUN/25</t>
-  </si>
-  <si>
-    <t>2025NE001828</t>
-  </si>
-  <si>
-    <t>C25869</t>
-  </si>
-  <si>
-    <t>25E1667</t>
   </si>
   <si>
     <t>2025NE000005,
@@ -375,55 +351,55 @@
 2025NE000774</t>
   </si>
   <si>
+    <t>2025NE001690</t>
+  </si>
+  <si>
+    <t>2025NP400522</t>
+  </si>
+  <si>
+    <t>25E1538</t>
+  </si>
+  <si>
+    <t>JUL/25</t>
+  </si>
+  <si>
+    <t>2025NE001823</t>
+  </si>
+  <si>
+    <t>C25865</t>
+  </si>
+  <si>
+    <t>25E1666</t>
+  </si>
+  <si>
+    <t>2025NE000843, 2025NE001200</t>
+  </si>
+  <si>
+    <t>2025NP003724</t>
+  </si>
+  <si>
+    <t>2025NE001828</t>
+  </si>
+  <si>
+    <t>C25869</t>
+  </si>
+  <si>
+    <t>AGO/25</t>
+  </si>
+  <si>
+    <t>25E1667</t>
+  </si>
+  <si>
     <t>20YJ</t>
   </si>
   <si>
-    <t>2025NP400522</t>
+    <t>2025NP004558</t>
   </si>
   <si>
     <t>2025NE001830</t>
   </si>
   <si>
     <t>25E1669</t>
-  </si>
-  <si>
-    <t>JUL/25</t>
-  </si>
-  <si>
-    <t>2025NE002200</t>
-  </si>
-  <si>
-    <t>C25863</t>
-  </si>
-  <si>
-    <t>2025NE000843, 2025NE001200</t>
-  </si>
-  <si>
-    <t>25E2021</t>
-  </si>
-  <si>
-    <t>2025NP003724</t>
-  </si>
-  <si>
-    <t>2025NE002237</t>
-  </si>
-  <si>
-    <t>25E2058</t>
-  </si>
-  <si>
-    <t>AGO/25</t>
-  </si>
-  <si>
-    <t>2026NE000330</t>
-  </si>
-  <si>
-    <t>C26163</t>
-  </si>
-  <si>
-    <t>2025NP004558</t>
-  </si>
-  <si>
-    <t>26E0320</t>
   </si>
   <si>
     <t>SET/25</t>
@@ -433,6 +409,51 @@
 2025NE001828</t>
   </si>
   <si>
+    <t>2025NE002200</t>
+  </si>
+  <si>
+    <t>C25863</t>
+  </si>
+  <si>
+    <t>25E2021</t>
+  </si>
+  <si>
+    <t>2025NP004897</t>
+  </si>
+  <si>
+    <t>OUT/25</t>
+  </si>
+  <si>
+    <t>2025NE002237</t>
+  </si>
+  <si>
+    <t>25E2058</t>
+  </si>
+  <si>
+    <t>2025NE001688, 2025NE001828, 2025NE002200</t>
+  </si>
+  <si>
+    <t>2025NP004932</t>
+  </si>
+  <si>
+    <t>2026NE000330</t>
+  </si>
+  <si>
+    <t>C26163</t>
+  </si>
+  <si>
+    <t>26E0320</t>
+  </si>
+  <si>
+    <t>NOV/25</t>
+  </si>
+  <si>
+    <t>2025NE001687, 2025NE001689, 2025NE001690, 2025NE001823, 2025NE001830, 2025NE002237</t>
+  </si>
+  <si>
+    <t>2026NP400440</t>
+  </si>
+  <si>
     <t>2026NE000388</t>
   </si>
   <si>
@@ -442,25 +463,25 @@
     <t>26E0375</t>
   </si>
   <si>
-    <t>2025NP004897</t>
-  </si>
-  <si>
-    <t>OUT/25</t>
-  </si>
-  <si>
-    <t>2025NE001688, 2025NE001828, 2025NE002200</t>
+    <t>DEZ/25</t>
   </si>
   <si>
     <t>2026NE000748</t>
   </si>
   <si>
+    <t>2025NE001065, 2025NE002200</t>
+  </si>
+  <si>
     <t>C26312</t>
   </si>
   <si>
     <t>26E0709</t>
   </si>
   <si>
-    <t>2025NP004932</t>
+    <t>2026NP400412</t>
+  </si>
+  <si>
+    <t>JAN/26</t>
   </si>
   <si>
     <t>2026NE000816</t>
@@ -472,7 +493,7 @@
     <t>26E0776</t>
   </si>
   <si>
-    <t>NOV/25</t>
+    <t>2026NP401035</t>
   </si>
   <si>
     <t>2026NE000817</t>
@@ -484,10 +505,13 @@
     <t>26E0777</t>
   </si>
   <si>
-    <t>2025NE001687, 2025NE001689, 2025NE001690, 2025NE001823, 2025NE001830, 2025NE002237</t>
-  </si>
-  <si>
-    <t>2026NP400440</t>
+    <t>FEV/26</t>
+  </si>
+  <si>
+    <t>2025NE001627, 2025NE001629, 2025NE001823</t>
+  </si>
+  <si>
+    <t>2026NP402272</t>
   </si>
   <si>
     <t>2026NE000842</t>
@@ -496,19 +520,28 @@
     <t>26E0803</t>
   </si>
   <si>
-    <t>DEZ/25</t>
+    <t>MAR/26</t>
+  </si>
+  <si>
+    <t>2025NE000770, 2025NE001627</t>
+  </si>
+  <si>
+    <t>R$ 1.350.542,52</t>
   </si>
   <si>
     <t>2026NE000944</t>
   </si>
   <si>
+    <t>2026NP401762</t>
+  </si>
+  <si>
     <t>26E0906</t>
   </si>
   <si>
-    <t>2025NE001065, 2025NE002200</t>
-  </si>
-  <si>
-    <t>2026NP400412</t>
+    <t>ABR/26</t>
+  </si>
+  <si>
+    <t>2025NE000770, 2025NE001065, 2025NE001627</t>
   </si>
   <si>
     <t>2026NE001015</t>
@@ -521,39 +554,6 @@
   </si>
   <si>
     <t>20XV</t>
-  </si>
-  <si>
-    <t>JAN/26</t>
-  </si>
-  <si>
-    <t>2026NP401035</t>
-  </si>
-  <si>
-    <t>FEV/26</t>
-  </si>
-  <si>
-    <t>2025NE001627, 2025NE001629, 2025NE001823</t>
-  </si>
-  <si>
-    <t>2026NP402272</t>
-  </si>
-  <si>
-    <t>MAR/26</t>
-  </si>
-  <si>
-    <t>2025NE000770, 2025NE001627</t>
-  </si>
-  <si>
-    <t>R$ 1.350.542,52</t>
-  </si>
-  <si>
-    <t>2026NP401762</t>
-  </si>
-  <si>
-    <t>ABR/26</t>
-  </si>
-  <si>
-    <t>2025NE000770, 2025NE001065, 2025NE001627</t>
   </si>
   <si>
     <t>REAJUSTE</t>
@@ -740,13 +740,13 @@
       <b/>
       <sz val="10.0"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Century Gothic"/>
     </font>
     <font>
       <b/>
       <sz val="10.0"/>
       <color theme="1"/>
-      <name val="Century Gothic"/>
+      <name val="Arial"/>
     </font>
     <font>
       <sz val="10.0"/>
@@ -904,11 +904,11 @@
     <xf borderId="0" fillId="5" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
     <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="center"/>
@@ -916,10 +916,10 @@
     <xf borderId="0" fillId="0" fontId="2" numFmtId="11" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="4" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
@@ -962,22 +962,22 @@
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="0" fontId="6" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="7" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="2" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="6" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="7" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -992,11 +992,11 @@
     <xf borderId="1" fillId="7" fontId="9" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="165" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="1" fillId="5" fontId="9" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="165" xfId="0" applyFont="1" applyNumberFormat="1"/>
-    <xf borderId="1" fillId="8" fontId="6" numFmtId="168" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="8" fontId="7" numFmtId="168" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="3" fillId="0" fontId="10" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
@@ -1018,14 +1018,14 @@
     <xf borderId="1" fillId="8" fontId="9" numFmtId="168" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="170" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="6" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="7" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="170" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="1" fillId="9" fontId="9" numFmtId="168" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
@@ -1040,13 +1040,13 @@
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="4" fillId="0" fontId="10" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="1" fillId="0" fontId="6" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="7" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="6" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="7" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="6" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="7" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="5" fontId="9" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
@@ -1055,7 +1055,7 @@
     <xf borderId="1" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="6" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="7" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="5" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -1450,7 +1450,7 @@
       <c r="B2" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="V2" s="8"/>
+      <c r="V2" s="9"/>
       <c r="W2" s="10"/>
       <c r="X2" s="10"/>
       <c r="Y2" s="10"/>
@@ -1463,38 +1463,38 @@
     <row r="3" ht="12.75" customHeight="1">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
-      <c r="C3" s="12"/>
-      <c r="D3" s="12"/>
-      <c r="E3" s="12"/>
-      <c r="F3" s="12"/>
-      <c r="G3" s="12"/>
-      <c r="H3" s="12"/>
-      <c r="I3" s="12"/>
-      <c r="J3" s="12"/>
-      <c r="K3" s="12"/>
-      <c r="L3" s="12"/>
-      <c r="M3" s="12"/>
-      <c r="N3" s="12"/>
-      <c r="O3" s="12"/>
-      <c r="P3" s="12"/>
-      <c r="Q3" s="12"/>
-      <c r="R3" s="12"/>
-      <c r="S3" s="12"/>
-      <c r="T3" s="12"/>
-      <c r="U3" s="12"/>
+      <c r="C3" s="13"/>
+      <c r="D3" s="13"/>
+      <c r="E3" s="13"/>
+      <c r="F3" s="13"/>
+      <c r="G3" s="13"/>
+      <c r="H3" s="13"/>
+      <c r="I3" s="13"/>
+      <c r="J3" s="13"/>
+      <c r="K3" s="13"/>
+      <c r="L3" s="13"/>
+      <c r="M3" s="13"/>
+      <c r="N3" s="13"/>
+      <c r="O3" s="13"/>
+      <c r="P3" s="13"/>
+      <c r="Q3" s="13"/>
+      <c r="R3" s="13"/>
+      <c r="S3" s="13"/>
+      <c r="T3" s="13"/>
+      <c r="U3" s="13"/>
       <c r="V3" s="3"/>
     </row>
     <row r="4" ht="12.75" customHeight="1">
       <c r="A4" s="15"/>
       <c r="B4" s="15"/>
       <c r="C4" s="16" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D4" s="16" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E4" s="16" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F4" s="16" t="s">
         <v>12</v>
@@ -1503,46 +1503,46 @@
         <v>13</v>
       </c>
       <c r="H4" s="17" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="I4" s="16" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="J4" s="16" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="K4" s="16" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="L4" s="16" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="M4" s="17" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="N4" s="17" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="O4" s="17" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="P4" s="17" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="Q4" s="17" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="R4" s="16" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="S4" s="16" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="T4" s="16" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="U4" s="16" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="V4" s="3"/>
     </row>
@@ -1551,16 +1551,16 @@
       <c r="B5" s="15"/>
       <c r="C5" s="18"/>
       <c r="D5" s="19" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="E5" s="19" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F5" s="19" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="G5" s="19" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="H5" s="20">
         <v>1564.0</v>
@@ -1569,16 +1569,16 @@
         <v>1564.0</v>
       </c>
       <c r="J5" s="19" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="K5" s="19" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="L5" s="19" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="M5" s="19" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="N5" s="21">
         <v>9.165159737E7</v>
@@ -1596,7 +1596,7 @@
         <v>1.085943044E7</v>
       </c>
       <c r="S5" s="19" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="V5" s="3"/>
     </row>
@@ -1628,43 +1628,43 @@
     <row r="8" ht="12.75" customHeight="1">
       <c r="A8" s="23"/>
       <c r="B8" s="23"/>
-      <c r="C8" s="28" t="s">
-        <v>45</v>
-      </c>
-      <c r="D8" s="28" t="s">
-        <v>46</v>
-      </c>
-      <c r="E8" s="29" t="s">
-        <v>47</v>
-      </c>
-      <c r="F8" s="28" t="s">
-        <v>52</v>
-      </c>
-      <c r="G8" s="28" t="s">
-        <v>53</v>
-      </c>
-      <c r="H8" s="28" t="s">
+      <c r="C8" s="29" t="s">
+        <v>49</v>
+      </c>
+      <c r="D8" s="29" t="s">
+        <v>51</v>
+      </c>
+      <c r="E8" s="30" t="s">
         <v>54</v>
       </c>
-      <c r="I8" s="29" t="s">
+      <c r="F8" s="29" t="s">
         <v>55</v>
       </c>
-      <c r="J8" s="28" t="s">
-        <v>56</v>
-      </c>
-      <c r="K8" s="28" t="s">
+      <c r="G8" s="29" t="s">
         <v>57</v>
       </c>
+      <c r="H8" s="29" t="s">
+        <v>58</v>
+      </c>
+      <c r="I8" s="30" t="s">
+        <v>59</v>
+      </c>
+      <c r="J8" s="29" t="s">
+        <v>60</v>
+      </c>
+      <c r="K8" s="29" t="s">
+        <v>62</v>
+      </c>
       <c r="L8" s="31" t="s">
-        <v>58</v>
-      </c>
-      <c r="M8" s="29" t="s">
-        <v>59</v>
-      </c>
-      <c r="N8" s="28" t="s">
-        <v>62</v>
-      </c>
-      <c r="O8" s="28"/>
+        <v>64</v>
+      </c>
+      <c r="M8" s="30" t="s">
+        <v>65</v>
+      </c>
+      <c r="N8" s="29" t="s">
+        <v>66</v>
+      </c>
+      <c r="O8" s="29"/>
       <c r="P8" s="27"/>
       <c r="V8" s="3"/>
     </row>
@@ -1675,10 +1675,10 @@
         <v>1.0</v>
       </c>
       <c r="D9" s="33" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E9" s="34" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="F9" s="35">
         <v>594.0</v>
@@ -1687,7 +1687,7 @@
         <v>45740.0</v>
       </c>
       <c r="H9" s="35" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="I9" s="36"/>
       <c r="J9" s="36">
@@ -1699,7 +1699,7 @@
       <c r="L9" s="35" t="s">
         <v>76</v>
       </c>
-      <c r="M9" s="38">
+      <c r="M9" s="39">
         <f t="shared" ref="M9:M10" si="1">K9</f>
         <v>748504.24</v>
       </c>
@@ -1716,7 +1716,7 @@
         <v>82</v>
       </c>
       <c r="E10" s="34" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="F10" s="35">
         <v>620.0</v>
@@ -1737,7 +1737,7 @@
       <c r="L10" s="35" t="s">
         <v>87</v>
       </c>
-      <c r="M10" s="38">
+      <c r="M10" s="39">
         <f t="shared" si="1"/>
         <v>1110378.24</v>
       </c>
@@ -1751,10 +1751,10 @@
       <c r="B11" s="23"/>
       <c r="C11" s="41"/>
       <c r="D11" s="33" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="E11" s="34" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="F11" s="35">
         <v>634.0</v>
@@ -1763,7 +1763,7 @@
         <v>45799.0</v>
       </c>
       <c r="H11" s="35" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="I11" s="36"/>
       <c r="J11" s="36">
@@ -1773,9 +1773,9 @@
         <v>974557.12</v>
       </c>
       <c r="L11" s="34" t="s">
-        <v>97</v>
-      </c>
-      <c r="M11" s="38">
+        <v>95</v>
+      </c>
+      <c r="M11" s="39">
         <v>974557.12</v>
       </c>
       <c r="N11" s="42"/>
@@ -1788,10 +1788,10 @@
       <c r="B12" s="23"/>
       <c r="C12" s="41"/>
       <c r="D12" s="33" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="E12" s="34" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="F12" s="34">
         <v>660.0</v>
@@ -1800,7 +1800,7 @@
         <v>45856.0</v>
       </c>
       <c r="H12" s="44" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I12" s="36"/>
       <c r="J12" s="36">
@@ -1810,9 +1810,9 @@
         <v>1402001.34</v>
       </c>
       <c r="L12" s="46" t="s">
-        <v>104</v>
-      </c>
-      <c r="M12" s="38">
+        <v>101</v>
+      </c>
+      <c r="M12" s="39">
         <v>1402001.34</v>
       </c>
       <c r="N12" s="47"/>
@@ -1824,11 +1824,11 @@
       <c r="A13" s="23"/>
       <c r="B13" s="23"/>
       <c r="C13" s="41"/>
-      <c r="D13" s="49" t="s">
-        <v>109</v>
+      <c r="D13" s="48" t="s">
+        <v>104</v>
       </c>
       <c r="E13" s="34" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="F13" s="35">
         <v>661.0</v>
@@ -1837,7 +1837,7 @@
         <v>45856.0</v>
       </c>
       <c r="H13" s="35" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="I13" s="43"/>
       <c r="J13" s="43">
@@ -1847,25 +1847,25 @@
         <v>1223702.3</v>
       </c>
       <c r="L13" s="34" t="s">
-        <v>115</v>
-      </c>
-      <c r="M13" s="38">
+        <v>107</v>
+      </c>
+      <c r="M13" s="39">
         <v>1223702.3</v>
       </c>
       <c r="N13" s="47"/>
       <c r="O13" s="25"/>
-      <c r="P13" s="50"/>
+      <c r="P13" s="49"/>
       <c r="V13" s="3"/>
     </row>
     <row r="14">
       <c r="A14" s="23"/>
       <c r="B14" s="23"/>
       <c r="C14" s="41"/>
-      <c r="D14" s="49" t="s">
-        <v>118</v>
+      <c r="D14" s="48" t="s">
+        <v>109</v>
       </c>
       <c r="E14" s="34" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="F14" s="34">
         <v>688.0</v>
@@ -1874,7 +1874,7 @@
         <v>45901.0</v>
       </c>
       <c r="H14" s="34" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
       <c r="I14" s="43"/>
       <c r="J14" s="43">
@@ -1884,9 +1884,9 @@
         <v>1011677.95</v>
       </c>
       <c r="L14" s="34" t="s">
-        <v>123</v>
-      </c>
-      <c r="M14" s="38">
+        <v>114</v>
+      </c>
+      <c r="M14" s="39">
         <v>1011677.95</v>
       </c>
       <c r="N14" s="42"/>
@@ -1898,11 +1898,11 @@
       <c r="A15" s="23"/>
       <c r="B15" s="23"/>
       <c r="C15" s="41"/>
-      <c r="D15" s="49" t="s">
-        <v>126</v>
+      <c r="D15" s="48" t="s">
+        <v>117</v>
       </c>
       <c r="E15" s="34" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="F15" s="34">
         <v>696.0</v>
@@ -1921,9 +1921,9 @@
         <v>896744.06</v>
       </c>
       <c r="L15" s="34" t="s">
-        <v>129</v>
-      </c>
-      <c r="M15" s="38">
+        <v>120</v>
+      </c>
+      <c r="M15" s="39">
         <v>896744.06</v>
       </c>
       <c r="N15" s="47"/>
@@ -1934,11 +1934,11 @@
       <c r="A16" s="23"/>
       <c r="B16" s="23"/>
       <c r="C16" s="41"/>
-      <c r="D16" s="49" t="s">
-        <v>131</v>
+      <c r="D16" s="48" t="s">
+        <v>123</v>
       </c>
       <c r="E16" s="34" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="F16" s="34">
         <v>704.0</v>
@@ -1947,7 +1947,7 @@
         <v>45957.0</v>
       </c>
       <c r="H16" s="34" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
       <c r="I16" s="43"/>
       <c r="J16" s="43">
@@ -1957,9 +1957,9 @@
         <v>919329.06</v>
       </c>
       <c r="L16" s="34" t="s">
-        <v>136</v>
-      </c>
-      <c r="M16" s="38">
+        <v>128</v>
+      </c>
+      <c r="M16" s="39">
         <v>919329.06</v>
       </c>
       <c r="N16" s="42"/>
@@ -1970,8 +1970,8 @@
       <c r="A17" s="23"/>
       <c r="B17" s="23"/>
       <c r="C17" s="41"/>
-      <c r="D17" s="49" t="s">
-        <v>137</v>
+      <c r="D17" s="48" t="s">
+        <v>129</v>
       </c>
       <c r="E17" s="34"/>
       <c r="F17" s="34">
@@ -1981,7 +1981,7 @@
         <v>45972.0</v>
       </c>
       <c r="H17" s="34" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="I17" s="34"/>
       <c r="J17" s="43">
@@ -1991,9 +1991,9 @@
         <v>1157009.26</v>
       </c>
       <c r="L17" s="34" t="s">
-        <v>142</v>
-      </c>
-      <c r="M17" s="38">
+        <v>133</v>
+      </c>
+      <c r="M17" s="39">
         <v>1157009.26</v>
       </c>
       <c r="N17" s="51"/>
@@ -2004,11 +2004,11 @@
       <c r="A18" s="23"/>
       <c r="B18" s="23"/>
       <c r="C18" s="41"/>
-      <c r="D18" s="49" t="s">
-        <v>146</v>
+      <c r="D18" s="48" t="s">
+        <v>137</v>
       </c>
       <c r="E18" s="34" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="F18" s="34">
         <v>728.0</v>
@@ -2017,7 +2017,7 @@
         <v>46008.0</v>
       </c>
       <c r="H18" s="34" t="s">
-        <v>150</v>
+        <v>138</v>
       </c>
       <c r="I18" s="34"/>
       <c r="J18" s="43">
@@ -2027,9 +2027,9 @@
         <v>1214597.952</v>
       </c>
       <c r="L18" s="34" t="s">
-        <v>151</v>
-      </c>
-      <c r="M18" s="38">
+        <v>139</v>
+      </c>
+      <c r="M18" s="39">
         <v>1214597.952</v>
       </c>
       <c r="N18" s="51"/>
@@ -2044,11 +2044,11 @@
       <c r="A19" s="23"/>
       <c r="B19" s="23"/>
       <c r="C19" s="41"/>
-      <c r="D19" s="49" t="s">
-        <v>154</v>
+      <c r="D19" s="48" t="s">
+        <v>143</v>
       </c>
       <c r="E19" s="34" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="F19" s="34">
         <v>278.0</v>
@@ -2057,7 +2057,7 @@
         <v>46042.0</v>
       </c>
       <c r="H19" s="34" t="s">
-        <v>157</v>
+        <v>145</v>
       </c>
       <c r="I19" s="43"/>
       <c r="J19" s="43">
@@ -2067,9 +2067,9 @@
         <v>967082.09</v>
       </c>
       <c r="L19" s="34" t="s">
-        <v>158</v>
-      </c>
-      <c r="M19" s="38">
+        <v>148</v>
+      </c>
+      <c r="M19" s="39">
         <v>967082.09</v>
       </c>
       <c r="N19" s="51"/>
@@ -2084,8 +2084,8 @@
       <c r="A20" s="23"/>
       <c r="B20" s="23"/>
       <c r="C20" s="41"/>
-      <c r="D20" s="49" t="s">
-        <v>163</v>
+      <c r="D20" s="48" t="s">
+        <v>149</v>
       </c>
       <c r="E20" s="34"/>
       <c r="F20" s="34">
@@ -2095,7 +2095,7 @@
         <v>46078.0</v>
       </c>
       <c r="H20" s="34" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="I20" s="43"/>
       <c r="J20" s="43">
@@ -2105,9 +2105,9 @@
         <v>719561.08</v>
       </c>
       <c r="L20" s="34" t="s">
-        <v>164</v>
-      </c>
-      <c r="M20" s="38">
+        <v>153</v>
+      </c>
+      <c r="M20" s="39">
         <v>719561.08</v>
       </c>
       <c r="N20" s="51"/>
@@ -2122,8 +2122,8 @@
       <c r="A21" s="23"/>
       <c r="B21" s="23"/>
       <c r="C21" s="41"/>
-      <c r="D21" s="49" t="s">
-        <v>165</v>
+      <c r="D21" s="48" t="s">
+        <v>157</v>
       </c>
       <c r="E21" s="34"/>
       <c r="F21" s="34">
@@ -2133,7 +2133,7 @@
         <v>46094.0</v>
       </c>
       <c r="H21" s="34" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="I21" s="43"/>
       <c r="J21" s="43">
@@ -2143,9 +2143,9 @@
         <v>885881.08</v>
       </c>
       <c r="L21" s="34" t="s">
-        <v>167</v>
-      </c>
-      <c r="M21" s="38">
+        <v>159</v>
+      </c>
+      <c r="M21" s="39">
         <v>885881.08</v>
       </c>
       <c r="N21" s="51"/>
@@ -2160,8 +2160,8 @@
       <c r="A22" s="23"/>
       <c r="B22" s="23"/>
       <c r="C22" s="41"/>
-      <c r="D22" s="49" t="s">
-        <v>168</v>
+      <c r="D22" s="48" t="s">
+        <v>162</v>
       </c>
       <c r="E22" s="34"/>
       <c r="F22" s="34">
@@ -2171,20 +2171,20 @@
         <v>46128.0</v>
       </c>
       <c r="H22" s="34" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
       <c r="I22" s="43"/>
       <c r="J22" s="43">
         <v>46164.0</v>
       </c>
       <c r="K22" s="45" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="L22" s="34" t="s">
-        <v>171</v>
-      </c>
-      <c r="M22" s="38" t="s">
-        <v>170</v>
+        <v>166</v>
+      </c>
+      <c r="M22" s="39" t="s">
+        <v>164</v>
       </c>
       <c r="N22" s="51"/>
       <c r="O22" s="25"/>
@@ -2198,8 +2198,8 @@
       <c r="A23" s="23"/>
       <c r="B23" s="23"/>
       <c r="C23" s="41"/>
-      <c r="D23" s="49" t="s">
-        <v>172</v>
+      <c r="D23" s="48" t="s">
+        <v>168</v>
       </c>
       <c r="E23" s="34"/>
       <c r="F23" s="34">
@@ -2209,7 +2209,7 @@
         <v>46156.0</v>
       </c>
       <c r="H23" s="34" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="I23" s="43"/>
       <c r="J23" s="43">
@@ -2219,9 +2219,9 @@
         <v>1108954.4358333333</v>
       </c>
       <c r="L23" s="34" t="s">
-        <v>167</v>
-      </c>
-      <c r="M23" s="38">
+        <v>159</v>
+      </c>
+      <c r="M23" s="39">
         <v>1108954.4358333333</v>
       </c>
       <c r="N23" s="53"/>
@@ -2236,7 +2236,7 @@
       <c r="A24" s="23"/>
       <c r="B24" s="23"/>
       <c r="C24" s="41"/>
-      <c r="D24" s="49" t="s">
+      <c r="D24" s="48" t="s">
         <v>174</v>
       </c>
       <c r="E24" s="34"/>
@@ -2247,7 +2247,7 @@
         <v>46149.0</v>
       </c>
       <c r="H24" s="34" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="I24" s="43"/>
       <c r="J24" s="43">
@@ -2259,7 +2259,7 @@
       <c r="L24" s="34" t="s">
         <v>175</v>
       </c>
-      <c r="M24" s="38">
+      <c r="M24" s="39">
         <v>218206.1</v>
       </c>
       <c r="N24" s="54"/>
@@ -2274,7 +2274,7 @@
       <c r="A25" s="23"/>
       <c r="B25" s="23"/>
       <c r="C25" s="41"/>
-      <c r="D25" s="49" t="s">
+      <c r="D25" s="48" t="s">
         <v>176</v>
       </c>
       <c r="E25" s="34"/>
@@ -2285,7 +2285,7 @@
         <v>46156.0</v>
       </c>
       <c r="H25" s="34" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="I25" s="43"/>
       <c r="J25" s="43">
@@ -2297,7 +2297,7 @@
       <c r="L25" s="34" t="s">
         <v>177</v>
       </c>
-      <c r="M25" s="38">
+      <c r="M25" s="39">
         <v>1549250.84</v>
       </c>
       <c r="N25" s="54"/>
@@ -2312,7 +2312,7 @@
       <c r="A26" s="23"/>
       <c r="B26" s="23"/>
       <c r="C26" s="55"/>
-      <c r="D26" s="49" t="s">
+      <c r="D26" s="48" t="s">
         <v>178</v>
       </c>
       <c r="E26" s="34"/>
@@ -2335,7 +2335,7 @@
       <c r="L26" s="34" t="s">
         <v>181</v>
       </c>
-      <c r="M26" s="38" t="s">
+      <c r="M26" s="39" t="s">
         <v>180</v>
       </c>
       <c r="N26" s="54"/>
@@ -2350,7 +2350,7 @@
       <c r="A27" s="23"/>
       <c r="B27" s="23"/>
       <c r="C27" s="35"/>
-      <c r="D27" s="49" t="s">
+      <c r="D27" s="48" t="s">
         <v>182</v>
       </c>
       <c r="E27" s="34"/>
@@ -2361,7 +2361,7 @@
       <c r="J27" s="43"/>
       <c r="K27" s="45"/>
       <c r="L27" s="34"/>
-      <c r="M27" s="38"/>
+      <c r="M27" s="39"/>
       <c r="N27" s="54" t="s">
         <v>183</v>
       </c>
@@ -2375,35 +2375,35 @@
     <row r="28" ht="30.75" customHeight="1">
       <c r="A28" s="23"/>
       <c r="B28" s="23"/>
-      <c r="C28" s="28" t="s">
-        <v>45</v>
-      </c>
-      <c r="D28" s="28" t="s">
-        <v>46</v>
-      </c>
-      <c r="E28" s="29" t="s">
-        <v>47</v>
-      </c>
-      <c r="F28" s="28" t="s">
-        <v>52</v>
-      </c>
-      <c r="G28" s="28"/>
-      <c r="H28" s="28" t="s">
+      <c r="C28" s="29" t="s">
+        <v>49</v>
+      </c>
+      <c r="D28" s="29" t="s">
+        <v>51</v>
+      </c>
+      <c r="E28" s="30" t="s">
         <v>54</v>
       </c>
-      <c r="I28" s="28"/>
-      <c r="J28" s="28"/>
+      <c r="F28" s="29" t="s">
+        <v>55</v>
+      </c>
+      <c r="G28" s="29"/>
+      <c r="H28" s="29" t="s">
+        <v>58</v>
+      </c>
+      <c r="I28" s="29"/>
+      <c r="J28" s="29"/>
       <c r="K28" s="56" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="L28" s="31" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="M28" s="57" t="s">
-        <v>59</v>
-      </c>
-      <c r="N28" s="28" t="s">
-        <v>62</v>
+        <v>65</v>
+      </c>
+      <c r="N28" s="29" t="s">
+        <v>66</v>
       </c>
       <c r="O28" s="25"/>
       <c r="P28" s="27"/>
@@ -2437,7 +2437,7 @@
         <v>45791.0</v>
       </c>
       <c r="H29" s="35" t="s">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="I29" s="36"/>
       <c r="J29" s="36">
@@ -2498,7 +2498,7 @@
       <c r="L30" s="34" t="s">
         <v>188</v>
       </c>
-      <c r="M30" s="38">
+      <c r="M30" s="39">
         <v>112720.77</v>
       </c>
       <c r="N30" s="51"/>
@@ -2535,7 +2535,7 @@
         <v>45853.0</v>
       </c>
       <c r="H31" s="34" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="I31" s="43"/>
       <c r="J31" s="43">
@@ -2547,7 +2547,7 @@
       <c r="L31" s="34" t="s">
         <v>191</v>
       </c>
-      <c r="M31" s="38">
+      <c r="M31" s="39">
         <v>378307.61</v>
       </c>
       <c r="N31" s="51"/>
@@ -2584,7 +2584,7 @@
         <v>45910.0</v>
       </c>
       <c r="H32" s="34" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="I32" s="43"/>
       <c r="J32" s="43">
@@ -2596,7 +2596,7 @@
       <c r="L32" s="34" t="s">
         <v>193</v>
       </c>
-      <c r="M32" s="38">
+      <c r="M32" s="39">
         <v>3315.04710000003</v>
       </c>
       <c r="N32" s="51"/>
@@ -2633,7 +2633,7 @@
         <v>45904.0</v>
       </c>
       <c r="H33" s="34" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I33" s="66"/>
       <c r="J33" s="66">
@@ -2645,7 +2645,7 @@
       <c r="L33" s="34" t="s">
         <v>195</v>
       </c>
-      <c r="M33" s="38">
+      <c r="M33" s="39">
         <v>198332.75</v>
       </c>
       <c r="N33" s="51"/>
@@ -2682,7 +2682,7 @@
         <v>46008.0</v>
       </c>
       <c r="H34" s="34" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="I34" s="66"/>
       <c r="J34" s="66">
@@ -2731,7 +2731,7 @@
         <v>45930.0</v>
       </c>
       <c r="H35" s="34" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I35" s="66"/>
       <c r="J35" s="66">
@@ -2780,7 +2780,7 @@
         <v>45968.0</v>
       </c>
       <c r="H36" s="34" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="I36" s="66"/>
       <c r="J36" s="66">
@@ -2829,7 +2829,7 @@
         <v>46043.0</v>
       </c>
       <c r="H37" s="65" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="I37" s="70"/>
       <c r="J37" s="69">
@@ -2841,7 +2841,7 @@
       <c r="L37" s="34" t="s">
         <v>207</v>
       </c>
-      <c r="M37" s="38">
+      <c r="M37" s="39">
         <v>11372.9</v>
       </c>
       <c r="N37" s="51"/>
@@ -2878,7 +2878,7 @@
       <c r="J38" s="69"/>
       <c r="K38" s="45"/>
       <c r="L38" s="34"/>
-      <c r="M38" s="38"/>
+      <c r="M38" s="39"/>
       <c r="N38" s="51">
         <v>15854.78</v>
       </c>
@@ -2915,7 +2915,7 @@
       <c r="J39" s="69"/>
       <c r="K39" s="45"/>
       <c r="L39" s="34"/>
-      <c r="M39" s="38"/>
+      <c r="M39" s="39"/>
       <c r="N39" s="71">
         <v>42229.72325</v>
       </c>
@@ -2952,7 +2952,7 @@
       <c r="J40" s="69"/>
       <c r="K40" s="45"/>
       <c r="L40" s="46"/>
-      <c r="M40" s="38"/>
+      <c r="M40" s="39"/>
       <c r="N40" s="72">
         <v>48857.395500000006</v>
       </c>
@@ -2989,7 +2989,7 @@
       <c r="J41" s="69"/>
       <c r="K41" s="45"/>
       <c r="L41" s="46"/>
-      <c r="M41" s="38"/>
+      <c r="M41" s="39"/>
       <c r="N41" s="72"/>
       <c r="O41" s="25"/>
       <c r="P41" s="27"/>
@@ -3024,7 +3024,7 @@
         <v>46104.0</v>
       </c>
       <c r="H42" s="65" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="I42" s="70"/>
       <c r="J42" s="69">
@@ -3081,7 +3081,7 @@
         <v>58868.35</v>
       </c>
       <c r="L43" s="34" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="M43" s="74">
         <v>58868.35</v>
@@ -8055,31 +8055,31 @@
       <c r="AH2" s="2"/>
     </row>
     <row r="3">
-      <c r="A3" s="9" t="s">
+      <c r="A3" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="9" t="s">
+      <c r="B3" s="8" t="s">
         <v>3</v>
       </c>
       <c r="C3" s="11">
         <v>2.5E32</v>
       </c>
-      <c r="D3" s="9" t="s">
+      <c r="D3" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="13">
+      <c r="E3" s="12">
         <v>45686.0</v>
       </c>
-      <c r="F3" s="9" t="s">
+      <c r="F3" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G3" s="9">
+      <c r="G3" s="8">
         <v>12.0</v>
       </c>
-      <c r="H3" s="9">
+      <c r="H3" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I3" s="9">
+      <c r="I3" s="8">
         <v>2048.0</v>
       </c>
       <c r="J3" s="14">
@@ -8088,7 +8088,7 @@
       <c r="K3" s="14">
         <v>1000.0</v>
       </c>
-      <c r="L3" s="9">
+      <c r="L3" s="8">
         <v>0.0</v>
       </c>
       <c r="AB3" s="2"/>
@@ -8100,31 +8100,31 @@
       <c r="AH3" s="2"/>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="s">
+      <c r="A4" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="C4" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="D4" s="9" t="s">
+      <c r="C4" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="13">
+      <c r="E4" s="12">
         <v>45762.0</v>
       </c>
-      <c r="F4" s="9" t="s">
+      <c r="F4" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G4" s="9">
+      <c r="G4" s="8">
         <v>12.0</v>
       </c>
-      <c r="H4" s="9">
+      <c r="H4" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I4" s="9">
+      <c r="I4" s="8">
         <v>2048.0</v>
       </c>
       <c r="J4" s="14">
@@ -8133,7 +8133,7 @@
       <c r="K4" s="14">
         <v>52250.04</v>
       </c>
-      <c r="L4" s="9">
+      <c r="L4" s="8">
         <v>0.0</v>
       </c>
       <c r="AB4" s="2"/>
@@ -8145,31 +8145,31 @@
       <c r="AH4" s="2"/>
     </row>
     <row r="5">
-      <c r="A5" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="B5" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="C5" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="D5" s="9" t="s">
+      <c r="A5" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="D5" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E5" s="13">
+      <c r="E5" s="12">
         <v>45762.0</v>
       </c>
-      <c r="F5" s="9" t="s">
+      <c r="F5" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G5" s="9">
+      <c r="G5" s="8">
         <v>12.0</v>
       </c>
-      <c r="H5" s="9">
+      <c r="H5" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I5" s="9">
+      <c r="I5" s="8">
         <v>2048.0</v>
       </c>
       <c r="J5" s="14">
@@ -8178,7 +8178,7 @@
       <c r="K5" s="14">
         <v>881914.18</v>
       </c>
-      <c r="L5" s="9">
+      <c r="L5" s="8">
         <v>0.0</v>
       </c>
       <c r="AB5" s="2"/>
@@ -8190,31 +8190,31 @@
       <c r="AH5" s="2"/>
     </row>
     <row r="6">
-      <c r="A6" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="B6" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="C6" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="D6" s="9" t="s">
+      <c r="A6" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="D6" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E6" s="13">
+      <c r="E6" s="12">
         <v>45762.0</v>
       </c>
-      <c r="F6" s="9" t="s">
+      <c r="F6" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G6" s="9">
+      <c r="G6" s="8">
         <v>12.0</v>
       </c>
-      <c r="H6" s="9">
+      <c r="H6" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I6" s="9">
+      <c r="I6" s="8">
         <v>2048.0</v>
       </c>
       <c r="J6" s="14">
@@ -8223,7 +8223,7 @@
       <c r="K6" s="14">
         <v>750000.0</v>
       </c>
-      <c r="L6" s="9">
+      <c r="L6" s="8">
         <v>0.0</v>
       </c>
       <c r="AB6" s="2"/>
@@ -8235,31 +8235,31 @@
       <c r="AH6" s="2"/>
     </row>
     <row r="7">
-      <c r="A7" s="9" t="s">
+      <c r="A7" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="B7" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="B7" s="9" t="s">
+      <c r="C7" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="C7" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="D7" s="9" t="s">
+      <c r="D7" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E7" s="13">
+      <c r="E7" s="12">
         <v>45763.0</v>
       </c>
-      <c r="F7" s="9" t="s">
+      <c r="F7" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G7" s="9">
+      <c r="G7" s="8">
         <v>12.0</v>
       </c>
-      <c r="H7" s="9">
+      <c r="H7" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I7" s="9" t="s">
+      <c r="I7" s="8" t="s">
         <v>44</v>
       </c>
       <c r="J7" s="14">
@@ -8268,7 +8268,7 @@
       <c r="K7" s="14">
         <v>949835.78</v>
       </c>
-      <c r="L7" s="9">
+      <c r="L7" s="8">
         <v>0.0</v>
       </c>
       <c r="AB7" s="2"/>
@@ -8280,32 +8280,32 @@
       <c r="AH7" s="2"/>
     </row>
     <row r="8">
-      <c r="A8" s="9" t="s">
+      <c r="A8" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="E8" s="12">
+        <v>45763.0</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="G8" s="8">
+        <v>12.0</v>
+      </c>
+      <c r="H8" s="8">
+        <v>339039.0</v>
+      </c>
+      <c r="I8" s="8" t="s">
         <v>48</v>
-      </c>
-      <c r="B8" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="C8" s="9" t="s">
-        <v>50</v>
-      </c>
-      <c r="D8" s="9" t="s">
-        <v>4</v>
-      </c>
-      <c r="E8" s="13">
-        <v>45763.0</v>
-      </c>
-      <c r="F8" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="G8" s="9">
-        <v>12.0</v>
-      </c>
-      <c r="H8" s="9">
-        <v>339039.0</v>
-      </c>
-      <c r="I8" s="9" t="s">
-        <v>51</v>
       </c>
       <c r="J8" s="14">
         <v>524584.95</v>
@@ -8313,10 +8313,10 @@
       <c r="K8" s="14">
         <v>524584.95</v>
       </c>
-      <c r="L8" s="9">
+      <c r="L8" s="8">
         <v>0.0</v>
       </c>
-      <c r="O8" s="30"/>
+      <c r="O8" s="28"/>
       <c r="AB8" s="2"/>
       <c r="AC8" s="2"/>
       <c r="AD8" s="2"/>
@@ -8326,32 +8326,32 @@
       <c r="AH8" s="2"/>
     </row>
     <row r="9">
-      <c r="A9" s="9" t="s">
-        <v>60</v>
-      </c>
-      <c r="B9" s="9" t="s">
-        <v>61</v>
-      </c>
-      <c r="C9" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="D9" s="9" t="s">
+      <c r="A9" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="D9" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E9" s="13">
+      <c r="E9" s="12">
         <v>45792.0</v>
       </c>
-      <c r="F9" s="9" t="s">
+      <c r="F9" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G9" s="9">
+      <c r="G9" s="8">
         <v>12.0</v>
       </c>
-      <c r="H9" s="9">
+      <c r="H9" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I9" s="9" t="s">
-        <v>64</v>
+      <c r="I9" s="8" t="s">
+        <v>56</v>
       </c>
       <c r="J9" s="14">
         <v>211614.23</v>
@@ -8359,7 +8359,7 @@
       <c r="K9" s="14">
         <v>211614.23</v>
       </c>
-      <c r="L9" s="9">
+      <c r="L9" s="8">
         <v>0.0</v>
       </c>
       <c r="AB9" s="2"/>
@@ -8371,31 +8371,31 @@
       <c r="AH9" s="2"/>
     </row>
     <row r="10">
-      <c r="A10" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="B10" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="C10" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="D10" s="9" t="s">
+      <c r="A10" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="D10" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E10" s="13">
+      <c r="E10" s="12">
         <v>45825.0</v>
       </c>
-      <c r="F10" s="9" t="s">
+      <c r="F10" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G10" s="9">
+      <c r="G10" s="8">
         <v>12.0</v>
       </c>
-      <c r="H10" s="9">
+      <c r="H10" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I10" s="9">
+      <c r="I10" s="8">
         <v>2048.0</v>
       </c>
       <c r="J10" s="14">
@@ -8416,31 +8416,31 @@
       <c r="AH10" s="2"/>
     </row>
     <row r="11">
-      <c r="A11" s="9" t="s">
-        <v>69</v>
-      </c>
-      <c r="B11" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="C11" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="D11" s="9" t="s">
+      <c r="A11" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="D11" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E11" s="13">
+      <c r="E11" s="12">
         <v>45825.0</v>
       </c>
-      <c r="F11" s="9" t="s">
+      <c r="F11" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G11" s="9">
+      <c r="G11" s="8">
         <v>12.0</v>
       </c>
-      <c r="H11" s="9">
+      <c r="H11" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I11" s="9">
+      <c r="I11" s="8">
         <v>2048.0</v>
       </c>
       <c r="J11" s="14">
@@ -8449,7 +8449,7 @@
       <c r="K11" s="14">
         <v>618154.38</v>
       </c>
-      <c r="L11" s="9">
+      <c r="L11" s="8">
         <v>0.01</v>
       </c>
       <c r="AB11" s="2"/>
@@ -8461,31 +8461,31 @@
       <c r="AH11" s="2"/>
     </row>
     <row r="12">
-      <c r="A12" s="9" t="s">
+      <c r="A12" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="B12" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="B12" s="9" t="s">
+      <c r="C12" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="C12" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="D12" s="9" t="s">
+      <c r="D12" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E12" s="13">
+      <c r="E12" s="12">
         <v>45832.0</v>
       </c>
-      <c r="F12" s="9" t="s">
+      <c r="F12" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G12" s="9">
+      <c r="G12" s="8">
         <v>12.0</v>
       </c>
-      <c r="H12" s="9">
+      <c r="H12" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I12" s="9" t="s">
+      <c r="I12" s="8" t="s">
         <v>75</v>
       </c>
       <c r="J12" s="14">
@@ -8494,7 +8494,7 @@
       <c r="K12" s="14">
         <v>1600334.09</v>
       </c>
-      <c r="L12" s="9">
+      <c r="L12" s="8">
         <v>0.0</v>
       </c>
       <c r="AB12" s="2"/>
@@ -8506,31 +8506,31 @@
       <c r="AH12" s="2"/>
     </row>
     <row r="13">
-      <c r="A13" s="9" t="s">
+      <c r="A13" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="B13" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="C13" s="9" t="s">
+      <c r="B13" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="C13" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="D13" s="9" t="s">
+      <c r="D13" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E13" s="13">
+      <c r="E13" s="12">
         <v>45863.0</v>
       </c>
-      <c r="F13" s="9" t="s">
+      <c r="F13" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G13" s="9">
+      <c r="G13" s="8">
         <v>12.0</v>
       </c>
-      <c r="H13" s="9">
+      <c r="H13" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I13" s="9">
+      <c r="I13" s="8">
         <v>2048.0</v>
       </c>
       <c r="J13" s="14">
@@ -8542,7 +8542,7 @@
       <c r="L13" s="14">
         <v>0.0</v>
       </c>
-      <c r="M13" s="39"/>
+      <c r="M13" s="38"/>
       <c r="AB13" s="2"/>
       <c r="AC13" s="2"/>
       <c r="AD13" s="2"/>
@@ -8552,32 +8552,32 @@
       <c r="AH13" s="2"/>
     </row>
     <row r="14">
-      <c r="A14" s="9" t="s">
+      <c r="A14" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="B14" s="9" t="s">
+      <c r="B14" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="C14" s="9" t="s">
+      <c r="C14" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="D14" s="9" t="s">
+      <c r="D14" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E14" s="13">
+      <c r="E14" s="12">
         <v>45887.0</v>
       </c>
-      <c r="F14" s="9" t="s">
+      <c r="F14" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G14" s="9">
+      <c r="G14" s="8">
         <v>12.0</v>
       </c>
-      <c r="H14" s="9">
+      <c r="H14" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I14" s="9" t="s">
-        <v>64</v>
+      <c r="I14" s="8" t="s">
+        <v>56</v>
       </c>
       <c r="J14" s="14">
         <v>968237.39</v>
@@ -8585,7 +8585,7 @@
       <c r="K14" s="14">
         <v>968237.39</v>
       </c>
-      <c r="L14" s="9">
+      <c r="L14" s="8">
         <v>0.0</v>
       </c>
       <c r="AB14" s="2"/>
@@ -8597,31 +8597,31 @@
       <c r="AH14" s="2"/>
     </row>
     <row r="15">
-      <c r="A15" s="9" t="s">
+      <c r="A15" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="B15" s="9" t="s">
+      <c r="B15" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="C15" s="9" t="s">
+      <c r="C15" s="8" t="s">
         <v>85</v>
       </c>
-      <c r="D15" s="9" t="s">
+      <c r="D15" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E15" s="13">
+      <c r="E15" s="12">
         <v>45924.0</v>
       </c>
-      <c r="F15" s="9" t="s">
+      <c r="F15" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G15" s="9">
+      <c r="G15" s="8">
         <v>12.0</v>
       </c>
-      <c r="H15" s="9">
+      <c r="H15" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I15" s="9" t="s">
+      <c r="I15" s="8" t="s">
         <v>44</v>
       </c>
       <c r="J15" s="14">
@@ -8630,7 +8630,7 @@
       <c r="K15" s="14">
         <v>1011677.95</v>
       </c>
-      <c r="L15" s="9">
+      <c r="L15" s="8">
         <v>0.0</v>
       </c>
       <c r="AB15" s="2"/>
@@ -8642,31 +8642,31 @@
       <c r="AH15" s="2"/>
     </row>
     <row r="16">
-      <c r="A16" s="9" t="s">
+      <c r="A16" s="8" t="s">
         <v>88</v>
       </c>
-      <c r="B16" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="C16" s="9" t="s">
+      <c r="B16" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="C16" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="D16" s="9" t="s">
+      <c r="D16" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E16" s="13">
+      <c r="E16" s="12">
         <v>45929.0</v>
       </c>
-      <c r="F16" s="9" t="s">
+      <c r="F16" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G16" s="9">
+      <c r="G16" s="8">
         <v>12.0</v>
       </c>
-      <c r="H16" s="9">
+      <c r="H16" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I16" s="9">
+      <c r="I16" s="8">
         <v>2048.0</v>
       </c>
       <c r="J16" s="14">
@@ -8687,37 +8687,37 @@
       <c r="AH16" s="2"/>
     </row>
     <row r="17">
-      <c r="A17" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="B17" s="9" t="s">
-        <v>91</v>
-      </c>
-      <c r="C17" s="9" t="s">
+      <c r="A17" s="8" t="s">
         <v>92</v>
       </c>
-      <c r="D17" s="9" t="s">
+      <c r="B17" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="C17" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="D17" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E17" s="13">
+      <c r="E17" s="12">
         <v>45930.0</v>
       </c>
-      <c r="F17" s="9" t="s">
+      <c r="F17" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G17" s="9">
+      <c r="G17" s="8">
         <v>12.0</v>
       </c>
-      <c r="H17" s="9">
+      <c r="H17" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I17" s="9">
+      <c r="I17" s="8">
         <v>2048.0</v>
       </c>
       <c r="J17" s="14">
         <v>34065.36</v>
       </c>
-      <c r="K17" s="9">
+      <c r="K17" s="8">
         <v>0.0</v>
       </c>
       <c r="L17" s="14">
@@ -8732,32 +8732,32 @@
       <c r="AH17" s="2"/>
     </row>
     <row r="18">
-      <c r="A18" s="9" t="s">
-        <v>95</v>
-      </c>
-      <c r="B18" s="9" t="s">
+      <c r="A18" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="B18" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="C18" s="9" t="s">
-        <v>96</v>
-      </c>
-      <c r="D18" s="9" t="s">
+      <c r="C18" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="D18" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E18" s="13">
+      <c r="E18" s="12">
         <v>45938.0</v>
       </c>
-      <c r="F18" s="9" t="s">
+      <c r="F18" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G18" s="9">
+      <c r="G18" s="8">
         <v>12.0</v>
       </c>
-      <c r="H18" s="9">
+      <c r="H18" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I18" s="9" t="s">
-        <v>64</v>
+      <c r="I18" s="8" t="s">
+        <v>56</v>
       </c>
       <c r="J18" s="14">
         <v>63746.85</v>
@@ -8765,7 +8765,7 @@
       <c r="K18" s="14">
         <v>63746.85</v>
       </c>
-      <c r="L18" s="9">
+      <c r="L18" s="8">
         <v>0.0</v>
       </c>
       <c r="AB18" s="2"/>
@@ -8777,31 +8777,31 @@
       <c r="AH18" s="2"/>
     </row>
     <row r="19">
-      <c r="A19" s="9" t="s">
+      <c r="A19" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="B19" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="C19" s="9" t="s">
+      <c r="B19" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="C19" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="D19" s="9" t="s">
+      <c r="D19" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E19" s="13">
+      <c r="E19" s="12">
         <v>45938.0</v>
       </c>
-      <c r="F19" s="9" t="s">
+      <c r="F19" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G19" s="9">
+      <c r="G19" s="8">
         <v>12.0</v>
       </c>
-      <c r="H19" s="9">
+      <c r="H19" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I19" s="9" t="s">
+      <c r="I19" s="8" t="s">
         <v>75</v>
       </c>
       <c r="J19" s="14">
@@ -8810,7 +8810,7 @@
       <c r="K19" s="14">
         <v>947931.1</v>
       </c>
-      <c r="L19" s="9">
+      <c r="L19" s="8">
         <v>0.0</v>
       </c>
       <c r="AB19" s="2"/>
@@ -8822,31 +8822,31 @@
       <c r="AH19" s="2"/>
     </row>
     <row r="20">
-      <c r="A20" s="9" t="s">
-        <v>101</v>
-      </c>
-      <c r="B20" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="C20" s="9" t="s">
+      <c r="A20" s="8" t="s">
         <v>102</v>
       </c>
-      <c r="D20" s="9" t="s">
+      <c r="B20" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="C20" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="D20" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E20" s="13">
+      <c r="E20" s="12">
         <v>45938.0</v>
       </c>
-      <c r="F20" s="9" t="s">
+      <c r="F20" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G20" s="9">
+      <c r="G20" s="8">
         <v>12.0</v>
       </c>
-      <c r="H20" s="9">
+      <c r="H20" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I20" s="9">
+      <c r="I20" s="8">
         <v>2048.0</v>
       </c>
       <c r="J20" s="14">
@@ -8855,7 +8855,7 @@
       <c r="K20" s="14">
         <v>259790.57</v>
       </c>
-      <c r="L20" s="9">
+      <c r="L20" s="8">
         <v>0.0</v>
       </c>
       <c r="AB20" s="2"/>
@@ -8867,31 +8867,31 @@
       <c r="AH20" s="2"/>
     </row>
     <row r="21">
-      <c r="A21" s="9" t="s">
-        <v>103</v>
-      </c>
-      <c r="B21" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="C21" s="9" t="s">
-        <v>105</v>
-      </c>
-      <c r="D21" s="9" t="s">
+      <c r="A21" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="B21" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C21" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="D21" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E21" s="13">
+      <c r="E21" s="12">
         <v>45938.0</v>
       </c>
-      <c r="F21" s="9" t="s">
+      <c r="F21" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G21" s="9">
+      <c r="G21" s="8">
         <v>12.0</v>
       </c>
-      <c r="H21" s="9">
+      <c r="H21" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I21" s="9">
+      <c r="I21" s="8">
         <v>2048.0</v>
       </c>
       <c r="J21" s="14">
@@ -8900,7 +8900,7 @@
       <c r="K21" s="14">
         <v>170479.3</v>
       </c>
-      <c r="L21" s="9">
+      <c r="L21" s="8">
         <v>0.0</v>
       </c>
       <c r="AB21" s="2"/>
@@ -8912,31 +8912,31 @@
       <c r="AH21" s="2"/>
     </row>
     <row r="22">
-      <c r="A22" s="9" t="s">
-        <v>106</v>
-      </c>
-      <c r="B22" s="9" t="s">
-        <v>107</v>
-      </c>
-      <c r="C22" s="9" t="s">
-        <v>108</v>
-      </c>
-      <c r="D22" s="9" t="s">
+      <c r="A22" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="B22" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="C22" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="D22" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E22" s="48">
+      <c r="E22" s="50">
         <v>45953.0</v>
       </c>
-      <c r="F22" s="9" t="s">
+      <c r="F22" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G22" s="9">
+      <c r="G22" s="8">
         <v>12.0</v>
       </c>
-      <c r="H22" s="9">
+      <c r="H22" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I22" s="9">
+      <c r="I22" s="8">
         <v>2000.0</v>
       </c>
       <c r="J22" s="14">
@@ -8957,32 +8957,32 @@
       <c r="AH22" s="2"/>
     </row>
     <row r="23">
-      <c r="A23" s="9" t="s">
-        <v>110</v>
-      </c>
-      <c r="B23" s="9" t="s">
-        <v>111</v>
-      </c>
-      <c r="C23" s="9" t="s">
-        <v>112</v>
-      </c>
-      <c r="D23" s="9" t="s">
+      <c r="A23" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="B23" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="C23" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="D23" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E23" s="48">
+      <c r="E23" s="50">
         <v>45953.0</v>
       </c>
-      <c r="F23" s="9" t="s">
+      <c r="F23" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G23" s="9">
+      <c r="G23" s="8">
         <v>12.0</v>
       </c>
-      <c r="H23" s="9">
+      <c r="H23" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I23" s="9" t="s">
-        <v>114</v>
+      <c r="I23" s="8" t="s">
+        <v>119</v>
       </c>
       <c r="J23" s="14">
         <v>1000001.64</v>
@@ -8990,7 +8990,7 @@
       <c r="K23" s="14">
         <v>1000001.64</v>
       </c>
-      <c r="L23" s="9">
+      <c r="L23" s="8">
         <v>0.0</v>
       </c>
       <c r="AB23" s="2"/>
@@ -9002,31 +9002,31 @@
       <c r="AH23" s="2"/>
     </row>
     <row r="24">
-      <c r="A24" s="9" t="s">
-        <v>116</v>
-      </c>
-      <c r="B24" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="C24" s="9" t="s">
-        <v>117</v>
-      </c>
-      <c r="D24" s="9" t="s">
+      <c r="A24" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="B24" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C24" s="8" t="s">
+        <v>122</v>
+      </c>
+      <c r="D24" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E24" s="48">
+      <c r="E24" s="50">
         <v>45953.0</v>
       </c>
-      <c r="F24" s="9" t="s">
+      <c r="F24" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G24" s="9">
+      <c r="G24" s="8">
         <v>12.0</v>
       </c>
-      <c r="H24" s="9">
+      <c r="H24" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I24" s="9">
+      <c r="I24" s="8">
         <v>2048.0</v>
       </c>
       <c r="J24" s="14">
@@ -9035,7 +9035,7 @@
       <c r="K24" s="14">
         <v>68405.66</v>
       </c>
-      <c r="L24" s="9">
+      <c r="L24" s="8">
         <v>0.0</v>
       </c>
       <c r="AB24" s="2"/>
@@ -9047,32 +9047,32 @@
       <c r="AH24" s="2"/>
     </row>
     <row r="25">
-      <c r="A25" s="9" t="s">
+      <c r="A25" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="B25" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="C25" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="D25" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="E25" s="50">
+        <v>45975.0</v>
+      </c>
+      <c r="F25" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="G25" s="8">
+        <v>12.0</v>
+      </c>
+      <c r="H25" s="8">
+        <v>339039.0</v>
+      </c>
+      <c r="I25" s="8" t="s">
         <v>119</v>
-      </c>
-      <c r="B25" s="9" t="s">
-        <v>120</v>
-      </c>
-      <c r="C25" s="9" t="s">
-        <v>122</v>
-      </c>
-      <c r="D25" s="9" t="s">
-        <v>4</v>
-      </c>
-      <c r="E25" s="48">
-        <v>45975.0</v>
-      </c>
-      <c r="F25" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="G25" s="9">
-        <v>12.0</v>
-      </c>
-      <c r="H25" s="9">
-        <v>339039.0</v>
-      </c>
-      <c r="I25" s="9" t="s">
-        <v>114</v>
       </c>
       <c r="J25" s="14">
         <v>1157673.06</v>
@@ -9080,7 +9080,7 @@
       <c r="K25" s="14">
         <v>1157673.06</v>
       </c>
-      <c r="L25" s="9">
+      <c r="L25" s="8">
         <v>0.0</v>
       </c>
       <c r="AB25" s="2"/>
@@ -9092,31 +9092,31 @@
       <c r="AH25" s="2"/>
     </row>
     <row r="26">
-      <c r="A26" s="9" t="s">
-        <v>124</v>
-      </c>
-      <c r="B26" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="C26" s="9" t="s">
-        <v>125</v>
-      </c>
-      <c r="D26" s="9" t="s">
+      <c r="A26" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="B26" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="C26" s="8" t="s">
+        <v>131</v>
+      </c>
+      <c r="D26" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E26" s="48">
+      <c r="E26" s="50">
         <v>45989.0</v>
       </c>
-      <c r="F26" s="9" t="s">
+      <c r="F26" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G26" s="9">
+      <c r="G26" s="8">
         <v>12.0</v>
       </c>
-      <c r="H26" s="9">
+      <c r="H26" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I26" s="9">
+      <c r="I26" s="8">
         <v>2048.0</v>
       </c>
       <c r="J26" s="14">
@@ -9125,7 +9125,7 @@
       <c r="K26" s="14">
         <v>34065.36</v>
       </c>
-      <c r="L26" s="9">
+      <c r="L26" s="8">
         <v>0.0</v>
       </c>
       <c r="AB26" s="2"/>
@@ -9137,31 +9137,31 @@
       <c r="AH26" s="2"/>
     </row>
     <row r="27">
-      <c r="A27" s="9" t="s">
-        <v>127</v>
-      </c>
-      <c r="B27" s="9" t="s">
-        <v>128</v>
-      </c>
-      <c r="C27" s="9" t="s">
-        <v>130</v>
-      </c>
-      <c r="D27" s="9" t="s">
+      <c r="A27" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="B27" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="C27" s="8" t="s">
+        <v>136</v>
+      </c>
+      <c r="D27" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E27" s="13">
+      <c r="E27" s="12">
         <v>46104.0</v>
       </c>
-      <c r="F27" s="9" t="s">
+      <c r="F27" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G27" s="9">
+      <c r="G27" s="8">
         <v>12.0</v>
       </c>
-      <c r="H27" s="9">
+      <c r="H27" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I27" s="9">
+      <c r="I27" s="8">
         <v>2048.0</v>
       </c>
       <c r="J27" s="14">
@@ -9182,37 +9182,37 @@
       <c r="AH27" s="2"/>
     </row>
     <row r="28">
-      <c r="A28" s="9" t="s">
-        <v>133</v>
-      </c>
-      <c r="B28" s="9" t="s">
-        <v>134</v>
-      </c>
-      <c r="C28" s="9" t="s">
-        <v>135</v>
-      </c>
-      <c r="D28" s="9" t="s">
+      <c r="A28" s="8" t="s">
+        <v>140</v>
+      </c>
+      <c r="B28" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="C28" s="8" t="s">
+        <v>142</v>
+      </c>
+      <c r="D28" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E28" s="13">
+      <c r="E28" s="12">
         <v>46120.0</v>
       </c>
-      <c r="F28" s="9" t="s">
+      <c r="F28" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G28" s="9">
+      <c r="G28" s="8">
         <v>12.0</v>
       </c>
-      <c r="H28" s="9">
+      <c r="H28" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I28" s="9" t="s">
-        <v>51</v>
+      <c r="I28" s="8" t="s">
+        <v>48</v>
       </c>
       <c r="J28" s="14">
         <v>1912292.52</v>
       </c>
-      <c r="K28" s="9">
+      <c r="K28" s="8">
         <v>0.0</v>
       </c>
       <c r="L28" s="14">
@@ -9227,37 +9227,37 @@
       <c r="AH28" s="2"/>
     </row>
     <row r="29">
-      <c r="A29" s="9" t="s">
-        <v>139</v>
-      </c>
-      <c r="B29" s="9" t="s">
-        <v>140</v>
-      </c>
-      <c r="C29" s="9" t="s">
-        <v>141</v>
-      </c>
-      <c r="D29" s="9" t="s">
+      <c r="A29" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="B29" s="8" t="s">
+        <v>146</v>
+      </c>
+      <c r="C29" s="8" t="s">
+        <v>147</v>
+      </c>
+      <c r="D29" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E29" s="13">
+      <c r="E29" s="12">
         <v>46196.0</v>
       </c>
-      <c r="F29" s="9" t="s">
+      <c r="F29" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G29" s="9">
+      <c r="G29" s="8">
         <v>12.0</v>
       </c>
-      <c r="H29" s="9">
+      <c r="H29" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I29" s="9">
+      <c r="I29" s="8">
         <v>2048.0</v>
       </c>
       <c r="J29" s="14">
         <v>1496713.48</v>
       </c>
-      <c r="K29" s="9">
+      <c r="K29" s="8">
         <v>0.0</v>
       </c>
       <c r="L29" s="14">
@@ -9272,37 +9272,37 @@
       <c r="AH29" s="2"/>
     </row>
     <row r="30">
-      <c r="A30" s="9" t="s">
-        <v>143</v>
-      </c>
-      <c r="B30" s="9" t="s">
-        <v>144</v>
-      </c>
-      <c r="C30" s="9" t="s">
-        <v>145</v>
-      </c>
-      <c r="D30" s="9" t="s">
+      <c r="A30" s="8" t="s">
+        <v>150</v>
+      </c>
+      <c r="B30" s="8" t="s">
+        <v>151</v>
+      </c>
+      <c r="C30" s="8" t="s">
+        <v>152</v>
+      </c>
+      <c r="D30" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E30" s="13">
+      <c r="E30" s="12">
         <v>46205.0</v>
       </c>
-      <c r="F30" s="9" t="s">
+      <c r="F30" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G30" s="9">
+      <c r="G30" s="8">
         <v>12.0</v>
       </c>
-      <c r="H30" s="9">
+      <c r="H30" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I30" s="9" t="s">
+      <c r="I30" s="8" t="s">
         <v>44</v>
       </c>
       <c r="J30" s="14">
         <v>624166.14</v>
       </c>
-      <c r="K30" s="9">
+      <c r="K30" s="8">
         <v>0.0</v>
       </c>
       <c r="L30" s="14">
@@ -9317,37 +9317,37 @@
       <c r="AH30" s="2"/>
     </row>
     <row r="31">
-      <c r="A31" s="9" t="s">
-        <v>147</v>
-      </c>
-      <c r="B31" s="9" t="s">
-        <v>148</v>
-      </c>
-      <c r="C31" s="9" t="s">
-        <v>149</v>
-      </c>
-      <c r="D31" s="9" t="s">
+      <c r="A31" s="8" t="s">
+        <v>154</v>
+      </c>
+      <c r="B31" s="8" t="s">
+        <v>155</v>
+      </c>
+      <c r="C31" s="8" t="s">
+        <v>156</v>
+      </c>
+      <c r="D31" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E31" s="13">
+      <c r="E31" s="12">
         <v>46205.0</v>
       </c>
-      <c r="F31" s="9" t="s">
+      <c r="F31" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G31" s="9">
+      <c r="G31" s="8">
         <v>12.0</v>
       </c>
-      <c r="H31" s="9">
+      <c r="H31" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I31" s="9" t="s">
-        <v>114</v>
+      <c r="I31" s="8" t="s">
+        <v>119</v>
       </c>
       <c r="J31" s="14">
         <v>18462.36</v>
       </c>
-      <c r="K31" s="9">
+      <c r="K31" s="8">
         <v>0.0</v>
       </c>
       <c r="L31" s="14">
@@ -9362,37 +9362,37 @@
       <c r="AH31" s="2"/>
     </row>
     <row r="32">
-      <c r="A32" s="9" t="s">
-        <v>152</v>
-      </c>
-      <c r="B32" s="9" t="s">
-        <v>148</v>
+      <c r="A32" s="8" t="s">
+        <v>160</v>
+      </c>
+      <c r="B32" s="8" t="s">
+        <v>155</v>
       </c>
       <c r="C32" s="14" t="s">
-        <v>153</v>
-      </c>
-      <c r="D32" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="D32" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E32" s="13">
+      <c r="E32" s="12">
         <v>46213.0</v>
       </c>
-      <c r="F32" s="9" t="s">
+      <c r="F32" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G32" s="9">
+      <c r="G32" s="8">
         <v>12.0</v>
       </c>
-      <c r="H32" s="9">
+      <c r="H32" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I32" s="9" t="s">
-        <v>114</v>
+      <c r="I32" s="8" t="s">
+        <v>119</v>
       </c>
       <c r="J32" s="14">
         <v>1530656.62</v>
       </c>
-      <c r="K32" s="9">
+      <c r="K32" s="8">
         <v>0.0</v>
       </c>
       <c r="L32" s="14">
@@ -9407,37 +9407,37 @@
       <c r="AH32" s="2"/>
     </row>
     <row r="33">
-      <c r="A33" s="9" t="s">
-        <v>155</v>
-      </c>
-      <c r="B33" s="9" t="s">
-        <v>140</v>
+      <c r="A33" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="B33" s="8" t="s">
+        <v>146</v>
       </c>
       <c r="C33" s="14" t="s">
-        <v>156</v>
-      </c>
-      <c r="D33" s="9" t="s">
+        <v>167</v>
+      </c>
+      <c r="D33" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E33" s="13">
+      <c r="E33" s="12">
         <v>46227.0</v>
       </c>
-      <c r="F33" s="9" t="s">
+      <c r="F33" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G33" s="9">
+      <c r="G33" s="8">
         <v>12.0</v>
       </c>
-      <c r="H33" s="9">
+      <c r="H33" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I33" s="9">
+      <c r="I33" s="8">
         <v>2048.0</v>
       </c>
       <c r="J33" s="14">
         <v>173846.38</v>
       </c>
-      <c r="K33" s="9">
+      <c r="K33" s="8">
         <v>0.0</v>
       </c>
       <c r="L33" s="14">
@@ -9452,37 +9452,37 @@
       <c r="AH33" s="2"/>
     </row>
     <row r="34">
-      <c r="A34" s="9" t="s">
-        <v>159</v>
-      </c>
-      <c r="B34" s="9" t="s">
-        <v>160</v>
-      </c>
-      <c r="C34" s="9" t="s">
-        <v>161</v>
-      </c>
-      <c r="D34" s="9" t="s">
+      <c r="A34" s="8" t="s">
+        <v>170</v>
+      </c>
+      <c r="B34" s="8" t="s">
+        <v>171</v>
+      </c>
+      <c r="C34" s="8" t="s">
+        <v>172</v>
+      </c>
+      <c r="D34" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E34" s="13">
+      <c r="E34" s="12">
         <v>46240.0</v>
       </c>
-      <c r="F34" s="9" t="s">
+      <c r="F34" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G34" s="9">
+      <c r="G34" s="8">
         <v>12.0</v>
       </c>
-      <c r="H34" s="9">
+      <c r="H34" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I34" s="9" t="s">
-        <v>162</v>
+      <c r="I34" s="8" t="s">
+        <v>173</v>
       </c>
       <c r="J34" s="14">
         <v>236343.68</v>
       </c>
-      <c r="K34" s="9">
+      <c r="K34" s="8">
         <v>0.0</v>
       </c>
       <c r="L34" s="14">

</xml_diff>

<commit_message>
Atualização automática: pagamentos (21/08/2026 20:32)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/01_Bases_Originais/005_CELOG_2025/005_CELOG-PAMALS_2025 online.xlsx
+++ b/Contrato 005/Dashboard/01_Bases_Originais/005_CELOG_2025/005_CELOG-PAMALS_2025 online.xlsx
@@ -30,12 +30,12 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="342" uniqueCount="217">
   <si>
+    <t>Controle de pagamentos</t>
+  </si>
+  <si>
     <t>Saldo</t>
   </si>
   <si>
-    <t>Controle de pagamentos</t>
-  </si>
-  <si>
     <t>2025NE000005</t>
   </si>
   <si>
@@ -60,27 +60,27 @@
     <t>Número Contrato</t>
   </si>
   <si>
+    <t>2025NE000369</t>
+  </si>
+  <si>
     <t>UG Executora</t>
   </si>
   <si>
+    <t>C25516</t>
+  </si>
+  <si>
     <t>UG Responsável</t>
   </si>
   <si>
-    <t>2025NE000369</t>
+    <t>25E0387</t>
   </si>
   <si>
     <t>UG Fiscalizadora</t>
   </si>
   <si>
-    <t>C25516</t>
-  </si>
-  <si>
     <t>Prazo Final de Execução</t>
   </si>
   <si>
-    <t>25E0387</t>
-  </si>
-  <si>
     <t>Prazo Final de Vigência</t>
   </si>
   <si>
@@ -102,12 +102,18 @@
     <t>Valor a Empenhar</t>
   </si>
   <si>
+    <t>2025NE000371</t>
+  </si>
+  <si>
     <t>Valor Empenhado</t>
   </si>
   <si>
     <t>Valor Liquidado</t>
   </si>
   <si>
+    <t>25E0389</t>
+  </si>
+  <si>
     <t>Saldo (Valor a Faturar)</t>
   </si>
   <si>
@@ -123,21 +129,27 @@
     <t>Editar</t>
   </si>
   <si>
-    <t>2025NE000371</t>
-  </si>
-  <si>
-    <t>25E0389</t>
-  </si>
-  <si>
     <t>005/CELOG-PAMALS/2025</t>
   </si>
   <si>
+    <t>2025NE000413</t>
+  </si>
+  <si>
     <t>CELOG</t>
   </si>
   <si>
+    <t>C25501</t>
+  </si>
+  <si>
+    <t>25E0403</t>
+  </si>
+  <si>
     <t>PAMALS</t>
   </si>
   <si>
+    <t>20SP</t>
+  </si>
+  <si>
     <t>Vigente</t>
   </si>
   <si>
@@ -147,33 +159,21 @@
     <t>67101.001510/2024-12</t>
   </si>
   <si>
-    <t>2025NE000413</t>
-  </si>
-  <si>
-    <t>C25501</t>
-  </si>
-  <si>
-    <t>25E0403</t>
-  </si>
-  <si>
     <t>R$</t>
   </si>
   <si>
-    <t>20SP</t>
+    <t>2025NE000414</t>
+  </si>
+  <si>
+    <t>C25525</t>
+  </si>
+  <si>
+    <t>25E0431</t>
   </si>
   <si>
     <t>VEE ONE-MANUTENCAO E SERVICOS TECNICOS LTDA</t>
   </si>
   <si>
-    <t>2025NE000414</t>
-  </si>
-  <si>
-    <t>C25525</t>
-  </si>
-  <si>
-    <t>25E0431</t>
-  </si>
-  <si>
     <t>21EM</t>
   </si>
   <si>
@@ -192,10 +192,16 @@
     <t>2025NE000770</t>
   </si>
   <si>
+    <t>25E0731</t>
+  </si>
+  <si>
     <t>Módulo</t>
   </si>
   <si>
-    <t>25E0731</t>
+    <t>2025NE000774</t>
+  </si>
+  <si>
+    <t>25E0737</t>
   </si>
   <si>
     <t>Referência</t>
@@ -210,15 +216,9 @@
     <t>Data</t>
   </si>
   <si>
-    <t>2025NE000774</t>
-  </si>
-  <si>
     <t>Empenho</t>
   </si>
   <si>
-    <t>25E0737</t>
-  </si>
-  <si>
     <t>Observações</t>
   </si>
   <si>
@@ -228,21 +228,21 @@
     <t>Valor das Nfs</t>
   </si>
   <si>
+    <t>2025NE000843</t>
+  </si>
+  <si>
+    <t>C25630</t>
+  </si>
+  <si>
     <t>Ordem de Pagamento</t>
   </si>
   <si>
+    <t>25E0787</t>
+  </si>
+  <si>
     <t>Faturado</t>
   </si>
   <si>
-    <t>2025NE000843</t>
-  </si>
-  <si>
-    <t>C25630</t>
-  </si>
-  <si>
-    <t>25E0787</t>
-  </si>
-  <si>
     <t>Pendente</t>
   </si>
   <si>
@@ -291,6 +291,9 @@
     <t>25E1475</t>
   </si>
   <si>
+    <t>MAR/25</t>
+  </si>
+  <si>
     <t>2025NE001629</t>
   </si>
   <si>
@@ -300,7 +303,10 @@
     <t>25E1477</t>
   </si>
   <si>
-    <t>MAR/25</t>
+    <t>2025NE000367, 2025NE000369, 2025NE000371, 2025NE000413</t>
+  </si>
+  <si>
+    <t>2025NP001979</t>
   </si>
   <si>
     <t>2025NE001687</t>
@@ -312,13 +318,13 @@
     <t>2025NE001688</t>
   </si>
   <si>
-    <t>2025NE000367, 2025NE000369, 2025NE000371, 2025NE000413</t>
-  </si>
-  <si>
     <t>25E1536</t>
   </si>
   <si>
-    <t>2025NP001979</t>
+    <t>ABR/25</t>
+  </si>
+  <si>
+    <t>2025NE000413, 2025NE000414, 2025NE000559</t>
   </si>
   <si>
     <t>2025NE001689</t>
@@ -327,16 +333,19 @@
     <t>25E1537</t>
   </si>
   <si>
+    <t>2025NP002341</t>
+  </si>
+  <si>
+    <t>MAI/25</t>
+  </si>
+  <si>
     <t>2025NE001690</t>
   </si>
   <si>
     <t>25E1538</t>
   </si>
   <si>
-    <t>ABR/25</t>
-  </si>
-  <si>
-    <t>2025NE000413, 2025NE000414, 2025NE000559</t>
+    <t>2025NP002884</t>
   </si>
   <si>
     <t>2025NE001823</t>
@@ -346,48 +355,6 @@
   </si>
   <si>
     <t>25E1666</t>
-  </si>
-  <si>
-    <t>2025NP002341</t>
-  </si>
-  <si>
-    <t>2025NE001828</t>
-  </si>
-  <si>
-    <t>C25869</t>
-  </si>
-  <si>
-    <t>25E1667</t>
-  </si>
-  <si>
-    <t>20YJ</t>
-  </si>
-  <si>
-    <t>MAI/25</t>
-  </si>
-  <si>
-    <t>2025NE001830</t>
-  </si>
-  <si>
-    <t>25E1669</t>
-  </si>
-  <si>
-    <t>2025NP002884</t>
-  </si>
-  <si>
-    <t>2025NE002200</t>
-  </si>
-  <si>
-    <t>C25863</t>
-  </si>
-  <si>
-    <t>25E2021</t>
-  </si>
-  <si>
-    <t>2025NE002237</t>
-  </si>
-  <si>
-    <t>25E2058</t>
   </si>
   <si>
     <t>JUN/25</t>
@@ -399,37 +366,28 @@
 2025NE000774</t>
   </si>
   <si>
-    <t>2026NE000330</t>
-  </si>
-  <si>
-    <t>C26163</t>
-  </si>
-  <si>
-    <t>26E0320</t>
+    <t>2025NE001828</t>
+  </si>
+  <si>
+    <t>C25869</t>
+  </si>
+  <si>
+    <t>25E1667</t>
   </si>
   <si>
     <t>2025NP400522</t>
   </si>
   <si>
-    <t>2026NE000388</t>
-  </si>
-  <si>
-    <t>C26193</t>
-  </si>
-  <si>
-    <t>26E0375</t>
+    <t>20YJ</t>
   </si>
   <si>
     <t>JUL/25</t>
   </si>
   <si>
-    <t>2026NE000748</t>
-  </si>
-  <si>
-    <t>C26312</t>
-  </si>
-  <si>
-    <t>26E0709</t>
+    <t>2025NE001830</t>
+  </si>
+  <si>
+    <t>25E1669</t>
   </si>
   <si>
     <t>2025NE000843, 2025NE001200</t>
@@ -438,34 +396,25 @@
     <t>2025NP003724</t>
   </si>
   <si>
-    <t>2026NE000816</t>
-  </si>
-  <si>
-    <t>C26324</t>
-  </si>
-  <si>
-    <t>26E0776</t>
-  </si>
-  <si>
     <t>AGO/25</t>
   </si>
   <si>
-    <t>2026NE000817</t>
-  </si>
-  <si>
-    <t>C26326</t>
-  </si>
-  <si>
-    <t>26E0777</t>
+    <t>2025NE002200</t>
+  </si>
+  <si>
+    <t>C25863</t>
+  </si>
+  <si>
+    <t>25E2021</t>
   </si>
   <si>
     <t>2025NP004558</t>
   </si>
   <si>
-    <t>2026NE000842</t>
-  </si>
-  <si>
-    <t>26E0803</t>
+    <t>2025NE002237</t>
+  </si>
+  <si>
+    <t>25E2058</t>
   </si>
   <si>
     <t>SET/25</t>
@@ -475,16 +424,121 @@
 2025NE001828</t>
   </si>
   <si>
+    <t>2025NP004897</t>
+  </si>
+  <si>
+    <t>2026NE000330</t>
+  </si>
+  <si>
+    <t>C26163</t>
+  </si>
+  <si>
+    <t>26E0320</t>
+  </si>
+  <si>
+    <t>OUT/25</t>
+  </si>
+  <si>
+    <t>2025NE001688, 2025NE001828, 2025NE002200</t>
+  </si>
+  <si>
+    <t>2026NE000388</t>
+  </si>
+  <si>
+    <t>C26193</t>
+  </si>
+  <si>
+    <t>2025NP004932</t>
+  </si>
+  <si>
+    <t>26E0375</t>
+  </si>
+  <si>
+    <t>NOV/25</t>
+  </si>
+  <si>
+    <t>2025NE001687, 2025NE001689, 2025NE001690, 2025NE001823, 2025NE001830, 2025NE002237</t>
+  </si>
+  <si>
+    <t>2026NE000748</t>
+  </si>
+  <si>
+    <t>C26312</t>
+  </si>
+  <si>
+    <t>26E0709</t>
+  </si>
+  <si>
+    <t>2026NP400440</t>
+  </si>
+  <si>
+    <t>DEZ/25</t>
+  </si>
+  <si>
+    <t>2026NE000816</t>
+  </si>
+  <si>
+    <t>C26324</t>
+  </si>
+  <si>
+    <t>26E0776</t>
+  </si>
+  <si>
+    <t>2025NE001065, 2025NE002200</t>
+  </si>
+  <si>
+    <t>2026NP400412</t>
+  </si>
+  <si>
+    <t>2026NE000817</t>
+  </si>
+  <si>
+    <t>C26326</t>
+  </si>
+  <si>
+    <t>26E0777</t>
+  </si>
+  <si>
+    <t>JAN/26</t>
+  </si>
+  <si>
+    <t>2026NP401035</t>
+  </si>
+  <si>
+    <t>2026NE000842</t>
+  </si>
+  <si>
+    <t>FEV/26</t>
+  </si>
+  <si>
+    <t>26E0803</t>
+  </si>
+  <si>
+    <t>2025NE001627, 2025NE001629, 2025NE001823</t>
+  </si>
+  <si>
+    <t>2026NP402272</t>
+  </si>
+  <si>
+    <t>MAR/26</t>
+  </si>
+  <si>
     <t>2026NE000944</t>
   </si>
   <si>
     <t>26E0906</t>
   </si>
   <si>
-    <t>2025NP004897</t>
-  </si>
-  <si>
-    <t>OUT/25</t>
+    <t>2025NE000770, 2025NE001627</t>
+  </si>
+  <si>
+    <t>R$ 1.350.542,52</t>
+  </si>
+  <si>
+    <t>2026NP401762</t>
+  </si>
+  <si>
+    <t>ABR/26</t>
   </si>
   <si>
     <t>2026NE001015</t>
@@ -496,64 +550,10 @@
     <t>26E0959</t>
   </si>
   <si>
-    <t>2025NE001688, 2025NE001828, 2025NE002200</t>
+    <t>2025NE000770, 2025NE001065, 2025NE001627</t>
   </si>
   <si>
     <t>20XV</t>
-  </si>
-  <si>
-    <t>2025NP004932</t>
-  </si>
-  <si>
-    <t>NOV/25</t>
-  </si>
-  <si>
-    <t>2025NE001687, 2025NE001689, 2025NE001690, 2025NE001823, 2025NE001830, 2025NE002237</t>
-  </si>
-  <si>
-    <t>2026NP400440</t>
-  </si>
-  <si>
-    <t>DEZ/25</t>
-  </si>
-  <si>
-    <t>2025NE001065, 2025NE002200</t>
-  </si>
-  <si>
-    <t>2026NP400412</t>
-  </si>
-  <si>
-    <t>JAN/26</t>
-  </si>
-  <si>
-    <t>2026NP401035</t>
-  </si>
-  <si>
-    <t>FEV/26</t>
-  </si>
-  <si>
-    <t>2025NE001627, 2025NE001629, 2025NE001823</t>
-  </si>
-  <si>
-    <t>2026NP402272</t>
-  </si>
-  <si>
-    <t>MAR/26</t>
-  </si>
-  <si>
-    <t>2025NE000770, 2025NE001627</t>
-  </si>
-  <si>
-    <t>R$ 1.350.542,52</t>
-  </si>
-  <si>
-    <t>2026NP401762</t>
-  </si>
-  <si>
-    <t>ABR/26</t>
-  </si>
-  <si>
-    <t>2025NE000770, 2025NE001065, 2025NE001627</t>
   </si>
   <si>
     <t>REAJUSTE</t>
@@ -695,8 +695,8 @@
     <numFmt numFmtId="166" formatCode="dd/MM/yyyy"/>
     <numFmt numFmtId="167" formatCode="R$ #,##0.00"/>
     <numFmt numFmtId="168" formatCode="[$R$-416]\ #,##0.00;[RED]\-[$R$-416]\ #,##0.00"/>
-    <numFmt numFmtId="169" formatCode="d/m/yyyy"/>
-    <numFmt numFmtId="170" formatCode="MM/DD/YY"/>
+    <numFmt numFmtId="169" formatCode="MM/DD/YY"/>
+    <numFmt numFmtId="170" formatCode="d/m/yyyy"/>
     <numFmt numFmtId="171" formatCode="[$R$ -416]#,##0.00"/>
     <numFmt numFmtId="172" formatCode="_([$R$ -416]* #,##0.00_);_([$R$ -416]* \(#,##0.00\);_([$R$ -416]* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
@@ -732,15 +732,15 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="10.0"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-    </font>
-    <font>
       <b/>
       <sz val="10.0"/>
       <color theme="1"/>
       <name val="Century Gothic"/>
+    </font>
+    <font>
+      <sz val="10.0"/>
+      <color theme="1"/>
+      <name val="Arial"/>
     </font>
     <font>
       <b/>
@@ -892,26 +892,26 @@
     </xf>
     <xf borderId="0" fillId="3" fontId="2" numFmtId="0" xfId="0" applyFill="1" applyFont="1"/>
     <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyFill="1" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0"/>
-    </xf>
     <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="5" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
+      <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="11" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
@@ -947,22 +947,22 @@
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="0" fontId="5" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf borderId="0" fillId="2" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="6" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -980,7 +980,6 @@
     <xf borderId="1" fillId="0" fontId="7" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="165" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="1" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
@@ -990,6 +989,7 @@
     <xf borderId="1" fillId="0" fontId="8" numFmtId="166" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="165" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="1" fillId="7" fontId="9" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
@@ -1003,13 +1003,10 @@
     <xf borderId="1" fillId="8" fontId="9" numFmtId="168" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="169" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
     <xf borderId="1" fillId="0" fontId="8" numFmtId="166" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="8" numFmtId="170" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="8" numFmtId="169" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="7" fontId="9" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
@@ -1021,16 +1018,19 @@
     <xf borderId="1" fillId="8" fontId="9" numFmtId="168" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="170" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
     <xf borderId="1" fillId="0" fontId="7" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="9" fontId="9" numFmtId="168" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="4" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="4" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="9" fontId="9" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
@@ -1446,19 +1446,19 @@
       <c r="V1" s="3"/>
     </row>
     <row r="2" ht="59.25" customHeight="1">
-      <c r="A2" s="5"/>
-      <c r="B2" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="V2" s="9"/>
-      <c r="W2" s="10"/>
-      <c r="X2" s="10"/>
-      <c r="Y2" s="10"/>
-      <c r="Z2" s="10"/>
-      <c r="AA2" s="10"/>
-      <c r="AB2" s="10"/>
-      <c r="AC2" s="10"/>
-      <c r="AD2" s="10"/>
+      <c r="A2" s="4"/>
+      <c r="B2" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="V2" s="8"/>
+      <c r="W2" s="9"/>
+      <c r="X2" s="9"/>
+      <c r="Y2" s="9"/>
+      <c r="Z2" s="9"/>
+      <c r="AA2" s="9"/>
+      <c r="AB2" s="9"/>
+      <c r="AC2" s="9"/>
+      <c r="AD2" s="9"/>
     </row>
     <row r="3" ht="12.75" customHeight="1">
       <c r="A3" s="1"/>
@@ -1491,16 +1491,16 @@
         <v>9</v>
       </c>
       <c r="D4" s="16" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E4" s="16" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F4" s="16" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G4" s="17" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H4" s="17" t="s">
         <v>17</v>
@@ -1524,25 +1524,25 @@
         <v>23</v>
       </c>
       <c r="O4" s="17" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="P4" s="17" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="Q4" s="17" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="R4" s="16" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="S4" s="16" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="T4" s="16" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="U4" s="16" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="V4" s="3"/>
     </row>
@@ -1554,13 +1554,13 @@
         <v>33</v>
       </c>
       <c r="E5" s="19" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F5" s="19" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="G5" s="19" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="H5" s="20">
         <v>1564.0</v>
@@ -1569,16 +1569,16 @@
         <v>1564.0</v>
       </c>
       <c r="J5" s="19" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="K5" s="19" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="L5" s="19" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="M5" s="19" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="N5" s="21">
         <v>9.165159737E7</v>
@@ -1596,7 +1596,7 @@
         <v>1.085943044E7</v>
       </c>
       <c r="S5" s="19" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="V5" s="3"/>
     </row>
@@ -1607,8 +1607,8 @@
       <c r="V6" s="3"/>
     </row>
     <row r="7" ht="12.75" customHeight="1">
-      <c r="A7" s="23"/>
-      <c r="B7" s="23"/>
+      <c r="A7" s="24"/>
+      <c r="B7" s="24"/>
       <c r="C7" s="25"/>
       <c r="D7" s="26"/>
       <c r="E7" s="26"/>
@@ -1626,25 +1626,25 @@
       <c r="V7" s="3"/>
     </row>
     <row r="8" ht="12.75" customHeight="1">
-      <c r="A8" s="23"/>
-      <c r="B8" s="23"/>
+      <c r="A8" s="24"/>
+      <c r="B8" s="24"/>
       <c r="C8" s="29" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D8" s="29" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E8" s="30" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F8" s="29" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="G8" s="29" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="H8" s="29" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="I8" s="30" t="s">
         <v>63</v>
@@ -1656,10 +1656,10 @@
         <v>65</v>
       </c>
       <c r="L8" s="31" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="M8" s="30" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="N8" s="29" t="s">
         <v>71</v>
@@ -1669,34 +1669,34 @@
       <c r="V8" s="3"/>
     </row>
     <row r="9" ht="19.5" customHeight="1">
-      <c r="A9" s="23"/>
-      <c r="B9" s="23"/>
+      <c r="A9" s="24"/>
+      <c r="B9" s="24"/>
       <c r="C9" s="32">
         <v>1.0</v>
       </c>
       <c r="D9" s="33" t="s">
         <v>75</v>
       </c>
-      <c r="E9" s="35" t="s">
+      <c r="E9" s="34" t="s">
         <v>76</v>
       </c>
-      <c r="F9" s="36">
+      <c r="F9" s="35">
         <v>594.0</v>
       </c>
-      <c r="G9" s="37">
+      <c r="G9" s="36">
         <v>45740.0</v>
       </c>
-      <c r="H9" s="36" t="s">
+      <c r="H9" s="35" t="s">
         <v>77</v>
       </c>
-      <c r="I9" s="37"/>
-      <c r="J9" s="37">
+      <c r="I9" s="36"/>
+      <c r="J9" s="36">
         <v>45778.0</v>
       </c>
       <c r="K9" s="38">
         <v>748504.24</v>
       </c>
-      <c r="L9" s="36" t="s">
+      <c r="L9" s="35" t="s">
         <v>81</v>
       </c>
       <c r="M9" s="39">
@@ -1709,33 +1709,33 @@
       <c r="V9" s="3"/>
     </row>
     <row r="10" ht="51.0" customHeight="1">
-      <c r="A10" s="23"/>
-      <c r="B10" s="23"/>
+      <c r="A10" s="24"/>
+      <c r="B10" s="24"/>
       <c r="C10" s="41"/>
       <c r="D10" s="33" t="s">
-        <v>90</v>
-      </c>
-      <c r="E10" s="35" t="s">
+        <v>87</v>
+      </c>
+      <c r="E10" s="34" t="s">
         <v>76</v>
       </c>
-      <c r="F10" s="36">
+      <c r="F10" s="35">
         <v>620.0</v>
       </c>
-      <c r="G10" s="37">
+      <c r="G10" s="36">
         <v>45775.0</v>
       </c>
-      <c r="H10" s="36" t="s">
-        <v>94</v>
-      </c>
-      <c r="I10" s="37"/>
-      <c r="J10" s="37">
+      <c r="H10" s="35" t="s">
+        <v>91</v>
+      </c>
+      <c r="I10" s="36"/>
+      <c r="J10" s="36">
         <v>45806.0</v>
       </c>
       <c r="K10" s="38">
         <v>1110378.24</v>
       </c>
-      <c r="L10" s="36" t="s">
-        <v>96</v>
+      <c r="L10" s="35" t="s">
+        <v>92</v>
       </c>
       <c r="M10" s="39">
         <f t="shared" si="1"/>
@@ -1747,33 +1747,33 @@
       <c r="V10" s="3"/>
     </row>
     <row r="11" ht="12.75" customHeight="1">
-      <c r="A11" s="23"/>
-      <c r="B11" s="23"/>
+      <c r="A11" s="24"/>
+      <c r="B11" s="24"/>
       <c r="C11" s="41"/>
       <c r="D11" s="33" t="s">
-        <v>101</v>
-      </c>
-      <c r="E11" s="35" t="s">
+        <v>97</v>
+      </c>
+      <c r="E11" s="34" t="s">
         <v>76</v>
       </c>
-      <c r="F11" s="36">
+      <c r="F11" s="35">
         <v>634.0</v>
       </c>
-      <c r="G11" s="37">
+      <c r="G11" s="36">
         <v>45799.0</v>
       </c>
-      <c r="H11" s="36" t="s">
-        <v>102</v>
-      </c>
-      <c r="I11" s="37"/>
-      <c r="J11" s="37">
+      <c r="H11" s="35" t="s">
+        <v>98</v>
+      </c>
+      <c r="I11" s="36"/>
+      <c r="J11" s="36">
         <v>45844.0</v>
       </c>
       <c r="K11" s="38">
         <v>974557.12</v>
       </c>
-      <c r="L11" s="35" t="s">
-        <v>106</v>
+      <c r="L11" s="34" t="s">
+        <v>101</v>
       </c>
       <c r="M11" s="39">
         <v>974557.12</v>
@@ -1784,107 +1784,107 @@
       <c r="V11" s="3"/>
     </row>
     <row r="12" ht="27.75" customHeight="1">
-      <c r="A12" s="23"/>
-      <c r="B12" s="23"/>
+      <c r="A12" s="24"/>
+      <c r="B12" s="24"/>
       <c r="C12" s="41"/>
       <c r="D12" s="33" t="s">
-        <v>111</v>
-      </c>
-      <c r="E12" s="35" t="s">
+        <v>102</v>
+      </c>
+      <c r="E12" s="34" t="s">
         <v>76</v>
       </c>
-      <c r="F12" s="35">
+      <c r="F12" s="34">
         <v>660.0</v>
       </c>
-      <c r="G12" s="44">
+      <c r="G12" s="43">
         <v>45856.0</v>
       </c>
-      <c r="H12" s="45" t="s">
-        <v>68</v>
-      </c>
-      <c r="I12" s="37"/>
-      <c r="J12" s="37">
+      <c r="H12" s="44" t="s">
+        <v>66</v>
+      </c>
+      <c r="I12" s="36"/>
+      <c r="J12" s="36">
         <v>45891.0</v>
       </c>
-      <c r="K12" s="46">
+      <c r="K12" s="45">
         <v>1402001.34</v>
       </c>
-      <c r="L12" s="47" t="s">
-        <v>114</v>
+      <c r="L12" s="46" t="s">
+        <v>105</v>
       </c>
       <c r="M12" s="39">
         <v>1402001.34</v>
       </c>
-      <c r="N12" s="48"/>
+      <c r="N12" s="47"/>
       <c r="O12" s="26"/>
       <c r="P12" s="28"/>
       <c r="V12" s="3"/>
     </row>
     <row r="13">
-      <c r="A13" s="23"/>
-      <c r="B13" s="23"/>
+      <c r="A13" s="24"/>
+      <c r="B13" s="24"/>
       <c r="C13" s="41"/>
       <c r="D13" s="49" t="s">
-        <v>120</v>
-      </c>
-      <c r="E13" s="35" t="s">
+        <v>109</v>
+      </c>
+      <c r="E13" s="34" t="s">
         <v>76</v>
       </c>
-      <c r="F13" s="36">
+      <c r="F13" s="35">
         <v>661.0</v>
       </c>
-      <c r="G13" s="37">
+      <c r="G13" s="36">
         <v>45856.0</v>
       </c>
-      <c r="H13" s="36" t="s">
-        <v>121</v>
-      </c>
-      <c r="I13" s="44"/>
-      <c r="J13" s="44">
+      <c r="H13" s="35" t="s">
+        <v>110</v>
+      </c>
+      <c r="I13" s="43"/>
+      <c r="J13" s="43">
         <v>45891.0</v>
       </c>
-      <c r="K13" s="46">
+      <c r="K13" s="45">
         <v>1223702.3</v>
       </c>
-      <c r="L13" s="35" t="s">
-        <v>125</v>
+      <c r="L13" s="34" t="s">
+        <v>114</v>
       </c>
       <c r="M13" s="39">
         <v>1223702.3</v>
       </c>
-      <c r="N13" s="48"/>
+      <c r="N13" s="47"/>
       <c r="O13" s="26"/>
       <c r="P13" s="50"/>
       <c r="V13" s="3"/>
     </row>
     <row r="14">
-      <c r="A14" s="23"/>
-      <c r="B14" s="23"/>
+      <c r="A14" s="24"/>
+      <c r="B14" s="24"/>
       <c r="C14" s="41"/>
       <c r="D14" s="49" t="s">
-        <v>129</v>
-      </c>
-      <c r="E14" s="35" t="s">
+        <v>116</v>
+      </c>
+      <c r="E14" s="34" t="s">
         <v>76</v>
       </c>
-      <c r="F14" s="35">
+      <c r="F14" s="34">
         <v>688.0</v>
       </c>
-      <c r="G14" s="37">
+      <c r="G14" s="36">
         <v>45901.0</v>
       </c>
-      <c r="H14" s="35" t="s">
-        <v>133</v>
-      </c>
-      <c r="I14" s="44"/>
-      <c r="J14" s="44">
+      <c r="H14" s="34" t="s">
+        <v>119</v>
+      </c>
+      <c r="I14" s="43"/>
+      <c r="J14" s="43">
         <v>45938.0</v>
       </c>
-      <c r="K14" s="46">
+      <c r="K14" s="45">
         <v>1011677.95</v>
       </c>
-      <c r="L14" s="35" t="s">
-        <v>134</v>
+      <c r="L14" s="34" t="s">
+        <v>120</v>
       </c>
       <c r="M14" s="39">
         <v>1011677.95</v>
@@ -1895,69 +1895,69 @@
       <c r="V14" s="3"/>
     </row>
     <row r="15">
-      <c r="A15" s="23"/>
-      <c r="B15" s="23"/>
+      <c r="A15" s="24"/>
+      <c r="B15" s="24"/>
       <c r="C15" s="41"/>
       <c r="D15" s="49" t="s">
-        <v>138</v>
-      </c>
-      <c r="E15" s="35" t="s">
+        <v>121</v>
+      </c>
+      <c r="E15" s="34" t="s">
         <v>76</v>
       </c>
-      <c r="F15" s="35">
+      <c r="F15" s="34">
         <v>696.0</v>
       </c>
-      <c r="G15" s="37">
+      <c r="G15" s="36">
         <v>45923.0</v>
       </c>
-      <c r="H15" s="35" t="s">
+      <c r="H15" s="34" t="s">
         <v>78</v>
       </c>
-      <c r="I15" s="44"/>
-      <c r="J15" s="44">
+      <c r="I15" s="43"/>
+      <c r="J15" s="43">
         <v>45938.0</v>
       </c>
-      <c r="K15" s="46">
+      <c r="K15" s="45">
         <v>896744.06</v>
       </c>
-      <c r="L15" s="35" t="s">
-        <v>142</v>
+      <c r="L15" s="34" t="s">
+        <v>125</v>
       </c>
       <c r="M15" s="39">
         <v>896744.06</v>
       </c>
-      <c r="N15" s="48"/>
+      <c r="N15" s="47"/>
       <c r="O15" s="26"/>
       <c r="V15" s="3"/>
     </row>
     <row r="16">
-      <c r="A16" s="23"/>
-      <c r="B16" s="23"/>
+      <c r="A16" s="24"/>
+      <c r="B16" s="24"/>
       <c r="C16" s="41"/>
       <c r="D16" s="49" t="s">
-        <v>145</v>
-      </c>
-      <c r="E16" s="35" t="s">
+        <v>128</v>
+      </c>
+      <c r="E16" s="34" t="s">
         <v>76</v>
       </c>
-      <c r="F16" s="35">
+      <c r="F16" s="34">
         <v>704.0</v>
       </c>
-      <c r="G16" s="37">
+      <c r="G16" s="36">
         <v>45957.0</v>
       </c>
-      <c r="H16" s="35" t="s">
-        <v>146</v>
-      </c>
-      <c r="I16" s="44"/>
-      <c r="J16" s="44">
+      <c r="H16" s="34" t="s">
+        <v>129</v>
+      </c>
+      <c r="I16" s="43"/>
+      <c r="J16" s="43">
         <v>46003.0</v>
       </c>
-      <c r="K16" s="46">
+      <c r="K16" s="45">
         <v>919329.06</v>
       </c>
-      <c r="L16" s="35" t="s">
-        <v>149</v>
+      <c r="L16" s="34" t="s">
+        <v>130</v>
       </c>
       <c r="M16" s="39">
         <v>919329.06</v>
@@ -1967,31 +1967,31 @@
       <c r="V16" s="3"/>
     </row>
     <row r="17">
-      <c r="A17" s="23"/>
-      <c r="B17" s="23"/>
+      <c r="A17" s="24"/>
+      <c r="B17" s="24"/>
       <c r="C17" s="41"/>
       <c r="D17" s="49" t="s">
-        <v>150</v>
-      </c>
-      <c r="E17" s="35"/>
-      <c r="F17" s="35">
+        <v>134</v>
+      </c>
+      <c r="E17" s="34"/>
+      <c r="F17" s="34">
         <v>705.0</v>
       </c>
-      <c r="G17" s="44">
+      <c r="G17" s="43">
         <v>45972.0</v>
       </c>
-      <c r="H17" s="35" t="s">
-        <v>154</v>
-      </c>
-      <c r="I17" s="35"/>
-      <c r="J17" s="44">
+      <c r="H17" s="34" t="s">
+        <v>135</v>
+      </c>
+      <c r="I17" s="34"/>
+      <c r="J17" s="43">
         <v>46016.0</v>
       </c>
-      <c r="K17" s="46">
+      <c r="K17" s="45">
         <v>1157009.26</v>
       </c>
-      <c r="L17" s="35" t="s">
-        <v>156</v>
+      <c r="L17" s="34" t="s">
+        <v>138</v>
       </c>
       <c r="M17" s="39">
         <v>1157009.26</v>
@@ -2001,33 +2001,33 @@
       <c r="V17" s="3"/>
     </row>
     <row r="18">
-      <c r="A18" s="23"/>
-      <c r="B18" s="23"/>
+      <c r="A18" s="24"/>
+      <c r="B18" s="24"/>
       <c r="C18" s="41"/>
       <c r="D18" s="49" t="s">
-        <v>157</v>
-      </c>
-      <c r="E18" s="35" t="s">
+        <v>140</v>
+      </c>
+      <c r="E18" s="34" t="s">
         <v>76</v>
       </c>
-      <c r="F18" s="35">
+      <c r="F18" s="34">
         <v>728.0</v>
       </c>
-      <c r="G18" s="44">
+      <c r="G18" s="43">
         <v>46008.0</v>
       </c>
-      <c r="H18" s="35" t="s">
-        <v>158</v>
-      </c>
-      <c r="I18" s="35"/>
-      <c r="J18" s="44">
+      <c r="H18" s="34" t="s">
+        <v>141</v>
+      </c>
+      <c r="I18" s="34"/>
+      <c r="J18" s="43">
         <v>46040.0</v>
       </c>
-      <c r="K18" s="46">
+      <c r="K18" s="45">
         <v>1214597.952</v>
       </c>
-      <c r="L18" s="35" t="s">
-        <v>159</v>
+      <c r="L18" s="34" t="s">
+        <v>145</v>
       </c>
       <c r="M18" s="39">
         <v>1214597.952</v>
@@ -2041,33 +2041,33 @@
       <c r="V18" s="52"/>
     </row>
     <row r="19">
-      <c r="A19" s="23"/>
-      <c r="B19" s="23"/>
+      <c r="A19" s="24"/>
+      <c r="B19" s="24"/>
       <c r="C19" s="41"/>
       <c r="D19" s="49" t="s">
-        <v>160</v>
-      </c>
-      <c r="E19" s="35" t="s">
+        <v>146</v>
+      </c>
+      <c r="E19" s="34" t="s">
         <v>76</v>
       </c>
-      <c r="F19" s="35">
+      <c r="F19" s="34">
         <v>278.0</v>
       </c>
-      <c r="G19" s="44">
+      <c r="G19" s="43">
         <v>46042.0</v>
       </c>
-      <c r="H19" s="35" t="s">
-        <v>161</v>
-      </c>
-      <c r="I19" s="44"/>
-      <c r="J19" s="44">
+      <c r="H19" s="34" t="s">
+        <v>150</v>
+      </c>
+      <c r="I19" s="43"/>
+      <c r="J19" s="43">
         <v>46074.0</v>
       </c>
-      <c r="K19" s="46">
+      <c r="K19" s="45">
         <v>967082.09</v>
       </c>
-      <c r="L19" s="35" t="s">
-        <v>162</v>
+      <c r="L19" s="34" t="s">
+        <v>151</v>
       </c>
       <c r="M19" s="39">
         <v>967082.09</v>
@@ -2081,31 +2081,31 @@
       <c r="V19" s="52"/>
     </row>
     <row r="20">
-      <c r="A20" s="23"/>
-      <c r="B20" s="23"/>
+      <c r="A20" s="24"/>
+      <c r="B20" s="24"/>
       <c r="C20" s="41"/>
       <c r="D20" s="49" t="s">
-        <v>163</v>
-      </c>
-      <c r="E20" s="35"/>
-      <c r="F20" s="35">
+        <v>155</v>
+      </c>
+      <c r="E20" s="34"/>
+      <c r="F20" s="34">
         <v>10.0</v>
       </c>
-      <c r="G20" s="44">
+      <c r="G20" s="43">
         <v>46078.0</v>
       </c>
-      <c r="H20" s="35" t="s">
-        <v>103</v>
-      </c>
-      <c r="I20" s="44"/>
-      <c r="J20" s="44">
+      <c r="H20" s="34" t="s">
+        <v>106</v>
+      </c>
+      <c r="I20" s="43"/>
+      <c r="J20" s="43">
         <v>46106.0</v>
       </c>
-      <c r="K20" s="46">
+      <c r="K20" s="45">
         <v>719561.08</v>
       </c>
-      <c r="L20" s="35" t="s">
-        <v>164</v>
+      <c r="L20" s="34" t="s">
+        <v>156</v>
       </c>
       <c r="M20" s="39">
         <v>719561.08</v>
@@ -2119,31 +2119,31 @@
       <c r="V20" s="52"/>
     </row>
     <row r="21">
-      <c r="A21" s="23"/>
-      <c r="B21" s="23"/>
+      <c r="A21" s="24"/>
+      <c r="B21" s="24"/>
       <c r="C21" s="41"/>
       <c r="D21" s="49" t="s">
-        <v>165</v>
-      </c>
-      <c r="E21" s="35"/>
-      <c r="F21" s="35">
+        <v>158</v>
+      </c>
+      <c r="E21" s="34"/>
+      <c r="F21" s="34">
         <v>15.0</v>
       </c>
-      <c r="G21" s="44">
+      <c r="G21" s="43">
         <v>46094.0</v>
       </c>
-      <c r="H21" s="35" t="s">
-        <v>166</v>
-      </c>
-      <c r="I21" s="44"/>
-      <c r="J21" s="44">
+      <c r="H21" s="34" t="s">
+        <v>160</v>
+      </c>
+      <c r="I21" s="43"/>
+      <c r="J21" s="43">
         <v>46128.0</v>
       </c>
-      <c r="K21" s="46">
+      <c r="K21" s="45">
         <v>885881.08</v>
       </c>
-      <c r="L21" s="35" t="s">
-        <v>167</v>
+      <c r="L21" s="34" t="s">
+        <v>161</v>
       </c>
       <c r="M21" s="39">
         <v>885881.08</v>
@@ -2157,34 +2157,34 @@
       <c r="V21" s="52"/>
     </row>
     <row r="22">
-      <c r="A22" s="23"/>
-      <c r="B22" s="23"/>
+      <c r="A22" s="24"/>
+      <c r="B22" s="24"/>
       <c r="C22" s="41"/>
       <c r="D22" s="49" t="s">
-        <v>168</v>
-      </c>
-      <c r="E22" s="35"/>
-      <c r="F22" s="35">
+        <v>162</v>
+      </c>
+      <c r="E22" s="34"/>
+      <c r="F22" s="34">
         <v>28.0</v>
       </c>
-      <c r="G22" s="44">
+      <c r="G22" s="43">
         <v>46128.0</v>
       </c>
-      <c r="H22" s="35" t="s">
-        <v>169</v>
-      </c>
-      <c r="I22" s="44"/>
-      <c r="J22" s="44">
+      <c r="H22" s="34" t="s">
+        <v>165</v>
+      </c>
+      <c r="I22" s="43"/>
+      <c r="J22" s="43">
         <v>46164.0</v>
       </c>
-      <c r="K22" s="46" t="s">
-        <v>170</v>
-      </c>
-      <c r="L22" s="35" t="s">
-        <v>171</v>
+      <c r="K22" s="45" t="s">
+        <v>166</v>
+      </c>
+      <c r="L22" s="34" t="s">
+        <v>167</v>
       </c>
       <c r="M22" s="39" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="N22" s="51"/>
       <c r="O22" s="26"/>
@@ -2195,31 +2195,31 @@
       <c r="V22" s="52"/>
     </row>
     <row r="23">
-      <c r="A23" s="23"/>
-      <c r="B23" s="23"/>
+      <c r="A23" s="24"/>
+      <c r="B23" s="24"/>
       <c r="C23" s="41"/>
       <c r="D23" s="49" t="s">
+        <v>168</v>
+      </c>
+      <c r="E23" s="34"/>
+      <c r="F23" s="34">
+        <v>33.0</v>
+      </c>
+      <c r="G23" s="43">
+        <v>46156.0</v>
+      </c>
+      <c r="H23" s="34" t="s">
         <v>172</v>
       </c>
-      <c r="E23" s="35"/>
-      <c r="F23" s="35">
-        <v>33.0</v>
-      </c>
-      <c r="G23" s="44">
-        <v>46156.0</v>
-      </c>
-      <c r="H23" s="35" t="s">
-        <v>173</v>
-      </c>
-      <c r="I23" s="44"/>
-      <c r="J23" s="44">
+      <c r="I23" s="43"/>
+      <c r="J23" s="43">
         <v>46191.0</v>
       </c>
-      <c r="K23" s="46">
+      <c r="K23" s="45">
         <v>1108954.4358333333</v>
       </c>
-      <c r="L23" s="35" t="s">
-        <v>167</v>
+      <c r="L23" s="34" t="s">
+        <v>161</v>
       </c>
       <c r="M23" s="39">
         <v>1108954.4358333333</v>
@@ -2233,30 +2233,30 @@
       <c r="V23" s="52"/>
     </row>
     <row r="24">
-      <c r="A24" s="23"/>
-      <c r="B24" s="23"/>
+      <c r="A24" s="24"/>
+      <c r="B24" s="24"/>
       <c r="C24" s="41"/>
       <c r="D24" s="49" t="s">
         <v>174</v>
       </c>
-      <c r="E24" s="35"/>
-      <c r="F24" s="35">
+      <c r="E24" s="34"/>
+      <c r="F24" s="34">
         <v>29.0</v>
       </c>
-      <c r="G24" s="44">
+      <c r="G24" s="43">
         <v>46149.0</v>
       </c>
-      <c r="H24" s="35" t="s">
-        <v>173</v>
-      </c>
-      <c r="I24" s="44"/>
-      <c r="J24" s="44">
+      <c r="H24" s="34" t="s">
+        <v>172</v>
+      </c>
+      <c r="I24" s="43"/>
+      <c r="J24" s="43">
         <v>46185.0</v>
       </c>
-      <c r="K24" s="46">
+      <c r="K24" s="45">
         <v>218206.1</v>
       </c>
-      <c r="L24" s="35" t="s">
+      <c r="L24" s="34" t="s">
         <v>175</v>
       </c>
       <c r="M24" s="39">
@@ -2271,30 +2271,30 @@
       <c r="V24" s="52"/>
     </row>
     <row r="25">
-      <c r="A25" s="23"/>
-      <c r="B25" s="23"/>
+      <c r="A25" s="24"/>
+      <c r="B25" s="24"/>
       <c r="C25" s="41"/>
       <c r="D25" s="49" t="s">
         <v>176</v>
       </c>
-      <c r="E25" s="35"/>
-      <c r="F25" s="35">
+      <c r="E25" s="34"/>
+      <c r="F25" s="34">
         <v>40.0</v>
       </c>
-      <c r="G25" s="44">
+      <c r="G25" s="43">
         <v>46156.0</v>
       </c>
-      <c r="H25" s="35" t="s">
-        <v>173</v>
-      </c>
-      <c r="I25" s="44"/>
-      <c r="J25" s="44">
+      <c r="H25" s="34" t="s">
+        <v>172</v>
+      </c>
+      <c r="I25" s="43"/>
+      <c r="J25" s="43">
         <v>46191.0</v>
       </c>
-      <c r="K25" s="46">
+      <c r="K25" s="45">
         <v>1549250.84</v>
       </c>
-      <c r="L25" s="35" t="s">
+      <c r="L25" s="34" t="s">
         <v>177</v>
       </c>
       <c r="M25" s="39">
@@ -2309,30 +2309,30 @@
       <c r="V25" s="52"/>
     </row>
     <row r="26">
-      <c r="A26" s="23"/>
-      <c r="B26" s="23"/>
+      <c r="A26" s="24"/>
+      <c r="B26" s="24"/>
       <c r="C26" s="55"/>
       <c r="D26" s="49" t="s">
         <v>178</v>
       </c>
-      <c r="E26" s="35"/>
-      <c r="F26" s="35">
+      <c r="E26" s="34"/>
+      <c r="F26" s="34">
         <v>48.0</v>
       </c>
-      <c r="G26" s="44">
+      <c r="G26" s="43">
         <v>46230.0</v>
       </c>
-      <c r="H26" s="35" t="s">
+      <c r="H26" s="34" t="s">
         <v>179</v>
       </c>
-      <c r="I26" s="44"/>
-      <c r="J26" s="44">
+      <c r="I26" s="43"/>
+      <c r="J26" s="43">
         <v>46262.0</v>
       </c>
-      <c r="K26" s="46" t="s">
+      <c r="K26" s="45" t="s">
         <v>180</v>
       </c>
-      <c r="L26" s="35" t="s">
+      <c r="L26" s="34" t="s">
         <v>181</v>
       </c>
       <c r="M26" s="39" t="s">
@@ -2347,20 +2347,20 @@
       <c r="V26" s="52"/>
     </row>
     <row r="27">
-      <c r="A27" s="23"/>
-      <c r="B27" s="23"/>
-      <c r="C27" s="36"/>
+      <c r="A27" s="24"/>
+      <c r="B27" s="24"/>
+      <c r="C27" s="35"/>
       <c r="D27" s="49" t="s">
         <v>182</v>
       </c>
-      <c r="E27" s="35"/>
-      <c r="F27" s="35"/>
-      <c r="G27" s="44"/>
-      <c r="H27" s="35"/>
-      <c r="I27" s="44"/>
-      <c r="J27" s="44"/>
-      <c r="K27" s="46"/>
-      <c r="L27" s="35"/>
+      <c r="E27" s="34"/>
+      <c r="F27" s="34"/>
+      <c r="G27" s="43"/>
+      <c r="H27" s="34"/>
+      <c r="I27" s="43"/>
+      <c r="J27" s="43"/>
+      <c r="K27" s="45"/>
+      <c r="L27" s="34"/>
       <c r="M27" s="39"/>
       <c r="N27" s="54" t="s">
         <v>183</v>
@@ -2373,23 +2373,23 @@
       <c r="V27" s="52"/>
     </row>
     <row r="28" ht="30.75" customHeight="1">
-      <c r="A28" s="23"/>
-      <c r="B28" s="23"/>
+      <c r="A28" s="24"/>
+      <c r="B28" s="24"/>
       <c r="C28" s="29" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D28" s="29" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E28" s="30" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F28" s="29" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="G28" s="29"/>
       <c r="H28" s="29" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="I28" s="29"/>
       <c r="J28" s="29"/>
@@ -2397,10 +2397,10 @@
         <v>65</v>
       </c>
       <c r="L28" s="31" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="M28" s="57" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="N28" s="29" t="s">
         <v>71</v>
@@ -2421,32 +2421,32 @@
       <c r="AC28" s="28"/>
     </row>
     <row r="29" ht="12.75" customHeight="1">
-      <c r="A29" s="23"/>
-      <c r="B29" s="23"/>
+      <c r="A29" s="24"/>
+      <c r="B29" s="24"/>
       <c r="C29" s="32">
         <v>2.0</v>
       </c>
       <c r="D29" s="58" t="s">
         <v>184</v>
       </c>
-      <c r="E29" s="36"/>
-      <c r="F29" s="36">
+      <c r="E29" s="35"/>
+      <c r="F29" s="35">
         <v>402.0</v>
       </c>
-      <c r="G29" s="37">
+      <c r="G29" s="36">
         <v>45791.0</v>
       </c>
-      <c r="H29" s="36" t="s">
+      <c r="H29" s="35" t="s">
         <v>49</v>
       </c>
-      <c r="I29" s="37"/>
-      <c r="J29" s="37">
+      <c r="I29" s="36"/>
+      <c r="J29" s="36">
         <v>45834.0</v>
       </c>
       <c r="K29" s="38">
         <v>188246.17</v>
       </c>
-      <c r="L29" s="35" t="s">
+      <c r="L29" s="34" t="s">
         <v>185</v>
       </c>
       <c r="M29" s="59">
@@ -2470,8 +2470,8 @@
       <c r="AC29" s="28"/>
     </row>
     <row r="30">
-      <c r="A30" s="23"/>
-      <c r="B30" s="23"/>
+      <c r="A30" s="24"/>
+      <c r="B30" s="24"/>
       <c r="C30" s="41"/>
       <c r="D30" s="58" t="s">
         <v>186</v>
@@ -2479,23 +2479,23 @@
       <c r="E30" s="60">
         <v>46.0</v>
       </c>
-      <c r="F30" s="36">
+      <c r="F30" s="35">
         <v>447.0</v>
       </c>
-      <c r="G30" s="37">
+      <c r="G30" s="36">
         <v>45814.0</v>
       </c>
-      <c r="H30" s="35" t="s">
+      <c r="H30" s="34" t="s">
         <v>187</v>
       </c>
-      <c r="I30" s="44"/>
-      <c r="J30" s="44">
+      <c r="I30" s="43"/>
+      <c r="J30" s="43">
         <v>45955.0</v>
       </c>
       <c r="K30" s="38">
         <v>112720.77</v>
       </c>
-      <c r="L30" s="35" t="s">
+      <c r="L30" s="34" t="s">
         <v>188</v>
       </c>
       <c r="M30" s="39">
@@ -2519,8 +2519,8 @@
       <c r="AC30" s="28"/>
     </row>
     <row r="31" ht="12.75" customHeight="1">
-      <c r="A31" s="23"/>
-      <c r="B31" s="23"/>
+      <c r="A31" s="24"/>
+      <c r="B31" s="24"/>
       <c r="C31" s="41"/>
       <c r="D31" s="61" t="s">
         <v>189</v>
@@ -2528,23 +2528,23 @@
       <c r="E31" s="62" t="s">
         <v>190</v>
       </c>
-      <c r="F31" s="36">
+      <c r="F31" s="35">
         <v>529.0</v>
       </c>
       <c r="G31" s="63">
         <v>45853.0</v>
       </c>
-      <c r="H31" s="35" t="s">
+      <c r="H31" s="34" t="s">
         <v>53</v>
       </c>
-      <c r="I31" s="44"/>
-      <c r="J31" s="44">
+      <c r="I31" s="43"/>
+      <c r="J31" s="43">
         <v>45939.0</v>
       </c>
-      <c r="K31" s="46">
+      <c r="K31" s="45">
         <v>378307.61</v>
       </c>
-      <c r="L31" s="35" t="s">
+      <c r="L31" s="34" t="s">
         <v>191</v>
       </c>
       <c r="M31" s="39">
@@ -2568,8 +2568,8 @@
       <c r="AC31" s="28"/>
     </row>
     <row r="32" ht="60.0" customHeight="1">
-      <c r="A32" s="23"/>
-      <c r="B32" s="23"/>
+      <c r="A32" s="24"/>
+      <c r="B32" s="24"/>
       <c r="C32" s="41"/>
       <c r="D32" s="61" t="s">
         <v>192</v>
@@ -2577,23 +2577,23 @@
       <c r="E32" s="62" t="s">
         <v>190</v>
       </c>
-      <c r="F32" s="35">
+      <c r="F32" s="34">
         <v>691.0</v>
       </c>
       <c r="G32" s="63">
         <v>45910.0</v>
       </c>
-      <c r="H32" s="35" t="s">
+      <c r="H32" s="34" t="s">
         <v>53</v>
       </c>
-      <c r="I32" s="44"/>
-      <c r="J32" s="44">
+      <c r="I32" s="43"/>
+      <c r="J32" s="43">
         <v>45941.0</v>
       </c>
       <c r="K32" s="38">
         <v>3315.0471000000252</v>
       </c>
-      <c r="L32" s="35" t="s">
+      <c r="L32" s="34" t="s">
         <v>193</v>
       </c>
       <c r="M32" s="39">
@@ -2617,8 +2617,8 @@
       <c r="AC32" s="28"/>
     </row>
     <row r="33" ht="12.75" customHeight="1">
-      <c r="A33" s="23"/>
-      <c r="B33" s="23"/>
+      <c r="A33" s="24"/>
+      <c r="B33" s="24"/>
       <c r="C33" s="41"/>
       <c r="D33" s="61" t="s">
         <v>194</v>
@@ -2626,23 +2626,23 @@
       <c r="E33" s="65">
         <v>135.0</v>
       </c>
-      <c r="F33" s="35">
+      <c r="F33" s="34">
         <v>677.0</v>
       </c>
       <c r="G33" s="63">
         <v>45904.0</v>
       </c>
-      <c r="H33" s="35" t="s">
-        <v>68</v>
+      <c r="H33" s="34" t="s">
+        <v>66</v>
       </c>
       <c r="I33" s="66"/>
       <c r="J33" s="66">
         <v>45935.0</v>
       </c>
-      <c r="K33" s="46">
+      <c r="K33" s="45">
         <v>198332.75</v>
       </c>
-      <c r="L33" s="35" t="s">
+      <c r="L33" s="34" t="s">
         <v>195</v>
       </c>
       <c r="M33" s="39">
@@ -2666,8 +2666,8 @@
       <c r="AC33" s="28"/>
     </row>
     <row r="34" ht="12.75" customHeight="1">
-      <c r="A34" s="23"/>
-      <c r="B34" s="23"/>
+      <c r="A34" s="24"/>
+      <c r="B34" s="24"/>
       <c r="C34" s="41"/>
       <c r="D34" s="61" t="s">
         <v>196</v>
@@ -2675,20 +2675,20 @@
       <c r="E34" s="65">
         <v>40.0</v>
       </c>
-      <c r="F34" s="35">
+      <c r="F34" s="34">
         <v>278.0</v>
       </c>
       <c r="G34" s="63">
         <v>46008.0</v>
       </c>
-      <c r="H34" s="35" t="s">
-        <v>115</v>
+      <c r="H34" s="34" t="s">
+        <v>122</v>
       </c>
       <c r="I34" s="66"/>
       <c r="J34" s="66">
         <v>46066.0</v>
       </c>
-      <c r="K34" s="46">
+      <c r="K34" s="45">
         <v>1528.62</v>
       </c>
       <c r="L34" s="67" t="s">
@@ -2715,8 +2715,8 @@
       <c r="AC34" s="28"/>
     </row>
     <row r="35" ht="12.75" customHeight="1">
-      <c r="A35" s="23"/>
-      <c r="B35" s="23"/>
+      <c r="A35" s="24"/>
+      <c r="B35" s="24"/>
       <c r="C35" s="41"/>
       <c r="D35" s="61" t="s">
         <v>199</v>
@@ -2724,23 +2724,23 @@
       <c r="E35" s="65" t="s">
         <v>200</v>
       </c>
-      <c r="F35" s="35">
+      <c r="F35" s="34">
         <v>748.0</v>
       </c>
       <c r="G35" s="63">
         <v>45930.0</v>
       </c>
-      <c r="H35" s="35" t="s">
-        <v>91</v>
+      <c r="H35" s="34" t="s">
+        <v>93</v>
       </c>
       <c r="I35" s="66"/>
       <c r="J35" s="66">
         <v>45935.0</v>
       </c>
-      <c r="K35" s="46">
+      <c r="K35" s="45">
         <v>38718.58</v>
       </c>
-      <c r="L35" s="35" t="s">
+      <c r="L35" s="34" t="s">
         <v>201</v>
       </c>
       <c r="M35" s="59" t="s">
@@ -2764,8 +2764,8 @@
       <c r="AC35" s="28"/>
     </row>
     <row r="36" ht="12.75" customHeight="1">
-      <c r="A36" s="23"/>
-      <c r="B36" s="23"/>
+      <c r="A36" s="24"/>
+      <c r="B36" s="24"/>
       <c r="C36" s="41"/>
       <c r="D36" s="61" t="s">
         <v>203</v>
@@ -2773,23 +2773,23 @@
       <c r="E36" s="65">
         <v>154.0</v>
       </c>
-      <c r="F36" s="35">
+      <c r="F36" s="34">
         <v>822.0</v>
       </c>
       <c r="G36" s="63">
         <v>45968.0</v>
       </c>
-      <c r="H36" s="35" t="s">
-        <v>107</v>
+      <c r="H36" s="34" t="s">
+        <v>111</v>
       </c>
       <c r="I36" s="66"/>
       <c r="J36" s="66">
         <v>45935.0</v>
       </c>
-      <c r="K36" s="46">
+      <c r="K36" s="45">
         <v>133124.11</v>
       </c>
-      <c r="L36" s="35" t="s">
+      <c r="L36" s="34" t="s">
         <v>204</v>
       </c>
       <c r="M36" s="59" t="s">
@@ -2813,8 +2813,8 @@
       <c r="AC36" s="28"/>
     </row>
     <row r="37" ht="12.75" customHeight="1">
-      <c r="A37" s="23"/>
-      <c r="B37" s="23"/>
+      <c r="A37" s="24"/>
+      <c r="B37" s="24"/>
       <c r="C37" s="41"/>
       <c r="D37" s="61" t="s">
         <v>206</v>
@@ -2829,16 +2829,16 @@
         <v>46043.0</v>
       </c>
       <c r="H37" s="65" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="I37" s="70"/>
       <c r="J37" s="69">
         <v>46075.0</v>
       </c>
-      <c r="K37" s="46">
+      <c r="K37" s="45">
         <v>11372.9</v>
       </c>
-      <c r="L37" s="35" t="s">
+      <c r="L37" s="34" t="s">
         <v>207</v>
       </c>
       <c r="M37" s="39">
@@ -2862,8 +2862,8 @@
       <c r="AC37" s="28"/>
     </row>
     <row r="38" ht="12.75" customHeight="1">
-      <c r="A38" s="23"/>
-      <c r="B38" s="23"/>
+      <c r="A38" s="24"/>
+      <c r="B38" s="24"/>
       <c r="C38" s="41"/>
       <c r="D38" s="61" t="s">
         <v>208</v>
@@ -2876,8 +2876,8 @@
         <v>209</v>
       </c>
       <c r="J38" s="69"/>
-      <c r="K38" s="46"/>
-      <c r="L38" s="35"/>
+      <c r="K38" s="45"/>
+      <c r="L38" s="34"/>
       <c r="M38" s="39"/>
       <c r="N38" s="51">
         <v>15854.78</v>
@@ -2899,8 +2899,8 @@
       <c r="AC38" s="28"/>
     </row>
     <row r="39" ht="12.75" customHeight="1">
-      <c r="A39" s="23"/>
-      <c r="B39" s="23"/>
+      <c r="A39" s="24"/>
+      <c r="B39" s="24"/>
       <c r="C39" s="55"/>
       <c r="D39" s="61" t="s">
         <v>210</v>
@@ -2913,8 +2913,8 @@
         <v>209</v>
       </c>
       <c r="J39" s="69"/>
-      <c r="K39" s="46"/>
-      <c r="L39" s="35"/>
+      <c r="K39" s="45"/>
+      <c r="L39" s="34"/>
       <c r="M39" s="39"/>
       <c r="N39" s="71">
         <v>42229.72325</v>
@@ -2936,9 +2936,9 @@
       <c r="AC39" s="28"/>
     </row>
     <row r="40" ht="12.75" customHeight="1">
-      <c r="A40" s="23"/>
-      <c r="B40" s="23"/>
-      <c r="C40" s="36"/>
+      <c r="A40" s="24"/>
+      <c r="B40" s="24"/>
+      <c r="C40" s="35"/>
       <c r="D40" s="61" t="s">
         <v>211</v>
       </c>
@@ -2950,8 +2950,8 @@
         <v>209</v>
       </c>
       <c r="J40" s="69"/>
-      <c r="K40" s="46"/>
-      <c r="L40" s="47"/>
+      <c r="K40" s="45"/>
+      <c r="L40" s="46"/>
       <c r="M40" s="39"/>
       <c r="N40" s="72">
         <v>48857.395500000006</v>
@@ -2973,9 +2973,9 @@
       <c r="AC40" s="28"/>
     </row>
     <row r="41" ht="12.75" customHeight="1">
-      <c r="A41" s="23"/>
-      <c r="B41" s="23"/>
-      <c r="C41" s="36"/>
+      <c r="A41" s="24"/>
+      <c r="B41" s="24"/>
+      <c r="C41" s="35"/>
       <c r="D41" s="61" t="s">
         <v>212</v>
       </c>
@@ -2987,8 +2987,8 @@
         <v>213</v>
       </c>
       <c r="J41" s="69"/>
-      <c r="K41" s="46"/>
-      <c r="L41" s="47"/>
+      <c r="K41" s="45"/>
+      <c r="L41" s="46"/>
       <c r="M41" s="39"/>
       <c r="N41" s="72"/>
       <c r="O41" s="26"/>
@@ -3008,8 +3008,8 @@
       <c r="AC41" s="28"/>
     </row>
     <row r="42" ht="12.75" customHeight="1">
-      <c r="A42" s="23"/>
-      <c r="B42" s="23"/>
+      <c r="A42" s="24"/>
+      <c r="B42" s="24"/>
       <c r="C42" s="32">
         <v>3.0</v>
       </c>
@@ -3024,13 +3024,13 @@
         <v>46104.0</v>
       </c>
       <c r="H42" s="65" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="I42" s="70"/>
       <c r="J42" s="69">
         <v>46106.0</v>
       </c>
-      <c r="K42" s="46">
+      <c r="K42" s="45">
         <v>27801.11</v>
       </c>
       <c r="L42" s="73" t="s">
@@ -3077,11 +3077,11 @@
       <c r="J43" s="69">
         <v>46233.0</v>
       </c>
-      <c r="K43" s="46">
+      <c r="K43" s="45">
         <v>58868.35</v>
       </c>
-      <c r="L43" s="35" t="s">
-        <v>67</v>
+      <c r="L43" s="34" t="s">
+        <v>70</v>
       </c>
       <c r="M43" s="74">
         <v>58868.35</v>
@@ -8040,11 +8040,11 @@
       <c r="AH1" s="2"/>
     </row>
     <row r="2">
-      <c r="A2" s="4">
+      <c r="A2" s="5">
         <v>46212.0</v>
       </c>
-      <c r="L2" s="6" t="s">
-        <v>0</v>
+      <c r="L2" s="7" t="s">
+        <v>1</v>
       </c>
       <c r="AB2" s="2"/>
       <c r="AC2" s="2"/>
@@ -8055,31 +8055,31 @@
       <c r="AH2" s="2"/>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="10" t="s">
         <v>3</v>
       </c>
       <c r="C3" s="11">
         <v>2.5E32</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="D3" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E3" s="12">
         <v>45686.0</v>
       </c>
-      <c r="F3" s="8" t="s">
+      <c r="F3" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G3" s="8">
+      <c r="G3" s="10">
         <v>12.0</v>
       </c>
-      <c r="H3" s="8">
+      <c r="H3" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I3" s="8">
+      <c r="I3" s="10">
         <v>2048.0</v>
       </c>
       <c r="J3" s="14">
@@ -8088,7 +8088,7 @@
       <c r="K3" s="14">
         <v>1000.0</v>
       </c>
-      <c r="L3" s="8">
+      <c r="L3" s="10">
         <v>0.0</v>
       </c>
       <c r="AB3" s="2"/>
@@ -8100,31 +8100,31 @@
       <c r="AH3" s="2"/>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="C4" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="D4" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E4" s="12">
         <v>45762.0</v>
       </c>
-      <c r="F4" s="8" t="s">
+      <c r="F4" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G4" s="8">
+      <c r="G4" s="10">
         <v>12.0</v>
       </c>
-      <c r="H4" s="8">
+      <c r="H4" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I4" s="8">
+      <c r="I4" s="10">
         <v>2048.0</v>
       </c>
       <c r="J4" s="14">
@@ -8133,7 +8133,7 @@
       <c r="K4" s="14">
         <v>52250.04</v>
       </c>
-      <c r="L4" s="8">
+      <c r="L4" s="10">
         <v>0.0</v>
       </c>
       <c r="AB4" s="2"/>
@@ -8145,31 +8145,31 @@
       <c r="AH4" s="2"/>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="C5" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="D5" s="8" t="s">
+      <c r="D5" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E5" s="12">
         <v>45762.0</v>
       </c>
-      <c r="F5" s="8" t="s">
+      <c r="F5" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G5" s="8">
+      <c r="G5" s="10">
         <v>12.0</v>
       </c>
-      <c r="H5" s="8">
+      <c r="H5" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I5" s="8">
+      <c r="I5" s="10">
         <v>2048.0</v>
       </c>
       <c r="J5" s="14">
@@ -8178,7 +8178,7 @@
       <c r="K5" s="14">
         <v>881914.18</v>
       </c>
-      <c r="L5" s="8">
+      <c r="L5" s="10">
         <v>0.0</v>
       </c>
       <c r="AB5" s="2"/>
@@ -8190,31 +8190,31 @@
       <c r="AH5" s="2"/>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="B6" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="C6" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="D6" s="8" t="s">
+      <c r="A6" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="D6" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E6" s="12">
         <v>45762.0</v>
       </c>
-      <c r="F6" s="8" t="s">
+      <c r="F6" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G6" s="8">
+      <c r="G6" s="10">
         <v>12.0</v>
       </c>
-      <c r="H6" s="8">
+      <c r="H6" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I6" s="8">
+      <c r="I6" s="10">
         <v>2048.0</v>
       </c>
       <c r="J6" s="14">
@@ -8223,7 +8223,7 @@
       <c r="K6" s="14">
         <v>750000.0</v>
       </c>
-      <c r="L6" s="8">
+      <c r="L6" s="10">
         <v>0.0</v>
       </c>
       <c r="AB6" s="2"/>
@@ -8235,32 +8235,32 @@
       <c r="AH6" s="2"/>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="B7" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="C7" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="D7" s="8" t="s">
+      <c r="A7" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="D7" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E7" s="12">
         <v>45763.0</v>
       </c>
-      <c r="F7" s="8" t="s">
+      <c r="F7" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G7" s="8">
+      <c r="G7" s="10">
         <v>12.0</v>
       </c>
-      <c r="H7" s="8">
+      <c r="H7" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I7" s="8" t="s">
-        <v>43</v>
+      <c r="I7" s="10" t="s">
+        <v>39</v>
       </c>
       <c r="J7" s="14">
         <v>949835.78</v>
@@ -8268,7 +8268,7 @@
       <c r="K7" s="14">
         <v>949835.78</v>
       </c>
-      <c r="L7" s="8">
+      <c r="L7" s="10">
         <v>0.0</v>
       </c>
       <c r="AB7" s="2"/>
@@ -8280,31 +8280,31 @@
       <c r="AH7" s="2"/>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="s">
+      <c r="A8" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="B8" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="C8" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="C8" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="D8" s="8" t="s">
+      <c r="D8" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E8" s="12">
         <v>45763.0</v>
       </c>
-      <c r="F8" s="8" t="s">
+      <c r="F8" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G8" s="8">
+      <c r="G8" s="10">
         <v>12.0</v>
       </c>
-      <c r="H8" s="8">
+      <c r="H8" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I8" s="8" t="s">
+      <c r="I8" s="10" t="s">
         <v>48</v>
       </c>
       <c r="J8" s="14">
@@ -8313,10 +8313,10 @@
       <c r="K8" s="14">
         <v>524584.95</v>
       </c>
-      <c r="L8" s="8">
+      <c r="L8" s="10">
         <v>0.0</v>
       </c>
-      <c r="O8" s="24"/>
+      <c r="O8" s="23"/>
       <c r="AB8" s="2"/>
       <c r="AC8" s="2"/>
       <c r="AD8" s="2"/>
@@ -8326,31 +8326,31 @@
       <c r="AH8" s="2"/>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="s">
+      <c r="A9" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="B9" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="C9" s="8" t="s">
+      <c r="C9" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="D9" s="8" t="s">
+      <c r="D9" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E9" s="12">
         <v>45792.0</v>
       </c>
-      <c r="F9" s="8" t="s">
+      <c r="F9" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G9" s="8">
+      <c r="G9" s="10">
         <v>12.0</v>
       </c>
-      <c r="H9" s="8">
+      <c r="H9" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I9" s="8" t="s">
+      <c r="I9" s="10" t="s">
         <v>52</v>
       </c>
       <c r="J9" s="14">
@@ -8359,7 +8359,7 @@
       <c r="K9" s="14">
         <v>211614.23</v>
       </c>
-      <c r="L9" s="8">
+      <c r="L9" s="10">
         <v>0.0</v>
       </c>
       <c r="AB9" s="2"/>
@@ -8371,31 +8371,31 @@
       <c r="AH9" s="2"/>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="s">
+      <c r="A10" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="B10" s="8" t="s">
+      <c r="B10" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="C10" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="D10" s="8" t="s">
+      <c r="C10" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="D10" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E10" s="12">
         <v>45825.0</v>
       </c>
-      <c r="F10" s="8" t="s">
+      <c r="F10" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G10" s="8">
+      <c r="G10" s="10">
         <v>12.0</v>
       </c>
-      <c r="H10" s="8">
+      <c r="H10" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I10" s="8">
+      <c r="I10" s="10">
         <v>2048.0</v>
       </c>
       <c r="J10" s="14">
@@ -8416,31 +8416,31 @@
       <c r="AH10" s="2"/>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="B11" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="C11" s="8" t="s">
-        <v>62</v>
-      </c>
-      <c r="D11" s="8" t="s">
+      <c r="A11" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="C11" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="D11" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E11" s="12">
         <v>45825.0</v>
       </c>
-      <c r="F11" s="8" t="s">
+      <c r="F11" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G11" s="8">
+      <c r="G11" s="10">
         <v>12.0</v>
       </c>
-      <c r="H11" s="8">
+      <c r="H11" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I11" s="8">
+      <c r="I11" s="10">
         <v>2048.0</v>
       </c>
       <c r="J11" s="14">
@@ -8449,7 +8449,7 @@
       <c r="K11" s="14">
         <v>618154.38</v>
       </c>
-      <c r="L11" s="8">
+      <c r="L11" s="10">
         <v>0.01</v>
       </c>
       <c r="AB11" s="2"/>
@@ -8461,31 +8461,31 @@
       <c r="AH11" s="2"/>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="s">
-        <v>68</v>
-      </c>
-      <c r="B12" s="8" t="s">
+      <c r="A12" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="B12" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="C12" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="C12" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="D12" s="8" t="s">
+      <c r="D12" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E12" s="12">
         <v>45832.0</v>
       </c>
-      <c r="F12" s="8" t="s">
+      <c r="F12" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G12" s="8">
+      <c r="G12" s="10">
         <v>12.0</v>
       </c>
-      <c r="H12" s="8">
+      <c r="H12" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I12" s="8" t="s">
+      <c r="I12" s="10" t="s">
         <v>72</v>
       </c>
       <c r="J12" s="14">
@@ -8494,7 +8494,7 @@
       <c r="K12" s="14">
         <v>1600334.09</v>
       </c>
-      <c r="L12" s="8">
+      <c r="L12" s="10">
         <v>0.0</v>
       </c>
       <c r="AB12" s="2"/>
@@ -8506,31 +8506,31 @@
       <c r="AH12" s="2"/>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="s">
+      <c r="A13" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="B13" s="8" t="s">
+      <c r="B13" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="C13" s="8" t="s">
+      <c r="C13" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="D13" s="8" t="s">
+      <c r="D13" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E13" s="12">
         <v>45863.0</v>
       </c>
-      <c r="F13" s="8" t="s">
+      <c r="F13" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G13" s="8">
+      <c r="G13" s="10">
         <v>12.0</v>
       </c>
-      <c r="H13" s="8">
+      <c r="H13" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I13" s="8">
+      <c r="I13" s="10">
         <v>2048.0</v>
       </c>
       <c r="J13" s="14">
@@ -8542,7 +8542,7 @@
       <c r="L13" s="14">
         <v>0.0</v>
       </c>
-      <c r="M13" s="34"/>
+      <c r="M13" s="37"/>
       <c r="AB13" s="2"/>
       <c r="AC13" s="2"/>
       <c r="AD13" s="2"/>
@@ -8552,31 +8552,31 @@
       <c r="AH13" s="2"/>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="s">
+      <c r="A14" s="10" t="s">
         <v>78</v>
       </c>
-      <c r="B14" s="8" t="s">
+      <c r="B14" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="C14" s="8" t="s">
+      <c r="C14" s="10" t="s">
         <v>80</v>
       </c>
-      <c r="D14" s="8" t="s">
+      <c r="D14" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E14" s="12">
         <v>45887.0</v>
       </c>
-      <c r="F14" s="8" t="s">
+      <c r="F14" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G14" s="8">
+      <c r="G14" s="10">
         <v>12.0</v>
       </c>
-      <c r="H14" s="8">
+      <c r="H14" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I14" s="8" t="s">
+      <c r="I14" s="10" t="s">
         <v>52</v>
       </c>
       <c r="J14" s="14">
@@ -8585,7 +8585,7 @@
       <c r="K14" s="14">
         <v>968237.39</v>
       </c>
-      <c r="L14" s="8">
+      <c r="L14" s="10">
         <v>0.0</v>
       </c>
       <c r="AB14" s="2"/>
@@ -8597,32 +8597,32 @@
       <c r="AH14" s="2"/>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="s">
+      <c r="A15" s="10" t="s">
         <v>82</v>
       </c>
-      <c r="B15" s="8" t="s">
+      <c r="B15" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="C15" s="8" t="s">
+      <c r="C15" s="10" t="s">
         <v>84</v>
       </c>
-      <c r="D15" s="8" t="s">
+      <c r="D15" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E15" s="12">
         <v>45924.0</v>
       </c>
-      <c r="F15" s="8" t="s">
+      <c r="F15" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G15" s="8">
+      <c r="G15" s="10">
         <v>12.0</v>
       </c>
-      <c r="H15" s="8">
+      <c r="H15" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I15" s="8" t="s">
-        <v>43</v>
+      <c r="I15" s="10" t="s">
+        <v>39</v>
       </c>
       <c r="J15" s="14">
         <v>1011677.95</v>
@@ -8630,7 +8630,7 @@
       <c r="K15" s="14">
         <v>1011677.95</v>
       </c>
-      <c r="L15" s="8">
+      <c r="L15" s="10">
         <v>0.0</v>
       </c>
       <c r="AB15" s="2"/>
@@ -8642,31 +8642,31 @@
       <c r="AH15" s="2"/>
     </row>
     <row r="16">
-      <c r="A16" s="8" t="s">
+      <c r="A16" s="10" t="s">
         <v>85</v>
       </c>
-      <c r="B16" s="8" t="s">
+      <c r="B16" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="C16" s="8" t="s">
+      <c r="C16" s="10" t="s">
         <v>86</v>
       </c>
-      <c r="D16" s="8" t="s">
+      <c r="D16" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E16" s="12">
         <v>45929.0</v>
       </c>
-      <c r="F16" s="8" t="s">
+      <c r="F16" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G16" s="8">
+      <c r="G16" s="10">
         <v>12.0</v>
       </c>
-      <c r="H16" s="8">
+      <c r="H16" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I16" s="8">
+      <c r="I16" s="10">
         <v>2048.0</v>
       </c>
       <c r="J16" s="14">
@@ -8687,37 +8687,37 @@
       <c r="AH16" s="2"/>
     </row>
     <row r="17">
-      <c r="A17" s="8" t="s">
-        <v>87</v>
-      </c>
-      <c r="B17" s="8" t="s">
+      <c r="A17" s="10" t="s">
         <v>88</v>
       </c>
-      <c r="C17" s="8" t="s">
+      <c r="B17" s="10" t="s">
         <v>89</v>
       </c>
-      <c r="D17" s="8" t="s">
+      <c r="C17" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="D17" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E17" s="12">
         <v>45930.0</v>
       </c>
-      <c r="F17" s="8" t="s">
+      <c r="F17" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G17" s="8">
+      <c r="G17" s="10">
         <v>12.0</v>
       </c>
-      <c r="H17" s="8">
+      <c r="H17" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I17" s="8">
+      <c r="I17" s="10">
         <v>2048.0</v>
       </c>
       <c r="J17" s="14">
         <v>34065.36</v>
       </c>
-      <c r="K17" s="8">
+      <c r="K17" s="10">
         <v>0.0</v>
       </c>
       <c r="L17" s="14">
@@ -8732,31 +8732,31 @@
       <c r="AH17" s="2"/>
     </row>
     <row r="18">
-      <c r="A18" s="8" t="s">
-        <v>91</v>
-      </c>
-      <c r="B18" s="8" t="s">
+      <c r="A18" s="10" t="s">
+        <v>93</v>
+      </c>
+      <c r="B18" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="C18" s="8" t="s">
-        <v>92</v>
-      </c>
-      <c r="D18" s="8" t="s">
+      <c r="C18" s="10" t="s">
+        <v>94</v>
+      </c>
+      <c r="D18" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E18" s="12">
         <v>45938.0</v>
       </c>
-      <c r="F18" s="8" t="s">
+      <c r="F18" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G18" s="8">
+      <c r="G18" s="10">
         <v>12.0</v>
       </c>
-      <c r="H18" s="8">
+      <c r="H18" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I18" s="8" t="s">
+      <c r="I18" s="10" t="s">
         <v>52</v>
       </c>
       <c r="J18" s="14">
@@ -8765,7 +8765,7 @@
       <c r="K18" s="14">
         <v>63746.85</v>
       </c>
-      <c r="L18" s="8">
+      <c r="L18" s="10">
         <v>0.0</v>
       </c>
       <c r="AB18" s="2"/>
@@ -8777,31 +8777,31 @@
       <c r="AH18" s="2"/>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="s">
-        <v>93</v>
-      </c>
-      <c r="B19" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="C19" s="8" t="s">
+      <c r="A19" s="10" t="s">
         <v>95</v>
       </c>
-      <c r="D19" s="8" t="s">
+      <c r="B19" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="C19" s="10" t="s">
+        <v>96</v>
+      </c>
+      <c r="D19" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E19" s="12">
         <v>45938.0</v>
       </c>
-      <c r="F19" s="8" t="s">
+      <c r="F19" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G19" s="8">
+      <c r="G19" s="10">
         <v>12.0</v>
       </c>
-      <c r="H19" s="8">
+      <c r="H19" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I19" s="8" t="s">
+      <c r="I19" s="10" t="s">
         <v>72</v>
       </c>
       <c r="J19" s="14">
@@ -8810,7 +8810,7 @@
       <c r="K19" s="14">
         <v>947931.1</v>
       </c>
-      <c r="L19" s="8">
+      <c r="L19" s="10">
         <v>0.0</v>
       </c>
       <c r="AB19" s="2"/>
@@ -8822,31 +8822,31 @@
       <c r="AH19" s="2"/>
     </row>
     <row r="20">
-      <c r="A20" s="8" t="s">
-        <v>97</v>
-      </c>
-      <c r="B20" s="8" t="s">
+      <c r="A20" s="10" t="s">
+        <v>99</v>
+      </c>
+      <c r="B20" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="C20" s="8" t="s">
-        <v>98</v>
-      </c>
-      <c r="D20" s="8" t="s">
+      <c r="C20" s="10" t="s">
+        <v>100</v>
+      </c>
+      <c r="D20" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E20" s="12">
         <v>45938.0</v>
       </c>
-      <c r="F20" s="8" t="s">
+      <c r="F20" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G20" s="8">
+      <c r="G20" s="10">
         <v>12.0</v>
       </c>
-      <c r="H20" s="8">
+      <c r="H20" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I20" s="8">
+      <c r="I20" s="10">
         <v>2048.0</v>
       </c>
       <c r="J20" s="14">
@@ -8855,7 +8855,7 @@
       <c r="K20" s="14">
         <v>259790.57</v>
       </c>
-      <c r="L20" s="8">
+      <c r="L20" s="10">
         <v>0.0</v>
       </c>
       <c r="AB20" s="2"/>
@@ -8867,31 +8867,31 @@
       <c r="AH20" s="2"/>
     </row>
     <row r="21">
-      <c r="A21" s="8" t="s">
-        <v>99</v>
-      </c>
-      <c r="B21" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="C21" s="8" t="s">
-        <v>100</v>
-      </c>
-      <c r="D21" s="8" t="s">
+      <c r="A21" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="B21" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="C21" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="D21" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E21" s="12">
         <v>45938.0</v>
       </c>
-      <c r="F21" s="8" t="s">
+      <c r="F21" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G21" s="8">
+      <c r="G21" s="10">
         <v>12.0</v>
       </c>
-      <c r="H21" s="8">
+      <c r="H21" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I21" s="8">
+      <c r="I21" s="10">
         <v>2048.0</v>
       </c>
       <c r="J21" s="14">
@@ -8900,7 +8900,7 @@
       <c r="K21" s="14">
         <v>170479.3</v>
       </c>
-      <c r="L21" s="8">
+      <c r="L21" s="10">
         <v>0.0</v>
       </c>
       <c r="AB21" s="2"/>
@@ -8912,31 +8912,31 @@
       <c r="AH21" s="2"/>
     </row>
     <row r="22">
-      <c r="A22" s="8" t="s">
-        <v>103</v>
-      </c>
-      <c r="B22" s="8" t="s">
-        <v>104</v>
-      </c>
-      <c r="C22" s="8" t="s">
-        <v>105</v>
-      </c>
-      <c r="D22" s="8" t="s">
+      <c r="A22" s="10" t="s">
+        <v>106</v>
+      </c>
+      <c r="B22" s="10" t="s">
+        <v>107</v>
+      </c>
+      <c r="C22" s="10" t="s">
+        <v>108</v>
+      </c>
+      <c r="D22" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E22" s="43">
+      <c r="E22" s="48">
         <v>45953.0</v>
       </c>
-      <c r="F22" s="8" t="s">
+      <c r="F22" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G22" s="8">
+      <c r="G22" s="10">
         <v>12.0</v>
       </c>
-      <c r="H22" s="8">
+      <c r="H22" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I22" s="8">
+      <c r="I22" s="10">
         <v>2000.0</v>
       </c>
       <c r="J22" s="14">
@@ -8957,32 +8957,32 @@
       <c r="AH22" s="2"/>
     </row>
     <row r="23">
-      <c r="A23" s="8" t="s">
-        <v>107</v>
-      </c>
-      <c r="B23" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="C23" s="8" t="s">
-        <v>109</v>
-      </c>
-      <c r="D23" s="8" t="s">
+      <c r="A23" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="B23" s="10" t="s">
+        <v>112</v>
+      </c>
+      <c r="C23" s="10" t="s">
+        <v>113</v>
+      </c>
+      <c r="D23" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E23" s="43">
+      <c r="E23" s="48">
         <v>45953.0</v>
       </c>
-      <c r="F23" s="8" t="s">
+      <c r="F23" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G23" s="8">
+      <c r="G23" s="10">
         <v>12.0</v>
       </c>
-      <c r="H23" s="8">
+      <c r="H23" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I23" s="8" t="s">
-        <v>110</v>
+      <c r="I23" s="10" t="s">
+        <v>115</v>
       </c>
       <c r="J23" s="14">
         <v>1000001.64</v>
@@ -8990,7 +8990,7 @@
       <c r="K23" s="14">
         <v>1000001.64</v>
       </c>
-      <c r="L23" s="8">
+      <c r="L23" s="10">
         <v>0.0</v>
       </c>
       <c r="AB23" s="2"/>
@@ -9002,31 +9002,31 @@
       <c r="AH23" s="2"/>
     </row>
     <row r="24">
-      <c r="A24" s="8" t="s">
-        <v>112</v>
-      </c>
-      <c r="B24" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="C24" s="8" t="s">
-        <v>113</v>
-      </c>
-      <c r="D24" s="8" t="s">
+      <c r="A24" s="10" t="s">
+        <v>117</v>
+      </c>
+      <c r="B24" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="C24" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="D24" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E24" s="43">
+      <c r="E24" s="48">
         <v>45953.0</v>
       </c>
-      <c r="F24" s="8" t="s">
+      <c r="F24" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G24" s="8">
+      <c r="G24" s="10">
         <v>12.0</v>
       </c>
-      <c r="H24" s="8">
+      <c r="H24" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I24" s="8">
+      <c r="I24" s="10">
         <v>2048.0</v>
       </c>
       <c r="J24" s="14">
@@ -9035,7 +9035,7 @@
       <c r="K24" s="14">
         <v>68405.66</v>
       </c>
-      <c r="L24" s="8">
+      <c r="L24" s="10">
         <v>0.0</v>
       </c>
       <c r="AB24" s="2"/>
@@ -9047,32 +9047,32 @@
       <c r="AH24" s="2"/>
     </row>
     <row r="25">
-      <c r="A25" s="8" t="s">
+      <c r="A25" s="10" t="s">
+        <v>122</v>
+      </c>
+      <c r="B25" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="C25" s="10" t="s">
+        <v>124</v>
+      </c>
+      <c r="D25" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="E25" s="48">
+        <v>45975.0</v>
+      </c>
+      <c r="F25" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="G25" s="10">
+        <v>12.0</v>
+      </c>
+      <c r="H25" s="10">
+        <v>339039.0</v>
+      </c>
+      <c r="I25" s="10" t="s">
         <v>115</v>
-      </c>
-      <c r="B25" s="8" t="s">
-        <v>116</v>
-      </c>
-      <c r="C25" s="8" t="s">
-        <v>117</v>
-      </c>
-      <c r="D25" s="8" t="s">
-        <v>4</v>
-      </c>
-      <c r="E25" s="43">
-        <v>45975.0</v>
-      </c>
-      <c r="F25" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="G25" s="8">
-        <v>12.0</v>
-      </c>
-      <c r="H25" s="8">
-        <v>339039.0</v>
-      </c>
-      <c r="I25" s="8" t="s">
-        <v>110</v>
       </c>
       <c r="J25" s="14">
         <v>1157673.06</v>
@@ -9080,7 +9080,7 @@
       <c r="K25" s="14">
         <v>1157673.06</v>
       </c>
-      <c r="L25" s="8">
+      <c r="L25" s="10">
         <v>0.0</v>
       </c>
       <c r="AB25" s="2"/>
@@ -9092,31 +9092,31 @@
       <c r="AH25" s="2"/>
     </row>
     <row r="26">
-      <c r="A26" s="8" t="s">
-        <v>118</v>
-      </c>
-      <c r="B26" s="8" t="s">
+      <c r="A26" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="B26" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="C26" s="8" t="s">
-        <v>119</v>
-      </c>
-      <c r="D26" s="8" t="s">
+      <c r="C26" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="D26" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E26" s="43">
+      <c r="E26" s="48">
         <v>45989.0</v>
       </c>
-      <c r="F26" s="8" t="s">
+      <c r="F26" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G26" s="8">
+      <c r="G26" s="10">
         <v>12.0</v>
       </c>
-      <c r="H26" s="8">
+      <c r="H26" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I26" s="8">
+      <c r="I26" s="10">
         <v>2048.0</v>
       </c>
       <c r="J26" s="14">
@@ -9125,7 +9125,7 @@
       <c r="K26" s="14">
         <v>34065.36</v>
       </c>
-      <c r="L26" s="8">
+      <c r="L26" s="10">
         <v>0.0</v>
       </c>
       <c r="AB26" s="2"/>
@@ -9137,31 +9137,31 @@
       <c r="AH26" s="2"/>
     </row>
     <row r="27">
-      <c r="A27" s="8" t="s">
-        <v>122</v>
-      </c>
-      <c r="B27" s="8" t="s">
-        <v>123</v>
-      </c>
-      <c r="C27" s="8" t="s">
-        <v>124</v>
-      </c>
-      <c r="D27" s="8" t="s">
+      <c r="A27" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="B27" s="10" t="s">
+        <v>132</v>
+      </c>
+      <c r="C27" s="10" t="s">
+        <v>133</v>
+      </c>
+      <c r="D27" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E27" s="12">
         <v>46104.0</v>
       </c>
-      <c r="F27" s="8" t="s">
+      <c r="F27" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G27" s="8">
+      <c r="G27" s="10">
         <v>12.0</v>
       </c>
-      <c r="H27" s="8">
+      <c r="H27" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I27" s="8">
+      <c r="I27" s="10">
         <v>2048.0</v>
       </c>
       <c r="J27" s="14">
@@ -9182,37 +9182,37 @@
       <c r="AH27" s="2"/>
     </row>
     <row r="28">
-      <c r="A28" s="8" t="s">
-        <v>126</v>
-      </c>
-      <c r="B28" s="8" t="s">
-        <v>127</v>
-      </c>
-      <c r="C28" s="8" t="s">
-        <v>128</v>
-      </c>
-      <c r="D28" s="8" t="s">
+      <c r="A28" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="B28" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="C28" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="D28" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E28" s="12">
         <v>46120.0</v>
       </c>
-      <c r="F28" s="8" t="s">
+      <c r="F28" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G28" s="8">
+      <c r="G28" s="10">
         <v>12.0</v>
       </c>
-      <c r="H28" s="8">
+      <c r="H28" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I28" s="8" t="s">
+      <c r="I28" s="10" t="s">
         <v>48</v>
       </c>
       <c r="J28" s="14">
         <v>1912292.52</v>
       </c>
-      <c r="K28" s="8">
+      <c r="K28" s="10">
         <v>0.0</v>
       </c>
       <c r="L28" s="14">
@@ -9227,37 +9227,37 @@
       <c r="AH28" s="2"/>
     </row>
     <row r="29">
-      <c r="A29" s="8" t="s">
-        <v>130</v>
-      </c>
-      <c r="B29" s="8" t="s">
-        <v>131</v>
-      </c>
-      <c r="C29" s="8" t="s">
-        <v>132</v>
-      </c>
-      <c r="D29" s="8" t="s">
+      <c r="A29" s="10" t="s">
+        <v>142</v>
+      </c>
+      <c r="B29" s="10" t="s">
+        <v>143</v>
+      </c>
+      <c r="C29" s="10" t="s">
+        <v>144</v>
+      </c>
+      <c r="D29" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E29" s="12">
         <v>46196.0</v>
       </c>
-      <c r="F29" s="8" t="s">
+      <c r="F29" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G29" s="8">
+      <c r="G29" s="10">
         <v>12.0</v>
       </c>
-      <c r="H29" s="8">
+      <c r="H29" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I29" s="8">
+      <c r="I29" s="10">
         <v>2048.0</v>
       </c>
       <c r="J29" s="14">
         <v>1496713.48</v>
       </c>
-      <c r="K29" s="8">
+      <c r="K29" s="10">
         <v>0.0</v>
       </c>
       <c r="L29" s="14">
@@ -9272,37 +9272,37 @@
       <c r="AH29" s="2"/>
     </row>
     <row r="30">
-      <c r="A30" s="8" t="s">
-        <v>135</v>
-      </c>
-      <c r="B30" s="8" t="s">
-        <v>136</v>
-      </c>
-      <c r="C30" s="8" t="s">
-        <v>137</v>
-      </c>
-      <c r="D30" s="8" t="s">
+      <c r="A30" s="10" t="s">
+        <v>147</v>
+      </c>
+      <c r="B30" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="C30" s="10" t="s">
+        <v>149</v>
+      </c>
+      <c r="D30" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E30" s="12">
         <v>46205.0</v>
       </c>
-      <c r="F30" s="8" t="s">
+      <c r="F30" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G30" s="8">
+      <c r="G30" s="10">
         <v>12.0</v>
       </c>
-      <c r="H30" s="8">
+      <c r="H30" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I30" s="8" t="s">
-        <v>43</v>
+      <c r="I30" s="10" t="s">
+        <v>39</v>
       </c>
       <c r="J30" s="14">
         <v>624166.14</v>
       </c>
-      <c r="K30" s="8">
+      <c r="K30" s="10">
         <v>0.0</v>
       </c>
       <c r="L30" s="14">
@@ -9317,37 +9317,37 @@
       <c r="AH30" s="2"/>
     </row>
     <row r="31">
-      <c r="A31" s="8" t="s">
-        <v>139</v>
-      </c>
-      <c r="B31" s="8" t="s">
-        <v>140</v>
-      </c>
-      <c r="C31" s="8" t="s">
-        <v>141</v>
-      </c>
-      <c r="D31" s="8" t="s">
+      <c r="A31" s="10" t="s">
+        <v>152</v>
+      </c>
+      <c r="B31" s="10" t="s">
+        <v>153</v>
+      </c>
+      <c r="C31" s="10" t="s">
+        <v>154</v>
+      </c>
+      <c r="D31" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E31" s="12">
         <v>46205.0</v>
       </c>
-      <c r="F31" s="8" t="s">
+      <c r="F31" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G31" s="8">
+      <c r="G31" s="10">
         <v>12.0</v>
       </c>
-      <c r="H31" s="8">
+      <c r="H31" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I31" s="8" t="s">
-        <v>110</v>
+      <c r="I31" s="10" t="s">
+        <v>115</v>
       </c>
       <c r="J31" s="14">
         <v>18462.36</v>
       </c>
-      <c r="K31" s="8">
+      <c r="K31" s="10">
         <v>0.0</v>
       </c>
       <c r="L31" s="14">
@@ -9362,37 +9362,37 @@
       <c r="AH31" s="2"/>
     </row>
     <row r="32">
-      <c r="A32" s="8" t="s">
-        <v>143</v>
-      </c>
-      <c r="B32" s="8" t="s">
-        <v>140</v>
+      <c r="A32" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="B32" s="10" t="s">
+        <v>153</v>
       </c>
       <c r="C32" s="14" t="s">
-        <v>144</v>
-      </c>
-      <c r="D32" s="8" t="s">
+        <v>159</v>
+      </c>
+      <c r="D32" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E32" s="12">
         <v>46213.0</v>
       </c>
-      <c r="F32" s="8" t="s">
+      <c r="F32" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G32" s="8">
+      <c r="G32" s="10">
         <v>12.0</v>
       </c>
-      <c r="H32" s="8">
+      <c r="H32" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I32" s="8" t="s">
-        <v>110</v>
+      <c r="I32" s="10" t="s">
+        <v>115</v>
       </c>
       <c r="J32" s="14">
         <v>1530656.62</v>
       </c>
-      <c r="K32" s="8">
+      <c r="K32" s="10">
         <v>0.0</v>
       </c>
       <c r="L32" s="14">
@@ -9407,37 +9407,37 @@
       <c r="AH32" s="2"/>
     </row>
     <row r="33">
-      <c r="A33" s="8" t="s">
-        <v>147</v>
-      </c>
-      <c r="B33" s="8" t="s">
-        <v>131</v>
+      <c r="A33" s="10" t="s">
+        <v>163</v>
+      </c>
+      <c r="B33" s="10" t="s">
+        <v>143</v>
       </c>
       <c r="C33" s="14" t="s">
-        <v>148</v>
-      </c>
-      <c r="D33" s="8" t="s">
+        <v>164</v>
+      </c>
+      <c r="D33" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E33" s="12">
         <v>46227.0</v>
       </c>
-      <c r="F33" s="8" t="s">
+      <c r="F33" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G33" s="8">
+      <c r="G33" s="10">
         <v>12.0</v>
       </c>
-      <c r="H33" s="8">
+      <c r="H33" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I33" s="8">
+      <c r="I33" s="10">
         <v>2048.0</v>
       </c>
       <c r="J33" s="14">
         <v>173846.38</v>
       </c>
-      <c r="K33" s="8">
+      <c r="K33" s="10">
         <v>0.0</v>
       </c>
       <c r="L33" s="14">
@@ -9452,37 +9452,37 @@
       <c r="AH33" s="2"/>
     </row>
     <row r="34">
-      <c r="A34" s="8" t="s">
-        <v>151</v>
-      </c>
-      <c r="B34" s="8" t="s">
-        <v>152</v>
-      </c>
-      <c r="C34" s="8" t="s">
-        <v>153</v>
-      </c>
-      <c r="D34" s="8" t="s">
+      <c r="A34" s="10" t="s">
+        <v>169</v>
+      </c>
+      <c r="B34" s="10" t="s">
+        <v>170</v>
+      </c>
+      <c r="C34" s="10" t="s">
+        <v>171</v>
+      </c>
+      <c r="D34" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E34" s="12">
         <v>46240.0</v>
       </c>
-      <c r="F34" s="8" t="s">
+      <c r="F34" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G34" s="8">
+      <c r="G34" s="10">
         <v>12.0</v>
       </c>
-      <c r="H34" s="8">
+      <c r="H34" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I34" s="8" t="s">
-        <v>155</v>
+      <c r="I34" s="10" t="s">
+        <v>173</v>
       </c>
       <c r="J34" s="14">
         <v>236343.68</v>
       </c>
-      <c r="K34" s="8">
+      <c r="K34" s="10">
         <v>0.0</v>
       </c>
       <c r="L34" s="14">

</xml_diff>

<commit_message>
Atualização automática: pagamentos (24/08/2026 10:56)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/01_Bases_Originais/005_CELOG_2025/005_CELOG-PAMALS_2025 online.xlsx
+++ b/Contrato 005/Dashboard/01_Bases_Originais/005_CELOG_2025/005_CELOG-PAMALS_2025 online.xlsx
@@ -33,15 +33,15 @@
     <t>Saldo</t>
   </si>
   <si>
+    <t>Controle de pagamentos</t>
+  </si>
+  <si>
     <t>2025NE000005</t>
   </si>
   <si>
     <t>C25375</t>
   </si>
   <si>
-    <t>Controle de pagamentos</t>
-  </si>
-  <si>
     <t>Ordenador de Despesas</t>
   </si>
   <si>
@@ -69,109 +69,112 @@
     <t>Número Contrato</t>
   </si>
   <si>
+    <t>UG Executora</t>
+  </si>
+  <si>
+    <t>UG Responsável</t>
+  </si>
+  <si>
+    <t>UG Fiscalizadora</t>
+  </si>
+  <si>
+    <t>Prazo Final de Execução</t>
+  </si>
+  <si>
     <t>2025NE000371</t>
   </si>
   <si>
+    <t>Prazo Final de Vigência</t>
+  </si>
+  <si>
     <t>25E0389</t>
   </si>
   <si>
-    <t>UG Executora</t>
-  </si>
-  <si>
-    <t>UG Responsável</t>
-  </si>
-  <si>
-    <t>UG Fiscalizadora</t>
-  </si>
-  <si>
-    <t>Prazo Final de Execução</t>
-  </si>
-  <si>
-    <t>Prazo Final de Vigência</t>
-  </si>
-  <si>
     <t>Status</t>
   </si>
   <si>
     <t>Ação</t>
   </si>
   <si>
+    <t>PAG</t>
+  </si>
+  <si>
+    <t>Moeda</t>
+  </si>
+  <si>
+    <t>Valor Total do Contrato</t>
+  </si>
+  <si>
+    <t>Valor a Empenhar</t>
+  </si>
+  <si>
+    <t>Valor Empenhado</t>
+  </si>
+  <si>
+    <t>Valor Liquidado</t>
+  </si>
+  <si>
+    <t>Saldo (Valor a Faturar)</t>
+  </si>
+  <si>
+    <t>Fornecedor</t>
+  </si>
+  <si>
+    <t>Tipo Despesa /Receita</t>
+  </si>
+  <si>
+    <t>Abrir</t>
+  </si>
+  <si>
+    <t>Editar</t>
+  </si>
+  <si>
     <t>2025NE000413</t>
   </si>
   <si>
     <t>C25501</t>
   </si>
   <si>
-    <t>PAG</t>
-  </si>
-  <si>
     <t>25E0403</t>
   </si>
   <si>
-    <t>Moeda</t>
-  </si>
-  <si>
-    <t>Valor Total do Contrato</t>
-  </si>
-  <si>
-    <t>Valor a Empenhar</t>
+    <t>005/CELOG-PAMALS/2025</t>
+  </si>
+  <si>
+    <t>CELOG</t>
   </si>
   <si>
     <t>20SP</t>
   </si>
   <si>
-    <t>Valor Empenhado</t>
-  </si>
-  <si>
-    <t>Valor Liquidado</t>
-  </si>
-  <si>
-    <t>Saldo (Valor a Faturar)</t>
-  </si>
-  <si>
-    <t>Fornecedor</t>
-  </si>
-  <si>
-    <t>Tipo Despesa /Receita</t>
-  </si>
-  <si>
-    <t>Abrir</t>
-  </si>
-  <si>
-    <t>Editar</t>
+    <t>PAMALS</t>
   </si>
   <si>
     <t>2025NE000414</t>
   </si>
   <si>
-    <t>005/CELOG-PAMALS/2025</t>
+    <t>Vigente</t>
   </si>
   <si>
     <t>C25525</t>
   </si>
   <si>
+    <t>2048 20YJ 21EM 219C 20SP 20X7 2000</t>
+  </si>
+  <si>
     <t>25E0431</t>
   </si>
   <si>
-    <t>CELOG</t>
-  </si>
-  <si>
-    <t>PAMALS</t>
+    <t>67101.001510/2024-12</t>
+  </si>
+  <si>
+    <t>R$</t>
   </si>
   <si>
     <t>21EM</t>
   </si>
   <si>
-    <t>Vigente</t>
-  </si>
-  <si>
-    <t>2048 20YJ 21EM 219C 20SP 20X7 2000</t>
-  </si>
-  <si>
-    <t>67101.001510/2024-12</t>
-  </si>
-  <si>
-    <t>R$</t>
+    <t>VEE ONE-MANUTENCAO E SERVICOS TECNICOS LTDA</t>
   </si>
   <si>
     <t>2025NE000559</t>
@@ -183,9 +186,6 @@
     <t>25E0524</t>
   </si>
   <si>
-    <t>VEE ONE-MANUTENCAO E SERVICOS TECNICOS LTDA</t>
-  </si>
-  <si>
     <t>20X7</t>
   </si>
   <si>
@@ -195,12 +195,48 @@
     <t>25E0731</t>
   </si>
   <si>
+    <t>Módulo</t>
+  </si>
+  <si>
+    <t>Referência</t>
+  </si>
+  <si>
+    <t>Nº recibo</t>
+  </si>
+  <si>
+    <t>Nº</t>
+  </si>
+  <si>
+    <t>Data</t>
+  </si>
+  <si>
     <t>2025NE000774</t>
   </si>
   <si>
     <t>25E0737</t>
   </si>
   <si>
+    <t>Empenho</t>
+  </si>
+  <si>
+    <t>Observações</t>
+  </si>
+  <si>
+    <t>Vencimento</t>
+  </si>
+  <si>
+    <t>Valor das Nfs</t>
+  </si>
+  <si>
+    <t>Ordem de Pagamento</t>
+  </si>
+  <si>
+    <t>Faturado</t>
+  </si>
+  <si>
+    <t>Pendente</t>
+  </si>
+  <si>
     <t>2025NE000843</t>
   </si>
   <si>
@@ -213,34 +249,19 @@
     <t>219C</t>
   </si>
   <si>
-    <t>Módulo</t>
-  </si>
-  <si>
-    <t>Referência</t>
+    <t>FEV/25</t>
   </si>
   <si>
     <t>2025NE001065</t>
   </si>
   <si>
-    <t>Nº recibo</t>
-  </si>
-  <si>
     <t>25E0999</t>
   </si>
   <si>
-    <t>Nº</t>
-  </si>
-  <si>
-    <t>Data</t>
-  </si>
-  <si>
-    <t>Empenho</t>
-  </si>
-  <si>
-    <t>Observações</t>
-  </si>
-  <si>
-    <t>Vencimento</t>
+    <t>-</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025NE000369 </t>
   </si>
   <si>
     <t>2025NE001200</t>
@@ -252,16 +273,7 @@
     <t>25E1128</t>
   </si>
   <si>
-    <t>Valor das Nfs</t>
-  </si>
-  <si>
-    <t>Ordem de Pagamento</t>
-  </si>
-  <si>
-    <t>Faturado</t>
-  </si>
-  <si>
-    <t>Pendente</t>
+    <t>2025NP001980</t>
   </si>
   <si>
     <t>2025NE001598</t>
@@ -273,31 +285,25 @@
     <t>25E1446</t>
   </si>
   <si>
-    <t>FEV/25</t>
-  </si>
-  <si>
     <t>2025NE001627</t>
   </si>
   <si>
-    <t>-</t>
-  </si>
-  <si>
     <t>25E1475</t>
   </si>
   <si>
+    <t>MAR/25</t>
+  </si>
+  <si>
     <t>2025NE001629</t>
   </si>
   <si>
-    <t xml:space="preserve">2025NE000369 </t>
-  </si>
-  <si>
     <t>C25820</t>
   </si>
   <si>
     <t>25E1477</t>
   </si>
   <si>
-    <t>2025NP001980</t>
+    <t>2025NE000367, 2025NE000369, 2025NE000371, 2025NE000413</t>
   </si>
   <si>
     <t>2025NE001687</t>
@@ -306,22 +312,28 @@
     <t>25E1535</t>
   </si>
   <si>
+    <t>2025NP001979</t>
+  </si>
+  <si>
     <t>2025NE001688</t>
   </si>
   <si>
     <t>25E1536</t>
   </si>
   <si>
+    <t>ABR/25</t>
+  </si>
+  <si>
+    <t>2025NE000413, 2025NE000414, 2025NE000559</t>
+  </si>
+  <si>
     <t>2025NE001689</t>
   </si>
   <si>
     <t>25E1537</t>
   </si>
   <si>
-    <t>MAR/25</t>
-  </si>
-  <si>
-    <t>2025NE000367, 2025NE000369, 2025NE000371, 2025NE000413</t>
+    <t>2025NP002341</t>
   </si>
   <si>
     <t>2025NE001690</t>
@@ -330,7 +342,7 @@
     <t>25E1538</t>
   </si>
   <si>
-    <t>2025NP001979</t>
+    <t>MAI/25</t>
   </si>
   <si>
     <t>2025NE001823</t>
@@ -342,10 +354,7 @@
     <t>25E1666</t>
   </si>
   <si>
-    <t>ABR/25</t>
-  </si>
-  <si>
-    <t>2025NE000413, 2025NE000414, 2025NE000559</t>
+    <t>2025NP002884</t>
   </si>
   <si>
     <t>2025NE001828</t>
@@ -357,40 +366,10 @@
     <t>25E1667</t>
   </si>
   <si>
-    <t>2025NP002341</t>
+    <t>JUN/25</t>
   </si>
   <si>
     <t>20YJ</t>
-  </si>
-  <si>
-    <t>MAI/25</t>
-  </si>
-  <si>
-    <t>2025NE001830</t>
-  </si>
-  <si>
-    <t>25E1669</t>
-  </si>
-  <si>
-    <t>2025NP002884</t>
-  </si>
-  <si>
-    <t>2025NE002200</t>
-  </si>
-  <si>
-    <t>C25863</t>
-  </si>
-  <si>
-    <t>25E2021</t>
-  </si>
-  <si>
-    <t>JUN/25</t>
-  </si>
-  <si>
-    <t>2025NE002237</t>
-  </si>
-  <si>
-    <t>25E2058</t>
   </si>
   <si>
     <t>2025NE000005,
@@ -399,25 +378,52 @@
 2025NE000774</t>
   </si>
   <si>
+    <t>2025NE001830</t>
+  </si>
+  <si>
+    <t>25E1669</t>
+  </si>
+  <si>
     <t>2025NP400522</t>
   </si>
   <si>
+    <t>JUL/25</t>
+  </si>
+  <si>
+    <t>2025NE002200</t>
+  </si>
+  <si>
+    <t>C25863</t>
+  </si>
+  <si>
+    <t>25E2021</t>
+  </si>
+  <si>
+    <t>2025NE000843, 2025NE001200</t>
+  </si>
+  <si>
+    <t>2025NP003724</t>
+  </si>
+  <si>
+    <t>2025NE002237</t>
+  </si>
+  <si>
+    <t>25E2058</t>
+  </si>
+  <si>
+    <t>AGO/25</t>
+  </si>
+  <si>
     <t>2026NE000330</t>
   </si>
   <si>
-    <t>JUL/25</t>
-  </si>
-  <si>
     <t>C26163</t>
   </si>
   <si>
     <t>26E0320</t>
   </si>
   <si>
-    <t>2025NE000843, 2025NE001200</t>
-  </si>
-  <si>
-    <t>2025NP003724</t>
+    <t>2025NP004558</t>
   </si>
   <si>
     <t>2026NE000388</t>
@@ -429,28 +435,22 @@
     <t>26E0375</t>
   </si>
   <si>
-    <t>AGO/25</t>
-  </si>
-  <si>
-    <t>2025NP004558</t>
+    <t>SET/25</t>
   </si>
   <si>
     <t>2026NE000748</t>
-  </si>
-  <si>
-    <t>C26312</t>
-  </si>
-  <si>
-    <t>26E0709</t>
-  </si>
-  <si>
-    <t>SET/25</t>
   </si>
   <si>
     <t>2025NE001688 
 2025NE001828</t>
   </si>
   <si>
+    <t>C26312</t>
+  </si>
+  <si>
+    <t>26E0709</t>
+  </si>
+  <si>
     <t>2025NP004897</t>
   </si>
   <si>
@@ -460,73 +460,73 @@
     <t>C26324</t>
   </si>
   <si>
+    <t>26E0776</t>
+  </si>
+  <si>
     <t>OUT/25</t>
   </si>
   <si>
-    <t>26E0776</t>
-  </si>
-  <si>
     <t>2025NE001688, 2025NE001828, 2025NE002200</t>
   </si>
   <si>
+    <t>2026NE000817</t>
+  </si>
+  <si>
+    <t>C26326</t>
+  </si>
+  <si>
+    <t>26E0777</t>
+  </si>
+  <si>
     <t>2025NP004932</t>
   </si>
   <si>
-    <t>2026NE000817</t>
-  </si>
-  <si>
-    <t>C26326</t>
+    <t>2026NE000842</t>
   </si>
   <si>
     <t>NOV/25</t>
   </si>
   <si>
-    <t>26E0777</t>
+    <t>26E0803</t>
   </si>
   <si>
     <t>2025NE001687, 2025NE001689, 2025NE001690, 2025NE001823, 2025NE001830, 2025NE002237</t>
   </si>
   <si>
+    <t>2026NE000944</t>
+  </si>
+  <si>
     <t>2026NP400440</t>
   </si>
   <si>
-    <t>2026NE000842</t>
-  </si>
-  <si>
-    <t>26E0803</t>
+    <t>26E0906</t>
+  </si>
+  <si>
+    <t>2026NE001015</t>
+  </si>
+  <si>
+    <t>C26363</t>
+  </si>
+  <si>
+    <t>26E0959</t>
   </si>
   <si>
     <t>DEZ/25</t>
   </si>
   <si>
+    <t>20XV</t>
+  </si>
+  <si>
     <t>2025NE001065, 2025NE002200</t>
   </si>
   <si>
     <t>2026NP400412</t>
   </si>
   <si>
-    <t>2026NE000944</t>
-  </si>
-  <si>
-    <t>26E0906</t>
-  </si>
-  <si>
     <t>JAN/26</t>
   </si>
   <si>
     <t>2026NP401035</t>
-  </si>
-  <si>
-    <t>2026NE001015</t>
-  </si>
-  <si>
-    <t>C26363</t>
-  </si>
-  <si>
-    <t>26E0959</t>
-  </si>
-  <si>
-    <t>20XV</t>
   </si>
   <si>
     <t>FEV/26</t>
@@ -695,8 +695,8 @@
     <numFmt numFmtId="166" formatCode="dd/MM/yyyy"/>
     <numFmt numFmtId="167" formatCode="R$ #,##0.00"/>
     <numFmt numFmtId="168" formatCode="[$R$-416]\ #,##0.00;[RED]\-[$R$-416]\ #,##0.00"/>
-    <numFmt numFmtId="169" formatCode="d/m/yyyy"/>
-    <numFmt numFmtId="170" formatCode="MM/DD/YY"/>
+    <numFmt numFmtId="169" formatCode="MM/DD/YY"/>
+    <numFmt numFmtId="170" formatCode="d/m/yyyy"/>
     <numFmt numFmtId="171" formatCode="[$R$ -416]#,##0.00"/>
     <numFmt numFmtId="172" formatCode="_([$R$ -416]* #,##0.00_);_([$R$ -416]* \(#,##0.00\);_([$R$ -416]* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
@@ -891,36 +891,36 @@
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="3" fontId="2" numFmtId="0" xfId="0" applyFill="1" applyFont="1"/>
+    <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyFill="1" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyFill="1" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="11" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
     <xf borderId="0" fillId="5" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="4" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="11" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="4" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
@@ -941,11 +941,11 @@
     <xf borderId="0" fillId="6" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="right" readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="4" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="right" readingOrder="0"/>
+    </xf>
     <xf borderId="1" fillId="0" fontId="5" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="4" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="right" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="1"/>
@@ -971,7 +971,6 @@
     <xf borderId="1" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="165" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="1" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
@@ -990,6 +989,7 @@
     <xf borderId="1" fillId="0" fontId="8" numFmtId="166" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="165" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="1" fillId="7" fontId="9" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
@@ -1003,17 +1003,17 @@
     <xf borderId="1" fillId="8" fontId="9" numFmtId="168" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="169" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
     <xf borderId="1" fillId="0" fontId="8" numFmtId="166" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="8" numFmtId="170" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="8" numFmtId="169" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="7" fontId="9" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="170" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
@@ -1437,22 +1437,22 @@
       <c r="S1" s="1"/>
       <c r="T1" s="1"/>
       <c r="U1" s="1"/>
-      <c r="V1" s="5"/>
+      <c r="V1" s="3"/>
     </row>
     <row r="2" ht="59.25" customHeight="1">
-      <c r="A2" s="7"/>
-      <c r="B2" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="V2" s="11"/>
-      <c r="W2" s="13"/>
-      <c r="X2" s="13"/>
-      <c r="Y2" s="13"/>
-      <c r="Z2" s="13"/>
-      <c r="AA2" s="13"/>
-      <c r="AB2" s="13"/>
-      <c r="AC2" s="13"/>
-      <c r="AD2" s="13"/>
+      <c r="A2" s="5"/>
+      <c r="B2" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="V2" s="9"/>
+      <c r="W2" s="11"/>
+      <c r="X2" s="11"/>
+      <c r="Y2" s="11"/>
+      <c r="Z2" s="11"/>
+      <c r="AA2" s="11"/>
+      <c r="AB2" s="11"/>
+      <c r="AC2" s="11"/>
+      <c r="AD2" s="11"/>
     </row>
     <row r="3" ht="12.75" customHeight="1">
       <c r="A3" s="1"/>
@@ -1476,7 +1476,7 @@
       <c r="S3" s="14"/>
       <c r="T3" s="14"/>
       <c r="U3" s="14"/>
-      <c r="V3" s="5"/>
+      <c r="V3" s="3"/>
     </row>
     <row r="4" ht="12.75" customHeight="1">
       <c r="A4" s="15"/>
@@ -1485,19 +1485,19 @@
         <v>12</v>
       </c>
       <c r="D4" s="16" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="16" t="s">
+      <c r="G4" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="F4" s="16" t="s">
-        <v>17</v>
-      </c>
-      <c r="G4" s="17" t="s">
+      <c r="H4" s="17" t="s">
         <v>18</v>
-      </c>
-      <c r="H4" s="17" t="s">
-        <v>19</v>
       </c>
       <c r="I4" s="16" t="s">
         <v>20</v>
@@ -1506,55 +1506,55 @@
         <v>21</v>
       </c>
       <c r="K4" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="L4" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="M4" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="L4" s="16" t="s">
+      <c r="N4" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="O4" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="M4" s="17" t="s">
+      <c r="P4" s="17" t="s">
         <v>27</v>
       </c>
-      <c r="N4" s="17" t="s">
+      <c r="Q4" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="O4" s="17" t="s">
+      <c r="R4" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="S4" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="P4" s="17" t="s">
+      <c r="T4" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="Q4" s="17" t="s">
+      <c r="U4" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="R4" s="16" t="s">
-        <v>33</v>
-      </c>
-      <c r="S4" s="16" t="s">
-        <v>34</v>
-      </c>
-      <c r="T4" s="16" t="s">
-        <v>35</v>
-      </c>
-      <c r="U4" s="16" t="s">
-        <v>36</v>
-      </c>
-      <c r="V4" s="5"/>
+      <c r="V4" s="3"/>
     </row>
     <row r="5" ht="12.75" customHeight="1">
       <c r="A5" s="15"/>
       <c r="B5" s="15"/>
       <c r="C5" s="18"/>
       <c r="D5" s="19" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="E5" s="19" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="F5" s="19" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G5" s="19" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="H5" s="20">
         <v>1564.0</v>
@@ -1563,42 +1563,42 @@
         <v>1564.0</v>
       </c>
       <c r="J5" s="19" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="K5" s="19" t="s">
+        <v>43</v>
+      </c>
+      <c r="L5" s="19" t="s">
         <v>45</v>
       </c>
-      <c r="L5" s="19" t="s">
+      <c r="M5" s="19" t="s">
         <v>46</v>
       </c>
-      <c r="M5" s="19" t="s">
-        <v>47</v>
-      </c>
-      <c r="N5" s="22">
+      <c r="N5" s="21">
         <v>9.165159737E7</v>
       </c>
-      <c r="O5" s="22">
+      <c r="O5" s="21">
         <v>7.254367932E7</v>
       </c>
-      <c r="P5" s="22">
+      <c r="P5" s="21">
         <v>1.910791805E7</v>
       </c>
-      <c r="Q5" s="22">
+      <c r="Q5" s="21">
         <v>8248487.61</v>
       </c>
-      <c r="R5" s="22">
+      <c r="R5" s="21">
         <v>1.085943044E7</v>
       </c>
       <c r="S5" s="19" t="s">
-        <v>51</v>
-      </c>
-      <c r="V5" s="5"/>
+        <v>48</v>
+      </c>
+      <c r="V5" s="3"/>
     </row>
     <row r="6" ht="12.75" customHeight="1">
       <c r="A6" s="15"/>
       <c r="B6" s="15"/>
       <c r="L6" s="23"/>
-      <c r="V6" s="5"/>
+      <c r="V6" s="3"/>
     </row>
     <row r="7" ht="12.75" customHeight="1">
       <c r="A7" s="24"/>
@@ -1617,81 +1617,81 @@
       <c r="N7" s="26"/>
       <c r="O7" s="26"/>
       <c r="P7" s="28"/>
-      <c r="V7" s="5"/>
+      <c r="V7" s="3"/>
     </row>
     <row r="8" ht="12.75" customHeight="1">
       <c r="A8" s="24"/>
       <c r="B8" s="24"/>
       <c r="C8" s="29" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="D8" s="29" t="s">
+        <v>56</v>
+      </c>
+      <c r="E8" s="30" t="s">
+        <v>57</v>
+      </c>
+      <c r="F8" s="29" t="s">
+        <v>58</v>
+      </c>
+      <c r="G8" s="29" t="s">
+        <v>59</v>
+      </c>
+      <c r="H8" s="29" t="s">
         <v>62</v>
       </c>
-      <c r="E8" s="30" t="s">
+      <c r="I8" s="30" t="s">
+        <v>63</v>
+      </c>
+      <c r="J8" s="29" t="s">
         <v>64</v>
       </c>
-      <c r="F8" s="29" t="s">
+      <c r="K8" s="29" t="s">
+        <v>65</v>
+      </c>
+      <c r="L8" s="31" t="s">
         <v>66</v>
       </c>
-      <c r="G8" s="29" t="s">
+      <c r="M8" s="30" t="s">
         <v>67</v>
       </c>
-      <c r="H8" s="29" t="s">
+      <c r="N8" s="29" t="s">
         <v>68</v>
-      </c>
-      <c r="I8" s="30" t="s">
-        <v>69</v>
-      </c>
-      <c r="J8" s="29" t="s">
-        <v>70</v>
-      </c>
-      <c r="K8" s="29" t="s">
-        <v>74</v>
-      </c>
-      <c r="L8" s="32" t="s">
-        <v>75</v>
-      </c>
-      <c r="M8" s="30" t="s">
-        <v>76</v>
-      </c>
-      <c r="N8" s="29" t="s">
-        <v>77</v>
       </c>
       <c r="O8" s="29"/>
       <c r="P8" s="28"/>
-      <c r="V8" s="5"/>
+      <c r="V8" s="3"/>
     </row>
     <row r="9" ht="19.5" customHeight="1">
       <c r="A9" s="24"/>
       <c r="B9" s="24"/>
-      <c r="C9" s="33">
+      <c r="C9" s="32">
         <v>1.0</v>
       </c>
-      <c r="D9" s="34" t="s">
-        <v>81</v>
-      </c>
-      <c r="E9" s="35" t="s">
-        <v>83</v>
-      </c>
-      <c r="F9" s="36">
+      <c r="D9" s="33" t="s">
+        <v>73</v>
+      </c>
+      <c r="E9" s="34" t="s">
+        <v>76</v>
+      </c>
+      <c r="F9" s="35">
         <v>594.0</v>
       </c>
-      <c r="G9" s="37">
+      <c r="G9" s="36">
         <v>45740.0</v>
       </c>
-      <c r="H9" s="36" t="s">
-        <v>86</v>
-      </c>
-      <c r="I9" s="37"/>
-      <c r="J9" s="37">
+      <c r="H9" s="35" t="s">
+        <v>77</v>
+      </c>
+      <c r="I9" s="36"/>
+      <c r="J9" s="36">
         <v>45778.0</v>
       </c>
       <c r="K9" s="38">
         <v>748504.24</v>
       </c>
-      <c r="L9" s="36" t="s">
-        <v>89</v>
+      <c r="L9" s="35" t="s">
+        <v>81</v>
       </c>
       <c r="M9" s="39">
         <f t="shared" ref="M9:M10" si="1">K9</f>
@@ -1700,36 +1700,36 @@
       <c r="N9" s="40"/>
       <c r="O9" s="26"/>
       <c r="P9" s="28"/>
-      <c r="V9" s="5"/>
+      <c r="V9" s="3"/>
     </row>
     <row r="10" ht="51.0" customHeight="1">
       <c r="A10" s="24"/>
       <c r="B10" s="24"/>
       <c r="C10" s="41"/>
-      <c r="D10" s="34" t="s">
-        <v>96</v>
-      </c>
-      <c r="E10" s="35" t="s">
-        <v>83</v>
-      </c>
-      <c r="F10" s="36">
+      <c r="D10" s="33" t="s">
+        <v>87</v>
+      </c>
+      <c r="E10" s="34" t="s">
+        <v>76</v>
+      </c>
+      <c r="F10" s="35">
         <v>620.0</v>
       </c>
-      <c r="G10" s="37">
+      <c r="G10" s="36">
         <v>45775.0</v>
       </c>
-      <c r="H10" s="36" t="s">
-        <v>97</v>
-      </c>
-      <c r="I10" s="37"/>
-      <c r="J10" s="37">
+      <c r="H10" s="35" t="s">
+        <v>91</v>
+      </c>
+      <c r="I10" s="36"/>
+      <c r="J10" s="36">
         <v>45806.0</v>
       </c>
       <c r="K10" s="38">
         <v>1110378.24</v>
       </c>
-      <c r="L10" s="36" t="s">
-        <v>100</v>
+      <c r="L10" s="35" t="s">
+        <v>94</v>
       </c>
       <c r="M10" s="39">
         <f t="shared" si="1"/>
@@ -1738,36 +1738,36 @@
       <c r="N10" s="42"/>
       <c r="O10" s="26"/>
       <c r="P10" s="28"/>
-      <c r="V10" s="5"/>
+      <c r="V10" s="3"/>
     </row>
     <row r="11" ht="12.75" customHeight="1">
       <c r="A11" s="24"/>
       <c r="B11" s="24"/>
       <c r="C11" s="41"/>
-      <c r="D11" s="34" t="s">
-        <v>104</v>
-      </c>
-      <c r="E11" s="35" t="s">
-        <v>83</v>
-      </c>
-      <c r="F11" s="36">
+      <c r="D11" s="33" t="s">
+        <v>97</v>
+      </c>
+      <c r="E11" s="34" t="s">
+        <v>76</v>
+      </c>
+      <c r="F11" s="35">
         <v>634.0</v>
       </c>
-      <c r="G11" s="37">
+      <c r="G11" s="36">
         <v>45799.0</v>
       </c>
-      <c r="H11" s="36" t="s">
-        <v>105</v>
-      </c>
-      <c r="I11" s="37"/>
-      <c r="J11" s="37">
+      <c r="H11" s="35" t="s">
+        <v>98</v>
+      </c>
+      <c r="I11" s="36"/>
+      <c r="J11" s="36">
         <v>45844.0</v>
       </c>
       <c r="K11" s="38">
         <v>974557.12</v>
       </c>
-      <c r="L11" s="35" t="s">
-        <v>109</v>
+      <c r="L11" s="34" t="s">
+        <v>101</v>
       </c>
       <c r="M11" s="39">
         <v>974557.12</v>
@@ -1775,36 +1775,36 @@
       <c r="N11" s="42"/>
       <c r="O11" s="26"/>
       <c r="P11" s="28"/>
-      <c r="V11" s="5"/>
+      <c r="V11" s="3"/>
     </row>
     <row r="12" ht="27.75" customHeight="1">
       <c r="A12" s="24"/>
       <c r="B12" s="24"/>
       <c r="C12" s="41"/>
-      <c r="D12" s="34" t="s">
-        <v>111</v>
-      </c>
-      <c r="E12" s="35" t="s">
-        <v>83</v>
-      </c>
-      <c r="F12" s="35">
+      <c r="D12" s="33" t="s">
+        <v>104</v>
+      </c>
+      <c r="E12" s="34" t="s">
+        <v>76</v>
+      </c>
+      <c r="F12" s="34">
         <v>660.0</v>
       </c>
-      <c r="G12" s="44">
+      <c r="G12" s="43">
         <v>45856.0</v>
       </c>
-      <c r="H12" s="45" t="s">
-        <v>57</v>
-      </c>
-      <c r="I12" s="37"/>
-      <c r="J12" s="37">
+      <c r="H12" s="44" t="s">
+        <v>69</v>
+      </c>
+      <c r="I12" s="36"/>
+      <c r="J12" s="36">
         <v>45891.0</v>
       </c>
-      <c r="K12" s="46">
+      <c r="K12" s="45">
         <v>1402001.34</v>
       </c>
       <c r="L12" s="47" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="M12" s="39">
         <v>1402001.34</v>
@@ -1812,36 +1812,36 @@
       <c r="N12" s="48"/>
       <c r="O12" s="26"/>
       <c r="P12" s="28"/>
-      <c r="V12" s="5"/>
+      <c r="V12" s="3"/>
     </row>
     <row r="13">
       <c r="A13" s="24"/>
       <c r="B13" s="24"/>
       <c r="C13" s="41"/>
       <c r="D13" s="49" t="s">
-        <v>118</v>
-      </c>
-      <c r="E13" s="35" t="s">
-        <v>83</v>
-      </c>
-      <c r="F13" s="36">
+        <v>112</v>
+      </c>
+      <c r="E13" s="34" t="s">
+        <v>76</v>
+      </c>
+      <c r="F13" s="35">
         <v>661.0</v>
       </c>
-      <c r="G13" s="37">
+      <c r="G13" s="36">
         <v>45856.0</v>
       </c>
-      <c r="H13" s="36" t="s">
-        <v>121</v>
-      </c>
-      <c r="I13" s="44"/>
-      <c r="J13" s="44">
+      <c r="H13" s="35" t="s">
+        <v>114</v>
+      </c>
+      <c r="I13" s="43"/>
+      <c r="J13" s="43">
         <v>45891.0</v>
       </c>
-      <c r="K13" s="46">
+      <c r="K13" s="45">
         <v>1223702.3</v>
       </c>
-      <c r="L13" s="35" t="s">
-        <v>122</v>
+      <c r="L13" s="34" t="s">
+        <v>117</v>
       </c>
       <c r="M13" s="39">
         <v>1223702.3</v>
@@ -1849,36 +1849,36 @@
       <c r="N13" s="48"/>
       <c r="O13" s="26"/>
       <c r="P13" s="50"/>
-      <c r="V13" s="5"/>
+      <c r="V13" s="3"/>
     </row>
     <row r="14">
       <c r="A14" s="24"/>
       <c r="B14" s="24"/>
       <c r="C14" s="41"/>
       <c r="D14" s="49" t="s">
-        <v>124</v>
-      </c>
-      <c r="E14" s="35" t="s">
-        <v>83</v>
-      </c>
-      <c r="F14" s="35">
+        <v>118</v>
+      </c>
+      <c r="E14" s="34" t="s">
+        <v>76</v>
+      </c>
+      <c r="F14" s="34">
         <v>688.0</v>
       </c>
-      <c r="G14" s="37">
+      <c r="G14" s="36">
         <v>45901.0</v>
       </c>
-      <c r="H14" s="35" t="s">
-        <v>127</v>
-      </c>
-      <c r="I14" s="44"/>
-      <c r="J14" s="44">
+      <c r="H14" s="34" t="s">
+        <v>122</v>
+      </c>
+      <c r="I14" s="43"/>
+      <c r="J14" s="43">
         <v>45938.0</v>
       </c>
-      <c r="K14" s="46">
+      <c r="K14" s="45">
         <v>1011677.95</v>
       </c>
-      <c r="L14" s="35" t="s">
-        <v>128</v>
+      <c r="L14" s="34" t="s">
+        <v>123</v>
       </c>
       <c r="M14" s="39">
         <v>1011677.95</v>
@@ -1886,71 +1886,71 @@
       <c r="N14" s="42"/>
       <c r="O14" s="26"/>
       <c r="P14" s="28"/>
-      <c r="V14" s="5"/>
+      <c r="V14" s="3"/>
     </row>
     <row r="15">
       <c r="A15" s="24"/>
       <c r="B15" s="24"/>
       <c r="C15" s="41"/>
       <c r="D15" s="49" t="s">
-        <v>132</v>
-      </c>
-      <c r="E15" s="35" t="s">
-        <v>83</v>
-      </c>
-      <c r="F15" s="35">
+        <v>126</v>
+      </c>
+      <c r="E15" s="34" t="s">
+        <v>76</v>
+      </c>
+      <c r="F15" s="34">
         <v>696.0</v>
       </c>
-      <c r="G15" s="37">
+      <c r="G15" s="36">
         <v>45923.0</v>
       </c>
-      <c r="H15" s="35" t="s">
-        <v>71</v>
-      </c>
-      <c r="I15" s="44"/>
-      <c r="J15" s="44">
+      <c r="H15" s="34" t="s">
+        <v>78</v>
+      </c>
+      <c r="I15" s="43"/>
+      <c r="J15" s="43">
         <v>45938.0</v>
       </c>
-      <c r="K15" s="46">
+      <c r="K15" s="45">
         <v>896744.06</v>
       </c>
-      <c r="L15" s="35" t="s">
-        <v>133</v>
+      <c r="L15" s="34" t="s">
+        <v>130</v>
       </c>
       <c r="M15" s="39">
         <v>896744.06</v>
       </c>
       <c r="N15" s="48"/>
       <c r="O15" s="26"/>
-      <c r="V15" s="5"/>
+      <c r="V15" s="3"/>
     </row>
     <row r="16">
       <c r="A16" s="24"/>
       <c r="B16" s="24"/>
       <c r="C16" s="41"/>
       <c r="D16" s="49" t="s">
-        <v>137</v>
-      </c>
-      <c r="E16" s="35" t="s">
-        <v>83</v>
-      </c>
-      <c r="F16" s="35">
+        <v>134</v>
+      </c>
+      <c r="E16" s="34" t="s">
+        <v>76</v>
+      </c>
+      <c r="F16" s="34">
         <v>704.0</v>
       </c>
-      <c r="G16" s="37">
+      <c r="G16" s="36">
         <v>45957.0</v>
       </c>
-      <c r="H16" s="35" t="s">
-        <v>138</v>
-      </c>
-      <c r="I16" s="44"/>
-      <c r="J16" s="44">
+      <c r="H16" s="34" t="s">
+        <v>136</v>
+      </c>
+      <c r="I16" s="43"/>
+      <c r="J16" s="43">
         <v>46003.0</v>
       </c>
-      <c r="K16" s="46">
+      <c r="K16" s="45">
         <v>919329.06</v>
       </c>
-      <c r="L16" s="35" t="s">
+      <c r="L16" s="34" t="s">
         <v>139</v>
       </c>
       <c r="M16" s="39">
@@ -1958,70 +1958,70 @@
       </c>
       <c r="N16" s="42"/>
       <c r="O16" s="26"/>
-      <c r="V16" s="5"/>
+      <c r="V16" s="3"/>
     </row>
     <row r="17">
       <c r="A17" s="24"/>
       <c r="B17" s="24"/>
       <c r="C17" s="41"/>
       <c r="D17" s="49" t="s">
-        <v>142</v>
-      </c>
-      <c r="E17" s="35"/>
-      <c r="F17" s="35">
+        <v>143</v>
+      </c>
+      <c r="E17" s="34"/>
+      <c r="F17" s="34">
         <v>705.0</v>
       </c>
-      <c r="G17" s="44">
+      <c r="G17" s="43">
         <v>45972.0</v>
       </c>
-      <c r="H17" s="35" t="s">
+      <c r="H17" s="34" t="s">
         <v>144</v>
       </c>
-      <c r="I17" s="35"/>
-      <c r="J17" s="44">
+      <c r="I17" s="34"/>
+      <c r="J17" s="43">
         <v>46016.0</v>
       </c>
-      <c r="K17" s="46">
+      <c r="K17" s="45">
         <v>1157009.26</v>
       </c>
-      <c r="L17" s="35" t="s">
-        <v>145</v>
+      <c r="L17" s="34" t="s">
+        <v>148</v>
       </c>
       <c r="M17" s="39">
         <v>1157009.26</v>
       </c>
       <c r="N17" s="51"/>
       <c r="O17" s="26"/>
-      <c r="V17" s="5"/>
+      <c r="V17" s="3"/>
     </row>
     <row r="18">
       <c r="A18" s="24"/>
       <c r="B18" s="24"/>
       <c r="C18" s="41"/>
       <c r="D18" s="49" t="s">
-        <v>148</v>
-      </c>
-      <c r="E18" s="35" t="s">
-        <v>83</v>
-      </c>
-      <c r="F18" s="35">
+        <v>150</v>
+      </c>
+      <c r="E18" s="34" t="s">
+        <v>76</v>
+      </c>
+      <c r="F18" s="34">
         <v>728.0</v>
       </c>
-      <c r="G18" s="44">
+      <c r="G18" s="43">
         <v>46008.0</v>
       </c>
-      <c r="H18" s="35" t="s">
-        <v>150</v>
-      </c>
-      <c r="I18" s="35"/>
-      <c r="J18" s="44">
+      <c r="H18" s="34" t="s">
+        <v>152</v>
+      </c>
+      <c r="I18" s="34"/>
+      <c r="J18" s="43">
         <v>46040.0</v>
       </c>
-      <c r="K18" s="46">
+      <c r="K18" s="45">
         <v>1214597.952</v>
       </c>
-      <c r="L18" s="35" t="s">
-        <v>151</v>
+      <c r="L18" s="34" t="s">
+        <v>154</v>
       </c>
       <c r="M18" s="39">
         <v>1214597.952</v>
@@ -2039,29 +2039,29 @@
       <c r="B19" s="24"/>
       <c r="C19" s="41"/>
       <c r="D19" s="49" t="s">
-        <v>154</v>
-      </c>
-      <c r="E19" s="35" t="s">
-        <v>83</v>
-      </c>
-      <c r="F19" s="35">
+        <v>159</v>
+      </c>
+      <c r="E19" s="34" t="s">
+        <v>76</v>
+      </c>
+      <c r="F19" s="34">
         <v>278.0</v>
       </c>
-      <c r="G19" s="44">
+      <c r="G19" s="43">
         <v>46042.0</v>
       </c>
-      <c r="H19" s="35" t="s">
-        <v>155</v>
-      </c>
-      <c r="I19" s="44"/>
-      <c r="J19" s="44">
+      <c r="H19" s="34" t="s">
+        <v>161</v>
+      </c>
+      <c r="I19" s="43"/>
+      <c r="J19" s="43">
         <v>46074.0</v>
       </c>
-      <c r="K19" s="46">
+      <c r="K19" s="45">
         <v>967082.09</v>
       </c>
-      <c r="L19" s="35" t="s">
-        <v>156</v>
+      <c r="L19" s="34" t="s">
+        <v>162</v>
       </c>
       <c r="M19" s="39">
         <v>967082.09</v>
@@ -2079,27 +2079,27 @@
       <c r="B20" s="24"/>
       <c r="C20" s="41"/>
       <c r="D20" s="49" t="s">
-        <v>159</v>
-      </c>
-      <c r="E20" s="35"/>
-      <c r="F20" s="35">
+        <v>163</v>
+      </c>
+      <c r="E20" s="34"/>
+      <c r="F20" s="34">
         <v>10.0</v>
       </c>
-      <c r="G20" s="44">
+      <c r="G20" s="43">
         <v>46078.0</v>
       </c>
-      <c r="H20" s="35" t="s">
-        <v>101</v>
-      </c>
-      <c r="I20" s="44"/>
-      <c r="J20" s="44">
+      <c r="H20" s="34" t="s">
+        <v>105</v>
+      </c>
+      <c r="I20" s="43"/>
+      <c r="J20" s="43">
         <v>46106.0</v>
       </c>
-      <c r="K20" s="46">
+      <c r="K20" s="45">
         <v>719561.08</v>
       </c>
-      <c r="L20" s="35" t="s">
-        <v>160</v>
+      <c r="L20" s="34" t="s">
+        <v>164</v>
       </c>
       <c r="M20" s="39">
         <v>719561.08</v>
@@ -2119,24 +2119,24 @@
       <c r="D21" s="49" t="s">
         <v>165</v>
       </c>
-      <c r="E21" s="35"/>
-      <c r="F21" s="35">
+      <c r="E21" s="34"/>
+      <c r="F21" s="34">
         <v>15.0</v>
       </c>
-      <c r="G21" s="44">
+      <c r="G21" s="43">
         <v>46094.0</v>
       </c>
-      <c r="H21" s="35" t="s">
+      <c r="H21" s="34" t="s">
         <v>166</v>
       </c>
-      <c r="I21" s="44"/>
-      <c r="J21" s="44">
+      <c r="I21" s="43"/>
+      <c r="J21" s="43">
         <v>46128.0</v>
       </c>
-      <c r="K21" s="46">
+      <c r="K21" s="45">
         <v>885881.08</v>
       </c>
-      <c r="L21" s="35" t="s">
+      <c r="L21" s="34" t="s">
         <v>167</v>
       </c>
       <c r="M21" s="39">
@@ -2157,24 +2157,24 @@
       <c r="D22" s="49" t="s">
         <v>168</v>
       </c>
-      <c r="E22" s="35"/>
-      <c r="F22" s="35">
+      <c r="E22" s="34"/>
+      <c r="F22" s="34">
         <v>28.0</v>
       </c>
-      <c r="G22" s="44">
+      <c r="G22" s="43">
         <v>46128.0</v>
       </c>
-      <c r="H22" s="35" t="s">
+      <c r="H22" s="34" t="s">
         <v>169</v>
       </c>
-      <c r="I22" s="44"/>
-      <c r="J22" s="44">
+      <c r="I22" s="43"/>
+      <c r="J22" s="43">
         <v>46164.0</v>
       </c>
-      <c r="K22" s="46" t="s">
+      <c r="K22" s="45" t="s">
         <v>170</v>
       </c>
-      <c r="L22" s="35" t="s">
+      <c r="L22" s="34" t="s">
         <v>171</v>
       </c>
       <c r="M22" s="39" t="s">
@@ -2195,24 +2195,24 @@
       <c r="D23" s="49" t="s">
         <v>172</v>
       </c>
-      <c r="E23" s="35"/>
-      <c r="F23" s="35">
+      <c r="E23" s="34"/>
+      <c r="F23" s="34">
         <v>33.0</v>
       </c>
-      <c r="G23" s="44">
+      <c r="G23" s="43">
         <v>46156.0</v>
       </c>
-      <c r="H23" s="35" t="s">
+      <c r="H23" s="34" t="s">
         <v>173</v>
       </c>
-      <c r="I23" s="44"/>
-      <c r="J23" s="44">
+      <c r="I23" s="43"/>
+      <c r="J23" s="43">
         <v>46191.0</v>
       </c>
-      <c r="K23" s="46">
+      <c r="K23" s="45">
         <v>1108954.4358333333</v>
       </c>
-      <c r="L23" s="35" t="s">
+      <c r="L23" s="34" t="s">
         <v>167</v>
       </c>
       <c r="M23" s="39">
@@ -2233,24 +2233,24 @@
       <c r="D24" s="49" t="s">
         <v>174</v>
       </c>
-      <c r="E24" s="35"/>
-      <c r="F24" s="35">
+      <c r="E24" s="34"/>
+      <c r="F24" s="34">
         <v>29.0</v>
       </c>
-      <c r="G24" s="44">
+      <c r="G24" s="43">
         <v>46149.0</v>
       </c>
-      <c r="H24" s="35" t="s">
+      <c r="H24" s="34" t="s">
         <v>173</v>
       </c>
-      <c r="I24" s="44"/>
-      <c r="J24" s="44">
+      <c r="I24" s="43"/>
+      <c r="J24" s="43">
         <v>46185.0</v>
       </c>
-      <c r="K24" s="46">
+      <c r="K24" s="45">
         <v>218206.1</v>
       </c>
-      <c r="L24" s="35" t="s">
+      <c r="L24" s="34" t="s">
         <v>175</v>
       </c>
       <c r="M24" s="39">
@@ -2271,24 +2271,24 @@
       <c r="D25" s="49" t="s">
         <v>176</v>
       </c>
-      <c r="E25" s="35"/>
-      <c r="F25" s="35">
+      <c r="E25" s="34"/>
+      <c r="F25" s="34">
         <v>40.0</v>
       </c>
-      <c r="G25" s="44">
+      <c r="G25" s="43">
         <v>46156.0</v>
       </c>
-      <c r="H25" s="35" t="s">
+      <c r="H25" s="34" t="s">
         <v>173</v>
       </c>
-      <c r="I25" s="44"/>
-      <c r="J25" s="44">
+      <c r="I25" s="43"/>
+      <c r="J25" s="43">
         <v>46191.0</v>
       </c>
-      <c r="K25" s="46">
+      <c r="K25" s="45">
         <v>1549250.84</v>
       </c>
-      <c r="L25" s="35" t="s">
+      <c r="L25" s="34" t="s">
         <v>177</v>
       </c>
       <c r="M25" s="39">
@@ -2309,24 +2309,24 @@
       <c r="D26" s="49" t="s">
         <v>178</v>
       </c>
-      <c r="E26" s="35"/>
-      <c r="F26" s="35">
+      <c r="E26" s="34"/>
+      <c r="F26" s="34">
         <v>48.0</v>
       </c>
-      <c r="G26" s="44">
+      <c r="G26" s="43">
         <v>46230.0</v>
       </c>
-      <c r="H26" s="35" t="s">
+      <c r="H26" s="34" t="s">
         <v>179</v>
       </c>
-      <c r="I26" s="44"/>
-      <c r="J26" s="44">
+      <c r="I26" s="43"/>
+      <c r="J26" s="43">
         <v>46262.0</v>
       </c>
-      <c r="K26" s="46" t="s">
+      <c r="K26" s="45" t="s">
         <v>180</v>
       </c>
-      <c r="L26" s="35" t="s">
+      <c r="L26" s="34" t="s">
         <v>181</v>
       </c>
       <c r="M26" s="39" t="s">
@@ -2343,26 +2343,26 @@
     <row r="27">
       <c r="A27" s="24"/>
       <c r="B27" s="24"/>
-      <c r="C27" s="36"/>
+      <c r="C27" s="35"/>
       <c r="D27" s="49" t="s">
         <v>182</v>
       </c>
-      <c r="E27" s="35"/>
-      <c r="F27" s="35">
+      <c r="E27" s="34"/>
+      <c r="F27" s="34">
         <v>49.0</v>
       </c>
-      <c r="G27" s="44">
+      <c r="G27" s="43">
         <v>46252.0</v>
       </c>
-      <c r="H27" s="35" t="s">
-        <v>129</v>
-      </c>
-      <c r="I27" s="44"/>
-      <c r="J27" s="44">
+      <c r="H27" s="34" t="s">
+        <v>131</v>
+      </c>
+      <c r="I27" s="43"/>
+      <c r="J27" s="43">
         <v>46284.0</v>
       </c>
-      <c r="K27" s="46"/>
-      <c r="L27" s="35"/>
+      <c r="K27" s="45"/>
+      <c r="L27" s="34"/>
       <c r="M27" s="39" t="s">
         <v>183</v>
       </c>
@@ -2378,34 +2378,34 @@
       <c r="A28" s="24"/>
       <c r="B28" s="24"/>
       <c r="C28" s="29" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="D28" s="29" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="E28" s="30" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="F28" s="30" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="G28" s="30"/>
       <c r="H28" s="30" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="I28" s="30"/>
       <c r="J28" s="30"/>
       <c r="K28" s="30" t="s">
-        <v>74</v>
+        <v>65</v>
       </c>
       <c r="L28" s="30" t="s">
-        <v>75</v>
+        <v>66</v>
       </c>
       <c r="M28" s="30" t="s">
-        <v>76</v>
+        <v>67</v>
       </c>
       <c r="N28" s="30" t="s">
-        <v>77</v>
+        <v>68</v>
       </c>
       <c r="O28" s="26"/>
       <c r="P28" s="28"/>
@@ -2425,30 +2425,30 @@
     <row r="29" ht="12.75" customHeight="1">
       <c r="A29" s="24"/>
       <c r="B29" s="24"/>
-      <c r="C29" s="33">
+      <c r="C29" s="32">
         <v>2.0</v>
       </c>
       <c r="D29" s="56" t="s">
         <v>184</v>
       </c>
-      <c r="E29" s="36"/>
-      <c r="F29" s="36">
+      <c r="E29" s="35"/>
+      <c r="F29" s="35">
         <v>402.0</v>
       </c>
-      <c r="G29" s="37">
+      <c r="G29" s="36">
         <v>45791.0</v>
       </c>
-      <c r="H29" s="36" t="s">
-        <v>48</v>
-      </c>
-      <c r="I29" s="37"/>
-      <c r="J29" s="37">
+      <c r="H29" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="I29" s="36"/>
+      <c r="J29" s="36">
         <v>45834.0</v>
       </c>
       <c r="K29" s="38">
         <v>188246.17</v>
       </c>
-      <c r="L29" s="35" t="s">
+      <c r="L29" s="34" t="s">
         <v>185</v>
       </c>
       <c r="M29" s="57">
@@ -2481,23 +2481,23 @@
       <c r="E30" s="58">
         <v>46.0</v>
       </c>
-      <c r="F30" s="36">
+      <c r="F30" s="35">
         <v>447.0</v>
       </c>
-      <c r="G30" s="37">
+      <c r="G30" s="36">
         <v>45814.0</v>
       </c>
-      <c r="H30" s="35" t="s">
+      <c r="H30" s="34" t="s">
         <v>187</v>
       </c>
-      <c r="I30" s="44"/>
-      <c r="J30" s="44">
+      <c r="I30" s="43"/>
+      <c r="J30" s="43">
         <v>45955.0</v>
       </c>
       <c r="K30" s="38">
         <v>112720.77</v>
       </c>
-      <c r="L30" s="35" t="s">
+      <c r="L30" s="34" t="s">
         <v>188</v>
       </c>
       <c r="M30" s="39">
@@ -2530,23 +2530,23 @@
       <c r="E31" s="60" t="s">
         <v>190</v>
       </c>
-      <c r="F31" s="36">
+      <c r="F31" s="35">
         <v>529.0</v>
       </c>
       <c r="G31" s="61">
         <v>45853.0</v>
       </c>
-      <c r="H31" s="35" t="s">
+      <c r="H31" s="34" t="s">
         <v>53</v>
       </c>
-      <c r="I31" s="44"/>
-      <c r="J31" s="44">
+      <c r="I31" s="43"/>
+      <c r="J31" s="43">
         <v>45939.0</v>
       </c>
-      <c r="K31" s="46">
+      <c r="K31" s="45">
         <v>378307.61</v>
       </c>
-      <c r="L31" s="35" t="s">
+      <c r="L31" s="34" t="s">
         <v>191</v>
       </c>
       <c r="M31" s="39">
@@ -2579,23 +2579,23 @@
       <c r="E32" s="60" t="s">
         <v>190</v>
       </c>
-      <c r="F32" s="35">
+      <c r="F32" s="34">
         <v>691.0</v>
       </c>
       <c r="G32" s="61">
         <v>45910.0</v>
       </c>
-      <c r="H32" s="35" t="s">
+      <c r="H32" s="34" t="s">
         <v>53</v>
       </c>
-      <c r="I32" s="44"/>
-      <c r="J32" s="44">
+      <c r="I32" s="43"/>
+      <c r="J32" s="43">
         <v>45941.0</v>
       </c>
       <c r="K32" s="38">
         <v>3315.0471000000252</v>
       </c>
-      <c r="L32" s="35" t="s">
+      <c r="L32" s="34" t="s">
         <v>193</v>
       </c>
       <c r="M32" s="39">
@@ -2628,23 +2628,23 @@
       <c r="E33" s="63">
         <v>135.0</v>
       </c>
-      <c r="F33" s="35">
+      <c r="F33" s="34">
         <v>677.0</v>
       </c>
       <c r="G33" s="61">
         <v>45904.0</v>
       </c>
-      <c r="H33" s="35" t="s">
-        <v>57</v>
+      <c r="H33" s="34" t="s">
+        <v>69</v>
       </c>
       <c r="I33" s="64"/>
       <c r="J33" s="64">
         <v>45935.0</v>
       </c>
-      <c r="K33" s="46">
+      <c r="K33" s="45">
         <v>198332.75</v>
       </c>
-      <c r="L33" s="35" t="s">
+      <c r="L33" s="34" t="s">
         <v>195</v>
       </c>
       <c r="M33" s="39">
@@ -2677,20 +2677,20 @@
       <c r="E34" s="63">
         <v>40.0</v>
       </c>
-      <c r="F34" s="35">
+      <c r="F34" s="34">
         <v>278.0</v>
       </c>
       <c r="G34" s="61">
         <v>46008.0</v>
       </c>
-      <c r="H34" s="35" t="s">
-        <v>115</v>
+      <c r="H34" s="34" t="s">
+        <v>119</v>
       </c>
       <c r="I34" s="64"/>
       <c r="J34" s="64">
         <v>46066.0</v>
       </c>
-      <c r="K34" s="46">
+      <c r="K34" s="45">
         <v>1528.62</v>
       </c>
       <c r="L34" s="65" t="s">
@@ -2726,23 +2726,23 @@
       <c r="E35" s="63" t="s">
         <v>200</v>
       </c>
-      <c r="F35" s="35">
+      <c r="F35" s="34">
         <v>748.0</v>
       </c>
       <c r="G35" s="61">
         <v>45930.0</v>
       </c>
-      <c r="H35" s="35" t="s">
-        <v>90</v>
+      <c r="H35" s="34" t="s">
+        <v>92</v>
       </c>
       <c r="I35" s="64"/>
       <c r="J35" s="64">
         <v>45935.0</v>
       </c>
-      <c r="K35" s="46">
+      <c r="K35" s="45">
         <v>38718.58</v>
       </c>
-      <c r="L35" s="35" t="s">
+      <c r="L35" s="34" t="s">
         <v>201</v>
       </c>
       <c r="M35" s="57" t="s">
@@ -2775,23 +2775,23 @@
       <c r="E36" s="63">
         <v>154.0</v>
       </c>
-      <c r="F36" s="35">
+      <c r="F36" s="34">
         <v>822.0</v>
       </c>
       <c r="G36" s="61">
         <v>45968.0</v>
       </c>
-      <c r="H36" s="35" t="s">
-        <v>106</v>
+      <c r="H36" s="34" t="s">
+        <v>109</v>
       </c>
       <c r="I36" s="64"/>
       <c r="J36" s="64">
         <v>45935.0</v>
       </c>
-      <c r="K36" s="46">
+      <c r="K36" s="45">
         <v>133124.11</v>
       </c>
-      <c r="L36" s="35" t="s">
+      <c r="L36" s="34" t="s">
         <v>204</v>
       </c>
       <c r="M36" s="57" t="s">
@@ -2831,16 +2831,16 @@
         <v>46043.0</v>
       </c>
       <c r="H37" s="63" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="I37" s="68"/>
       <c r="J37" s="67">
         <v>46075.0</v>
       </c>
-      <c r="K37" s="46">
+      <c r="K37" s="45">
         <v>11372.9</v>
       </c>
-      <c r="L37" s="35" t="s">
+      <c r="L37" s="34" t="s">
         <v>207</v>
       </c>
       <c r="M37" s="39">
@@ -2878,8 +2878,8 @@
         <v>209</v>
       </c>
       <c r="J38" s="67"/>
-      <c r="K38" s="46"/>
-      <c r="L38" s="35"/>
+      <c r="K38" s="45"/>
+      <c r="L38" s="34"/>
       <c r="M38" s="39"/>
       <c r="N38" s="51">
         <v>15854.78</v>
@@ -2915,8 +2915,8 @@
         <v>209</v>
       </c>
       <c r="J39" s="67"/>
-      <c r="K39" s="46"/>
-      <c r="L39" s="35"/>
+      <c r="K39" s="45"/>
+      <c r="L39" s="34"/>
       <c r="M39" s="39"/>
       <c r="N39" s="69">
         <v>42229.72325</v>
@@ -2940,7 +2940,7 @@
     <row r="40" ht="12.75" customHeight="1">
       <c r="A40" s="24"/>
       <c r="B40" s="24"/>
-      <c r="C40" s="36"/>
+      <c r="C40" s="35"/>
       <c r="D40" s="59" t="s">
         <v>211</v>
       </c>
@@ -2952,7 +2952,7 @@
         <v>209</v>
       </c>
       <c r="J40" s="67"/>
-      <c r="K40" s="46"/>
+      <c r="K40" s="45"/>
       <c r="L40" s="47"/>
       <c r="M40" s="39"/>
       <c r="N40" s="70">
@@ -2977,7 +2977,7 @@
     <row r="41" ht="12.75" customHeight="1">
       <c r="A41" s="24"/>
       <c r="B41" s="24"/>
-      <c r="C41" s="36"/>
+      <c r="C41" s="35"/>
       <c r="D41" s="59" t="s">
         <v>212</v>
       </c>
@@ -2989,7 +2989,7 @@
         <v>213</v>
       </c>
       <c r="J41" s="67"/>
-      <c r="K41" s="46"/>
+      <c r="K41" s="45"/>
       <c r="L41" s="47"/>
       <c r="M41" s="39"/>
       <c r="N41" s="70"/>
@@ -3012,7 +3012,7 @@
     <row r="42" ht="12.75" customHeight="1">
       <c r="A42" s="24"/>
       <c r="B42" s="24"/>
-      <c r="C42" s="33">
+      <c r="C42" s="32">
         <v>3.0</v>
       </c>
       <c r="D42" s="59" t="s">
@@ -3026,13 +3026,13 @@
         <v>46104.0</v>
       </c>
       <c r="H42" s="63" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="I42" s="68"/>
       <c r="J42" s="67">
         <v>46106.0</v>
       </c>
-      <c r="K42" s="46">
+      <c r="K42" s="45">
         <v>27801.11</v>
       </c>
       <c r="L42" s="71" t="s">
@@ -3073,23 +3073,23 @@
         <v>46199.0</v>
       </c>
       <c r="H43" s="63" t="s">
-        <v>63</v>
+        <v>74</v>
       </c>
       <c r="I43" s="68"/>
       <c r="J43" s="67">
         <v>46233.0</v>
       </c>
-      <c r="K43" s="46">
+      <c r="K43" s="45">
         <v>58868.35</v>
       </c>
-      <c r="L43" s="35" t="s">
-        <v>76</v>
+      <c r="L43" s="34" t="s">
+        <v>67</v>
       </c>
       <c r="M43" s="72">
         <v>58868.35</v>
       </c>
       <c r="N43" s="51"/>
-      <c r="V43" s="5"/>
+      <c r="V43" s="3"/>
     </row>
     <row r="44" ht="12.75" customHeight="1">
       <c r="A44" s="15"/>
@@ -3097,7 +3097,7 @@
       <c r="C44" s="41"/>
       <c r="K44" s="73"/>
       <c r="M44" s="73"/>
-      <c r="V44" s="5"/>
+      <c r="V44" s="3"/>
     </row>
     <row r="45" ht="12.75" customHeight="1">
       <c r="A45" s="15"/>
@@ -3105,31 +3105,31 @@
       <c r="C45" s="41"/>
       <c r="K45" s="73"/>
       <c r="M45" s="73"/>
-      <c r="V45" s="5"/>
+      <c r="V45" s="3"/>
     </row>
     <row r="46" ht="12.75" customHeight="1">
       <c r="A46" s="15"/>
       <c r="B46" s="15"/>
       <c r="C46" s="41"/>
-      <c r="V46" s="5"/>
+      <c r="V46" s="3"/>
     </row>
     <row r="47" ht="12.75" customHeight="1">
       <c r="A47" s="15"/>
       <c r="B47" s="15"/>
       <c r="C47" s="41"/>
-      <c r="V47" s="5"/>
+      <c r="V47" s="3"/>
     </row>
     <row r="48" ht="12.75" customHeight="1">
       <c r="A48" s="15"/>
       <c r="B48" s="15"/>
       <c r="C48" s="41"/>
-      <c r="V48" s="5"/>
+      <c r="V48" s="3"/>
     </row>
     <row r="49" ht="12.75" customHeight="1">
       <c r="A49" s="15"/>
       <c r="B49" s="15"/>
       <c r="C49" s="41"/>
-      <c r="V49" s="5"/>
+      <c r="V49" s="3"/>
     </row>
     <row r="50" ht="12.75" customHeight="1">
       <c r="A50" s="15"/>
@@ -3137,7 +3137,7 @@
       <c r="C50" s="55"/>
       <c r="K50" s="73"/>
       <c r="M50" s="73"/>
-      <c r="V50" s="5"/>
+      <c r="V50" s="3"/>
     </row>
     <row r="51" ht="12.75" customHeight="1">
       <c r="A51" s="15"/>
@@ -3161,7 +3161,7 @@
       <c r="S51" s="74"/>
       <c r="T51" s="74"/>
       <c r="U51" s="74"/>
-      <c r="V51" s="5"/>
+      <c r="V51" s="3"/>
     </row>
     <row r="52" ht="12.75" customHeight="1">
       <c r="A52" s="15"/>
@@ -8042,10 +8042,10 @@
       <c r="AH1" s="2"/>
     </row>
     <row r="2">
-      <c r="A2" s="3">
+      <c r="A2" s="4">
         <v>46258.0</v>
       </c>
-      <c r="L2" s="4" t="s">
+      <c r="L2" s="6" t="s">
         <v>0</v>
       </c>
       <c r="AB2" s="2"/>
@@ -8057,40 +8057,40 @@
       <c r="AH2" s="2"/>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="6" t="s">
+      <c r="A3" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="8">
+      <c r="B3" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3" s="10">
         <v>2.5E32</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="10">
+      <c r="E3" s="12">
         <v>45686.0</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="F3" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G3" s="6">
+      <c r="G3" s="8">
         <v>12.0</v>
       </c>
-      <c r="H3" s="6">
+      <c r="H3" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I3" s="6">
+      <c r="I3" s="8">
         <v>2048.0</v>
       </c>
-      <c r="J3" s="12">
+      <c r="J3" s="13">
         <v>1000.0</v>
       </c>
-      <c r="K3" s="12">
+      <c r="K3" s="13">
         <v>1000.0</v>
       </c>
-      <c r="L3" s="6">
+      <c r="L3" s="8">
         <v>0.0</v>
       </c>
       <c r="AB3" s="2"/>
@@ -8102,40 +8102,40 @@
       <c r="AH3" s="2"/>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="10">
+      <c r="E4" s="12">
         <v>45762.0</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="F4" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G4" s="6">
+      <c r="G4" s="8">
         <v>12.0</v>
       </c>
-      <c r="H4" s="6">
+      <c r="H4" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I4" s="6">
+      <c r="I4" s="8">
         <v>2048.0</v>
       </c>
-      <c r="J4" s="12">
+      <c r="J4" s="13">
         <v>52250.04</v>
       </c>
-      <c r="K4" s="12">
+      <c r="K4" s="13">
         <v>52250.04</v>
       </c>
-      <c r="L4" s="6">
+      <c r="L4" s="8">
         <v>0.0</v>
       </c>
       <c r="AB4" s="2"/>
@@ -8147,40 +8147,40 @@
       <c r="AH4" s="2"/>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="s">
+      <c r="A5" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E5" s="10">
+      <c r="E5" s="12">
         <v>45762.0</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="F5" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G5" s="6">
+      <c r="G5" s="8">
         <v>12.0</v>
       </c>
-      <c r="H5" s="6">
+      <c r="H5" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I5" s="6">
+      <c r="I5" s="8">
         <v>2048.0</v>
       </c>
-      <c r="J5" s="12">
+      <c r="J5" s="13">
         <v>881914.18</v>
       </c>
-      <c r="K5" s="12">
+      <c r="K5" s="13">
         <v>881914.18</v>
       </c>
-      <c r="L5" s="6">
+      <c r="L5" s="8">
         <v>0.0</v>
       </c>
       <c r="AB5" s="2"/>
@@ -8192,40 +8192,40 @@
       <c r="AH5" s="2"/>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="B6" s="6" t="s">
+      <c r="A6" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="D6" s="6" t="s">
+      <c r="C6" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="D6" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E6" s="10">
+      <c r="E6" s="12">
         <v>45762.0</v>
       </c>
-      <c r="F6" s="6" t="s">
+      <c r="F6" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G6" s="6">
+      <c r="G6" s="8">
         <v>12.0</v>
       </c>
-      <c r="H6" s="6">
+      <c r="H6" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I6" s="6">
+      <c r="I6" s="8">
         <v>2048.0</v>
       </c>
-      <c r="J6" s="12">
+      <c r="J6" s="13">
         <v>750000.0</v>
       </c>
-      <c r="K6" s="12">
+      <c r="K6" s="13">
         <v>750000.0</v>
       </c>
-      <c r="L6" s="6">
+      <c r="L6" s="8">
         <v>0.0</v>
       </c>
       <c r="AB6" s="2"/>
@@ -8237,40 +8237,40 @@
       <c r="AH6" s="2"/>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="D7" s="6" t="s">
+      <c r="A7" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="D7" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E7" s="10">
+      <c r="E7" s="12">
         <v>45763.0</v>
       </c>
-      <c r="F7" s="6" t="s">
+      <c r="F7" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G7" s="6">
+      <c r="G7" s="8">
         <v>12.0</v>
       </c>
-      <c r="H7" s="6">
+      <c r="H7" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I7" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="J7" s="12">
+      <c r="I7" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="J7" s="13">
         <v>949835.78</v>
       </c>
-      <c r="K7" s="12">
+      <c r="K7" s="13">
         <v>949835.78</v>
       </c>
-      <c r="L7" s="6">
+      <c r="L7" s="8">
         <v>0.0</v>
       </c>
       <c r="AB7" s="2"/>
@@ -8282,43 +8282,43 @@
       <c r="AH7" s="2"/>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="C8" s="6" t="s">
+      <c r="A8" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="B8" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="D8" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E8" s="10">
+      <c r="E8" s="12">
         <v>45763.0</v>
       </c>
-      <c r="F8" s="6" t="s">
+      <c r="F8" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G8" s="6">
+      <c r="G8" s="8">
         <v>12.0</v>
       </c>
-      <c r="H8" s="6">
+      <c r="H8" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I8" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="J8" s="12">
+      <c r="I8" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="J8" s="13">
         <v>524584.95</v>
       </c>
-      <c r="K8" s="12">
+      <c r="K8" s="13">
         <v>524584.95</v>
       </c>
-      <c r="L8" s="6">
+      <c r="L8" s="8">
         <v>0.0</v>
       </c>
-      <c r="O8" s="21"/>
+      <c r="O8" s="22"/>
       <c r="AB8" s="2"/>
       <c r="AC8" s="2"/>
       <c r="AD8" s="2"/>
@@ -8328,40 +8328,40 @@
       <c r="AH8" s="2"/>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="B9" s="6" t="s">
+      <c r="A9" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="B9" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="C9" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="D9" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E9" s="10">
+      <c r="E9" s="12">
         <v>45792.0</v>
       </c>
-      <c r="F9" s="6" t="s">
+      <c r="F9" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G9" s="6">
+      <c r="G9" s="8">
         <v>12.0</v>
       </c>
-      <c r="H9" s="6">
+      <c r="H9" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I9" s="6" t="s">
+      <c r="I9" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="J9" s="12">
+      <c r="J9" s="13">
         <v>211614.23</v>
       </c>
-      <c r="K9" s="12">
+      <c r="K9" s="13">
         <v>211614.23</v>
       </c>
-      <c r="L9" s="6">
+      <c r="L9" s="8">
         <v>0.0</v>
       </c>
       <c r="AB9" s="2"/>
@@ -8373,40 +8373,40 @@
       <c r="AH9" s="2"/>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="s">
+      <c r="A10" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="B10" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="C10" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="D10" s="6" t="s">
+      <c r="D10" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E10" s="10">
+      <c r="E10" s="12">
         <v>45825.0</v>
       </c>
-      <c r="F10" s="6" t="s">
+      <c r="F10" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G10" s="6">
+      <c r="G10" s="8">
         <v>12.0</v>
       </c>
-      <c r="H10" s="6">
+      <c r="H10" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I10" s="6">
+      <c r="I10" s="8">
         <v>2048.0</v>
       </c>
-      <c r="J10" s="12">
+      <c r="J10" s="13">
         <v>2391157.42</v>
       </c>
-      <c r="K10" s="12">
+      <c r="K10" s="13">
         <v>2391157.41</v>
       </c>
-      <c r="L10" s="12">
+      <c r="L10" s="13">
         <v>0.01</v>
       </c>
       <c r="AB10" s="2"/>
@@ -8418,40 +8418,40 @@
       <c r="AH10" s="2"/>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="B11" s="6" t="s">
+      <c r="A11" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="B11" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C11" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="D11" s="6" t="s">
+      <c r="C11" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="D11" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E11" s="10">
+      <c r="E11" s="12">
         <v>45825.0</v>
       </c>
-      <c r="F11" s="6" t="s">
+      <c r="F11" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G11" s="6">
+      <c r="G11" s="8">
         <v>12.0</v>
       </c>
-      <c r="H11" s="6">
+      <c r="H11" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I11" s="6">
+      <c r="I11" s="8">
         <v>2048.0</v>
       </c>
-      <c r="J11" s="12">
+      <c r="J11" s="13">
         <v>618154.39</v>
       </c>
-      <c r="K11" s="12">
+      <c r="K11" s="13">
         <v>618154.38</v>
       </c>
-      <c r="L11" s="6">
+      <c r="L11" s="8">
         <v>0.01</v>
       </c>
       <c r="AB11" s="2"/>
@@ -8463,40 +8463,40 @@
       <c r="AH11" s="2"/>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="B12" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="C12" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="D12" s="6" t="s">
+      <c r="A12" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="D12" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E12" s="10">
+      <c r="E12" s="12">
         <v>45832.0</v>
       </c>
-      <c r="F12" s="6" t="s">
+      <c r="F12" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G12" s="6">
+      <c r="G12" s="8">
         <v>12.0</v>
       </c>
-      <c r="H12" s="6">
+      <c r="H12" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I12" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="J12" s="12">
+      <c r="I12" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="J12" s="13">
         <v>1600334.09</v>
       </c>
-      <c r="K12" s="12">
+      <c r="K12" s="13">
         <v>1600334.09</v>
       </c>
-      <c r="L12" s="6">
+      <c r="L12" s="8">
         <v>0.0</v>
       </c>
       <c r="AB12" s="2"/>
@@ -8508,43 +8508,43 @@
       <c r="AH12" s="2"/>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="B13" s="6" t="s">
+      <c r="A13" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="B13" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="C13" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="D13" s="6" t="s">
+      <c r="C13" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="D13" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E13" s="10">
+      <c r="E13" s="12">
         <v>45863.0</v>
       </c>
-      <c r="F13" s="6" t="s">
+      <c r="F13" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G13" s="6">
+      <c r="G13" s="8">
         <v>12.0</v>
       </c>
-      <c r="H13" s="6">
+      <c r="H13" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I13" s="6">
+      <c r="I13" s="8">
         <v>2048.0</v>
       </c>
-      <c r="J13" s="12">
+      <c r="J13" s="13">
         <v>2364771.07</v>
       </c>
-      <c r="K13" s="12">
+      <c r="K13" s="13">
         <v>2364771.07</v>
       </c>
-      <c r="L13" s="12">
+      <c r="L13" s="13">
         <v>0.0</v>
       </c>
-      <c r="M13" s="31"/>
+      <c r="M13" s="37"/>
       <c r="AB13" s="2"/>
       <c r="AC13" s="2"/>
       <c r="AD13" s="2"/>
@@ -8554,40 +8554,40 @@
       <c r="AH13" s="2"/>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="B14" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="C14" s="6" t="s">
-        <v>73</v>
-      </c>
-      <c r="D14" s="6" t="s">
+      <c r="A14" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="D14" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E14" s="10">
+      <c r="E14" s="12">
         <v>45887.0</v>
       </c>
-      <c r="F14" s="6" t="s">
+      <c r="F14" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G14" s="6">
+      <c r="G14" s="8">
         <v>12.0</v>
       </c>
-      <c r="H14" s="6">
+      <c r="H14" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I14" s="6" t="s">
+      <c r="I14" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="J14" s="12">
+      <c r="J14" s="13">
         <v>968237.39</v>
       </c>
-      <c r="K14" s="12">
+      <c r="K14" s="13">
         <v>968237.39</v>
       </c>
-      <c r="L14" s="6">
+      <c r="L14" s="8">
         <v>0.0</v>
       </c>
       <c r="AB14" s="2"/>
@@ -8599,40 +8599,40 @@
       <c r="AH14" s="2"/>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="B15" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="C15" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="D15" s="6" t="s">
+      <c r="A15" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="B15" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="C15" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="D15" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E15" s="10">
+      <c r="E15" s="12">
         <v>45924.0</v>
       </c>
-      <c r="F15" s="6" t="s">
+      <c r="F15" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G15" s="6">
+      <c r="G15" s="8">
         <v>12.0</v>
       </c>
-      <c r="H15" s="6">
+      <c r="H15" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I15" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="J15" s="12">
+      <c r="I15" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="J15" s="13">
         <v>1011677.95</v>
       </c>
-      <c r="K15" s="12">
+      <c r="K15" s="13">
         <v>1011677.95</v>
       </c>
-      <c r="L15" s="6">
+      <c r="L15" s="8">
         <v>0.0</v>
       </c>
       <c r="AB15" s="2"/>
@@ -8644,40 +8644,40 @@
       <c r="AH15" s="2"/>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="B16" s="6" t="s">
+      <c r="A16" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="B16" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="C16" s="6" t="s">
-        <v>84</v>
-      </c>
-      <c r="D16" s="6" t="s">
+      <c r="C16" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="D16" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E16" s="10">
+      <c r="E16" s="12">
         <v>45929.0</v>
       </c>
-      <c r="F16" s="6" t="s">
+      <c r="F16" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G16" s="6">
+      <c r="G16" s="8">
         <v>12.0</v>
       </c>
-      <c r="H16" s="6">
+      <c r="H16" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I16" s="6">
+      <c r="I16" s="8">
         <v>2048.0</v>
       </c>
-      <c r="J16" s="12">
+      <c r="J16" s="13">
         <v>1580293.02</v>
       </c>
-      <c r="K16" s="12">
+      <c r="K16" s="13">
         <v>1580293.02</v>
       </c>
-      <c r="L16" s="12">
+      <c r="L16" s="13">
         <v>0.0</v>
       </c>
       <c r="AB16" s="2"/>
@@ -8689,40 +8689,40 @@
       <c r="AH16" s="2"/>
     </row>
     <row r="17">
-      <c r="A17" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="B17" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="C17" s="6" t="s">
+      <c r="A17" s="8" t="s">
         <v>88</v>
       </c>
-      <c r="D17" s="6" t="s">
+      <c r="B17" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="C17" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="D17" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E17" s="10">
+      <c r="E17" s="12">
         <v>45930.0</v>
       </c>
-      <c r="F17" s="6" t="s">
+      <c r="F17" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G17" s="6">
+      <c r="G17" s="8">
         <v>12.0</v>
       </c>
-      <c r="H17" s="6">
+      <c r="H17" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I17" s="6">
+      <c r="I17" s="8">
         <v>2048.0</v>
       </c>
-      <c r="J17" s="12">
+      <c r="J17" s="13">
         <v>34065.36</v>
       </c>
-      <c r="K17" s="6">
+      <c r="K17" s="8">
         <v>0.0</v>
       </c>
-      <c r="L17" s="12">
+      <c r="L17" s="13">
         <v>34065.36</v>
       </c>
       <c r="AB17" s="2"/>
@@ -8734,40 +8734,40 @@
       <c r="AH17" s="2"/>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="B18" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="C18" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="D18" s="6" t="s">
+      <c r="A18" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="B18" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="C18" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="D18" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E18" s="10">
+      <c r="E18" s="12">
         <v>45938.0</v>
       </c>
-      <c r="F18" s="6" t="s">
+      <c r="F18" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G18" s="6">
+      <c r="G18" s="8">
         <v>12.0</v>
       </c>
-      <c r="H18" s="6">
+      <c r="H18" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I18" s="6" t="s">
+      <c r="I18" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="J18" s="12">
+      <c r="J18" s="13">
         <v>63746.85</v>
       </c>
-      <c r="K18" s="12">
+      <c r="K18" s="13">
         <v>63746.85</v>
       </c>
-      <c r="L18" s="6">
+      <c r="L18" s="8">
         <v>0.0</v>
       </c>
       <c r="AB18" s="2"/>
@@ -8779,40 +8779,40 @@
       <c r="AH18" s="2"/>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="B19" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="C19" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="D19" s="6" t="s">
+      <c r="A19" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="B19" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="C19" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="D19" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E19" s="10">
+      <c r="E19" s="12">
         <v>45938.0</v>
       </c>
-      <c r="F19" s="6" t="s">
+      <c r="F19" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G19" s="6">
+      <c r="G19" s="8">
         <v>12.0</v>
       </c>
-      <c r="H19" s="6">
+      <c r="H19" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I19" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="J19" s="12">
+      <c r="I19" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="J19" s="13">
         <v>947931.1</v>
       </c>
-      <c r="K19" s="12">
+      <c r="K19" s="13">
         <v>947931.1</v>
       </c>
-      <c r="L19" s="6">
+      <c r="L19" s="8">
         <v>0.0</v>
       </c>
       <c r="AB19" s="2"/>
@@ -8824,40 +8824,40 @@
       <c r="AH19" s="2"/>
     </row>
     <row r="20">
-      <c r="A20" s="6" t="s">
-        <v>94</v>
-      </c>
-      <c r="B20" s="6" t="s">
+      <c r="A20" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="B20" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="C20" s="6" t="s">
-        <v>95</v>
-      </c>
-      <c r="D20" s="6" t="s">
+      <c r="C20" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="D20" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E20" s="10">
+      <c r="E20" s="12">
         <v>45938.0</v>
       </c>
-      <c r="F20" s="6" t="s">
+      <c r="F20" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G20" s="6">
+      <c r="G20" s="8">
         <v>12.0</v>
       </c>
-      <c r="H20" s="6">
+      <c r="H20" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I20" s="6">
+      <c r="I20" s="8">
         <v>2048.0</v>
       </c>
-      <c r="J20" s="12">
+      <c r="J20" s="13">
         <v>259790.57</v>
       </c>
-      <c r="K20" s="12">
+      <c r="K20" s="13">
         <v>259790.57</v>
       </c>
-      <c r="L20" s="6">
+      <c r="L20" s="8">
         <v>0.0</v>
       </c>
       <c r="AB20" s="2"/>
@@ -8869,40 +8869,40 @@
       <c r="AH20" s="2"/>
     </row>
     <row r="21">
-      <c r="A21" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="B21" s="6" t="s">
+      <c r="A21" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="B21" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C21" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="D21" s="6" t="s">
+      <c r="C21" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="D21" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E21" s="10">
+      <c r="E21" s="12">
         <v>45938.0</v>
       </c>
-      <c r="F21" s="6" t="s">
+      <c r="F21" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G21" s="6">
+      <c r="G21" s="8">
         <v>12.0</v>
       </c>
-      <c r="H21" s="6">
+      <c r="H21" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I21" s="6">
+      <c r="I21" s="8">
         <v>2048.0</v>
       </c>
-      <c r="J21" s="12">
+      <c r="J21" s="13">
         <v>170479.3</v>
       </c>
-      <c r="K21" s="12">
+      <c r="K21" s="13">
         <v>170479.3</v>
       </c>
-      <c r="L21" s="6">
+      <c r="L21" s="8">
         <v>0.0</v>
       </c>
       <c r="AB21" s="2"/>
@@ -8914,40 +8914,40 @@
       <c r="AH21" s="2"/>
     </row>
     <row r="22">
-      <c r="A22" s="6" t="s">
-        <v>101</v>
-      </c>
-      <c r="B22" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="C22" s="6" t="s">
-        <v>103</v>
-      </c>
-      <c r="D22" s="6" t="s">
+      <c r="A22" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="B22" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="C22" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="D22" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E22" s="43">
+      <c r="E22" s="46">
         <v>45953.0</v>
       </c>
-      <c r="F22" s="6" t="s">
+      <c r="F22" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G22" s="6">
+      <c r="G22" s="8">
         <v>12.0</v>
       </c>
-      <c r="H22" s="6">
+      <c r="H22" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I22" s="6">
+      <c r="I22" s="8">
         <v>2000.0</v>
       </c>
-      <c r="J22" s="12">
+      <c r="J22" s="13">
         <v>1500000.0</v>
       </c>
-      <c r="K22" s="12">
+      <c r="K22" s="13">
         <v>1500000.0</v>
       </c>
-      <c r="L22" s="12">
+      <c r="L22" s="13">
         <v>0.0</v>
       </c>
       <c r="AB22" s="2"/>
@@ -8959,40 +8959,40 @@
       <c r="AH22" s="2"/>
     </row>
     <row r="23">
-      <c r="A23" s="6" t="s">
-        <v>106</v>
-      </c>
-      <c r="B23" s="6" t="s">
-        <v>107</v>
-      </c>
-      <c r="C23" s="6" t="s">
-        <v>108</v>
-      </c>
-      <c r="D23" s="6" t="s">
+      <c r="A23" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="B23" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="C23" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="D23" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E23" s="43">
+      <c r="E23" s="46">
         <v>45953.0</v>
       </c>
-      <c r="F23" s="6" t="s">
+      <c r="F23" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G23" s="6">
+      <c r="G23" s="8">
         <v>12.0</v>
       </c>
-      <c r="H23" s="6">
+      <c r="H23" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I23" s="6" t="s">
-        <v>110</v>
-      </c>
-      <c r="J23" s="12">
+      <c r="I23" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="J23" s="13">
         <v>1000001.64</v>
       </c>
-      <c r="K23" s="12">
+      <c r="K23" s="13">
         <v>1000001.64</v>
       </c>
-      <c r="L23" s="6">
+      <c r="L23" s="8">
         <v>0.0</v>
       </c>
       <c r="AB23" s="2"/>
@@ -9004,40 +9004,40 @@
       <c r="AH23" s="2"/>
     </row>
     <row r="24">
-      <c r="A24" s="6" t="s">
-        <v>112</v>
-      </c>
-      <c r="B24" s="6" t="s">
+      <c r="A24" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="B24" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C24" s="6" t="s">
-        <v>113</v>
-      </c>
-      <c r="D24" s="6" t="s">
+      <c r="C24" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="D24" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E24" s="43">
+      <c r="E24" s="46">
         <v>45953.0</v>
       </c>
-      <c r="F24" s="6" t="s">
+      <c r="F24" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G24" s="6">
+      <c r="G24" s="8">
         <v>12.0</v>
       </c>
-      <c r="H24" s="6">
+      <c r="H24" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I24" s="6">
+      <c r="I24" s="8">
         <v>2048.0</v>
       </c>
-      <c r="J24" s="12">
+      <c r="J24" s="13">
         <v>68405.66</v>
       </c>
-      <c r="K24" s="12">
+      <c r="K24" s="13">
         <v>68405.66</v>
       </c>
-      <c r="L24" s="6">
+      <c r="L24" s="8">
         <v>0.0</v>
       </c>
       <c r="AB24" s="2"/>
@@ -9049,40 +9049,40 @@
       <c r="AH24" s="2"/>
     </row>
     <row r="25">
-      <c r="A25" s="6" t="s">
-        <v>115</v>
-      </c>
-      <c r="B25" s="6" t="s">
-        <v>116</v>
-      </c>
-      <c r="C25" s="6" t="s">
-        <v>117</v>
-      </c>
-      <c r="D25" s="6" t="s">
+      <c r="A25" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="B25" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="C25" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="D25" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E25" s="43">
+      <c r="E25" s="46">
         <v>45975.0</v>
       </c>
-      <c r="F25" s="6" t="s">
+      <c r="F25" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G25" s="6">
+      <c r="G25" s="8">
         <v>12.0</v>
       </c>
-      <c r="H25" s="6">
+      <c r="H25" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I25" s="6" t="s">
-        <v>110</v>
-      </c>
-      <c r="J25" s="12">
+      <c r="I25" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="J25" s="13">
         <v>1157673.06</v>
       </c>
-      <c r="K25" s="12">
+      <c r="K25" s="13">
         <v>1157673.06</v>
       </c>
-      <c r="L25" s="6">
+      <c r="L25" s="8">
         <v>0.0</v>
       </c>
       <c r="AB25" s="2"/>
@@ -9094,40 +9094,40 @@
       <c r="AH25" s="2"/>
     </row>
     <row r="26">
-      <c r="A26" s="6" t="s">
-        <v>119</v>
-      </c>
-      <c r="B26" s="6" t="s">
+      <c r="A26" s="8" t="s">
+        <v>124</v>
+      </c>
+      <c r="B26" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="C26" s="6" t="s">
-        <v>120</v>
-      </c>
-      <c r="D26" s="6" t="s">
+      <c r="C26" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="D26" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E26" s="43">
+      <c r="E26" s="46">
         <v>45989.0</v>
       </c>
-      <c r="F26" s="6" t="s">
+      <c r="F26" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G26" s="6">
+      <c r="G26" s="8">
         <v>12.0</v>
       </c>
-      <c r="H26" s="6">
+      <c r="H26" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I26" s="6">
+      <c r="I26" s="8">
         <v>2048.0</v>
       </c>
-      <c r="J26" s="12">
+      <c r="J26" s="13">
         <v>34065.36</v>
       </c>
-      <c r="K26" s="12">
+      <c r="K26" s="13">
         <v>34065.36</v>
       </c>
-      <c r="L26" s="6">
+      <c r="L26" s="8">
         <v>0.0</v>
       </c>
       <c r="AB26" s="2"/>
@@ -9139,40 +9139,40 @@
       <c r="AH26" s="2"/>
     </row>
     <row r="27">
-      <c r="A27" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="B27" s="6" t="s">
-        <v>125</v>
-      </c>
-      <c r="C27" s="6" t="s">
-        <v>126</v>
-      </c>
-      <c r="D27" s="6" t="s">
+      <c r="A27" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="B27" s="8" t="s">
+        <v>128</v>
+      </c>
+      <c r="C27" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="D27" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E27" s="10">
+      <c r="E27" s="12">
         <v>46104.0</v>
       </c>
-      <c r="F27" s="6" t="s">
+      <c r="F27" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G27" s="6">
+      <c r="G27" s="8">
         <v>12.0</v>
       </c>
-      <c r="H27" s="6">
+      <c r="H27" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I27" s="6">
+      <c r="I27" s="8">
         <v>2048.0</v>
       </c>
-      <c r="J27" s="12">
+      <c r="J27" s="13">
         <v>1770880.5</v>
       </c>
-      <c r="K27" s="12">
+      <c r="K27" s="13">
         <v>843261.89</v>
       </c>
-      <c r="L27" s="12">
+      <c r="L27" s="13">
         <v>927618.61</v>
       </c>
       <c r="AB27" s="2"/>
@@ -9184,40 +9184,40 @@
       <c r="AH27" s="2"/>
     </row>
     <row r="28">
-      <c r="A28" s="6" t="s">
-        <v>129</v>
-      </c>
-      <c r="B28" s="6" t="s">
-        <v>130</v>
-      </c>
-      <c r="C28" s="6" t="s">
+      <c r="A28" s="8" t="s">
         <v>131</v>
       </c>
-      <c r="D28" s="6" t="s">
+      <c r="B28" s="8" t="s">
+        <v>132</v>
+      </c>
+      <c r="C28" s="8" t="s">
+        <v>133</v>
+      </c>
+      <c r="D28" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E28" s="10">
+      <c r="E28" s="12">
         <v>46120.0</v>
       </c>
-      <c r="F28" s="6" t="s">
+      <c r="F28" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G28" s="6">
+      <c r="G28" s="8">
         <v>12.0</v>
       </c>
-      <c r="H28" s="6">
+      <c r="H28" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I28" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="J28" s="12">
+      <c r="I28" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="J28" s="13">
         <v>1912292.52</v>
       </c>
-      <c r="K28" s="12">
+      <c r="K28" s="13">
         <v>1629834.48</v>
       </c>
-      <c r="L28" s="12">
+      <c r="L28" s="13">
         <v>282458.04</v>
       </c>
       <c r="AB28" s="2"/>
@@ -9229,40 +9229,40 @@
       <c r="AH28" s="2"/>
     </row>
     <row r="29">
-      <c r="A29" s="6" t="s">
-        <v>134</v>
-      </c>
-      <c r="B29" s="6" t="s">
+      <c r="A29" s="8" t="s">
         <v>135</v>
       </c>
-      <c r="C29" s="6" t="s">
-        <v>136</v>
-      </c>
-      <c r="D29" s="6" t="s">
+      <c r="B29" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="C29" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="D29" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E29" s="10">
+      <c r="E29" s="12">
         <v>46196.0</v>
       </c>
-      <c r="F29" s="6" t="s">
+      <c r="F29" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G29" s="6">
+      <c r="G29" s="8">
         <v>12.0</v>
       </c>
-      <c r="H29" s="6">
+      <c r="H29" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I29" s="6">
+      <c r="I29" s="8">
         <v>2048.0</v>
       </c>
-      <c r="J29" s="12">
+      <c r="J29" s="13">
         <v>1496713.48</v>
       </c>
-      <c r="K29" s="6">
+      <c r="K29" s="8">
         <v>0.0</v>
       </c>
-      <c r="L29" s="12">
+      <c r="L29" s="13">
         <v>1496713.48</v>
       </c>
       <c r="AB29" s="2"/>
@@ -9274,40 +9274,40 @@
       <c r="AH29" s="2"/>
     </row>
     <row r="30">
-      <c r="A30" s="6" t="s">
+      <c r="A30" s="8" t="s">
         <v>140</v>
       </c>
-      <c r="B30" s="6" t="s">
+      <c r="B30" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="C30" s="6" t="s">
-        <v>143</v>
-      </c>
-      <c r="D30" s="6" t="s">
+      <c r="C30" s="8" t="s">
+        <v>142</v>
+      </c>
+      <c r="D30" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E30" s="10">
+      <c r="E30" s="12">
         <v>46205.0</v>
       </c>
-      <c r="F30" s="6" t="s">
+      <c r="F30" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G30" s="6">
+      <c r="G30" s="8">
         <v>12.0</v>
       </c>
-      <c r="H30" s="6">
+      <c r="H30" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I30" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="J30" s="12">
+      <c r="I30" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="J30" s="13">
         <v>624166.14</v>
       </c>
-      <c r="K30" s="6">
+      <c r="K30" s="8">
         <v>0.0</v>
       </c>
-      <c r="L30" s="12">
+      <c r="L30" s="13">
         <v>624166.14</v>
       </c>
       <c r="AB30" s="2"/>
@@ -9319,40 +9319,40 @@
       <c r="AH30" s="2"/>
     </row>
     <row r="31">
-      <c r="A31" s="6" t="s">
+      <c r="A31" s="8" t="s">
+        <v>145</v>
+      </c>
+      <c r="B31" s="8" t="s">
         <v>146</v>
       </c>
-      <c r="B31" s="6" t="s">
+      <c r="C31" s="8" t="s">
         <v>147</v>
       </c>
-      <c r="C31" s="6" t="s">
-        <v>149</v>
-      </c>
-      <c r="D31" s="6" t="s">
+      <c r="D31" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E31" s="10">
+      <c r="E31" s="12">
         <v>46205.0</v>
       </c>
-      <c r="F31" s="6" t="s">
+      <c r="F31" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G31" s="6">
+      <c r="G31" s="8">
         <v>12.0</v>
       </c>
-      <c r="H31" s="6">
+      <c r="H31" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I31" s="6" t="s">
-        <v>110</v>
-      </c>
-      <c r="J31" s="12">
+      <c r="I31" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="J31" s="13">
         <v>18462.36</v>
       </c>
-      <c r="K31" s="6">
+      <c r="K31" s="8">
         <v>0.0</v>
       </c>
-      <c r="L31" s="12">
+      <c r="L31" s="13">
         <v>18462.36</v>
       </c>
       <c r="AB31" s="2"/>
@@ -9364,40 +9364,40 @@
       <c r="AH31" s="2"/>
     </row>
     <row r="32">
-      <c r="A32" s="6" t="s">
-        <v>152</v>
-      </c>
-      <c r="B32" s="6" t="s">
-        <v>147</v>
-      </c>
-      <c r="C32" s="12" t="s">
-        <v>153</v>
-      </c>
-      <c r="D32" s="6" t="s">
+      <c r="A32" s="8" t="s">
+        <v>149</v>
+      </c>
+      <c r="B32" s="8" t="s">
+        <v>146</v>
+      </c>
+      <c r="C32" s="13" t="s">
+        <v>151</v>
+      </c>
+      <c r="D32" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E32" s="10">
+      <c r="E32" s="12">
         <v>46213.0</v>
       </c>
-      <c r="F32" s="6" t="s">
+      <c r="F32" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G32" s="6">
+      <c r="G32" s="8">
         <v>12.0</v>
       </c>
-      <c r="H32" s="6">
+      <c r="H32" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I32" s="6" t="s">
-        <v>110</v>
-      </c>
-      <c r="J32" s="12">
+      <c r="I32" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="J32" s="13">
         <v>1530656.62</v>
       </c>
-      <c r="K32" s="6">
+      <c r="K32" s="8">
         <v>0.0</v>
       </c>
-      <c r="L32" s="12">
+      <c r="L32" s="13">
         <v>1530656.62</v>
       </c>
       <c r="AB32" s="2"/>
@@ -9409,40 +9409,40 @@
       <c r="AH32" s="2"/>
     </row>
     <row r="33">
-      <c r="A33" s="6" t="s">
-        <v>157</v>
-      </c>
-      <c r="B33" s="6" t="s">
-        <v>135</v>
-      </c>
-      <c r="C33" s="12" t="s">
-        <v>158</v>
-      </c>
-      <c r="D33" s="6" t="s">
+      <c r="A33" s="8" t="s">
+        <v>153</v>
+      </c>
+      <c r="B33" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="C33" s="13" t="s">
+        <v>155</v>
+      </c>
+      <c r="D33" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E33" s="10">
+      <c r="E33" s="12">
         <v>46227.0</v>
       </c>
-      <c r="F33" s="6" t="s">
+      <c r="F33" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G33" s="6">
+      <c r="G33" s="8">
         <v>12.0</v>
       </c>
-      <c r="H33" s="6">
+      <c r="H33" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I33" s="6">
+      <c r="I33" s="8">
         <v>2048.0</v>
       </c>
-      <c r="J33" s="12">
+      <c r="J33" s="13">
         <v>173846.38</v>
       </c>
-      <c r="K33" s="6">
+      <c r="K33" s="8">
         <v>0.0</v>
       </c>
-      <c r="L33" s="12">
+      <c r="L33" s="13">
         <v>173846.38</v>
       </c>
       <c r="AB33" s="2"/>
@@ -9454,40 +9454,40 @@
       <c r="AH33" s="2"/>
     </row>
     <row r="34">
-      <c r="A34" s="6" t="s">
-        <v>161</v>
-      </c>
-      <c r="B34" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="C34" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="D34" s="6" t="s">
+      <c r="A34" s="8" t="s">
+        <v>156</v>
+      </c>
+      <c r="B34" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="C34" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="D34" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E34" s="10">
+      <c r="E34" s="12">
         <v>46240.0</v>
       </c>
-      <c r="F34" s="6" t="s">
+      <c r="F34" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G34" s="6">
+      <c r="G34" s="8">
         <v>12.0</v>
       </c>
-      <c r="H34" s="6">
+      <c r="H34" s="8">
         <v>339039.0</v>
       </c>
-      <c r="I34" s="6" t="s">
-        <v>164</v>
-      </c>
-      <c r="J34" s="12">
+      <c r="I34" s="8" t="s">
+        <v>160</v>
+      </c>
+      <c r="J34" s="13">
         <v>236343.68</v>
       </c>
-      <c r="K34" s="6">
+      <c r="K34" s="8">
         <v>0.0</v>
       </c>
-      <c r="L34" s="12">
+      <c r="L34" s="13">
         <v>236343.68</v>
       </c>
       <c r="AB34" s="2"/>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (25/08/2026 08:36)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/01_Bases_Originais/005_CELOG_2025/005_CELOG-PAMALS_2025 online.xlsx
+++ b/Contrato 005/Dashboard/01_Bases_Originais/005_CELOG_2025/005_CELOG-PAMALS_2025 online.xlsx
@@ -66,12 +66,21 @@
     <t>Prazo Final de Vigência</t>
   </si>
   <si>
+    <t>2025NE000367</t>
+  </si>
+  <si>
     <t>Status</t>
   </si>
   <si>
+    <t>C25512</t>
+  </si>
+  <si>
     <t>Ação</t>
   </si>
   <si>
+    <t>25E0385</t>
+  </si>
+  <si>
     <t>PAG</t>
   </si>
   <si>
@@ -96,24 +105,15 @@
     <t>Fornecedor</t>
   </si>
   <si>
-    <t>2025NE000367</t>
-  </si>
-  <si>
     <t>Tipo Despesa /Receita</t>
   </si>
   <si>
-    <t>C25512</t>
-  </si>
-  <si>
     <t>Abrir</t>
   </si>
   <si>
     <t>Editar</t>
   </si>
   <si>
-    <t>25E0385</t>
-  </si>
-  <si>
     <t>005/CELOG-PAMALS/2025</t>
   </si>
   <si>
@@ -135,148 +135,166 @@
     <t>R$</t>
   </si>
   <si>
+    <t>2025NE000369</t>
+  </si>
+  <si>
+    <t>C25516</t>
+  </si>
+  <si>
+    <t>25E0387</t>
+  </si>
+  <si>
     <t>VEE ONE-MANUTENCAO E SERVICOS TECNICOS LTDA</t>
   </si>
   <si>
-    <t>2025NE000369</t>
-  </si>
-  <si>
-    <t>C25516</t>
-  </si>
-  <si>
-    <t>25E0387</t>
-  </si>
-  <si>
     <t>2025NE000371</t>
   </si>
   <si>
     <t>25E0389</t>
   </si>
   <si>
+    <t>2025NE000413</t>
+  </si>
+  <si>
+    <t>C25501</t>
+  </si>
+  <si>
+    <t>25E0403</t>
+  </si>
+  <si>
     <t>Módulo</t>
   </si>
   <si>
+    <t>20SP</t>
+  </si>
+  <si>
     <t>Referência</t>
   </si>
   <si>
     <t>Nº recibo</t>
   </si>
   <si>
-    <t>2025NE000413</t>
-  </si>
-  <si>
-    <t>C25501</t>
-  </si>
-  <si>
     <t>Nº</t>
   </si>
   <si>
-    <t>25E0403</t>
-  </si>
-  <si>
     <t>Data</t>
   </si>
   <si>
+    <t>2025NE000414</t>
+  </si>
+  <si>
+    <t>C25525</t>
+  </si>
+  <si>
     <t>Empenho</t>
   </si>
   <si>
+    <t>25E0431</t>
+  </si>
+  <si>
     <t>Observações</t>
   </si>
   <si>
-    <t>20SP</t>
-  </si>
-  <si>
     <t>Vencimento</t>
   </si>
   <si>
     <t>Valor das Nfs</t>
   </si>
   <si>
+    <t>21EM</t>
+  </si>
+  <si>
     <t>Ordem de Pagamento</t>
   </si>
   <si>
     <t>Faturado</t>
   </si>
   <si>
-    <t>2025NE000414</t>
-  </si>
-  <si>
     <t>Pendente</t>
   </si>
   <si>
-    <t>C25525</t>
-  </si>
-  <si>
-    <t>25E0431</t>
-  </si>
-  <si>
-    <t>21EM</t>
+    <t>2025NE000559</t>
+  </si>
+  <si>
+    <t>C25545</t>
+  </si>
+  <si>
+    <t>25E0524</t>
   </si>
   <si>
     <t>FEV/25</t>
   </si>
   <si>
+    <t>20X7</t>
+  </si>
+  <si>
     <t>-</t>
   </si>
   <si>
-    <t>2025NE000559</t>
-  </si>
-  <si>
-    <t>C25545</t>
+    <t>2025NE000770</t>
+  </si>
+  <si>
+    <t>25E0731</t>
   </si>
   <si>
     <t xml:space="preserve">2025NE000369 </t>
   </si>
   <si>
-    <t>25E0524</t>
-  </si>
-  <si>
-    <t>20X7</t>
+    <t>2025NE000774</t>
+  </si>
+  <si>
+    <t>25E0737</t>
   </si>
   <si>
     <t>2025NP001980</t>
   </si>
   <si>
-    <t>2025NE000770</t>
-  </si>
-  <si>
-    <t>25E0731</t>
-  </si>
-  <si>
-    <t>2025NE000774</t>
-  </si>
-  <si>
-    <t>25E0737</t>
+    <t>2025NE000843</t>
+  </si>
+  <si>
+    <t>C25630</t>
+  </si>
+  <si>
+    <t>25E0787</t>
+  </si>
+  <si>
+    <t>219C</t>
+  </si>
+  <si>
+    <t>2025NE001065</t>
+  </si>
+  <si>
+    <t>25E0999</t>
   </si>
   <si>
     <t>MAR/25</t>
   </si>
   <si>
-    <t>2025NE000843</t>
-  </si>
-  <si>
-    <t>C25630</t>
-  </si>
-  <si>
-    <t>25E0787</t>
-  </si>
-  <si>
     <t>2025NE000367, 2025NE000369, 2025NE000371, 2025NE000413</t>
   </si>
   <si>
-    <t>219C</t>
+    <t>2025NE001200</t>
+  </si>
+  <si>
+    <t>C25590</t>
+  </si>
+  <si>
+    <t>25E1128</t>
   </si>
   <si>
     <t>2025NP001979</t>
   </si>
   <si>
-    <t>2025NE001065</t>
-  </si>
-  <si>
     <t>ABR/25</t>
   </si>
   <si>
-    <t>25E0999</t>
+    <t>2025NE001598</t>
+  </si>
+  <si>
+    <t>C25814</t>
+  </si>
+  <si>
+    <t>25E1446</t>
   </si>
   <si>
     <t>2025NE000413, 2025NE000414, 2025NE000559</t>
@@ -285,34 +303,34 @@
     <t>2025NP002341</t>
   </si>
   <si>
+    <t>2025NE001627</t>
+  </si>
+  <si>
+    <t>25E1475</t>
+  </si>
+  <si>
     <t>MAI/25</t>
   </si>
   <si>
-    <t>2025NE001200</t>
-  </si>
-  <si>
-    <t>C25590</t>
-  </si>
-  <si>
-    <t>25E1128</t>
+    <t>2025NE001629</t>
+  </si>
+  <si>
+    <t>C25820</t>
+  </si>
+  <si>
+    <t>25E1477</t>
   </si>
   <si>
     <t>2025NP002884</t>
   </si>
   <si>
-    <t>2025NE001598</t>
-  </si>
-  <si>
-    <t>C25814</t>
-  </si>
-  <si>
-    <t>25E1446</t>
+    <t>2025NE001687</t>
+  </si>
+  <si>
+    <t>25E1535</t>
   </si>
   <si>
     <t>JUN/25</t>
-  </si>
-  <si>
-    <t>2025NE001627</t>
   </si>
   <si>
     <t>2025NE000005,
@@ -321,86 +339,128 @@
 2025NE000774</t>
   </si>
   <si>
-    <t>25E1475</t>
-  </si>
-  <si>
     <t>2025NP400522</t>
   </si>
   <si>
+    <t>2025NE001688</t>
+  </si>
+  <si>
+    <t>25E1536</t>
+  </si>
+  <si>
     <t>JUL/25</t>
   </si>
   <si>
+    <t>2025NE001689</t>
+  </si>
+  <si>
     <t>2025NE000843, 2025NE001200</t>
   </si>
   <si>
-    <t>2025NE001629</t>
-  </si>
-  <si>
-    <t>C25820</t>
-  </si>
-  <si>
-    <t>25E1477</t>
+    <t>25E1537</t>
   </si>
   <si>
     <t>2025NP003724</t>
   </si>
   <si>
+    <t>2025NE001690</t>
+  </si>
+  <si>
+    <t>25E1538</t>
+  </si>
+  <si>
     <t>AGO/25</t>
   </si>
   <si>
+    <t>2025NE001823</t>
+  </si>
+  <si>
+    <t>C25865</t>
+  </si>
+  <si>
+    <t>25E1666</t>
+  </si>
+  <si>
     <t>2025NP004558</t>
   </si>
   <si>
-    <t>2025NE001687</t>
-  </si>
-  <si>
-    <t>25E1535</t>
+    <t>2025NE001828</t>
+  </si>
+  <si>
+    <t>C25869</t>
+  </si>
+  <si>
+    <t>25E1667</t>
+  </si>
+  <si>
+    <t>20YJ</t>
   </si>
   <si>
     <t>SET/25</t>
+  </si>
+  <si>
+    <t>2025NE001830</t>
   </si>
   <si>
     <t>2025NE001688 
 2025NE001828</t>
   </si>
   <si>
+    <t>25E1669</t>
+  </si>
+  <si>
     <t>2025NP004897</t>
   </si>
   <si>
-    <t>2025NE001688</t>
+    <t>2025NE002200</t>
+  </si>
+  <si>
+    <t>C25863</t>
   </si>
   <si>
     <t>OUT/25</t>
   </si>
   <si>
-    <t>25E1536</t>
+    <t>25E2021</t>
   </si>
   <si>
     <t>2025NE001688, 2025NE001828, 2025NE002200</t>
   </si>
   <si>
+    <t>2025NE002237</t>
+  </si>
+  <si>
     <t>2025NP004932</t>
   </si>
   <si>
-    <t>2025NE001689</t>
-  </si>
-  <si>
-    <t>25E1537</t>
+    <t>25E2058</t>
   </si>
   <si>
     <t>NOV/25</t>
   </si>
   <si>
+    <t>2026NE000330</t>
+  </si>
+  <si>
+    <t>C26163</t>
+  </si>
+  <si>
+    <t>26E0320</t>
+  </si>
+  <si>
     <t>2025NE001687, 2025NE001689, 2025NE001690, 2025NE001823, 2025NE001830, 2025NE002237</t>
   </si>
   <si>
     <t>2026NP400440</t>
   </si>
   <si>
-    <t>2025NE001690</t>
-  </si>
-  <si>
-    <t>25E1538</t>
+    <t>2026NE000388</t>
+  </si>
+  <si>
+    <t>C26193</t>
+  </si>
+  <si>
+    <t>26E0375</t>
   </si>
   <si>
     <t>DEZ/25</t>
@@ -409,76 +469,76 @@
     <t>2025NE001065, 2025NE002200</t>
   </si>
   <si>
-    <t>2025NE001823</t>
+    <t>2026NE000748</t>
+  </si>
+  <si>
+    <t>C26312</t>
+  </si>
+  <si>
+    <t>26E0709</t>
   </si>
   <si>
     <t>2026NP400412</t>
   </si>
   <si>
-    <t>C25865</t>
-  </si>
-  <si>
-    <t>25E1666</t>
+    <t>2026NE000816</t>
+  </si>
+  <si>
+    <t>C26324</t>
+  </si>
+  <si>
+    <t>26E0776</t>
   </si>
   <si>
     <t>JAN/26</t>
   </si>
   <si>
-    <t>2025NE001828</t>
-  </si>
-  <si>
-    <t>C25869</t>
-  </si>
-  <si>
-    <t>25E1667</t>
-  </si>
-  <si>
-    <t>20YJ</t>
+    <t>2026NE000817</t>
+  </si>
+  <si>
+    <t>C26326</t>
+  </si>
+  <si>
+    <t>26E0777</t>
   </si>
   <si>
     <t>2026NP401035</t>
   </si>
   <si>
-    <t>2025NE001830</t>
-  </si>
-  <si>
-    <t>25E1669</t>
+    <t>2026NE000842</t>
+  </si>
+  <si>
+    <t>26E0803</t>
   </si>
   <si>
     <t>FEV/26</t>
   </si>
   <si>
-    <t>2025NE002200</t>
-  </si>
-  <si>
-    <t>C25863</t>
-  </si>
-  <si>
-    <t>25E2021</t>
-  </si>
-  <si>
     <t>2025NE001627, 2025NE001629, 2025NE001823</t>
   </si>
   <si>
+    <t>2026NE000944</t>
+  </si>
+  <si>
+    <t>26E0906</t>
+  </si>
+  <si>
     <t>2026NP402272</t>
   </si>
   <si>
-    <t>2025NE002237</t>
-  </si>
-  <si>
-    <t>25E2058</t>
+    <t>2026NE001015</t>
+  </si>
+  <si>
+    <t>C26363</t>
+  </si>
+  <si>
+    <t>26E0959</t>
   </si>
   <si>
     <t>MAR/26</t>
   </si>
   <si>
-    <t>2026NE000330</t>
-  </si>
-  <si>
-    <t>C26163</t>
-  </si>
-  <si>
-    <t>26E0320</t>
+    <t>20XV</t>
   </si>
   <si>
     <t>2025NE000770, 2025NE001627</t>
@@ -490,66 +550,24 @@
     <t>2026NP401762</t>
   </si>
   <si>
-    <t>2026NE000388</t>
-  </si>
-  <si>
-    <t>C26193</t>
-  </si>
-  <si>
-    <t>26E0375</t>
-  </si>
-  <si>
     <t>ABR/26</t>
   </si>
   <si>
-    <t>2026NE000748</t>
-  </si>
-  <si>
     <t>2025NE000770, 2025NE001065, 2025NE001627</t>
   </si>
   <si>
-    <t>C26312</t>
-  </si>
-  <si>
-    <t>26E0709</t>
-  </si>
-  <si>
-    <t>2026NE000816</t>
-  </si>
-  <si>
-    <t>C26324</t>
-  </si>
-  <si>
-    <t>26E0776</t>
-  </si>
-  <si>
     <t>REAJUSTE</t>
   </si>
   <si>
     <t>2026NP402148</t>
   </si>
   <si>
-    <t>2026NE000817</t>
-  </si>
-  <si>
-    <t>C26326</t>
-  </si>
-  <si>
-    <t>26E0777</t>
-  </si>
-  <si>
     <t>MAIO/26</t>
   </si>
   <si>
     <t>2026NP402373</t>
   </si>
   <si>
-    <t>2026NE000842</t>
-  </si>
-  <si>
-    <t>26E0803</t>
-  </si>
-  <si>
     <t>JUNHO/26</t>
   </si>
   <si>
@@ -562,28 +580,10 @@
     <t>2026NP402899</t>
   </si>
   <si>
-    <t>2026NE000944</t>
-  </si>
-  <si>
-    <t>26E0906</t>
-  </si>
-  <si>
     <t>JULHO/26</t>
   </si>
   <si>
     <t>R$ 1.629.834,48</t>
-  </si>
-  <si>
-    <t>2026NE001015</t>
-  </si>
-  <si>
-    <t>C26363</t>
-  </si>
-  <si>
-    <t>26E0959</t>
-  </si>
-  <si>
-    <t>20XV</t>
   </si>
   <si>
     <t>Módulo II – Parcial Orçamento 10 (FAB 2728)</t>
@@ -743,15 +743,15 @@
       <name val="Arial"/>
     </font>
     <font>
-      <sz val="10.0"/>
-      <color theme="1"/>
-      <name val="Times New Roman"/>
-    </font>
-    <font>
       <b/>
       <sz val="10.0"/>
       <color theme="1"/>
       <name val="Century Gothic"/>
+    </font>
+    <font>
+      <sz val="10.0"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
     </font>
     <font>
       <b/>
@@ -901,11 +901,11 @@
     <xf borderId="0" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="center"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
@@ -923,11 +923,11 @@
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="2" numFmtId="0" xfId="0" applyFill="1" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="4" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="4" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="right" readingOrder="0"/>
@@ -971,22 +971,22 @@
     <xf borderId="1" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="2" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="0" fontId="7" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf borderId="2" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="6" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="8" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="7" numFmtId="166" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="8" numFmtId="166" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="7" fontId="9" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
@@ -999,20 +999,20 @@
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="3" fillId="0" fontId="10" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="165" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="1" fillId="8" fontId="9" numFmtId="168" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="165" xfId="0" applyFont="1" applyNumberFormat="1"/>
-    <xf borderId="1" fillId="0" fontId="7" numFmtId="166" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="8" numFmtId="166" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="7" numFmtId="169" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="8" numFmtId="169" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="7" fontId="9" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="8" fontId="9" numFmtId="168" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
@@ -1024,14 +1024,14 @@
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="170" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
     <xf borderId="1" fillId="9" fontId="9" numFmtId="168" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="3" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="170" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="1" fillId="9" fontId="9" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
@@ -1055,7 +1055,7 @@
     <xf borderId="5" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="7" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="8" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="4" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
@@ -1064,10 +1064,10 @@
     <xf borderId="1" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="7" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="8" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="7" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="8" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="5" fontId="9" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
@@ -1445,14 +1445,14 @@
         <v>0</v>
       </c>
       <c r="V2" s="6"/>
-      <c r="W2" s="8"/>
-      <c r="X2" s="8"/>
-      <c r="Y2" s="8"/>
-      <c r="Z2" s="8"/>
-      <c r="AA2" s="8"/>
-      <c r="AB2" s="8"/>
-      <c r="AC2" s="8"/>
-      <c r="AD2" s="8"/>
+      <c r="W2" s="7"/>
+      <c r="X2" s="7"/>
+      <c r="Y2" s="7"/>
+      <c r="Z2" s="7"/>
+      <c r="AA2" s="7"/>
+      <c r="AB2" s="7"/>
+      <c r="AC2" s="7"/>
+      <c r="AD2" s="7"/>
     </row>
     <row r="3" ht="12.75" customHeight="1">
       <c r="A3" s="1"/>
@@ -1481,16 +1481,16 @@
     <row r="4" ht="12.75" customHeight="1">
       <c r="A4" s="14"/>
       <c r="B4" s="14"/>
-      <c r="C4" s="15" t="s">
+      <c r="C4" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="D4" s="15" t="s">
+      <c r="D4" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="E4" s="15" t="s">
+      <c r="E4" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="F4" s="15" t="s">
+      <c r="F4" s="16" t="s">
         <v>9</v>
       </c>
       <c r="G4" s="17" t="s">
@@ -1499,44 +1499,44 @@
       <c r="H4" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="I4" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="J4" s="15" t="s">
+      <c r="I4" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="K4" s="15" t="s">
-        <v>14</v>
-      </c>
-      <c r="L4" s="15" t="s">
+      <c r="J4" s="16" t="s">
         <v>15</v>
       </c>
+      <c r="K4" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="L4" s="16" t="s">
+        <v>18</v>
+      </c>
       <c r="M4" s="17" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="N4" s="17" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="O4" s="17" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="P4" s="17" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="Q4" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="R4" s="15" t="s">
-        <v>21</v>
-      </c>
-      <c r="S4" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="T4" s="15" t="s">
+      <c r="R4" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="S4" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="U4" s="15" t="s">
+      <c r="T4" s="16" t="s">
         <v>26</v>
+      </c>
+      <c r="U4" s="16" t="s">
+        <v>27</v>
       </c>
       <c r="V4" s="2"/>
     </row>
@@ -1590,7 +1590,7 @@
         <v>1.085943044E7</v>
       </c>
       <c r="S5" s="19" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="V5" s="2"/>
     </row>
@@ -1623,40 +1623,40 @@
       <c r="A8" s="23"/>
       <c r="B8" s="23"/>
       <c r="C8" s="28" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="D8" s="28" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="E8" s="29" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="F8" s="28" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="G8" s="28" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H8" s="28" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="I8" s="29" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="J8" s="28" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="K8" s="28" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="L8" s="30" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="M8" s="29" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="N8" s="28" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="O8" s="28"/>
       <c r="P8" s="27"/>
@@ -1665,14 +1665,14 @@
     <row r="9" ht="19.5" customHeight="1">
       <c r="A9" s="23"/>
       <c r="B9" s="23"/>
-      <c r="C9" s="31">
+      <c r="C9" s="32">
         <v>1.0</v>
       </c>
-      <c r="D9" s="32" t="s">
-        <v>61</v>
+      <c r="D9" s="33" t="s">
+        <v>64</v>
       </c>
       <c r="E9" s="34" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="F9" s="35">
         <v>594.0</v>
@@ -1681,7 +1681,7 @@
         <v>45740.0</v>
       </c>
       <c r="H9" s="35" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="I9" s="36"/>
       <c r="J9" s="36">
@@ -1691,7 +1691,7 @@
         <v>748504.24</v>
       </c>
       <c r="L9" s="35" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="M9" s="38">
         <f t="shared" ref="M9:M10" si="1">K9</f>
@@ -1706,11 +1706,11 @@
       <c r="A10" s="23"/>
       <c r="B10" s="23"/>
       <c r="C10" s="40"/>
-      <c r="D10" s="32" t="s">
-        <v>73</v>
+      <c r="D10" s="33" t="s">
+        <v>79</v>
       </c>
       <c r="E10" s="34" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="F10" s="35">
         <v>620.0</v>
@@ -1719,7 +1719,7 @@
         <v>45775.0</v>
       </c>
       <c r="H10" s="35" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="I10" s="36"/>
       <c r="J10" s="36">
@@ -1729,13 +1729,13 @@
         <v>1110378.24</v>
       </c>
       <c r="L10" s="35" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="M10" s="38">
         <f t="shared" si="1"/>
         <v>1110378.24</v>
       </c>
-      <c r="N10" s="41"/>
+      <c r="N10" s="42"/>
       <c r="O10" s="25"/>
       <c r="P10" s="27"/>
       <c r="V10" s="2"/>
@@ -1744,11 +1744,11 @@
       <c r="A11" s="23"/>
       <c r="B11" s="23"/>
       <c r="C11" s="40"/>
-      <c r="D11" s="32" t="s">
-        <v>81</v>
+      <c r="D11" s="33" t="s">
+        <v>85</v>
       </c>
       <c r="E11" s="34" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="F11" s="35">
         <v>634.0</v>
@@ -1757,7 +1757,7 @@
         <v>45799.0</v>
       </c>
       <c r="H11" s="35" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="I11" s="36"/>
       <c r="J11" s="36">
@@ -1767,12 +1767,12 @@
         <v>974557.12</v>
       </c>
       <c r="L11" s="34" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="M11" s="38">
         <v>974557.12</v>
       </c>
-      <c r="N11" s="41"/>
+      <c r="N11" s="42"/>
       <c r="O11" s="25"/>
       <c r="P11" s="27"/>
       <c r="V11" s="2"/>
@@ -1781,11 +1781,11 @@
       <c r="A12" s="23"/>
       <c r="B12" s="23"/>
       <c r="C12" s="40"/>
-      <c r="D12" s="32" t="s">
-        <v>85</v>
+      <c r="D12" s="33" t="s">
+        <v>93</v>
       </c>
       <c r="E12" s="34" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="F12" s="34">
         <v>660.0</v>
@@ -1794,7 +1794,7 @@
         <v>45856.0</v>
       </c>
       <c r="H12" s="44" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="I12" s="36"/>
       <c r="J12" s="36">
@@ -1804,7 +1804,7 @@
         <v>1402001.34</v>
       </c>
       <c r="L12" s="46" t="s">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="M12" s="38">
         <v>1402001.34</v>
@@ -1819,10 +1819,10 @@
       <c r="B13" s="23"/>
       <c r="C13" s="40"/>
       <c r="D13" s="48" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="E13" s="34" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="F13" s="35">
         <v>661.0</v>
@@ -1831,7 +1831,7 @@
         <v>45856.0</v>
       </c>
       <c r="H13" s="35" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="I13" s="43"/>
       <c r="J13" s="43">
@@ -1841,7 +1841,7 @@
         <v>1223702.3</v>
       </c>
       <c r="L13" s="34" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="M13" s="38">
         <v>1223702.3</v>
@@ -1856,10 +1856,10 @@
       <c r="B14" s="23"/>
       <c r="C14" s="40"/>
       <c r="D14" s="48" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="E14" s="34" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="F14" s="34">
         <v>688.0</v>
@@ -1868,7 +1868,7 @@
         <v>45901.0</v>
       </c>
       <c r="H14" s="34" t="s">
-        <v>99</v>
+        <v>107</v>
       </c>
       <c r="I14" s="43"/>
       <c r="J14" s="43">
@@ -1878,12 +1878,12 @@
         <v>1011677.95</v>
       </c>
       <c r="L14" s="34" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="M14" s="38">
         <v>1011677.95</v>
       </c>
-      <c r="N14" s="41"/>
+      <c r="N14" s="42"/>
       <c r="O14" s="25"/>
       <c r="P14" s="27"/>
       <c r="V14" s="2"/>
@@ -1893,10 +1893,10 @@
       <c r="B15" s="23"/>
       <c r="C15" s="40"/>
       <c r="D15" s="48" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="E15" s="34" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="F15" s="34">
         <v>696.0</v>
@@ -1905,7 +1905,7 @@
         <v>45923.0</v>
       </c>
       <c r="H15" s="34" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="I15" s="43"/>
       <c r="J15" s="43">
@@ -1915,7 +1915,7 @@
         <v>896744.06</v>
       </c>
       <c r="L15" s="34" t="s">
-        <v>105</v>
+        <v>116</v>
       </c>
       <c r="M15" s="38">
         <v>896744.06</v>
@@ -1929,10 +1929,10 @@
       <c r="B16" s="23"/>
       <c r="C16" s="40"/>
       <c r="D16" s="48" t="s">
-        <v>108</v>
+        <v>121</v>
       </c>
       <c r="E16" s="34" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="F16" s="34">
         <v>704.0</v>
@@ -1941,7 +1941,7 @@
         <v>45957.0</v>
       </c>
       <c r="H16" s="34" t="s">
-        <v>109</v>
+        <v>123</v>
       </c>
       <c r="I16" s="43"/>
       <c r="J16" s="43">
@@ -1951,12 +1951,12 @@
         <v>919329.06</v>
       </c>
       <c r="L16" s="34" t="s">
-        <v>110</v>
+        <v>125</v>
       </c>
       <c r="M16" s="38">
         <v>919329.06</v>
       </c>
-      <c r="N16" s="41"/>
+      <c r="N16" s="42"/>
       <c r="O16" s="25"/>
       <c r="V16" s="2"/>
     </row>
@@ -1965,7 +1965,7 @@
       <c r="B17" s="23"/>
       <c r="C17" s="40"/>
       <c r="D17" s="48" t="s">
-        <v>112</v>
+        <v>128</v>
       </c>
       <c r="E17" s="34"/>
       <c r="F17" s="34">
@@ -1975,7 +1975,7 @@
         <v>45972.0</v>
       </c>
       <c r="H17" s="34" t="s">
-        <v>114</v>
+        <v>130</v>
       </c>
       <c r="I17" s="34"/>
       <c r="J17" s="43">
@@ -1985,12 +1985,12 @@
         <v>1157009.26</v>
       </c>
       <c r="L17" s="34" t="s">
-        <v>115</v>
+        <v>132</v>
       </c>
       <c r="M17" s="38">
         <v>1157009.26</v>
       </c>
-      <c r="N17" s="50"/>
+      <c r="N17" s="51"/>
       <c r="O17" s="25"/>
       <c r="V17" s="2"/>
     </row>
@@ -1999,10 +1999,10 @@
       <c r="B18" s="23"/>
       <c r="C18" s="40"/>
       <c r="D18" s="48" t="s">
-        <v>118</v>
+        <v>134</v>
       </c>
       <c r="E18" s="34" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="F18" s="34">
         <v>728.0</v>
@@ -2011,7 +2011,7 @@
         <v>46008.0</v>
       </c>
       <c r="H18" s="34" t="s">
-        <v>119</v>
+        <v>138</v>
       </c>
       <c r="I18" s="34"/>
       <c r="J18" s="43">
@@ -2021,28 +2021,28 @@
         <v>1214597.952</v>
       </c>
       <c r="L18" s="34" t="s">
-        <v>120</v>
+        <v>139</v>
       </c>
       <c r="M18" s="38">
         <v>1214597.952</v>
       </c>
-      <c r="N18" s="50"/>
+      <c r="N18" s="51"/>
       <c r="O18" s="25"/>
       <c r="R18" s="27"/>
       <c r="S18" s="27"/>
       <c r="T18" s="27"/>
       <c r="U18" s="27"/>
-      <c r="V18" s="51"/>
+      <c r="V18" s="52"/>
     </row>
     <row r="19">
       <c r="A19" s="23"/>
       <c r="B19" s="23"/>
       <c r="C19" s="40"/>
       <c r="D19" s="48" t="s">
-        <v>123</v>
+        <v>143</v>
       </c>
       <c r="E19" s="34" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="F19" s="34">
         <v>278.0</v>
@@ -2051,7 +2051,7 @@
         <v>46042.0</v>
       </c>
       <c r="H19" s="34" t="s">
-        <v>124</v>
+        <v>144</v>
       </c>
       <c r="I19" s="43"/>
       <c r="J19" s="43">
@@ -2061,25 +2061,25 @@
         <v>967082.09</v>
       </c>
       <c r="L19" s="34" t="s">
-        <v>126</v>
+        <v>148</v>
       </c>
       <c r="M19" s="38">
         <v>967082.09</v>
       </c>
-      <c r="N19" s="50"/>
+      <c r="N19" s="51"/>
       <c r="O19" s="25"/>
       <c r="R19" s="27"/>
       <c r="S19" s="27"/>
       <c r="T19" s="27"/>
       <c r="U19" s="27"/>
-      <c r="V19" s="51"/>
+      <c r="V19" s="52"/>
     </row>
     <row r="20">
       <c r="A20" s="23"/>
       <c r="B20" s="23"/>
       <c r="C20" s="40"/>
       <c r="D20" s="48" t="s">
-        <v>129</v>
+        <v>152</v>
       </c>
       <c r="E20" s="34"/>
       <c r="F20" s="34">
@@ -2089,7 +2089,7 @@
         <v>46078.0</v>
       </c>
       <c r="H20" s="34" t="s">
-        <v>125</v>
+        <v>113</v>
       </c>
       <c r="I20" s="43"/>
       <c r="J20" s="43">
@@ -2099,25 +2099,25 @@
         <v>719561.08</v>
       </c>
       <c r="L20" s="34" t="s">
-        <v>134</v>
+        <v>156</v>
       </c>
       <c r="M20" s="38">
         <v>719561.08</v>
       </c>
-      <c r="N20" s="50"/>
+      <c r="N20" s="51"/>
       <c r="O20" s="25"/>
       <c r="R20" s="27"/>
       <c r="S20" s="27"/>
       <c r="T20" s="27"/>
       <c r="U20" s="27"/>
-      <c r="V20" s="51"/>
+      <c r="V20" s="52"/>
     </row>
     <row r="21">
       <c r="A21" s="23"/>
       <c r="B21" s="23"/>
       <c r="C21" s="40"/>
       <c r="D21" s="48" t="s">
-        <v>137</v>
+        <v>159</v>
       </c>
       <c r="E21" s="34"/>
       <c r="F21" s="34">
@@ -2127,7 +2127,7 @@
         <v>46094.0</v>
       </c>
       <c r="H21" s="34" t="s">
-        <v>141</v>
+        <v>160</v>
       </c>
       <c r="I21" s="43"/>
       <c r="J21" s="43">
@@ -2137,25 +2137,25 @@
         <v>885881.08</v>
       </c>
       <c r="L21" s="34" t="s">
-        <v>142</v>
+        <v>163</v>
       </c>
       <c r="M21" s="38">
         <v>885881.08</v>
       </c>
-      <c r="N21" s="50"/>
+      <c r="N21" s="51"/>
       <c r="O21" s="25"/>
       <c r="R21" s="27"/>
       <c r="S21" s="27"/>
       <c r="T21" s="27"/>
       <c r="U21" s="27"/>
-      <c r="V21" s="51"/>
+      <c r="V21" s="52"/>
     </row>
     <row r="22">
       <c r="A22" s="23"/>
       <c r="B22" s="23"/>
       <c r="C22" s="40"/>
       <c r="D22" s="48" t="s">
-        <v>145</v>
+        <v>167</v>
       </c>
       <c r="E22" s="34"/>
       <c r="F22" s="34">
@@ -2165,35 +2165,35 @@
         <v>46128.0</v>
       </c>
       <c r="H22" s="34" t="s">
-        <v>149</v>
+        <v>169</v>
       </c>
       <c r="I22" s="43"/>
       <c r="J22" s="43">
         <v>46164.0</v>
       </c>
       <c r="K22" s="45" t="s">
-        <v>150</v>
+        <v>170</v>
       </c>
       <c r="L22" s="34" t="s">
-        <v>151</v>
+        <v>171</v>
       </c>
       <c r="M22" s="38" t="s">
-        <v>150</v>
-      </c>
-      <c r="N22" s="50"/>
+        <v>170</v>
+      </c>
+      <c r="N22" s="51"/>
       <c r="O22" s="25"/>
       <c r="R22" s="27"/>
       <c r="S22" s="27"/>
       <c r="T22" s="27"/>
       <c r="U22" s="27"/>
-      <c r="V22" s="51"/>
+      <c r="V22" s="52"/>
     </row>
     <row r="23">
       <c r="A23" s="23"/>
       <c r="B23" s="23"/>
       <c r="C23" s="40"/>
       <c r="D23" s="48" t="s">
-        <v>155</v>
+        <v>172</v>
       </c>
       <c r="E23" s="34"/>
       <c r="F23" s="34">
@@ -2203,7 +2203,7 @@
         <v>46156.0</v>
       </c>
       <c r="H23" s="34" t="s">
-        <v>157</v>
+        <v>173</v>
       </c>
       <c r="I23" s="43"/>
       <c r="J23" s="43">
@@ -2213,7 +2213,7 @@
         <v>1108954.4358333333</v>
       </c>
       <c r="L23" s="34" t="s">
-        <v>142</v>
+        <v>163</v>
       </c>
       <c r="M23" s="38">
         <v>1108954.4358333333</v>
@@ -2224,14 +2224,14 @@
       <c r="S23" s="27"/>
       <c r="T23" s="27"/>
       <c r="U23" s="27"/>
-      <c r="V23" s="51"/>
+      <c r="V23" s="52"/>
     </row>
     <row r="24">
       <c r="A24" s="23"/>
       <c r="B24" s="23"/>
       <c r="C24" s="40"/>
       <c r="D24" s="48" t="s">
-        <v>163</v>
+        <v>174</v>
       </c>
       <c r="E24" s="34"/>
       <c r="F24" s="34">
@@ -2241,7 +2241,7 @@
         <v>46149.0</v>
       </c>
       <c r="H24" s="34" t="s">
-        <v>157</v>
+        <v>173</v>
       </c>
       <c r="I24" s="43"/>
       <c r="J24" s="43">
@@ -2251,7 +2251,7 @@
         <v>218206.1</v>
       </c>
       <c r="L24" s="34" t="s">
-        <v>164</v>
+        <v>175</v>
       </c>
       <c r="M24" s="38">
         <v>218206.1</v>
@@ -2262,14 +2262,14 @@
       <c r="S24" s="27"/>
       <c r="T24" s="27"/>
       <c r="U24" s="27"/>
-      <c r="V24" s="51"/>
+      <c r="V24" s="52"/>
     </row>
     <row r="25">
       <c r="A25" s="23"/>
       <c r="B25" s="23"/>
       <c r="C25" s="40"/>
       <c r="D25" s="48" t="s">
-        <v>168</v>
+        <v>176</v>
       </c>
       <c r="E25" s="34"/>
       <c r="F25" s="34">
@@ -2279,7 +2279,7 @@
         <v>46156.0</v>
       </c>
       <c r="H25" s="34" t="s">
-        <v>157</v>
+        <v>173</v>
       </c>
       <c r="I25" s="43"/>
       <c r="J25" s="43">
@@ -2289,7 +2289,7 @@
         <v>1549250.84</v>
       </c>
       <c r="L25" s="34" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="M25" s="38">
         <v>1549250.84</v>
@@ -2300,14 +2300,14 @@
       <c r="S25" s="27"/>
       <c r="T25" s="27"/>
       <c r="U25" s="27"/>
-      <c r="V25" s="51"/>
+      <c r="V25" s="52"/>
     </row>
     <row r="26">
       <c r="A26" s="23"/>
       <c r="B26" s="23"/>
       <c r="C26" s="55"/>
       <c r="D26" s="48" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="E26" s="34"/>
       <c r="F26" s="34">
@@ -2317,20 +2317,20 @@
         <v>46230.0</v>
       </c>
       <c r="H26" s="34" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="I26" s="43"/>
       <c r="J26" s="43">
         <v>46262.0</v>
       </c>
       <c r="K26" s="45" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="L26" s="34" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="M26" s="38" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="N26" s="54"/>
       <c r="O26" s="25"/>
@@ -2338,14 +2338,14 @@
       <c r="S26" s="27"/>
       <c r="T26" s="27"/>
       <c r="U26" s="27"/>
-      <c r="V26" s="51"/>
+      <c r="V26" s="52"/>
     </row>
     <row r="27">
       <c r="A27" s="23"/>
       <c r="B27" s="23"/>
       <c r="C27" s="35"/>
       <c r="D27" s="48" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="E27" s="34"/>
       <c r="F27" s="34">
@@ -2355,7 +2355,7 @@
         <v>46252.0</v>
       </c>
       <c r="H27" s="34" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="I27" s="43"/>
       <c r="J27" s="43">
@@ -2364,7 +2364,7 @@
       <c r="K27" s="45"/>
       <c r="L27" s="34"/>
       <c r="M27" s="38" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="N27" s="54"/>
       <c r="O27" s="25"/>
@@ -2372,40 +2372,40 @@
       <c r="S27" s="27"/>
       <c r="T27" s="27"/>
       <c r="U27" s="27"/>
-      <c r="V27" s="51"/>
+      <c r="V27" s="52"/>
     </row>
     <row r="28" ht="30.75" customHeight="1">
       <c r="A28" s="23"/>
       <c r="B28" s="23"/>
       <c r="C28" s="28" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="D28" s="28" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="E28" s="29" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="F28" s="29" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="G28" s="29"/>
       <c r="H28" s="29" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="I28" s="29"/>
       <c r="J28" s="29"/>
       <c r="K28" s="29" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="L28" s="29" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="M28" s="29" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="N28" s="29" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="O28" s="25"/>
       <c r="P28" s="27"/>
@@ -2413,7 +2413,7 @@
       <c r="S28" s="27"/>
       <c r="T28" s="27"/>
       <c r="U28" s="27"/>
-      <c r="V28" s="51"/>
+      <c r="V28" s="52"/>
       <c r="W28" s="27"/>
       <c r="X28" s="27"/>
       <c r="Y28" s="27"/>
@@ -2425,7 +2425,7 @@
     <row r="29" ht="12.75" customHeight="1">
       <c r="A29" s="23"/>
       <c r="B29" s="23"/>
-      <c r="C29" s="31">
+      <c r="C29" s="32">
         <v>2.0</v>
       </c>
       <c r="D29" s="56" t="s">
@@ -2439,7 +2439,7 @@
         <v>45791.0</v>
       </c>
       <c r="H29" s="35" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="I29" s="36"/>
       <c r="J29" s="36">
@@ -2454,7 +2454,7 @@
       <c r="M29" s="57">
         <v>188246.17</v>
       </c>
-      <c r="N29" s="50"/>
+      <c r="N29" s="51"/>
       <c r="O29" s="25"/>
       <c r="P29" s="27"/>
       <c r="Q29" s="27"/>
@@ -2462,7 +2462,7 @@
       <c r="S29" s="27"/>
       <c r="T29" s="27"/>
       <c r="U29" s="27"/>
-      <c r="V29" s="51"/>
+      <c r="V29" s="52"/>
       <c r="W29" s="27"/>
       <c r="X29" s="27"/>
       <c r="Y29" s="27"/>
@@ -2503,7 +2503,7 @@
       <c r="M30" s="38">
         <v>112720.77</v>
       </c>
-      <c r="N30" s="50"/>
+      <c r="N30" s="51"/>
       <c r="O30" s="25"/>
       <c r="P30" s="27"/>
       <c r="Q30" s="27"/>
@@ -2511,7 +2511,7 @@
       <c r="S30" s="27"/>
       <c r="T30" s="27"/>
       <c r="U30" s="27"/>
-      <c r="V30" s="51"/>
+      <c r="V30" s="52"/>
       <c r="W30" s="27"/>
       <c r="X30" s="27"/>
       <c r="Y30" s="27"/>
@@ -2537,7 +2537,7 @@
         <v>45853.0</v>
       </c>
       <c r="H31" s="34" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I31" s="43"/>
       <c r="J31" s="43">
@@ -2552,7 +2552,7 @@
       <c r="M31" s="38">
         <v>378307.61</v>
       </c>
-      <c r="N31" s="50"/>
+      <c r="N31" s="51"/>
       <c r="O31" s="25"/>
       <c r="P31" s="62"/>
       <c r="Q31" s="27"/>
@@ -2560,7 +2560,7 @@
       <c r="S31" s="27"/>
       <c r="T31" s="27"/>
       <c r="U31" s="27"/>
-      <c r="V31" s="51"/>
+      <c r="V31" s="52"/>
       <c r="W31" s="27"/>
       <c r="X31" s="27"/>
       <c r="Y31" s="27"/>
@@ -2586,7 +2586,7 @@
         <v>45910.0</v>
       </c>
       <c r="H32" s="34" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I32" s="43"/>
       <c r="J32" s="43">
@@ -2601,7 +2601,7 @@
       <c r="M32" s="38">
         <v>3315.04710000003</v>
       </c>
-      <c r="N32" s="50"/>
+      <c r="N32" s="51"/>
       <c r="O32" s="25"/>
       <c r="P32" s="62"/>
       <c r="Q32" s="27"/>
@@ -2609,7 +2609,7 @@
       <c r="S32" s="27"/>
       <c r="T32" s="27"/>
       <c r="U32" s="27"/>
-      <c r="V32" s="51"/>
+      <c r="V32" s="52"/>
       <c r="W32" s="27"/>
       <c r="X32" s="27"/>
       <c r="Y32" s="27"/>
@@ -2635,7 +2635,7 @@
         <v>45904.0</v>
       </c>
       <c r="H33" s="34" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="I33" s="64"/>
       <c r="J33" s="64">
@@ -2650,7 +2650,7 @@
       <c r="M33" s="38">
         <v>198332.75</v>
       </c>
-      <c r="N33" s="50"/>
+      <c r="N33" s="51"/>
       <c r="O33" s="25"/>
       <c r="P33" s="62"/>
       <c r="Q33" s="27"/>
@@ -2658,7 +2658,7 @@
       <c r="S33" s="27"/>
       <c r="T33" s="27"/>
       <c r="U33" s="27"/>
-      <c r="V33" s="51"/>
+      <c r="V33" s="52"/>
       <c r="W33" s="27"/>
       <c r="X33" s="27"/>
       <c r="Y33" s="27"/>
@@ -2684,7 +2684,7 @@
         <v>46008.0</v>
       </c>
       <c r="H34" s="34" t="s">
-        <v>138</v>
+        <v>126</v>
       </c>
       <c r="I34" s="64"/>
       <c r="J34" s="64">
@@ -2699,7 +2699,7 @@
       <c r="M34" s="66" t="s">
         <v>198</v>
       </c>
-      <c r="N34" s="50"/>
+      <c r="N34" s="51"/>
       <c r="O34" s="25"/>
       <c r="P34" s="62"/>
       <c r="Q34" s="27"/>
@@ -2707,7 +2707,7 @@
       <c r="S34" s="27"/>
       <c r="T34" s="27"/>
       <c r="U34" s="27"/>
-      <c r="V34" s="51"/>
+      <c r="V34" s="52"/>
       <c r="W34" s="27"/>
       <c r="X34" s="27"/>
       <c r="Y34" s="27"/>
@@ -2733,7 +2733,7 @@
         <v>45930.0</v>
       </c>
       <c r="H35" s="34" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="I35" s="64"/>
       <c r="J35" s="64">
@@ -2748,7 +2748,7 @@
       <c r="M35" s="57" t="s">
         <v>202</v>
       </c>
-      <c r="N35" s="50"/>
+      <c r="N35" s="51"/>
       <c r="O35" s="25"/>
       <c r="P35" s="62"/>
       <c r="Q35" s="27"/>
@@ -2756,7 +2756,7 @@
       <c r="S35" s="27"/>
       <c r="T35" s="27"/>
       <c r="U35" s="27"/>
-      <c r="V35" s="51"/>
+      <c r="V35" s="52"/>
       <c r="W35" s="27"/>
       <c r="X35" s="27"/>
       <c r="Y35" s="27"/>
@@ -2782,7 +2782,7 @@
         <v>45968.0</v>
       </c>
       <c r="H36" s="34" t="s">
-        <v>130</v>
+        <v>117</v>
       </c>
       <c r="I36" s="64"/>
       <c r="J36" s="64">
@@ -2797,7 +2797,7 @@
       <c r="M36" s="57" t="s">
         <v>205</v>
       </c>
-      <c r="N36" s="50"/>
+      <c r="N36" s="51"/>
       <c r="O36" s="25"/>
       <c r="P36" s="62"/>
       <c r="Q36" s="27"/>
@@ -2805,7 +2805,7 @@
       <c r="S36" s="27"/>
       <c r="T36" s="27"/>
       <c r="U36" s="27"/>
-      <c r="V36" s="51"/>
+      <c r="V36" s="52"/>
       <c r="W36" s="27"/>
       <c r="X36" s="27"/>
       <c r="Y36" s="27"/>
@@ -2831,7 +2831,7 @@
         <v>46043.0</v>
       </c>
       <c r="H37" s="63" t="s">
-        <v>125</v>
+        <v>113</v>
       </c>
       <c r="I37" s="68"/>
       <c r="J37" s="67">
@@ -2846,7 +2846,7 @@
       <c r="M37" s="38">
         <v>11372.9</v>
       </c>
-      <c r="N37" s="50"/>
+      <c r="N37" s="51"/>
       <c r="O37" s="25"/>
       <c r="P37" s="27"/>
       <c r="Q37" s="27"/>
@@ -2854,7 +2854,7 @@
       <c r="S37" s="27"/>
       <c r="T37" s="27"/>
       <c r="U37" s="27"/>
-      <c r="V37" s="51"/>
+      <c r="V37" s="52"/>
       <c r="W37" s="27"/>
       <c r="X37" s="27"/>
       <c r="Y37" s="27"/>
@@ -2881,7 +2881,7 @@
       <c r="K38" s="45"/>
       <c r="L38" s="34"/>
       <c r="M38" s="38"/>
-      <c r="N38" s="50">
+      <c r="N38" s="51">
         <v>15854.78</v>
       </c>
       <c r="O38" s="25"/>
@@ -2891,7 +2891,7 @@
       <c r="S38" s="27"/>
       <c r="T38" s="27"/>
       <c r="U38" s="27"/>
-      <c r="V38" s="51"/>
+      <c r="V38" s="52"/>
       <c r="W38" s="27"/>
       <c r="X38" s="27"/>
       <c r="Y38" s="27"/>
@@ -2928,7 +2928,7 @@
       <c r="S39" s="27"/>
       <c r="T39" s="27"/>
       <c r="U39" s="27"/>
-      <c r="V39" s="51"/>
+      <c r="V39" s="52"/>
       <c r="W39" s="27"/>
       <c r="X39" s="27"/>
       <c r="Y39" s="27"/>
@@ -2965,7 +2965,7 @@
       <c r="S40" s="27"/>
       <c r="T40" s="27"/>
       <c r="U40" s="27"/>
-      <c r="V40" s="51"/>
+      <c r="V40" s="52"/>
       <c r="W40" s="27"/>
       <c r="X40" s="27"/>
       <c r="Y40" s="27"/>
@@ -3000,7 +3000,7 @@
       <c r="S41" s="27"/>
       <c r="T41" s="27"/>
       <c r="U41" s="27"/>
-      <c r="V41" s="51"/>
+      <c r="V41" s="52"/>
       <c r="W41" s="27"/>
       <c r="X41" s="27"/>
       <c r="Y41" s="27"/>
@@ -3012,7 +3012,7 @@
     <row r="42" ht="12.75" customHeight="1">
       <c r="A42" s="23"/>
       <c r="B42" s="23"/>
-      <c r="C42" s="31">
+      <c r="C42" s="32">
         <v>3.0</v>
       </c>
       <c r="D42" s="59" t="s">
@@ -3026,7 +3026,7 @@
         <v>46104.0</v>
       </c>
       <c r="H42" s="63" t="s">
-        <v>125</v>
+        <v>113</v>
       </c>
       <c r="I42" s="68"/>
       <c r="J42" s="67">
@@ -3041,7 +3041,7 @@
       <c r="M42" s="72">
         <v>27801.11</v>
       </c>
-      <c r="N42" s="50"/>
+      <c r="N42" s="51"/>
       <c r="O42" s="25"/>
       <c r="P42" s="27"/>
       <c r="Q42" s="27"/>
@@ -3049,7 +3049,7 @@
       <c r="S42" s="27"/>
       <c r="T42" s="27"/>
       <c r="U42" s="27"/>
-      <c r="V42" s="51"/>
+      <c r="V42" s="52"/>
       <c r="W42" s="27"/>
       <c r="X42" s="27"/>
       <c r="Y42" s="27"/>
@@ -3073,7 +3073,7 @@
         <v>46199.0</v>
       </c>
       <c r="H43" s="63" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="I43" s="68"/>
       <c r="J43" s="67">
@@ -3083,12 +3083,12 @@
         <v>58868.35</v>
       </c>
       <c r="L43" s="34" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="M43" s="72">
         <v>58868.35</v>
       </c>
-      <c r="N43" s="50"/>
+      <c r="N43" s="51"/>
       <c r="V43" s="2"/>
     </row>
     <row r="44" ht="12.75" customHeight="1">
@@ -8042,7 +8042,7 @@
       <c r="AH1" s="4"/>
     </row>
     <row r="2">
-      <c r="A2" s="7">
+      <c r="A2" s="8">
         <v>46258.0</v>
       </c>
       <c r="L2" s="9" t="s">
@@ -8084,10 +8084,10 @@
       <c r="I3" s="11">
         <v>2048.0</v>
       </c>
-      <c r="J3" s="16">
+      <c r="J3" s="15">
         <v>1000.0</v>
       </c>
-      <c r="K3" s="16">
+      <c r="K3" s="15">
         <v>1000.0</v>
       </c>
       <c r="L3" s="11">
@@ -8103,13 +8103,13 @@
     </row>
     <row r="4">
       <c r="A4" s="11" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="D4" s="11" t="s">
         <v>4</v>
@@ -8129,10 +8129,10 @@
       <c r="I4" s="11">
         <v>2048.0</v>
       </c>
-      <c r="J4" s="16">
+      <c r="J4" s="15">
         <v>52250.04</v>
       </c>
-      <c r="K4" s="16">
+      <c r="K4" s="15">
         <v>52250.04</v>
       </c>
       <c r="L4" s="11">
@@ -8148,13 +8148,13 @@
     </row>
     <row r="5">
       <c r="A5" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="B5" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="B5" s="11" t="s">
+      <c r="C5" s="11" t="s">
         <v>37</v>
-      </c>
-      <c r="C5" s="11" t="s">
-        <v>38</v>
       </c>
       <c r="D5" s="11" t="s">
         <v>4</v>
@@ -8174,10 +8174,10 @@
       <c r="I5" s="11">
         <v>2048.0</v>
       </c>
-      <c r="J5" s="16">
+      <c r="J5" s="15">
         <v>881914.18</v>
       </c>
-      <c r="K5" s="16">
+      <c r="K5" s="15">
         <v>881914.18</v>
       </c>
       <c r="L5" s="11">
@@ -8196,7 +8196,7 @@
         <v>39</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C6" s="11" t="s">
         <v>40</v>
@@ -8219,10 +8219,10 @@
       <c r="I6" s="11">
         <v>2048.0</v>
       </c>
-      <c r="J6" s="16">
+      <c r="J6" s="15">
         <v>750000.0</v>
       </c>
-      <c r="K6" s="16">
+      <c r="K6" s="15">
         <v>750000.0</v>
       </c>
       <c r="L6" s="11">
@@ -8238,13 +8238,13 @@
     </row>
     <row r="7">
       <c r="A7" s="11" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="D7" s="11" t="s">
         <v>4</v>
@@ -8262,12 +8262,12 @@
         <v>339039.0</v>
       </c>
       <c r="I7" s="11" t="s">
-        <v>51</v>
-      </c>
-      <c r="J7" s="16">
+        <v>45</v>
+      </c>
+      <c r="J7" s="15">
         <v>949835.78</v>
       </c>
-      <c r="K7" s="16">
+      <c r="K7" s="15">
         <v>949835.78</v>
       </c>
       <c r="L7" s="11">
@@ -8283,13 +8283,13 @@
     </row>
     <row r="8">
       <c r="A8" s="11" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="D8" s="11" t="s">
         <v>4</v>
@@ -8307,18 +8307,18 @@
         <v>339039.0</v>
       </c>
       <c r="I8" s="11" t="s">
-        <v>60</v>
-      </c>
-      <c r="J8" s="16">
+        <v>57</v>
+      </c>
+      <c r="J8" s="15">
         <v>524584.95</v>
       </c>
-      <c r="K8" s="16">
+      <c r="K8" s="15">
         <v>524584.95</v>
       </c>
       <c r="L8" s="11">
         <v>0.0</v>
       </c>
-      <c r="O8" s="33"/>
+      <c r="O8" s="31"/>
       <c r="AB8" s="4"/>
       <c r="AC8" s="4"/>
       <c r="AD8" s="4"/>
@@ -8329,13 +8329,13 @@
     </row>
     <row r="9">
       <c r="A9" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="C9" s="11" t="s">
         <v>63</v>
-      </c>
-      <c r="B9" s="11" t="s">
-        <v>64</v>
-      </c>
-      <c r="C9" s="11" t="s">
-        <v>66</v>
       </c>
       <c r="D9" s="11" t="s">
         <v>4</v>
@@ -8353,12 +8353,12 @@
         <v>339039.0</v>
       </c>
       <c r="I9" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="J9" s="16">
+        <v>65</v>
+      </c>
+      <c r="J9" s="15">
         <v>211614.23</v>
       </c>
-      <c r="K9" s="16">
+      <c r="K9" s="15">
         <v>211614.23</v>
       </c>
       <c r="L9" s="11">
@@ -8374,13 +8374,13 @@
     </row>
     <row r="10">
       <c r="A10" s="11" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="D10" s="11" t="s">
         <v>4</v>
@@ -8400,13 +8400,13 @@
       <c r="I10" s="11">
         <v>2048.0</v>
       </c>
-      <c r="J10" s="16">
+      <c r="J10" s="15">
         <v>2391157.42</v>
       </c>
-      <c r="K10" s="16">
+      <c r="K10" s="15">
         <v>2391157.41</v>
       </c>
-      <c r="L10" s="16">
+      <c r="L10" s="15">
         <v>0.01</v>
       </c>
       <c r="AB10" s="4"/>
@@ -8419,13 +8419,13 @@
     </row>
     <row r="11">
       <c r="A11" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="B11" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="C11" s="11" t="s">
         <v>71</v>
-      </c>
-      <c r="B11" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="C11" s="11" t="s">
-        <v>72</v>
       </c>
       <c r="D11" s="11" t="s">
         <v>4</v>
@@ -8445,10 +8445,10 @@
       <c r="I11" s="11">
         <v>2048.0</v>
       </c>
-      <c r="J11" s="16">
+      <c r="J11" s="15">
         <v>618154.39</v>
       </c>
-      <c r="K11" s="16">
+      <c r="K11" s="15">
         <v>618154.38</v>
       </c>
       <c r="L11" s="11">
@@ -8464,13 +8464,13 @@
     </row>
     <row r="12">
       <c r="A12" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="B12" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="B12" s="11" t="s">
+      <c r="C12" s="11" t="s">
         <v>75</v>
-      </c>
-      <c r="C12" s="11" t="s">
-        <v>76</v>
       </c>
       <c r="D12" s="11" t="s">
         <v>4</v>
@@ -8488,12 +8488,12 @@
         <v>339039.0</v>
       </c>
       <c r="I12" s="11" t="s">
-        <v>78</v>
-      </c>
-      <c r="J12" s="16">
+        <v>76</v>
+      </c>
+      <c r="J12" s="15">
         <v>1600334.09</v>
       </c>
-      <c r="K12" s="16">
+      <c r="K12" s="15">
         <v>1600334.09</v>
       </c>
       <c r="L12" s="11">
@@ -8509,13 +8509,13 @@
     </row>
     <row r="13">
       <c r="A13" s="11" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="D13" s="11" t="s">
         <v>4</v>
@@ -8535,16 +8535,16 @@
       <c r="I13" s="11">
         <v>2048.0</v>
       </c>
-      <c r="J13" s="16">
+      <c r="J13" s="15">
         <v>2364771.07</v>
       </c>
-      <c r="K13" s="16">
+      <c r="K13" s="15">
         <v>2364771.07</v>
       </c>
-      <c r="L13" s="16">
+      <c r="L13" s="15">
         <v>0.0</v>
       </c>
-      <c r="M13" s="42"/>
+      <c r="M13" s="41"/>
       <c r="AB13" s="4"/>
       <c r="AC13" s="4"/>
       <c r="AD13" s="4"/>
@@ -8555,13 +8555,13 @@
     </row>
     <row r="14">
       <c r="A14" s="11" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="D14" s="11" t="s">
         <v>4</v>
@@ -8579,12 +8579,12 @@
         <v>339039.0</v>
       </c>
       <c r="I14" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="J14" s="16">
+        <v>65</v>
+      </c>
+      <c r="J14" s="15">
         <v>968237.39</v>
       </c>
-      <c r="K14" s="16">
+      <c r="K14" s="15">
         <v>968237.39</v>
       </c>
       <c r="L14" s="11">
@@ -8600,13 +8600,13 @@
     </row>
     <row r="15">
       <c r="A15" s="11" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="D15" s="11" t="s">
         <v>4</v>
@@ -8624,12 +8624,12 @@
         <v>339039.0</v>
       </c>
       <c r="I15" s="11" t="s">
-        <v>51</v>
-      </c>
-      <c r="J15" s="16">
+        <v>45</v>
+      </c>
+      <c r="J15" s="15">
         <v>1011677.95</v>
       </c>
-      <c r="K15" s="16">
+      <c r="K15" s="15">
         <v>1011677.95</v>
       </c>
       <c r="L15" s="11">
@@ -8645,13 +8645,13 @@
     </row>
     <row r="16">
       <c r="A16" s="11" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="C16" s="11" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D16" s="11" t="s">
         <v>4</v>
@@ -8671,13 +8671,13 @@
       <c r="I16" s="11">
         <v>2048.0</v>
       </c>
-      <c r="J16" s="16">
+      <c r="J16" s="15">
         <v>1580293.02</v>
       </c>
-      <c r="K16" s="16">
+      <c r="K16" s="15">
         <v>1580293.02</v>
       </c>
-      <c r="L16" s="16">
+      <c r="L16" s="15">
         <v>0.0</v>
       </c>
       <c r="AB16" s="4"/>
@@ -8690,13 +8690,13 @@
     </row>
     <row r="17">
       <c r="A17" s="11" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="B17" s="11" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="C17" s="11" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="D17" s="11" t="s">
         <v>4</v>
@@ -8716,13 +8716,13 @@
       <c r="I17" s="11">
         <v>2048.0</v>
       </c>
-      <c r="J17" s="16">
+      <c r="J17" s="15">
         <v>34065.36</v>
       </c>
       <c r="K17" s="11">
         <v>0.0</v>
       </c>
-      <c r="L17" s="16">
+      <c r="L17" s="15">
         <v>34065.36</v>
       </c>
       <c r="AB17" s="4"/>
@@ -8735,13 +8735,13 @@
     </row>
     <row r="18">
       <c r="A18" s="11" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="C18" s="11" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="D18" s="11" t="s">
         <v>4</v>
@@ -8759,12 +8759,12 @@
         <v>339039.0</v>
       </c>
       <c r="I18" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="J18" s="16">
+        <v>65</v>
+      </c>
+      <c r="J18" s="15">
         <v>63746.85</v>
       </c>
-      <c r="K18" s="16">
+      <c r="K18" s="15">
         <v>63746.85</v>
       </c>
       <c r="L18" s="11">
@@ -8780,13 +8780,13 @@
     </row>
     <row r="19">
       <c r="A19" s="11" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C19" s="11" t="s">
-        <v>113</v>
+        <v>104</v>
       </c>
       <c r="D19" s="11" t="s">
         <v>4</v>
@@ -8804,12 +8804,12 @@
         <v>339039.0</v>
       </c>
       <c r="I19" s="11" t="s">
-        <v>78</v>
-      </c>
-      <c r="J19" s="16">
+        <v>76</v>
+      </c>
+      <c r="J19" s="15">
         <v>947931.1</v>
       </c>
-      <c r="K19" s="16">
+      <c r="K19" s="15">
         <v>947931.1</v>
       </c>
       <c r="L19" s="11">
@@ -8825,13 +8825,13 @@
     </row>
     <row r="20">
       <c r="A20" s="11" t="s">
-        <v>116</v>
+        <v>106</v>
       </c>
       <c r="B20" s="11" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="C20" s="11" t="s">
-        <v>117</v>
+        <v>108</v>
       </c>
       <c r="D20" s="11" t="s">
         <v>4</v>
@@ -8851,10 +8851,10 @@
       <c r="I20" s="11">
         <v>2048.0</v>
       </c>
-      <c r="J20" s="16">
+      <c r="J20" s="15">
         <v>259790.57</v>
       </c>
-      <c r="K20" s="16">
+      <c r="K20" s="15">
         <v>259790.57</v>
       </c>
       <c r="L20" s="11">
@@ -8870,13 +8870,13 @@
     </row>
     <row r="21">
       <c r="A21" s="11" t="s">
-        <v>121</v>
+        <v>110</v>
       </c>
       <c r="B21" s="11" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>122</v>
+        <v>111</v>
       </c>
       <c r="D21" s="11" t="s">
         <v>4</v>
@@ -8896,10 +8896,10 @@
       <c r="I21" s="11">
         <v>2048.0</v>
       </c>
-      <c r="J21" s="16">
+      <c r="J21" s="15">
         <v>170479.3</v>
       </c>
-      <c r="K21" s="16">
+      <c r="K21" s="15">
         <v>170479.3</v>
       </c>
       <c r="L21" s="11">
@@ -8915,18 +8915,18 @@
     </row>
     <row r="22">
       <c r="A22" s="11" t="s">
-        <v>125</v>
+        <v>113</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>127</v>
+        <v>114</v>
       </c>
       <c r="C22" s="11" t="s">
-        <v>128</v>
+        <v>115</v>
       </c>
       <c r="D22" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="E22" s="52">
+      <c r="E22" s="50">
         <v>45953.0</v>
       </c>
       <c r="F22" s="11" t="s">
@@ -8941,13 +8941,13 @@
       <c r="I22" s="11">
         <v>2000.0</v>
       </c>
-      <c r="J22" s="16">
+      <c r="J22" s="15">
         <v>1500000.0</v>
       </c>
-      <c r="K22" s="16">
+      <c r="K22" s="15">
         <v>1500000.0</v>
       </c>
-      <c r="L22" s="16">
+      <c r="L22" s="15">
         <v>0.0</v>
       </c>
       <c r="AB22" s="4"/>
@@ -8960,18 +8960,18 @@
     </row>
     <row r="23">
       <c r="A23" s="11" t="s">
-        <v>130</v>
+        <v>117</v>
       </c>
       <c r="B23" s="11" t="s">
-        <v>131</v>
+        <v>118</v>
       </c>
       <c r="C23" s="11" t="s">
-        <v>132</v>
+        <v>119</v>
       </c>
       <c r="D23" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="E23" s="52">
+      <c r="E23" s="50">
         <v>45953.0</v>
       </c>
       <c r="F23" s="11" t="s">
@@ -8984,12 +8984,12 @@
         <v>339039.0</v>
       </c>
       <c r="I23" s="11" t="s">
-        <v>133</v>
-      </c>
-      <c r="J23" s="16">
+        <v>120</v>
+      </c>
+      <c r="J23" s="15">
         <v>1000001.64</v>
       </c>
-      <c r="K23" s="16">
+      <c r="K23" s="15">
         <v>1000001.64</v>
       </c>
       <c r="L23" s="11">
@@ -9005,18 +9005,18 @@
     </row>
     <row r="24">
       <c r="A24" s="11" t="s">
-        <v>135</v>
+        <v>122</v>
       </c>
       <c r="B24" s="11" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C24" s="11" t="s">
-        <v>136</v>
+        <v>124</v>
       </c>
       <c r="D24" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="E24" s="52">
+      <c r="E24" s="50">
         <v>45953.0</v>
       </c>
       <c r="F24" s="11" t="s">
@@ -9031,10 +9031,10 @@
       <c r="I24" s="11">
         <v>2048.0</v>
       </c>
-      <c r="J24" s="16">
+      <c r="J24" s="15">
         <v>68405.66</v>
       </c>
-      <c r="K24" s="16">
+      <c r="K24" s="15">
         <v>68405.66</v>
       </c>
       <c r="L24" s="11">
@@ -9050,18 +9050,18 @@
     </row>
     <row r="25">
       <c r="A25" s="11" t="s">
-        <v>138</v>
+        <v>126</v>
       </c>
       <c r="B25" s="11" t="s">
-        <v>139</v>
+        <v>127</v>
       </c>
       <c r="C25" s="11" t="s">
-        <v>140</v>
+        <v>129</v>
       </c>
       <c r="D25" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="E25" s="52">
+      <c r="E25" s="50">
         <v>45975.0</v>
       </c>
       <c r="F25" s="11" t="s">
@@ -9074,12 +9074,12 @@
         <v>339039.0</v>
       </c>
       <c r="I25" s="11" t="s">
-        <v>133</v>
-      </c>
-      <c r="J25" s="16">
+        <v>120</v>
+      </c>
+      <c r="J25" s="15">
         <v>1157673.06</v>
       </c>
-      <c r="K25" s="16">
+      <c r="K25" s="15">
         <v>1157673.06</v>
       </c>
       <c r="L25" s="11">
@@ -9095,18 +9095,18 @@
     </row>
     <row r="26">
       <c r="A26" s="11" t="s">
-        <v>143</v>
+        <v>131</v>
       </c>
       <c r="B26" s="11" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="C26" s="11" t="s">
-        <v>144</v>
+        <v>133</v>
       </c>
       <c r="D26" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="E26" s="52">
+      <c r="E26" s="50">
         <v>45989.0</v>
       </c>
       <c r="F26" s="11" t="s">
@@ -9121,10 +9121,10 @@
       <c r="I26" s="11">
         <v>2048.0</v>
       </c>
-      <c r="J26" s="16">
+      <c r="J26" s="15">
         <v>34065.36</v>
       </c>
-      <c r="K26" s="16">
+      <c r="K26" s="15">
         <v>34065.36</v>
       </c>
       <c r="L26" s="11">
@@ -9140,13 +9140,13 @@
     </row>
     <row r="27">
       <c r="A27" s="11" t="s">
-        <v>146</v>
+        <v>135</v>
       </c>
       <c r="B27" s="11" t="s">
-        <v>147</v>
+        <v>136</v>
       </c>
       <c r="C27" s="11" t="s">
-        <v>148</v>
+        <v>137</v>
       </c>
       <c r="D27" s="11" t="s">
         <v>4</v>
@@ -9166,13 +9166,13 @@
       <c r="I27" s="11">
         <v>2048.0</v>
       </c>
-      <c r="J27" s="16">
+      <c r="J27" s="15">
         <v>1770880.5</v>
       </c>
-      <c r="K27" s="16">
+      <c r="K27" s="15">
         <v>843261.89</v>
       </c>
-      <c r="L27" s="16">
+      <c r="L27" s="15">
         <v>927618.61</v>
       </c>
       <c r="AB27" s="4"/>
@@ -9185,13 +9185,13 @@
     </row>
     <row r="28">
       <c r="A28" s="11" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="B28" s="11" t="s">
-        <v>153</v>
+        <v>141</v>
       </c>
       <c r="C28" s="11" t="s">
-        <v>154</v>
+        <v>142</v>
       </c>
       <c r="D28" s="11" t="s">
         <v>4</v>
@@ -9209,15 +9209,15 @@
         <v>339039.0</v>
       </c>
       <c r="I28" s="11" t="s">
-        <v>60</v>
-      </c>
-      <c r="J28" s="16">
+        <v>57</v>
+      </c>
+      <c r="J28" s="15">
         <v>1912292.52</v>
       </c>
-      <c r="K28" s="16">
+      <c r="K28" s="15">
         <v>1629834.48</v>
       </c>
-      <c r="L28" s="16">
+      <c r="L28" s="15">
         <v>282458.04</v>
       </c>
       <c r="AB28" s="4"/>
@@ -9230,13 +9230,13 @@
     </row>
     <row r="29">
       <c r="A29" s="11" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="B29" s="11" t="s">
-        <v>158</v>
+        <v>146</v>
       </c>
       <c r="C29" s="11" t="s">
-        <v>159</v>
+        <v>147</v>
       </c>
       <c r="D29" s="11" t="s">
         <v>4</v>
@@ -9256,13 +9256,13 @@
       <c r="I29" s="11">
         <v>2048.0</v>
       </c>
-      <c r="J29" s="16">
+      <c r="J29" s="15">
         <v>1496713.48</v>
       </c>
       <c r="K29" s="11">
         <v>0.0</v>
       </c>
-      <c r="L29" s="16">
+      <c r="L29" s="15">
         <v>1496713.48</v>
       </c>
       <c r="AB29" s="4"/>
@@ -9275,13 +9275,13 @@
     </row>
     <row r="30">
       <c r="A30" s="11" t="s">
-        <v>160</v>
+        <v>149</v>
       </c>
       <c r="B30" s="11" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="C30" s="11" t="s">
-        <v>162</v>
+        <v>151</v>
       </c>
       <c r="D30" s="11" t="s">
         <v>4</v>
@@ -9299,15 +9299,15 @@
         <v>339039.0</v>
       </c>
       <c r="I30" s="11" t="s">
-        <v>51</v>
-      </c>
-      <c r="J30" s="16">
+        <v>45</v>
+      </c>
+      <c r="J30" s="15">
         <v>624166.14</v>
       </c>
       <c r="K30" s="11">
         <v>0.0</v>
       </c>
-      <c r="L30" s="16">
+      <c r="L30" s="15">
         <v>624166.14</v>
       </c>
       <c r="AB30" s="4"/>
@@ -9320,13 +9320,13 @@
     </row>
     <row r="31">
       <c r="A31" s="11" t="s">
-        <v>165</v>
+        <v>153</v>
       </c>
       <c r="B31" s="11" t="s">
-        <v>166</v>
+        <v>154</v>
       </c>
       <c r="C31" s="11" t="s">
-        <v>167</v>
+        <v>155</v>
       </c>
       <c r="D31" s="11" t="s">
         <v>4</v>
@@ -9344,15 +9344,15 @@
         <v>339039.0</v>
       </c>
       <c r="I31" s="11" t="s">
-        <v>133</v>
-      </c>
-      <c r="J31" s="16">
+        <v>120</v>
+      </c>
+      <c r="J31" s="15">
         <v>18462.36</v>
       </c>
       <c r="K31" s="11">
         <v>0.0</v>
       </c>
-      <c r="L31" s="16">
+      <c r="L31" s="15">
         <v>18462.36</v>
       </c>
       <c r="AB31" s="4"/>
@@ -9365,13 +9365,13 @@
     </row>
     <row r="32">
       <c r="A32" s="11" t="s">
-        <v>170</v>
+        <v>157</v>
       </c>
       <c r="B32" s="11" t="s">
-        <v>166</v>
-      </c>
-      <c r="C32" s="16" t="s">
-        <v>171</v>
+        <v>154</v>
+      </c>
+      <c r="C32" s="15" t="s">
+        <v>158</v>
       </c>
       <c r="D32" s="11" t="s">
         <v>4</v>
@@ -9389,15 +9389,15 @@
         <v>339039.0</v>
       </c>
       <c r="I32" s="11" t="s">
-        <v>133</v>
-      </c>
-      <c r="J32" s="16">
+        <v>120</v>
+      </c>
+      <c r="J32" s="15">
         <v>1530656.62</v>
       </c>
       <c r="K32" s="11">
         <v>0.0</v>
       </c>
-      <c r="L32" s="16">
+      <c r="L32" s="15">
         <v>1530656.62</v>
       </c>
       <c r="AB32" s="4"/>
@@ -9410,13 +9410,13 @@
     </row>
     <row r="33">
       <c r="A33" s="11" t="s">
-        <v>176</v>
+        <v>161</v>
       </c>
       <c r="B33" s="11" t="s">
-        <v>158</v>
-      </c>
-      <c r="C33" s="16" t="s">
-        <v>177</v>
+        <v>146</v>
+      </c>
+      <c r="C33" s="15" t="s">
+        <v>162</v>
       </c>
       <c r="D33" s="11" t="s">
         <v>4</v>
@@ -9436,13 +9436,13 @@
       <c r="I33" s="11">
         <v>2048.0</v>
       </c>
-      <c r="J33" s="16">
+      <c r="J33" s="15">
         <v>173846.38</v>
       </c>
       <c r="K33" s="11">
         <v>0.0</v>
       </c>
-      <c r="L33" s="16">
+      <c r="L33" s="15">
         <v>173846.38</v>
       </c>
       <c r="AB33" s="4"/>
@@ -9455,13 +9455,13 @@
     </row>
     <row r="34">
       <c r="A34" s="11" t="s">
-        <v>180</v>
+        <v>164</v>
       </c>
       <c r="B34" s="11" t="s">
-        <v>181</v>
+        <v>165</v>
       </c>
       <c r="C34" s="11" t="s">
-        <v>182</v>
+        <v>166</v>
       </c>
       <c r="D34" s="11" t="s">
         <v>4</v>
@@ -9479,15 +9479,15 @@
         <v>339039.0</v>
       </c>
       <c r="I34" s="11" t="s">
-        <v>183</v>
-      </c>
-      <c r="J34" s="16">
+        <v>168</v>
+      </c>
+      <c r="J34" s="15">
         <v>236343.68</v>
       </c>
       <c r="K34" s="11">
         <v>0.0</v>
       </c>
-      <c r="L34" s="16">
+      <c r="L34" s="15">
         <v>236343.68</v>
       </c>
       <c r="AB34" s="4"/>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (26/08/2026 10:59)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/01_Bases_Originais/005_CELOG_2025/005_CELOG-PAMALS_2025 online.xlsx
+++ b/Contrato 005/Dashboard/01_Bases_Originais/005_CELOG_2025/005_CELOG-PAMALS_2025 online.xlsx
@@ -30,12 +30,12 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="343" uniqueCount="217">
   <si>
+    <t>Controle de pagamentos</t>
+  </si>
+  <si>
     <t>Saldo</t>
   </si>
   <si>
-    <t>Controle de pagamentos</t>
-  </si>
-  <si>
     <t>2025NE000005</t>
   </si>
   <si>
@@ -60,12 +60,21 @@
     <t>Número Contrato</t>
   </si>
   <si>
+    <t>2025NE000369</t>
+  </si>
+  <si>
     <t>UG Executora</t>
   </si>
   <si>
+    <t>C25516</t>
+  </si>
+  <si>
     <t>UG Responsável</t>
   </si>
   <si>
+    <t>25E0387</t>
+  </si>
+  <si>
     <t>UG Fiscalizadora</t>
   </si>
   <si>
@@ -78,21 +87,12 @@
     <t>Status</t>
   </si>
   <si>
-    <t>2025NE000369</t>
-  </si>
-  <si>
     <t>Ação</t>
   </si>
   <si>
-    <t>C25516</t>
-  </si>
-  <si>
     <t>PAG</t>
   </si>
   <si>
-    <t>25E0387</t>
-  </si>
-  <si>
     <t>Moeda</t>
   </si>
   <si>
@@ -114,93 +114,102 @@
     <t>Fornecedor</t>
   </si>
   <si>
+    <t>2025NE000371</t>
+  </si>
+  <si>
     <t>Tipo Despesa /Receita</t>
   </si>
   <si>
     <t>Abrir</t>
   </si>
   <si>
+    <t>25E0389</t>
+  </si>
+  <si>
     <t>Editar</t>
   </si>
   <si>
+    <t>2025NE000413</t>
+  </si>
+  <si>
+    <t>C25501</t>
+  </si>
+  <si>
+    <t>25E0403</t>
+  </si>
+  <si>
     <t>005/CELOG-PAMALS/2025</t>
   </si>
   <si>
-    <t>2025NE000371</t>
-  </si>
-  <si>
     <t>CELOG</t>
   </si>
   <si>
     <t>PAMALS</t>
   </si>
   <si>
-    <t>25E0389</t>
+    <t>20SP</t>
   </si>
   <si>
     <t>Vigente</t>
   </si>
   <si>
+    <t>2025NE000414</t>
+  </si>
+  <si>
+    <t>C25525</t>
+  </si>
+  <si>
     <t>2048 20YJ 21EM 219C 20SP 20X7 2000</t>
   </si>
   <si>
     <t>67101.001510/2024-12</t>
   </si>
   <si>
+    <t>25E0431</t>
+  </si>
+  <si>
     <t>R$</t>
   </si>
   <si>
     <t>VEE ONE-MANUTENCAO E SERVICOS TECNICOS LTDA</t>
   </si>
   <si>
-    <t>2025NE000413</t>
-  </si>
-  <si>
-    <t>C25501</t>
-  </si>
-  <si>
-    <t>25E0403</t>
-  </si>
-  <si>
-    <t>20SP</t>
-  </si>
-  <si>
-    <t>2025NE000414</t>
-  </si>
-  <si>
-    <t>C25525</t>
-  </si>
-  <si>
-    <t>25E0431</t>
-  </si>
-  <si>
     <t>21EM</t>
   </si>
   <si>
+    <t>2025NE000559</t>
+  </si>
+  <si>
+    <t>C25545</t>
+  </si>
+  <si>
+    <t>25E0524</t>
+  </si>
+  <si>
+    <t>20X7</t>
+  </si>
+  <si>
     <t>Módulo</t>
   </si>
   <si>
     <t>Referência</t>
   </si>
   <si>
+    <t>2025NE000770</t>
+  </si>
+  <si>
     <t>Nº recibo</t>
   </si>
   <si>
+    <t>25E0731</t>
+  </si>
+  <si>
     <t>Nº</t>
   </si>
   <si>
-    <t>2025NE000559</t>
-  </si>
-  <si>
     <t>Data</t>
   </si>
   <si>
-    <t>C25545</t>
-  </si>
-  <si>
-    <t>25E0524</t>
-  </si>
-  <si>
     <t>Empenho</t>
   </si>
   <si>
@@ -210,9 +219,6 @@
     <t>Vencimento</t>
   </si>
   <si>
-    <t>20X7</t>
-  </si>
-  <si>
     <t>Valor das Nfs</t>
   </si>
   <si>
@@ -222,127 +228,121 @@
     <t>Faturado</t>
   </si>
   <si>
+    <t>2025NE000774</t>
+  </si>
+  <si>
     <t>Pendente</t>
   </si>
   <si>
-    <t>2025NE000770</t>
-  </si>
-  <si>
-    <t>25E0731</t>
+    <t>25E0737</t>
   </si>
   <si>
     <t>FEV/25</t>
   </si>
   <si>
-    <t>2025NE000774</t>
-  </si>
-  <si>
     <t>-</t>
   </si>
   <si>
-    <t>25E0737</t>
+    <t>2025NE000843</t>
+  </si>
+  <si>
+    <t>C25630</t>
+  </si>
+  <si>
+    <t>25E0787</t>
+  </si>
+  <si>
+    <t>219C</t>
   </si>
   <si>
     <t xml:space="preserve">2025NE000369 </t>
   </si>
   <si>
-    <t>2025NE000843</t>
-  </si>
-  <si>
-    <t>C25630</t>
-  </si>
-  <si>
-    <t>25E0787</t>
-  </si>
-  <si>
     <t>2025NP001980</t>
   </si>
   <si>
-    <t>219C</t>
-  </si>
-  <si>
     <t>2025NE001065</t>
   </si>
   <si>
     <t>25E0999</t>
   </si>
   <si>
+    <t>2025NE001200</t>
+  </si>
+  <si>
+    <t>C25590</t>
+  </si>
+  <si>
+    <t>25E1128</t>
+  </si>
+  <si>
+    <t>2025NE001598</t>
+  </si>
+  <si>
+    <t>C25814</t>
+  </si>
+  <si>
+    <t>25E1446</t>
+  </si>
+  <si>
     <t>MAR/25</t>
   </si>
   <si>
-    <t>2025NE001200</t>
-  </si>
-  <si>
-    <t>C25590</t>
-  </si>
-  <si>
-    <t>25E1128</t>
-  </si>
-  <si>
     <t>2025NE000367, 2025NE000369, 2025NE000371, 2025NE000413</t>
   </si>
   <si>
+    <t>2025NE001627</t>
+  </si>
+  <si>
+    <t>25E1475</t>
+  </si>
+  <si>
     <t>2025NP001979</t>
   </si>
   <si>
-    <t>2025NE001598</t>
-  </si>
-  <si>
-    <t>C25814</t>
-  </si>
-  <si>
-    <t>25E1446</t>
+    <t>2025NE001629</t>
+  </si>
+  <si>
+    <t>C25820</t>
   </si>
   <si>
     <t>ABR/25</t>
   </si>
   <si>
-    <t>2025NE001627</t>
-  </si>
-  <si>
-    <t>25E1475</t>
+    <t>25E1477</t>
   </si>
   <si>
     <t>2025NE000413, 2025NE000414, 2025NE000559</t>
   </si>
   <si>
+    <t>2025NE001687</t>
+  </si>
+  <si>
     <t>2025NP002341</t>
   </si>
   <si>
-    <t>2025NE001629</t>
-  </si>
-  <si>
-    <t>C25820</t>
-  </si>
-  <si>
-    <t>25E1477</t>
+    <t>25E1535</t>
   </si>
   <si>
     <t>MAI/25</t>
   </si>
   <si>
-    <t>2025NE001687</t>
-  </si>
-  <si>
-    <t>25E1535</t>
+    <t>2025NE001688</t>
+  </si>
+  <si>
+    <t>25E1536</t>
   </si>
   <si>
     <t>2025NP002884</t>
   </si>
   <si>
-    <t>2025NE001688</t>
-  </si>
-  <si>
-    <t>25E1536</t>
+    <t>2025NE001689</t>
+  </si>
+  <si>
+    <t>25E1537</t>
   </si>
   <si>
     <t>JUN/25</t>
-  </si>
-  <si>
-    <t>2025NE001689</t>
-  </si>
-  <si>
-    <t>25E1537</t>
   </si>
   <si>
     <t>2025NE000005,
@@ -351,12 +351,12 @@
 2025NE000774</t>
   </si>
   <si>
+    <t>2025NE001690</t>
+  </si>
+  <si>
     <t>2025NP400522</t>
   </si>
   <si>
-    <t>2025NE001690</t>
-  </si>
-  <si>
     <t>25E1538</t>
   </si>
   <si>
@@ -378,40 +378,40 @@
     <t>2025NP003724</t>
   </si>
   <si>
+    <t>AGO/25</t>
+  </si>
+  <si>
     <t>2025NE001828</t>
   </si>
   <si>
     <t>C25869</t>
   </si>
   <si>
-    <t>AGO/25</t>
-  </si>
-  <si>
     <t>25E1667</t>
   </si>
   <si>
     <t>20YJ</t>
   </si>
   <si>
+    <t>2025NP004558</t>
+  </si>
+  <si>
     <t>2025NE001830</t>
   </si>
   <si>
-    <t>2025NP004558</t>
-  </si>
-  <si>
     <t>25E1669</t>
   </si>
   <si>
     <t>SET/25</t>
+  </si>
+  <si>
+    <t>2025NE002200</t>
   </si>
   <si>
     <t>2025NE001688 
 2025NE001828</t>
   </si>
   <si>
-    <t>2025NE002200</t>
-  </si>
-  <si>
     <t>C25863</t>
   </si>
   <si>
@@ -421,13 +421,22 @@
     <t>2025NP004897</t>
   </si>
   <si>
+    <t>2025NE002237</t>
+  </si>
+  <si>
+    <t>25E2058</t>
+  </si>
+  <si>
     <t>OUT/25</t>
   </si>
   <si>
-    <t>2025NE002237</t>
-  </si>
-  <si>
-    <t>25E2058</t>
+    <t>2026NE000330</t>
+  </si>
+  <si>
+    <t>C26163</t>
+  </si>
+  <si>
+    <t>26E0320</t>
   </si>
   <si>
     <t>2025NE001688, 2025NE001828, 2025NE002200</t>
@@ -436,43 +445,58 @@
     <t>2025NP004932</t>
   </si>
   <si>
-    <t>2026NE000330</t>
-  </si>
-  <si>
-    <t>C26163</t>
-  </si>
-  <si>
-    <t>26E0320</t>
+    <t>2026NE000388</t>
+  </si>
+  <si>
+    <t>C26193</t>
+  </si>
+  <si>
+    <t>26E0375</t>
   </si>
   <si>
     <t>NOV/25</t>
   </si>
   <si>
+    <t>2026NE000748</t>
+  </si>
+  <si>
+    <t>C26312</t>
+  </si>
+  <si>
     <t>2025NE001687, 2025NE001689, 2025NE001690, 2025NE001823, 2025NE001830, 2025NE002237</t>
   </si>
   <si>
-    <t>2026NE000388</t>
-  </si>
-  <si>
-    <t>C26193</t>
-  </si>
-  <si>
-    <t>26E0375</t>
+    <t>26E0709</t>
   </si>
   <si>
     <t>2026NP400440</t>
   </si>
   <si>
-    <t>2026NE000748</t>
-  </si>
-  <si>
-    <t>C26312</t>
+    <t>2026NE000816</t>
+  </si>
+  <si>
+    <t>C26324</t>
+  </si>
+  <si>
+    <t>26E0776</t>
+  </si>
+  <si>
+    <t>2026NE000817</t>
+  </si>
+  <si>
+    <t>C26326</t>
+  </si>
+  <si>
+    <t>26E0777</t>
   </si>
   <si>
     <t>DEZ/25</t>
   </si>
   <si>
-    <t>26E0709</t>
+    <t>2026NE000842</t>
+  </si>
+  <si>
+    <t>26E0803</t>
   </si>
   <si>
     <t>2025NE001065, 2025NE002200</t>
@@ -481,34 +505,28 @@
     <t>2026NP400412</t>
   </si>
   <si>
-    <t>2026NE000816</t>
-  </si>
-  <si>
-    <t>C26324</t>
-  </si>
-  <si>
-    <t>26E0776</t>
+    <t>2026NE000944</t>
+  </si>
+  <si>
+    <t>26E0906</t>
   </si>
   <si>
     <t>JAN/26</t>
   </si>
   <si>
-    <t>2026NE000817</t>
-  </si>
-  <si>
-    <t>C26326</t>
-  </si>
-  <si>
-    <t>26E0777</t>
+    <t>2026NE001015</t>
+  </si>
+  <si>
+    <t>C26363</t>
+  </si>
+  <si>
+    <t>26E0959</t>
   </si>
   <si>
     <t>2026NP401035</t>
   </si>
   <si>
-    <t>2026NE000842</t>
-  </si>
-  <si>
-    <t>26E0803</t>
+    <t>20XV</t>
   </si>
   <si>
     <t>FEV/26</t>
@@ -517,28 +535,10 @@
     <t>2025NE001627, 2025NE001629, 2025NE001823</t>
   </si>
   <si>
-    <t>2026NE000944</t>
-  </si>
-  <si>
-    <t>26E0906</t>
-  </si>
-  <si>
     <t>2026NP402272</t>
   </si>
   <si>
-    <t>2026NE001015</t>
-  </si>
-  <si>
-    <t>C26363</t>
-  </si>
-  <si>
-    <t>26E0959</t>
-  </si>
-  <si>
     <t>MAR/26</t>
-  </si>
-  <si>
-    <t>20XV</t>
   </si>
   <si>
     <t>2025NE000770, 2025NE001627</t>
@@ -732,6 +732,12 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="10.0"/>
+      <color theme="1"/>
+      <name val="Century Gothic"/>
+    </font>
+    <font>
       <sz val="10.0"/>
       <color theme="1"/>
       <name val="Arial"/>
@@ -741,12 +747,6 @@
       <sz val="10.0"/>
       <color theme="1"/>
       <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10.0"/>
-      <color theme="1"/>
-      <name val="Century Gothic"/>
     </font>
     <font>
       <sz val="10.0"/>
@@ -891,27 +891,27 @@
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="3" fontId="2" numFmtId="0" xfId="0" applyFill="1" applyFont="1"/>
+    <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyFill="1" applyFont="1"/>
+    <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyFill="1" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
     <xf borderId="0" fillId="5" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
+      <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="11" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
@@ -947,37 +947,37 @@
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="0" fontId="5" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf borderId="0" fillId="2" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="7" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="2" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="6" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="7" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -992,13 +992,13 @@
     <xf borderId="1" fillId="7" fontId="9" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="165" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="1" fillId="5" fontId="9" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="8" fontId="6" numFmtId="168" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="8" fontId="7" numFmtId="168" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="165" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="3" fillId="0" fontId="10" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="1" fillId="8" fontId="9" numFmtId="168" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
@@ -1018,10 +1018,10 @@
     <xf borderId="1" fillId="8" fontId="9" numFmtId="168" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="6" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="7" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="170" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
@@ -1030,7 +1030,7 @@
     <xf borderId="1" fillId="9" fontId="9" numFmtId="168" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="4" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="4" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="9" fontId="9" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
@@ -1040,7 +1040,7 @@
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="4" fillId="0" fontId="10" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="1" fillId="0" fontId="6" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="7" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="5" fontId="9" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
@@ -1049,7 +1049,7 @@
     <xf borderId="1" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="6" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="7" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="5" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -1437,22 +1437,22 @@
       <c r="S1" s="1"/>
       <c r="T1" s="1"/>
       <c r="U1" s="1"/>
-      <c r="V1" s="4"/>
+      <c r="V1" s="3"/>
     </row>
     <row r="2" ht="59.25" customHeight="1">
-      <c r="A2" s="6"/>
-      <c r="B2" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="V2" s="9"/>
-      <c r="W2" s="10"/>
-      <c r="X2" s="10"/>
-      <c r="Y2" s="10"/>
-      <c r="Z2" s="10"/>
-      <c r="AA2" s="10"/>
-      <c r="AB2" s="10"/>
-      <c r="AC2" s="10"/>
-      <c r="AD2" s="10"/>
+      <c r="A2" s="4"/>
+      <c r="B2" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="V2" s="8"/>
+      <c r="W2" s="9"/>
+      <c r="X2" s="9"/>
+      <c r="Y2" s="9"/>
+      <c r="Z2" s="9"/>
+      <c r="AA2" s="9"/>
+      <c r="AB2" s="9"/>
+      <c r="AC2" s="9"/>
+      <c r="AD2" s="9"/>
     </row>
     <row r="3" ht="12.75" customHeight="1">
       <c r="A3" s="1"/>
@@ -1476,7 +1476,7 @@
       <c r="S3" s="13"/>
       <c r="T3" s="13"/>
       <c r="U3" s="13"/>
-      <c r="V3" s="4"/>
+      <c r="V3" s="3"/>
     </row>
     <row r="4" ht="12.75" customHeight="1">
       <c r="A4" s="15"/>
@@ -1485,28 +1485,28 @@
         <v>9</v>
       </c>
       <c r="D4" s="16" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E4" s="16" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F4" s="16" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="G4" s="17" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="H4" s="17" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="I4" s="16" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="J4" s="16" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="K4" s="16" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L4" s="16" t="s">
         <v>21</v>
@@ -1530,31 +1530,31 @@
         <v>27</v>
       </c>
       <c r="S4" s="16" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="T4" s="16" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="U4" s="16" t="s">
-        <v>30</v>
-      </c>
-      <c r="V4" s="4"/>
+        <v>32</v>
+      </c>
+      <c r="V4" s="3"/>
     </row>
     <row r="5" ht="12.75" customHeight="1">
       <c r="A5" s="15"/>
       <c r="B5" s="15"/>
       <c r="C5" s="18"/>
       <c r="D5" s="19" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="E5" s="19" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="F5" s="19" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="G5" s="19" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="H5" s="20">
         <v>1564.0</v>
@@ -1563,16 +1563,16 @@
         <v>1564.0</v>
       </c>
       <c r="J5" s="19" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="K5" s="19" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="L5" s="19" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="M5" s="19" t="s">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="N5" s="21">
         <v>9.165159737E7</v>
@@ -1590,89 +1590,89 @@
         <v>1.085943044E7</v>
       </c>
       <c r="S5" s="19" t="s">
-        <v>40</v>
-      </c>
-      <c r="V5" s="4"/>
+        <v>47</v>
+      </c>
+      <c r="V5" s="3"/>
     </row>
     <row r="6" ht="12.75" customHeight="1">
       <c r="A6" s="15"/>
       <c r="B6" s="15"/>
       <c r="L6" s="22"/>
-      <c r="V6" s="4"/>
+      <c r="V6" s="3"/>
     </row>
     <row r="7" ht="12.75" customHeight="1">
-      <c r="A7" s="23"/>
-      <c r="B7" s="23"/>
-      <c r="C7" s="24"/>
-      <c r="D7" s="25"/>
-      <c r="E7" s="25"/>
-      <c r="F7" s="25"/>
-      <c r="G7" s="25"/>
-      <c r="H7" s="25"/>
-      <c r="I7" s="25"/>
-      <c r="J7" s="25"/>
-      <c r="K7" s="25"/>
-      <c r="L7" s="26"/>
-      <c r="M7" s="25"/>
-      <c r="N7" s="25"/>
-      <c r="O7" s="25"/>
-      <c r="P7" s="27"/>
-      <c r="V7" s="4"/>
+      <c r="A7" s="24"/>
+      <c r="B7" s="24"/>
+      <c r="C7" s="25"/>
+      <c r="D7" s="26"/>
+      <c r="E7" s="26"/>
+      <c r="F7" s="26"/>
+      <c r="G7" s="26"/>
+      <c r="H7" s="26"/>
+      <c r="I7" s="26"/>
+      <c r="J7" s="26"/>
+      <c r="K7" s="26"/>
+      <c r="L7" s="27"/>
+      <c r="M7" s="26"/>
+      <c r="N7" s="26"/>
+      <c r="O7" s="26"/>
+      <c r="P7" s="28"/>
+      <c r="V7" s="3"/>
     </row>
     <row r="8" ht="12.75" customHeight="1">
-      <c r="A8" s="23"/>
-      <c r="B8" s="23"/>
-      <c r="C8" s="28" t="s">
-        <v>49</v>
-      </c>
-      <c r="D8" s="28" t="s">
-        <v>50</v>
+      <c r="A8" s="24"/>
+      <c r="B8" s="24"/>
+      <c r="C8" s="29" t="s">
+        <v>53</v>
+      </c>
+      <c r="D8" s="29" t="s">
+        <v>54</v>
       </c>
       <c r="E8" s="30" t="s">
-        <v>51</v>
-      </c>
-      <c r="F8" s="28" t="s">
-        <v>52</v>
-      </c>
-      <c r="G8" s="28" t="s">
-        <v>54</v>
-      </c>
-      <c r="H8" s="28" t="s">
-        <v>57</v>
+        <v>56</v>
+      </c>
+      <c r="F8" s="29" t="s">
+        <v>58</v>
+      </c>
+      <c r="G8" s="29" t="s">
+        <v>59</v>
+      </c>
+      <c r="H8" s="29" t="s">
+        <v>60</v>
       </c>
       <c r="I8" s="30" t="s">
-        <v>58</v>
-      </c>
-      <c r="J8" s="28" t="s">
-        <v>59</v>
-      </c>
-      <c r="K8" s="28" t="s">
         <v>61</v>
       </c>
+      <c r="J8" s="29" t="s">
+        <v>62</v>
+      </c>
+      <c r="K8" s="29" t="s">
+        <v>63</v>
+      </c>
       <c r="L8" s="31" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="M8" s="30" t="s">
-        <v>63</v>
-      </c>
-      <c r="N8" s="28" t="s">
-        <v>64</v>
-      </c>
-      <c r="O8" s="28"/>
-      <c r="P8" s="27"/>
-      <c r="V8" s="4"/>
+        <v>65</v>
+      </c>
+      <c r="N8" s="29" t="s">
+        <v>67</v>
+      </c>
+      <c r="O8" s="29"/>
+      <c r="P8" s="28"/>
+      <c r="V8" s="3"/>
     </row>
     <row r="9" ht="19.5" customHeight="1">
-      <c r="A9" s="23"/>
-      <c r="B9" s="23"/>
+      <c r="A9" s="24"/>
+      <c r="B9" s="24"/>
       <c r="C9" s="32">
         <v>1.0</v>
       </c>
       <c r="D9" s="33" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E9" s="34" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F9" s="35">
         <v>594.0</v>
@@ -1681,7 +1681,7 @@
         <v>45740.0</v>
       </c>
       <c r="H9" s="35" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="I9" s="36"/>
       <c r="J9" s="36">
@@ -1691,26 +1691,26 @@
         <v>748504.24</v>
       </c>
       <c r="L9" s="35" t="s">
-        <v>75</v>
-      </c>
-      <c r="M9" s="38">
+        <v>76</v>
+      </c>
+      <c r="M9" s="39">
         <f t="shared" ref="M9:M10" si="1">K9</f>
         <v>748504.24</v>
       </c>
-      <c r="N9" s="39"/>
-      <c r="O9" s="25"/>
-      <c r="P9" s="27"/>
-      <c r="V9" s="4"/>
+      <c r="N9" s="40"/>
+      <c r="O9" s="26"/>
+      <c r="P9" s="28"/>
+      <c r="V9" s="3"/>
     </row>
     <row r="10" ht="51.0" customHeight="1">
-      <c r="A10" s="23"/>
-      <c r="B10" s="23"/>
+      <c r="A10" s="24"/>
+      <c r="B10" s="24"/>
       <c r="C10" s="41"/>
       <c r="D10" s="33" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="E10" s="34" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F10" s="35">
         <v>620.0</v>
@@ -1719,7 +1719,7 @@
         <v>45775.0</v>
       </c>
       <c r="H10" s="35" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="I10" s="36"/>
       <c r="J10" s="36">
@@ -1729,26 +1729,26 @@
         <v>1110378.24</v>
       </c>
       <c r="L10" s="35" t="s">
-        <v>84</v>
-      </c>
-      <c r="M10" s="38">
+        <v>89</v>
+      </c>
+      <c r="M10" s="39">
         <f t="shared" si="1"/>
         <v>1110378.24</v>
       </c>
       <c r="N10" s="42"/>
-      <c r="O10" s="25"/>
-      <c r="P10" s="27"/>
-      <c r="V10" s="4"/>
+      <c r="O10" s="26"/>
+      <c r="P10" s="28"/>
+      <c r="V10" s="3"/>
     </row>
     <row r="11" ht="12.75" customHeight="1">
-      <c r="A11" s="23"/>
-      <c r="B11" s="23"/>
+      <c r="A11" s="24"/>
+      <c r="B11" s="24"/>
       <c r="C11" s="41"/>
       <c r="D11" s="33" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="E11" s="34" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F11" s="35">
         <v>634.0</v>
@@ -1757,7 +1757,7 @@
         <v>45799.0</v>
       </c>
       <c r="H11" s="35" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="I11" s="36"/>
       <c r="J11" s="36">
@@ -1767,25 +1767,25 @@
         <v>974557.12</v>
       </c>
       <c r="L11" s="34" t="s">
-        <v>92</v>
-      </c>
-      <c r="M11" s="38">
+        <v>96</v>
+      </c>
+      <c r="M11" s="39">
         <v>974557.12</v>
       </c>
       <c r="N11" s="42"/>
-      <c r="O11" s="25"/>
-      <c r="P11" s="27"/>
-      <c r="V11" s="4"/>
+      <c r="O11" s="26"/>
+      <c r="P11" s="28"/>
+      <c r="V11" s="3"/>
     </row>
     <row r="12" ht="27.75" customHeight="1">
-      <c r="A12" s="23"/>
-      <c r="B12" s="23"/>
+      <c r="A12" s="24"/>
+      <c r="B12" s="24"/>
       <c r="C12" s="41"/>
       <c r="D12" s="33" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E12" s="34" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F12" s="34">
         <v>660.0</v>
@@ -1794,7 +1794,7 @@
         <v>45856.0</v>
       </c>
       <c r="H12" s="44" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I12" s="36"/>
       <c r="J12" s="36">
@@ -1804,25 +1804,25 @@
         <v>1402001.34</v>
       </c>
       <c r="L12" s="46" t="s">
-        <v>99</v>
-      </c>
-      <c r="M12" s="38">
+        <v>101</v>
+      </c>
+      <c r="M12" s="39">
         <v>1402001.34</v>
       </c>
       <c r="N12" s="47"/>
-      <c r="O12" s="25"/>
-      <c r="P12" s="27"/>
-      <c r="V12" s="4"/>
+      <c r="O12" s="26"/>
+      <c r="P12" s="28"/>
+      <c r="V12" s="3"/>
     </row>
     <row r="13">
-      <c r="A13" s="23"/>
-      <c r="B13" s="23"/>
+      <c r="A13" s="24"/>
+      <c r="B13" s="24"/>
       <c r="C13" s="41"/>
       <c r="D13" s="48" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="E13" s="34" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F13" s="35">
         <v>661.0</v>
@@ -1841,25 +1841,25 @@
         <v>1223702.3</v>
       </c>
       <c r="L13" s="34" t="s">
-        <v>106</v>
-      </c>
-      <c r="M13" s="38">
+        <v>107</v>
+      </c>
+      <c r="M13" s="39">
         <v>1223702.3</v>
       </c>
       <c r="N13" s="47"/>
-      <c r="O13" s="25"/>
+      <c r="O13" s="26"/>
       <c r="P13" s="49"/>
-      <c r="V13" s="4"/>
+      <c r="V13" s="3"/>
     </row>
     <row r="14">
-      <c r="A14" s="23"/>
-      <c r="B14" s="23"/>
+      <c r="A14" s="24"/>
+      <c r="B14" s="24"/>
       <c r="C14" s="41"/>
       <c r="D14" s="48" t="s">
         <v>109</v>
       </c>
       <c r="E14" s="34" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F14" s="34">
         <v>688.0</v>
@@ -1880,23 +1880,23 @@
       <c r="L14" s="34" t="s">
         <v>114</v>
       </c>
-      <c r="M14" s="38">
+      <c r="M14" s="39">
         <v>1011677.95</v>
       </c>
       <c r="N14" s="42"/>
-      <c r="O14" s="25"/>
-      <c r="P14" s="27"/>
-      <c r="V14" s="4"/>
+      <c r="O14" s="26"/>
+      <c r="P14" s="28"/>
+      <c r="V14" s="3"/>
     </row>
     <row r="15">
-      <c r="A15" s="23"/>
-      <c r="B15" s="23"/>
+      <c r="A15" s="24"/>
+      <c r="B15" s="24"/>
       <c r="C15" s="41"/>
       <c r="D15" s="48" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="E15" s="34" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F15" s="34">
         <v>696.0</v>
@@ -1905,7 +1905,7 @@
         <v>45923.0</v>
       </c>
       <c r="H15" s="34" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I15" s="43"/>
       <c r="J15" s="43">
@@ -1915,24 +1915,24 @@
         <v>896744.06</v>
       </c>
       <c r="L15" s="34" t="s">
-        <v>121</v>
-      </c>
-      <c r="M15" s="38">
+        <v>120</v>
+      </c>
+      <c r="M15" s="39">
         <v>896744.06</v>
       </c>
       <c r="N15" s="47"/>
-      <c r="O15" s="25"/>
-      <c r="V15" s="4"/>
+      <c r="O15" s="26"/>
+      <c r="V15" s="3"/>
     </row>
     <row r="16">
-      <c r="A16" s="23"/>
-      <c r="B16" s="23"/>
+      <c r="A16" s="24"/>
+      <c r="B16" s="24"/>
       <c r="C16" s="41"/>
       <c r="D16" s="48" t="s">
         <v>123</v>
       </c>
       <c r="E16" s="34" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F16" s="34">
         <v>704.0</v>
@@ -1941,7 +1941,7 @@
         <v>45957.0</v>
       </c>
       <c r="H16" s="34" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="I16" s="43"/>
       <c r="J16" s="43">
@@ -1953,19 +1953,19 @@
       <c r="L16" s="34" t="s">
         <v>128</v>
       </c>
-      <c r="M16" s="38">
+      <c r="M16" s="39">
         <v>919329.06</v>
       </c>
       <c r="N16" s="42"/>
-      <c r="O16" s="25"/>
-      <c r="V16" s="4"/>
+      <c r="O16" s="26"/>
+      <c r="V16" s="3"/>
     </row>
     <row r="17">
-      <c r="A17" s="23"/>
-      <c r="B17" s="23"/>
+      <c r="A17" s="24"/>
+      <c r="B17" s="24"/>
       <c r="C17" s="41"/>
       <c r="D17" s="48" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="E17" s="34"/>
       <c r="F17" s="34">
@@ -1975,7 +1975,7 @@
         <v>45972.0</v>
       </c>
       <c r="H17" s="34" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="I17" s="34"/>
       <c r="J17" s="43">
@@ -1985,24 +1985,24 @@
         <v>1157009.26</v>
       </c>
       <c r="L17" s="34" t="s">
-        <v>133</v>
-      </c>
-      <c r="M17" s="38">
+        <v>136</v>
+      </c>
+      <c r="M17" s="39">
         <v>1157009.26</v>
       </c>
       <c r="N17" s="51"/>
-      <c r="O17" s="25"/>
-      <c r="V17" s="4"/>
+      <c r="O17" s="26"/>
+      <c r="V17" s="3"/>
     </row>
     <row r="18">
-      <c r="A18" s="23"/>
-      <c r="B18" s="23"/>
+      <c r="A18" s="24"/>
+      <c r="B18" s="24"/>
       <c r="C18" s="41"/>
       <c r="D18" s="48" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="E18" s="34" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F18" s="34">
         <v>728.0</v>
@@ -2011,7 +2011,7 @@
         <v>46008.0</v>
       </c>
       <c r="H18" s="34" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="I18" s="34"/>
       <c r="J18" s="43">
@@ -2021,28 +2021,28 @@
         <v>1214597.952</v>
       </c>
       <c r="L18" s="34" t="s">
-        <v>142</v>
-      </c>
-      <c r="M18" s="38">
+        <v>145</v>
+      </c>
+      <c r="M18" s="39">
         <v>1214597.952</v>
       </c>
       <c r="N18" s="51"/>
-      <c r="O18" s="25"/>
-      <c r="R18" s="27"/>
-      <c r="S18" s="27"/>
-      <c r="T18" s="27"/>
-      <c r="U18" s="27"/>
+      <c r="O18" s="26"/>
+      <c r="R18" s="28"/>
+      <c r="S18" s="28"/>
+      <c r="T18" s="28"/>
+      <c r="U18" s="28"/>
       <c r="V18" s="52"/>
     </row>
     <row r="19">
-      <c r="A19" s="23"/>
-      <c r="B19" s="23"/>
+      <c r="A19" s="24"/>
+      <c r="B19" s="24"/>
       <c r="C19" s="41"/>
       <c r="D19" s="48" t="s">
-        <v>145</v>
+        <v>152</v>
       </c>
       <c r="E19" s="34" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F19" s="34">
         <v>278.0</v>
@@ -2051,7 +2051,7 @@
         <v>46042.0</v>
       </c>
       <c r="H19" s="34" t="s">
-        <v>147</v>
+        <v>155</v>
       </c>
       <c r="I19" s="43"/>
       <c r="J19" s="43">
@@ -2061,25 +2061,25 @@
         <v>967082.09</v>
       </c>
       <c r="L19" s="34" t="s">
-        <v>148</v>
-      </c>
-      <c r="M19" s="38">
+        <v>156</v>
+      </c>
+      <c r="M19" s="39">
         <v>967082.09</v>
       </c>
       <c r="N19" s="51"/>
-      <c r="O19" s="25"/>
-      <c r="R19" s="27"/>
-      <c r="S19" s="27"/>
-      <c r="T19" s="27"/>
-      <c r="U19" s="27"/>
+      <c r="O19" s="26"/>
+      <c r="R19" s="28"/>
+      <c r="S19" s="28"/>
+      <c r="T19" s="28"/>
+      <c r="U19" s="28"/>
       <c r="V19" s="52"/>
     </row>
     <row r="20">
-      <c r="A20" s="23"/>
-      <c r="B20" s="23"/>
+      <c r="A20" s="24"/>
+      <c r="B20" s="24"/>
       <c r="C20" s="41"/>
       <c r="D20" s="48" t="s">
-        <v>152</v>
+        <v>159</v>
       </c>
       <c r="E20" s="34"/>
       <c r="F20" s="34">
@@ -2099,25 +2099,25 @@
         <v>719561.08</v>
       </c>
       <c r="L20" s="34" t="s">
-        <v>156</v>
-      </c>
-      <c r="M20" s="38">
+        <v>163</v>
+      </c>
+      <c r="M20" s="39">
         <v>719561.08</v>
       </c>
       <c r="N20" s="51"/>
-      <c r="O20" s="25"/>
-      <c r="R20" s="27"/>
-      <c r="S20" s="27"/>
-      <c r="T20" s="27"/>
-      <c r="U20" s="27"/>
+      <c r="O20" s="26"/>
+      <c r="R20" s="28"/>
+      <c r="S20" s="28"/>
+      <c r="T20" s="28"/>
+      <c r="U20" s="28"/>
       <c r="V20" s="52"/>
     </row>
     <row r="21">
-      <c r="A21" s="23"/>
-      <c r="B21" s="23"/>
+      <c r="A21" s="24"/>
+      <c r="B21" s="24"/>
       <c r="C21" s="41"/>
       <c r="D21" s="48" t="s">
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="E21" s="34"/>
       <c r="F21" s="34">
@@ -2127,7 +2127,7 @@
         <v>46094.0</v>
       </c>
       <c r="H21" s="34" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="I21" s="43"/>
       <c r="J21" s="43">
@@ -2137,25 +2137,25 @@
         <v>885881.08</v>
       </c>
       <c r="L21" s="34" t="s">
-        <v>163</v>
-      </c>
-      <c r="M21" s="38">
+        <v>167</v>
+      </c>
+      <c r="M21" s="39">
         <v>885881.08</v>
       </c>
       <c r="N21" s="51"/>
-      <c r="O21" s="25"/>
-      <c r="R21" s="27"/>
-      <c r="S21" s="27"/>
-      <c r="T21" s="27"/>
-      <c r="U21" s="27"/>
+      <c r="O21" s="26"/>
+      <c r="R21" s="28"/>
+      <c r="S21" s="28"/>
+      <c r="T21" s="28"/>
+      <c r="U21" s="28"/>
       <c r="V21" s="52"/>
     </row>
     <row r="22">
-      <c r="A22" s="23"/>
-      <c r="B22" s="23"/>
+      <c r="A22" s="24"/>
+      <c r="B22" s="24"/>
       <c r="C22" s="41"/>
       <c r="D22" s="48" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="E22" s="34"/>
       <c r="F22" s="34">
@@ -2177,20 +2177,20 @@
       <c r="L22" s="34" t="s">
         <v>171</v>
       </c>
-      <c r="M22" s="38" t="s">
+      <c r="M22" s="39" t="s">
         <v>170</v>
       </c>
       <c r="N22" s="51"/>
-      <c r="O22" s="25"/>
-      <c r="R22" s="27"/>
-      <c r="S22" s="27"/>
-      <c r="T22" s="27"/>
-      <c r="U22" s="27"/>
+      <c r="O22" s="26"/>
+      <c r="R22" s="28"/>
+      <c r="S22" s="28"/>
+      <c r="T22" s="28"/>
+      <c r="U22" s="28"/>
       <c r="V22" s="52"/>
     </row>
     <row r="23">
-      <c r="A23" s="23"/>
-      <c r="B23" s="23"/>
+      <c r="A23" s="24"/>
+      <c r="B23" s="24"/>
       <c r="C23" s="41"/>
       <c r="D23" s="48" t="s">
         <v>172</v>
@@ -2213,22 +2213,22 @@
         <v>1108954.4358333333</v>
       </c>
       <c r="L23" s="34" t="s">
-        <v>163</v>
-      </c>
-      <c r="M23" s="38">
+        <v>167</v>
+      </c>
+      <c r="M23" s="39">
         <v>1108954.4358333333</v>
       </c>
       <c r="N23" s="53"/>
-      <c r="O23" s="25"/>
-      <c r="R23" s="27"/>
-      <c r="S23" s="27"/>
-      <c r="T23" s="27"/>
-      <c r="U23" s="27"/>
+      <c r="O23" s="26"/>
+      <c r="R23" s="28"/>
+      <c r="S23" s="28"/>
+      <c r="T23" s="28"/>
+      <c r="U23" s="28"/>
       <c r="V23" s="52"/>
     </row>
     <row r="24">
-      <c r="A24" s="23"/>
-      <c r="B24" s="23"/>
+      <c r="A24" s="24"/>
+      <c r="B24" s="24"/>
       <c r="C24" s="41"/>
       <c r="D24" s="48" t="s">
         <v>174</v>
@@ -2253,20 +2253,20 @@
       <c r="L24" s="34" t="s">
         <v>175</v>
       </c>
-      <c r="M24" s="38">
+      <c r="M24" s="39">
         <v>218206.1</v>
       </c>
       <c r="N24" s="54"/>
-      <c r="O24" s="25"/>
-      <c r="R24" s="27"/>
-      <c r="S24" s="27"/>
-      <c r="T24" s="27"/>
-      <c r="U24" s="27"/>
+      <c r="O24" s="26"/>
+      <c r="R24" s="28"/>
+      <c r="S24" s="28"/>
+      <c r="T24" s="28"/>
+      <c r="U24" s="28"/>
       <c r="V24" s="52"/>
     </row>
     <row r="25">
-      <c r="A25" s="23"/>
-      <c r="B25" s="23"/>
+      <c r="A25" s="24"/>
+      <c r="B25" s="24"/>
       <c r="C25" s="41"/>
       <c r="D25" s="48" t="s">
         <v>176</v>
@@ -2291,20 +2291,20 @@
       <c r="L25" s="34" t="s">
         <v>177</v>
       </c>
-      <c r="M25" s="38">
+      <c r="M25" s="39">
         <v>1549250.84</v>
       </c>
       <c r="N25" s="54"/>
-      <c r="O25" s="25"/>
-      <c r="R25" s="27"/>
-      <c r="S25" s="27"/>
-      <c r="T25" s="27"/>
-      <c r="U25" s="27"/>
+      <c r="O25" s="26"/>
+      <c r="R25" s="28"/>
+      <c r="S25" s="28"/>
+      <c r="T25" s="28"/>
+      <c r="U25" s="28"/>
       <c r="V25" s="52"/>
     </row>
     <row r="26">
-      <c r="A26" s="23"/>
-      <c r="B26" s="23"/>
+      <c r="A26" s="24"/>
+      <c r="B26" s="24"/>
       <c r="C26" s="55"/>
       <c r="D26" s="48" t="s">
         <v>178</v>
@@ -2329,20 +2329,20 @@
       <c r="L26" s="34" t="s">
         <v>181</v>
       </c>
-      <c r="M26" s="38" t="s">
+      <c r="M26" s="39" t="s">
         <v>180</v>
       </c>
       <c r="N26" s="54"/>
-      <c r="O26" s="25"/>
-      <c r="R26" s="27"/>
-      <c r="S26" s="27"/>
-      <c r="T26" s="27"/>
-      <c r="U26" s="27"/>
+      <c r="O26" s="26"/>
+      <c r="R26" s="28"/>
+      <c r="S26" s="28"/>
+      <c r="T26" s="28"/>
+      <c r="U26" s="28"/>
       <c r="V26" s="52"/>
     </row>
     <row r="27">
-      <c r="A27" s="23"/>
-      <c r="B27" s="23"/>
+      <c r="A27" s="24"/>
+      <c r="B27" s="24"/>
       <c r="C27" s="35"/>
       <c r="D27" s="48" t="s">
         <v>182</v>
@@ -2355,7 +2355,7 @@
         <v>46252.0</v>
       </c>
       <c r="H27" s="34" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="I27" s="43"/>
       <c r="J27" s="43">
@@ -2363,68 +2363,68 @@
       </c>
       <c r="K27" s="45"/>
       <c r="L27" s="34"/>
-      <c r="M27" s="38" t="s">
+      <c r="M27" s="39" t="s">
         <v>183</v>
       </c>
       <c r="N27" s="54"/>
-      <c r="O27" s="25"/>
-      <c r="R27" s="27"/>
-      <c r="S27" s="27"/>
-      <c r="T27" s="27"/>
-      <c r="U27" s="27"/>
+      <c r="O27" s="26"/>
+      <c r="R27" s="28"/>
+      <c r="S27" s="28"/>
+      <c r="T27" s="28"/>
+      <c r="U27" s="28"/>
       <c r="V27" s="52"/>
     </row>
     <row r="28" ht="30.75" customHeight="1">
-      <c r="A28" s="23"/>
-      <c r="B28" s="23"/>
-      <c r="C28" s="28" t="s">
-        <v>49</v>
-      </c>
-      <c r="D28" s="28" t="s">
-        <v>50</v>
+      <c r="A28" s="24"/>
+      <c r="B28" s="24"/>
+      <c r="C28" s="29" t="s">
+        <v>53</v>
+      </c>
+      <c r="D28" s="29" t="s">
+        <v>54</v>
       </c>
       <c r="E28" s="30" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="F28" s="30" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="G28" s="30"/>
       <c r="H28" s="30" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="I28" s="30"/>
       <c r="J28" s="30"/>
       <c r="K28" s="30" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="L28" s="30" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="M28" s="30" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="N28" s="30" t="s">
-        <v>64</v>
-      </c>
-      <c r="O28" s="25"/>
-      <c r="P28" s="27"/>
-      <c r="R28" s="27"/>
-      <c r="S28" s="27"/>
-      <c r="T28" s="27"/>
-      <c r="U28" s="27"/>
+        <v>67</v>
+      </c>
+      <c r="O28" s="26"/>
+      <c r="P28" s="28"/>
+      <c r="R28" s="28"/>
+      <c r="S28" s="28"/>
+      <c r="T28" s="28"/>
+      <c r="U28" s="28"/>
       <c r="V28" s="52"/>
-      <c r="W28" s="27"/>
-      <c r="X28" s="27"/>
-      <c r="Y28" s="27"/>
-      <c r="Z28" s="27"/>
-      <c r="AA28" s="27"/>
-      <c r="AB28" s="27"/>
-      <c r="AC28" s="27"/>
+      <c r="W28" s="28"/>
+      <c r="X28" s="28"/>
+      <c r="Y28" s="28"/>
+      <c r="Z28" s="28"/>
+      <c r="AA28" s="28"/>
+      <c r="AB28" s="28"/>
+      <c r="AC28" s="28"/>
     </row>
     <row r="29" ht="12.75" customHeight="1">
-      <c r="A29" s="23"/>
-      <c r="B29" s="23"/>
+      <c r="A29" s="24"/>
+      <c r="B29" s="24"/>
       <c r="C29" s="32">
         <v>2.0</v>
       </c>
@@ -2439,7 +2439,7 @@
         <v>45791.0</v>
       </c>
       <c r="H29" s="35" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="I29" s="36"/>
       <c r="J29" s="36">
@@ -2455,25 +2455,25 @@
         <v>188246.17</v>
       </c>
       <c r="N29" s="51"/>
-      <c r="O29" s="25"/>
-      <c r="P29" s="27"/>
-      <c r="Q29" s="27"/>
-      <c r="R29" s="27"/>
-      <c r="S29" s="27"/>
-      <c r="T29" s="27"/>
-      <c r="U29" s="27"/>
+      <c r="O29" s="26"/>
+      <c r="P29" s="28"/>
+      <c r="Q29" s="28"/>
+      <c r="R29" s="28"/>
+      <c r="S29" s="28"/>
+      <c r="T29" s="28"/>
+      <c r="U29" s="28"/>
       <c r="V29" s="52"/>
-      <c r="W29" s="27"/>
-      <c r="X29" s="27"/>
-      <c r="Y29" s="27"/>
-      <c r="Z29" s="27"/>
-      <c r="AA29" s="27"/>
-      <c r="AB29" s="27"/>
-      <c r="AC29" s="27"/>
+      <c r="W29" s="28"/>
+      <c r="X29" s="28"/>
+      <c r="Y29" s="28"/>
+      <c r="Z29" s="28"/>
+      <c r="AA29" s="28"/>
+      <c r="AB29" s="28"/>
+      <c r="AC29" s="28"/>
     </row>
     <row r="30">
-      <c r="A30" s="23"/>
-      <c r="B30" s="23"/>
+      <c r="A30" s="24"/>
+      <c r="B30" s="24"/>
       <c r="C30" s="41"/>
       <c r="D30" s="56" t="s">
         <v>186</v>
@@ -2500,29 +2500,29 @@
       <c r="L30" s="34" t="s">
         <v>188</v>
       </c>
-      <c r="M30" s="38">
+      <c r="M30" s="39">
         <v>112720.77</v>
       </c>
       <c r="N30" s="51"/>
-      <c r="O30" s="25"/>
-      <c r="P30" s="27"/>
-      <c r="Q30" s="27"/>
-      <c r="R30" s="27"/>
-      <c r="S30" s="27"/>
-      <c r="T30" s="27"/>
-      <c r="U30" s="27"/>
+      <c r="O30" s="26"/>
+      <c r="P30" s="28"/>
+      <c r="Q30" s="28"/>
+      <c r="R30" s="28"/>
+      <c r="S30" s="28"/>
+      <c r="T30" s="28"/>
+      <c r="U30" s="28"/>
       <c r="V30" s="52"/>
-      <c r="W30" s="27"/>
-      <c r="X30" s="27"/>
-      <c r="Y30" s="27"/>
-      <c r="Z30" s="27"/>
-      <c r="AA30" s="27"/>
-      <c r="AB30" s="27"/>
-      <c r="AC30" s="27"/>
+      <c r="W30" s="28"/>
+      <c r="X30" s="28"/>
+      <c r="Y30" s="28"/>
+      <c r="Z30" s="28"/>
+      <c r="AA30" s="28"/>
+      <c r="AB30" s="28"/>
+      <c r="AC30" s="28"/>
     </row>
     <row r="31" ht="12.75" customHeight="1">
-      <c r="A31" s="23"/>
-      <c r="B31" s="23"/>
+      <c r="A31" s="24"/>
+      <c r="B31" s="24"/>
       <c r="C31" s="41"/>
       <c r="D31" s="59" t="s">
         <v>189</v>
@@ -2537,7 +2537,7 @@
         <v>45853.0</v>
       </c>
       <c r="H31" s="34" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="I31" s="43"/>
       <c r="J31" s="43">
@@ -2549,29 +2549,29 @@
       <c r="L31" s="34" t="s">
         <v>191</v>
       </c>
-      <c r="M31" s="38">
+      <c r="M31" s="39">
         <v>378307.61</v>
       </c>
       <c r="N31" s="51"/>
-      <c r="O31" s="25"/>
+      <c r="O31" s="26"/>
       <c r="P31" s="62"/>
-      <c r="Q31" s="27"/>
-      <c r="R31" s="27"/>
-      <c r="S31" s="27"/>
-      <c r="T31" s="27"/>
-      <c r="U31" s="27"/>
+      <c r="Q31" s="28"/>
+      <c r="R31" s="28"/>
+      <c r="S31" s="28"/>
+      <c r="T31" s="28"/>
+      <c r="U31" s="28"/>
       <c r="V31" s="52"/>
-      <c r="W31" s="27"/>
-      <c r="X31" s="27"/>
-      <c r="Y31" s="27"/>
-      <c r="Z31" s="27"/>
-      <c r="AA31" s="27"/>
-      <c r="AB31" s="27"/>
-      <c r="AC31" s="27"/>
+      <c r="W31" s="28"/>
+      <c r="X31" s="28"/>
+      <c r="Y31" s="28"/>
+      <c r="Z31" s="28"/>
+      <c r="AA31" s="28"/>
+      <c r="AB31" s="28"/>
+      <c r="AC31" s="28"/>
     </row>
     <row r="32" ht="60.0" customHeight="1">
-      <c r="A32" s="23"/>
-      <c r="B32" s="23"/>
+      <c r="A32" s="24"/>
+      <c r="B32" s="24"/>
       <c r="C32" s="41"/>
       <c r="D32" s="59" t="s">
         <v>192</v>
@@ -2586,7 +2586,7 @@
         <v>45910.0</v>
       </c>
       <c r="H32" s="34" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="I32" s="43"/>
       <c r="J32" s="43">
@@ -2598,29 +2598,29 @@
       <c r="L32" s="34" t="s">
         <v>193</v>
       </c>
-      <c r="M32" s="38">
+      <c r="M32" s="39">
         <v>3315.04710000003</v>
       </c>
       <c r="N32" s="51"/>
-      <c r="O32" s="25"/>
+      <c r="O32" s="26"/>
       <c r="P32" s="62"/>
-      <c r="Q32" s="27"/>
-      <c r="R32" s="27"/>
-      <c r="S32" s="27"/>
-      <c r="T32" s="27"/>
-      <c r="U32" s="27"/>
+      <c r="Q32" s="28"/>
+      <c r="R32" s="28"/>
+      <c r="S32" s="28"/>
+      <c r="T32" s="28"/>
+      <c r="U32" s="28"/>
       <c r="V32" s="52"/>
-      <c r="W32" s="27"/>
-      <c r="X32" s="27"/>
-      <c r="Y32" s="27"/>
-      <c r="Z32" s="27"/>
-      <c r="AA32" s="27"/>
-      <c r="AB32" s="27"/>
-      <c r="AC32" s="27"/>
+      <c r="W32" s="28"/>
+      <c r="X32" s="28"/>
+      <c r="Y32" s="28"/>
+      <c r="Z32" s="28"/>
+      <c r="AA32" s="28"/>
+      <c r="AB32" s="28"/>
+      <c r="AC32" s="28"/>
     </row>
     <row r="33" ht="12.75" customHeight="1">
-      <c r="A33" s="23"/>
-      <c r="B33" s="23"/>
+      <c r="A33" s="24"/>
+      <c r="B33" s="24"/>
       <c r="C33" s="41"/>
       <c r="D33" s="59" t="s">
         <v>194</v>
@@ -2635,7 +2635,7 @@
         <v>45904.0</v>
       </c>
       <c r="H33" s="34" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I33" s="64"/>
       <c r="J33" s="64">
@@ -2647,29 +2647,29 @@
       <c r="L33" s="34" t="s">
         <v>195</v>
       </c>
-      <c r="M33" s="38">
+      <c r="M33" s="39">
         <v>198332.75</v>
       </c>
       <c r="N33" s="51"/>
-      <c r="O33" s="25"/>
+      <c r="O33" s="26"/>
       <c r="P33" s="62"/>
-      <c r="Q33" s="27"/>
-      <c r="R33" s="27"/>
-      <c r="S33" s="27"/>
-      <c r="T33" s="27"/>
-      <c r="U33" s="27"/>
+      <c r="Q33" s="28"/>
+      <c r="R33" s="28"/>
+      <c r="S33" s="28"/>
+      <c r="T33" s="28"/>
+      <c r="U33" s="28"/>
       <c r="V33" s="52"/>
-      <c r="W33" s="27"/>
-      <c r="X33" s="27"/>
-      <c r="Y33" s="27"/>
-      <c r="Z33" s="27"/>
-      <c r="AA33" s="27"/>
-      <c r="AB33" s="27"/>
-      <c r="AC33" s="27"/>
+      <c r="W33" s="28"/>
+      <c r="X33" s="28"/>
+      <c r="Y33" s="28"/>
+      <c r="Z33" s="28"/>
+      <c r="AA33" s="28"/>
+      <c r="AB33" s="28"/>
+      <c r="AC33" s="28"/>
     </row>
     <row r="34" ht="12.75" customHeight="1">
-      <c r="A34" s="23"/>
-      <c r="B34" s="23"/>
+      <c r="A34" s="24"/>
+      <c r="B34" s="24"/>
       <c r="C34" s="41"/>
       <c r="D34" s="59" t="s">
         <v>196</v>
@@ -2684,7 +2684,7 @@
         <v>46008.0</v>
       </c>
       <c r="H34" s="34" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="I34" s="64"/>
       <c r="J34" s="64">
@@ -2700,25 +2700,25 @@
         <v>198</v>
       </c>
       <c r="N34" s="51"/>
-      <c r="O34" s="25"/>
+      <c r="O34" s="26"/>
       <c r="P34" s="62"/>
-      <c r="Q34" s="27"/>
-      <c r="R34" s="27"/>
-      <c r="S34" s="27"/>
-      <c r="T34" s="27"/>
-      <c r="U34" s="27"/>
+      <c r="Q34" s="28"/>
+      <c r="R34" s="28"/>
+      <c r="S34" s="28"/>
+      <c r="T34" s="28"/>
+      <c r="U34" s="28"/>
       <c r="V34" s="52"/>
-      <c r="W34" s="27"/>
-      <c r="X34" s="27"/>
-      <c r="Y34" s="27"/>
-      <c r="Z34" s="27"/>
-      <c r="AA34" s="27"/>
-      <c r="AB34" s="27"/>
-      <c r="AC34" s="27"/>
+      <c r="W34" s="28"/>
+      <c r="X34" s="28"/>
+      <c r="Y34" s="28"/>
+      <c r="Z34" s="28"/>
+      <c r="AA34" s="28"/>
+      <c r="AB34" s="28"/>
+      <c r="AC34" s="28"/>
     </row>
     <row r="35" ht="12.75" customHeight="1">
-      <c r="A35" s="23"/>
-      <c r="B35" s="23"/>
+      <c r="A35" s="24"/>
+      <c r="B35" s="24"/>
       <c r="C35" s="41"/>
       <c r="D35" s="59" t="s">
         <v>199</v>
@@ -2733,7 +2733,7 @@
         <v>45930.0</v>
       </c>
       <c r="H35" s="34" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="I35" s="64"/>
       <c r="J35" s="64">
@@ -2749,25 +2749,25 @@
         <v>202</v>
       </c>
       <c r="N35" s="51"/>
-      <c r="O35" s="25"/>
+      <c r="O35" s="26"/>
       <c r="P35" s="62"/>
-      <c r="Q35" s="27"/>
-      <c r="R35" s="27"/>
-      <c r="S35" s="27"/>
-      <c r="T35" s="27"/>
-      <c r="U35" s="27"/>
+      <c r="Q35" s="28"/>
+      <c r="R35" s="28"/>
+      <c r="S35" s="28"/>
+      <c r="T35" s="28"/>
+      <c r="U35" s="28"/>
       <c r="V35" s="52"/>
-      <c r="W35" s="27"/>
-      <c r="X35" s="27"/>
-      <c r="Y35" s="27"/>
-      <c r="Z35" s="27"/>
-      <c r="AA35" s="27"/>
-      <c r="AB35" s="27"/>
-      <c r="AC35" s="27"/>
+      <c r="W35" s="28"/>
+      <c r="X35" s="28"/>
+      <c r="Y35" s="28"/>
+      <c r="Z35" s="28"/>
+      <c r="AA35" s="28"/>
+      <c r="AB35" s="28"/>
+      <c r="AC35" s="28"/>
     </row>
     <row r="36" ht="12.75" customHeight="1">
-      <c r="A36" s="23"/>
-      <c r="B36" s="23"/>
+      <c r="A36" s="24"/>
+      <c r="B36" s="24"/>
       <c r="C36" s="41"/>
       <c r="D36" s="59" t="s">
         <v>203</v>
@@ -2782,7 +2782,7 @@
         <v>45968.0</v>
       </c>
       <c r="H36" s="34" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="I36" s="64"/>
       <c r="J36" s="64">
@@ -2798,25 +2798,25 @@
         <v>205</v>
       </c>
       <c r="N36" s="51"/>
-      <c r="O36" s="25"/>
+      <c r="O36" s="26"/>
       <c r="P36" s="62"/>
-      <c r="Q36" s="27"/>
-      <c r="R36" s="27"/>
-      <c r="S36" s="27"/>
-      <c r="T36" s="27"/>
-      <c r="U36" s="27"/>
+      <c r="Q36" s="28"/>
+      <c r="R36" s="28"/>
+      <c r="S36" s="28"/>
+      <c r="T36" s="28"/>
+      <c r="U36" s="28"/>
       <c r="V36" s="52"/>
-      <c r="W36" s="27"/>
-      <c r="X36" s="27"/>
-      <c r="Y36" s="27"/>
-      <c r="Z36" s="27"/>
-      <c r="AA36" s="27"/>
-      <c r="AB36" s="27"/>
-      <c r="AC36" s="27"/>
+      <c r="W36" s="28"/>
+      <c r="X36" s="28"/>
+      <c r="Y36" s="28"/>
+      <c r="Z36" s="28"/>
+      <c r="AA36" s="28"/>
+      <c r="AB36" s="28"/>
+      <c r="AC36" s="28"/>
     </row>
     <row r="37" ht="12.75" customHeight="1">
-      <c r="A37" s="23"/>
-      <c r="B37" s="23"/>
+      <c r="A37" s="24"/>
+      <c r="B37" s="24"/>
       <c r="C37" s="41"/>
       <c r="D37" s="59" t="s">
         <v>206</v>
@@ -2843,29 +2843,29 @@
       <c r="L37" s="34" t="s">
         <v>207</v>
       </c>
-      <c r="M37" s="38">
+      <c r="M37" s="39">
         <v>11372.9</v>
       </c>
       <c r="N37" s="51"/>
-      <c r="O37" s="25"/>
-      <c r="P37" s="27"/>
-      <c r="Q37" s="27"/>
-      <c r="R37" s="27"/>
-      <c r="S37" s="27"/>
-      <c r="T37" s="27"/>
-      <c r="U37" s="27"/>
+      <c r="O37" s="26"/>
+      <c r="P37" s="28"/>
+      <c r="Q37" s="28"/>
+      <c r="R37" s="28"/>
+      <c r="S37" s="28"/>
+      <c r="T37" s="28"/>
+      <c r="U37" s="28"/>
       <c r="V37" s="52"/>
-      <c r="W37" s="27"/>
-      <c r="X37" s="27"/>
-      <c r="Y37" s="27"/>
-      <c r="Z37" s="27"/>
-      <c r="AA37" s="27"/>
-      <c r="AB37" s="27"/>
-      <c r="AC37" s="27"/>
+      <c r="W37" s="28"/>
+      <c r="X37" s="28"/>
+      <c r="Y37" s="28"/>
+      <c r="Z37" s="28"/>
+      <c r="AA37" s="28"/>
+      <c r="AB37" s="28"/>
+      <c r="AC37" s="28"/>
     </row>
     <row r="38" ht="12.75" customHeight="1">
-      <c r="A38" s="23"/>
-      <c r="B38" s="23"/>
+      <c r="A38" s="24"/>
+      <c r="B38" s="24"/>
       <c r="C38" s="41"/>
       <c r="D38" s="59" t="s">
         <v>208</v>
@@ -2880,29 +2880,29 @@
       <c r="J38" s="67"/>
       <c r="K38" s="45"/>
       <c r="L38" s="34"/>
-      <c r="M38" s="38"/>
+      <c r="M38" s="39"/>
       <c r="N38" s="51">
         <v>15854.78</v>
       </c>
-      <c r="O38" s="25"/>
-      <c r="P38" s="27"/>
-      <c r="Q38" s="27"/>
-      <c r="R38" s="27"/>
-      <c r="S38" s="27"/>
-      <c r="T38" s="27"/>
-      <c r="U38" s="27"/>
+      <c r="O38" s="26"/>
+      <c r="P38" s="28"/>
+      <c r="Q38" s="28"/>
+      <c r="R38" s="28"/>
+      <c r="S38" s="28"/>
+      <c r="T38" s="28"/>
+      <c r="U38" s="28"/>
       <c r="V38" s="52"/>
-      <c r="W38" s="27"/>
-      <c r="X38" s="27"/>
-      <c r="Y38" s="27"/>
-      <c r="Z38" s="27"/>
-      <c r="AA38" s="27"/>
-      <c r="AB38" s="27"/>
-      <c r="AC38" s="27"/>
+      <c r="W38" s="28"/>
+      <c r="X38" s="28"/>
+      <c r="Y38" s="28"/>
+      <c r="Z38" s="28"/>
+      <c r="AA38" s="28"/>
+      <c r="AB38" s="28"/>
+      <c r="AC38" s="28"/>
     </row>
     <row r="39" ht="12.75" customHeight="1">
-      <c r="A39" s="23"/>
-      <c r="B39" s="23"/>
+      <c r="A39" s="24"/>
+      <c r="B39" s="24"/>
       <c r="C39" s="55"/>
       <c r="D39" s="59" t="s">
         <v>210</v>
@@ -2917,29 +2917,29 @@
       <c r="J39" s="67"/>
       <c r="K39" s="45"/>
       <c r="L39" s="34"/>
-      <c r="M39" s="38"/>
+      <c r="M39" s="39"/>
       <c r="N39" s="69">
         <v>42229.72325</v>
       </c>
-      <c r="O39" s="25"/>
-      <c r="P39" s="27"/>
-      <c r="Q39" s="27"/>
-      <c r="R39" s="27"/>
-      <c r="S39" s="27"/>
-      <c r="T39" s="27"/>
-      <c r="U39" s="27"/>
+      <c r="O39" s="26"/>
+      <c r="P39" s="28"/>
+      <c r="Q39" s="28"/>
+      <c r="R39" s="28"/>
+      <c r="S39" s="28"/>
+      <c r="T39" s="28"/>
+      <c r="U39" s="28"/>
       <c r="V39" s="52"/>
-      <c r="W39" s="27"/>
-      <c r="X39" s="27"/>
-      <c r="Y39" s="27"/>
-      <c r="Z39" s="27"/>
-      <c r="AA39" s="27"/>
-      <c r="AB39" s="27"/>
-      <c r="AC39" s="27"/>
+      <c r="W39" s="28"/>
+      <c r="X39" s="28"/>
+      <c r="Y39" s="28"/>
+      <c r="Z39" s="28"/>
+      <c r="AA39" s="28"/>
+      <c r="AB39" s="28"/>
+      <c r="AC39" s="28"/>
     </row>
     <row r="40" ht="12.75" customHeight="1">
-      <c r="A40" s="23"/>
-      <c r="B40" s="23"/>
+      <c r="A40" s="24"/>
+      <c r="B40" s="24"/>
       <c r="C40" s="35"/>
       <c r="D40" s="59" t="s">
         <v>211</v>
@@ -2954,29 +2954,29 @@
       <c r="J40" s="67"/>
       <c r="K40" s="45"/>
       <c r="L40" s="46"/>
-      <c r="M40" s="38"/>
+      <c r="M40" s="39"/>
       <c r="N40" s="70">
         <v>48857.395500000006</v>
       </c>
-      <c r="O40" s="25"/>
-      <c r="P40" s="27"/>
-      <c r="Q40" s="27"/>
-      <c r="R40" s="27"/>
-      <c r="S40" s="27"/>
-      <c r="T40" s="27"/>
-      <c r="U40" s="27"/>
+      <c r="O40" s="26"/>
+      <c r="P40" s="28"/>
+      <c r="Q40" s="28"/>
+      <c r="R40" s="28"/>
+      <c r="S40" s="28"/>
+      <c r="T40" s="28"/>
+      <c r="U40" s="28"/>
       <c r="V40" s="52"/>
-      <c r="W40" s="27"/>
-      <c r="X40" s="27"/>
-      <c r="Y40" s="27"/>
-      <c r="Z40" s="27"/>
-      <c r="AA40" s="27"/>
-      <c r="AB40" s="27"/>
-      <c r="AC40" s="27"/>
+      <c r="W40" s="28"/>
+      <c r="X40" s="28"/>
+      <c r="Y40" s="28"/>
+      <c r="Z40" s="28"/>
+      <c r="AA40" s="28"/>
+      <c r="AB40" s="28"/>
+      <c r="AC40" s="28"/>
     </row>
     <row r="41" ht="12.75" customHeight="1">
-      <c r="A41" s="23"/>
-      <c r="B41" s="23"/>
+      <c r="A41" s="24"/>
+      <c r="B41" s="24"/>
       <c r="C41" s="35"/>
       <c r="D41" s="59" t="s">
         <v>212</v>
@@ -2991,27 +2991,27 @@
       <c r="J41" s="67"/>
       <c r="K41" s="45"/>
       <c r="L41" s="46"/>
-      <c r="M41" s="38"/>
+      <c r="M41" s="39"/>
       <c r="N41" s="70"/>
-      <c r="O41" s="25"/>
-      <c r="P41" s="27"/>
-      <c r="Q41" s="27"/>
-      <c r="R41" s="27"/>
-      <c r="S41" s="27"/>
-      <c r="T41" s="27"/>
-      <c r="U41" s="27"/>
+      <c r="O41" s="26"/>
+      <c r="P41" s="28"/>
+      <c r="Q41" s="28"/>
+      <c r="R41" s="28"/>
+      <c r="S41" s="28"/>
+      <c r="T41" s="28"/>
+      <c r="U41" s="28"/>
       <c r="V41" s="52"/>
-      <c r="W41" s="27"/>
-      <c r="X41" s="27"/>
-      <c r="Y41" s="27"/>
-      <c r="Z41" s="27"/>
-      <c r="AA41" s="27"/>
-      <c r="AB41" s="27"/>
-      <c r="AC41" s="27"/>
+      <c r="W41" s="28"/>
+      <c r="X41" s="28"/>
+      <c r="Y41" s="28"/>
+      <c r="Z41" s="28"/>
+      <c r="AA41" s="28"/>
+      <c r="AB41" s="28"/>
+      <c r="AC41" s="28"/>
     </row>
     <row r="42" ht="12.75" customHeight="1">
-      <c r="A42" s="23"/>
-      <c r="B42" s="23"/>
+      <c r="A42" s="24"/>
+      <c r="B42" s="24"/>
       <c r="C42" s="32">
         <v>3.0</v>
       </c>
@@ -3042,21 +3042,21 @@
         <v>27801.11</v>
       </c>
       <c r="N42" s="51"/>
-      <c r="O42" s="25"/>
-      <c r="P42" s="27"/>
-      <c r="Q42" s="27"/>
-      <c r="R42" s="27"/>
-      <c r="S42" s="27"/>
-      <c r="T42" s="27"/>
-      <c r="U42" s="27"/>
+      <c r="O42" s="26"/>
+      <c r="P42" s="28"/>
+      <c r="Q42" s="28"/>
+      <c r="R42" s="28"/>
+      <c r="S42" s="28"/>
+      <c r="T42" s="28"/>
+      <c r="U42" s="28"/>
       <c r="V42" s="52"/>
-      <c r="W42" s="27"/>
-      <c r="X42" s="27"/>
-      <c r="Y42" s="27"/>
-      <c r="Z42" s="27"/>
-      <c r="AA42" s="27"/>
-      <c r="AB42" s="27"/>
-      <c r="AC42" s="27"/>
+      <c r="W42" s="28"/>
+      <c r="X42" s="28"/>
+      <c r="Y42" s="28"/>
+      <c r="Z42" s="28"/>
+      <c r="AA42" s="28"/>
+      <c r="AB42" s="28"/>
+      <c r="AC42" s="28"/>
     </row>
     <row r="43" ht="12.75" customHeight="1">
       <c r="A43" s="15"/>
@@ -3083,13 +3083,13 @@
         <v>58868.35</v>
       </c>
       <c r="L43" s="34" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="M43" s="72">
         <v>58868.35</v>
       </c>
       <c r="N43" s="51"/>
-      <c r="V43" s="4"/>
+      <c r="V43" s="3"/>
     </row>
     <row r="44" ht="12.75" customHeight="1">
       <c r="A44" s="15"/>
@@ -3097,7 +3097,7 @@
       <c r="C44" s="41"/>
       <c r="K44" s="73"/>
       <c r="M44" s="73"/>
-      <c r="V44" s="4"/>
+      <c r="V44" s="3"/>
     </row>
     <row r="45" ht="12.75" customHeight="1">
       <c r="A45" s="15"/>
@@ -3105,31 +3105,31 @@
       <c r="C45" s="41"/>
       <c r="K45" s="73"/>
       <c r="M45" s="73"/>
-      <c r="V45" s="4"/>
+      <c r="V45" s="3"/>
     </row>
     <row r="46" ht="12.75" customHeight="1">
       <c r="A46" s="15"/>
       <c r="B46" s="15"/>
       <c r="C46" s="41"/>
-      <c r="V46" s="4"/>
+      <c r="V46" s="3"/>
     </row>
     <row r="47" ht="12.75" customHeight="1">
       <c r="A47" s="15"/>
       <c r="B47" s="15"/>
       <c r="C47" s="41"/>
-      <c r="V47" s="4"/>
+      <c r="V47" s="3"/>
     </row>
     <row r="48" ht="12.75" customHeight="1">
       <c r="A48" s="15"/>
       <c r="B48" s="15"/>
       <c r="C48" s="41"/>
-      <c r="V48" s="4"/>
+      <c r="V48" s="3"/>
     </row>
     <row r="49" ht="12.75" customHeight="1">
       <c r="A49" s="15"/>
       <c r="B49" s="15"/>
       <c r="C49" s="41"/>
-      <c r="V49" s="4"/>
+      <c r="V49" s="3"/>
     </row>
     <row r="50" ht="12.75" customHeight="1">
       <c r="A50" s="15"/>
@@ -3137,7 +3137,7 @@
       <c r="C50" s="55"/>
       <c r="K50" s="73"/>
       <c r="M50" s="73"/>
-      <c r="V50" s="4"/>
+      <c r="V50" s="3"/>
     </row>
     <row r="51" ht="12.75" customHeight="1">
       <c r="A51" s="15"/>
@@ -3161,7 +3161,7 @@
       <c r="S51" s="74"/>
       <c r="T51" s="74"/>
       <c r="U51" s="74"/>
-      <c r="V51" s="4"/>
+      <c r="V51" s="3"/>
     </row>
     <row r="52" ht="12.75" customHeight="1">
       <c r="A52" s="15"/>
@@ -8042,11 +8042,11 @@
       <c r="AH1" s="2"/>
     </row>
     <row r="2">
-      <c r="A2" s="3">
+      <c r="A2" s="5">
         <v>46258.0</v>
       </c>
-      <c r="L2" s="5" t="s">
-        <v>0</v>
+      <c r="L2" s="7" t="s">
+        <v>1</v>
       </c>
       <c r="AB2" s="2"/>
       <c r="AC2" s="2"/>
@@ -8057,31 +8057,31 @@
       <c r="AH2" s="2"/>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="10" t="s">
         <v>3</v>
       </c>
       <c r="C3" s="11">
         <v>2.5E32</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="D3" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E3" s="12">
         <v>45686.0</v>
       </c>
-      <c r="F3" s="8" t="s">
+      <c r="F3" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G3" s="8">
+      <c r="G3" s="10">
         <v>12.0</v>
       </c>
-      <c r="H3" s="8">
+      <c r="H3" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I3" s="8">
+      <c r="I3" s="10">
         <v>2048.0</v>
       </c>
       <c r="J3" s="14">
@@ -8090,7 +8090,7 @@
       <c r="K3" s="14">
         <v>1000.0</v>
       </c>
-      <c r="L3" s="8">
+      <c r="L3" s="10">
         <v>0.0</v>
       </c>
       <c r="AB3" s="2"/>
@@ -8102,31 +8102,31 @@
       <c r="AH3" s="2"/>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="C4" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="D4" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E4" s="12">
         <v>45762.0</v>
       </c>
-      <c r="F4" s="8" t="s">
+      <c r="F4" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G4" s="8">
+      <c r="G4" s="10">
         <v>12.0</v>
       </c>
-      <c r="H4" s="8">
+      <c r="H4" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I4" s="8">
+      <c r="I4" s="10">
         <v>2048.0</v>
       </c>
       <c r="J4" s="14">
@@ -8135,7 +8135,7 @@
       <c r="K4" s="14">
         <v>52250.04</v>
       </c>
-      <c r="L4" s="8">
+      <c r="L4" s="10">
         <v>0.0</v>
       </c>
       <c r="AB4" s="2"/>
@@ -8147,31 +8147,31 @@
       <c r="AH4" s="2"/>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="B5" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="C5" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="D5" s="8" t="s">
+      <c r="A5" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E5" s="12">
         <v>45762.0</v>
       </c>
-      <c r="F5" s="8" t="s">
+      <c r="F5" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G5" s="8">
+      <c r="G5" s="10">
         <v>12.0</v>
       </c>
-      <c r="H5" s="8">
+      <c r="H5" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I5" s="8">
+      <c r="I5" s="10">
         <v>2048.0</v>
       </c>
       <c r="J5" s="14">
@@ -8180,7 +8180,7 @@
       <c r="K5" s="14">
         <v>881914.18</v>
       </c>
-      <c r="L5" s="8">
+      <c r="L5" s="10">
         <v>0.0</v>
       </c>
       <c r="AB5" s="2"/>
@@ -8192,31 +8192,31 @@
       <c r="AH5" s="2"/>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="B6" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="C6" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="D6" s="8" t="s">
+      <c r="A6" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="D6" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E6" s="12">
         <v>45762.0</v>
       </c>
-      <c r="F6" s="8" t="s">
+      <c r="F6" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G6" s="8">
+      <c r="G6" s="10">
         <v>12.0</v>
       </c>
-      <c r="H6" s="8">
+      <c r="H6" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I6" s="8">
+      <c r="I6" s="10">
         <v>2048.0</v>
       </c>
       <c r="J6" s="14">
@@ -8225,7 +8225,7 @@
       <c r="K6" s="14">
         <v>750000.0</v>
       </c>
-      <c r="L6" s="8">
+      <c r="L6" s="10">
         <v>0.0</v>
       </c>
       <c r="AB6" s="2"/>
@@ -8237,32 +8237,32 @@
       <c r="AH6" s="2"/>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="B7" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="C7" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="D7" s="8" t="s">
+      <c r="A7" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="D7" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E7" s="12">
         <v>45763.0</v>
       </c>
-      <c r="F7" s="8" t="s">
+      <c r="F7" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G7" s="8">
+      <c r="G7" s="10">
         <v>12.0</v>
       </c>
-      <c r="H7" s="8">
+      <c r="H7" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I7" s="8" t="s">
-        <v>44</v>
+      <c r="I7" s="10" t="s">
+        <v>39</v>
       </c>
       <c r="J7" s="14">
         <v>949835.78</v>
@@ -8270,7 +8270,7 @@
       <c r="K7" s="14">
         <v>949835.78</v>
       </c>
-      <c r="L7" s="8">
+      <c r="L7" s="10">
         <v>0.0</v>
       </c>
       <c r="AB7" s="2"/>
@@ -8282,31 +8282,31 @@
       <c r="AH7" s="2"/>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="s">
+      <c r="A8" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="B8" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="C8" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="B8" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="C8" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="D8" s="8" t="s">
+      <c r="D8" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E8" s="12">
         <v>45763.0</v>
       </c>
-      <c r="F8" s="8" t="s">
+      <c r="F8" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G8" s="8">
+      <c r="G8" s="10">
         <v>12.0</v>
       </c>
-      <c r="H8" s="8">
+      <c r="H8" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I8" s="8" t="s">
+      <c r="I8" s="10" t="s">
         <v>48</v>
       </c>
       <c r="J8" s="14">
@@ -8315,10 +8315,10 @@
       <c r="K8" s="14">
         <v>524584.95</v>
       </c>
-      <c r="L8" s="8">
+      <c r="L8" s="10">
         <v>0.0</v>
       </c>
-      <c r="O8" s="29"/>
+      <c r="O8" s="23"/>
       <c r="AB8" s="2"/>
       <c r="AC8" s="2"/>
       <c r="AD8" s="2"/>
@@ -8328,32 +8328,32 @@
       <c r="AH8" s="2"/>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="B9" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="C9" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="D9" s="8" t="s">
+      <c r="A9" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="C9" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="D9" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E9" s="12">
         <v>45792.0</v>
       </c>
-      <c r="F9" s="8" t="s">
+      <c r="F9" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G9" s="8">
+      <c r="G9" s="10">
         <v>12.0</v>
       </c>
-      <c r="H9" s="8">
+      <c r="H9" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I9" s="8" t="s">
-        <v>60</v>
+      <c r="I9" s="10" t="s">
+        <v>52</v>
       </c>
       <c r="J9" s="14">
         <v>211614.23</v>
@@ -8361,7 +8361,7 @@
       <c r="K9" s="14">
         <v>211614.23</v>
       </c>
-      <c r="L9" s="8">
+      <c r="L9" s="10">
         <v>0.0</v>
       </c>
       <c r="AB9" s="2"/>
@@ -8373,31 +8373,31 @@
       <c r="AH9" s="2"/>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="s">
-        <v>65</v>
-      </c>
-      <c r="B10" s="8" t="s">
+      <c r="A10" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="B10" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="C10" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="D10" s="8" t="s">
+      <c r="C10" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="D10" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E10" s="12">
         <v>45825.0</v>
       </c>
-      <c r="F10" s="8" t="s">
+      <c r="F10" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G10" s="8">
+      <c r="G10" s="10">
         <v>12.0</v>
       </c>
-      <c r="H10" s="8">
+      <c r="H10" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I10" s="8">
+      <c r="I10" s="10">
         <v>2048.0</v>
       </c>
       <c r="J10" s="14">
@@ -8418,31 +8418,31 @@
       <c r="AH10" s="2"/>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="s">
+      <c r="A11" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="C11" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="B11" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="C11" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="D11" s="8" t="s">
+      <c r="D11" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E11" s="12">
         <v>45825.0</v>
       </c>
-      <c r="F11" s="8" t="s">
+      <c r="F11" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G11" s="8">
+      <c r="G11" s="10">
         <v>12.0</v>
       </c>
-      <c r="H11" s="8">
+      <c r="H11" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I11" s="8">
+      <c r="I11" s="10">
         <v>2048.0</v>
       </c>
       <c r="J11" s="14">
@@ -8451,7 +8451,7 @@
       <c r="K11" s="14">
         <v>618154.38</v>
       </c>
-      <c r="L11" s="8">
+      <c r="L11" s="10">
         <v>0.01</v>
       </c>
       <c r="AB11" s="2"/>
@@ -8463,32 +8463,32 @@
       <c r="AH11" s="2"/>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="s">
+      <c r="A12" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="B12" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="B12" s="8" t="s">
+      <c r="C12" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="C12" s="8" t="s">
-        <v>74</v>
-      </c>
-      <c r="D12" s="8" t="s">
+      <c r="D12" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E12" s="12">
         <v>45832.0</v>
       </c>
-      <c r="F12" s="8" t="s">
+      <c r="F12" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G12" s="8">
+      <c r="G12" s="10">
         <v>12.0</v>
       </c>
-      <c r="H12" s="8">
+      <c r="H12" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I12" s="8" t="s">
-        <v>76</v>
+      <c r="I12" s="10" t="s">
+        <v>74</v>
       </c>
       <c r="J12" s="14">
         <v>1600334.09</v>
@@ -8496,7 +8496,7 @@
       <c r="K12" s="14">
         <v>1600334.09</v>
       </c>
-      <c r="L12" s="8">
+      <c r="L12" s="10">
         <v>0.0</v>
       </c>
       <c r="AB12" s="2"/>
@@ -8508,31 +8508,31 @@
       <c r="AH12" s="2"/>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="s">
+      <c r="A13" s="10" t="s">
         <v>77</v>
       </c>
-      <c r="B13" s="8" t="s">
+      <c r="B13" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="C13" s="8" t="s">
+      <c r="C13" s="10" t="s">
         <v>78</v>
       </c>
-      <c r="D13" s="8" t="s">
+      <c r="D13" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E13" s="12">
         <v>45863.0</v>
       </c>
-      <c r="F13" s="8" t="s">
+      <c r="F13" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G13" s="8">
+      <c r="G13" s="10">
         <v>12.0</v>
       </c>
-      <c r="H13" s="8">
+      <c r="H13" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I13" s="8">
+      <c r="I13" s="10">
         <v>2048.0</v>
       </c>
       <c r="J13" s="14">
@@ -8544,7 +8544,7 @@
       <c r="L13" s="14">
         <v>0.0</v>
       </c>
-      <c r="M13" s="40"/>
+      <c r="M13" s="38"/>
       <c r="AB13" s="2"/>
       <c r="AC13" s="2"/>
       <c r="AD13" s="2"/>
@@ -8554,32 +8554,32 @@
       <c r="AH13" s="2"/>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="s">
+      <c r="A14" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="B14" s="10" t="s">
         <v>80</v>
       </c>
-      <c r="B14" s="8" t="s">
+      <c r="C14" s="10" t="s">
         <v>81</v>
       </c>
-      <c r="C14" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="D14" s="8" t="s">
+      <c r="D14" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E14" s="12">
         <v>45887.0</v>
       </c>
-      <c r="F14" s="8" t="s">
+      <c r="F14" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G14" s="8">
+      <c r="G14" s="10">
         <v>12.0</v>
       </c>
-      <c r="H14" s="8">
+      <c r="H14" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I14" s="8" t="s">
-        <v>60</v>
+      <c r="I14" s="10" t="s">
+        <v>52</v>
       </c>
       <c r="J14" s="14">
         <v>968237.39</v>
@@ -8587,7 +8587,7 @@
       <c r="K14" s="14">
         <v>968237.39</v>
       </c>
-      <c r="L14" s="8">
+      <c r="L14" s="10">
         <v>0.0</v>
       </c>
       <c r="AB14" s="2"/>
@@ -8599,32 +8599,32 @@
       <c r="AH14" s="2"/>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="s">
-        <v>85</v>
-      </c>
-      <c r="B15" s="8" t="s">
-        <v>86</v>
-      </c>
-      <c r="C15" s="8" t="s">
-        <v>87</v>
-      </c>
-      <c r="D15" s="8" t="s">
+      <c r="A15" s="10" t="s">
+        <v>82</v>
+      </c>
+      <c r="B15" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="D15" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E15" s="12">
         <v>45924.0</v>
       </c>
-      <c r="F15" s="8" t="s">
+      <c r="F15" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G15" s="8">
+      <c r="G15" s="10">
         <v>12.0</v>
       </c>
-      <c r="H15" s="8">
+      <c r="H15" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I15" s="8" t="s">
-        <v>44</v>
+      <c r="I15" s="10" t="s">
+        <v>39</v>
       </c>
       <c r="J15" s="14">
         <v>1011677.95</v>
@@ -8632,7 +8632,7 @@
       <c r="K15" s="14">
         <v>1011677.95</v>
       </c>
-      <c r="L15" s="8">
+      <c r="L15" s="10">
         <v>0.0</v>
       </c>
       <c r="AB15" s="2"/>
@@ -8644,31 +8644,31 @@
       <c r="AH15" s="2"/>
     </row>
     <row r="16">
-      <c r="A16" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="B16" s="8" t="s">
+      <c r="A16" s="10" t="s">
+        <v>87</v>
+      </c>
+      <c r="B16" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="C16" s="8" t="s">
-        <v>90</v>
-      </c>
-      <c r="D16" s="8" t="s">
+      <c r="C16" s="10" t="s">
+        <v>88</v>
+      </c>
+      <c r="D16" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E16" s="12">
         <v>45929.0</v>
       </c>
-      <c r="F16" s="8" t="s">
+      <c r="F16" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G16" s="8">
+      <c r="G16" s="10">
         <v>12.0</v>
       </c>
-      <c r="H16" s="8">
+      <c r="H16" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I16" s="8">
+      <c r="I16" s="10">
         <v>2048.0</v>
       </c>
       <c r="J16" s="14">
@@ -8689,37 +8689,37 @@
       <c r="AH16" s="2"/>
     </row>
     <row r="17">
-      <c r="A17" s="8" t="s">
+      <c r="A17" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="B17" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="C17" s="10" t="s">
         <v>93</v>
       </c>
-      <c r="B17" s="8" t="s">
-        <v>94</v>
-      </c>
-      <c r="C17" s="8" t="s">
-        <v>95</v>
-      </c>
-      <c r="D17" s="8" t="s">
+      <c r="D17" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E17" s="12">
         <v>45930.0</v>
       </c>
-      <c r="F17" s="8" t="s">
+      <c r="F17" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G17" s="8">
+      <c r="G17" s="10">
         <v>12.0</v>
       </c>
-      <c r="H17" s="8">
+      <c r="H17" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I17" s="8">
+      <c r="I17" s="10">
         <v>2048.0</v>
       </c>
       <c r="J17" s="14">
         <v>34065.36</v>
       </c>
-      <c r="K17" s="8">
+      <c r="K17" s="10">
         <v>0.0</v>
       </c>
       <c r="L17" s="14">
@@ -8734,32 +8734,32 @@
       <c r="AH17" s="2"/>
     </row>
     <row r="18">
-      <c r="A18" s="8" t="s">
+      <c r="A18" s="10" t="s">
+        <v>95</v>
+      </c>
+      <c r="B18" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="C18" s="10" t="s">
         <v>97</v>
       </c>
-      <c r="B18" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="C18" s="8" t="s">
-        <v>98</v>
-      </c>
-      <c r="D18" s="8" t="s">
+      <c r="D18" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E18" s="12">
         <v>45938.0</v>
       </c>
-      <c r="F18" s="8" t="s">
+      <c r="F18" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G18" s="8">
+      <c r="G18" s="10">
         <v>12.0</v>
       </c>
-      <c r="H18" s="8">
+      <c r="H18" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I18" s="8" t="s">
-        <v>60</v>
+      <c r="I18" s="10" t="s">
+        <v>52</v>
       </c>
       <c r="J18" s="14">
         <v>63746.85</v>
@@ -8767,7 +8767,7 @@
       <c r="K18" s="14">
         <v>63746.85</v>
       </c>
-      <c r="L18" s="8">
+      <c r="L18" s="10">
         <v>0.0</v>
       </c>
       <c r="AB18" s="2"/>
@@ -8779,32 +8779,32 @@
       <c r="AH18" s="2"/>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="s">
+      <c r="A19" s="10" t="s">
+        <v>99</v>
+      </c>
+      <c r="B19" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="C19" s="10" t="s">
         <v>100</v>
       </c>
-      <c r="B19" s="8" t="s">
-        <v>73</v>
-      </c>
-      <c r="C19" s="8" t="s">
-        <v>101</v>
-      </c>
-      <c r="D19" s="8" t="s">
+      <c r="D19" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E19" s="12">
         <v>45938.0</v>
       </c>
-      <c r="F19" s="8" t="s">
+      <c r="F19" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G19" s="8">
+      <c r="G19" s="10">
         <v>12.0</v>
       </c>
-      <c r="H19" s="8">
+      <c r="H19" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I19" s="8" t="s">
-        <v>76</v>
+      <c r="I19" s="10" t="s">
+        <v>74</v>
       </c>
       <c r="J19" s="14">
         <v>947931.1</v>
@@ -8812,7 +8812,7 @@
       <c r="K19" s="14">
         <v>947931.1</v>
       </c>
-      <c r="L19" s="8">
+      <c r="L19" s="10">
         <v>0.0</v>
       </c>
       <c r="AB19" s="2"/>
@@ -8824,31 +8824,31 @@
       <c r="AH19" s="2"/>
     </row>
     <row r="20">
-      <c r="A20" s="8" t="s">
+      <c r="A20" s="10" t="s">
+        <v>102</v>
+      </c>
+      <c r="B20" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C20" s="10" t="s">
         <v>103</v>
       </c>
-      <c r="B20" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="C20" s="8" t="s">
-        <v>104</v>
-      </c>
-      <c r="D20" s="8" t="s">
+      <c r="D20" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E20" s="12">
         <v>45938.0</v>
       </c>
-      <c r="F20" s="8" t="s">
+      <c r="F20" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G20" s="8">
+      <c r="G20" s="10">
         <v>12.0</v>
       </c>
-      <c r="H20" s="8">
+      <c r="H20" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I20" s="8">
+      <c r="I20" s="10">
         <v>2048.0</v>
       </c>
       <c r="J20" s="14">
@@ -8857,7 +8857,7 @@
       <c r="K20" s="14">
         <v>259790.57</v>
       </c>
-      <c r="L20" s="8">
+      <c r="L20" s="10">
         <v>0.0</v>
       </c>
       <c r="AB20" s="2"/>
@@ -8869,31 +8869,31 @@
       <c r="AH20" s="2"/>
     </row>
     <row r="21">
-      <c r="A21" s="8" t="s">
-        <v>107</v>
-      </c>
-      <c r="B21" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="C21" s="8" t="s">
+      <c r="A21" s="10" t="s">
+        <v>106</v>
+      </c>
+      <c r="B21" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="C21" s="10" t="s">
         <v>108</v>
       </c>
-      <c r="D21" s="8" t="s">
+      <c r="D21" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E21" s="12">
         <v>45938.0</v>
       </c>
-      <c r="F21" s="8" t="s">
+      <c r="F21" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G21" s="8">
+      <c r="G21" s="10">
         <v>12.0</v>
       </c>
-      <c r="H21" s="8">
+      <c r="H21" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I21" s="8">
+      <c r="I21" s="10">
         <v>2048.0</v>
       </c>
       <c r="J21" s="14">
@@ -8902,7 +8902,7 @@
       <c r="K21" s="14">
         <v>170479.3</v>
       </c>
-      <c r="L21" s="8">
+      <c r="L21" s="10">
         <v>0.0</v>
       </c>
       <c r="AB21" s="2"/>
@@ -8914,31 +8914,31 @@
       <c r="AH21" s="2"/>
     </row>
     <row r="22">
-      <c r="A22" s="8" t="s">
+      <c r="A22" s="10" t="s">
         <v>111</v>
       </c>
-      <c r="B22" s="8" t="s">
+      <c r="B22" s="10" t="s">
         <v>112</v>
       </c>
-      <c r="C22" s="8" t="s">
+      <c r="C22" s="10" t="s">
         <v>113</v>
       </c>
-      <c r="D22" s="8" t="s">
+      <c r="D22" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E22" s="50">
         <v>45953.0</v>
       </c>
-      <c r="F22" s="8" t="s">
+      <c r="F22" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G22" s="8">
+      <c r="G22" s="10">
         <v>12.0</v>
       </c>
-      <c r="H22" s="8">
+      <c r="H22" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I22" s="8">
+      <c r="I22" s="10">
         <v>2000.0</v>
       </c>
       <c r="J22" s="14">
@@ -8959,31 +8959,31 @@
       <c r="AH22" s="2"/>
     </row>
     <row r="23">
-      <c r="A23" s="8" t="s">
-        <v>115</v>
-      </c>
-      <c r="B23" s="8" t="s">
+      <c r="A23" s="10" t="s">
         <v>116</v>
       </c>
-      <c r="C23" s="8" t="s">
+      <c r="B23" s="10" t="s">
+        <v>117</v>
+      </c>
+      <c r="C23" s="10" t="s">
         <v>118</v>
       </c>
-      <c r="D23" s="8" t="s">
+      <c r="D23" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E23" s="50">
         <v>45953.0</v>
       </c>
-      <c r="F23" s="8" t="s">
+      <c r="F23" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G23" s="8">
+      <c r="G23" s="10">
         <v>12.0</v>
       </c>
-      <c r="H23" s="8">
+      <c r="H23" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I23" s="8" t="s">
+      <c r="I23" s="10" t="s">
         <v>119</v>
       </c>
       <c r="J23" s="14">
@@ -8992,7 +8992,7 @@
       <c r="K23" s="14">
         <v>1000001.64</v>
       </c>
-      <c r="L23" s="8">
+      <c r="L23" s="10">
         <v>0.0</v>
       </c>
       <c r="AB23" s="2"/>
@@ -9004,31 +9004,31 @@
       <c r="AH23" s="2"/>
     </row>
     <row r="24">
-      <c r="A24" s="8" t="s">
-        <v>120</v>
-      </c>
-      <c r="B24" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="C24" s="8" t="s">
+      <c r="A24" s="10" t="s">
+        <v>121</v>
+      </c>
+      <c r="B24" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="C24" s="10" t="s">
         <v>122</v>
       </c>
-      <c r="D24" s="8" t="s">
+      <c r="D24" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E24" s="50">
         <v>45953.0</v>
       </c>
-      <c r="F24" s="8" t="s">
+      <c r="F24" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G24" s="8">
+      <c r="G24" s="10">
         <v>12.0</v>
       </c>
-      <c r="H24" s="8">
+      <c r="H24" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I24" s="8">
+      <c r="I24" s="10">
         <v>2048.0</v>
       </c>
       <c r="J24" s="14">
@@ -9037,7 +9037,7 @@
       <c r="K24" s="14">
         <v>68405.66</v>
       </c>
-      <c r="L24" s="8">
+      <c r="L24" s="10">
         <v>0.0</v>
       </c>
       <c r="AB24" s="2"/>
@@ -9049,31 +9049,31 @@
       <c r="AH24" s="2"/>
     </row>
     <row r="25">
-      <c r="A25" s="8" t="s">
-        <v>125</v>
-      </c>
-      <c r="B25" s="8" t="s">
+      <c r="A25" s="10" t="s">
+        <v>124</v>
+      </c>
+      <c r="B25" s="10" t="s">
         <v>126</v>
       </c>
-      <c r="C25" s="8" t="s">
+      <c r="C25" s="10" t="s">
         <v>127</v>
       </c>
-      <c r="D25" s="8" t="s">
+      <c r="D25" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E25" s="50">
         <v>45975.0</v>
       </c>
-      <c r="F25" s="8" t="s">
+      <c r="F25" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G25" s="8">
+      <c r="G25" s="10">
         <v>12.0</v>
       </c>
-      <c r="H25" s="8">
+      <c r="H25" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I25" s="8" t="s">
+      <c r="I25" s="10" t="s">
         <v>119</v>
       </c>
       <c r="J25" s="14">
@@ -9082,7 +9082,7 @@
       <c r="K25" s="14">
         <v>1157673.06</v>
       </c>
-      <c r="L25" s="8">
+      <c r="L25" s="10">
         <v>0.0</v>
       </c>
       <c r="AB25" s="2"/>
@@ -9094,31 +9094,31 @@
       <c r="AH25" s="2"/>
     </row>
     <row r="26">
-      <c r="A26" s="8" t="s">
+      <c r="A26" s="10" t="s">
+        <v>129</v>
+      </c>
+      <c r="B26" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C26" s="10" t="s">
         <v>130</v>
       </c>
-      <c r="B26" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="C26" s="8" t="s">
-        <v>131</v>
-      </c>
-      <c r="D26" s="8" t="s">
+      <c r="D26" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E26" s="50">
         <v>45989.0</v>
       </c>
-      <c r="F26" s="8" t="s">
+      <c r="F26" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G26" s="8">
+      <c r="G26" s="10">
         <v>12.0</v>
       </c>
-      <c r="H26" s="8">
+      <c r="H26" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I26" s="8">
+      <c r="I26" s="10">
         <v>2048.0</v>
       </c>
       <c r="J26" s="14">
@@ -9127,7 +9127,7 @@
       <c r="K26" s="14">
         <v>34065.36</v>
       </c>
-      <c r="L26" s="8">
+      <c r="L26" s="10">
         <v>0.0</v>
       </c>
       <c r="AB26" s="2"/>
@@ -9139,31 +9139,31 @@
       <c r="AH26" s="2"/>
     </row>
     <row r="27">
-      <c r="A27" s="8" t="s">
+      <c r="A27" s="10" t="s">
+        <v>132</v>
+      </c>
+      <c r="B27" s="10" t="s">
+        <v>133</v>
+      </c>
+      <c r="C27" s="10" t="s">
         <v>134</v>
       </c>
-      <c r="B27" s="8" t="s">
-        <v>135</v>
-      </c>
-      <c r="C27" s="8" t="s">
-        <v>136</v>
-      </c>
-      <c r="D27" s="8" t="s">
+      <c r="D27" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E27" s="12">
         <v>46104.0</v>
       </c>
-      <c r="F27" s="8" t="s">
+      <c r="F27" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G27" s="8">
+      <c r="G27" s="10">
         <v>12.0</v>
       </c>
-      <c r="H27" s="8">
+      <c r="H27" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I27" s="8">
+      <c r="I27" s="10">
         <v>2048.0</v>
       </c>
       <c r="J27" s="14">
@@ -9184,31 +9184,31 @@
       <c r="AH27" s="2"/>
     </row>
     <row r="28">
-      <c r="A28" s="8" t="s">
+      <c r="A28" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="B28" s="10" t="s">
+        <v>138</v>
+      </c>
+      <c r="C28" s="10" t="s">
         <v>139</v>
       </c>
-      <c r="B28" s="8" t="s">
-        <v>140</v>
-      </c>
-      <c r="C28" s="8" t="s">
-        <v>141</v>
-      </c>
-      <c r="D28" s="8" t="s">
+      <c r="D28" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E28" s="12">
         <v>46120.0</v>
       </c>
-      <c r="F28" s="8" t="s">
+      <c r="F28" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G28" s="8">
+      <c r="G28" s="10">
         <v>12.0</v>
       </c>
-      <c r="H28" s="8">
+      <c r="H28" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I28" s="8" t="s">
+      <c r="I28" s="10" t="s">
         <v>48</v>
       </c>
       <c r="J28" s="14">
@@ -9229,37 +9229,37 @@
       <c r="AH28" s="2"/>
     </row>
     <row r="29">
-      <c r="A29" s="8" t="s">
-        <v>143</v>
-      </c>
-      <c r="B29" s="8" t="s">
+      <c r="A29" s="10" t="s">
+        <v>141</v>
+      </c>
+      <c r="B29" s="10" t="s">
+        <v>142</v>
+      </c>
+      <c r="C29" s="10" t="s">
         <v>144</v>
       </c>
-      <c r="C29" s="8" t="s">
-        <v>146</v>
-      </c>
-      <c r="D29" s="8" t="s">
+      <c r="D29" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E29" s="12">
         <v>46196.0</v>
       </c>
-      <c r="F29" s="8" t="s">
+      <c r="F29" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G29" s="8">
+      <c r="G29" s="10">
         <v>12.0</v>
       </c>
-      <c r="H29" s="8">
+      <c r="H29" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I29" s="8">
+      <c r="I29" s="10">
         <v>2048.0</v>
       </c>
       <c r="J29" s="14">
         <v>1496713.48</v>
       </c>
-      <c r="K29" s="8">
+      <c r="K29" s="10">
         <v>0.0</v>
       </c>
       <c r="L29" s="14">
@@ -9274,37 +9274,37 @@
       <c r="AH29" s="2"/>
     </row>
     <row r="30">
-      <c r="A30" s="8" t="s">
-        <v>149</v>
-      </c>
-      <c r="B30" s="8" t="s">
-        <v>150</v>
-      </c>
-      <c r="C30" s="8" t="s">
-        <v>151</v>
-      </c>
-      <c r="D30" s="8" t="s">
+      <c r="A30" s="10" t="s">
+        <v>146</v>
+      </c>
+      <c r="B30" s="10" t="s">
+        <v>147</v>
+      </c>
+      <c r="C30" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="D30" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E30" s="12">
         <v>46205.0</v>
       </c>
-      <c r="F30" s="8" t="s">
+      <c r="F30" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G30" s="8">
+      <c r="G30" s="10">
         <v>12.0</v>
       </c>
-      <c r="H30" s="8">
+      <c r="H30" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I30" s="8" t="s">
-        <v>44</v>
+      <c r="I30" s="10" t="s">
+        <v>39</v>
       </c>
       <c r="J30" s="14">
         <v>624166.14</v>
       </c>
-      <c r="K30" s="8">
+      <c r="K30" s="10">
         <v>0.0</v>
       </c>
       <c r="L30" s="14">
@@ -9319,37 +9319,37 @@
       <c r="AH30" s="2"/>
     </row>
     <row r="31">
-      <c r="A31" s="8" t="s">
-        <v>153</v>
-      </c>
-      <c r="B31" s="8" t="s">
-        <v>154</v>
-      </c>
-      <c r="C31" s="8" t="s">
-        <v>155</v>
-      </c>
-      <c r="D31" s="8" t="s">
+      <c r="A31" s="10" t="s">
+        <v>149</v>
+      </c>
+      <c r="B31" s="10" t="s">
+        <v>150</v>
+      </c>
+      <c r="C31" s="10" t="s">
+        <v>151</v>
+      </c>
+      <c r="D31" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E31" s="12">
         <v>46205.0</v>
       </c>
-      <c r="F31" s="8" t="s">
+      <c r="F31" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G31" s="8">
+      <c r="G31" s="10">
         <v>12.0</v>
       </c>
-      <c r="H31" s="8">
+      <c r="H31" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I31" s="8" t="s">
+      <c r="I31" s="10" t="s">
         <v>119</v>
       </c>
       <c r="J31" s="14">
         <v>18462.36</v>
       </c>
-      <c r="K31" s="8">
+      <c r="K31" s="10">
         <v>0.0</v>
       </c>
       <c r="L31" s="14">
@@ -9364,37 +9364,37 @@
       <c r="AH31" s="2"/>
     </row>
     <row r="32">
-      <c r="A32" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="B32" s="8" t="s">
+      <c r="A32" s="10" t="s">
+        <v>153</v>
+      </c>
+      <c r="B32" s="10" t="s">
+        <v>150</v>
+      </c>
+      <c r="C32" s="14" t="s">
         <v>154</v>
       </c>
-      <c r="C32" s="14" t="s">
-        <v>158</v>
-      </c>
-      <c r="D32" s="8" t="s">
+      <c r="D32" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E32" s="12">
         <v>46213.0</v>
       </c>
-      <c r="F32" s="8" t="s">
+      <c r="F32" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G32" s="8">
+      <c r="G32" s="10">
         <v>12.0</v>
       </c>
-      <c r="H32" s="8">
+      <c r="H32" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I32" s="8" t="s">
+      <c r="I32" s="10" t="s">
         <v>119</v>
       </c>
       <c r="J32" s="14">
         <v>1530656.62</v>
       </c>
-      <c r="K32" s="8">
+      <c r="K32" s="10">
         <v>0.0</v>
       </c>
       <c r="L32" s="14">
@@ -9409,37 +9409,37 @@
       <c r="AH32" s="2"/>
     </row>
     <row r="33">
-      <c r="A33" s="8" t="s">
-        <v>161</v>
-      </c>
-      <c r="B33" s="8" t="s">
-        <v>144</v>
+      <c r="A33" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="B33" s="10" t="s">
+        <v>142</v>
       </c>
       <c r="C33" s="14" t="s">
-        <v>162</v>
-      </c>
-      <c r="D33" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="D33" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E33" s="12">
         <v>46227.0</v>
       </c>
-      <c r="F33" s="8" t="s">
+      <c r="F33" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G33" s="8">
+      <c r="G33" s="10">
         <v>12.0</v>
       </c>
-      <c r="H33" s="8">
+      <c r="H33" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I33" s="8">
+      <c r="I33" s="10">
         <v>2048.0</v>
       </c>
       <c r="J33" s="14">
         <v>173846.38</v>
       </c>
-      <c r="K33" s="8">
+      <c r="K33" s="10">
         <v>0.0</v>
       </c>
       <c r="L33" s="14">
@@ -9454,37 +9454,37 @@
       <c r="AH33" s="2"/>
     </row>
     <row r="34">
-      <c r="A34" s="8" t="s">
-        <v>164</v>
-      </c>
-      <c r="B34" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="C34" s="8" t="s">
-        <v>166</v>
-      </c>
-      <c r="D34" s="8" t="s">
+      <c r="A34" s="10" t="s">
+        <v>160</v>
+      </c>
+      <c r="B34" s="10" t="s">
+        <v>161</v>
+      </c>
+      <c r="C34" s="10" t="s">
+        <v>162</v>
+      </c>
+      <c r="D34" s="10" t="s">
         <v>4</v>
       </c>
       <c r="E34" s="12">
         <v>46240.0</v>
       </c>
-      <c r="F34" s="8" t="s">
+      <c r="F34" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G34" s="8">
+      <c r="G34" s="10">
         <v>12.0</v>
       </c>
-      <c r="H34" s="8">
+      <c r="H34" s="10">
         <v>339039.0</v>
       </c>
-      <c r="I34" s="8" t="s">
-        <v>168</v>
+      <c r="I34" s="10" t="s">
+        <v>164</v>
       </c>
       <c r="J34" s="14">
         <v>236343.68</v>
       </c>
-      <c r="K34" s="8">
+      <c r="K34" s="10">
         <v>0.0</v>
       </c>
       <c r="L34" s="14">

</xml_diff>

<commit_message>
Atualização automática: pagamentos (03/09/2026 13:42)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/01_Bases_Originais/005_CELOG_2025/005_CELOG-PAMALS_2025 online.xlsx
+++ b/Contrato 005/Dashboard/01_Bases_Originais/005_CELOG_2025/005_CELOG-PAMALS_2025 online.xlsx
@@ -81,42 +81,42 @@
     <t>Ação</t>
   </si>
   <si>
+    <t>PAG</t>
+  </si>
+  <si>
+    <t>Moeda</t>
+  </si>
+  <si>
+    <t>Valor Total do Contrato</t>
+  </si>
+  <si>
+    <t>Valor a Empenhar</t>
+  </si>
+  <si>
+    <t>Valor Empenhado</t>
+  </si>
+  <si>
+    <t>Valor Liquidado</t>
+  </si>
+  <si>
     <t>2025NE000369</t>
   </si>
   <si>
-    <t>PAG</t>
+    <t>Saldo (Valor a Faturar)</t>
   </si>
   <si>
     <t>C25516</t>
   </si>
   <si>
-    <t>Moeda</t>
+    <t>Fornecedor</t>
+  </si>
+  <si>
+    <t>Tipo Despesa /Receita</t>
   </si>
   <si>
     <t>25E0387</t>
   </si>
   <si>
-    <t>Valor Total do Contrato</t>
-  </si>
-  <si>
-    <t>Valor a Empenhar</t>
-  </si>
-  <si>
-    <t>Valor Empenhado</t>
-  </si>
-  <si>
-    <t>Valor Liquidado</t>
-  </si>
-  <si>
-    <t>Saldo (Valor a Faturar)</t>
-  </si>
-  <si>
-    <t>Fornecedor</t>
-  </si>
-  <si>
-    <t>Tipo Despesa /Receita</t>
-  </si>
-  <si>
     <t>Abrir</t>
   </si>
   <si>
@@ -126,15 +126,15 @@
     <t>005/CELOG-PAMALS/2025</t>
   </si>
   <si>
+    <t>CELOG</t>
+  </si>
+  <si>
+    <t>PAMALS</t>
+  </si>
+  <si>
     <t>2025NE000371</t>
   </si>
   <si>
-    <t>CELOG</t>
-  </si>
-  <si>
-    <t>PAMALS</t>
-  </si>
-  <si>
     <t>25E0389</t>
   </si>
   <si>
@@ -150,12 +150,12 @@
     <t>R$</t>
   </si>
   <si>
+    <t>VEE ONE-MANUTENCAO E SERVICOS TECNICOS LTDA</t>
+  </si>
+  <si>
     <t>2025NE000413</t>
   </si>
   <si>
-    <t>VEE ONE-MANUTENCAO E SERVICOS TECNICOS LTDA</t>
-  </si>
-  <si>
     <t>C25501</t>
   </si>
   <si>
@@ -180,57 +180,57 @@
     <t>Módulo</t>
   </si>
   <si>
+    <t>Referência</t>
+  </si>
+  <si>
+    <t>Nº recibo</t>
+  </si>
+  <si>
+    <t>Nº</t>
+  </si>
+  <si>
     <t>2025NE000559</t>
   </si>
   <si>
+    <t>Data</t>
+  </si>
+  <si>
     <t>C25545</t>
   </si>
   <si>
-    <t>Referência</t>
-  </si>
-  <si>
     <t>25E0524</t>
   </si>
   <si>
-    <t>Nº recibo</t>
-  </si>
-  <si>
-    <t>Nº</t>
+    <t>Empenho</t>
+  </si>
+  <si>
+    <t>Observações</t>
+  </si>
+  <si>
+    <t>Vencimento</t>
+  </si>
+  <si>
+    <t>Valor das Nfs</t>
   </si>
   <si>
     <t>20X7</t>
   </si>
   <si>
-    <t>Data</t>
-  </si>
-  <si>
-    <t>Empenho</t>
-  </si>
-  <si>
-    <t>Observações</t>
-  </si>
-  <si>
-    <t>Vencimento</t>
+    <t>Ordem de Pagamento</t>
+  </si>
+  <si>
+    <t>Faturado</t>
+  </si>
+  <si>
+    <t>Pendente</t>
   </si>
   <si>
     <t>2025NE000770</t>
   </si>
   <si>
-    <t>Valor das Nfs</t>
-  </si>
-  <si>
     <t>25E0731</t>
   </si>
   <si>
-    <t>Ordem de Pagamento</t>
-  </si>
-  <si>
-    <t>Faturado</t>
-  </si>
-  <si>
-    <t>Pendente</t>
-  </si>
-  <si>
     <t>2025NE000774</t>
   </si>
   <si>
@@ -255,12 +255,12 @@
     <t>219C</t>
   </si>
   <si>
+    <t>2025NE001065</t>
+  </si>
+  <si>
     <t xml:space="preserve">2025NE000369 </t>
   </si>
   <si>
-    <t>2025NE001065</t>
-  </si>
-  <si>
     <t>25E0999</t>
   </si>
   <si>
@@ -288,31 +288,49 @@
     <t>2025NE001627</t>
   </si>
   <si>
+    <t>25E1475</t>
+  </si>
+  <si>
+    <t>2025NE001629</t>
+  </si>
+  <si>
+    <t>C25820</t>
+  </si>
+  <si>
+    <t>25E1477</t>
+  </si>
+  <si>
     <t>MAR/25</t>
   </si>
   <si>
-    <t>25E1475</t>
+    <t>2025NE001687</t>
+  </si>
+  <si>
+    <t>25E1535</t>
   </si>
   <si>
     <t>2025NE000367, 2025NE000369, 2025NE000371, 2025NE000413</t>
   </si>
   <si>
-    <t>2025NE001629</t>
-  </si>
-  <si>
-    <t>C25820</t>
-  </si>
-  <si>
-    <t>25E1477</t>
-  </si>
-  <si>
     <t>2025NP001979</t>
   </si>
   <si>
-    <t>2025NE001687</t>
-  </si>
-  <si>
-    <t>25E1535</t>
+    <t>2025NE001688</t>
+  </si>
+  <si>
+    <t>25E1536</t>
+  </si>
+  <si>
+    <t>2025NE001689</t>
+  </si>
+  <si>
+    <t>25E1537</t>
+  </si>
+  <si>
+    <t>2025NE001690</t>
+  </si>
+  <si>
+    <t>25E1538</t>
   </si>
   <si>
     <t>ABR/25</t>
@@ -321,55 +339,58 @@
     <t>2025NE000413, 2025NE000414, 2025NE000559</t>
   </si>
   <si>
-    <t>2025NE001688</t>
-  </si>
-  <si>
-    <t>25E1536</t>
+    <t>2025NE001823</t>
+  </si>
+  <si>
+    <t>C25865</t>
+  </si>
+  <si>
+    <t>25E1666</t>
   </si>
   <si>
     <t>2025NP002341</t>
   </si>
   <si>
-    <t>2025NE001689</t>
-  </si>
-  <si>
-    <t>25E1537</t>
-  </si>
-  <si>
     <t>MAI/25</t>
   </si>
   <si>
-    <t>2025NE001690</t>
-  </si>
-  <si>
-    <t>25E1538</t>
-  </si>
-  <si>
-    <t>2025NE001823</t>
-  </si>
-  <si>
-    <t>C25865</t>
-  </si>
-  <si>
-    <t>25E1666</t>
+    <t>2025NE001828</t>
+  </si>
+  <si>
+    <t>C25869</t>
+  </si>
+  <si>
+    <t>25E1667</t>
+  </si>
+  <si>
+    <t>20YJ</t>
+  </si>
+  <si>
+    <t>2025NE001830</t>
+  </si>
+  <si>
+    <t>25E1669</t>
   </si>
   <si>
     <t>2025NP002884</t>
   </si>
   <si>
-    <t>2025NE001828</t>
-  </si>
-  <si>
-    <t>C25869</t>
-  </si>
-  <si>
-    <t>25E1667</t>
+    <t>2025NE002200</t>
+  </si>
+  <si>
+    <t>C25863</t>
+  </si>
+  <si>
+    <t>25E2021</t>
   </si>
   <si>
     <t>JUN/25</t>
   </si>
   <si>
-    <t>20YJ</t>
+    <t>2025NE002237</t>
+  </si>
+  <si>
+    <t>25E2058</t>
   </si>
   <si>
     <t>2025NE000005,
@@ -378,134 +399,116 @@
 2025NE000774</t>
   </si>
   <si>
-    <t>2025NE001830</t>
-  </si>
-  <si>
-    <t>25E1669</t>
-  </si>
-  <si>
     <t>2025NP400522</t>
   </si>
   <si>
-    <t>2025NE002200</t>
-  </si>
-  <si>
-    <t>C25863</t>
-  </si>
-  <si>
-    <t>25E2021</t>
+    <t>2026NE000330</t>
+  </si>
+  <si>
+    <t>C26163</t>
+  </si>
+  <si>
+    <t>26E0320</t>
   </si>
   <si>
     <t>JUL/25</t>
   </si>
   <si>
-    <t>2025NE002237</t>
-  </si>
-  <si>
     <t>2025NE000843, 2025NE001200</t>
   </si>
   <si>
-    <t>25E2058</t>
+    <t>2026NE000388</t>
+  </si>
+  <si>
+    <t>C26193</t>
+  </si>
+  <si>
+    <t>26E0375</t>
   </si>
   <si>
     <t>2025NP003724</t>
   </si>
   <si>
-    <t>2026NE000330</t>
-  </si>
-  <si>
-    <t>C26163</t>
-  </si>
-  <si>
-    <t>26E0320</t>
-  </si>
-  <si>
     <t>AGO/25</t>
   </si>
   <si>
-    <t>2026NE000388</t>
-  </si>
-  <si>
-    <t>C26193</t>
-  </si>
-  <si>
-    <t>26E0375</t>
+    <t>2026NE000748</t>
+  </si>
+  <si>
+    <t>C26312</t>
+  </si>
+  <si>
+    <t>26E0709</t>
   </si>
   <si>
     <t>2025NP004558</t>
   </si>
   <si>
+    <t>2026NE000816</t>
+  </si>
+  <si>
+    <t>C26324</t>
+  </si>
+  <si>
+    <t>26E0776</t>
+  </si>
+  <si>
     <t>SET/25</t>
-  </si>
-  <si>
-    <t>2026NE000748</t>
-  </si>
-  <si>
-    <t>C26312</t>
-  </si>
-  <si>
-    <t>26E0709</t>
   </si>
   <si>
     <t>2025NE001688 
 2025NE001828</t>
   </si>
   <si>
+    <t>2026NE000817</t>
+  </si>
+  <si>
+    <t>C26326</t>
+  </si>
+  <si>
+    <t>26E0777</t>
+  </si>
+  <si>
     <t>2025NP004897</t>
   </si>
   <si>
-    <t>2026NE000816</t>
-  </si>
-  <si>
-    <t>C26324</t>
-  </si>
-  <si>
     <t>OUT/25</t>
   </si>
   <si>
-    <t>26E0776</t>
-  </si>
-  <si>
     <t>2025NE001688, 2025NE001828, 2025NE002200</t>
   </si>
   <si>
     <t>2025NP004932</t>
   </si>
   <si>
-    <t>2026NE000817</t>
-  </si>
-  <si>
-    <t>C26326</t>
-  </si>
-  <si>
-    <t>26E0777</t>
+    <t>2026NE000842</t>
+  </si>
+  <si>
+    <t>26E0803</t>
   </si>
   <si>
     <t>NOV/25</t>
   </si>
   <si>
-    <t>2026NE000842</t>
-  </si>
-  <si>
-    <t>26E0803</t>
-  </si>
-  <si>
     <t>2025NE001687, 2025NE001689, 2025NE001690, 2025NE001823, 2025NE001830, 2025NE002237</t>
   </si>
   <si>
+    <t>2026NP400440</t>
+  </si>
+  <si>
     <t>2026NE000944</t>
   </si>
   <si>
-    <t>2026NP400440</t>
-  </si>
-  <si>
     <t>26E0906</t>
   </si>
   <si>
+    <t>DEZ/25</t>
+  </si>
+  <si>
     <t>2026NE001015</t>
   </si>
   <si>
-    <t>DEZ/25</t>
+    <t>2025NE001065, 2025NE002200</t>
   </si>
   <si>
     <t>C26363</t>
@@ -514,13 +517,10 @@
     <t>26E0959</t>
   </si>
   <si>
-    <t>2025NE001065, 2025NE002200</t>
+    <t>2026NP400412</t>
   </si>
   <si>
     <t>20XV</t>
-  </si>
-  <si>
-    <t>2026NP400412</t>
   </si>
   <si>
     <t>JAN/26</t>
@@ -695,8 +695,8 @@
     <numFmt numFmtId="166" formatCode="dd/MM/yyyy"/>
     <numFmt numFmtId="167" formatCode="R$ #,##0.00"/>
     <numFmt numFmtId="168" formatCode="[$R$-416]\ #,##0.00;[RED]\-[$R$-416]\ #,##0.00"/>
-    <numFmt numFmtId="169" formatCode="MM/DD/YY"/>
-    <numFmt numFmtId="170" formatCode="d/m/yyyy"/>
+    <numFmt numFmtId="169" formatCode="d/m/yyyy"/>
+    <numFmt numFmtId="170" formatCode="MM/DD/YY"/>
     <numFmt numFmtId="171" formatCode="[$R$ -416]#,##0.00"/>
     <numFmt numFmtId="172" formatCode="_([$R$ -416]* #,##0.00_);_([$R$ -416]* \(#,##0.00\);_([$R$ -416]* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
@@ -740,13 +740,13 @@
       <b/>
       <sz val="10.0"/>
       <color theme="1"/>
-      <name val="Century Gothic"/>
+      <name val="Arial"/>
     </font>
     <font>
       <b/>
       <sz val="10.0"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Century Gothic"/>
     </font>
     <font>
       <sz val="10.0"/>
@@ -901,17 +901,17 @@
     <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
     <xf borderId="0" fillId="5" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
+    <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment vertical="center"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="11" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment vertical="center"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="center"/>
@@ -919,10 +919,10 @@
     <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="4" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="4" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="2" numFmtId="0" xfId="0" applyFill="1" applyFont="1"/>
@@ -962,22 +962,22 @@
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="6" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="7" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="2" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="7" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="6" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -996,17 +996,20 @@
     <xf borderId="1" fillId="5" fontId="9" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="8" fontId="7" numFmtId="168" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="8" fontId="6" numFmtId="168" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="3" fillId="0" fontId="10" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="1" fillId="8" fontId="9" numFmtId="168" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="169" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
     <xf borderId="1" fillId="0" fontId="8" numFmtId="166" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="8" numFmtId="169" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="8" numFmtId="170" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="7" fontId="9" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
@@ -1015,13 +1018,10 @@
     <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="170" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
     <xf borderId="1" fillId="8" fontId="9" numFmtId="168" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="7" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="6" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -1040,7 +1040,7 @@
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="4" fillId="0" fontId="10" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="1" fillId="0" fontId="7" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="6" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="5" fontId="9" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
@@ -1049,7 +1049,7 @@
     <xf borderId="1" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="7" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="6" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="5" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -1441,10 +1441,10 @@
     </row>
     <row r="2" ht="59.25" customHeight="1">
       <c r="A2" s="6"/>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="V2" s="10"/>
+      <c r="V2" s="9"/>
       <c r="W2" s="11"/>
       <c r="X2" s="11"/>
       <c r="Y2" s="11"/>
@@ -1457,25 +1457,25 @@
     <row r="3" ht="12.75" customHeight="1">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
-      <c r="C3" s="14"/>
-      <c r="D3" s="14"/>
-      <c r="E3" s="14"/>
-      <c r="F3" s="14"/>
-      <c r="G3" s="14"/>
-      <c r="H3" s="14"/>
-      <c r="I3" s="14"/>
-      <c r="J3" s="14"/>
-      <c r="K3" s="14"/>
-      <c r="L3" s="14"/>
-      <c r="M3" s="14"/>
-      <c r="N3" s="14"/>
-      <c r="O3" s="14"/>
-      <c r="P3" s="14"/>
-      <c r="Q3" s="14"/>
-      <c r="R3" s="14"/>
-      <c r="S3" s="14"/>
-      <c r="T3" s="14"/>
-      <c r="U3" s="14"/>
+      <c r="C3" s="13"/>
+      <c r="D3" s="13"/>
+      <c r="E3" s="13"/>
+      <c r="F3" s="13"/>
+      <c r="G3" s="13"/>
+      <c r="H3" s="13"/>
+      <c r="I3" s="13"/>
+      <c r="J3" s="13"/>
+      <c r="K3" s="13"/>
+      <c r="L3" s="13"/>
+      <c r="M3" s="13"/>
+      <c r="N3" s="13"/>
+      <c r="O3" s="13"/>
+      <c r="P3" s="13"/>
+      <c r="Q3" s="13"/>
+      <c r="R3" s="13"/>
+      <c r="S3" s="13"/>
+      <c r="T3" s="13"/>
+      <c r="U3" s="13"/>
       <c r="V3" s="4"/>
     </row>
     <row r="4" ht="12.75" customHeight="1">
@@ -1506,31 +1506,31 @@
         <v>16</v>
       </c>
       <c r="K4" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="L4" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="L4" s="16" t="s">
+      <c r="M4" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="N4" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="M4" s="17" t="s">
+      <c r="O4" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="P4" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="N4" s="17" t="s">
-        <v>23</v>
-      </c>
-      <c r="O4" s="17" t="s">
+      <c r="Q4" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="P4" s="17" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q4" s="17" t="s">
+      <c r="R4" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="R4" s="16" t="s">
+      <c r="S4" s="16" t="s">
         <v>27</v>
-      </c>
-      <c r="S4" s="16" t="s">
-        <v>28</v>
       </c>
       <c r="T4" s="16" t="s">
         <v>29</v>
@@ -1548,13 +1548,13 @@
         <v>31</v>
       </c>
       <c r="E5" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="F5" s="19" t="s">
         <v>33</v>
       </c>
-      <c r="F5" s="19" t="s">
-        <v>34</v>
-      </c>
       <c r="G5" s="19" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H5" s="20">
         <v>1564.0</v>
@@ -1590,7 +1590,7 @@
         <v>1.085943044E7</v>
       </c>
       <c r="S5" s="19" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="V5" s="4"/>
     </row>
@@ -1622,43 +1622,43 @@
     <row r="8" ht="12.75" customHeight="1">
       <c r="A8" s="23"/>
       <c r="B8" s="23"/>
-      <c r="C8" s="29" t="s">
+      <c r="C8" s="28" t="s">
         <v>49</v>
       </c>
-      <c r="D8" s="29" t="s">
+      <c r="D8" s="28" t="s">
+        <v>50</v>
+      </c>
+      <c r="E8" s="30" t="s">
+        <v>51</v>
+      </c>
+      <c r="F8" s="28" t="s">
         <v>52</v>
       </c>
-      <c r="E8" s="30" t="s">
+      <c r="G8" s="28" t="s">
         <v>54</v>
       </c>
-      <c r="F8" s="29" t="s">
-        <v>55</v>
-      </c>
-      <c r="G8" s="29" t="s">
+      <c r="H8" s="28" t="s">
         <v>57</v>
       </c>
-      <c r="H8" s="29" t="s">
+      <c r="I8" s="30" t="s">
         <v>58</v>
       </c>
-      <c r="I8" s="30" t="s">
+      <c r="J8" s="28" t="s">
         <v>59</v>
       </c>
-      <c r="J8" s="29" t="s">
+      <c r="K8" s="28" t="s">
         <v>60</v>
       </c>
-      <c r="K8" s="29" t="s">
+      <c r="L8" s="31" t="s">
         <v>62</v>
       </c>
-      <c r="L8" s="31" t="s">
+      <c r="M8" s="30" t="s">
+        <v>63</v>
+      </c>
+      <c r="N8" s="28" t="s">
         <v>64</v>
       </c>
-      <c r="M8" s="30" t="s">
-        <v>65</v>
-      </c>
-      <c r="N8" s="29" t="s">
-        <v>66</v>
-      </c>
-      <c r="O8" s="29"/>
+      <c r="O8" s="28"/>
       <c r="P8" s="27"/>
       <c r="V8" s="4"/>
     </row>
@@ -1681,7 +1681,7 @@
         <v>45740.0</v>
       </c>
       <c r="H9" s="35" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="I9" s="36"/>
       <c r="J9" s="36">
@@ -1707,7 +1707,7 @@
       <c r="B10" s="23"/>
       <c r="C10" s="41"/>
       <c r="D10" s="33" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="E10" s="34" t="s">
         <v>70</v>
@@ -1719,7 +1719,7 @@
         <v>45775.0</v>
       </c>
       <c r="H10" s="35" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="I10" s="36"/>
       <c r="J10" s="36">
@@ -1729,7 +1729,7 @@
         <v>1110378.24</v>
       </c>
       <c r="L10" s="35" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="M10" s="39">
         <f t="shared" si="1"/>
@@ -1745,7 +1745,7 @@
       <c r="B11" s="23"/>
       <c r="C11" s="41"/>
       <c r="D11" s="33" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="E11" s="34" t="s">
         <v>70</v>
@@ -1757,7 +1757,7 @@
         <v>45799.0</v>
       </c>
       <c r="H11" s="35" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="I11" s="36"/>
       <c r="J11" s="36">
@@ -1767,7 +1767,7 @@
         <v>974557.12</v>
       </c>
       <c r="L11" s="34" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="M11" s="39">
         <v>974557.12</v>
@@ -1782,7 +1782,7 @@
       <c r="B12" s="23"/>
       <c r="C12" s="41"/>
       <c r="D12" s="33" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="E12" s="34" t="s">
         <v>70</v>
@@ -1790,21 +1790,21 @@
       <c r="F12" s="34">
         <v>660.0</v>
       </c>
-      <c r="G12" s="43">
+      <c r="G12" s="44">
         <v>45856.0</v>
       </c>
-      <c r="H12" s="44" t="s">
+      <c r="H12" s="45" t="s">
         <v>71</v>
       </c>
       <c r="I12" s="36"/>
       <c r="J12" s="36">
         <v>45891.0</v>
       </c>
-      <c r="K12" s="45">
+      <c r="K12" s="46">
         <v>1402001.34</v>
       </c>
-      <c r="L12" s="46" t="s">
-        <v>108</v>
+      <c r="L12" s="47" t="s">
+        <v>114</v>
       </c>
       <c r="M12" s="39">
         <v>1402001.34</v>
@@ -1819,7 +1819,7 @@
       <c r="B13" s="23"/>
       <c r="C13" s="41"/>
       <c r="D13" s="49" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="E13" s="34" t="s">
         <v>70</v>
@@ -1831,17 +1831,17 @@
         <v>45856.0</v>
       </c>
       <c r="H13" s="35" t="s">
-        <v>114</v>
-      </c>
-      <c r="I13" s="43"/>
-      <c r="J13" s="43">
+        <v>121</v>
+      </c>
+      <c r="I13" s="44"/>
+      <c r="J13" s="44">
         <v>45891.0</v>
       </c>
-      <c r="K13" s="45">
+      <c r="K13" s="46">
         <v>1223702.3</v>
       </c>
       <c r="L13" s="34" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="M13" s="39">
         <v>1223702.3</v>
@@ -1856,7 +1856,7 @@
       <c r="B14" s="23"/>
       <c r="C14" s="41"/>
       <c r="D14" s="49" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="E14" s="34" t="s">
         <v>70</v>
@@ -1868,17 +1868,17 @@
         <v>45901.0</v>
       </c>
       <c r="H14" s="34" t="s">
-        <v>123</v>
-      </c>
-      <c r="I14" s="43"/>
-      <c r="J14" s="43">
+        <v>127</v>
+      </c>
+      <c r="I14" s="44"/>
+      <c r="J14" s="44">
         <v>45938.0</v>
       </c>
-      <c r="K14" s="45">
+      <c r="K14" s="46">
         <v>1011677.95</v>
       </c>
       <c r="L14" s="34" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="M14" s="39">
         <v>1011677.95</v>
@@ -1893,7 +1893,7 @@
       <c r="B15" s="23"/>
       <c r="C15" s="41"/>
       <c r="D15" s="49" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="E15" s="34" t="s">
         <v>70</v>
@@ -1907,15 +1907,15 @@
       <c r="H15" s="34" t="s">
         <v>79</v>
       </c>
-      <c r="I15" s="43"/>
-      <c r="J15" s="43">
+      <c r="I15" s="44"/>
+      <c r="J15" s="44">
         <v>45938.0</v>
       </c>
-      <c r="K15" s="45">
+      <c r="K15" s="46">
         <v>896744.06</v>
       </c>
       <c r="L15" s="34" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="M15" s="39">
         <v>896744.06</v>
@@ -1929,7 +1929,7 @@
       <c r="B16" s="23"/>
       <c r="C16" s="41"/>
       <c r="D16" s="49" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="E16" s="34" t="s">
         <v>70</v>
@@ -1941,17 +1941,17 @@
         <v>45957.0</v>
       </c>
       <c r="H16" s="34" t="s">
-        <v>138</v>
-      </c>
-      <c r="I16" s="43"/>
-      <c r="J16" s="43">
+        <v>141</v>
+      </c>
+      <c r="I16" s="44"/>
+      <c r="J16" s="44">
         <v>46003.0</v>
       </c>
-      <c r="K16" s="45">
+      <c r="K16" s="46">
         <v>919329.06</v>
       </c>
       <c r="L16" s="34" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="M16" s="39">
         <v>919329.06</v>
@@ -1965,27 +1965,27 @@
       <c r="B17" s="23"/>
       <c r="C17" s="41"/>
       <c r="D17" s="49" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="E17" s="34"/>
       <c r="F17" s="34">
         <v>705.0</v>
       </c>
-      <c r="G17" s="43">
+      <c r="G17" s="44">
         <v>45972.0</v>
       </c>
       <c r="H17" s="34" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="I17" s="34"/>
-      <c r="J17" s="43">
+      <c r="J17" s="44">
         <v>46016.0</v>
       </c>
-      <c r="K17" s="45">
+      <c r="K17" s="46">
         <v>1157009.26</v>
       </c>
       <c r="L17" s="34" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="M17" s="39">
         <v>1157009.26</v>
@@ -1999,7 +1999,7 @@
       <c r="B18" s="23"/>
       <c r="C18" s="41"/>
       <c r="D18" s="49" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="E18" s="34" t="s">
         <v>70</v>
@@ -2007,21 +2007,21 @@
       <c r="F18" s="34">
         <v>728.0</v>
       </c>
-      <c r="G18" s="43">
+      <c r="G18" s="44">
         <v>46008.0</v>
       </c>
       <c r="H18" s="34" t="s">
         <v>152</v>
       </c>
       <c r="I18" s="34"/>
-      <c r="J18" s="43">
+      <c r="J18" s="44">
         <v>46040.0</v>
       </c>
-      <c r="K18" s="45">
+      <c r="K18" s="46">
         <v>1214597.952</v>
       </c>
       <c r="L18" s="34" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="M18" s="39">
         <v>1214597.952</v>
@@ -2039,7 +2039,7 @@
       <c r="B19" s="23"/>
       <c r="C19" s="41"/>
       <c r="D19" s="49" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="E19" s="34" t="s">
         <v>70</v>
@@ -2047,21 +2047,21 @@
       <c r="F19" s="34">
         <v>278.0</v>
       </c>
-      <c r="G19" s="43">
+      <c r="G19" s="44">
         <v>46042.0</v>
       </c>
       <c r="H19" s="34" t="s">
-        <v>160</v>
-      </c>
-      <c r="I19" s="43"/>
-      <c r="J19" s="43">
+        <v>158</v>
+      </c>
+      <c r="I19" s="44"/>
+      <c r="J19" s="44">
         <v>46074.0</v>
       </c>
-      <c r="K19" s="45">
+      <c r="K19" s="46">
         <v>967082.09</v>
       </c>
       <c r="L19" s="34" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="M19" s="39">
         <v>967082.09</v>
@@ -2085,17 +2085,17 @@
       <c r="F20" s="34">
         <v>10.0</v>
       </c>
-      <c r="G20" s="43">
+      <c r="G20" s="44">
         <v>46078.0</v>
       </c>
       <c r="H20" s="34" t="s">
-        <v>105</v>
-      </c>
-      <c r="I20" s="43"/>
-      <c r="J20" s="43">
+        <v>103</v>
+      </c>
+      <c r="I20" s="44"/>
+      <c r="J20" s="44">
         <v>46106.0</v>
       </c>
-      <c r="K20" s="45">
+      <c r="K20" s="46">
         <v>719561.08</v>
       </c>
       <c r="L20" s="34" t="s">
@@ -2123,17 +2123,17 @@
       <c r="F21" s="34">
         <v>15.0</v>
       </c>
-      <c r="G21" s="43">
+      <c r="G21" s="44">
         <v>46094.0</v>
       </c>
       <c r="H21" s="34" t="s">
         <v>166</v>
       </c>
-      <c r="I21" s="43"/>
-      <c r="J21" s="43">
+      <c r="I21" s="44"/>
+      <c r="J21" s="44">
         <v>46128.0</v>
       </c>
-      <c r="K21" s="45">
+      <c r="K21" s="46">
         <v>885881.08</v>
       </c>
       <c r="L21" s="34" t="s">
@@ -2161,17 +2161,17 @@
       <c r="F22" s="34">
         <v>28.0</v>
       </c>
-      <c r="G22" s="43">
+      <c r="G22" s="44">
         <v>46128.0</v>
       </c>
       <c r="H22" s="34" t="s">
         <v>169</v>
       </c>
-      <c r="I22" s="43"/>
-      <c r="J22" s="43">
+      <c r="I22" s="44"/>
+      <c r="J22" s="44">
         <v>46164.0</v>
       </c>
-      <c r="K22" s="45" t="s">
+      <c r="K22" s="46" t="s">
         <v>170</v>
       </c>
       <c r="L22" s="34" t="s">
@@ -2199,17 +2199,17 @@
       <c r="F23" s="34">
         <v>33.0</v>
       </c>
-      <c r="G23" s="43">
+      <c r="G23" s="44">
         <v>46156.0</v>
       </c>
       <c r="H23" s="34" t="s">
         <v>173</v>
       </c>
-      <c r="I23" s="43"/>
-      <c r="J23" s="43">
+      <c r="I23" s="44"/>
+      <c r="J23" s="44">
         <v>46191.0</v>
       </c>
-      <c r="K23" s="45">
+      <c r="K23" s="46">
         <v>1108954.4358333333</v>
       </c>
       <c r="L23" s="34" t="s">
@@ -2237,17 +2237,17 @@
       <c r="F24" s="34">
         <v>29.0</v>
       </c>
-      <c r="G24" s="43">
+      <c r="G24" s="44">
         <v>46149.0</v>
       </c>
       <c r="H24" s="34" t="s">
         <v>173</v>
       </c>
-      <c r="I24" s="43"/>
-      <c r="J24" s="43">
+      <c r="I24" s="44"/>
+      <c r="J24" s="44">
         <v>46185.0</v>
       </c>
-      <c r="K24" s="45">
+      <c r="K24" s="46">
         <v>218206.1</v>
       </c>
       <c r="L24" s="34" t="s">
@@ -2275,17 +2275,17 @@
       <c r="F25" s="34">
         <v>40.0</v>
       </c>
-      <c r="G25" s="43">
+      <c r="G25" s="44">
         <v>46156.0</v>
       </c>
       <c r="H25" s="34" t="s">
         <v>173</v>
       </c>
-      <c r="I25" s="43"/>
-      <c r="J25" s="43">
+      <c r="I25" s="44"/>
+      <c r="J25" s="44">
         <v>46191.0</v>
       </c>
-      <c r="K25" s="45">
+      <c r="K25" s="46">
         <v>1549250.84</v>
       </c>
       <c r="L25" s="34" t="s">
@@ -2313,17 +2313,17 @@
       <c r="F26" s="34">
         <v>48.0</v>
       </c>
-      <c r="G26" s="43">
+      <c r="G26" s="44">
         <v>46230.0</v>
       </c>
       <c r="H26" s="34" t="s">
         <v>179</v>
       </c>
-      <c r="I26" s="43"/>
-      <c r="J26" s="43">
+      <c r="I26" s="44"/>
+      <c r="J26" s="44">
         <v>46262.0</v>
       </c>
-      <c r="K26" s="45" t="s">
+      <c r="K26" s="46" t="s">
         <v>180</v>
       </c>
       <c r="L26" s="34" t="s">
@@ -2351,17 +2351,17 @@
       <c r="F27" s="34">
         <v>49.0</v>
       </c>
-      <c r="G27" s="43">
+      <c r="G27" s="44">
         <v>46252.0</v>
       </c>
       <c r="H27" s="34" t="s">
-        <v>130</v>
-      </c>
-      <c r="I27" s="43"/>
-      <c r="J27" s="43">
+        <v>128</v>
+      </c>
+      <c r="I27" s="44"/>
+      <c r="J27" s="44">
         <v>46284.0</v>
       </c>
-      <c r="K27" s="45"/>
+      <c r="K27" s="46"/>
       <c r="L27" s="34"/>
       <c r="M27" s="39" t="s">
         <v>183</v>
@@ -2377,35 +2377,35 @@
     <row r="28" ht="30.75" customHeight="1">
       <c r="A28" s="23"/>
       <c r="B28" s="23"/>
-      <c r="C28" s="29" t="s">
+      <c r="C28" s="28" t="s">
         <v>49</v>
       </c>
-      <c r="D28" s="29" t="s">
+      <c r="D28" s="28" t="s">
+        <v>50</v>
+      </c>
+      <c r="E28" s="30" t="s">
+        <v>51</v>
+      </c>
+      <c r="F28" s="30" t="s">
         <v>52</v>
-      </c>
-      <c r="E28" s="30" t="s">
-        <v>54</v>
-      </c>
-      <c r="F28" s="30" t="s">
-        <v>55</v>
       </c>
       <c r="G28" s="30"/>
       <c r="H28" s="30" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="I28" s="30"/>
       <c r="J28" s="30"/>
       <c r="K28" s="30" t="s">
+        <v>60</v>
+      </c>
+      <c r="L28" s="30" t="s">
         <v>62</v>
       </c>
-      <c r="L28" s="30" t="s">
+      <c r="M28" s="30" t="s">
+        <v>63</v>
+      </c>
+      <c r="N28" s="30" t="s">
         <v>64</v>
-      </c>
-      <c r="M28" s="30" t="s">
-        <v>65</v>
-      </c>
-      <c r="N28" s="30" t="s">
-        <v>66</v>
       </c>
       <c r="O28" s="25"/>
       <c r="P28" s="27"/>
@@ -2439,7 +2439,7 @@
         <v>45791.0</v>
       </c>
       <c r="H29" s="35" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="I29" s="36"/>
       <c r="J29" s="36">
@@ -2490,8 +2490,8 @@
       <c r="H30" s="34" t="s">
         <v>187</v>
       </c>
-      <c r="I30" s="43"/>
-      <c r="J30" s="43">
+      <c r="I30" s="44"/>
+      <c r="J30" s="44">
         <v>45955.0</v>
       </c>
       <c r="K30" s="37">
@@ -2537,13 +2537,13 @@
         <v>45853.0</v>
       </c>
       <c r="H31" s="34" t="s">
-        <v>61</v>
-      </c>
-      <c r="I31" s="43"/>
-      <c r="J31" s="43">
+        <v>65</v>
+      </c>
+      <c r="I31" s="44"/>
+      <c r="J31" s="44">
         <v>45939.0</v>
       </c>
-      <c r="K31" s="45">
+      <c r="K31" s="46">
         <v>378307.61</v>
       </c>
       <c r="L31" s="34" t="s">
@@ -2586,10 +2586,10 @@
         <v>45910.0</v>
       </c>
       <c r="H32" s="34" t="s">
-        <v>61</v>
-      </c>
-      <c r="I32" s="43"/>
-      <c r="J32" s="43">
+        <v>65</v>
+      </c>
+      <c r="I32" s="44"/>
+      <c r="J32" s="44">
         <v>45941.0</v>
       </c>
       <c r="K32" s="37">
@@ -2641,7 +2641,7 @@
       <c r="J33" s="64">
         <v>45935.0</v>
       </c>
-      <c r="K33" s="45">
+      <c r="K33" s="46">
         <v>198332.75</v>
       </c>
       <c r="L33" s="34" t="s">
@@ -2684,13 +2684,13 @@
         <v>46008.0</v>
       </c>
       <c r="H34" s="34" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="I34" s="64"/>
       <c r="J34" s="64">
         <v>46066.0</v>
       </c>
-      <c r="K34" s="45">
+      <c r="K34" s="46">
         <v>1528.62</v>
       </c>
       <c r="L34" s="65" t="s">
@@ -2733,13 +2733,13 @@
         <v>45930.0</v>
       </c>
       <c r="H35" s="34" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="I35" s="64"/>
       <c r="J35" s="64">
         <v>45935.0</v>
       </c>
-      <c r="K35" s="45">
+      <c r="K35" s="46">
         <v>38718.58</v>
       </c>
       <c r="L35" s="34" t="s">
@@ -2782,13 +2782,13 @@
         <v>45968.0</v>
       </c>
       <c r="H36" s="34" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="I36" s="64"/>
       <c r="J36" s="64">
         <v>45935.0</v>
       </c>
-      <c r="K36" s="45">
+      <c r="K36" s="46">
         <v>133124.11</v>
       </c>
       <c r="L36" s="34" t="s">
@@ -2831,13 +2831,13 @@
         <v>46043.0</v>
       </c>
       <c r="H37" s="63" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I37" s="68"/>
       <c r="J37" s="67">
         <v>46075.0</v>
       </c>
-      <c r="K37" s="45">
+      <c r="K37" s="46">
         <v>11372.9</v>
       </c>
       <c r="L37" s="34" t="s">
@@ -2878,7 +2878,7 @@
         <v>209</v>
       </c>
       <c r="J38" s="67"/>
-      <c r="K38" s="45"/>
+      <c r="K38" s="46"/>
       <c r="L38" s="34"/>
       <c r="M38" s="39"/>
       <c r="N38" s="51">
@@ -2915,7 +2915,7 @@
         <v>209</v>
       </c>
       <c r="J39" s="67"/>
-      <c r="K39" s="45"/>
+      <c r="K39" s="46"/>
       <c r="L39" s="34"/>
       <c r="M39" s="39"/>
       <c r="N39" s="69">
@@ -2952,8 +2952,8 @@
         <v>209</v>
       </c>
       <c r="J40" s="67"/>
-      <c r="K40" s="45"/>
-      <c r="L40" s="46"/>
+      <c r="K40" s="46"/>
+      <c r="L40" s="47"/>
       <c r="M40" s="39"/>
       <c r="N40" s="70">
         <v>48857.395500000006</v>
@@ -2989,8 +2989,8 @@
         <v>213</v>
       </c>
       <c r="J41" s="67"/>
-      <c r="K41" s="45"/>
-      <c r="L41" s="46"/>
+      <c r="K41" s="46"/>
+      <c r="L41" s="47"/>
       <c r="M41" s="39"/>
       <c r="N41" s="70"/>
       <c r="O41" s="25"/>
@@ -3026,13 +3026,13 @@
         <v>46104.0</v>
       </c>
       <c r="H42" s="63" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I42" s="68"/>
       <c r="J42" s="67">
         <v>46106.0</v>
       </c>
-      <c r="K42" s="45">
+      <c r="K42" s="46">
         <v>27801.11</v>
       </c>
       <c r="L42" s="71" t="s">
@@ -3073,17 +3073,17 @@
         <v>46199.0</v>
       </c>
       <c r="H43" s="63" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I43" s="68"/>
       <c r="J43" s="67">
         <v>46233.0</v>
       </c>
-      <c r="K43" s="45">
+      <c r="K43" s="46">
         <v>58868.35</v>
       </c>
       <c r="L43" s="34" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="M43" s="72">
         <v>58868.35</v>
@@ -8057,40 +8057,40 @@
       <c r="AH2" s="2"/>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="9">
+      <c r="C3" s="10">
         <v>2.5E32</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="D3" s="7" t="s">
         <v>4</v>
       </c>
       <c r="E3" s="12">
         <v>45686.0</v>
       </c>
-      <c r="F3" s="8" t="s">
+      <c r="F3" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G3" s="8">
+      <c r="G3" s="7">
         <v>12.0</v>
       </c>
-      <c r="H3" s="8">
+      <c r="H3" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I3" s="8">
+      <c r="I3" s="7">
         <v>2048.0</v>
       </c>
-      <c r="J3" s="13">
+      <c r="J3" s="14">
         <v>1000.0</v>
       </c>
-      <c r="K3" s="13">
+      <c r="K3" s="14">
         <v>1000.0</v>
       </c>
-      <c r="L3" s="8">
+      <c r="L3" s="7">
         <v>0.0</v>
       </c>
       <c r="AB3" s="2"/>
@@ -8102,40 +8102,40 @@
       <c r="AH3" s="2"/>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="C4" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="D4" s="7" t="s">
         <v>4</v>
       </c>
       <c r="E4" s="12">
         <v>45762.0</v>
       </c>
-      <c r="F4" s="8" t="s">
+      <c r="F4" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G4" s="8">
+      <c r="G4" s="7">
         <v>12.0</v>
       </c>
-      <c r="H4" s="8">
+      <c r="H4" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I4" s="8">
+      <c r="I4" s="7">
         <v>2048.0</v>
       </c>
-      <c r="J4" s="13">
+      <c r="J4" s="14">
         <v>52250.04</v>
       </c>
-      <c r="K4" s="13">
+      <c r="K4" s="14">
         <v>52250.04</v>
       </c>
-      <c r="L4" s="8">
+      <c r="L4" s="7">
         <v>0.0</v>
       </c>
       <c r="AB4" s="2"/>
@@ -8147,40 +8147,40 @@
       <c r="AH4" s="2"/>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="B5" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="C5" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="D5" s="8" t="s">
+      <c r="A5" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="D5" s="7" t="s">
         <v>4</v>
       </c>
       <c r="E5" s="12">
         <v>45762.0</v>
       </c>
-      <c r="F5" s="8" t="s">
+      <c r="F5" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G5" s="8">
+      <c r="G5" s="7">
         <v>12.0</v>
       </c>
-      <c r="H5" s="8">
+      <c r="H5" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I5" s="8">
+      <c r="I5" s="7">
         <v>2048.0</v>
       </c>
-      <c r="J5" s="13">
+      <c r="J5" s="14">
         <v>881914.18</v>
       </c>
-      <c r="K5" s="13">
+      <c r="K5" s="14">
         <v>881914.18</v>
       </c>
-      <c r="L5" s="8">
+      <c r="L5" s="7">
         <v>0.0</v>
       </c>
       <c r="AB5" s="2"/>
@@ -8192,40 +8192,40 @@
       <c r="AH5" s="2"/>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="B6" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="C6" s="8" t="s">
+      <c r="A6" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="C6" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="D6" s="8" t="s">
+      <c r="D6" s="7" t="s">
         <v>4</v>
       </c>
       <c r="E6" s="12">
         <v>45762.0</v>
       </c>
-      <c r="F6" s="8" t="s">
+      <c r="F6" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G6" s="8">
+      <c r="G6" s="7">
         <v>12.0</v>
       </c>
-      <c r="H6" s="8">
+      <c r="H6" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I6" s="8">
+      <c r="I6" s="7">
         <v>2048.0</v>
       </c>
-      <c r="J6" s="13">
+      <c r="J6" s="14">
         <v>750000.0</v>
       </c>
-      <c r="K6" s="13">
+      <c r="K6" s="14">
         <v>750000.0</v>
       </c>
-      <c r="L6" s="8">
+      <c r="L6" s="7">
         <v>0.0</v>
       </c>
       <c r="AB6" s="2"/>
@@ -8237,40 +8237,40 @@
       <c r="AH6" s="2"/>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="B7" s="8" t="s">
+      <c r="A7" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="B7" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="C7" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="D7" s="8" t="s">
+      <c r="D7" s="7" t="s">
         <v>4</v>
       </c>
       <c r="E7" s="12">
         <v>45763.0</v>
       </c>
-      <c r="F7" s="8" t="s">
+      <c r="F7" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G7" s="8">
+      <c r="G7" s="7">
         <v>12.0</v>
       </c>
-      <c r="H7" s="8">
+      <c r="H7" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I7" s="8" t="s">
+      <c r="I7" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="J7" s="13">
+      <c r="J7" s="14">
         <v>949835.78</v>
       </c>
-      <c r="K7" s="13">
+      <c r="K7" s="14">
         <v>949835.78</v>
       </c>
-      <c r="L7" s="8">
+      <c r="L7" s="7">
         <v>0.0</v>
       </c>
       <c r="AB7" s="2"/>
@@ -8282,43 +8282,43 @@
       <c r="AH7" s="2"/>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="s">
+      <c r="A8" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="B8" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="C8" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="D8" s="7" t="s">
         <v>4</v>
       </c>
       <c r="E8" s="12">
         <v>45763.0</v>
       </c>
-      <c r="F8" s="8" t="s">
+      <c r="F8" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G8" s="8">
+      <c r="G8" s="7">
         <v>12.0</v>
       </c>
-      <c r="H8" s="8">
+      <c r="H8" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I8" s="8" t="s">
+      <c r="I8" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="J8" s="13">
+      <c r="J8" s="14">
         <v>524584.95</v>
       </c>
-      <c r="K8" s="13">
+      <c r="K8" s="14">
         <v>524584.95</v>
       </c>
-      <c r="L8" s="8">
+      <c r="L8" s="7">
         <v>0.0</v>
       </c>
-      <c r="O8" s="28"/>
+      <c r="O8" s="29"/>
       <c r="AB8" s="2"/>
       <c r="AC8" s="2"/>
       <c r="AD8" s="2"/>
@@ -8328,40 +8328,40 @@
       <c r="AH8" s="2"/>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="B9" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="C9" s="8" t="s">
+      <c r="A9" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="D9" s="8" t="s">
+      <c r="B9" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="D9" s="7" t="s">
         <v>4</v>
       </c>
       <c r="E9" s="12">
         <v>45792.0</v>
       </c>
-      <c r="F9" s="8" t="s">
+      <c r="F9" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G9" s="8">
+      <c r="G9" s="7">
         <v>12.0</v>
       </c>
-      <c r="H9" s="8">
+      <c r="H9" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I9" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="J9" s="13">
+      <c r="I9" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="J9" s="14">
         <v>211614.23</v>
       </c>
-      <c r="K9" s="13">
+      <c r="K9" s="14">
         <v>211614.23</v>
       </c>
-      <c r="L9" s="8">
+      <c r="L9" s="7">
         <v>0.0</v>
       </c>
       <c r="AB9" s="2"/>
@@ -8373,40 +8373,40 @@
       <c r="AH9" s="2"/>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="s">
-        <v>61</v>
-      </c>
-      <c r="B10" s="8" t="s">
+      <c r="A10" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="B10" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="C10" s="8" t="s">
-        <v>63</v>
-      </c>
-      <c r="D10" s="8" t="s">
+      <c r="C10" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="D10" s="7" t="s">
         <v>4</v>
       </c>
       <c r="E10" s="12">
         <v>45825.0</v>
       </c>
-      <c r="F10" s="8" t="s">
+      <c r="F10" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G10" s="8">
+      <c r="G10" s="7">
         <v>12.0</v>
       </c>
-      <c r="H10" s="8">
+      <c r="H10" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I10" s="8">
+      <c r="I10" s="7">
         <v>2048.0</v>
       </c>
-      <c r="J10" s="13">
+      <c r="J10" s="14">
         <v>2391157.42</v>
       </c>
-      <c r="K10" s="13">
+      <c r="K10" s="14">
         <v>2391157.41</v>
       </c>
-      <c r="L10" s="13">
+      <c r="L10" s="14">
         <v>0.01</v>
       </c>
       <c r="AB10" s="2"/>
@@ -8418,40 +8418,40 @@
       <c r="AH10" s="2"/>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="s">
+      <c r="A11" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="B11" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="C11" s="8" t="s">
+      <c r="B11" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="C11" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="D11" s="8" t="s">
+      <c r="D11" s="7" t="s">
         <v>4</v>
       </c>
       <c r="E11" s="12">
         <v>45825.0</v>
       </c>
-      <c r="F11" s="8" t="s">
+      <c r="F11" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G11" s="8">
+      <c r="G11" s="7">
         <v>12.0</v>
       </c>
-      <c r="H11" s="8">
+      <c r="H11" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I11" s="8">
+      <c r="I11" s="7">
         <v>2048.0</v>
       </c>
-      <c r="J11" s="13">
+      <c r="J11" s="14">
         <v>618154.39</v>
       </c>
-      <c r="K11" s="13">
+      <c r="K11" s="14">
         <v>618154.38</v>
       </c>
-      <c r="L11" s="8">
+      <c r="L11" s="7">
         <v>0.01</v>
       </c>
       <c r="AB11" s="2"/>
@@ -8463,40 +8463,40 @@
       <c r="AH11" s="2"/>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="s">
+      <c r="A12" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="B12" s="8" t="s">
+      <c r="B12" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="C12" s="8" t="s">
+      <c r="C12" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="D12" s="8" t="s">
+      <c r="D12" s="7" t="s">
         <v>4</v>
       </c>
       <c r="E12" s="12">
         <v>45832.0</v>
       </c>
-      <c r="F12" s="8" t="s">
+      <c r="F12" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G12" s="8">
+      <c r="G12" s="7">
         <v>12.0</v>
       </c>
-      <c r="H12" s="8">
+      <c r="H12" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I12" s="8" t="s">
+      <c r="I12" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="J12" s="13">
+      <c r="J12" s="14">
         <v>1600334.09</v>
       </c>
-      <c r="K12" s="13">
+      <c r="K12" s="14">
         <v>1600334.09</v>
       </c>
-      <c r="L12" s="8">
+      <c r="L12" s="7">
         <v>0.0</v>
       </c>
       <c r="AB12" s="2"/>
@@ -8508,40 +8508,40 @@
       <c r="AH12" s="2"/>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="s">
-        <v>76</v>
-      </c>
-      <c r="B13" s="8" t="s">
+      <c r="A13" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="B13" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="C13" s="8" t="s">
+      <c r="C13" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="D13" s="8" t="s">
+      <c r="D13" s="7" t="s">
         <v>4</v>
       </c>
       <c r="E13" s="12">
         <v>45863.0</v>
       </c>
-      <c r="F13" s="8" t="s">
+      <c r="F13" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G13" s="8">
+      <c r="G13" s="7">
         <v>12.0</v>
       </c>
-      <c r="H13" s="8">
+      <c r="H13" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I13" s="8">
+      <c r="I13" s="7">
         <v>2048.0</v>
       </c>
-      <c r="J13" s="13">
+      <c r="J13" s="14">
         <v>2364771.07</v>
       </c>
-      <c r="K13" s="13">
+      <c r="K13" s="14">
         <v>2364771.07</v>
       </c>
-      <c r="L13" s="13">
+      <c r="L13" s="14">
         <v>0.0</v>
       </c>
       <c r="M13" s="38"/>
@@ -8554,40 +8554,40 @@
       <c r="AH13" s="2"/>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="s">
+      <c r="A14" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="B14" s="8" t="s">
+      <c r="B14" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="C14" s="8" t="s">
+      <c r="C14" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="D14" s="8" t="s">
+      <c r="D14" s="7" t="s">
         <v>4</v>
       </c>
       <c r="E14" s="12">
         <v>45887.0</v>
       </c>
-      <c r="F14" s="8" t="s">
+      <c r="F14" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G14" s="8">
+      <c r="G14" s="7">
         <v>12.0</v>
       </c>
-      <c r="H14" s="8">
+      <c r="H14" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I14" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="J14" s="13">
+      <c r="I14" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="J14" s="14">
         <v>968237.39</v>
       </c>
-      <c r="K14" s="13">
+      <c r="K14" s="14">
         <v>968237.39</v>
       </c>
-      <c r="L14" s="8">
+      <c r="L14" s="7">
         <v>0.0</v>
       </c>
       <c r="AB14" s="2"/>
@@ -8599,40 +8599,40 @@
       <c r="AH14" s="2"/>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="s">
+      <c r="A15" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="B15" s="8" t="s">
+      <c r="B15" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="C15" s="8" t="s">
+      <c r="C15" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="D15" s="8" t="s">
+      <c r="D15" s="7" t="s">
         <v>4</v>
       </c>
       <c r="E15" s="12">
         <v>45924.0</v>
       </c>
-      <c r="F15" s="8" t="s">
+      <c r="F15" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G15" s="8">
+      <c r="G15" s="7">
         <v>12.0</v>
       </c>
-      <c r="H15" s="8">
+      <c r="H15" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I15" s="8" t="s">
+      <c r="I15" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="J15" s="13">
+      <c r="J15" s="14">
         <v>1011677.95</v>
       </c>
-      <c r="K15" s="13">
+      <c r="K15" s="14">
         <v>1011677.95</v>
       </c>
-      <c r="L15" s="8">
+      <c r="L15" s="7">
         <v>0.0</v>
       </c>
       <c r="AB15" s="2"/>
@@ -8644,40 +8644,40 @@
       <c r="AH15" s="2"/>
     </row>
     <row r="16">
-      <c r="A16" s="8" t="s">
+      <c r="A16" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="B16" s="8" t="s">
+      <c r="B16" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="C16" s="8" t="s">
-        <v>87</v>
-      </c>
-      <c r="D16" s="8" t="s">
+      <c r="C16" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="D16" s="7" t="s">
         <v>4</v>
       </c>
       <c r="E16" s="12">
         <v>45929.0</v>
       </c>
-      <c r="F16" s="8" t="s">
+      <c r="F16" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G16" s="8">
+      <c r="G16" s="7">
         <v>12.0</v>
       </c>
-      <c r="H16" s="8">
+      <c r="H16" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I16" s="8">
+      <c r="I16" s="7">
         <v>2048.0</v>
       </c>
-      <c r="J16" s="13">
+      <c r="J16" s="14">
         <v>1580293.02</v>
       </c>
-      <c r="K16" s="13">
+      <c r="K16" s="14">
         <v>1580293.02</v>
       </c>
-      <c r="L16" s="13">
+      <c r="L16" s="14">
         <v>0.0</v>
       </c>
       <c r="AB16" s="2"/>
@@ -8689,40 +8689,40 @@
       <c r="AH16" s="2"/>
     </row>
     <row r="17">
-      <c r="A17" s="8" t="s">
+      <c r="A17" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="C17" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="B17" s="8" t="s">
-        <v>90</v>
-      </c>
-      <c r="C17" s="8" t="s">
-        <v>91</v>
-      </c>
-      <c r="D17" s="8" t="s">
+      <c r="D17" s="7" t="s">
         <v>4</v>
       </c>
       <c r="E17" s="12">
         <v>45930.0</v>
       </c>
-      <c r="F17" s="8" t="s">
+      <c r="F17" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G17" s="8">
+      <c r="G17" s="7">
         <v>12.0</v>
       </c>
-      <c r="H17" s="8">
+      <c r="H17" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I17" s="8">
+      <c r="I17" s="7">
         <v>2048.0</v>
       </c>
-      <c r="J17" s="13">
+      <c r="J17" s="14">
         <v>34065.36</v>
       </c>
-      <c r="K17" s="8">
+      <c r="K17" s="7">
         <v>0.0</v>
       </c>
-      <c r="L17" s="13">
+      <c r="L17" s="14">
         <v>34065.36</v>
       </c>
       <c r="AB17" s="2"/>
@@ -8734,40 +8734,40 @@
       <c r="AH17" s="2"/>
     </row>
     <row r="18">
-      <c r="A18" s="8" t="s">
-        <v>93</v>
-      </c>
-      <c r="B18" s="8" t="s">
+      <c r="A18" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="B18" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="C18" s="8" t="s">
-        <v>94</v>
-      </c>
-      <c r="D18" s="8" t="s">
+      <c r="C18" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="D18" s="7" t="s">
         <v>4</v>
       </c>
       <c r="E18" s="12">
         <v>45938.0</v>
       </c>
-      <c r="F18" s="8" t="s">
+      <c r="F18" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G18" s="8">
+      <c r="G18" s="7">
         <v>12.0</v>
       </c>
-      <c r="H18" s="8">
+      <c r="H18" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I18" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="J18" s="13">
+      <c r="I18" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="J18" s="14">
         <v>63746.85</v>
       </c>
-      <c r="K18" s="13">
+      <c r="K18" s="14">
         <v>63746.85</v>
       </c>
-      <c r="L18" s="8">
+      <c r="L18" s="7">
         <v>0.0</v>
       </c>
       <c r="AB18" s="2"/>
@@ -8779,40 +8779,40 @@
       <c r="AH18" s="2"/>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="s">
-        <v>97</v>
-      </c>
-      <c r="B19" s="8" t="s">
+      <c r="A19" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="B19" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="C19" s="8" t="s">
-        <v>98</v>
-      </c>
-      <c r="D19" s="8" t="s">
+      <c r="C19" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="D19" s="7" t="s">
         <v>4</v>
       </c>
       <c r="E19" s="12">
         <v>45938.0</v>
       </c>
-      <c r="F19" s="8" t="s">
+      <c r="F19" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G19" s="8">
+      <c r="G19" s="7">
         <v>12.0</v>
       </c>
-      <c r="H19" s="8">
+      <c r="H19" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I19" s="8" t="s">
+      <c r="I19" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="J19" s="13">
+      <c r="J19" s="14">
         <v>947931.1</v>
       </c>
-      <c r="K19" s="13">
+      <c r="K19" s="14">
         <v>947931.1</v>
       </c>
-      <c r="L19" s="8">
+      <c r="L19" s="7">
         <v>0.0</v>
       </c>
       <c r="AB19" s="2"/>
@@ -8824,40 +8824,40 @@
       <c r="AH19" s="2"/>
     </row>
     <row r="20">
-      <c r="A20" s="8" t="s">
-        <v>100</v>
-      </c>
-      <c r="B20" s="8" t="s">
+      <c r="A20" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="B20" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="C20" s="8" t="s">
-        <v>101</v>
-      </c>
-      <c r="D20" s="8" t="s">
+      <c r="C20" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="D20" s="7" t="s">
         <v>4</v>
       </c>
       <c r="E20" s="12">
         <v>45938.0</v>
       </c>
-      <c r="F20" s="8" t="s">
+      <c r="F20" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G20" s="8">
+      <c r="G20" s="7">
         <v>12.0</v>
       </c>
-      <c r="H20" s="8">
+      <c r="H20" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I20" s="8">
+      <c r="I20" s="7">
         <v>2048.0</v>
       </c>
-      <c r="J20" s="13">
+      <c r="J20" s="14">
         <v>259790.57</v>
       </c>
-      <c r="K20" s="13">
+      <c r="K20" s="14">
         <v>259790.57</v>
       </c>
-      <c r="L20" s="8">
+      <c r="L20" s="7">
         <v>0.0</v>
       </c>
       <c r="AB20" s="2"/>
@@ -8869,40 +8869,40 @@
       <c r="AH20" s="2"/>
     </row>
     <row r="21">
-      <c r="A21" s="8" t="s">
-        <v>103</v>
-      </c>
-      <c r="B21" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="C21" s="8" t="s">
-        <v>104</v>
-      </c>
-      <c r="D21" s="8" t="s">
+      <c r="A21" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="B21" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="C21" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="D21" s="7" t="s">
         <v>4</v>
       </c>
       <c r="E21" s="12">
         <v>45938.0</v>
       </c>
-      <c r="F21" s="8" t="s">
+      <c r="F21" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G21" s="8">
+      <c r="G21" s="7">
         <v>12.0</v>
       </c>
-      <c r="H21" s="8">
+      <c r="H21" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I21" s="8">
+      <c r="I21" s="7">
         <v>2048.0</v>
       </c>
-      <c r="J21" s="13">
+      <c r="J21" s="14">
         <v>170479.3</v>
       </c>
-      <c r="K21" s="13">
+      <c r="K21" s="14">
         <v>170479.3</v>
       </c>
-      <c r="L21" s="8">
+      <c r="L21" s="7">
         <v>0.0</v>
       </c>
       <c r="AB21" s="2"/>
@@ -8914,40 +8914,40 @@
       <c r="AH21" s="2"/>
     </row>
     <row r="22">
-      <c r="A22" s="8" t="s">
+      <c r="A22" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="B22" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="C22" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="B22" s="8" t="s">
-        <v>106</v>
-      </c>
-      <c r="C22" s="8" t="s">
-        <v>107</v>
-      </c>
-      <c r="D22" s="8" t="s">
+      <c r="D22" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="E22" s="47">
+      <c r="E22" s="43">
         <v>45953.0</v>
       </c>
-      <c r="F22" s="8" t="s">
+      <c r="F22" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G22" s="8">
+      <c r="G22" s="7">
         <v>12.0</v>
       </c>
-      <c r="H22" s="8">
+      <c r="H22" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I22" s="8">
+      <c r="I22" s="7">
         <v>2000.0</v>
       </c>
-      <c r="J22" s="13">
+      <c r="J22" s="14">
         <v>1500000.0</v>
       </c>
-      <c r="K22" s="13">
+      <c r="K22" s="14">
         <v>1500000.0</v>
       </c>
-      <c r="L22" s="13">
+      <c r="L22" s="14">
         <v>0.0</v>
       </c>
       <c r="AB22" s="2"/>
@@ -8959,40 +8959,40 @@
       <c r="AH22" s="2"/>
     </row>
     <row r="23">
-      <c r="A23" s="8" t="s">
+      <c r="A23" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="B23" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="B23" s="8" t="s">
+      <c r="C23" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="C23" s="8" t="s">
+      <c r="D23" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="E23" s="43">
+        <v>45953.0</v>
+      </c>
+      <c r="F23" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="G23" s="7">
+        <v>12.0</v>
+      </c>
+      <c r="H23" s="7">
+        <v>339039.0</v>
+      </c>
+      <c r="I23" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="D23" s="8" t="s">
-        <v>4</v>
-      </c>
-      <c r="E23" s="47">
-        <v>45953.0</v>
-      </c>
-      <c r="F23" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="G23" s="8">
-        <v>12.0</v>
-      </c>
-      <c r="H23" s="8">
-        <v>339039.0</v>
-      </c>
-      <c r="I23" s="8" t="s">
-        <v>113</v>
-      </c>
-      <c r="J23" s="13">
+      <c r="J23" s="14">
         <v>1000001.64</v>
       </c>
-      <c r="K23" s="13">
+      <c r="K23" s="14">
         <v>1000001.64</v>
       </c>
-      <c r="L23" s="8">
+      <c r="L23" s="7">
         <v>0.0</v>
       </c>
       <c r="AB23" s="2"/>
@@ -9004,40 +9004,40 @@
       <c r="AH23" s="2"/>
     </row>
     <row r="24">
-      <c r="A24" s="8" t="s">
-        <v>115</v>
-      </c>
-      <c r="B24" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="C24" s="8" t="s">
-        <v>116</v>
-      </c>
-      <c r="D24" s="8" t="s">
+      <c r="A24" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="B24" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="C24" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="D24" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="E24" s="47">
+      <c r="E24" s="43">
         <v>45953.0</v>
       </c>
-      <c r="F24" s="8" t="s">
+      <c r="F24" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G24" s="8">
+      <c r="G24" s="7">
         <v>12.0</v>
       </c>
-      <c r="H24" s="8">
+      <c r="H24" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I24" s="8">
+      <c r="I24" s="7">
         <v>2048.0</v>
       </c>
-      <c r="J24" s="13">
+      <c r="J24" s="14">
         <v>68405.66</v>
       </c>
-      <c r="K24" s="13">
+      <c r="K24" s="14">
         <v>68405.66</v>
       </c>
-      <c r="L24" s="8">
+      <c r="L24" s="7">
         <v>0.0</v>
       </c>
       <c r="AB24" s="2"/>
@@ -9049,40 +9049,40 @@
       <c r="AH24" s="2"/>
     </row>
     <row r="25">
-      <c r="A25" s="8" t="s">
-        <v>118</v>
-      </c>
-      <c r="B25" s="8" t="s">
-        <v>119</v>
-      </c>
-      <c r="C25" s="8" t="s">
-        <v>120</v>
-      </c>
-      <c r="D25" s="8" t="s">
+      <c r="A25" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="B25" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="C25" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="D25" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="E25" s="47">
+      <c r="E25" s="43">
         <v>45975.0</v>
       </c>
-      <c r="F25" s="8" t="s">
+      <c r="F25" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G25" s="8">
+      <c r="G25" s="7">
         <v>12.0</v>
       </c>
-      <c r="H25" s="8">
+      <c r="H25" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I25" s="8" t="s">
-        <v>113</v>
-      </c>
-      <c r="J25" s="13">
+      <c r="I25" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="J25" s="14">
         <v>1157673.06</v>
       </c>
-      <c r="K25" s="13">
+      <c r="K25" s="14">
         <v>1157673.06</v>
       </c>
-      <c r="L25" s="8">
+      <c r="L25" s="7">
         <v>0.0</v>
       </c>
       <c r="AB25" s="2"/>
@@ -9094,40 +9094,40 @@
       <c r="AH25" s="2"/>
     </row>
     <row r="26">
-      <c r="A26" s="8" t="s">
-        <v>122</v>
-      </c>
-      <c r="B26" s="8" t="s">
+      <c r="A26" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="B26" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="C26" s="8" t="s">
-        <v>124</v>
-      </c>
-      <c r="D26" s="8" t="s">
+      <c r="C26" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="D26" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="E26" s="47">
+      <c r="E26" s="43">
         <v>45989.0</v>
       </c>
-      <c r="F26" s="8" t="s">
+      <c r="F26" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G26" s="8">
+      <c r="G26" s="7">
         <v>12.0</v>
       </c>
-      <c r="H26" s="8">
+      <c r="H26" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I26" s="8">
+      <c r="I26" s="7">
         <v>2048.0</v>
       </c>
-      <c r="J26" s="13">
+      <c r="J26" s="14">
         <v>34065.36</v>
       </c>
-      <c r="K26" s="13">
+      <c r="K26" s="14">
         <v>34065.36</v>
       </c>
-      <c r="L26" s="8">
+      <c r="L26" s="7">
         <v>0.0</v>
       </c>
       <c r="AB26" s="2"/>
@@ -9139,40 +9139,40 @@
       <c r="AH26" s="2"/>
     </row>
     <row r="27">
-      <c r="A27" s="8" t="s">
-        <v>126</v>
-      </c>
-      <c r="B27" s="8" t="s">
-        <v>127</v>
-      </c>
-      <c r="C27" s="8" t="s">
-        <v>128</v>
-      </c>
-      <c r="D27" s="8" t="s">
+      <c r="A27" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="B27" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="C27" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="D27" s="7" t="s">
         <v>4</v>
       </c>
       <c r="E27" s="12">
         <v>46104.0</v>
       </c>
-      <c r="F27" s="8" t="s">
+      <c r="F27" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G27" s="8">
+      <c r="G27" s="7">
         <v>12.0</v>
       </c>
-      <c r="H27" s="8">
+      <c r="H27" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I27" s="8">
+      <c r="I27" s="7">
         <v>2048.0</v>
       </c>
-      <c r="J27" s="13">
+      <c r="J27" s="14">
         <v>1770880.5</v>
       </c>
-      <c r="K27" s="13">
+      <c r="K27" s="14">
         <v>843261.89</v>
       </c>
-      <c r="L27" s="13">
+      <c r="L27" s="14">
         <v>927618.61</v>
       </c>
       <c r="AB27" s="2"/>
@@ -9184,40 +9184,40 @@
       <c r="AH27" s="2"/>
     </row>
     <row r="28">
-      <c r="A28" s="8" t="s">
+      <c r="A28" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="B28" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="C28" s="7" t="s">
         <v>130</v>
       </c>
-      <c r="B28" s="8" t="s">
-        <v>131</v>
-      </c>
-      <c r="C28" s="8" t="s">
-        <v>132</v>
-      </c>
-      <c r="D28" s="8" t="s">
+      <c r="D28" s="7" t="s">
         <v>4</v>
       </c>
       <c r="E28" s="12">
         <v>46120.0</v>
       </c>
-      <c r="F28" s="8" t="s">
+      <c r="F28" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G28" s="8">
+      <c r="G28" s="7">
         <v>12.0</v>
       </c>
-      <c r="H28" s="8">
+      <c r="H28" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I28" s="8" t="s">
+      <c r="I28" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="J28" s="13">
+      <c r="J28" s="14">
         <v>1912292.52</v>
       </c>
-      <c r="K28" s="13">
+      <c r="K28" s="14">
         <v>1629834.48</v>
       </c>
-      <c r="L28" s="13">
+      <c r="L28" s="14">
         <v>282458.04</v>
       </c>
       <c r="AB28" s="2"/>
@@ -9229,40 +9229,40 @@
       <c r="AH28" s="2"/>
     </row>
     <row r="29">
-      <c r="A29" s="8" t="s">
+      <c r="A29" s="7" t="s">
+        <v>133</v>
+      </c>
+      <c r="B29" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="C29" s="7" t="s">
         <v>135</v>
       </c>
-      <c r="B29" s="8" t="s">
-        <v>136</v>
-      </c>
-      <c r="C29" s="8" t="s">
-        <v>137</v>
-      </c>
-      <c r="D29" s="8" t="s">
+      <c r="D29" s="7" t="s">
         <v>4</v>
       </c>
       <c r="E29" s="12">
         <v>46196.0</v>
       </c>
-      <c r="F29" s="8" t="s">
+      <c r="F29" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G29" s="8">
+      <c r="G29" s="7">
         <v>12.0</v>
       </c>
-      <c r="H29" s="8">
+      <c r="H29" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I29" s="8">
+      <c r="I29" s="7">
         <v>2048.0</v>
       </c>
-      <c r="J29" s="13">
+      <c r="J29" s="14">
         <v>1496713.48</v>
       </c>
-      <c r="K29" s="8">
+      <c r="K29" s="7">
         <v>0.0</v>
       </c>
-      <c r="L29" s="13">
+      <c r="L29" s="14">
         <v>1496713.48</v>
       </c>
       <c r="AB29" s="2"/>
@@ -9274,40 +9274,40 @@
       <c r="AH29" s="2"/>
     </row>
     <row r="30">
-      <c r="A30" s="8" t="s">
-        <v>140</v>
-      </c>
-      <c r="B30" s="8" t="s">
-        <v>141</v>
-      </c>
-      <c r="C30" s="8" t="s">
-        <v>143</v>
-      </c>
-      <c r="D30" s="8" t="s">
+      <c r="A30" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="B30" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="C30" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="D30" s="7" t="s">
         <v>4</v>
       </c>
       <c r="E30" s="12">
         <v>46205.0</v>
       </c>
-      <c r="F30" s="8" t="s">
+      <c r="F30" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G30" s="8">
+      <c r="G30" s="7">
         <v>12.0</v>
       </c>
-      <c r="H30" s="8">
+      <c r="H30" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I30" s="8" t="s">
+      <c r="I30" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="J30" s="13">
+      <c r="J30" s="14">
         <v>624166.14</v>
       </c>
-      <c r="K30" s="8">
+      <c r="K30" s="7">
         <v>0.0</v>
       </c>
-      <c r="L30" s="13">
+      <c r="L30" s="14">
         <v>624166.14</v>
       </c>
       <c r="AB30" s="2"/>
@@ -9319,40 +9319,40 @@
       <c r="AH30" s="2"/>
     </row>
     <row r="31">
-      <c r="A31" s="8" t="s">
-        <v>146</v>
-      </c>
-      <c r="B31" s="8" t="s">
-        <v>147</v>
-      </c>
-      <c r="C31" s="8" t="s">
-        <v>148</v>
-      </c>
-      <c r="D31" s="8" t="s">
+      <c r="A31" s="7" t="s">
+        <v>142</v>
+      </c>
+      <c r="B31" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="C31" s="7" t="s">
+        <v>144</v>
+      </c>
+      <c r="D31" s="7" t="s">
         <v>4</v>
       </c>
       <c r="E31" s="12">
         <v>46205.0</v>
       </c>
-      <c r="F31" s="8" t="s">
+      <c r="F31" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G31" s="8">
+      <c r="G31" s="7">
         <v>12.0</v>
       </c>
-      <c r="H31" s="8">
+      <c r="H31" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I31" s="8" t="s">
-        <v>113</v>
-      </c>
-      <c r="J31" s="13">
+      <c r="I31" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="J31" s="14">
         <v>18462.36</v>
       </c>
-      <c r="K31" s="8">
+      <c r="K31" s="7">
         <v>0.0</v>
       </c>
-      <c r="L31" s="13">
+      <c r="L31" s="14">
         <v>18462.36</v>
       </c>
       <c r="AB31" s="2"/>
@@ -9364,40 +9364,40 @@
       <c r="AH31" s="2"/>
     </row>
     <row r="32">
-      <c r="A32" s="8" t="s">
+      <c r="A32" s="7" t="s">
+        <v>149</v>
+      </c>
+      <c r="B32" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="C32" s="14" t="s">
         <v>150</v>
       </c>
-      <c r="B32" s="8" t="s">
-        <v>147</v>
-      </c>
-      <c r="C32" s="13" t="s">
-        <v>151</v>
-      </c>
-      <c r="D32" s="8" t="s">
+      <c r="D32" s="7" t="s">
         <v>4</v>
       </c>
       <c r="E32" s="12">
         <v>46213.0</v>
       </c>
-      <c r="F32" s="8" t="s">
+      <c r="F32" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G32" s="8">
+      <c r="G32" s="7">
         <v>12.0</v>
       </c>
-      <c r="H32" s="8">
+      <c r="H32" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I32" s="8" t="s">
-        <v>113</v>
-      </c>
-      <c r="J32" s="13">
+      <c r="I32" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="J32" s="14">
         <v>1530656.62</v>
       </c>
-      <c r="K32" s="8">
+      <c r="K32" s="7">
         <v>0.0</v>
       </c>
-      <c r="L32" s="13">
+      <c r="L32" s="14">
         <v>1530656.62</v>
       </c>
       <c r="AB32" s="2"/>
@@ -9409,40 +9409,40 @@
       <c r="AH32" s="2"/>
     </row>
     <row r="33">
-      <c r="A33" s="8" t="s">
-        <v>153</v>
-      </c>
-      <c r="B33" s="8" t="s">
-        <v>136</v>
-      </c>
-      <c r="C33" s="13" t="s">
+      <c r="A33" s="7" t="s">
+        <v>154</v>
+      </c>
+      <c r="B33" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="C33" s="14" t="s">
         <v>155</v>
       </c>
-      <c r="D33" s="8" t="s">
+      <c r="D33" s="7" t="s">
         <v>4</v>
       </c>
       <c r="E33" s="12">
         <v>46227.0</v>
       </c>
-      <c r="F33" s="8" t="s">
+      <c r="F33" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G33" s="8">
+      <c r="G33" s="7">
         <v>12.0</v>
       </c>
-      <c r="H33" s="8">
+      <c r="H33" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I33" s="8">
+      <c r="I33" s="7">
         <v>2048.0</v>
       </c>
-      <c r="J33" s="13">
+      <c r="J33" s="14">
         <v>173846.38</v>
       </c>
-      <c r="K33" s="8">
+      <c r="K33" s="7">
         <v>0.0</v>
       </c>
-      <c r="L33" s="13">
+      <c r="L33" s="14">
         <v>173846.38</v>
       </c>
       <c r="AB33" s="2"/>
@@ -9454,40 +9454,40 @@
       <c r="AH33" s="2"/>
     </row>
     <row r="34">
-      <c r="A34" s="8" t="s">
-        <v>156</v>
-      </c>
-      <c r="B34" s="8" t="s">
-        <v>158</v>
-      </c>
-      <c r="C34" s="8" t="s">
+      <c r="A34" s="7" t="s">
+        <v>157</v>
+      </c>
+      <c r="B34" s="7" t="s">
         <v>159</v>
       </c>
-      <c r="D34" s="8" t="s">
+      <c r="C34" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="D34" s="7" t="s">
         <v>4</v>
       </c>
       <c r="E34" s="12">
         <v>46240.0</v>
       </c>
-      <c r="F34" s="8" t="s">
+      <c r="F34" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G34" s="8">
+      <c r="G34" s="7">
         <v>12.0</v>
       </c>
-      <c r="H34" s="8">
+      <c r="H34" s="7">
         <v>339039.0</v>
       </c>
-      <c r="I34" s="8" t="s">
-        <v>161</v>
-      </c>
-      <c r="J34" s="13">
+      <c r="I34" s="7" t="s">
+        <v>162</v>
+      </c>
+      <c r="J34" s="14">
         <v>236343.68</v>
       </c>
-      <c r="K34" s="8">
+      <c r="K34" s="7">
         <v>0.0</v>
       </c>
-      <c r="L34" s="13">
+      <c r="L34" s="14">
         <v>236343.68</v>
       </c>
       <c r="AB34" s="2"/>

</xml_diff>